<commit_message>
chore(data): batch update intraday meta_faturamento - 08:01:00
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1276"/>
+  <dimension ref="A1:C1278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11289,10 +11289,10 @@
         <v>46266</v>
       </c>
       <c r="B987" t="n">
-        <v>2830</v>
+        <v>2824</v>
       </c>
       <c r="C987" t="n">
-        <v>32720</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="988">
@@ -11300,10 +11300,10 @@
         <v>46266</v>
       </c>
       <c r="B988" t="n">
-        <v>816</v>
+        <v>2787</v>
       </c>
       <c r="C988" t="n">
-        <v>97400</v>
+        <v>59090</v>
       </c>
     </row>
     <row r="989">
@@ -11311,10 +11311,10 @@
         <v>46266</v>
       </c>
       <c r="B989" t="n">
-        <v>2671</v>
+        <v>2830</v>
       </c>
       <c r="C989" t="n">
-        <v>29088</v>
+        <v>40900</v>
       </c>
     </row>
     <row r="990">
@@ -11322,10 +11322,10 @@
         <v>46266</v>
       </c>
       <c r="B990" t="n">
-        <v>2705</v>
+        <v>816</v>
       </c>
       <c r="C990" t="n">
-        <v>65160</v>
+        <v>121750</v>
       </c>
     </row>
     <row r="991">
@@ -11333,10 +11333,10 @@
         <v>46266</v>
       </c>
       <c r="B991" t="n">
-        <v>2333</v>
+        <v>2671</v>
       </c>
       <c r="C991" t="n">
-        <v>56128</v>
+        <v>36360</v>
       </c>
     </row>
     <row r="992">
@@ -11344,10 +11344,10 @@
         <v>46266</v>
       </c>
       <c r="B992" t="n">
-        <v>2440</v>
+        <v>2705</v>
       </c>
       <c r="C992" t="n">
-        <v>32720</v>
+        <v>81450</v>
       </c>
     </row>
     <row r="993">
@@ -11355,10 +11355,10 @@
         <v>46266</v>
       </c>
       <c r="B993" t="n">
-        <v>2448</v>
+        <v>2333</v>
       </c>
       <c r="C993" t="n">
-        <v>7272</v>
+        <v>70160</v>
       </c>
     </row>
     <row r="994">
@@ -11366,10 +11366,10 @@
         <v>46266</v>
       </c>
       <c r="B994" t="n">
-        <v>2310</v>
+        <v>2440</v>
       </c>
       <c r="C994" t="n">
-        <v>24976</v>
+        <v>40900</v>
       </c>
     </row>
     <row r="995">
@@ -11377,10 +11377,10 @@
         <v>46266</v>
       </c>
       <c r="B995" t="n">
-        <v>2809</v>
+        <v>2448</v>
       </c>
       <c r="C995" t="n">
-        <v>24976</v>
+        <v>9090</v>
       </c>
     </row>
     <row r="996">
@@ -11388,10 +11388,10 @@
         <v>46266</v>
       </c>
       <c r="B996" t="n">
-        <v>2548</v>
+        <v>2310</v>
       </c>
       <c r="C996" t="n">
-        <v>21280</v>
+        <v>31220</v>
       </c>
     </row>
     <row r="997">
@@ -11399,10 +11399,10 @@
         <v>46266</v>
       </c>
       <c r="B997" t="n">
-        <v>451</v>
+        <v>2809</v>
       </c>
       <c r="C997" t="n">
-        <v>87272</v>
+        <v>31220</v>
       </c>
     </row>
     <row r="998">
@@ -11410,10 +11410,10 @@
         <v>46266</v>
       </c>
       <c r="B998" t="n">
-        <v>933</v>
+        <v>2548</v>
       </c>
       <c r="C998" t="n">
-        <v>29632</v>
+        <v>26600</v>
       </c>
     </row>
     <row r="999">
@@ -11421,10 +11421,10 @@
         <v>46266</v>
       </c>
       <c r="B999" t="n">
-        <v>2702</v>
+        <v>451</v>
       </c>
       <c r="C999" t="n">
-        <v>29632</v>
+        <v>109090</v>
       </c>
     </row>
     <row r="1000">
@@ -11432,10 +11432,10 @@
         <v>46266</v>
       </c>
       <c r="B1000" t="n">
-        <v>2549</v>
+        <v>933</v>
       </c>
       <c r="C1000" t="n">
-        <v>10304</v>
+        <v>37040</v>
       </c>
     </row>
     <row r="1001">
@@ -11443,10 +11443,10 @@
         <v>46266</v>
       </c>
       <c r="B1001" t="n">
-        <v>535</v>
+        <v>2702</v>
       </c>
       <c r="C1001" t="n">
-        <v>134544</v>
+        <v>37040</v>
       </c>
     </row>
     <row r="1002">
@@ -11454,10 +11454,10 @@
         <v>46266</v>
       </c>
       <c r="B1002" t="n">
-        <v>1117</v>
+        <v>2549</v>
       </c>
       <c r="C1002" t="n">
-        <v>126504</v>
+        <v>12880</v>
       </c>
     </row>
     <row r="1003">
@@ -11465,10 +11465,10 @@
         <v>46266</v>
       </c>
       <c r="B1003" t="n">
-        <v>530</v>
+        <v>535</v>
       </c>
       <c r="C1003" t="n">
-        <v>88752</v>
+        <v>168180</v>
       </c>
     </row>
     <row r="1004">
@@ -11476,10 +11476,10 @@
         <v>46266</v>
       </c>
       <c r="B1004" t="n">
-        <v>358</v>
+        <v>1117</v>
       </c>
       <c r="C1004" t="n">
-        <v>123632</v>
+        <v>158130</v>
       </c>
     </row>
     <row r="1005">
@@ -11487,10 +11487,10 @@
         <v>46266</v>
       </c>
       <c r="B1005" t="n">
-        <v>2498</v>
+        <v>530</v>
       </c>
       <c r="C1005" t="n">
-        <v>20192</v>
+        <v>110940</v>
       </c>
     </row>
     <row r="1006">
@@ -11498,10 +11498,10 @@
         <v>46266</v>
       </c>
       <c r="B1006" t="n">
-        <v>2381</v>
+        <v>358</v>
       </c>
       <c r="C1006" t="n">
-        <v>28848</v>
+        <v>154540</v>
       </c>
     </row>
     <row r="1007">
@@ -11509,10 +11509,10 @@
         <v>46266</v>
       </c>
       <c r="B1007" t="n">
-        <v>2695</v>
+        <v>2498</v>
       </c>
       <c r="C1007" t="n">
-        <v>17352</v>
+        <v>25240</v>
       </c>
     </row>
     <row r="1008">
@@ -11520,10 +11520,10 @@
         <v>46266</v>
       </c>
       <c r="B1008" t="n">
-        <v>2744</v>
+        <v>2381</v>
       </c>
       <c r="C1008" t="n">
-        <v>21816</v>
+        <v>36060</v>
       </c>
     </row>
     <row r="1009">
@@ -11531,10 +11531,10 @@
         <v>46266</v>
       </c>
       <c r="B1009" t="n">
-        <v>2750</v>
+        <v>2695</v>
       </c>
       <c r="C1009" t="n">
-        <v>21816</v>
+        <v>21690</v>
       </c>
     </row>
     <row r="1010">
@@ -11542,10 +11542,10 @@
         <v>46266</v>
       </c>
       <c r="B1010" t="n">
-        <v>2131</v>
+        <v>2744</v>
       </c>
       <c r="C1010" t="n">
-        <v>43632</v>
+        <v>27272.76</v>
       </c>
     </row>
     <row r="1011">
@@ -11553,10 +11553,10 @@
         <v>46266</v>
       </c>
       <c r="B1011" t="n">
-        <v>818</v>
+        <v>2750</v>
       </c>
       <c r="C1011" t="n">
-        <v>145448</v>
+        <v>27270</v>
       </c>
     </row>
     <row r="1012">
@@ -11564,10 +11564,10 @@
         <v>46266</v>
       </c>
       <c r="B1012" t="n">
-        <v>2566</v>
+        <v>2131</v>
       </c>
       <c r="C1012" t="n">
-        <v>29088</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1013">
@@ -11575,10 +11575,10 @@
         <v>46266</v>
       </c>
       <c r="B1013" t="n">
-        <v>132</v>
+        <v>818</v>
       </c>
       <c r="C1013" t="n">
-        <v>272720</v>
+        <v>181810</v>
       </c>
     </row>
     <row r="1014">
@@ -11586,10 +11586,10 @@
         <v>46266</v>
       </c>
       <c r="B1014" t="n">
-        <v>2431</v>
+        <v>2566</v>
       </c>
       <c r="C1014" t="n">
-        <v>66904</v>
+        <v>36360</v>
       </c>
     </row>
     <row r="1015">
@@ -11597,10 +11597,10 @@
         <v>46266</v>
       </c>
       <c r="B1015" t="n">
-        <v>2249</v>
+        <v>132</v>
       </c>
       <c r="C1015" t="n">
-        <v>71024</v>
+        <v>340900</v>
       </c>
     </row>
     <row r="1016">
@@ -11608,10 +11608,10 @@
         <v>46266</v>
       </c>
       <c r="B1016" t="n">
-        <v>1585</v>
+        <v>2431</v>
       </c>
       <c r="C1016" t="n">
-        <v>60016</v>
+        <v>83630</v>
       </c>
     </row>
     <row r="1017">
@@ -11619,10 +11619,10 @@
         <v>46266</v>
       </c>
       <c r="B1017" t="n">
-        <v>2325</v>
+        <v>2249</v>
       </c>
       <c r="C1017" t="n">
-        <v>58016</v>
+        <v>88780</v>
       </c>
     </row>
     <row r="1018">
@@ -11630,10 +11630,10 @@
         <v>46266</v>
       </c>
       <c r="B1018" t="n">
-        <v>2190</v>
+        <v>1585</v>
       </c>
       <c r="C1018" t="n">
-        <v>81816</v>
+        <v>75020</v>
       </c>
     </row>
     <row r="1019">
@@ -11641,10 +11641,10 @@
         <v>46266</v>
       </c>
       <c r="B1019" t="n">
-        <v>1466</v>
+        <v>2325</v>
       </c>
       <c r="C1019" t="n">
-        <v>147272</v>
+        <v>72520</v>
       </c>
     </row>
     <row r="1020">
@@ -11652,10 +11652,10 @@
         <v>46266</v>
       </c>
       <c r="B1020" t="n">
-        <v>2659</v>
+        <v>2190</v>
       </c>
       <c r="C1020" t="n">
-        <v>44728</v>
+        <v>102270</v>
       </c>
     </row>
     <row r="1021">
@@ -11663,10 +11663,10 @@
         <v>46266</v>
       </c>
       <c r="B1021" t="n">
-        <v>1064</v>
+        <v>1466</v>
       </c>
       <c r="C1021" t="n">
-        <v>217952</v>
+        <v>184090</v>
       </c>
     </row>
     <row r="1022">
@@ -11674,10 +11674,10 @@
         <v>46266</v>
       </c>
       <c r="B1022" t="n">
-        <v>2308</v>
+        <v>2659</v>
       </c>
       <c r="C1022" t="n">
-        <v>74544</v>
+        <v>55910</v>
       </c>
     </row>
     <row r="1023">
@@ -11685,10 +11685,10 @@
         <v>46266</v>
       </c>
       <c r="B1023" t="n">
-        <v>1137</v>
+        <v>619</v>
       </c>
       <c r="C1023" t="n">
-        <v>232720</v>
+        <v>140560</v>
       </c>
     </row>
     <row r="1024">
@@ -11696,10 +11696,10 @@
         <v>46266</v>
       </c>
       <c r="B1024" t="n">
-        <v>2747</v>
+        <v>1299</v>
       </c>
       <c r="C1024" t="n">
-        <v>21816</v>
+        <v>236520</v>
       </c>
     </row>
     <row r="1025">
@@ -11707,10 +11707,10 @@
         <v>46266</v>
       </c>
       <c r="B1025" t="n">
-        <v>2819</v>
+        <v>1064</v>
       </c>
       <c r="C1025" t="n">
-        <v>21816</v>
+        <v>272440</v>
       </c>
     </row>
     <row r="1026">
@@ -11718,10 +11718,10 @@
         <v>46266</v>
       </c>
       <c r="B1026" t="n">
-        <v>1259</v>
+        <v>2308</v>
       </c>
       <c r="C1026" t="n">
-        <v>36360</v>
+        <v>93180</v>
       </c>
     </row>
     <row r="1027">
@@ -11729,10 +11729,10 @@
         <v>46266</v>
       </c>
       <c r="B1027" t="n">
-        <v>2544</v>
+        <v>1137</v>
       </c>
       <c r="C1027" t="n">
-        <v>29088</v>
+        <v>290900</v>
       </c>
     </row>
     <row r="1028">
@@ -11740,10 +11740,10 @@
         <v>46266</v>
       </c>
       <c r="B1028" t="n">
-        <v>2261</v>
+        <v>2747</v>
       </c>
       <c r="C1028" t="n">
-        <v>54544</v>
+        <v>27272.76</v>
       </c>
     </row>
     <row r="1029">
@@ -11751,10 +11751,10 @@
         <v>46266</v>
       </c>
       <c r="B1029" t="n">
-        <v>2729</v>
+        <v>2819</v>
       </c>
       <c r="C1029" t="n">
-        <v>29088</v>
+        <v>27272.76</v>
       </c>
     </row>
     <row r="1030">
@@ -11762,10 +11762,10 @@
         <v>46266</v>
       </c>
       <c r="B1030" t="n">
-        <v>2649</v>
+        <v>1259</v>
       </c>
       <c r="C1030" t="n">
-        <v>10736</v>
+        <v>45454.6</v>
       </c>
     </row>
     <row r="1031">
@@ -11773,10 +11773,10 @@
         <v>46266</v>
       </c>
       <c r="B1031" t="n">
-        <v>2494</v>
+        <v>2544</v>
       </c>
       <c r="C1031" t="n">
-        <v>47272</v>
+        <v>36360</v>
       </c>
     </row>
     <row r="1032">
@@ -11784,10 +11784,10 @@
         <v>46266</v>
       </c>
       <c r="B1032" t="n">
-        <v>1384</v>
+        <v>2261</v>
       </c>
       <c r="C1032" t="n">
-        <v>163632</v>
+        <v>68180</v>
       </c>
     </row>
     <row r="1033">
@@ -11795,10 +11795,10 @@
         <v>46266</v>
       </c>
       <c r="B1033" t="n">
-        <v>634</v>
+        <v>2729</v>
       </c>
       <c r="C1033" t="n">
-        <v>200000</v>
+        <v>36360</v>
       </c>
     </row>
     <row r="1034">
@@ -11806,10 +11806,10 @@
         <v>46266</v>
       </c>
       <c r="B1034" t="n">
-        <v>2804</v>
+        <v>2649</v>
       </c>
       <c r="C1034" t="n">
-        <v>36360</v>
+        <v>13420</v>
       </c>
     </row>
     <row r="1035">
@@ -11817,10 +11817,10 @@
         <v>46266</v>
       </c>
       <c r="B1035" t="n">
-        <v>2375</v>
+        <v>2494</v>
       </c>
       <c r="C1035" t="n">
-        <v>120000</v>
+        <v>59090</v>
       </c>
     </row>
     <row r="1036">
@@ -11828,10 +11828,10 @@
         <v>46266</v>
       </c>
       <c r="B1036" t="n">
-        <v>2601</v>
+        <v>1384</v>
       </c>
       <c r="C1036" t="n">
-        <v>100000</v>
+        <v>204540</v>
       </c>
     </row>
     <row r="1037">
@@ -11839,10 +11839,10 @@
         <v>46266</v>
       </c>
       <c r="B1037" t="n">
-        <v>952</v>
+        <v>634</v>
       </c>
       <c r="C1037" t="n">
-        <v>36360</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="1038">
@@ -11850,10 +11850,10 @@
         <v>46266</v>
       </c>
       <c r="B1038" t="n">
-        <v>571</v>
+        <v>2804</v>
       </c>
       <c r="C1038" t="n">
-        <v>231448</v>
+        <v>45450</v>
       </c>
     </row>
     <row r="1039">
@@ -11861,10 +11861,10 @@
         <v>46266</v>
       </c>
       <c r="B1039" t="n">
-        <v>1380</v>
+        <v>2375</v>
       </c>
       <c r="C1039" t="n">
-        <v>36360</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="1040">
@@ -11872,10 +11872,10 @@
         <v>46266</v>
       </c>
       <c r="B1040" t="n">
-        <v>1105</v>
+        <v>2601</v>
       </c>
       <c r="C1040" t="n">
-        <v>36360</v>
+        <v>125000</v>
       </c>
     </row>
     <row r="1041">
@@ -11883,10 +11883,10 @@
         <v>46266</v>
       </c>
       <c r="B1041" t="n">
-        <v>2789</v>
+        <v>952</v>
       </c>
       <c r="C1041" t="n">
-        <v>61816</v>
+        <v>45450</v>
       </c>
     </row>
     <row r="1042">
@@ -11894,10 +11894,10 @@
         <v>46266</v>
       </c>
       <c r="B1042" t="n">
-        <v>2822</v>
+        <v>571</v>
       </c>
       <c r="C1042" t="n">
-        <v>49088</v>
+        <v>289310</v>
       </c>
     </row>
     <row r="1043">
@@ -11905,10 +11905,10 @@
         <v>46266</v>
       </c>
       <c r="B1043" t="n">
-        <v>2728</v>
+        <v>1380</v>
       </c>
       <c r="C1043" t="n">
-        <v>3632</v>
+        <v>45450</v>
       </c>
     </row>
     <row r="1044">
@@ -11916,10 +11916,10 @@
         <v>46266</v>
       </c>
       <c r="B1044" t="n">
-        <v>2488</v>
+        <v>1105</v>
       </c>
       <c r="C1044" t="n">
-        <v>36360</v>
+        <v>45450</v>
       </c>
     </row>
     <row r="1045">
@@ -11927,10 +11927,10 @@
         <v>46266</v>
       </c>
       <c r="B1045" t="n">
-        <v>2069</v>
+        <v>2789</v>
       </c>
       <c r="C1045" t="n">
-        <v>65448</v>
+        <v>77270</v>
       </c>
     </row>
     <row r="1046">
@@ -11938,10 +11938,10 @@
         <v>46266</v>
       </c>
       <c r="B1046" t="n">
-        <v>2082</v>
+        <v>2822</v>
       </c>
       <c r="C1046" t="n">
-        <v>60568</v>
+        <v>61360</v>
       </c>
     </row>
     <row r="1047">
@@ -11949,10 +11949,10 @@
         <v>46266</v>
       </c>
       <c r="B1047" t="n">
-        <v>781</v>
+        <v>2728</v>
       </c>
       <c r="C1047" t="n">
-        <v>47272</v>
+        <v>4540</v>
       </c>
     </row>
     <row r="1048">
@@ -11960,10 +11960,10 @@
         <v>46266</v>
       </c>
       <c r="B1048" t="n">
-        <v>744</v>
+        <v>2488</v>
       </c>
       <c r="C1048" t="n">
-        <v>15128</v>
+        <v>45450</v>
       </c>
     </row>
     <row r="1049">
@@ -11971,10 +11971,10 @@
         <v>46266</v>
       </c>
       <c r="B1049" t="n">
-        <v>2223</v>
+        <v>2069</v>
       </c>
       <c r="C1049" t="n">
-        <v>47976</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1050">
@@ -11982,10 +11982,10 @@
         <v>46266</v>
       </c>
       <c r="B1050" t="n">
-        <v>2452</v>
+        <v>2082</v>
       </c>
       <c r="C1050" t="n">
-        <v>25448</v>
+        <v>75710</v>
       </c>
     </row>
     <row r="1051">
@@ -11993,10 +11993,10 @@
         <v>46266</v>
       </c>
       <c r="B1051" t="n">
-        <v>970</v>
+        <v>781</v>
       </c>
       <c r="C1051" t="n">
-        <v>24976</v>
+        <v>59090</v>
       </c>
     </row>
     <row r="1052">
@@ -12004,10 +12004,10 @@
         <v>46266</v>
       </c>
       <c r="B1052" t="n">
-        <v>2550</v>
+        <v>744</v>
       </c>
       <c r="C1052" t="n">
-        <v>22176</v>
+        <v>18910</v>
       </c>
     </row>
     <row r="1053">
@@ -12015,10 +12015,10 @@
         <v>46266</v>
       </c>
       <c r="B1053" t="n">
-        <v>768</v>
+        <v>2223</v>
       </c>
       <c r="C1053" t="n">
-        <v>47272</v>
+        <v>59970</v>
       </c>
     </row>
     <row r="1054">
@@ -12026,10 +12026,10 @@
         <v>46266</v>
       </c>
       <c r="B1054" t="n">
-        <v>1075</v>
+        <v>2452</v>
       </c>
       <c r="C1054" t="n">
-        <v>164720</v>
+        <v>31810</v>
       </c>
     </row>
     <row r="1055">
@@ -12037,10 +12037,10 @@
         <v>46266</v>
       </c>
       <c r="B1055" t="n">
-        <v>664</v>
+        <v>970</v>
       </c>
       <c r="C1055" t="n">
-        <v>94176</v>
+        <v>31220</v>
       </c>
     </row>
     <row r="1056">
@@ -12048,10 +12048,10 @@
         <v>46266</v>
       </c>
       <c r="B1056" t="n">
-        <v>2555</v>
+        <v>2550</v>
       </c>
       <c r="C1056" t="n">
-        <v>15096</v>
+        <v>27720</v>
       </c>
     </row>
     <row r="1057">
@@ -12059,10 +12059,10 @@
         <v>46266</v>
       </c>
       <c r="B1057" t="n">
-        <v>2627</v>
+        <v>768</v>
       </c>
       <c r="C1057" t="n">
-        <v>8864</v>
+        <v>59090</v>
       </c>
     </row>
     <row r="1058">
@@ -12070,10 +12070,10 @@
         <v>46266</v>
       </c>
       <c r="B1058" t="n">
-        <v>2557</v>
+        <v>1075</v>
       </c>
       <c r="C1058" t="n">
-        <v>9376</v>
+        <v>205900</v>
       </c>
     </row>
     <row r="1059">
@@ -12081,10 +12081,10 @@
         <v>46266</v>
       </c>
       <c r="B1059" t="n">
-        <v>2551</v>
+        <v>664</v>
       </c>
       <c r="C1059" t="n">
-        <v>7448</v>
+        <v>117720</v>
       </c>
     </row>
     <row r="1060">
@@ -12092,10 +12092,10 @@
         <v>46266</v>
       </c>
       <c r="B1060" t="n">
-        <v>2463</v>
+        <v>2555</v>
       </c>
       <c r="C1060" t="n">
-        <v>116440</v>
+        <v>18870</v>
       </c>
     </row>
     <row r="1061">
@@ -12103,10 +12103,10 @@
         <v>46266</v>
       </c>
       <c r="B1061" t="n">
-        <v>2279</v>
+        <v>2627</v>
       </c>
       <c r="C1061" t="n">
-        <v>87848</v>
+        <v>11080</v>
       </c>
     </row>
     <row r="1062">
@@ -12114,10 +12114,10 @@
         <v>46266</v>
       </c>
       <c r="B1062" t="n">
-        <v>631</v>
+        <v>2557</v>
       </c>
       <c r="C1062" t="n">
-        <v>127272</v>
+        <v>11720</v>
       </c>
     </row>
     <row r="1063">
@@ -12125,10 +12125,10 @@
         <v>46266</v>
       </c>
       <c r="B1063" t="n">
-        <v>2251</v>
+        <v>2551</v>
       </c>
       <c r="C1063" t="n">
-        <v>77936</v>
+        <v>9310</v>
       </c>
     </row>
     <row r="1064">
@@ -12136,10 +12136,10 @@
         <v>46266</v>
       </c>
       <c r="B1064" t="n">
-        <v>1653</v>
+        <v>2463</v>
       </c>
       <c r="C1064" t="n">
-        <v>118176</v>
+        <v>145550</v>
       </c>
     </row>
     <row r="1065">
@@ -12147,10 +12147,10 @@
         <v>46266</v>
       </c>
       <c r="B1065" t="n">
-        <v>1293</v>
+        <v>2279</v>
       </c>
       <c r="C1065" t="n">
-        <v>150904</v>
+        <v>109810</v>
       </c>
     </row>
     <row r="1066">
@@ -12158,10 +12158,10 @@
         <v>46266</v>
       </c>
       <c r="B1066" t="n">
-        <v>360</v>
+        <v>631</v>
       </c>
       <c r="C1066" t="n">
-        <v>181816</v>
+        <v>159090</v>
       </c>
     </row>
     <row r="1067">
@@ -12169,10 +12169,10 @@
         <v>46266</v>
       </c>
       <c r="B1067" t="n">
-        <v>1063</v>
+        <v>2251</v>
       </c>
       <c r="C1067" t="n">
-        <v>132200</v>
+        <v>97420</v>
       </c>
     </row>
     <row r="1068">
@@ -12180,10 +12180,10 @@
         <v>46266</v>
       </c>
       <c r="B1068" t="n">
-        <v>2273</v>
+        <v>1653</v>
       </c>
       <c r="C1068" t="n">
-        <v>77120</v>
+        <v>147720</v>
       </c>
     </row>
     <row r="1069">
@@ -12191,10 +12191,10 @@
         <v>46266</v>
       </c>
       <c r="B1069" t="n">
-        <v>2757</v>
+        <v>1293</v>
       </c>
       <c r="C1069" t="n">
-        <v>25448</v>
+        <v>188630</v>
       </c>
     </row>
     <row r="1070">
@@ -12202,10 +12202,10 @@
         <v>46266</v>
       </c>
       <c r="B1070" t="n">
-        <v>2795</v>
+        <v>360</v>
       </c>
       <c r="C1070" t="n">
-        <v>21816</v>
+        <v>227270</v>
       </c>
     </row>
     <row r="1071">
@@ -12213,10 +12213,10 @@
         <v>46266</v>
       </c>
       <c r="B1071" t="n">
-        <v>2722</v>
+        <v>1063</v>
       </c>
       <c r="C1071" t="n">
-        <v>21816</v>
+        <v>165250</v>
       </c>
     </row>
     <row r="1072">
@@ -12224,10 +12224,10 @@
         <v>46266</v>
       </c>
       <c r="B1072" t="n">
-        <v>2718</v>
+        <v>2273</v>
       </c>
       <c r="C1072" t="n">
-        <v>29088</v>
+        <v>96400</v>
       </c>
     </row>
     <row r="1073">
@@ -12235,10 +12235,10 @@
         <v>46266</v>
       </c>
       <c r="B1073" t="n">
-        <v>595</v>
+        <v>2757</v>
       </c>
       <c r="C1073" t="n">
-        <v>200000</v>
+        <v>31818.28</v>
       </c>
     </row>
     <row r="1074">
@@ -12246,10 +12246,10 @@
         <v>46266</v>
       </c>
       <c r="B1074" t="n">
-        <v>890</v>
+        <v>2795</v>
       </c>
       <c r="C1074" t="n">
-        <v>254544</v>
+        <v>27272.76</v>
       </c>
     </row>
     <row r="1075">
@@ -12257,10 +12257,10 @@
         <v>46266</v>
       </c>
       <c r="B1075" t="n">
-        <v>2652</v>
+        <v>2722</v>
       </c>
       <c r="C1075" t="n">
-        <v>47272</v>
+        <v>27270</v>
       </c>
     </row>
     <row r="1076">
@@ -12268,10 +12268,10 @@
         <v>46266</v>
       </c>
       <c r="B1076" t="n">
-        <v>2714</v>
+        <v>2718</v>
       </c>
       <c r="C1076" t="n">
-        <v>130904</v>
+        <v>36360</v>
       </c>
     </row>
     <row r="1077">
@@ -12279,10 +12279,10 @@
         <v>46266</v>
       </c>
       <c r="B1077" t="n">
-        <v>1869</v>
+        <v>595</v>
       </c>
       <c r="C1077" t="n">
-        <v>83632</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="1078">
@@ -12290,10 +12290,10 @@
         <v>46266</v>
       </c>
       <c r="B1078" t="n">
-        <v>400</v>
+        <v>890</v>
       </c>
       <c r="C1078" t="n">
-        <v>69088</v>
+        <v>318180</v>
       </c>
     </row>
     <row r="1079">
@@ -12301,10 +12301,10 @@
         <v>46266</v>
       </c>
       <c r="B1079" t="n">
-        <v>1907</v>
+        <v>2652</v>
       </c>
       <c r="C1079" t="n">
-        <v>134904</v>
+        <v>59090</v>
       </c>
     </row>
     <row r="1080">
@@ -12312,10 +12312,10 @@
         <v>46266</v>
       </c>
       <c r="B1080" t="n">
-        <v>1996</v>
+        <v>2714</v>
       </c>
       <c r="C1080" t="n">
-        <v>85272</v>
+        <v>163630</v>
       </c>
     </row>
     <row r="1081">
@@ -12323,10 +12323,10 @@
         <v>46266</v>
       </c>
       <c r="B1081" t="n">
-        <v>947</v>
+        <v>1869</v>
       </c>
       <c r="C1081" t="n">
-        <v>158008</v>
+        <v>104540</v>
       </c>
     </row>
     <row r="1082">
@@ -12334,10 +12334,10 @@
         <v>46266</v>
       </c>
       <c r="B1082" t="n">
-        <v>1956</v>
+        <v>400</v>
       </c>
       <c r="C1082" t="n">
-        <v>91808</v>
+        <v>86360</v>
       </c>
     </row>
     <row r="1083">
@@ -12345,10 +12345,10 @@
         <v>46266</v>
       </c>
       <c r="B1083" t="n">
-        <v>2824</v>
+        <v>1907</v>
       </c>
       <c r="C1083" t="n">
-        <v>40000</v>
+        <v>168630</v>
       </c>
     </row>
     <row r="1084">
@@ -12356,10 +12356,10 @@
         <v>46266</v>
       </c>
       <c r="B1084" t="n">
-        <v>2787</v>
+        <v>1996</v>
       </c>
       <c r="C1084" t="n">
-        <v>47272</v>
+        <v>106590</v>
       </c>
     </row>
     <row r="1085">
@@ -12367,10 +12367,10 @@
         <v>46266</v>
       </c>
       <c r="B1085" t="n">
-        <v>2510</v>
+        <v>947</v>
       </c>
       <c r="C1085" t="n">
-        <v>201904</v>
+        <v>197510</v>
       </c>
     </row>
     <row r="1086">
@@ -12378,10 +12378,10 @@
         <v>46266</v>
       </c>
       <c r="B1086" t="n">
-        <v>2392</v>
+        <v>1956</v>
       </c>
       <c r="C1086" t="n">
-        <v>60568</v>
+        <v>114760</v>
       </c>
     </row>
     <row r="1087">
@@ -12389,10 +12389,10 @@
         <v>46266</v>
       </c>
       <c r="B1087" t="n">
-        <v>415</v>
+        <v>2178</v>
       </c>
       <c r="C1087" t="n">
-        <v>207088</v>
+        <v>127270</v>
       </c>
     </row>
     <row r="1088">
@@ -12400,10 +12400,10 @@
         <v>46266</v>
       </c>
       <c r="B1088" t="n">
-        <v>1289</v>
+        <v>2827</v>
       </c>
       <c r="C1088" t="n">
-        <v>90904</v>
+        <v>45450</v>
       </c>
     </row>
     <row r="1089">
@@ -12411,10 +12411,10 @@
         <v>46266</v>
       </c>
       <c r="B1089" t="n">
-        <v>2801</v>
+        <v>2510</v>
       </c>
       <c r="C1089" t="n">
-        <v>29088</v>
+        <v>252380</v>
       </c>
     </row>
     <row r="1090">
@@ -12422,10 +12422,10 @@
         <v>46266</v>
       </c>
       <c r="B1090" t="n">
-        <v>2810</v>
+        <v>2392</v>
       </c>
       <c r="C1090" t="n">
-        <v>49088</v>
+        <v>75710</v>
       </c>
     </row>
     <row r="1091">
@@ -12433,10 +12433,10 @@
         <v>46266</v>
       </c>
       <c r="B1091" t="n">
-        <v>767</v>
+        <v>415</v>
       </c>
       <c r="C1091" t="n">
-        <v>65448</v>
+        <v>258860</v>
       </c>
     </row>
     <row r="1092">
@@ -12444,10 +12444,10 @@
         <v>46266</v>
       </c>
       <c r="B1092" t="n">
-        <v>2687</v>
+        <v>1289</v>
       </c>
       <c r="C1092" t="n">
-        <v>36360</v>
+        <v>113630</v>
       </c>
     </row>
     <row r="1093">
@@ -12455,10 +12455,10 @@
         <v>46266</v>
       </c>
       <c r="B1093" t="n">
-        <v>2686</v>
+        <v>2801</v>
       </c>
       <c r="C1093" t="n">
-        <v>47272</v>
+        <v>36360</v>
       </c>
     </row>
     <row r="1094">
@@ -12466,10 +12466,10 @@
         <v>46266</v>
       </c>
       <c r="B1094" t="n">
-        <v>2730</v>
+        <v>2810</v>
       </c>
       <c r="C1094" t="n">
-        <v>32720</v>
+        <v>61360</v>
       </c>
     </row>
     <row r="1095">
@@ -12477,10 +12477,10 @@
         <v>46266</v>
       </c>
       <c r="B1095" t="n">
-        <v>1642</v>
+        <v>767</v>
       </c>
       <c r="C1095" t="n">
-        <v>96360</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1096">
@@ -12488,10 +12488,10 @@
         <v>46266</v>
       </c>
       <c r="B1096" t="n">
-        <v>2613</v>
+        <v>2687</v>
       </c>
       <c r="C1096" t="n">
-        <v>65160</v>
+        <v>45450</v>
       </c>
     </row>
     <row r="1097">
@@ -12499,10 +12499,10 @@
         <v>46266</v>
       </c>
       <c r="B1097" t="n">
-        <v>1020</v>
+        <v>2686</v>
       </c>
       <c r="C1097" t="n">
-        <v>32720</v>
+        <v>59090</v>
       </c>
     </row>
     <row r="1098">
@@ -12510,10 +12510,10 @@
         <v>46266</v>
       </c>
       <c r="B1098" t="n">
-        <v>2785</v>
+        <v>2730</v>
       </c>
       <c r="C1098" t="n">
-        <v>15128</v>
+        <v>40900</v>
       </c>
     </row>
     <row r="1099">
@@ -12521,10 +12521,10 @@
         <v>46266</v>
       </c>
       <c r="B1099" t="n">
-        <v>1327</v>
+        <v>1642</v>
       </c>
       <c r="C1099" t="n">
-        <v>21816</v>
+        <v>120450</v>
       </c>
     </row>
     <row r="1100">
@@ -12532,10 +12532,10 @@
         <v>46266</v>
       </c>
       <c r="B1100" t="n">
-        <v>2629</v>
+        <v>2613</v>
       </c>
       <c r="C1100" t="n">
-        <v>24976</v>
+        <v>81450</v>
       </c>
     </row>
     <row r="1101">
@@ -12543,10 +12543,10 @@
         <v>46266</v>
       </c>
       <c r="B1101" t="n">
-        <v>951</v>
+        <v>1020</v>
       </c>
       <c r="C1101" t="n">
-        <v>41816</v>
+        <v>40900</v>
       </c>
     </row>
     <row r="1102">
@@ -12554,10 +12554,10 @@
         <v>46266</v>
       </c>
       <c r="B1102" t="n">
-        <v>2449</v>
+        <v>2785</v>
       </c>
       <c r="C1102" t="n">
-        <v>14544</v>
+        <v>18910</v>
       </c>
     </row>
     <row r="1103">
@@ -12565,10 +12565,10 @@
         <v>46266</v>
       </c>
       <c r="B1103" t="n">
-        <v>610</v>
+        <v>1327</v>
       </c>
       <c r="C1103" t="n">
-        <v>296360</v>
+        <v>27270</v>
       </c>
     </row>
     <row r="1104">
@@ -12576,10 +12576,10 @@
         <v>46266</v>
       </c>
       <c r="B1104" t="n">
-        <v>2761</v>
+        <v>2629</v>
       </c>
       <c r="C1104" t="n">
-        <v>29632</v>
+        <v>31220</v>
       </c>
     </row>
     <row r="1105">
@@ -12587,10 +12587,10 @@
         <v>46266</v>
       </c>
       <c r="B1105" t="n">
-        <v>483</v>
+        <v>951</v>
       </c>
       <c r="C1105" t="n">
-        <v>161088</v>
+        <v>52270</v>
       </c>
     </row>
     <row r="1106">
@@ -12598,10 +12598,10 @@
         <v>46266</v>
       </c>
       <c r="B1106" t="n">
-        <v>2015</v>
+        <v>2449</v>
       </c>
       <c r="C1106" t="n">
-        <v>134544</v>
+        <v>18180</v>
       </c>
     </row>
     <row r="1107">
@@ -12609,10 +12609,10 @@
         <v>46266</v>
       </c>
       <c r="B1107" t="n">
-        <v>1478</v>
+        <v>610</v>
       </c>
       <c r="C1107" t="n">
-        <v>196784</v>
+        <v>370450</v>
       </c>
     </row>
     <row r="1108">
@@ -12620,10 +12620,10 @@
         <v>46266</v>
       </c>
       <c r="B1108" t="n">
-        <v>424</v>
+        <v>2761</v>
       </c>
       <c r="C1108" t="n">
-        <v>87848</v>
+        <v>37040</v>
       </c>
     </row>
     <row r="1109">
@@ -12631,10 +12631,10 @@
         <v>46266</v>
       </c>
       <c r="B1109" t="n">
-        <v>477</v>
+        <v>483</v>
       </c>
       <c r="C1109" t="n">
-        <v>94056</v>
+        <v>201360</v>
       </c>
     </row>
     <row r="1110">
@@ -12642,10 +12642,10 @@
         <v>46266</v>
       </c>
       <c r="B1110" t="n">
-        <v>1810</v>
+        <v>2015</v>
       </c>
       <c r="C1110" t="n">
-        <v>14568</v>
+        <v>168180</v>
       </c>
     </row>
     <row r="1111">
@@ -12653,10 +12653,10 @@
         <v>46266</v>
       </c>
       <c r="B1111" t="n">
-        <v>2826</v>
+        <v>1478</v>
       </c>
       <c r="C1111" t="n">
-        <v>25448</v>
+        <v>245980</v>
       </c>
     </row>
     <row r="1112">
@@ -12664,10 +12664,10 @@
         <v>46266</v>
       </c>
       <c r="B1112" t="n">
-        <v>2561</v>
+        <v>424</v>
       </c>
       <c r="C1112" t="n">
-        <v>5344</v>
+        <v>109810</v>
       </c>
     </row>
     <row r="1113">
@@ -12675,10 +12675,10 @@
         <v>46266</v>
       </c>
       <c r="B1113" t="n">
-        <v>2653</v>
+        <v>477</v>
       </c>
       <c r="C1113" t="n">
-        <v>21816</v>
+        <v>117570</v>
       </c>
     </row>
     <row r="1114">
@@ -12686,10 +12686,10 @@
         <v>46266</v>
       </c>
       <c r="B1114" t="n">
-        <v>2829</v>
+        <v>1810</v>
       </c>
       <c r="C1114" t="n">
-        <v>21816</v>
+        <v>18210</v>
       </c>
     </row>
     <row r="1115">
@@ -12697,10 +12697,10 @@
         <v>46266</v>
       </c>
       <c r="B1115" t="n">
-        <v>2643</v>
+        <v>2826</v>
       </c>
       <c r="C1115" t="n">
-        <v>10736</v>
+        <v>31818.28</v>
       </c>
     </row>
     <row r="1116">
@@ -12708,10 +12708,10 @@
         <v>46266</v>
       </c>
       <c r="B1116" t="n">
-        <v>2794</v>
+        <v>2561</v>
       </c>
       <c r="C1116" t="n">
-        <v>32720</v>
+        <v>6680</v>
       </c>
     </row>
     <row r="1117">
@@ -12719,10 +12719,10 @@
         <v>46266</v>
       </c>
       <c r="B1117" t="n">
-        <v>2655</v>
+        <v>2653</v>
       </c>
       <c r="C1117" t="n">
-        <v>40000</v>
+        <v>27272.76</v>
       </c>
     </row>
     <row r="1118">
@@ -12730,10 +12730,10 @@
         <v>46266</v>
       </c>
       <c r="B1118" t="n">
-        <v>1456</v>
+        <v>2829</v>
       </c>
       <c r="C1118" t="n">
-        <v>280104</v>
+        <v>27272.76</v>
       </c>
     </row>
     <row r="1119">
@@ -12741,10 +12741,10 @@
         <v>46266</v>
       </c>
       <c r="B1119" t="n">
-        <v>2606</v>
+        <v>2643</v>
       </c>
       <c r="C1119" t="n">
-        <v>86032</v>
+        <v>13420</v>
       </c>
     </row>
     <row r="1120">
@@ -12752,10 +12752,10 @@
         <v>46266</v>
       </c>
       <c r="B1120" t="n">
-        <v>1142</v>
+        <v>2794</v>
       </c>
       <c r="C1120" t="n">
-        <v>156016</v>
+        <v>40900</v>
       </c>
     </row>
     <row r="1121">
@@ -12763,10 +12763,10 @@
         <v>46266</v>
       </c>
       <c r="B1121" t="n">
-        <v>1450</v>
+        <v>2655</v>
       </c>
       <c r="C1121" t="n">
-        <v>99112</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="1122">
@@ -12774,10 +12774,10 @@
         <v>46266</v>
       </c>
       <c r="B1122" t="n">
-        <v>2133</v>
+        <v>1456</v>
       </c>
       <c r="C1122" t="n">
-        <v>231448</v>
+        <v>350130</v>
       </c>
     </row>
     <row r="1123">
@@ -12785,10 +12785,10 @@
         <v>46266</v>
       </c>
       <c r="B1123" t="n">
-        <v>522</v>
+        <v>2606</v>
       </c>
       <c r="C1123" t="n">
-        <v>70904</v>
+        <v>107540</v>
       </c>
     </row>
     <row r="1124">
@@ -12796,10 +12796,10 @@
         <v>46266</v>
       </c>
       <c r="B1124" t="n">
-        <v>2692</v>
+        <v>1142</v>
       </c>
       <c r="C1124" t="n">
-        <v>36360</v>
+        <v>195020</v>
       </c>
     </row>
     <row r="1125">
@@ -12807,10 +12807,10 @@
         <v>46266</v>
       </c>
       <c r="B1125" t="n">
-        <v>2691</v>
+        <v>1450</v>
       </c>
       <c r="C1125" t="n">
-        <v>43632</v>
+        <v>123890</v>
       </c>
     </row>
     <row r="1126">
@@ -12818,10 +12818,10 @@
         <v>46266</v>
       </c>
       <c r="B1126" t="n">
-        <v>1632</v>
+        <v>2133</v>
       </c>
       <c r="C1126" t="n">
-        <v>90904</v>
+        <v>289310</v>
       </c>
     </row>
     <row r="1127">
@@ -12829,10 +12829,10 @@
         <v>46266</v>
       </c>
       <c r="B1127" t="n">
-        <v>2641</v>
+        <v>522</v>
       </c>
       <c r="C1127" t="n">
-        <v>29088</v>
+        <v>88630</v>
       </c>
     </row>
     <row r="1128">
@@ -12840,10 +12840,10 @@
         <v>46266</v>
       </c>
       <c r="B1128" t="n">
-        <v>2197</v>
+        <v>2692</v>
       </c>
       <c r="C1128" t="n">
-        <v>72720</v>
+        <v>45450</v>
       </c>
     </row>
     <row r="1129">
@@ -12851,10 +12851,10 @@
         <v>46266</v>
       </c>
       <c r="B1129" t="n">
-        <v>609</v>
+        <v>2691</v>
       </c>
       <c r="C1129" t="n">
-        <v>80000</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1130">
@@ -12862,10 +12862,10 @@
         <v>46266</v>
       </c>
       <c r="B1130" t="n">
-        <v>104</v>
+        <v>1632</v>
       </c>
       <c r="C1130" t="n">
-        <v>109088</v>
+        <v>113630</v>
       </c>
     </row>
     <row r="1131">
@@ -12873,10 +12873,10 @@
         <v>46266</v>
       </c>
       <c r="B1131" t="n">
-        <v>2621</v>
+        <v>2641</v>
       </c>
       <c r="C1131" t="n">
-        <v>25448</v>
+        <v>36360</v>
       </c>
     </row>
     <row r="1132">
@@ -12884,10 +12884,10 @@
         <v>46266</v>
       </c>
       <c r="B1132" t="n">
-        <v>2786</v>
+        <v>2197</v>
       </c>
       <c r="C1132" t="n">
-        <v>25448</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1133">
@@ -12895,10 +12895,10 @@
         <v>46266</v>
       </c>
       <c r="B1133" t="n">
-        <v>2784</v>
+        <v>609</v>
       </c>
       <c r="C1133" t="n">
-        <v>15128</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1134">
@@ -12906,10 +12906,10 @@
         <v>46266</v>
       </c>
       <c r="B1134" t="n">
-        <v>2586</v>
+        <v>104</v>
       </c>
       <c r="C1134" t="n">
-        <v>15128</v>
+        <v>136360</v>
       </c>
     </row>
     <row r="1135">
@@ -12917,10 +12917,10 @@
         <v>46266</v>
       </c>
       <c r="B1135" t="n">
-        <v>2145</v>
+        <v>2621</v>
       </c>
       <c r="C1135" t="n">
-        <v>47072</v>
+        <v>31810</v>
       </c>
     </row>
     <row r="1136">
@@ -12928,10 +12928,10 @@
         <v>46266</v>
       </c>
       <c r="B1136" t="n">
-        <v>2574</v>
+        <v>2786</v>
       </c>
       <c r="C1136" t="n">
-        <v>47072</v>
+        <v>31810</v>
       </c>
     </row>
     <row r="1137">
@@ -12939,10 +12939,10 @@
         <v>46266</v>
       </c>
       <c r="B1137" t="n">
-        <v>2492</v>
+        <v>2784</v>
       </c>
       <c r="C1137" t="n">
-        <v>51600</v>
+        <v>18910</v>
       </c>
     </row>
     <row r="1138">
@@ -12950,10 +12950,10 @@
         <v>46266</v>
       </c>
       <c r="B1138" t="n">
-        <v>629</v>
+        <v>2586</v>
       </c>
       <c r="C1138" t="n">
-        <v>160720</v>
+        <v>18910</v>
       </c>
     </row>
     <row r="1139">
@@ -12961,10 +12961,10 @@
         <v>46266</v>
       </c>
       <c r="B1139" t="n">
-        <v>966</v>
+        <v>2145</v>
       </c>
       <c r="C1139" t="n">
-        <v>29632</v>
+        <v>58840</v>
       </c>
     </row>
     <row r="1140">
@@ -12972,10 +12972,10 @@
         <v>46266</v>
       </c>
       <c r="B1140" t="n">
-        <v>2721</v>
+        <v>2574</v>
       </c>
       <c r="C1140" t="n">
-        <v>29632</v>
+        <v>58840</v>
       </c>
     </row>
     <row r="1141">
@@ -12983,10 +12983,10 @@
         <v>46266</v>
       </c>
       <c r="B1141" t="n">
-        <v>2554</v>
+        <v>2492</v>
       </c>
       <c r="C1141" t="n">
-        <v>8928</v>
+        <v>64500</v>
       </c>
     </row>
     <row r="1142">
@@ -12994,10 +12994,10 @@
         <v>46266</v>
       </c>
       <c r="B1142" t="n">
-        <v>2556</v>
+        <v>629</v>
       </c>
       <c r="C1142" t="n">
-        <v>13128</v>
+        <v>200900</v>
       </c>
     </row>
     <row r="1143">
@@ -13005,10 +13005,10 @@
         <v>46266</v>
       </c>
       <c r="B1143" t="n">
-        <v>2546</v>
+        <v>966</v>
       </c>
       <c r="C1143" t="n">
-        <v>8672</v>
+        <v>37040</v>
       </c>
     </row>
     <row r="1144">
@@ -13016,10 +13016,10 @@
         <v>46266</v>
       </c>
       <c r="B1144" t="n">
-        <v>42</v>
+        <v>2721</v>
       </c>
       <c r="C1144" t="n">
-        <v>687272</v>
+        <v>37040</v>
       </c>
     </row>
     <row r="1145">
@@ -13027,10 +13027,10 @@
         <v>46266</v>
       </c>
       <c r="B1145" t="n">
-        <v>953</v>
+        <v>2554</v>
       </c>
       <c r="C1145" t="n">
-        <v>248240</v>
+        <v>11160</v>
       </c>
     </row>
     <row r="1146">
@@ -13038,10 +13038,10 @@
         <v>46266</v>
       </c>
       <c r="B1146" t="n">
-        <v>675</v>
+        <v>2556</v>
       </c>
       <c r="C1146" t="n">
-        <v>72720</v>
+        <v>16410</v>
       </c>
     </row>
     <row r="1147">
@@ -13049,10 +13049,10 @@
         <v>46266</v>
       </c>
       <c r="B1147" t="n">
-        <v>619</v>
+        <v>2546</v>
       </c>
       <c r="C1147" t="n">
-        <v>112448</v>
+        <v>10840</v>
       </c>
     </row>
     <row r="1148">
@@ -13060,10 +13060,10 @@
         <v>46266</v>
       </c>
       <c r="B1148" t="n">
-        <v>1299</v>
+        <v>42</v>
       </c>
       <c r="C1148" t="n">
-        <v>189216</v>
+        <v>859090</v>
       </c>
     </row>
     <row r="1149">
@@ -13071,10 +13071,10 @@
         <v>46266</v>
       </c>
       <c r="B1149" t="n">
-        <v>525</v>
+        <v>953</v>
       </c>
       <c r="C1149" t="n">
-        <v>81816</v>
+        <v>310300</v>
       </c>
     </row>
     <row r="1150">
@@ -13082,10 +13082,10 @@
         <v>46266</v>
       </c>
       <c r="B1150" t="n">
-        <v>2727</v>
+        <v>675</v>
       </c>
       <c r="C1150" t="n">
-        <v>14720</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1151">
@@ -13093,10 +13093,10 @@
         <v>46266</v>
       </c>
       <c r="B1151" t="n">
-        <v>2341</v>
+        <v>630</v>
       </c>
       <c r="C1151" t="n">
-        <v>51600</v>
+        <v>68040</v>
       </c>
     </row>
     <row r="1152">
@@ -13104,10 +13104,10 @@
         <v>46266</v>
       </c>
       <c r="B1152" t="n">
-        <v>1374</v>
+        <v>525</v>
       </c>
       <c r="C1152" t="n">
-        <v>65448</v>
+        <v>102270</v>
       </c>
     </row>
     <row r="1153">
@@ -13115,10 +13115,10 @@
         <v>46266</v>
       </c>
       <c r="B1153" t="n">
-        <v>793</v>
+        <v>2727</v>
       </c>
       <c r="C1153" t="n">
-        <v>15128</v>
+        <v>18400</v>
       </c>
     </row>
     <row r="1154">
@@ -13126,10 +13126,10 @@
         <v>46266</v>
       </c>
       <c r="B1154" t="n">
-        <v>794</v>
+        <v>2341</v>
       </c>
       <c r="C1154" t="n">
-        <v>15128</v>
+        <v>64500</v>
       </c>
     </row>
     <row r="1155">
@@ -13137,10 +13137,10 @@
         <v>46266</v>
       </c>
       <c r="B1155" t="n">
-        <v>1834</v>
+        <v>1374</v>
       </c>
       <c r="C1155" t="n">
-        <v>42544</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1156">
@@ -13148,10 +13148,10 @@
         <v>46266</v>
       </c>
       <c r="B1156" t="n">
-        <v>802</v>
+        <v>793</v>
       </c>
       <c r="C1156" t="n">
-        <v>27272</v>
+        <v>18910</v>
       </c>
     </row>
     <row r="1157">
@@ -13159,10 +13159,10 @@
         <v>46266</v>
       </c>
       <c r="B1157" t="n">
-        <v>1344</v>
+        <v>794</v>
       </c>
       <c r="C1157" t="n">
-        <v>54544</v>
+        <v>18910</v>
       </c>
     </row>
     <row r="1158">
@@ -13170,10 +13170,10 @@
         <v>46266</v>
       </c>
       <c r="B1158" t="n">
-        <v>1881</v>
+        <v>1834</v>
       </c>
       <c r="C1158" t="n">
-        <v>24976</v>
+        <v>53180</v>
       </c>
     </row>
     <row r="1159">
@@ -13181,10 +13181,10 @@
         <v>46266</v>
       </c>
       <c r="B1159" t="n">
-        <v>2365</v>
+        <v>802</v>
       </c>
       <c r="C1159" t="n">
-        <v>28968</v>
+        <v>34090</v>
       </c>
     </row>
     <row r="1160">
@@ -13192,10 +13192,10 @@
         <v>46266</v>
       </c>
       <c r="B1160" t="n">
-        <v>2411</v>
+        <v>1344</v>
       </c>
       <c r="C1160" t="n">
-        <v>51600</v>
+        <v>68180</v>
       </c>
     </row>
     <row r="1161">
@@ -13203,10 +13203,10 @@
         <v>46266</v>
       </c>
       <c r="B1161" t="n">
-        <v>2363</v>
+        <v>1881</v>
       </c>
       <c r="C1161" t="n">
-        <v>54544</v>
+        <v>31220</v>
       </c>
     </row>
     <row r="1162">
@@ -13214,10 +13214,10 @@
         <v>46266</v>
       </c>
       <c r="B1162" t="n">
-        <v>2124</v>
+        <v>2365</v>
       </c>
       <c r="C1162" t="n">
-        <v>127272</v>
+        <v>36210</v>
       </c>
     </row>
     <row r="1163">
@@ -13225,10 +13225,10 @@
         <v>46266</v>
       </c>
       <c r="B1163" t="n">
-        <v>1937</v>
+        <v>2411</v>
       </c>
       <c r="C1163" t="n">
-        <v>92720</v>
+        <v>64500</v>
       </c>
     </row>
     <row r="1164">
@@ -13236,10 +13236,10 @@
         <v>46266</v>
       </c>
       <c r="B1164" t="n">
-        <v>2709</v>
+        <v>2363</v>
       </c>
       <c r="C1164" t="n">
-        <v>65448</v>
+        <v>68180</v>
       </c>
     </row>
     <row r="1165">
@@ -13247,10 +13247,10 @@
         <v>46266</v>
       </c>
       <c r="B1165" t="n">
-        <v>2558</v>
+        <v>2124</v>
       </c>
       <c r="C1165" t="n">
-        <v>10928</v>
+        <v>159090</v>
       </c>
     </row>
     <row r="1166">
@@ -13258,10 +13258,10 @@
         <v>46266</v>
       </c>
       <c r="B1166" t="n">
-        <v>663</v>
+        <v>1937</v>
       </c>
       <c r="C1166" t="n">
-        <v>92720</v>
+        <v>115900</v>
       </c>
     </row>
     <row r="1167">
@@ -13269,10 +13269,10 @@
         <v>46266</v>
       </c>
       <c r="B1167" t="n">
-        <v>40</v>
+        <v>2709</v>
       </c>
       <c r="C1167" t="n">
-        <v>80000</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1168">
@@ -13280,10 +13280,10 @@
         <v>46266</v>
       </c>
       <c r="B1168" t="n">
-        <v>1756</v>
+        <v>2558</v>
       </c>
       <c r="C1168" t="n">
-        <v>158728</v>
+        <v>13660</v>
       </c>
     </row>
     <row r="1169">
@@ -13291,10 +13291,10 @@
         <v>46266</v>
       </c>
       <c r="B1169" t="n">
-        <v>1116</v>
+        <v>663</v>
       </c>
       <c r="C1169" t="n">
-        <v>92232</v>
+        <v>115900</v>
       </c>
     </row>
     <row r="1170">
@@ -13302,10 +13302,10 @@
         <v>46266</v>
       </c>
       <c r="B1170" t="n">
-        <v>636</v>
+        <v>40</v>
       </c>
       <c r="C1170" t="n">
-        <v>90904</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1171">
@@ -13313,10 +13313,10 @@
         <v>46266</v>
       </c>
       <c r="B1171" t="n">
-        <v>1800</v>
+        <v>2833</v>
       </c>
       <c r="C1171" t="n">
-        <v>10176</v>
+        <v>31818.28</v>
       </c>
     </row>
     <row r="1172">
@@ -13324,10 +13324,10 @@
         <v>46266</v>
       </c>
       <c r="B1172" t="n">
-        <v>2815</v>
+        <v>1756</v>
       </c>
       <c r="C1172" t="n">
-        <v>21816</v>
+        <v>198410</v>
       </c>
     </row>
     <row r="1173">
@@ -13335,10 +13335,10 @@
         <v>46266</v>
       </c>
       <c r="B1173" t="n">
-        <v>1658</v>
+        <v>1116</v>
       </c>
       <c r="C1173" t="n">
-        <v>48000</v>
+        <v>115290</v>
       </c>
     </row>
     <row r="1174">
@@ -13346,10 +13346,10 @@
         <v>46266</v>
       </c>
       <c r="B1174" t="n">
-        <v>2635</v>
+        <v>636</v>
       </c>
       <c r="C1174" t="n">
-        <v>47272</v>
+        <v>113630</v>
       </c>
     </row>
     <row r="1175">
@@ -13357,10 +13357,10 @@
         <v>46266</v>
       </c>
       <c r="B1175" t="n">
-        <v>2402</v>
+        <v>1800</v>
       </c>
       <c r="C1175" t="n">
-        <v>237088</v>
+        <v>12720</v>
       </c>
     </row>
     <row r="1176">
@@ -13368,10 +13368,10 @@
         <v>46266</v>
       </c>
       <c r="B1176" t="n">
-        <v>452</v>
+        <v>2815</v>
       </c>
       <c r="C1176" t="n">
-        <v>98176</v>
+        <v>27272.76</v>
       </c>
     </row>
     <row r="1177">
@@ -13379,10 +13379,10 @@
         <v>46266</v>
       </c>
       <c r="B1177" t="n">
-        <v>2085</v>
+        <v>1658</v>
       </c>
       <c r="C1177" t="n">
-        <v>48016</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1178">
@@ -13390,10 +13390,10 @@
         <v>46266</v>
       </c>
       <c r="B1178" t="n">
-        <v>2568</v>
+        <v>2635</v>
       </c>
       <c r="C1178" t="n">
-        <v>74336</v>
+        <v>59090</v>
       </c>
     </row>
     <row r="1179">
@@ -13401,10 +13401,10 @@
         <v>46266</v>
       </c>
       <c r="B1179" t="n">
-        <v>2726</v>
+        <v>2402</v>
       </c>
       <c r="C1179" t="n">
-        <v>54544</v>
+        <v>296360</v>
       </c>
     </row>
     <row r="1180">
@@ -13412,10 +13412,10 @@
         <v>46266</v>
       </c>
       <c r="B1180" t="n">
-        <v>2820</v>
+        <v>452</v>
       </c>
       <c r="C1180" t="n">
-        <v>65448</v>
+        <v>122720</v>
       </c>
     </row>
     <row r="1181">
@@ -13423,10 +13423,10 @@
         <v>46266</v>
       </c>
       <c r="B1181" t="n">
-        <v>1007</v>
+        <v>2085</v>
       </c>
       <c r="C1181" t="n">
-        <v>69088</v>
+        <v>60020</v>
       </c>
     </row>
     <row r="1182">
@@ -13434,10 +13434,10 @@
         <v>46266</v>
       </c>
       <c r="B1182" t="n">
-        <v>20</v>
+        <v>2568</v>
       </c>
       <c r="C1182" t="n">
-        <v>140000</v>
+        <v>92920</v>
       </c>
     </row>
     <row r="1183">
@@ -13445,10 +13445,10 @@
         <v>46266</v>
       </c>
       <c r="B1183" t="n">
-        <v>1372</v>
+        <v>2726</v>
       </c>
       <c r="C1183" t="n">
-        <v>105448</v>
+        <v>68180</v>
       </c>
     </row>
     <row r="1184">
@@ -13456,10 +13456,10 @@
         <v>46266</v>
       </c>
       <c r="B1184" t="n">
-        <v>2735</v>
+        <v>2820</v>
       </c>
       <c r="C1184" t="n">
-        <v>43632</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1185">
@@ -13467,10 +13467,10 @@
         <v>46266</v>
       </c>
       <c r="B1185" t="n">
-        <v>2811</v>
+        <v>1007</v>
       </c>
       <c r="C1185" t="n">
-        <v>15128</v>
+        <v>86360</v>
       </c>
     </row>
     <row r="1186">
@@ -13478,10 +13478,10 @@
         <v>46266</v>
       </c>
       <c r="B1186" t="n">
-        <v>1871</v>
+        <v>20</v>
       </c>
       <c r="C1186" t="n">
-        <v>64272</v>
+        <v>175000</v>
       </c>
     </row>
     <row r="1187">
@@ -13489,10 +13489,10 @@
         <v>46266</v>
       </c>
       <c r="B1187" t="n">
-        <v>2541</v>
+        <v>1372</v>
       </c>
       <c r="C1187" t="n">
-        <v>76944</v>
+        <v>131810</v>
       </c>
     </row>
     <row r="1188">
@@ -13500,10 +13500,10 @@
         <v>46266</v>
       </c>
       <c r="B1188" t="n">
-        <v>2362</v>
+        <v>2735</v>
       </c>
       <c r="C1188" t="n">
-        <v>27272</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1189">
@@ -13511,10 +13511,10 @@
         <v>46266</v>
       </c>
       <c r="B1189" t="n">
-        <v>1324</v>
+        <v>2811</v>
       </c>
       <c r="C1189" t="n">
-        <v>101816</v>
+        <v>18910</v>
       </c>
     </row>
     <row r="1190">
@@ -13522,10 +13522,10 @@
         <v>46266</v>
       </c>
       <c r="B1190" t="n">
-        <v>2323</v>
+        <v>1871</v>
       </c>
       <c r="C1190" t="n">
-        <v>24976</v>
+        <v>80340</v>
       </c>
     </row>
     <row r="1191">
@@ -13533,10 +13533,10 @@
         <v>46266</v>
       </c>
       <c r="B1191" t="n">
-        <v>2647</v>
+        <v>2541</v>
       </c>
       <c r="C1191" t="n">
-        <v>51600</v>
+        <v>96180</v>
       </c>
     </row>
     <row r="1192">
@@ -13544,10 +13544,10 @@
         <v>46266</v>
       </c>
       <c r="B1192" t="n">
-        <v>559</v>
+        <v>2362</v>
       </c>
       <c r="C1192" t="n">
-        <v>83432</v>
+        <v>34090</v>
       </c>
     </row>
     <row r="1193">
@@ -13555,10 +13555,10 @@
         <v>46266</v>
       </c>
       <c r="B1193" t="n">
-        <v>2762</v>
+        <v>1324</v>
       </c>
       <c r="C1193" t="n">
-        <v>29632</v>
+        <v>127270</v>
       </c>
     </row>
     <row r="1194">
@@ -13566,10 +13566,10 @@
         <v>46266</v>
       </c>
       <c r="B1194" t="n">
-        <v>2501</v>
+        <v>2323</v>
       </c>
       <c r="C1194" t="n">
-        <v>29632</v>
+        <v>31220</v>
       </c>
     </row>
     <row r="1195">
@@ -13577,10 +13577,10 @@
         <v>46266</v>
       </c>
       <c r="B1195" t="n">
-        <v>2562</v>
+        <v>2647</v>
       </c>
       <c r="C1195" t="n">
-        <v>5752</v>
+        <v>64500</v>
       </c>
     </row>
     <row r="1196">
@@ -13588,10 +13588,10 @@
         <v>46266</v>
       </c>
       <c r="B1196" t="n">
-        <v>429</v>
+        <v>559</v>
       </c>
       <c r="C1196" t="n">
-        <v>141816</v>
+        <v>104290</v>
       </c>
     </row>
     <row r="1197">
@@ -13599,10 +13599,10 @@
         <v>46266</v>
       </c>
       <c r="B1197" t="n">
-        <v>58</v>
+        <v>2762</v>
       </c>
       <c r="C1197" t="n">
-        <v>98392</v>
+        <v>37040</v>
       </c>
     </row>
     <row r="1198">
@@ -13610,10 +13610,10 @@
         <v>46266</v>
       </c>
       <c r="B1198" t="n">
-        <v>2245</v>
+        <v>2501</v>
       </c>
       <c r="C1198" t="n">
-        <v>87848</v>
+        <v>37040</v>
       </c>
     </row>
     <row r="1199">
@@ -13621,10 +13621,10 @@
         <v>46266</v>
       </c>
       <c r="B1199" t="n">
-        <v>285</v>
+        <v>2562</v>
       </c>
       <c r="C1199" t="n">
-        <v>196784</v>
+        <v>7190</v>
       </c>
     </row>
     <row r="1200">
@@ -13632,10 +13632,10 @@
         <v>46266</v>
       </c>
       <c r="B1200" t="n">
-        <v>363</v>
+        <v>429</v>
       </c>
       <c r="C1200" t="n">
-        <v>109088</v>
+        <v>177270</v>
       </c>
     </row>
     <row r="1201">
@@ -13643,10 +13643,10 @@
         <v>46266</v>
       </c>
       <c r="B1201" t="n">
-        <v>2651</v>
+        <v>58</v>
       </c>
       <c r="C1201" t="n">
-        <v>61496</v>
+        <v>122990</v>
       </c>
     </row>
     <row r="1202">
@@ -13654,10 +13654,10 @@
         <v>46266</v>
       </c>
       <c r="B1202" t="n">
-        <v>2142</v>
+        <v>2245</v>
       </c>
       <c r="C1202" t="n">
-        <v>19408</v>
+        <v>109810</v>
       </c>
     </row>
     <row r="1203">
@@ -13665,10 +13665,10 @@
         <v>46266</v>
       </c>
       <c r="B1203" t="n">
-        <v>2258</v>
+        <v>285</v>
       </c>
       <c r="C1203" t="n">
-        <v>29088</v>
+        <v>245980</v>
       </c>
     </row>
     <row r="1204">
@@ -13676,10 +13676,10 @@
         <v>46266</v>
       </c>
       <c r="B1204" t="n">
-        <v>2772</v>
+        <v>363</v>
       </c>
       <c r="C1204" t="n">
-        <v>21816</v>
+        <v>136360</v>
       </c>
     </row>
     <row r="1205">
@@ -13687,10 +13687,10 @@
         <v>46266</v>
       </c>
       <c r="B1205" t="n">
-        <v>2346</v>
+        <v>2651</v>
       </c>
       <c r="C1205" t="n">
-        <v>40000</v>
+        <v>76870</v>
       </c>
     </row>
     <row r="1206">
@@ -13698,10 +13698,10 @@
         <v>46266</v>
       </c>
       <c r="B1206" t="n">
-        <v>2442</v>
+        <v>2142</v>
       </c>
       <c r="C1206" t="n">
-        <v>29088</v>
+        <v>24260</v>
       </c>
     </row>
     <row r="1207">
@@ -13709,10 +13709,10 @@
         <v>46266</v>
       </c>
       <c r="B1207" t="n">
-        <v>772</v>
+        <v>2258</v>
       </c>
       <c r="C1207" t="n">
-        <v>120000</v>
+        <v>36363.68</v>
       </c>
     </row>
     <row r="1208">
@@ -13720,10 +13720,10 @@
         <v>46266</v>
       </c>
       <c r="B1208" t="n">
-        <v>2684</v>
+        <v>2772</v>
       </c>
       <c r="C1208" t="n">
-        <v>34544</v>
+        <v>27272.76</v>
       </c>
     </row>
     <row r="1209">
@@ -13731,10 +13731,10 @@
         <v>46266</v>
       </c>
       <c r="B1209" t="n">
-        <v>2765</v>
+        <v>2346</v>
       </c>
       <c r="C1209" t="n">
-        <v>32720</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="1210">
@@ -13742,10 +13742,10 @@
         <v>46266</v>
       </c>
       <c r="B1210" t="n">
-        <v>2567</v>
+        <v>2442</v>
       </c>
       <c r="C1210" t="n">
-        <v>60016</v>
+        <v>36360</v>
       </c>
     </row>
     <row r="1211">
@@ -13753,10 +13753,10 @@
         <v>46266</v>
       </c>
       <c r="B1211" t="n">
-        <v>2178</v>
+        <v>772</v>
       </c>
       <c r="C1211" t="n">
-        <v>101816</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="1212">
@@ -13764,10 +13764,10 @@
         <v>46266</v>
       </c>
       <c r="B1212" t="n">
-        <v>2827</v>
+        <v>2684</v>
       </c>
       <c r="C1212" t="n">
-        <v>36360</v>
+        <v>43180</v>
       </c>
     </row>
     <row r="1213">
@@ -13775,10 +13775,10 @@
         <v>46266</v>
       </c>
       <c r="B1213" t="n">
-        <v>2831</v>
+        <v>2765</v>
       </c>
       <c r="C1213" t="n">
-        <v>21816</v>
+        <v>40900</v>
       </c>
     </row>
     <row r="1214">
@@ -13786,10 +13786,10 @@
         <v>46266</v>
       </c>
       <c r="B1214" t="n">
-        <v>580</v>
+        <v>2567</v>
       </c>
       <c r="C1214" t="n">
-        <v>49088</v>
+        <v>75020</v>
       </c>
     </row>
     <row r="1215">
@@ -13797,10 +13797,10 @@
         <v>46266</v>
       </c>
       <c r="B1215" t="n">
-        <v>438</v>
+        <v>2831</v>
       </c>
       <c r="C1215" t="n">
-        <v>56360</v>
+        <v>27270</v>
       </c>
     </row>
     <row r="1216">
@@ -13808,10 +13808,10 @@
         <v>46266</v>
       </c>
       <c r="B1216" t="n">
-        <v>1539</v>
+        <v>580</v>
       </c>
       <c r="C1216" t="n">
-        <v>61816</v>
+        <v>61360</v>
       </c>
     </row>
     <row r="1217">
@@ -13819,10 +13819,10 @@
         <v>46266</v>
       </c>
       <c r="B1217" t="n">
-        <v>2817</v>
+        <v>438</v>
       </c>
       <c r="C1217" t="n">
-        <v>21816</v>
+        <v>70450</v>
       </c>
     </row>
     <row r="1218">
@@ -13830,10 +13830,10 @@
         <v>46266</v>
       </c>
       <c r="B1218" t="n">
-        <v>2816</v>
+        <v>1539</v>
       </c>
       <c r="C1218" t="n">
-        <v>47272</v>
+        <v>77270</v>
       </c>
     </row>
     <row r="1219">
@@ -13841,10 +13841,10 @@
         <v>46266</v>
       </c>
       <c r="B1219" t="n">
-        <v>2146</v>
+        <v>2817</v>
       </c>
       <c r="C1219" t="n">
-        <v>73328</v>
+        <v>27270</v>
       </c>
     </row>
     <row r="1220">
@@ -13852,10 +13852,10 @@
         <v>46266</v>
       </c>
       <c r="B1220" t="n">
-        <v>2276</v>
+        <v>2816</v>
       </c>
       <c r="C1220" t="n">
-        <v>81472</v>
+        <v>59090</v>
       </c>
     </row>
     <row r="1221">
@@ -13863,10 +13863,10 @@
         <v>46266</v>
       </c>
       <c r="B1221" t="n">
-        <v>1381</v>
+        <v>2146</v>
       </c>
       <c r="C1221" t="n">
-        <v>107272</v>
+        <v>91660</v>
       </c>
     </row>
     <row r="1222">
@@ -13874,10 +13874,10 @@
         <v>46266</v>
       </c>
       <c r="B1222" t="n">
-        <v>2081</v>
+        <v>2276</v>
       </c>
       <c r="C1222" t="n">
-        <v>54544</v>
+        <v>101840</v>
       </c>
     </row>
     <row r="1223">
@@ -13885,10 +13885,10 @@
         <v>46266</v>
       </c>
       <c r="B1223" t="n">
-        <v>14</v>
+        <v>1381</v>
       </c>
       <c r="C1223" t="n">
-        <v>158176</v>
+        <v>134090</v>
       </c>
     </row>
     <row r="1224">
@@ -13896,10 +13896,10 @@
         <v>46266</v>
       </c>
       <c r="B1224" t="n">
-        <v>766</v>
+        <v>2081</v>
       </c>
       <c r="C1224" t="n">
-        <v>24976</v>
+        <v>68180</v>
       </c>
     </row>
     <row r="1225">
@@ -13907,10 +13907,10 @@
         <v>46266</v>
       </c>
       <c r="B1225" t="n">
-        <v>2547</v>
+        <v>14</v>
       </c>
       <c r="C1225" t="n">
-        <v>14952</v>
+        <v>197720</v>
       </c>
     </row>
     <row r="1226">
@@ -13918,10 +13918,10 @@
         <v>46266</v>
       </c>
       <c r="B1226" t="n">
-        <v>2552</v>
+        <v>766</v>
       </c>
       <c r="C1226" t="n">
-        <v>10752</v>
+        <v>31220</v>
       </c>
     </row>
     <row r="1227">
@@ -13929,10 +13929,10 @@
         <v>46266</v>
       </c>
       <c r="B1227" t="n">
-        <v>131</v>
+        <v>2547</v>
       </c>
       <c r="C1227" t="n">
-        <v>148720</v>
+        <v>18690</v>
       </c>
     </row>
     <row r="1228">
@@ -13940,10 +13940,10 @@
         <v>46266</v>
       </c>
       <c r="B1228" t="n">
-        <v>2250</v>
+        <v>2552</v>
       </c>
       <c r="C1228" t="n">
-        <v>120328</v>
+        <v>13440</v>
       </c>
     </row>
     <row r="1229">
@@ -13951,10 +13951,10 @@
         <v>46266</v>
       </c>
       <c r="B1229" t="n">
-        <v>89</v>
+        <v>131</v>
       </c>
       <c r="C1229" t="n">
-        <v>122976</v>
+        <v>185900</v>
       </c>
     </row>
     <row r="1230">
@@ -13962,10 +13962,10 @@
         <v>46266</v>
       </c>
       <c r="B1230" t="n">
-        <v>2141</v>
+        <v>2250</v>
       </c>
       <c r="C1230" t="n">
-        <v>11504</v>
+        <v>150410</v>
       </c>
     </row>
     <row r="1231">
@@ -13973,10 +13973,10 @@
         <v>46266</v>
       </c>
       <c r="B1231" t="n">
-        <v>2798</v>
+        <v>89</v>
       </c>
       <c r="C1231" t="n">
-        <v>21816</v>
+        <v>153720</v>
       </c>
     </row>
     <row r="1232">
@@ -13984,10 +13984,10 @@
         <v>46266</v>
       </c>
       <c r="B1232" t="n">
-        <v>2797</v>
+        <v>2141</v>
       </c>
       <c r="C1232" t="n">
-        <v>21816</v>
+        <v>14380</v>
       </c>
     </row>
     <row r="1233">
@@ -13995,10 +13995,10 @@
         <v>46266</v>
       </c>
       <c r="B1233" t="n">
-        <v>2266</v>
+        <v>2798</v>
       </c>
       <c r="C1233" t="n">
-        <v>29088</v>
+        <v>27272.76</v>
       </c>
     </row>
     <row r="1234">
@@ -14006,10 +14006,10 @@
         <v>46266</v>
       </c>
       <c r="B1234" t="n">
-        <v>1499</v>
+        <v>2797</v>
       </c>
       <c r="C1234" t="n">
-        <v>50904</v>
+        <v>27272.76</v>
       </c>
     </row>
     <row r="1235">
@@ -14017,10 +14017,10 @@
         <v>46266</v>
       </c>
       <c r="B1235" t="n">
-        <v>2496</v>
+        <v>2266</v>
       </c>
       <c r="C1235" t="n">
-        <v>58176</v>
+        <v>36363.68</v>
       </c>
     </row>
     <row r="1236">
@@ -14028,10 +14028,10 @@
         <v>46266</v>
       </c>
       <c r="B1236" t="n">
-        <v>949</v>
+        <v>1499</v>
       </c>
       <c r="C1236" t="n">
-        <v>35688</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1237">
@@ -14039,10 +14039,10 @@
         <v>46266</v>
       </c>
       <c r="B1237" t="n">
-        <v>1853</v>
+        <v>2496</v>
       </c>
       <c r="C1237" t="n">
-        <v>43632</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1238">
@@ -14050,10 +14050,10 @@
         <v>46266</v>
       </c>
       <c r="B1238" t="n">
-        <v>854</v>
+        <v>949</v>
       </c>
       <c r="C1238" t="n">
-        <v>40000</v>
+        <v>44610</v>
       </c>
     </row>
     <row r="1239">
@@ -14061,10 +14061,10 @@
         <v>46266</v>
       </c>
       <c r="B1239" t="n">
-        <v>2674</v>
+        <v>1853</v>
       </c>
       <c r="C1239" t="n">
-        <v>94544</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1240">
@@ -14072,10 +14072,10 @@
         <v>46266</v>
       </c>
       <c r="B1240" t="n">
-        <v>2803</v>
+        <v>854</v>
       </c>
       <c r="C1240" t="n">
-        <v>43632</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="1241">
@@ -14083,10 +14083,10 @@
         <v>46266</v>
       </c>
       <c r="B1241" t="n">
-        <v>2599</v>
+        <v>2674</v>
       </c>
       <c r="C1241" t="n">
-        <v>69088</v>
+        <v>118180</v>
       </c>
     </row>
     <row r="1242">
@@ -14094,10 +14094,10 @@
         <v>46266</v>
       </c>
       <c r="B1242" t="n">
-        <v>783</v>
+        <v>2803</v>
       </c>
       <c r="C1242" t="n">
-        <v>18904</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1243">
@@ -14105,10 +14105,10 @@
         <v>46266</v>
       </c>
       <c r="B1243" t="n">
-        <v>27</v>
+        <v>2599</v>
       </c>
       <c r="C1243" t="n">
-        <v>36360</v>
+        <v>86360</v>
       </c>
     </row>
     <row r="1244">
@@ -14116,10 +14116,10 @@
         <v>46266</v>
       </c>
       <c r="B1244" t="n">
-        <v>2823</v>
+        <v>783</v>
       </c>
       <c r="C1244" t="n">
-        <v>34000</v>
+        <v>23630</v>
       </c>
     </row>
     <row r="1245">
@@ -14127,10 +14127,10 @@
         <v>46266</v>
       </c>
       <c r="B1245" t="n">
-        <v>945</v>
+        <v>27</v>
       </c>
       <c r="C1245" t="n">
-        <v>103024</v>
+        <v>45450</v>
       </c>
     </row>
     <row r="1246">
@@ -14138,10 +14138,10 @@
         <v>46266</v>
       </c>
       <c r="B1246" t="n">
-        <v>2660</v>
+        <v>2823</v>
       </c>
       <c r="C1246" t="n">
-        <v>112720</v>
+        <v>42500</v>
       </c>
     </row>
     <row r="1247">
@@ -14149,10 +14149,10 @@
         <v>46266</v>
       </c>
       <c r="B1247" t="n">
-        <v>1317</v>
+        <v>945</v>
       </c>
       <c r="C1247" t="n">
-        <v>109088</v>
+        <v>128780</v>
       </c>
     </row>
     <row r="1248">
@@ -14160,10 +14160,10 @@
         <v>46266</v>
       </c>
       <c r="B1248" t="n">
-        <v>1278</v>
+        <v>2660</v>
       </c>
       <c r="C1248" t="n">
-        <v>36360</v>
+        <v>140900</v>
       </c>
     </row>
     <row r="1249">
@@ -14171,10 +14171,10 @@
         <v>46266</v>
       </c>
       <c r="B1249" t="n">
-        <v>2745</v>
+        <v>1317</v>
       </c>
       <c r="C1249" t="n">
-        <v>40000</v>
+        <v>136360</v>
       </c>
     </row>
     <row r="1250">
@@ -14182,10 +14182,10 @@
         <v>46266</v>
       </c>
       <c r="B1250" t="n">
-        <v>2753</v>
+        <v>1278</v>
       </c>
       <c r="C1250" t="n">
-        <v>27272</v>
+        <v>45450</v>
       </c>
     </row>
     <row r="1251">
@@ -14193,10 +14193,10 @@
         <v>46266</v>
       </c>
       <c r="B1251" t="n">
-        <v>2183</v>
+        <v>2745</v>
       </c>
       <c r="C1251" t="n">
-        <v>133072</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="1252">
@@ -14204,10 +14204,10 @@
         <v>46266</v>
       </c>
       <c r="B1252" t="n">
-        <v>1340</v>
+        <v>2753</v>
       </c>
       <c r="C1252" t="n">
-        <v>52720</v>
+        <v>34090</v>
       </c>
     </row>
     <row r="1253">
@@ -14215,10 +14215,10 @@
         <v>46266</v>
       </c>
       <c r="B1253" t="n">
-        <v>2583</v>
+        <v>2183</v>
       </c>
       <c r="C1253" t="n">
-        <v>15128</v>
+        <v>166340</v>
       </c>
     </row>
     <row r="1254">
@@ -14226,10 +14226,10 @@
         <v>46266</v>
       </c>
       <c r="B1254" t="n">
-        <v>2090</v>
+        <v>1340</v>
       </c>
       <c r="C1254" t="n">
-        <v>15128</v>
+        <v>65900</v>
       </c>
     </row>
     <row r="1255">
@@ -14237,10 +14237,10 @@
         <v>46266</v>
       </c>
       <c r="B1255" t="n">
-        <v>1277</v>
+        <v>2583</v>
       </c>
       <c r="C1255" t="n">
-        <v>80000</v>
+        <v>18910</v>
       </c>
     </row>
     <row r="1256">
@@ -14248,10 +14248,10 @@
         <v>46266</v>
       </c>
       <c r="B1256" t="n">
-        <v>1501</v>
+        <v>2090</v>
       </c>
       <c r="C1256" t="n">
-        <v>34544</v>
+        <v>18910</v>
       </c>
     </row>
     <row r="1257">
@@ -14259,10 +14259,10 @@
         <v>46266</v>
       </c>
       <c r="B1257" t="n">
-        <v>703</v>
+        <v>1277</v>
       </c>
       <c r="C1257" t="n">
-        <v>90904</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1258">
@@ -14270,10 +14270,10 @@
         <v>46266</v>
       </c>
       <c r="B1258" t="n">
-        <v>749</v>
+        <v>1501</v>
       </c>
       <c r="C1258" t="n">
-        <v>29632</v>
+        <v>43180</v>
       </c>
     </row>
     <row r="1259">
@@ -14281,10 +14281,10 @@
         <v>46266</v>
       </c>
       <c r="B1259" t="n">
-        <v>1983</v>
+        <v>703</v>
       </c>
       <c r="C1259" t="n">
-        <v>196784</v>
+        <v>113630</v>
       </c>
     </row>
     <row r="1260">
@@ -14292,10 +14292,10 @@
         <v>46266</v>
       </c>
       <c r="B1260" t="n">
-        <v>1993</v>
+        <v>749</v>
       </c>
       <c r="C1260" t="n">
-        <v>126504</v>
+        <v>37040</v>
       </c>
     </row>
     <row r="1261">
@@ -14303,10 +14303,10 @@
         <v>46266</v>
       </c>
       <c r="B1261" t="n">
-        <v>2767</v>
+        <v>1983</v>
       </c>
       <c r="C1261" t="n">
-        <v>70152</v>
+        <v>245980</v>
       </c>
     </row>
     <row r="1262">
@@ -14314,10 +14314,10 @@
         <v>46266</v>
       </c>
       <c r="B1262" t="n">
-        <v>1102</v>
+        <v>1993</v>
       </c>
       <c r="C1262" t="n">
-        <v>87848</v>
+        <v>158130</v>
       </c>
     </row>
     <row r="1263">
@@ -14325,10 +14325,10 @@
         <v>46266</v>
       </c>
       <c r="B1263" t="n">
-        <v>1465</v>
+        <v>2767</v>
       </c>
       <c r="C1263" t="n">
-        <v>130832</v>
+        <v>87690</v>
       </c>
     </row>
     <row r="1264">
@@ -14336,10 +14336,10 @@
         <v>46266</v>
       </c>
       <c r="B1264" t="n">
-        <v>2758</v>
+        <v>2646</v>
       </c>
       <c r="C1264" t="n">
-        <v>21816</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1265">
@@ -14347,10 +14347,10 @@
         <v>46266</v>
       </c>
       <c r="B1265" t="n">
-        <v>2742</v>
+        <v>1102</v>
       </c>
       <c r="C1265" t="n">
-        <v>21816</v>
+        <v>109810</v>
       </c>
     </row>
     <row r="1266">
@@ -14358,10 +14358,10 @@
         <v>46266</v>
       </c>
       <c r="B1266" t="n">
-        <v>2748</v>
+        <v>1465</v>
       </c>
       <c r="C1266" t="n">
-        <v>25448</v>
+        <v>163540</v>
       </c>
     </row>
     <row r="1267">
@@ -14369,10 +14369,10 @@
         <v>46266</v>
       </c>
       <c r="B1267" t="n">
-        <v>1873</v>
+        <v>2758</v>
       </c>
       <c r="C1267" t="n">
-        <v>116360</v>
+        <v>27272.76</v>
       </c>
     </row>
     <row r="1268">
@@ -14380,10 +14380,10 @@
         <v>46266</v>
       </c>
       <c r="B1268" t="n">
-        <v>2163</v>
+        <v>2742</v>
       </c>
       <c r="C1268" t="n">
-        <v>54544</v>
+        <v>27272.76</v>
       </c>
     </row>
     <row r="1269">
@@ -14391,10 +14391,10 @@
         <v>46266</v>
       </c>
       <c r="B1269" t="n">
-        <v>2394</v>
+        <v>2748</v>
       </c>
       <c r="C1269" t="n">
-        <v>56016</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1270">
@@ -14402,10 +14402,10 @@
         <v>46266</v>
       </c>
       <c r="B1270" t="n">
-        <v>33</v>
+        <v>1873</v>
       </c>
       <c r="C1270" t="n">
-        <v>141088</v>
+        <v>145450</v>
       </c>
     </row>
     <row r="1271">
@@ -14413,10 +14413,10 @@
         <v>46266</v>
       </c>
       <c r="B1271" t="n">
-        <v>2421</v>
+        <v>2163</v>
       </c>
       <c r="C1271" t="n">
-        <v>23632</v>
+        <v>68180</v>
       </c>
     </row>
     <row r="1272">
@@ -14424,10 +14424,10 @@
         <v>46266</v>
       </c>
       <c r="B1272" t="n">
-        <v>2663</v>
+        <v>2394</v>
       </c>
       <c r="C1272" t="n">
-        <v>100000</v>
+        <v>70020</v>
       </c>
     </row>
     <row r="1273">
@@ -14435,10 +14435,10 @@
         <v>46266</v>
       </c>
       <c r="B1273" t="n">
-        <v>2413</v>
+        <v>33</v>
       </c>
       <c r="C1273" t="n">
-        <v>44016</v>
+        <v>176360</v>
       </c>
     </row>
     <row r="1274">
@@ -14446,10 +14446,10 @@
         <v>46266</v>
       </c>
       <c r="B1274" t="n">
-        <v>351</v>
+        <v>2421</v>
       </c>
       <c r="C1274" t="n">
-        <v>66904</v>
+        <v>29540</v>
       </c>
     </row>
     <row r="1275">
@@ -14457,10 +14457,10 @@
         <v>46266</v>
       </c>
       <c r="B1275" t="n">
-        <v>1298</v>
+        <v>2663</v>
       </c>
       <c r="C1275" t="n">
-        <v>462904</v>
+        <v>125000</v>
       </c>
     </row>
     <row r="1276">
@@ -14468,10 +14468,32 @@
         <v>46266</v>
       </c>
       <c r="B1276" t="n">
-        <v>630</v>
+        <v>2413</v>
       </c>
       <c r="C1276" t="n">
-        <v>54432</v>
+        <v>55020</v>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1277" t="n">
+        <v>351</v>
+      </c>
+      <c r="C1277" t="n">
+        <v>83630</v>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1278" t="n">
+        <v>1298</v>
+      </c>
+      <c r="C1278" t="n">
+        <v>578630</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:01:11
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1332"/>
+  <dimension ref="A1:C1346"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11289,10 +11289,10 @@
         <v>46266</v>
       </c>
       <c r="B987" t="n">
-        <v>2548</v>
+        <v>1956</v>
       </c>
       <c r="C987" t="n">
-        <v>26600</v>
+        <v>126236</v>
       </c>
     </row>
     <row r="988">
@@ -11300,10 +11300,10 @@
         <v>46266</v>
       </c>
       <c r="B988" t="n">
-        <v>451</v>
+        <v>2824</v>
       </c>
       <c r="C988" t="n">
-        <v>109090</v>
+        <v>55000</v>
       </c>
     </row>
     <row r="989">
@@ -11311,10 +11311,10 @@
         <v>46266</v>
       </c>
       <c r="B989" t="n">
-        <v>933</v>
+        <v>2787</v>
       </c>
       <c r="C989" t="n">
-        <v>37040</v>
+        <v>64999</v>
       </c>
     </row>
     <row r="990">
@@ -11322,10 +11322,10 @@
         <v>46266</v>
       </c>
       <c r="B990" t="n">
-        <v>2702</v>
+        <v>2830</v>
       </c>
       <c r="C990" t="n">
-        <v>37040</v>
+        <v>44990</v>
       </c>
     </row>
     <row r="991">
@@ -11333,10 +11333,10 @@
         <v>46266</v>
       </c>
       <c r="B991" t="n">
-        <v>2549</v>
+        <v>1254</v>
       </c>
       <c r="C991" t="n">
-        <v>12880</v>
+        <v>97098.00999999999</v>
       </c>
     </row>
     <row r="992">
@@ -11344,10 +11344,10 @@
         <v>46266</v>
       </c>
       <c r="B992" t="n">
-        <v>535</v>
+        <v>1890</v>
       </c>
       <c r="C992" t="n">
-        <v>168180</v>
+        <v>158071.42</v>
       </c>
     </row>
     <row r="993">
@@ -11355,10 +11355,10 @@
         <v>46266</v>
       </c>
       <c r="B993" t="n">
-        <v>1117</v>
+        <v>816</v>
       </c>
       <c r="C993" t="n">
-        <v>158130</v>
+        <v>133925</v>
       </c>
     </row>
     <row r="994">
@@ -11366,10 +11366,10 @@
         <v>46266</v>
       </c>
       <c r="B994" t="n">
-        <v>2109</v>
+        <v>2671</v>
       </c>
       <c r="C994" t="n">
-        <v>0</v>
+        <v>39996</v>
       </c>
     </row>
     <row r="995">
@@ -11377,10 +11377,10 @@
         <v>46266</v>
       </c>
       <c r="B995" t="n">
-        <v>530</v>
+        <v>2705</v>
       </c>
       <c r="C995" t="n">
-        <v>110940</v>
+        <v>89595</v>
       </c>
     </row>
     <row r="996">
@@ -11388,10 +11388,10 @@
         <v>46266</v>
       </c>
       <c r="B996" t="n">
-        <v>358</v>
+        <v>2333</v>
       </c>
       <c r="C996" t="n">
-        <v>154540</v>
+        <v>77176</v>
       </c>
     </row>
     <row r="997">
@@ -11399,10 +11399,10 @@
         <v>46266</v>
       </c>
       <c r="B997" t="n">
-        <v>2498</v>
+        <v>2440</v>
       </c>
       <c r="C997" t="n">
-        <v>25240</v>
+        <v>44990</v>
       </c>
     </row>
     <row r="998">
@@ -11410,10 +11410,10 @@
         <v>46266</v>
       </c>
       <c r="B998" t="n">
-        <v>2381</v>
+        <v>2448</v>
       </c>
       <c r="C998" t="n">
-        <v>36060</v>
+        <v>9999</v>
       </c>
     </row>
     <row r="999">
@@ -11421,10 +11421,10 @@
         <v>46266</v>
       </c>
       <c r="B999" t="n">
-        <v>2695</v>
+        <v>2310</v>
       </c>
       <c r="C999" t="n">
-        <v>21690</v>
+        <v>34342</v>
       </c>
     </row>
     <row r="1000">
@@ -11432,10 +11432,10 @@
         <v>46266</v>
       </c>
       <c r="B1000" t="n">
-        <v>2744</v>
+        <v>2809</v>
       </c>
       <c r="C1000" t="n">
-        <v>27272.76</v>
+        <v>34342</v>
       </c>
     </row>
     <row r="1001">
@@ -11443,10 +11443,10 @@
         <v>46266</v>
       </c>
       <c r="B1001" t="n">
-        <v>2750</v>
+        <v>2548</v>
       </c>
       <c r="C1001" t="n">
-        <v>27270</v>
+        <v>29260</v>
       </c>
     </row>
     <row r="1002">
@@ -11454,10 +11454,10 @@
         <v>46266</v>
       </c>
       <c r="B1002" t="n">
-        <v>2131</v>
+        <v>451</v>
       </c>
       <c r="C1002" t="n">
-        <v>54540</v>
+        <v>119999</v>
       </c>
     </row>
     <row r="1003">
@@ -11465,10 +11465,10 @@
         <v>46266</v>
       </c>
       <c r="B1003" t="n">
-        <v>818</v>
+        <v>933</v>
       </c>
       <c r="C1003" t="n">
-        <v>181810</v>
+        <v>40744</v>
       </c>
     </row>
     <row r="1004">
@@ -11476,10 +11476,10 @@
         <v>46266</v>
       </c>
       <c r="B1004" t="n">
-        <v>2566</v>
+        <v>2702</v>
       </c>
       <c r="C1004" t="n">
-        <v>36360</v>
+        <v>40744</v>
       </c>
     </row>
     <row r="1005">
@@ -11487,10 +11487,10 @@
         <v>46266</v>
       </c>
       <c r="B1005" t="n">
-        <v>132</v>
+        <v>2549</v>
       </c>
       <c r="C1005" t="n">
-        <v>340900</v>
+        <v>14168</v>
       </c>
     </row>
     <row r="1006">
@@ -11498,10 +11498,10 @@
         <v>46266</v>
       </c>
       <c r="B1006" t="n">
-        <v>2431</v>
+        <v>535</v>
       </c>
       <c r="C1006" t="n">
-        <v>83630</v>
+        <v>184998</v>
       </c>
     </row>
     <row r="1007">
@@ -11509,10 +11509,10 @@
         <v>46266</v>
       </c>
       <c r="B1007" t="n">
-        <v>2249</v>
+        <v>1117</v>
       </c>
       <c r="C1007" t="n">
-        <v>88780</v>
+        <v>173943</v>
       </c>
     </row>
     <row r="1008">
@@ -11520,10 +11520,10 @@
         <v>46266</v>
       </c>
       <c r="B1008" t="n">
-        <v>1585</v>
+        <v>2109</v>
       </c>
       <c r="C1008" t="n">
-        <v>75020</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1009">
@@ -11531,10 +11531,10 @@
         <v>46266</v>
       </c>
       <c r="B1009" t="n">
-        <v>2325</v>
+        <v>530</v>
       </c>
       <c r="C1009" t="n">
-        <v>72520</v>
+        <v>122034</v>
       </c>
     </row>
     <row r="1010">
@@ -11542,10 +11542,10 @@
         <v>46266</v>
       </c>
       <c r="B1010" t="n">
-        <v>2190</v>
+        <v>358</v>
       </c>
       <c r="C1010" t="n">
-        <v>102270</v>
+        <v>169994</v>
       </c>
     </row>
     <row r="1011">
@@ -11553,10 +11553,10 @@
         <v>46266</v>
       </c>
       <c r="B1011" t="n">
-        <v>1466</v>
+        <v>2498</v>
       </c>
       <c r="C1011" t="n">
-        <v>184090</v>
+        <v>27764</v>
       </c>
     </row>
     <row r="1012">
@@ -11564,10 +11564,10 @@
         <v>46266</v>
       </c>
       <c r="B1012" t="n">
-        <v>2659</v>
+        <v>2381</v>
       </c>
       <c r="C1012" t="n">
-        <v>55910</v>
+        <v>39666</v>
       </c>
     </row>
     <row r="1013">
@@ -11575,10 +11575,10 @@
         <v>46266</v>
       </c>
       <c r="B1013" t="n">
-        <v>1105</v>
+        <v>2695</v>
       </c>
       <c r="C1013" t="n">
-        <v>0</v>
+        <v>23859</v>
       </c>
     </row>
     <row r="1014">
@@ -11586,10 +11586,10 @@
         <v>46266</v>
       </c>
       <c r="B1014" t="n">
-        <v>2789</v>
+        <v>2744</v>
       </c>
       <c r="C1014" t="n">
-        <v>77270</v>
+        <v>30000.03</v>
       </c>
     </row>
     <row r="1015">
@@ -11597,10 +11597,10 @@
         <v>46266</v>
       </c>
       <c r="B1015" t="n">
-        <v>569</v>
+        <v>2750</v>
       </c>
       <c r="C1015" t="n">
-        <v>1301780</v>
+        <v>29997</v>
       </c>
     </row>
     <row r="1016">
@@ -11608,10 +11608,10 @@
         <v>46266</v>
       </c>
       <c r="B1016" t="n">
-        <v>2822</v>
+        <v>2131</v>
       </c>
       <c r="C1016" t="n">
-        <v>61360</v>
+        <v>59994</v>
       </c>
     </row>
     <row r="1017">
@@ -11619,10 +11619,10 @@
         <v>46266</v>
       </c>
       <c r="B1017" t="n">
-        <v>2728</v>
+        <v>818</v>
       </c>
       <c r="C1017" t="n">
-        <v>4540</v>
+        <v>199991</v>
       </c>
     </row>
     <row r="1018">
@@ -11630,10 +11630,10 @@
         <v>46266</v>
       </c>
       <c r="B1018" t="n">
-        <v>2488</v>
+        <v>2566</v>
       </c>
       <c r="C1018" t="n">
-        <v>45450</v>
+        <v>39996</v>
       </c>
     </row>
     <row r="1019">
@@ -11641,10 +11641,10 @@
         <v>46266</v>
       </c>
       <c r="B1019" t="n">
-        <v>2791</v>
+        <v>132</v>
       </c>
       <c r="C1019" t="n">
-        <v>44859.2</v>
+        <v>374990</v>
       </c>
     </row>
     <row r="1020">
@@ -11652,10 +11652,10 @@
         <v>46266</v>
       </c>
       <c r="B1020" t="n">
-        <v>2577</v>
+        <v>2431</v>
       </c>
       <c r="C1020" t="n">
-        <v>40531.93</v>
+        <v>91993</v>
       </c>
     </row>
     <row r="1021">
@@ -11663,10 +11663,10 @@
         <v>46266</v>
       </c>
       <c r="B1021" t="n">
-        <v>2069</v>
+        <v>2249</v>
       </c>
       <c r="C1021" t="n">
-        <v>81810</v>
+        <v>97658</v>
       </c>
     </row>
     <row r="1022">
@@ -11674,10 +11674,10 @@
         <v>46266</v>
       </c>
       <c r="B1022" t="n">
-        <v>2082</v>
+        <v>1585</v>
       </c>
       <c r="C1022" t="n">
-        <v>75710</v>
+        <v>82522</v>
       </c>
     </row>
     <row r="1023">
@@ -11685,10 +11685,10 @@
         <v>46266</v>
       </c>
       <c r="B1023" t="n">
-        <v>781</v>
+        <v>2325</v>
       </c>
       <c r="C1023" t="n">
-        <v>59090</v>
+        <v>79772</v>
       </c>
     </row>
     <row r="1024">
@@ -11696,10 +11696,10 @@
         <v>46266</v>
       </c>
       <c r="B1024" t="n">
-        <v>744</v>
+        <v>2190</v>
       </c>
       <c r="C1024" t="n">
-        <v>18910</v>
+        <v>112497</v>
       </c>
     </row>
     <row r="1025">
@@ -11707,10 +11707,10 @@
         <v>46266</v>
       </c>
       <c r="B1025" t="n">
-        <v>2223</v>
+        <v>1466</v>
       </c>
       <c r="C1025" t="n">
-        <v>59970</v>
+        <v>202499</v>
       </c>
     </row>
     <row r="1026">
@@ -11718,10 +11718,10 @@
         <v>46266</v>
       </c>
       <c r="B1026" t="n">
-        <v>2452</v>
+        <v>2659</v>
       </c>
       <c r="C1026" t="n">
-        <v>31810</v>
+        <v>61501</v>
       </c>
     </row>
     <row r="1027">
@@ -11729,10 +11729,10 @@
         <v>46266</v>
       </c>
       <c r="B1027" t="n">
-        <v>970</v>
+        <v>634</v>
       </c>
       <c r="C1027" t="n">
-        <v>31220</v>
+        <v>275000</v>
       </c>
     </row>
     <row r="1028">
@@ -11740,10 +11740,10 @@
         <v>46266</v>
       </c>
       <c r="B1028" t="n">
-        <v>2550</v>
+        <v>2804</v>
       </c>
       <c r="C1028" t="n">
-        <v>27720</v>
+        <v>49995</v>
       </c>
     </row>
     <row r="1029">
@@ -11751,10 +11751,10 @@
         <v>46266</v>
       </c>
       <c r="B1029" t="n">
-        <v>768</v>
+        <v>2375</v>
       </c>
       <c r="C1029" t="n">
-        <v>59090</v>
+        <v>165000</v>
       </c>
     </row>
     <row r="1030">
@@ -11762,10 +11762,10 @@
         <v>46266</v>
       </c>
       <c r="B1030" t="n">
-        <v>1075</v>
+        <v>2601</v>
       </c>
       <c r="C1030" t="n">
-        <v>205900</v>
+        <v>137500</v>
       </c>
     </row>
     <row r="1031">
@@ -11773,10 +11773,10 @@
         <v>46266</v>
       </c>
       <c r="B1031" t="n">
-        <v>664</v>
+        <v>952</v>
       </c>
       <c r="C1031" t="n">
-        <v>117720</v>
+        <v>49995</v>
       </c>
     </row>
     <row r="1032">
@@ -11784,10 +11784,10 @@
         <v>46266</v>
       </c>
       <c r="B1032" t="n">
-        <v>2555</v>
+        <v>571</v>
       </c>
       <c r="C1032" t="n">
-        <v>18870</v>
+        <v>318241</v>
       </c>
     </row>
     <row r="1033">
@@ -11795,10 +11795,10 @@
         <v>46266</v>
       </c>
       <c r="B1033" t="n">
-        <v>2627</v>
+        <v>2697</v>
       </c>
       <c r="C1033" t="n">
-        <v>11080</v>
+        <v>96965</v>
       </c>
     </row>
     <row r="1034">
@@ -11806,10 +11806,10 @@
         <v>46266</v>
       </c>
       <c r="B1034" t="n">
-        <v>2557</v>
+        <v>2678</v>
       </c>
       <c r="C1034" t="n">
-        <v>11720</v>
+        <v>167761</v>
       </c>
     </row>
     <row r="1035">
@@ -11817,10 +11817,10 @@
         <v>46266</v>
       </c>
       <c r="B1035" t="n">
-        <v>2551</v>
+        <v>2768</v>
       </c>
       <c r="C1035" t="n">
-        <v>9310</v>
+        <v>175571</v>
       </c>
     </row>
     <row r="1036">
@@ -11828,10 +11828,10 @@
         <v>46266</v>
       </c>
       <c r="B1036" t="n">
-        <v>2463</v>
+        <v>2359</v>
       </c>
       <c r="C1036" t="n">
-        <v>145550</v>
+        <v>53251</v>
       </c>
     </row>
     <row r="1037">
@@ -11839,10 +11839,10 @@
         <v>46266</v>
       </c>
       <c r="B1037" t="n">
-        <v>2279</v>
+        <v>353</v>
       </c>
       <c r="C1037" t="n">
-        <v>109810</v>
+        <v>172986</v>
       </c>
     </row>
     <row r="1038">
@@ -11850,10 +11850,10 @@
         <v>46266</v>
       </c>
       <c r="B1038" t="n">
-        <v>631</v>
+        <v>2026</v>
       </c>
       <c r="C1038" t="n">
-        <v>159090</v>
+        <v>143330</v>
       </c>
     </row>
     <row r="1039">
@@ -11861,10 +11861,10 @@
         <v>46266</v>
       </c>
       <c r="B1039" t="n">
-        <v>2251</v>
+        <v>1105</v>
       </c>
       <c r="C1039" t="n">
-        <v>97420</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1040">
@@ -11872,10 +11872,10 @@
         <v>46266</v>
       </c>
       <c r="B1040" t="n">
-        <v>1653</v>
+        <v>2345</v>
       </c>
       <c r="C1040" t="n">
-        <v>147720</v>
+        <v>31471</v>
       </c>
     </row>
     <row r="1041">
@@ -11883,10 +11883,10 @@
         <v>46266</v>
       </c>
       <c r="B1041" t="n">
-        <v>1293</v>
+        <v>2789</v>
       </c>
       <c r="C1041" t="n">
-        <v>188630</v>
+        <v>84997</v>
       </c>
     </row>
     <row r="1042">
@@ -11894,10 +11894,10 @@
         <v>46266</v>
       </c>
       <c r="B1042" t="n">
-        <v>360</v>
+        <v>569</v>
       </c>
       <c r="C1042" t="n">
-        <v>227270</v>
+        <v>1431958</v>
       </c>
     </row>
     <row r="1043">
@@ -11905,10 +11905,10 @@
         <v>46266</v>
       </c>
       <c r="B1043" t="n">
-        <v>1063</v>
+        <v>2822</v>
       </c>
       <c r="C1043" t="n">
-        <v>165250</v>
+        <v>67496</v>
       </c>
     </row>
     <row r="1044">
@@ -11916,10 +11916,10 @@
         <v>46266</v>
       </c>
       <c r="B1044" t="n">
-        <v>2273</v>
+        <v>2728</v>
       </c>
       <c r="C1044" t="n">
-        <v>96400</v>
+        <v>4994</v>
       </c>
     </row>
     <row r="1045">
@@ -11927,10 +11927,10 @@
         <v>46266</v>
       </c>
       <c r="B1045" t="n">
-        <v>2757</v>
+        <v>2488</v>
       </c>
       <c r="C1045" t="n">
-        <v>31818.28</v>
+        <v>49995</v>
       </c>
     </row>
     <row r="1046">
@@ -11938,10 +11938,10 @@
         <v>46266</v>
       </c>
       <c r="B1046" t="n">
-        <v>2795</v>
+        <v>2791</v>
       </c>
       <c r="C1046" t="n">
-        <v>27272.76</v>
+        <v>49345.1</v>
       </c>
     </row>
     <row r="1047">
@@ -11949,10 +11949,10 @@
         <v>46266</v>
       </c>
       <c r="B1047" t="n">
-        <v>2722</v>
+        <v>2577</v>
       </c>
       <c r="C1047" t="n">
-        <v>27270</v>
+        <v>44585.11</v>
       </c>
     </row>
     <row r="1048">
@@ -11960,10 +11960,10 @@
         <v>46266</v>
       </c>
       <c r="B1048" t="n">
-        <v>2718</v>
+        <v>2069</v>
       </c>
       <c r="C1048" t="n">
-        <v>36360</v>
+        <v>89991</v>
       </c>
     </row>
     <row r="1049">
@@ -11971,10 +11971,10 @@
         <v>46266</v>
       </c>
       <c r="B1049" t="n">
-        <v>595</v>
+        <v>2082</v>
       </c>
       <c r="C1049" t="n">
-        <v>250000</v>
+        <v>83281</v>
       </c>
     </row>
     <row r="1050">
@@ -11982,10 +11982,10 @@
         <v>46266</v>
       </c>
       <c r="B1050" t="n">
-        <v>890</v>
+        <v>781</v>
       </c>
       <c r="C1050" t="n">
-        <v>318180</v>
+        <v>64999</v>
       </c>
     </row>
     <row r="1051">
@@ -11993,10 +11993,10 @@
         <v>46266</v>
       </c>
       <c r="B1051" t="n">
-        <v>2652</v>
+        <v>744</v>
       </c>
       <c r="C1051" t="n">
-        <v>59090</v>
+        <v>20801</v>
       </c>
     </row>
     <row r="1052">
@@ -12004,10 +12004,10 @@
         <v>46266</v>
       </c>
       <c r="B1052" t="n">
-        <v>2714</v>
+        <v>2223</v>
       </c>
       <c r="C1052" t="n">
-        <v>163630</v>
+        <v>65967</v>
       </c>
     </row>
     <row r="1053">
@@ -12015,10 +12015,10 @@
         <v>46266</v>
       </c>
       <c r="B1053" t="n">
-        <v>1869</v>
+        <v>2452</v>
       </c>
       <c r="C1053" t="n">
-        <v>104540</v>
+        <v>34991</v>
       </c>
     </row>
     <row r="1054">
@@ -12026,10 +12026,10 @@
         <v>46266</v>
       </c>
       <c r="B1054" t="n">
-        <v>400</v>
+        <v>970</v>
       </c>
       <c r="C1054" t="n">
-        <v>86360</v>
+        <v>34342</v>
       </c>
     </row>
     <row r="1055">
@@ -12037,10 +12037,10 @@
         <v>46266</v>
       </c>
       <c r="B1055" t="n">
-        <v>1907</v>
+        <v>2550</v>
       </c>
       <c r="C1055" t="n">
-        <v>168630</v>
+        <v>30492</v>
       </c>
     </row>
     <row r="1056">
@@ -12048,10 +12048,10 @@
         <v>46266</v>
       </c>
       <c r="B1056" t="n">
-        <v>1996</v>
+        <v>768</v>
       </c>
       <c r="C1056" t="n">
-        <v>106590</v>
+        <v>64999</v>
       </c>
     </row>
     <row r="1057">
@@ -12059,10 +12059,10 @@
         <v>46266</v>
       </c>
       <c r="B1057" t="n">
-        <v>2114</v>
+        <v>1075</v>
       </c>
       <c r="C1057" t="n">
-        <v>83500</v>
+        <v>226490</v>
       </c>
     </row>
     <row r="1058">
@@ -12070,10 +12070,10 @@
         <v>46266</v>
       </c>
       <c r="B1058" t="n">
-        <v>2330</v>
+        <v>664</v>
       </c>
       <c r="C1058" t="n">
-        <v>122170</v>
+        <v>129492</v>
       </c>
     </row>
     <row r="1059">
@@ -12081,10 +12081,10 @@
         <v>46266</v>
       </c>
       <c r="B1059" t="n">
-        <v>2000</v>
+        <v>2555</v>
       </c>
       <c r="C1059" t="n">
-        <v>0</v>
+        <v>20757</v>
       </c>
     </row>
     <row r="1060">
@@ -12092,10 +12092,10 @@
         <v>46266</v>
       </c>
       <c r="B1060" t="n">
-        <v>2591</v>
+        <v>2627</v>
       </c>
       <c r="C1060" t="n">
-        <v>0</v>
+        <v>12188</v>
       </c>
     </row>
     <row r="1061">
@@ -12103,10 +12103,10 @@
         <v>46266</v>
       </c>
       <c r="B1061" t="n">
-        <v>2639</v>
+        <v>2557</v>
       </c>
       <c r="C1061" t="n">
-        <v>0</v>
+        <v>12892</v>
       </c>
     </row>
     <row r="1062">
@@ -12114,10 +12114,10 @@
         <v>46266</v>
       </c>
       <c r="B1062" t="n">
-        <v>947</v>
+        <v>2551</v>
       </c>
       <c r="C1062" t="n">
-        <v>197510</v>
+        <v>10241</v>
       </c>
     </row>
     <row r="1063">
@@ -12125,10 +12125,10 @@
         <v>46266</v>
       </c>
       <c r="B1063" t="n">
-        <v>1956</v>
+        <v>2463</v>
       </c>
       <c r="C1063" t="n">
-        <v>114760</v>
+        <v>160105</v>
       </c>
     </row>
     <row r="1064">
@@ -12136,10 +12136,10 @@
         <v>46266</v>
       </c>
       <c r="B1064" t="n">
-        <v>2824</v>
+        <v>2279</v>
       </c>
       <c r="C1064" t="n">
-        <v>50000</v>
+        <v>120791</v>
       </c>
     </row>
     <row r="1065">
@@ -12147,10 +12147,10 @@
         <v>46266</v>
       </c>
       <c r="B1065" t="n">
-        <v>2787</v>
+        <v>631</v>
       </c>
       <c r="C1065" t="n">
-        <v>59090</v>
+        <v>174999</v>
       </c>
     </row>
     <row r="1066">
@@ -12158,10 +12158,10 @@
         <v>46266</v>
       </c>
       <c r="B1066" t="n">
-        <v>2830</v>
+        <v>2251</v>
       </c>
       <c r="C1066" t="n">
-        <v>40900</v>
+        <v>107162</v>
       </c>
     </row>
     <row r="1067">
@@ -12169,10 +12169,10 @@
         <v>46266</v>
       </c>
       <c r="B1067" t="n">
-        <v>1254</v>
+        <v>1653</v>
       </c>
       <c r="C1067" t="n">
-        <v>88270.92</v>
+        <v>162492</v>
       </c>
     </row>
     <row r="1068">
@@ -12180,10 +12180,10 @@
         <v>46266</v>
       </c>
       <c r="B1068" t="n">
-        <v>1890</v>
+        <v>1293</v>
       </c>
       <c r="C1068" t="n">
-        <v>143701.31</v>
+        <v>207493</v>
       </c>
     </row>
     <row r="1069">
@@ -12191,10 +12191,10 @@
         <v>46266</v>
       </c>
       <c r="B1069" t="n">
-        <v>816</v>
+        <v>360</v>
       </c>
       <c r="C1069" t="n">
-        <v>121750</v>
+        <v>249997</v>
       </c>
     </row>
     <row r="1070">
@@ -12202,10 +12202,10 @@
         <v>46266</v>
       </c>
       <c r="B1070" t="n">
-        <v>2671</v>
+        <v>1063</v>
       </c>
       <c r="C1070" t="n">
-        <v>36360</v>
+        <v>181775</v>
       </c>
     </row>
     <row r="1071">
@@ -12213,10 +12213,10 @@
         <v>46266</v>
       </c>
       <c r="B1071" t="n">
-        <v>2705</v>
+        <v>2273</v>
       </c>
       <c r="C1071" t="n">
-        <v>81450</v>
+        <v>106040</v>
       </c>
     </row>
     <row r="1072">
@@ -12224,10 +12224,10 @@
         <v>46266</v>
       </c>
       <c r="B1072" t="n">
-        <v>2333</v>
+        <v>2757</v>
       </c>
       <c r="C1072" t="n">
-        <v>70160</v>
+        <v>35000.09</v>
       </c>
     </row>
     <row r="1073">
@@ -12235,10 +12235,10 @@
         <v>46266</v>
       </c>
       <c r="B1073" t="n">
-        <v>2440</v>
+        <v>2795</v>
       </c>
       <c r="C1073" t="n">
-        <v>40900</v>
+        <v>30000.03</v>
       </c>
     </row>
     <row r="1074">
@@ -12246,10 +12246,10 @@
         <v>46266</v>
       </c>
       <c r="B1074" t="n">
-        <v>2448</v>
+        <v>2722</v>
       </c>
       <c r="C1074" t="n">
-        <v>9090</v>
+        <v>29997</v>
       </c>
     </row>
     <row r="1075">
@@ -12257,10 +12257,10 @@
         <v>46266</v>
       </c>
       <c r="B1075" t="n">
-        <v>2310</v>
+        <v>2718</v>
       </c>
       <c r="C1075" t="n">
-        <v>31220</v>
+        <v>39996</v>
       </c>
     </row>
     <row r="1076">
@@ -12268,10 +12268,10 @@
         <v>46266</v>
       </c>
       <c r="B1076" t="n">
-        <v>2809</v>
+        <v>595</v>
       </c>
       <c r="C1076" t="n">
-        <v>31220</v>
+        <v>275000</v>
       </c>
     </row>
     <row r="1077">
@@ -12279,10 +12279,10 @@
         <v>46266</v>
       </c>
       <c r="B1077" t="n">
-        <v>1810</v>
+        <v>890</v>
       </c>
       <c r="C1077" t="n">
-        <v>18210</v>
+        <v>349998</v>
       </c>
     </row>
     <row r="1078">
@@ -12290,10 +12290,10 @@
         <v>46266</v>
       </c>
       <c r="B1078" t="n">
-        <v>2826</v>
+        <v>2652</v>
       </c>
       <c r="C1078" t="n">
-        <v>31818.28</v>
+        <v>64999</v>
       </c>
     </row>
     <row r="1079">
@@ -12301,10 +12301,10 @@
         <v>46266</v>
       </c>
       <c r="B1079" t="n">
-        <v>2561</v>
+        <v>2714</v>
       </c>
       <c r="C1079" t="n">
-        <v>6680</v>
+        <v>179993</v>
       </c>
     </row>
     <row r="1080">
@@ -12312,10 +12312,10 @@
         <v>46266</v>
       </c>
       <c r="B1080" t="n">
-        <v>2653</v>
+        <v>1869</v>
       </c>
       <c r="C1080" t="n">
-        <v>27272.76</v>
+        <v>114994</v>
       </c>
     </row>
     <row r="1081">
@@ -12323,10 +12323,10 @@
         <v>46266</v>
       </c>
       <c r="B1081" t="n">
-        <v>2829</v>
+        <v>400</v>
       </c>
       <c r="C1081" t="n">
-        <v>27272.76</v>
+        <v>94996</v>
       </c>
     </row>
     <row r="1082">
@@ -12334,10 +12334,10 @@
         <v>46266</v>
       </c>
       <c r="B1082" t="n">
-        <v>2643</v>
+        <v>1907</v>
       </c>
       <c r="C1082" t="n">
-        <v>13420</v>
+        <v>185493</v>
       </c>
     </row>
     <row r="1083">
@@ -12345,10 +12345,10 @@
         <v>46266</v>
       </c>
       <c r="B1083" t="n">
-        <v>2794</v>
+        <v>1996</v>
       </c>
       <c r="C1083" t="n">
-        <v>40900</v>
+        <v>117249</v>
       </c>
     </row>
     <row r="1084">
@@ -12356,10 +12356,10 @@
         <v>46266</v>
       </c>
       <c r="B1084" t="n">
-        <v>2655</v>
+        <v>2114</v>
       </c>
       <c r="C1084" t="n">
-        <v>50000</v>
+        <v>91850</v>
       </c>
     </row>
     <row r="1085">
@@ -12367,10 +12367,10 @@
         <v>46266</v>
       </c>
       <c r="B1085" t="n">
-        <v>1456</v>
+        <v>2330</v>
       </c>
       <c r="C1085" t="n">
-        <v>350130</v>
+        <v>134387</v>
       </c>
     </row>
     <row r="1086">
@@ -12378,10 +12378,10 @@
         <v>46266</v>
       </c>
       <c r="B1086" t="n">
-        <v>2606</v>
+        <v>2000</v>
       </c>
       <c r="C1086" t="n">
-        <v>107540</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1087">
@@ -12389,10 +12389,10 @@
         <v>46266</v>
       </c>
       <c r="B1087" t="n">
-        <v>1142</v>
+        <v>2591</v>
       </c>
       <c r="C1087" t="n">
-        <v>195020</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1088">
@@ -12400,10 +12400,10 @@
         <v>46266</v>
       </c>
       <c r="B1088" t="n">
-        <v>1450</v>
+        <v>2639</v>
       </c>
       <c r="C1088" t="n">
-        <v>123890</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1089">
@@ -12411,10 +12411,10 @@
         <v>46266</v>
       </c>
       <c r="B1089" t="n">
-        <v>2133</v>
+        <v>931</v>
       </c>
       <c r="C1089" t="n">
-        <v>289310</v>
+        <v>47212</v>
       </c>
     </row>
     <row r="1090">
@@ -12422,10 +12422,10 @@
         <v>46266</v>
       </c>
       <c r="B1090" t="n">
-        <v>522</v>
+        <v>947</v>
       </c>
       <c r="C1090" t="n">
-        <v>88630</v>
+        <v>217261</v>
       </c>
     </row>
     <row r="1091">
@@ -12433,10 +12433,10 @@
         <v>46266</v>
       </c>
       <c r="B1091" t="n">
-        <v>2696</v>
+        <v>951</v>
       </c>
       <c r="C1091" t="n">
-        <v>119600</v>
+        <v>57497</v>
       </c>
     </row>
     <row r="1092">
@@ -12444,10 +12444,10 @@
         <v>46266</v>
       </c>
       <c r="B1092" t="n">
-        <v>2693</v>
+        <v>2449</v>
       </c>
       <c r="C1092" t="n">
-        <v>0</v>
+        <v>19998</v>
       </c>
     </row>
     <row r="1093">
@@ -12455,10 +12455,10 @@
         <v>46266</v>
       </c>
       <c r="B1093" t="n">
-        <v>2692</v>
+        <v>610</v>
       </c>
       <c r="C1093" t="n">
-        <v>34090</v>
+        <v>407495</v>
       </c>
     </row>
     <row r="1094">
@@ -12466,10 +12466,10 @@
         <v>46266</v>
       </c>
       <c r="B1094" t="n">
-        <v>2691</v>
+        <v>2761</v>
       </c>
       <c r="C1094" t="n">
-        <v>61360</v>
+        <v>40744</v>
       </c>
     </row>
     <row r="1095">
@@ -12477,10 +12477,10 @@
         <v>46266</v>
       </c>
       <c r="B1095" t="n">
-        <v>1632</v>
+        <v>483</v>
       </c>
       <c r="C1095" t="n">
-        <v>113630</v>
+        <v>221496</v>
       </c>
     </row>
     <row r="1096">
@@ -12488,10 +12488,10 @@
         <v>46266</v>
       </c>
       <c r="B1096" t="n">
-        <v>2641</v>
+        <v>2015</v>
       </c>
       <c r="C1096" t="n">
-        <v>36360</v>
+        <v>184998</v>
       </c>
     </row>
     <row r="1097">
@@ -12499,10 +12499,10 @@
         <v>46266</v>
       </c>
       <c r="B1097" t="n">
-        <v>2197</v>
+        <v>1478</v>
       </c>
       <c r="C1097" t="n">
-        <v>90900</v>
+        <v>270578</v>
       </c>
     </row>
     <row r="1098">
@@ -12510,10 +12510,10 @@
         <v>46266</v>
       </c>
       <c r="B1098" t="n">
-        <v>609</v>
+        <v>424</v>
       </c>
       <c r="C1098" t="n">
-        <v>100000</v>
+        <v>120791</v>
       </c>
     </row>
     <row r="1099">
@@ -12521,10 +12521,10 @@
         <v>46266</v>
       </c>
       <c r="B1099" t="n">
-        <v>104</v>
+        <v>1261</v>
       </c>
       <c r="C1099" t="n">
-        <v>136360</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1100">
@@ -12532,10 +12532,10 @@
         <v>46266</v>
       </c>
       <c r="B1100" t="n">
-        <v>2621</v>
+        <v>477</v>
       </c>
       <c r="C1100" t="n">
-        <v>31810</v>
+        <v>129327</v>
       </c>
     </row>
     <row r="1101">
@@ -12543,10 +12543,10 @@
         <v>46266</v>
       </c>
       <c r="B1101" t="n">
-        <v>2786</v>
+        <v>1810</v>
       </c>
       <c r="C1101" t="n">
-        <v>31810</v>
+        <v>20031</v>
       </c>
     </row>
     <row r="1102">
@@ -12554,10 +12554,10 @@
         <v>46266</v>
       </c>
       <c r="B1102" t="n">
-        <v>2784</v>
+        <v>2826</v>
       </c>
       <c r="C1102" t="n">
-        <v>18910</v>
+        <v>35000.09</v>
       </c>
     </row>
     <row r="1103">
@@ -12565,10 +12565,10 @@
         <v>46266</v>
       </c>
       <c r="B1103" t="n">
-        <v>2586</v>
+        <v>2561</v>
       </c>
       <c r="C1103" t="n">
-        <v>18910</v>
+        <v>7348</v>
       </c>
     </row>
     <row r="1104">
@@ -12576,10 +12576,10 @@
         <v>46266</v>
       </c>
       <c r="B1104" t="n">
-        <v>2145</v>
+        <v>2653</v>
       </c>
       <c r="C1104" t="n">
-        <v>58840</v>
+        <v>30000.03</v>
       </c>
     </row>
     <row r="1105">
@@ -12587,10 +12587,10 @@
         <v>46266</v>
       </c>
       <c r="B1105" t="n">
-        <v>2574</v>
+        <v>2829</v>
       </c>
       <c r="C1105" t="n">
-        <v>58840</v>
+        <v>30000.03</v>
       </c>
     </row>
     <row r="1106">
@@ -12598,10 +12598,10 @@
         <v>46266</v>
       </c>
       <c r="B1106" t="n">
-        <v>2492</v>
+        <v>2643</v>
       </c>
       <c r="C1106" t="n">
-        <v>64500</v>
+        <v>14762</v>
       </c>
     </row>
     <row r="1107">
@@ -12609,10 +12609,10 @@
         <v>46266</v>
       </c>
       <c r="B1107" t="n">
-        <v>629</v>
+        <v>2794</v>
       </c>
       <c r="C1107" t="n">
-        <v>200900</v>
+        <v>44990</v>
       </c>
     </row>
     <row r="1108">
@@ -12620,10 +12620,10 @@
         <v>46266</v>
       </c>
       <c r="B1108" t="n">
-        <v>966</v>
+        <v>2655</v>
       </c>
       <c r="C1108" t="n">
-        <v>37040</v>
+        <v>55000</v>
       </c>
     </row>
     <row r="1109">
@@ -12631,10 +12631,10 @@
         <v>46266</v>
       </c>
       <c r="B1109" t="n">
-        <v>2721</v>
+        <v>1456</v>
       </c>
       <c r="C1109" t="n">
-        <v>37040</v>
+        <v>385143</v>
       </c>
     </row>
     <row r="1110">
@@ -12642,10 +12642,10 @@
         <v>46266</v>
       </c>
       <c r="B1110" t="n">
-        <v>2554</v>
+        <v>2606</v>
       </c>
       <c r="C1110" t="n">
-        <v>11160</v>
+        <v>118294</v>
       </c>
     </row>
     <row r="1111">
@@ -12653,10 +12653,10 @@
         <v>46266</v>
       </c>
       <c r="B1111" t="n">
-        <v>2556</v>
+        <v>1142</v>
       </c>
       <c r="C1111" t="n">
-        <v>16410</v>
+        <v>214522</v>
       </c>
     </row>
     <row r="1112">
@@ -12664,10 +12664,10 @@
         <v>46266</v>
       </c>
       <c r="B1112" t="n">
-        <v>2546</v>
+        <v>1450</v>
       </c>
       <c r="C1112" t="n">
-        <v>10840</v>
+        <v>136279</v>
       </c>
     </row>
     <row r="1113">
@@ -12675,10 +12675,10 @@
         <v>46266</v>
       </c>
       <c r="B1113" t="n">
-        <v>42</v>
+        <v>2133</v>
       </c>
       <c r="C1113" t="n">
-        <v>859090</v>
+        <v>318241</v>
       </c>
     </row>
     <row r="1114">
@@ -12686,10 +12686,10 @@
         <v>46266</v>
       </c>
       <c r="B1114" t="n">
-        <v>953</v>
+        <v>522</v>
       </c>
       <c r="C1114" t="n">
-        <v>310300</v>
+        <v>97493</v>
       </c>
     </row>
     <row r="1115">
@@ -12697,10 +12697,10 @@
         <v>46266</v>
       </c>
       <c r="B1115" t="n">
-        <v>675</v>
+        <v>2696</v>
       </c>
       <c r="C1115" t="n">
-        <v>90900</v>
+        <v>131560</v>
       </c>
     </row>
     <row r="1116">
@@ -12708,10 +12708,10 @@
         <v>46266</v>
       </c>
       <c r="B1116" t="n">
-        <v>619</v>
+        <v>2693</v>
       </c>
       <c r="C1116" t="n">
-        <v>140560</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1117">
@@ -12719,10 +12719,10 @@
         <v>46266</v>
       </c>
       <c r="B1117" t="n">
-        <v>1299</v>
+        <v>2692</v>
       </c>
       <c r="C1117" t="n">
-        <v>236520</v>
+        <v>37499</v>
       </c>
     </row>
     <row r="1118">
@@ -12730,10 +12730,10 @@
         <v>46266</v>
       </c>
       <c r="B1118" t="n">
-        <v>1064</v>
+        <v>2691</v>
       </c>
       <c r="C1118" t="n">
-        <v>272440</v>
+        <v>67496</v>
       </c>
     </row>
     <row r="1119">
@@ -12741,10 +12741,10 @@
         <v>46266</v>
       </c>
       <c r="B1119" t="n">
-        <v>2308</v>
+        <v>1632</v>
       </c>
       <c r="C1119" t="n">
-        <v>93180</v>
+        <v>124993</v>
       </c>
     </row>
     <row r="1120">
@@ -12752,10 +12752,10 @@
         <v>46266</v>
       </c>
       <c r="B1120" t="n">
-        <v>1137</v>
+        <v>2641</v>
       </c>
       <c r="C1120" t="n">
-        <v>290900</v>
+        <v>39996</v>
       </c>
     </row>
     <row r="1121">
@@ -12763,10 +12763,10 @@
         <v>46266</v>
       </c>
       <c r="B1121" t="n">
-        <v>2747</v>
+        <v>2197</v>
       </c>
       <c r="C1121" t="n">
-        <v>27272.76</v>
+        <v>99990</v>
       </c>
     </row>
     <row r="1122">
@@ -12774,10 +12774,10 @@
         <v>46266</v>
       </c>
       <c r="B1122" t="n">
-        <v>2819</v>
+        <v>609</v>
       </c>
       <c r="C1122" t="n">
-        <v>27272.76</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="1123">
@@ -12785,10 +12785,10 @@
         <v>46266</v>
       </c>
       <c r="B1123" t="n">
-        <v>1259</v>
+        <v>1380</v>
       </c>
       <c r="C1123" t="n">
-        <v>45454.6</v>
+        <v>49995</v>
       </c>
     </row>
     <row r="1124">
@@ -12796,10 +12796,10 @@
         <v>46266</v>
       </c>
       <c r="B1124" t="n">
-        <v>2544</v>
+        <v>104</v>
       </c>
       <c r="C1124" t="n">
-        <v>36360</v>
+        <v>149996</v>
       </c>
     </row>
     <row r="1125">
@@ -12807,10 +12807,10 @@
         <v>46266</v>
       </c>
       <c r="B1125" t="n">
-        <v>2261</v>
+        <v>2621</v>
       </c>
       <c r="C1125" t="n">
-        <v>68180</v>
+        <v>34991</v>
       </c>
     </row>
     <row r="1126">
@@ -12818,10 +12818,10 @@
         <v>46266</v>
       </c>
       <c r="B1126" t="n">
-        <v>2729</v>
+        <v>2786</v>
       </c>
       <c r="C1126" t="n">
-        <v>36360</v>
+        <v>34991</v>
       </c>
     </row>
     <row r="1127">
@@ -12829,10 +12829,10 @@
         <v>46266</v>
       </c>
       <c r="B1127" t="n">
-        <v>2649</v>
+        <v>2784</v>
       </c>
       <c r="C1127" t="n">
-        <v>13420</v>
+        <v>20801</v>
       </c>
     </row>
     <row r="1128">
@@ -12840,10 +12840,10 @@
         <v>46266</v>
       </c>
       <c r="B1128" t="n">
-        <v>2494</v>
+        <v>2586</v>
       </c>
       <c r="C1128" t="n">
-        <v>59090</v>
+        <v>20801</v>
       </c>
     </row>
     <row r="1129">
@@ -12851,10 +12851,10 @@
         <v>46266</v>
       </c>
       <c r="B1129" t="n">
-        <v>1384</v>
+        <v>2145</v>
       </c>
       <c r="C1129" t="n">
-        <v>204540</v>
+        <v>64724</v>
       </c>
     </row>
     <row r="1130">
@@ -12862,10 +12862,10 @@
         <v>46266</v>
       </c>
       <c r="B1130" t="n">
-        <v>634</v>
+        <v>2574</v>
       </c>
       <c r="C1130" t="n">
-        <v>250000</v>
+        <v>64724</v>
       </c>
     </row>
     <row r="1131">
@@ -12873,10 +12873,10 @@
         <v>46266</v>
       </c>
       <c r="B1131" t="n">
-        <v>2804</v>
+        <v>2492</v>
       </c>
       <c r="C1131" t="n">
-        <v>45450</v>
+        <v>70950</v>
       </c>
     </row>
     <row r="1132">
@@ -12884,10 +12884,10 @@
         <v>46266</v>
       </c>
       <c r="B1132" t="n">
-        <v>2375</v>
+        <v>629</v>
       </c>
       <c r="C1132" t="n">
-        <v>150000</v>
+        <v>220990</v>
       </c>
     </row>
     <row r="1133">
@@ -12895,10 +12895,10 @@
         <v>46266</v>
       </c>
       <c r="B1133" t="n">
-        <v>2601</v>
+        <v>966</v>
       </c>
       <c r="C1133" t="n">
-        <v>125000</v>
+        <v>40744</v>
       </c>
     </row>
     <row r="1134">
@@ -12906,10 +12906,10 @@
         <v>46266</v>
       </c>
       <c r="B1134" t="n">
-        <v>952</v>
+        <v>2721</v>
       </c>
       <c r="C1134" t="n">
-        <v>45450</v>
+        <v>40744</v>
       </c>
     </row>
     <row r="1135">
@@ -12917,10 +12917,10 @@
         <v>46266</v>
       </c>
       <c r="B1135" t="n">
-        <v>571</v>
+        <v>2554</v>
       </c>
       <c r="C1135" t="n">
-        <v>289310</v>
+        <v>12276</v>
       </c>
     </row>
     <row r="1136">
@@ -12928,10 +12928,10 @@
         <v>46266</v>
       </c>
       <c r="B1136" t="n">
-        <v>1380</v>
+        <v>2556</v>
       </c>
       <c r="C1136" t="n">
-        <v>45450</v>
+        <v>18051</v>
       </c>
     </row>
     <row r="1137">
@@ -12939,10 +12939,10 @@
         <v>46266</v>
       </c>
       <c r="B1137" t="n">
-        <v>2697</v>
+        <v>2546</v>
       </c>
       <c r="C1137" t="n">
-        <v>88150</v>
+        <v>11924</v>
       </c>
     </row>
     <row r="1138">
@@ -12950,10 +12950,10 @@
         <v>46266</v>
       </c>
       <c r="B1138" t="n">
-        <v>2678</v>
+        <v>42</v>
       </c>
       <c r="C1138" t="n">
-        <v>152510</v>
+        <v>944999</v>
       </c>
     </row>
     <row r="1139">
@@ -12961,10 +12961,10 @@
         <v>46266</v>
       </c>
       <c r="B1139" t="n">
-        <v>2768</v>
+        <v>953</v>
       </c>
       <c r="C1139" t="n">
-        <v>159610</v>
+        <v>341330</v>
       </c>
     </row>
     <row r="1140">
@@ -12972,10 +12972,10 @@
         <v>46266</v>
       </c>
       <c r="B1140" t="n">
-        <v>2359</v>
+        <v>675</v>
       </c>
       <c r="C1140" t="n">
-        <v>48410</v>
+        <v>99990</v>
       </c>
     </row>
     <row r="1141">
@@ -12983,10 +12983,10 @@
         <v>46266</v>
       </c>
       <c r="B1141" t="n">
-        <v>2811</v>
+        <v>619</v>
       </c>
       <c r="C1141" t="n">
-        <v>18910</v>
+        <v>154616</v>
       </c>
     </row>
     <row r="1142">
@@ -12994,10 +12994,10 @@
         <v>46266</v>
       </c>
       <c r="B1142" t="n">
-        <v>1871</v>
+        <v>1299</v>
       </c>
       <c r="C1142" t="n">
-        <v>80340</v>
+        <v>260172</v>
       </c>
     </row>
     <row r="1143">
@@ -13005,10 +13005,10 @@
         <v>46266</v>
       </c>
       <c r="B1143" t="n">
-        <v>2541</v>
+        <v>1064</v>
       </c>
       <c r="C1143" t="n">
-        <v>96180</v>
+        <v>299684</v>
       </c>
     </row>
     <row r="1144">
@@ -13016,10 +13016,10 @@
         <v>46266</v>
       </c>
       <c r="B1144" t="n">
-        <v>2362</v>
+        <v>2308</v>
       </c>
       <c r="C1144" t="n">
-        <v>34090</v>
+        <v>102498</v>
       </c>
     </row>
     <row r="1145">
@@ -13027,10 +13027,10 @@
         <v>46266</v>
       </c>
       <c r="B1145" t="n">
-        <v>1324</v>
+        <v>1137</v>
       </c>
       <c r="C1145" t="n">
-        <v>127270</v>
+        <v>319990</v>
       </c>
     </row>
     <row r="1146">
@@ -13038,10 +13038,10 @@
         <v>46266</v>
       </c>
       <c r="B1146" t="n">
-        <v>2323</v>
+        <v>2747</v>
       </c>
       <c r="C1146" t="n">
-        <v>31220</v>
+        <v>30000.03</v>
       </c>
     </row>
     <row r="1147">
@@ -13049,10 +13049,10 @@
         <v>46266</v>
       </c>
       <c r="B1147" t="n">
-        <v>2647</v>
+        <v>2819</v>
       </c>
       <c r="C1147" t="n">
-        <v>64500</v>
+        <v>30000.03</v>
       </c>
     </row>
     <row r="1148">
@@ -13060,10 +13060,10 @@
         <v>46266</v>
       </c>
       <c r="B1148" t="n">
-        <v>559</v>
+        <v>1259</v>
       </c>
       <c r="C1148" t="n">
-        <v>104290</v>
+        <v>50000.05</v>
       </c>
     </row>
     <row r="1149">
@@ -13071,10 +13071,10 @@
         <v>46266</v>
       </c>
       <c r="B1149" t="n">
-        <v>2762</v>
+        <v>2544</v>
       </c>
       <c r="C1149" t="n">
-        <v>37040</v>
+        <v>39996</v>
       </c>
     </row>
     <row r="1150">
@@ -13082,10 +13082,10 @@
         <v>46266</v>
       </c>
       <c r="B1150" t="n">
-        <v>2501</v>
+        <v>2261</v>
       </c>
       <c r="C1150" t="n">
-        <v>37040</v>
+        <v>74998</v>
       </c>
     </row>
     <row r="1151">
@@ -13093,10 +13093,10 @@
         <v>46266</v>
       </c>
       <c r="B1151" t="n">
-        <v>2562</v>
+        <v>2729</v>
       </c>
       <c r="C1151" t="n">
-        <v>7190</v>
+        <v>39996</v>
       </c>
     </row>
     <row r="1152">
@@ -13104,10 +13104,10 @@
         <v>46266</v>
       </c>
       <c r="B1152" t="n">
-        <v>429</v>
+        <v>2649</v>
       </c>
       <c r="C1152" t="n">
-        <v>177270</v>
+        <v>14762</v>
       </c>
     </row>
     <row r="1153">
@@ -13115,10 +13115,10 @@
         <v>46266</v>
       </c>
       <c r="B1153" t="n">
-        <v>58</v>
+        <v>2494</v>
       </c>
       <c r="C1153" t="n">
-        <v>122990</v>
+        <v>64999</v>
       </c>
     </row>
     <row r="1154">
@@ -13126,10 +13126,10 @@
         <v>46266</v>
       </c>
       <c r="B1154" t="n">
-        <v>2245</v>
+        <v>1384</v>
       </c>
       <c r="C1154" t="n">
-        <v>109810</v>
+        <v>224994</v>
       </c>
     </row>
     <row r="1155">
@@ -13137,10 +13137,10 @@
         <v>46266</v>
       </c>
       <c r="B1155" t="n">
-        <v>285</v>
+        <v>2633</v>
       </c>
       <c r="C1155" t="n">
-        <v>245980</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1156">
@@ -13148,10 +13148,10 @@
         <v>46266</v>
       </c>
       <c r="B1156" t="n">
-        <v>1464</v>
+        <v>2802</v>
       </c>
       <c r="C1156" t="n">
-        <v>0</v>
+        <v>35409</v>
       </c>
     </row>
     <row r="1157">
@@ -13159,10 +13159,10 @@
         <v>46266</v>
       </c>
       <c r="B1157" t="n">
-        <v>363</v>
+        <v>2726</v>
       </c>
       <c r="C1157" t="n">
-        <v>136360</v>
+        <v>74998</v>
       </c>
     </row>
     <row r="1158">
@@ -13170,10 +13170,10 @@
         <v>46266</v>
       </c>
       <c r="B1158" t="n">
-        <v>2651</v>
+        <v>2820</v>
       </c>
       <c r="C1158" t="n">
-        <v>76870</v>
+        <v>89991</v>
       </c>
     </row>
     <row r="1159">
@@ -13181,10 +13181,10 @@
         <v>46266</v>
       </c>
       <c r="B1159" t="n">
-        <v>2142</v>
+        <v>1007</v>
       </c>
       <c r="C1159" t="n">
-        <v>24260</v>
+        <v>94996</v>
       </c>
     </row>
     <row r="1160">
@@ -13192,10 +13192,10 @@
         <v>46266</v>
       </c>
       <c r="B1160" t="n">
-        <v>2258</v>
+        <v>20</v>
       </c>
       <c r="C1160" t="n">
-        <v>36363.68</v>
+        <v>192500</v>
       </c>
     </row>
     <row r="1161">
@@ -13203,10 +13203,10 @@
         <v>46266</v>
       </c>
       <c r="B1161" t="n">
-        <v>2772</v>
+        <v>1372</v>
       </c>
       <c r="C1161" t="n">
-        <v>27272.76</v>
+        <v>144991</v>
       </c>
     </row>
     <row r="1162">
@@ -13214,10 +13214,10 @@
         <v>46266</v>
       </c>
       <c r="B1162" t="n">
-        <v>2346</v>
+        <v>2735</v>
       </c>
       <c r="C1162" t="n">
-        <v>50000</v>
+        <v>59994</v>
       </c>
     </row>
     <row r="1163">
@@ -13225,10 +13225,10 @@
         <v>46266</v>
       </c>
       <c r="B1163" t="n">
-        <v>2442</v>
+        <v>2811</v>
       </c>
       <c r="C1163" t="n">
-        <v>36360</v>
+        <v>20801</v>
       </c>
     </row>
     <row r="1164">
@@ -13236,10 +13236,10 @@
         <v>46266</v>
       </c>
       <c r="B1164" t="n">
-        <v>772</v>
+        <v>1871</v>
       </c>
       <c r="C1164" t="n">
-        <v>150000</v>
+        <v>88374</v>
       </c>
     </row>
     <row r="1165">
@@ -13247,10 +13247,10 @@
         <v>46266</v>
       </c>
       <c r="B1165" t="n">
-        <v>2684</v>
+        <v>2541</v>
       </c>
       <c r="C1165" t="n">
-        <v>43180</v>
+        <v>105798</v>
       </c>
     </row>
     <row r="1166">
@@ -13258,10 +13258,10 @@
         <v>46266</v>
       </c>
       <c r="B1166" t="n">
-        <v>2765</v>
+        <v>2362</v>
       </c>
       <c r="C1166" t="n">
-        <v>40900</v>
+        <v>37499</v>
       </c>
     </row>
     <row r="1167">
@@ -13269,10 +13269,10 @@
         <v>46266</v>
       </c>
       <c r="B1167" t="n">
-        <v>2567</v>
+        <v>1324</v>
       </c>
       <c r="C1167" t="n">
-        <v>75020</v>
+        <v>139997</v>
       </c>
     </row>
     <row r="1168">
@@ -13280,10 +13280,10 @@
         <v>46266</v>
       </c>
       <c r="B1168" t="n">
-        <v>2178</v>
+        <v>2323</v>
       </c>
       <c r="C1168" t="n">
-        <v>127270</v>
+        <v>34342</v>
       </c>
     </row>
     <row r="1169">
@@ -13291,10 +13291,10 @@
         <v>46266</v>
       </c>
       <c r="B1169" t="n">
-        <v>2827</v>
+        <v>2647</v>
       </c>
       <c r="C1169" t="n">
-        <v>45450</v>
+        <v>70950</v>
       </c>
     </row>
     <row r="1170">
@@ -13302,10 +13302,10 @@
         <v>46266</v>
       </c>
       <c r="B1170" t="n">
-        <v>2510</v>
+        <v>559</v>
       </c>
       <c r="C1170" t="n">
-        <v>252380</v>
+        <v>114719</v>
       </c>
     </row>
     <row r="1171">
@@ -13313,10 +13313,10 @@
         <v>46266</v>
       </c>
       <c r="B1171" t="n">
-        <v>2392</v>
+        <v>2762</v>
       </c>
       <c r="C1171" t="n">
-        <v>75710</v>
+        <v>40744</v>
       </c>
     </row>
     <row r="1172">
@@ -13324,10 +13324,10 @@
         <v>46266</v>
       </c>
       <c r="B1172" t="n">
-        <v>415</v>
+        <v>2501</v>
       </c>
       <c r="C1172" t="n">
-        <v>258860</v>
+        <v>40744</v>
       </c>
     </row>
     <row r="1173">
@@ -13335,10 +13335,10 @@
         <v>46266</v>
       </c>
       <c r="B1173" t="n">
-        <v>2107</v>
+        <v>2562</v>
       </c>
       <c r="C1173" t="n">
-        <v>133670</v>
+        <v>7909</v>
       </c>
     </row>
     <row r="1174">
@@ -13346,10 +13346,10 @@
         <v>46266</v>
       </c>
       <c r="B1174" t="n">
-        <v>2211</v>
+        <v>429</v>
       </c>
       <c r="C1174" t="n">
-        <v>110820</v>
+        <v>194997</v>
       </c>
     </row>
     <row r="1175">
@@ -13357,10 +13357,10 @@
         <v>46266</v>
       </c>
       <c r="B1175" t="n">
-        <v>2682</v>
+        <v>58</v>
       </c>
       <c r="C1175" t="n">
-        <v>68170</v>
+        <v>135289</v>
       </c>
     </row>
     <row r="1176">
@@ -13368,10 +13368,10 @@
         <v>46266</v>
       </c>
       <c r="B1176" t="n">
-        <v>2781</v>
+        <v>2245</v>
       </c>
       <c r="C1176" t="n">
-        <v>0</v>
+        <v>120791</v>
       </c>
     </row>
     <row r="1177">
@@ -13379,10 +13379,10 @@
         <v>46266</v>
       </c>
       <c r="B1177" t="n">
-        <v>2576</v>
+        <v>285</v>
       </c>
       <c r="C1177" t="n">
-        <v>0</v>
+        <v>270578</v>
       </c>
     </row>
     <row r="1178">
@@ -13390,10 +13390,10 @@
         <v>46266</v>
       </c>
       <c r="B1178" t="n">
-        <v>2755</v>
+        <v>1464</v>
       </c>
       <c r="C1178" t="n">
-        <v>27270</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1179">
@@ -13401,10 +13401,10 @@
         <v>46266</v>
       </c>
       <c r="B1179" t="n">
-        <v>1289</v>
+        <v>363</v>
       </c>
       <c r="C1179" t="n">
-        <v>113630</v>
+        <v>149996</v>
       </c>
     </row>
     <row r="1180">
@@ -13412,10 +13412,10 @@
         <v>46266</v>
       </c>
       <c r="B1180" t="n">
-        <v>2801</v>
+        <v>2651</v>
       </c>
       <c r="C1180" t="n">
-        <v>36360</v>
+        <v>84557</v>
       </c>
     </row>
     <row r="1181">
@@ -13423,10 +13423,10 @@
         <v>46266</v>
       </c>
       <c r="B1181" t="n">
-        <v>2810</v>
+        <v>2142</v>
       </c>
       <c r="C1181" t="n">
-        <v>61360</v>
+        <v>26686</v>
       </c>
     </row>
     <row r="1182">
@@ -13434,10 +13434,10 @@
         <v>46266</v>
       </c>
       <c r="B1182" t="n">
-        <v>767</v>
+        <v>2258</v>
       </c>
       <c r="C1182" t="n">
-        <v>81810</v>
+        <v>40000.04</v>
       </c>
     </row>
     <row r="1183">
@@ -13445,10 +13445,10 @@
         <v>46266</v>
       </c>
       <c r="B1183" t="n">
-        <v>2687</v>
+        <v>2772</v>
       </c>
       <c r="C1183" t="n">
-        <v>45450</v>
+        <v>30000.03</v>
       </c>
     </row>
     <row r="1184">
@@ -13456,10 +13456,10 @@
         <v>46266</v>
       </c>
       <c r="B1184" t="n">
-        <v>2686</v>
+        <v>2346</v>
       </c>
       <c r="C1184" t="n">
-        <v>59090</v>
+        <v>55000</v>
       </c>
     </row>
     <row r="1185">
@@ -13467,10 +13467,10 @@
         <v>46266</v>
       </c>
       <c r="B1185" t="n">
-        <v>2730</v>
+        <v>2442</v>
       </c>
       <c r="C1185" t="n">
-        <v>40900</v>
+        <v>39996</v>
       </c>
     </row>
     <row r="1186">
@@ -13478,10 +13478,10 @@
         <v>46266</v>
       </c>
       <c r="B1186" t="n">
-        <v>2580</v>
+        <v>772</v>
       </c>
       <c r="C1186" t="n">
-        <v>15250</v>
+        <v>165000</v>
       </c>
     </row>
     <row r="1187">
@@ -13489,10 +13489,10 @@
         <v>46266</v>
       </c>
       <c r="B1187" t="n">
-        <v>2472</v>
+        <v>2684</v>
       </c>
       <c r="C1187" t="n">
-        <v>24064.6</v>
+        <v>47498</v>
       </c>
     </row>
     <row r="1188">
@@ -13500,10 +13500,10 @@
         <v>46266</v>
       </c>
       <c r="B1188" t="n">
-        <v>2631</v>
+        <v>2765</v>
       </c>
       <c r="C1188" t="n">
-        <v>11150.92</v>
+        <v>44990</v>
       </c>
     </row>
     <row r="1189">
@@ -13511,10 +13511,10 @@
         <v>46266</v>
       </c>
       <c r="B1189" t="n">
-        <v>1642</v>
+        <v>2567</v>
       </c>
       <c r="C1189" t="n">
-        <v>120450</v>
+        <v>82522</v>
       </c>
     </row>
     <row r="1190">
@@ -13522,10 +13522,10 @@
         <v>46266</v>
       </c>
       <c r="B1190" t="n">
-        <v>2613</v>
+        <v>2178</v>
       </c>
       <c r="C1190" t="n">
-        <v>81450</v>
+        <v>139997</v>
       </c>
     </row>
     <row r="1191">
@@ -13533,10 +13533,10 @@
         <v>46266</v>
       </c>
       <c r="B1191" t="n">
-        <v>1020</v>
+        <v>2827</v>
       </c>
       <c r="C1191" t="n">
-        <v>40900</v>
+        <v>49995</v>
       </c>
     </row>
     <row r="1192">
@@ -13544,10 +13544,10 @@
         <v>46266</v>
       </c>
       <c r="B1192" t="n">
-        <v>2785</v>
+        <v>2510</v>
       </c>
       <c r="C1192" t="n">
-        <v>18910</v>
+        <v>277618</v>
       </c>
     </row>
     <row r="1193">
@@ -13555,10 +13555,10 @@
         <v>46266</v>
       </c>
       <c r="B1193" t="n">
-        <v>1327</v>
+        <v>2392</v>
       </c>
       <c r="C1193" t="n">
-        <v>27270</v>
+        <v>83281</v>
       </c>
     </row>
     <row r="1194">
@@ -13566,10 +13566,10 @@
         <v>46266</v>
       </c>
       <c r="B1194" t="n">
-        <v>2629</v>
+        <v>415</v>
       </c>
       <c r="C1194" t="n">
-        <v>31220</v>
+        <v>284746</v>
       </c>
     </row>
     <row r="1195">
@@ -13577,10 +13577,10 @@
         <v>46266</v>
       </c>
       <c r="B1195" t="n">
-        <v>951</v>
+        <v>2107</v>
       </c>
       <c r="C1195" t="n">
-        <v>52270</v>
+        <v>147037</v>
       </c>
     </row>
     <row r="1196">
@@ -13588,10 +13588,10 @@
         <v>46266</v>
       </c>
       <c r="B1196" t="n">
-        <v>2449</v>
+        <v>2211</v>
       </c>
       <c r="C1196" t="n">
-        <v>18180</v>
+        <v>121902</v>
       </c>
     </row>
     <row r="1197">
@@ -13599,10 +13599,10 @@
         <v>46266</v>
       </c>
       <c r="B1197" t="n">
-        <v>610</v>
+        <v>2682</v>
       </c>
       <c r="C1197" t="n">
-        <v>370450</v>
+        <v>74987</v>
       </c>
     </row>
     <row r="1198">
@@ -13610,10 +13610,10 @@
         <v>46266</v>
       </c>
       <c r="B1198" t="n">
-        <v>2761</v>
+        <v>2781</v>
       </c>
       <c r="C1198" t="n">
-        <v>37040</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1199">
@@ -13621,10 +13621,10 @@
         <v>46266</v>
       </c>
       <c r="B1199" t="n">
-        <v>483</v>
+        <v>2576</v>
       </c>
       <c r="C1199" t="n">
-        <v>201360</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1200">
@@ -13632,10 +13632,10 @@
         <v>46266</v>
       </c>
       <c r="B1200" t="n">
-        <v>2015</v>
+        <v>2755</v>
       </c>
       <c r="C1200" t="n">
-        <v>168180</v>
+        <v>29997</v>
       </c>
     </row>
     <row r="1201">
@@ -13643,10 +13643,10 @@
         <v>46266</v>
       </c>
       <c r="B1201" t="n">
-        <v>1478</v>
+        <v>941</v>
       </c>
       <c r="C1201" t="n">
-        <v>245980</v>
+        <v>196438</v>
       </c>
     </row>
     <row r="1202">
@@ -13654,10 +13654,10 @@
         <v>46266</v>
       </c>
       <c r="B1202" t="n">
-        <v>424</v>
+        <v>2734</v>
       </c>
       <c r="C1202" t="n">
-        <v>109810</v>
+        <v>27533</v>
       </c>
     </row>
     <row r="1203">
@@ -13665,10 +13665,10 @@
         <v>46266</v>
       </c>
       <c r="B1203" t="n">
-        <v>1261</v>
+        <v>1289</v>
       </c>
       <c r="C1203" t="n">
-        <v>0</v>
+        <v>124993</v>
       </c>
     </row>
     <row r="1204">
@@ -13676,10 +13676,10 @@
         <v>46266</v>
       </c>
       <c r="B1204" t="n">
-        <v>477</v>
+        <v>2801</v>
       </c>
       <c r="C1204" t="n">
-        <v>117570</v>
+        <v>39996</v>
       </c>
     </row>
     <row r="1205">
@@ -13687,10 +13687,10 @@
         <v>46266</v>
       </c>
       <c r="B1205" t="n">
-        <v>1102</v>
+        <v>2810</v>
       </c>
       <c r="C1205" t="n">
-        <v>109810</v>
+        <v>67496</v>
       </c>
     </row>
     <row r="1206">
@@ -13698,10 +13698,10 @@
         <v>46266</v>
       </c>
       <c r="B1206" t="n">
-        <v>626</v>
+        <v>767</v>
       </c>
       <c r="C1206" t="n">
-        <v>774688.6800000001</v>
+        <v>89991</v>
       </c>
     </row>
     <row r="1207">
@@ -13709,10 +13709,10 @@
         <v>46266</v>
       </c>
       <c r="B1207" t="n">
-        <v>1465</v>
+        <v>2687</v>
       </c>
       <c r="C1207" t="n">
-        <v>163540</v>
+        <v>49995</v>
       </c>
     </row>
     <row r="1208">
@@ -13720,10 +13720,10 @@
         <v>46266</v>
       </c>
       <c r="B1208" t="n">
-        <v>2758</v>
+        <v>2686</v>
       </c>
       <c r="C1208" t="n">
-        <v>27272.76</v>
+        <v>64999</v>
       </c>
     </row>
     <row r="1209">
@@ -13731,10 +13731,10 @@
         <v>46266</v>
       </c>
       <c r="B1209" t="n">
-        <v>2742</v>
+        <v>2730</v>
       </c>
       <c r="C1209" t="n">
-        <v>27272.76</v>
+        <v>44990</v>
       </c>
     </row>
     <row r="1210">
@@ -13742,10 +13742,10 @@
         <v>46266</v>
       </c>
       <c r="B1210" t="n">
-        <v>2748</v>
+        <v>2580</v>
       </c>
       <c r="C1210" t="n">
-        <v>0</v>
+        <v>16775</v>
       </c>
     </row>
     <row r="1211">
@@ -13753,10 +13753,10 @@
         <v>46266</v>
       </c>
       <c r="B1211" t="n">
-        <v>1873</v>
+        <v>2472</v>
       </c>
       <c r="C1211" t="n">
-        <v>145450</v>
+        <v>26471.05</v>
       </c>
     </row>
     <row r="1212">
@@ -13764,10 +13764,10 @@
         <v>46266</v>
       </c>
       <c r="B1212" t="n">
-        <v>2163</v>
+        <v>2631</v>
       </c>
       <c r="C1212" t="n">
-        <v>68180</v>
+        <v>12266.01</v>
       </c>
     </row>
     <row r="1213">
@@ -13775,10 +13775,10 @@
         <v>46266</v>
       </c>
       <c r="B1213" t="n">
-        <v>2394</v>
+        <v>1642</v>
       </c>
       <c r="C1213" t="n">
-        <v>70020</v>
+        <v>132495</v>
       </c>
     </row>
     <row r="1214">
@@ -13786,10 +13786,10 @@
         <v>46266</v>
       </c>
       <c r="B1214" t="n">
-        <v>33</v>
+        <v>2613</v>
       </c>
       <c r="C1214" t="n">
-        <v>176360</v>
+        <v>89595</v>
       </c>
     </row>
     <row r="1215">
@@ -13797,10 +13797,10 @@
         <v>46266</v>
       </c>
       <c r="B1215" t="n">
-        <v>2421</v>
+        <v>1020</v>
       </c>
       <c r="C1215" t="n">
-        <v>29540</v>
+        <v>44990</v>
       </c>
     </row>
     <row r="1216">
@@ -13808,10 +13808,10 @@
         <v>46266</v>
       </c>
       <c r="B1216" t="n">
-        <v>2663</v>
+        <v>2785</v>
       </c>
       <c r="C1216" t="n">
-        <v>125000</v>
+        <v>20801</v>
       </c>
     </row>
     <row r="1217">
@@ -13819,10 +13819,10 @@
         <v>46266</v>
       </c>
       <c r="B1217" t="n">
-        <v>2413</v>
+        <v>1327</v>
       </c>
       <c r="C1217" t="n">
-        <v>55020</v>
+        <v>29997</v>
       </c>
     </row>
     <row r="1218">
@@ -13830,10 +13830,10 @@
         <v>46266</v>
       </c>
       <c r="B1218" t="n">
-        <v>351</v>
+        <v>2629</v>
       </c>
       <c r="C1218" t="n">
-        <v>83630</v>
+        <v>34342</v>
       </c>
     </row>
     <row r="1219">
@@ -13841,10 +13841,10 @@
         <v>46266</v>
       </c>
       <c r="B1219" t="n">
-        <v>1298</v>
+        <v>749</v>
       </c>
       <c r="C1219" t="n">
-        <v>578630</v>
+        <v>40744</v>
       </c>
     </row>
     <row r="1220">
@@ -13852,10 +13852,10 @@
         <v>46266</v>
       </c>
       <c r="B1220" t="n">
-        <v>2491</v>
+        <v>1983</v>
       </c>
       <c r="C1220" t="n">
-        <v>46760</v>
+        <v>270578</v>
       </c>
     </row>
     <row r="1221">
@@ -13863,10 +13863,10 @@
         <v>46266</v>
       </c>
       <c r="B1221" t="n">
-        <v>2571</v>
+        <v>1993</v>
       </c>
       <c r="C1221" t="n">
-        <v>66030</v>
+        <v>173943</v>
       </c>
     </row>
     <row r="1222">
@@ -13874,10 +13874,10 @@
         <v>46266</v>
       </c>
       <c r="B1222" t="n">
-        <v>2507</v>
+        <v>2767</v>
       </c>
       <c r="C1222" t="n">
-        <v>40120</v>
+        <v>96459</v>
       </c>
     </row>
     <row r="1223">
@@ -13885,10 +13885,10 @@
         <v>46266</v>
       </c>
       <c r="B1223" t="n">
-        <v>2799</v>
+        <v>2646</v>
       </c>
       <c r="C1223" t="n">
-        <v>51640</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1224">
@@ -13896,10 +13896,10 @@
         <v>46266</v>
       </c>
       <c r="B1224" t="n">
-        <v>2253</v>
+        <v>1102</v>
       </c>
       <c r="C1224" t="n">
-        <v>0</v>
+        <v>120791</v>
       </c>
     </row>
     <row r="1225">
@@ -13907,10 +13907,10 @@
         <v>46266</v>
       </c>
       <c r="B1225" t="n">
-        <v>630</v>
+        <v>626</v>
       </c>
       <c r="C1225" t="n">
-        <v>68040</v>
+        <v>852157.54</v>
       </c>
     </row>
     <row r="1226">
@@ -13918,10 +13918,10 @@
         <v>46266</v>
       </c>
       <c r="B1226" t="n">
-        <v>525</v>
+        <v>1465</v>
       </c>
       <c r="C1226" t="n">
-        <v>102270</v>
+        <v>179894</v>
       </c>
     </row>
     <row r="1227">
@@ -13929,10 +13929,10 @@
         <v>46266</v>
       </c>
       <c r="B1227" t="n">
-        <v>2727</v>
+        <v>2758</v>
       </c>
       <c r="C1227" t="n">
-        <v>18400</v>
+        <v>30000.03</v>
       </c>
     </row>
     <row r="1228">
@@ -13940,10 +13940,10 @@
         <v>46266</v>
       </c>
       <c r="B1228" t="n">
-        <v>2707</v>
+        <v>2742</v>
       </c>
       <c r="C1228" t="n">
-        <v>14560</v>
+        <v>30000.03</v>
       </c>
     </row>
     <row r="1229">
@@ -13951,10 +13951,10 @@
         <v>46266</v>
       </c>
       <c r="B1229" t="n">
-        <v>2834</v>
+        <v>2748</v>
       </c>
       <c r="C1229" t="n">
-        <v>7521.84</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1230">
@@ -13962,10 +13962,10 @@
         <v>46266</v>
       </c>
       <c r="B1230" t="n">
-        <v>2773</v>
+        <v>1873</v>
       </c>
       <c r="C1230" t="n">
-        <v>36678.28</v>
+        <v>159995</v>
       </c>
     </row>
     <row r="1231">
@@ -13973,10 +13973,10 @@
         <v>46266</v>
       </c>
       <c r="B1231" t="n">
-        <v>2341</v>
+        <v>2163</v>
       </c>
       <c r="C1231" t="n">
-        <v>64500</v>
+        <v>74998</v>
       </c>
     </row>
     <row r="1232">
@@ -13984,10 +13984,10 @@
         <v>46266</v>
       </c>
       <c r="B1232" t="n">
-        <v>1374</v>
+        <v>2394</v>
       </c>
       <c r="C1232" t="n">
-        <v>81810</v>
+        <v>77022</v>
       </c>
     </row>
     <row r="1233">
@@ -13995,10 +13995,10 @@
         <v>46266</v>
       </c>
       <c r="B1233" t="n">
-        <v>793</v>
+        <v>33</v>
       </c>
       <c r="C1233" t="n">
-        <v>18910</v>
+        <v>193996</v>
       </c>
     </row>
     <row r="1234">
@@ -14006,10 +14006,10 @@
         <v>46266</v>
       </c>
       <c r="B1234" t="n">
-        <v>794</v>
+        <v>2421</v>
       </c>
       <c r="C1234" t="n">
-        <v>18910</v>
+        <v>32494</v>
       </c>
     </row>
     <row r="1235">
@@ -14017,10 +14017,10 @@
         <v>46266</v>
       </c>
       <c r="B1235" t="n">
-        <v>1834</v>
+        <v>2663</v>
       </c>
       <c r="C1235" t="n">
-        <v>53180</v>
+        <v>137500</v>
       </c>
     </row>
     <row r="1236">
@@ -14028,10 +14028,10 @@
         <v>46266</v>
       </c>
       <c r="B1236" t="n">
-        <v>802</v>
+        <v>2413</v>
       </c>
       <c r="C1236" t="n">
-        <v>34090</v>
+        <v>60522</v>
       </c>
     </row>
     <row r="1237">
@@ -14039,10 +14039,10 @@
         <v>46266</v>
       </c>
       <c r="B1237" t="n">
-        <v>1344</v>
+        <v>351</v>
       </c>
       <c r="C1237" t="n">
-        <v>68180</v>
+        <v>91993</v>
       </c>
     </row>
     <row r="1238">
@@ -14050,10 +14050,10 @@
         <v>46266</v>
       </c>
       <c r="B1238" t="n">
-        <v>1881</v>
+        <v>1298</v>
       </c>
       <c r="C1238" t="n">
-        <v>31220</v>
+        <v>636493</v>
       </c>
     </row>
     <row r="1239">
@@ -14061,10 +14061,10 @@
         <v>46266</v>
       </c>
       <c r="B1239" t="n">
-        <v>2365</v>
+        <v>2491</v>
       </c>
       <c r="C1239" t="n">
-        <v>36210</v>
+        <v>51436</v>
       </c>
     </row>
     <row r="1240">
@@ -14072,10 +14072,10 @@
         <v>46266</v>
       </c>
       <c r="B1240" t="n">
-        <v>2411</v>
+        <v>2571</v>
       </c>
       <c r="C1240" t="n">
-        <v>64500</v>
+        <v>72633</v>
       </c>
     </row>
     <row r="1241">
@@ -14083,10 +14083,10 @@
         <v>46266</v>
       </c>
       <c r="B1241" t="n">
-        <v>2363</v>
+        <v>2507</v>
       </c>
       <c r="C1241" t="n">
-        <v>68180</v>
+        <v>44132</v>
       </c>
     </row>
     <row r="1242">
@@ -14094,10 +14094,10 @@
         <v>46266</v>
       </c>
       <c r="B1242" t="n">
-        <v>2124</v>
+        <v>2799</v>
       </c>
       <c r="C1242" t="n">
-        <v>159090</v>
+        <v>56804</v>
       </c>
     </row>
     <row r="1243">
@@ -14105,10 +14105,10 @@
         <v>46266</v>
       </c>
       <c r="B1243" t="n">
-        <v>1937</v>
+        <v>2253</v>
       </c>
       <c r="C1243" t="n">
-        <v>115900</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1244">
@@ -14116,10 +14116,10 @@
         <v>46266</v>
       </c>
       <c r="B1244" t="n">
-        <v>2709</v>
+        <v>2582</v>
       </c>
       <c r="C1244" t="n">
-        <v>81810</v>
+        <v>43274</v>
       </c>
     </row>
     <row r="1245">
@@ -14127,10 +14127,10 @@
         <v>46266</v>
       </c>
       <c r="B1245" t="n">
-        <v>2558</v>
+        <v>2637</v>
       </c>
       <c r="C1245" t="n">
-        <v>13660</v>
+        <v>31471</v>
       </c>
     </row>
     <row r="1246">
@@ -14138,10 +14138,10 @@
         <v>46266</v>
       </c>
       <c r="B1246" t="n">
-        <v>663</v>
+        <v>630</v>
       </c>
       <c r="C1246" t="n">
-        <v>115900</v>
+        <v>74844</v>
       </c>
     </row>
     <row r="1247">
@@ -14149,10 +14149,10 @@
         <v>46266</v>
       </c>
       <c r="B1247" t="n">
-        <v>40</v>
+        <v>525</v>
       </c>
       <c r="C1247" t="n">
-        <v>100000</v>
+        <v>112497</v>
       </c>
     </row>
     <row r="1248">
@@ -14160,10 +14160,10 @@
         <v>46266</v>
       </c>
       <c r="B1248" t="n">
-        <v>2833</v>
+        <v>2727</v>
       </c>
       <c r="C1248" t="n">
-        <v>31818.28</v>
+        <v>20240</v>
       </c>
     </row>
     <row r="1249">
@@ -14171,10 +14171,10 @@
         <v>46266</v>
       </c>
       <c r="B1249" t="n">
-        <v>1756</v>
+        <v>2707</v>
       </c>
       <c r="C1249" t="n">
-        <v>198410</v>
+        <v>16016</v>
       </c>
     </row>
     <row r="1250">
@@ -14182,10 +14182,10 @@
         <v>46266</v>
       </c>
       <c r="B1250" t="n">
-        <v>1116</v>
+        <v>2834</v>
       </c>
       <c r="C1250" t="n">
-        <v>115290</v>
+        <v>8274.02</v>
       </c>
     </row>
     <row r="1251">
@@ -14193,10 +14193,10 @@
         <v>46266</v>
       </c>
       <c r="B1251" t="n">
-        <v>636</v>
+        <v>2773</v>
       </c>
       <c r="C1251" t="n">
-        <v>113630</v>
+        <v>40346.09</v>
       </c>
     </row>
     <row r="1252">
@@ -14204,10 +14204,10 @@
         <v>46266</v>
       </c>
       <c r="B1252" t="n">
-        <v>1800</v>
+        <v>2341</v>
       </c>
       <c r="C1252" t="n">
-        <v>12720</v>
+        <v>70950</v>
       </c>
     </row>
     <row r="1253">
@@ -14215,10 +14215,10 @@
         <v>46266</v>
       </c>
       <c r="B1253" t="n">
-        <v>2815</v>
+        <v>1374</v>
       </c>
       <c r="C1253" t="n">
-        <v>27272.76</v>
+        <v>89991</v>
       </c>
     </row>
     <row r="1254">
@@ -14226,10 +14226,10 @@
         <v>46266</v>
       </c>
       <c r="B1254" t="n">
-        <v>1658</v>
+        <v>793</v>
       </c>
       <c r="C1254" t="n">
-        <v>60000</v>
+        <v>20801</v>
       </c>
     </row>
     <row r="1255">
@@ -14237,10 +14237,10 @@
         <v>46266</v>
       </c>
       <c r="B1255" t="n">
-        <v>2635</v>
+        <v>794</v>
       </c>
       <c r="C1255" t="n">
-        <v>59090</v>
+        <v>20801</v>
       </c>
     </row>
     <row r="1256">
@@ -14248,10 +14248,10 @@
         <v>46266</v>
       </c>
       <c r="B1256" t="n">
-        <v>2402</v>
+        <v>1834</v>
       </c>
       <c r="C1256" t="n">
-        <v>296360</v>
+        <v>58498</v>
       </c>
     </row>
     <row r="1257">
@@ -14259,10 +14259,10 @@
         <v>46266</v>
       </c>
       <c r="B1257" t="n">
-        <v>452</v>
+        <v>802</v>
       </c>
       <c r="C1257" t="n">
-        <v>122720</v>
+        <v>37499</v>
       </c>
     </row>
     <row r="1258">
@@ -14270,10 +14270,10 @@
         <v>46266</v>
       </c>
       <c r="B1258" t="n">
-        <v>2085</v>
+        <v>1344</v>
       </c>
       <c r="C1258" t="n">
-        <v>60020</v>
+        <v>74998</v>
       </c>
     </row>
     <row r="1259">
@@ -14281,10 +14281,10 @@
         <v>46266</v>
       </c>
       <c r="B1259" t="n">
-        <v>2568</v>
+        <v>1881</v>
       </c>
       <c r="C1259" t="n">
-        <v>92920</v>
+        <v>34342</v>
       </c>
     </row>
     <row r="1260">
@@ -14292,10 +14292,10 @@
         <v>46266</v>
       </c>
       <c r="B1260" t="n">
-        <v>1906</v>
+        <v>2365</v>
       </c>
       <c r="C1260" t="n">
-        <v>52740</v>
+        <v>39831</v>
       </c>
     </row>
     <row r="1261">
@@ -14303,10 +14303,10 @@
         <v>46266</v>
       </c>
       <c r="B1261" t="n">
-        <v>2821</v>
+        <v>2411</v>
       </c>
       <c r="C1261" t="n">
-        <v>45860</v>
+        <v>70950</v>
       </c>
     </row>
     <row r="1262">
@@ -14314,10 +14314,10 @@
         <v>46266</v>
       </c>
       <c r="B1262" t="n">
-        <v>2633</v>
+        <v>2363</v>
       </c>
       <c r="C1262" t="n">
-        <v>0</v>
+        <v>74998</v>
       </c>
     </row>
     <row r="1263">
@@ -14325,10 +14325,10 @@
         <v>46266</v>
       </c>
       <c r="B1263" t="n">
-        <v>2726</v>
+        <v>2124</v>
       </c>
       <c r="C1263" t="n">
-        <v>68180</v>
+        <v>174999</v>
       </c>
     </row>
     <row r="1264">
@@ -14336,10 +14336,10 @@
         <v>46266</v>
       </c>
       <c r="B1264" t="n">
-        <v>2820</v>
+        <v>1937</v>
       </c>
       <c r="C1264" t="n">
-        <v>81810</v>
+        <v>127490</v>
       </c>
     </row>
     <row r="1265">
@@ -14347,10 +14347,10 @@
         <v>46266</v>
       </c>
       <c r="B1265" t="n">
-        <v>1007</v>
+        <v>2709</v>
       </c>
       <c r="C1265" t="n">
-        <v>86360</v>
+        <v>89991</v>
       </c>
     </row>
     <row r="1266">
@@ -14358,10 +14358,10 @@
         <v>46266</v>
       </c>
       <c r="B1266" t="n">
-        <v>20</v>
+        <v>2558</v>
       </c>
       <c r="C1266" t="n">
-        <v>175000</v>
+        <v>15026</v>
       </c>
     </row>
     <row r="1267">
@@ -14369,10 +14369,10 @@
         <v>46266</v>
       </c>
       <c r="B1267" t="n">
-        <v>1372</v>
+        <v>663</v>
       </c>
       <c r="C1267" t="n">
-        <v>131810</v>
+        <v>127490</v>
       </c>
     </row>
     <row r="1268">
@@ -14380,10 +14380,10 @@
         <v>46266</v>
       </c>
       <c r="B1268" t="n">
-        <v>2735</v>
+        <v>40</v>
       </c>
       <c r="C1268" t="n">
-        <v>54540</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="1269">
@@ -14391,10 +14391,10 @@
         <v>46266</v>
       </c>
       <c r="B1269" t="n">
-        <v>2698</v>
+        <v>2833</v>
       </c>
       <c r="C1269" t="n">
-        <v>56210</v>
+        <v>35000.09</v>
       </c>
     </row>
     <row r="1270">
@@ -14402,10 +14402,10 @@
         <v>46266</v>
       </c>
       <c r="B1270" t="n">
-        <v>2118</v>
+        <v>1756</v>
       </c>
       <c r="C1270" t="n">
-        <v>107800</v>
+        <v>218251</v>
       </c>
     </row>
     <row r="1271">
@@ -14413,10 +14413,10 @@
         <v>46266</v>
       </c>
       <c r="B1271" t="n">
-        <v>2383</v>
+        <v>1116</v>
       </c>
       <c r="C1271" t="n">
-        <v>62940</v>
+        <v>126819</v>
       </c>
     </row>
     <row r="1272">
@@ -14424,10 +14424,10 @@
         <v>46266</v>
       </c>
       <c r="B1272" t="n">
-        <v>2831</v>
+        <v>636</v>
       </c>
       <c r="C1272" t="n">
-        <v>27270</v>
+        <v>124993</v>
       </c>
     </row>
     <row r="1273">
@@ -14435,10 +14435,10 @@
         <v>46266</v>
       </c>
       <c r="B1273" t="n">
-        <v>2045</v>
+        <v>1800</v>
       </c>
       <c r="C1273" t="n">
-        <v>152934.46</v>
+        <v>13992</v>
       </c>
     </row>
     <row r="1274">
@@ -14446,10 +14446,10 @@
         <v>46266</v>
       </c>
       <c r="B1274" t="n">
-        <v>580</v>
+        <v>2815</v>
       </c>
       <c r="C1274" t="n">
-        <v>61360</v>
+        <v>30000.03</v>
       </c>
     </row>
     <row r="1275">
@@ -14457,10 +14457,10 @@
         <v>46266</v>
       </c>
       <c r="B1275" t="n">
-        <v>438</v>
+        <v>1658</v>
       </c>
       <c r="C1275" t="n">
-        <v>70450</v>
+        <v>66000</v>
       </c>
     </row>
     <row r="1276">
@@ -14468,10 +14468,10 @@
         <v>46266</v>
       </c>
       <c r="B1276" t="n">
-        <v>1539</v>
+        <v>2635</v>
       </c>
       <c r="C1276" t="n">
-        <v>77270</v>
+        <v>64999</v>
       </c>
     </row>
     <row r="1277">
@@ -14479,10 +14479,10 @@
         <v>46266</v>
       </c>
       <c r="B1277" t="n">
-        <v>2817</v>
+        <v>2402</v>
       </c>
       <c r="C1277" t="n">
-        <v>27270</v>
+        <v>325996</v>
       </c>
     </row>
     <row r="1278">
@@ -14490,10 +14490,10 @@
         <v>46266</v>
       </c>
       <c r="B1278" t="n">
-        <v>2816</v>
+        <v>452</v>
       </c>
       <c r="C1278" t="n">
-        <v>59090</v>
+        <v>134992</v>
       </c>
     </row>
     <row r="1279">
@@ -14501,10 +14501,10 @@
         <v>46266</v>
       </c>
       <c r="B1279" t="n">
-        <v>2146</v>
+        <v>2085</v>
       </c>
       <c r="C1279" t="n">
-        <v>91660</v>
+        <v>66022</v>
       </c>
     </row>
     <row r="1280">
@@ -14512,10 +14512,10 @@
         <v>46266</v>
       </c>
       <c r="B1280" t="n">
-        <v>2276</v>
+        <v>2568</v>
       </c>
       <c r="C1280" t="n">
-        <v>101840</v>
+        <v>102212</v>
       </c>
     </row>
     <row r="1281">
@@ -14523,10 +14523,10 @@
         <v>46266</v>
       </c>
       <c r="B1281" t="n">
-        <v>1381</v>
+        <v>1906</v>
       </c>
       <c r="C1281" t="n">
-        <v>134090</v>
+        <v>58014</v>
       </c>
     </row>
     <row r="1282">
@@ -14534,10 +14534,10 @@
         <v>46266</v>
       </c>
       <c r="B1282" t="n">
-        <v>2081</v>
+        <v>2821</v>
       </c>
       <c r="C1282" t="n">
-        <v>68180</v>
+        <v>50446</v>
       </c>
     </row>
     <row r="1283">
@@ -14545,10 +14545,10 @@
         <v>46266</v>
       </c>
       <c r="B1283" t="n">
-        <v>14</v>
+        <v>2698</v>
       </c>
       <c r="C1283" t="n">
-        <v>197720</v>
+        <v>61831</v>
       </c>
     </row>
     <row r="1284">
@@ -14556,10 +14556,10 @@
         <v>46266</v>
       </c>
       <c r="B1284" t="n">
-        <v>766</v>
+        <v>2118</v>
       </c>
       <c r="C1284" t="n">
-        <v>31220</v>
+        <v>118580</v>
       </c>
     </row>
     <row r="1285">
@@ -14567,10 +14567,10 @@
         <v>46266</v>
       </c>
       <c r="B1285" t="n">
-        <v>2547</v>
+        <v>2383</v>
       </c>
       <c r="C1285" t="n">
-        <v>18690</v>
+        <v>69234</v>
       </c>
     </row>
     <row r="1286">
@@ -14578,10 +14578,10 @@
         <v>46266</v>
       </c>
       <c r="B1286" t="n">
-        <v>2552</v>
+        <v>2813</v>
       </c>
       <c r="C1286" t="n">
-        <v>13440</v>
+        <v>31471</v>
       </c>
     </row>
     <row r="1287">
@@ -14589,10 +14589,10 @@
         <v>46266</v>
       </c>
       <c r="B1287" t="n">
-        <v>131</v>
+        <v>925</v>
       </c>
       <c r="C1287" t="n">
-        <v>185900</v>
+        <v>39336</v>
       </c>
     </row>
     <row r="1288">
@@ -14600,10 +14600,10 @@
         <v>46266</v>
       </c>
       <c r="B1288" t="n">
-        <v>2250</v>
+        <v>2689</v>
       </c>
       <c r="C1288" t="n">
-        <v>150410</v>
+        <v>31471</v>
       </c>
     </row>
     <row r="1289">
@@ -14611,10 +14611,10 @@
         <v>46266</v>
       </c>
       <c r="B1289" t="n">
-        <v>89</v>
+        <v>2716</v>
       </c>
       <c r="C1289" t="n">
-        <v>153720</v>
+        <v>43274</v>
       </c>
     </row>
     <row r="1290">
@@ -14622,10 +14622,10 @@
         <v>46266</v>
       </c>
       <c r="B1290" t="n">
-        <v>2141</v>
+        <v>2831</v>
       </c>
       <c r="C1290" t="n">
-        <v>14380</v>
+        <v>29997</v>
       </c>
     </row>
     <row r="1291">
@@ -14633,10 +14633,10 @@
         <v>46266</v>
       </c>
       <c r="B1291" t="n">
-        <v>2798</v>
+        <v>2045</v>
       </c>
       <c r="C1291" t="n">
-        <v>27272.76</v>
+        <v>168227.89</v>
       </c>
     </row>
     <row r="1292">
@@ -14644,10 +14644,10 @@
         <v>46266</v>
       </c>
       <c r="B1292" t="n">
-        <v>2797</v>
+        <v>580</v>
       </c>
       <c r="C1292" t="n">
-        <v>27272.76</v>
+        <v>67496</v>
       </c>
     </row>
     <row r="1293">
@@ -14655,10 +14655,10 @@
         <v>46266</v>
       </c>
       <c r="B1293" t="n">
-        <v>2266</v>
+        <v>438</v>
       </c>
       <c r="C1293" t="n">
-        <v>36363.68</v>
+        <v>77495</v>
       </c>
     </row>
     <row r="1294">
@@ -14666,10 +14666,10 @@
         <v>46266</v>
       </c>
       <c r="B1294" t="n">
-        <v>1499</v>
+        <v>1539</v>
       </c>
       <c r="C1294" t="n">
-        <v>63630</v>
+        <v>84997</v>
       </c>
     </row>
     <row r="1295">
@@ -14677,10 +14677,10 @@
         <v>46266</v>
       </c>
       <c r="B1295" t="n">
-        <v>2496</v>
+        <v>2817</v>
       </c>
       <c r="C1295" t="n">
-        <v>72720</v>
+        <v>29997</v>
       </c>
     </row>
     <row r="1296">
@@ -14688,10 +14688,10 @@
         <v>46266</v>
       </c>
       <c r="B1296" t="n">
-        <v>949</v>
+        <v>2816</v>
       </c>
       <c r="C1296" t="n">
-        <v>44610</v>
+        <v>64999</v>
       </c>
     </row>
     <row r="1297">
@@ -14699,10 +14699,10 @@
         <v>46266</v>
       </c>
       <c r="B1297" t="n">
-        <v>1853</v>
+        <v>2146</v>
       </c>
       <c r="C1297" t="n">
-        <v>54540</v>
+        <v>100826</v>
       </c>
     </row>
     <row r="1298">
@@ -14710,10 +14710,10 @@
         <v>46266</v>
       </c>
       <c r="B1298" t="n">
-        <v>854</v>
+        <v>2276</v>
       </c>
       <c r="C1298" t="n">
-        <v>50000</v>
+        <v>112024</v>
       </c>
     </row>
     <row r="1299">
@@ -14721,10 +14721,10 @@
         <v>46266</v>
       </c>
       <c r="B1299" t="n">
-        <v>2674</v>
+        <v>1381</v>
       </c>
       <c r="C1299" t="n">
-        <v>118180</v>
+        <v>147499</v>
       </c>
     </row>
     <row r="1300">
@@ -14732,10 +14732,10 @@
         <v>46266</v>
       </c>
       <c r="B1300" t="n">
-        <v>2803</v>
+        <v>2081</v>
       </c>
       <c r="C1300" t="n">
-        <v>54540</v>
+        <v>74998</v>
       </c>
     </row>
     <row r="1301">
@@ -14743,10 +14743,10 @@
         <v>46266</v>
       </c>
       <c r="B1301" t="n">
-        <v>2599</v>
+        <v>14</v>
       </c>
       <c r="C1301" t="n">
-        <v>86360</v>
+        <v>217492</v>
       </c>
     </row>
     <row r="1302">
@@ -14754,10 +14754,10 @@
         <v>46266</v>
       </c>
       <c r="B1302" t="n">
-        <v>783</v>
+        <v>766</v>
       </c>
       <c r="C1302" t="n">
-        <v>23630</v>
+        <v>34342</v>
       </c>
     </row>
     <row r="1303">
@@ -14765,10 +14765,10 @@
         <v>46266</v>
       </c>
       <c r="B1303" t="n">
-        <v>27</v>
+        <v>2547</v>
       </c>
       <c r="C1303" t="n">
-        <v>45450</v>
+        <v>20559</v>
       </c>
     </row>
     <row r="1304">
@@ -14776,10 +14776,10 @@
         <v>46266</v>
       </c>
       <c r="B1304" t="n">
-        <v>531</v>
+        <v>2552</v>
       </c>
       <c r="C1304" t="n">
-        <v>159090</v>
+        <v>14784</v>
       </c>
     </row>
     <row r="1305">
@@ -14787,10 +14787,10 @@
         <v>46266</v>
       </c>
       <c r="B1305" t="n">
-        <v>1308</v>
+        <v>131</v>
       </c>
       <c r="C1305" t="n">
-        <v>73420</v>
+        <v>204490</v>
       </c>
     </row>
     <row r="1306">
@@ -14798,10 +14798,10 @@
         <v>46266</v>
       </c>
       <c r="B1306" t="n">
-        <v>2792</v>
+        <v>2250</v>
       </c>
       <c r="C1306" t="n">
-        <v>52950</v>
+        <v>165451</v>
       </c>
     </row>
     <row r="1307">
@@ -14809,10 +14809,10 @@
         <v>46266</v>
       </c>
       <c r="B1307" t="n">
-        <v>2828</v>
+        <v>89</v>
       </c>
       <c r="C1307" t="n">
-        <v>0</v>
+        <v>169092</v>
       </c>
     </row>
     <row r="1308">
@@ -14820,10 +14820,10 @@
         <v>46266</v>
       </c>
       <c r="B1308" t="n">
-        <v>2823</v>
+        <v>2141</v>
       </c>
       <c r="C1308" t="n">
-        <v>42500</v>
+        <v>15818</v>
       </c>
     </row>
     <row r="1309">
@@ -14831,10 +14831,10 @@
         <v>46266</v>
       </c>
       <c r="B1309" t="n">
-        <v>945</v>
+        <v>2798</v>
       </c>
       <c r="C1309" t="n">
-        <v>128780</v>
+        <v>30000.03</v>
       </c>
     </row>
     <row r="1310">
@@ -14842,10 +14842,10 @@
         <v>46266</v>
       </c>
       <c r="B1310" t="n">
-        <v>2660</v>
+        <v>2797</v>
       </c>
       <c r="C1310" t="n">
-        <v>140900</v>
+        <v>30000.03</v>
       </c>
     </row>
     <row r="1311">
@@ -14853,10 +14853,10 @@
         <v>46266</v>
       </c>
       <c r="B1311" t="n">
-        <v>1317</v>
+        <v>2266</v>
       </c>
       <c r="C1311" t="n">
-        <v>136360</v>
+        <v>40000.04</v>
       </c>
     </row>
     <row r="1312">
@@ -14864,10 +14864,10 @@
         <v>46266</v>
       </c>
       <c r="B1312" t="n">
-        <v>2790</v>
+        <v>1499</v>
       </c>
       <c r="C1312" t="n">
-        <v>28950</v>
+        <v>69993</v>
       </c>
     </row>
     <row r="1313">
@@ -14875,10 +14875,10 @@
         <v>46266</v>
       </c>
       <c r="B1313" t="n">
-        <v>2711</v>
+        <v>2496</v>
       </c>
       <c r="C1313" t="n">
-        <v>39403.68</v>
+        <v>79992</v>
       </c>
     </row>
     <row r="1314">
@@ -14886,10 +14886,10 @@
         <v>46266</v>
       </c>
       <c r="B1314" t="n">
-        <v>2607</v>
+        <v>949</v>
       </c>
       <c r="C1314" t="n">
-        <v>22583.68</v>
+        <v>49071</v>
       </c>
     </row>
     <row r="1315">
@@ -14897,10 +14897,10 @@
         <v>46266</v>
       </c>
       <c r="B1315" t="n">
-        <v>2667</v>
+        <v>1853</v>
       </c>
       <c r="C1315" t="n">
-        <v>20772.76</v>
+        <v>59994</v>
       </c>
     </row>
     <row r="1316">
@@ -14908,10 +14908,10 @@
         <v>46266</v>
       </c>
       <c r="B1316" t="n">
-        <v>2706</v>
+        <v>854</v>
       </c>
       <c r="C1316" t="n">
-        <v>10014.6</v>
+        <v>55000</v>
       </c>
     </row>
     <row r="1317">
@@ -14919,10 +14919,10 @@
         <v>46266</v>
       </c>
       <c r="B1317" t="n">
-        <v>2657</v>
+        <v>2674</v>
       </c>
       <c r="C1317" t="n">
-        <v>35998.28</v>
+        <v>129998</v>
       </c>
     </row>
     <row r="1318">
@@ -14930,10 +14930,10 @@
         <v>46266</v>
       </c>
       <c r="B1318" t="n">
-        <v>1278</v>
+        <v>2803</v>
       </c>
       <c r="C1318" t="n">
-        <v>45450</v>
+        <v>59994</v>
       </c>
     </row>
     <row r="1319">
@@ -14941,10 +14941,10 @@
         <v>46266</v>
       </c>
       <c r="B1319" t="n">
-        <v>2745</v>
+        <v>2599</v>
       </c>
       <c r="C1319" t="n">
-        <v>50000</v>
+        <v>94996</v>
       </c>
     </row>
     <row r="1320">
@@ -14952,10 +14952,10 @@
         <v>46266</v>
       </c>
       <c r="B1320" t="n">
-        <v>2753</v>
+        <v>783</v>
       </c>
       <c r="C1320" t="n">
-        <v>34090</v>
+        <v>25993</v>
       </c>
     </row>
     <row r="1321">
@@ -14963,10 +14963,10 @@
         <v>46266</v>
       </c>
       <c r="B1321" t="n">
-        <v>2183</v>
+        <v>27</v>
       </c>
       <c r="C1321" t="n">
-        <v>166340</v>
+        <v>49995</v>
       </c>
     </row>
     <row r="1322">
@@ -14974,10 +14974,10 @@
         <v>46266</v>
       </c>
       <c r="B1322" t="n">
-        <v>1340</v>
+        <v>531</v>
       </c>
       <c r="C1322" t="n">
-        <v>65900</v>
+        <v>174999</v>
       </c>
     </row>
     <row r="1323">
@@ -14985,10 +14985,10 @@
         <v>46266</v>
       </c>
       <c r="B1323" t="n">
-        <v>2583</v>
+        <v>1308</v>
       </c>
       <c r="C1323" t="n">
-        <v>18910</v>
+        <v>80762</v>
       </c>
     </row>
     <row r="1324">
@@ -14996,10 +14996,10 @@
         <v>46266</v>
       </c>
       <c r="B1324" t="n">
-        <v>2090</v>
+        <v>2792</v>
       </c>
       <c r="C1324" t="n">
-        <v>18910</v>
+        <v>58245</v>
       </c>
     </row>
     <row r="1325">
@@ -15007,10 +15007,10 @@
         <v>46266</v>
       </c>
       <c r="B1325" t="n">
-        <v>1277</v>
+        <v>2828</v>
       </c>
       <c r="C1325" t="n">
-        <v>100000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1326">
@@ -15018,10 +15018,10 @@
         <v>46266</v>
       </c>
       <c r="B1326" t="n">
-        <v>1501</v>
+        <v>2823</v>
       </c>
       <c r="C1326" t="n">
-        <v>43180</v>
+        <v>46750</v>
       </c>
     </row>
     <row r="1327">
@@ -15029,10 +15029,10 @@
         <v>46266</v>
       </c>
       <c r="B1327" t="n">
-        <v>703</v>
+        <v>2584</v>
       </c>
       <c r="C1327" t="n">
-        <v>113630</v>
+        <v>31471</v>
       </c>
     </row>
     <row r="1328">
@@ -15040,10 +15040,10 @@
         <v>46266</v>
       </c>
       <c r="B1328" t="n">
-        <v>749</v>
+        <v>945</v>
       </c>
       <c r="C1328" t="n">
-        <v>37040</v>
+        <v>141658</v>
       </c>
     </row>
     <row r="1329">
@@ -15051,10 +15051,10 @@
         <v>46266</v>
       </c>
       <c r="B1329" t="n">
-        <v>1983</v>
+        <v>2660</v>
       </c>
       <c r="C1329" t="n">
-        <v>245980</v>
+        <v>154990</v>
       </c>
     </row>
     <row r="1330">
@@ -15062,10 +15062,10 @@
         <v>46266</v>
       </c>
       <c r="B1330" t="n">
-        <v>1993</v>
+        <v>1317</v>
       </c>
       <c r="C1330" t="n">
-        <v>158130</v>
+        <v>149996</v>
       </c>
     </row>
     <row r="1331">
@@ -15073,10 +15073,10 @@
         <v>46266</v>
       </c>
       <c r="B1331" t="n">
-        <v>2767</v>
+        <v>2790</v>
       </c>
       <c r="C1331" t="n">
-        <v>87690</v>
+        <v>31845</v>
       </c>
     </row>
     <row r="1332">
@@ -15084,10 +15084,164 @@
         <v>46266</v>
       </c>
       <c r="B1332" t="n">
-        <v>2646</v>
+        <v>2711</v>
       </c>
       <c r="C1332" t="n">
-        <v>0</v>
+        <v>43344.04</v>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1333" t="n">
+        <v>2607</v>
+      </c>
+      <c r="C1333" t="n">
+        <v>24842.04</v>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1334" t="n">
+        <v>2667</v>
+      </c>
+      <c r="C1334" t="n">
+        <v>22850.03</v>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1335" t="n">
+        <v>2706</v>
+      </c>
+      <c r="C1335" t="n">
+        <v>11016.05</v>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1336" t="n">
+        <v>2657</v>
+      </c>
+      <c r="C1336" t="n">
+        <v>39598.09</v>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1337" t="n">
+        <v>1278</v>
+      </c>
+      <c r="C1337" t="n">
+        <v>49995</v>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1338" t="n">
+        <v>2745</v>
+      </c>
+      <c r="C1338" t="n">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1339" t="n">
+        <v>2753</v>
+      </c>
+      <c r="C1339" t="n">
+        <v>37499</v>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1340" t="n">
+        <v>2183</v>
+      </c>
+      <c r="C1340" t="n">
+        <v>182974</v>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1341" t="n">
+        <v>1340</v>
+      </c>
+      <c r="C1341" t="n">
+        <v>72490</v>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1342" t="n">
+        <v>2583</v>
+      </c>
+      <c r="C1342" t="n">
+        <v>20801</v>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1343" t="n">
+        <v>2090</v>
+      </c>
+      <c r="C1343" t="n">
+        <v>20801</v>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1344" t="n">
+        <v>1277</v>
+      </c>
+      <c r="C1344" t="n">
+        <v>110000</v>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1345" t="n">
+        <v>1501</v>
+      </c>
+      <c r="C1345" t="n">
+        <v>47498</v>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1346" t="n">
+        <v>703</v>
+      </c>
+      <c r="C1346" t="n">
+        <v>124993</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 10:03:32
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -11292,7 +11292,7 @@
         <v>1956</v>
       </c>
       <c r="C987" t="n">
-        <v>126236</v>
+        <v>137712</v>
       </c>
     </row>
     <row r="988">
@@ -11303,7 +11303,7 @@
         <v>2824</v>
       </c>
       <c r="C988" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="989">
@@ -11314,7 +11314,7 @@
         <v>2787</v>
       </c>
       <c r="C989" t="n">
-        <v>64999</v>
+        <v>70908</v>
       </c>
     </row>
     <row r="990">
@@ -11325,7 +11325,7 @@
         <v>2830</v>
       </c>
       <c r="C990" t="n">
-        <v>44990</v>
+        <v>49080</v>
       </c>
     </row>
     <row r="991">
@@ -11336,7 +11336,7 @@
         <v>1254</v>
       </c>
       <c r="C991" t="n">
-        <v>97098.00999999999</v>
+        <v>105925.1</v>
       </c>
     </row>
     <row r="992">
@@ -11347,7 +11347,7 @@
         <v>1890</v>
       </c>
       <c r="C992" t="n">
-        <v>158071.42</v>
+        <v>172441.53</v>
       </c>
     </row>
     <row r="993">
@@ -11358,7 +11358,7 @@
         <v>816</v>
       </c>
       <c r="C993" t="n">
-        <v>133925</v>
+        <v>146100</v>
       </c>
     </row>
     <row r="994">
@@ -11369,7 +11369,7 @@
         <v>2671</v>
       </c>
       <c r="C994" t="n">
-        <v>39996</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="995">
@@ -11380,7 +11380,7 @@
         <v>2705</v>
       </c>
       <c r="C995" t="n">
-        <v>89595</v>
+        <v>97740</v>
       </c>
     </row>
     <row r="996">
@@ -11391,7 +11391,7 @@
         <v>2333</v>
       </c>
       <c r="C996" t="n">
-        <v>77176</v>
+        <v>84192</v>
       </c>
     </row>
     <row r="997">
@@ -11402,7 +11402,7 @@
         <v>2440</v>
       </c>
       <c r="C997" t="n">
-        <v>44990</v>
+        <v>49080</v>
       </c>
     </row>
     <row r="998">
@@ -11413,7 +11413,7 @@
         <v>2448</v>
       </c>
       <c r="C998" t="n">
-        <v>9999</v>
+        <v>10908</v>
       </c>
     </row>
     <row r="999">
@@ -11424,7 +11424,7 @@
         <v>2310</v>
       </c>
       <c r="C999" t="n">
-        <v>34342</v>
+        <v>37464</v>
       </c>
     </row>
     <row r="1000">
@@ -11435,7 +11435,7 @@
         <v>2809</v>
       </c>
       <c r="C1000" t="n">
-        <v>34342</v>
+        <v>37464</v>
       </c>
     </row>
     <row r="1001">
@@ -11446,7 +11446,7 @@
         <v>2548</v>
       </c>
       <c r="C1001" t="n">
-        <v>29260</v>
+        <v>31920</v>
       </c>
     </row>
     <row r="1002">
@@ -11457,7 +11457,7 @@
         <v>451</v>
       </c>
       <c r="C1002" t="n">
-        <v>119999</v>
+        <v>130908</v>
       </c>
     </row>
     <row r="1003">
@@ -11468,7 +11468,7 @@
         <v>933</v>
       </c>
       <c r="C1003" t="n">
-        <v>40744</v>
+        <v>44448</v>
       </c>
     </row>
     <row r="1004">
@@ -11479,7 +11479,7 @@
         <v>2702</v>
       </c>
       <c r="C1004" t="n">
-        <v>40744</v>
+        <v>44448</v>
       </c>
     </row>
     <row r="1005">
@@ -11490,7 +11490,7 @@
         <v>2549</v>
       </c>
       <c r="C1005" t="n">
-        <v>14168</v>
+        <v>15456</v>
       </c>
     </row>
     <row r="1006">
@@ -11501,7 +11501,7 @@
         <v>535</v>
       </c>
       <c r="C1006" t="n">
-        <v>184998</v>
+        <v>201816</v>
       </c>
     </row>
     <row r="1007">
@@ -11512,7 +11512,7 @@
         <v>1117</v>
       </c>
       <c r="C1007" t="n">
-        <v>173943</v>
+        <v>189756</v>
       </c>
     </row>
     <row r="1008">
@@ -11534,7 +11534,7 @@
         <v>530</v>
       </c>
       <c r="C1009" t="n">
-        <v>122034</v>
+        <v>133128</v>
       </c>
     </row>
     <row r="1010">
@@ -11545,7 +11545,7 @@
         <v>358</v>
       </c>
       <c r="C1010" t="n">
-        <v>169994</v>
+        <v>185448</v>
       </c>
     </row>
     <row r="1011">
@@ -11556,7 +11556,7 @@
         <v>2498</v>
       </c>
       <c r="C1011" t="n">
-        <v>27764</v>
+        <v>30288</v>
       </c>
     </row>
     <row r="1012">
@@ -11567,7 +11567,7 @@
         <v>2381</v>
       </c>
       <c r="C1012" t="n">
-        <v>39666</v>
+        <v>43272</v>
       </c>
     </row>
     <row r="1013">
@@ -11578,7 +11578,7 @@
         <v>2695</v>
       </c>
       <c r="C1013" t="n">
-        <v>23859</v>
+        <v>26028</v>
       </c>
     </row>
     <row r="1014">
@@ -11589,7 +11589,7 @@
         <v>2744</v>
       </c>
       <c r="C1014" t="n">
-        <v>30000.03</v>
+        <v>32727.3</v>
       </c>
     </row>
     <row r="1015">
@@ -11600,7 +11600,7 @@
         <v>2750</v>
       </c>
       <c r="C1015" t="n">
-        <v>29997</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1016">
@@ -11611,7 +11611,7 @@
         <v>2131</v>
       </c>
       <c r="C1016" t="n">
-        <v>59994</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1017">
@@ -11622,7 +11622,7 @@
         <v>818</v>
       </c>
       <c r="C1017" t="n">
-        <v>199991</v>
+        <v>218172</v>
       </c>
     </row>
     <row r="1018">
@@ -11633,7 +11633,7 @@
         <v>2566</v>
       </c>
       <c r="C1018" t="n">
-        <v>39996</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1019">
@@ -11644,7 +11644,7 @@
         <v>132</v>
       </c>
       <c r="C1019" t="n">
-        <v>374990</v>
+        <v>409080</v>
       </c>
     </row>
     <row r="1020">
@@ -11655,7 +11655,7 @@
         <v>2431</v>
       </c>
       <c r="C1020" t="n">
-        <v>91993</v>
+        <v>100356</v>
       </c>
     </row>
     <row r="1021">
@@ -11666,7 +11666,7 @@
         <v>2249</v>
       </c>
       <c r="C1021" t="n">
-        <v>97658</v>
+        <v>106536</v>
       </c>
     </row>
     <row r="1022">
@@ -11677,7 +11677,7 @@
         <v>1585</v>
       </c>
       <c r="C1022" t="n">
-        <v>82522</v>
+        <v>90024</v>
       </c>
     </row>
     <row r="1023">
@@ -11688,7 +11688,7 @@
         <v>2325</v>
       </c>
       <c r="C1023" t="n">
-        <v>79772</v>
+        <v>87024</v>
       </c>
     </row>
     <row r="1024">
@@ -11699,7 +11699,7 @@
         <v>2190</v>
       </c>
       <c r="C1024" t="n">
-        <v>112497</v>
+        <v>122724</v>
       </c>
     </row>
     <row r="1025">
@@ -11710,7 +11710,7 @@
         <v>1466</v>
       </c>
       <c r="C1025" t="n">
-        <v>202499</v>
+        <v>220908</v>
       </c>
     </row>
     <row r="1026">
@@ -11721,7 +11721,7 @@
         <v>2659</v>
       </c>
       <c r="C1026" t="n">
-        <v>61501</v>
+        <v>67092</v>
       </c>
     </row>
     <row r="1027">
@@ -11732,7 +11732,7 @@
         <v>634</v>
       </c>
       <c r="C1027" t="n">
-        <v>275000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="1028">
@@ -11743,7 +11743,7 @@
         <v>2804</v>
       </c>
       <c r="C1028" t="n">
-        <v>49995</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1029">
@@ -11754,7 +11754,7 @@
         <v>2375</v>
       </c>
       <c r="C1029" t="n">
-        <v>165000</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="1030">
@@ -11765,7 +11765,7 @@
         <v>2601</v>
       </c>
       <c r="C1030" t="n">
-        <v>137500</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="1031">
@@ -11776,7 +11776,7 @@
         <v>952</v>
       </c>
       <c r="C1031" t="n">
-        <v>49995</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1032">
@@ -11787,7 +11787,7 @@
         <v>571</v>
       </c>
       <c r="C1032" t="n">
-        <v>318241</v>
+        <v>347172</v>
       </c>
     </row>
     <row r="1033">
@@ -11798,7 +11798,7 @@
         <v>2697</v>
       </c>
       <c r="C1033" t="n">
-        <v>96965</v>
+        <v>105780</v>
       </c>
     </row>
     <row r="1034">
@@ -11809,7 +11809,7 @@
         <v>2678</v>
       </c>
       <c r="C1034" t="n">
-        <v>167761</v>
+        <v>183012</v>
       </c>
     </row>
     <row r="1035">
@@ -11820,7 +11820,7 @@
         <v>2768</v>
       </c>
       <c r="C1035" t="n">
-        <v>175571</v>
+        <v>191532</v>
       </c>
     </row>
     <row r="1036">
@@ -11831,7 +11831,7 @@
         <v>2359</v>
       </c>
       <c r="C1036" t="n">
-        <v>53251</v>
+        <v>58092</v>
       </c>
     </row>
     <row r="1037">
@@ -11842,7 +11842,7 @@
         <v>353</v>
       </c>
       <c r="C1037" t="n">
-        <v>172986</v>
+        <v>188712</v>
       </c>
     </row>
     <row r="1038">
@@ -11853,7 +11853,7 @@
         <v>2026</v>
       </c>
       <c r="C1038" t="n">
-        <v>143330</v>
+        <v>156360</v>
       </c>
     </row>
     <row r="1039">
@@ -11875,7 +11875,7 @@
         <v>2345</v>
       </c>
       <c r="C1040" t="n">
-        <v>31471</v>
+        <v>34332</v>
       </c>
     </row>
     <row r="1041">
@@ -11886,7 +11886,7 @@
         <v>2789</v>
       </c>
       <c r="C1041" t="n">
-        <v>84997</v>
+        <v>92724</v>
       </c>
     </row>
     <row r="1042">
@@ -11897,7 +11897,7 @@
         <v>569</v>
       </c>
       <c r="C1042" t="n">
-        <v>1431958</v>
+        <v>1562136</v>
       </c>
     </row>
     <row r="1043">
@@ -11908,7 +11908,7 @@
         <v>2822</v>
       </c>
       <c r="C1043" t="n">
-        <v>67496</v>
+        <v>73632</v>
       </c>
     </row>
     <row r="1044">
@@ -11919,7 +11919,7 @@
         <v>2728</v>
       </c>
       <c r="C1044" t="n">
-        <v>4994</v>
+        <v>5448</v>
       </c>
     </row>
     <row r="1045">
@@ -11930,7 +11930,7 @@
         <v>2488</v>
       </c>
       <c r="C1045" t="n">
-        <v>49995</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1046">
@@ -11941,7 +11941,7 @@
         <v>2791</v>
       </c>
       <c r="C1046" t="n">
-        <v>49345.1</v>
+        <v>53831</v>
       </c>
     </row>
     <row r="1047">
@@ -11952,7 +11952,7 @@
         <v>2577</v>
       </c>
       <c r="C1047" t="n">
-        <v>44585.11</v>
+        <v>48638.29</v>
       </c>
     </row>
     <row r="1048">
@@ -11963,7 +11963,7 @@
         <v>2069</v>
       </c>
       <c r="C1048" t="n">
-        <v>89991</v>
+        <v>98172</v>
       </c>
     </row>
     <row r="1049">
@@ -11974,7 +11974,7 @@
         <v>2082</v>
       </c>
       <c r="C1049" t="n">
-        <v>83281</v>
+        <v>90852</v>
       </c>
     </row>
     <row r="1050">
@@ -11985,7 +11985,7 @@
         <v>781</v>
       </c>
       <c r="C1050" t="n">
-        <v>64999</v>
+        <v>70908</v>
       </c>
     </row>
     <row r="1051">
@@ -11996,7 +11996,7 @@
         <v>744</v>
       </c>
       <c r="C1051" t="n">
-        <v>20801</v>
+        <v>22692</v>
       </c>
     </row>
     <row r="1052">
@@ -12007,7 +12007,7 @@
         <v>2223</v>
       </c>
       <c r="C1052" t="n">
-        <v>65967</v>
+        <v>71964</v>
       </c>
     </row>
     <row r="1053">
@@ -12018,7 +12018,7 @@
         <v>2452</v>
       </c>
       <c r="C1053" t="n">
-        <v>34991</v>
+        <v>38172</v>
       </c>
     </row>
     <row r="1054">
@@ -12029,7 +12029,7 @@
         <v>970</v>
       </c>
       <c r="C1054" t="n">
-        <v>34342</v>
+        <v>37464</v>
       </c>
     </row>
     <row r="1055">
@@ -12040,7 +12040,7 @@
         <v>2550</v>
       </c>
       <c r="C1055" t="n">
-        <v>30492</v>
+        <v>33264</v>
       </c>
     </row>
     <row r="1056">
@@ -12051,7 +12051,7 @@
         <v>768</v>
       </c>
       <c r="C1056" t="n">
-        <v>64999</v>
+        <v>70908</v>
       </c>
     </row>
     <row r="1057">
@@ -12062,7 +12062,7 @@
         <v>1075</v>
       </c>
       <c r="C1057" t="n">
-        <v>226490</v>
+        <v>247080</v>
       </c>
     </row>
     <row r="1058">
@@ -12073,7 +12073,7 @@
         <v>664</v>
       </c>
       <c r="C1058" t="n">
-        <v>129492</v>
+        <v>141264</v>
       </c>
     </row>
     <row r="1059">
@@ -12084,7 +12084,7 @@
         <v>2555</v>
       </c>
       <c r="C1059" t="n">
-        <v>20757</v>
+        <v>22644</v>
       </c>
     </row>
     <row r="1060">
@@ -12095,7 +12095,7 @@
         <v>2627</v>
       </c>
       <c r="C1060" t="n">
-        <v>12188</v>
+        <v>13296</v>
       </c>
     </row>
     <row r="1061">
@@ -12106,7 +12106,7 @@
         <v>2557</v>
       </c>
       <c r="C1061" t="n">
-        <v>12892</v>
+        <v>14064</v>
       </c>
     </row>
     <row r="1062">
@@ -12117,7 +12117,7 @@
         <v>2551</v>
       </c>
       <c r="C1062" t="n">
-        <v>10241</v>
+        <v>11172</v>
       </c>
     </row>
     <row r="1063">
@@ -12128,7 +12128,7 @@
         <v>2463</v>
       </c>
       <c r="C1063" t="n">
-        <v>160105</v>
+        <v>174660</v>
       </c>
     </row>
     <row r="1064">
@@ -12139,7 +12139,7 @@
         <v>2279</v>
       </c>
       <c r="C1064" t="n">
-        <v>120791</v>
+        <v>131772</v>
       </c>
     </row>
     <row r="1065">
@@ -12150,7 +12150,7 @@
         <v>631</v>
       </c>
       <c r="C1065" t="n">
-        <v>174999</v>
+        <v>190908</v>
       </c>
     </row>
     <row r="1066">
@@ -12161,7 +12161,7 @@
         <v>2251</v>
       </c>
       <c r="C1066" t="n">
-        <v>107162</v>
+        <v>116904</v>
       </c>
     </row>
     <row r="1067">
@@ -12172,7 +12172,7 @@
         <v>1653</v>
       </c>
       <c r="C1067" t="n">
-        <v>162492</v>
+        <v>177264</v>
       </c>
     </row>
     <row r="1068">
@@ -12183,7 +12183,7 @@
         <v>1293</v>
       </c>
       <c r="C1068" t="n">
-        <v>207493</v>
+        <v>226356</v>
       </c>
     </row>
     <row r="1069">
@@ -12194,7 +12194,7 @@
         <v>360</v>
       </c>
       <c r="C1069" t="n">
-        <v>249997</v>
+        <v>272724</v>
       </c>
     </row>
     <row r="1070">
@@ -12205,7 +12205,7 @@
         <v>1063</v>
       </c>
       <c r="C1070" t="n">
-        <v>181775</v>
+        <v>198300</v>
       </c>
     </row>
     <row r="1071">
@@ -12216,7 +12216,7 @@
         <v>2273</v>
       </c>
       <c r="C1071" t="n">
-        <v>106040</v>
+        <v>115680</v>
       </c>
     </row>
     <row r="1072">
@@ -12227,7 +12227,7 @@
         <v>2757</v>
       </c>
       <c r="C1072" t="n">
-        <v>35000.09</v>
+        <v>38181.9</v>
       </c>
     </row>
     <row r="1073">
@@ -12238,7 +12238,7 @@
         <v>2795</v>
       </c>
       <c r="C1073" t="n">
-        <v>30000.03</v>
+        <v>32727.3</v>
       </c>
     </row>
     <row r="1074">
@@ -12249,7 +12249,7 @@
         <v>2722</v>
       </c>
       <c r="C1074" t="n">
-        <v>29997</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1075">
@@ -12260,7 +12260,7 @@
         <v>2718</v>
       </c>
       <c r="C1075" t="n">
-        <v>39996</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1076">
@@ -12271,7 +12271,7 @@
         <v>595</v>
       </c>
       <c r="C1076" t="n">
-        <v>275000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="1077">
@@ -12282,7 +12282,7 @@
         <v>890</v>
       </c>
       <c r="C1077" t="n">
-        <v>349998</v>
+        <v>381816</v>
       </c>
     </row>
     <row r="1078">
@@ -12293,7 +12293,7 @@
         <v>2652</v>
       </c>
       <c r="C1078" t="n">
-        <v>64999</v>
+        <v>70908</v>
       </c>
     </row>
     <row r="1079">
@@ -12304,7 +12304,7 @@
         <v>2714</v>
       </c>
       <c r="C1079" t="n">
-        <v>179993</v>
+        <v>196356</v>
       </c>
     </row>
     <row r="1080">
@@ -12315,7 +12315,7 @@
         <v>1869</v>
       </c>
       <c r="C1080" t="n">
-        <v>114994</v>
+        <v>125448</v>
       </c>
     </row>
     <row r="1081">
@@ -12326,7 +12326,7 @@
         <v>400</v>
       </c>
       <c r="C1081" t="n">
-        <v>94996</v>
+        <v>103632</v>
       </c>
     </row>
     <row r="1082">
@@ -12337,7 +12337,7 @@
         <v>1907</v>
       </c>
       <c r="C1082" t="n">
-        <v>185493</v>
+        <v>202356</v>
       </c>
     </row>
     <row r="1083">
@@ -12348,7 +12348,7 @@
         <v>1996</v>
       </c>
       <c r="C1083" t="n">
-        <v>117249</v>
+        <v>127908</v>
       </c>
     </row>
     <row r="1084">
@@ -12359,7 +12359,7 @@
         <v>2114</v>
       </c>
       <c r="C1084" t="n">
-        <v>91850</v>
+        <v>100200</v>
       </c>
     </row>
     <row r="1085">
@@ -12370,7 +12370,7 @@
         <v>2330</v>
       </c>
       <c r="C1085" t="n">
-        <v>134387</v>
+        <v>146604</v>
       </c>
     </row>
     <row r="1086">
@@ -12414,7 +12414,7 @@
         <v>931</v>
       </c>
       <c r="C1089" t="n">
-        <v>47212</v>
+        <v>51504</v>
       </c>
     </row>
     <row r="1090">
@@ -12425,7 +12425,7 @@
         <v>947</v>
       </c>
       <c r="C1090" t="n">
-        <v>217261</v>
+        <v>237012</v>
       </c>
     </row>
     <row r="1091">
@@ -12436,7 +12436,7 @@
         <v>951</v>
       </c>
       <c r="C1091" t="n">
-        <v>57497</v>
+        <v>62724</v>
       </c>
     </row>
     <row r="1092">
@@ -12447,7 +12447,7 @@
         <v>2449</v>
       </c>
       <c r="C1092" t="n">
-        <v>19998</v>
+        <v>21816</v>
       </c>
     </row>
     <row r="1093">
@@ -12458,7 +12458,7 @@
         <v>610</v>
       </c>
       <c r="C1093" t="n">
-        <v>407495</v>
+        <v>444540</v>
       </c>
     </row>
     <row r="1094">
@@ -12469,7 +12469,7 @@
         <v>2761</v>
       </c>
       <c r="C1094" t="n">
-        <v>40744</v>
+        <v>44448</v>
       </c>
     </row>
     <row r="1095">
@@ -12480,7 +12480,7 @@
         <v>483</v>
       </c>
       <c r="C1095" t="n">
-        <v>221496</v>
+        <v>241632</v>
       </c>
     </row>
     <row r="1096">
@@ -12491,7 +12491,7 @@
         <v>2015</v>
       </c>
       <c r="C1096" t="n">
-        <v>184998</v>
+        <v>201816</v>
       </c>
     </row>
     <row r="1097">
@@ -12502,7 +12502,7 @@
         <v>1478</v>
       </c>
       <c r="C1097" t="n">
-        <v>270578</v>
+        <v>295176</v>
       </c>
     </row>
     <row r="1098">
@@ -12513,7 +12513,7 @@
         <v>424</v>
       </c>
       <c r="C1098" t="n">
-        <v>120791</v>
+        <v>131772</v>
       </c>
     </row>
     <row r="1099">
@@ -12535,7 +12535,7 @@
         <v>477</v>
       </c>
       <c r="C1100" t="n">
-        <v>129327</v>
+        <v>141084</v>
       </c>
     </row>
     <row r="1101">
@@ -12546,7 +12546,7 @@
         <v>1810</v>
       </c>
       <c r="C1101" t="n">
-        <v>20031</v>
+        <v>21852</v>
       </c>
     </row>
     <row r="1102">
@@ -12557,7 +12557,7 @@
         <v>2826</v>
       </c>
       <c r="C1102" t="n">
-        <v>35000.09</v>
+        <v>38181.9</v>
       </c>
     </row>
     <row r="1103">
@@ -12568,7 +12568,7 @@
         <v>2561</v>
       </c>
       <c r="C1103" t="n">
-        <v>7348</v>
+        <v>8016</v>
       </c>
     </row>
     <row r="1104">
@@ -12579,7 +12579,7 @@
         <v>2653</v>
       </c>
       <c r="C1104" t="n">
-        <v>30000.03</v>
+        <v>32727.3</v>
       </c>
     </row>
     <row r="1105">
@@ -12590,7 +12590,7 @@
         <v>2829</v>
       </c>
       <c r="C1105" t="n">
-        <v>30000.03</v>
+        <v>32727.3</v>
       </c>
     </row>
     <row r="1106">
@@ -12601,7 +12601,7 @@
         <v>2643</v>
       </c>
       <c r="C1106" t="n">
-        <v>14762</v>
+        <v>16104</v>
       </c>
     </row>
     <row r="1107">
@@ -12612,7 +12612,7 @@
         <v>2794</v>
       </c>
       <c r="C1107" t="n">
-        <v>44990</v>
+        <v>49080</v>
       </c>
     </row>
     <row r="1108">
@@ -12623,7 +12623,7 @@
         <v>2655</v>
       </c>
       <c r="C1108" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1109">
@@ -12634,7 +12634,7 @@
         <v>1456</v>
       </c>
       <c r="C1109" t="n">
-        <v>385143</v>
+        <v>420156</v>
       </c>
     </row>
     <row r="1110">
@@ -12645,7 +12645,7 @@
         <v>2606</v>
       </c>
       <c r="C1110" t="n">
-        <v>118294</v>
+        <v>129048</v>
       </c>
     </row>
     <row r="1111">
@@ -12656,7 +12656,7 @@
         <v>1142</v>
       </c>
       <c r="C1111" t="n">
-        <v>214522</v>
+        <v>234024</v>
       </c>
     </row>
     <row r="1112">
@@ -12667,7 +12667,7 @@
         <v>1450</v>
       </c>
       <c r="C1112" t="n">
-        <v>136279</v>
+        <v>148668</v>
       </c>
     </row>
     <row r="1113">
@@ -12678,7 +12678,7 @@
         <v>2133</v>
       </c>
       <c r="C1113" t="n">
-        <v>318241</v>
+        <v>347172</v>
       </c>
     </row>
     <row r="1114">
@@ -12689,7 +12689,7 @@
         <v>522</v>
       </c>
       <c r="C1114" t="n">
-        <v>97493</v>
+        <v>106356</v>
       </c>
     </row>
     <row r="1115">
@@ -12700,7 +12700,7 @@
         <v>2696</v>
       </c>
       <c r="C1115" t="n">
-        <v>131560</v>
+        <v>143520</v>
       </c>
     </row>
     <row r="1116">
@@ -12722,7 +12722,7 @@
         <v>2692</v>
       </c>
       <c r="C1117" t="n">
-        <v>37499</v>
+        <v>40908</v>
       </c>
     </row>
     <row r="1118">
@@ -12733,7 +12733,7 @@
         <v>2691</v>
       </c>
       <c r="C1118" t="n">
-        <v>67496</v>
+        <v>73632</v>
       </c>
     </row>
     <row r="1119">
@@ -12744,7 +12744,7 @@
         <v>1632</v>
       </c>
       <c r="C1119" t="n">
-        <v>124993</v>
+        <v>136356</v>
       </c>
     </row>
     <row r="1120">
@@ -12755,7 +12755,7 @@
         <v>2641</v>
       </c>
       <c r="C1120" t="n">
-        <v>39996</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1121">
@@ -12766,7 +12766,7 @@
         <v>2197</v>
       </c>
       <c r="C1121" t="n">
-        <v>99990</v>
+        <v>109080</v>
       </c>
     </row>
     <row r="1122">
@@ -12777,7 +12777,7 @@
         <v>609</v>
       </c>
       <c r="C1122" t="n">
-        <v>110000</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="1123">
@@ -12788,7 +12788,7 @@
         <v>1380</v>
       </c>
       <c r="C1123" t="n">
-        <v>49995</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1124">
@@ -12799,7 +12799,7 @@
         <v>104</v>
       </c>
       <c r="C1124" t="n">
-        <v>149996</v>
+        <v>163632</v>
       </c>
     </row>
     <row r="1125">
@@ -12810,7 +12810,7 @@
         <v>2621</v>
       </c>
       <c r="C1125" t="n">
-        <v>34991</v>
+        <v>38172</v>
       </c>
     </row>
     <row r="1126">
@@ -12821,7 +12821,7 @@
         <v>2786</v>
       </c>
       <c r="C1126" t="n">
-        <v>34991</v>
+        <v>38172</v>
       </c>
     </row>
     <row r="1127">
@@ -12832,7 +12832,7 @@
         <v>2784</v>
       </c>
       <c r="C1127" t="n">
-        <v>20801</v>
+        <v>22692</v>
       </c>
     </row>
     <row r="1128">
@@ -12843,7 +12843,7 @@
         <v>2586</v>
       </c>
       <c r="C1128" t="n">
-        <v>20801</v>
+        <v>22692</v>
       </c>
     </row>
     <row r="1129">
@@ -12854,7 +12854,7 @@
         <v>2145</v>
       </c>
       <c r="C1129" t="n">
-        <v>64724</v>
+        <v>70608</v>
       </c>
     </row>
     <row r="1130">
@@ -12865,7 +12865,7 @@
         <v>2574</v>
       </c>
       <c r="C1130" t="n">
-        <v>64724</v>
+        <v>70608</v>
       </c>
     </row>
     <row r="1131">
@@ -12876,7 +12876,7 @@
         <v>2492</v>
       </c>
       <c r="C1131" t="n">
-        <v>70950</v>
+        <v>77400</v>
       </c>
     </row>
     <row r="1132">
@@ -12887,7 +12887,7 @@
         <v>629</v>
       </c>
       <c r="C1132" t="n">
-        <v>220990</v>
+        <v>241080</v>
       </c>
     </row>
     <row r="1133">
@@ -12898,7 +12898,7 @@
         <v>966</v>
       </c>
       <c r="C1133" t="n">
-        <v>40744</v>
+        <v>44448</v>
       </c>
     </row>
     <row r="1134">
@@ -12909,7 +12909,7 @@
         <v>2721</v>
       </c>
       <c r="C1134" t="n">
-        <v>40744</v>
+        <v>44448</v>
       </c>
     </row>
     <row r="1135">
@@ -12920,7 +12920,7 @@
         <v>2554</v>
       </c>
       <c r="C1135" t="n">
-        <v>12276</v>
+        <v>13392</v>
       </c>
     </row>
     <row r="1136">
@@ -12931,7 +12931,7 @@
         <v>2556</v>
       </c>
       <c r="C1136" t="n">
-        <v>18051</v>
+        <v>19692</v>
       </c>
     </row>
     <row r="1137">
@@ -12942,7 +12942,7 @@
         <v>2546</v>
       </c>
       <c r="C1137" t="n">
-        <v>11924</v>
+        <v>13008</v>
       </c>
     </row>
     <row r="1138">
@@ -12953,7 +12953,7 @@
         <v>42</v>
       </c>
       <c r="C1138" t="n">
-        <v>944999</v>
+        <v>1030908</v>
       </c>
     </row>
     <row r="1139">
@@ -12964,7 +12964,7 @@
         <v>953</v>
       </c>
       <c r="C1139" t="n">
-        <v>341330</v>
+        <v>372360</v>
       </c>
     </row>
     <row r="1140">
@@ -12975,7 +12975,7 @@
         <v>675</v>
       </c>
       <c r="C1140" t="n">
-        <v>99990</v>
+        <v>109080</v>
       </c>
     </row>
     <row r="1141">
@@ -12986,7 +12986,7 @@
         <v>619</v>
       </c>
       <c r="C1141" t="n">
-        <v>154616</v>
+        <v>168672</v>
       </c>
     </row>
     <row r="1142">
@@ -12997,7 +12997,7 @@
         <v>1299</v>
       </c>
       <c r="C1142" t="n">
-        <v>260172</v>
+        <v>283824</v>
       </c>
     </row>
     <row r="1143">
@@ -13008,7 +13008,7 @@
         <v>1064</v>
       </c>
       <c r="C1143" t="n">
-        <v>299684</v>
+        <v>326928</v>
       </c>
     </row>
     <row r="1144">
@@ -13019,7 +13019,7 @@
         <v>2308</v>
       </c>
       <c r="C1144" t="n">
-        <v>102498</v>
+        <v>111816</v>
       </c>
     </row>
     <row r="1145">
@@ -13030,7 +13030,7 @@
         <v>1137</v>
       </c>
       <c r="C1145" t="n">
-        <v>319990</v>
+        <v>349080</v>
       </c>
     </row>
     <row r="1146">
@@ -13041,7 +13041,7 @@
         <v>2747</v>
       </c>
       <c r="C1146" t="n">
-        <v>30000.03</v>
+        <v>32727.3</v>
       </c>
     </row>
     <row r="1147">
@@ -13052,7 +13052,7 @@
         <v>2819</v>
       </c>
       <c r="C1147" t="n">
-        <v>30000.03</v>
+        <v>32727.3</v>
       </c>
     </row>
     <row r="1148">
@@ -13063,7 +13063,7 @@
         <v>1259</v>
       </c>
       <c r="C1148" t="n">
-        <v>50000.05</v>
+        <v>54545.5</v>
       </c>
     </row>
     <row r="1149">
@@ -13074,7 +13074,7 @@
         <v>2544</v>
       </c>
       <c r="C1149" t="n">
-        <v>39996</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1150">
@@ -13085,7 +13085,7 @@
         <v>2261</v>
       </c>
       <c r="C1150" t="n">
-        <v>74998</v>
+        <v>81816</v>
       </c>
     </row>
     <row r="1151">
@@ -13096,7 +13096,7 @@
         <v>2729</v>
       </c>
       <c r="C1151" t="n">
-        <v>39996</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1152">
@@ -13107,7 +13107,7 @@
         <v>2649</v>
       </c>
       <c r="C1152" t="n">
-        <v>14762</v>
+        <v>16104</v>
       </c>
     </row>
     <row r="1153">
@@ -13118,7 +13118,7 @@
         <v>2494</v>
       </c>
       <c r="C1153" t="n">
-        <v>64999</v>
+        <v>70908</v>
       </c>
     </row>
     <row r="1154">
@@ -13129,7 +13129,7 @@
         <v>1384</v>
       </c>
       <c r="C1154" t="n">
-        <v>224994</v>
+        <v>245448</v>
       </c>
     </row>
     <row r="1155">
@@ -13151,7 +13151,7 @@
         <v>2802</v>
       </c>
       <c r="C1156" t="n">
-        <v>35409</v>
+        <v>38628</v>
       </c>
     </row>
     <row r="1157">
@@ -13162,7 +13162,7 @@
         <v>2726</v>
       </c>
       <c r="C1157" t="n">
-        <v>74998</v>
+        <v>81816</v>
       </c>
     </row>
     <row r="1158">
@@ -13173,7 +13173,7 @@
         <v>2820</v>
       </c>
       <c r="C1158" t="n">
-        <v>89991</v>
+        <v>98172</v>
       </c>
     </row>
     <row r="1159">
@@ -13184,7 +13184,7 @@
         <v>1007</v>
       </c>
       <c r="C1159" t="n">
-        <v>94996</v>
+        <v>103632</v>
       </c>
     </row>
     <row r="1160">
@@ -13195,7 +13195,7 @@
         <v>20</v>
       </c>
       <c r="C1160" t="n">
-        <v>192500</v>
+        <v>210000</v>
       </c>
     </row>
     <row r="1161">
@@ -13206,7 +13206,7 @@
         <v>1372</v>
       </c>
       <c r="C1161" t="n">
-        <v>144991</v>
+        <v>158172</v>
       </c>
     </row>
     <row r="1162">
@@ -13217,7 +13217,7 @@
         <v>2735</v>
       </c>
       <c r="C1162" t="n">
-        <v>59994</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1163">
@@ -13228,7 +13228,7 @@
         <v>2811</v>
       </c>
       <c r="C1163" t="n">
-        <v>20801</v>
+        <v>22692</v>
       </c>
     </row>
     <row r="1164">
@@ -13239,7 +13239,7 @@
         <v>1871</v>
       </c>
       <c r="C1164" t="n">
-        <v>88374</v>
+        <v>96408</v>
       </c>
     </row>
     <row r="1165">
@@ -13250,7 +13250,7 @@
         <v>2541</v>
       </c>
       <c r="C1165" t="n">
-        <v>105798</v>
+        <v>115416</v>
       </c>
     </row>
     <row r="1166">
@@ -13261,7 +13261,7 @@
         <v>2362</v>
       </c>
       <c r="C1166" t="n">
-        <v>37499</v>
+        <v>40908</v>
       </c>
     </row>
     <row r="1167">
@@ -13272,7 +13272,7 @@
         <v>1324</v>
       </c>
       <c r="C1167" t="n">
-        <v>139997</v>
+        <v>152724</v>
       </c>
     </row>
     <row r="1168">
@@ -13283,7 +13283,7 @@
         <v>2323</v>
       </c>
       <c r="C1168" t="n">
-        <v>34342</v>
+        <v>37464</v>
       </c>
     </row>
     <row r="1169">
@@ -13294,7 +13294,7 @@
         <v>2647</v>
       </c>
       <c r="C1169" t="n">
-        <v>70950</v>
+        <v>77400</v>
       </c>
     </row>
     <row r="1170">
@@ -13305,7 +13305,7 @@
         <v>559</v>
       </c>
       <c r="C1170" t="n">
-        <v>114719</v>
+        <v>125148</v>
       </c>
     </row>
     <row r="1171">
@@ -13316,7 +13316,7 @@
         <v>2762</v>
       </c>
       <c r="C1171" t="n">
-        <v>40744</v>
+        <v>44448</v>
       </c>
     </row>
     <row r="1172">
@@ -13327,7 +13327,7 @@
         <v>2501</v>
       </c>
       <c r="C1172" t="n">
-        <v>40744</v>
+        <v>44448</v>
       </c>
     </row>
     <row r="1173">
@@ -13338,7 +13338,7 @@
         <v>2562</v>
       </c>
       <c r="C1173" t="n">
-        <v>7909</v>
+        <v>8628</v>
       </c>
     </row>
     <row r="1174">
@@ -13349,7 +13349,7 @@
         <v>429</v>
       </c>
       <c r="C1174" t="n">
-        <v>194997</v>
+        <v>212724</v>
       </c>
     </row>
     <row r="1175">
@@ -13360,7 +13360,7 @@
         <v>58</v>
       </c>
       <c r="C1175" t="n">
-        <v>135289</v>
+        <v>147588</v>
       </c>
     </row>
     <row r="1176">
@@ -13371,7 +13371,7 @@
         <v>2245</v>
       </c>
       <c r="C1176" t="n">
-        <v>120791</v>
+        <v>131772</v>
       </c>
     </row>
     <row r="1177">
@@ -13382,7 +13382,7 @@
         <v>285</v>
       </c>
       <c r="C1177" t="n">
-        <v>270578</v>
+        <v>295176</v>
       </c>
     </row>
     <row r="1178">
@@ -13404,7 +13404,7 @@
         <v>363</v>
       </c>
       <c r="C1179" t="n">
-        <v>149996</v>
+        <v>163632</v>
       </c>
     </row>
     <row r="1180">
@@ -13415,7 +13415,7 @@
         <v>2651</v>
       </c>
       <c r="C1180" t="n">
-        <v>84557</v>
+        <v>92244</v>
       </c>
     </row>
     <row r="1181">
@@ -13426,7 +13426,7 @@
         <v>2142</v>
       </c>
       <c r="C1181" t="n">
-        <v>26686</v>
+        <v>29112</v>
       </c>
     </row>
     <row r="1182">
@@ -13437,7 +13437,7 @@
         <v>2258</v>
       </c>
       <c r="C1182" t="n">
-        <v>40000.04</v>
+        <v>43636.4</v>
       </c>
     </row>
     <row r="1183">
@@ -13448,7 +13448,7 @@
         <v>2772</v>
       </c>
       <c r="C1183" t="n">
-        <v>30000.03</v>
+        <v>32727.3</v>
       </c>
     </row>
     <row r="1184">
@@ -13459,7 +13459,7 @@
         <v>2346</v>
       </c>
       <c r="C1184" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1185">
@@ -13470,7 +13470,7 @@
         <v>2442</v>
       </c>
       <c r="C1185" t="n">
-        <v>39996</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1186">
@@ -13481,7 +13481,7 @@
         <v>772</v>
       </c>
       <c r="C1186" t="n">
-        <v>165000</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="1187">
@@ -13492,7 +13492,7 @@
         <v>2684</v>
       </c>
       <c r="C1187" t="n">
-        <v>47498</v>
+        <v>51816</v>
       </c>
     </row>
     <row r="1188">
@@ -13503,7 +13503,7 @@
         <v>2765</v>
       </c>
       <c r="C1188" t="n">
-        <v>44990</v>
+        <v>49080</v>
       </c>
     </row>
     <row r="1189">
@@ -13514,7 +13514,7 @@
         <v>2567</v>
       </c>
       <c r="C1189" t="n">
-        <v>82522</v>
+        <v>90024</v>
       </c>
     </row>
     <row r="1190">
@@ -13525,7 +13525,7 @@
         <v>2178</v>
       </c>
       <c r="C1190" t="n">
-        <v>139997</v>
+        <v>152724</v>
       </c>
     </row>
     <row r="1191">
@@ -13536,7 +13536,7 @@
         <v>2827</v>
       </c>
       <c r="C1191" t="n">
-        <v>49995</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1192">
@@ -13547,7 +13547,7 @@
         <v>2510</v>
       </c>
       <c r="C1192" t="n">
-        <v>277618</v>
+        <v>302856</v>
       </c>
     </row>
     <row r="1193">
@@ -13558,7 +13558,7 @@
         <v>2392</v>
       </c>
       <c r="C1193" t="n">
-        <v>83281</v>
+        <v>90852</v>
       </c>
     </row>
     <row r="1194">
@@ -13569,7 +13569,7 @@
         <v>415</v>
       </c>
       <c r="C1194" t="n">
-        <v>284746</v>
+        <v>310632</v>
       </c>
     </row>
     <row r="1195">
@@ -13580,7 +13580,7 @@
         <v>2107</v>
       </c>
       <c r="C1195" t="n">
-        <v>147037</v>
+        <v>160404</v>
       </c>
     </row>
     <row r="1196">
@@ -13591,7 +13591,7 @@
         <v>2211</v>
       </c>
       <c r="C1196" t="n">
-        <v>121902</v>
+        <v>132984</v>
       </c>
     </row>
     <row r="1197">
@@ -13602,7 +13602,7 @@
         <v>2682</v>
       </c>
       <c r="C1197" t="n">
-        <v>74987</v>
+        <v>81804</v>
       </c>
     </row>
     <row r="1198">
@@ -13635,7 +13635,7 @@
         <v>2755</v>
       </c>
       <c r="C1200" t="n">
-        <v>29997</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1201">
@@ -13646,7 +13646,7 @@
         <v>941</v>
       </c>
       <c r="C1201" t="n">
-        <v>196438</v>
+        <v>214296</v>
       </c>
     </row>
     <row r="1202">
@@ -13657,7 +13657,7 @@
         <v>2734</v>
       </c>
       <c r="C1202" t="n">
-        <v>27533</v>
+        <v>30036</v>
       </c>
     </row>
     <row r="1203">
@@ -13668,7 +13668,7 @@
         <v>1289</v>
       </c>
       <c r="C1203" t="n">
-        <v>124993</v>
+        <v>136356</v>
       </c>
     </row>
     <row r="1204">
@@ -13679,7 +13679,7 @@
         <v>2801</v>
       </c>
       <c r="C1204" t="n">
-        <v>39996</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1205">
@@ -13690,7 +13690,7 @@
         <v>2810</v>
       </c>
       <c r="C1205" t="n">
-        <v>67496</v>
+        <v>73632</v>
       </c>
     </row>
     <row r="1206">
@@ -13701,7 +13701,7 @@
         <v>767</v>
       </c>
       <c r="C1206" t="n">
-        <v>89991</v>
+        <v>98172</v>
       </c>
     </row>
     <row r="1207">
@@ -13712,7 +13712,7 @@
         <v>2687</v>
       </c>
       <c r="C1207" t="n">
-        <v>49995</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1208">
@@ -13723,7 +13723,7 @@
         <v>2686</v>
       </c>
       <c r="C1208" t="n">
-        <v>64999</v>
+        <v>70908</v>
       </c>
     </row>
     <row r="1209">
@@ -13734,7 +13734,7 @@
         <v>2730</v>
       </c>
       <c r="C1209" t="n">
-        <v>44990</v>
+        <v>49080</v>
       </c>
     </row>
     <row r="1210">
@@ -13745,7 +13745,7 @@
         <v>2580</v>
       </c>
       <c r="C1210" t="n">
-        <v>16775</v>
+        <v>18300</v>
       </c>
     </row>
     <row r="1211">
@@ -13756,7 +13756,7 @@
         <v>2472</v>
       </c>
       <c r="C1211" t="n">
-        <v>26471.05</v>
+        <v>28877.5</v>
       </c>
     </row>
     <row r="1212">
@@ -13767,7 +13767,7 @@
         <v>2631</v>
       </c>
       <c r="C1212" t="n">
-        <v>12266.01</v>
+        <v>13381.1</v>
       </c>
     </row>
     <row r="1213">
@@ -13778,7 +13778,7 @@
         <v>1642</v>
       </c>
       <c r="C1213" t="n">
-        <v>132495</v>
+        <v>144540</v>
       </c>
     </row>
     <row r="1214">
@@ -13789,7 +13789,7 @@
         <v>2613</v>
       </c>
       <c r="C1214" t="n">
-        <v>89595</v>
+        <v>97740</v>
       </c>
     </row>
     <row r="1215">
@@ -13800,7 +13800,7 @@
         <v>1020</v>
       </c>
       <c r="C1215" t="n">
-        <v>44990</v>
+        <v>49080</v>
       </c>
     </row>
     <row r="1216">
@@ -13811,7 +13811,7 @@
         <v>2785</v>
       </c>
       <c r="C1216" t="n">
-        <v>20801</v>
+        <v>22692</v>
       </c>
     </row>
     <row r="1217">
@@ -13822,7 +13822,7 @@
         <v>1327</v>
       </c>
       <c r="C1217" t="n">
-        <v>29997</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1218">
@@ -13833,7 +13833,7 @@
         <v>2629</v>
       </c>
       <c r="C1218" t="n">
-        <v>34342</v>
+        <v>37464</v>
       </c>
     </row>
     <row r="1219">
@@ -13844,7 +13844,7 @@
         <v>749</v>
       </c>
       <c r="C1219" t="n">
-        <v>40744</v>
+        <v>44448</v>
       </c>
     </row>
     <row r="1220">
@@ -13855,7 +13855,7 @@
         <v>1983</v>
       </c>
       <c r="C1220" t="n">
-        <v>270578</v>
+        <v>295176</v>
       </c>
     </row>
     <row r="1221">
@@ -13866,7 +13866,7 @@
         <v>1993</v>
       </c>
       <c r="C1221" t="n">
-        <v>173943</v>
+        <v>189756</v>
       </c>
     </row>
     <row r="1222">
@@ -13877,7 +13877,7 @@
         <v>2767</v>
       </c>
       <c r="C1222" t="n">
-        <v>96459</v>
+        <v>105228</v>
       </c>
     </row>
     <row r="1223">
@@ -13899,7 +13899,7 @@
         <v>1102</v>
       </c>
       <c r="C1224" t="n">
-        <v>120791</v>
+        <v>131772</v>
       </c>
     </row>
     <row r="1225">
@@ -13910,7 +13910,7 @@
         <v>626</v>
       </c>
       <c r="C1225" t="n">
-        <v>852157.54</v>
+        <v>929626.4</v>
       </c>
     </row>
     <row r="1226">
@@ -13921,7 +13921,7 @@
         <v>1465</v>
       </c>
       <c r="C1226" t="n">
-        <v>179894</v>
+        <v>196248</v>
       </c>
     </row>
     <row r="1227">
@@ -13932,7 +13932,7 @@
         <v>2758</v>
       </c>
       <c r="C1227" t="n">
-        <v>30000.03</v>
+        <v>32727.3</v>
       </c>
     </row>
     <row r="1228">
@@ -13943,7 +13943,7 @@
         <v>2742</v>
       </c>
       <c r="C1228" t="n">
-        <v>30000.03</v>
+        <v>32727.3</v>
       </c>
     </row>
     <row r="1229">
@@ -13965,7 +13965,7 @@
         <v>1873</v>
       </c>
       <c r="C1230" t="n">
-        <v>159995</v>
+        <v>174540</v>
       </c>
     </row>
     <row r="1231">
@@ -13976,7 +13976,7 @@
         <v>2163</v>
       </c>
       <c r="C1231" t="n">
-        <v>74998</v>
+        <v>81816</v>
       </c>
     </row>
     <row r="1232">
@@ -13987,7 +13987,7 @@
         <v>2394</v>
       </c>
       <c r="C1232" t="n">
-        <v>77022</v>
+        <v>84024</v>
       </c>
     </row>
     <row r="1233">
@@ -13998,7 +13998,7 @@
         <v>33</v>
       </c>
       <c r="C1233" t="n">
-        <v>193996</v>
+        <v>211632</v>
       </c>
     </row>
     <row r="1234">
@@ -14009,7 +14009,7 @@
         <v>2421</v>
       </c>
       <c r="C1234" t="n">
-        <v>32494</v>
+        <v>35448</v>
       </c>
     </row>
     <row r="1235">
@@ -14020,7 +14020,7 @@
         <v>2663</v>
       </c>
       <c r="C1235" t="n">
-        <v>137500</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="1236">
@@ -14031,7 +14031,7 @@
         <v>2413</v>
       </c>
       <c r="C1236" t="n">
-        <v>60522</v>
+        <v>66024</v>
       </c>
     </row>
     <row r="1237">
@@ -14042,7 +14042,7 @@
         <v>351</v>
       </c>
       <c r="C1237" t="n">
-        <v>91993</v>
+        <v>100356</v>
       </c>
     </row>
     <row r="1238">
@@ -14053,7 +14053,7 @@
         <v>1298</v>
       </c>
       <c r="C1238" t="n">
-        <v>636493</v>
+        <v>694356</v>
       </c>
     </row>
     <row r="1239">
@@ -14064,7 +14064,7 @@
         <v>2491</v>
       </c>
       <c r="C1239" t="n">
-        <v>51436</v>
+        <v>56112</v>
       </c>
     </row>
     <row r="1240">
@@ -14075,7 +14075,7 @@
         <v>2571</v>
       </c>
       <c r="C1240" t="n">
-        <v>72633</v>
+        <v>79236</v>
       </c>
     </row>
     <row r="1241">
@@ -14086,7 +14086,7 @@
         <v>2507</v>
       </c>
       <c r="C1241" t="n">
-        <v>44132</v>
+        <v>48144</v>
       </c>
     </row>
     <row r="1242">
@@ -14097,7 +14097,7 @@
         <v>2799</v>
       </c>
       <c r="C1242" t="n">
-        <v>56804</v>
+        <v>61968</v>
       </c>
     </row>
     <row r="1243">
@@ -14119,7 +14119,7 @@
         <v>2582</v>
       </c>
       <c r="C1244" t="n">
-        <v>43274</v>
+        <v>47208</v>
       </c>
     </row>
     <row r="1245">
@@ -14130,7 +14130,7 @@
         <v>2637</v>
       </c>
       <c r="C1245" t="n">
-        <v>31471</v>
+        <v>34332</v>
       </c>
     </row>
     <row r="1246">
@@ -14141,7 +14141,7 @@
         <v>630</v>
       </c>
       <c r="C1246" t="n">
-        <v>74844</v>
+        <v>81648</v>
       </c>
     </row>
     <row r="1247">
@@ -14152,7 +14152,7 @@
         <v>525</v>
       </c>
       <c r="C1247" t="n">
-        <v>112497</v>
+        <v>122724</v>
       </c>
     </row>
     <row r="1248">
@@ -14163,7 +14163,7 @@
         <v>2727</v>
       </c>
       <c r="C1248" t="n">
-        <v>20240</v>
+        <v>22080</v>
       </c>
     </row>
     <row r="1249">
@@ -14174,7 +14174,7 @@
         <v>2707</v>
       </c>
       <c r="C1249" t="n">
-        <v>16016</v>
+        <v>17472</v>
       </c>
     </row>
     <row r="1250">
@@ -14185,7 +14185,7 @@
         <v>2834</v>
       </c>
       <c r="C1250" t="n">
-        <v>8274.02</v>
+        <v>9026.200000000001</v>
       </c>
     </row>
     <row r="1251">
@@ -14196,7 +14196,7 @@
         <v>2773</v>
       </c>
       <c r="C1251" t="n">
-        <v>40346.09</v>
+        <v>44013.9</v>
       </c>
     </row>
     <row r="1252">
@@ -14207,7 +14207,7 @@
         <v>2341</v>
       </c>
       <c r="C1252" t="n">
-        <v>70950</v>
+        <v>77400</v>
       </c>
     </row>
     <row r="1253">
@@ -14218,7 +14218,7 @@
         <v>1374</v>
       </c>
       <c r="C1253" t="n">
-        <v>89991</v>
+        <v>98172</v>
       </c>
     </row>
     <row r="1254">
@@ -14229,7 +14229,7 @@
         <v>793</v>
       </c>
       <c r="C1254" t="n">
-        <v>20801</v>
+        <v>22692</v>
       </c>
     </row>
     <row r="1255">
@@ -14240,7 +14240,7 @@
         <v>794</v>
       </c>
       <c r="C1255" t="n">
-        <v>20801</v>
+        <v>22692</v>
       </c>
     </row>
     <row r="1256">
@@ -14251,7 +14251,7 @@
         <v>1834</v>
       </c>
       <c r="C1256" t="n">
-        <v>58498</v>
+        <v>63816</v>
       </c>
     </row>
     <row r="1257">
@@ -14262,7 +14262,7 @@
         <v>802</v>
       </c>
       <c r="C1257" t="n">
-        <v>37499</v>
+        <v>40908</v>
       </c>
     </row>
     <row r="1258">
@@ -14273,7 +14273,7 @@
         <v>1344</v>
       </c>
       <c r="C1258" t="n">
-        <v>74998</v>
+        <v>81816</v>
       </c>
     </row>
     <row r="1259">
@@ -14284,7 +14284,7 @@
         <v>1881</v>
       </c>
       <c r="C1259" t="n">
-        <v>34342</v>
+        <v>37464</v>
       </c>
     </row>
     <row r="1260">
@@ -14295,7 +14295,7 @@
         <v>2365</v>
       </c>
       <c r="C1260" t="n">
-        <v>39831</v>
+        <v>43452</v>
       </c>
     </row>
     <row r="1261">
@@ -14306,7 +14306,7 @@
         <v>2411</v>
       </c>
       <c r="C1261" t="n">
-        <v>70950</v>
+        <v>77400</v>
       </c>
     </row>
     <row r="1262">
@@ -14317,7 +14317,7 @@
         <v>2363</v>
       </c>
       <c r="C1262" t="n">
-        <v>74998</v>
+        <v>81816</v>
       </c>
     </row>
     <row r="1263">
@@ -14328,7 +14328,7 @@
         <v>2124</v>
       </c>
       <c r="C1263" t="n">
-        <v>174999</v>
+        <v>190908</v>
       </c>
     </row>
     <row r="1264">
@@ -14339,7 +14339,7 @@
         <v>1937</v>
       </c>
       <c r="C1264" t="n">
-        <v>127490</v>
+        <v>139080</v>
       </c>
     </row>
     <row r="1265">
@@ -14350,7 +14350,7 @@
         <v>2709</v>
       </c>
       <c r="C1265" t="n">
-        <v>89991</v>
+        <v>98172</v>
       </c>
     </row>
     <row r="1266">
@@ -14361,7 +14361,7 @@
         <v>2558</v>
       </c>
       <c r="C1266" t="n">
-        <v>15026</v>
+        <v>16392</v>
       </c>
     </row>
     <row r="1267">
@@ -14372,7 +14372,7 @@
         <v>663</v>
       </c>
       <c r="C1267" t="n">
-        <v>127490</v>
+        <v>139080</v>
       </c>
     </row>
     <row r="1268">
@@ -14383,7 +14383,7 @@
         <v>40</v>
       </c>
       <c r="C1268" t="n">
-        <v>110000</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="1269">
@@ -14394,7 +14394,7 @@
         <v>2833</v>
       </c>
       <c r="C1269" t="n">
-        <v>35000.09</v>
+        <v>38181.9</v>
       </c>
     </row>
     <row r="1270">
@@ -14405,7 +14405,7 @@
         <v>1756</v>
       </c>
       <c r="C1270" t="n">
-        <v>218251</v>
+        <v>238092</v>
       </c>
     </row>
     <row r="1271">
@@ -14416,7 +14416,7 @@
         <v>1116</v>
       </c>
       <c r="C1271" t="n">
-        <v>126819</v>
+        <v>138348</v>
       </c>
     </row>
     <row r="1272">
@@ -14427,7 +14427,7 @@
         <v>636</v>
       </c>
       <c r="C1272" t="n">
-        <v>124993</v>
+        <v>136356</v>
       </c>
     </row>
     <row r="1273">
@@ -14438,7 +14438,7 @@
         <v>1800</v>
       </c>
       <c r="C1273" t="n">
-        <v>13992</v>
+        <v>15264</v>
       </c>
     </row>
     <row r="1274">
@@ -14449,7 +14449,7 @@
         <v>2815</v>
       </c>
       <c r="C1274" t="n">
-        <v>30000.03</v>
+        <v>32727.3</v>
       </c>
     </row>
     <row r="1275">
@@ -14460,7 +14460,7 @@
         <v>1658</v>
       </c>
       <c r="C1275" t="n">
-        <v>66000</v>
+        <v>72000</v>
       </c>
     </row>
     <row r="1276">
@@ -14471,7 +14471,7 @@
         <v>2635</v>
       </c>
       <c r="C1276" t="n">
-        <v>64999</v>
+        <v>70908</v>
       </c>
     </row>
     <row r="1277">
@@ -14482,7 +14482,7 @@
         <v>2402</v>
       </c>
       <c r="C1277" t="n">
-        <v>325996</v>
+        <v>355632</v>
       </c>
     </row>
     <row r="1278">
@@ -14493,7 +14493,7 @@
         <v>452</v>
       </c>
       <c r="C1278" t="n">
-        <v>134992</v>
+        <v>147264</v>
       </c>
     </row>
     <row r="1279">
@@ -14504,7 +14504,7 @@
         <v>2085</v>
       </c>
       <c r="C1279" t="n">
-        <v>66022</v>
+        <v>72024</v>
       </c>
     </row>
     <row r="1280">
@@ -14515,7 +14515,7 @@
         <v>2568</v>
       </c>
       <c r="C1280" t="n">
-        <v>102212</v>
+        <v>111504</v>
       </c>
     </row>
     <row r="1281">
@@ -14526,7 +14526,7 @@
         <v>1906</v>
       </c>
       <c r="C1281" t="n">
-        <v>58014</v>
+        <v>63288</v>
       </c>
     </row>
     <row r="1282">
@@ -14537,7 +14537,7 @@
         <v>2821</v>
       </c>
       <c r="C1282" t="n">
-        <v>50446</v>
+        <v>55032</v>
       </c>
     </row>
     <row r="1283">
@@ -14548,7 +14548,7 @@
         <v>2698</v>
       </c>
       <c r="C1283" t="n">
-        <v>61831</v>
+        <v>67452</v>
       </c>
     </row>
     <row r="1284">
@@ -14559,7 +14559,7 @@
         <v>2118</v>
       </c>
       <c r="C1284" t="n">
-        <v>118580</v>
+        <v>129360</v>
       </c>
     </row>
     <row r="1285">
@@ -14570,7 +14570,7 @@
         <v>2383</v>
       </c>
       <c r="C1285" t="n">
-        <v>69234</v>
+        <v>75528</v>
       </c>
     </row>
     <row r="1286">
@@ -14581,7 +14581,7 @@
         <v>2813</v>
       </c>
       <c r="C1286" t="n">
-        <v>31471</v>
+        <v>34332</v>
       </c>
     </row>
     <row r="1287">
@@ -14592,7 +14592,7 @@
         <v>925</v>
       </c>
       <c r="C1287" t="n">
-        <v>39336</v>
+        <v>42912</v>
       </c>
     </row>
     <row r="1288">
@@ -14603,7 +14603,7 @@
         <v>2689</v>
       </c>
       <c r="C1288" t="n">
-        <v>31471</v>
+        <v>34332</v>
       </c>
     </row>
     <row r="1289">
@@ -14614,7 +14614,7 @@
         <v>2716</v>
       </c>
       <c r="C1289" t="n">
-        <v>43274</v>
+        <v>47208</v>
       </c>
     </row>
     <row r="1290">
@@ -14625,7 +14625,7 @@
         <v>2831</v>
       </c>
       <c r="C1290" t="n">
-        <v>29997</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1291">
@@ -14636,7 +14636,7 @@
         <v>2045</v>
       </c>
       <c r="C1291" t="n">
-        <v>168227.89</v>
+        <v>183521.32</v>
       </c>
     </row>
     <row r="1292">
@@ -14647,7 +14647,7 @@
         <v>580</v>
       </c>
       <c r="C1292" t="n">
-        <v>67496</v>
+        <v>73632</v>
       </c>
     </row>
     <row r="1293">
@@ -14658,7 +14658,7 @@
         <v>438</v>
       </c>
       <c r="C1293" t="n">
-        <v>77495</v>
+        <v>84540</v>
       </c>
     </row>
     <row r="1294">
@@ -14669,7 +14669,7 @@
         <v>1539</v>
       </c>
       <c r="C1294" t="n">
-        <v>84997</v>
+        <v>92724</v>
       </c>
     </row>
     <row r="1295">
@@ -14680,7 +14680,7 @@
         <v>2817</v>
       </c>
       <c r="C1295" t="n">
-        <v>29997</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1296">
@@ -14691,7 +14691,7 @@
         <v>2816</v>
       </c>
       <c r="C1296" t="n">
-        <v>64999</v>
+        <v>70908</v>
       </c>
     </row>
     <row r="1297">
@@ -14702,7 +14702,7 @@
         <v>2146</v>
       </c>
       <c r="C1297" t="n">
-        <v>100826</v>
+        <v>109992</v>
       </c>
     </row>
     <row r="1298">
@@ -14713,7 +14713,7 @@
         <v>2276</v>
       </c>
       <c r="C1298" t="n">
-        <v>112024</v>
+        <v>122208</v>
       </c>
     </row>
     <row r="1299">
@@ -14724,7 +14724,7 @@
         <v>1381</v>
       </c>
       <c r="C1299" t="n">
-        <v>147499</v>
+        <v>160908</v>
       </c>
     </row>
     <row r="1300">
@@ -14735,7 +14735,7 @@
         <v>2081</v>
       </c>
       <c r="C1300" t="n">
-        <v>74998</v>
+        <v>81816</v>
       </c>
     </row>
     <row r="1301">
@@ -14746,7 +14746,7 @@
         <v>14</v>
       </c>
       <c r="C1301" t="n">
-        <v>217492</v>
+        <v>237264</v>
       </c>
     </row>
     <row r="1302">
@@ -14757,7 +14757,7 @@
         <v>766</v>
       </c>
       <c r="C1302" t="n">
-        <v>34342</v>
+        <v>37464</v>
       </c>
     </row>
     <row r="1303">
@@ -14768,7 +14768,7 @@
         <v>2547</v>
       </c>
       <c r="C1303" t="n">
-        <v>20559</v>
+        <v>22428</v>
       </c>
     </row>
     <row r="1304">
@@ -14779,7 +14779,7 @@
         <v>2552</v>
       </c>
       <c r="C1304" t="n">
-        <v>14784</v>
+        <v>16128</v>
       </c>
     </row>
     <row r="1305">
@@ -14790,7 +14790,7 @@
         <v>131</v>
       </c>
       <c r="C1305" t="n">
-        <v>204490</v>
+        <v>223080</v>
       </c>
     </row>
     <row r="1306">
@@ -14801,7 +14801,7 @@
         <v>2250</v>
       </c>
       <c r="C1306" t="n">
-        <v>165451</v>
+        <v>180492</v>
       </c>
     </row>
     <row r="1307">
@@ -14812,7 +14812,7 @@
         <v>89</v>
       </c>
       <c r="C1307" t="n">
-        <v>169092</v>
+        <v>184464</v>
       </c>
     </row>
     <row r="1308">
@@ -14823,7 +14823,7 @@
         <v>2141</v>
       </c>
       <c r="C1308" t="n">
-        <v>15818</v>
+        <v>17256</v>
       </c>
     </row>
     <row r="1309">
@@ -14834,7 +14834,7 @@
         <v>2798</v>
       </c>
       <c r="C1309" t="n">
-        <v>30000.03</v>
+        <v>32727.3</v>
       </c>
     </row>
     <row r="1310">
@@ -14845,7 +14845,7 @@
         <v>2797</v>
       </c>
       <c r="C1310" t="n">
-        <v>30000.03</v>
+        <v>32727.3</v>
       </c>
     </row>
     <row r="1311">
@@ -14856,7 +14856,7 @@
         <v>2266</v>
       </c>
       <c r="C1311" t="n">
-        <v>40000.04</v>
+        <v>43636.4</v>
       </c>
     </row>
     <row r="1312">
@@ -14867,7 +14867,7 @@
         <v>1499</v>
       </c>
       <c r="C1312" t="n">
-        <v>69993</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1313">
@@ -14878,7 +14878,7 @@
         <v>2496</v>
       </c>
       <c r="C1313" t="n">
-        <v>79992</v>
+        <v>87264</v>
       </c>
     </row>
     <row r="1314">
@@ -14889,7 +14889,7 @@
         <v>949</v>
       </c>
       <c r="C1314" t="n">
-        <v>49071</v>
+        <v>53532</v>
       </c>
     </row>
     <row r="1315">
@@ -14900,7 +14900,7 @@
         <v>1853</v>
       </c>
       <c r="C1315" t="n">
-        <v>59994</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1316">
@@ -14911,7 +14911,7 @@
         <v>854</v>
       </c>
       <c r="C1316" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1317">
@@ -14922,7 +14922,7 @@
         <v>2674</v>
       </c>
       <c r="C1317" t="n">
-        <v>129998</v>
+        <v>141816</v>
       </c>
     </row>
     <row r="1318">
@@ -14933,7 +14933,7 @@
         <v>2803</v>
       </c>
       <c r="C1318" t="n">
-        <v>59994</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1319">
@@ -14944,7 +14944,7 @@
         <v>2599</v>
       </c>
       <c r="C1319" t="n">
-        <v>94996</v>
+        <v>103632</v>
       </c>
     </row>
     <row r="1320">
@@ -14955,7 +14955,7 @@
         <v>783</v>
       </c>
       <c r="C1320" t="n">
-        <v>25993</v>
+        <v>28356</v>
       </c>
     </row>
     <row r="1321">
@@ -14966,7 +14966,7 @@
         <v>27</v>
       </c>
       <c r="C1321" t="n">
-        <v>49995</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1322">
@@ -14977,7 +14977,7 @@
         <v>531</v>
       </c>
       <c r="C1322" t="n">
-        <v>174999</v>
+        <v>190908</v>
       </c>
     </row>
     <row r="1323">
@@ -14988,7 +14988,7 @@
         <v>1308</v>
       </c>
       <c r="C1323" t="n">
-        <v>80762</v>
+        <v>88104</v>
       </c>
     </row>
     <row r="1324">
@@ -14999,7 +14999,7 @@
         <v>2792</v>
       </c>
       <c r="C1324" t="n">
-        <v>58245</v>
+        <v>63540</v>
       </c>
     </row>
     <row r="1325">
@@ -15021,7 +15021,7 @@
         <v>2823</v>
       </c>
       <c r="C1326" t="n">
-        <v>46750</v>
+        <v>51000</v>
       </c>
     </row>
     <row r="1327">
@@ -15032,7 +15032,7 @@
         <v>2584</v>
       </c>
       <c r="C1327" t="n">
-        <v>31471</v>
+        <v>34332</v>
       </c>
     </row>
     <row r="1328">
@@ -15043,7 +15043,7 @@
         <v>945</v>
       </c>
       <c r="C1328" t="n">
-        <v>141658</v>
+        <v>154536</v>
       </c>
     </row>
     <row r="1329">
@@ -15054,7 +15054,7 @@
         <v>2660</v>
       </c>
       <c r="C1329" t="n">
-        <v>154990</v>
+        <v>169080</v>
       </c>
     </row>
     <row r="1330">
@@ -15065,7 +15065,7 @@
         <v>1317</v>
       </c>
       <c r="C1330" t="n">
-        <v>149996</v>
+        <v>163632</v>
       </c>
     </row>
     <row r="1331">
@@ -15076,7 +15076,7 @@
         <v>2790</v>
       </c>
       <c r="C1331" t="n">
-        <v>31845</v>
+        <v>34740</v>
       </c>
     </row>
     <row r="1332">
@@ -15087,7 +15087,7 @@
         <v>2711</v>
       </c>
       <c r="C1332" t="n">
-        <v>43344.04</v>
+        <v>47284.4</v>
       </c>
     </row>
     <row r="1333">
@@ -15098,7 +15098,7 @@
         <v>2607</v>
       </c>
       <c r="C1333" t="n">
-        <v>24842.04</v>
+        <v>27100.4</v>
       </c>
     </row>
     <row r="1334">
@@ -15109,7 +15109,7 @@
         <v>2667</v>
       </c>
       <c r="C1334" t="n">
-        <v>22850.03</v>
+        <v>24927.3</v>
       </c>
     </row>
     <row r="1335">
@@ -15120,7 +15120,7 @@
         <v>2706</v>
       </c>
       <c r="C1335" t="n">
-        <v>11016.05</v>
+        <v>12017.5</v>
       </c>
     </row>
     <row r="1336">
@@ -15131,7 +15131,7 @@
         <v>2657</v>
       </c>
       <c r="C1336" t="n">
-        <v>39598.09</v>
+        <v>43197.9</v>
       </c>
     </row>
     <row r="1337">
@@ -15142,7 +15142,7 @@
         <v>1278</v>
       </c>
       <c r="C1337" t="n">
-        <v>49995</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1338">
@@ -15153,7 +15153,7 @@
         <v>2745</v>
       </c>
       <c r="C1338" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1339">
@@ -15164,7 +15164,7 @@
         <v>2753</v>
       </c>
       <c r="C1339" t="n">
-        <v>37499</v>
+        <v>40908</v>
       </c>
     </row>
     <row r="1340">
@@ -15175,7 +15175,7 @@
         <v>2183</v>
       </c>
       <c r="C1340" t="n">
-        <v>182974</v>
+        <v>199608</v>
       </c>
     </row>
     <row r="1341">
@@ -15186,7 +15186,7 @@
         <v>1340</v>
       </c>
       <c r="C1341" t="n">
-        <v>72490</v>
+        <v>79080</v>
       </c>
     </row>
     <row r="1342">
@@ -15197,7 +15197,7 @@
         <v>2583</v>
       </c>
       <c r="C1342" t="n">
-        <v>20801</v>
+        <v>22692</v>
       </c>
     </row>
     <row r="1343">
@@ -15208,7 +15208,7 @@
         <v>2090</v>
       </c>
       <c r="C1343" t="n">
-        <v>20801</v>
+        <v>22692</v>
       </c>
     </row>
     <row r="1344">
@@ -15219,7 +15219,7 @@
         <v>1277</v>
       </c>
       <c r="C1344" t="n">
-        <v>110000</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="1345">
@@ -15230,7 +15230,7 @@
         <v>1501</v>
       </c>
       <c r="C1345" t="n">
-        <v>47498</v>
+        <v>51816</v>
       </c>
     </row>
     <row r="1346">
@@ -15241,7 +15241,7 @@
         <v>703</v>
       </c>
       <c r="C1346" t="n">
-        <v>124993</v>
+        <v>136356</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:00:56
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -11289,10 +11289,10 @@
         <v>46266</v>
       </c>
       <c r="B987" t="n">
-        <v>1956</v>
+        <v>947</v>
       </c>
       <c r="C987" t="n">
-        <v>137712</v>
+        <v>256763</v>
       </c>
     </row>
     <row r="988">
@@ -11300,10 +11300,10 @@
         <v>46266</v>
       </c>
       <c r="B988" t="n">
-        <v>2824</v>
+        <v>1956</v>
       </c>
       <c r="C988" t="n">
-        <v>60000</v>
+        <v>149188</v>
       </c>
     </row>
     <row r="989">
@@ -11311,10 +11311,10 @@
         <v>46266</v>
       </c>
       <c r="B989" t="n">
-        <v>2787</v>
+        <v>2824</v>
       </c>
       <c r="C989" t="n">
-        <v>70908</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="990">
@@ -11322,10 +11322,10 @@
         <v>46266</v>
       </c>
       <c r="B990" t="n">
-        <v>2830</v>
+        <v>2787</v>
       </c>
       <c r="C990" t="n">
-        <v>49080</v>
+        <v>76817</v>
       </c>
     </row>
     <row r="991">
@@ -11333,10 +11333,10 @@
         <v>46266</v>
       </c>
       <c r="B991" t="n">
-        <v>1254</v>
+        <v>2830</v>
       </c>
       <c r="C991" t="n">
-        <v>105925.1</v>
+        <v>53170</v>
       </c>
     </row>
     <row r="992">
@@ -11344,10 +11344,10 @@
         <v>46266</v>
       </c>
       <c r="B992" t="n">
-        <v>1890</v>
+        <v>1254</v>
       </c>
       <c r="C992" t="n">
-        <v>172441.53</v>
+        <v>114752.19</v>
       </c>
     </row>
     <row r="993">
@@ -11358,7 +11358,7 @@
         <v>816</v>
       </c>
       <c r="C993" t="n">
-        <v>146100</v>
+        <v>158275</v>
       </c>
     </row>
     <row r="994">
@@ -11369,7 +11369,7 @@
         <v>2671</v>
       </c>
       <c r="C994" t="n">
-        <v>43632</v>
+        <v>47268</v>
       </c>
     </row>
     <row r="995">
@@ -11380,7 +11380,7 @@
         <v>2705</v>
       </c>
       <c r="C995" t="n">
-        <v>97740</v>
+        <v>105885</v>
       </c>
     </row>
     <row r="996">
@@ -11391,7 +11391,7 @@
         <v>2333</v>
       </c>
       <c r="C996" t="n">
-        <v>84192</v>
+        <v>91208</v>
       </c>
     </row>
     <row r="997">
@@ -11402,7 +11402,7 @@
         <v>2440</v>
       </c>
       <c r="C997" t="n">
-        <v>49080</v>
+        <v>53170</v>
       </c>
     </row>
     <row r="998">
@@ -11413,7 +11413,7 @@
         <v>2448</v>
       </c>
       <c r="C998" t="n">
-        <v>10908</v>
+        <v>11817</v>
       </c>
     </row>
     <row r="999">
@@ -11424,7 +11424,7 @@
         <v>2310</v>
       </c>
       <c r="C999" t="n">
-        <v>37464</v>
+        <v>40586</v>
       </c>
     </row>
     <row r="1000">
@@ -11435,7 +11435,7 @@
         <v>2809</v>
       </c>
       <c r="C1000" t="n">
-        <v>37464</v>
+        <v>40586</v>
       </c>
     </row>
     <row r="1001">
@@ -11446,7 +11446,7 @@
         <v>2548</v>
       </c>
       <c r="C1001" t="n">
-        <v>31920</v>
+        <v>34580</v>
       </c>
     </row>
     <row r="1002">
@@ -11457,7 +11457,7 @@
         <v>451</v>
       </c>
       <c r="C1002" t="n">
-        <v>130908</v>
+        <v>141817</v>
       </c>
     </row>
     <row r="1003">
@@ -11468,7 +11468,7 @@
         <v>933</v>
       </c>
       <c r="C1003" t="n">
-        <v>44448</v>
+        <v>48152</v>
       </c>
     </row>
     <row r="1004">
@@ -11479,7 +11479,7 @@
         <v>2702</v>
       </c>
       <c r="C1004" t="n">
-        <v>44448</v>
+        <v>48152</v>
       </c>
     </row>
     <row r="1005">
@@ -11490,7 +11490,7 @@
         <v>2549</v>
       </c>
       <c r="C1005" t="n">
-        <v>15456</v>
+        <v>16744</v>
       </c>
     </row>
     <row r="1006">
@@ -11501,7 +11501,7 @@
         <v>535</v>
       </c>
       <c r="C1006" t="n">
-        <v>201816</v>
+        <v>218634</v>
       </c>
     </row>
     <row r="1007">
@@ -11512,7 +11512,7 @@
         <v>1117</v>
       </c>
       <c r="C1007" t="n">
-        <v>189756</v>
+        <v>205569</v>
       </c>
     </row>
     <row r="1008">
@@ -11534,7 +11534,7 @@
         <v>530</v>
       </c>
       <c r="C1009" t="n">
-        <v>133128</v>
+        <v>144222</v>
       </c>
     </row>
     <row r="1010">
@@ -11545,7 +11545,7 @@
         <v>358</v>
       </c>
       <c r="C1010" t="n">
-        <v>185448</v>
+        <v>200902</v>
       </c>
     </row>
     <row r="1011">
@@ -11556,7 +11556,7 @@
         <v>2498</v>
       </c>
       <c r="C1011" t="n">
-        <v>30288</v>
+        <v>32812</v>
       </c>
     </row>
     <row r="1012">
@@ -11567,7 +11567,7 @@
         <v>2381</v>
       </c>
       <c r="C1012" t="n">
-        <v>43272</v>
+        <v>46878</v>
       </c>
     </row>
     <row r="1013">
@@ -11578,7 +11578,7 @@
         <v>2695</v>
       </c>
       <c r="C1013" t="n">
-        <v>26028</v>
+        <v>28197</v>
       </c>
     </row>
     <row r="1014">
@@ -11589,7 +11589,7 @@
         <v>2744</v>
       </c>
       <c r="C1014" t="n">
-        <v>32727.3</v>
+        <v>35454.57</v>
       </c>
     </row>
     <row r="1015">
@@ -11600,7 +11600,7 @@
         <v>2750</v>
       </c>
       <c r="C1015" t="n">
-        <v>32724</v>
+        <v>35451</v>
       </c>
     </row>
     <row r="1016">
@@ -11611,7 +11611,7 @@
         <v>2131</v>
       </c>
       <c r="C1016" t="n">
-        <v>65448</v>
+        <v>70902</v>
       </c>
     </row>
     <row r="1017">
@@ -11622,7 +11622,7 @@
         <v>818</v>
       </c>
       <c r="C1017" t="n">
-        <v>218172</v>
+        <v>236353</v>
       </c>
     </row>
     <row r="1018">
@@ -11633,7 +11633,7 @@
         <v>2566</v>
       </c>
       <c r="C1018" t="n">
-        <v>43632</v>
+        <v>47268</v>
       </c>
     </row>
     <row r="1019">
@@ -11644,7 +11644,7 @@
         <v>132</v>
       </c>
       <c r="C1019" t="n">
-        <v>409080</v>
+        <v>443170</v>
       </c>
     </row>
     <row r="1020">
@@ -11655,7 +11655,7 @@
         <v>2431</v>
       </c>
       <c r="C1020" t="n">
-        <v>100356</v>
+        <v>108719</v>
       </c>
     </row>
     <row r="1021">
@@ -11666,7 +11666,7 @@
         <v>2249</v>
       </c>
       <c r="C1021" t="n">
-        <v>106536</v>
+        <v>115414</v>
       </c>
     </row>
     <row r="1022">
@@ -11677,7 +11677,7 @@
         <v>1585</v>
       </c>
       <c r="C1022" t="n">
-        <v>90024</v>
+        <v>97526</v>
       </c>
     </row>
     <row r="1023">
@@ -11688,7 +11688,7 @@
         <v>2325</v>
       </c>
       <c r="C1023" t="n">
-        <v>87024</v>
+        <v>94276</v>
       </c>
     </row>
     <row r="1024">
@@ -11699,7 +11699,7 @@
         <v>2190</v>
       </c>
       <c r="C1024" t="n">
-        <v>122724</v>
+        <v>132951</v>
       </c>
     </row>
     <row r="1025">
@@ -11710,7 +11710,7 @@
         <v>1466</v>
       </c>
       <c r="C1025" t="n">
-        <v>220908</v>
+        <v>239317</v>
       </c>
     </row>
     <row r="1026">
@@ -11721,7 +11721,7 @@
         <v>2659</v>
       </c>
       <c r="C1026" t="n">
-        <v>67092</v>
+        <v>72683</v>
       </c>
     </row>
     <row r="1027">
@@ -11732,7 +11732,7 @@
         <v>634</v>
       </c>
       <c r="C1027" t="n">
-        <v>300000</v>
+        <v>325000</v>
       </c>
     </row>
     <row r="1028">
@@ -11743,7 +11743,7 @@
         <v>2804</v>
       </c>
       <c r="C1028" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1029">
@@ -11754,7 +11754,7 @@
         <v>2375</v>
       </c>
       <c r="C1029" t="n">
-        <v>180000</v>
+        <v>195000</v>
       </c>
     </row>
     <row r="1030">
@@ -11765,7 +11765,7 @@
         <v>2601</v>
       </c>
       <c r="C1030" t="n">
-        <v>150000</v>
+        <v>162500</v>
       </c>
     </row>
     <row r="1031">
@@ -11776,7 +11776,7 @@
         <v>952</v>
       </c>
       <c r="C1031" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1032">
@@ -11787,7 +11787,7 @@
         <v>571</v>
       </c>
       <c r="C1032" t="n">
-        <v>347172</v>
+        <v>376103</v>
       </c>
     </row>
     <row r="1033">
@@ -11798,7 +11798,7 @@
         <v>2697</v>
       </c>
       <c r="C1033" t="n">
-        <v>105780</v>
+        <v>114595</v>
       </c>
     </row>
     <row r="1034">
@@ -11809,7 +11809,7 @@
         <v>2678</v>
       </c>
       <c r="C1034" t="n">
-        <v>183012</v>
+        <v>198263</v>
       </c>
     </row>
     <row r="1035">
@@ -11820,7 +11820,7 @@
         <v>2768</v>
       </c>
       <c r="C1035" t="n">
-        <v>191532</v>
+        <v>207493</v>
       </c>
     </row>
     <row r="1036">
@@ -11831,7 +11831,7 @@
         <v>2359</v>
       </c>
       <c r="C1036" t="n">
-        <v>58092</v>
+        <v>62933</v>
       </c>
     </row>
     <row r="1037">
@@ -11842,7 +11842,7 @@
         <v>353</v>
       </c>
       <c r="C1037" t="n">
-        <v>188712</v>
+        <v>204438</v>
       </c>
     </row>
     <row r="1038">
@@ -11853,7 +11853,7 @@
         <v>2026</v>
       </c>
       <c r="C1038" t="n">
-        <v>156360</v>
+        <v>169390</v>
       </c>
     </row>
     <row r="1039">
@@ -11875,7 +11875,7 @@
         <v>2345</v>
       </c>
       <c r="C1040" t="n">
-        <v>34332</v>
+        <v>37193</v>
       </c>
     </row>
     <row r="1041">
@@ -11886,7 +11886,7 @@
         <v>2789</v>
       </c>
       <c r="C1041" t="n">
-        <v>92724</v>
+        <v>100451</v>
       </c>
     </row>
     <row r="1042">
@@ -11897,7 +11897,7 @@
         <v>569</v>
       </c>
       <c r="C1042" t="n">
-        <v>1562136</v>
+        <v>1692314</v>
       </c>
     </row>
     <row r="1043">
@@ -11908,7 +11908,7 @@
         <v>2822</v>
       </c>
       <c r="C1043" t="n">
-        <v>73632</v>
+        <v>79768</v>
       </c>
     </row>
     <row r="1044">
@@ -11919,7 +11919,7 @@
         <v>2728</v>
       </c>
       <c r="C1044" t="n">
-        <v>5448</v>
+        <v>5902</v>
       </c>
     </row>
     <row r="1045">
@@ -11930,7 +11930,7 @@
         <v>2488</v>
       </c>
       <c r="C1045" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1046">
@@ -11941,7 +11941,7 @@
         <v>2791</v>
       </c>
       <c r="C1046" t="n">
-        <v>53831</v>
+        <v>58316.9</v>
       </c>
     </row>
     <row r="1047">
@@ -11952,7 +11952,7 @@
         <v>2577</v>
       </c>
       <c r="C1047" t="n">
-        <v>48638.29</v>
+        <v>52691.47</v>
       </c>
     </row>
     <row r="1048">
@@ -11963,7 +11963,7 @@
         <v>2069</v>
       </c>
       <c r="C1048" t="n">
-        <v>98172</v>
+        <v>106353</v>
       </c>
     </row>
     <row r="1049">
@@ -11974,7 +11974,7 @@
         <v>2082</v>
       </c>
       <c r="C1049" t="n">
-        <v>90852</v>
+        <v>98423</v>
       </c>
     </row>
     <row r="1050">
@@ -11985,7 +11985,7 @@
         <v>781</v>
       </c>
       <c r="C1050" t="n">
-        <v>70908</v>
+        <v>76817</v>
       </c>
     </row>
     <row r="1051">
@@ -11996,7 +11996,7 @@
         <v>744</v>
       </c>
       <c r="C1051" t="n">
-        <v>22692</v>
+        <v>24583</v>
       </c>
     </row>
     <row r="1052">
@@ -12007,7 +12007,7 @@
         <v>2223</v>
       </c>
       <c r="C1052" t="n">
-        <v>71964</v>
+        <v>77961</v>
       </c>
     </row>
     <row r="1053">
@@ -12018,7 +12018,7 @@
         <v>2452</v>
       </c>
       <c r="C1053" t="n">
-        <v>38172</v>
+        <v>41353</v>
       </c>
     </row>
     <row r="1054">
@@ -12029,7 +12029,7 @@
         <v>970</v>
       </c>
       <c r="C1054" t="n">
-        <v>37464</v>
+        <v>40586</v>
       </c>
     </row>
     <row r="1055">
@@ -12040,7 +12040,7 @@
         <v>2550</v>
       </c>
       <c r="C1055" t="n">
-        <v>33264</v>
+        <v>36036</v>
       </c>
     </row>
     <row r="1056">
@@ -12051,7 +12051,7 @@
         <v>768</v>
       </c>
       <c r="C1056" t="n">
-        <v>70908</v>
+        <v>76817</v>
       </c>
     </row>
     <row r="1057">
@@ -12062,7 +12062,7 @@
         <v>1075</v>
       </c>
       <c r="C1057" t="n">
-        <v>247080</v>
+        <v>267670</v>
       </c>
     </row>
     <row r="1058">
@@ -12073,7 +12073,7 @@
         <v>664</v>
       </c>
       <c r="C1058" t="n">
-        <v>141264</v>
+        <v>153036</v>
       </c>
     </row>
     <row r="1059">
@@ -12084,7 +12084,7 @@
         <v>2555</v>
       </c>
       <c r="C1059" t="n">
-        <v>22644</v>
+        <v>24531</v>
       </c>
     </row>
     <row r="1060">
@@ -12095,7 +12095,7 @@
         <v>2627</v>
       </c>
       <c r="C1060" t="n">
-        <v>13296</v>
+        <v>14404</v>
       </c>
     </row>
     <row r="1061">
@@ -12106,7 +12106,7 @@
         <v>2557</v>
       </c>
       <c r="C1061" t="n">
-        <v>14064</v>
+        <v>15236</v>
       </c>
     </row>
     <row r="1062">
@@ -12117,7 +12117,7 @@
         <v>2551</v>
       </c>
       <c r="C1062" t="n">
-        <v>11172</v>
+        <v>12103</v>
       </c>
     </row>
     <row r="1063">
@@ -12128,7 +12128,7 @@
         <v>2463</v>
       </c>
       <c r="C1063" t="n">
-        <v>174660</v>
+        <v>189215</v>
       </c>
     </row>
     <row r="1064">
@@ -12139,7 +12139,7 @@
         <v>2279</v>
       </c>
       <c r="C1064" t="n">
-        <v>131772</v>
+        <v>142753</v>
       </c>
     </row>
     <row r="1065">
@@ -12150,7 +12150,7 @@
         <v>631</v>
       </c>
       <c r="C1065" t="n">
-        <v>190908</v>
+        <v>206817</v>
       </c>
     </row>
     <row r="1066">
@@ -12161,7 +12161,7 @@
         <v>2251</v>
       </c>
       <c r="C1066" t="n">
-        <v>116904</v>
+        <v>126646</v>
       </c>
     </row>
     <row r="1067">
@@ -12172,7 +12172,7 @@
         <v>1653</v>
       </c>
       <c r="C1067" t="n">
-        <v>177264</v>
+        <v>192036</v>
       </c>
     </row>
     <row r="1068">
@@ -12183,7 +12183,7 @@
         <v>1293</v>
       </c>
       <c r="C1068" t="n">
-        <v>226356</v>
+        <v>245219</v>
       </c>
     </row>
     <row r="1069">
@@ -12194,7 +12194,7 @@
         <v>360</v>
       </c>
       <c r="C1069" t="n">
-        <v>272724</v>
+        <v>295451</v>
       </c>
     </row>
     <row r="1070">
@@ -12205,7 +12205,7 @@
         <v>1063</v>
       </c>
       <c r="C1070" t="n">
-        <v>198300</v>
+        <v>214825</v>
       </c>
     </row>
     <row r="1071">
@@ -12216,7 +12216,7 @@
         <v>2273</v>
       </c>
       <c r="C1071" t="n">
-        <v>115680</v>
+        <v>125320</v>
       </c>
     </row>
     <row r="1072">
@@ -12227,7 +12227,7 @@
         <v>2757</v>
       </c>
       <c r="C1072" t="n">
-        <v>38181.9</v>
+        <v>41363.71</v>
       </c>
     </row>
     <row r="1073">
@@ -12238,7 +12238,7 @@
         <v>2795</v>
       </c>
       <c r="C1073" t="n">
-        <v>32727.3</v>
+        <v>35454.57</v>
       </c>
     </row>
     <row r="1074">
@@ -12249,7 +12249,7 @@
         <v>2722</v>
       </c>
       <c r="C1074" t="n">
-        <v>32724</v>
+        <v>35451</v>
       </c>
     </row>
     <row r="1075">
@@ -12260,7 +12260,7 @@
         <v>2718</v>
       </c>
       <c r="C1075" t="n">
-        <v>43632</v>
+        <v>47268</v>
       </c>
     </row>
     <row r="1076">
@@ -12271,7 +12271,7 @@
         <v>595</v>
       </c>
       <c r="C1076" t="n">
-        <v>300000</v>
+        <v>325000</v>
       </c>
     </row>
     <row r="1077">
@@ -12282,7 +12282,7 @@
         <v>890</v>
       </c>
       <c r="C1077" t="n">
-        <v>381816</v>
+        <v>413634</v>
       </c>
     </row>
     <row r="1078">
@@ -12293,7 +12293,7 @@
         <v>2652</v>
       </c>
       <c r="C1078" t="n">
-        <v>70908</v>
+        <v>76817</v>
       </c>
     </row>
     <row r="1079">
@@ -12304,7 +12304,7 @@
         <v>2714</v>
       </c>
       <c r="C1079" t="n">
-        <v>196356</v>
+        <v>212719</v>
       </c>
     </row>
     <row r="1080">
@@ -12315,7 +12315,7 @@
         <v>1869</v>
       </c>
       <c r="C1080" t="n">
-        <v>125448</v>
+        <v>135902</v>
       </c>
     </row>
     <row r="1081">
@@ -12326,7 +12326,7 @@
         <v>400</v>
       </c>
       <c r="C1081" t="n">
-        <v>103632</v>
+        <v>112268</v>
       </c>
     </row>
     <row r="1082">
@@ -12337,7 +12337,7 @@
         <v>1907</v>
       </c>
       <c r="C1082" t="n">
-        <v>202356</v>
+        <v>219219</v>
       </c>
     </row>
     <row r="1083">
@@ -12348,7 +12348,7 @@
         <v>1996</v>
       </c>
       <c r="C1083" t="n">
-        <v>127908</v>
+        <v>138567</v>
       </c>
     </row>
     <row r="1084">
@@ -12356,10 +12356,10 @@
         <v>46266</v>
       </c>
       <c r="B1084" t="n">
-        <v>2114</v>
+        <v>1890</v>
       </c>
       <c r="C1084" t="n">
-        <v>100200</v>
+        <v>186811.64</v>
       </c>
     </row>
     <row r="1085">
@@ -12367,10 +12367,10 @@
         <v>46266</v>
       </c>
       <c r="B1085" t="n">
-        <v>2330</v>
+        <v>2114</v>
       </c>
       <c r="C1085" t="n">
-        <v>146604</v>
+        <v>108550</v>
       </c>
     </row>
     <row r="1086">
@@ -12378,10 +12378,10 @@
         <v>46266</v>
       </c>
       <c r="B1086" t="n">
-        <v>2000</v>
+        <v>2330</v>
       </c>
       <c r="C1086" t="n">
-        <v>0</v>
+        <v>158821</v>
       </c>
     </row>
     <row r="1087">
@@ -12389,7 +12389,7 @@
         <v>46266</v>
       </c>
       <c r="B1087" t="n">
-        <v>2591</v>
+        <v>2000</v>
       </c>
       <c r="C1087" t="n">
         <v>0</v>
@@ -12400,7 +12400,7 @@
         <v>46266</v>
       </c>
       <c r="B1088" t="n">
-        <v>2639</v>
+        <v>2591</v>
       </c>
       <c r="C1088" t="n">
         <v>0</v>
@@ -12411,10 +12411,10 @@
         <v>46266</v>
       </c>
       <c r="B1089" t="n">
-        <v>931</v>
+        <v>2639</v>
       </c>
       <c r="C1089" t="n">
-        <v>51504</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1090">
@@ -12422,10 +12422,10 @@
         <v>46266</v>
       </c>
       <c r="B1090" t="n">
-        <v>947</v>
+        <v>931</v>
       </c>
       <c r="C1090" t="n">
-        <v>237012</v>
+        <v>55796</v>
       </c>
     </row>
     <row r="1091">
@@ -12436,7 +12436,7 @@
         <v>951</v>
       </c>
       <c r="C1091" t="n">
-        <v>62724</v>
+        <v>67951</v>
       </c>
     </row>
     <row r="1092">
@@ -12447,7 +12447,7 @@
         <v>2449</v>
       </c>
       <c r="C1092" t="n">
-        <v>21816</v>
+        <v>23634</v>
       </c>
     </row>
     <row r="1093">
@@ -12458,7 +12458,7 @@
         <v>610</v>
       </c>
       <c r="C1093" t="n">
-        <v>444540</v>
+        <v>481585</v>
       </c>
     </row>
     <row r="1094">
@@ -12469,7 +12469,7 @@
         <v>2761</v>
       </c>
       <c r="C1094" t="n">
-        <v>44448</v>
+        <v>48152</v>
       </c>
     </row>
     <row r="1095">
@@ -12480,7 +12480,7 @@
         <v>483</v>
       </c>
       <c r="C1095" t="n">
-        <v>241632</v>
+        <v>261768</v>
       </c>
     </row>
     <row r="1096">
@@ -12491,7 +12491,7 @@
         <v>2015</v>
       </c>
       <c r="C1096" t="n">
-        <v>201816</v>
+        <v>218634</v>
       </c>
     </row>
     <row r="1097">
@@ -12502,7 +12502,7 @@
         <v>1478</v>
       </c>
       <c r="C1097" t="n">
-        <v>295176</v>
+        <v>319774</v>
       </c>
     </row>
     <row r="1098">
@@ -12513,7 +12513,7 @@
         <v>424</v>
       </c>
       <c r="C1098" t="n">
-        <v>131772</v>
+        <v>142753</v>
       </c>
     </row>
     <row r="1099">
@@ -12535,7 +12535,7 @@
         <v>477</v>
       </c>
       <c r="C1100" t="n">
-        <v>141084</v>
+        <v>152841</v>
       </c>
     </row>
     <row r="1101">
@@ -12546,7 +12546,7 @@
         <v>1810</v>
       </c>
       <c r="C1101" t="n">
-        <v>21852</v>
+        <v>23673</v>
       </c>
     </row>
     <row r="1102">
@@ -12557,7 +12557,7 @@
         <v>2826</v>
       </c>
       <c r="C1102" t="n">
-        <v>38181.9</v>
+        <v>41363.71</v>
       </c>
     </row>
     <row r="1103">
@@ -12568,7 +12568,7 @@
         <v>2561</v>
       </c>
       <c r="C1103" t="n">
-        <v>8016</v>
+        <v>8684</v>
       </c>
     </row>
     <row r="1104">
@@ -12579,7 +12579,7 @@
         <v>2653</v>
       </c>
       <c r="C1104" t="n">
-        <v>32727.3</v>
+        <v>35454.57</v>
       </c>
     </row>
     <row r="1105">
@@ -12590,7 +12590,7 @@
         <v>2829</v>
       </c>
       <c r="C1105" t="n">
-        <v>32727.3</v>
+        <v>35454.57</v>
       </c>
     </row>
     <row r="1106">
@@ -12601,7 +12601,7 @@
         <v>2643</v>
       </c>
       <c r="C1106" t="n">
-        <v>16104</v>
+        <v>17446</v>
       </c>
     </row>
     <row r="1107">
@@ -12612,7 +12612,7 @@
         <v>2794</v>
       </c>
       <c r="C1107" t="n">
-        <v>49080</v>
+        <v>53170</v>
       </c>
     </row>
     <row r="1108">
@@ -12623,7 +12623,7 @@
         <v>2655</v>
       </c>
       <c r="C1108" t="n">
-        <v>60000</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="1109">
@@ -12634,7 +12634,7 @@
         <v>1456</v>
       </c>
       <c r="C1109" t="n">
-        <v>420156</v>
+        <v>455169</v>
       </c>
     </row>
     <row r="1110">
@@ -12645,7 +12645,7 @@
         <v>2606</v>
       </c>
       <c r="C1110" t="n">
-        <v>129048</v>
+        <v>139802</v>
       </c>
     </row>
     <row r="1111">
@@ -12656,7 +12656,7 @@
         <v>1142</v>
       </c>
       <c r="C1111" t="n">
-        <v>234024</v>
+        <v>253526</v>
       </c>
     </row>
     <row r="1112">
@@ -12667,7 +12667,7 @@
         <v>1450</v>
       </c>
       <c r="C1112" t="n">
-        <v>148668</v>
+        <v>161057</v>
       </c>
     </row>
     <row r="1113">
@@ -12678,7 +12678,7 @@
         <v>2133</v>
       </c>
       <c r="C1113" t="n">
-        <v>347172</v>
+        <v>376103</v>
       </c>
     </row>
     <row r="1114">
@@ -12689,7 +12689,7 @@
         <v>522</v>
       </c>
       <c r="C1114" t="n">
-        <v>106356</v>
+        <v>115219</v>
       </c>
     </row>
     <row r="1115">
@@ -12700,7 +12700,7 @@
         <v>2696</v>
       </c>
       <c r="C1115" t="n">
-        <v>143520</v>
+        <v>155480</v>
       </c>
     </row>
     <row r="1116">
@@ -12722,7 +12722,7 @@
         <v>2692</v>
       </c>
       <c r="C1117" t="n">
-        <v>40908</v>
+        <v>44317</v>
       </c>
     </row>
     <row r="1118">
@@ -12733,7 +12733,7 @@
         <v>2691</v>
       </c>
       <c r="C1118" t="n">
-        <v>73632</v>
+        <v>79768</v>
       </c>
     </row>
     <row r="1119">
@@ -12744,7 +12744,7 @@
         <v>1632</v>
       </c>
       <c r="C1119" t="n">
-        <v>136356</v>
+        <v>147719</v>
       </c>
     </row>
     <row r="1120">
@@ -12755,7 +12755,7 @@
         <v>2641</v>
       </c>
       <c r="C1120" t="n">
-        <v>43632</v>
+        <v>47268</v>
       </c>
     </row>
     <row r="1121">
@@ -12766,7 +12766,7 @@
         <v>2197</v>
       </c>
       <c r="C1121" t="n">
-        <v>109080</v>
+        <v>118170</v>
       </c>
     </row>
     <row r="1122">
@@ -12777,7 +12777,7 @@
         <v>609</v>
       </c>
       <c r="C1122" t="n">
-        <v>120000</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="1123">
@@ -12788,7 +12788,7 @@
         <v>1380</v>
       </c>
       <c r="C1123" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1124">
@@ -12799,7 +12799,7 @@
         <v>104</v>
       </c>
       <c r="C1124" t="n">
-        <v>163632</v>
+        <v>177268</v>
       </c>
     </row>
     <row r="1125">
@@ -12810,7 +12810,7 @@
         <v>2621</v>
       </c>
       <c r="C1125" t="n">
-        <v>38172</v>
+        <v>41353</v>
       </c>
     </row>
     <row r="1126">
@@ -12821,7 +12821,7 @@
         <v>2786</v>
       </c>
       <c r="C1126" t="n">
-        <v>38172</v>
+        <v>41353</v>
       </c>
     </row>
     <row r="1127">
@@ -12832,7 +12832,7 @@
         <v>2784</v>
       </c>
       <c r="C1127" t="n">
-        <v>22692</v>
+        <v>24583</v>
       </c>
     </row>
     <row r="1128">
@@ -12843,7 +12843,7 @@
         <v>2586</v>
       </c>
       <c r="C1128" t="n">
-        <v>22692</v>
+        <v>24583</v>
       </c>
     </row>
     <row r="1129">
@@ -12854,7 +12854,7 @@
         <v>2145</v>
       </c>
       <c r="C1129" t="n">
-        <v>70608</v>
+        <v>76492</v>
       </c>
     </row>
     <row r="1130">
@@ -12865,7 +12865,7 @@
         <v>2574</v>
       </c>
       <c r="C1130" t="n">
-        <v>70608</v>
+        <v>76492</v>
       </c>
     </row>
     <row r="1131">
@@ -12876,7 +12876,7 @@
         <v>2492</v>
       </c>
       <c r="C1131" t="n">
-        <v>77400</v>
+        <v>83850</v>
       </c>
     </row>
     <row r="1132">
@@ -12887,7 +12887,7 @@
         <v>629</v>
       </c>
       <c r="C1132" t="n">
-        <v>241080</v>
+        <v>261170</v>
       </c>
     </row>
     <row r="1133">
@@ -12898,7 +12898,7 @@
         <v>966</v>
       </c>
       <c r="C1133" t="n">
-        <v>44448</v>
+        <v>48152</v>
       </c>
     </row>
     <row r="1134">
@@ -12909,7 +12909,7 @@
         <v>2721</v>
       </c>
       <c r="C1134" t="n">
-        <v>44448</v>
+        <v>48152</v>
       </c>
     </row>
     <row r="1135">
@@ -12920,7 +12920,7 @@
         <v>2554</v>
       </c>
       <c r="C1135" t="n">
-        <v>13392</v>
+        <v>14508</v>
       </c>
     </row>
     <row r="1136">
@@ -12931,7 +12931,7 @@
         <v>2556</v>
       </c>
       <c r="C1136" t="n">
-        <v>19692</v>
+        <v>21333</v>
       </c>
     </row>
     <row r="1137">
@@ -12942,7 +12942,7 @@
         <v>2546</v>
       </c>
       <c r="C1137" t="n">
-        <v>13008</v>
+        <v>14092</v>
       </c>
     </row>
     <row r="1138">
@@ -12953,7 +12953,7 @@
         <v>42</v>
       </c>
       <c r="C1138" t="n">
-        <v>1030908</v>
+        <v>1116817</v>
       </c>
     </row>
     <row r="1139">
@@ -12964,7 +12964,7 @@
         <v>953</v>
       </c>
       <c r="C1139" t="n">
-        <v>372360</v>
+        <v>403390</v>
       </c>
     </row>
     <row r="1140">
@@ -12975,7 +12975,7 @@
         <v>675</v>
       </c>
       <c r="C1140" t="n">
-        <v>109080</v>
+        <v>118170</v>
       </c>
     </row>
     <row r="1141">
@@ -12986,7 +12986,7 @@
         <v>619</v>
       </c>
       <c r="C1141" t="n">
-        <v>168672</v>
+        <v>182728</v>
       </c>
     </row>
     <row r="1142">
@@ -12997,7 +12997,7 @@
         <v>1299</v>
       </c>
       <c r="C1142" t="n">
-        <v>283824</v>
+        <v>307476</v>
       </c>
     </row>
     <row r="1143">
@@ -13008,7 +13008,7 @@
         <v>1064</v>
       </c>
       <c r="C1143" t="n">
-        <v>326928</v>
+        <v>354172</v>
       </c>
     </row>
     <row r="1144">
@@ -13019,7 +13019,7 @@
         <v>2308</v>
       </c>
       <c r="C1144" t="n">
-        <v>111816</v>
+        <v>121134</v>
       </c>
     </row>
     <row r="1145">
@@ -13030,7 +13030,7 @@
         <v>1137</v>
       </c>
       <c r="C1145" t="n">
-        <v>349080</v>
+        <v>378170</v>
       </c>
     </row>
     <row r="1146">
@@ -13041,7 +13041,7 @@
         <v>2747</v>
       </c>
       <c r="C1146" t="n">
-        <v>32727.3</v>
+        <v>35454.57</v>
       </c>
     </row>
     <row r="1147">
@@ -13052,7 +13052,7 @@
         <v>2819</v>
       </c>
       <c r="C1147" t="n">
-        <v>32727.3</v>
+        <v>35454.57</v>
       </c>
     </row>
     <row r="1148">
@@ -13063,7 +13063,7 @@
         <v>1259</v>
       </c>
       <c r="C1148" t="n">
-        <v>54545.5</v>
+        <v>59090.95</v>
       </c>
     </row>
     <row r="1149">
@@ -13074,7 +13074,7 @@
         <v>2544</v>
       </c>
       <c r="C1149" t="n">
-        <v>43632</v>
+        <v>47268</v>
       </c>
     </row>
     <row r="1150">
@@ -13085,7 +13085,7 @@
         <v>2261</v>
       </c>
       <c r="C1150" t="n">
-        <v>81816</v>
+        <v>88634</v>
       </c>
     </row>
     <row r="1151">
@@ -13096,7 +13096,7 @@
         <v>2729</v>
       </c>
       <c r="C1151" t="n">
-        <v>43632</v>
+        <v>47268</v>
       </c>
     </row>
     <row r="1152">
@@ -13107,7 +13107,7 @@
         <v>2649</v>
       </c>
       <c r="C1152" t="n">
-        <v>16104</v>
+        <v>17446</v>
       </c>
     </row>
     <row r="1153">
@@ -13118,7 +13118,7 @@
         <v>2494</v>
       </c>
       <c r="C1153" t="n">
-        <v>70908</v>
+        <v>76817</v>
       </c>
     </row>
     <row r="1154">
@@ -13129,7 +13129,7 @@
         <v>1384</v>
       </c>
       <c r="C1154" t="n">
-        <v>245448</v>
+        <v>265902</v>
       </c>
     </row>
     <row r="1155">
@@ -13151,7 +13151,7 @@
         <v>2802</v>
       </c>
       <c r="C1156" t="n">
-        <v>38628</v>
+        <v>41847</v>
       </c>
     </row>
     <row r="1157">
@@ -13162,7 +13162,7 @@
         <v>2726</v>
       </c>
       <c r="C1157" t="n">
-        <v>81816</v>
+        <v>88634</v>
       </c>
     </row>
     <row r="1158">
@@ -13173,7 +13173,7 @@
         <v>2820</v>
       </c>
       <c r="C1158" t="n">
-        <v>98172</v>
+        <v>106353</v>
       </c>
     </row>
     <row r="1159">
@@ -13184,7 +13184,7 @@
         <v>1007</v>
       </c>
       <c r="C1159" t="n">
-        <v>103632</v>
+        <v>112268</v>
       </c>
     </row>
     <row r="1160">
@@ -13195,7 +13195,7 @@
         <v>20</v>
       </c>
       <c r="C1160" t="n">
-        <v>210000</v>
+        <v>227500</v>
       </c>
     </row>
     <row r="1161">
@@ -13206,7 +13206,7 @@
         <v>1372</v>
       </c>
       <c r="C1161" t="n">
-        <v>158172</v>
+        <v>171353</v>
       </c>
     </row>
     <row r="1162">
@@ -13217,7 +13217,7 @@
         <v>2735</v>
       </c>
       <c r="C1162" t="n">
-        <v>65448</v>
+        <v>70902</v>
       </c>
     </row>
     <row r="1163">
@@ -13228,7 +13228,7 @@
         <v>2811</v>
       </c>
       <c r="C1163" t="n">
-        <v>22692</v>
+        <v>24583</v>
       </c>
     </row>
     <row r="1164">
@@ -13239,7 +13239,7 @@
         <v>1871</v>
       </c>
       <c r="C1164" t="n">
-        <v>96408</v>
+        <v>104442</v>
       </c>
     </row>
     <row r="1165">
@@ -13250,7 +13250,7 @@
         <v>2541</v>
       </c>
       <c r="C1165" t="n">
-        <v>115416</v>
+        <v>125034</v>
       </c>
     </row>
     <row r="1166">
@@ -13261,7 +13261,7 @@
         <v>2362</v>
       </c>
       <c r="C1166" t="n">
-        <v>40908</v>
+        <v>44317</v>
       </c>
     </row>
     <row r="1167">
@@ -13272,7 +13272,7 @@
         <v>1324</v>
       </c>
       <c r="C1167" t="n">
-        <v>152724</v>
+        <v>165451</v>
       </c>
     </row>
     <row r="1168">
@@ -13283,7 +13283,7 @@
         <v>2323</v>
       </c>
       <c r="C1168" t="n">
-        <v>37464</v>
+        <v>40586</v>
       </c>
     </row>
     <row r="1169">
@@ -13294,7 +13294,7 @@
         <v>2647</v>
       </c>
       <c r="C1169" t="n">
-        <v>77400</v>
+        <v>83850</v>
       </c>
     </row>
     <row r="1170">
@@ -13305,7 +13305,7 @@
         <v>559</v>
       </c>
       <c r="C1170" t="n">
-        <v>125148</v>
+        <v>135577</v>
       </c>
     </row>
     <row r="1171">
@@ -13316,7 +13316,7 @@
         <v>2762</v>
       </c>
       <c r="C1171" t="n">
-        <v>44448</v>
+        <v>48152</v>
       </c>
     </row>
     <row r="1172">
@@ -13327,7 +13327,7 @@
         <v>2501</v>
       </c>
       <c r="C1172" t="n">
-        <v>44448</v>
+        <v>48152</v>
       </c>
     </row>
     <row r="1173">
@@ -13338,7 +13338,7 @@
         <v>2562</v>
       </c>
       <c r="C1173" t="n">
-        <v>8628</v>
+        <v>9347</v>
       </c>
     </row>
     <row r="1174">
@@ -13349,7 +13349,7 @@
         <v>429</v>
       </c>
       <c r="C1174" t="n">
-        <v>212724</v>
+        <v>230451</v>
       </c>
     </row>
     <row r="1175">
@@ -13360,7 +13360,7 @@
         <v>58</v>
       </c>
       <c r="C1175" t="n">
-        <v>147588</v>
+        <v>159887</v>
       </c>
     </row>
     <row r="1176">
@@ -13371,7 +13371,7 @@
         <v>2245</v>
       </c>
       <c r="C1176" t="n">
-        <v>131772</v>
+        <v>142753</v>
       </c>
     </row>
     <row r="1177">
@@ -13382,7 +13382,7 @@
         <v>285</v>
       </c>
       <c r="C1177" t="n">
-        <v>295176</v>
+        <v>319774</v>
       </c>
     </row>
     <row r="1178">
@@ -13404,7 +13404,7 @@
         <v>363</v>
       </c>
       <c r="C1179" t="n">
-        <v>163632</v>
+        <v>177268</v>
       </c>
     </row>
     <row r="1180">
@@ -13415,7 +13415,7 @@
         <v>2651</v>
       </c>
       <c r="C1180" t="n">
-        <v>92244</v>
+        <v>99931</v>
       </c>
     </row>
     <row r="1181">
@@ -13426,7 +13426,7 @@
         <v>2142</v>
       </c>
       <c r="C1181" t="n">
-        <v>29112</v>
+        <v>31538</v>
       </c>
     </row>
     <row r="1182">
@@ -13437,7 +13437,7 @@
         <v>2258</v>
       </c>
       <c r="C1182" t="n">
-        <v>43636.4</v>
+        <v>47272.76</v>
       </c>
     </row>
     <row r="1183">
@@ -13448,7 +13448,7 @@
         <v>2772</v>
       </c>
       <c r="C1183" t="n">
-        <v>32727.3</v>
+        <v>35454.57</v>
       </c>
     </row>
     <row r="1184">
@@ -13459,7 +13459,7 @@
         <v>2346</v>
       </c>
       <c r="C1184" t="n">
-        <v>60000</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="1185">
@@ -13470,7 +13470,7 @@
         <v>2442</v>
       </c>
       <c r="C1185" t="n">
-        <v>43632</v>
+        <v>47268</v>
       </c>
     </row>
     <row r="1186">
@@ -13481,7 +13481,7 @@
         <v>772</v>
       </c>
       <c r="C1186" t="n">
-        <v>180000</v>
+        <v>195000</v>
       </c>
     </row>
     <row r="1187">
@@ -13492,7 +13492,7 @@
         <v>2684</v>
       </c>
       <c r="C1187" t="n">
-        <v>51816</v>
+        <v>56134</v>
       </c>
     </row>
     <row r="1188">
@@ -13503,7 +13503,7 @@
         <v>2765</v>
       </c>
       <c r="C1188" t="n">
-        <v>49080</v>
+        <v>53170</v>
       </c>
     </row>
     <row r="1189">
@@ -13514,7 +13514,7 @@
         <v>2567</v>
       </c>
       <c r="C1189" t="n">
-        <v>90024</v>
+        <v>97526</v>
       </c>
     </row>
     <row r="1190">
@@ -13525,7 +13525,7 @@
         <v>2178</v>
       </c>
       <c r="C1190" t="n">
-        <v>152724</v>
+        <v>165451</v>
       </c>
     </row>
     <row r="1191">
@@ -13536,7 +13536,7 @@
         <v>2827</v>
       </c>
       <c r="C1191" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1192">
@@ -13547,7 +13547,7 @@
         <v>2510</v>
       </c>
       <c r="C1192" t="n">
-        <v>302856</v>
+        <v>328094</v>
       </c>
     </row>
     <row r="1193">
@@ -13558,7 +13558,7 @@
         <v>2392</v>
       </c>
       <c r="C1193" t="n">
-        <v>90852</v>
+        <v>98423</v>
       </c>
     </row>
     <row r="1194">
@@ -13569,7 +13569,7 @@
         <v>415</v>
       </c>
       <c r="C1194" t="n">
-        <v>310632</v>
+        <v>336518</v>
       </c>
     </row>
     <row r="1195">
@@ -13580,7 +13580,7 @@
         <v>2107</v>
       </c>
       <c r="C1195" t="n">
-        <v>160404</v>
+        <v>173771</v>
       </c>
     </row>
     <row r="1196">
@@ -13591,7 +13591,7 @@
         <v>2211</v>
       </c>
       <c r="C1196" t="n">
-        <v>132984</v>
+        <v>144066</v>
       </c>
     </row>
     <row r="1197">
@@ -13602,7 +13602,7 @@
         <v>2682</v>
       </c>
       <c r="C1197" t="n">
-        <v>81804</v>
+        <v>88621</v>
       </c>
     </row>
     <row r="1198">
@@ -13635,7 +13635,7 @@
         <v>2755</v>
       </c>
       <c r="C1200" t="n">
-        <v>32724</v>
+        <v>35451</v>
       </c>
     </row>
     <row r="1201">
@@ -13646,7 +13646,7 @@
         <v>941</v>
       </c>
       <c r="C1201" t="n">
-        <v>214296</v>
+        <v>232154</v>
       </c>
     </row>
     <row r="1202">
@@ -13657,7 +13657,7 @@
         <v>2734</v>
       </c>
       <c r="C1202" t="n">
-        <v>30036</v>
+        <v>32539</v>
       </c>
     </row>
     <row r="1203">
@@ -13668,7 +13668,7 @@
         <v>1289</v>
       </c>
       <c r="C1203" t="n">
-        <v>136356</v>
+        <v>147719</v>
       </c>
     </row>
     <row r="1204">
@@ -13679,7 +13679,7 @@
         <v>2801</v>
       </c>
       <c r="C1204" t="n">
-        <v>43632</v>
+        <v>47268</v>
       </c>
     </row>
     <row r="1205">
@@ -13690,7 +13690,7 @@
         <v>2810</v>
       </c>
       <c r="C1205" t="n">
-        <v>73632</v>
+        <v>79768</v>
       </c>
     </row>
     <row r="1206">
@@ -13701,7 +13701,7 @@
         <v>767</v>
       </c>
       <c r="C1206" t="n">
-        <v>98172</v>
+        <v>106353</v>
       </c>
     </row>
     <row r="1207">
@@ -13712,7 +13712,7 @@
         <v>2687</v>
       </c>
       <c r="C1207" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1208">
@@ -13723,7 +13723,7 @@
         <v>2686</v>
       </c>
       <c r="C1208" t="n">
-        <v>70908</v>
+        <v>76817</v>
       </c>
     </row>
     <row r="1209">
@@ -13734,7 +13734,7 @@
         <v>2730</v>
       </c>
       <c r="C1209" t="n">
-        <v>49080</v>
+        <v>53170</v>
       </c>
     </row>
     <row r="1210">
@@ -13745,7 +13745,7 @@
         <v>2580</v>
       </c>
       <c r="C1210" t="n">
-        <v>18300</v>
+        <v>19825</v>
       </c>
     </row>
     <row r="1211">
@@ -13756,7 +13756,7 @@
         <v>2472</v>
       </c>
       <c r="C1211" t="n">
-        <v>28877.5</v>
+        <v>31283.95</v>
       </c>
     </row>
     <row r="1212">
@@ -13767,7 +13767,7 @@
         <v>2631</v>
       </c>
       <c r="C1212" t="n">
-        <v>13381.1</v>
+        <v>14496.19</v>
       </c>
     </row>
     <row r="1213">
@@ -13778,7 +13778,7 @@
         <v>1642</v>
       </c>
       <c r="C1213" t="n">
-        <v>144540</v>
+        <v>156585</v>
       </c>
     </row>
     <row r="1214">
@@ -13789,7 +13789,7 @@
         <v>2613</v>
       </c>
       <c r="C1214" t="n">
-        <v>97740</v>
+        <v>105885</v>
       </c>
     </row>
     <row r="1215">
@@ -13800,7 +13800,7 @@
         <v>1020</v>
       </c>
       <c r="C1215" t="n">
-        <v>49080</v>
+        <v>53170</v>
       </c>
     </row>
     <row r="1216">
@@ -13811,7 +13811,7 @@
         <v>2785</v>
       </c>
       <c r="C1216" t="n">
-        <v>22692</v>
+        <v>24583</v>
       </c>
     </row>
     <row r="1217">
@@ -13822,7 +13822,7 @@
         <v>1327</v>
       </c>
       <c r="C1217" t="n">
-        <v>32724</v>
+        <v>35451</v>
       </c>
     </row>
     <row r="1218">
@@ -13833,7 +13833,7 @@
         <v>2629</v>
       </c>
       <c r="C1218" t="n">
-        <v>37464</v>
+        <v>40586</v>
       </c>
     </row>
     <row r="1219">
@@ -13844,7 +13844,7 @@
         <v>749</v>
       </c>
       <c r="C1219" t="n">
-        <v>44448</v>
+        <v>48152</v>
       </c>
     </row>
     <row r="1220">
@@ -13855,7 +13855,7 @@
         <v>1983</v>
       </c>
       <c r="C1220" t="n">
-        <v>295176</v>
+        <v>319774</v>
       </c>
     </row>
     <row r="1221">
@@ -13866,7 +13866,7 @@
         <v>1993</v>
       </c>
       <c r="C1221" t="n">
-        <v>189756</v>
+        <v>205569</v>
       </c>
     </row>
     <row r="1222">
@@ -13877,7 +13877,7 @@
         <v>2767</v>
       </c>
       <c r="C1222" t="n">
-        <v>105228</v>
+        <v>113997</v>
       </c>
     </row>
     <row r="1223">
@@ -13899,7 +13899,7 @@
         <v>1102</v>
       </c>
       <c r="C1224" t="n">
-        <v>131772</v>
+        <v>142753</v>
       </c>
     </row>
     <row r="1225">
@@ -13910,7 +13910,7 @@
         <v>626</v>
       </c>
       <c r="C1225" t="n">
-        <v>929626.4</v>
+        <v>1007095.26</v>
       </c>
     </row>
     <row r="1226">
@@ -13921,7 +13921,7 @@
         <v>1465</v>
       </c>
       <c r="C1226" t="n">
-        <v>196248</v>
+        <v>212602</v>
       </c>
     </row>
     <row r="1227">
@@ -13932,7 +13932,7 @@
         <v>2758</v>
       </c>
       <c r="C1227" t="n">
-        <v>32727.3</v>
+        <v>35454.57</v>
       </c>
     </row>
     <row r="1228">
@@ -13943,7 +13943,7 @@
         <v>2742</v>
       </c>
       <c r="C1228" t="n">
-        <v>32727.3</v>
+        <v>35454.57</v>
       </c>
     </row>
     <row r="1229">
@@ -13965,7 +13965,7 @@
         <v>1873</v>
       </c>
       <c r="C1230" t="n">
-        <v>174540</v>
+        <v>189085</v>
       </c>
     </row>
     <row r="1231">
@@ -13976,7 +13976,7 @@
         <v>2163</v>
       </c>
       <c r="C1231" t="n">
-        <v>81816</v>
+        <v>88634</v>
       </c>
     </row>
     <row r="1232">
@@ -13987,7 +13987,7 @@
         <v>2394</v>
       </c>
       <c r="C1232" t="n">
-        <v>84024</v>
+        <v>91026</v>
       </c>
     </row>
     <row r="1233">
@@ -13998,7 +13998,7 @@
         <v>33</v>
       </c>
       <c r="C1233" t="n">
-        <v>211632</v>
+        <v>229268</v>
       </c>
     </row>
     <row r="1234">
@@ -14009,7 +14009,7 @@
         <v>2421</v>
       </c>
       <c r="C1234" t="n">
-        <v>35448</v>
+        <v>38402</v>
       </c>
     </row>
     <row r="1235">
@@ -14020,7 +14020,7 @@
         <v>2663</v>
       </c>
       <c r="C1235" t="n">
-        <v>150000</v>
+        <v>162500</v>
       </c>
     </row>
     <row r="1236">
@@ -14031,7 +14031,7 @@
         <v>2413</v>
       </c>
       <c r="C1236" t="n">
-        <v>66024</v>
+        <v>71526</v>
       </c>
     </row>
     <row r="1237">
@@ -14042,7 +14042,7 @@
         <v>351</v>
       </c>
       <c r="C1237" t="n">
-        <v>100356</v>
+        <v>108719</v>
       </c>
     </row>
     <row r="1238">
@@ -14053,7 +14053,7 @@
         <v>1298</v>
       </c>
       <c r="C1238" t="n">
-        <v>694356</v>
+        <v>752219</v>
       </c>
     </row>
     <row r="1239">
@@ -14064,7 +14064,7 @@
         <v>2491</v>
       </c>
       <c r="C1239" t="n">
-        <v>56112</v>
+        <v>60788</v>
       </c>
     </row>
     <row r="1240">
@@ -14075,7 +14075,7 @@
         <v>2571</v>
       </c>
       <c r="C1240" t="n">
-        <v>79236</v>
+        <v>85839</v>
       </c>
     </row>
     <row r="1241">
@@ -14086,7 +14086,7 @@
         <v>2507</v>
       </c>
       <c r="C1241" t="n">
-        <v>48144</v>
+        <v>52156</v>
       </c>
     </row>
     <row r="1242">
@@ -14097,7 +14097,7 @@
         <v>2799</v>
       </c>
       <c r="C1242" t="n">
-        <v>61968</v>
+        <v>67132</v>
       </c>
     </row>
     <row r="1243">
@@ -14119,7 +14119,7 @@
         <v>2582</v>
       </c>
       <c r="C1244" t="n">
-        <v>47208</v>
+        <v>51142</v>
       </c>
     </row>
     <row r="1245">
@@ -14130,7 +14130,7 @@
         <v>2637</v>
       </c>
       <c r="C1245" t="n">
-        <v>34332</v>
+        <v>37193</v>
       </c>
     </row>
     <row r="1246">
@@ -14141,7 +14141,7 @@
         <v>630</v>
       </c>
       <c r="C1246" t="n">
-        <v>81648</v>
+        <v>88452</v>
       </c>
     </row>
     <row r="1247">
@@ -14152,7 +14152,7 @@
         <v>525</v>
       </c>
       <c r="C1247" t="n">
-        <v>122724</v>
+        <v>132951</v>
       </c>
     </row>
     <row r="1248">
@@ -14163,7 +14163,7 @@
         <v>2727</v>
       </c>
       <c r="C1248" t="n">
-        <v>22080</v>
+        <v>23920</v>
       </c>
     </row>
     <row r="1249">
@@ -14174,7 +14174,7 @@
         <v>2707</v>
       </c>
       <c r="C1249" t="n">
-        <v>17472</v>
+        <v>18928</v>
       </c>
     </row>
     <row r="1250">
@@ -14185,7 +14185,7 @@
         <v>2834</v>
       </c>
       <c r="C1250" t="n">
-        <v>9026.200000000001</v>
+        <v>9778.379999999999</v>
       </c>
     </row>
     <row r="1251">
@@ -14196,7 +14196,7 @@
         <v>2773</v>
       </c>
       <c r="C1251" t="n">
-        <v>44013.9</v>
+        <v>47681.71</v>
       </c>
     </row>
     <row r="1252">
@@ -14207,7 +14207,7 @@
         <v>2341</v>
       </c>
       <c r="C1252" t="n">
-        <v>77400</v>
+        <v>83850</v>
       </c>
     </row>
     <row r="1253">
@@ -14218,7 +14218,7 @@
         <v>1374</v>
       </c>
       <c r="C1253" t="n">
-        <v>98172</v>
+        <v>106353</v>
       </c>
     </row>
     <row r="1254">
@@ -14229,7 +14229,7 @@
         <v>793</v>
       </c>
       <c r="C1254" t="n">
-        <v>22692</v>
+        <v>24583</v>
       </c>
     </row>
     <row r="1255">
@@ -14240,7 +14240,7 @@
         <v>794</v>
       </c>
       <c r="C1255" t="n">
-        <v>22692</v>
+        <v>24583</v>
       </c>
     </row>
     <row r="1256">
@@ -14251,7 +14251,7 @@
         <v>1834</v>
       </c>
       <c r="C1256" t="n">
-        <v>63816</v>
+        <v>69134</v>
       </c>
     </row>
     <row r="1257">
@@ -14262,7 +14262,7 @@
         <v>802</v>
       </c>
       <c r="C1257" t="n">
-        <v>40908</v>
+        <v>44317</v>
       </c>
     </row>
     <row r="1258">
@@ -14273,7 +14273,7 @@
         <v>1344</v>
       </c>
       <c r="C1258" t="n">
-        <v>81816</v>
+        <v>88634</v>
       </c>
     </row>
     <row r="1259">
@@ -14284,7 +14284,7 @@
         <v>1881</v>
       </c>
       <c r="C1259" t="n">
-        <v>37464</v>
+        <v>40586</v>
       </c>
     </row>
     <row r="1260">
@@ -14295,7 +14295,7 @@
         <v>2365</v>
       </c>
       <c r="C1260" t="n">
-        <v>43452</v>
+        <v>47073</v>
       </c>
     </row>
     <row r="1261">
@@ -14306,7 +14306,7 @@
         <v>2411</v>
       </c>
       <c r="C1261" t="n">
-        <v>77400</v>
+        <v>83850</v>
       </c>
     </row>
     <row r="1262">
@@ -14317,7 +14317,7 @@
         <v>2363</v>
       </c>
       <c r="C1262" t="n">
-        <v>81816</v>
+        <v>88634</v>
       </c>
     </row>
     <row r="1263">
@@ -14328,7 +14328,7 @@
         <v>2124</v>
       </c>
       <c r="C1263" t="n">
-        <v>190908</v>
+        <v>206817</v>
       </c>
     </row>
     <row r="1264">
@@ -14339,7 +14339,7 @@
         <v>1937</v>
       </c>
       <c r="C1264" t="n">
-        <v>139080</v>
+        <v>150670</v>
       </c>
     </row>
     <row r="1265">
@@ -14350,7 +14350,7 @@
         <v>2709</v>
       </c>
       <c r="C1265" t="n">
-        <v>98172</v>
+        <v>106353</v>
       </c>
     </row>
     <row r="1266">
@@ -14361,7 +14361,7 @@
         <v>2558</v>
       </c>
       <c r="C1266" t="n">
-        <v>16392</v>
+        <v>17758</v>
       </c>
     </row>
     <row r="1267">
@@ -14372,7 +14372,7 @@
         <v>663</v>
       </c>
       <c r="C1267" t="n">
-        <v>139080</v>
+        <v>150670</v>
       </c>
     </row>
     <row r="1268">
@@ -14383,7 +14383,7 @@
         <v>40</v>
       </c>
       <c r="C1268" t="n">
-        <v>120000</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="1269">
@@ -14394,7 +14394,7 @@
         <v>2833</v>
       </c>
       <c r="C1269" t="n">
-        <v>38181.9</v>
+        <v>41363.71</v>
       </c>
     </row>
     <row r="1270">
@@ -14405,7 +14405,7 @@
         <v>1756</v>
       </c>
       <c r="C1270" t="n">
-        <v>238092</v>
+        <v>257933</v>
       </c>
     </row>
     <row r="1271">
@@ -14416,7 +14416,7 @@
         <v>1116</v>
       </c>
       <c r="C1271" t="n">
-        <v>138348</v>
+        <v>149877</v>
       </c>
     </row>
     <row r="1272">
@@ -14427,7 +14427,7 @@
         <v>636</v>
       </c>
       <c r="C1272" t="n">
-        <v>136356</v>
+        <v>147719</v>
       </c>
     </row>
     <row r="1273">
@@ -14438,7 +14438,7 @@
         <v>1800</v>
       </c>
       <c r="C1273" t="n">
-        <v>15264</v>
+        <v>16536</v>
       </c>
     </row>
     <row r="1274">
@@ -14449,7 +14449,7 @@
         <v>2815</v>
       </c>
       <c r="C1274" t="n">
-        <v>32727.3</v>
+        <v>35454.57</v>
       </c>
     </row>
     <row r="1275">
@@ -14460,7 +14460,7 @@
         <v>1658</v>
       </c>
       <c r="C1275" t="n">
-        <v>72000</v>
+        <v>78000</v>
       </c>
     </row>
     <row r="1276">
@@ -14471,7 +14471,7 @@
         <v>2635</v>
       </c>
       <c r="C1276" t="n">
-        <v>70908</v>
+        <v>76817</v>
       </c>
     </row>
     <row r="1277">
@@ -14482,7 +14482,7 @@
         <v>2402</v>
       </c>
       <c r="C1277" t="n">
-        <v>355632</v>
+        <v>385268</v>
       </c>
     </row>
     <row r="1278">
@@ -14493,7 +14493,7 @@
         <v>452</v>
       </c>
       <c r="C1278" t="n">
-        <v>147264</v>
+        <v>159536</v>
       </c>
     </row>
     <row r="1279">
@@ -14504,7 +14504,7 @@
         <v>2085</v>
       </c>
       <c r="C1279" t="n">
-        <v>72024</v>
+        <v>78026</v>
       </c>
     </row>
     <row r="1280">
@@ -14515,7 +14515,7 @@
         <v>2568</v>
       </c>
       <c r="C1280" t="n">
-        <v>111504</v>
+        <v>120796</v>
       </c>
     </row>
     <row r="1281">
@@ -14526,7 +14526,7 @@
         <v>1906</v>
       </c>
       <c r="C1281" t="n">
-        <v>63288</v>
+        <v>68562</v>
       </c>
     </row>
     <row r="1282">
@@ -14537,7 +14537,7 @@
         <v>2821</v>
       </c>
       <c r="C1282" t="n">
-        <v>55032</v>
+        <v>59618</v>
       </c>
     </row>
     <row r="1283">
@@ -14548,7 +14548,7 @@
         <v>2698</v>
       </c>
       <c r="C1283" t="n">
-        <v>67452</v>
+        <v>73073</v>
       </c>
     </row>
     <row r="1284">
@@ -14559,7 +14559,7 @@
         <v>2118</v>
       </c>
       <c r="C1284" t="n">
-        <v>129360</v>
+        <v>140140</v>
       </c>
     </row>
     <row r="1285">
@@ -14570,7 +14570,7 @@
         <v>2383</v>
       </c>
       <c r="C1285" t="n">
-        <v>75528</v>
+        <v>81822</v>
       </c>
     </row>
     <row r="1286">
@@ -14581,7 +14581,7 @@
         <v>2813</v>
       </c>
       <c r="C1286" t="n">
-        <v>34332</v>
+        <v>37193</v>
       </c>
     </row>
     <row r="1287">
@@ -14592,7 +14592,7 @@
         <v>925</v>
       </c>
       <c r="C1287" t="n">
-        <v>42912</v>
+        <v>46488</v>
       </c>
     </row>
     <row r="1288">
@@ -14603,7 +14603,7 @@
         <v>2689</v>
       </c>
       <c r="C1288" t="n">
-        <v>34332</v>
+        <v>37193</v>
       </c>
     </row>
     <row r="1289">
@@ -14614,7 +14614,7 @@
         <v>2716</v>
       </c>
       <c r="C1289" t="n">
-        <v>47208</v>
+        <v>51142</v>
       </c>
     </row>
     <row r="1290">
@@ -14625,7 +14625,7 @@
         <v>2831</v>
       </c>
       <c r="C1290" t="n">
-        <v>32724</v>
+        <v>35451</v>
       </c>
     </row>
     <row r="1291">
@@ -14636,7 +14636,7 @@
         <v>2045</v>
       </c>
       <c r="C1291" t="n">
-        <v>183521.32</v>
+        <v>198814.75</v>
       </c>
     </row>
     <row r="1292">
@@ -14647,7 +14647,7 @@
         <v>580</v>
       </c>
       <c r="C1292" t="n">
-        <v>73632</v>
+        <v>79768</v>
       </c>
     </row>
     <row r="1293">
@@ -14658,7 +14658,7 @@
         <v>438</v>
       </c>
       <c r="C1293" t="n">
-        <v>84540</v>
+        <v>91585</v>
       </c>
     </row>
     <row r="1294">
@@ -14669,7 +14669,7 @@
         <v>1539</v>
       </c>
       <c r="C1294" t="n">
-        <v>92724</v>
+        <v>100451</v>
       </c>
     </row>
     <row r="1295">
@@ -14680,7 +14680,7 @@
         <v>2817</v>
       </c>
       <c r="C1295" t="n">
-        <v>32724</v>
+        <v>35451</v>
       </c>
     </row>
     <row r="1296">
@@ -14691,7 +14691,7 @@
         <v>2816</v>
       </c>
       <c r="C1296" t="n">
-        <v>70908</v>
+        <v>76817</v>
       </c>
     </row>
     <row r="1297">
@@ -14702,7 +14702,7 @@
         <v>2146</v>
       </c>
       <c r="C1297" t="n">
-        <v>109992</v>
+        <v>119158</v>
       </c>
     </row>
     <row r="1298">
@@ -14713,7 +14713,7 @@
         <v>2276</v>
       </c>
       <c r="C1298" t="n">
-        <v>122208</v>
+        <v>132392</v>
       </c>
     </row>
     <row r="1299">
@@ -14724,7 +14724,7 @@
         <v>1381</v>
       </c>
       <c r="C1299" t="n">
-        <v>160908</v>
+        <v>174317</v>
       </c>
     </row>
     <row r="1300">
@@ -14735,7 +14735,7 @@
         <v>2081</v>
       </c>
       <c r="C1300" t="n">
-        <v>81816</v>
+        <v>88634</v>
       </c>
     </row>
     <row r="1301">
@@ -14746,7 +14746,7 @@
         <v>14</v>
       </c>
       <c r="C1301" t="n">
-        <v>237264</v>
+        <v>257036</v>
       </c>
     </row>
     <row r="1302">
@@ -14757,7 +14757,7 @@
         <v>766</v>
       </c>
       <c r="C1302" t="n">
-        <v>37464</v>
+        <v>40586</v>
       </c>
     </row>
     <row r="1303">
@@ -14768,7 +14768,7 @@
         <v>2547</v>
       </c>
       <c r="C1303" t="n">
-        <v>22428</v>
+        <v>24297</v>
       </c>
     </row>
     <row r="1304">
@@ -14779,7 +14779,7 @@
         <v>2552</v>
       </c>
       <c r="C1304" t="n">
-        <v>16128</v>
+        <v>17472</v>
       </c>
     </row>
     <row r="1305">
@@ -14790,7 +14790,7 @@
         <v>131</v>
       </c>
       <c r="C1305" t="n">
-        <v>223080</v>
+        <v>241670</v>
       </c>
     </row>
     <row r="1306">
@@ -14801,7 +14801,7 @@
         <v>2250</v>
       </c>
       <c r="C1306" t="n">
-        <v>180492</v>
+        <v>195533</v>
       </c>
     </row>
     <row r="1307">
@@ -14812,7 +14812,7 @@
         <v>89</v>
       </c>
       <c r="C1307" t="n">
-        <v>184464</v>
+        <v>199836</v>
       </c>
     </row>
     <row r="1308">
@@ -14823,7 +14823,7 @@
         <v>2141</v>
       </c>
       <c r="C1308" t="n">
-        <v>17256</v>
+        <v>18694</v>
       </c>
     </row>
     <row r="1309">
@@ -14834,7 +14834,7 @@
         <v>2798</v>
       </c>
       <c r="C1309" t="n">
-        <v>32727.3</v>
+        <v>35454.57</v>
       </c>
     </row>
     <row r="1310">
@@ -14845,7 +14845,7 @@
         <v>2797</v>
       </c>
       <c r="C1310" t="n">
-        <v>32727.3</v>
+        <v>35454.57</v>
       </c>
     </row>
     <row r="1311">
@@ -14856,7 +14856,7 @@
         <v>2266</v>
       </c>
       <c r="C1311" t="n">
-        <v>43636.4</v>
+        <v>47272.76</v>
       </c>
     </row>
     <row r="1312">
@@ -14867,7 +14867,7 @@
         <v>1499</v>
       </c>
       <c r="C1312" t="n">
-        <v>76356</v>
+        <v>82719</v>
       </c>
     </row>
     <row r="1313">
@@ -14878,7 +14878,7 @@
         <v>2496</v>
       </c>
       <c r="C1313" t="n">
-        <v>87264</v>
+        <v>94536</v>
       </c>
     </row>
     <row r="1314">
@@ -14889,7 +14889,7 @@
         <v>949</v>
       </c>
       <c r="C1314" t="n">
-        <v>53532</v>
+        <v>57993</v>
       </c>
     </row>
     <row r="1315">
@@ -14900,7 +14900,7 @@
         <v>1853</v>
       </c>
       <c r="C1315" t="n">
-        <v>65448</v>
+        <v>70902</v>
       </c>
     </row>
     <row r="1316">
@@ -14911,7 +14911,7 @@
         <v>854</v>
       </c>
       <c r="C1316" t="n">
-        <v>60000</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="1317">
@@ -14922,7 +14922,7 @@
         <v>2674</v>
       </c>
       <c r="C1317" t="n">
-        <v>141816</v>
+        <v>153634</v>
       </c>
     </row>
     <row r="1318">
@@ -14933,7 +14933,7 @@
         <v>2803</v>
       </c>
       <c r="C1318" t="n">
-        <v>65448</v>
+        <v>70902</v>
       </c>
     </row>
     <row r="1319">
@@ -14944,7 +14944,7 @@
         <v>2599</v>
       </c>
       <c r="C1319" t="n">
-        <v>103632</v>
+        <v>112268</v>
       </c>
     </row>
     <row r="1320">
@@ -14955,7 +14955,7 @@
         <v>783</v>
       </c>
       <c r="C1320" t="n">
-        <v>28356</v>
+        <v>30719</v>
       </c>
     </row>
     <row r="1321">
@@ -14966,7 +14966,7 @@
         <v>27</v>
       </c>
       <c r="C1321" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1322">
@@ -14977,7 +14977,7 @@
         <v>531</v>
       </c>
       <c r="C1322" t="n">
-        <v>190908</v>
+        <v>206817</v>
       </c>
     </row>
     <row r="1323">
@@ -14988,7 +14988,7 @@
         <v>1308</v>
       </c>
       <c r="C1323" t="n">
-        <v>88104</v>
+        <v>95446</v>
       </c>
     </row>
     <row r="1324">
@@ -14999,7 +14999,7 @@
         <v>2792</v>
       </c>
       <c r="C1324" t="n">
-        <v>63540</v>
+        <v>68835</v>
       </c>
     </row>
     <row r="1325">
@@ -15021,7 +15021,7 @@
         <v>2823</v>
       </c>
       <c r="C1326" t="n">
-        <v>51000</v>
+        <v>55250</v>
       </c>
     </row>
     <row r="1327">
@@ -15032,7 +15032,7 @@
         <v>2584</v>
       </c>
       <c r="C1327" t="n">
-        <v>34332</v>
+        <v>37193</v>
       </c>
     </row>
     <row r="1328">
@@ -15043,7 +15043,7 @@
         <v>945</v>
       </c>
       <c r="C1328" t="n">
-        <v>154536</v>
+        <v>167414</v>
       </c>
     </row>
     <row r="1329">
@@ -15054,7 +15054,7 @@
         <v>2660</v>
       </c>
       <c r="C1329" t="n">
-        <v>169080</v>
+        <v>183170</v>
       </c>
     </row>
     <row r="1330">
@@ -15065,7 +15065,7 @@
         <v>1317</v>
       </c>
       <c r="C1330" t="n">
-        <v>163632</v>
+        <v>177268</v>
       </c>
     </row>
     <row r="1331">
@@ -15076,7 +15076,7 @@
         <v>2790</v>
       </c>
       <c r="C1331" t="n">
-        <v>34740</v>
+        <v>37635</v>
       </c>
     </row>
     <row r="1332">
@@ -15087,7 +15087,7 @@
         <v>2711</v>
       </c>
       <c r="C1332" t="n">
-        <v>47284.4</v>
+        <v>51224.76</v>
       </c>
     </row>
     <row r="1333">
@@ -15098,7 +15098,7 @@
         <v>2607</v>
       </c>
       <c r="C1333" t="n">
-        <v>27100.4</v>
+        <v>29358.76</v>
       </c>
     </row>
     <row r="1334">
@@ -15109,7 +15109,7 @@
         <v>2667</v>
       </c>
       <c r="C1334" t="n">
-        <v>24927.3</v>
+        <v>27004.57</v>
       </c>
     </row>
     <row r="1335">
@@ -15120,7 +15120,7 @@
         <v>2706</v>
       </c>
       <c r="C1335" t="n">
-        <v>12017.5</v>
+        <v>13018.95</v>
       </c>
     </row>
     <row r="1336">
@@ -15131,7 +15131,7 @@
         <v>2657</v>
       </c>
       <c r="C1336" t="n">
-        <v>43197.9</v>
+        <v>46797.71</v>
       </c>
     </row>
     <row r="1337">
@@ -15142,7 +15142,7 @@
         <v>1278</v>
       </c>
       <c r="C1337" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1338">
@@ -15153,7 +15153,7 @@
         <v>2745</v>
       </c>
       <c r="C1338" t="n">
-        <v>60000</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="1339">
@@ -15164,7 +15164,7 @@
         <v>2753</v>
       </c>
       <c r="C1339" t="n">
-        <v>40908</v>
+        <v>44317</v>
       </c>
     </row>
     <row r="1340">
@@ -15175,7 +15175,7 @@
         <v>2183</v>
       </c>
       <c r="C1340" t="n">
-        <v>199608</v>
+        <v>216242</v>
       </c>
     </row>
     <row r="1341">
@@ -15186,7 +15186,7 @@
         <v>1340</v>
       </c>
       <c r="C1341" t="n">
-        <v>79080</v>
+        <v>85670</v>
       </c>
     </row>
     <row r="1342">
@@ -15197,7 +15197,7 @@
         <v>2583</v>
       </c>
       <c r="C1342" t="n">
-        <v>22692</v>
+        <v>24583</v>
       </c>
     </row>
     <row r="1343">
@@ -15208,7 +15208,7 @@
         <v>2090</v>
       </c>
       <c r="C1343" t="n">
-        <v>22692</v>
+        <v>24583</v>
       </c>
     </row>
     <row r="1344">
@@ -15219,7 +15219,7 @@
         <v>1277</v>
       </c>
       <c r="C1344" t="n">
-        <v>120000</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="1345">
@@ -15230,7 +15230,7 @@
         <v>1501</v>
       </c>
       <c r="C1345" t="n">
-        <v>51816</v>
+        <v>56134</v>
       </c>
     </row>
     <row r="1346">
@@ -15241,7 +15241,7 @@
         <v>703</v>
       </c>
       <c r="C1346" t="n">
-        <v>136356</v>
+        <v>147719</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:02:54
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -11292,7 +11292,7 @@
         <v>947</v>
       </c>
       <c r="C987" t="n">
-        <v>256763</v>
+        <v>276514</v>
       </c>
     </row>
     <row r="988">
@@ -11303,7 +11303,7 @@
         <v>1956</v>
       </c>
       <c r="C988" t="n">
-        <v>149188</v>
+        <v>160664</v>
       </c>
     </row>
     <row r="989">
@@ -11314,7 +11314,7 @@
         <v>2824</v>
       </c>
       <c r="C989" t="n">
-        <v>65000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="990">
@@ -11325,7 +11325,7 @@
         <v>2787</v>
       </c>
       <c r="C990" t="n">
-        <v>76817</v>
+        <v>82726</v>
       </c>
     </row>
     <row r="991">
@@ -11336,7 +11336,7 @@
         <v>2830</v>
       </c>
       <c r="C991" t="n">
-        <v>53170</v>
+        <v>57260</v>
       </c>
     </row>
     <row r="992">
@@ -11347,7 +11347,7 @@
         <v>1254</v>
       </c>
       <c r="C992" t="n">
-        <v>114752.19</v>
+        <v>123579.28</v>
       </c>
     </row>
     <row r="993">
@@ -11358,7 +11358,7 @@
         <v>816</v>
       </c>
       <c r="C993" t="n">
-        <v>158275</v>
+        <v>170450</v>
       </c>
     </row>
     <row r="994">
@@ -11369,7 +11369,7 @@
         <v>2671</v>
       </c>
       <c r="C994" t="n">
-        <v>47268</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="995">
@@ -11380,7 +11380,7 @@
         <v>2705</v>
       </c>
       <c r="C995" t="n">
-        <v>105885</v>
+        <v>114030</v>
       </c>
     </row>
     <row r="996">
@@ -11391,7 +11391,7 @@
         <v>2333</v>
       </c>
       <c r="C996" t="n">
-        <v>91208</v>
+        <v>98224</v>
       </c>
     </row>
     <row r="997">
@@ -11402,7 +11402,7 @@
         <v>2440</v>
       </c>
       <c r="C997" t="n">
-        <v>53170</v>
+        <v>57260</v>
       </c>
     </row>
     <row r="998">
@@ -11413,7 +11413,7 @@
         <v>2448</v>
       </c>
       <c r="C998" t="n">
-        <v>11817</v>
+        <v>12726</v>
       </c>
     </row>
     <row r="999">
@@ -11424,7 +11424,7 @@
         <v>2310</v>
       </c>
       <c r="C999" t="n">
-        <v>40586</v>
+        <v>43708</v>
       </c>
     </row>
     <row r="1000">
@@ -11435,7 +11435,7 @@
         <v>2809</v>
       </c>
       <c r="C1000" t="n">
-        <v>40586</v>
+        <v>43708</v>
       </c>
     </row>
     <row r="1001">
@@ -11446,7 +11446,7 @@
         <v>2548</v>
       </c>
       <c r="C1001" t="n">
-        <v>34580</v>
+        <v>37240</v>
       </c>
     </row>
     <row r="1002">
@@ -11457,7 +11457,7 @@
         <v>451</v>
       </c>
       <c r="C1002" t="n">
-        <v>141817</v>
+        <v>152726</v>
       </c>
     </row>
     <row r="1003">
@@ -11468,7 +11468,7 @@
         <v>933</v>
       </c>
       <c r="C1003" t="n">
-        <v>48152</v>
+        <v>51856</v>
       </c>
     </row>
     <row r="1004">
@@ -11479,7 +11479,7 @@
         <v>2702</v>
       </c>
       <c r="C1004" t="n">
-        <v>48152</v>
+        <v>51856</v>
       </c>
     </row>
     <row r="1005">
@@ -11490,7 +11490,7 @@
         <v>2549</v>
       </c>
       <c r="C1005" t="n">
-        <v>16744</v>
+        <v>18032</v>
       </c>
     </row>
     <row r="1006">
@@ -11501,7 +11501,7 @@
         <v>535</v>
       </c>
       <c r="C1006" t="n">
-        <v>218634</v>
+        <v>235452</v>
       </c>
     </row>
     <row r="1007">
@@ -11512,7 +11512,7 @@
         <v>1117</v>
       </c>
       <c r="C1007" t="n">
-        <v>205569</v>
+        <v>221382</v>
       </c>
     </row>
     <row r="1008">
@@ -11534,7 +11534,7 @@
         <v>530</v>
       </c>
       <c r="C1009" t="n">
-        <v>144222</v>
+        <v>155316</v>
       </c>
     </row>
     <row r="1010">
@@ -11545,7 +11545,7 @@
         <v>358</v>
       </c>
       <c r="C1010" t="n">
-        <v>200902</v>
+        <v>216356</v>
       </c>
     </row>
     <row r="1011">
@@ -11556,7 +11556,7 @@
         <v>2498</v>
       </c>
       <c r="C1011" t="n">
-        <v>32812</v>
+        <v>35336</v>
       </c>
     </row>
     <row r="1012">
@@ -11567,7 +11567,7 @@
         <v>2381</v>
       </c>
       <c r="C1012" t="n">
-        <v>46878</v>
+        <v>50484</v>
       </c>
     </row>
     <row r="1013">
@@ -11578,7 +11578,7 @@
         <v>2695</v>
       </c>
       <c r="C1013" t="n">
-        <v>28197</v>
+        <v>30366</v>
       </c>
     </row>
     <row r="1014">
@@ -11589,7 +11589,7 @@
         <v>2744</v>
       </c>
       <c r="C1014" t="n">
-        <v>35454.57</v>
+        <v>38181.84</v>
       </c>
     </row>
     <row r="1015">
@@ -11600,7 +11600,7 @@
         <v>2750</v>
       </c>
       <c r="C1015" t="n">
-        <v>35451</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1016">
@@ -11611,7 +11611,7 @@
         <v>2131</v>
       </c>
       <c r="C1016" t="n">
-        <v>70902</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1017">
@@ -11622,7 +11622,7 @@
         <v>818</v>
       </c>
       <c r="C1017" t="n">
-        <v>236353</v>
+        <v>254534</v>
       </c>
     </row>
     <row r="1018">
@@ -11633,7 +11633,7 @@
         <v>2566</v>
       </c>
       <c r="C1018" t="n">
-        <v>47268</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1019">
@@ -11644,7 +11644,7 @@
         <v>132</v>
       </c>
       <c r="C1019" t="n">
-        <v>443170</v>
+        <v>477260</v>
       </c>
     </row>
     <row r="1020">
@@ -11655,7 +11655,7 @@
         <v>2431</v>
       </c>
       <c r="C1020" t="n">
-        <v>108719</v>
+        <v>117082</v>
       </c>
     </row>
     <row r="1021">
@@ -11666,7 +11666,7 @@
         <v>2249</v>
       </c>
       <c r="C1021" t="n">
-        <v>115414</v>
+        <v>124292</v>
       </c>
     </row>
     <row r="1022">
@@ -11677,7 +11677,7 @@
         <v>1585</v>
       </c>
       <c r="C1022" t="n">
-        <v>97526</v>
+        <v>105028</v>
       </c>
     </row>
     <row r="1023">
@@ -11688,7 +11688,7 @@
         <v>2325</v>
       </c>
       <c r="C1023" t="n">
-        <v>94276</v>
+        <v>101528</v>
       </c>
     </row>
     <row r="1024">
@@ -11699,7 +11699,7 @@
         <v>2190</v>
       </c>
       <c r="C1024" t="n">
-        <v>132951</v>
+        <v>143178</v>
       </c>
     </row>
     <row r="1025">
@@ -11710,7 +11710,7 @@
         <v>1466</v>
       </c>
       <c r="C1025" t="n">
-        <v>239317</v>
+        <v>257726</v>
       </c>
     </row>
     <row r="1026">
@@ -11721,7 +11721,7 @@
         <v>2659</v>
       </c>
       <c r="C1026" t="n">
-        <v>72683</v>
+        <v>78274</v>
       </c>
     </row>
     <row r="1027">
@@ -11732,7 +11732,7 @@
         <v>634</v>
       </c>
       <c r="C1027" t="n">
-        <v>325000</v>
+        <v>350000</v>
       </c>
     </row>
     <row r="1028">
@@ -11743,7 +11743,7 @@
         <v>2804</v>
       </c>
       <c r="C1028" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1029">
@@ -11754,7 +11754,7 @@
         <v>2375</v>
       </c>
       <c r="C1029" t="n">
-        <v>195000</v>
+        <v>210000</v>
       </c>
     </row>
     <row r="1030">
@@ -11765,7 +11765,7 @@
         <v>2601</v>
       </c>
       <c r="C1030" t="n">
-        <v>162500</v>
+        <v>175000</v>
       </c>
     </row>
     <row r="1031">
@@ -11776,7 +11776,7 @@
         <v>952</v>
       </c>
       <c r="C1031" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1032">
@@ -11787,7 +11787,7 @@
         <v>571</v>
       </c>
       <c r="C1032" t="n">
-        <v>376103</v>
+        <v>405034</v>
       </c>
     </row>
     <row r="1033">
@@ -11798,7 +11798,7 @@
         <v>2697</v>
       </c>
       <c r="C1033" t="n">
-        <v>114595</v>
+        <v>123410</v>
       </c>
     </row>
     <row r="1034">
@@ -11809,7 +11809,7 @@
         <v>2678</v>
       </c>
       <c r="C1034" t="n">
-        <v>198263</v>
+        <v>213514</v>
       </c>
     </row>
     <row r="1035">
@@ -11820,7 +11820,7 @@
         <v>2768</v>
       </c>
       <c r="C1035" t="n">
-        <v>207493</v>
+        <v>223454</v>
       </c>
     </row>
     <row r="1036">
@@ -11831,7 +11831,7 @@
         <v>2359</v>
       </c>
       <c r="C1036" t="n">
-        <v>62933</v>
+        <v>67774</v>
       </c>
     </row>
     <row r="1037">
@@ -11842,7 +11842,7 @@
         <v>353</v>
       </c>
       <c r="C1037" t="n">
-        <v>204438</v>
+        <v>220164</v>
       </c>
     </row>
     <row r="1038">
@@ -11853,7 +11853,7 @@
         <v>2026</v>
       </c>
       <c r="C1038" t="n">
-        <v>169390</v>
+        <v>182420</v>
       </c>
     </row>
     <row r="1039">
@@ -11875,7 +11875,7 @@
         <v>2345</v>
       </c>
       <c r="C1040" t="n">
-        <v>37193</v>
+        <v>40054</v>
       </c>
     </row>
     <row r="1041">
@@ -11886,7 +11886,7 @@
         <v>2789</v>
       </c>
       <c r="C1041" t="n">
-        <v>100451</v>
+        <v>108178</v>
       </c>
     </row>
     <row r="1042">
@@ -11897,7 +11897,7 @@
         <v>569</v>
       </c>
       <c r="C1042" t="n">
-        <v>1692314</v>
+        <v>1822492</v>
       </c>
     </row>
     <row r="1043">
@@ -11908,7 +11908,7 @@
         <v>2822</v>
       </c>
       <c r="C1043" t="n">
-        <v>79768</v>
+        <v>85904</v>
       </c>
     </row>
     <row r="1044">
@@ -11919,7 +11919,7 @@
         <v>2728</v>
       </c>
       <c r="C1044" t="n">
-        <v>5902</v>
+        <v>6356</v>
       </c>
     </row>
     <row r="1045">
@@ -11930,7 +11930,7 @@
         <v>2488</v>
       </c>
       <c r="C1045" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1046">
@@ -11941,7 +11941,7 @@
         <v>2791</v>
       </c>
       <c r="C1046" t="n">
-        <v>58316.9</v>
+        <v>62802.8</v>
       </c>
     </row>
     <row r="1047">
@@ -11952,7 +11952,7 @@
         <v>2577</v>
       </c>
       <c r="C1047" t="n">
-        <v>52691.47</v>
+        <v>56744.65</v>
       </c>
     </row>
     <row r="1048">
@@ -11963,7 +11963,7 @@
         <v>2069</v>
       </c>
       <c r="C1048" t="n">
-        <v>106353</v>
+        <v>114534</v>
       </c>
     </row>
     <row r="1049">
@@ -11974,7 +11974,7 @@
         <v>2082</v>
       </c>
       <c r="C1049" t="n">
-        <v>98423</v>
+        <v>105994</v>
       </c>
     </row>
     <row r="1050">
@@ -11985,7 +11985,7 @@
         <v>781</v>
       </c>
       <c r="C1050" t="n">
-        <v>76817</v>
+        <v>82726</v>
       </c>
     </row>
     <row r="1051">
@@ -11996,7 +11996,7 @@
         <v>744</v>
       </c>
       <c r="C1051" t="n">
-        <v>24583</v>
+        <v>26474</v>
       </c>
     </row>
     <row r="1052">
@@ -12007,7 +12007,7 @@
         <v>2223</v>
       </c>
       <c r="C1052" t="n">
-        <v>77961</v>
+        <v>83958</v>
       </c>
     </row>
     <row r="1053">
@@ -12018,7 +12018,7 @@
         <v>2452</v>
       </c>
       <c r="C1053" t="n">
-        <v>41353</v>
+        <v>44534</v>
       </c>
     </row>
     <row r="1054">
@@ -12029,7 +12029,7 @@
         <v>970</v>
       </c>
       <c r="C1054" t="n">
-        <v>40586</v>
+        <v>43708</v>
       </c>
     </row>
     <row r="1055">
@@ -12040,7 +12040,7 @@
         <v>2550</v>
       </c>
       <c r="C1055" t="n">
-        <v>36036</v>
+        <v>38808</v>
       </c>
     </row>
     <row r="1056">
@@ -12051,7 +12051,7 @@
         <v>768</v>
       </c>
       <c r="C1056" t="n">
-        <v>76817</v>
+        <v>82726</v>
       </c>
     </row>
     <row r="1057">
@@ -12062,7 +12062,7 @@
         <v>1075</v>
       </c>
       <c r="C1057" t="n">
-        <v>267670</v>
+        <v>288260</v>
       </c>
     </row>
     <row r="1058">
@@ -12073,7 +12073,7 @@
         <v>664</v>
       </c>
       <c r="C1058" t="n">
-        <v>153036</v>
+        <v>164808</v>
       </c>
     </row>
     <row r="1059">
@@ -12084,7 +12084,7 @@
         <v>2555</v>
       </c>
       <c r="C1059" t="n">
-        <v>24531</v>
+        <v>26418</v>
       </c>
     </row>
     <row r="1060">
@@ -12095,7 +12095,7 @@
         <v>2627</v>
       </c>
       <c r="C1060" t="n">
-        <v>14404</v>
+        <v>15512</v>
       </c>
     </row>
     <row r="1061">
@@ -12106,7 +12106,7 @@
         <v>2557</v>
       </c>
       <c r="C1061" t="n">
-        <v>15236</v>
+        <v>16408</v>
       </c>
     </row>
     <row r="1062">
@@ -12117,7 +12117,7 @@
         <v>2551</v>
       </c>
       <c r="C1062" t="n">
-        <v>12103</v>
+        <v>13034</v>
       </c>
     </row>
     <row r="1063">
@@ -12128,7 +12128,7 @@
         <v>2463</v>
       </c>
       <c r="C1063" t="n">
-        <v>189215</v>
+        <v>203770</v>
       </c>
     </row>
     <row r="1064">
@@ -12139,7 +12139,7 @@
         <v>2279</v>
       </c>
       <c r="C1064" t="n">
-        <v>142753</v>
+        <v>153734</v>
       </c>
     </row>
     <row r="1065">
@@ -12150,7 +12150,7 @@
         <v>631</v>
       </c>
       <c r="C1065" t="n">
-        <v>206817</v>
+        <v>222726</v>
       </c>
     </row>
     <row r="1066">
@@ -12161,7 +12161,7 @@
         <v>2251</v>
       </c>
       <c r="C1066" t="n">
-        <v>126646</v>
+        <v>136388</v>
       </c>
     </row>
     <row r="1067">
@@ -12172,7 +12172,7 @@
         <v>1653</v>
       </c>
       <c r="C1067" t="n">
-        <v>192036</v>
+        <v>206808</v>
       </c>
     </row>
     <row r="1068">
@@ -12183,7 +12183,7 @@
         <v>1293</v>
       </c>
       <c r="C1068" t="n">
-        <v>245219</v>
+        <v>264082</v>
       </c>
     </row>
     <row r="1069">
@@ -12194,7 +12194,7 @@
         <v>360</v>
       </c>
       <c r="C1069" t="n">
-        <v>295451</v>
+        <v>318178</v>
       </c>
     </row>
     <row r="1070">
@@ -12205,7 +12205,7 @@
         <v>1063</v>
       </c>
       <c r="C1070" t="n">
-        <v>214825</v>
+        <v>231350</v>
       </c>
     </row>
     <row r="1071">
@@ -12216,7 +12216,7 @@
         <v>2273</v>
       </c>
       <c r="C1071" t="n">
-        <v>125320</v>
+        <v>134960</v>
       </c>
     </row>
     <row r="1072">
@@ -12227,7 +12227,7 @@
         <v>2757</v>
       </c>
       <c r="C1072" t="n">
-        <v>41363.71</v>
+        <v>44545.52</v>
       </c>
     </row>
     <row r="1073">
@@ -12238,7 +12238,7 @@
         <v>2795</v>
       </c>
       <c r="C1073" t="n">
-        <v>35454.57</v>
+        <v>38181.84</v>
       </c>
     </row>
     <row r="1074">
@@ -12249,7 +12249,7 @@
         <v>2722</v>
       </c>
       <c r="C1074" t="n">
-        <v>35451</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1075">
@@ -12260,7 +12260,7 @@
         <v>2718</v>
       </c>
       <c r="C1075" t="n">
-        <v>47268</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1076">
@@ -12271,7 +12271,7 @@
         <v>595</v>
       </c>
       <c r="C1076" t="n">
-        <v>325000</v>
+        <v>350000</v>
       </c>
     </row>
     <row r="1077">
@@ -12282,7 +12282,7 @@
         <v>890</v>
       </c>
       <c r="C1077" t="n">
-        <v>413634</v>
+        <v>445452</v>
       </c>
     </row>
     <row r="1078">
@@ -12293,7 +12293,7 @@
         <v>2652</v>
       </c>
       <c r="C1078" t="n">
-        <v>76817</v>
+        <v>82726</v>
       </c>
     </row>
     <row r="1079">
@@ -12304,7 +12304,7 @@
         <v>2714</v>
       </c>
       <c r="C1079" t="n">
-        <v>212719</v>
+        <v>229082</v>
       </c>
     </row>
     <row r="1080">
@@ -12315,7 +12315,7 @@
         <v>1869</v>
       </c>
       <c r="C1080" t="n">
-        <v>135902</v>
+        <v>146356</v>
       </c>
     </row>
     <row r="1081">
@@ -12326,7 +12326,7 @@
         <v>400</v>
       </c>
       <c r="C1081" t="n">
-        <v>112268</v>
+        <v>120904</v>
       </c>
     </row>
     <row r="1082">
@@ -12337,7 +12337,7 @@
         <v>1907</v>
       </c>
       <c r="C1082" t="n">
-        <v>219219</v>
+        <v>236082</v>
       </c>
     </row>
     <row r="1083">
@@ -12348,7 +12348,7 @@
         <v>1996</v>
       </c>
       <c r="C1083" t="n">
-        <v>138567</v>
+        <v>149226</v>
       </c>
     </row>
     <row r="1084">
@@ -12359,7 +12359,7 @@
         <v>1890</v>
       </c>
       <c r="C1084" t="n">
-        <v>186811.64</v>
+        <v>201181.75</v>
       </c>
     </row>
     <row r="1085">
@@ -12370,7 +12370,7 @@
         <v>2114</v>
       </c>
       <c r="C1085" t="n">
-        <v>108550</v>
+        <v>116900</v>
       </c>
     </row>
     <row r="1086">
@@ -12381,7 +12381,7 @@
         <v>2330</v>
       </c>
       <c r="C1086" t="n">
-        <v>158821</v>
+        <v>171038</v>
       </c>
     </row>
     <row r="1087">
@@ -12425,7 +12425,7 @@
         <v>931</v>
       </c>
       <c r="C1090" t="n">
-        <v>55796</v>
+        <v>60088</v>
       </c>
     </row>
     <row r="1091">
@@ -12436,7 +12436,7 @@
         <v>951</v>
       </c>
       <c r="C1091" t="n">
-        <v>67951</v>
+        <v>73178</v>
       </c>
     </row>
     <row r="1092">
@@ -12447,7 +12447,7 @@
         <v>2449</v>
       </c>
       <c r="C1092" t="n">
-        <v>23634</v>
+        <v>25452</v>
       </c>
     </row>
     <row r="1093">
@@ -12458,7 +12458,7 @@
         <v>610</v>
       </c>
       <c r="C1093" t="n">
-        <v>481585</v>
+        <v>518630</v>
       </c>
     </row>
     <row r="1094">
@@ -12469,7 +12469,7 @@
         <v>2761</v>
       </c>
       <c r="C1094" t="n">
-        <v>48152</v>
+        <v>51856</v>
       </c>
     </row>
     <row r="1095">
@@ -12480,7 +12480,7 @@
         <v>483</v>
       </c>
       <c r="C1095" t="n">
-        <v>261768</v>
+        <v>281904</v>
       </c>
     </row>
     <row r="1096">
@@ -12491,7 +12491,7 @@
         <v>2015</v>
       </c>
       <c r="C1096" t="n">
-        <v>218634</v>
+        <v>235452</v>
       </c>
     </row>
     <row r="1097">
@@ -12502,7 +12502,7 @@
         <v>1478</v>
       </c>
       <c r="C1097" t="n">
-        <v>319774</v>
+        <v>344372</v>
       </c>
     </row>
     <row r="1098">
@@ -12513,7 +12513,7 @@
         <v>424</v>
       </c>
       <c r="C1098" t="n">
-        <v>142753</v>
+        <v>153734</v>
       </c>
     </row>
     <row r="1099">
@@ -12535,7 +12535,7 @@
         <v>477</v>
       </c>
       <c r="C1100" t="n">
-        <v>152841</v>
+        <v>164598</v>
       </c>
     </row>
     <row r="1101">
@@ -12546,7 +12546,7 @@
         <v>1810</v>
       </c>
       <c r="C1101" t="n">
-        <v>23673</v>
+        <v>25494</v>
       </c>
     </row>
     <row r="1102">
@@ -12557,7 +12557,7 @@
         <v>2826</v>
       </c>
       <c r="C1102" t="n">
-        <v>41363.71</v>
+        <v>44545.52</v>
       </c>
     </row>
     <row r="1103">
@@ -12568,7 +12568,7 @@
         <v>2561</v>
       </c>
       <c r="C1103" t="n">
-        <v>8684</v>
+        <v>9352</v>
       </c>
     </row>
     <row r="1104">
@@ -12579,7 +12579,7 @@
         <v>2653</v>
       </c>
       <c r="C1104" t="n">
-        <v>35454.57</v>
+        <v>38181.84</v>
       </c>
     </row>
     <row r="1105">
@@ -12590,7 +12590,7 @@
         <v>2829</v>
       </c>
       <c r="C1105" t="n">
-        <v>35454.57</v>
+        <v>38181.84</v>
       </c>
     </row>
     <row r="1106">
@@ -12601,7 +12601,7 @@
         <v>2643</v>
       </c>
       <c r="C1106" t="n">
-        <v>17446</v>
+        <v>18788</v>
       </c>
     </row>
     <row r="1107">
@@ -12612,7 +12612,7 @@
         <v>2794</v>
       </c>
       <c r="C1107" t="n">
-        <v>53170</v>
+        <v>57260</v>
       </c>
     </row>
     <row r="1108">
@@ -12623,7 +12623,7 @@
         <v>2655</v>
       </c>
       <c r="C1108" t="n">
-        <v>65000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="1109">
@@ -12634,7 +12634,7 @@
         <v>1456</v>
       </c>
       <c r="C1109" t="n">
-        <v>455169</v>
+        <v>490182</v>
       </c>
     </row>
     <row r="1110">
@@ -12645,7 +12645,7 @@
         <v>2606</v>
       </c>
       <c r="C1110" t="n">
-        <v>139802</v>
+        <v>150556</v>
       </c>
     </row>
     <row r="1111">
@@ -12656,7 +12656,7 @@
         <v>1142</v>
       </c>
       <c r="C1111" t="n">
-        <v>253526</v>
+        <v>273028</v>
       </c>
     </row>
     <row r="1112">
@@ -12667,7 +12667,7 @@
         <v>1450</v>
       </c>
       <c r="C1112" t="n">
-        <v>161057</v>
+        <v>173446</v>
       </c>
     </row>
     <row r="1113">
@@ -12678,7 +12678,7 @@
         <v>2133</v>
       </c>
       <c r="C1113" t="n">
-        <v>376103</v>
+        <v>405034</v>
       </c>
     </row>
     <row r="1114">
@@ -12689,7 +12689,7 @@
         <v>522</v>
       </c>
       <c r="C1114" t="n">
-        <v>115219</v>
+        <v>124082</v>
       </c>
     </row>
     <row r="1115">
@@ -12700,7 +12700,7 @@
         <v>2696</v>
       </c>
       <c r="C1115" t="n">
-        <v>155480</v>
+        <v>167440</v>
       </c>
     </row>
     <row r="1116">
@@ -12722,7 +12722,7 @@
         <v>2692</v>
       </c>
       <c r="C1117" t="n">
-        <v>44317</v>
+        <v>47726</v>
       </c>
     </row>
     <row r="1118">
@@ -12733,7 +12733,7 @@
         <v>2691</v>
       </c>
       <c r="C1118" t="n">
-        <v>79768</v>
+        <v>85904</v>
       </c>
     </row>
     <row r="1119">
@@ -12744,7 +12744,7 @@
         <v>1632</v>
       </c>
       <c r="C1119" t="n">
-        <v>147719</v>
+        <v>159082</v>
       </c>
     </row>
     <row r="1120">
@@ -12755,7 +12755,7 @@
         <v>2641</v>
       </c>
       <c r="C1120" t="n">
-        <v>47268</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1121">
@@ -12766,7 +12766,7 @@
         <v>2197</v>
       </c>
       <c r="C1121" t="n">
-        <v>118170</v>
+        <v>127260</v>
       </c>
     </row>
     <row r="1122">
@@ -12777,7 +12777,7 @@
         <v>609</v>
       </c>
       <c r="C1122" t="n">
-        <v>130000</v>
+        <v>140000</v>
       </c>
     </row>
     <row r="1123">
@@ -12788,7 +12788,7 @@
         <v>1380</v>
       </c>
       <c r="C1123" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1124">
@@ -12799,7 +12799,7 @@
         <v>104</v>
       </c>
       <c r="C1124" t="n">
-        <v>177268</v>
+        <v>190904</v>
       </c>
     </row>
     <row r="1125">
@@ -12810,7 +12810,7 @@
         <v>2621</v>
       </c>
       <c r="C1125" t="n">
-        <v>41353</v>
+        <v>44534</v>
       </c>
     </row>
     <row r="1126">
@@ -12821,7 +12821,7 @@
         <v>2786</v>
       </c>
       <c r="C1126" t="n">
-        <v>41353</v>
+        <v>44534</v>
       </c>
     </row>
     <row r="1127">
@@ -12832,7 +12832,7 @@
         <v>2784</v>
       </c>
       <c r="C1127" t="n">
-        <v>24583</v>
+        <v>26474</v>
       </c>
     </row>
     <row r="1128">
@@ -12843,7 +12843,7 @@
         <v>2586</v>
       </c>
       <c r="C1128" t="n">
-        <v>24583</v>
+        <v>26474</v>
       </c>
     </row>
     <row r="1129">
@@ -12854,7 +12854,7 @@
         <v>2145</v>
       </c>
       <c r="C1129" t="n">
-        <v>76492</v>
+        <v>82376</v>
       </c>
     </row>
     <row r="1130">
@@ -12865,7 +12865,7 @@
         <v>2574</v>
       </c>
       <c r="C1130" t="n">
-        <v>76492</v>
+        <v>82376</v>
       </c>
     </row>
     <row r="1131">
@@ -12876,7 +12876,7 @@
         <v>2492</v>
       </c>
       <c r="C1131" t="n">
-        <v>83850</v>
+        <v>90300</v>
       </c>
     </row>
     <row r="1132">
@@ -12887,7 +12887,7 @@
         <v>629</v>
       </c>
       <c r="C1132" t="n">
-        <v>261170</v>
+        <v>281260</v>
       </c>
     </row>
     <row r="1133">
@@ -12898,7 +12898,7 @@
         <v>966</v>
       </c>
       <c r="C1133" t="n">
-        <v>48152</v>
+        <v>51856</v>
       </c>
     </row>
     <row r="1134">
@@ -12909,7 +12909,7 @@
         <v>2721</v>
       </c>
       <c r="C1134" t="n">
-        <v>48152</v>
+        <v>51856</v>
       </c>
     </row>
     <row r="1135">
@@ -12920,7 +12920,7 @@
         <v>2554</v>
       </c>
       <c r="C1135" t="n">
-        <v>14508</v>
+        <v>15624</v>
       </c>
     </row>
     <row r="1136">
@@ -12931,7 +12931,7 @@
         <v>2556</v>
       </c>
       <c r="C1136" t="n">
-        <v>21333</v>
+        <v>22974</v>
       </c>
     </row>
     <row r="1137">
@@ -12942,7 +12942,7 @@
         <v>2546</v>
       </c>
       <c r="C1137" t="n">
-        <v>14092</v>
+        <v>15176</v>
       </c>
     </row>
     <row r="1138">
@@ -12953,7 +12953,7 @@
         <v>42</v>
       </c>
       <c r="C1138" t="n">
-        <v>1116817</v>
+        <v>1202726</v>
       </c>
     </row>
     <row r="1139">
@@ -12964,7 +12964,7 @@
         <v>953</v>
       </c>
       <c r="C1139" t="n">
-        <v>403390</v>
+        <v>434420</v>
       </c>
     </row>
     <row r="1140">
@@ -12975,7 +12975,7 @@
         <v>675</v>
       </c>
       <c r="C1140" t="n">
-        <v>118170</v>
+        <v>127260</v>
       </c>
     </row>
     <row r="1141">
@@ -12986,7 +12986,7 @@
         <v>619</v>
       </c>
       <c r="C1141" t="n">
-        <v>182728</v>
+        <v>196784</v>
       </c>
     </row>
     <row r="1142">
@@ -12997,7 +12997,7 @@
         <v>1299</v>
       </c>
       <c r="C1142" t="n">
-        <v>307476</v>
+        <v>331128</v>
       </c>
     </row>
     <row r="1143">
@@ -13008,7 +13008,7 @@
         <v>1064</v>
       </c>
       <c r="C1143" t="n">
-        <v>354172</v>
+        <v>381416</v>
       </c>
     </row>
     <row r="1144">
@@ -13019,7 +13019,7 @@
         <v>2308</v>
       </c>
       <c r="C1144" t="n">
-        <v>121134</v>
+        <v>130452</v>
       </c>
     </row>
     <row r="1145">
@@ -13030,7 +13030,7 @@
         <v>1137</v>
       </c>
       <c r="C1145" t="n">
-        <v>378170</v>
+        <v>407260</v>
       </c>
     </row>
     <row r="1146">
@@ -13041,7 +13041,7 @@
         <v>2747</v>
       </c>
       <c r="C1146" t="n">
-        <v>35454.57</v>
+        <v>38181.84</v>
       </c>
     </row>
     <row r="1147">
@@ -13052,7 +13052,7 @@
         <v>2819</v>
       </c>
       <c r="C1147" t="n">
-        <v>35454.57</v>
+        <v>38181.84</v>
       </c>
     </row>
     <row r="1148">
@@ -13063,7 +13063,7 @@
         <v>1259</v>
       </c>
       <c r="C1148" t="n">
-        <v>59090.95</v>
+        <v>63636.4</v>
       </c>
     </row>
     <row r="1149">
@@ -13074,7 +13074,7 @@
         <v>2544</v>
       </c>
       <c r="C1149" t="n">
-        <v>47268</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1150">
@@ -13085,7 +13085,7 @@
         <v>2261</v>
       </c>
       <c r="C1150" t="n">
-        <v>88634</v>
+        <v>95452</v>
       </c>
     </row>
     <row r="1151">
@@ -13096,7 +13096,7 @@
         <v>2729</v>
       </c>
       <c r="C1151" t="n">
-        <v>47268</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1152">
@@ -13107,7 +13107,7 @@
         <v>2649</v>
       </c>
       <c r="C1152" t="n">
-        <v>17446</v>
+        <v>18788</v>
       </c>
     </row>
     <row r="1153">
@@ -13118,7 +13118,7 @@
         <v>2494</v>
       </c>
       <c r="C1153" t="n">
-        <v>76817</v>
+        <v>82726</v>
       </c>
     </row>
     <row r="1154">
@@ -13129,7 +13129,7 @@
         <v>1384</v>
       </c>
       <c r="C1154" t="n">
-        <v>265902</v>
+        <v>286356</v>
       </c>
     </row>
     <row r="1155">
@@ -13151,7 +13151,7 @@
         <v>2802</v>
       </c>
       <c r="C1156" t="n">
-        <v>41847</v>
+        <v>45066</v>
       </c>
     </row>
     <row r="1157">
@@ -13162,7 +13162,7 @@
         <v>2726</v>
       </c>
       <c r="C1157" t="n">
-        <v>88634</v>
+        <v>95452</v>
       </c>
     </row>
     <row r="1158">
@@ -13173,7 +13173,7 @@
         <v>2820</v>
       </c>
       <c r="C1158" t="n">
-        <v>106353</v>
+        <v>114534</v>
       </c>
     </row>
     <row r="1159">
@@ -13184,7 +13184,7 @@
         <v>1007</v>
       </c>
       <c r="C1159" t="n">
-        <v>112268</v>
+        <v>120904</v>
       </c>
     </row>
     <row r="1160">
@@ -13195,7 +13195,7 @@
         <v>20</v>
       </c>
       <c r="C1160" t="n">
-        <v>227500</v>
+        <v>245000</v>
       </c>
     </row>
     <row r="1161">
@@ -13206,7 +13206,7 @@
         <v>1372</v>
       </c>
       <c r="C1161" t="n">
-        <v>171353</v>
+        <v>184534</v>
       </c>
     </row>
     <row r="1162">
@@ -13217,7 +13217,7 @@
         <v>2735</v>
       </c>
       <c r="C1162" t="n">
-        <v>70902</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1163">
@@ -13228,7 +13228,7 @@
         <v>2811</v>
       </c>
       <c r="C1163" t="n">
-        <v>24583</v>
+        <v>26474</v>
       </c>
     </row>
     <row r="1164">
@@ -13239,7 +13239,7 @@
         <v>1871</v>
       </c>
       <c r="C1164" t="n">
-        <v>104442</v>
+        <v>112476</v>
       </c>
     </row>
     <row r="1165">
@@ -13250,7 +13250,7 @@
         <v>2541</v>
       </c>
       <c r="C1165" t="n">
-        <v>125034</v>
+        <v>134652</v>
       </c>
     </row>
     <row r="1166">
@@ -13261,7 +13261,7 @@
         <v>2362</v>
       </c>
       <c r="C1166" t="n">
-        <v>44317</v>
+        <v>47726</v>
       </c>
     </row>
     <row r="1167">
@@ -13272,7 +13272,7 @@
         <v>1324</v>
       </c>
       <c r="C1167" t="n">
-        <v>165451</v>
+        <v>178178</v>
       </c>
     </row>
     <row r="1168">
@@ -13283,7 +13283,7 @@
         <v>2323</v>
       </c>
       <c r="C1168" t="n">
-        <v>40586</v>
+        <v>43708</v>
       </c>
     </row>
     <row r="1169">
@@ -13294,7 +13294,7 @@
         <v>2647</v>
       </c>
       <c r="C1169" t="n">
-        <v>83850</v>
+        <v>90300</v>
       </c>
     </row>
     <row r="1170">
@@ -13305,7 +13305,7 @@
         <v>559</v>
       </c>
       <c r="C1170" t="n">
-        <v>135577</v>
+        <v>146006</v>
       </c>
     </row>
     <row r="1171">
@@ -13316,7 +13316,7 @@
         <v>2762</v>
       </c>
       <c r="C1171" t="n">
-        <v>48152</v>
+        <v>51856</v>
       </c>
     </row>
     <row r="1172">
@@ -13327,7 +13327,7 @@
         <v>2501</v>
       </c>
       <c r="C1172" t="n">
-        <v>48152</v>
+        <v>51856</v>
       </c>
     </row>
     <row r="1173">
@@ -13338,7 +13338,7 @@
         <v>2562</v>
       </c>
       <c r="C1173" t="n">
-        <v>9347</v>
+        <v>10066</v>
       </c>
     </row>
     <row r="1174">
@@ -13349,7 +13349,7 @@
         <v>429</v>
       </c>
       <c r="C1174" t="n">
-        <v>230451</v>
+        <v>248178</v>
       </c>
     </row>
     <row r="1175">
@@ -13360,7 +13360,7 @@
         <v>58</v>
       </c>
       <c r="C1175" t="n">
-        <v>159887</v>
+        <v>172186</v>
       </c>
     </row>
     <row r="1176">
@@ -13371,7 +13371,7 @@
         <v>2245</v>
       </c>
       <c r="C1176" t="n">
-        <v>142753</v>
+        <v>153734</v>
       </c>
     </row>
     <row r="1177">
@@ -13382,7 +13382,7 @@
         <v>285</v>
       </c>
       <c r="C1177" t="n">
-        <v>319774</v>
+        <v>344372</v>
       </c>
     </row>
     <row r="1178">
@@ -13404,7 +13404,7 @@
         <v>363</v>
       </c>
       <c r="C1179" t="n">
-        <v>177268</v>
+        <v>190904</v>
       </c>
     </row>
     <row r="1180">
@@ -13415,7 +13415,7 @@
         <v>2651</v>
       </c>
       <c r="C1180" t="n">
-        <v>99931</v>
+        <v>107618</v>
       </c>
     </row>
     <row r="1181">
@@ -13426,7 +13426,7 @@
         <v>2142</v>
       </c>
       <c r="C1181" t="n">
-        <v>31538</v>
+        <v>33964</v>
       </c>
     </row>
     <row r="1182">
@@ -13437,7 +13437,7 @@
         <v>2258</v>
       </c>
       <c r="C1182" t="n">
-        <v>47272.76</v>
+        <v>50909.12</v>
       </c>
     </row>
     <row r="1183">
@@ -13448,7 +13448,7 @@
         <v>2772</v>
       </c>
       <c r="C1183" t="n">
-        <v>35454.57</v>
+        <v>38181.84</v>
       </c>
     </row>
     <row r="1184">
@@ -13459,7 +13459,7 @@
         <v>2346</v>
       </c>
       <c r="C1184" t="n">
-        <v>65000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="1185">
@@ -13470,7 +13470,7 @@
         <v>2442</v>
       </c>
       <c r="C1185" t="n">
-        <v>47268</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1186">
@@ -13481,7 +13481,7 @@
         <v>772</v>
       </c>
       <c r="C1186" t="n">
-        <v>195000</v>
+        <v>210000</v>
       </c>
     </row>
     <row r="1187">
@@ -13492,7 +13492,7 @@
         <v>2684</v>
       </c>
       <c r="C1187" t="n">
-        <v>56134</v>
+        <v>60452</v>
       </c>
     </row>
     <row r="1188">
@@ -13503,7 +13503,7 @@
         <v>2765</v>
       </c>
       <c r="C1188" t="n">
-        <v>53170</v>
+        <v>57260</v>
       </c>
     </row>
     <row r="1189">
@@ -13514,7 +13514,7 @@
         <v>2567</v>
       </c>
       <c r="C1189" t="n">
-        <v>97526</v>
+        <v>105028</v>
       </c>
     </row>
     <row r="1190">
@@ -13525,7 +13525,7 @@
         <v>2178</v>
       </c>
       <c r="C1190" t="n">
-        <v>165451</v>
+        <v>178178</v>
       </c>
     </row>
     <row r="1191">
@@ -13536,7 +13536,7 @@
         <v>2827</v>
       </c>
       <c r="C1191" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1192">
@@ -13547,7 +13547,7 @@
         <v>2510</v>
       </c>
       <c r="C1192" t="n">
-        <v>328094</v>
+        <v>353332</v>
       </c>
     </row>
     <row r="1193">
@@ -13558,7 +13558,7 @@
         <v>2392</v>
       </c>
       <c r="C1193" t="n">
-        <v>98423</v>
+        <v>105994</v>
       </c>
     </row>
     <row r="1194">
@@ -13569,7 +13569,7 @@
         <v>415</v>
       </c>
       <c r="C1194" t="n">
-        <v>336518</v>
+        <v>362404</v>
       </c>
     </row>
     <row r="1195">
@@ -13580,7 +13580,7 @@
         <v>2107</v>
       </c>
       <c r="C1195" t="n">
-        <v>173771</v>
+        <v>187138</v>
       </c>
     </row>
     <row r="1196">
@@ -13591,7 +13591,7 @@
         <v>2211</v>
       </c>
       <c r="C1196" t="n">
-        <v>144066</v>
+        <v>155148</v>
       </c>
     </row>
     <row r="1197">
@@ -13602,7 +13602,7 @@
         <v>2682</v>
       </c>
       <c r="C1197" t="n">
-        <v>88621</v>
+        <v>95438</v>
       </c>
     </row>
     <row r="1198">
@@ -13635,7 +13635,7 @@
         <v>2755</v>
       </c>
       <c r="C1200" t="n">
-        <v>35451</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1201">
@@ -13646,7 +13646,7 @@
         <v>941</v>
       </c>
       <c r="C1201" t="n">
-        <v>232154</v>
+        <v>250012</v>
       </c>
     </row>
     <row r="1202">
@@ -13657,7 +13657,7 @@
         <v>2734</v>
       </c>
       <c r="C1202" t="n">
-        <v>32539</v>
+        <v>35042</v>
       </c>
     </row>
     <row r="1203">
@@ -13668,7 +13668,7 @@
         <v>1289</v>
       </c>
       <c r="C1203" t="n">
-        <v>147719</v>
+        <v>159082</v>
       </c>
     </row>
     <row r="1204">
@@ -13679,7 +13679,7 @@
         <v>2801</v>
       </c>
       <c r="C1204" t="n">
-        <v>47268</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1205">
@@ -13690,7 +13690,7 @@
         <v>2810</v>
       </c>
       <c r="C1205" t="n">
-        <v>79768</v>
+        <v>85904</v>
       </c>
     </row>
     <row r="1206">
@@ -13701,7 +13701,7 @@
         <v>767</v>
       </c>
       <c r="C1206" t="n">
-        <v>106353</v>
+        <v>114534</v>
       </c>
     </row>
     <row r="1207">
@@ -13712,7 +13712,7 @@
         <v>2687</v>
       </c>
       <c r="C1207" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1208">
@@ -13723,7 +13723,7 @@
         <v>2686</v>
       </c>
       <c r="C1208" t="n">
-        <v>76817</v>
+        <v>82726</v>
       </c>
     </row>
     <row r="1209">
@@ -13734,7 +13734,7 @@
         <v>2730</v>
       </c>
       <c r="C1209" t="n">
-        <v>53170</v>
+        <v>57260</v>
       </c>
     </row>
     <row r="1210">
@@ -13745,7 +13745,7 @@
         <v>2580</v>
       </c>
       <c r="C1210" t="n">
-        <v>19825</v>
+        <v>21350</v>
       </c>
     </row>
     <row r="1211">
@@ -13756,7 +13756,7 @@
         <v>2472</v>
       </c>
       <c r="C1211" t="n">
-        <v>31283.95</v>
+        <v>33690.4</v>
       </c>
     </row>
     <row r="1212">
@@ -13767,7 +13767,7 @@
         <v>2631</v>
       </c>
       <c r="C1212" t="n">
-        <v>14496.19</v>
+        <v>15611.28</v>
       </c>
     </row>
     <row r="1213">
@@ -13778,7 +13778,7 @@
         <v>1642</v>
       </c>
       <c r="C1213" t="n">
-        <v>156585</v>
+        <v>168630</v>
       </c>
     </row>
     <row r="1214">
@@ -13789,7 +13789,7 @@
         <v>2613</v>
       </c>
       <c r="C1214" t="n">
-        <v>105885</v>
+        <v>114030</v>
       </c>
     </row>
     <row r="1215">
@@ -13800,7 +13800,7 @@
         <v>1020</v>
       </c>
       <c r="C1215" t="n">
-        <v>53170</v>
+        <v>57260</v>
       </c>
     </row>
     <row r="1216">
@@ -13811,7 +13811,7 @@
         <v>2785</v>
       </c>
       <c r="C1216" t="n">
-        <v>24583</v>
+        <v>26474</v>
       </c>
     </row>
     <row r="1217">
@@ -13822,7 +13822,7 @@
         <v>1327</v>
       </c>
       <c r="C1217" t="n">
-        <v>35451</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1218">
@@ -13833,7 +13833,7 @@
         <v>2629</v>
       </c>
       <c r="C1218" t="n">
-        <v>40586</v>
+        <v>43708</v>
       </c>
     </row>
     <row r="1219">
@@ -13844,7 +13844,7 @@
         <v>749</v>
       </c>
       <c r="C1219" t="n">
-        <v>48152</v>
+        <v>51856</v>
       </c>
     </row>
     <row r="1220">
@@ -13855,7 +13855,7 @@
         <v>1983</v>
       </c>
       <c r="C1220" t="n">
-        <v>319774</v>
+        <v>344372</v>
       </c>
     </row>
     <row r="1221">
@@ -13866,7 +13866,7 @@
         <v>1993</v>
       </c>
       <c r="C1221" t="n">
-        <v>205569</v>
+        <v>221382</v>
       </c>
     </row>
     <row r="1222">
@@ -13877,7 +13877,7 @@
         <v>2767</v>
       </c>
       <c r="C1222" t="n">
-        <v>113997</v>
+        <v>122766</v>
       </c>
     </row>
     <row r="1223">
@@ -13899,7 +13899,7 @@
         <v>1102</v>
       </c>
       <c r="C1224" t="n">
-        <v>142753</v>
+        <v>153734</v>
       </c>
     </row>
     <row r="1225">
@@ -13910,7 +13910,7 @@
         <v>626</v>
       </c>
       <c r="C1225" t="n">
-        <v>1007095.26</v>
+        <v>1084564.12</v>
       </c>
     </row>
     <row r="1226">
@@ -13921,7 +13921,7 @@
         <v>1465</v>
       </c>
       <c r="C1226" t="n">
-        <v>212602</v>
+        <v>228956</v>
       </c>
     </row>
     <row r="1227">
@@ -13932,7 +13932,7 @@
         <v>2758</v>
       </c>
       <c r="C1227" t="n">
-        <v>35454.57</v>
+        <v>38181.84</v>
       </c>
     </row>
     <row r="1228">
@@ -13943,7 +13943,7 @@
         <v>2742</v>
       </c>
       <c r="C1228" t="n">
-        <v>35454.57</v>
+        <v>38181.84</v>
       </c>
     </row>
     <row r="1229">
@@ -13965,7 +13965,7 @@
         <v>1873</v>
       </c>
       <c r="C1230" t="n">
-        <v>189085</v>
+        <v>203630</v>
       </c>
     </row>
     <row r="1231">
@@ -13976,7 +13976,7 @@
         <v>2163</v>
       </c>
       <c r="C1231" t="n">
-        <v>88634</v>
+        <v>95452</v>
       </c>
     </row>
     <row r="1232">
@@ -13987,7 +13987,7 @@
         <v>2394</v>
       </c>
       <c r="C1232" t="n">
-        <v>91026</v>
+        <v>98028</v>
       </c>
     </row>
     <row r="1233">
@@ -13998,7 +13998,7 @@
         <v>33</v>
       </c>
       <c r="C1233" t="n">
-        <v>229268</v>
+        <v>246904</v>
       </c>
     </row>
     <row r="1234">
@@ -14009,7 +14009,7 @@
         <v>2421</v>
       </c>
       <c r="C1234" t="n">
-        <v>38402</v>
+        <v>41356</v>
       </c>
     </row>
     <row r="1235">
@@ -14020,7 +14020,7 @@
         <v>2663</v>
       </c>
       <c r="C1235" t="n">
-        <v>162500</v>
+        <v>175000</v>
       </c>
     </row>
     <row r="1236">
@@ -14031,7 +14031,7 @@
         <v>2413</v>
       </c>
       <c r="C1236" t="n">
-        <v>71526</v>
+        <v>77028</v>
       </c>
     </row>
     <row r="1237">
@@ -14042,7 +14042,7 @@
         <v>351</v>
       </c>
       <c r="C1237" t="n">
-        <v>108719</v>
+        <v>117082</v>
       </c>
     </row>
     <row r="1238">
@@ -14053,7 +14053,7 @@
         <v>1298</v>
       </c>
       <c r="C1238" t="n">
-        <v>752219</v>
+        <v>810082</v>
       </c>
     </row>
     <row r="1239">
@@ -14064,7 +14064,7 @@
         <v>2491</v>
       </c>
       <c r="C1239" t="n">
-        <v>60788</v>
+        <v>65464</v>
       </c>
     </row>
     <row r="1240">
@@ -14075,7 +14075,7 @@
         <v>2571</v>
       </c>
       <c r="C1240" t="n">
-        <v>85839</v>
+        <v>92442</v>
       </c>
     </row>
     <row r="1241">
@@ -14086,7 +14086,7 @@
         <v>2507</v>
       </c>
       <c r="C1241" t="n">
-        <v>52156</v>
+        <v>56168</v>
       </c>
     </row>
     <row r="1242">
@@ -14097,7 +14097,7 @@
         <v>2799</v>
       </c>
       <c r="C1242" t="n">
-        <v>67132</v>
+        <v>72296</v>
       </c>
     </row>
     <row r="1243">
@@ -14119,7 +14119,7 @@
         <v>2582</v>
       </c>
       <c r="C1244" t="n">
-        <v>51142</v>
+        <v>55076</v>
       </c>
     </row>
     <row r="1245">
@@ -14130,7 +14130,7 @@
         <v>2637</v>
       </c>
       <c r="C1245" t="n">
-        <v>37193</v>
+        <v>40054</v>
       </c>
     </row>
     <row r="1246">
@@ -14141,7 +14141,7 @@
         <v>630</v>
       </c>
       <c r="C1246" t="n">
-        <v>88452</v>
+        <v>95256</v>
       </c>
     </row>
     <row r="1247">
@@ -14152,7 +14152,7 @@
         <v>525</v>
       </c>
       <c r="C1247" t="n">
-        <v>132951</v>
+        <v>143178</v>
       </c>
     </row>
     <row r="1248">
@@ -14163,7 +14163,7 @@
         <v>2727</v>
       </c>
       <c r="C1248" t="n">
-        <v>23920</v>
+        <v>25760</v>
       </c>
     </row>
     <row r="1249">
@@ -14174,7 +14174,7 @@
         <v>2707</v>
       </c>
       <c r="C1249" t="n">
-        <v>18928</v>
+        <v>20384</v>
       </c>
     </row>
     <row r="1250">
@@ -14185,7 +14185,7 @@
         <v>2834</v>
       </c>
       <c r="C1250" t="n">
-        <v>9778.379999999999</v>
+        <v>10530.56</v>
       </c>
     </row>
     <row r="1251">
@@ -14196,7 +14196,7 @@
         <v>2773</v>
       </c>
       <c r="C1251" t="n">
-        <v>47681.71</v>
+        <v>51349.52</v>
       </c>
     </row>
     <row r="1252">
@@ -14207,7 +14207,7 @@
         <v>2341</v>
       </c>
       <c r="C1252" t="n">
-        <v>83850</v>
+        <v>90300</v>
       </c>
     </row>
     <row r="1253">
@@ -14218,7 +14218,7 @@
         <v>1374</v>
       </c>
       <c r="C1253" t="n">
-        <v>106353</v>
+        <v>114534</v>
       </c>
     </row>
     <row r="1254">
@@ -14229,7 +14229,7 @@
         <v>793</v>
       </c>
       <c r="C1254" t="n">
-        <v>24583</v>
+        <v>26474</v>
       </c>
     </row>
     <row r="1255">
@@ -14240,7 +14240,7 @@
         <v>794</v>
       </c>
       <c r="C1255" t="n">
-        <v>24583</v>
+        <v>26474</v>
       </c>
     </row>
     <row r="1256">
@@ -14251,7 +14251,7 @@
         <v>1834</v>
       </c>
       <c r="C1256" t="n">
-        <v>69134</v>
+        <v>74452</v>
       </c>
     </row>
     <row r="1257">
@@ -14262,7 +14262,7 @@
         <v>802</v>
       </c>
       <c r="C1257" t="n">
-        <v>44317</v>
+        <v>47726</v>
       </c>
     </row>
     <row r="1258">
@@ -14273,7 +14273,7 @@
         <v>1344</v>
       </c>
       <c r="C1258" t="n">
-        <v>88634</v>
+        <v>95452</v>
       </c>
     </row>
     <row r="1259">
@@ -14284,7 +14284,7 @@
         <v>1881</v>
       </c>
       <c r="C1259" t="n">
-        <v>40586</v>
+        <v>43708</v>
       </c>
     </row>
     <row r="1260">
@@ -14295,7 +14295,7 @@
         <v>2365</v>
       </c>
       <c r="C1260" t="n">
-        <v>47073</v>
+        <v>50694</v>
       </c>
     </row>
     <row r="1261">
@@ -14306,7 +14306,7 @@
         <v>2411</v>
       </c>
       <c r="C1261" t="n">
-        <v>83850</v>
+        <v>90300</v>
       </c>
     </row>
     <row r="1262">
@@ -14317,7 +14317,7 @@
         <v>2363</v>
       </c>
       <c r="C1262" t="n">
-        <v>88634</v>
+        <v>95452</v>
       </c>
     </row>
     <row r="1263">
@@ -14328,7 +14328,7 @@
         <v>2124</v>
       </c>
       <c r="C1263" t="n">
-        <v>206817</v>
+        <v>222726</v>
       </c>
     </row>
     <row r="1264">
@@ -14339,7 +14339,7 @@
         <v>1937</v>
       </c>
       <c r="C1264" t="n">
-        <v>150670</v>
+        <v>162260</v>
       </c>
     </row>
     <row r="1265">
@@ -14350,7 +14350,7 @@
         <v>2709</v>
       </c>
       <c r="C1265" t="n">
-        <v>106353</v>
+        <v>114534</v>
       </c>
     </row>
     <row r="1266">
@@ -14361,7 +14361,7 @@
         <v>2558</v>
       </c>
       <c r="C1266" t="n">
-        <v>17758</v>
+        <v>19124</v>
       </c>
     </row>
     <row r="1267">
@@ -14372,7 +14372,7 @@
         <v>663</v>
       </c>
       <c r="C1267" t="n">
-        <v>150670</v>
+        <v>162260</v>
       </c>
     </row>
     <row r="1268">
@@ -14383,7 +14383,7 @@
         <v>40</v>
       </c>
       <c r="C1268" t="n">
-        <v>130000</v>
+        <v>140000</v>
       </c>
     </row>
     <row r="1269">
@@ -14394,7 +14394,7 @@
         <v>2833</v>
       </c>
       <c r="C1269" t="n">
-        <v>41363.71</v>
+        <v>44545.52</v>
       </c>
     </row>
     <row r="1270">
@@ -14405,7 +14405,7 @@
         <v>1756</v>
       </c>
       <c r="C1270" t="n">
-        <v>257933</v>
+        <v>277774</v>
       </c>
     </row>
     <row r="1271">
@@ -14416,7 +14416,7 @@
         <v>1116</v>
       </c>
       <c r="C1271" t="n">
-        <v>149877</v>
+        <v>161406</v>
       </c>
     </row>
     <row r="1272">
@@ -14427,7 +14427,7 @@
         <v>636</v>
       </c>
       <c r="C1272" t="n">
-        <v>147719</v>
+        <v>159082</v>
       </c>
     </row>
     <row r="1273">
@@ -14438,7 +14438,7 @@
         <v>1800</v>
       </c>
       <c r="C1273" t="n">
-        <v>16536</v>
+        <v>17808</v>
       </c>
     </row>
     <row r="1274">
@@ -14449,7 +14449,7 @@
         <v>2815</v>
       </c>
       <c r="C1274" t="n">
-        <v>35454.57</v>
+        <v>38181.84</v>
       </c>
     </row>
     <row r="1275">
@@ -14460,7 +14460,7 @@
         <v>1658</v>
       </c>
       <c r="C1275" t="n">
-        <v>78000</v>
+        <v>84000</v>
       </c>
     </row>
     <row r="1276">
@@ -14471,7 +14471,7 @@
         <v>2635</v>
       </c>
       <c r="C1276" t="n">
-        <v>76817</v>
+        <v>82726</v>
       </c>
     </row>
     <row r="1277">
@@ -14482,7 +14482,7 @@
         <v>2402</v>
       </c>
       <c r="C1277" t="n">
-        <v>385268</v>
+        <v>414904</v>
       </c>
     </row>
     <row r="1278">
@@ -14493,7 +14493,7 @@
         <v>452</v>
       </c>
       <c r="C1278" t="n">
-        <v>159536</v>
+        <v>171808</v>
       </c>
     </row>
     <row r="1279">
@@ -14504,7 +14504,7 @@
         <v>2085</v>
       </c>
       <c r="C1279" t="n">
-        <v>78026</v>
+        <v>84028</v>
       </c>
     </row>
     <row r="1280">
@@ -14515,7 +14515,7 @@
         <v>2568</v>
       </c>
       <c r="C1280" t="n">
-        <v>120796</v>
+        <v>130088</v>
       </c>
     </row>
     <row r="1281">
@@ -14526,7 +14526,7 @@
         <v>1906</v>
       </c>
       <c r="C1281" t="n">
-        <v>68562</v>
+        <v>73836</v>
       </c>
     </row>
     <row r="1282">
@@ -14537,7 +14537,7 @@
         <v>2821</v>
       </c>
       <c r="C1282" t="n">
-        <v>59618</v>
+        <v>64204</v>
       </c>
     </row>
     <row r="1283">
@@ -14548,7 +14548,7 @@
         <v>2698</v>
       </c>
       <c r="C1283" t="n">
-        <v>73073</v>
+        <v>78694</v>
       </c>
     </row>
     <row r="1284">
@@ -14559,7 +14559,7 @@
         <v>2118</v>
       </c>
       <c r="C1284" t="n">
-        <v>140140</v>
+        <v>150920</v>
       </c>
     </row>
     <row r="1285">
@@ -14570,7 +14570,7 @@
         <v>2383</v>
       </c>
       <c r="C1285" t="n">
-        <v>81822</v>
+        <v>88116</v>
       </c>
     </row>
     <row r="1286">
@@ -14581,7 +14581,7 @@
         <v>2813</v>
       </c>
       <c r="C1286" t="n">
-        <v>37193</v>
+        <v>40054</v>
       </c>
     </row>
     <row r="1287">
@@ -14592,7 +14592,7 @@
         <v>925</v>
       </c>
       <c r="C1287" t="n">
-        <v>46488</v>
+        <v>50064</v>
       </c>
     </row>
     <row r="1288">
@@ -14603,7 +14603,7 @@
         <v>2689</v>
       </c>
       <c r="C1288" t="n">
-        <v>37193</v>
+        <v>40054</v>
       </c>
     </row>
     <row r="1289">
@@ -14614,7 +14614,7 @@
         <v>2716</v>
       </c>
       <c r="C1289" t="n">
-        <v>51142</v>
+        <v>55076</v>
       </c>
     </row>
     <row r="1290">
@@ -14625,7 +14625,7 @@
         <v>2831</v>
       </c>
       <c r="C1290" t="n">
-        <v>35451</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1291">
@@ -14636,7 +14636,7 @@
         <v>2045</v>
       </c>
       <c r="C1291" t="n">
-        <v>198814.75</v>
+        <v>214108.18</v>
       </c>
     </row>
     <row r="1292">
@@ -14647,7 +14647,7 @@
         <v>580</v>
       </c>
       <c r="C1292" t="n">
-        <v>79768</v>
+        <v>85904</v>
       </c>
     </row>
     <row r="1293">
@@ -14658,7 +14658,7 @@
         <v>438</v>
       </c>
       <c r="C1293" t="n">
-        <v>91585</v>
+        <v>98630</v>
       </c>
     </row>
     <row r="1294">
@@ -14669,7 +14669,7 @@
         <v>1539</v>
       </c>
       <c r="C1294" t="n">
-        <v>100451</v>
+        <v>108178</v>
       </c>
     </row>
     <row r="1295">
@@ -14680,7 +14680,7 @@
         <v>2817</v>
       </c>
       <c r="C1295" t="n">
-        <v>35451</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1296">
@@ -14691,7 +14691,7 @@
         <v>2816</v>
       </c>
       <c r="C1296" t="n">
-        <v>76817</v>
+        <v>82726</v>
       </c>
     </row>
     <row r="1297">
@@ -14702,7 +14702,7 @@
         <v>2146</v>
       </c>
       <c r="C1297" t="n">
-        <v>119158</v>
+        <v>128324</v>
       </c>
     </row>
     <row r="1298">
@@ -14713,7 +14713,7 @@
         <v>2276</v>
       </c>
       <c r="C1298" t="n">
-        <v>132392</v>
+        <v>142576</v>
       </c>
     </row>
     <row r="1299">
@@ -14724,7 +14724,7 @@
         <v>1381</v>
       </c>
       <c r="C1299" t="n">
-        <v>174317</v>
+        <v>187726</v>
       </c>
     </row>
     <row r="1300">
@@ -14735,7 +14735,7 @@
         <v>2081</v>
       </c>
       <c r="C1300" t="n">
-        <v>88634</v>
+        <v>95452</v>
       </c>
     </row>
     <row r="1301">
@@ -14746,7 +14746,7 @@
         <v>14</v>
       </c>
       <c r="C1301" t="n">
-        <v>257036</v>
+        <v>276808</v>
       </c>
     </row>
     <row r="1302">
@@ -14757,7 +14757,7 @@
         <v>766</v>
       </c>
       <c r="C1302" t="n">
-        <v>40586</v>
+        <v>43708</v>
       </c>
     </row>
     <row r="1303">
@@ -14768,7 +14768,7 @@
         <v>2547</v>
       </c>
       <c r="C1303" t="n">
-        <v>24297</v>
+        <v>26166</v>
       </c>
     </row>
     <row r="1304">
@@ -14779,7 +14779,7 @@
         <v>2552</v>
       </c>
       <c r="C1304" t="n">
-        <v>17472</v>
+        <v>18816</v>
       </c>
     </row>
     <row r="1305">
@@ -14790,7 +14790,7 @@
         <v>131</v>
       </c>
       <c r="C1305" t="n">
-        <v>241670</v>
+        <v>260260</v>
       </c>
     </row>
     <row r="1306">
@@ -14801,7 +14801,7 @@
         <v>2250</v>
       </c>
       <c r="C1306" t="n">
-        <v>195533</v>
+        <v>210574</v>
       </c>
     </row>
     <row r="1307">
@@ -14812,7 +14812,7 @@
         <v>89</v>
       </c>
       <c r="C1307" t="n">
-        <v>199836</v>
+        <v>215208</v>
       </c>
     </row>
     <row r="1308">
@@ -14823,7 +14823,7 @@
         <v>2141</v>
       </c>
       <c r="C1308" t="n">
-        <v>18694</v>
+        <v>20132</v>
       </c>
     </row>
     <row r="1309">
@@ -14834,7 +14834,7 @@
         <v>2798</v>
       </c>
       <c r="C1309" t="n">
-        <v>35454.57</v>
+        <v>38181.84</v>
       </c>
     </row>
     <row r="1310">
@@ -14845,7 +14845,7 @@
         <v>2797</v>
       </c>
       <c r="C1310" t="n">
-        <v>35454.57</v>
+        <v>38181.84</v>
       </c>
     </row>
     <row r="1311">
@@ -14856,7 +14856,7 @@
         <v>2266</v>
       </c>
       <c r="C1311" t="n">
-        <v>47272.76</v>
+        <v>50909.12</v>
       </c>
     </row>
     <row r="1312">
@@ -14867,7 +14867,7 @@
         <v>1499</v>
       </c>
       <c r="C1312" t="n">
-        <v>82719</v>
+        <v>89082</v>
       </c>
     </row>
     <row r="1313">
@@ -14878,7 +14878,7 @@
         <v>2496</v>
       </c>
       <c r="C1313" t="n">
-        <v>94536</v>
+        <v>101808</v>
       </c>
     </row>
     <row r="1314">
@@ -14889,7 +14889,7 @@
         <v>949</v>
       </c>
       <c r="C1314" t="n">
-        <v>57993</v>
+        <v>62454</v>
       </c>
     </row>
     <row r="1315">
@@ -14900,7 +14900,7 @@
         <v>1853</v>
       </c>
       <c r="C1315" t="n">
-        <v>70902</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1316">
@@ -14911,7 +14911,7 @@
         <v>854</v>
       </c>
       <c r="C1316" t="n">
-        <v>65000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="1317">
@@ -14922,7 +14922,7 @@
         <v>2674</v>
       </c>
       <c r="C1317" t="n">
-        <v>153634</v>
+        <v>165452</v>
       </c>
     </row>
     <row r="1318">
@@ -14933,7 +14933,7 @@
         <v>2803</v>
       </c>
       <c r="C1318" t="n">
-        <v>70902</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1319">
@@ -14944,7 +14944,7 @@
         <v>2599</v>
       </c>
       <c r="C1319" t="n">
-        <v>112268</v>
+        <v>120904</v>
       </c>
     </row>
     <row r="1320">
@@ -14955,7 +14955,7 @@
         <v>783</v>
       </c>
       <c r="C1320" t="n">
-        <v>30719</v>
+        <v>33082</v>
       </c>
     </row>
     <row r="1321">
@@ -14966,7 +14966,7 @@
         <v>27</v>
       </c>
       <c r="C1321" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1322">
@@ -14977,7 +14977,7 @@
         <v>531</v>
       </c>
       <c r="C1322" t="n">
-        <v>206817</v>
+        <v>222726</v>
       </c>
     </row>
     <row r="1323">
@@ -14988,7 +14988,7 @@
         <v>1308</v>
       </c>
       <c r="C1323" t="n">
-        <v>95446</v>
+        <v>102788</v>
       </c>
     </row>
     <row r="1324">
@@ -14999,7 +14999,7 @@
         <v>2792</v>
       </c>
       <c r="C1324" t="n">
-        <v>68835</v>
+        <v>74130</v>
       </c>
     </row>
     <row r="1325">
@@ -15021,7 +15021,7 @@
         <v>2823</v>
       </c>
       <c r="C1326" t="n">
-        <v>55250</v>
+        <v>59500</v>
       </c>
     </row>
     <row r="1327">
@@ -15032,7 +15032,7 @@
         <v>2584</v>
       </c>
       <c r="C1327" t="n">
-        <v>37193</v>
+        <v>40054</v>
       </c>
     </row>
     <row r="1328">
@@ -15043,7 +15043,7 @@
         <v>945</v>
       </c>
       <c r="C1328" t="n">
-        <v>167414</v>
+        <v>180292</v>
       </c>
     </row>
     <row r="1329">
@@ -15054,7 +15054,7 @@
         <v>2660</v>
       </c>
       <c r="C1329" t="n">
-        <v>183170</v>
+        <v>197260</v>
       </c>
     </row>
     <row r="1330">
@@ -15065,7 +15065,7 @@
         <v>1317</v>
       </c>
       <c r="C1330" t="n">
-        <v>177268</v>
+        <v>190904</v>
       </c>
     </row>
     <row r="1331">
@@ -15076,7 +15076,7 @@
         <v>2790</v>
       </c>
       <c r="C1331" t="n">
-        <v>37635</v>
+        <v>40530</v>
       </c>
     </row>
     <row r="1332">
@@ -15087,7 +15087,7 @@
         <v>2711</v>
       </c>
       <c r="C1332" t="n">
-        <v>51224.76</v>
+        <v>55165.12</v>
       </c>
     </row>
     <row r="1333">
@@ -15098,7 +15098,7 @@
         <v>2607</v>
       </c>
       <c r="C1333" t="n">
-        <v>29358.76</v>
+        <v>31617.12</v>
       </c>
     </row>
     <row r="1334">
@@ -15109,7 +15109,7 @@
         <v>2667</v>
       </c>
       <c r="C1334" t="n">
-        <v>27004.57</v>
+        <v>29081.84</v>
       </c>
     </row>
     <row r="1335">
@@ -15120,7 +15120,7 @@
         <v>2706</v>
       </c>
       <c r="C1335" t="n">
-        <v>13018.95</v>
+        <v>14020.4</v>
       </c>
     </row>
     <row r="1336">
@@ -15131,7 +15131,7 @@
         <v>2657</v>
       </c>
       <c r="C1336" t="n">
-        <v>46797.71</v>
+        <v>50397.52</v>
       </c>
     </row>
     <row r="1337">
@@ -15142,7 +15142,7 @@
         <v>1278</v>
       </c>
       <c r="C1337" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1338">
@@ -15153,7 +15153,7 @@
         <v>2745</v>
       </c>
       <c r="C1338" t="n">
-        <v>65000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="1339">
@@ -15164,7 +15164,7 @@
         <v>2753</v>
       </c>
       <c r="C1339" t="n">
-        <v>44317</v>
+        <v>47726</v>
       </c>
     </row>
     <row r="1340">
@@ -15175,7 +15175,7 @@
         <v>2183</v>
       </c>
       <c r="C1340" t="n">
-        <v>216242</v>
+        <v>232876</v>
       </c>
     </row>
     <row r="1341">
@@ -15186,7 +15186,7 @@
         <v>1340</v>
       </c>
       <c r="C1341" t="n">
-        <v>85670</v>
+        <v>92260</v>
       </c>
     </row>
     <row r="1342">
@@ -15197,7 +15197,7 @@
         <v>2583</v>
       </c>
       <c r="C1342" t="n">
-        <v>24583</v>
+        <v>26474</v>
       </c>
     </row>
     <row r="1343">
@@ -15208,7 +15208,7 @@
         <v>2090</v>
       </c>
       <c r="C1343" t="n">
-        <v>24583</v>
+        <v>26474</v>
       </c>
     </row>
     <row r="1344">
@@ -15219,7 +15219,7 @@
         <v>1277</v>
       </c>
       <c r="C1344" t="n">
-        <v>130000</v>
+        <v>140000</v>
       </c>
     </row>
     <row r="1345">
@@ -15230,7 +15230,7 @@
         <v>1501</v>
       </c>
       <c r="C1345" t="n">
-        <v>56134</v>
+        <v>60452</v>
       </c>
     </row>
     <row r="1346">
@@ -15241,7 +15241,7 @@
         <v>703</v>
       </c>
       <c r="C1346" t="n">
-        <v>147719</v>
+        <v>159082</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:02:56
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -11292,7 +11292,7 @@
         <v>947</v>
       </c>
       <c r="C987" t="n">
-        <v>276514</v>
+        <v>296265</v>
       </c>
     </row>
     <row r="988">
@@ -11303,7 +11303,7 @@
         <v>1956</v>
       </c>
       <c r="C988" t="n">
-        <v>160664</v>
+        <v>172140</v>
       </c>
     </row>
     <row r="989">
@@ -11314,7 +11314,7 @@
         <v>2824</v>
       </c>
       <c r="C989" t="n">
-        <v>70000</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="990">
@@ -11325,7 +11325,7 @@
         <v>2787</v>
       </c>
       <c r="C990" t="n">
-        <v>82726</v>
+        <v>88635</v>
       </c>
     </row>
     <row r="991">
@@ -11336,7 +11336,7 @@
         <v>2830</v>
       </c>
       <c r="C991" t="n">
-        <v>57260</v>
+        <v>61350</v>
       </c>
     </row>
     <row r="992">
@@ -11347,7 +11347,7 @@
         <v>1254</v>
       </c>
       <c r="C992" t="n">
-        <v>123579.28</v>
+        <v>132406.37</v>
       </c>
     </row>
     <row r="993">
@@ -11358,7 +11358,7 @@
         <v>816</v>
       </c>
       <c r="C993" t="n">
-        <v>170450</v>
+        <v>182625</v>
       </c>
     </row>
     <row r="994">
@@ -11369,7 +11369,7 @@
         <v>2671</v>
       </c>
       <c r="C994" t="n">
-        <v>50904</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="995">
@@ -11380,7 +11380,7 @@
         <v>2705</v>
       </c>
       <c r="C995" t="n">
-        <v>114030</v>
+        <v>122175</v>
       </c>
     </row>
     <row r="996">
@@ -11391,7 +11391,7 @@
         <v>2333</v>
       </c>
       <c r="C996" t="n">
-        <v>98224</v>
+        <v>105240</v>
       </c>
     </row>
     <row r="997">
@@ -11402,7 +11402,7 @@
         <v>2440</v>
       </c>
       <c r="C997" t="n">
-        <v>57260</v>
+        <v>61350</v>
       </c>
     </row>
     <row r="998">
@@ -11413,7 +11413,7 @@
         <v>2448</v>
       </c>
       <c r="C998" t="n">
-        <v>12726</v>
+        <v>13635</v>
       </c>
     </row>
     <row r="999">
@@ -11424,7 +11424,7 @@
         <v>2310</v>
       </c>
       <c r="C999" t="n">
-        <v>43708</v>
+        <v>46830</v>
       </c>
     </row>
     <row r="1000">
@@ -11435,7 +11435,7 @@
         <v>2809</v>
       </c>
       <c r="C1000" t="n">
-        <v>43708</v>
+        <v>46830</v>
       </c>
     </row>
     <row r="1001">
@@ -11446,7 +11446,7 @@
         <v>2548</v>
       </c>
       <c r="C1001" t="n">
-        <v>37240</v>
+        <v>39900</v>
       </c>
     </row>
     <row r="1002">
@@ -11457,7 +11457,7 @@
         <v>451</v>
       </c>
       <c r="C1002" t="n">
-        <v>152726</v>
+        <v>163635</v>
       </c>
     </row>
     <row r="1003">
@@ -11468,7 +11468,7 @@
         <v>933</v>
       </c>
       <c r="C1003" t="n">
-        <v>51856</v>
+        <v>55560</v>
       </c>
     </row>
     <row r="1004">
@@ -11479,7 +11479,7 @@
         <v>2702</v>
       </c>
       <c r="C1004" t="n">
-        <v>51856</v>
+        <v>55560</v>
       </c>
     </row>
     <row r="1005">
@@ -11490,7 +11490,7 @@
         <v>2549</v>
       </c>
       <c r="C1005" t="n">
-        <v>18032</v>
+        <v>19320</v>
       </c>
     </row>
     <row r="1006">
@@ -11501,7 +11501,7 @@
         <v>535</v>
       </c>
       <c r="C1006" t="n">
-        <v>235452</v>
+        <v>252270</v>
       </c>
     </row>
     <row r="1007">
@@ -11512,7 +11512,7 @@
         <v>1117</v>
       </c>
       <c r="C1007" t="n">
-        <v>221382</v>
+        <v>237195</v>
       </c>
     </row>
     <row r="1008">
@@ -11534,7 +11534,7 @@
         <v>530</v>
       </c>
       <c r="C1009" t="n">
-        <v>155316</v>
+        <v>166410</v>
       </c>
     </row>
     <row r="1010">
@@ -11545,7 +11545,7 @@
         <v>358</v>
       </c>
       <c r="C1010" t="n">
-        <v>216356</v>
+        <v>231810</v>
       </c>
     </row>
     <row r="1011">
@@ -11556,7 +11556,7 @@
         <v>2498</v>
       </c>
       <c r="C1011" t="n">
-        <v>35336</v>
+        <v>37860</v>
       </c>
     </row>
     <row r="1012">
@@ -11567,7 +11567,7 @@
         <v>2381</v>
       </c>
       <c r="C1012" t="n">
-        <v>50484</v>
+        <v>54090</v>
       </c>
     </row>
     <row r="1013">
@@ -11578,7 +11578,7 @@
         <v>2695</v>
       </c>
       <c r="C1013" t="n">
-        <v>30366</v>
+        <v>32535</v>
       </c>
     </row>
     <row r="1014">
@@ -11589,7 +11589,7 @@
         <v>2744</v>
       </c>
       <c r="C1014" t="n">
-        <v>38181.84</v>
+        <v>40909.11</v>
       </c>
     </row>
     <row r="1015">
@@ -11600,7 +11600,7 @@
         <v>2750</v>
       </c>
       <c r="C1015" t="n">
-        <v>38178</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1016">
@@ -11611,7 +11611,7 @@
         <v>2131</v>
       </c>
       <c r="C1016" t="n">
-        <v>76356</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1017">
@@ -11622,7 +11622,7 @@
         <v>818</v>
       </c>
       <c r="C1017" t="n">
-        <v>254534</v>
+        <v>272715</v>
       </c>
     </row>
     <row r="1018">
@@ -11633,7 +11633,7 @@
         <v>2566</v>
       </c>
       <c r="C1018" t="n">
-        <v>50904</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1019">
@@ -11644,7 +11644,7 @@
         <v>132</v>
       </c>
       <c r="C1019" t="n">
-        <v>477260</v>
+        <v>511350</v>
       </c>
     </row>
     <row r="1020">
@@ -11655,7 +11655,7 @@
         <v>2431</v>
       </c>
       <c r="C1020" t="n">
-        <v>117082</v>
+        <v>125445</v>
       </c>
     </row>
     <row r="1021">
@@ -11666,7 +11666,7 @@
         <v>2249</v>
       </c>
       <c r="C1021" t="n">
-        <v>124292</v>
+        <v>133170</v>
       </c>
     </row>
     <row r="1022">
@@ -11677,7 +11677,7 @@
         <v>1585</v>
       </c>
       <c r="C1022" t="n">
-        <v>105028</v>
+        <v>112530</v>
       </c>
     </row>
     <row r="1023">
@@ -11688,7 +11688,7 @@
         <v>2325</v>
       </c>
       <c r="C1023" t="n">
-        <v>101528</v>
+        <v>108780</v>
       </c>
     </row>
     <row r="1024">
@@ -11699,7 +11699,7 @@
         <v>2190</v>
       </c>
       <c r="C1024" t="n">
-        <v>143178</v>
+        <v>153405</v>
       </c>
     </row>
     <row r="1025">
@@ -11710,7 +11710,7 @@
         <v>1466</v>
       </c>
       <c r="C1025" t="n">
-        <v>257726</v>
+        <v>276135</v>
       </c>
     </row>
     <row r="1026">
@@ -11721,7 +11721,7 @@
         <v>2659</v>
       </c>
       <c r="C1026" t="n">
-        <v>78274</v>
+        <v>83865</v>
       </c>
     </row>
     <row r="1027">
@@ -11732,7 +11732,7 @@
         <v>634</v>
       </c>
       <c r="C1027" t="n">
-        <v>350000</v>
+        <v>375000</v>
       </c>
     </row>
     <row r="1028">
@@ -11743,7 +11743,7 @@
         <v>2804</v>
       </c>
       <c r="C1028" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1029">
@@ -11754,7 +11754,7 @@
         <v>2375</v>
       </c>
       <c r="C1029" t="n">
-        <v>210000</v>
+        <v>225000</v>
       </c>
     </row>
     <row r="1030">
@@ -11765,7 +11765,7 @@
         <v>2601</v>
       </c>
       <c r="C1030" t="n">
-        <v>175000</v>
+        <v>187500</v>
       </c>
     </row>
     <row r="1031">
@@ -11776,7 +11776,7 @@
         <v>952</v>
       </c>
       <c r="C1031" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1032">
@@ -11787,7 +11787,7 @@
         <v>571</v>
       </c>
       <c r="C1032" t="n">
-        <v>405034</v>
+        <v>433965</v>
       </c>
     </row>
     <row r="1033">
@@ -11798,7 +11798,7 @@
         <v>2697</v>
       </c>
       <c r="C1033" t="n">
-        <v>123410</v>
+        <v>132225</v>
       </c>
     </row>
     <row r="1034">
@@ -11809,7 +11809,7 @@
         <v>2678</v>
       </c>
       <c r="C1034" t="n">
-        <v>213514</v>
+        <v>228765</v>
       </c>
     </row>
     <row r="1035">
@@ -11820,7 +11820,7 @@
         <v>2768</v>
       </c>
       <c r="C1035" t="n">
-        <v>223454</v>
+        <v>239415</v>
       </c>
     </row>
     <row r="1036">
@@ -11831,7 +11831,7 @@
         <v>2359</v>
       </c>
       <c r="C1036" t="n">
-        <v>67774</v>
+        <v>72615</v>
       </c>
     </row>
     <row r="1037">
@@ -11842,7 +11842,7 @@
         <v>353</v>
       </c>
       <c r="C1037" t="n">
-        <v>220164</v>
+        <v>235890</v>
       </c>
     </row>
     <row r="1038">
@@ -11853,7 +11853,7 @@
         <v>2026</v>
       </c>
       <c r="C1038" t="n">
-        <v>182420</v>
+        <v>195450</v>
       </c>
     </row>
     <row r="1039">
@@ -11875,7 +11875,7 @@
         <v>2345</v>
       </c>
       <c r="C1040" t="n">
-        <v>40054</v>
+        <v>42915</v>
       </c>
     </row>
     <row r="1041">
@@ -11886,7 +11886,7 @@
         <v>2789</v>
       </c>
       <c r="C1041" t="n">
-        <v>108178</v>
+        <v>115905</v>
       </c>
     </row>
     <row r="1042">
@@ -11897,7 +11897,7 @@
         <v>569</v>
       </c>
       <c r="C1042" t="n">
-        <v>1822492</v>
+        <v>1952670</v>
       </c>
     </row>
     <row r="1043">
@@ -11908,7 +11908,7 @@
         <v>2822</v>
       </c>
       <c r="C1043" t="n">
-        <v>85904</v>
+        <v>92040</v>
       </c>
     </row>
     <row r="1044">
@@ -11919,7 +11919,7 @@
         <v>2728</v>
       </c>
       <c r="C1044" t="n">
-        <v>6356</v>
+        <v>6810</v>
       </c>
     </row>
     <row r="1045">
@@ -11930,7 +11930,7 @@
         <v>2488</v>
       </c>
       <c r="C1045" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1046">
@@ -11941,7 +11941,7 @@
         <v>2791</v>
       </c>
       <c r="C1046" t="n">
-        <v>62802.8</v>
+        <v>67288.7</v>
       </c>
     </row>
     <row r="1047">
@@ -11952,7 +11952,7 @@
         <v>2577</v>
       </c>
       <c r="C1047" t="n">
-        <v>56744.65</v>
+        <v>60797.83</v>
       </c>
     </row>
     <row r="1048">
@@ -11963,7 +11963,7 @@
         <v>2069</v>
       </c>
       <c r="C1048" t="n">
-        <v>114534</v>
+        <v>122715</v>
       </c>
     </row>
     <row r="1049">
@@ -11974,7 +11974,7 @@
         <v>2082</v>
       </c>
       <c r="C1049" t="n">
-        <v>105994</v>
+        <v>113565</v>
       </c>
     </row>
     <row r="1050">
@@ -11985,7 +11985,7 @@
         <v>781</v>
       </c>
       <c r="C1050" t="n">
-        <v>82726</v>
+        <v>88635</v>
       </c>
     </row>
     <row r="1051">
@@ -11996,7 +11996,7 @@
         <v>744</v>
       </c>
       <c r="C1051" t="n">
-        <v>26474</v>
+        <v>28365</v>
       </c>
     </row>
     <row r="1052">
@@ -12007,7 +12007,7 @@
         <v>2223</v>
       </c>
       <c r="C1052" t="n">
-        <v>83958</v>
+        <v>89955</v>
       </c>
     </row>
     <row r="1053">
@@ -12018,7 +12018,7 @@
         <v>2452</v>
       </c>
       <c r="C1053" t="n">
-        <v>44534</v>
+        <v>47715</v>
       </c>
     </row>
     <row r="1054">
@@ -12029,7 +12029,7 @@
         <v>970</v>
       </c>
       <c r="C1054" t="n">
-        <v>43708</v>
+        <v>46830</v>
       </c>
     </row>
     <row r="1055">
@@ -12040,7 +12040,7 @@
         <v>2550</v>
       </c>
       <c r="C1055" t="n">
-        <v>38808</v>
+        <v>41580</v>
       </c>
     </row>
     <row r="1056">
@@ -12051,7 +12051,7 @@
         <v>768</v>
       </c>
       <c r="C1056" t="n">
-        <v>82726</v>
+        <v>88635</v>
       </c>
     </row>
     <row r="1057">
@@ -12062,7 +12062,7 @@
         <v>1075</v>
       </c>
       <c r="C1057" t="n">
-        <v>288260</v>
+        <v>308850</v>
       </c>
     </row>
     <row r="1058">
@@ -12073,7 +12073,7 @@
         <v>664</v>
       </c>
       <c r="C1058" t="n">
-        <v>164808</v>
+        <v>176580</v>
       </c>
     </row>
     <row r="1059">
@@ -12084,7 +12084,7 @@
         <v>2555</v>
       </c>
       <c r="C1059" t="n">
-        <v>26418</v>
+        <v>28305</v>
       </c>
     </row>
     <row r="1060">
@@ -12095,7 +12095,7 @@
         <v>2627</v>
       </c>
       <c r="C1060" t="n">
-        <v>15512</v>
+        <v>16620</v>
       </c>
     </row>
     <row r="1061">
@@ -12106,7 +12106,7 @@
         <v>2557</v>
       </c>
       <c r="C1061" t="n">
-        <v>16408</v>
+        <v>17580</v>
       </c>
     </row>
     <row r="1062">
@@ -12117,7 +12117,7 @@
         <v>2551</v>
       </c>
       <c r="C1062" t="n">
-        <v>13034</v>
+        <v>13965</v>
       </c>
     </row>
     <row r="1063">
@@ -12128,7 +12128,7 @@
         <v>2463</v>
       </c>
       <c r="C1063" t="n">
-        <v>203770</v>
+        <v>218325</v>
       </c>
     </row>
     <row r="1064">
@@ -12139,7 +12139,7 @@
         <v>2279</v>
       </c>
       <c r="C1064" t="n">
-        <v>153734</v>
+        <v>164715</v>
       </c>
     </row>
     <row r="1065">
@@ -12150,7 +12150,7 @@
         <v>631</v>
       </c>
       <c r="C1065" t="n">
-        <v>222726</v>
+        <v>238635</v>
       </c>
     </row>
     <row r="1066">
@@ -12161,7 +12161,7 @@
         <v>2251</v>
       </c>
       <c r="C1066" t="n">
-        <v>136388</v>
+        <v>146130</v>
       </c>
     </row>
     <row r="1067">
@@ -12172,7 +12172,7 @@
         <v>1653</v>
       </c>
       <c r="C1067" t="n">
-        <v>206808</v>
+        <v>221580</v>
       </c>
     </row>
     <row r="1068">
@@ -12183,7 +12183,7 @@
         <v>1293</v>
       </c>
       <c r="C1068" t="n">
-        <v>264082</v>
+        <v>282945</v>
       </c>
     </row>
     <row r="1069">
@@ -12194,7 +12194,7 @@
         <v>360</v>
       </c>
       <c r="C1069" t="n">
-        <v>318178</v>
+        <v>340905</v>
       </c>
     </row>
     <row r="1070">
@@ -12205,7 +12205,7 @@
         <v>1063</v>
       </c>
       <c r="C1070" t="n">
-        <v>231350</v>
+        <v>247875</v>
       </c>
     </row>
     <row r="1071">
@@ -12216,7 +12216,7 @@
         <v>2273</v>
       </c>
       <c r="C1071" t="n">
-        <v>134960</v>
+        <v>144600</v>
       </c>
     </row>
     <row r="1072">
@@ -12227,7 +12227,7 @@
         <v>2757</v>
       </c>
       <c r="C1072" t="n">
-        <v>44545.52</v>
+        <v>47727.33</v>
       </c>
     </row>
     <row r="1073">
@@ -12238,7 +12238,7 @@
         <v>2795</v>
       </c>
       <c r="C1073" t="n">
-        <v>38181.84</v>
+        <v>40909.11</v>
       </c>
     </row>
     <row r="1074">
@@ -12249,7 +12249,7 @@
         <v>2722</v>
       </c>
       <c r="C1074" t="n">
-        <v>38178</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1075">
@@ -12260,7 +12260,7 @@
         <v>2718</v>
       </c>
       <c r="C1075" t="n">
-        <v>50904</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1076">
@@ -12271,7 +12271,7 @@
         <v>595</v>
       </c>
       <c r="C1076" t="n">
-        <v>350000</v>
+        <v>375000</v>
       </c>
     </row>
     <row r="1077">
@@ -12282,7 +12282,7 @@
         <v>890</v>
       </c>
       <c r="C1077" t="n">
-        <v>445452</v>
+        <v>477270</v>
       </c>
     </row>
     <row r="1078">
@@ -12293,7 +12293,7 @@
         <v>2652</v>
       </c>
       <c r="C1078" t="n">
-        <v>82726</v>
+        <v>88635</v>
       </c>
     </row>
     <row r="1079">
@@ -12304,7 +12304,7 @@
         <v>2714</v>
       </c>
       <c r="C1079" t="n">
-        <v>229082</v>
+        <v>245445</v>
       </c>
     </row>
     <row r="1080">
@@ -12315,7 +12315,7 @@
         <v>1869</v>
       </c>
       <c r="C1080" t="n">
-        <v>146356</v>
+        <v>156810</v>
       </c>
     </row>
     <row r="1081">
@@ -12326,7 +12326,7 @@
         <v>400</v>
       </c>
       <c r="C1081" t="n">
-        <v>120904</v>
+        <v>129540</v>
       </c>
     </row>
     <row r="1082">
@@ -12337,7 +12337,7 @@
         <v>1907</v>
       </c>
       <c r="C1082" t="n">
-        <v>236082</v>
+        <v>252945</v>
       </c>
     </row>
     <row r="1083">
@@ -12348,7 +12348,7 @@
         <v>1996</v>
       </c>
       <c r="C1083" t="n">
-        <v>149226</v>
+        <v>159885</v>
       </c>
     </row>
     <row r="1084">
@@ -12359,7 +12359,7 @@
         <v>1890</v>
       </c>
       <c r="C1084" t="n">
-        <v>201181.75</v>
+        <v>215551.86</v>
       </c>
     </row>
     <row r="1085">
@@ -12370,7 +12370,7 @@
         <v>2114</v>
       </c>
       <c r="C1085" t="n">
-        <v>116900</v>
+        <v>125250</v>
       </c>
     </row>
     <row r="1086">
@@ -12381,7 +12381,7 @@
         <v>2330</v>
       </c>
       <c r="C1086" t="n">
-        <v>171038</v>
+        <v>183255</v>
       </c>
     </row>
     <row r="1087">
@@ -12425,7 +12425,7 @@
         <v>931</v>
       </c>
       <c r="C1090" t="n">
-        <v>60088</v>
+        <v>64380</v>
       </c>
     </row>
     <row r="1091">
@@ -12436,7 +12436,7 @@
         <v>951</v>
       </c>
       <c r="C1091" t="n">
-        <v>73178</v>
+        <v>78405</v>
       </c>
     </row>
     <row r="1092">
@@ -12447,7 +12447,7 @@
         <v>2449</v>
       </c>
       <c r="C1092" t="n">
-        <v>25452</v>
+        <v>27270</v>
       </c>
     </row>
     <row r="1093">
@@ -12458,7 +12458,7 @@
         <v>610</v>
       </c>
       <c r="C1093" t="n">
-        <v>518630</v>
+        <v>555675</v>
       </c>
     </row>
     <row r="1094">
@@ -12469,7 +12469,7 @@
         <v>2761</v>
       </c>
       <c r="C1094" t="n">
-        <v>51856</v>
+        <v>55560</v>
       </c>
     </row>
     <row r="1095">
@@ -12480,7 +12480,7 @@
         <v>483</v>
       </c>
       <c r="C1095" t="n">
-        <v>281904</v>
+        <v>302040</v>
       </c>
     </row>
     <row r="1096">
@@ -12491,7 +12491,7 @@
         <v>2015</v>
       </c>
       <c r="C1096" t="n">
-        <v>235452</v>
+        <v>252270</v>
       </c>
     </row>
     <row r="1097">
@@ -12502,7 +12502,7 @@
         <v>1478</v>
       </c>
       <c r="C1097" t="n">
-        <v>344372</v>
+        <v>368970</v>
       </c>
     </row>
     <row r="1098">
@@ -12513,7 +12513,7 @@
         <v>424</v>
       </c>
       <c r="C1098" t="n">
-        <v>153734</v>
+        <v>164715</v>
       </c>
     </row>
     <row r="1099">
@@ -12535,7 +12535,7 @@
         <v>477</v>
       </c>
       <c r="C1100" t="n">
-        <v>164598</v>
+        <v>176355</v>
       </c>
     </row>
     <row r="1101">
@@ -12546,7 +12546,7 @@
         <v>1810</v>
       </c>
       <c r="C1101" t="n">
-        <v>25494</v>
+        <v>27315</v>
       </c>
     </row>
     <row r="1102">
@@ -12557,7 +12557,7 @@
         <v>2826</v>
       </c>
       <c r="C1102" t="n">
-        <v>44545.52</v>
+        <v>47727.33</v>
       </c>
     </row>
     <row r="1103">
@@ -12568,7 +12568,7 @@
         <v>2561</v>
       </c>
       <c r="C1103" t="n">
-        <v>9352</v>
+        <v>10020</v>
       </c>
     </row>
     <row r="1104">
@@ -12579,7 +12579,7 @@
         <v>2653</v>
       </c>
       <c r="C1104" t="n">
-        <v>38181.84</v>
+        <v>40909.11</v>
       </c>
     </row>
     <row r="1105">
@@ -12590,7 +12590,7 @@
         <v>2829</v>
       </c>
       <c r="C1105" t="n">
-        <v>38181.84</v>
+        <v>40909.11</v>
       </c>
     </row>
     <row r="1106">
@@ -12601,7 +12601,7 @@
         <v>2643</v>
       </c>
       <c r="C1106" t="n">
-        <v>18788</v>
+        <v>20130</v>
       </c>
     </row>
     <row r="1107">
@@ -12612,7 +12612,7 @@
         <v>2794</v>
       </c>
       <c r="C1107" t="n">
-        <v>57260</v>
+        <v>61350</v>
       </c>
     </row>
     <row r="1108">
@@ -12623,7 +12623,7 @@
         <v>2655</v>
       </c>
       <c r="C1108" t="n">
-        <v>70000</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="1109">
@@ -12634,7 +12634,7 @@
         <v>1456</v>
       </c>
       <c r="C1109" t="n">
-        <v>490182</v>
+        <v>525195</v>
       </c>
     </row>
     <row r="1110">
@@ -12645,7 +12645,7 @@
         <v>2606</v>
       </c>
       <c r="C1110" t="n">
-        <v>150556</v>
+        <v>161310</v>
       </c>
     </row>
     <row r="1111">
@@ -12656,7 +12656,7 @@
         <v>1142</v>
       </c>
       <c r="C1111" t="n">
-        <v>273028</v>
+        <v>292530</v>
       </c>
     </row>
     <row r="1112">
@@ -12667,7 +12667,7 @@
         <v>1450</v>
       </c>
       <c r="C1112" t="n">
-        <v>173446</v>
+        <v>185835</v>
       </c>
     </row>
     <row r="1113">
@@ -12678,7 +12678,7 @@
         <v>2133</v>
       </c>
       <c r="C1113" t="n">
-        <v>405034</v>
+        <v>433965</v>
       </c>
     </row>
     <row r="1114">
@@ -12689,7 +12689,7 @@
         <v>522</v>
       </c>
       <c r="C1114" t="n">
-        <v>124082</v>
+        <v>132945</v>
       </c>
     </row>
     <row r="1115">
@@ -12700,7 +12700,7 @@
         <v>2696</v>
       </c>
       <c r="C1115" t="n">
-        <v>167440</v>
+        <v>179400</v>
       </c>
     </row>
     <row r="1116">
@@ -12722,7 +12722,7 @@
         <v>2692</v>
       </c>
       <c r="C1117" t="n">
-        <v>47726</v>
+        <v>51135</v>
       </c>
     </row>
     <row r="1118">
@@ -12733,7 +12733,7 @@
         <v>2691</v>
       </c>
       <c r="C1118" t="n">
-        <v>85904</v>
+        <v>92040</v>
       </c>
     </row>
     <row r="1119">
@@ -12744,7 +12744,7 @@
         <v>1632</v>
       </c>
       <c r="C1119" t="n">
-        <v>159082</v>
+        <v>170445</v>
       </c>
     </row>
     <row r="1120">
@@ -12755,7 +12755,7 @@
         <v>2641</v>
       </c>
       <c r="C1120" t="n">
-        <v>50904</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1121">
@@ -12766,7 +12766,7 @@
         <v>2197</v>
       </c>
       <c r="C1121" t="n">
-        <v>127260</v>
+        <v>136350</v>
       </c>
     </row>
     <row r="1122">
@@ -12777,7 +12777,7 @@
         <v>609</v>
       </c>
       <c r="C1122" t="n">
-        <v>140000</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="1123">
@@ -12788,7 +12788,7 @@
         <v>1380</v>
       </c>
       <c r="C1123" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1124">
@@ -12799,7 +12799,7 @@
         <v>104</v>
       </c>
       <c r="C1124" t="n">
-        <v>190904</v>
+        <v>204540</v>
       </c>
     </row>
     <row r="1125">
@@ -12810,7 +12810,7 @@
         <v>2621</v>
       </c>
       <c r="C1125" t="n">
-        <v>44534</v>
+        <v>47715</v>
       </c>
     </row>
     <row r="1126">
@@ -12821,7 +12821,7 @@
         <v>2786</v>
       </c>
       <c r="C1126" t="n">
-        <v>44534</v>
+        <v>47715</v>
       </c>
     </row>
     <row r="1127">
@@ -12832,7 +12832,7 @@
         <v>2784</v>
       </c>
       <c r="C1127" t="n">
-        <v>26474</v>
+        <v>28365</v>
       </c>
     </row>
     <row r="1128">
@@ -12843,7 +12843,7 @@
         <v>2586</v>
       </c>
       <c r="C1128" t="n">
-        <v>26474</v>
+        <v>28365</v>
       </c>
     </row>
     <row r="1129">
@@ -12854,7 +12854,7 @@
         <v>2145</v>
       </c>
       <c r="C1129" t="n">
-        <v>82376</v>
+        <v>88260</v>
       </c>
     </row>
     <row r="1130">
@@ -12865,7 +12865,7 @@
         <v>2574</v>
       </c>
       <c r="C1130" t="n">
-        <v>82376</v>
+        <v>88260</v>
       </c>
     </row>
     <row r="1131">
@@ -12876,7 +12876,7 @@
         <v>2492</v>
       </c>
       <c r="C1131" t="n">
-        <v>90300</v>
+        <v>96750</v>
       </c>
     </row>
     <row r="1132">
@@ -12887,7 +12887,7 @@
         <v>629</v>
       </c>
       <c r="C1132" t="n">
-        <v>281260</v>
+        <v>301350</v>
       </c>
     </row>
     <row r="1133">
@@ -12898,7 +12898,7 @@
         <v>966</v>
       </c>
       <c r="C1133" t="n">
-        <v>51856</v>
+        <v>55560</v>
       </c>
     </row>
     <row r="1134">
@@ -12909,7 +12909,7 @@
         <v>2721</v>
       </c>
       <c r="C1134" t="n">
-        <v>51856</v>
+        <v>55560</v>
       </c>
     </row>
     <row r="1135">
@@ -12920,7 +12920,7 @@
         <v>2554</v>
       </c>
       <c r="C1135" t="n">
-        <v>15624</v>
+        <v>16740</v>
       </c>
     </row>
     <row r="1136">
@@ -12931,7 +12931,7 @@
         <v>2556</v>
       </c>
       <c r="C1136" t="n">
-        <v>22974</v>
+        <v>24615</v>
       </c>
     </row>
     <row r="1137">
@@ -12942,7 +12942,7 @@
         <v>2546</v>
       </c>
       <c r="C1137" t="n">
-        <v>15176</v>
+        <v>16260</v>
       </c>
     </row>
     <row r="1138">
@@ -12953,7 +12953,7 @@
         <v>42</v>
       </c>
       <c r="C1138" t="n">
-        <v>1202726</v>
+        <v>1288635</v>
       </c>
     </row>
     <row r="1139">
@@ -12964,7 +12964,7 @@
         <v>953</v>
       </c>
       <c r="C1139" t="n">
-        <v>434420</v>
+        <v>465450</v>
       </c>
     </row>
     <row r="1140">
@@ -12975,7 +12975,7 @@
         <v>675</v>
       </c>
       <c r="C1140" t="n">
-        <v>127260</v>
+        <v>136350</v>
       </c>
     </row>
     <row r="1141">
@@ -12986,7 +12986,7 @@
         <v>619</v>
       </c>
       <c r="C1141" t="n">
-        <v>196784</v>
+        <v>210840</v>
       </c>
     </row>
     <row r="1142">
@@ -12997,7 +12997,7 @@
         <v>1299</v>
       </c>
       <c r="C1142" t="n">
-        <v>331128</v>
+        <v>354780</v>
       </c>
     </row>
     <row r="1143">
@@ -13008,7 +13008,7 @@
         <v>1064</v>
       </c>
       <c r="C1143" t="n">
-        <v>381416</v>
+        <v>408660</v>
       </c>
     </row>
     <row r="1144">
@@ -13019,7 +13019,7 @@
         <v>2308</v>
       </c>
       <c r="C1144" t="n">
-        <v>130452</v>
+        <v>139770</v>
       </c>
     </row>
     <row r="1145">
@@ -13030,7 +13030,7 @@
         <v>1137</v>
       </c>
       <c r="C1145" t="n">
-        <v>407260</v>
+        <v>436350</v>
       </c>
     </row>
     <row r="1146">
@@ -13041,7 +13041,7 @@
         <v>2747</v>
       </c>
       <c r="C1146" t="n">
-        <v>38181.84</v>
+        <v>40909.11</v>
       </c>
     </row>
     <row r="1147">
@@ -13052,7 +13052,7 @@
         <v>2819</v>
       </c>
       <c r="C1147" t="n">
-        <v>38181.84</v>
+        <v>40909.11</v>
       </c>
     </row>
     <row r="1148">
@@ -13063,7 +13063,7 @@
         <v>1259</v>
       </c>
       <c r="C1148" t="n">
-        <v>63636.4</v>
+        <v>68181.85000000001</v>
       </c>
     </row>
     <row r="1149">
@@ -13074,7 +13074,7 @@
         <v>2544</v>
       </c>
       <c r="C1149" t="n">
-        <v>50904</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1150">
@@ -13085,7 +13085,7 @@
         <v>2261</v>
       </c>
       <c r="C1150" t="n">
-        <v>95452</v>
+        <v>102270</v>
       </c>
     </row>
     <row r="1151">
@@ -13096,7 +13096,7 @@
         <v>2729</v>
       </c>
       <c r="C1151" t="n">
-        <v>50904</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1152">
@@ -13107,7 +13107,7 @@
         <v>2649</v>
       </c>
       <c r="C1152" t="n">
-        <v>18788</v>
+        <v>20130</v>
       </c>
     </row>
     <row r="1153">
@@ -13118,7 +13118,7 @@
         <v>2494</v>
       </c>
       <c r="C1153" t="n">
-        <v>82726</v>
+        <v>88635</v>
       </c>
     </row>
     <row r="1154">
@@ -13129,7 +13129,7 @@
         <v>1384</v>
       </c>
       <c r="C1154" t="n">
-        <v>286356</v>
+        <v>306810</v>
       </c>
     </row>
     <row r="1155">
@@ -13151,7 +13151,7 @@
         <v>2802</v>
       </c>
       <c r="C1156" t="n">
-        <v>45066</v>
+        <v>48285</v>
       </c>
     </row>
     <row r="1157">
@@ -13162,7 +13162,7 @@
         <v>2726</v>
       </c>
       <c r="C1157" t="n">
-        <v>95452</v>
+        <v>102270</v>
       </c>
     </row>
     <row r="1158">
@@ -13173,7 +13173,7 @@
         <v>2820</v>
       </c>
       <c r="C1158" t="n">
-        <v>114534</v>
+        <v>122715</v>
       </c>
     </row>
     <row r="1159">
@@ -13184,7 +13184,7 @@
         <v>1007</v>
       </c>
       <c r="C1159" t="n">
-        <v>120904</v>
+        <v>129540</v>
       </c>
     </row>
     <row r="1160">
@@ -13195,7 +13195,7 @@
         <v>20</v>
       </c>
       <c r="C1160" t="n">
-        <v>245000</v>
+        <v>262500</v>
       </c>
     </row>
     <row r="1161">
@@ -13206,7 +13206,7 @@
         <v>1372</v>
       </c>
       <c r="C1161" t="n">
-        <v>184534</v>
+        <v>197715</v>
       </c>
     </row>
     <row r="1162">
@@ -13217,7 +13217,7 @@
         <v>2735</v>
       </c>
       <c r="C1162" t="n">
-        <v>76356</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1163">
@@ -13228,7 +13228,7 @@
         <v>2811</v>
       </c>
       <c r="C1163" t="n">
-        <v>26474</v>
+        <v>28365</v>
       </c>
     </row>
     <row r="1164">
@@ -13239,7 +13239,7 @@
         <v>1871</v>
       </c>
       <c r="C1164" t="n">
-        <v>112476</v>
+        <v>120510</v>
       </c>
     </row>
     <row r="1165">
@@ -13250,7 +13250,7 @@
         <v>2541</v>
       </c>
       <c r="C1165" t="n">
-        <v>134652</v>
+        <v>144270</v>
       </c>
     </row>
     <row r="1166">
@@ -13261,7 +13261,7 @@
         <v>2362</v>
       </c>
       <c r="C1166" t="n">
-        <v>47726</v>
+        <v>51135</v>
       </c>
     </row>
     <row r="1167">
@@ -13272,7 +13272,7 @@
         <v>1324</v>
       </c>
       <c r="C1167" t="n">
-        <v>178178</v>
+        <v>190905</v>
       </c>
     </row>
     <row r="1168">
@@ -13283,7 +13283,7 @@
         <v>2323</v>
       </c>
       <c r="C1168" t="n">
-        <v>43708</v>
+        <v>46830</v>
       </c>
     </row>
     <row r="1169">
@@ -13294,7 +13294,7 @@
         <v>2647</v>
       </c>
       <c r="C1169" t="n">
-        <v>90300</v>
+        <v>96750</v>
       </c>
     </row>
     <row r="1170">
@@ -13305,7 +13305,7 @@
         <v>559</v>
       </c>
       <c r="C1170" t="n">
-        <v>146006</v>
+        <v>156435</v>
       </c>
     </row>
     <row r="1171">
@@ -13316,7 +13316,7 @@
         <v>2762</v>
       </c>
       <c r="C1171" t="n">
-        <v>51856</v>
+        <v>55560</v>
       </c>
     </row>
     <row r="1172">
@@ -13327,7 +13327,7 @@
         <v>2501</v>
       </c>
       <c r="C1172" t="n">
-        <v>51856</v>
+        <v>55560</v>
       </c>
     </row>
     <row r="1173">
@@ -13338,7 +13338,7 @@
         <v>2562</v>
       </c>
       <c r="C1173" t="n">
-        <v>10066</v>
+        <v>10785</v>
       </c>
     </row>
     <row r="1174">
@@ -13349,7 +13349,7 @@
         <v>429</v>
       </c>
       <c r="C1174" t="n">
-        <v>248178</v>
+        <v>265905</v>
       </c>
     </row>
     <row r="1175">
@@ -13360,7 +13360,7 @@
         <v>58</v>
       </c>
       <c r="C1175" t="n">
-        <v>172186</v>
+        <v>184485</v>
       </c>
     </row>
     <row r="1176">
@@ -13371,7 +13371,7 @@
         <v>2245</v>
       </c>
       <c r="C1176" t="n">
-        <v>153734</v>
+        <v>164715</v>
       </c>
     </row>
     <row r="1177">
@@ -13382,7 +13382,7 @@
         <v>285</v>
       </c>
       <c r="C1177" t="n">
-        <v>344372</v>
+        <v>368970</v>
       </c>
     </row>
     <row r="1178">
@@ -13404,7 +13404,7 @@
         <v>363</v>
       </c>
       <c r="C1179" t="n">
-        <v>190904</v>
+        <v>204540</v>
       </c>
     </row>
     <row r="1180">
@@ -13415,7 +13415,7 @@
         <v>2651</v>
       </c>
       <c r="C1180" t="n">
-        <v>107618</v>
+        <v>115305</v>
       </c>
     </row>
     <row r="1181">
@@ -13426,7 +13426,7 @@
         <v>2142</v>
       </c>
       <c r="C1181" t="n">
-        <v>33964</v>
+        <v>36390</v>
       </c>
     </row>
     <row r="1182">
@@ -13437,7 +13437,7 @@
         <v>2258</v>
       </c>
       <c r="C1182" t="n">
-        <v>50909.12</v>
+        <v>54545.48</v>
       </c>
     </row>
     <row r="1183">
@@ -13448,7 +13448,7 @@
         <v>2772</v>
       </c>
       <c r="C1183" t="n">
-        <v>38181.84</v>
+        <v>40909.11</v>
       </c>
     </row>
     <row r="1184">
@@ -13459,7 +13459,7 @@
         <v>2346</v>
       </c>
       <c r="C1184" t="n">
-        <v>70000</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="1185">
@@ -13470,7 +13470,7 @@
         <v>2442</v>
       </c>
       <c r="C1185" t="n">
-        <v>50904</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1186">
@@ -13481,7 +13481,7 @@
         <v>772</v>
       </c>
       <c r="C1186" t="n">
-        <v>210000</v>
+        <v>225000</v>
       </c>
     </row>
     <row r="1187">
@@ -13492,7 +13492,7 @@
         <v>2684</v>
       </c>
       <c r="C1187" t="n">
-        <v>60452</v>
+        <v>64770</v>
       </c>
     </row>
     <row r="1188">
@@ -13503,7 +13503,7 @@
         <v>2765</v>
       </c>
       <c r="C1188" t="n">
-        <v>57260</v>
+        <v>61350</v>
       </c>
     </row>
     <row r="1189">
@@ -13514,7 +13514,7 @@
         <v>2567</v>
       </c>
       <c r="C1189" t="n">
-        <v>105028</v>
+        <v>112530</v>
       </c>
     </row>
     <row r="1190">
@@ -13525,7 +13525,7 @@
         <v>2178</v>
       </c>
       <c r="C1190" t="n">
-        <v>178178</v>
+        <v>190905</v>
       </c>
     </row>
     <row r="1191">
@@ -13536,7 +13536,7 @@
         <v>2827</v>
       </c>
       <c r="C1191" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1192">
@@ -13547,7 +13547,7 @@
         <v>2510</v>
       </c>
       <c r="C1192" t="n">
-        <v>353332</v>
+        <v>378570</v>
       </c>
     </row>
     <row r="1193">
@@ -13558,7 +13558,7 @@
         <v>2392</v>
       </c>
       <c r="C1193" t="n">
-        <v>105994</v>
+        <v>113565</v>
       </c>
     </row>
     <row r="1194">
@@ -13569,7 +13569,7 @@
         <v>415</v>
       </c>
       <c r="C1194" t="n">
-        <v>362404</v>
+        <v>388290</v>
       </c>
     </row>
     <row r="1195">
@@ -13580,7 +13580,7 @@
         <v>2107</v>
       </c>
       <c r="C1195" t="n">
-        <v>187138</v>
+        <v>200505</v>
       </c>
     </row>
     <row r="1196">
@@ -13591,7 +13591,7 @@
         <v>2211</v>
       </c>
       <c r="C1196" t="n">
-        <v>155148</v>
+        <v>166230</v>
       </c>
     </row>
     <row r="1197">
@@ -13602,7 +13602,7 @@
         <v>2682</v>
       </c>
       <c r="C1197" t="n">
-        <v>95438</v>
+        <v>102255</v>
       </c>
     </row>
     <row r="1198">
@@ -13635,7 +13635,7 @@
         <v>2755</v>
       </c>
       <c r="C1200" t="n">
-        <v>38178</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1201">
@@ -13646,7 +13646,7 @@
         <v>941</v>
       </c>
       <c r="C1201" t="n">
-        <v>250012</v>
+        <v>267870</v>
       </c>
     </row>
     <row r="1202">
@@ -13657,7 +13657,7 @@
         <v>2734</v>
       </c>
       <c r="C1202" t="n">
-        <v>35042</v>
+        <v>37545</v>
       </c>
     </row>
     <row r="1203">
@@ -13668,7 +13668,7 @@
         <v>1289</v>
       </c>
       <c r="C1203" t="n">
-        <v>159082</v>
+        <v>170445</v>
       </c>
     </row>
     <row r="1204">
@@ -13679,7 +13679,7 @@
         <v>2801</v>
       </c>
       <c r="C1204" t="n">
-        <v>50904</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1205">
@@ -13690,7 +13690,7 @@
         <v>2810</v>
       </c>
       <c r="C1205" t="n">
-        <v>85904</v>
+        <v>92040</v>
       </c>
     </row>
     <row r="1206">
@@ -13701,7 +13701,7 @@
         <v>767</v>
       </c>
       <c r="C1206" t="n">
-        <v>114534</v>
+        <v>122715</v>
       </c>
     </row>
     <row r="1207">
@@ -13712,7 +13712,7 @@
         <v>2687</v>
       </c>
       <c r="C1207" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1208">
@@ -13723,7 +13723,7 @@
         <v>2686</v>
       </c>
       <c r="C1208" t="n">
-        <v>82726</v>
+        <v>88635</v>
       </c>
     </row>
     <row r="1209">
@@ -13734,7 +13734,7 @@
         <v>2730</v>
       </c>
       <c r="C1209" t="n">
-        <v>57260</v>
+        <v>61350</v>
       </c>
     </row>
     <row r="1210">
@@ -13745,7 +13745,7 @@
         <v>2580</v>
       </c>
       <c r="C1210" t="n">
-        <v>21350</v>
+        <v>22875</v>
       </c>
     </row>
     <row r="1211">
@@ -13756,7 +13756,7 @@
         <v>2472</v>
       </c>
       <c r="C1211" t="n">
-        <v>33690.4</v>
+        <v>36096.85</v>
       </c>
     </row>
     <row r="1212">
@@ -13767,7 +13767,7 @@
         <v>2631</v>
       </c>
       <c r="C1212" t="n">
-        <v>15611.28</v>
+        <v>16726.37</v>
       </c>
     </row>
     <row r="1213">
@@ -13778,7 +13778,7 @@
         <v>1642</v>
       </c>
       <c r="C1213" t="n">
-        <v>168630</v>
+        <v>180675</v>
       </c>
     </row>
     <row r="1214">
@@ -13789,7 +13789,7 @@
         <v>2613</v>
       </c>
       <c r="C1214" t="n">
-        <v>114030</v>
+        <v>122175</v>
       </c>
     </row>
     <row r="1215">
@@ -13800,7 +13800,7 @@
         <v>1020</v>
       </c>
       <c r="C1215" t="n">
-        <v>57260</v>
+        <v>61350</v>
       </c>
     </row>
     <row r="1216">
@@ -13811,7 +13811,7 @@
         <v>2785</v>
       </c>
       <c r="C1216" t="n">
-        <v>26474</v>
+        <v>28365</v>
       </c>
     </row>
     <row r="1217">
@@ -13822,7 +13822,7 @@
         <v>1327</v>
       </c>
       <c r="C1217" t="n">
-        <v>38178</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1218">
@@ -13833,7 +13833,7 @@
         <v>2629</v>
       </c>
       <c r="C1218" t="n">
-        <v>43708</v>
+        <v>46830</v>
       </c>
     </row>
     <row r="1219">
@@ -13844,7 +13844,7 @@
         <v>749</v>
       </c>
       <c r="C1219" t="n">
-        <v>51856</v>
+        <v>55560</v>
       </c>
     </row>
     <row r="1220">
@@ -13855,7 +13855,7 @@
         <v>1983</v>
       </c>
       <c r="C1220" t="n">
-        <v>344372</v>
+        <v>368970</v>
       </c>
     </row>
     <row r="1221">
@@ -13866,7 +13866,7 @@
         <v>1993</v>
       </c>
       <c r="C1221" t="n">
-        <v>221382</v>
+        <v>237195</v>
       </c>
     </row>
     <row r="1222">
@@ -13877,7 +13877,7 @@
         <v>2767</v>
       </c>
       <c r="C1222" t="n">
-        <v>122766</v>
+        <v>131535</v>
       </c>
     </row>
     <row r="1223">
@@ -13899,7 +13899,7 @@
         <v>1102</v>
       </c>
       <c r="C1224" t="n">
-        <v>153734</v>
+        <v>164715</v>
       </c>
     </row>
     <row r="1225">
@@ -13910,7 +13910,7 @@
         <v>626</v>
       </c>
       <c r="C1225" t="n">
-        <v>1084564.12</v>
+        <v>1162032.98</v>
       </c>
     </row>
     <row r="1226">
@@ -13921,7 +13921,7 @@
         <v>1465</v>
       </c>
       <c r="C1226" t="n">
-        <v>228956</v>
+        <v>245310</v>
       </c>
     </row>
     <row r="1227">
@@ -13932,7 +13932,7 @@
         <v>2758</v>
       </c>
       <c r="C1227" t="n">
-        <v>38181.84</v>
+        <v>40909.11</v>
       </c>
     </row>
     <row r="1228">
@@ -13943,7 +13943,7 @@
         <v>2742</v>
       </c>
       <c r="C1228" t="n">
-        <v>38181.84</v>
+        <v>40909.11</v>
       </c>
     </row>
     <row r="1229">
@@ -13965,7 +13965,7 @@
         <v>1873</v>
       </c>
       <c r="C1230" t="n">
-        <v>203630</v>
+        <v>218175</v>
       </c>
     </row>
     <row r="1231">
@@ -13976,7 +13976,7 @@
         <v>2163</v>
       </c>
       <c r="C1231" t="n">
-        <v>95452</v>
+        <v>102270</v>
       </c>
     </row>
     <row r="1232">
@@ -13987,7 +13987,7 @@
         <v>2394</v>
       </c>
       <c r="C1232" t="n">
-        <v>98028</v>
+        <v>105030</v>
       </c>
     </row>
     <row r="1233">
@@ -13998,7 +13998,7 @@
         <v>33</v>
       </c>
       <c r="C1233" t="n">
-        <v>246904</v>
+        <v>264540</v>
       </c>
     </row>
     <row r="1234">
@@ -14009,7 +14009,7 @@
         <v>2421</v>
       </c>
       <c r="C1234" t="n">
-        <v>41356</v>
+        <v>44310</v>
       </c>
     </row>
     <row r="1235">
@@ -14020,7 +14020,7 @@
         <v>2663</v>
       </c>
       <c r="C1235" t="n">
-        <v>175000</v>
+        <v>187500</v>
       </c>
     </row>
     <row r="1236">
@@ -14031,7 +14031,7 @@
         <v>2413</v>
       </c>
       <c r="C1236" t="n">
-        <v>77028</v>
+        <v>82530</v>
       </c>
     </row>
     <row r="1237">
@@ -14042,7 +14042,7 @@
         <v>351</v>
       </c>
       <c r="C1237" t="n">
-        <v>117082</v>
+        <v>125445</v>
       </c>
     </row>
     <row r="1238">
@@ -14053,7 +14053,7 @@
         <v>1298</v>
       </c>
       <c r="C1238" t="n">
-        <v>810082</v>
+        <v>867945</v>
       </c>
     </row>
     <row r="1239">
@@ -14064,7 +14064,7 @@
         <v>2491</v>
       </c>
       <c r="C1239" t="n">
-        <v>65464</v>
+        <v>70140</v>
       </c>
     </row>
     <row r="1240">
@@ -14075,7 +14075,7 @@
         <v>2571</v>
       </c>
       <c r="C1240" t="n">
-        <v>92442</v>
+        <v>99045</v>
       </c>
     </row>
     <row r="1241">
@@ -14086,7 +14086,7 @@
         <v>2507</v>
       </c>
       <c r="C1241" t="n">
-        <v>56168</v>
+        <v>60180</v>
       </c>
     </row>
     <row r="1242">
@@ -14097,7 +14097,7 @@
         <v>2799</v>
       </c>
       <c r="C1242" t="n">
-        <v>72296</v>
+        <v>77460</v>
       </c>
     </row>
     <row r="1243">
@@ -14119,7 +14119,7 @@
         <v>2582</v>
       </c>
       <c r="C1244" t="n">
-        <v>55076</v>
+        <v>59010</v>
       </c>
     </row>
     <row r="1245">
@@ -14130,7 +14130,7 @@
         <v>2637</v>
       </c>
       <c r="C1245" t="n">
-        <v>40054</v>
+        <v>42915</v>
       </c>
     </row>
     <row r="1246">
@@ -14141,7 +14141,7 @@
         <v>630</v>
       </c>
       <c r="C1246" t="n">
-        <v>95256</v>
+        <v>102060</v>
       </c>
     </row>
     <row r="1247">
@@ -14152,7 +14152,7 @@
         <v>525</v>
       </c>
       <c r="C1247" t="n">
-        <v>143178</v>
+        <v>153405</v>
       </c>
     </row>
     <row r="1248">
@@ -14163,7 +14163,7 @@
         <v>2727</v>
       </c>
       <c r="C1248" t="n">
-        <v>25760</v>
+        <v>27600</v>
       </c>
     </row>
     <row r="1249">
@@ -14174,7 +14174,7 @@
         <v>2707</v>
       </c>
       <c r="C1249" t="n">
-        <v>20384</v>
+        <v>21840</v>
       </c>
     </row>
     <row r="1250">
@@ -14185,7 +14185,7 @@
         <v>2834</v>
       </c>
       <c r="C1250" t="n">
-        <v>10530.56</v>
+        <v>11282.74</v>
       </c>
     </row>
     <row r="1251">
@@ -14196,7 +14196,7 @@
         <v>2773</v>
       </c>
       <c r="C1251" t="n">
-        <v>51349.52</v>
+        <v>55017.33</v>
       </c>
     </row>
     <row r="1252">
@@ -14207,7 +14207,7 @@
         <v>2341</v>
       </c>
       <c r="C1252" t="n">
-        <v>90300</v>
+        <v>96750</v>
       </c>
     </row>
     <row r="1253">
@@ -14218,7 +14218,7 @@
         <v>1374</v>
       </c>
       <c r="C1253" t="n">
-        <v>114534</v>
+        <v>122715</v>
       </c>
     </row>
     <row r="1254">
@@ -14229,7 +14229,7 @@
         <v>793</v>
       </c>
       <c r="C1254" t="n">
-        <v>26474</v>
+        <v>28365</v>
       </c>
     </row>
     <row r="1255">
@@ -14240,7 +14240,7 @@
         <v>794</v>
       </c>
       <c r="C1255" t="n">
-        <v>26474</v>
+        <v>28365</v>
       </c>
     </row>
     <row r="1256">
@@ -14251,7 +14251,7 @@
         <v>1834</v>
       </c>
       <c r="C1256" t="n">
-        <v>74452</v>
+        <v>79770</v>
       </c>
     </row>
     <row r="1257">
@@ -14262,7 +14262,7 @@
         <v>802</v>
       </c>
       <c r="C1257" t="n">
-        <v>47726</v>
+        <v>51135</v>
       </c>
     </row>
     <row r="1258">
@@ -14273,7 +14273,7 @@
         <v>1344</v>
       </c>
       <c r="C1258" t="n">
-        <v>95452</v>
+        <v>102270</v>
       </c>
     </row>
     <row r="1259">
@@ -14284,7 +14284,7 @@
         <v>1881</v>
       </c>
       <c r="C1259" t="n">
-        <v>43708</v>
+        <v>46830</v>
       </c>
     </row>
     <row r="1260">
@@ -14295,7 +14295,7 @@
         <v>2365</v>
       </c>
       <c r="C1260" t="n">
-        <v>50694</v>
+        <v>54315</v>
       </c>
     </row>
     <row r="1261">
@@ -14306,7 +14306,7 @@
         <v>2411</v>
       </c>
       <c r="C1261" t="n">
-        <v>90300</v>
+        <v>96750</v>
       </c>
     </row>
     <row r="1262">
@@ -14317,7 +14317,7 @@
         <v>2363</v>
       </c>
       <c r="C1262" t="n">
-        <v>95452</v>
+        <v>102270</v>
       </c>
     </row>
     <row r="1263">
@@ -14328,7 +14328,7 @@
         <v>2124</v>
       </c>
       <c r="C1263" t="n">
-        <v>222726</v>
+        <v>238635</v>
       </c>
     </row>
     <row r="1264">
@@ -14339,7 +14339,7 @@
         <v>1937</v>
       </c>
       <c r="C1264" t="n">
-        <v>162260</v>
+        <v>173850</v>
       </c>
     </row>
     <row r="1265">
@@ -14350,7 +14350,7 @@
         <v>2709</v>
       </c>
       <c r="C1265" t="n">
-        <v>114534</v>
+        <v>122715</v>
       </c>
     </row>
     <row r="1266">
@@ -14361,7 +14361,7 @@
         <v>2558</v>
       </c>
       <c r="C1266" t="n">
-        <v>19124</v>
+        <v>20490</v>
       </c>
     </row>
     <row r="1267">
@@ -14372,7 +14372,7 @@
         <v>663</v>
       </c>
       <c r="C1267" t="n">
-        <v>162260</v>
+        <v>173850</v>
       </c>
     </row>
     <row r="1268">
@@ -14383,7 +14383,7 @@
         <v>40</v>
       </c>
       <c r="C1268" t="n">
-        <v>140000</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="1269">
@@ -14394,7 +14394,7 @@
         <v>2833</v>
       </c>
       <c r="C1269" t="n">
-        <v>44545.52</v>
+        <v>47727.33</v>
       </c>
     </row>
     <row r="1270">
@@ -14405,7 +14405,7 @@
         <v>1756</v>
       </c>
       <c r="C1270" t="n">
-        <v>277774</v>
+        <v>297615</v>
       </c>
     </row>
     <row r="1271">
@@ -14416,7 +14416,7 @@
         <v>1116</v>
       </c>
       <c r="C1271" t="n">
-        <v>161406</v>
+        <v>172935</v>
       </c>
     </row>
     <row r="1272">
@@ -14427,7 +14427,7 @@
         <v>636</v>
       </c>
       <c r="C1272" t="n">
-        <v>159082</v>
+        <v>170445</v>
       </c>
     </row>
     <row r="1273">
@@ -14438,7 +14438,7 @@
         <v>1800</v>
       </c>
       <c r="C1273" t="n">
-        <v>17808</v>
+        <v>19080</v>
       </c>
     </row>
     <row r="1274">
@@ -14449,7 +14449,7 @@
         <v>2815</v>
       </c>
       <c r="C1274" t="n">
-        <v>38181.84</v>
+        <v>40909.11</v>
       </c>
     </row>
     <row r="1275">
@@ -14460,7 +14460,7 @@
         <v>1658</v>
       </c>
       <c r="C1275" t="n">
-        <v>84000</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="1276">
@@ -14471,7 +14471,7 @@
         <v>2635</v>
       </c>
       <c r="C1276" t="n">
-        <v>82726</v>
+        <v>88635</v>
       </c>
     </row>
     <row r="1277">
@@ -14482,7 +14482,7 @@
         <v>2402</v>
       </c>
       <c r="C1277" t="n">
-        <v>414904</v>
+        <v>444540</v>
       </c>
     </row>
     <row r="1278">
@@ -14493,7 +14493,7 @@
         <v>452</v>
       </c>
       <c r="C1278" t="n">
-        <v>171808</v>
+        <v>184080</v>
       </c>
     </row>
     <row r="1279">
@@ -14504,7 +14504,7 @@
         <v>2085</v>
       </c>
       <c r="C1279" t="n">
-        <v>84028</v>
+        <v>90030</v>
       </c>
     </row>
     <row r="1280">
@@ -14515,7 +14515,7 @@
         <v>2568</v>
       </c>
       <c r="C1280" t="n">
-        <v>130088</v>
+        <v>139380</v>
       </c>
     </row>
     <row r="1281">
@@ -14526,7 +14526,7 @@
         <v>1906</v>
       </c>
       <c r="C1281" t="n">
-        <v>73836</v>
+        <v>79110</v>
       </c>
     </row>
     <row r="1282">
@@ -14537,7 +14537,7 @@
         <v>2821</v>
       </c>
       <c r="C1282" t="n">
-        <v>64204</v>
+        <v>68790</v>
       </c>
     </row>
     <row r="1283">
@@ -14548,7 +14548,7 @@
         <v>2698</v>
       </c>
       <c r="C1283" t="n">
-        <v>78694</v>
+        <v>84315</v>
       </c>
     </row>
     <row r="1284">
@@ -14559,7 +14559,7 @@
         <v>2118</v>
       </c>
       <c r="C1284" t="n">
-        <v>150920</v>
+        <v>161700</v>
       </c>
     </row>
     <row r="1285">
@@ -14570,7 +14570,7 @@
         <v>2383</v>
       </c>
       <c r="C1285" t="n">
-        <v>88116</v>
+        <v>94410</v>
       </c>
     </row>
     <row r="1286">
@@ -14581,7 +14581,7 @@
         <v>2813</v>
       </c>
       <c r="C1286" t="n">
-        <v>40054</v>
+        <v>42915</v>
       </c>
     </row>
     <row r="1287">
@@ -14592,7 +14592,7 @@
         <v>925</v>
       </c>
       <c r="C1287" t="n">
-        <v>50064</v>
+        <v>53640</v>
       </c>
     </row>
     <row r="1288">
@@ -14603,7 +14603,7 @@
         <v>2689</v>
       </c>
       <c r="C1288" t="n">
-        <v>40054</v>
+        <v>42915</v>
       </c>
     </row>
     <row r="1289">
@@ -14614,7 +14614,7 @@
         <v>2716</v>
       </c>
       <c r="C1289" t="n">
-        <v>55076</v>
+        <v>59010</v>
       </c>
     </row>
     <row r="1290">
@@ -14625,7 +14625,7 @@
         <v>2831</v>
       </c>
       <c r="C1290" t="n">
-        <v>38178</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1291">
@@ -14636,7 +14636,7 @@
         <v>2045</v>
       </c>
       <c r="C1291" t="n">
-        <v>214108.18</v>
+        <v>229401.61</v>
       </c>
     </row>
     <row r="1292">
@@ -14647,7 +14647,7 @@
         <v>580</v>
       </c>
       <c r="C1292" t="n">
-        <v>85904</v>
+        <v>92040</v>
       </c>
     </row>
     <row r="1293">
@@ -14658,7 +14658,7 @@
         <v>438</v>
       </c>
       <c r="C1293" t="n">
-        <v>98630</v>
+        <v>105675</v>
       </c>
     </row>
     <row r="1294">
@@ -14669,7 +14669,7 @@
         <v>1539</v>
       </c>
       <c r="C1294" t="n">
-        <v>108178</v>
+        <v>115905</v>
       </c>
     </row>
     <row r="1295">
@@ -14680,7 +14680,7 @@
         <v>2817</v>
       </c>
       <c r="C1295" t="n">
-        <v>38178</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1296">
@@ -14691,7 +14691,7 @@
         <v>2816</v>
       </c>
       <c r="C1296" t="n">
-        <v>82726</v>
+        <v>88635</v>
       </c>
     </row>
     <row r="1297">
@@ -14702,7 +14702,7 @@
         <v>2146</v>
       </c>
       <c r="C1297" t="n">
-        <v>128324</v>
+        <v>137490</v>
       </c>
     </row>
     <row r="1298">
@@ -14713,7 +14713,7 @@
         <v>2276</v>
       </c>
       <c r="C1298" t="n">
-        <v>142576</v>
+        <v>152760</v>
       </c>
     </row>
     <row r="1299">
@@ -14724,7 +14724,7 @@
         <v>1381</v>
       </c>
       <c r="C1299" t="n">
-        <v>187726</v>
+        <v>201135</v>
       </c>
     </row>
     <row r="1300">
@@ -14735,7 +14735,7 @@
         <v>2081</v>
       </c>
       <c r="C1300" t="n">
-        <v>95452</v>
+        <v>102270</v>
       </c>
     </row>
     <row r="1301">
@@ -14746,7 +14746,7 @@
         <v>14</v>
       </c>
       <c r="C1301" t="n">
-        <v>276808</v>
+        <v>296580</v>
       </c>
     </row>
     <row r="1302">
@@ -14757,7 +14757,7 @@
         <v>766</v>
       </c>
       <c r="C1302" t="n">
-        <v>43708</v>
+        <v>46830</v>
       </c>
     </row>
     <row r="1303">
@@ -14768,7 +14768,7 @@
         <v>2547</v>
       </c>
       <c r="C1303" t="n">
-        <v>26166</v>
+        <v>28035</v>
       </c>
     </row>
     <row r="1304">
@@ -14779,7 +14779,7 @@
         <v>2552</v>
       </c>
       <c r="C1304" t="n">
-        <v>18816</v>
+        <v>20160</v>
       </c>
     </row>
     <row r="1305">
@@ -14790,7 +14790,7 @@
         <v>131</v>
       </c>
       <c r="C1305" t="n">
-        <v>260260</v>
+        <v>278850</v>
       </c>
     </row>
     <row r="1306">
@@ -14801,7 +14801,7 @@
         <v>2250</v>
       </c>
       <c r="C1306" t="n">
-        <v>210574</v>
+        <v>225615</v>
       </c>
     </row>
     <row r="1307">
@@ -14812,7 +14812,7 @@
         <v>89</v>
       </c>
       <c r="C1307" t="n">
-        <v>215208</v>
+        <v>230580</v>
       </c>
     </row>
     <row r="1308">
@@ -14823,7 +14823,7 @@
         <v>2141</v>
       </c>
       <c r="C1308" t="n">
-        <v>20132</v>
+        <v>21570</v>
       </c>
     </row>
     <row r="1309">
@@ -14834,7 +14834,7 @@
         <v>2798</v>
       </c>
       <c r="C1309" t="n">
-        <v>38181.84</v>
+        <v>40909.11</v>
       </c>
     </row>
     <row r="1310">
@@ -14845,7 +14845,7 @@
         <v>2797</v>
       </c>
       <c r="C1310" t="n">
-        <v>38181.84</v>
+        <v>40909.11</v>
       </c>
     </row>
     <row r="1311">
@@ -14856,7 +14856,7 @@
         <v>2266</v>
       </c>
       <c r="C1311" t="n">
-        <v>50909.12</v>
+        <v>54545.48</v>
       </c>
     </row>
     <row r="1312">
@@ -14867,7 +14867,7 @@
         <v>1499</v>
       </c>
       <c r="C1312" t="n">
-        <v>89082</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1313">
@@ -14878,7 +14878,7 @@
         <v>2496</v>
       </c>
       <c r="C1313" t="n">
-        <v>101808</v>
+        <v>109080</v>
       </c>
     </row>
     <row r="1314">
@@ -14889,7 +14889,7 @@
         <v>949</v>
       </c>
       <c r="C1314" t="n">
-        <v>62454</v>
+        <v>66915</v>
       </c>
     </row>
     <row r="1315">
@@ -14900,7 +14900,7 @@
         <v>1853</v>
       </c>
       <c r="C1315" t="n">
-        <v>76356</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1316">
@@ -14911,7 +14911,7 @@
         <v>854</v>
       </c>
       <c r="C1316" t="n">
-        <v>70000</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="1317">
@@ -14922,7 +14922,7 @@
         <v>2674</v>
       </c>
       <c r="C1317" t="n">
-        <v>165452</v>
+        <v>177270</v>
       </c>
     </row>
     <row r="1318">
@@ -14933,7 +14933,7 @@
         <v>2803</v>
       </c>
       <c r="C1318" t="n">
-        <v>76356</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1319">
@@ -14944,7 +14944,7 @@
         <v>2599</v>
       </c>
       <c r="C1319" t="n">
-        <v>120904</v>
+        <v>129540</v>
       </c>
     </row>
     <row r="1320">
@@ -14955,7 +14955,7 @@
         <v>783</v>
       </c>
       <c r="C1320" t="n">
-        <v>33082</v>
+        <v>35445</v>
       </c>
     </row>
     <row r="1321">
@@ -14966,7 +14966,7 @@
         <v>27</v>
       </c>
       <c r="C1321" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1322">
@@ -14977,7 +14977,7 @@
         <v>531</v>
       </c>
       <c r="C1322" t="n">
-        <v>222726</v>
+        <v>238635</v>
       </c>
     </row>
     <row r="1323">
@@ -14988,7 +14988,7 @@
         <v>1308</v>
       </c>
       <c r="C1323" t="n">
-        <v>102788</v>
+        <v>110130</v>
       </c>
     </row>
     <row r="1324">
@@ -14999,7 +14999,7 @@
         <v>2792</v>
       </c>
       <c r="C1324" t="n">
-        <v>74130</v>
+        <v>79425</v>
       </c>
     </row>
     <row r="1325">
@@ -15021,7 +15021,7 @@
         <v>2823</v>
       </c>
       <c r="C1326" t="n">
-        <v>59500</v>
+        <v>63750</v>
       </c>
     </row>
     <row r="1327">
@@ -15032,7 +15032,7 @@
         <v>2584</v>
       </c>
       <c r="C1327" t="n">
-        <v>40054</v>
+        <v>42915</v>
       </c>
     </row>
     <row r="1328">
@@ -15043,7 +15043,7 @@
         <v>945</v>
       </c>
       <c r="C1328" t="n">
-        <v>180292</v>
+        <v>193170</v>
       </c>
     </row>
     <row r="1329">
@@ -15054,7 +15054,7 @@
         <v>2660</v>
       </c>
       <c r="C1329" t="n">
-        <v>197260</v>
+        <v>211350</v>
       </c>
     </row>
     <row r="1330">
@@ -15065,7 +15065,7 @@
         <v>1317</v>
       </c>
       <c r="C1330" t="n">
-        <v>190904</v>
+        <v>204540</v>
       </c>
     </row>
     <row r="1331">
@@ -15076,7 +15076,7 @@
         <v>2790</v>
       </c>
       <c r="C1331" t="n">
-        <v>40530</v>
+        <v>43425</v>
       </c>
     </row>
     <row r="1332">
@@ -15087,7 +15087,7 @@
         <v>2711</v>
       </c>
       <c r="C1332" t="n">
-        <v>55165.12</v>
+        <v>59105.48</v>
       </c>
     </row>
     <row r="1333">
@@ -15098,7 +15098,7 @@
         <v>2607</v>
       </c>
       <c r="C1333" t="n">
-        <v>31617.12</v>
+        <v>33875.48</v>
       </c>
     </row>
     <row r="1334">
@@ -15109,7 +15109,7 @@
         <v>2667</v>
       </c>
       <c r="C1334" t="n">
-        <v>29081.84</v>
+        <v>31159.11</v>
       </c>
     </row>
     <row r="1335">
@@ -15120,7 +15120,7 @@
         <v>2706</v>
       </c>
       <c r="C1335" t="n">
-        <v>14020.4</v>
+        <v>15021.85</v>
       </c>
     </row>
     <row r="1336">
@@ -15131,7 +15131,7 @@
         <v>2657</v>
       </c>
       <c r="C1336" t="n">
-        <v>50397.52</v>
+        <v>53997.33</v>
       </c>
     </row>
     <row r="1337">
@@ -15142,7 +15142,7 @@
         <v>1278</v>
       </c>
       <c r="C1337" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1338">
@@ -15153,7 +15153,7 @@
         <v>2745</v>
       </c>
       <c r="C1338" t="n">
-        <v>70000</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="1339">
@@ -15164,7 +15164,7 @@
         <v>2753</v>
       </c>
       <c r="C1339" t="n">
-        <v>47726</v>
+        <v>51135</v>
       </c>
     </row>
     <row r="1340">
@@ -15175,7 +15175,7 @@
         <v>2183</v>
       </c>
       <c r="C1340" t="n">
-        <v>232876</v>
+        <v>249510</v>
       </c>
     </row>
     <row r="1341">
@@ -15186,7 +15186,7 @@
         <v>1340</v>
       </c>
       <c r="C1341" t="n">
-        <v>92260</v>
+        <v>98850</v>
       </c>
     </row>
     <row r="1342">
@@ -15197,7 +15197,7 @@
         <v>2583</v>
       </c>
       <c r="C1342" t="n">
-        <v>26474</v>
+        <v>28365</v>
       </c>
     </row>
     <row r="1343">
@@ -15208,7 +15208,7 @@
         <v>2090</v>
       </c>
       <c r="C1343" t="n">
-        <v>26474</v>
+        <v>28365</v>
       </c>
     </row>
     <row r="1344">
@@ -15219,7 +15219,7 @@
         <v>1277</v>
       </c>
       <c r="C1344" t="n">
-        <v>140000</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="1345">
@@ -15230,7 +15230,7 @@
         <v>1501</v>
       </c>
       <c r="C1345" t="n">
-        <v>60452</v>
+        <v>64770</v>
       </c>
     </row>
     <row r="1346">
@@ -15241,7 +15241,7 @@
         <v>703</v>
       </c>
       <c r="C1346" t="n">
-        <v>159082</v>
+        <v>170445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:01:35
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -11292,7 +11292,7 @@
         <v>947</v>
       </c>
       <c r="C987" t="n">
-        <v>296265</v>
+        <v>316016</v>
       </c>
     </row>
     <row r="988">
@@ -11303,7 +11303,7 @@
         <v>1956</v>
       </c>
       <c r="C988" t="n">
-        <v>172140</v>
+        <v>183616</v>
       </c>
     </row>
     <row r="989">
@@ -11314,7 +11314,7 @@
         <v>2824</v>
       </c>
       <c r="C989" t="n">
-        <v>75000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="990">
@@ -11325,7 +11325,7 @@
         <v>2787</v>
       </c>
       <c r="C990" t="n">
-        <v>88635</v>
+        <v>94544</v>
       </c>
     </row>
     <row r="991">
@@ -11336,7 +11336,7 @@
         <v>2830</v>
       </c>
       <c r="C991" t="n">
-        <v>61350</v>
+        <v>65440</v>
       </c>
     </row>
     <row r="992">
@@ -11347,7 +11347,7 @@
         <v>1254</v>
       </c>
       <c r="C992" t="n">
-        <v>132406.37</v>
+        <v>141233.46</v>
       </c>
     </row>
     <row r="993">
@@ -11358,7 +11358,7 @@
         <v>816</v>
       </c>
       <c r="C993" t="n">
-        <v>182625</v>
+        <v>194800</v>
       </c>
     </row>
     <row r="994">
@@ -11369,7 +11369,7 @@
         <v>2671</v>
       </c>
       <c r="C994" t="n">
-        <v>54540</v>
+        <v>58176</v>
       </c>
     </row>
     <row r="995">
@@ -11380,7 +11380,7 @@
         <v>2705</v>
       </c>
       <c r="C995" t="n">
-        <v>122175</v>
+        <v>130320</v>
       </c>
     </row>
     <row r="996">
@@ -11391,7 +11391,7 @@
         <v>2333</v>
       </c>
       <c r="C996" t="n">
-        <v>105240</v>
+        <v>112256</v>
       </c>
     </row>
     <row r="997">
@@ -11402,7 +11402,7 @@
         <v>2440</v>
       </c>
       <c r="C997" t="n">
-        <v>61350</v>
+        <v>65440</v>
       </c>
     </row>
     <row r="998">
@@ -11413,7 +11413,7 @@
         <v>2448</v>
       </c>
       <c r="C998" t="n">
-        <v>13635</v>
+        <v>14544</v>
       </c>
     </row>
     <row r="999">
@@ -11424,7 +11424,7 @@
         <v>2310</v>
       </c>
       <c r="C999" t="n">
-        <v>46830</v>
+        <v>49952</v>
       </c>
     </row>
     <row r="1000">
@@ -11435,7 +11435,7 @@
         <v>2809</v>
       </c>
       <c r="C1000" t="n">
-        <v>46830</v>
+        <v>49952</v>
       </c>
     </row>
     <row r="1001">
@@ -11446,7 +11446,7 @@
         <v>2548</v>
       </c>
       <c r="C1001" t="n">
-        <v>39900</v>
+        <v>42560</v>
       </c>
     </row>
     <row r="1002">
@@ -11457,7 +11457,7 @@
         <v>451</v>
       </c>
       <c r="C1002" t="n">
-        <v>163635</v>
+        <v>174544</v>
       </c>
     </row>
     <row r="1003">
@@ -11468,7 +11468,7 @@
         <v>933</v>
       </c>
       <c r="C1003" t="n">
-        <v>55560</v>
+        <v>59264</v>
       </c>
     </row>
     <row r="1004">
@@ -11479,7 +11479,7 @@
         <v>2702</v>
       </c>
       <c r="C1004" t="n">
-        <v>55560</v>
+        <v>59264</v>
       </c>
     </row>
     <row r="1005">
@@ -11490,7 +11490,7 @@
         <v>2549</v>
       </c>
       <c r="C1005" t="n">
-        <v>19320</v>
+        <v>20608</v>
       </c>
     </row>
     <row r="1006">
@@ -11501,7 +11501,7 @@
         <v>535</v>
       </c>
       <c r="C1006" t="n">
-        <v>252270</v>
+        <v>269088</v>
       </c>
     </row>
     <row r="1007">
@@ -11512,7 +11512,7 @@
         <v>1117</v>
       </c>
       <c r="C1007" t="n">
-        <v>237195</v>
+        <v>253008</v>
       </c>
     </row>
     <row r="1008">
@@ -11534,7 +11534,7 @@
         <v>530</v>
       </c>
       <c r="C1009" t="n">
-        <v>166410</v>
+        <v>177504</v>
       </c>
     </row>
     <row r="1010">
@@ -11545,7 +11545,7 @@
         <v>358</v>
       </c>
       <c r="C1010" t="n">
-        <v>231810</v>
+        <v>247264</v>
       </c>
     </row>
     <row r="1011">
@@ -11556,7 +11556,7 @@
         <v>2498</v>
       </c>
       <c r="C1011" t="n">
-        <v>37860</v>
+        <v>40384</v>
       </c>
     </row>
     <row r="1012">
@@ -11567,7 +11567,7 @@
         <v>2381</v>
       </c>
       <c r="C1012" t="n">
-        <v>54090</v>
+        <v>57696</v>
       </c>
     </row>
     <row r="1013">
@@ -11578,7 +11578,7 @@
         <v>2695</v>
       </c>
       <c r="C1013" t="n">
-        <v>32535</v>
+        <v>34704</v>
       </c>
     </row>
     <row r="1014">
@@ -11589,7 +11589,7 @@
         <v>2744</v>
       </c>
       <c r="C1014" t="n">
-        <v>40909.11</v>
+        <v>43636.38</v>
       </c>
     </row>
     <row r="1015">
@@ -11600,7 +11600,7 @@
         <v>2750</v>
       </c>
       <c r="C1015" t="n">
-        <v>40905</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1016">
@@ -11611,7 +11611,7 @@
         <v>2131</v>
       </c>
       <c r="C1016" t="n">
-        <v>81810</v>
+        <v>87264</v>
       </c>
     </row>
     <row r="1017">
@@ -11622,7 +11622,7 @@
         <v>818</v>
       </c>
       <c r="C1017" t="n">
-        <v>272715</v>
+        <v>290896</v>
       </c>
     </row>
     <row r="1018">
@@ -11633,7 +11633,7 @@
         <v>2566</v>
       </c>
       <c r="C1018" t="n">
-        <v>54540</v>
+        <v>58176</v>
       </c>
     </row>
     <row r="1019">
@@ -11644,7 +11644,7 @@
         <v>132</v>
       </c>
       <c r="C1019" t="n">
-        <v>511350</v>
+        <v>545440</v>
       </c>
     </row>
     <row r="1020">
@@ -11655,7 +11655,7 @@
         <v>2431</v>
       </c>
       <c r="C1020" t="n">
-        <v>125445</v>
+        <v>133808</v>
       </c>
     </row>
     <row r="1021">
@@ -11666,7 +11666,7 @@
         <v>2249</v>
       </c>
       <c r="C1021" t="n">
-        <v>133170</v>
+        <v>142048</v>
       </c>
     </row>
     <row r="1022">
@@ -11677,7 +11677,7 @@
         <v>1585</v>
       </c>
       <c r="C1022" t="n">
-        <v>112530</v>
+        <v>120032</v>
       </c>
     </row>
     <row r="1023">
@@ -11688,7 +11688,7 @@
         <v>2325</v>
       </c>
       <c r="C1023" t="n">
-        <v>108780</v>
+        <v>116032</v>
       </c>
     </row>
     <row r="1024">
@@ -11699,7 +11699,7 @@
         <v>2190</v>
       </c>
       <c r="C1024" t="n">
-        <v>153405</v>
+        <v>163632</v>
       </c>
     </row>
     <row r="1025">
@@ -11710,7 +11710,7 @@
         <v>1466</v>
       </c>
       <c r="C1025" t="n">
-        <v>276135</v>
+        <v>294544</v>
       </c>
     </row>
     <row r="1026">
@@ -11721,7 +11721,7 @@
         <v>2659</v>
       </c>
       <c r="C1026" t="n">
-        <v>83865</v>
+        <v>89456</v>
       </c>
     </row>
     <row r="1027">
@@ -11732,7 +11732,7 @@
         <v>634</v>
       </c>
       <c r="C1027" t="n">
-        <v>375000</v>
+        <v>400000</v>
       </c>
     </row>
     <row r="1028">
@@ -11743,7 +11743,7 @@
         <v>2804</v>
       </c>
       <c r="C1028" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1029">
@@ -11754,7 +11754,7 @@
         <v>2375</v>
       </c>
       <c r="C1029" t="n">
-        <v>225000</v>
+        <v>240000</v>
       </c>
     </row>
     <row r="1030">
@@ -11765,7 +11765,7 @@
         <v>2601</v>
       </c>
       <c r="C1030" t="n">
-        <v>187500</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="1031">
@@ -11776,7 +11776,7 @@
         <v>952</v>
       </c>
       <c r="C1031" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1032">
@@ -11787,7 +11787,7 @@
         <v>571</v>
       </c>
       <c r="C1032" t="n">
-        <v>433965</v>
+        <v>462896</v>
       </c>
     </row>
     <row r="1033">
@@ -11798,7 +11798,7 @@
         <v>2697</v>
       </c>
       <c r="C1033" t="n">
-        <v>132225</v>
+        <v>141040</v>
       </c>
     </row>
     <row r="1034">
@@ -11809,7 +11809,7 @@
         <v>2678</v>
       </c>
       <c r="C1034" t="n">
-        <v>228765</v>
+        <v>244016</v>
       </c>
     </row>
     <row r="1035">
@@ -11820,7 +11820,7 @@
         <v>2768</v>
       </c>
       <c r="C1035" t="n">
-        <v>239415</v>
+        <v>255376</v>
       </c>
     </row>
     <row r="1036">
@@ -11831,7 +11831,7 @@
         <v>2359</v>
       </c>
       <c r="C1036" t="n">
-        <v>72615</v>
+        <v>77456</v>
       </c>
     </row>
     <row r="1037">
@@ -11842,7 +11842,7 @@
         <v>353</v>
       </c>
       <c r="C1037" t="n">
-        <v>235890</v>
+        <v>251616</v>
       </c>
     </row>
     <row r="1038">
@@ -11853,7 +11853,7 @@
         <v>2026</v>
       </c>
       <c r="C1038" t="n">
-        <v>195450</v>
+        <v>208480</v>
       </c>
     </row>
     <row r="1039">
@@ -11875,7 +11875,7 @@
         <v>2345</v>
       </c>
       <c r="C1040" t="n">
-        <v>42915</v>
+        <v>45776</v>
       </c>
     </row>
     <row r="1041">
@@ -11886,7 +11886,7 @@
         <v>2789</v>
       </c>
       <c r="C1041" t="n">
-        <v>115905</v>
+        <v>123632</v>
       </c>
     </row>
     <row r="1042">
@@ -11897,7 +11897,7 @@
         <v>569</v>
       </c>
       <c r="C1042" t="n">
-        <v>1952670</v>
+        <v>2082848</v>
       </c>
     </row>
     <row r="1043">
@@ -11908,7 +11908,7 @@
         <v>2822</v>
       </c>
       <c r="C1043" t="n">
-        <v>92040</v>
+        <v>98176</v>
       </c>
     </row>
     <row r="1044">
@@ -11919,7 +11919,7 @@
         <v>2728</v>
       </c>
       <c r="C1044" t="n">
-        <v>6810</v>
+        <v>7264</v>
       </c>
     </row>
     <row r="1045">
@@ -11930,7 +11930,7 @@
         <v>2488</v>
       </c>
       <c r="C1045" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1046">
@@ -11941,7 +11941,7 @@
         <v>2791</v>
       </c>
       <c r="C1046" t="n">
-        <v>67288.7</v>
+        <v>71774.60000000001</v>
       </c>
     </row>
     <row r="1047">
@@ -11952,7 +11952,7 @@
         <v>2577</v>
       </c>
       <c r="C1047" t="n">
-        <v>60797.83</v>
+        <v>64851.01</v>
       </c>
     </row>
     <row r="1048">
@@ -11963,7 +11963,7 @@
         <v>2069</v>
       </c>
       <c r="C1048" t="n">
-        <v>122715</v>
+        <v>130896</v>
       </c>
     </row>
     <row r="1049">
@@ -11974,7 +11974,7 @@
         <v>2082</v>
       </c>
       <c r="C1049" t="n">
-        <v>113565</v>
+        <v>121136</v>
       </c>
     </row>
     <row r="1050">
@@ -11985,7 +11985,7 @@
         <v>781</v>
       </c>
       <c r="C1050" t="n">
-        <v>88635</v>
+        <v>94544</v>
       </c>
     </row>
     <row r="1051">
@@ -11996,7 +11996,7 @@
         <v>744</v>
       </c>
       <c r="C1051" t="n">
-        <v>28365</v>
+        <v>30256</v>
       </c>
     </row>
     <row r="1052">
@@ -12007,7 +12007,7 @@
         <v>2223</v>
       </c>
       <c r="C1052" t="n">
-        <v>89955</v>
+        <v>95952</v>
       </c>
     </row>
     <row r="1053">
@@ -12018,7 +12018,7 @@
         <v>2452</v>
       </c>
       <c r="C1053" t="n">
-        <v>47715</v>
+        <v>50896</v>
       </c>
     </row>
     <row r="1054">
@@ -12029,7 +12029,7 @@
         <v>970</v>
       </c>
       <c r="C1054" t="n">
-        <v>46830</v>
+        <v>49952</v>
       </c>
     </row>
     <row r="1055">
@@ -12040,7 +12040,7 @@
         <v>2550</v>
       </c>
       <c r="C1055" t="n">
-        <v>41580</v>
+        <v>44352</v>
       </c>
     </row>
     <row r="1056">
@@ -12051,7 +12051,7 @@
         <v>768</v>
       </c>
       <c r="C1056" t="n">
-        <v>88635</v>
+        <v>94544</v>
       </c>
     </row>
     <row r="1057">
@@ -12062,7 +12062,7 @@
         <v>1075</v>
       </c>
       <c r="C1057" t="n">
-        <v>308850</v>
+        <v>329440</v>
       </c>
     </row>
     <row r="1058">
@@ -12073,7 +12073,7 @@
         <v>664</v>
       </c>
       <c r="C1058" t="n">
-        <v>176580</v>
+        <v>188352</v>
       </c>
     </row>
     <row r="1059">
@@ -12084,7 +12084,7 @@
         <v>2555</v>
       </c>
       <c r="C1059" t="n">
-        <v>28305</v>
+        <v>30192</v>
       </c>
     </row>
     <row r="1060">
@@ -12095,7 +12095,7 @@
         <v>2627</v>
       </c>
       <c r="C1060" t="n">
-        <v>16620</v>
+        <v>17728</v>
       </c>
     </row>
     <row r="1061">
@@ -12106,7 +12106,7 @@
         <v>2557</v>
       </c>
       <c r="C1061" t="n">
-        <v>17580</v>
+        <v>18752</v>
       </c>
     </row>
     <row r="1062">
@@ -12117,7 +12117,7 @@
         <v>2551</v>
       </c>
       <c r="C1062" t="n">
-        <v>13965</v>
+        <v>14896</v>
       </c>
     </row>
     <row r="1063">
@@ -12128,7 +12128,7 @@
         <v>2463</v>
       </c>
       <c r="C1063" t="n">
-        <v>218325</v>
+        <v>232880</v>
       </c>
     </row>
     <row r="1064">
@@ -12139,7 +12139,7 @@
         <v>2279</v>
       </c>
       <c r="C1064" t="n">
-        <v>164715</v>
+        <v>175696</v>
       </c>
     </row>
     <row r="1065">
@@ -12150,7 +12150,7 @@
         <v>631</v>
       </c>
       <c r="C1065" t="n">
-        <v>238635</v>
+        <v>254544</v>
       </c>
     </row>
     <row r="1066">
@@ -12161,7 +12161,7 @@
         <v>2251</v>
       </c>
       <c r="C1066" t="n">
-        <v>146130</v>
+        <v>155872</v>
       </c>
     </row>
     <row r="1067">
@@ -12172,7 +12172,7 @@
         <v>1653</v>
       </c>
       <c r="C1067" t="n">
-        <v>221580</v>
+        <v>236352</v>
       </c>
     </row>
     <row r="1068">
@@ -12183,7 +12183,7 @@
         <v>1293</v>
       </c>
       <c r="C1068" t="n">
-        <v>282945</v>
+        <v>301808</v>
       </c>
     </row>
     <row r="1069">
@@ -12194,7 +12194,7 @@
         <v>360</v>
       </c>
       <c r="C1069" t="n">
-        <v>340905</v>
+        <v>363632</v>
       </c>
     </row>
     <row r="1070">
@@ -12205,7 +12205,7 @@
         <v>1063</v>
       </c>
       <c r="C1070" t="n">
-        <v>247875</v>
+        <v>264400</v>
       </c>
     </row>
     <row r="1071">
@@ -12216,7 +12216,7 @@
         <v>2273</v>
       </c>
       <c r="C1071" t="n">
-        <v>144600</v>
+        <v>154240</v>
       </c>
     </row>
     <row r="1072">
@@ -12227,7 +12227,7 @@
         <v>2757</v>
       </c>
       <c r="C1072" t="n">
-        <v>47727.33</v>
+        <v>50909.14</v>
       </c>
     </row>
     <row r="1073">
@@ -12238,7 +12238,7 @@
         <v>2795</v>
       </c>
       <c r="C1073" t="n">
-        <v>40909.11</v>
+        <v>43636.38</v>
       </c>
     </row>
     <row r="1074">
@@ -12249,7 +12249,7 @@
         <v>2722</v>
       </c>
       <c r="C1074" t="n">
-        <v>40905</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1075">
@@ -12260,7 +12260,7 @@
         <v>2718</v>
       </c>
       <c r="C1075" t="n">
-        <v>54540</v>
+        <v>58176</v>
       </c>
     </row>
     <row r="1076">
@@ -12271,7 +12271,7 @@
         <v>595</v>
       </c>
       <c r="C1076" t="n">
-        <v>375000</v>
+        <v>400000</v>
       </c>
     </row>
     <row r="1077">
@@ -12282,7 +12282,7 @@
         <v>890</v>
       </c>
       <c r="C1077" t="n">
-        <v>477270</v>
+        <v>509088</v>
       </c>
     </row>
     <row r="1078">
@@ -12293,7 +12293,7 @@
         <v>2652</v>
       </c>
       <c r="C1078" t="n">
-        <v>88635</v>
+        <v>94544</v>
       </c>
     </row>
     <row r="1079">
@@ -12304,7 +12304,7 @@
         <v>2714</v>
       </c>
       <c r="C1079" t="n">
-        <v>245445</v>
+        <v>261808</v>
       </c>
     </row>
     <row r="1080">
@@ -12315,7 +12315,7 @@
         <v>1869</v>
       </c>
       <c r="C1080" t="n">
-        <v>156810</v>
+        <v>167264</v>
       </c>
     </row>
     <row r="1081">
@@ -12326,7 +12326,7 @@
         <v>400</v>
       </c>
       <c r="C1081" t="n">
-        <v>129540</v>
+        <v>138176</v>
       </c>
     </row>
     <row r="1082">
@@ -12337,7 +12337,7 @@
         <v>1907</v>
       </c>
       <c r="C1082" t="n">
-        <v>252945</v>
+        <v>269808</v>
       </c>
     </row>
     <row r="1083">
@@ -12348,7 +12348,7 @@
         <v>1996</v>
       </c>
       <c r="C1083" t="n">
-        <v>159885</v>
+        <v>170544</v>
       </c>
     </row>
     <row r="1084">
@@ -12359,7 +12359,7 @@
         <v>1890</v>
       </c>
       <c r="C1084" t="n">
-        <v>215551.86</v>
+        <v>229921.97</v>
       </c>
     </row>
     <row r="1085">
@@ -12370,7 +12370,7 @@
         <v>2114</v>
       </c>
       <c r="C1085" t="n">
-        <v>125250</v>
+        <v>133600</v>
       </c>
     </row>
     <row r="1086">
@@ -12381,7 +12381,7 @@
         <v>2330</v>
       </c>
       <c r="C1086" t="n">
-        <v>183255</v>
+        <v>195472</v>
       </c>
     </row>
     <row r="1087">
@@ -12425,7 +12425,7 @@
         <v>931</v>
       </c>
       <c r="C1090" t="n">
-        <v>64380</v>
+        <v>68672</v>
       </c>
     </row>
     <row r="1091">
@@ -12436,7 +12436,7 @@
         <v>951</v>
       </c>
       <c r="C1091" t="n">
-        <v>78405</v>
+        <v>83632</v>
       </c>
     </row>
     <row r="1092">
@@ -12447,7 +12447,7 @@
         <v>2449</v>
       </c>
       <c r="C1092" t="n">
-        <v>27270</v>
+        <v>29088</v>
       </c>
     </row>
     <row r="1093">
@@ -12458,7 +12458,7 @@
         <v>610</v>
       </c>
       <c r="C1093" t="n">
-        <v>555675</v>
+        <v>592720</v>
       </c>
     </row>
     <row r="1094">
@@ -12469,7 +12469,7 @@
         <v>2761</v>
       </c>
       <c r="C1094" t="n">
-        <v>55560</v>
+        <v>59264</v>
       </c>
     </row>
     <row r="1095">
@@ -12480,7 +12480,7 @@
         <v>483</v>
       </c>
       <c r="C1095" t="n">
-        <v>302040</v>
+        <v>322176</v>
       </c>
     </row>
     <row r="1096">
@@ -12491,7 +12491,7 @@
         <v>2015</v>
       </c>
       <c r="C1096" t="n">
-        <v>252270</v>
+        <v>269088</v>
       </c>
     </row>
     <row r="1097">
@@ -12502,7 +12502,7 @@
         <v>1478</v>
       </c>
       <c r="C1097" t="n">
-        <v>368970</v>
+        <v>393568</v>
       </c>
     </row>
     <row r="1098">
@@ -12513,7 +12513,7 @@
         <v>424</v>
       </c>
       <c r="C1098" t="n">
-        <v>164715</v>
+        <v>175696</v>
       </c>
     </row>
     <row r="1099">
@@ -12535,7 +12535,7 @@
         <v>477</v>
       </c>
       <c r="C1100" t="n">
-        <v>176355</v>
+        <v>188112</v>
       </c>
     </row>
     <row r="1101">
@@ -12546,7 +12546,7 @@
         <v>1810</v>
       </c>
       <c r="C1101" t="n">
-        <v>27315</v>
+        <v>29136</v>
       </c>
     </row>
     <row r="1102">
@@ -12557,7 +12557,7 @@
         <v>2826</v>
       </c>
       <c r="C1102" t="n">
-        <v>47727.33</v>
+        <v>50909.14</v>
       </c>
     </row>
     <row r="1103">
@@ -12568,7 +12568,7 @@
         <v>2561</v>
       </c>
       <c r="C1103" t="n">
-        <v>10020</v>
+        <v>10688</v>
       </c>
     </row>
     <row r="1104">
@@ -12579,7 +12579,7 @@
         <v>2653</v>
       </c>
       <c r="C1104" t="n">
-        <v>40909.11</v>
+        <v>43636.38</v>
       </c>
     </row>
     <row r="1105">
@@ -12590,7 +12590,7 @@
         <v>2829</v>
       </c>
       <c r="C1105" t="n">
-        <v>40909.11</v>
+        <v>43636.38</v>
       </c>
     </row>
     <row r="1106">
@@ -12601,7 +12601,7 @@
         <v>2643</v>
       </c>
       <c r="C1106" t="n">
-        <v>20130</v>
+        <v>21472</v>
       </c>
     </row>
     <row r="1107">
@@ -12612,7 +12612,7 @@
         <v>2794</v>
       </c>
       <c r="C1107" t="n">
-        <v>61350</v>
+        <v>65440</v>
       </c>
     </row>
     <row r="1108">
@@ -12623,7 +12623,7 @@
         <v>2655</v>
       </c>
       <c r="C1108" t="n">
-        <v>75000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="1109">
@@ -12634,7 +12634,7 @@
         <v>1456</v>
       </c>
       <c r="C1109" t="n">
-        <v>525195</v>
+        <v>560208</v>
       </c>
     </row>
     <row r="1110">
@@ -12645,7 +12645,7 @@
         <v>2606</v>
       </c>
       <c r="C1110" t="n">
-        <v>161310</v>
+        <v>172064</v>
       </c>
     </row>
     <row r="1111">
@@ -12656,7 +12656,7 @@
         <v>1142</v>
       </c>
       <c r="C1111" t="n">
-        <v>292530</v>
+        <v>312032</v>
       </c>
     </row>
     <row r="1112">
@@ -12667,7 +12667,7 @@
         <v>1450</v>
       </c>
       <c r="C1112" t="n">
-        <v>185835</v>
+        <v>198224</v>
       </c>
     </row>
     <row r="1113">
@@ -12678,7 +12678,7 @@
         <v>2133</v>
       </c>
       <c r="C1113" t="n">
-        <v>433965</v>
+        <v>462896</v>
       </c>
     </row>
     <row r="1114">
@@ -12689,7 +12689,7 @@
         <v>522</v>
       </c>
       <c r="C1114" t="n">
-        <v>132945</v>
+        <v>141808</v>
       </c>
     </row>
     <row r="1115">
@@ -12700,7 +12700,7 @@
         <v>2696</v>
       </c>
       <c r="C1115" t="n">
-        <v>179400</v>
+        <v>191360</v>
       </c>
     </row>
     <row r="1116">
@@ -12722,7 +12722,7 @@
         <v>2692</v>
       </c>
       <c r="C1117" t="n">
-        <v>51135</v>
+        <v>54544</v>
       </c>
     </row>
     <row r="1118">
@@ -12733,7 +12733,7 @@
         <v>2691</v>
       </c>
       <c r="C1118" t="n">
-        <v>92040</v>
+        <v>98176</v>
       </c>
     </row>
     <row r="1119">
@@ -12744,7 +12744,7 @@
         <v>1632</v>
       </c>
       <c r="C1119" t="n">
-        <v>170445</v>
+        <v>181808</v>
       </c>
     </row>
     <row r="1120">
@@ -12755,7 +12755,7 @@
         <v>2641</v>
       </c>
       <c r="C1120" t="n">
-        <v>54540</v>
+        <v>58176</v>
       </c>
     </row>
     <row r="1121">
@@ -12766,7 +12766,7 @@
         <v>2197</v>
       </c>
       <c r="C1121" t="n">
-        <v>136350</v>
+        <v>145440</v>
       </c>
     </row>
     <row r="1122">
@@ -12777,7 +12777,7 @@
         <v>609</v>
       </c>
       <c r="C1122" t="n">
-        <v>150000</v>
+        <v>160000</v>
       </c>
     </row>
     <row r="1123">
@@ -12788,7 +12788,7 @@
         <v>1380</v>
       </c>
       <c r="C1123" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1124">
@@ -12799,7 +12799,7 @@
         <v>104</v>
       </c>
       <c r="C1124" t="n">
-        <v>204540</v>
+        <v>218176</v>
       </c>
     </row>
     <row r="1125">
@@ -12810,7 +12810,7 @@
         <v>2621</v>
       </c>
       <c r="C1125" t="n">
-        <v>47715</v>
+        <v>50896</v>
       </c>
     </row>
     <row r="1126">
@@ -12821,7 +12821,7 @@
         <v>2786</v>
       </c>
       <c r="C1126" t="n">
-        <v>47715</v>
+        <v>50896</v>
       </c>
     </row>
     <row r="1127">
@@ -12832,7 +12832,7 @@
         <v>2784</v>
       </c>
       <c r="C1127" t="n">
-        <v>28365</v>
+        <v>30256</v>
       </c>
     </row>
     <row r="1128">
@@ -12843,7 +12843,7 @@
         <v>2586</v>
       </c>
       <c r="C1128" t="n">
-        <v>28365</v>
+        <v>30256</v>
       </c>
     </row>
     <row r="1129">
@@ -12854,7 +12854,7 @@
         <v>2145</v>
       </c>
       <c r="C1129" t="n">
-        <v>88260</v>
+        <v>94144</v>
       </c>
     </row>
     <row r="1130">
@@ -12865,7 +12865,7 @@
         <v>2574</v>
       </c>
       <c r="C1130" t="n">
-        <v>88260</v>
+        <v>94144</v>
       </c>
     </row>
     <row r="1131">
@@ -12876,7 +12876,7 @@
         <v>2492</v>
       </c>
       <c r="C1131" t="n">
-        <v>96750</v>
+        <v>103200</v>
       </c>
     </row>
     <row r="1132">
@@ -12887,7 +12887,7 @@
         <v>629</v>
       </c>
       <c r="C1132" t="n">
-        <v>301350</v>
+        <v>321440</v>
       </c>
     </row>
     <row r="1133">
@@ -12898,7 +12898,7 @@
         <v>966</v>
       </c>
       <c r="C1133" t="n">
-        <v>55560</v>
+        <v>59264</v>
       </c>
     </row>
     <row r="1134">
@@ -12909,7 +12909,7 @@
         <v>2721</v>
       </c>
       <c r="C1134" t="n">
-        <v>55560</v>
+        <v>59264</v>
       </c>
     </row>
     <row r="1135">
@@ -12920,7 +12920,7 @@
         <v>2554</v>
       </c>
       <c r="C1135" t="n">
-        <v>16740</v>
+        <v>17856</v>
       </c>
     </row>
     <row r="1136">
@@ -12931,7 +12931,7 @@
         <v>2556</v>
       </c>
       <c r="C1136" t="n">
-        <v>24615</v>
+        <v>26256</v>
       </c>
     </row>
     <row r="1137">
@@ -12942,7 +12942,7 @@
         <v>2546</v>
       </c>
       <c r="C1137" t="n">
-        <v>16260</v>
+        <v>17344</v>
       </c>
     </row>
     <row r="1138">
@@ -12953,7 +12953,7 @@
         <v>42</v>
       </c>
       <c r="C1138" t="n">
-        <v>1288635</v>
+        <v>1374544</v>
       </c>
     </row>
     <row r="1139">
@@ -12964,7 +12964,7 @@
         <v>953</v>
       </c>
       <c r="C1139" t="n">
-        <v>465450</v>
+        <v>496480</v>
       </c>
     </row>
     <row r="1140">
@@ -12972,10 +12972,10 @@
         <v>46266</v>
       </c>
       <c r="B1140" t="n">
-        <v>675</v>
+        <v>1137</v>
       </c>
       <c r="C1140" t="n">
-        <v>136350</v>
+        <v>465440</v>
       </c>
     </row>
     <row r="1141">
@@ -12983,10 +12983,10 @@
         <v>46266</v>
       </c>
       <c r="B1141" t="n">
-        <v>619</v>
+        <v>675</v>
       </c>
       <c r="C1141" t="n">
-        <v>210840</v>
+        <v>145440</v>
       </c>
     </row>
     <row r="1142">
@@ -12994,10 +12994,10 @@
         <v>46266</v>
       </c>
       <c r="B1142" t="n">
-        <v>1299</v>
+        <v>619</v>
       </c>
       <c r="C1142" t="n">
-        <v>354780</v>
+        <v>224896</v>
       </c>
     </row>
     <row r="1143">
@@ -13005,10 +13005,10 @@
         <v>46266</v>
       </c>
       <c r="B1143" t="n">
-        <v>1064</v>
+        <v>1299</v>
       </c>
       <c r="C1143" t="n">
-        <v>408660</v>
+        <v>378432</v>
       </c>
     </row>
     <row r="1144">
@@ -13016,10 +13016,10 @@
         <v>46266</v>
       </c>
       <c r="B1144" t="n">
-        <v>2308</v>
+        <v>1064</v>
       </c>
       <c r="C1144" t="n">
-        <v>139770</v>
+        <v>435904</v>
       </c>
     </row>
     <row r="1145">
@@ -13027,10 +13027,10 @@
         <v>46266</v>
       </c>
       <c r="B1145" t="n">
-        <v>1137</v>
+        <v>2308</v>
       </c>
       <c r="C1145" t="n">
-        <v>436350</v>
+        <v>149088</v>
       </c>
     </row>
     <row r="1146">
@@ -13041,7 +13041,7 @@
         <v>2747</v>
       </c>
       <c r="C1146" t="n">
-        <v>40909.11</v>
+        <v>43636.38</v>
       </c>
     </row>
     <row r="1147">
@@ -13052,7 +13052,7 @@
         <v>2819</v>
       </c>
       <c r="C1147" t="n">
-        <v>40909.11</v>
+        <v>43636.38</v>
       </c>
     </row>
     <row r="1148">
@@ -13063,7 +13063,7 @@
         <v>1259</v>
       </c>
       <c r="C1148" t="n">
-        <v>68181.85000000001</v>
+        <v>72727.3</v>
       </c>
     </row>
     <row r="1149">
@@ -13074,7 +13074,7 @@
         <v>2544</v>
       </c>
       <c r="C1149" t="n">
-        <v>54540</v>
+        <v>58176</v>
       </c>
     </row>
     <row r="1150">
@@ -13085,7 +13085,7 @@
         <v>2261</v>
       </c>
       <c r="C1150" t="n">
-        <v>102270</v>
+        <v>109088</v>
       </c>
     </row>
     <row r="1151">
@@ -13096,7 +13096,7 @@
         <v>2729</v>
       </c>
       <c r="C1151" t="n">
-        <v>54540</v>
+        <v>58176</v>
       </c>
     </row>
     <row r="1152">
@@ -13107,7 +13107,7 @@
         <v>2649</v>
       </c>
       <c r="C1152" t="n">
-        <v>20130</v>
+        <v>21472</v>
       </c>
     </row>
     <row r="1153">
@@ -13118,7 +13118,7 @@
         <v>2494</v>
       </c>
       <c r="C1153" t="n">
-        <v>88635</v>
+        <v>94544</v>
       </c>
     </row>
     <row r="1154">
@@ -13129,7 +13129,7 @@
         <v>1384</v>
       </c>
       <c r="C1154" t="n">
-        <v>306810</v>
+        <v>327264</v>
       </c>
     </row>
     <row r="1155">
@@ -13151,7 +13151,7 @@
         <v>2802</v>
       </c>
       <c r="C1156" t="n">
-        <v>48285</v>
+        <v>51504</v>
       </c>
     </row>
     <row r="1157">
@@ -13162,7 +13162,7 @@
         <v>2726</v>
       </c>
       <c r="C1157" t="n">
-        <v>102270</v>
+        <v>109088</v>
       </c>
     </row>
     <row r="1158">
@@ -13173,7 +13173,7 @@
         <v>2820</v>
       </c>
       <c r="C1158" t="n">
-        <v>122715</v>
+        <v>130896</v>
       </c>
     </row>
     <row r="1159">
@@ -13184,7 +13184,7 @@
         <v>1007</v>
       </c>
       <c r="C1159" t="n">
-        <v>129540</v>
+        <v>138176</v>
       </c>
     </row>
     <row r="1160">
@@ -13195,7 +13195,7 @@
         <v>20</v>
       </c>
       <c r="C1160" t="n">
-        <v>262500</v>
+        <v>280000</v>
       </c>
     </row>
     <row r="1161">
@@ -13206,7 +13206,7 @@
         <v>1372</v>
       </c>
       <c r="C1161" t="n">
-        <v>197715</v>
+        <v>210896</v>
       </c>
     </row>
     <row r="1162">
@@ -13217,7 +13217,7 @@
         <v>2735</v>
       </c>
       <c r="C1162" t="n">
-        <v>81810</v>
+        <v>87264</v>
       </c>
     </row>
     <row r="1163">
@@ -13228,7 +13228,7 @@
         <v>2811</v>
       </c>
       <c r="C1163" t="n">
-        <v>28365</v>
+        <v>30256</v>
       </c>
     </row>
     <row r="1164">
@@ -13239,7 +13239,7 @@
         <v>1871</v>
       </c>
       <c r="C1164" t="n">
-        <v>120510</v>
+        <v>128544</v>
       </c>
     </row>
     <row r="1165">
@@ -13250,7 +13250,7 @@
         <v>2541</v>
       </c>
       <c r="C1165" t="n">
-        <v>144270</v>
+        <v>153888</v>
       </c>
     </row>
     <row r="1166">
@@ -13261,7 +13261,7 @@
         <v>2362</v>
       </c>
       <c r="C1166" t="n">
-        <v>51135</v>
+        <v>54544</v>
       </c>
     </row>
     <row r="1167">
@@ -13272,7 +13272,7 @@
         <v>1324</v>
       </c>
       <c r="C1167" t="n">
-        <v>190905</v>
+        <v>203632</v>
       </c>
     </row>
     <row r="1168">
@@ -13283,7 +13283,7 @@
         <v>2323</v>
       </c>
       <c r="C1168" t="n">
-        <v>46830</v>
+        <v>49952</v>
       </c>
     </row>
     <row r="1169">
@@ -13294,7 +13294,7 @@
         <v>2647</v>
       </c>
       <c r="C1169" t="n">
-        <v>96750</v>
+        <v>103200</v>
       </c>
     </row>
     <row r="1170">
@@ -13305,7 +13305,7 @@
         <v>559</v>
       </c>
       <c r="C1170" t="n">
-        <v>156435</v>
+        <v>166864</v>
       </c>
     </row>
     <row r="1171">
@@ -13316,7 +13316,7 @@
         <v>2762</v>
       </c>
       <c r="C1171" t="n">
-        <v>55560</v>
+        <v>59264</v>
       </c>
     </row>
     <row r="1172">
@@ -13327,7 +13327,7 @@
         <v>2501</v>
       </c>
       <c r="C1172" t="n">
-        <v>55560</v>
+        <v>59264</v>
       </c>
     </row>
     <row r="1173">
@@ -13338,7 +13338,7 @@
         <v>2562</v>
       </c>
       <c r="C1173" t="n">
-        <v>10785</v>
+        <v>11504</v>
       </c>
     </row>
     <row r="1174">
@@ -13349,7 +13349,7 @@
         <v>429</v>
       </c>
       <c r="C1174" t="n">
-        <v>265905</v>
+        <v>283632</v>
       </c>
     </row>
     <row r="1175">
@@ -13360,7 +13360,7 @@
         <v>58</v>
       </c>
       <c r="C1175" t="n">
-        <v>184485</v>
+        <v>196784</v>
       </c>
     </row>
     <row r="1176">
@@ -13371,7 +13371,7 @@
         <v>2245</v>
       </c>
       <c r="C1176" t="n">
-        <v>164715</v>
+        <v>175696</v>
       </c>
     </row>
     <row r="1177">
@@ -13382,7 +13382,7 @@
         <v>285</v>
       </c>
       <c r="C1177" t="n">
-        <v>368970</v>
+        <v>393568</v>
       </c>
     </row>
     <row r="1178">
@@ -13404,7 +13404,7 @@
         <v>363</v>
       </c>
       <c r="C1179" t="n">
-        <v>204540</v>
+        <v>218176</v>
       </c>
     </row>
     <row r="1180">
@@ -13415,7 +13415,7 @@
         <v>2651</v>
       </c>
       <c r="C1180" t="n">
-        <v>115305</v>
+        <v>122992</v>
       </c>
     </row>
     <row r="1181">
@@ -13426,7 +13426,7 @@
         <v>2142</v>
       </c>
       <c r="C1181" t="n">
-        <v>36390</v>
+        <v>38816</v>
       </c>
     </row>
     <row r="1182">
@@ -13437,7 +13437,7 @@
         <v>2258</v>
       </c>
       <c r="C1182" t="n">
-        <v>54545.48</v>
+        <v>58181.84</v>
       </c>
     </row>
     <row r="1183">
@@ -13448,7 +13448,7 @@
         <v>2772</v>
       </c>
       <c r="C1183" t="n">
-        <v>40909.11</v>
+        <v>43636.38</v>
       </c>
     </row>
     <row r="1184">
@@ -13459,7 +13459,7 @@
         <v>2346</v>
       </c>
       <c r="C1184" t="n">
-        <v>75000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="1185">
@@ -13470,7 +13470,7 @@
         <v>2442</v>
       </c>
       <c r="C1185" t="n">
-        <v>54540</v>
+        <v>58176</v>
       </c>
     </row>
     <row r="1186">
@@ -13481,7 +13481,7 @@
         <v>772</v>
       </c>
       <c r="C1186" t="n">
-        <v>225000</v>
+        <v>240000</v>
       </c>
     </row>
     <row r="1187">
@@ -13492,7 +13492,7 @@
         <v>2684</v>
       </c>
       <c r="C1187" t="n">
-        <v>64770</v>
+        <v>69088</v>
       </c>
     </row>
     <row r="1188">
@@ -13503,7 +13503,7 @@
         <v>2765</v>
       </c>
       <c r="C1188" t="n">
-        <v>61350</v>
+        <v>65440</v>
       </c>
     </row>
     <row r="1189">
@@ -13514,7 +13514,7 @@
         <v>2567</v>
       </c>
       <c r="C1189" t="n">
-        <v>112530</v>
+        <v>120032</v>
       </c>
     </row>
     <row r="1190">
@@ -13525,7 +13525,7 @@
         <v>2178</v>
       </c>
       <c r="C1190" t="n">
-        <v>190905</v>
+        <v>203632</v>
       </c>
     </row>
     <row r="1191">
@@ -13536,7 +13536,7 @@
         <v>2827</v>
       </c>
       <c r="C1191" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1192">
@@ -13547,7 +13547,7 @@
         <v>2510</v>
       </c>
       <c r="C1192" t="n">
-        <v>378570</v>
+        <v>403808</v>
       </c>
     </row>
     <row r="1193">
@@ -13558,7 +13558,7 @@
         <v>2392</v>
       </c>
       <c r="C1193" t="n">
-        <v>113565</v>
+        <v>121136</v>
       </c>
     </row>
     <row r="1194">
@@ -13569,7 +13569,7 @@
         <v>415</v>
       </c>
       <c r="C1194" t="n">
-        <v>388290</v>
+        <v>414176</v>
       </c>
     </row>
     <row r="1195">
@@ -13580,7 +13580,7 @@
         <v>2107</v>
       </c>
       <c r="C1195" t="n">
-        <v>200505</v>
+        <v>213872</v>
       </c>
     </row>
     <row r="1196">
@@ -13591,7 +13591,7 @@
         <v>2211</v>
       </c>
       <c r="C1196" t="n">
-        <v>166230</v>
+        <v>177312</v>
       </c>
     </row>
     <row r="1197">
@@ -13602,7 +13602,7 @@
         <v>2682</v>
       </c>
       <c r="C1197" t="n">
-        <v>102255</v>
+        <v>109072</v>
       </c>
     </row>
     <row r="1198">
@@ -13635,7 +13635,7 @@
         <v>2755</v>
       </c>
       <c r="C1200" t="n">
-        <v>40905</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1201">
@@ -13646,7 +13646,7 @@
         <v>941</v>
       </c>
       <c r="C1201" t="n">
-        <v>267870</v>
+        <v>285728</v>
       </c>
     </row>
     <row r="1202">
@@ -13657,7 +13657,7 @@
         <v>2734</v>
       </c>
       <c r="C1202" t="n">
-        <v>37545</v>
+        <v>40048</v>
       </c>
     </row>
     <row r="1203">
@@ -13668,7 +13668,7 @@
         <v>1289</v>
       </c>
       <c r="C1203" t="n">
-        <v>170445</v>
+        <v>181808</v>
       </c>
     </row>
     <row r="1204">
@@ -13679,7 +13679,7 @@
         <v>2801</v>
       </c>
       <c r="C1204" t="n">
-        <v>54540</v>
+        <v>58176</v>
       </c>
     </row>
     <row r="1205">
@@ -13690,7 +13690,7 @@
         <v>2810</v>
       </c>
       <c r="C1205" t="n">
-        <v>92040</v>
+        <v>98176</v>
       </c>
     </row>
     <row r="1206">
@@ -13701,7 +13701,7 @@
         <v>767</v>
       </c>
       <c r="C1206" t="n">
-        <v>122715</v>
+        <v>130896</v>
       </c>
     </row>
     <row r="1207">
@@ -13712,7 +13712,7 @@
         <v>2687</v>
       </c>
       <c r="C1207" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1208">
@@ -13723,7 +13723,7 @@
         <v>2686</v>
       </c>
       <c r="C1208" t="n">
-        <v>88635</v>
+        <v>94544</v>
       </c>
     </row>
     <row r="1209">
@@ -13734,7 +13734,7 @@
         <v>2730</v>
       </c>
       <c r="C1209" t="n">
-        <v>61350</v>
+        <v>65440</v>
       </c>
     </row>
     <row r="1210">
@@ -13745,7 +13745,7 @@
         <v>2580</v>
       </c>
       <c r="C1210" t="n">
-        <v>22875</v>
+        <v>24400</v>
       </c>
     </row>
     <row r="1211">
@@ -13756,7 +13756,7 @@
         <v>2472</v>
       </c>
       <c r="C1211" t="n">
-        <v>36096.85</v>
+        <v>38503.3</v>
       </c>
     </row>
     <row r="1212">
@@ -13767,7 +13767,7 @@
         <v>2631</v>
       </c>
       <c r="C1212" t="n">
-        <v>16726.37</v>
+        <v>17841.46</v>
       </c>
     </row>
     <row r="1213">
@@ -13778,7 +13778,7 @@
         <v>1642</v>
       </c>
       <c r="C1213" t="n">
-        <v>180675</v>
+        <v>192720</v>
       </c>
     </row>
     <row r="1214">
@@ -13789,7 +13789,7 @@
         <v>2613</v>
       </c>
       <c r="C1214" t="n">
-        <v>122175</v>
+        <v>130320</v>
       </c>
     </row>
     <row r="1215">
@@ -13800,7 +13800,7 @@
         <v>1020</v>
       </c>
       <c r="C1215" t="n">
-        <v>61350</v>
+        <v>65440</v>
       </c>
     </row>
     <row r="1216">
@@ -13811,7 +13811,7 @@
         <v>2785</v>
       </c>
       <c r="C1216" t="n">
-        <v>28365</v>
+        <v>30256</v>
       </c>
     </row>
     <row r="1217">
@@ -13822,7 +13822,7 @@
         <v>1327</v>
       </c>
       <c r="C1217" t="n">
-        <v>40905</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1218">
@@ -13833,7 +13833,7 @@
         <v>2629</v>
       </c>
       <c r="C1218" t="n">
-        <v>46830</v>
+        <v>49952</v>
       </c>
     </row>
     <row r="1219">
@@ -13844,7 +13844,7 @@
         <v>749</v>
       </c>
       <c r="C1219" t="n">
-        <v>55560</v>
+        <v>59264</v>
       </c>
     </row>
     <row r="1220">
@@ -13855,7 +13855,7 @@
         <v>1983</v>
       </c>
       <c r="C1220" t="n">
-        <v>368970</v>
+        <v>393568</v>
       </c>
     </row>
     <row r="1221">
@@ -13866,7 +13866,7 @@
         <v>1993</v>
       </c>
       <c r="C1221" t="n">
-        <v>237195</v>
+        <v>253008</v>
       </c>
     </row>
     <row r="1222">
@@ -13877,7 +13877,7 @@
         <v>2767</v>
       </c>
       <c r="C1222" t="n">
-        <v>131535</v>
+        <v>140304</v>
       </c>
     </row>
     <row r="1223">
@@ -13899,7 +13899,7 @@
         <v>1102</v>
       </c>
       <c r="C1224" t="n">
-        <v>164715</v>
+        <v>175696</v>
       </c>
     </row>
     <row r="1225">
@@ -13910,7 +13910,7 @@
         <v>626</v>
       </c>
       <c r="C1225" t="n">
-        <v>1162032.98</v>
+        <v>1239501.84</v>
       </c>
     </row>
     <row r="1226">
@@ -13921,7 +13921,7 @@
         <v>1465</v>
       </c>
       <c r="C1226" t="n">
-        <v>245310</v>
+        <v>261664</v>
       </c>
     </row>
     <row r="1227">
@@ -13932,7 +13932,7 @@
         <v>2758</v>
       </c>
       <c r="C1227" t="n">
-        <v>40909.11</v>
+        <v>43636.38</v>
       </c>
     </row>
     <row r="1228">
@@ -13943,7 +13943,7 @@
         <v>2742</v>
       </c>
       <c r="C1228" t="n">
-        <v>40909.11</v>
+        <v>43636.38</v>
       </c>
     </row>
     <row r="1229">
@@ -13965,7 +13965,7 @@
         <v>1873</v>
       </c>
       <c r="C1230" t="n">
-        <v>218175</v>
+        <v>232720</v>
       </c>
     </row>
     <row r="1231">
@@ -13976,7 +13976,7 @@
         <v>2163</v>
       </c>
       <c r="C1231" t="n">
-        <v>102270</v>
+        <v>109088</v>
       </c>
     </row>
     <row r="1232">
@@ -13987,7 +13987,7 @@
         <v>2394</v>
       </c>
       <c r="C1232" t="n">
-        <v>105030</v>
+        <v>112032</v>
       </c>
     </row>
     <row r="1233">
@@ -13998,7 +13998,7 @@
         <v>33</v>
       </c>
       <c r="C1233" t="n">
-        <v>264540</v>
+        <v>282176</v>
       </c>
     </row>
     <row r="1234">
@@ -14009,7 +14009,7 @@
         <v>2421</v>
       </c>
       <c r="C1234" t="n">
-        <v>44310</v>
+        <v>47264</v>
       </c>
     </row>
     <row r="1235">
@@ -14020,7 +14020,7 @@
         <v>2663</v>
       </c>
       <c r="C1235" t="n">
-        <v>187500</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="1236">
@@ -14031,7 +14031,7 @@
         <v>2413</v>
       </c>
       <c r="C1236" t="n">
-        <v>82530</v>
+        <v>88032</v>
       </c>
     </row>
     <row r="1237">
@@ -14042,7 +14042,7 @@
         <v>351</v>
       </c>
       <c r="C1237" t="n">
-        <v>125445</v>
+        <v>133808</v>
       </c>
     </row>
     <row r="1238">
@@ -14053,7 +14053,7 @@
         <v>1298</v>
       </c>
       <c r="C1238" t="n">
-        <v>867945</v>
+        <v>925808</v>
       </c>
     </row>
     <row r="1239">
@@ -14064,7 +14064,7 @@
         <v>2491</v>
       </c>
       <c r="C1239" t="n">
-        <v>70140</v>
+        <v>74816</v>
       </c>
     </row>
     <row r="1240">
@@ -14075,7 +14075,7 @@
         <v>2571</v>
       </c>
       <c r="C1240" t="n">
-        <v>99045</v>
+        <v>105648</v>
       </c>
     </row>
     <row r="1241">
@@ -14086,7 +14086,7 @@
         <v>2507</v>
       </c>
       <c r="C1241" t="n">
-        <v>60180</v>
+        <v>64192</v>
       </c>
     </row>
     <row r="1242">
@@ -14097,7 +14097,7 @@
         <v>2799</v>
       </c>
       <c r="C1242" t="n">
-        <v>77460</v>
+        <v>82624</v>
       </c>
     </row>
     <row r="1243">
@@ -14119,7 +14119,7 @@
         <v>2582</v>
       </c>
       <c r="C1244" t="n">
-        <v>59010</v>
+        <v>62944</v>
       </c>
     </row>
     <row r="1245">
@@ -14130,7 +14130,7 @@
         <v>2637</v>
       </c>
       <c r="C1245" t="n">
-        <v>42915</v>
+        <v>45776</v>
       </c>
     </row>
     <row r="1246">
@@ -14141,7 +14141,7 @@
         <v>630</v>
       </c>
       <c r="C1246" t="n">
-        <v>102060</v>
+        <v>108864</v>
       </c>
     </row>
     <row r="1247">
@@ -14152,7 +14152,7 @@
         <v>525</v>
       </c>
       <c r="C1247" t="n">
-        <v>153405</v>
+        <v>163632</v>
       </c>
     </row>
     <row r="1248">
@@ -14163,7 +14163,7 @@
         <v>2727</v>
       </c>
       <c r="C1248" t="n">
-        <v>27600</v>
+        <v>29440</v>
       </c>
     </row>
     <row r="1249">
@@ -14174,7 +14174,7 @@
         <v>2707</v>
       </c>
       <c r="C1249" t="n">
-        <v>21840</v>
+        <v>23296</v>
       </c>
     </row>
     <row r="1250">
@@ -14185,7 +14185,7 @@
         <v>2834</v>
       </c>
       <c r="C1250" t="n">
-        <v>11282.74</v>
+        <v>12034.92</v>
       </c>
     </row>
     <row r="1251">
@@ -14196,7 +14196,7 @@
         <v>2773</v>
       </c>
       <c r="C1251" t="n">
-        <v>55017.33</v>
+        <v>58685.14</v>
       </c>
     </row>
     <row r="1252">
@@ -14207,7 +14207,7 @@
         <v>2341</v>
       </c>
       <c r="C1252" t="n">
-        <v>96750</v>
+        <v>103200</v>
       </c>
     </row>
     <row r="1253">
@@ -14218,7 +14218,7 @@
         <v>1374</v>
       </c>
       <c r="C1253" t="n">
-        <v>122715</v>
+        <v>130896</v>
       </c>
     </row>
     <row r="1254">
@@ -14229,7 +14229,7 @@
         <v>793</v>
       </c>
       <c r="C1254" t="n">
-        <v>28365</v>
+        <v>30256</v>
       </c>
     </row>
     <row r="1255">
@@ -14240,7 +14240,7 @@
         <v>794</v>
       </c>
       <c r="C1255" t="n">
-        <v>28365</v>
+        <v>30256</v>
       </c>
     </row>
     <row r="1256">
@@ -14251,7 +14251,7 @@
         <v>1834</v>
       </c>
       <c r="C1256" t="n">
-        <v>79770</v>
+        <v>85088</v>
       </c>
     </row>
     <row r="1257">
@@ -14262,7 +14262,7 @@
         <v>802</v>
       </c>
       <c r="C1257" t="n">
-        <v>51135</v>
+        <v>54544</v>
       </c>
     </row>
     <row r="1258">
@@ -14273,7 +14273,7 @@
         <v>1344</v>
       </c>
       <c r="C1258" t="n">
-        <v>102270</v>
+        <v>109088</v>
       </c>
     </row>
     <row r="1259">
@@ -14284,7 +14284,7 @@
         <v>1881</v>
       </c>
       <c r="C1259" t="n">
-        <v>46830</v>
+        <v>49952</v>
       </c>
     </row>
     <row r="1260">
@@ -14295,7 +14295,7 @@
         <v>2365</v>
       </c>
       <c r="C1260" t="n">
-        <v>54315</v>
+        <v>57936</v>
       </c>
     </row>
     <row r="1261">
@@ -14306,7 +14306,7 @@
         <v>2411</v>
       </c>
       <c r="C1261" t="n">
-        <v>96750</v>
+        <v>103200</v>
       </c>
     </row>
     <row r="1262">
@@ -14317,7 +14317,7 @@
         <v>2363</v>
       </c>
       <c r="C1262" t="n">
-        <v>102270</v>
+        <v>109088</v>
       </c>
     </row>
     <row r="1263">
@@ -14328,7 +14328,7 @@
         <v>2124</v>
       </c>
       <c r="C1263" t="n">
-        <v>238635</v>
+        <v>254544</v>
       </c>
     </row>
     <row r="1264">
@@ -14339,7 +14339,7 @@
         <v>1937</v>
       </c>
       <c r="C1264" t="n">
-        <v>173850</v>
+        <v>185440</v>
       </c>
     </row>
     <row r="1265">
@@ -14350,7 +14350,7 @@
         <v>2709</v>
       </c>
       <c r="C1265" t="n">
-        <v>122715</v>
+        <v>130896</v>
       </c>
     </row>
     <row r="1266">
@@ -14361,7 +14361,7 @@
         <v>2558</v>
       </c>
       <c r="C1266" t="n">
-        <v>20490</v>
+        <v>21856</v>
       </c>
     </row>
     <row r="1267">
@@ -14372,7 +14372,7 @@
         <v>663</v>
       </c>
       <c r="C1267" t="n">
-        <v>173850</v>
+        <v>185440</v>
       </c>
     </row>
     <row r="1268">
@@ -14383,7 +14383,7 @@
         <v>40</v>
       </c>
       <c r="C1268" t="n">
-        <v>150000</v>
+        <v>160000</v>
       </c>
     </row>
     <row r="1269">
@@ -14394,7 +14394,7 @@
         <v>2833</v>
       </c>
       <c r="C1269" t="n">
-        <v>47727.33</v>
+        <v>50909.14</v>
       </c>
     </row>
     <row r="1270">
@@ -14405,7 +14405,7 @@
         <v>1756</v>
       </c>
       <c r="C1270" t="n">
-        <v>297615</v>
+        <v>317456</v>
       </c>
     </row>
     <row r="1271">
@@ -14416,7 +14416,7 @@
         <v>1116</v>
       </c>
       <c r="C1271" t="n">
-        <v>172935</v>
+        <v>184464</v>
       </c>
     </row>
     <row r="1272">
@@ -14427,7 +14427,7 @@
         <v>636</v>
       </c>
       <c r="C1272" t="n">
-        <v>170445</v>
+        <v>181808</v>
       </c>
     </row>
     <row r="1273">
@@ -14438,7 +14438,7 @@
         <v>1800</v>
       </c>
       <c r="C1273" t="n">
-        <v>19080</v>
+        <v>20352</v>
       </c>
     </row>
     <row r="1274">
@@ -14449,7 +14449,7 @@
         <v>2815</v>
       </c>
       <c r="C1274" t="n">
-        <v>40909.11</v>
+        <v>43636.38</v>
       </c>
     </row>
     <row r="1275">
@@ -14460,7 +14460,7 @@
         <v>1658</v>
       </c>
       <c r="C1275" t="n">
-        <v>90000</v>
+        <v>96000</v>
       </c>
     </row>
     <row r="1276">
@@ -14471,7 +14471,7 @@
         <v>2635</v>
       </c>
       <c r="C1276" t="n">
-        <v>88635</v>
+        <v>94544</v>
       </c>
     </row>
     <row r="1277">
@@ -14482,7 +14482,7 @@
         <v>2402</v>
       </c>
       <c r="C1277" t="n">
-        <v>444540</v>
+        <v>474176</v>
       </c>
     </row>
     <row r="1278">
@@ -14493,7 +14493,7 @@
         <v>452</v>
       </c>
       <c r="C1278" t="n">
-        <v>184080</v>
+        <v>196352</v>
       </c>
     </row>
     <row r="1279">
@@ -14504,7 +14504,7 @@
         <v>2085</v>
       </c>
       <c r="C1279" t="n">
-        <v>90030</v>
+        <v>96032</v>
       </c>
     </row>
     <row r="1280">
@@ -14515,7 +14515,7 @@
         <v>2568</v>
       </c>
       <c r="C1280" t="n">
-        <v>139380</v>
+        <v>148672</v>
       </c>
     </row>
     <row r="1281">
@@ -14526,7 +14526,7 @@
         <v>1906</v>
       </c>
       <c r="C1281" t="n">
-        <v>79110</v>
+        <v>84384</v>
       </c>
     </row>
     <row r="1282">
@@ -14537,7 +14537,7 @@
         <v>2821</v>
       </c>
       <c r="C1282" t="n">
-        <v>68790</v>
+        <v>73376</v>
       </c>
     </row>
     <row r="1283">
@@ -14548,7 +14548,7 @@
         <v>2698</v>
       </c>
       <c r="C1283" t="n">
-        <v>84315</v>
+        <v>89936</v>
       </c>
     </row>
     <row r="1284">
@@ -14559,7 +14559,7 @@
         <v>2118</v>
       </c>
       <c r="C1284" t="n">
-        <v>161700</v>
+        <v>172480</v>
       </c>
     </row>
     <row r="1285">
@@ -14570,7 +14570,7 @@
         <v>2383</v>
       </c>
       <c r="C1285" t="n">
-        <v>94410</v>
+        <v>100704</v>
       </c>
     </row>
     <row r="1286">
@@ -14581,7 +14581,7 @@
         <v>2813</v>
       </c>
       <c r="C1286" t="n">
-        <v>42915</v>
+        <v>45776</v>
       </c>
     </row>
     <row r="1287">
@@ -14592,7 +14592,7 @@
         <v>925</v>
       </c>
       <c r="C1287" t="n">
-        <v>53640</v>
+        <v>57216</v>
       </c>
     </row>
     <row r="1288">
@@ -14603,7 +14603,7 @@
         <v>2689</v>
       </c>
       <c r="C1288" t="n">
-        <v>42915</v>
+        <v>45776</v>
       </c>
     </row>
     <row r="1289">
@@ -14614,7 +14614,7 @@
         <v>2716</v>
       </c>
       <c r="C1289" t="n">
-        <v>59010</v>
+        <v>62944</v>
       </c>
     </row>
     <row r="1290">
@@ -14625,7 +14625,7 @@
         <v>2831</v>
       </c>
       <c r="C1290" t="n">
-        <v>40905</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1291">
@@ -14636,7 +14636,7 @@
         <v>2045</v>
       </c>
       <c r="C1291" t="n">
-        <v>229401.61</v>
+        <v>244695.04</v>
       </c>
     </row>
     <row r="1292">
@@ -14647,7 +14647,7 @@
         <v>580</v>
       </c>
       <c r="C1292" t="n">
-        <v>92040</v>
+        <v>98176</v>
       </c>
     </row>
     <row r="1293">
@@ -14658,7 +14658,7 @@
         <v>438</v>
       </c>
       <c r="C1293" t="n">
-        <v>105675</v>
+        <v>112720</v>
       </c>
     </row>
     <row r="1294">
@@ -14669,7 +14669,7 @@
         <v>1539</v>
       </c>
       <c r="C1294" t="n">
-        <v>115905</v>
+        <v>123632</v>
       </c>
     </row>
     <row r="1295">
@@ -14680,7 +14680,7 @@
         <v>2817</v>
       </c>
       <c r="C1295" t="n">
-        <v>40905</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1296">
@@ -14691,7 +14691,7 @@
         <v>2816</v>
       </c>
       <c r="C1296" t="n">
-        <v>88635</v>
+        <v>94544</v>
       </c>
     </row>
     <row r="1297">
@@ -14702,7 +14702,7 @@
         <v>2146</v>
       </c>
       <c r="C1297" t="n">
-        <v>137490</v>
+        <v>146656</v>
       </c>
     </row>
     <row r="1298">
@@ -14713,7 +14713,7 @@
         <v>2276</v>
       </c>
       <c r="C1298" t="n">
-        <v>152760</v>
+        <v>162944</v>
       </c>
     </row>
     <row r="1299">
@@ -14724,7 +14724,7 @@
         <v>1381</v>
       </c>
       <c r="C1299" t="n">
-        <v>201135</v>
+        <v>214544</v>
       </c>
     </row>
     <row r="1300">
@@ -14735,7 +14735,7 @@
         <v>2081</v>
       </c>
       <c r="C1300" t="n">
-        <v>102270</v>
+        <v>109088</v>
       </c>
     </row>
     <row r="1301">
@@ -14746,7 +14746,7 @@
         <v>14</v>
       </c>
       <c r="C1301" t="n">
-        <v>296580</v>
+        <v>316352</v>
       </c>
     </row>
     <row r="1302">
@@ -14757,7 +14757,7 @@
         <v>766</v>
       </c>
       <c r="C1302" t="n">
-        <v>46830</v>
+        <v>49952</v>
       </c>
     </row>
     <row r="1303">
@@ -14768,7 +14768,7 @@
         <v>2547</v>
       </c>
       <c r="C1303" t="n">
-        <v>28035</v>
+        <v>29904</v>
       </c>
     </row>
     <row r="1304">
@@ -14779,7 +14779,7 @@
         <v>2552</v>
       </c>
       <c r="C1304" t="n">
-        <v>20160</v>
+        <v>21504</v>
       </c>
     </row>
     <row r="1305">
@@ -14790,7 +14790,7 @@
         <v>131</v>
       </c>
       <c r="C1305" t="n">
-        <v>278850</v>
+        <v>297440</v>
       </c>
     </row>
     <row r="1306">
@@ -14801,7 +14801,7 @@
         <v>2250</v>
       </c>
       <c r="C1306" t="n">
-        <v>225615</v>
+        <v>240656</v>
       </c>
     </row>
     <row r="1307">
@@ -14812,7 +14812,7 @@
         <v>89</v>
       </c>
       <c r="C1307" t="n">
-        <v>230580</v>
+        <v>245952</v>
       </c>
     </row>
     <row r="1308">
@@ -14823,7 +14823,7 @@
         <v>2141</v>
       </c>
       <c r="C1308" t="n">
-        <v>21570</v>
+        <v>23008</v>
       </c>
     </row>
     <row r="1309">
@@ -14834,7 +14834,7 @@
         <v>2798</v>
       </c>
       <c r="C1309" t="n">
-        <v>40909.11</v>
+        <v>43636.38</v>
       </c>
     </row>
     <row r="1310">
@@ -14845,7 +14845,7 @@
         <v>2797</v>
       </c>
       <c r="C1310" t="n">
-        <v>40909.11</v>
+        <v>43636.38</v>
       </c>
     </row>
     <row r="1311">
@@ -14856,7 +14856,7 @@
         <v>2266</v>
       </c>
       <c r="C1311" t="n">
-        <v>54545.48</v>
+        <v>58181.84</v>
       </c>
     </row>
     <row r="1312">
@@ -14867,7 +14867,7 @@
         <v>1499</v>
       </c>
       <c r="C1312" t="n">
-        <v>95445</v>
+        <v>101808</v>
       </c>
     </row>
     <row r="1313">
@@ -14878,7 +14878,7 @@
         <v>2496</v>
       </c>
       <c r="C1313" t="n">
-        <v>109080</v>
+        <v>116352</v>
       </c>
     </row>
     <row r="1314">
@@ -14889,7 +14889,7 @@
         <v>949</v>
       </c>
       <c r="C1314" t="n">
-        <v>66915</v>
+        <v>71376</v>
       </c>
     </row>
     <row r="1315">
@@ -14900,7 +14900,7 @@
         <v>1853</v>
       </c>
       <c r="C1315" t="n">
-        <v>81810</v>
+        <v>87264</v>
       </c>
     </row>
     <row r="1316">
@@ -14911,7 +14911,7 @@
         <v>854</v>
       </c>
       <c r="C1316" t="n">
-        <v>75000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="1317">
@@ -14922,7 +14922,7 @@
         <v>2674</v>
       </c>
       <c r="C1317" t="n">
-        <v>177270</v>
+        <v>189088</v>
       </c>
     </row>
     <row r="1318">
@@ -14933,7 +14933,7 @@
         <v>2803</v>
       </c>
       <c r="C1318" t="n">
-        <v>81810</v>
+        <v>87264</v>
       </c>
     </row>
     <row r="1319">
@@ -14944,7 +14944,7 @@
         <v>2599</v>
       </c>
       <c r="C1319" t="n">
-        <v>129540</v>
+        <v>138176</v>
       </c>
     </row>
     <row r="1320">
@@ -14955,7 +14955,7 @@
         <v>783</v>
       </c>
       <c r="C1320" t="n">
-        <v>35445</v>
+        <v>37808</v>
       </c>
     </row>
     <row r="1321">
@@ -14966,7 +14966,7 @@
         <v>27</v>
       </c>
       <c r="C1321" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1322">
@@ -14977,7 +14977,7 @@
         <v>531</v>
       </c>
       <c r="C1322" t="n">
-        <v>238635</v>
+        <v>254544</v>
       </c>
     </row>
     <row r="1323">
@@ -14988,7 +14988,7 @@
         <v>1308</v>
       </c>
       <c r="C1323" t="n">
-        <v>110130</v>
+        <v>117472</v>
       </c>
     </row>
     <row r="1324">
@@ -14999,7 +14999,7 @@
         <v>2792</v>
       </c>
       <c r="C1324" t="n">
-        <v>79425</v>
+        <v>84720</v>
       </c>
     </row>
     <row r="1325">
@@ -15021,7 +15021,7 @@
         <v>2823</v>
       </c>
       <c r="C1326" t="n">
-        <v>63750</v>
+        <v>68000</v>
       </c>
     </row>
     <row r="1327">
@@ -15032,7 +15032,7 @@
         <v>2584</v>
       </c>
       <c r="C1327" t="n">
-        <v>42915</v>
+        <v>45776</v>
       </c>
     </row>
     <row r="1328">
@@ -15043,7 +15043,7 @@
         <v>945</v>
       </c>
       <c r="C1328" t="n">
-        <v>193170</v>
+        <v>206048</v>
       </c>
     </row>
     <row r="1329">
@@ -15054,7 +15054,7 @@
         <v>2660</v>
       </c>
       <c r="C1329" t="n">
-        <v>211350</v>
+        <v>225440</v>
       </c>
     </row>
     <row r="1330">
@@ -15065,7 +15065,7 @@
         <v>1317</v>
       </c>
       <c r="C1330" t="n">
-        <v>204540</v>
+        <v>218176</v>
       </c>
     </row>
     <row r="1331">
@@ -15076,7 +15076,7 @@
         <v>2790</v>
       </c>
       <c r="C1331" t="n">
-        <v>43425</v>
+        <v>46320</v>
       </c>
     </row>
     <row r="1332">
@@ -15087,7 +15087,7 @@
         <v>2711</v>
       </c>
       <c r="C1332" t="n">
-        <v>59105.48</v>
+        <v>63045.84</v>
       </c>
     </row>
     <row r="1333">
@@ -15098,7 +15098,7 @@
         <v>2607</v>
       </c>
       <c r="C1333" t="n">
-        <v>33875.48</v>
+        <v>36133.84</v>
       </c>
     </row>
     <row r="1334">
@@ -15109,7 +15109,7 @@
         <v>2667</v>
       </c>
       <c r="C1334" t="n">
-        <v>31159.11</v>
+        <v>33236.38</v>
       </c>
     </row>
     <row r="1335">
@@ -15120,7 +15120,7 @@
         <v>2706</v>
       </c>
       <c r="C1335" t="n">
-        <v>15021.85</v>
+        <v>16023.3</v>
       </c>
     </row>
     <row r="1336">
@@ -15131,7 +15131,7 @@
         <v>2657</v>
       </c>
       <c r="C1336" t="n">
-        <v>53997.33</v>
+        <v>57597.14</v>
       </c>
     </row>
     <row r="1337">
@@ -15142,7 +15142,7 @@
         <v>1278</v>
       </c>
       <c r="C1337" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1338">
@@ -15153,7 +15153,7 @@
         <v>2745</v>
       </c>
       <c r="C1338" t="n">
-        <v>75000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="1339">
@@ -15164,7 +15164,7 @@
         <v>2753</v>
       </c>
       <c r="C1339" t="n">
-        <v>51135</v>
+        <v>54544</v>
       </c>
     </row>
     <row r="1340">
@@ -15175,7 +15175,7 @@
         <v>2183</v>
       </c>
       <c r="C1340" t="n">
-        <v>249510</v>
+        <v>266144</v>
       </c>
     </row>
     <row r="1341">
@@ -15186,7 +15186,7 @@
         <v>1340</v>
       </c>
       <c r="C1341" t="n">
-        <v>98850</v>
+        <v>105440</v>
       </c>
     </row>
     <row r="1342">
@@ -15197,7 +15197,7 @@
         <v>2583</v>
       </c>
       <c r="C1342" t="n">
-        <v>28365</v>
+        <v>30256</v>
       </c>
     </row>
     <row r="1343">
@@ -15208,7 +15208,7 @@
         <v>2090</v>
       </c>
       <c r="C1343" t="n">
-        <v>28365</v>
+        <v>30256</v>
       </c>
     </row>
     <row r="1344">
@@ -15219,7 +15219,7 @@
         <v>1277</v>
       </c>
       <c r="C1344" t="n">
-        <v>150000</v>
+        <v>160000</v>
       </c>
     </row>
     <row r="1345">
@@ -15230,7 +15230,7 @@
         <v>1501</v>
       </c>
       <c r="C1345" t="n">
-        <v>64770</v>
+        <v>69088</v>
       </c>
     </row>
     <row r="1346">
@@ -15241,7 +15241,7 @@
         <v>703</v>
       </c>
       <c r="C1346" t="n">
-        <v>170445</v>
+        <v>181808</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:01:59
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -11292,7 +11292,7 @@
         <v>947</v>
       </c>
       <c r="C987" t="n">
-        <v>316016</v>
+        <v>335767</v>
       </c>
     </row>
     <row r="988">
@@ -11303,7 +11303,7 @@
         <v>1956</v>
       </c>
       <c r="C988" t="n">
-        <v>183616</v>
+        <v>195092</v>
       </c>
     </row>
     <row r="989">
@@ -11314,7 +11314,7 @@
         <v>2824</v>
       </c>
       <c r="C989" t="n">
-        <v>80000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="990">
@@ -11325,7 +11325,7 @@
         <v>2787</v>
       </c>
       <c r="C990" t="n">
-        <v>94544</v>
+        <v>100453</v>
       </c>
     </row>
     <row r="991">
@@ -11336,7 +11336,7 @@
         <v>2830</v>
       </c>
       <c r="C991" t="n">
-        <v>65440</v>
+        <v>69530</v>
       </c>
     </row>
     <row r="992">
@@ -11347,7 +11347,7 @@
         <v>1254</v>
       </c>
       <c r="C992" t="n">
-        <v>141233.46</v>
+        <v>150060.55</v>
       </c>
     </row>
     <row r="993">
@@ -11358,7 +11358,7 @@
         <v>816</v>
       </c>
       <c r="C993" t="n">
-        <v>194800</v>
+        <v>206975</v>
       </c>
     </row>
     <row r="994">
@@ -11369,7 +11369,7 @@
         <v>2671</v>
       </c>
       <c r="C994" t="n">
-        <v>58176</v>
+        <v>61812</v>
       </c>
     </row>
     <row r="995">
@@ -11380,7 +11380,7 @@
         <v>2705</v>
       </c>
       <c r="C995" t="n">
-        <v>130320</v>
+        <v>138465</v>
       </c>
     </row>
     <row r="996">
@@ -11391,7 +11391,7 @@
         <v>2333</v>
       </c>
       <c r="C996" t="n">
-        <v>112256</v>
+        <v>119272</v>
       </c>
     </row>
     <row r="997">
@@ -11402,7 +11402,7 @@
         <v>2440</v>
       </c>
       <c r="C997" t="n">
-        <v>65440</v>
+        <v>69530</v>
       </c>
     </row>
     <row r="998">
@@ -11413,7 +11413,7 @@
         <v>2448</v>
       </c>
       <c r="C998" t="n">
-        <v>14544</v>
+        <v>15453</v>
       </c>
     </row>
     <row r="999">
@@ -11424,7 +11424,7 @@
         <v>2310</v>
       </c>
       <c r="C999" t="n">
-        <v>49952</v>
+        <v>53074</v>
       </c>
     </row>
     <row r="1000">
@@ -11435,7 +11435,7 @@
         <v>2809</v>
       </c>
       <c r="C1000" t="n">
-        <v>49952</v>
+        <v>53074</v>
       </c>
     </row>
     <row r="1001">
@@ -11446,7 +11446,7 @@
         <v>2548</v>
       </c>
       <c r="C1001" t="n">
-        <v>42560</v>
+        <v>45220</v>
       </c>
     </row>
     <row r="1002">
@@ -11457,7 +11457,7 @@
         <v>451</v>
       </c>
       <c r="C1002" t="n">
-        <v>174544</v>
+        <v>185453</v>
       </c>
     </row>
     <row r="1003">
@@ -11468,7 +11468,7 @@
         <v>933</v>
       </c>
       <c r="C1003" t="n">
-        <v>59264</v>
+        <v>62968</v>
       </c>
     </row>
     <row r="1004">
@@ -11479,7 +11479,7 @@
         <v>2702</v>
       </c>
       <c r="C1004" t="n">
-        <v>59264</v>
+        <v>62968</v>
       </c>
     </row>
     <row r="1005">
@@ -11490,7 +11490,7 @@
         <v>2549</v>
       </c>
       <c r="C1005" t="n">
-        <v>20608</v>
+        <v>21896</v>
       </c>
     </row>
     <row r="1006">
@@ -11501,7 +11501,7 @@
         <v>535</v>
       </c>
       <c r="C1006" t="n">
-        <v>269088</v>
+        <v>285906</v>
       </c>
     </row>
     <row r="1007">
@@ -11512,7 +11512,7 @@
         <v>1117</v>
       </c>
       <c r="C1007" t="n">
-        <v>253008</v>
+        <v>268821</v>
       </c>
     </row>
     <row r="1008">
@@ -11534,7 +11534,7 @@
         <v>530</v>
       </c>
       <c r="C1009" t="n">
-        <v>177504</v>
+        <v>188598</v>
       </c>
     </row>
     <row r="1010">
@@ -11545,7 +11545,7 @@
         <v>358</v>
       </c>
       <c r="C1010" t="n">
-        <v>247264</v>
+        <v>262718</v>
       </c>
     </row>
     <row r="1011">
@@ -11556,7 +11556,7 @@
         <v>2498</v>
       </c>
       <c r="C1011" t="n">
-        <v>40384</v>
+        <v>42908</v>
       </c>
     </row>
     <row r="1012">
@@ -11567,7 +11567,7 @@
         <v>2381</v>
       </c>
       <c r="C1012" t="n">
-        <v>57696</v>
+        <v>61302</v>
       </c>
     </row>
     <row r="1013">
@@ -11578,7 +11578,7 @@
         <v>2695</v>
       </c>
       <c r="C1013" t="n">
-        <v>34704</v>
+        <v>36873</v>
       </c>
     </row>
     <row r="1014">
@@ -11589,7 +11589,7 @@
         <v>2744</v>
       </c>
       <c r="C1014" t="n">
-        <v>43636.38</v>
+        <v>46363.65</v>
       </c>
     </row>
     <row r="1015">
@@ -11600,7 +11600,7 @@
         <v>2750</v>
       </c>
       <c r="C1015" t="n">
-        <v>43632</v>
+        <v>46359</v>
       </c>
     </row>
     <row r="1016">
@@ -11611,7 +11611,7 @@
         <v>2131</v>
       </c>
       <c r="C1016" t="n">
-        <v>87264</v>
+        <v>92718</v>
       </c>
     </row>
     <row r="1017">
@@ -11622,7 +11622,7 @@
         <v>818</v>
       </c>
       <c r="C1017" t="n">
-        <v>290896</v>
+        <v>309077</v>
       </c>
     </row>
     <row r="1018">
@@ -11633,7 +11633,7 @@
         <v>2566</v>
       </c>
       <c r="C1018" t="n">
-        <v>58176</v>
+        <v>61812</v>
       </c>
     </row>
     <row r="1019">
@@ -11644,7 +11644,7 @@
         <v>132</v>
       </c>
       <c r="C1019" t="n">
-        <v>545440</v>
+        <v>579530</v>
       </c>
     </row>
     <row r="1020">
@@ -11655,7 +11655,7 @@
         <v>2431</v>
       </c>
       <c r="C1020" t="n">
-        <v>133808</v>
+        <v>142171</v>
       </c>
     </row>
     <row r="1021">
@@ -11666,7 +11666,7 @@
         <v>2249</v>
       </c>
       <c r="C1021" t="n">
-        <v>142048</v>
+        <v>150926</v>
       </c>
     </row>
     <row r="1022">
@@ -11677,7 +11677,7 @@
         <v>1585</v>
       </c>
       <c r="C1022" t="n">
-        <v>120032</v>
+        <v>127534</v>
       </c>
     </row>
     <row r="1023">
@@ -11688,7 +11688,7 @@
         <v>2325</v>
       </c>
       <c r="C1023" t="n">
-        <v>116032</v>
+        <v>123284</v>
       </c>
     </row>
     <row r="1024">
@@ -11699,7 +11699,7 @@
         <v>2190</v>
       </c>
       <c r="C1024" t="n">
-        <v>163632</v>
+        <v>173859</v>
       </c>
     </row>
     <row r="1025">
@@ -11710,7 +11710,7 @@
         <v>1466</v>
       </c>
       <c r="C1025" t="n">
-        <v>294544</v>
+        <v>312953</v>
       </c>
     </row>
     <row r="1026">
@@ -11721,7 +11721,7 @@
         <v>2659</v>
       </c>
       <c r="C1026" t="n">
-        <v>89456</v>
+        <v>95047</v>
       </c>
     </row>
     <row r="1027">
@@ -11732,7 +11732,7 @@
         <v>634</v>
       </c>
       <c r="C1027" t="n">
-        <v>400000</v>
+        <v>425000</v>
       </c>
     </row>
     <row r="1028">
@@ -11743,7 +11743,7 @@
         <v>2804</v>
       </c>
       <c r="C1028" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1029">
@@ -11754,7 +11754,7 @@
         <v>2375</v>
       </c>
       <c r="C1029" t="n">
-        <v>240000</v>
+        <v>255000</v>
       </c>
     </row>
     <row r="1030">
@@ -11765,7 +11765,7 @@
         <v>2601</v>
       </c>
       <c r="C1030" t="n">
-        <v>200000</v>
+        <v>212500</v>
       </c>
     </row>
     <row r="1031">
@@ -11776,7 +11776,7 @@
         <v>952</v>
       </c>
       <c r="C1031" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1032">
@@ -11787,7 +11787,7 @@
         <v>571</v>
       </c>
       <c r="C1032" t="n">
-        <v>462896</v>
+        <v>491827</v>
       </c>
     </row>
     <row r="1033">
@@ -11798,7 +11798,7 @@
         <v>2697</v>
       </c>
       <c r="C1033" t="n">
-        <v>141040</v>
+        <v>149855</v>
       </c>
     </row>
     <row r="1034">
@@ -11809,7 +11809,7 @@
         <v>2678</v>
       </c>
       <c r="C1034" t="n">
-        <v>244016</v>
+        <v>259267</v>
       </c>
     </row>
     <row r="1035">
@@ -11820,7 +11820,7 @@
         <v>2768</v>
       </c>
       <c r="C1035" t="n">
-        <v>255376</v>
+        <v>271337</v>
       </c>
     </row>
     <row r="1036">
@@ -11831,7 +11831,7 @@
         <v>2359</v>
       </c>
       <c r="C1036" t="n">
-        <v>77456</v>
+        <v>82297</v>
       </c>
     </row>
     <row r="1037">
@@ -11842,7 +11842,7 @@
         <v>353</v>
       </c>
       <c r="C1037" t="n">
-        <v>251616</v>
+        <v>267342</v>
       </c>
     </row>
     <row r="1038">
@@ -11853,7 +11853,7 @@
         <v>2026</v>
       </c>
       <c r="C1038" t="n">
-        <v>208480</v>
+        <v>221510</v>
       </c>
     </row>
     <row r="1039">
@@ -11875,7 +11875,7 @@
         <v>2345</v>
       </c>
       <c r="C1040" t="n">
-        <v>45776</v>
+        <v>48637</v>
       </c>
     </row>
     <row r="1041">
@@ -11886,7 +11886,7 @@
         <v>2789</v>
       </c>
       <c r="C1041" t="n">
-        <v>123632</v>
+        <v>131359</v>
       </c>
     </row>
     <row r="1042">
@@ -11897,7 +11897,7 @@
         <v>569</v>
       </c>
       <c r="C1042" t="n">
-        <v>2082848</v>
+        <v>2213026</v>
       </c>
     </row>
     <row r="1043">
@@ -11908,7 +11908,7 @@
         <v>2822</v>
       </c>
       <c r="C1043" t="n">
-        <v>98176</v>
+        <v>104312</v>
       </c>
     </row>
     <row r="1044">
@@ -11919,7 +11919,7 @@
         <v>2728</v>
       </c>
       <c r="C1044" t="n">
-        <v>7264</v>
+        <v>7718</v>
       </c>
     </row>
     <row r="1045">
@@ -11930,7 +11930,7 @@
         <v>2488</v>
       </c>
       <c r="C1045" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1046">
@@ -11941,7 +11941,7 @@
         <v>2791</v>
       </c>
       <c r="C1046" t="n">
-        <v>71774.60000000001</v>
+        <v>76260.5</v>
       </c>
     </row>
     <row r="1047">
@@ -11952,7 +11952,7 @@
         <v>2577</v>
       </c>
       <c r="C1047" t="n">
-        <v>64851.01</v>
+        <v>68904.19</v>
       </c>
     </row>
     <row r="1048">
@@ -11963,7 +11963,7 @@
         <v>2069</v>
       </c>
       <c r="C1048" t="n">
-        <v>130896</v>
+        <v>139077</v>
       </c>
     </row>
     <row r="1049">
@@ -11974,7 +11974,7 @@
         <v>2082</v>
       </c>
       <c r="C1049" t="n">
-        <v>121136</v>
+        <v>128707</v>
       </c>
     </row>
     <row r="1050">
@@ -11985,7 +11985,7 @@
         <v>781</v>
       </c>
       <c r="C1050" t="n">
-        <v>94544</v>
+        <v>100453</v>
       </c>
     </row>
     <row r="1051">
@@ -11996,7 +11996,7 @@
         <v>744</v>
       </c>
       <c r="C1051" t="n">
-        <v>30256</v>
+        <v>32147</v>
       </c>
     </row>
     <row r="1052">
@@ -12007,7 +12007,7 @@
         <v>2223</v>
       </c>
       <c r="C1052" t="n">
-        <v>95952</v>
+        <v>101949</v>
       </c>
     </row>
     <row r="1053">
@@ -12018,7 +12018,7 @@
         <v>2452</v>
       </c>
       <c r="C1053" t="n">
-        <v>50896</v>
+        <v>54077</v>
       </c>
     </row>
     <row r="1054">
@@ -12029,7 +12029,7 @@
         <v>970</v>
       </c>
       <c r="C1054" t="n">
-        <v>49952</v>
+        <v>53074</v>
       </c>
     </row>
     <row r="1055">
@@ -12040,7 +12040,7 @@
         <v>2550</v>
       </c>
       <c r="C1055" t="n">
-        <v>44352</v>
+        <v>47124</v>
       </c>
     </row>
     <row r="1056">
@@ -12051,7 +12051,7 @@
         <v>768</v>
       </c>
       <c r="C1056" t="n">
-        <v>94544</v>
+        <v>100453</v>
       </c>
     </row>
     <row r="1057">
@@ -12062,7 +12062,7 @@
         <v>1075</v>
       </c>
       <c r="C1057" t="n">
-        <v>329440</v>
+        <v>350030</v>
       </c>
     </row>
     <row r="1058">
@@ -12073,7 +12073,7 @@
         <v>664</v>
       </c>
       <c r="C1058" t="n">
-        <v>188352</v>
+        <v>200124</v>
       </c>
     </row>
     <row r="1059">
@@ -12084,7 +12084,7 @@
         <v>2555</v>
       </c>
       <c r="C1059" t="n">
-        <v>30192</v>
+        <v>32079</v>
       </c>
     </row>
     <row r="1060">
@@ -12095,7 +12095,7 @@
         <v>2627</v>
       </c>
       <c r="C1060" t="n">
-        <v>17728</v>
+        <v>18836</v>
       </c>
     </row>
     <row r="1061">
@@ -12106,7 +12106,7 @@
         <v>2557</v>
       </c>
       <c r="C1061" t="n">
-        <v>18752</v>
+        <v>19924</v>
       </c>
     </row>
     <row r="1062">
@@ -12117,7 +12117,7 @@
         <v>2551</v>
       </c>
       <c r="C1062" t="n">
-        <v>14896</v>
+        <v>15827</v>
       </c>
     </row>
     <row r="1063">
@@ -12128,7 +12128,7 @@
         <v>2463</v>
       </c>
       <c r="C1063" t="n">
-        <v>232880</v>
+        <v>247435</v>
       </c>
     </row>
     <row r="1064">
@@ -12139,7 +12139,7 @@
         <v>2279</v>
       </c>
       <c r="C1064" t="n">
-        <v>175696</v>
+        <v>186677</v>
       </c>
     </row>
     <row r="1065">
@@ -12150,7 +12150,7 @@
         <v>631</v>
       </c>
       <c r="C1065" t="n">
-        <v>254544</v>
+        <v>270453</v>
       </c>
     </row>
     <row r="1066">
@@ -12161,7 +12161,7 @@
         <v>2251</v>
       </c>
       <c r="C1066" t="n">
-        <v>155872</v>
+        <v>165614</v>
       </c>
     </row>
     <row r="1067">
@@ -12172,7 +12172,7 @@
         <v>1653</v>
       </c>
       <c r="C1067" t="n">
-        <v>236352</v>
+        <v>251124</v>
       </c>
     </row>
     <row r="1068">
@@ -12183,7 +12183,7 @@
         <v>1293</v>
       </c>
       <c r="C1068" t="n">
-        <v>301808</v>
+        <v>320671</v>
       </c>
     </row>
     <row r="1069">
@@ -12194,7 +12194,7 @@
         <v>360</v>
       </c>
       <c r="C1069" t="n">
-        <v>363632</v>
+        <v>386359</v>
       </c>
     </row>
     <row r="1070">
@@ -12205,7 +12205,7 @@
         <v>1063</v>
       </c>
       <c r="C1070" t="n">
-        <v>264400</v>
+        <v>280925</v>
       </c>
     </row>
     <row r="1071">
@@ -12216,7 +12216,7 @@
         <v>2273</v>
       </c>
       <c r="C1071" t="n">
-        <v>154240</v>
+        <v>163880</v>
       </c>
     </row>
     <row r="1072">
@@ -12227,7 +12227,7 @@
         <v>2757</v>
       </c>
       <c r="C1072" t="n">
-        <v>50909.14</v>
+        <v>54090.95</v>
       </c>
     </row>
     <row r="1073">
@@ -12238,7 +12238,7 @@
         <v>2795</v>
       </c>
       <c r="C1073" t="n">
-        <v>43636.38</v>
+        <v>46363.65</v>
       </c>
     </row>
     <row r="1074">
@@ -12249,7 +12249,7 @@
         <v>2722</v>
       </c>
       <c r="C1074" t="n">
-        <v>43632</v>
+        <v>46359</v>
       </c>
     </row>
     <row r="1075">
@@ -12260,7 +12260,7 @@
         <v>2718</v>
       </c>
       <c r="C1075" t="n">
-        <v>58176</v>
+        <v>61812</v>
       </c>
     </row>
     <row r="1076">
@@ -12271,7 +12271,7 @@
         <v>595</v>
       </c>
       <c r="C1076" t="n">
-        <v>400000</v>
+        <v>425000</v>
       </c>
     </row>
     <row r="1077">
@@ -12282,7 +12282,7 @@
         <v>890</v>
       </c>
       <c r="C1077" t="n">
-        <v>509088</v>
+        <v>540906</v>
       </c>
     </row>
     <row r="1078">
@@ -12293,7 +12293,7 @@
         <v>2652</v>
       </c>
       <c r="C1078" t="n">
-        <v>94544</v>
+        <v>100453</v>
       </c>
     </row>
     <row r="1079">
@@ -12304,7 +12304,7 @@
         <v>2714</v>
       </c>
       <c r="C1079" t="n">
-        <v>261808</v>
+        <v>278171</v>
       </c>
     </row>
     <row r="1080">
@@ -12315,7 +12315,7 @@
         <v>1869</v>
       </c>
       <c r="C1080" t="n">
-        <v>167264</v>
+        <v>177718</v>
       </c>
     </row>
     <row r="1081">
@@ -12326,7 +12326,7 @@
         <v>400</v>
       </c>
       <c r="C1081" t="n">
-        <v>138176</v>
+        <v>146812</v>
       </c>
     </row>
     <row r="1082">
@@ -12337,7 +12337,7 @@
         <v>1907</v>
       </c>
       <c r="C1082" t="n">
-        <v>269808</v>
+        <v>286671</v>
       </c>
     </row>
     <row r="1083">
@@ -12348,7 +12348,7 @@
         <v>1996</v>
       </c>
       <c r="C1083" t="n">
-        <v>170544</v>
+        <v>181203</v>
       </c>
     </row>
     <row r="1084">
@@ -12359,7 +12359,7 @@
         <v>1890</v>
       </c>
       <c r="C1084" t="n">
-        <v>229921.97</v>
+        <v>244292.08</v>
       </c>
     </row>
     <row r="1085">
@@ -12370,7 +12370,7 @@
         <v>2114</v>
       </c>
       <c r="C1085" t="n">
-        <v>133600</v>
+        <v>141950</v>
       </c>
     </row>
     <row r="1086">
@@ -12381,7 +12381,7 @@
         <v>2330</v>
       </c>
       <c r="C1086" t="n">
-        <v>195472</v>
+        <v>207689</v>
       </c>
     </row>
     <row r="1087">
@@ -12425,7 +12425,7 @@
         <v>931</v>
       </c>
       <c r="C1090" t="n">
-        <v>68672</v>
+        <v>72964</v>
       </c>
     </row>
     <row r="1091">
@@ -12436,7 +12436,7 @@
         <v>951</v>
       </c>
       <c r="C1091" t="n">
-        <v>83632</v>
+        <v>88859</v>
       </c>
     </row>
     <row r="1092">
@@ -12447,7 +12447,7 @@
         <v>2449</v>
       </c>
       <c r="C1092" t="n">
-        <v>29088</v>
+        <v>30906</v>
       </c>
     </row>
     <row r="1093">
@@ -12458,7 +12458,7 @@
         <v>610</v>
       </c>
       <c r="C1093" t="n">
-        <v>592720</v>
+        <v>629765</v>
       </c>
     </row>
     <row r="1094">
@@ -12469,7 +12469,7 @@
         <v>2761</v>
       </c>
       <c r="C1094" t="n">
-        <v>59264</v>
+        <v>62968</v>
       </c>
     </row>
     <row r="1095">
@@ -12480,7 +12480,7 @@
         <v>483</v>
       </c>
       <c r="C1095" t="n">
-        <v>322176</v>
+        <v>342312</v>
       </c>
     </row>
     <row r="1096">
@@ -12491,7 +12491,7 @@
         <v>2015</v>
       </c>
       <c r="C1096" t="n">
-        <v>269088</v>
+        <v>285906</v>
       </c>
     </row>
     <row r="1097">
@@ -12502,7 +12502,7 @@
         <v>1478</v>
       </c>
       <c r="C1097" t="n">
-        <v>393568</v>
+        <v>418166</v>
       </c>
     </row>
     <row r="1098">
@@ -12513,7 +12513,7 @@
         <v>424</v>
       </c>
       <c r="C1098" t="n">
-        <v>175696</v>
+        <v>186677</v>
       </c>
     </row>
     <row r="1099">
@@ -12535,7 +12535,7 @@
         <v>477</v>
       </c>
       <c r="C1100" t="n">
-        <v>188112</v>
+        <v>199869</v>
       </c>
     </row>
     <row r="1101">
@@ -12546,7 +12546,7 @@
         <v>1810</v>
       </c>
       <c r="C1101" t="n">
-        <v>29136</v>
+        <v>30957</v>
       </c>
     </row>
     <row r="1102">
@@ -12557,7 +12557,7 @@
         <v>2826</v>
       </c>
       <c r="C1102" t="n">
-        <v>50909.14</v>
+        <v>54090.95</v>
       </c>
     </row>
     <row r="1103">
@@ -12568,7 +12568,7 @@
         <v>2561</v>
       </c>
       <c r="C1103" t="n">
-        <v>10688</v>
+        <v>11356</v>
       </c>
     </row>
     <row r="1104">
@@ -12579,7 +12579,7 @@
         <v>2653</v>
       </c>
       <c r="C1104" t="n">
-        <v>43636.38</v>
+        <v>46363.65</v>
       </c>
     </row>
     <row r="1105">
@@ -12590,7 +12590,7 @@
         <v>2829</v>
       </c>
       <c r="C1105" t="n">
-        <v>43636.38</v>
+        <v>46363.65</v>
       </c>
     </row>
     <row r="1106">
@@ -12601,7 +12601,7 @@
         <v>2643</v>
       </c>
       <c r="C1106" t="n">
-        <v>21472</v>
+        <v>22814</v>
       </c>
     </row>
     <row r="1107">
@@ -12612,7 +12612,7 @@
         <v>2794</v>
       </c>
       <c r="C1107" t="n">
-        <v>65440</v>
+        <v>69530</v>
       </c>
     </row>
     <row r="1108">
@@ -12623,7 +12623,7 @@
         <v>2655</v>
       </c>
       <c r="C1108" t="n">
-        <v>80000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="1109">
@@ -12634,7 +12634,7 @@
         <v>1456</v>
       </c>
       <c r="C1109" t="n">
-        <v>560208</v>
+        <v>595221</v>
       </c>
     </row>
     <row r="1110">
@@ -12645,7 +12645,7 @@
         <v>2606</v>
       </c>
       <c r="C1110" t="n">
-        <v>172064</v>
+        <v>182818</v>
       </c>
     </row>
     <row r="1111">
@@ -12656,7 +12656,7 @@
         <v>1142</v>
       </c>
       <c r="C1111" t="n">
-        <v>312032</v>
+        <v>331534</v>
       </c>
     </row>
     <row r="1112">
@@ -12667,7 +12667,7 @@
         <v>1450</v>
       </c>
       <c r="C1112" t="n">
-        <v>198224</v>
+        <v>210613</v>
       </c>
     </row>
     <row r="1113">
@@ -12678,7 +12678,7 @@
         <v>2133</v>
       </c>
       <c r="C1113" t="n">
-        <v>462896</v>
+        <v>491827</v>
       </c>
     </row>
     <row r="1114">
@@ -12689,7 +12689,7 @@
         <v>522</v>
       </c>
       <c r="C1114" t="n">
-        <v>141808</v>
+        <v>150671</v>
       </c>
     </row>
     <row r="1115">
@@ -12700,7 +12700,7 @@
         <v>2696</v>
       </c>
       <c r="C1115" t="n">
-        <v>191360</v>
+        <v>203320</v>
       </c>
     </row>
     <row r="1116">
@@ -12722,7 +12722,7 @@
         <v>2692</v>
       </c>
       <c r="C1117" t="n">
-        <v>54544</v>
+        <v>57953</v>
       </c>
     </row>
     <row r="1118">
@@ -12733,7 +12733,7 @@
         <v>2691</v>
       </c>
       <c r="C1118" t="n">
-        <v>98176</v>
+        <v>104312</v>
       </c>
     </row>
     <row r="1119">
@@ -12744,7 +12744,7 @@
         <v>1632</v>
       </c>
       <c r="C1119" t="n">
-        <v>181808</v>
+        <v>193171</v>
       </c>
     </row>
     <row r="1120">
@@ -12755,7 +12755,7 @@
         <v>2641</v>
       </c>
       <c r="C1120" t="n">
-        <v>58176</v>
+        <v>61812</v>
       </c>
     </row>
     <row r="1121">
@@ -12766,7 +12766,7 @@
         <v>2197</v>
       </c>
       <c r="C1121" t="n">
-        <v>145440</v>
+        <v>154530</v>
       </c>
     </row>
     <row r="1122">
@@ -12777,7 +12777,7 @@
         <v>609</v>
       </c>
       <c r="C1122" t="n">
-        <v>160000</v>
+        <v>170000</v>
       </c>
     </row>
     <row r="1123">
@@ -12788,7 +12788,7 @@
         <v>1380</v>
       </c>
       <c r="C1123" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1124">
@@ -12799,7 +12799,7 @@
         <v>104</v>
       </c>
       <c r="C1124" t="n">
-        <v>218176</v>
+        <v>231812</v>
       </c>
     </row>
     <row r="1125">
@@ -12810,7 +12810,7 @@
         <v>2621</v>
       </c>
       <c r="C1125" t="n">
-        <v>50896</v>
+        <v>54077</v>
       </c>
     </row>
     <row r="1126">
@@ -12821,7 +12821,7 @@
         <v>2786</v>
       </c>
       <c r="C1126" t="n">
-        <v>50896</v>
+        <v>54077</v>
       </c>
     </row>
     <row r="1127">
@@ -12832,7 +12832,7 @@
         <v>2784</v>
       </c>
       <c r="C1127" t="n">
-        <v>30256</v>
+        <v>32147</v>
       </c>
     </row>
     <row r="1128">
@@ -12843,7 +12843,7 @@
         <v>2586</v>
       </c>
       <c r="C1128" t="n">
-        <v>30256</v>
+        <v>32147</v>
       </c>
     </row>
     <row r="1129">
@@ -12854,7 +12854,7 @@
         <v>2145</v>
       </c>
       <c r="C1129" t="n">
-        <v>94144</v>
+        <v>100028</v>
       </c>
     </row>
     <row r="1130">
@@ -12865,7 +12865,7 @@
         <v>2574</v>
       </c>
       <c r="C1130" t="n">
-        <v>94144</v>
+        <v>100028</v>
       </c>
     </row>
     <row r="1131">
@@ -12876,7 +12876,7 @@
         <v>2492</v>
       </c>
       <c r="C1131" t="n">
-        <v>103200</v>
+        <v>109650</v>
       </c>
     </row>
     <row r="1132">
@@ -12887,7 +12887,7 @@
         <v>629</v>
       </c>
       <c r="C1132" t="n">
-        <v>321440</v>
+        <v>341530</v>
       </c>
     </row>
     <row r="1133">
@@ -12898,7 +12898,7 @@
         <v>966</v>
       </c>
       <c r="C1133" t="n">
-        <v>59264</v>
+        <v>62968</v>
       </c>
     </row>
     <row r="1134">
@@ -12909,7 +12909,7 @@
         <v>2721</v>
       </c>
       <c r="C1134" t="n">
-        <v>59264</v>
+        <v>62968</v>
       </c>
     </row>
     <row r="1135">
@@ -12920,7 +12920,7 @@
         <v>2554</v>
       </c>
       <c r="C1135" t="n">
-        <v>17856</v>
+        <v>18972</v>
       </c>
     </row>
     <row r="1136">
@@ -12931,7 +12931,7 @@
         <v>2556</v>
       </c>
       <c r="C1136" t="n">
-        <v>26256</v>
+        <v>27897</v>
       </c>
     </row>
     <row r="1137">
@@ -12942,7 +12942,7 @@
         <v>2546</v>
       </c>
       <c r="C1137" t="n">
-        <v>17344</v>
+        <v>18428</v>
       </c>
     </row>
     <row r="1138">
@@ -12953,7 +12953,7 @@
         <v>42</v>
       </c>
       <c r="C1138" t="n">
-        <v>1374544</v>
+        <v>1460453</v>
       </c>
     </row>
     <row r="1139">
@@ -12964,7 +12964,7 @@
         <v>953</v>
       </c>
       <c r="C1139" t="n">
-        <v>496480</v>
+        <v>527510</v>
       </c>
     </row>
     <row r="1140">
@@ -12975,7 +12975,7 @@
         <v>1137</v>
       </c>
       <c r="C1140" t="n">
-        <v>465440</v>
+        <v>494530</v>
       </c>
     </row>
     <row r="1141">
@@ -12986,7 +12986,7 @@
         <v>675</v>
       </c>
       <c r="C1141" t="n">
-        <v>145440</v>
+        <v>154530</v>
       </c>
     </row>
     <row r="1142">
@@ -12997,7 +12997,7 @@
         <v>619</v>
       </c>
       <c r="C1142" t="n">
-        <v>224896</v>
+        <v>238952</v>
       </c>
     </row>
     <row r="1143">
@@ -13008,7 +13008,7 @@
         <v>1299</v>
       </c>
       <c r="C1143" t="n">
-        <v>378432</v>
+        <v>402084</v>
       </c>
     </row>
     <row r="1144">
@@ -13019,7 +13019,7 @@
         <v>1064</v>
       </c>
       <c r="C1144" t="n">
-        <v>435904</v>
+        <v>463148</v>
       </c>
     </row>
     <row r="1145">
@@ -13030,7 +13030,7 @@
         <v>2308</v>
       </c>
       <c r="C1145" t="n">
-        <v>149088</v>
+        <v>158406</v>
       </c>
     </row>
     <row r="1146">
@@ -13041,7 +13041,7 @@
         <v>2747</v>
       </c>
       <c r="C1146" t="n">
-        <v>43636.38</v>
+        <v>46363.65</v>
       </c>
     </row>
     <row r="1147">
@@ -13052,7 +13052,7 @@
         <v>2819</v>
       </c>
       <c r="C1147" t="n">
-        <v>43636.38</v>
+        <v>46363.65</v>
       </c>
     </row>
     <row r="1148">
@@ -13063,7 +13063,7 @@
         <v>1259</v>
       </c>
       <c r="C1148" t="n">
-        <v>72727.3</v>
+        <v>77272.75</v>
       </c>
     </row>
     <row r="1149">
@@ -13074,7 +13074,7 @@
         <v>2544</v>
       </c>
       <c r="C1149" t="n">
-        <v>58176</v>
+        <v>61812</v>
       </c>
     </row>
     <row r="1150">
@@ -13085,7 +13085,7 @@
         <v>2261</v>
       </c>
       <c r="C1150" t="n">
-        <v>109088</v>
+        <v>115906</v>
       </c>
     </row>
     <row r="1151">
@@ -13096,7 +13096,7 @@
         <v>2729</v>
       </c>
       <c r="C1151" t="n">
-        <v>58176</v>
+        <v>61812</v>
       </c>
     </row>
     <row r="1152">
@@ -13107,7 +13107,7 @@
         <v>2649</v>
       </c>
       <c r="C1152" t="n">
-        <v>21472</v>
+        <v>22814</v>
       </c>
     </row>
     <row r="1153">
@@ -13118,7 +13118,7 @@
         <v>2494</v>
       </c>
       <c r="C1153" t="n">
-        <v>94544</v>
+        <v>100453</v>
       </c>
     </row>
     <row r="1154">
@@ -13129,7 +13129,7 @@
         <v>1384</v>
       </c>
       <c r="C1154" t="n">
-        <v>327264</v>
+        <v>347718</v>
       </c>
     </row>
     <row r="1155">
@@ -13151,7 +13151,7 @@
         <v>2802</v>
       </c>
       <c r="C1156" t="n">
-        <v>51504</v>
+        <v>54723</v>
       </c>
     </row>
     <row r="1157">
@@ -13162,7 +13162,7 @@
         <v>2726</v>
       </c>
       <c r="C1157" t="n">
-        <v>109088</v>
+        <v>115906</v>
       </c>
     </row>
     <row r="1158">
@@ -13173,7 +13173,7 @@
         <v>2820</v>
       </c>
       <c r="C1158" t="n">
-        <v>130896</v>
+        <v>139077</v>
       </c>
     </row>
     <row r="1159">
@@ -13184,7 +13184,7 @@
         <v>1007</v>
       </c>
       <c r="C1159" t="n">
-        <v>138176</v>
+        <v>146812</v>
       </c>
     </row>
     <row r="1160">
@@ -13195,7 +13195,7 @@
         <v>20</v>
       </c>
       <c r="C1160" t="n">
-        <v>280000</v>
+        <v>297500</v>
       </c>
     </row>
     <row r="1161">
@@ -13206,7 +13206,7 @@
         <v>1372</v>
       </c>
       <c r="C1161" t="n">
-        <v>210896</v>
+        <v>224077</v>
       </c>
     </row>
     <row r="1162">
@@ -13217,7 +13217,7 @@
         <v>2735</v>
       </c>
       <c r="C1162" t="n">
-        <v>87264</v>
+        <v>92718</v>
       </c>
     </row>
     <row r="1163">
@@ -13228,7 +13228,7 @@
         <v>2811</v>
       </c>
       <c r="C1163" t="n">
-        <v>30256</v>
+        <v>32147</v>
       </c>
     </row>
     <row r="1164">
@@ -13239,7 +13239,7 @@
         <v>1871</v>
       </c>
       <c r="C1164" t="n">
-        <v>128544</v>
+        <v>136578</v>
       </c>
     </row>
     <row r="1165">
@@ -13250,7 +13250,7 @@
         <v>2541</v>
       </c>
       <c r="C1165" t="n">
-        <v>153888</v>
+        <v>163506</v>
       </c>
     </row>
     <row r="1166">
@@ -13261,7 +13261,7 @@
         <v>2362</v>
       </c>
       <c r="C1166" t="n">
-        <v>54544</v>
+        <v>57953</v>
       </c>
     </row>
     <row r="1167">
@@ -13272,7 +13272,7 @@
         <v>1324</v>
       </c>
       <c r="C1167" t="n">
-        <v>203632</v>
+        <v>216359</v>
       </c>
     </row>
     <row r="1168">
@@ -13283,7 +13283,7 @@
         <v>2323</v>
       </c>
       <c r="C1168" t="n">
-        <v>49952</v>
+        <v>53074</v>
       </c>
     </row>
     <row r="1169">
@@ -13294,7 +13294,7 @@
         <v>2647</v>
       </c>
       <c r="C1169" t="n">
-        <v>103200</v>
+        <v>109650</v>
       </c>
     </row>
     <row r="1170">
@@ -13305,7 +13305,7 @@
         <v>559</v>
       </c>
       <c r="C1170" t="n">
-        <v>166864</v>
+        <v>177293</v>
       </c>
     </row>
     <row r="1171">
@@ -13316,7 +13316,7 @@
         <v>2762</v>
       </c>
       <c r="C1171" t="n">
-        <v>59264</v>
+        <v>62968</v>
       </c>
     </row>
     <row r="1172">
@@ -13327,7 +13327,7 @@
         <v>2501</v>
       </c>
       <c r="C1172" t="n">
-        <v>59264</v>
+        <v>62968</v>
       </c>
     </row>
     <row r="1173">
@@ -13338,7 +13338,7 @@
         <v>2562</v>
       </c>
       <c r="C1173" t="n">
-        <v>11504</v>
+        <v>12223</v>
       </c>
     </row>
     <row r="1174">
@@ -13349,7 +13349,7 @@
         <v>429</v>
       </c>
       <c r="C1174" t="n">
-        <v>283632</v>
+        <v>301359</v>
       </c>
     </row>
     <row r="1175">
@@ -13360,7 +13360,7 @@
         <v>58</v>
       </c>
       <c r="C1175" t="n">
-        <v>196784</v>
+        <v>209083</v>
       </c>
     </row>
     <row r="1176">
@@ -13371,7 +13371,7 @@
         <v>2245</v>
       </c>
       <c r="C1176" t="n">
-        <v>175696</v>
+        <v>186677</v>
       </c>
     </row>
     <row r="1177">
@@ -13382,7 +13382,7 @@
         <v>285</v>
       </c>
       <c r="C1177" t="n">
-        <v>393568</v>
+        <v>418166</v>
       </c>
     </row>
     <row r="1178">
@@ -13404,7 +13404,7 @@
         <v>363</v>
       </c>
       <c r="C1179" t="n">
-        <v>218176</v>
+        <v>231812</v>
       </c>
     </row>
     <row r="1180">
@@ -13415,7 +13415,7 @@
         <v>2651</v>
       </c>
       <c r="C1180" t="n">
-        <v>122992</v>
+        <v>130679</v>
       </c>
     </row>
     <row r="1181">
@@ -13426,7 +13426,7 @@
         <v>2142</v>
       </c>
       <c r="C1181" t="n">
-        <v>38816</v>
+        <v>41242</v>
       </c>
     </row>
     <row r="1182">
@@ -13437,7 +13437,7 @@
         <v>2258</v>
       </c>
       <c r="C1182" t="n">
-        <v>58181.84</v>
+        <v>61818.2</v>
       </c>
     </row>
     <row r="1183">
@@ -13448,7 +13448,7 @@
         <v>2772</v>
       </c>
       <c r="C1183" t="n">
-        <v>43636.38</v>
+        <v>46363.65</v>
       </c>
     </row>
     <row r="1184">
@@ -13459,7 +13459,7 @@
         <v>2346</v>
       </c>
       <c r="C1184" t="n">
-        <v>80000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="1185">
@@ -13470,7 +13470,7 @@
         <v>2442</v>
       </c>
       <c r="C1185" t="n">
-        <v>58176</v>
+        <v>61812</v>
       </c>
     </row>
     <row r="1186">
@@ -13481,7 +13481,7 @@
         <v>772</v>
       </c>
       <c r="C1186" t="n">
-        <v>240000</v>
+        <v>255000</v>
       </c>
     </row>
     <row r="1187">
@@ -13492,7 +13492,7 @@
         <v>2684</v>
       </c>
       <c r="C1187" t="n">
-        <v>69088</v>
+        <v>73406</v>
       </c>
     </row>
     <row r="1188">
@@ -13503,7 +13503,7 @@
         <v>2765</v>
       </c>
       <c r="C1188" t="n">
-        <v>65440</v>
+        <v>69530</v>
       </c>
     </row>
     <row r="1189">
@@ -13514,7 +13514,7 @@
         <v>2567</v>
       </c>
       <c r="C1189" t="n">
-        <v>120032</v>
+        <v>127534</v>
       </c>
     </row>
     <row r="1190">
@@ -13525,7 +13525,7 @@
         <v>2178</v>
       </c>
       <c r="C1190" t="n">
-        <v>203632</v>
+        <v>216359</v>
       </c>
     </row>
     <row r="1191">
@@ -13536,7 +13536,7 @@
         <v>2827</v>
       </c>
       <c r="C1191" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1192">
@@ -13547,7 +13547,7 @@
         <v>2510</v>
       </c>
       <c r="C1192" t="n">
-        <v>403808</v>
+        <v>429046</v>
       </c>
     </row>
     <row r="1193">
@@ -13558,7 +13558,7 @@
         <v>2392</v>
       </c>
       <c r="C1193" t="n">
-        <v>121136</v>
+        <v>128707</v>
       </c>
     </row>
     <row r="1194">
@@ -13569,7 +13569,7 @@
         <v>415</v>
       </c>
       <c r="C1194" t="n">
-        <v>414176</v>
+        <v>440062</v>
       </c>
     </row>
     <row r="1195">
@@ -13580,7 +13580,7 @@
         <v>2107</v>
       </c>
       <c r="C1195" t="n">
-        <v>213872</v>
+        <v>227239</v>
       </c>
     </row>
     <row r="1196">
@@ -13591,7 +13591,7 @@
         <v>2211</v>
       </c>
       <c r="C1196" t="n">
-        <v>177312</v>
+        <v>188394</v>
       </c>
     </row>
     <row r="1197">
@@ -13602,7 +13602,7 @@
         <v>2682</v>
       </c>
       <c r="C1197" t="n">
-        <v>109072</v>
+        <v>115889</v>
       </c>
     </row>
     <row r="1198">
@@ -13635,7 +13635,7 @@
         <v>2755</v>
       </c>
       <c r="C1200" t="n">
-        <v>43632</v>
+        <v>46359</v>
       </c>
     </row>
     <row r="1201">
@@ -13646,7 +13646,7 @@
         <v>941</v>
       </c>
       <c r="C1201" t="n">
-        <v>285728</v>
+        <v>303586</v>
       </c>
     </row>
     <row r="1202">
@@ -13657,7 +13657,7 @@
         <v>2734</v>
       </c>
       <c r="C1202" t="n">
-        <v>40048</v>
+        <v>42551</v>
       </c>
     </row>
     <row r="1203">
@@ -13668,7 +13668,7 @@
         <v>1289</v>
       </c>
       <c r="C1203" t="n">
-        <v>181808</v>
+        <v>193171</v>
       </c>
     </row>
     <row r="1204">
@@ -13679,7 +13679,7 @@
         <v>2801</v>
       </c>
       <c r="C1204" t="n">
-        <v>58176</v>
+        <v>61812</v>
       </c>
     </row>
     <row r="1205">
@@ -13690,7 +13690,7 @@
         <v>2810</v>
       </c>
       <c r="C1205" t="n">
-        <v>98176</v>
+        <v>104312</v>
       </c>
     </row>
     <row r="1206">
@@ -13701,7 +13701,7 @@
         <v>767</v>
       </c>
       <c r="C1206" t="n">
-        <v>130896</v>
+        <v>139077</v>
       </c>
     </row>
     <row r="1207">
@@ -13712,7 +13712,7 @@
         <v>2687</v>
       </c>
       <c r="C1207" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1208">
@@ -13723,7 +13723,7 @@
         <v>2686</v>
       </c>
       <c r="C1208" t="n">
-        <v>94544</v>
+        <v>100453</v>
       </c>
     </row>
     <row r="1209">
@@ -13734,7 +13734,7 @@
         <v>2730</v>
       </c>
       <c r="C1209" t="n">
-        <v>65440</v>
+        <v>69530</v>
       </c>
     </row>
     <row r="1210">
@@ -13745,7 +13745,7 @@
         <v>2580</v>
       </c>
       <c r="C1210" t="n">
-        <v>24400</v>
+        <v>25925</v>
       </c>
     </row>
     <row r="1211">
@@ -13756,7 +13756,7 @@
         <v>2472</v>
       </c>
       <c r="C1211" t="n">
-        <v>38503.3</v>
+        <v>40909.75</v>
       </c>
     </row>
     <row r="1212">
@@ -13767,7 +13767,7 @@
         <v>2631</v>
       </c>
       <c r="C1212" t="n">
-        <v>17841.46</v>
+        <v>18956.55</v>
       </c>
     </row>
     <row r="1213">
@@ -13778,7 +13778,7 @@
         <v>1642</v>
       </c>
       <c r="C1213" t="n">
-        <v>192720</v>
+        <v>204765</v>
       </c>
     </row>
     <row r="1214">
@@ -13789,7 +13789,7 @@
         <v>2613</v>
       </c>
       <c r="C1214" t="n">
-        <v>130320</v>
+        <v>138465</v>
       </c>
     </row>
     <row r="1215">
@@ -13800,7 +13800,7 @@
         <v>1020</v>
       </c>
       <c r="C1215" t="n">
-        <v>65440</v>
+        <v>69530</v>
       </c>
     </row>
     <row r="1216">
@@ -13811,7 +13811,7 @@
         <v>2785</v>
       </c>
       <c r="C1216" t="n">
-        <v>30256</v>
+        <v>32147</v>
       </c>
     </row>
     <row r="1217">
@@ -13822,7 +13822,7 @@
         <v>1327</v>
       </c>
       <c r="C1217" t="n">
-        <v>43632</v>
+        <v>46359</v>
       </c>
     </row>
     <row r="1218">
@@ -13833,7 +13833,7 @@
         <v>2629</v>
       </c>
       <c r="C1218" t="n">
-        <v>49952</v>
+        <v>53074</v>
       </c>
     </row>
     <row r="1219">
@@ -13844,7 +13844,7 @@
         <v>749</v>
       </c>
       <c r="C1219" t="n">
-        <v>59264</v>
+        <v>62968</v>
       </c>
     </row>
     <row r="1220">
@@ -13855,7 +13855,7 @@
         <v>1983</v>
       </c>
       <c r="C1220" t="n">
-        <v>393568</v>
+        <v>418166</v>
       </c>
     </row>
     <row r="1221">
@@ -13866,7 +13866,7 @@
         <v>1993</v>
       </c>
       <c r="C1221" t="n">
-        <v>253008</v>
+        <v>268821</v>
       </c>
     </row>
     <row r="1222">
@@ -13877,7 +13877,7 @@
         <v>2767</v>
       </c>
       <c r="C1222" t="n">
-        <v>140304</v>
+        <v>149073</v>
       </c>
     </row>
     <row r="1223">
@@ -13899,7 +13899,7 @@
         <v>1102</v>
       </c>
       <c r="C1224" t="n">
-        <v>175696</v>
+        <v>186677</v>
       </c>
     </row>
     <row r="1225">
@@ -13910,7 +13910,7 @@
         <v>626</v>
       </c>
       <c r="C1225" t="n">
-        <v>1239501.84</v>
+        <v>1316970.7</v>
       </c>
     </row>
     <row r="1226">
@@ -13921,7 +13921,7 @@
         <v>1465</v>
       </c>
       <c r="C1226" t="n">
-        <v>261664</v>
+        <v>278018</v>
       </c>
     </row>
     <row r="1227">
@@ -13932,7 +13932,7 @@
         <v>2758</v>
       </c>
       <c r="C1227" t="n">
-        <v>43636.38</v>
+        <v>46363.65</v>
       </c>
     </row>
     <row r="1228">
@@ -13943,7 +13943,7 @@
         <v>2742</v>
       </c>
       <c r="C1228" t="n">
-        <v>43636.38</v>
+        <v>46363.65</v>
       </c>
     </row>
     <row r="1229">
@@ -13965,7 +13965,7 @@
         <v>1873</v>
       </c>
       <c r="C1230" t="n">
-        <v>232720</v>
+        <v>247265</v>
       </c>
     </row>
     <row r="1231">
@@ -13976,7 +13976,7 @@
         <v>2163</v>
       </c>
       <c r="C1231" t="n">
-        <v>109088</v>
+        <v>115906</v>
       </c>
     </row>
     <row r="1232">
@@ -13987,7 +13987,7 @@
         <v>2394</v>
       </c>
       <c r="C1232" t="n">
-        <v>112032</v>
+        <v>119034</v>
       </c>
     </row>
     <row r="1233">
@@ -13998,7 +13998,7 @@
         <v>33</v>
       </c>
       <c r="C1233" t="n">
-        <v>282176</v>
+        <v>299812</v>
       </c>
     </row>
     <row r="1234">
@@ -14009,7 +14009,7 @@
         <v>2421</v>
       </c>
       <c r="C1234" t="n">
-        <v>47264</v>
+        <v>50218</v>
       </c>
     </row>
     <row r="1235">
@@ -14020,7 +14020,7 @@
         <v>2663</v>
       </c>
       <c r="C1235" t="n">
-        <v>200000</v>
+        <v>212500</v>
       </c>
     </row>
     <row r="1236">
@@ -14031,7 +14031,7 @@
         <v>2413</v>
       </c>
       <c r="C1236" t="n">
-        <v>88032</v>
+        <v>93534</v>
       </c>
     </row>
     <row r="1237">
@@ -14042,7 +14042,7 @@
         <v>351</v>
       </c>
       <c r="C1237" t="n">
-        <v>133808</v>
+        <v>142171</v>
       </c>
     </row>
     <row r="1238">
@@ -14053,7 +14053,7 @@
         <v>1298</v>
       </c>
       <c r="C1238" t="n">
-        <v>925808</v>
+        <v>983671</v>
       </c>
     </row>
     <row r="1239">
@@ -14064,7 +14064,7 @@
         <v>2491</v>
       </c>
       <c r="C1239" t="n">
-        <v>74816</v>
+        <v>79492</v>
       </c>
     </row>
     <row r="1240">
@@ -14075,7 +14075,7 @@
         <v>2571</v>
       </c>
       <c r="C1240" t="n">
-        <v>105648</v>
+        <v>112251</v>
       </c>
     </row>
     <row r="1241">
@@ -14086,7 +14086,7 @@
         <v>2507</v>
       </c>
       <c r="C1241" t="n">
-        <v>64192</v>
+        <v>68204</v>
       </c>
     </row>
     <row r="1242">
@@ -14097,7 +14097,7 @@
         <v>2799</v>
       </c>
       <c r="C1242" t="n">
-        <v>82624</v>
+        <v>87788</v>
       </c>
     </row>
     <row r="1243">
@@ -14119,7 +14119,7 @@
         <v>2582</v>
       </c>
       <c r="C1244" t="n">
-        <v>62944</v>
+        <v>66878</v>
       </c>
     </row>
     <row r="1245">
@@ -14130,7 +14130,7 @@
         <v>2637</v>
       </c>
       <c r="C1245" t="n">
-        <v>45776</v>
+        <v>48637</v>
       </c>
     </row>
     <row r="1246">
@@ -14141,7 +14141,7 @@
         <v>630</v>
       </c>
       <c r="C1246" t="n">
-        <v>108864</v>
+        <v>115668</v>
       </c>
     </row>
     <row r="1247">
@@ -14152,7 +14152,7 @@
         <v>525</v>
       </c>
       <c r="C1247" t="n">
-        <v>163632</v>
+        <v>173859</v>
       </c>
     </row>
     <row r="1248">
@@ -14163,7 +14163,7 @@
         <v>2727</v>
       </c>
       <c r="C1248" t="n">
-        <v>29440</v>
+        <v>31280</v>
       </c>
     </row>
     <row r="1249">
@@ -14174,7 +14174,7 @@
         <v>2707</v>
       </c>
       <c r="C1249" t="n">
-        <v>23296</v>
+        <v>24752</v>
       </c>
     </row>
     <row r="1250">
@@ -14185,7 +14185,7 @@
         <v>2834</v>
       </c>
       <c r="C1250" t="n">
-        <v>12034.92</v>
+        <v>12787.1</v>
       </c>
     </row>
     <row r="1251">
@@ -14196,7 +14196,7 @@
         <v>2773</v>
       </c>
       <c r="C1251" t="n">
-        <v>58685.14</v>
+        <v>62352.95</v>
       </c>
     </row>
     <row r="1252">
@@ -14207,7 +14207,7 @@
         <v>2341</v>
       </c>
       <c r="C1252" t="n">
-        <v>103200</v>
+        <v>109650</v>
       </c>
     </row>
     <row r="1253">
@@ -14218,7 +14218,7 @@
         <v>1374</v>
       </c>
       <c r="C1253" t="n">
-        <v>130896</v>
+        <v>139077</v>
       </c>
     </row>
     <row r="1254">
@@ -14229,7 +14229,7 @@
         <v>793</v>
       </c>
       <c r="C1254" t="n">
-        <v>30256</v>
+        <v>32147</v>
       </c>
     </row>
     <row r="1255">
@@ -14240,7 +14240,7 @@
         <v>794</v>
       </c>
       <c r="C1255" t="n">
-        <v>30256</v>
+        <v>32147</v>
       </c>
     </row>
     <row r="1256">
@@ -14251,7 +14251,7 @@
         <v>1834</v>
       </c>
       <c r="C1256" t="n">
-        <v>85088</v>
+        <v>90406</v>
       </c>
     </row>
     <row r="1257">
@@ -14262,7 +14262,7 @@
         <v>802</v>
       </c>
       <c r="C1257" t="n">
-        <v>54544</v>
+        <v>57953</v>
       </c>
     </row>
     <row r="1258">
@@ -14273,7 +14273,7 @@
         <v>1344</v>
       </c>
       <c r="C1258" t="n">
-        <v>109088</v>
+        <v>115906</v>
       </c>
     </row>
     <row r="1259">
@@ -14284,7 +14284,7 @@
         <v>1881</v>
       </c>
       <c r="C1259" t="n">
-        <v>49952</v>
+        <v>53074</v>
       </c>
     </row>
     <row r="1260">
@@ -14295,7 +14295,7 @@
         <v>2365</v>
       </c>
       <c r="C1260" t="n">
-        <v>57936</v>
+        <v>61557</v>
       </c>
     </row>
     <row r="1261">
@@ -14306,7 +14306,7 @@
         <v>2411</v>
       </c>
       <c r="C1261" t="n">
-        <v>103200</v>
+        <v>109650</v>
       </c>
     </row>
     <row r="1262">
@@ -14317,7 +14317,7 @@
         <v>2363</v>
       </c>
       <c r="C1262" t="n">
-        <v>109088</v>
+        <v>115906</v>
       </c>
     </row>
     <row r="1263">
@@ -14328,7 +14328,7 @@
         <v>2124</v>
       </c>
       <c r="C1263" t="n">
-        <v>254544</v>
+        <v>270453</v>
       </c>
     </row>
     <row r="1264">
@@ -14339,7 +14339,7 @@
         <v>1937</v>
       </c>
       <c r="C1264" t="n">
-        <v>185440</v>
+        <v>197030</v>
       </c>
     </row>
     <row r="1265">
@@ -14350,7 +14350,7 @@
         <v>2709</v>
       </c>
       <c r="C1265" t="n">
-        <v>130896</v>
+        <v>139077</v>
       </c>
     </row>
     <row r="1266">
@@ -14361,7 +14361,7 @@
         <v>2558</v>
       </c>
       <c r="C1266" t="n">
-        <v>21856</v>
+        <v>23222</v>
       </c>
     </row>
     <row r="1267">
@@ -14372,7 +14372,7 @@
         <v>663</v>
       </c>
       <c r="C1267" t="n">
-        <v>185440</v>
+        <v>197030</v>
       </c>
     </row>
     <row r="1268">
@@ -14383,7 +14383,7 @@
         <v>40</v>
       </c>
       <c r="C1268" t="n">
-        <v>160000</v>
+        <v>170000</v>
       </c>
     </row>
     <row r="1269">
@@ -14394,7 +14394,7 @@
         <v>2833</v>
       </c>
       <c r="C1269" t="n">
-        <v>50909.14</v>
+        <v>54090.95</v>
       </c>
     </row>
     <row r="1270">
@@ -14405,7 +14405,7 @@
         <v>1756</v>
       </c>
       <c r="C1270" t="n">
-        <v>317456</v>
+        <v>337297</v>
       </c>
     </row>
     <row r="1271">
@@ -14416,7 +14416,7 @@
         <v>1116</v>
       </c>
       <c r="C1271" t="n">
-        <v>184464</v>
+        <v>195993</v>
       </c>
     </row>
     <row r="1272">
@@ -14427,7 +14427,7 @@
         <v>636</v>
       </c>
       <c r="C1272" t="n">
-        <v>181808</v>
+        <v>193171</v>
       </c>
     </row>
     <row r="1273">
@@ -14438,7 +14438,7 @@
         <v>1800</v>
       </c>
       <c r="C1273" t="n">
-        <v>20352</v>
+        <v>21624</v>
       </c>
     </row>
     <row r="1274">
@@ -14449,7 +14449,7 @@
         <v>2815</v>
       </c>
       <c r="C1274" t="n">
-        <v>43636.38</v>
+        <v>46363.65</v>
       </c>
     </row>
     <row r="1275">
@@ -14460,7 +14460,7 @@
         <v>1658</v>
       </c>
       <c r="C1275" t="n">
-        <v>96000</v>
+        <v>102000</v>
       </c>
     </row>
     <row r="1276">
@@ -14471,7 +14471,7 @@
         <v>2635</v>
       </c>
       <c r="C1276" t="n">
-        <v>94544</v>
+        <v>100453</v>
       </c>
     </row>
     <row r="1277">
@@ -14482,7 +14482,7 @@
         <v>2402</v>
       </c>
       <c r="C1277" t="n">
-        <v>474176</v>
+        <v>503812</v>
       </c>
     </row>
     <row r="1278">
@@ -14493,7 +14493,7 @@
         <v>452</v>
       </c>
       <c r="C1278" t="n">
-        <v>196352</v>
+        <v>208624</v>
       </c>
     </row>
     <row r="1279">
@@ -14504,7 +14504,7 @@
         <v>2085</v>
       </c>
       <c r="C1279" t="n">
-        <v>96032</v>
+        <v>102034</v>
       </c>
     </row>
     <row r="1280">
@@ -14515,7 +14515,7 @@
         <v>2568</v>
       </c>
       <c r="C1280" t="n">
-        <v>148672</v>
+        <v>157964</v>
       </c>
     </row>
     <row r="1281">
@@ -14526,7 +14526,7 @@
         <v>1906</v>
       </c>
       <c r="C1281" t="n">
-        <v>84384</v>
+        <v>89658</v>
       </c>
     </row>
     <row r="1282">
@@ -14537,7 +14537,7 @@
         <v>2821</v>
       </c>
       <c r="C1282" t="n">
-        <v>73376</v>
+        <v>77962</v>
       </c>
     </row>
     <row r="1283">
@@ -14548,7 +14548,7 @@
         <v>2698</v>
       </c>
       <c r="C1283" t="n">
-        <v>89936</v>
+        <v>95557</v>
       </c>
     </row>
     <row r="1284">
@@ -14559,7 +14559,7 @@
         <v>2118</v>
       </c>
       <c r="C1284" t="n">
-        <v>172480</v>
+        <v>183260</v>
       </c>
     </row>
     <row r="1285">
@@ -14570,7 +14570,7 @@
         <v>2383</v>
       </c>
       <c r="C1285" t="n">
-        <v>100704</v>
+        <v>106998</v>
       </c>
     </row>
     <row r="1286">
@@ -14581,7 +14581,7 @@
         <v>2813</v>
       </c>
       <c r="C1286" t="n">
-        <v>45776</v>
+        <v>48637</v>
       </c>
     </row>
     <row r="1287">
@@ -14592,7 +14592,7 @@
         <v>925</v>
       </c>
       <c r="C1287" t="n">
-        <v>57216</v>
+        <v>60792</v>
       </c>
     </row>
     <row r="1288">
@@ -14603,7 +14603,7 @@
         <v>2689</v>
       </c>
       <c r="C1288" t="n">
-        <v>45776</v>
+        <v>48637</v>
       </c>
     </row>
     <row r="1289">
@@ -14614,7 +14614,7 @@
         <v>2716</v>
       </c>
       <c r="C1289" t="n">
-        <v>62944</v>
+        <v>66878</v>
       </c>
     </row>
     <row r="1290">
@@ -14625,7 +14625,7 @@
         <v>2831</v>
       </c>
       <c r="C1290" t="n">
-        <v>43632</v>
+        <v>46359</v>
       </c>
     </row>
     <row r="1291">
@@ -14636,7 +14636,7 @@
         <v>2045</v>
       </c>
       <c r="C1291" t="n">
-        <v>244695.04</v>
+        <v>259988.47</v>
       </c>
     </row>
     <row r="1292">
@@ -14647,7 +14647,7 @@
         <v>580</v>
       </c>
       <c r="C1292" t="n">
-        <v>98176</v>
+        <v>104312</v>
       </c>
     </row>
     <row r="1293">
@@ -14658,7 +14658,7 @@
         <v>438</v>
       </c>
       <c r="C1293" t="n">
-        <v>112720</v>
+        <v>119765</v>
       </c>
     </row>
     <row r="1294">
@@ -14669,7 +14669,7 @@
         <v>1539</v>
       </c>
       <c r="C1294" t="n">
-        <v>123632</v>
+        <v>131359</v>
       </c>
     </row>
     <row r="1295">
@@ -14680,7 +14680,7 @@
         <v>2817</v>
       </c>
       <c r="C1295" t="n">
-        <v>43632</v>
+        <v>46359</v>
       </c>
     </row>
     <row r="1296">
@@ -14691,7 +14691,7 @@
         <v>2816</v>
       </c>
       <c r="C1296" t="n">
-        <v>94544</v>
+        <v>100453</v>
       </c>
     </row>
     <row r="1297">
@@ -14702,7 +14702,7 @@
         <v>2146</v>
       </c>
       <c r="C1297" t="n">
-        <v>146656</v>
+        <v>155822</v>
       </c>
     </row>
     <row r="1298">
@@ -14713,7 +14713,7 @@
         <v>2276</v>
       </c>
       <c r="C1298" t="n">
-        <v>162944</v>
+        <v>173128</v>
       </c>
     </row>
     <row r="1299">
@@ -14724,7 +14724,7 @@
         <v>1381</v>
       </c>
       <c r="C1299" t="n">
-        <v>214544</v>
+        <v>227953</v>
       </c>
     </row>
     <row r="1300">
@@ -14735,7 +14735,7 @@
         <v>2081</v>
       </c>
       <c r="C1300" t="n">
-        <v>109088</v>
+        <v>115906</v>
       </c>
     </row>
     <row r="1301">
@@ -14746,7 +14746,7 @@
         <v>14</v>
       </c>
       <c r="C1301" t="n">
-        <v>316352</v>
+        <v>336124</v>
       </c>
     </row>
     <row r="1302">
@@ -14757,7 +14757,7 @@
         <v>766</v>
       </c>
       <c r="C1302" t="n">
-        <v>49952</v>
+        <v>53074</v>
       </c>
     </row>
     <row r="1303">
@@ -14768,7 +14768,7 @@
         <v>2547</v>
       </c>
       <c r="C1303" t="n">
-        <v>29904</v>
+        <v>31773</v>
       </c>
     </row>
     <row r="1304">
@@ -14779,7 +14779,7 @@
         <v>2552</v>
       </c>
       <c r="C1304" t="n">
-        <v>21504</v>
+        <v>22848</v>
       </c>
     </row>
     <row r="1305">
@@ -14790,7 +14790,7 @@
         <v>131</v>
       </c>
       <c r="C1305" t="n">
-        <v>297440</v>
+        <v>316030</v>
       </c>
     </row>
     <row r="1306">
@@ -14801,7 +14801,7 @@
         <v>2250</v>
       </c>
       <c r="C1306" t="n">
-        <v>240656</v>
+        <v>255697</v>
       </c>
     </row>
     <row r="1307">
@@ -14812,7 +14812,7 @@
         <v>89</v>
       </c>
       <c r="C1307" t="n">
-        <v>245952</v>
+        <v>261324</v>
       </c>
     </row>
     <row r="1308">
@@ -14823,7 +14823,7 @@
         <v>2141</v>
       </c>
       <c r="C1308" t="n">
-        <v>23008</v>
+        <v>24446</v>
       </c>
     </row>
     <row r="1309">
@@ -14834,7 +14834,7 @@
         <v>2798</v>
       </c>
       <c r="C1309" t="n">
-        <v>43636.38</v>
+        <v>46363.65</v>
       </c>
     </row>
     <row r="1310">
@@ -14845,7 +14845,7 @@
         <v>2797</v>
       </c>
       <c r="C1310" t="n">
-        <v>43636.38</v>
+        <v>46363.65</v>
       </c>
     </row>
     <row r="1311">
@@ -14856,7 +14856,7 @@
         <v>2266</v>
       </c>
       <c r="C1311" t="n">
-        <v>58181.84</v>
+        <v>61818.2</v>
       </c>
     </row>
     <row r="1312">
@@ -14867,7 +14867,7 @@
         <v>1499</v>
       </c>
       <c r="C1312" t="n">
-        <v>101808</v>
+        <v>108171</v>
       </c>
     </row>
     <row r="1313">
@@ -14878,7 +14878,7 @@
         <v>2496</v>
       </c>
       <c r="C1313" t="n">
-        <v>116352</v>
+        <v>123624</v>
       </c>
     </row>
     <row r="1314">
@@ -14889,7 +14889,7 @@
         <v>949</v>
       </c>
       <c r="C1314" t="n">
-        <v>71376</v>
+        <v>75837</v>
       </c>
     </row>
     <row r="1315">
@@ -14900,7 +14900,7 @@
         <v>1853</v>
       </c>
       <c r="C1315" t="n">
-        <v>87264</v>
+        <v>92718</v>
       </c>
     </row>
     <row r="1316">
@@ -14911,7 +14911,7 @@
         <v>854</v>
       </c>
       <c r="C1316" t="n">
-        <v>80000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="1317">
@@ -14922,7 +14922,7 @@
         <v>2674</v>
       </c>
       <c r="C1317" t="n">
-        <v>189088</v>
+        <v>200906</v>
       </c>
     </row>
     <row r="1318">
@@ -14933,7 +14933,7 @@
         <v>2803</v>
       </c>
       <c r="C1318" t="n">
-        <v>87264</v>
+        <v>92718</v>
       </c>
     </row>
     <row r="1319">
@@ -14944,7 +14944,7 @@
         <v>2599</v>
       </c>
       <c r="C1319" t="n">
-        <v>138176</v>
+        <v>146812</v>
       </c>
     </row>
     <row r="1320">
@@ -14955,7 +14955,7 @@
         <v>783</v>
       </c>
       <c r="C1320" t="n">
-        <v>37808</v>
+        <v>40171</v>
       </c>
     </row>
     <row r="1321">
@@ -14966,7 +14966,7 @@
         <v>27</v>
       </c>
       <c r="C1321" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1322">
@@ -14977,7 +14977,7 @@
         <v>531</v>
       </c>
       <c r="C1322" t="n">
-        <v>254544</v>
+        <v>270453</v>
       </c>
     </row>
     <row r="1323">
@@ -14988,7 +14988,7 @@
         <v>1308</v>
       </c>
       <c r="C1323" t="n">
-        <v>117472</v>
+        <v>124814</v>
       </c>
     </row>
     <row r="1324">
@@ -14999,7 +14999,7 @@
         <v>2792</v>
       </c>
       <c r="C1324" t="n">
-        <v>84720</v>
+        <v>90015</v>
       </c>
     </row>
     <row r="1325">
@@ -15021,7 +15021,7 @@
         <v>2823</v>
       </c>
       <c r="C1326" t="n">
-        <v>68000</v>
+        <v>72250</v>
       </c>
     </row>
     <row r="1327">
@@ -15032,7 +15032,7 @@
         <v>2584</v>
       </c>
       <c r="C1327" t="n">
-        <v>45776</v>
+        <v>48637</v>
       </c>
     </row>
     <row r="1328">
@@ -15043,7 +15043,7 @@
         <v>945</v>
       </c>
       <c r="C1328" t="n">
-        <v>206048</v>
+        <v>218926</v>
       </c>
     </row>
     <row r="1329">
@@ -15054,7 +15054,7 @@
         <v>2660</v>
       </c>
       <c r="C1329" t="n">
-        <v>225440</v>
+        <v>239530</v>
       </c>
     </row>
     <row r="1330">
@@ -15065,7 +15065,7 @@
         <v>1317</v>
       </c>
       <c r="C1330" t="n">
-        <v>218176</v>
+        <v>231812</v>
       </c>
     </row>
     <row r="1331">
@@ -15076,7 +15076,7 @@
         <v>2790</v>
       </c>
       <c r="C1331" t="n">
-        <v>46320</v>
+        <v>49215</v>
       </c>
     </row>
     <row r="1332">
@@ -15087,7 +15087,7 @@
         <v>2711</v>
       </c>
       <c r="C1332" t="n">
-        <v>63045.84</v>
+        <v>66986.2</v>
       </c>
     </row>
     <row r="1333">
@@ -15098,7 +15098,7 @@
         <v>2607</v>
       </c>
       <c r="C1333" t="n">
-        <v>36133.84</v>
+        <v>38392.2</v>
       </c>
     </row>
     <row r="1334">
@@ -15109,7 +15109,7 @@
         <v>2667</v>
       </c>
       <c r="C1334" t="n">
-        <v>33236.38</v>
+        <v>35313.65</v>
       </c>
     </row>
     <row r="1335">
@@ -15120,7 +15120,7 @@
         <v>2706</v>
       </c>
       <c r="C1335" t="n">
-        <v>16023.3</v>
+        <v>17024.75</v>
       </c>
     </row>
     <row r="1336">
@@ -15131,7 +15131,7 @@
         <v>2657</v>
       </c>
       <c r="C1336" t="n">
-        <v>57597.14</v>
+        <v>61196.95</v>
       </c>
     </row>
     <row r="1337">
@@ -15142,7 +15142,7 @@
         <v>1278</v>
       </c>
       <c r="C1337" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1338">
@@ -15153,7 +15153,7 @@
         <v>2745</v>
       </c>
       <c r="C1338" t="n">
-        <v>80000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="1339">
@@ -15164,7 +15164,7 @@
         <v>2753</v>
       </c>
       <c r="C1339" t="n">
-        <v>54544</v>
+        <v>57953</v>
       </c>
     </row>
     <row r="1340">
@@ -15175,7 +15175,7 @@
         <v>2183</v>
       </c>
       <c r="C1340" t="n">
-        <v>266144</v>
+        <v>282778</v>
       </c>
     </row>
     <row r="1341">
@@ -15186,7 +15186,7 @@
         <v>1340</v>
       </c>
       <c r="C1341" t="n">
-        <v>105440</v>
+        <v>112030</v>
       </c>
     </row>
     <row r="1342">
@@ -15197,7 +15197,7 @@
         <v>2583</v>
       </c>
       <c r="C1342" t="n">
-        <v>30256</v>
+        <v>32147</v>
       </c>
     </row>
     <row r="1343">
@@ -15208,7 +15208,7 @@
         <v>2090</v>
       </c>
       <c r="C1343" t="n">
-        <v>30256</v>
+        <v>32147</v>
       </c>
     </row>
     <row r="1344">
@@ -15219,7 +15219,7 @@
         <v>1277</v>
       </c>
       <c r="C1344" t="n">
-        <v>160000</v>
+        <v>170000</v>
       </c>
     </row>
     <row r="1345">
@@ -15230,7 +15230,7 @@
         <v>1501</v>
       </c>
       <c r="C1345" t="n">
-        <v>69088</v>
+        <v>73406</v>
       </c>
     </row>
     <row r="1346">
@@ -15241,7 +15241,7 @@
         <v>703</v>
       </c>
       <c r="C1346" t="n">
-        <v>181808</v>
+        <v>193171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:18:12
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -11292,7 +11292,7 @@
         <v>947</v>
       </c>
       <c r="C987" t="n">
-        <v>335767</v>
+        <v>355518</v>
       </c>
     </row>
     <row r="988">
@@ -11303,7 +11303,7 @@
         <v>1956</v>
       </c>
       <c r="C988" t="n">
-        <v>195092</v>
+        <v>206568</v>
       </c>
     </row>
     <row r="989">
@@ -11314,7 +11314,7 @@
         <v>2824</v>
       </c>
       <c r="C989" t="n">
-        <v>85000</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="990">
@@ -11325,7 +11325,7 @@
         <v>2787</v>
       </c>
       <c r="C990" t="n">
-        <v>100453</v>
+        <v>106362</v>
       </c>
     </row>
     <row r="991">
@@ -11336,7 +11336,7 @@
         <v>2830</v>
       </c>
       <c r="C991" t="n">
-        <v>69530</v>
+        <v>73620</v>
       </c>
     </row>
     <row r="992">
@@ -11347,7 +11347,7 @@
         <v>1254</v>
       </c>
       <c r="C992" t="n">
-        <v>150060.55</v>
+        <v>158887.64</v>
       </c>
     </row>
     <row r="993">
@@ -11358,7 +11358,7 @@
         <v>816</v>
       </c>
       <c r="C993" t="n">
-        <v>206975</v>
+        <v>219150</v>
       </c>
     </row>
     <row r="994">
@@ -11369,7 +11369,7 @@
         <v>2671</v>
       </c>
       <c r="C994" t="n">
-        <v>61812</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="995">
@@ -11380,7 +11380,7 @@
         <v>2705</v>
       </c>
       <c r="C995" t="n">
-        <v>138465</v>
+        <v>146610</v>
       </c>
     </row>
     <row r="996">
@@ -11391,7 +11391,7 @@
         <v>2333</v>
       </c>
       <c r="C996" t="n">
-        <v>119272</v>
+        <v>126288</v>
       </c>
     </row>
     <row r="997">
@@ -11402,7 +11402,7 @@
         <v>2440</v>
       </c>
       <c r="C997" t="n">
-        <v>69530</v>
+        <v>73620</v>
       </c>
     </row>
     <row r="998">
@@ -11413,7 +11413,7 @@
         <v>2448</v>
       </c>
       <c r="C998" t="n">
-        <v>15453</v>
+        <v>16362</v>
       </c>
     </row>
     <row r="999">
@@ -11424,7 +11424,7 @@
         <v>2310</v>
       </c>
       <c r="C999" t="n">
-        <v>53074</v>
+        <v>56196</v>
       </c>
     </row>
     <row r="1000">
@@ -11435,7 +11435,7 @@
         <v>2809</v>
       </c>
       <c r="C1000" t="n">
-        <v>53074</v>
+        <v>56196</v>
       </c>
     </row>
     <row r="1001">
@@ -11446,7 +11446,7 @@
         <v>2548</v>
       </c>
       <c r="C1001" t="n">
-        <v>45220</v>
+        <v>47880</v>
       </c>
     </row>
     <row r="1002">
@@ -11457,7 +11457,7 @@
         <v>451</v>
       </c>
       <c r="C1002" t="n">
-        <v>185453</v>
+        <v>196362</v>
       </c>
     </row>
     <row r="1003">
@@ -11468,7 +11468,7 @@
         <v>933</v>
       </c>
       <c r="C1003" t="n">
-        <v>62968</v>
+        <v>66672</v>
       </c>
     </row>
     <row r="1004">
@@ -11479,7 +11479,7 @@
         <v>2702</v>
       </c>
       <c r="C1004" t="n">
-        <v>62968</v>
+        <v>66672</v>
       </c>
     </row>
     <row r="1005">
@@ -11490,7 +11490,7 @@
         <v>2549</v>
       </c>
       <c r="C1005" t="n">
-        <v>21896</v>
+        <v>23184</v>
       </c>
     </row>
     <row r="1006">
@@ -11501,7 +11501,7 @@
         <v>535</v>
       </c>
       <c r="C1006" t="n">
-        <v>285906</v>
+        <v>302724</v>
       </c>
     </row>
     <row r="1007">
@@ -11512,7 +11512,7 @@
         <v>1117</v>
       </c>
       <c r="C1007" t="n">
-        <v>268821</v>
+        <v>284634</v>
       </c>
     </row>
     <row r="1008">
@@ -11534,7 +11534,7 @@
         <v>530</v>
       </c>
       <c r="C1009" t="n">
-        <v>188598</v>
+        <v>199692</v>
       </c>
     </row>
     <row r="1010">
@@ -11545,7 +11545,7 @@
         <v>358</v>
       </c>
       <c r="C1010" t="n">
-        <v>262718</v>
+        <v>278172</v>
       </c>
     </row>
     <row r="1011">
@@ -11556,7 +11556,7 @@
         <v>2498</v>
       </c>
       <c r="C1011" t="n">
-        <v>42908</v>
+        <v>45432</v>
       </c>
     </row>
     <row r="1012">
@@ -11567,7 +11567,7 @@
         <v>2381</v>
       </c>
       <c r="C1012" t="n">
-        <v>61302</v>
+        <v>64908</v>
       </c>
     </row>
     <row r="1013">
@@ -11578,7 +11578,7 @@
         <v>2695</v>
       </c>
       <c r="C1013" t="n">
-        <v>36873</v>
+        <v>39042</v>
       </c>
     </row>
     <row r="1014">
@@ -11589,7 +11589,7 @@
         <v>2744</v>
       </c>
       <c r="C1014" t="n">
-        <v>46363.65</v>
+        <v>49090.92</v>
       </c>
     </row>
     <row r="1015">
@@ -11600,7 +11600,7 @@
         <v>2750</v>
       </c>
       <c r="C1015" t="n">
-        <v>46359</v>
+        <v>49086</v>
       </c>
     </row>
     <row r="1016">
@@ -11611,7 +11611,7 @@
         <v>2131</v>
       </c>
       <c r="C1016" t="n">
-        <v>92718</v>
+        <v>98172</v>
       </c>
     </row>
     <row r="1017">
@@ -11622,7 +11622,7 @@
         <v>818</v>
       </c>
       <c r="C1017" t="n">
-        <v>309077</v>
+        <v>327258</v>
       </c>
     </row>
     <row r="1018">
@@ -11633,7 +11633,7 @@
         <v>2566</v>
       </c>
       <c r="C1018" t="n">
-        <v>61812</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1019">
@@ -11644,7 +11644,7 @@
         <v>132</v>
       </c>
       <c r="C1019" t="n">
-        <v>579530</v>
+        <v>613620</v>
       </c>
     </row>
     <row r="1020">
@@ -11655,7 +11655,7 @@
         <v>2431</v>
       </c>
       <c r="C1020" t="n">
-        <v>142171</v>
+        <v>150534</v>
       </c>
     </row>
     <row r="1021">
@@ -11666,7 +11666,7 @@
         <v>2249</v>
       </c>
       <c r="C1021" t="n">
-        <v>150926</v>
+        <v>159804</v>
       </c>
     </row>
     <row r="1022">
@@ -11677,7 +11677,7 @@
         <v>1585</v>
       </c>
       <c r="C1022" t="n">
-        <v>127534</v>
+        <v>135036</v>
       </c>
     </row>
     <row r="1023">
@@ -11688,7 +11688,7 @@
         <v>2325</v>
       </c>
       <c r="C1023" t="n">
-        <v>123284</v>
+        <v>130536</v>
       </c>
     </row>
     <row r="1024">
@@ -11699,7 +11699,7 @@
         <v>2190</v>
       </c>
       <c r="C1024" t="n">
-        <v>173859</v>
+        <v>184086</v>
       </c>
     </row>
     <row r="1025">
@@ -11710,7 +11710,7 @@
         <v>1466</v>
       </c>
       <c r="C1025" t="n">
-        <v>312953</v>
+        <v>331362</v>
       </c>
     </row>
     <row r="1026">
@@ -11721,7 +11721,7 @@
         <v>2659</v>
       </c>
       <c r="C1026" t="n">
-        <v>95047</v>
+        <v>100638</v>
       </c>
     </row>
     <row r="1027">
@@ -11732,7 +11732,7 @@
         <v>634</v>
       </c>
       <c r="C1027" t="n">
-        <v>425000</v>
+        <v>450000</v>
       </c>
     </row>
     <row r="1028">
@@ -11743,7 +11743,7 @@
         <v>2804</v>
       </c>
       <c r="C1028" t="n">
-        <v>77265</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1029">
@@ -11754,7 +11754,7 @@
         <v>2375</v>
       </c>
       <c r="C1029" t="n">
-        <v>255000</v>
+        <v>270000</v>
       </c>
     </row>
     <row r="1030">
@@ -11765,7 +11765,7 @@
         <v>2601</v>
       </c>
       <c r="C1030" t="n">
-        <v>212500</v>
+        <v>225000</v>
       </c>
     </row>
     <row r="1031">
@@ -11776,7 +11776,7 @@
         <v>952</v>
       </c>
       <c r="C1031" t="n">
-        <v>77265</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1032">
@@ -11787,7 +11787,7 @@
         <v>571</v>
       </c>
       <c r="C1032" t="n">
-        <v>491827</v>
+        <v>520758</v>
       </c>
     </row>
     <row r="1033">
@@ -11798,7 +11798,7 @@
         <v>2697</v>
       </c>
       <c r="C1033" t="n">
-        <v>149855</v>
+        <v>158670</v>
       </c>
     </row>
     <row r="1034">
@@ -11809,7 +11809,7 @@
         <v>2678</v>
       </c>
       <c r="C1034" t="n">
-        <v>259267</v>
+        <v>274518</v>
       </c>
     </row>
     <row r="1035">
@@ -11820,7 +11820,7 @@
         <v>2768</v>
       </c>
       <c r="C1035" t="n">
-        <v>271337</v>
+        <v>287298</v>
       </c>
     </row>
     <row r="1036">
@@ -11831,7 +11831,7 @@
         <v>2359</v>
       </c>
       <c r="C1036" t="n">
-        <v>82297</v>
+        <v>87138</v>
       </c>
     </row>
     <row r="1037">
@@ -11842,7 +11842,7 @@
         <v>353</v>
       </c>
       <c r="C1037" t="n">
-        <v>267342</v>
+        <v>283068</v>
       </c>
     </row>
     <row r="1038">
@@ -11853,7 +11853,7 @@
         <v>2026</v>
       </c>
       <c r="C1038" t="n">
-        <v>221510</v>
+        <v>234540</v>
       </c>
     </row>
     <row r="1039">
@@ -11875,7 +11875,7 @@
         <v>2345</v>
       </c>
       <c r="C1040" t="n">
-        <v>48637</v>
+        <v>51498</v>
       </c>
     </row>
     <row r="1041">
@@ -11886,7 +11886,7 @@
         <v>2789</v>
       </c>
       <c r="C1041" t="n">
-        <v>131359</v>
+        <v>139086</v>
       </c>
     </row>
     <row r="1042">
@@ -11897,7 +11897,7 @@
         <v>569</v>
       </c>
       <c r="C1042" t="n">
-        <v>2213026</v>
+        <v>2343204</v>
       </c>
     </row>
     <row r="1043">
@@ -11908,7 +11908,7 @@
         <v>2822</v>
       </c>
       <c r="C1043" t="n">
-        <v>104312</v>
+        <v>110448</v>
       </c>
     </row>
     <row r="1044">
@@ -11919,7 +11919,7 @@
         <v>2728</v>
       </c>
       <c r="C1044" t="n">
-        <v>7718</v>
+        <v>8172</v>
       </c>
     </row>
     <row r="1045">
@@ -11930,7 +11930,7 @@
         <v>2488</v>
       </c>
       <c r="C1045" t="n">
-        <v>77265</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1046">
@@ -11941,7 +11941,7 @@
         <v>2791</v>
       </c>
       <c r="C1046" t="n">
-        <v>76260.5</v>
+        <v>80746.39999999999</v>
       </c>
     </row>
     <row r="1047">
@@ -11952,7 +11952,7 @@
         <v>2577</v>
       </c>
       <c r="C1047" t="n">
-        <v>68904.19</v>
+        <v>72957.37</v>
       </c>
     </row>
     <row r="1048">
@@ -11963,7 +11963,7 @@
         <v>2069</v>
       </c>
       <c r="C1048" t="n">
-        <v>139077</v>
+        <v>147258</v>
       </c>
     </row>
     <row r="1049">
@@ -11974,7 +11974,7 @@
         <v>2082</v>
       </c>
       <c r="C1049" t="n">
-        <v>128707</v>
+        <v>136278</v>
       </c>
     </row>
     <row r="1050">
@@ -11985,7 +11985,7 @@
         <v>781</v>
       </c>
       <c r="C1050" t="n">
-        <v>100453</v>
+        <v>106362</v>
       </c>
     </row>
     <row r="1051">
@@ -11996,7 +11996,7 @@
         <v>744</v>
       </c>
       <c r="C1051" t="n">
-        <v>32147</v>
+        <v>34038</v>
       </c>
     </row>
     <row r="1052">
@@ -12007,7 +12007,7 @@
         <v>2223</v>
       </c>
       <c r="C1052" t="n">
-        <v>101949</v>
+        <v>107946</v>
       </c>
     </row>
     <row r="1053">
@@ -12018,7 +12018,7 @@
         <v>2452</v>
       </c>
       <c r="C1053" t="n">
-        <v>54077</v>
+        <v>57258</v>
       </c>
     </row>
     <row r="1054">
@@ -12029,7 +12029,7 @@
         <v>970</v>
       </c>
       <c r="C1054" t="n">
-        <v>53074</v>
+        <v>56196</v>
       </c>
     </row>
     <row r="1055">
@@ -12040,7 +12040,7 @@
         <v>2550</v>
       </c>
       <c r="C1055" t="n">
-        <v>47124</v>
+        <v>49896</v>
       </c>
     </row>
     <row r="1056">
@@ -12051,7 +12051,7 @@
         <v>768</v>
       </c>
       <c r="C1056" t="n">
-        <v>100453</v>
+        <v>106362</v>
       </c>
     </row>
     <row r="1057">
@@ -12062,7 +12062,7 @@
         <v>1075</v>
       </c>
       <c r="C1057" t="n">
-        <v>350030</v>
+        <v>370620</v>
       </c>
     </row>
     <row r="1058">
@@ -12073,7 +12073,7 @@
         <v>664</v>
       </c>
       <c r="C1058" t="n">
-        <v>200124</v>
+        <v>211896</v>
       </c>
     </row>
     <row r="1059">
@@ -12084,7 +12084,7 @@
         <v>2555</v>
       </c>
       <c r="C1059" t="n">
-        <v>32079</v>
+        <v>33966</v>
       </c>
     </row>
     <row r="1060">
@@ -12095,7 +12095,7 @@
         <v>2627</v>
       </c>
       <c r="C1060" t="n">
-        <v>18836</v>
+        <v>19944</v>
       </c>
     </row>
     <row r="1061">
@@ -12106,7 +12106,7 @@
         <v>2557</v>
       </c>
       <c r="C1061" t="n">
-        <v>19924</v>
+        <v>21096</v>
       </c>
     </row>
     <row r="1062">
@@ -12117,7 +12117,7 @@
         <v>2551</v>
       </c>
       <c r="C1062" t="n">
-        <v>15827</v>
+        <v>16758</v>
       </c>
     </row>
     <row r="1063">
@@ -12128,7 +12128,7 @@
         <v>2463</v>
       </c>
       <c r="C1063" t="n">
-        <v>247435</v>
+        <v>261990</v>
       </c>
     </row>
     <row r="1064">
@@ -12139,7 +12139,7 @@
         <v>2279</v>
       </c>
       <c r="C1064" t="n">
-        <v>186677</v>
+        <v>197658</v>
       </c>
     </row>
     <row r="1065">
@@ -12150,7 +12150,7 @@
         <v>631</v>
       </c>
       <c r="C1065" t="n">
-        <v>270453</v>
+        <v>286362</v>
       </c>
     </row>
     <row r="1066">
@@ -12161,7 +12161,7 @@
         <v>2251</v>
       </c>
       <c r="C1066" t="n">
-        <v>165614</v>
+        <v>175356</v>
       </c>
     </row>
     <row r="1067">
@@ -12172,7 +12172,7 @@
         <v>1653</v>
       </c>
       <c r="C1067" t="n">
-        <v>251124</v>
+        <v>265896</v>
       </c>
     </row>
     <row r="1068">
@@ -12183,7 +12183,7 @@
         <v>1293</v>
       </c>
       <c r="C1068" t="n">
-        <v>320671</v>
+        <v>339534</v>
       </c>
     </row>
     <row r="1069">
@@ -12194,7 +12194,7 @@
         <v>360</v>
       </c>
       <c r="C1069" t="n">
-        <v>386359</v>
+        <v>409086</v>
       </c>
     </row>
     <row r="1070">
@@ -12205,7 +12205,7 @@
         <v>1063</v>
       </c>
       <c r="C1070" t="n">
-        <v>280925</v>
+        <v>297450</v>
       </c>
     </row>
     <row r="1071">
@@ -12216,7 +12216,7 @@
         <v>2273</v>
       </c>
       <c r="C1071" t="n">
-        <v>163880</v>
+        <v>173520</v>
       </c>
     </row>
     <row r="1072">
@@ -12227,7 +12227,7 @@
         <v>2757</v>
       </c>
       <c r="C1072" t="n">
-        <v>54090.95</v>
+        <v>57272.76</v>
       </c>
     </row>
     <row r="1073">
@@ -12238,7 +12238,7 @@
         <v>2795</v>
       </c>
       <c r="C1073" t="n">
-        <v>46363.65</v>
+        <v>49090.92</v>
       </c>
     </row>
     <row r="1074">
@@ -12249,7 +12249,7 @@
         <v>2722</v>
       </c>
       <c r="C1074" t="n">
-        <v>46359</v>
+        <v>49086</v>
       </c>
     </row>
     <row r="1075">
@@ -12260,7 +12260,7 @@
         <v>2718</v>
       </c>
       <c r="C1075" t="n">
-        <v>61812</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1076">
@@ -12271,7 +12271,7 @@
         <v>595</v>
       </c>
       <c r="C1076" t="n">
-        <v>425000</v>
+        <v>450000</v>
       </c>
     </row>
     <row r="1077">
@@ -12282,7 +12282,7 @@
         <v>890</v>
       </c>
       <c r="C1077" t="n">
-        <v>540906</v>
+        <v>572724</v>
       </c>
     </row>
     <row r="1078">
@@ -12293,7 +12293,7 @@
         <v>2652</v>
       </c>
       <c r="C1078" t="n">
-        <v>100453</v>
+        <v>106362</v>
       </c>
     </row>
     <row r="1079">
@@ -12304,7 +12304,7 @@
         <v>2714</v>
       </c>
       <c r="C1079" t="n">
-        <v>278171</v>
+        <v>294534</v>
       </c>
     </row>
     <row r="1080">
@@ -12315,7 +12315,7 @@
         <v>1869</v>
       </c>
       <c r="C1080" t="n">
-        <v>177718</v>
+        <v>188172</v>
       </c>
     </row>
     <row r="1081">
@@ -12326,7 +12326,7 @@
         <v>400</v>
       </c>
       <c r="C1081" t="n">
-        <v>146812</v>
+        <v>155448</v>
       </c>
     </row>
     <row r="1082">
@@ -12337,7 +12337,7 @@
         <v>1907</v>
       </c>
       <c r="C1082" t="n">
-        <v>286671</v>
+        <v>303534</v>
       </c>
     </row>
     <row r="1083">
@@ -12348,7 +12348,7 @@
         <v>1996</v>
       </c>
       <c r="C1083" t="n">
-        <v>181203</v>
+        <v>191862</v>
       </c>
     </row>
     <row r="1084">
@@ -12359,7 +12359,7 @@
         <v>1890</v>
       </c>
       <c r="C1084" t="n">
-        <v>244292.08</v>
+        <v>258662.19</v>
       </c>
     </row>
     <row r="1085">
@@ -12370,7 +12370,7 @@
         <v>2114</v>
       </c>
       <c r="C1085" t="n">
-        <v>141950</v>
+        <v>150300</v>
       </c>
     </row>
     <row r="1086">
@@ -12381,7 +12381,7 @@
         <v>2330</v>
       </c>
       <c r="C1086" t="n">
-        <v>207689</v>
+        <v>219906</v>
       </c>
     </row>
     <row r="1087">
@@ -12425,7 +12425,7 @@
         <v>931</v>
       </c>
       <c r="C1090" t="n">
-        <v>72964</v>
+        <v>77256</v>
       </c>
     </row>
     <row r="1091">
@@ -12436,7 +12436,7 @@
         <v>951</v>
       </c>
       <c r="C1091" t="n">
-        <v>88859</v>
+        <v>94086</v>
       </c>
     </row>
     <row r="1092">
@@ -12447,7 +12447,7 @@
         <v>2449</v>
       </c>
       <c r="C1092" t="n">
-        <v>30906</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1093">
@@ -12458,7 +12458,7 @@
         <v>610</v>
       </c>
       <c r="C1093" t="n">
-        <v>629765</v>
+        <v>666810</v>
       </c>
     </row>
     <row r="1094">
@@ -12469,7 +12469,7 @@
         <v>2761</v>
       </c>
       <c r="C1094" t="n">
-        <v>62968</v>
+        <v>66672</v>
       </c>
     </row>
     <row r="1095">
@@ -12480,7 +12480,7 @@
         <v>483</v>
       </c>
       <c r="C1095" t="n">
-        <v>342312</v>
+        <v>362448</v>
       </c>
     </row>
     <row r="1096">
@@ -12491,7 +12491,7 @@
         <v>2015</v>
       </c>
       <c r="C1096" t="n">
-        <v>285906</v>
+        <v>302724</v>
       </c>
     </row>
     <row r="1097">
@@ -12502,7 +12502,7 @@
         <v>1478</v>
       </c>
       <c r="C1097" t="n">
-        <v>418166</v>
+        <v>442764</v>
       </c>
     </row>
     <row r="1098">
@@ -12513,7 +12513,7 @@
         <v>424</v>
       </c>
       <c r="C1098" t="n">
-        <v>186677</v>
+        <v>197658</v>
       </c>
     </row>
     <row r="1099">
@@ -12535,7 +12535,7 @@
         <v>477</v>
       </c>
       <c r="C1100" t="n">
-        <v>199869</v>
+        <v>211626</v>
       </c>
     </row>
     <row r="1101">
@@ -12546,7 +12546,7 @@
         <v>1810</v>
       </c>
       <c r="C1101" t="n">
-        <v>30957</v>
+        <v>32778</v>
       </c>
     </row>
     <row r="1102">
@@ -12557,7 +12557,7 @@
         <v>2826</v>
       </c>
       <c r="C1102" t="n">
-        <v>54090.95</v>
+        <v>57272.76</v>
       </c>
     </row>
     <row r="1103">
@@ -12568,7 +12568,7 @@
         <v>2561</v>
       </c>
       <c r="C1103" t="n">
-        <v>11356</v>
+        <v>12024</v>
       </c>
     </row>
     <row r="1104">
@@ -12579,7 +12579,7 @@
         <v>2653</v>
       </c>
       <c r="C1104" t="n">
-        <v>46363.65</v>
+        <v>49090.92</v>
       </c>
     </row>
     <row r="1105">
@@ -12590,7 +12590,7 @@
         <v>2829</v>
       </c>
       <c r="C1105" t="n">
-        <v>46363.65</v>
+        <v>49090.92</v>
       </c>
     </row>
     <row r="1106">
@@ -12601,7 +12601,7 @@
         <v>2643</v>
       </c>
       <c r="C1106" t="n">
-        <v>22814</v>
+        <v>24156</v>
       </c>
     </row>
     <row r="1107">
@@ -12612,7 +12612,7 @@
         <v>2794</v>
       </c>
       <c r="C1107" t="n">
-        <v>69530</v>
+        <v>73620</v>
       </c>
     </row>
     <row r="1108">
@@ -12623,7 +12623,7 @@
         <v>2655</v>
       </c>
       <c r="C1108" t="n">
-        <v>85000</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="1109">
@@ -12634,7 +12634,7 @@
         <v>1456</v>
       </c>
       <c r="C1109" t="n">
-        <v>595221</v>
+        <v>630234</v>
       </c>
     </row>
     <row r="1110">
@@ -12645,7 +12645,7 @@
         <v>2606</v>
       </c>
       <c r="C1110" t="n">
-        <v>182818</v>
+        <v>193572</v>
       </c>
     </row>
     <row r="1111">
@@ -12656,7 +12656,7 @@
         <v>1142</v>
       </c>
       <c r="C1111" t="n">
-        <v>331534</v>
+        <v>351036</v>
       </c>
     </row>
     <row r="1112">
@@ -12667,7 +12667,7 @@
         <v>1450</v>
       </c>
       <c r="C1112" t="n">
-        <v>210613</v>
+        <v>223002</v>
       </c>
     </row>
     <row r="1113">
@@ -12678,7 +12678,7 @@
         <v>2133</v>
       </c>
       <c r="C1113" t="n">
-        <v>491827</v>
+        <v>520758</v>
       </c>
     </row>
     <row r="1114">
@@ -12689,7 +12689,7 @@
         <v>522</v>
       </c>
       <c r="C1114" t="n">
-        <v>150671</v>
+        <v>159534</v>
       </c>
     </row>
     <row r="1115">
@@ -12700,7 +12700,7 @@
         <v>2696</v>
       </c>
       <c r="C1115" t="n">
-        <v>203320</v>
+        <v>215280</v>
       </c>
     </row>
     <row r="1116">
@@ -12722,7 +12722,7 @@
         <v>2692</v>
       </c>
       <c r="C1117" t="n">
-        <v>57953</v>
+        <v>61362</v>
       </c>
     </row>
     <row r="1118">
@@ -12733,7 +12733,7 @@
         <v>2691</v>
       </c>
       <c r="C1118" t="n">
-        <v>104312</v>
+        <v>110448</v>
       </c>
     </row>
     <row r="1119">
@@ -12744,7 +12744,7 @@
         <v>1632</v>
       </c>
       <c r="C1119" t="n">
-        <v>193171</v>
+        <v>204534</v>
       </c>
     </row>
     <row r="1120">
@@ -12755,7 +12755,7 @@
         <v>2641</v>
       </c>
       <c r="C1120" t="n">
-        <v>61812</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1121">
@@ -12766,7 +12766,7 @@
         <v>2197</v>
       </c>
       <c r="C1121" t="n">
-        <v>154530</v>
+        <v>163620</v>
       </c>
     </row>
     <row r="1122">
@@ -12777,7 +12777,7 @@
         <v>609</v>
       </c>
       <c r="C1122" t="n">
-        <v>170000</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="1123">
@@ -12788,7 +12788,7 @@
         <v>1380</v>
       </c>
       <c r="C1123" t="n">
-        <v>77265</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1124">
@@ -12799,7 +12799,7 @@
         <v>104</v>
       </c>
       <c r="C1124" t="n">
-        <v>231812</v>
+        <v>245448</v>
       </c>
     </row>
     <row r="1125">
@@ -12810,7 +12810,7 @@
         <v>2621</v>
       </c>
       <c r="C1125" t="n">
-        <v>54077</v>
+        <v>57258</v>
       </c>
     </row>
     <row r="1126">
@@ -12821,7 +12821,7 @@
         <v>2786</v>
       </c>
       <c r="C1126" t="n">
-        <v>54077</v>
+        <v>57258</v>
       </c>
     </row>
     <row r="1127">
@@ -12832,7 +12832,7 @@
         <v>2784</v>
       </c>
       <c r="C1127" t="n">
-        <v>32147</v>
+        <v>34038</v>
       </c>
     </row>
     <row r="1128">
@@ -12843,7 +12843,7 @@
         <v>2586</v>
       </c>
       <c r="C1128" t="n">
-        <v>32147</v>
+        <v>34038</v>
       </c>
     </row>
     <row r="1129">
@@ -12854,7 +12854,7 @@
         <v>2145</v>
       </c>
       <c r="C1129" t="n">
-        <v>100028</v>
+        <v>105912</v>
       </c>
     </row>
     <row r="1130">
@@ -12865,7 +12865,7 @@
         <v>2574</v>
       </c>
       <c r="C1130" t="n">
-        <v>100028</v>
+        <v>105912</v>
       </c>
     </row>
     <row r="1131">
@@ -12876,7 +12876,7 @@
         <v>2492</v>
       </c>
       <c r="C1131" t="n">
-        <v>109650</v>
+        <v>116100</v>
       </c>
     </row>
     <row r="1132">
@@ -12887,7 +12887,7 @@
         <v>629</v>
       </c>
       <c r="C1132" t="n">
-        <v>341530</v>
+        <v>361620</v>
       </c>
     </row>
     <row r="1133">
@@ -12898,7 +12898,7 @@
         <v>966</v>
       </c>
       <c r="C1133" t="n">
-        <v>62968</v>
+        <v>66672</v>
       </c>
     </row>
     <row r="1134">
@@ -12909,7 +12909,7 @@
         <v>2721</v>
       </c>
       <c r="C1134" t="n">
-        <v>62968</v>
+        <v>66672</v>
       </c>
     </row>
     <row r="1135">
@@ -12920,7 +12920,7 @@
         <v>2554</v>
       </c>
       <c r="C1135" t="n">
-        <v>18972</v>
+        <v>20088</v>
       </c>
     </row>
     <row r="1136">
@@ -12931,7 +12931,7 @@
         <v>2556</v>
       </c>
       <c r="C1136" t="n">
-        <v>27897</v>
+        <v>29538</v>
       </c>
     </row>
     <row r="1137">
@@ -12942,7 +12942,7 @@
         <v>2546</v>
       </c>
       <c r="C1137" t="n">
-        <v>18428</v>
+        <v>19512</v>
       </c>
     </row>
     <row r="1138">
@@ -12953,7 +12953,7 @@
         <v>42</v>
       </c>
       <c r="C1138" t="n">
-        <v>1460453</v>
+        <v>1546362</v>
       </c>
     </row>
     <row r="1139">
@@ -12964,7 +12964,7 @@
         <v>953</v>
       </c>
       <c r="C1139" t="n">
-        <v>527510</v>
+        <v>558540</v>
       </c>
     </row>
     <row r="1140">
@@ -12975,7 +12975,7 @@
         <v>1137</v>
       </c>
       <c r="C1140" t="n">
-        <v>494530</v>
+        <v>523620</v>
       </c>
     </row>
     <row r="1141">
@@ -12986,7 +12986,7 @@
         <v>675</v>
       </c>
       <c r="C1141" t="n">
-        <v>154530</v>
+        <v>163620</v>
       </c>
     </row>
     <row r="1142">
@@ -12997,7 +12997,7 @@
         <v>619</v>
       </c>
       <c r="C1142" t="n">
-        <v>238952</v>
+        <v>253008</v>
       </c>
     </row>
     <row r="1143">
@@ -13008,7 +13008,7 @@
         <v>1299</v>
       </c>
       <c r="C1143" t="n">
-        <v>402084</v>
+        <v>425736</v>
       </c>
     </row>
     <row r="1144">
@@ -13019,7 +13019,7 @@
         <v>1064</v>
       </c>
       <c r="C1144" t="n">
-        <v>463148</v>
+        <v>490392</v>
       </c>
     </row>
     <row r="1145">
@@ -13030,7 +13030,7 @@
         <v>2308</v>
       </c>
       <c r="C1145" t="n">
-        <v>158406</v>
+        <v>167724</v>
       </c>
     </row>
     <row r="1146">
@@ -13041,7 +13041,7 @@
         <v>2747</v>
       </c>
       <c r="C1146" t="n">
-        <v>46363.65</v>
+        <v>49090.92</v>
       </c>
     </row>
     <row r="1147">
@@ -13052,7 +13052,7 @@
         <v>2819</v>
       </c>
       <c r="C1147" t="n">
-        <v>46363.65</v>
+        <v>49090.92</v>
       </c>
     </row>
     <row r="1148">
@@ -13063,7 +13063,7 @@
         <v>1259</v>
       </c>
       <c r="C1148" t="n">
-        <v>77272.75</v>
+        <v>81818.2</v>
       </c>
     </row>
     <row r="1149">
@@ -13074,7 +13074,7 @@
         <v>2544</v>
       </c>
       <c r="C1149" t="n">
-        <v>61812</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1150">
@@ -13085,7 +13085,7 @@
         <v>2261</v>
       </c>
       <c r="C1150" t="n">
-        <v>115906</v>
+        <v>122724</v>
       </c>
     </row>
     <row r="1151">
@@ -13096,7 +13096,7 @@
         <v>2729</v>
       </c>
       <c r="C1151" t="n">
-        <v>61812</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1152">
@@ -13107,7 +13107,7 @@
         <v>2649</v>
       </c>
       <c r="C1152" t="n">
-        <v>22814</v>
+        <v>24156</v>
       </c>
     </row>
     <row r="1153">
@@ -13118,7 +13118,7 @@
         <v>2494</v>
       </c>
       <c r="C1153" t="n">
-        <v>100453</v>
+        <v>106362</v>
       </c>
     </row>
     <row r="1154">
@@ -13129,7 +13129,7 @@
         <v>1384</v>
       </c>
       <c r="C1154" t="n">
-        <v>347718</v>
+        <v>368172</v>
       </c>
     </row>
     <row r="1155">
@@ -13151,7 +13151,7 @@
         <v>2802</v>
       </c>
       <c r="C1156" t="n">
-        <v>54723</v>
+        <v>57942</v>
       </c>
     </row>
     <row r="1157">
@@ -13162,7 +13162,7 @@
         <v>2726</v>
       </c>
       <c r="C1157" t="n">
-        <v>115906</v>
+        <v>122724</v>
       </c>
     </row>
     <row r="1158">
@@ -13173,7 +13173,7 @@
         <v>2820</v>
       </c>
       <c r="C1158" t="n">
-        <v>139077</v>
+        <v>147258</v>
       </c>
     </row>
     <row r="1159">
@@ -13184,7 +13184,7 @@
         <v>1007</v>
       </c>
       <c r="C1159" t="n">
-        <v>146812</v>
+        <v>155448</v>
       </c>
     </row>
     <row r="1160">
@@ -13195,7 +13195,7 @@
         <v>20</v>
       </c>
       <c r="C1160" t="n">
-        <v>297500</v>
+        <v>315000</v>
       </c>
     </row>
     <row r="1161">
@@ -13206,7 +13206,7 @@
         <v>1372</v>
       </c>
       <c r="C1161" t="n">
-        <v>224077</v>
+        <v>237258</v>
       </c>
     </row>
     <row r="1162">
@@ -13217,7 +13217,7 @@
         <v>2735</v>
       </c>
       <c r="C1162" t="n">
-        <v>92718</v>
+        <v>98172</v>
       </c>
     </row>
     <row r="1163">
@@ -13228,7 +13228,7 @@
         <v>2811</v>
       </c>
       <c r="C1163" t="n">
-        <v>32147</v>
+        <v>34038</v>
       </c>
     </row>
     <row r="1164">
@@ -13239,7 +13239,7 @@
         <v>1871</v>
       </c>
       <c r="C1164" t="n">
-        <v>136578</v>
+        <v>144612</v>
       </c>
     </row>
     <row r="1165">
@@ -13250,7 +13250,7 @@
         <v>2541</v>
       </c>
       <c r="C1165" t="n">
-        <v>163506</v>
+        <v>173124</v>
       </c>
     </row>
     <row r="1166">
@@ -13261,7 +13261,7 @@
         <v>2362</v>
       </c>
       <c r="C1166" t="n">
-        <v>57953</v>
+        <v>61362</v>
       </c>
     </row>
     <row r="1167">
@@ -13272,7 +13272,7 @@
         <v>1324</v>
       </c>
       <c r="C1167" t="n">
-        <v>216359</v>
+        <v>229086</v>
       </c>
     </row>
     <row r="1168">
@@ -13283,7 +13283,7 @@
         <v>2323</v>
       </c>
       <c r="C1168" t="n">
-        <v>53074</v>
+        <v>56196</v>
       </c>
     </row>
     <row r="1169">
@@ -13294,7 +13294,7 @@
         <v>2647</v>
       </c>
       <c r="C1169" t="n">
-        <v>109650</v>
+        <v>116100</v>
       </c>
     </row>
     <row r="1170">
@@ -13305,7 +13305,7 @@
         <v>559</v>
       </c>
       <c r="C1170" t="n">
-        <v>177293</v>
+        <v>187722</v>
       </c>
     </row>
     <row r="1171">
@@ -13316,7 +13316,7 @@
         <v>2762</v>
       </c>
       <c r="C1171" t="n">
-        <v>62968</v>
+        <v>66672</v>
       </c>
     </row>
     <row r="1172">
@@ -13327,7 +13327,7 @@
         <v>2501</v>
       </c>
       <c r="C1172" t="n">
-        <v>62968</v>
+        <v>66672</v>
       </c>
     </row>
     <row r="1173">
@@ -13338,7 +13338,7 @@
         <v>2562</v>
       </c>
       <c r="C1173" t="n">
-        <v>12223</v>
+        <v>12942</v>
       </c>
     </row>
     <row r="1174">
@@ -13349,7 +13349,7 @@
         <v>429</v>
       </c>
       <c r="C1174" t="n">
-        <v>301359</v>
+        <v>319086</v>
       </c>
     </row>
     <row r="1175">
@@ -13360,7 +13360,7 @@
         <v>58</v>
       </c>
       <c r="C1175" t="n">
-        <v>209083</v>
+        <v>221382</v>
       </c>
     </row>
     <row r="1176">
@@ -13371,7 +13371,7 @@
         <v>2245</v>
       </c>
       <c r="C1176" t="n">
-        <v>186677</v>
+        <v>197658</v>
       </c>
     </row>
     <row r="1177">
@@ -13382,7 +13382,7 @@
         <v>285</v>
       </c>
       <c r="C1177" t="n">
-        <v>418166</v>
+        <v>442764</v>
       </c>
     </row>
     <row r="1178">
@@ -13404,7 +13404,7 @@
         <v>363</v>
       </c>
       <c r="C1179" t="n">
-        <v>231812</v>
+        <v>245448</v>
       </c>
     </row>
     <row r="1180">
@@ -13415,7 +13415,7 @@
         <v>2651</v>
       </c>
       <c r="C1180" t="n">
-        <v>130679</v>
+        <v>138366</v>
       </c>
     </row>
     <row r="1181">
@@ -13426,7 +13426,7 @@
         <v>2142</v>
       </c>
       <c r="C1181" t="n">
-        <v>41242</v>
+        <v>43668</v>
       </c>
     </row>
     <row r="1182">
@@ -13437,7 +13437,7 @@
         <v>2258</v>
       </c>
       <c r="C1182" t="n">
-        <v>61818.2</v>
+        <v>65454.56</v>
       </c>
     </row>
     <row r="1183">
@@ -13448,7 +13448,7 @@
         <v>2772</v>
       </c>
       <c r="C1183" t="n">
-        <v>46363.65</v>
+        <v>49090.92</v>
       </c>
     </row>
     <row r="1184">
@@ -13459,7 +13459,7 @@
         <v>2346</v>
       </c>
       <c r="C1184" t="n">
-        <v>85000</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="1185">
@@ -13470,7 +13470,7 @@
         <v>2442</v>
       </c>
       <c r="C1185" t="n">
-        <v>61812</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1186">
@@ -13481,7 +13481,7 @@
         <v>772</v>
       </c>
       <c r="C1186" t="n">
-        <v>255000</v>
+        <v>270000</v>
       </c>
     </row>
     <row r="1187">
@@ -13492,7 +13492,7 @@
         <v>2684</v>
       </c>
       <c r="C1187" t="n">
-        <v>73406</v>
+        <v>77724</v>
       </c>
     </row>
     <row r="1188">
@@ -13503,7 +13503,7 @@
         <v>2765</v>
       </c>
       <c r="C1188" t="n">
-        <v>69530</v>
+        <v>73620</v>
       </c>
     </row>
     <row r="1189">
@@ -13514,7 +13514,7 @@
         <v>2567</v>
       </c>
       <c r="C1189" t="n">
-        <v>127534</v>
+        <v>135036</v>
       </c>
     </row>
     <row r="1190">
@@ -13525,7 +13525,7 @@
         <v>2178</v>
       </c>
       <c r="C1190" t="n">
-        <v>216359</v>
+        <v>229086</v>
       </c>
     </row>
     <row r="1191">
@@ -13536,7 +13536,7 @@
         <v>2827</v>
       </c>
       <c r="C1191" t="n">
-        <v>77265</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1192">
@@ -13547,7 +13547,7 @@
         <v>2510</v>
       </c>
       <c r="C1192" t="n">
-        <v>429046</v>
+        <v>454284</v>
       </c>
     </row>
     <row r="1193">
@@ -13558,7 +13558,7 @@
         <v>2392</v>
       </c>
       <c r="C1193" t="n">
-        <v>128707</v>
+        <v>136278</v>
       </c>
     </row>
     <row r="1194">
@@ -13569,7 +13569,7 @@
         <v>415</v>
       </c>
       <c r="C1194" t="n">
-        <v>440062</v>
+        <v>465948</v>
       </c>
     </row>
     <row r="1195">
@@ -13580,7 +13580,7 @@
         <v>2107</v>
       </c>
       <c r="C1195" t="n">
-        <v>227239</v>
+        <v>240606</v>
       </c>
     </row>
     <row r="1196">
@@ -13591,7 +13591,7 @@
         <v>2211</v>
       </c>
       <c r="C1196" t="n">
-        <v>188394</v>
+        <v>199476</v>
       </c>
     </row>
     <row r="1197">
@@ -13602,7 +13602,7 @@
         <v>2682</v>
       </c>
       <c r="C1197" t="n">
-        <v>115889</v>
+        <v>122706</v>
       </c>
     </row>
     <row r="1198">
@@ -13635,7 +13635,7 @@
         <v>2755</v>
       </c>
       <c r="C1200" t="n">
-        <v>46359</v>
+        <v>49086</v>
       </c>
     </row>
     <row r="1201">
@@ -13646,7 +13646,7 @@
         <v>941</v>
       </c>
       <c r="C1201" t="n">
-        <v>303586</v>
+        <v>321444</v>
       </c>
     </row>
     <row r="1202">
@@ -13657,7 +13657,7 @@
         <v>2734</v>
       </c>
       <c r="C1202" t="n">
-        <v>42551</v>
+        <v>45054</v>
       </c>
     </row>
     <row r="1203">
@@ -13668,7 +13668,7 @@
         <v>1289</v>
       </c>
       <c r="C1203" t="n">
-        <v>193171</v>
+        <v>204534</v>
       </c>
     </row>
     <row r="1204">
@@ -13679,7 +13679,7 @@
         <v>2801</v>
       </c>
       <c r="C1204" t="n">
-        <v>61812</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1205">
@@ -13690,7 +13690,7 @@
         <v>2810</v>
       </c>
       <c r="C1205" t="n">
-        <v>104312</v>
+        <v>110448</v>
       </c>
     </row>
     <row r="1206">
@@ -13701,7 +13701,7 @@
         <v>767</v>
       </c>
       <c r="C1206" t="n">
-        <v>139077</v>
+        <v>147258</v>
       </c>
     </row>
     <row r="1207">
@@ -13712,7 +13712,7 @@
         <v>2687</v>
       </c>
       <c r="C1207" t="n">
-        <v>77265</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1208">
@@ -13723,7 +13723,7 @@
         <v>2686</v>
       </c>
       <c r="C1208" t="n">
-        <v>100453</v>
+        <v>106362</v>
       </c>
     </row>
     <row r="1209">
@@ -13734,7 +13734,7 @@
         <v>2730</v>
       </c>
       <c r="C1209" t="n">
-        <v>69530</v>
+        <v>73620</v>
       </c>
     </row>
     <row r="1210">
@@ -13745,7 +13745,7 @@
         <v>2580</v>
       </c>
       <c r="C1210" t="n">
-        <v>25925</v>
+        <v>27450</v>
       </c>
     </row>
     <row r="1211">
@@ -13756,7 +13756,7 @@
         <v>2472</v>
       </c>
       <c r="C1211" t="n">
-        <v>40909.75</v>
+        <v>43316.2</v>
       </c>
     </row>
     <row r="1212">
@@ -13767,7 +13767,7 @@
         <v>2631</v>
       </c>
       <c r="C1212" t="n">
-        <v>18956.55</v>
+        <v>20071.64</v>
       </c>
     </row>
     <row r="1213">
@@ -13778,7 +13778,7 @@
         <v>1642</v>
       </c>
       <c r="C1213" t="n">
-        <v>204765</v>
+        <v>216810</v>
       </c>
     </row>
     <row r="1214">
@@ -13789,7 +13789,7 @@
         <v>2613</v>
       </c>
       <c r="C1214" t="n">
-        <v>138465</v>
+        <v>146610</v>
       </c>
     </row>
     <row r="1215">
@@ -13800,7 +13800,7 @@
         <v>1020</v>
       </c>
       <c r="C1215" t="n">
-        <v>69530</v>
+        <v>73620</v>
       </c>
     </row>
     <row r="1216">
@@ -13811,7 +13811,7 @@
         <v>2785</v>
       </c>
       <c r="C1216" t="n">
-        <v>32147</v>
+        <v>34038</v>
       </c>
     </row>
     <row r="1217">
@@ -13822,7 +13822,7 @@
         <v>1327</v>
       </c>
       <c r="C1217" t="n">
-        <v>46359</v>
+        <v>49086</v>
       </c>
     </row>
     <row r="1218">
@@ -13833,7 +13833,7 @@
         <v>2629</v>
       </c>
       <c r="C1218" t="n">
-        <v>53074</v>
+        <v>56196</v>
       </c>
     </row>
     <row r="1219">
@@ -13844,7 +13844,7 @@
         <v>749</v>
       </c>
       <c r="C1219" t="n">
-        <v>62968</v>
+        <v>66672</v>
       </c>
     </row>
     <row r="1220">
@@ -13855,7 +13855,7 @@
         <v>1983</v>
       </c>
       <c r="C1220" t="n">
-        <v>418166</v>
+        <v>442764</v>
       </c>
     </row>
     <row r="1221">
@@ -13866,7 +13866,7 @@
         <v>1993</v>
       </c>
       <c r="C1221" t="n">
-        <v>268821</v>
+        <v>284634</v>
       </c>
     </row>
     <row r="1222">
@@ -13877,7 +13877,7 @@
         <v>2767</v>
       </c>
       <c r="C1222" t="n">
-        <v>149073</v>
+        <v>157842</v>
       </c>
     </row>
     <row r="1223">
@@ -13899,7 +13899,7 @@
         <v>1102</v>
       </c>
       <c r="C1224" t="n">
-        <v>186677</v>
+        <v>197658</v>
       </c>
     </row>
     <row r="1225">
@@ -13910,7 +13910,7 @@
         <v>626</v>
       </c>
       <c r="C1225" t="n">
-        <v>1316970.7</v>
+        <v>1394439.56</v>
       </c>
     </row>
     <row r="1226">
@@ -13921,7 +13921,7 @@
         <v>1465</v>
       </c>
       <c r="C1226" t="n">
-        <v>278018</v>
+        <v>294372</v>
       </c>
     </row>
     <row r="1227">
@@ -13932,7 +13932,7 @@
         <v>2758</v>
       </c>
       <c r="C1227" t="n">
-        <v>46363.65</v>
+        <v>49090.92</v>
       </c>
     </row>
     <row r="1228">
@@ -13943,7 +13943,7 @@
         <v>2742</v>
       </c>
       <c r="C1228" t="n">
-        <v>46363.65</v>
+        <v>49090.92</v>
       </c>
     </row>
     <row r="1229">
@@ -13965,7 +13965,7 @@
         <v>1873</v>
       </c>
       <c r="C1230" t="n">
-        <v>247265</v>
+        <v>261810</v>
       </c>
     </row>
     <row r="1231">
@@ -13976,7 +13976,7 @@
         <v>2163</v>
       </c>
       <c r="C1231" t="n">
-        <v>115906</v>
+        <v>122724</v>
       </c>
     </row>
     <row r="1232">
@@ -13987,7 +13987,7 @@
         <v>2394</v>
       </c>
       <c r="C1232" t="n">
-        <v>119034</v>
+        <v>126036</v>
       </c>
     </row>
     <row r="1233">
@@ -13998,7 +13998,7 @@
         <v>33</v>
       </c>
       <c r="C1233" t="n">
-        <v>299812</v>
+        <v>317448</v>
       </c>
     </row>
     <row r="1234">
@@ -14009,7 +14009,7 @@
         <v>2421</v>
       </c>
       <c r="C1234" t="n">
-        <v>50218</v>
+        <v>53172</v>
       </c>
     </row>
     <row r="1235">
@@ -14020,7 +14020,7 @@
         <v>2663</v>
       </c>
       <c r="C1235" t="n">
-        <v>212500</v>
+        <v>225000</v>
       </c>
     </row>
     <row r="1236">
@@ -14031,7 +14031,7 @@
         <v>2413</v>
       </c>
       <c r="C1236" t="n">
-        <v>93534</v>
+        <v>99036</v>
       </c>
     </row>
     <row r="1237">
@@ -14042,7 +14042,7 @@
         <v>351</v>
       </c>
       <c r="C1237" t="n">
-        <v>142171</v>
+        <v>150534</v>
       </c>
     </row>
     <row r="1238">
@@ -14053,7 +14053,7 @@
         <v>1298</v>
       </c>
       <c r="C1238" t="n">
-        <v>983671</v>
+        <v>1041534</v>
       </c>
     </row>
     <row r="1239">
@@ -14064,7 +14064,7 @@
         <v>2491</v>
       </c>
       <c r="C1239" t="n">
-        <v>79492</v>
+        <v>84168</v>
       </c>
     </row>
     <row r="1240">
@@ -14075,7 +14075,7 @@
         <v>2571</v>
       </c>
       <c r="C1240" t="n">
-        <v>112251</v>
+        <v>118854</v>
       </c>
     </row>
     <row r="1241">
@@ -14086,7 +14086,7 @@
         <v>2507</v>
       </c>
       <c r="C1241" t="n">
-        <v>68204</v>
+        <v>72216</v>
       </c>
     </row>
     <row r="1242">
@@ -14097,7 +14097,7 @@
         <v>2799</v>
       </c>
       <c r="C1242" t="n">
-        <v>87788</v>
+        <v>92952</v>
       </c>
     </row>
     <row r="1243">
@@ -14119,7 +14119,7 @@
         <v>2582</v>
       </c>
       <c r="C1244" t="n">
-        <v>66878</v>
+        <v>70812</v>
       </c>
     </row>
     <row r="1245">
@@ -14130,7 +14130,7 @@
         <v>2637</v>
       </c>
       <c r="C1245" t="n">
-        <v>48637</v>
+        <v>51498</v>
       </c>
     </row>
     <row r="1246">
@@ -14141,7 +14141,7 @@
         <v>630</v>
       </c>
       <c r="C1246" t="n">
-        <v>115668</v>
+        <v>122472</v>
       </c>
     </row>
     <row r="1247">
@@ -14152,7 +14152,7 @@
         <v>525</v>
       </c>
       <c r="C1247" t="n">
-        <v>173859</v>
+        <v>184086</v>
       </c>
     </row>
     <row r="1248">
@@ -14163,7 +14163,7 @@
         <v>2727</v>
       </c>
       <c r="C1248" t="n">
-        <v>31280</v>
+        <v>33120</v>
       </c>
     </row>
     <row r="1249">
@@ -14174,7 +14174,7 @@
         <v>2707</v>
       </c>
       <c r="C1249" t="n">
-        <v>24752</v>
+        <v>26208</v>
       </c>
     </row>
     <row r="1250">
@@ -14185,7 +14185,7 @@
         <v>2834</v>
       </c>
       <c r="C1250" t="n">
-        <v>12787.1</v>
+        <v>13539.28</v>
       </c>
     </row>
     <row r="1251">
@@ -14196,7 +14196,7 @@
         <v>2773</v>
       </c>
       <c r="C1251" t="n">
-        <v>62352.95</v>
+        <v>66020.75999999999</v>
       </c>
     </row>
     <row r="1252">
@@ -14207,7 +14207,7 @@
         <v>2341</v>
       </c>
       <c r="C1252" t="n">
-        <v>109650</v>
+        <v>116100</v>
       </c>
     </row>
     <row r="1253">
@@ -14218,7 +14218,7 @@
         <v>1374</v>
       </c>
       <c r="C1253" t="n">
-        <v>139077</v>
+        <v>147258</v>
       </c>
     </row>
     <row r="1254">
@@ -14229,7 +14229,7 @@
         <v>793</v>
       </c>
       <c r="C1254" t="n">
-        <v>32147</v>
+        <v>34038</v>
       </c>
     </row>
     <row r="1255">
@@ -14240,7 +14240,7 @@
         <v>794</v>
       </c>
       <c r="C1255" t="n">
-        <v>32147</v>
+        <v>34038</v>
       </c>
     </row>
     <row r="1256">
@@ -14251,7 +14251,7 @@
         <v>1834</v>
       </c>
       <c r="C1256" t="n">
-        <v>90406</v>
+        <v>95724</v>
       </c>
     </row>
     <row r="1257">
@@ -14262,7 +14262,7 @@
         <v>802</v>
       </c>
       <c r="C1257" t="n">
-        <v>57953</v>
+        <v>61362</v>
       </c>
     </row>
     <row r="1258">
@@ -14273,7 +14273,7 @@
         <v>1344</v>
       </c>
       <c r="C1258" t="n">
-        <v>115906</v>
+        <v>122724</v>
       </c>
     </row>
     <row r="1259">
@@ -14284,7 +14284,7 @@
         <v>1881</v>
       </c>
       <c r="C1259" t="n">
-        <v>53074</v>
+        <v>56196</v>
       </c>
     </row>
     <row r="1260">
@@ -14295,7 +14295,7 @@
         <v>2365</v>
       </c>
       <c r="C1260" t="n">
-        <v>61557</v>
+        <v>65178</v>
       </c>
     </row>
     <row r="1261">
@@ -14306,7 +14306,7 @@
         <v>2411</v>
       </c>
       <c r="C1261" t="n">
-        <v>109650</v>
+        <v>116100</v>
       </c>
     </row>
     <row r="1262">
@@ -14317,7 +14317,7 @@
         <v>2363</v>
       </c>
       <c r="C1262" t="n">
-        <v>115906</v>
+        <v>122724</v>
       </c>
     </row>
     <row r="1263">
@@ -14328,7 +14328,7 @@
         <v>2124</v>
       </c>
       <c r="C1263" t="n">
-        <v>270453</v>
+        <v>286362</v>
       </c>
     </row>
     <row r="1264">
@@ -14339,7 +14339,7 @@
         <v>1937</v>
       </c>
       <c r="C1264" t="n">
-        <v>197030</v>
+        <v>208620</v>
       </c>
     </row>
     <row r="1265">
@@ -14350,7 +14350,7 @@
         <v>2709</v>
       </c>
       <c r="C1265" t="n">
-        <v>139077</v>
+        <v>147258</v>
       </c>
     </row>
     <row r="1266">
@@ -14361,7 +14361,7 @@
         <v>2558</v>
       </c>
       <c r="C1266" t="n">
-        <v>23222</v>
+        <v>24588</v>
       </c>
     </row>
     <row r="1267">
@@ -14372,7 +14372,7 @@
         <v>663</v>
       </c>
       <c r="C1267" t="n">
-        <v>197030</v>
+        <v>208620</v>
       </c>
     </row>
     <row r="1268">
@@ -14383,7 +14383,7 @@
         <v>40</v>
       </c>
       <c r="C1268" t="n">
-        <v>170000</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="1269">
@@ -14394,7 +14394,7 @@
         <v>2833</v>
       </c>
       <c r="C1269" t="n">
-        <v>54090.95</v>
+        <v>57272.76</v>
       </c>
     </row>
     <row r="1270">
@@ -14405,7 +14405,7 @@
         <v>1756</v>
       </c>
       <c r="C1270" t="n">
-        <v>337297</v>
+        <v>357138</v>
       </c>
     </row>
     <row r="1271">
@@ -14416,7 +14416,7 @@
         <v>1116</v>
       </c>
       <c r="C1271" t="n">
-        <v>195993</v>
+        <v>207522</v>
       </c>
     </row>
     <row r="1272">
@@ -14427,7 +14427,7 @@
         <v>636</v>
       </c>
       <c r="C1272" t="n">
-        <v>193171</v>
+        <v>204534</v>
       </c>
     </row>
     <row r="1273">
@@ -14438,7 +14438,7 @@
         <v>1800</v>
       </c>
       <c r="C1273" t="n">
-        <v>21624</v>
+        <v>22896</v>
       </c>
     </row>
     <row r="1274">
@@ -14449,7 +14449,7 @@
         <v>2815</v>
       </c>
       <c r="C1274" t="n">
-        <v>46363.65</v>
+        <v>49090.92</v>
       </c>
     </row>
     <row r="1275">
@@ -14460,7 +14460,7 @@
         <v>1658</v>
       </c>
       <c r="C1275" t="n">
-        <v>102000</v>
+        <v>108000</v>
       </c>
     </row>
     <row r="1276">
@@ -14471,7 +14471,7 @@
         <v>2635</v>
       </c>
       <c r="C1276" t="n">
-        <v>100453</v>
+        <v>106362</v>
       </c>
     </row>
     <row r="1277">
@@ -14482,7 +14482,7 @@
         <v>2402</v>
       </c>
       <c r="C1277" t="n">
-        <v>503812</v>
+        <v>533448</v>
       </c>
     </row>
     <row r="1278">
@@ -14493,7 +14493,7 @@
         <v>452</v>
       </c>
       <c r="C1278" t="n">
-        <v>208624</v>
+        <v>220896</v>
       </c>
     </row>
     <row r="1279">
@@ -14504,7 +14504,7 @@
         <v>2085</v>
       </c>
       <c r="C1279" t="n">
-        <v>102034</v>
+        <v>108036</v>
       </c>
     </row>
     <row r="1280">
@@ -14515,7 +14515,7 @@
         <v>2568</v>
       </c>
       <c r="C1280" t="n">
-        <v>157964</v>
+        <v>167256</v>
       </c>
     </row>
     <row r="1281">
@@ -14526,7 +14526,7 @@
         <v>1906</v>
       </c>
       <c r="C1281" t="n">
-        <v>89658</v>
+        <v>94932</v>
       </c>
     </row>
     <row r="1282">
@@ -14537,7 +14537,7 @@
         <v>2821</v>
       </c>
       <c r="C1282" t="n">
-        <v>77962</v>
+        <v>82548</v>
       </c>
     </row>
     <row r="1283">
@@ -14548,7 +14548,7 @@
         <v>2698</v>
       </c>
       <c r="C1283" t="n">
-        <v>95557</v>
+        <v>101178</v>
       </c>
     </row>
     <row r="1284">
@@ -14559,7 +14559,7 @@
         <v>2118</v>
       </c>
       <c r="C1284" t="n">
-        <v>183260</v>
+        <v>194040</v>
       </c>
     </row>
     <row r="1285">
@@ -14570,7 +14570,7 @@
         <v>2383</v>
       </c>
       <c r="C1285" t="n">
-        <v>106998</v>
+        <v>113292</v>
       </c>
     </row>
     <row r="1286">
@@ -14581,7 +14581,7 @@
         <v>2813</v>
       </c>
       <c r="C1286" t="n">
-        <v>48637</v>
+        <v>51498</v>
       </c>
     </row>
     <row r="1287">
@@ -14592,7 +14592,7 @@
         <v>925</v>
       </c>
       <c r="C1287" t="n">
-        <v>60792</v>
+        <v>64368</v>
       </c>
     </row>
     <row r="1288">
@@ -14603,7 +14603,7 @@
         <v>2689</v>
       </c>
       <c r="C1288" t="n">
-        <v>48637</v>
+        <v>51498</v>
       </c>
     </row>
     <row r="1289">
@@ -14614,7 +14614,7 @@
         <v>2716</v>
       </c>
       <c r="C1289" t="n">
-        <v>66878</v>
+        <v>70812</v>
       </c>
     </row>
     <row r="1290">
@@ -14625,7 +14625,7 @@
         <v>2831</v>
       </c>
       <c r="C1290" t="n">
-        <v>46359</v>
+        <v>49086</v>
       </c>
     </row>
     <row r="1291">
@@ -14636,7 +14636,7 @@
         <v>2045</v>
       </c>
       <c r="C1291" t="n">
-        <v>259988.47</v>
+        <v>275281.9</v>
       </c>
     </row>
     <row r="1292">
@@ -14647,7 +14647,7 @@
         <v>580</v>
       </c>
       <c r="C1292" t="n">
-        <v>104312</v>
+        <v>110448</v>
       </c>
     </row>
     <row r="1293">
@@ -14658,7 +14658,7 @@
         <v>438</v>
       </c>
       <c r="C1293" t="n">
-        <v>119765</v>
+        <v>126810</v>
       </c>
     </row>
     <row r="1294">
@@ -14669,7 +14669,7 @@
         <v>1539</v>
       </c>
       <c r="C1294" t="n">
-        <v>131359</v>
+        <v>139086</v>
       </c>
     </row>
     <row r="1295">
@@ -14680,7 +14680,7 @@
         <v>2817</v>
       </c>
       <c r="C1295" t="n">
-        <v>46359</v>
+        <v>49086</v>
       </c>
     </row>
     <row r="1296">
@@ -14691,7 +14691,7 @@
         <v>2816</v>
       </c>
       <c r="C1296" t="n">
-        <v>100453</v>
+        <v>106362</v>
       </c>
     </row>
     <row r="1297">
@@ -14702,7 +14702,7 @@
         <v>2146</v>
       </c>
       <c r="C1297" t="n">
-        <v>155822</v>
+        <v>164988</v>
       </c>
     </row>
     <row r="1298">
@@ -14713,7 +14713,7 @@
         <v>2276</v>
       </c>
       <c r="C1298" t="n">
-        <v>173128</v>
+        <v>183312</v>
       </c>
     </row>
     <row r="1299">
@@ -14724,7 +14724,7 @@
         <v>1381</v>
       </c>
       <c r="C1299" t="n">
-        <v>227953</v>
+        <v>241362</v>
       </c>
     </row>
     <row r="1300">
@@ -14735,7 +14735,7 @@
         <v>2081</v>
       </c>
       <c r="C1300" t="n">
-        <v>115906</v>
+        <v>122724</v>
       </c>
     </row>
     <row r="1301">
@@ -14746,7 +14746,7 @@
         <v>14</v>
       </c>
       <c r="C1301" t="n">
-        <v>336124</v>
+        <v>355896</v>
       </c>
     </row>
     <row r="1302">
@@ -14757,7 +14757,7 @@
         <v>766</v>
       </c>
       <c r="C1302" t="n">
-        <v>53074</v>
+        <v>56196</v>
       </c>
     </row>
     <row r="1303">
@@ -14768,7 +14768,7 @@
         <v>2547</v>
       </c>
       <c r="C1303" t="n">
-        <v>31773</v>
+        <v>33642</v>
       </c>
     </row>
     <row r="1304">
@@ -14779,7 +14779,7 @@
         <v>2552</v>
       </c>
       <c r="C1304" t="n">
-        <v>22848</v>
+        <v>24192</v>
       </c>
     </row>
     <row r="1305">
@@ -14790,7 +14790,7 @@
         <v>131</v>
       </c>
       <c r="C1305" t="n">
-        <v>316030</v>
+        <v>334620</v>
       </c>
     </row>
     <row r="1306">
@@ -14801,7 +14801,7 @@
         <v>2250</v>
       </c>
       <c r="C1306" t="n">
-        <v>255697</v>
+        <v>270738</v>
       </c>
     </row>
     <row r="1307">
@@ -14812,7 +14812,7 @@
         <v>89</v>
       </c>
       <c r="C1307" t="n">
-        <v>261324</v>
+        <v>276696</v>
       </c>
     </row>
     <row r="1308">
@@ -14823,7 +14823,7 @@
         <v>2141</v>
       </c>
       <c r="C1308" t="n">
-        <v>24446</v>
+        <v>25884</v>
       </c>
     </row>
     <row r="1309">
@@ -14834,7 +14834,7 @@
         <v>2798</v>
       </c>
       <c r="C1309" t="n">
-        <v>46363.65</v>
+        <v>49090.92</v>
       </c>
     </row>
     <row r="1310">
@@ -14845,7 +14845,7 @@
         <v>2797</v>
       </c>
       <c r="C1310" t="n">
-        <v>46363.65</v>
+        <v>49090.92</v>
       </c>
     </row>
     <row r="1311">
@@ -14856,7 +14856,7 @@
         <v>2266</v>
       </c>
       <c r="C1311" t="n">
-        <v>61818.2</v>
+        <v>65454.56</v>
       </c>
     </row>
     <row r="1312">
@@ -14867,7 +14867,7 @@
         <v>1499</v>
       </c>
       <c r="C1312" t="n">
-        <v>108171</v>
+        <v>114534</v>
       </c>
     </row>
     <row r="1313">
@@ -14878,7 +14878,7 @@
         <v>2496</v>
       </c>
       <c r="C1313" t="n">
-        <v>123624</v>
+        <v>130896</v>
       </c>
     </row>
     <row r="1314">
@@ -14889,7 +14889,7 @@
         <v>949</v>
       </c>
       <c r="C1314" t="n">
-        <v>75837</v>
+        <v>80298</v>
       </c>
     </row>
     <row r="1315">
@@ -14900,7 +14900,7 @@
         <v>1853</v>
       </c>
       <c r="C1315" t="n">
-        <v>92718</v>
+        <v>98172</v>
       </c>
     </row>
     <row r="1316">
@@ -14911,7 +14911,7 @@
         <v>854</v>
       </c>
       <c r="C1316" t="n">
-        <v>85000</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="1317">
@@ -14922,7 +14922,7 @@
         <v>2674</v>
       </c>
       <c r="C1317" t="n">
-        <v>200906</v>
+        <v>212724</v>
       </c>
     </row>
     <row r="1318">
@@ -14933,7 +14933,7 @@
         <v>2803</v>
       </c>
       <c r="C1318" t="n">
-        <v>92718</v>
+        <v>98172</v>
       </c>
     </row>
     <row r="1319">
@@ -14944,7 +14944,7 @@
         <v>2599</v>
       </c>
       <c r="C1319" t="n">
-        <v>146812</v>
+        <v>155448</v>
       </c>
     </row>
     <row r="1320">
@@ -14955,7 +14955,7 @@
         <v>783</v>
       </c>
       <c r="C1320" t="n">
-        <v>40171</v>
+        <v>42534</v>
       </c>
     </row>
     <row r="1321">
@@ -14966,7 +14966,7 @@
         <v>27</v>
       </c>
       <c r="C1321" t="n">
-        <v>77265</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1322">
@@ -14977,7 +14977,7 @@
         <v>531</v>
       </c>
       <c r="C1322" t="n">
-        <v>270453</v>
+        <v>286362</v>
       </c>
     </row>
     <row r="1323">
@@ -14988,7 +14988,7 @@
         <v>1308</v>
       </c>
       <c r="C1323" t="n">
-        <v>124814</v>
+        <v>132156</v>
       </c>
     </row>
     <row r="1324">
@@ -14999,7 +14999,7 @@
         <v>2792</v>
       </c>
       <c r="C1324" t="n">
-        <v>90015</v>
+        <v>95310</v>
       </c>
     </row>
     <row r="1325">
@@ -15021,7 +15021,7 @@
         <v>2823</v>
       </c>
       <c r="C1326" t="n">
-        <v>72250</v>
+        <v>76500</v>
       </c>
     </row>
     <row r="1327">
@@ -15032,7 +15032,7 @@
         <v>2584</v>
       </c>
       <c r="C1327" t="n">
-        <v>48637</v>
+        <v>51498</v>
       </c>
     </row>
     <row r="1328">
@@ -15043,7 +15043,7 @@
         <v>945</v>
       </c>
       <c r="C1328" t="n">
-        <v>218926</v>
+        <v>231804</v>
       </c>
     </row>
     <row r="1329">
@@ -15054,7 +15054,7 @@
         <v>2660</v>
       </c>
       <c r="C1329" t="n">
-        <v>239530</v>
+        <v>253620</v>
       </c>
     </row>
     <row r="1330">
@@ -15065,7 +15065,7 @@
         <v>1317</v>
       </c>
       <c r="C1330" t="n">
-        <v>231812</v>
+        <v>245448</v>
       </c>
     </row>
     <row r="1331">
@@ -15076,7 +15076,7 @@
         <v>2790</v>
       </c>
       <c r="C1331" t="n">
-        <v>49215</v>
+        <v>52110</v>
       </c>
     </row>
     <row r="1332">
@@ -15087,7 +15087,7 @@
         <v>2711</v>
       </c>
       <c r="C1332" t="n">
-        <v>66986.2</v>
+        <v>70926.56</v>
       </c>
     </row>
     <row r="1333">
@@ -15098,7 +15098,7 @@
         <v>2607</v>
       </c>
       <c r="C1333" t="n">
-        <v>38392.2</v>
+        <v>40650.56</v>
       </c>
     </row>
     <row r="1334">
@@ -15109,7 +15109,7 @@
         <v>2667</v>
       </c>
       <c r="C1334" t="n">
-        <v>35313.65</v>
+        <v>37390.92</v>
       </c>
     </row>
     <row r="1335">
@@ -15120,7 +15120,7 @@
         <v>2706</v>
       </c>
       <c r="C1335" t="n">
-        <v>17024.75</v>
+        <v>18026.2</v>
       </c>
     </row>
     <row r="1336">
@@ -15131,7 +15131,7 @@
         <v>2657</v>
       </c>
       <c r="C1336" t="n">
-        <v>61196.95</v>
+        <v>64796.76</v>
       </c>
     </row>
     <row r="1337">
@@ -15142,7 +15142,7 @@
         <v>1278</v>
       </c>
       <c r="C1337" t="n">
-        <v>77265</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1338">
@@ -15153,7 +15153,7 @@
         <v>2745</v>
       </c>
       <c r="C1338" t="n">
-        <v>85000</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="1339">
@@ -15164,7 +15164,7 @@
         <v>2753</v>
       </c>
       <c r="C1339" t="n">
-        <v>57953</v>
+        <v>61362</v>
       </c>
     </row>
     <row r="1340">
@@ -15175,7 +15175,7 @@
         <v>2183</v>
       </c>
       <c r="C1340" t="n">
-        <v>282778</v>
+        <v>299412</v>
       </c>
     </row>
     <row r="1341">
@@ -15186,7 +15186,7 @@
         <v>1340</v>
       </c>
       <c r="C1341" t="n">
-        <v>112030</v>
+        <v>118620</v>
       </c>
     </row>
     <row r="1342">
@@ -15197,7 +15197,7 @@
         <v>2583</v>
       </c>
       <c r="C1342" t="n">
-        <v>32147</v>
+        <v>34038</v>
       </c>
     </row>
     <row r="1343">
@@ -15208,7 +15208,7 @@
         <v>2090</v>
       </c>
       <c r="C1343" t="n">
-        <v>32147</v>
+        <v>34038</v>
       </c>
     </row>
     <row r="1344">
@@ -15219,7 +15219,7 @@
         <v>1277</v>
       </c>
       <c r="C1344" t="n">
-        <v>170000</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="1345">
@@ -15230,7 +15230,7 @@
         <v>1501</v>
       </c>
       <c r="C1345" t="n">
-        <v>73406</v>
+        <v>77724</v>
       </c>
     </row>
     <row r="1346">
@@ -15241,7 +15241,7 @@
         <v>703</v>
       </c>
       <c r="C1346" t="n">
-        <v>193171</v>
+        <v>204534</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:02:51
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1346"/>
+  <dimension ref="A1:C1347"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11289,10 +11289,10 @@
         <v>46266</v>
       </c>
       <c r="B987" t="n">
-        <v>947</v>
+        <v>931</v>
       </c>
       <c r="C987" t="n">
-        <v>355518</v>
+        <v>81548</v>
       </c>
     </row>
     <row r="988">
@@ -11300,10 +11300,10 @@
         <v>46266</v>
       </c>
       <c r="B988" t="n">
-        <v>1956</v>
+        <v>947</v>
       </c>
       <c r="C988" t="n">
-        <v>206568</v>
+        <v>375269</v>
       </c>
     </row>
     <row r="989">
@@ -11311,10 +11311,10 @@
         <v>46266</v>
       </c>
       <c r="B989" t="n">
-        <v>2824</v>
+        <v>1956</v>
       </c>
       <c r="C989" t="n">
-        <v>90000</v>
+        <v>218044</v>
       </c>
     </row>
     <row r="990">
@@ -11322,10 +11322,10 @@
         <v>46266</v>
       </c>
       <c r="B990" t="n">
-        <v>2787</v>
+        <v>2824</v>
       </c>
       <c r="C990" t="n">
-        <v>106362</v>
+        <v>95000</v>
       </c>
     </row>
     <row r="991">
@@ -11333,10 +11333,10 @@
         <v>46266</v>
       </c>
       <c r="B991" t="n">
-        <v>2830</v>
+        <v>2787</v>
       </c>
       <c r="C991" t="n">
-        <v>73620</v>
+        <v>112271</v>
       </c>
     </row>
     <row r="992">
@@ -11344,10 +11344,10 @@
         <v>46266</v>
       </c>
       <c r="B992" t="n">
-        <v>1254</v>
+        <v>2830</v>
       </c>
       <c r="C992" t="n">
-        <v>158887.64</v>
+        <v>77710</v>
       </c>
     </row>
     <row r="993">
@@ -11355,10 +11355,10 @@
         <v>46266</v>
       </c>
       <c r="B993" t="n">
-        <v>816</v>
+        <v>1254</v>
       </c>
       <c r="C993" t="n">
-        <v>219150</v>
+        <v>167714.73</v>
       </c>
     </row>
     <row r="994">
@@ -11366,10 +11366,10 @@
         <v>46266</v>
       </c>
       <c r="B994" t="n">
-        <v>2671</v>
+        <v>816</v>
       </c>
       <c r="C994" t="n">
-        <v>65448</v>
+        <v>231325</v>
       </c>
     </row>
     <row r="995">
@@ -11377,10 +11377,10 @@
         <v>46266</v>
       </c>
       <c r="B995" t="n">
-        <v>2705</v>
+        <v>2671</v>
       </c>
       <c r="C995" t="n">
-        <v>146610</v>
+        <v>69084</v>
       </c>
     </row>
     <row r="996">
@@ -11388,10 +11388,10 @@
         <v>46266</v>
       </c>
       <c r="B996" t="n">
-        <v>2333</v>
+        <v>2705</v>
       </c>
       <c r="C996" t="n">
-        <v>126288</v>
+        <v>154755</v>
       </c>
     </row>
     <row r="997">
@@ -11399,10 +11399,10 @@
         <v>46266</v>
       </c>
       <c r="B997" t="n">
-        <v>2440</v>
+        <v>2333</v>
       </c>
       <c r="C997" t="n">
-        <v>73620</v>
+        <v>133304</v>
       </c>
     </row>
     <row r="998">
@@ -11410,10 +11410,10 @@
         <v>46266</v>
       </c>
       <c r="B998" t="n">
-        <v>2448</v>
+        <v>2440</v>
       </c>
       <c r="C998" t="n">
-        <v>16362</v>
+        <v>77710</v>
       </c>
     </row>
     <row r="999">
@@ -11421,10 +11421,10 @@
         <v>46266</v>
       </c>
       <c r="B999" t="n">
-        <v>2310</v>
+        <v>2448</v>
       </c>
       <c r="C999" t="n">
-        <v>56196</v>
+        <v>17271</v>
       </c>
     </row>
     <row r="1000">
@@ -11432,10 +11432,10 @@
         <v>46266</v>
       </c>
       <c r="B1000" t="n">
-        <v>2809</v>
+        <v>2310</v>
       </c>
       <c r="C1000" t="n">
-        <v>56196</v>
+        <v>59318</v>
       </c>
     </row>
     <row r="1001">
@@ -11443,10 +11443,10 @@
         <v>46266</v>
       </c>
       <c r="B1001" t="n">
-        <v>2548</v>
+        <v>2809</v>
       </c>
       <c r="C1001" t="n">
-        <v>47880</v>
+        <v>59318</v>
       </c>
     </row>
     <row r="1002">
@@ -11454,10 +11454,10 @@
         <v>46266</v>
       </c>
       <c r="B1002" t="n">
-        <v>451</v>
+        <v>2548</v>
       </c>
       <c r="C1002" t="n">
-        <v>196362</v>
+        <v>50540</v>
       </c>
     </row>
     <row r="1003">
@@ -11465,10 +11465,10 @@
         <v>46266</v>
       </c>
       <c r="B1003" t="n">
-        <v>933</v>
+        <v>451</v>
       </c>
       <c r="C1003" t="n">
-        <v>66672</v>
+        <v>207271</v>
       </c>
     </row>
     <row r="1004">
@@ -11476,10 +11476,10 @@
         <v>46266</v>
       </c>
       <c r="B1004" t="n">
-        <v>2702</v>
+        <v>933</v>
       </c>
       <c r="C1004" t="n">
-        <v>66672</v>
+        <v>70376</v>
       </c>
     </row>
     <row r="1005">
@@ -11487,10 +11487,10 @@
         <v>46266</v>
       </c>
       <c r="B1005" t="n">
-        <v>2549</v>
+        <v>2702</v>
       </c>
       <c r="C1005" t="n">
-        <v>23184</v>
+        <v>70376</v>
       </c>
     </row>
     <row r="1006">
@@ -11498,10 +11498,10 @@
         <v>46266</v>
       </c>
       <c r="B1006" t="n">
-        <v>535</v>
+        <v>2549</v>
       </c>
       <c r="C1006" t="n">
-        <v>302724</v>
+        <v>24472</v>
       </c>
     </row>
     <row r="1007">
@@ -11509,10 +11509,10 @@
         <v>46266</v>
       </c>
       <c r="B1007" t="n">
-        <v>1117</v>
+        <v>535</v>
       </c>
       <c r="C1007" t="n">
-        <v>284634</v>
+        <v>319542</v>
       </c>
     </row>
     <row r="1008">
@@ -11520,10 +11520,10 @@
         <v>46266</v>
       </c>
       <c r="B1008" t="n">
-        <v>2109</v>
+        <v>1117</v>
       </c>
       <c r="C1008" t="n">
-        <v>0</v>
+        <v>300447</v>
       </c>
     </row>
     <row r="1009">
@@ -11531,10 +11531,10 @@
         <v>46266</v>
       </c>
       <c r="B1009" t="n">
-        <v>530</v>
+        <v>2109</v>
       </c>
       <c r="C1009" t="n">
-        <v>199692</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1010">
@@ -11542,10 +11542,10 @@
         <v>46266</v>
       </c>
       <c r="B1010" t="n">
-        <v>358</v>
+        <v>530</v>
       </c>
       <c r="C1010" t="n">
-        <v>278172</v>
+        <v>210786</v>
       </c>
     </row>
     <row r="1011">
@@ -11553,10 +11553,10 @@
         <v>46266</v>
       </c>
       <c r="B1011" t="n">
-        <v>2498</v>
+        <v>358</v>
       </c>
       <c r="C1011" t="n">
-        <v>45432</v>
+        <v>293626</v>
       </c>
     </row>
     <row r="1012">
@@ -11564,10 +11564,10 @@
         <v>46266</v>
       </c>
       <c r="B1012" t="n">
-        <v>2381</v>
+        <v>2498</v>
       </c>
       <c r="C1012" t="n">
-        <v>64908</v>
+        <v>47956</v>
       </c>
     </row>
     <row r="1013">
@@ -11575,10 +11575,10 @@
         <v>46266</v>
       </c>
       <c r="B1013" t="n">
-        <v>2695</v>
+        <v>2381</v>
       </c>
       <c r="C1013" t="n">
-        <v>39042</v>
+        <v>68514</v>
       </c>
     </row>
     <row r="1014">
@@ -11586,10 +11586,10 @@
         <v>46266</v>
       </c>
       <c r="B1014" t="n">
-        <v>2744</v>
+        <v>2695</v>
       </c>
       <c r="C1014" t="n">
-        <v>49090.92</v>
+        <v>41211</v>
       </c>
     </row>
     <row r="1015">
@@ -11597,10 +11597,10 @@
         <v>46266</v>
       </c>
       <c r="B1015" t="n">
-        <v>2750</v>
+        <v>2744</v>
       </c>
       <c r="C1015" t="n">
-        <v>49086</v>
+        <v>51818.19</v>
       </c>
     </row>
     <row r="1016">
@@ -11608,10 +11608,10 @@
         <v>46266</v>
       </c>
       <c r="B1016" t="n">
-        <v>2131</v>
+        <v>2750</v>
       </c>
       <c r="C1016" t="n">
-        <v>98172</v>
+        <v>51813</v>
       </c>
     </row>
     <row r="1017">
@@ -11619,10 +11619,10 @@
         <v>46266</v>
       </c>
       <c r="B1017" t="n">
-        <v>818</v>
+        <v>2131</v>
       </c>
       <c r="C1017" t="n">
-        <v>327258</v>
+        <v>103626</v>
       </c>
     </row>
     <row r="1018">
@@ -11630,10 +11630,10 @@
         <v>46266</v>
       </c>
       <c r="B1018" t="n">
-        <v>2566</v>
+        <v>818</v>
       </c>
       <c r="C1018" t="n">
-        <v>65448</v>
+        <v>345439</v>
       </c>
     </row>
     <row r="1019">
@@ -11641,10 +11641,10 @@
         <v>46266</v>
       </c>
       <c r="B1019" t="n">
-        <v>132</v>
+        <v>2566</v>
       </c>
       <c r="C1019" t="n">
-        <v>613620</v>
+        <v>69084</v>
       </c>
     </row>
     <row r="1020">
@@ -11652,10 +11652,10 @@
         <v>46266</v>
       </c>
       <c r="B1020" t="n">
-        <v>2431</v>
+        <v>132</v>
       </c>
       <c r="C1020" t="n">
-        <v>150534</v>
+        <v>647710</v>
       </c>
     </row>
     <row r="1021">
@@ -11663,10 +11663,10 @@
         <v>46266</v>
       </c>
       <c r="B1021" t="n">
-        <v>2249</v>
+        <v>2431</v>
       </c>
       <c r="C1021" t="n">
-        <v>159804</v>
+        <v>158897</v>
       </c>
     </row>
     <row r="1022">
@@ -11674,10 +11674,10 @@
         <v>46266</v>
       </c>
       <c r="B1022" t="n">
-        <v>1585</v>
+        <v>2249</v>
       </c>
       <c r="C1022" t="n">
-        <v>135036</v>
+        <v>168682</v>
       </c>
     </row>
     <row r="1023">
@@ -11685,10 +11685,10 @@
         <v>46266</v>
       </c>
       <c r="B1023" t="n">
-        <v>2325</v>
+        <v>1585</v>
       </c>
       <c r="C1023" t="n">
-        <v>130536</v>
+        <v>142538</v>
       </c>
     </row>
     <row r="1024">
@@ -11696,10 +11696,10 @@
         <v>46266</v>
       </c>
       <c r="B1024" t="n">
-        <v>2190</v>
+        <v>2325</v>
       </c>
       <c r="C1024" t="n">
-        <v>184086</v>
+        <v>137788</v>
       </c>
     </row>
     <row r="1025">
@@ -11707,10 +11707,10 @@
         <v>46266</v>
       </c>
       <c r="B1025" t="n">
-        <v>1466</v>
+        <v>2190</v>
       </c>
       <c r="C1025" t="n">
-        <v>331362</v>
+        <v>194313</v>
       </c>
     </row>
     <row r="1026">
@@ -11718,10 +11718,10 @@
         <v>46266</v>
       </c>
       <c r="B1026" t="n">
-        <v>2659</v>
+        <v>1466</v>
       </c>
       <c r="C1026" t="n">
-        <v>100638</v>
+        <v>349771</v>
       </c>
     </row>
     <row r="1027">
@@ -11729,10 +11729,10 @@
         <v>46266</v>
       </c>
       <c r="B1027" t="n">
-        <v>634</v>
+        <v>2659</v>
       </c>
       <c r="C1027" t="n">
-        <v>450000</v>
+        <v>106229</v>
       </c>
     </row>
     <row r="1028">
@@ -11740,10 +11740,10 @@
         <v>46266</v>
       </c>
       <c r="B1028" t="n">
-        <v>2804</v>
+        <v>1384</v>
       </c>
       <c r="C1028" t="n">
-        <v>81810</v>
+        <v>388626</v>
       </c>
     </row>
     <row r="1029">
@@ -11751,10 +11751,10 @@
         <v>46266</v>
       </c>
       <c r="B1029" t="n">
-        <v>2375</v>
+        <v>634</v>
       </c>
       <c r="C1029" t="n">
-        <v>270000</v>
+        <v>475000</v>
       </c>
     </row>
     <row r="1030">
@@ -11762,10 +11762,10 @@
         <v>46266</v>
       </c>
       <c r="B1030" t="n">
-        <v>2601</v>
+        <v>2804</v>
       </c>
       <c r="C1030" t="n">
-        <v>225000</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1031">
@@ -11773,10 +11773,10 @@
         <v>46266</v>
       </c>
       <c r="B1031" t="n">
-        <v>952</v>
+        <v>2375</v>
       </c>
       <c r="C1031" t="n">
-        <v>81810</v>
+        <v>285000</v>
       </c>
     </row>
     <row r="1032">
@@ -11784,10 +11784,10 @@
         <v>46266</v>
       </c>
       <c r="B1032" t="n">
-        <v>571</v>
+        <v>2601</v>
       </c>
       <c r="C1032" t="n">
-        <v>520758</v>
+        <v>237500</v>
       </c>
     </row>
     <row r="1033">
@@ -11795,10 +11795,10 @@
         <v>46266</v>
       </c>
       <c r="B1033" t="n">
-        <v>2697</v>
+        <v>952</v>
       </c>
       <c r="C1033" t="n">
-        <v>158670</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1034">
@@ -11806,10 +11806,10 @@
         <v>46266</v>
       </c>
       <c r="B1034" t="n">
-        <v>2678</v>
+        <v>571</v>
       </c>
       <c r="C1034" t="n">
-        <v>274518</v>
+        <v>549689</v>
       </c>
     </row>
     <row r="1035">
@@ -11817,10 +11817,10 @@
         <v>46266</v>
       </c>
       <c r="B1035" t="n">
-        <v>2768</v>
+        <v>2697</v>
       </c>
       <c r="C1035" t="n">
-        <v>287298</v>
+        <v>167485</v>
       </c>
     </row>
     <row r="1036">
@@ -11828,10 +11828,10 @@
         <v>46266</v>
       </c>
       <c r="B1036" t="n">
-        <v>2359</v>
+        <v>2678</v>
       </c>
       <c r="C1036" t="n">
-        <v>87138</v>
+        <v>289769</v>
       </c>
     </row>
     <row r="1037">
@@ -11839,10 +11839,10 @@
         <v>46266</v>
       </c>
       <c r="B1037" t="n">
-        <v>353</v>
+        <v>2768</v>
       </c>
       <c r="C1037" t="n">
-        <v>283068</v>
+        <v>303259</v>
       </c>
     </row>
     <row r="1038">
@@ -11850,10 +11850,10 @@
         <v>46266</v>
       </c>
       <c r="B1038" t="n">
-        <v>2026</v>
+        <v>2359</v>
       </c>
       <c r="C1038" t="n">
-        <v>234540</v>
+        <v>91979</v>
       </c>
     </row>
     <row r="1039">
@@ -11861,10 +11861,10 @@
         <v>46266</v>
       </c>
       <c r="B1039" t="n">
-        <v>1105</v>
+        <v>353</v>
       </c>
       <c r="C1039" t="n">
-        <v>0</v>
+        <v>298805.42</v>
       </c>
     </row>
     <row r="1040">
@@ -11872,10 +11872,10 @@
         <v>46266</v>
       </c>
       <c r="B1040" t="n">
-        <v>2345</v>
+        <v>2026</v>
       </c>
       <c r="C1040" t="n">
-        <v>51498</v>
+        <v>247581.62</v>
       </c>
     </row>
     <row r="1041">
@@ -11883,10 +11883,10 @@
         <v>46266</v>
       </c>
       <c r="B1041" t="n">
-        <v>2789</v>
+        <v>1105</v>
       </c>
       <c r="C1041" t="n">
-        <v>139086</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1042">
@@ -11894,10 +11894,10 @@
         <v>46266</v>
       </c>
       <c r="B1042" t="n">
-        <v>569</v>
+        <v>2345</v>
       </c>
       <c r="C1042" t="n">
-        <v>2343204</v>
+        <v>54359</v>
       </c>
     </row>
     <row r="1043">
@@ -11905,10 +11905,10 @@
         <v>46266</v>
       </c>
       <c r="B1043" t="n">
-        <v>2822</v>
+        <v>2789</v>
       </c>
       <c r="C1043" t="n">
-        <v>110448</v>
+        <v>146813</v>
       </c>
     </row>
     <row r="1044">
@@ -11916,10 +11916,10 @@
         <v>46266</v>
       </c>
       <c r="B1044" t="n">
-        <v>2728</v>
+        <v>569</v>
       </c>
       <c r="C1044" t="n">
-        <v>8172</v>
+        <v>2473382</v>
       </c>
     </row>
     <row r="1045">
@@ -11927,10 +11927,10 @@
         <v>46266</v>
       </c>
       <c r="B1045" t="n">
-        <v>2488</v>
+        <v>2822</v>
       </c>
       <c r="C1045" t="n">
-        <v>81810</v>
+        <v>116584</v>
       </c>
     </row>
     <row r="1046">
@@ -11938,10 +11938,10 @@
         <v>46266</v>
       </c>
       <c r="B1046" t="n">
-        <v>2791</v>
+        <v>2728</v>
       </c>
       <c r="C1046" t="n">
-        <v>80746.39999999999</v>
+        <v>8626</v>
       </c>
     </row>
     <row r="1047">
@@ -11949,10 +11949,10 @@
         <v>46266</v>
       </c>
       <c r="B1047" t="n">
-        <v>2577</v>
+        <v>2488</v>
       </c>
       <c r="C1047" t="n">
-        <v>72957.37</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1048">
@@ -11960,10 +11960,10 @@
         <v>46266</v>
       </c>
       <c r="B1048" t="n">
-        <v>2069</v>
+        <v>2791</v>
       </c>
       <c r="C1048" t="n">
-        <v>147258</v>
+        <v>85232.3</v>
       </c>
     </row>
     <row r="1049">
@@ -11971,10 +11971,10 @@
         <v>46266</v>
       </c>
       <c r="B1049" t="n">
-        <v>2082</v>
+        <v>2577</v>
       </c>
       <c r="C1049" t="n">
-        <v>136278</v>
+        <v>77010.55</v>
       </c>
     </row>
     <row r="1050">
@@ -11982,10 +11982,10 @@
         <v>46266</v>
       </c>
       <c r="B1050" t="n">
-        <v>781</v>
+        <v>2069</v>
       </c>
       <c r="C1050" t="n">
-        <v>106362</v>
+        <v>155439</v>
       </c>
     </row>
     <row r="1051">
@@ -11993,10 +11993,10 @@
         <v>46266</v>
       </c>
       <c r="B1051" t="n">
-        <v>744</v>
+        <v>2082</v>
       </c>
       <c r="C1051" t="n">
-        <v>34038</v>
+        <v>143849</v>
       </c>
     </row>
     <row r="1052">
@@ -12004,10 +12004,10 @@
         <v>46266</v>
       </c>
       <c r="B1052" t="n">
-        <v>2223</v>
+        <v>781</v>
       </c>
       <c r="C1052" t="n">
-        <v>107946</v>
+        <v>112271</v>
       </c>
     </row>
     <row r="1053">
@@ -12015,10 +12015,10 @@
         <v>46266</v>
       </c>
       <c r="B1053" t="n">
-        <v>2452</v>
+        <v>744</v>
       </c>
       <c r="C1053" t="n">
-        <v>57258</v>
+        <v>35929</v>
       </c>
     </row>
     <row r="1054">
@@ -12026,10 +12026,10 @@
         <v>46266</v>
       </c>
       <c r="B1054" t="n">
-        <v>970</v>
+        <v>2223</v>
       </c>
       <c r="C1054" t="n">
-        <v>56196</v>
+        <v>113943</v>
       </c>
     </row>
     <row r="1055">
@@ -12037,10 +12037,10 @@
         <v>46266</v>
       </c>
       <c r="B1055" t="n">
-        <v>2550</v>
+        <v>2452</v>
       </c>
       <c r="C1055" t="n">
-        <v>49896</v>
+        <v>60439</v>
       </c>
     </row>
     <row r="1056">
@@ -12048,10 +12048,10 @@
         <v>46266</v>
       </c>
       <c r="B1056" t="n">
-        <v>768</v>
+        <v>970</v>
       </c>
       <c r="C1056" t="n">
-        <v>106362</v>
+        <v>59318</v>
       </c>
     </row>
     <row r="1057">
@@ -12059,10 +12059,10 @@
         <v>46266</v>
       </c>
       <c r="B1057" t="n">
-        <v>1075</v>
+        <v>2550</v>
       </c>
       <c r="C1057" t="n">
-        <v>370620</v>
+        <v>52668</v>
       </c>
     </row>
     <row r="1058">
@@ -12070,10 +12070,10 @@
         <v>46266</v>
       </c>
       <c r="B1058" t="n">
-        <v>664</v>
+        <v>768</v>
       </c>
       <c r="C1058" t="n">
-        <v>211896</v>
+        <v>112271</v>
       </c>
     </row>
     <row r="1059">
@@ -12081,10 +12081,10 @@
         <v>46266</v>
       </c>
       <c r="B1059" t="n">
-        <v>2555</v>
+        <v>1075</v>
       </c>
       <c r="C1059" t="n">
-        <v>33966</v>
+        <v>391210</v>
       </c>
     </row>
     <row r="1060">
@@ -12092,10 +12092,10 @@
         <v>46266</v>
       </c>
       <c r="B1060" t="n">
-        <v>2627</v>
+        <v>664</v>
       </c>
       <c r="C1060" t="n">
-        <v>19944</v>
+        <v>223668</v>
       </c>
     </row>
     <row r="1061">
@@ -12103,10 +12103,10 @@
         <v>46266</v>
       </c>
       <c r="B1061" t="n">
-        <v>2557</v>
+        <v>2555</v>
       </c>
       <c r="C1061" t="n">
-        <v>21096</v>
+        <v>35853</v>
       </c>
     </row>
     <row r="1062">
@@ -12114,10 +12114,10 @@
         <v>46266</v>
       </c>
       <c r="B1062" t="n">
-        <v>2551</v>
+        <v>2627</v>
       </c>
       <c r="C1062" t="n">
-        <v>16758</v>
+        <v>21052</v>
       </c>
     </row>
     <row r="1063">
@@ -12125,10 +12125,10 @@
         <v>46266</v>
       </c>
       <c r="B1063" t="n">
-        <v>2463</v>
+        <v>2557</v>
       </c>
       <c r="C1063" t="n">
-        <v>261990</v>
+        <v>22268</v>
       </c>
     </row>
     <row r="1064">
@@ -12136,10 +12136,10 @@
         <v>46266</v>
       </c>
       <c r="B1064" t="n">
-        <v>2279</v>
+        <v>2551</v>
       </c>
       <c r="C1064" t="n">
-        <v>197658</v>
+        <v>17689</v>
       </c>
     </row>
     <row r="1065">
@@ -12147,10 +12147,10 @@
         <v>46266</v>
       </c>
       <c r="B1065" t="n">
-        <v>631</v>
+        <v>2463</v>
       </c>
       <c r="C1065" t="n">
-        <v>286362</v>
+        <v>276545</v>
       </c>
     </row>
     <row r="1066">
@@ -12158,10 +12158,10 @@
         <v>46266</v>
       </c>
       <c r="B1066" t="n">
-        <v>2251</v>
+        <v>2279</v>
       </c>
       <c r="C1066" t="n">
-        <v>175356</v>
+        <v>208639</v>
       </c>
     </row>
     <row r="1067">
@@ -12169,10 +12169,10 @@
         <v>46266</v>
       </c>
       <c r="B1067" t="n">
-        <v>1653</v>
+        <v>631</v>
       </c>
       <c r="C1067" t="n">
-        <v>265896</v>
+        <v>302271</v>
       </c>
     </row>
     <row r="1068">
@@ -12180,10 +12180,10 @@
         <v>46266</v>
       </c>
       <c r="B1068" t="n">
-        <v>1293</v>
+        <v>2251</v>
       </c>
       <c r="C1068" t="n">
-        <v>339534</v>
+        <v>185098</v>
       </c>
     </row>
     <row r="1069">
@@ -12191,10 +12191,10 @@
         <v>46266</v>
       </c>
       <c r="B1069" t="n">
-        <v>360</v>
+        <v>1653</v>
       </c>
       <c r="C1069" t="n">
-        <v>409086</v>
+        <v>280668</v>
       </c>
     </row>
     <row r="1070">
@@ -12202,10 +12202,10 @@
         <v>46266</v>
       </c>
       <c r="B1070" t="n">
-        <v>1063</v>
+        <v>1293</v>
       </c>
       <c r="C1070" t="n">
-        <v>297450</v>
+        <v>358397</v>
       </c>
     </row>
     <row r="1071">
@@ -12213,10 +12213,10 @@
         <v>46266</v>
       </c>
       <c r="B1071" t="n">
-        <v>2273</v>
+        <v>360</v>
       </c>
       <c r="C1071" t="n">
-        <v>173520</v>
+        <v>431813</v>
       </c>
     </row>
     <row r="1072">
@@ -12224,10 +12224,10 @@
         <v>46266</v>
       </c>
       <c r="B1072" t="n">
-        <v>2757</v>
+        <v>1063</v>
       </c>
       <c r="C1072" t="n">
-        <v>57272.76</v>
+        <v>313975</v>
       </c>
     </row>
     <row r="1073">
@@ -12235,10 +12235,10 @@
         <v>46266</v>
       </c>
       <c r="B1073" t="n">
-        <v>2795</v>
+        <v>2273</v>
       </c>
       <c r="C1073" t="n">
-        <v>49090.92</v>
+        <v>183160</v>
       </c>
     </row>
     <row r="1074">
@@ -12246,10 +12246,10 @@
         <v>46266</v>
       </c>
       <c r="B1074" t="n">
-        <v>2722</v>
+        <v>2757</v>
       </c>
       <c r="C1074" t="n">
-        <v>49086</v>
+        <v>60454.57</v>
       </c>
     </row>
     <row r="1075">
@@ -12257,10 +12257,10 @@
         <v>46266</v>
       </c>
       <c r="B1075" t="n">
-        <v>2718</v>
+        <v>2795</v>
       </c>
       <c r="C1075" t="n">
-        <v>65448</v>
+        <v>51818.19</v>
       </c>
     </row>
     <row r="1076">
@@ -12268,10 +12268,10 @@
         <v>46266</v>
       </c>
       <c r="B1076" t="n">
-        <v>595</v>
+        <v>2722</v>
       </c>
       <c r="C1076" t="n">
-        <v>450000</v>
+        <v>51813</v>
       </c>
     </row>
     <row r="1077">
@@ -12279,10 +12279,10 @@
         <v>46266</v>
       </c>
       <c r="B1077" t="n">
-        <v>890</v>
+        <v>2718</v>
       </c>
       <c r="C1077" t="n">
-        <v>572724</v>
+        <v>69084</v>
       </c>
     </row>
     <row r="1078">
@@ -12290,10 +12290,10 @@
         <v>46266</v>
       </c>
       <c r="B1078" t="n">
-        <v>2652</v>
+        <v>595</v>
       </c>
       <c r="C1078" t="n">
-        <v>106362</v>
+        <v>475000</v>
       </c>
     </row>
     <row r="1079">
@@ -12301,10 +12301,10 @@
         <v>46266</v>
       </c>
       <c r="B1079" t="n">
-        <v>2714</v>
+        <v>890</v>
       </c>
       <c r="C1079" t="n">
-        <v>294534</v>
+        <v>604542</v>
       </c>
     </row>
     <row r="1080">
@@ -12312,10 +12312,10 @@
         <v>46266</v>
       </c>
       <c r="B1080" t="n">
-        <v>1869</v>
+        <v>2652</v>
       </c>
       <c r="C1080" t="n">
-        <v>188172</v>
+        <v>112271</v>
       </c>
     </row>
     <row r="1081">
@@ -12323,10 +12323,10 @@
         <v>46266</v>
       </c>
       <c r="B1081" t="n">
-        <v>400</v>
+        <v>2714</v>
       </c>
       <c r="C1081" t="n">
-        <v>155448</v>
+        <v>310897</v>
       </c>
     </row>
     <row r="1082">
@@ -12334,10 +12334,10 @@
         <v>46266</v>
       </c>
       <c r="B1082" t="n">
-        <v>1907</v>
+        <v>1869</v>
       </c>
       <c r="C1082" t="n">
-        <v>303534</v>
+        <v>198626</v>
       </c>
     </row>
     <row r="1083">
@@ -12345,10 +12345,10 @@
         <v>46266</v>
       </c>
       <c r="B1083" t="n">
-        <v>1996</v>
+        <v>400</v>
       </c>
       <c r="C1083" t="n">
-        <v>191862</v>
+        <v>164084</v>
       </c>
     </row>
     <row r="1084">
@@ -12356,10 +12356,10 @@
         <v>46266</v>
       </c>
       <c r="B1084" t="n">
-        <v>1890</v>
+        <v>1907</v>
       </c>
       <c r="C1084" t="n">
-        <v>258662.19</v>
+        <v>320397</v>
       </c>
     </row>
     <row r="1085">
@@ -12367,10 +12367,10 @@
         <v>46266</v>
       </c>
       <c r="B1085" t="n">
-        <v>2114</v>
+        <v>1996</v>
       </c>
       <c r="C1085" t="n">
-        <v>150300</v>
+        <v>202521</v>
       </c>
     </row>
     <row r="1086">
@@ -12378,10 +12378,10 @@
         <v>46266</v>
       </c>
       <c r="B1086" t="n">
-        <v>2330</v>
+        <v>1890</v>
       </c>
       <c r="C1086" t="n">
-        <v>219906</v>
+        <v>273032.3</v>
       </c>
     </row>
     <row r="1087">
@@ -12389,10 +12389,10 @@
         <v>46266</v>
       </c>
       <c r="B1087" t="n">
-        <v>2000</v>
+        <v>2114</v>
       </c>
       <c r="C1087" t="n">
-        <v>0</v>
+        <v>158650</v>
       </c>
     </row>
     <row r="1088">
@@ -12400,10 +12400,10 @@
         <v>46266</v>
       </c>
       <c r="B1088" t="n">
-        <v>2591</v>
+        <v>2330</v>
       </c>
       <c r="C1088" t="n">
-        <v>0</v>
+        <v>232123</v>
       </c>
     </row>
     <row r="1089">
@@ -12411,7 +12411,7 @@
         <v>46266</v>
       </c>
       <c r="B1089" t="n">
-        <v>2639</v>
+        <v>2000</v>
       </c>
       <c r="C1089" t="n">
         <v>0</v>
@@ -12422,10 +12422,10 @@
         <v>46266</v>
       </c>
       <c r="B1090" t="n">
-        <v>931</v>
+        <v>2591</v>
       </c>
       <c r="C1090" t="n">
-        <v>77256</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1091">
@@ -12433,10 +12433,10 @@
         <v>46266</v>
       </c>
       <c r="B1091" t="n">
-        <v>951</v>
+        <v>2639</v>
       </c>
       <c r="C1091" t="n">
-        <v>94086</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1092">
@@ -12444,10 +12444,10 @@
         <v>46266</v>
       </c>
       <c r="B1092" t="n">
-        <v>2449</v>
+        <v>2629</v>
       </c>
       <c r="C1092" t="n">
-        <v>32724</v>
+        <v>59318</v>
       </c>
     </row>
     <row r="1093">
@@ -12455,10 +12455,10 @@
         <v>46266</v>
       </c>
       <c r="B1093" t="n">
-        <v>610</v>
+        <v>951</v>
       </c>
       <c r="C1093" t="n">
-        <v>666810</v>
+        <v>99313</v>
       </c>
     </row>
     <row r="1094">
@@ -12466,10 +12466,10 @@
         <v>46266</v>
       </c>
       <c r="B1094" t="n">
-        <v>2761</v>
+        <v>2449</v>
       </c>
       <c r="C1094" t="n">
-        <v>66672</v>
+        <v>34542</v>
       </c>
     </row>
     <row r="1095">
@@ -12477,10 +12477,10 @@
         <v>46266</v>
       </c>
       <c r="B1095" t="n">
-        <v>483</v>
+        <v>610</v>
       </c>
       <c r="C1095" t="n">
-        <v>362448</v>
+        <v>703855</v>
       </c>
     </row>
     <row r="1096">
@@ -12488,10 +12488,10 @@
         <v>46266</v>
       </c>
       <c r="B1096" t="n">
-        <v>2015</v>
+        <v>2761</v>
       </c>
       <c r="C1096" t="n">
-        <v>302724</v>
+        <v>70376</v>
       </c>
     </row>
     <row r="1097">
@@ -12499,10 +12499,10 @@
         <v>46266</v>
       </c>
       <c r="B1097" t="n">
-        <v>1478</v>
+        <v>483</v>
       </c>
       <c r="C1097" t="n">
-        <v>442764</v>
+        <v>382584</v>
       </c>
     </row>
     <row r="1098">
@@ -12510,10 +12510,10 @@
         <v>46266</v>
       </c>
       <c r="B1098" t="n">
-        <v>424</v>
+        <v>2015</v>
       </c>
       <c r="C1098" t="n">
-        <v>197658</v>
+        <v>319542</v>
       </c>
     </row>
     <row r="1099">
@@ -12521,10 +12521,10 @@
         <v>46266</v>
       </c>
       <c r="B1099" t="n">
-        <v>1261</v>
+        <v>1478</v>
       </c>
       <c r="C1099" t="n">
-        <v>0</v>
+        <v>467362</v>
       </c>
     </row>
     <row r="1100">
@@ -12532,10 +12532,10 @@
         <v>46266</v>
       </c>
       <c r="B1100" t="n">
-        <v>477</v>
+        <v>424</v>
       </c>
       <c r="C1100" t="n">
-        <v>211626</v>
+        <v>208639</v>
       </c>
     </row>
     <row r="1101">
@@ -12543,10 +12543,10 @@
         <v>46266</v>
       </c>
       <c r="B1101" t="n">
-        <v>1810</v>
+        <v>1261</v>
       </c>
       <c r="C1101" t="n">
-        <v>32778</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1102">
@@ -12554,10 +12554,10 @@
         <v>46266</v>
       </c>
       <c r="B1102" t="n">
-        <v>2826</v>
+        <v>477</v>
       </c>
       <c r="C1102" t="n">
-        <v>57272.76</v>
+        <v>223383</v>
       </c>
     </row>
     <row r="1103">
@@ -12565,10 +12565,10 @@
         <v>46266</v>
       </c>
       <c r="B1103" t="n">
-        <v>2561</v>
+        <v>1810</v>
       </c>
       <c r="C1103" t="n">
-        <v>12024</v>
+        <v>34599</v>
       </c>
     </row>
     <row r="1104">
@@ -12576,10 +12576,10 @@
         <v>46266</v>
       </c>
       <c r="B1104" t="n">
-        <v>2653</v>
+        <v>2826</v>
       </c>
       <c r="C1104" t="n">
-        <v>49090.92</v>
+        <v>60454.57</v>
       </c>
     </row>
     <row r="1105">
@@ -12587,10 +12587,10 @@
         <v>46266</v>
       </c>
       <c r="B1105" t="n">
-        <v>2829</v>
+        <v>2561</v>
       </c>
       <c r="C1105" t="n">
-        <v>49090.92</v>
+        <v>12692</v>
       </c>
     </row>
     <row r="1106">
@@ -12598,10 +12598,10 @@
         <v>46266</v>
       </c>
       <c r="B1106" t="n">
-        <v>2643</v>
+        <v>2653</v>
       </c>
       <c r="C1106" t="n">
-        <v>24156</v>
+        <v>51818.19</v>
       </c>
     </row>
     <row r="1107">
@@ -12609,10 +12609,10 @@
         <v>46266</v>
       </c>
       <c r="B1107" t="n">
-        <v>2794</v>
+        <v>2829</v>
       </c>
       <c r="C1107" t="n">
-        <v>73620</v>
+        <v>51818.19</v>
       </c>
     </row>
     <row r="1108">
@@ -12620,10 +12620,10 @@
         <v>46266</v>
       </c>
       <c r="B1108" t="n">
-        <v>2655</v>
+        <v>2643</v>
       </c>
       <c r="C1108" t="n">
-        <v>90000</v>
+        <v>25498</v>
       </c>
     </row>
     <row r="1109">
@@ -12631,10 +12631,10 @@
         <v>46266</v>
       </c>
       <c r="B1109" t="n">
-        <v>1456</v>
+        <v>2794</v>
       </c>
       <c r="C1109" t="n">
-        <v>630234</v>
+        <v>77710</v>
       </c>
     </row>
     <row r="1110">
@@ -12642,10 +12642,10 @@
         <v>46266</v>
       </c>
       <c r="B1110" t="n">
-        <v>2606</v>
+        <v>2655</v>
       </c>
       <c r="C1110" t="n">
-        <v>193572</v>
+        <v>95000</v>
       </c>
     </row>
     <row r="1111">
@@ -12653,10 +12653,10 @@
         <v>46266</v>
       </c>
       <c r="B1111" t="n">
-        <v>1142</v>
+        <v>1456</v>
       </c>
       <c r="C1111" t="n">
-        <v>351036</v>
+        <v>665247</v>
       </c>
     </row>
     <row r="1112">
@@ -12664,10 +12664,10 @@
         <v>46266</v>
       </c>
       <c r="B1112" t="n">
-        <v>1450</v>
+        <v>2606</v>
       </c>
       <c r="C1112" t="n">
-        <v>223002</v>
+        <v>204326</v>
       </c>
     </row>
     <row r="1113">
@@ -12675,10 +12675,10 @@
         <v>46266</v>
       </c>
       <c r="B1113" t="n">
-        <v>2133</v>
+        <v>1142</v>
       </c>
       <c r="C1113" t="n">
-        <v>520758</v>
+        <v>370538</v>
       </c>
     </row>
     <row r="1114">
@@ -12686,10 +12686,10 @@
         <v>46266</v>
       </c>
       <c r="B1114" t="n">
-        <v>522</v>
+        <v>1450</v>
       </c>
       <c r="C1114" t="n">
-        <v>159534</v>
+        <v>235391</v>
       </c>
     </row>
     <row r="1115">
@@ -12697,10 +12697,10 @@
         <v>46266</v>
       </c>
       <c r="B1115" t="n">
-        <v>2696</v>
+        <v>2133</v>
       </c>
       <c r="C1115" t="n">
-        <v>215280</v>
+        <v>549689</v>
       </c>
     </row>
     <row r="1116">
@@ -12708,10 +12708,10 @@
         <v>46266</v>
       </c>
       <c r="B1116" t="n">
-        <v>2693</v>
+        <v>522</v>
       </c>
       <c r="C1116" t="n">
-        <v>0</v>
+        <v>168397</v>
       </c>
     </row>
     <row r="1117">
@@ -12719,10 +12719,10 @@
         <v>46266</v>
       </c>
       <c r="B1117" t="n">
-        <v>2692</v>
+        <v>2696</v>
       </c>
       <c r="C1117" t="n">
-        <v>61362</v>
+        <v>227240</v>
       </c>
     </row>
     <row r="1118">
@@ -12730,10 +12730,10 @@
         <v>46266</v>
       </c>
       <c r="B1118" t="n">
-        <v>2691</v>
+        <v>2693</v>
       </c>
       <c r="C1118" t="n">
-        <v>110448</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1119">
@@ -12741,10 +12741,10 @@
         <v>46266</v>
       </c>
       <c r="B1119" t="n">
-        <v>1632</v>
+        <v>2692</v>
       </c>
       <c r="C1119" t="n">
-        <v>204534</v>
+        <v>64771</v>
       </c>
     </row>
     <row r="1120">
@@ -12752,10 +12752,10 @@
         <v>46266</v>
       </c>
       <c r="B1120" t="n">
-        <v>2641</v>
+        <v>2691</v>
       </c>
       <c r="C1120" t="n">
-        <v>65448</v>
+        <v>116584</v>
       </c>
     </row>
     <row r="1121">
@@ -12763,10 +12763,10 @@
         <v>46266</v>
       </c>
       <c r="B1121" t="n">
-        <v>2197</v>
+        <v>1632</v>
       </c>
       <c r="C1121" t="n">
-        <v>163620</v>
+        <v>215897</v>
       </c>
     </row>
     <row r="1122">
@@ -12774,10 +12774,10 @@
         <v>46266</v>
       </c>
       <c r="B1122" t="n">
-        <v>609</v>
+        <v>2641</v>
       </c>
       <c r="C1122" t="n">
-        <v>180000</v>
+        <v>69084</v>
       </c>
     </row>
     <row r="1123">
@@ -12785,10 +12785,10 @@
         <v>46266</v>
       </c>
       <c r="B1123" t="n">
-        <v>1380</v>
+        <v>2197</v>
       </c>
       <c r="C1123" t="n">
-        <v>81810</v>
+        <v>172710</v>
       </c>
     </row>
     <row r="1124">
@@ -12796,10 +12796,10 @@
         <v>46266</v>
       </c>
       <c r="B1124" t="n">
-        <v>104</v>
+        <v>609</v>
       </c>
       <c r="C1124" t="n">
-        <v>245448</v>
+        <v>190000</v>
       </c>
     </row>
     <row r="1125">
@@ -12807,10 +12807,10 @@
         <v>46266</v>
       </c>
       <c r="B1125" t="n">
-        <v>2621</v>
+        <v>1380</v>
       </c>
       <c r="C1125" t="n">
-        <v>57258</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1126">
@@ -12818,10 +12818,10 @@
         <v>46266</v>
       </c>
       <c r="B1126" t="n">
-        <v>2786</v>
+        <v>104</v>
       </c>
       <c r="C1126" t="n">
-        <v>57258</v>
+        <v>259084</v>
       </c>
     </row>
     <row r="1127">
@@ -12829,10 +12829,10 @@
         <v>46266</v>
       </c>
       <c r="B1127" t="n">
-        <v>2784</v>
+        <v>2621</v>
       </c>
       <c r="C1127" t="n">
-        <v>34038</v>
+        <v>60439</v>
       </c>
     </row>
     <row r="1128">
@@ -12840,10 +12840,10 @@
         <v>46266</v>
       </c>
       <c r="B1128" t="n">
-        <v>2586</v>
+        <v>2786</v>
       </c>
       <c r="C1128" t="n">
-        <v>34038</v>
+        <v>60439</v>
       </c>
     </row>
     <row r="1129">
@@ -12851,10 +12851,10 @@
         <v>46266</v>
       </c>
       <c r="B1129" t="n">
-        <v>2145</v>
+        <v>2784</v>
       </c>
       <c r="C1129" t="n">
-        <v>105912</v>
+        <v>35929</v>
       </c>
     </row>
     <row r="1130">
@@ -12862,10 +12862,10 @@
         <v>46266</v>
       </c>
       <c r="B1130" t="n">
-        <v>2574</v>
+        <v>2586</v>
       </c>
       <c r="C1130" t="n">
-        <v>105912</v>
+        <v>35929</v>
       </c>
     </row>
     <row r="1131">
@@ -12873,10 +12873,10 @@
         <v>46266</v>
       </c>
       <c r="B1131" t="n">
-        <v>2492</v>
+        <v>2145</v>
       </c>
       <c r="C1131" t="n">
-        <v>116100</v>
+        <v>111796</v>
       </c>
     </row>
     <row r="1132">
@@ -12884,10 +12884,10 @@
         <v>46266</v>
       </c>
       <c r="B1132" t="n">
-        <v>629</v>
+        <v>2574</v>
       </c>
       <c r="C1132" t="n">
-        <v>361620</v>
+        <v>111796</v>
       </c>
     </row>
     <row r="1133">
@@ -12895,10 +12895,10 @@
         <v>46266</v>
       </c>
       <c r="B1133" t="n">
-        <v>966</v>
+        <v>2492</v>
       </c>
       <c r="C1133" t="n">
-        <v>66672</v>
+        <v>122550</v>
       </c>
     </row>
     <row r="1134">
@@ -12906,10 +12906,10 @@
         <v>46266</v>
       </c>
       <c r="B1134" t="n">
-        <v>2721</v>
+        <v>629</v>
       </c>
       <c r="C1134" t="n">
-        <v>66672</v>
+        <v>381710</v>
       </c>
     </row>
     <row r="1135">
@@ -12917,10 +12917,10 @@
         <v>46266</v>
       </c>
       <c r="B1135" t="n">
-        <v>2554</v>
+        <v>966</v>
       </c>
       <c r="C1135" t="n">
-        <v>20088</v>
+        <v>70376</v>
       </c>
     </row>
     <row r="1136">
@@ -12928,10 +12928,10 @@
         <v>46266</v>
       </c>
       <c r="B1136" t="n">
-        <v>2556</v>
+        <v>2721</v>
       </c>
       <c r="C1136" t="n">
-        <v>29538</v>
+        <v>70376</v>
       </c>
     </row>
     <row r="1137">
@@ -12939,10 +12939,10 @@
         <v>46266</v>
       </c>
       <c r="B1137" t="n">
-        <v>2546</v>
+        <v>2554</v>
       </c>
       <c r="C1137" t="n">
-        <v>19512</v>
+        <v>21204</v>
       </c>
     </row>
     <row r="1138">
@@ -12950,10 +12950,10 @@
         <v>46266</v>
       </c>
       <c r="B1138" t="n">
-        <v>42</v>
+        <v>2556</v>
       </c>
       <c r="C1138" t="n">
-        <v>1546362</v>
+        <v>31179</v>
       </c>
     </row>
     <row r="1139">
@@ -12961,10 +12961,10 @@
         <v>46266</v>
       </c>
       <c r="B1139" t="n">
-        <v>953</v>
+        <v>2546</v>
       </c>
       <c r="C1139" t="n">
-        <v>558540</v>
+        <v>20596</v>
       </c>
     </row>
     <row r="1140">
@@ -12972,10 +12972,10 @@
         <v>46266</v>
       </c>
       <c r="B1140" t="n">
-        <v>1137</v>
+        <v>42</v>
       </c>
       <c r="C1140" t="n">
-        <v>523620</v>
+        <v>1632271</v>
       </c>
     </row>
     <row r="1141">
@@ -12983,10 +12983,10 @@
         <v>46266</v>
       </c>
       <c r="B1141" t="n">
-        <v>675</v>
+        <v>953</v>
       </c>
       <c r="C1141" t="n">
-        <v>163620</v>
+        <v>589570</v>
       </c>
     </row>
     <row r="1142">
@@ -12994,10 +12994,10 @@
         <v>46266</v>
       </c>
       <c r="B1142" t="n">
-        <v>619</v>
+        <v>1137</v>
       </c>
       <c r="C1142" t="n">
-        <v>253008</v>
+        <v>552710</v>
       </c>
     </row>
     <row r="1143">
@@ -13005,10 +13005,10 @@
         <v>46266</v>
       </c>
       <c r="B1143" t="n">
-        <v>1299</v>
+        <v>675</v>
       </c>
       <c r="C1143" t="n">
-        <v>425736</v>
+        <v>172710</v>
       </c>
     </row>
     <row r="1144">
@@ -13016,10 +13016,10 @@
         <v>46266</v>
       </c>
       <c r="B1144" t="n">
-        <v>1064</v>
+        <v>619</v>
       </c>
       <c r="C1144" t="n">
-        <v>490392</v>
+        <v>267064</v>
       </c>
     </row>
     <row r="1145">
@@ -13027,10 +13027,10 @@
         <v>46266</v>
       </c>
       <c r="B1145" t="n">
-        <v>2308</v>
+        <v>1299</v>
       </c>
       <c r="C1145" t="n">
-        <v>167724</v>
+        <v>449388</v>
       </c>
     </row>
     <row r="1146">
@@ -13038,10 +13038,10 @@
         <v>46266</v>
       </c>
       <c r="B1146" t="n">
-        <v>2747</v>
+        <v>1064</v>
       </c>
       <c r="C1146" t="n">
-        <v>49090.92</v>
+        <v>517636</v>
       </c>
     </row>
     <row r="1147">
@@ -13049,10 +13049,10 @@
         <v>46266</v>
       </c>
       <c r="B1147" t="n">
-        <v>2819</v>
+        <v>2308</v>
       </c>
       <c r="C1147" t="n">
-        <v>49090.92</v>
+        <v>177042</v>
       </c>
     </row>
     <row r="1148">
@@ -13060,10 +13060,10 @@
         <v>46266</v>
       </c>
       <c r="B1148" t="n">
-        <v>1259</v>
+        <v>2747</v>
       </c>
       <c r="C1148" t="n">
-        <v>81818.2</v>
+        <v>51818.19</v>
       </c>
     </row>
     <row r="1149">
@@ -13071,10 +13071,10 @@
         <v>46266</v>
       </c>
       <c r="B1149" t="n">
-        <v>2544</v>
+        <v>2819</v>
       </c>
       <c r="C1149" t="n">
-        <v>65448</v>
+        <v>51818.19</v>
       </c>
     </row>
     <row r="1150">
@@ -13082,10 +13082,10 @@
         <v>46266</v>
       </c>
       <c r="B1150" t="n">
-        <v>2261</v>
+        <v>1259</v>
       </c>
       <c r="C1150" t="n">
-        <v>122724</v>
+        <v>86363.64999999999</v>
       </c>
     </row>
     <row r="1151">
@@ -13093,10 +13093,10 @@
         <v>46266</v>
       </c>
       <c r="B1151" t="n">
-        <v>2729</v>
+        <v>2544</v>
       </c>
       <c r="C1151" t="n">
-        <v>65448</v>
+        <v>69084</v>
       </c>
     </row>
     <row r="1152">
@@ -13104,10 +13104,10 @@
         <v>46266</v>
       </c>
       <c r="B1152" t="n">
-        <v>2649</v>
+        <v>2261</v>
       </c>
       <c r="C1152" t="n">
-        <v>24156</v>
+        <v>129542</v>
       </c>
     </row>
     <row r="1153">
@@ -13115,10 +13115,10 @@
         <v>46266</v>
       </c>
       <c r="B1153" t="n">
-        <v>2494</v>
+        <v>2729</v>
       </c>
       <c r="C1153" t="n">
-        <v>106362</v>
+        <v>69084</v>
       </c>
     </row>
     <row r="1154">
@@ -13126,10 +13126,10 @@
         <v>46266</v>
       </c>
       <c r="B1154" t="n">
-        <v>1384</v>
+        <v>2649</v>
       </c>
       <c r="C1154" t="n">
-        <v>368172</v>
+        <v>25498</v>
       </c>
     </row>
     <row r="1155">
@@ -13137,10 +13137,10 @@
         <v>46266</v>
       </c>
       <c r="B1155" t="n">
-        <v>2633</v>
+        <v>2494</v>
       </c>
       <c r="C1155" t="n">
-        <v>0</v>
+        <v>112271</v>
       </c>
     </row>
     <row r="1156">
@@ -13148,10 +13148,10 @@
         <v>46266</v>
       </c>
       <c r="B1156" t="n">
-        <v>2802</v>
+        <v>2633</v>
       </c>
       <c r="C1156" t="n">
-        <v>57942</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1157">
@@ -13159,10 +13159,10 @@
         <v>46266</v>
       </c>
       <c r="B1157" t="n">
-        <v>2726</v>
+        <v>2802</v>
       </c>
       <c r="C1157" t="n">
-        <v>122724</v>
+        <v>61161</v>
       </c>
     </row>
     <row r="1158">
@@ -13170,10 +13170,10 @@
         <v>46266</v>
       </c>
       <c r="B1158" t="n">
-        <v>2820</v>
+        <v>2726</v>
       </c>
       <c r="C1158" t="n">
-        <v>147258</v>
+        <v>129542</v>
       </c>
     </row>
     <row r="1159">
@@ -13181,10 +13181,10 @@
         <v>46266</v>
       </c>
       <c r="B1159" t="n">
-        <v>1007</v>
+        <v>2820</v>
       </c>
       <c r="C1159" t="n">
-        <v>155448</v>
+        <v>155439</v>
       </c>
     </row>
     <row r="1160">
@@ -13192,10 +13192,10 @@
         <v>46266</v>
       </c>
       <c r="B1160" t="n">
-        <v>20</v>
+        <v>1007</v>
       </c>
       <c r="C1160" t="n">
-        <v>315000</v>
+        <v>164084</v>
       </c>
     </row>
     <row r="1161">
@@ -13203,10 +13203,10 @@
         <v>46266</v>
       </c>
       <c r="B1161" t="n">
-        <v>1372</v>
+        <v>20</v>
       </c>
       <c r="C1161" t="n">
-        <v>237258</v>
+        <v>332500</v>
       </c>
     </row>
     <row r="1162">
@@ -13214,10 +13214,10 @@
         <v>46266</v>
       </c>
       <c r="B1162" t="n">
-        <v>2735</v>
+        <v>1372</v>
       </c>
       <c r="C1162" t="n">
-        <v>98172</v>
+        <v>250439</v>
       </c>
     </row>
     <row r="1163">
@@ -13225,10 +13225,10 @@
         <v>46266</v>
       </c>
       <c r="B1163" t="n">
-        <v>2811</v>
+        <v>2735</v>
       </c>
       <c r="C1163" t="n">
-        <v>34038</v>
+        <v>103626</v>
       </c>
     </row>
     <row r="1164">
@@ -13236,10 +13236,10 @@
         <v>46266</v>
       </c>
       <c r="B1164" t="n">
-        <v>1871</v>
+        <v>2811</v>
       </c>
       <c r="C1164" t="n">
-        <v>144612</v>
+        <v>35929</v>
       </c>
     </row>
     <row r="1165">
@@ -13247,10 +13247,10 @@
         <v>46266</v>
       </c>
       <c r="B1165" t="n">
-        <v>2541</v>
+        <v>1871</v>
       </c>
       <c r="C1165" t="n">
-        <v>173124</v>
+        <v>152646</v>
       </c>
     </row>
     <row r="1166">
@@ -13258,10 +13258,10 @@
         <v>46266</v>
       </c>
       <c r="B1166" t="n">
-        <v>2362</v>
+        <v>2541</v>
       </c>
       <c r="C1166" t="n">
-        <v>61362</v>
+        <v>182742</v>
       </c>
     </row>
     <row r="1167">
@@ -13269,10 +13269,10 @@
         <v>46266</v>
       </c>
       <c r="B1167" t="n">
-        <v>1324</v>
+        <v>2362</v>
       </c>
       <c r="C1167" t="n">
-        <v>229086</v>
+        <v>64771</v>
       </c>
     </row>
     <row r="1168">
@@ -13280,10 +13280,10 @@
         <v>46266</v>
       </c>
       <c r="B1168" t="n">
-        <v>2323</v>
+        <v>1324</v>
       </c>
       <c r="C1168" t="n">
-        <v>56196</v>
+        <v>241813</v>
       </c>
     </row>
     <row r="1169">
@@ -13291,10 +13291,10 @@
         <v>46266</v>
       </c>
       <c r="B1169" t="n">
-        <v>2647</v>
+        <v>2323</v>
       </c>
       <c r="C1169" t="n">
-        <v>116100</v>
+        <v>59318</v>
       </c>
     </row>
     <row r="1170">
@@ -13302,10 +13302,10 @@
         <v>46266</v>
       </c>
       <c r="B1170" t="n">
-        <v>559</v>
+        <v>2647</v>
       </c>
       <c r="C1170" t="n">
-        <v>187722</v>
+        <v>122550</v>
       </c>
     </row>
     <row r="1171">
@@ -13313,10 +13313,10 @@
         <v>46266</v>
       </c>
       <c r="B1171" t="n">
-        <v>2762</v>
+        <v>559</v>
       </c>
       <c r="C1171" t="n">
-        <v>66672</v>
+        <v>198151</v>
       </c>
     </row>
     <row r="1172">
@@ -13324,10 +13324,10 @@
         <v>46266</v>
       </c>
       <c r="B1172" t="n">
-        <v>2501</v>
+        <v>2762</v>
       </c>
       <c r="C1172" t="n">
-        <v>66672</v>
+        <v>70376</v>
       </c>
     </row>
     <row r="1173">
@@ -13335,10 +13335,10 @@
         <v>46266</v>
       </c>
       <c r="B1173" t="n">
-        <v>2562</v>
+        <v>2501</v>
       </c>
       <c r="C1173" t="n">
-        <v>12942</v>
+        <v>70376</v>
       </c>
     </row>
     <row r="1174">
@@ -13346,10 +13346,10 @@
         <v>46266</v>
       </c>
       <c r="B1174" t="n">
-        <v>429</v>
+        <v>2562</v>
       </c>
       <c r="C1174" t="n">
-        <v>319086</v>
+        <v>13661</v>
       </c>
     </row>
     <row r="1175">
@@ -13357,10 +13357,10 @@
         <v>46266</v>
       </c>
       <c r="B1175" t="n">
-        <v>58</v>
+        <v>429</v>
       </c>
       <c r="C1175" t="n">
-        <v>221382</v>
+        <v>336813</v>
       </c>
     </row>
     <row r="1176">
@@ -13368,10 +13368,10 @@
         <v>46266</v>
       </c>
       <c r="B1176" t="n">
-        <v>2245</v>
+        <v>58</v>
       </c>
       <c r="C1176" t="n">
-        <v>197658</v>
+        <v>233681</v>
       </c>
     </row>
     <row r="1177">
@@ -13379,10 +13379,10 @@
         <v>46266</v>
       </c>
       <c r="B1177" t="n">
-        <v>285</v>
+        <v>2245</v>
       </c>
       <c r="C1177" t="n">
-        <v>442764</v>
+        <v>208639</v>
       </c>
     </row>
     <row r="1178">
@@ -13390,10 +13390,10 @@
         <v>46266</v>
       </c>
       <c r="B1178" t="n">
-        <v>1464</v>
+        <v>285</v>
       </c>
       <c r="C1178" t="n">
-        <v>0</v>
+        <v>467362</v>
       </c>
     </row>
     <row r="1179">
@@ -13401,10 +13401,10 @@
         <v>46266</v>
       </c>
       <c r="B1179" t="n">
-        <v>363</v>
+        <v>1464</v>
       </c>
       <c r="C1179" t="n">
-        <v>245448</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1180">
@@ -13412,10 +13412,10 @@
         <v>46266</v>
       </c>
       <c r="B1180" t="n">
-        <v>2651</v>
+        <v>363</v>
       </c>
       <c r="C1180" t="n">
-        <v>138366</v>
+        <v>259084</v>
       </c>
     </row>
     <row r="1181">
@@ -13423,10 +13423,10 @@
         <v>46266</v>
       </c>
       <c r="B1181" t="n">
-        <v>2142</v>
+        <v>2651</v>
       </c>
       <c r="C1181" t="n">
-        <v>43668</v>
+        <v>146053</v>
       </c>
     </row>
     <row r="1182">
@@ -13434,10 +13434,10 @@
         <v>46266</v>
       </c>
       <c r="B1182" t="n">
-        <v>2258</v>
+        <v>2142</v>
       </c>
       <c r="C1182" t="n">
-        <v>65454.56</v>
+        <v>46094</v>
       </c>
     </row>
     <row r="1183">
@@ -13445,10 +13445,10 @@
         <v>46266</v>
       </c>
       <c r="B1183" t="n">
-        <v>2772</v>
+        <v>2258</v>
       </c>
       <c r="C1183" t="n">
-        <v>49090.92</v>
+        <v>69090.92</v>
       </c>
     </row>
     <row r="1184">
@@ -13456,10 +13456,10 @@
         <v>46266</v>
       </c>
       <c r="B1184" t="n">
-        <v>2346</v>
+        <v>2772</v>
       </c>
       <c r="C1184" t="n">
-        <v>90000</v>
+        <v>51818.19</v>
       </c>
     </row>
     <row r="1185">
@@ -13467,10 +13467,10 @@
         <v>46266</v>
       </c>
       <c r="B1185" t="n">
-        <v>2442</v>
+        <v>2346</v>
       </c>
       <c r="C1185" t="n">
-        <v>65448</v>
+        <v>95000</v>
       </c>
     </row>
     <row r="1186">
@@ -13478,10 +13478,10 @@
         <v>46266</v>
       </c>
       <c r="B1186" t="n">
-        <v>772</v>
+        <v>2442</v>
       </c>
       <c r="C1186" t="n">
-        <v>270000</v>
+        <v>69084</v>
       </c>
     </row>
     <row r="1187">
@@ -13489,10 +13489,10 @@
         <v>46266</v>
       </c>
       <c r="B1187" t="n">
-        <v>2684</v>
+        <v>772</v>
       </c>
       <c r="C1187" t="n">
-        <v>77724</v>
+        <v>285000</v>
       </c>
     </row>
     <row r="1188">
@@ -13500,10 +13500,10 @@
         <v>46266</v>
       </c>
       <c r="B1188" t="n">
-        <v>2765</v>
+        <v>2684</v>
       </c>
       <c r="C1188" t="n">
-        <v>73620</v>
+        <v>82042</v>
       </c>
     </row>
     <row r="1189">
@@ -13511,10 +13511,10 @@
         <v>46266</v>
       </c>
       <c r="B1189" t="n">
-        <v>2567</v>
+        <v>2765</v>
       </c>
       <c r="C1189" t="n">
-        <v>135036</v>
+        <v>77710</v>
       </c>
     </row>
     <row r="1190">
@@ -13522,10 +13522,10 @@
         <v>46266</v>
       </c>
       <c r="B1190" t="n">
-        <v>2178</v>
+        <v>2567</v>
       </c>
       <c r="C1190" t="n">
-        <v>229086</v>
+        <v>142538</v>
       </c>
     </row>
     <row r="1191">
@@ -13533,10 +13533,10 @@
         <v>46266</v>
       </c>
       <c r="B1191" t="n">
-        <v>2827</v>
+        <v>2178</v>
       </c>
       <c r="C1191" t="n">
-        <v>81810</v>
+        <v>241813</v>
       </c>
     </row>
     <row r="1192">
@@ -13544,10 +13544,10 @@
         <v>46266</v>
       </c>
       <c r="B1192" t="n">
-        <v>2510</v>
+        <v>2827</v>
       </c>
       <c r="C1192" t="n">
-        <v>454284</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1193">
@@ -13555,10 +13555,10 @@
         <v>46266</v>
       </c>
       <c r="B1193" t="n">
-        <v>2392</v>
+        <v>2510</v>
       </c>
       <c r="C1193" t="n">
-        <v>136278</v>
+        <v>479522</v>
       </c>
     </row>
     <row r="1194">
@@ -13566,10 +13566,10 @@
         <v>46266</v>
       </c>
       <c r="B1194" t="n">
-        <v>415</v>
+        <v>2392</v>
       </c>
       <c r="C1194" t="n">
-        <v>465948</v>
+        <v>143849</v>
       </c>
     </row>
     <row r="1195">
@@ -13577,10 +13577,10 @@
         <v>46266</v>
       </c>
       <c r="B1195" t="n">
-        <v>2107</v>
+        <v>415</v>
       </c>
       <c r="C1195" t="n">
-        <v>240606</v>
+        <v>491834</v>
       </c>
     </row>
     <row r="1196">
@@ -13588,10 +13588,10 @@
         <v>46266</v>
       </c>
       <c r="B1196" t="n">
-        <v>2211</v>
+        <v>2107</v>
       </c>
       <c r="C1196" t="n">
-        <v>199476</v>
+        <v>253973</v>
       </c>
     </row>
     <row r="1197">
@@ -13599,10 +13599,10 @@
         <v>46266</v>
       </c>
       <c r="B1197" t="n">
-        <v>2682</v>
+        <v>2211</v>
       </c>
       <c r="C1197" t="n">
-        <v>122706</v>
+        <v>210558</v>
       </c>
     </row>
     <row r="1198">
@@ -13610,10 +13610,10 @@
         <v>46266</v>
       </c>
       <c r="B1198" t="n">
-        <v>2781</v>
+        <v>2682</v>
       </c>
       <c r="C1198" t="n">
-        <v>0</v>
+        <v>129523</v>
       </c>
     </row>
     <row r="1199">
@@ -13621,7 +13621,7 @@
         <v>46266</v>
       </c>
       <c r="B1199" t="n">
-        <v>2576</v>
+        <v>2781</v>
       </c>
       <c r="C1199" t="n">
         <v>0</v>
@@ -13632,10 +13632,10 @@
         <v>46266</v>
       </c>
       <c r="B1200" t="n">
-        <v>2755</v>
+        <v>2576</v>
       </c>
       <c r="C1200" t="n">
-        <v>49086</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1201">
@@ -13643,10 +13643,10 @@
         <v>46266</v>
       </c>
       <c r="B1201" t="n">
-        <v>941</v>
+        <v>2755</v>
       </c>
       <c r="C1201" t="n">
-        <v>321444</v>
+        <v>51813</v>
       </c>
     </row>
     <row r="1202">
@@ -13654,10 +13654,10 @@
         <v>46266</v>
       </c>
       <c r="B1202" t="n">
-        <v>2734</v>
+        <v>941</v>
       </c>
       <c r="C1202" t="n">
-        <v>45054</v>
+        <v>307342.7</v>
       </c>
     </row>
     <row r="1203">
@@ -13665,10 +13665,10 @@
         <v>46266</v>
       </c>
       <c r="B1203" t="n">
-        <v>1289</v>
+        <v>2734</v>
       </c>
       <c r="C1203" t="n">
-        <v>204534</v>
+        <v>47557</v>
       </c>
     </row>
     <row r="1204">
@@ -13676,10 +13676,10 @@
         <v>46266</v>
       </c>
       <c r="B1204" t="n">
-        <v>2801</v>
+        <v>1840</v>
       </c>
       <c r="C1204" t="n">
-        <v>65448</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1205">
@@ -13687,10 +13687,10 @@
         <v>46266</v>
       </c>
       <c r="B1205" t="n">
-        <v>2810</v>
+        <v>1289</v>
       </c>
       <c r="C1205" t="n">
-        <v>110448</v>
+        <v>215897</v>
       </c>
     </row>
     <row r="1206">
@@ -13698,10 +13698,10 @@
         <v>46266</v>
       </c>
       <c r="B1206" t="n">
-        <v>767</v>
+        <v>2801</v>
       </c>
       <c r="C1206" t="n">
-        <v>147258</v>
+        <v>69084</v>
       </c>
     </row>
     <row r="1207">
@@ -13709,10 +13709,10 @@
         <v>46266</v>
       </c>
       <c r="B1207" t="n">
-        <v>2687</v>
+        <v>2810</v>
       </c>
       <c r="C1207" t="n">
-        <v>81810</v>
+        <v>116584</v>
       </c>
     </row>
     <row r="1208">
@@ -13720,10 +13720,10 @@
         <v>46266</v>
       </c>
       <c r="B1208" t="n">
-        <v>2686</v>
+        <v>767</v>
       </c>
       <c r="C1208" t="n">
-        <v>106362</v>
+        <v>155439</v>
       </c>
     </row>
     <row r="1209">
@@ -13731,10 +13731,10 @@
         <v>46266</v>
       </c>
       <c r="B1209" t="n">
-        <v>2730</v>
+        <v>2687</v>
       </c>
       <c r="C1209" t="n">
-        <v>73620</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1210">
@@ -13742,10 +13742,10 @@
         <v>46266</v>
       </c>
       <c r="B1210" t="n">
-        <v>2580</v>
+        <v>2686</v>
       </c>
       <c r="C1210" t="n">
-        <v>27450</v>
+        <v>112271</v>
       </c>
     </row>
     <row r="1211">
@@ -13753,10 +13753,10 @@
         <v>46266</v>
       </c>
       <c r="B1211" t="n">
-        <v>2472</v>
+        <v>2730</v>
       </c>
       <c r="C1211" t="n">
-        <v>43316.2</v>
+        <v>77710</v>
       </c>
     </row>
     <row r="1212">
@@ -13764,10 +13764,10 @@
         <v>46266</v>
       </c>
       <c r="B1212" t="n">
-        <v>2631</v>
+        <v>2580</v>
       </c>
       <c r="C1212" t="n">
-        <v>20071.64</v>
+        <v>28975</v>
       </c>
     </row>
     <row r="1213">
@@ -13775,10 +13775,10 @@
         <v>46266</v>
       </c>
       <c r="B1213" t="n">
-        <v>1642</v>
+        <v>2472</v>
       </c>
       <c r="C1213" t="n">
-        <v>216810</v>
+        <v>45722.65</v>
       </c>
     </row>
     <row r="1214">
@@ -13786,10 +13786,10 @@
         <v>46266</v>
       </c>
       <c r="B1214" t="n">
-        <v>2613</v>
+        <v>2631</v>
       </c>
       <c r="C1214" t="n">
-        <v>146610</v>
+        <v>21186.73</v>
       </c>
     </row>
     <row r="1215">
@@ -13797,10 +13797,10 @@
         <v>46266</v>
       </c>
       <c r="B1215" t="n">
-        <v>1020</v>
+        <v>1642</v>
       </c>
       <c r="C1215" t="n">
-        <v>73620</v>
+        <v>228855</v>
       </c>
     </row>
     <row r="1216">
@@ -13808,10 +13808,10 @@
         <v>46266</v>
       </c>
       <c r="B1216" t="n">
-        <v>2785</v>
+        <v>2613</v>
       </c>
       <c r="C1216" t="n">
-        <v>34038</v>
+        <v>154755</v>
       </c>
     </row>
     <row r="1217">
@@ -13819,10 +13819,10 @@
         <v>46266</v>
       </c>
       <c r="B1217" t="n">
-        <v>1327</v>
+        <v>1020</v>
       </c>
       <c r="C1217" t="n">
-        <v>49086</v>
+        <v>77710</v>
       </c>
     </row>
     <row r="1218">
@@ -13830,10 +13830,10 @@
         <v>46266</v>
       </c>
       <c r="B1218" t="n">
-        <v>2629</v>
+        <v>2785</v>
       </c>
       <c r="C1218" t="n">
-        <v>56196</v>
+        <v>35929</v>
       </c>
     </row>
     <row r="1219">
@@ -13841,10 +13841,10 @@
         <v>46266</v>
       </c>
       <c r="B1219" t="n">
-        <v>749</v>
+        <v>1327</v>
       </c>
       <c r="C1219" t="n">
-        <v>66672</v>
+        <v>51813</v>
       </c>
     </row>
     <row r="1220">
@@ -13852,10 +13852,10 @@
         <v>46266</v>
       </c>
       <c r="B1220" t="n">
-        <v>1983</v>
+        <v>749</v>
       </c>
       <c r="C1220" t="n">
-        <v>442764</v>
+        <v>70376</v>
       </c>
     </row>
     <row r="1221">
@@ -13863,10 +13863,10 @@
         <v>46266</v>
       </c>
       <c r="B1221" t="n">
-        <v>1993</v>
+        <v>1983</v>
       </c>
       <c r="C1221" t="n">
-        <v>284634</v>
+        <v>467362</v>
       </c>
     </row>
     <row r="1222">
@@ -13874,10 +13874,10 @@
         <v>46266</v>
       </c>
       <c r="B1222" t="n">
-        <v>2767</v>
+        <v>1993</v>
       </c>
       <c r="C1222" t="n">
-        <v>157842</v>
+        <v>300447</v>
       </c>
     </row>
     <row r="1223">
@@ -13885,10 +13885,10 @@
         <v>46266</v>
       </c>
       <c r="B1223" t="n">
-        <v>2646</v>
+        <v>2767</v>
       </c>
       <c r="C1223" t="n">
-        <v>0</v>
+        <v>166611</v>
       </c>
     </row>
     <row r="1224">
@@ -13896,10 +13896,10 @@
         <v>46266</v>
       </c>
       <c r="B1224" t="n">
-        <v>1102</v>
+        <v>2646</v>
       </c>
       <c r="C1224" t="n">
-        <v>197658</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1225">
@@ -13907,10 +13907,10 @@
         <v>46266</v>
       </c>
       <c r="B1225" t="n">
-        <v>626</v>
+        <v>1102</v>
       </c>
       <c r="C1225" t="n">
-        <v>1394439.56</v>
+        <v>208639</v>
       </c>
     </row>
     <row r="1226">
@@ -13918,10 +13918,10 @@
         <v>46266</v>
       </c>
       <c r="B1226" t="n">
-        <v>1465</v>
+        <v>626</v>
       </c>
       <c r="C1226" t="n">
-        <v>294372</v>
+        <v>1471908.42</v>
       </c>
     </row>
     <row r="1227">
@@ -13929,10 +13929,10 @@
         <v>46266</v>
       </c>
       <c r="B1227" t="n">
-        <v>2758</v>
+        <v>1465</v>
       </c>
       <c r="C1227" t="n">
-        <v>49090.92</v>
+        <v>310726</v>
       </c>
     </row>
     <row r="1228">
@@ -13940,10 +13940,10 @@
         <v>46266</v>
       </c>
       <c r="B1228" t="n">
-        <v>2742</v>
+        <v>2758</v>
       </c>
       <c r="C1228" t="n">
-        <v>49090.92</v>
+        <v>51818.19</v>
       </c>
     </row>
     <row r="1229">
@@ -13951,10 +13951,10 @@
         <v>46266</v>
       </c>
       <c r="B1229" t="n">
-        <v>2748</v>
+        <v>2742</v>
       </c>
       <c r="C1229" t="n">
-        <v>0</v>
+        <v>51818.19</v>
       </c>
     </row>
     <row r="1230">
@@ -13962,10 +13962,10 @@
         <v>46266</v>
       </c>
       <c r="B1230" t="n">
-        <v>1873</v>
+        <v>2748</v>
       </c>
       <c r="C1230" t="n">
-        <v>261810</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1231">
@@ -13973,10 +13973,10 @@
         <v>46266</v>
       </c>
       <c r="B1231" t="n">
-        <v>2163</v>
+        <v>1873</v>
       </c>
       <c r="C1231" t="n">
-        <v>122724</v>
+        <v>276355</v>
       </c>
     </row>
     <row r="1232">
@@ -13984,10 +13984,10 @@
         <v>46266</v>
       </c>
       <c r="B1232" t="n">
-        <v>2394</v>
+        <v>2163</v>
       </c>
       <c r="C1232" t="n">
-        <v>126036</v>
+        <v>129542</v>
       </c>
     </row>
     <row r="1233">
@@ -13995,10 +13995,10 @@
         <v>46266</v>
       </c>
       <c r="B1233" t="n">
-        <v>33</v>
+        <v>2394</v>
       </c>
       <c r="C1233" t="n">
-        <v>317448</v>
+        <v>133038</v>
       </c>
     </row>
     <row r="1234">
@@ -14006,10 +14006,10 @@
         <v>46266</v>
       </c>
       <c r="B1234" t="n">
-        <v>2421</v>
+        <v>33</v>
       </c>
       <c r="C1234" t="n">
-        <v>53172</v>
+        <v>335084</v>
       </c>
     </row>
     <row r="1235">
@@ -14017,10 +14017,10 @@
         <v>46266</v>
       </c>
       <c r="B1235" t="n">
-        <v>2663</v>
+        <v>2421</v>
       </c>
       <c r="C1235" t="n">
-        <v>225000</v>
+        <v>56126</v>
       </c>
     </row>
     <row r="1236">
@@ -14028,10 +14028,10 @@
         <v>46266</v>
       </c>
       <c r="B1236" t="n">
-        <v>2413</v>
+        <v>2663</v>
       </c>
       <c r="C1236" t="n">
-        <v>99036</v>
+        <v>237500</v>
       </c>
     </row>
     <row r="1237">
@@ -14039,10 +14039,10 @@
         <v>46266</v>
       </c>
       <c r="B1237" t="n">
-        <v>351</v>
+        <v>2413</v>
       </c>
       <c r="C1237" t="n">
-        <v>150534</v>
+        <v>104538</v>
       </c>
     </row>
     <row r="1238">
@@ -14050,10 +14050,10 @@
         <v>46266</v>
       </c>
       <c r="B1238" t="n">
-        <v>1298</v>
+        <v>351</v>
       </c>
       <c r="C1238" t="n">
-        <v>1041534</v>
+        <v>158897</v>
       </c>
     </row>
     <row r="1239">
@@ -14061,10 +14061,10 @@
         <v>46266</v>
       </c>
       <c r="B1239" t="n">
-        <v>2491</v>
+        <v>1298</v>
       </c>
       <c r="C1239" t="n">
-        <v>84168</v>
+        <v>1099397</v>
       </c>
     </row>
     <row r="1240">
@@ -14072,10 +14072,10 @@
         <v>46266</v>
       </c>
       <c r="B1240" t="n">
-        <v>2571</v>
+        <v>2491</v>
       </c>
       <c r="C1240" t="n">
-        <v>118854</v>
+        <v>88844</v>
       </c>
     </row>
     <row r="1241">
@@ -14083,10 +14083,10 @@
         <v>46266</v>
       </c>
       <c r="B1241" t="n">
-        <v>2507</v>
+        <v>2571</v>
       </c>
       <c r="C1241" t="n">
-        <v>72216</v>
+        <v>125457</v>
       </c>
     </row>
     <row r="1242">
@@ -14094,10 +14094,10 @@
         <v>46266</v>
       </c>
       <c r="B1242" t="n">
-        <v>2799</v>
+        <v>2507</v>
       </c>
       <c r="C1242" t="n">
-        <v>92952</v>
+        <v>76228</v>
       </c>
     </row>
     <row r="1243">
@@ -14105,10 +14105,10 @@
         <v>46266</v>
       </c>
       <c r="B1243" t="n">
-        <v>2253</v>
+        <v>2799</v>
       </c>
       <c r="C1243" t="n">
-        <v>0</v>
+        <v>98116</v>
       </c>
     </row>
     <row r="1244">
@@ -14116,10 +14116,10 @@
         <v>46266</v>
       </c>
       <c r="B1244" t="n">
-        <v>2582</v>
+        <v>2253</v>
       </c>
       <c r="C1244" t="n">
-        <v>70812</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1245">
@@ -14127,10 +14127,10 @@
         <v>46266</v>
       </c>
       <c r="B1245" t="n">
-        <v>2637</v>
+        <v>2582</v>
       </c>
       <c r="C1245" t="n">
-        <v>51498</v>
+        <v>74746</v>
       </c>
     </row>
     <row r="1246">
@@ -14138,10 +14138,10 @@
         <v>46266</v>
       </c>
       <c r="B1246" t="n">
-        <v>630</v>
+        <v>2637</v>
       </c>
       <c r="C1246" t="n">
-        <v>122472</v>
+        <v>54359</v>
       </c>
     </row>
     <row r="1247">
@@ -14149,10 +14149,10 @@
         <v>46266</v>
       </c>
       <c r="B1247" t="n">
-        <v>525</v>
+        <v>630</v>
       </c>
       <c r="C1247" t="n">
-        <v>184086</v>
+        <v>129276</v>
       </c>
     </row>
     <row r="1248">
@@ -14160,10 +14160,10 @@
         <v>46266</v>
       </c>
       <c r="B1248" t="n">
-        <v>2727</v>
+        <v>525</v>
       </c>
       <c r="C1248" t="n">
-        <v>33120</v>
+        <v>194313</v>
       </c>
     </row>
     <row r="1249">
@@ -14171,10 +14171,10 @@
         <v>46266</v>
       </c>
       <c r="B1249" t="n">
-        <v>2707</v>
+        <v>2727</v>
       </c>
       <c r="C1249" t="n">
-        <v>26208</v>
+        <v>34960</v>
       </c>
     </row>
     <row r="1250">
@@ -14182,10 +14182,10 @@
         <v>46266</v>
       </c>
       <c r="B1250" t="n">
-        <v>2834</v>
+        <v>2707</v>
       </c>
       <c r="C1250" t="n">
-        <v>13539.28</v>
+        <v>27664</v>
       </c>
     </row>
     <row r="1251">
@@ -14193,10 +14193,10 @@
         <v>46266</v>
       </c>
       <c r="B1251" t="n">
-        <v>2773</v>
+        <v>2834</v>
       </c>
       <c r="C1251" t="n">
-        <v>66020.75999999999</v>
+        <v>14291.46</v>
       </c>
     </row>
     <row r="1252">
@@ -14204,10 +14204,10 @@
         <v>46266</v>
       </c>
       <c r="B1252" t="n">
-        <v>2341</v>
+        <v>2773</v>
       </c>
       <c r="C1252" t="n">
-        <v>116100</v>
+        <v>69688.57000000001</v>
       </c>
     </row>
     <row r="1253">
@@ -14215,10 +14215,10 @@
         <v>46266</v>
       </c>
       <c r="B1253" t="n">
-        <v>1374</v>
+        <v>2341</v>
       </c>
       <c r="C1253" t="n">
-        <v>147258</v>
+        <v>122550</v>
       </c>
     </row>
     <row r="1254">
@@ -14226,10 +14226,10 @@
         <v>46266</v>
       </c>
       <c r="B1254" t="n">
-        <v>793</v>
+        <v>1374</v>
       </c>
       <c r="C1254" t="n">
-        <v>34038</v>
+        <v>155439</v>
       </c>
     </row>
     <row r="1255">
@@ -14237,10 +14237,10 @@
         <v>46266</v>
       </c>
       <c r="B1255" t="n">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="C1255" t="n">
-        <v>34038</v>
+        <v>35929</v>
       </c>
     </row>
     <row r="1256">
@@ -14248,10 +14248,10 @@
         <v>46266</v>
       </c>
       <c r="B1256" t="n">
-        <v>1834</v>
+        <v>794</v>
       </c>
       <c r="C1256" t="n">
-        <v>95724</v>
+        <v>35929</v>
       </c>
     </row>
     <row r="1257">
@@ -14259,10 +14259,10 @@
         <v>46266</v>
       </c>
       <c r="B1257" t="n">
-        <v>802</v>
+        <v>1834</v>
       </c>
       <c r="C1257" t="n">
-        <v>61362</v>
+        <v>101042</v>
       </c>
     </row>
     <row r="1258">
@@ -14270,10 +14270,10 @@
         <v>46266</v>
       </c>
       <c r="B1258" t="n">
-        <v>1344</v>
+        <v>802</v>
       </c>
       <c r="C1258" t="n">
-        <v>122724</v>
+        <v>64771</v>
       </c>
     </row>
     <row r="1259">
@@ -14281,10 +14281,10 @@
         <v>46266</v>
       </c>
       <c r="B1259" t="n">
-        <v>1881</v>
+        <v>1344</v>
       </c>
       <c r="C1259" t="n">
-        <v>56196</v>
+        <v>129542</v>
       </c>
     </row>
     <row r="1260">
@@ -14292,10 +14292,10 @@
         <v>46266</v>
       </c>
       <c r="B1260" t="n">
-        <v>2365</v>
+        <v>1881</v>
       </c>
       <c r="C1260" t="n">
-        <v>65178</v>
+        <v>59318</v>
       </c>
     </row>
     <row r="1261">
@@ -14303,10 +14303,10 @@
         <v>46266</v>
       </c>
       <c r="B1261" t="n">
-        <v>2411</v>
+        <v>2365</v>
       </c>
       <c r="C1261" t="n">
-        <v>116100</v>
+        <v>68799</v>
       </c>
     </row>
     <row r="1262">
@@ -14314,10 +14314,10 @@
         <v>46266</v>
       </c>
       <c r="B1262" t="n">
-        <v>2363</v>
+        <v>2411</v>
       </c>
       <c r="C1262" t="n">
-        <v>122724</v>
+        <v>122550</v>
       </c>
     </row>
     <row r="1263">
@@ -14325,10 +14325,10 @@
         <v>46266</v>
       </c>
       <c r="B1263" t="n">
-        <v>2124</v>
+        <v>2363</v>
       </c>
       <c r="C1263" t="n">
-        <v>286362</v>
+        <v>129542</v>
       </c>
     </row>
     <row r="1264">
@@ -14336,10 +14336,10 @@
         <v>46266</v>
       </c>
       <c r="B1264" t="n">
-        <v>1937</v>
+        <v>2124</v>
       </c>
       <c r="C1264" t="n">
-        <v>208620</v>
+        <v>302271</v>
       </c>
     </row>
     <row r="1265">
@@ -14347,10 +14347,10 @@
         <v>46266</v>
       </c>
       <c r="B1265" t="n">
-        <v>2709</v>
+        <v>1937</v>
       </c>
       <c r="C1265" t="n">
-        <v>147258</v>
+        <v>220210</v>
       </c>
     </row>
     <row r="1266">
@@ -14358,10 +14358,10 @@
         <v>46266</v>
       </c>
       <c r="B1266" t="n">
-        <v>2558</v>
+        <v>2709</v>
       </c>
       <c r="C1266" t="n">
-        <v>24588</v>
+        <v>155439</v>
       </c>
     </row>
     <row r="1267">
@@ -14369,10 +14369,10 @@
         <v>46266</v>
       </c>
       <c r="B1267" t="n">
-        <v>663</v>
+        <v>2558</v>
       </c>
       <c r="C1267" t="n">
-        <v>208620</v>
+        <v>25954</v>
       </c>
     </row>
     <row r="1268">
@@ -14380,10 +14380,10 @@
         <v>46266</v>
       </c>
       <c r="B1268" t="n">
-        <v>40</v>
+        <v>663</v>
       </c>
       <c r="C1268" t="n">
-        <v>180000</v>
+        <v>220210</v>
       </c>
     </row>
     <row r="1269">
@@ -14391,10 +14391,10 @@
         <v>46266</v>
       </c>
       <c r="B1269" t="n">
-        <v>2833</v>
+        <v>40</v>
       </c>
       <c r="C1269" t="n">
-        <v>57272.76</v>
+        <v>190000</v>
       </c>
     </row>
     <row r="1270">
@@ -14402,10 +14402,10 @@
         <v>46266</v>
       </c>
       <c r="B1270" t="n">
-        <v>1756</v>
+        <v>2833</v>
       </c>
       <c r="C1270" t="n">
-        <v>357138</v>
+        <v>60454.57</v>
       </c>
     </row>
     <row r="1271">
@@ -14413,10 +14413,10 @@
         <v>46266</v>
       </c>
       <c r="B1271" t="n">
-        <v>1116</v>
+        <v>1756</v>
       </c>
       <c r="C1271" t="n">
-        <v>207522</v>
+        <v>376979</v>
       </c>
     </row>
     <row r="1272">
@@ -14424,10 +14424,10 @@
         <v>46266</v>
       </c>
       <c r="B1272" t="n">
-        <v>636</v>
+        <v>1116</v>
       </c>
       <c r="C1272" t="n">
-        <v>204534</v>
+        <v>219051</v>
       </c>
     </row>
     <row r="1273">
@@ -14435,10 +14435,10 @@
         <v>46266</v>
       </c>
       <c r="B1273" t="n">
-        <v>1800</v>
+        <v>636</v>
       </c>
       <c r="C1273" t="n">
-        <v>22896</v>
+        <v>215897</v>
       </c>
     </row>
     <row r="1274">
@@ -14446,10 +14446,10 @@
         <v>46266</v>
       </c>
       <c r="B1274" t="n">
-        <v>2815</v>
+        <v>1800</v>
       </c>
       <c r="C1274" t="n">
-        <v>49090.92</v>
+        <v>24168</v>
       </c>
     </row>
     <row r="1275">
@@ -14457,10 +14457,10 @@
         <v>46266</v>
       </c>
       <c r="B1275" t="n">
-        <v>1658</v>
+        <v>2815</v>
       </c>
       <c r="C1275" t="n">
-        <v>108000</v>
+        <v>51818.19</v>
       </c>
     </row>
     <row r="1276">
@@ -14468,10 +14468,10 @@
         <v>46266</v>
       </c>
       <c r="B1276" t="n">
-        <v>2635</v>
+        <v>1658</v>
       </c>
       <c r="C1276" t="n">
-        <v>106362</v>
+        <v>114000</v>
       </c>
     </row>
     <row r="1277">
@@ -14479,10 +14479,10 @@
         <v>46266</v>
       </c>
       <c r="B1277" t="n">
-        <v>2402</v>
+        <v>2635</v>
       </c>
       <c r="C1277" t="n">
-        <v>533448</v>
+        <v>112271</v>
       </c>
     </row>
     <row r="1278">
@@ -14490,10 +14490,10 @@
         <v>46266</v>
       </c>
       <c r="B1278" t="n">
-        <v>452</v>
+        <v>2402</v>
       </c>
       <c r="C1278" t="n">
-        <v>220896</v>
+        <v>563084</v>
       </c>
     </row>
     <row r="1279">
@@ -14501,10 +14501,10 @@
         <v>46266</v>
       </c>
       <c r="B1279" t="n">
-        <v>2085</v>
+        <v>452</v>
       </c>
       <c r="C1279" t="n">
-        <v>108036</v>
+        <v>233168</v>
       </c>
     </row>
     <row r="1280">
@@ -14512,10 +14512,10 @@
         <v>46266</v>
       </c>
       <c r="B1280" t="n">
-        <v>2568</v>
+        <v>2085</v>
       </c>
       <c r="C1280" t="n">
-        <v>167256</v>
+        <v>114038</v>
       </c>
     </row>
     <row r="1281">
@@ -14523,10 +14523,10 @@
         <v>46266</v>
       </c>
       <c r="B1281" t="n">
-        <v>1906</v>
+        <v>2568</v>
       </c>
       <c r="C1281" t="n">
-        <v>94932</v>
+        <v>176548</v>
       </c>
     </row>
     <row r="1282">
@@ -14534,10 +14534,10 @@
         <v>46266</v>
       </c>
       <c r="B1282" t="n">
-        <v>2821</v>
+        <v>1906</v>
       </c>
       <c r="C1282" t="n">
-        <v>82548</v>
+        <v>100206</v>
       </c>
     </row>
     <row r="1283">
@@ -14545,10 +14545,10 @@
         <v>46266</v>
       </c>
       <c r="B1283" t="n">
-        <v>2698</v>
+        <v>2821</v>
       </c>
       <c r="C1283" t="n">
-        <v>101178</v>
+        <v>87134</v>
       </c>
     </row>
     <row r="1284">
@@ -14556,10 +14556,10 @@
         <v>46266</v>
       </c>
       <c r="B1284" t="n">
-        <v>2118</v>
+        <v>2698</v>
       </c>
       <c r="C1284" t="n">
-        <v>194040</v>
+        <v>106799</v>
       </c>
     </row>
     <row r="1285">
@@ -14567,10 +14567,10 @@
         <v>46266</v>
       </c>
       <c r="B1285" t="n">
-        <v>2383</v>
+        <v>2118</v>
       </c>
       <c r="C1285" t="n">
-        <v>113292</v>
+        <v>204820</v>
       </c>
     </row>
     <row r="1286">
@@ -14578,10 +14578,10 @@
         <v>46266</v>
       </c>
       <c r="B1286" t="n">
-        <v>2813</v>
+        <v>2383</v>
       </c>
       <c r="C1286" t="n">
-        <v>51498</v>
+        <v>119586</v>
       </c>
     </row>
     <row r="1287">
@@ -14589,10 +14589,10 @@
         <v>46266</v>
       </c>
       <c r="B1287" t="n">
-        <v>925</v>
+        <v>2813</v>
       </c>
       <c r="C1287" t="n">
-        <v>64368</v>
+        <v>54359</v>
       </c>
     </row>
     <row r="1288">
@@ -14600,10 +14600,10 @@
         <v>46266</v>
       </c>
       <c r="B1288" t="n">
-        <v>2689</v>
+        <v>925</v>
       </c>
       <c r="C1288" t="n">
-        <v>51498</v>
+        <v>67944</v>
       </c>
     </row>
     <row r="1289">
@@ -14611,10 +14611,10 @@
         <v>46266</v>
       </c>
       <c r="B1289" t="n">
-        <v>2716</v>
+        <v>2689</v>
       </c>
       <c r="C1289" t="n">
-        <v>70812</v>
+        <v>54359</v>
       </c>
     </row>
     <row r="1290">
@@ -14622,10 +14622,10 @@
         <v>46266</v>
       </c>
       <c r="B1290" t="n">
-        <v>2831</v>
+        <v>2716</v>
       </c>
       <c r="C1290" t="n">
-        <v>49086</v>
+        <v>74746</v>
       </c>
     </row>
     <row r="1291">
@@ -14633,10 +14633,10 @@
         <v>46266</v>
       </c>
       <c r="B1291" t="n">
-        <v>2045</v>
+        <v>2831</v>
       </c>
       <c r="C1291" t="n">
-        <v>275281.9</v>
+        <v>51813</v>
       </c>
     </row>
     <row r="1292">
@@ -14644,10 +14644,10 @@
         <v>46266</v>
       </c>
       <c r="B1292" t="n">
-        <v>580</v>
+        <v>2045</v>
       </c>
       <c r="C1292" t="n">
-        <v>110448</v>
+        <v>290575.33</v>
       </c>
     </row>
     <row r="1293">
@@ -14655,10 +14655,10 @@
         <v>46266</v>
       </c>
       <c r="B1293" t="n">
-        <v>438</v>
+        <v>580</v>
       </c>
       <c r="C1293" t="n">
-        <v>126810</v>
+        <v>116584</v>
       </c>
     </row>
     <row r="1294">
@@ -14666,10 +14666,10 @@
         <v>46266</v>
       </c>
       <c r="B1294" t="n">
-        <v>1539</v>
+        <v>438</v>
       </c>
       <c r="C1294" t="n">
-        <v>139086</v>
+        <v>133855</v>
       </c>
     </row>
     <row r="1295">
@@ -14677,10 +14677,10 @@
         <v>46266</v>
       </c>
       <c r="B1295" t="n">
-        <v>2817</v>
+        <v>1539</v>
       </c>
       <c r="C1295" t="n">
-        <v>49086</v>
+        <v>146813</v>
       </c>
     </row>
     <row r="1296">
@@ -14688,10 +14688,10 @@
         <v>46266</v>
       </c>
       <c r="B1296" t="n">
-        <v>2816</v>
+        <v>2817</v>
       </c>
       <c r="C1296" t="n">
-        <v>106362</v>
+        <v>51813</v>
       </c>
     </row>
     <row r="1297">
@@ -14699,10 +14699,10 @@
         <v>46266</v>
       </c>
       <c r="B1297" t="n">
-        <v>2146</v>
+        <v>2816</v>
       </c>
       <c r="C1297" t="n">
-        <v>164988</v>
+        <v>112271</v>
       </c>
     </row>
     <row r="1298">
@@ -14710,10 +14710,10 @@
         <v>46266</v>
       </c>
       <c r="B1298" t="n">
-        <v>2276</v>
+        <v>2146</v>
       </c>
       <c r="C1298" t="n">
-        <v>183312</v>
+        <v>174154</v>
       </c>
     </row>
     <row r="1299">
@@ -14721,10 +14721,10 @@
         <v>46266</v>
       </c>
       <c r="B1299" t="n">
-        <v>1381</v>
+        <v>2276</v>
       </c>
       <c r="C1299" t="n">
-        <v>241362</v>
+        <v>193496</v>
       </c>
     </row>
     <row r="1300">
@@ -14732,10 +14732,10 @@
         <v>46266</v>
       </c>
       <c r="B1300" t="n">
-        <v>2081</v>
+        <v>1381</v>
       </c>
       <c r="C1300" t="n">
-        <v>122724</v>
+        <v>254771</v>
       </c>
     </row>
     <row r="1301">
@@ -14743,10 +14743,10 @@
         <v>46266</v>
       </c>
       <c r="B1301" t="n">
-        <v>14</v>
+        <v>2081</v>
       </c>
       <c r="C1301" t="n">
-        <v>355896</v>
+        <v>129542</v>
       </c>
     </row>
     <row r="1302">
@@ -14754,10 +14754,10 @@
         <v>46266</v>
       </c>
       <c r="B1302" t="n">
-        <v>766</v>
+        <v>14</v>
       </c>
       <c r="C1302" t="n">
-        <v>56196</v>
+        <v>375668</v>
       </c>
     </row>
     <row r="1303">
@@ -14765,10 +14765,10 @@
         <v>46266</v>
       </c>
       <c r="B1303" t="n">
-        <v>2547</v>
+        <v>766</v>
       </c>
       <c r="C1303" t="n">
-        <v>33642</v>
+        <v>59318</v>
       </c>
     </row>
     <row r="1304">
@@ -14776,10 +14776,10 @@
         <v>46266</v>
       </c>
       <c r="B1304" t="n">
-        <v>2552</v>
+        <v>2547</v>
       </c>
       <c r="C1304" t="n">
-        <v>24192</v>
+        <v>35511</v>
       </c>
     </row>
     <row r="1305">
@@ -14787,10 +14787,10 @@
         <v>46266</v>
       </c>
       <c r="B1305" t="n">
-        <v>131</v>
+        <v>2552</v>
       </c>
       <c r="C1305" t="n">
-        <v>334620</v>
+        <v>25536</v>
       </c>
     </row>
     <row r="1306">
@@ -14798,10 +14798,10 @@
         <v>46266</v>
       </c>
       <c r="B1306" t="n">
-        <v>2250</v>
+        <v>131</v>
       </c>
       <c r="C1306" t="n">
-        <v>270738</v>
+        <v>353210</v>
       </c>
     </row>
     <row r="1307">
@@ -14809,10 +14809,10 @@
         <v>46266</v>
       </c>
       <c r="B1307" t="n">
-        <v>89</v>
+        <v>2250</v>
       </c>
       <c r="C1307" t="n">
-        <v>276696</v>
+        <v>285779</v>
       </c>
     </row>
     <row r="1308">
@@ -14820,10 +14820,10 @@
         <v>46266</v>
       </c>
       <c r="B1308" t="n">
-        <v>2141</v>
+        <v>89</v>
       </c>
       <c r="C1308" t="n">
-        <v>25884</v>
+        <v>292068</v>
       </c>
     </row>
     <row r="1309">
@@ -14831,10 +14831,10 @@
         <v>46266</v>
       </c>
       <c r="B1309" t="n">
-        <v>2798</v>
+        <v>2141</v>
       </c>
       <c r="C1309" t="n">
-        <v>49090.92</v>
+        <v>27322</v>
       </c>
     </row>
     <row r="1310">
@@ -14842,10 +14842,10 @@
         <v>46266</v>
       </c>
       <c r="B1310" t="n">
-        <v>2797</v>
+        <v>2798</v>
       </c>
       <c r="C1310" t="n">
-        <v>49090.92</v>
+        <v>51818.19</v>
       </c>
     </row>
     <row r="1311">
@@ -14853,10 +14853,10 @@
         <v>46266</v>
       </c>
       <c r="B1311" t="n">
-        <v>2266</v>
+        <v>2797</v>
       </c>
       <c r="C1311" t="n">
-        <v>65454.56</v>
+        <v>51818.19</v>
       </c>
     </row>
     <row r="1312">
@@ -14864,10 +14864,10 @@
         <v>46266</v>
       </c>
       <c r="B1312" t="n">
-        <v>1499</v>
+        <v>2266</v>
       </c>
       <c r="C1312" t="n">
-        <v>114534</v>
+        <v>69090.92</v>
       </c>
     </row>
     <row r="1313">
@@ -14875,10 +14875,10 @@
         <v>46266</v>
       </c>
       <c r="B1313" t="n">
-        <v>2496</v>
+        <v>1499</v>
       </c>
       <c r="C1313" t="n">
-        <v>130896</v>
+        <v>120897</v>
       </c>
     </row>
     <row r="1314">
@@ -14886,10 +14886,10 @@
         <v>46266</v>
       </c>
       <c r="B1314" t="n">
-        <v>949</v>
+        <v>2496</v>
       </c>
       <c r="C1314" t="n">
-        <v>80298</v>
+        <v>138168</v>
       </c>
     </row>
     <row r="1315">
@@ -14897,10 +14897,10 @@
         <v>46266</v>
       </c>
       <c r="B1315" t="n">
-        <v>1853</v>
+        <v>949</v>
       </c>
       <c r="C1315" t="n">
-        <v>98172</v>
+        <v>84759</v>
       </c>
     </row>
     <row r="1316">
@@ -14908,10 +14908,10 @@
         <v>46266</v>
       </c>
       <c r="B1316" t="n">
-        <v>854</v>
+        <v>1853</v>
       </c>
       <c r="C1316" t="n">
-        <v>90000</v>
+        <v>103626</v>
       </c>
     </row>
     <row r="1317">
@@ -14919,10 +14919,10 @@
         <v>46266</v>
       </c>
       <c r="B1317" t="n">
-        <v>2674</v>
+        <v>854</v>
       </c>
       <c r="C1317" t="n">
-        <v>212724</v>
+        <v>95000</v>
       </c>
     </row>
     <row r="1318">
@@ -14930,10 +14930,10 @@
         <v>46266</v>
       </c>
       <c r="B1318" t="n">
-        <v>2803</v>
+        <v>2674</v>
       </c>
       <c r="C1318" t="n">
-        <v>98172</v>
+        <v>224542</v>
       </c>
     </row>
     <row r="1319">
@@ -14941,10 +14941,10 @@
         <v>46266</v>
       </c>
       <c r="B1319" t="n">
-        <v>2599</v>
+        <v>2803</v>
       </c>
       <c r="C1319" t="n">
-        <v>155448</v>
+        <v>103626</v>
       </c>
     </row>
     <row r="1320">
@@ -14952,10 +14952,10 @@
         <v>46266</v>
       </c>
       <c r="B1320" t="n">
-        <v>783</v>
+        <v>2599</v>
       </c>
       <c r="C1320" t="n">
-        <v>42534</v>
+        <v>164084</v>
       </c>
     </row>
     <row r="1321">
@@ -14963,10 +14963,10 @@
         <v>46266</v>
       </c>
       <c r="B1321" t="n">
-        <v>27</v>
+        <v>783</v>
       </c>
       <c r="C1321" t="n">
-        <v>81810</v>
+        <v>44897</v>
       </c>
     </row>
     <row r="1322">
@@ -14974,10 +14974,10 @@
         <v>46266</v>
       </c>
       <c r="B1322" t="n">
-        <v>531</v>
+        <v>27</v>
       </c>
       <c r="C1322" t="n">
-        <v>286362</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1323">
@@ -14985,10 +14985,10 @@
         <v>46266</v>
       </c>
       <c r="B1323" t="n">
-        <v>1308</v>
+        <v>531</v>
       </c>
       <c r="C1323" t="n">
-        <v>132156</v>
+        <v>302271</v>
       </c>
     </row>
     <row r="1324">
@@ -14996,10 +14996,10 @@
         <v>46266</v>
       </c>
       <c r="B1324" t="n">
-        <v>2792</v>
+        <v>1308</v>
       </c>
       <c r="C1324" t="n">
-        <v>95310</v>
+        <v>139498</v>
       </c>
     </row>
     <row r="1325">
@@ -15007,10 +15007,10 @@
         <v>46266</v>
       </c>
       <c r="B1325" t="n">
-        <v>2828</v>
+        <v>2792</v>
       </c>
       <c r="C1325" t="n">
-        <v>0</v>
+        <v>100605</v>
       </c>
     </row>
     <row r="1326">
@@ -15018,10 +15018,10 @@
         <v>46266</v>
       </c>
       <c r="B1326" t="n">
-        <v>2823</v>
+        <v>2828</v>
       </c>
       <c r="C1326" t="n">
-        <v>76500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1327">
@@ -15029,10 +15029,10 @@
         <v>46266</v>
       </c>
       <c r="B1327" t="n">
-        <v>2584</v>
+        <v>2823</v>
       </c>
       <c r="C1327" t="n">
-        <v>51498</v>
+        <v>80750</v>
       </c>
     </row>
     <row r="1328">
@@ -15040,10 +15040,10 @@
         <v>46266</v>
       </c>
       <c r="B1328" t="n">
-        <v>945</v>
+        <v>2584</v>
       </c>
       <c r="C1328" t="n">
-        <v>231804</v>
+        <v>54359</v>
       </c>
     </row>
     <row r="1329">
@@ -15051,10 +15051,10 @@
         <v>46266</v>
       </c>
       <c r="B1329" t="n">
-        <v>2660</v>
+        <v>945</v>
       </c>
       <c r="C1329" t="n">
-        <v>253620</v>
+        <v>244682</v>
       </c>
     </row>
     <row r="1330">
@@ -15062,10 +15062,10 @@
         <v>46266</v>
       </c>
       <c r="B1330" t="n">
-        <v>1317</v>
+        <v>2660</v>
       </c>
       <c r="C1330" t="n">
-        <v>245448</v>
+        <v>267710</v>
       </c>
     </row>
     <row r="1331">
@@ -15073,10 +15073,10 @@
         <v>46266</v>
       </c>
       <c r="B1331" t="n">
-        <v>2790</v>
+        <v>1317</v>
       </c>
       <c r="C1331" t="n">
-        <v>52110</v>
+        <v>259084</v>
       </c>
     </row>
     <row r="1332">
@@ -15084,10 +15084,10 @@
         <v>46266</v>
       </c>
       <c r="B1332" t="n">
-        <v>2711</v>
+        <v>2790</v>
       </c>
       <c r="C1332" t="n">
-        <v>70926.56</v>
+        <v>55005</v>
       </c>
     </row>
     <row r="1333">
@@ -15095,10 +15095,10 @@
         <v>46266</v>
       </c>
       <c r="B1333" t="n">
-        <v>2607</v>
+        <v>2711</v>
       </c>
       <c r="C1333" t="n">
-        <v>40650.56</v>
+        <v>74866.92</v>
       </c>
     </row>
     <row r="1334">
@@ -15106,10 +15106,10 @@
         <v>46266</v>
       </c>
       <c r="B1334" t="n">
-        <v>2667</v>
+        <v>2607</v>
       </c>
       <c r="C1334" t="n">
-        <v>37390.92</v>
+        <v>42908.92</v>
       </c>
     </row>
     <row r="1335">
@@ -15117,10 +15117,10 @@
         <v>46266</v>
       </c>
       <c r="B1335" t="n">
-        <v>2706</v>
+        <v>2667</v>
       </c>
       <c r="C1335" t="n">
-        <v>18026.2</v>
+        <v>39468.19</v>
       </c>
     </row>
     <row r="1336">
@@ -15128,10 +15128,10 @@
         <v>46266</v>
       </c>
       <c r="B1336" t="n">
-        <v>2657</v>
+        <v>2706</v>
       </c>
       <c r="C1336" t="n">
-        <v>64796.76</v>
+        <v>19027.65</v>
       </c>
     </row>
     <row r="1337">
@@ -15139,10 +15139,10 @@
         <v>46266</v>
       </c>
       <c r="B1337" t="n">
-        <v>1278</v>
+        <v>2657</v>
       </c>
       <c r="C1337" t="n">
-        <v>81810</v>
+        <v>68396.57000000001</v>
       </c>
     </row>
     <row r="1338">
@@ -15150,10 +15150,10 @@
         <v>46266</v>
       </c>
       <c r="B1338" t="n">
-        <v>2745</v>
+        <v>1278</v>
       </c>
       <c r="C1338" t="n">
-        <v>90000</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1339">
@@ -15161,10 +15161,10 @@
         <v>46266</v>
       </c>
       <c r="B1339" t="n">
-        <v>2753</v>
+        <v>2745</v>
       </c>
       <c r="C1339" t="n">
-        <v>61362</v>
+        <v>95000</v>
       </c>
     </row>
     <row r="1340">
@@ -15172,10 +15172,10 @@
         <v>46266</v>
       </c>
       <c r="B1340" t="n">
-        <v>2183</v>
+        <v>2753</v>
       </c>
       <c r="C1340" t="n">
-        <v>299412</v>
+        <v>64771</v>
       </c>
     </row>
     <row r="1341">
@@ -15183,10 +15183,10 @@
         <v>46266</v>
       </c>
       <c r="B1341" t="n">
-        <v>1340</v>
+        <v>2183</v>
       </c>
       <c r="C1341" t="n">
-        <v>118620</v>
+        <v>316046</v>
       </c>
     </row>
     <row r="1342">
@@ -15194,10 +15194,10 @@
         <v>46266</v>
       </c>
       <c r="B1342" t="n">
-        <v>2583</v>
+        <v>1340</v>
       </c>
       <c r="C1342" t="n">
-        <v>34038</v>
+        <v>125210</v>
       </c>
     </row>
     <row r="1343">
@@ -15205,10 +15205,10 @@
         <v>46266</v>
       </c>
       <c r="B1343" t="n">
-        <v>2090</v>
+        <v>2583</v>
       </c>
       <c r="C1343" t="n">
-        <v>34038</v>
+        <v>35929</v>
       </c>
     </row>
     <row r="1344">
@@ -15216,10 +15216,10 @@
         <v>46266</v>
       </c>
       <c r="B1344" t="n">
-        <v>1277</v>
+        <v>2090</v>
       </c>
       <c r="C1344" t="n">
-        <v>180000</v>
+        <v>35929</v>
       </c>
     </row>
     <row r="1345">
@@ -15227,10 +15227,10 @@
         <v>46266</v>
       </c>
       <c r="B1345" t="n">
-        <v>1501</v>
+        <v>1277</v>
       </c>
       <c r="C1345" t="n">
-        <v>77724</v>
+        <v>190000</v>
       </c>
     </row>
     <row r="1346">
@@ -15238,10 +15238,21 @@
         <v>46266</v>
       </c>
       <c r="B1346" t="n">
+        <v>1501</v>
+      </c>
+      <c r="C1346" t="n">
+        <v>82042</v>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1347" t="n">
         <v>703</v>
       </c>
-      <c r="C1346" t="n">
-        <v>204534</v>
+      <c r="C1347" t="n">
+        <v>215897</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:01:53
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -11292,7 +11292,7 @@
         <v>931</v>
       </c>
       <c r="C987" t="n">
-        <v>81548</v>
+        <v>85840</v>
       </c>
     </row>
     <row r="988">
@@ -11303,7 +11303,7 @@
         <v>947</v>
       </c>
       <c r="C988" t="n">
-        <v>375269</v>
+        <v>395020</v>
       </c>
     </row>
     <row r="989">
@@ -11314,7 +11314,7 @@
         <v>1956</v>
       </c>
       <c r="C989" t="n">
-        <v>218044</v>
+        <v>229520</v>
       </c>
     </row>
     <row r="990">
@@ -11325,7 +11325,7 @@
         <v>2824</v>
       </c>
       <c r="C990" t="n">
-        <v>95000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="991">
@@ -11336,7 +11336,7 @@
         <v>2787</v>
       </c>
       <c r="C991" t="n">
-        <v>112271</v>
+        <v>118180</v>
       </c>
     </row>
     <row r="992">
@@ -11347,7 +11347,7 @@
         <v>2830</v>
       </c>
       <c r="C992" t="n">
-        <v>77710</v>
+        <v>81800</v>
       </c>
     </row>
     <row r="993">
@@ -11358,7 +11358,7 @@
         <v>1254</v>
       </c>
       <c r="C993" t="n">
-        <v>167714.73</v>
+        <v>176541.82</v>
       </c>
     </row>
     <row r="994">
@@ -11369,7 +11369,7 @@
         <v>816</v>
       </c>
       <c r="C994" t="n">
-        <v>231325</v>
+        <v>243500</v>
       </c>
     </row>
     <row r="995">
@@ -11380,7 +11380,7 @@
         <v>2671</v>
       </c>
       <c r="C995" t="n">
-        <v>69084</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="996">
@@ -11391,7 +11391,7 @@
         <v>2705</v>
       </c>
       <c r="C996" t="n">
-        <v>154755</v>
+        <v>162900</v>
       </c>
     </row>
     <row r="997">
@@ -11402,7 +11402,7 @@
         <v>2333</v>
       </c>
       <c r="C997" t="n">
-        <v>133304</v>
+        <v>140320</v>
       </c>
     </row>
     <row r="998">
@@ -11413,7 +11413,7 @@
         <v>2440</v>
       </c>
       <c r="C998" t="n">
-        <v>77710</v>
+        <v>81800</v>
       </c>
     </row>
     <row r="999">
@@ -11424,7 +11424,7 @@
         <v>2448</v>
       </c>
       <c r="C999" t="n">
-        <v>17271</v>
+        <v>18180</v>
       </c>
     </row>
     <row r="1000">
@@ -11435,7 +11435,7 @@
         <v>2310</v>
       </c>
       <c r="C1000" t="n">
-        <v>59318</v>
+        <v>62440</v>
       </c>
     </row>
     <row r="1001">
@@ -11446,7 +11446,7 @@
         <v>2809</v>
       </c>
       <c r="C1001" t="n">
-        <v>59318</v>
+        <v>62440</v>
       </c>
     </row>
     <row r="1002">
@@ -11457,7 +11457,7 @@
         <v>2548</v>
       </c>
       <c r="C1002" t="n">
-        <v>50540</v>
+        <v>53200</v>
       </c>
     </row>
     <row r="1003">
@@ -11468,7 +11468,7 @@
         <v>451</v>
       </c>
       <c r="C1003" t="n">
-        <v>207271</v>
+        <v>218180</v>
       </c>
     </row>
     <row r="1004">
@@ -11479,7 +11479,7 @@
         <v>933</v>
       </c>
       <c r="C1004" t="n">
-        <v>70376</v>
+        <v>74080</v>
       </c>
     </row>
     <row r="1005">
@@ -11490,7 +11490,7 @@
         <v>2702</v>
       </c>
       <c r="C1005" t="n">
-        <v>70376</v>
+        <v>74080</v>
       </c>
     </row>
     <row r="1006">
@@ -11501,7 +11501,7 @@
         <v>2549</v>
       </c>
       <c r="C1006" t="n">
-        <v>24472</v>
+        <v>25760</v>
       </c>
     </row>
     <row r="1007">
@@ -11512,7 +11512,7 @@
         <v>535</v>
       </c>
       <c r="C1007" t="n">
-        <v>319542</v>
+        <v>336360</v>
       </c>
     </row>
     <row r="1008">
@@ -11523,7 +11523,7 @@
         <v>1117</v>
       </c>
       <c r="C1008" t="n">
-        <v>300447</v>
+        <v>316260</v>
       </c>
     </row>
     <row r="1009">
@@ -11545,7 +11545,7 @@
         <v>530</v>
       </c>
       <c r="C1010" t="n">
-        <v>210786</v>
+        <v>221880</v>
       </c>
     </row>
     <row r="1011">
@@ -11556,7 +11556,7 @@
         <v>358</v>
       </c>
       <c r="C1011" t="n">
-        <v>293626</v>
+        <v>309080</v>
       </c>
     </row>
     <row r="1012">
@@ -11567,7 +11567,7 @@
         <v>2498</v>
       </c>
       <c r="C1012" t="n">
-        <v>47956</v>
+        <v>50480</v>
       </c>
     </row>
     <row r="1013">
@@ -11578,7 +11578,7 @@
         <v>2381</v>
       </c>
       <c r="C1013" t="n">
-        <v>68514</v>
+        <v>72120</v>
       </c>
     </row>
     <row r="1014">
@@ -11589,7 +11589,7 @@
         <v>2695</v>
       </c>
       <c r="C1014" t="n">
-        <v>41211</v>
+        <v>43380</v>
       </c>
     </row>
     <row r="1015">
@@ -11600,7 +11600,7 @@
         <v>2744</v>
       </c>
       <c r="C1015" t="n">
-        <v>51818.19</v>
+        <v>54545.46</v>
       </c>
     </row>
     <row r="1016">
@@ -11611,7 +11611,7 @@
         <v>2750</v>
       </c>
       <c r="C1016" t="n">
-        <v>51813</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1017">
@@ -11622,7 +11622,7 @@
         <v>2131</v>
       </c>
       <c r="C1017" t="n">
-        <v>103626</v>
+        <v>109080</v>
       </c>
     </row>
     <row r="1018">
@@ -11633,7 +11633,7 @@
         <v>818</v>
       </c>
       <c r="C1018" t="n">
-        <v>345439</v>
+        <v>363620</v>
       </c>
     </row>
     <row r="1019">
@@ -11644,7 +11644,7 @@
         <v>2566</v>
       </c>
       <c r="C1019" t="n">
-        <v>69084</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1020">
@@ -11655,7 +11655,7 @@
         <v>132</v>
       </c>
       <c r="C1020" t="n">
-        <v>647710</v>
+        <v>681800</v>
       </c>
     </row>
     <row r="1021">
@@ -11666,7 +11666,7 @@
         <v>2431</v>
       </c>
       <c r="C1021" t="n">
-        <v>158897</v>
+        <v>167260</v>
       </c>
     </row>
     <row r="1022">
@@ -11677,7 +11677,7 @@
         <v>2249</v>
       </c>
       <c r="C1022" t="n">
-        <v>168682</v>
+        <v>177560</v>
       </c>
     </row>
     <row r="1023">
@@ -11688,7 +11688,7 @@
         <v>1585</v>
       </c>
       <c r="C1023" t="n">
-        <v>142538</v>
+        <v>150040</v>
       </c>
     </row>
     <row r="1024">
@@ -11699,7 +11699,7 @@
         <v>2325</v>
       </c>
       <c r="C1024" t="n">
-        <v>137788</v>
+        <v>145040</v>
       </c>
     </row>
     <row r="1025">
@@ -11710,7 +11710,7 @@
         <v>2190</v>
       </c>
       <c r="C1025" t="n">
-        <v>194313</v>
+        <v>204540</v>
       </c>
     </row>
     <row r="1026">
@@ -11721,7 +11721,7 @@
         <v>1466</v>
       </c>
       <c r="C1026" t="n">
-        <v>349771</v>
+        <v>368180</v>
       </c>
     </row>
     <row r="1027">
@@ -11732,7 +11732,7 @@
         <v>2659</v>
       </c>
       <c r="C1027" t="n">
-        <v>106229</v>
+        <v>111820</v>
       </c>
     </row>
     <row r="1028">
@@ -11743,7 +11743,7 @@
         <v>1384</v>
       </c>
       <c r="C1028" t="n">
-        <v>388626</v>
+        <v>409080</v>
       </c>
     </row>
     <row r="1029">
@@ -11754,7 +11754,7 @@
         <v>634</v>
       </c>
       <c r="C1029" t="n">
-        <v>475000</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="1030">
@@ -11765,7 +11765,7 @@
         <v>2804</v>
       </c>
       <c r="C1030" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1031">
@@ -11776,7 +11776,7 @@
         <v>2375</v>
       </c>
       <c r="C1031" t="n">
-        <v>285000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="1032">
@@ -11787,7 +11787,7 @@
         <v>2601</v>
       </c>
       <c r="C1032" t="n">
-        <v>237500</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="1033">
@@ -11798,7 +11798,7 @@
         <v>952</v>
       </c>
       <c r="C1033" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1034">
@@ -11809,7 +11809,7 @@
         <v>571</v>
       </c>
       <c r="C1034" t="n">
-        <v>549689</v>
+        <v>578620</v>
       </c>
     </row>
     <row r="1035">
@@ -11820,7 +11820,7 @@
         <v>2697</v>
       </c>
       <c r="C1035" t="n">
-        <v>167485</v>
+        <v>176300</v>
       </c>
     </row>
     <row r="1036">
@@ -11831,7 +11831,7 @@
         <v>2678</v>
       </c>
       <c r="C1036" t="n">
-        <v>289769</v>
+        <v>305020</v>
       </c>
     </row>
     <row r="1037">
@@ -11842,7 +11842,7 @@
         <v>2768</v>
       </c>
       <c r="C1037" t="n">
-        <v>303259</v>
+        <v>319220</v>
       </c>
     </row>
     <row r="1038">
@@ -11853,7 +11853,7 @@
         <v>2359</v>
       </c>
       <c r="C1038" t="n">
-        <v>91979</v>
+        <v>96820</v>
       </c>
     </row>
     <row r="1039">
@@ -11864,7 +11864,7 @@
         <v>353</v>
       </c>
       <c r="C1039" t="n">
-        <v>298805.42</v>
+        <v>314532.01</v>
       </c>
     </row>
     <row r="1040">
@@ -11875,7 +11875,7 @@
         <v>2026</v>
       </c>
       <c r="C1040" t="n">
-        <v>247581.62</v>
+        <v>260612.23</v>
       </c>
     </row>
     <row r="1041">
@@ -11897,7 +11897,7 @@
         <v>2345</v>
       </c>
       <c r="C1042" t="n">
-        <v>54359</v>
+        <v>57220</v>
       </c>
     </row>
     <row r="1043">
@@ -11908,7 +11908,7 @@
         <v>2789</v>
       </c>
       <c r="C1043" t="n">
-        <v>146813</v>
+        <v>154540</v>
       </c>
     </row>
     <row r="1044">
@@ -11919,7 +11919,7 @@
         <v>569</v>
       </c>
       <c r="C1044" t="n">
-        <v>2473382</v>
+        <v>2603560</v>
       </c>
     </row>
     <row r="1045">
@@ -11930,7 +11930,7 @@
         <v>2822</v>
       </c>
       <c r="C1045" t="n">
-        <v>116584</v>
+        <v>122720</v>
       </c>
     </row>
     <row r="1046">
@@ -11941,7 +11941,7 @@
         <v>2728</v>
       </c>
       <c r="C1046" t="n">
-        <v>8626</v>
+        <v>9080</v>
       </c>
     </row>
     <row r="1047">
@@ -11952,7 +11952,7 @@
         <v>2488</v>
       </c>
       <c r="C1047" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1048">
@@ -11963,7 +11963,7 @@
         <v>2791</v>
       </c>
       <c r="C1048" t="n">
-        <v>85232.3</v>
+        <v>89718.2</v>
       </c>
     </row>
     <row r="1049">
@@ -11974,7 +11974,7 @@
         <v>2577</v>
       </c>
       <c r="C1049" t="n">
-        <v>77010.55</v>
+        <v>81063.73</v>
       </c>
     </row>
     <row r="1050">
@@ -11985,7 +11985,7 @@
         <v>2069</v>
       </c>
       <c r="C1050" t="n">
-        <v>155439</v>
+        <v>163620</v>
       </c>
     </row>
     <row r="1051">
@@ -11996,7 +11996,7 @@
         <v>2082</v>
       </c>
       <c r="C1051" t="n">
-        <v>143849</v>
+        <v>151420</v>
       </c>
     </row>
     <row r="1052">
@@ -12007,7 +12007,7 @@
         <v>781</v>
       </c>
       <c r="C1052" t="n">
-        <v>112271</v>
+        <v>118180</v>
       </c>
     </row>
     <row r="1053">
@@ -12018,7 +12018,7 @@
         <v>744</v>
       </c>
       <c r="C1053" t="n">
-        <v>35929</v>
+        <v>37820</v>
       </c>
     </row>
     <row r="1054">
@@ -12029,7 +12029,7 @@
         <v>2223</v>
       </c>
       <c r="C1054" t="n">
-        <v>113943</v>
+        <v>119940</v>
       </c>
     </row>
     <row r="1055">
@@ -12040,7 +12040,7 @@
         <v>2452</v>
       </c>
       <c r="C1055" t="n">
-        <v>60439</v>
+        <v>63620</v>
       </c>
     </row>
     <row r="1056">
@@ -12051,7 +12051,7 @@
         <v>970</v>
       </c>
       <c r="C1056" t="n">
-        <v>59318</v>
+        <v>62440</v>
       </c>
     </row>
     <row r="1057">
@@ -12062,7 +12062,7 @@
         <v>2550</v>
       </c>
       <c r="C1057" t="n">
-        <v>52668</v>
+        <v>55440</v>
       </c>
     </row>
     <row r="1058">
@@ -12073,7 +12073,7 @@
         <v>768</v>
       </c>
       <c r="C1058" t="n">
-        <v>112271</v>
+        <v>118180</v>
       </c>
     </row>
     <row r="1059">
@@ -12084,7 +12084,7 @@
         <v>1075</v>
       </c>
       <c r="C1059" t="n">
-        <v>391210</v>
+        <v>411800</v>
       </c>
     </row>
     <row r="1060">
@@ -12095,7 +12095,7 @@
         <v>664</v>
       </c>
       <c r="C1060" t="n">
-        <v>223668</v>
+        <v>235440</v>
       </c>
     </row>
     <row r="1061">
@@ -12106,7 +12106,7 @@
         <v>2555</v>
       </c>
       <c r="C1061" t="n">
-        <v>35853</v>
+        <v>37740</v>
       </c>
     </row>
     <row r="1062">
@@ -12117,7 +12117,7 @@
         <v>2627</v>
       </c>
       <c r="C1062" t="n">
-        <v>21052</v>
+        <v>22160</v>
       </c>
     </row>
     <row r="1063">
@@ -12128,7 +12128,7 @@
         <v>2557</v>
       </c>
       <c r="C1063" t="n">
-        <v>22268</v>
+        <v>23440</v>
       </c>
     </row>
     <row r="1064">
@@ -12139,7 +12139,7 @@
         <v>2551</v>
       </c>
       <c r="C1064" t="n">
-        <v>17689</v>
+        <v>18620</v>
       </c>
     </row>
     <row r="1065">
@@ -12150,7 +12150,7 @@
         <v>2463</v>
       </c>
       <c r="C1065" t="n">
-        <v>276545</v>
+        <v>291100</v>
       </c>
     </row>
     <row r="1066">
@@ -12161,7 +12161,7 @@
         <v>2279</v>
       </c>
       <c r="C1066" t="n">
-        <v>208639</v>
+        <v>219620</v>
       </c>
     </row>
     <row r="1067">
@@ -12172,7 +12172,7 @@
         <v>631</v>
       </c>
       <c r="C1067" t="n">
-        <v>302271</v>
+        <v>318180</v>
       </c>
     </row>
     <row r="1068">
@@ -12183,7 +12183,7 @@
         <v>2251</v>
       </c>
       <c r="C1068" t="n">
-        <v>185098</v>
+        <v>194840</v>
       </c>
     </row>
     <row r="1069">
@@ -12194,7 +12194,7 @@
         <v>1653</v>
       </c>
       <c r="C1069" t="n">
-        <v>280668</v>
+        <v>295440</v>
       </c>
     </row>
     <row r="1070">
@@ -12205,7 +12205,7 @@
         <v>1293</v>
       </c>
       <c r="C1070" t="n">
-        <v>358397</v>
+        <v>377260</v>
       </c>
     </row>
     <row r="1071">
@@ -12216,7 +12216,7 @@
         <v>360</v>
       </c>
       <c r="C1071" t="n">
-        <v>431813</v>
+        <v>454540</v>
       </c>
     </row>
     <row r="1072">
@@ -12227,7 +12227,7 @@
         <v>1063</v>
       </c>
       <c r="C1072" t="n">
-        <v>313975</v>
+        <v>330500</v>
       </c>
     </row>
     <row r="1073">
@@ -12238,7 +12238,7 @@
         <v>2273</v>
       </c>
       <c r="C1073" t="n">
-        <v>183160</v>
+        <v>192800</v>
       </c>
     </row>
     <row r="1074">
@@ -12249,7 +12249,7 @@
         <v>2757</v>
       </c>
       <c r="C1074" t="n">
-        <v>60454.57</v>
+        <v>63636.38</v>
       </c>
     </row>
     <row r="1075">
@@ -12260,7 +12260,7 @@
         <v>2795</v>
       </c>
       <c r="C1075" t="n">
-        <v>51818.19</v>
+        <v>54545.46</v>
       </c>
     </row>
     <row r="1076">
@@ -12271,7 +12271,7 @@
         <v>2722</v>
       </c>
       <c r="C1076" t="n">
-        <v>51813</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1077">
@@ -12282,7 +12282,7 @@
         <v>2718</v>
       </c>
       <c r="C1077" t="n">
-        <v>69084</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1078">
@@ -12293,7 +12293,7 @@
         <v>595</v>
       </c>
       <c r="C1078" t="n">
-        <v>475000</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="1079">
@@ -12304,7 +12304,7 @@
         <v>890</v>
       </c>
       <c r="C1079" t="n">
-        <v>604542</v>
+        <v>636360</v>
       </c>
     </row>
     <row r="1080">
@@ -12315,7 +12315,7 @@
         <v>2652</v>
       </c>
       <c r="C1080" t="n">
-        <v>112271</v>
+        <v>118180</v>
       </c>
     </row>
     <row r="1081">
@@ -12326,7 +12326,7 @@
         <v>2714</v>
       </c>
       <c r="C1081" t="n">
-        <v>310897</v>
+        <v>327260</v>
       </c>
     </row>
     <row r="1082">
@@ -12337,7 +12337,7 @@
         <v>1869</v>
       </c>
       <c r="C1082" t="n">
-        <v>198626</v>
+        <v>209080</v>
       </c>
     </row>
     <row r="1083">
@@ -12348,7 +12348,7 @@
         <v>400</v>
       </c>
       <c r="C1083" t="n">
-        <v>164084</v>
+        <v>172720</v>
       </c>
     </row>
     <row r="1084">
@@ -12359,7 +12359,7 @@
         <v>1907</v>
       </c>
       <c r="C1084" t="n">
-        <v>320397</v>
+        <v>337260</v>
       </c>
     </row>
     <row r="1085">
@@ -12370,7 +12370,7 @@
         <v>1996</v>
       </c>
       <c r="C1085" t="n">
-        <v>202521</v>
+        <v>213180</v>
       </c>
     </row>
     <row r="1086">
@@ -12381,7 +12381,7 @@
         <v>1890</v>
       </c>
       <c r="C1086" t="n">
-        <v>273032.3</v>
+        <v>287402.41</v>
       </c>
     </row>
     <row r="1087">
@@ -12392,7 +12392,7 @@
         <v>2114</v>
       </c>
       <c r="C1087" t="n">
-        <v>158650</v>
+        <v>167000</v>
       </c>
     </row>
     <row r="1088">
@@ -12403,7 +12403,7 @@
         <v>2330</v>
       </c>
       <c r="C1088" t="n">
-        <v>232123</v>
+        <v>244340</v>
       </c>
     </row>
     <row r="1089">
@@ -12447,7 +12447,7 @@
         <v>2629</v>
       </c>
       <c r="C1092" t="n">
-        <v>59318</v>
+        <v>62440</v>
       </c>
     </row>
     <row r="1093">
@@ -12458,7 +12458,7 @@
         <v>951</v>
       </c>
       <c r="C1093" t="n">
-        <v>99313</v>
+        <v>104540</v>
       </c>
     </row>
     <row r="1094">
@@ -12469,7 +12469,7 @@
         <v>2449</v>
       </c>
       <c r="C1094" t="n">
-        <v>34542</v>
+        <v>36360</v>
       </c>
     </row>
     <row r="1095">
@@ -12480,7 +12480,7 @@
         <v>610</v>
       </c>
       <c r="C1095" t="n">
-        <v>703855</v>
+        <v>740900</v>
       </c>
     </row>
     <row r="1096">
@@ -12491,7 +12491,7 @@
         <v>2761</v>
       </c>
       <c r="C1096" t="n">
-        <v>70376</v>
+        <v>74080</v>
       </c>
     </row>
     <row r="1097">
@@ -12502,7 +12502,7 @@
         <v>483</v>
       </c>
       <c r="C1097" t="n">
-        <v>382584</v>
+        <v>402720</v>
       </c>
     </row>
     <row r="1098">
@@ -12513,7 +12513,7 @@
         <v>2015</v>
       </c>
       <c r="C1098" t="n">
-        <v>319542</v>
+        <v>336360</v>
       </c>
     </row>
     <row r="1099">
@@ -12524,7 +12524,7 @@
         <v>1478</v>
       </c>
       <c r="C1099" t="n">
-        <v>467362</v>
+        <v>491960</v>
       </c>
     </row>
     <row r="1100">
@@ -12535,7 +12535,7 @@
         <v>424</v>
       </c>
       <c r="C1100" t="n">
-        <v>208639</v>
+        <v>219620</v>
       </c>
     </row>
     <row r="1101">
@@ -12557,7 +12557,7 @@
         <v>477</v>
       </c>
       <c r="C1102" t="n">
-        <v>223383</v>
+        <v>235140</v>
       </c>
     </row>
     <row r="1103">
@@ -12568,7 +12568,7 @@
         <v>1810</v>
       </c>
       <c r="C1103" t="n">
-        <v>34599</v>
+        <v>36420</v>
       </c>
     </row>
     <row r="1104">
@@ -12579,7 +12579,7 @@
         <v>2826</v>
       </c>
       <c r="C1104" t="n">
-        <v>60454.57</v>
+        <v>63636.38</v>
       </c>
     </row>
     <row r="1105">
@@ -12590,7 +12590,7 @@
         <v>2561</v>
       </c>
       <c r="C1105" t="n">
-        <v>12692</v>
+        <v>13360</v>
       </c>
     </row>
     <row r="1106">
@@ -12601,7 +12601,7 @@
         <v>2653</v>
       </c>
       <c r="C1106" t="n">
-        <v>51818.19</v>
+        <v>54545.46</v>
       </c>
     </row>
     <row r="1107">
@@ -12612,7 +12612,7 @@
         <v>2829</v>
       </c>
       <c r="C1107" t="n">
-        <v>51818.19</v>
+        <v>54545.46</v>
       </c>
     </row>
     <row r="1108">
@@ -12623,7 +12623,7 @@
         <v>2643</v>
       </c>
       <c r="C1108" t="n">
-        <v>25498</v>
+        <v>26840</v>
       </c>
     </row>
     <row r="1109">
@@ -12634,7 +12634,7 @@
         <v>2794</v>
       </c>
       <c r="C1109" t="n">
-        <v>77710</v>
+        <v>81800</v>
       </c>
     </row>
     <row r="1110">
@@ -12645,7 +12645,7 @@
         <v>2655</v>
       </c>
       <c r="C1110" t="n">
-        <v>95000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1111">
@@ -12656,7 +12656,7 @@
         <v>1456</v>
       </c>
       <c r="C1111" t="n">
-        <v>665247</v>
+        <v>700260</v>
       </c>
     </row>
     <row r="1112">
@@ -12667,7 +12667,7 @@
         <v>2606</v>
       </c>
       <c r="C1112" t="n">
-        <v>204326</v>
+        <v>215080</v>
       </c>
     </row>
     <row r="1113">
@@ -12678,7 +12678,7 @@
         <v>1142</v>
       </c>
       <c r="C1113" t="n">
-        <v>370538</v>
+        <v>390040</v>
       </c>
     </row>
     <row r="1114">
@@ -12689,7 +12689,7 @@
         <v>1450</v>
       </c>
       <c r="C1114" t="n">
-        <v>235391</v>
+        <v>247780</v>
       </c>
     </row>
     <row r="1115">
@@ -12700,7 +12700,7 @@
         <v>2133</v>
       </c>
       <c r="C1115" t="n">
-        <v>549689</v>
+        <v>578620</v>
       </c>
     </row>
     <row r="1116">
@@ -12711,7 +12711,7 @@
         <v>522</v>
       </c>
       <c r="C1116" t="n">
-        <v>168397</v>
+        <v>177260</v>
       </c>
     </row>
     <row r="1117">
@@ -12722,7 +12722,7 @@
         <v>2696</v>
       </c>
       <c r="C1117" t="n">
-        <v>227240</v>
+        <v>239200</v>
       </c>
     </row>
     <row r="1118">
@@ -12744,7 +12744,7 @@
         <v>2692</v>
       </c>
       <c r="C1119" t="n">
-        <v>64771</v>
+        <v>68180</v>
       </c>
     </row>
     <row r="1120">
@@ -12755,7 +12755,7 @@
         <v>2691</v>
       </c>
       <c r="C1120" t="n">
-        <v>116584</v>
+        <v>122720</v>
       </c>
     </row>
     <row r="1121">
@@ -12766,7 +12766,7 @@
         <v>1632</v>
       </c>
       <c r="C1121" t="n">
-        <v>215897</v>
+        <v>227260</v>
       </c>
     </row>
     <row r="1122">
@@ -12777,7 +12777,7 @@
         <v>2641</v>
       </c>
       <c r="C1122" t="n">
-        <v>69084</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1123">
@@ -12788,7 +12788,7 @@
         <v>2197</v>
       </c>
       <c r="C1123" t="n">
-        <v>172710</v>
+        <v>181800</v>
       </c>
     </row>
     <row r="1124">
@@ -12799,7 +12799,7 @@
         <v>609</v>
       </c>
       <c r="C1124" t="n">
-        <v>190000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="1125">
@@ -12810,7 +12810,7 @@
         <v>1380</v>
       </c>
       <c r="C1125" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1126">
@@ -12821,7 +12821,7 @@
         <v>104</v>
       </c>
       <c r="C1126" t="n">
-        <v>259084</v>
+        <v>272720</v>
       </c>
     </row>
     <row r="1127">
@@ -12832,7 +12832,7 @@
         <v>2621</v>
       </c>
       <c r="C1127" t="n">
-        <v>60439</v>
+        <v>63620</v>
       </c>
     </row>
     <row r="1128">
@@ -12843,7 +12843,7 @@
         <v>2786</v>
       </c>
       <c r="C1128" t="n">
-        <v>60439</v>
+        <v>63620</v>
       </c>
     </row>
     <row r="1129">
@@ -12854,7 +12854,7 @@
         <v>2784</v>
       </c>
       <c r="C1129" t="n">
-        <v>35929</v>
+        <v>37820</v>
       </c>
     </row>
     <row r="1130">
@@ -12865,7 +12865,7 @@
         <v>2586</v>
       </c>
       <c r="C1130" t="n">
-        <v>35929</v>
+        <v>37820</v>
       </c>
     </row>
     <row r="1131">
@@ -12876,7 +12876,7 @@
         <v>2145</v>
       </c>
       <c r="C1131" t="n">
-        <v>111796</v>
+        <v>117680</v>
       </c>
     </row>
     <row r="1132">
@@ -12887,7 +12887,7 @@
         <v>2574</v>
       </c>
       <c r="C1132" t="n">
-        <v>111796</v>
+        <v>117680</v>
       </c>
     </row>
     <row r="1133">
@@ -12898,7 +12898,7 @@
         <v>2492</v>
       </c>
       <c r="C1133" t="n">
-        <v>122550</v>
+        <v>129000</v>
       </c>
     </row>
     <row r="1134">
@@ -12909,7 +12909,7 @@
         <v>629</v>
       </c>
       <c r="C1134" t="n">
-        <v>381710</v>
+        <v>401800</v>
       </c>
     </row>
     <row r="1135">
@@ -12920,7 +12920,7 @@
         <v>966</v>
       </c>
       <c r="C1135" t="n">
-        <v>70376</v>
+        <v>74080</v>
       </c>
     </row>
     <row r="1136">
@@ -12931,7 +12931,7 @@
         <v>2721</v>
       </c>
       <c r="C1136" t="n">
-        <v>70376</v>
+        <v>74080</v>
       </c>
     </row>
     <row r="1137">
@@ -12942,7 +12942,7 @@
         <v>2554</v>
       </c>
       <c r="C1137" t="n">
-        <v>21204</v>
+        <v>22320</v>
       </c>
     </row>
     <row r="1138">
@@ -12953,7 +12953,7 @@
         <v>2556</v>
       </c>
       <c r="C1138" t="n">
-        <v>31179</v>
+        <v>32820</v>
       </c>
     </row>
     <row r="1139">
@@ -12964,7 +12964,7 @@
         <v>2546</v>
       </c>
       <c r="C1139" t="n">
-        <v>20596</v>
+        <v>21680</v>
       </c>
     </row>
     <row r="1140">
@@ -12975,7 +12975,7 @@
         <v>42</v>
       </c>
       <c r="C1140" t="n">
-        <v>1632271</v>
+        <v>1718180</v>
       </c>
     </row>
     <row r="1141">
@@ -12986,7 +12986,7 @@
         <v>953</v>
       </c>
       <c r="C1141" t="n">
-        <v>589570</v>
+        <v>620600</v>
       </c>
     </row>
     <row r="1142">
@@ -12997,7 +12997,7 @@
         <v>1137</v>
       </c>
       <c r="C1142" t="n">
-        <v>552710</v>
+        <v>581800</v>
       </c>
     </row>
     <row r="1143">
@@ -13008,7 +13008,7 @@
         <v>675</v>
       </c>
       <c r="C1143" t="n">
-        <v>172710</v>
+        <v>181800</v>
       </c>
     </row>
     <row r="1144">
@@ -13019,7 +13019,7 @@
         <v>619</v>
       </c>
       <c r="C1144" t="n">
-        <v>267064</v>
+        <v>281120</v>
       </c>
     </row>
     <row r="1145">
@@ -13030,7 +13030,7 @@
         <v>1299</v>
       </c>
       <c r="C1145" t="n">
-        <v>449388</v>
+        <v>473040</v>
       </c>
     </row>
     <row r="1146">
@@ -13041,7 +13041,7 @@
         <v>1064</v>
       </c>
       <c r="C1146" t="n">
-        <v>517636</v>
+        <v>544880</v>
       </c>
     </row>
     <row r="1147">
@@ -13052,7 +13052,7 @@
         <v>2308</v>
       </c>
       <c r="C1147" t="n">
-        <v>177042</v>
+        <v>186360</v>
       </c>
     </row>
     <row r="1148">
@@ -13063,7 +13063,7 @@
         <v>2747</v>
       </c>
       <c r="C1148" t="n">
-        <v>51818.19</v>
+        <v>54545.46</v>
       </c>
     </row>
     <row r="1149">
@@ -13074,7 +13074,7 @@
         <v>2819</v>
       </c>
       <c r="C1149" t="n">
-        <v>51818.19</v>
+        <v>54545.46</v>
       </c>
     </row>
     <row r="1150">
@@ -13085,7 +13085,7 @@
         <v>1259</v>
       </c>
       <c r="C1150" t="n">
-        <v>86363.64999999999</v>
+        <v>90909.10000000001</v>
       </c>
     </row>
     <row r="1151">
@@ -13096,7 +13096,7 @@
         <v>2544</v>
       </c>
       <c r="C1151" t="n">
-        <v>69084</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1152">
@@ -13107,7 +13107,7 @@
         <v>2261</v>
       </c>
       <c r="C1152" t="n">
-        <v>129542</v>
+        <v>136360</v>
       </c>
     </row>
     <row r="1153">
@@ -13118,7 +13118,7 @@
         <v>2729</v>
       </c>
       <c r="C1153" t="n">
-        <v>69084</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1154">
@@ -13129,7 +13129,7 @@
         <v>2649</v>
       </c>
       <c r="C1154" t="n">
-        <v>25498</v>
+        <v>26840</v>
       </c>
     </row>
     <row r="1155">
@@ -13140,7 +13140,7 @@
         <v>2494</v>
       </c>
       <c r="C1155" t="n">
-        <v>112271</v>
+        <v>118180</v>
       </c>
     </row>
     <row r="1156">
@@ -13162,7 +13162,7 @@
         <v>2802</v>
       </c>
       <c r="C1157" t="n">
-        <v>61161</v>
+        <v>64380</v>
       </c>
     </row>
     <row r="1158">
@@ -13173,7 +13173,7 @@
         <v>2726</v>
       </c>
       <c r="C1158" t="n">
-        <v>129542</v>
+        <v>136360</v>
       </c>
     </row>
     <row r="1159">
@@ -13184,7 +13184,7 @@
         <v>2820</v>
       </c>
       <c r="C1159" t="n">
-        <v>155439</v>
+        <v>163620</v>
       </c>
     </row>
     <row r="1160">
@@ -13195,7 +13195,7 @@
         <v>1007</v>
       </c>
       <c r="C1160" t="n">
-        <v>164084</v>
+        <v>172720</v>
       </c>
     </row>
     <row r="1161">
@@ -13206,7 +13206,7 @@
         <v>20</v>
       </c>
       <c r="C1161" t="n">
-        <v>332500</v>
+        <v>350000</v>
       </c>
     </row>
     <row r="1162">
@@ -13217,7 +13217,7 @@
         <v>1372</v>
       </c>
       <c r="C1162" t="n">
-        <v>250439</v>
+        <v>263620</v>
       </c>
     </row>
     <row r="1163">
@@ -13228,7 +13228,7 @@
         <v>2735</v>
       </c>
       <c r="C1163" t="n">
-        <v>103626</v>
+        <v>109080</v>
       </c>
     </row>
     <row r="1164">
@@ -13239,7 +13239,7 @@
         <v>2811</v>
       </c>
       <c r="C1164" t="n">
-        <v>35929</v>
+        <v>37820</v>
       </c>
     </row>
     <row r="1165">
@@ -13250,7 +13250,7 @@
         <v>1871</v>
       </c>
       <c r="C1165" t="n">
-        <v>152646</v>
+        <v>160680</v>
       </c>
     </row>
     <row r="1166">
@@ -13261,7 +13261,7 @@
         <v>2541</v>
       </c>
       <c r="C1166" t="n">
-        <v>182742</v>
+        <v>192360</v>
       </c>
     </row>
     <row r="1167">
@@ -13272,7 +13272,7 @@
         <v>2362</v>
       </c>
       <c r="C1167" t="n">
-        <v>64771</v>
+        <v>68180</v>
       </c>
     </row>
     <row r="1168">
@@ -13283,7 +13283,7 @@
         <v>1324</v>
       </c>
       <c r="C1168" t="n">
-        <v>241813</v>
+        <v>254540</v>
       </c>
     </row>
     <row r="1169">
@@ -13294,7 +13294,7 @@
         <v>2323</v>
       </c>
       <c r="C1169" t="n">
-        <v>59318</v>
+        <v>62440</v>
       </c>
     </row>
     <row r="1170">
@@ -13305,7 +13305,7 @@
         <v>2647</v>
       </c>
       <c r="C1170" t="n">
-        <v>122550</v>
+        <v>129000</v>
       </c>
     </row>
     <row r="1171">
@@ -13316,7 +13316,7 @@
         <v>559</v>
       </c>
       <c r="C1171" t="n">
-        <v>198151</v>
+        <v>208580</v>
       </c>
     </row>
     <row r="1172">
@@ -13327,7 +13327,7 @@
         <v>2762</v>
       </c>
       <c r="C1172" t="n">
-        <v>70376</v>
+        <v>74080</v>
       </c>
     </row>
     <row r="1173">
@@ -13338,7 +13338,7 @@
         <v>2501</v>
       </c>
       <c r="C1173" t="n">
-        <v>70376</v>
+        <v>74080</v>
       </c>
     </row>
     <row r="1174">
@@ -13349,7 +13349,7 @@
         <v>2562</v>
       </c>
       <c r="C1174" t="n">
-        <v>13661</v>
+        <v>14380</v>
       </c>
     </row>
     <row r="1175">
@@ -13360,7 +13360,7 @@
         <v>429</v>
       </c>
       <c r="C1175" t="n">
-        <v>336813</v>
+        <v>354540</v>
       </c>
     </row>
     <row r="1176">
@@ -13371,7 +13371,7 @@
         <v>58</v>
       </c>
       <c r="C1176" t="n">
-        <v>233681</v>
+        <v>245980</v>
       </c>
     </row>
     <row r="1177">
@@ -13382,7 +13382,7 @@
         <v>2245</v>
       </c>
       <c r="C1177" t="n">
-        <v>208639</v>
+        <v>219620</v>
       </c>
     </row>
     <row r="1178">
@@ -13393,7 +13393,7 @@
         <v>285</v>
       </c>
       <c r="C1178" t="n">
-        <v>467362</v>
+        <v>491960</v>
       </c>
     </row>
     <row r="1179">
@@ -13415,7 +13415,7 @@
         <v>363</v>
       </c>
       <c r="C1180" t="n">
-        <v>259084</v>
+        <v>272720</v>
       </c>
     </row>
     <row r="1181">
@@ -13426,7 +13426,7 @@
         <v>2651</v>
       </c>
       <c r="C1181" t="n">
-        <v>146053</v>
+        <v>153740</v>
       </c>
     </row>
     <row r="1182">
@@ -13437,7 +13437,7 @@
         <v>2142</v>
       </c>
       <c r="C1182" t="n">
-        <v>46094</v>
+        <v>48520</v>
       </c>
     </row>
     <row r="1183">
@@ -13448,7 +13448,7 @@
         <v>2258</v>
       </c>
       <c r="C1183" t="n">
-        <v>69090.92</v>
+        <v>72727.28</v>
       </c>
     </row>
     <row r="1184">
@@ -13459,7 +13459,7 @@
         <v>2772</v>
       </c>
       <c r="C1184" t="n">
-        <v>51818.19</v>
+        <v>54545.46</v>
       </c>
     </row>
     <row r="1185">
@@ -13470,7 +13470,7 @@
         <v>2346</v>
       </c>
       <c r="C1185" t="n">
-        <v>95000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1186">
@@ -13481,7 +13481,7 @@
         <v>2442</v>
       </c>
       <c r="C1186" t="n">
-        <v>69084</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1187">
@@ -13492,7 +13492,7 @@
         <v>772</v>
       </c>
       <c r="C1187" t="n">
-        <v>285000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="1188">
@@ -13503,7 +13503,7 @@
         <v>2684</v>
       </c>
       <c r="C1188" t="n">
-        <v>82042</v>
+        <v>86360</v>
       </c>
     </row>
     <row r="1189">
@@ -13514,7 +13514,7 @@
         <v>2765</v>
       </c>
       <c r="C1189" t="n">
-        <v>77710</v>
+        <v>81800</v>
       </c>
     </row>
     <row r="1190">
@@ -13525,7 +13525,7 @@
         <v>2567</v>
       </c>
       <c r="C1190" t="n">
-        <v>142538</v>
+        <v>150040</v>
       </c>
     </row>
     <row r="1191">
@@ -13536,7 +13536,7 @@
         <v>2178</v>
       </c>
       <c r="C1191" t="n">
-        <v>241813</v>
+        <v>254540</v>
       </c>
     </row>
     <row r="1192">
@@ -13547,7 +13547,7 @@
         <v>2827</v>
       </c>
       <c r="C1192" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1193">
@@ -13558,7 +13558,7 @@
         <v>2510</v>
       </c>
       <c r="C1193" t="n">
-        <v>479522</v>
+        <v>504760</v>
       </c>
     </row>
     <row r="1194">
@@ -13569,7 +13569,7 @@
         <v>2392</v>
       </c>
       <c r="C1194" t="n">
-        <v>143849</v>
+        <v>151420</v>
       </c>
     </row>
     <row r="1195">
@@ -13580,7 +13580,7 @@
         <v>415</v>
       </c>
       <c r="C1195" t="n">
-        <v>491834</v>
+        <v>517720</v>
       </c>
     </row>
     <row r="1196">
@@ -13591,7 +13591,7 @@
         <v>2107</v>
       </c>
       <c r="C1196" t="n">
-        <v>253973</v>
+        <v>267340</v>
       </c>
     </row>
     <row r="1197">
@@ -13602,7 +13602,7 @@
         <v>2211</v>
       </c>
       <c r="C1197" t="n">
-        <v>210558</v>
+        <v>221640</v>
       </c>
     </row>
     <row r="1198">
@@ -13613,7 +13613,7 @@
         <v>2682</v>
       </c>
       <c r="C1198" t="n">
-        <v>129523</v>
+        <v>136340</v>
       </c>
     </row>
     <row r="1199">
@@ -13646,7 +13646,7 @@
         <v>2755</v>
       </c>
       <c r="C1201" t="n">
-        <v>51813</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1202">
@@ -13657,7 +13657,7 @@
         <v>941</v>
       </c>
       <c r="C1202" t="n">
-        <v>307342.7</v>
+        <v>323518.63</v>
       </c>
     </row>
     <row r="1203">
@@ -13668,7 +13668,7 @@
         <v>2734</v>
       </c>
       <c r="C1203" t="n">
-        <v>47557</v>
+        <v>50060</v>
       </c>
     </row>
     <row r="1204">
@@ -13690,7 +13690,7 @@
         <v>1289</v>
       </c>
       <c r="C1205" t="n">
-        <v>215897</v>
+        <v>227260</v>
       </c>
     </row>
     <row r="1206">
@@ -13701,7 +13701,7 @@
         <v>2801</v>
       </c>
       <c r="C1206" t="n">
-        <v>69084</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1207">
@@ -13712,7 +13712,7 @@
         <v>2810</v>
       </c>
       <c r="C1207" t="n">
-        <v>116584</v>
+        <v>122720</v>
       </c>
     </row>
     <row r="1208">
@@ -13723,7 +13723,7 @@
         <v>767</v>
       </c>
       <c r="C1208" t="n">
-        <v>155439</v>
+        <v>163620</v>
       </c>
     </row>
     <row r="1209">
@@ -13734,7 +13734,7 @@
         <v>2687</v>
       </c>
       <c r="C1209" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1210">
@@ -13745,7 +13745,7 @@
         <v>2686</v>
       </c>
       <c r="C1210" t="n">
-        <v>112271</v>
+        <v>118180</v>
       </c>
     </row>
     <row r="1211">
@@ -13756,7 +13756,7 @@
         <v>2730</v>
       </c>
       <c r="C1211" t="n">
-        <v>77710</v>
+        <v>81800</v>
       </c>
     </row>
     <row r="1212">
@@ -13767,7 +13767,7 @@
         <v>2580</v>
       </c>
       <c r="C1212" t="n">
-        <v>28975</v>
+        <v>30500</v>
       </c>
     </row>
     <row r="1213">
@@ -13778,7 +13778,7 @@
         <v>2472</v>
       </c>
       <c r="C1213" t="n">
-        <v>45722.65</v>
+        <v>48129.1</v>
       </c>
     </row>
     <row r="1214">
@@ -13789,7 +13789,7 @@
         <v>2631</v>
       </c>
       <c r="C1214" t="n">
-        <v>21186.73</v>
+        <v>22301.82</v>
       </c>
     </row>
     <row r="1215">
@@ -13800,7 +13800,7 @@
         <v>1642</v>
       </c>
       <c r="C1215" t="n">
-        <v>228855</v>
+        <v>240900</v>
       </c>
     </row>
     <row r="1216">
@@ -13811,7 +13811,7 @@
         <v>2613</v>
       </c>
       <c r="C1216" t="n">
-        <v>154755</v>
+        <v>162900</v>
       </c>
     </row>
     <row r="1217">
@@ -13822,7 +13822,7 @@
         <v>1020</v>
       </c>
       <c r="C1217" t="n">
-        <v>77710</v>
+        <v>81800</v>
       </c>
     </row>
     <row r="1218">
@@ -13833,7 +13833,7 @@
         <v>2785</v>
       </c>
       <c r="C1218" t="n">
-        <v>35929</v>
+        <v>37820</v>
       </c>
     </row>
     <row r="1219">
@@ -13844,7 +13844,7 @@
         <v>1327</v>
       </c>
       <c r="C1219" t="n">
-        <v>51813</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1220">
@@ -13855,7 +13855,7 @@
         <v>749</v>
       </c>
       <c r="C1220" t="n">
-        <v>70376</v>
+        <v>74080</v>
       </c>
     </row>
     <row r="1221">
@@ -13866,7 +13866,7 @@
         <v>1983</v>
       </c>
       <c r="C1221" t="n">
-        <v>467362</v>
+        <v>491960</v>
       </c>
     </row>
     <row r="1222">
@@ -13877,7 +13877,7 @@
         <v>1993</v>
       </c>
       <c r="C1222" t="n">
-        <v>300447</v>
+        <v>316260</v>
       </c>
     </row>
     <row r="1223">
@@ -13888,7 +13888,7 @@
         <v>2767</v>
       </c>
       <c r="C1223" t="n">
-        <v>166611</v>
+        <v>175380</v>
       </c>
     </row>
     <row r="1224">
@@ -13910,7 +13910,7 @@
         <v>1102</v>
       </c>
       <c r="C1225" t="n">
-        <v>208639</v>
+        <v>219620</v>
       </c>
     </row>
     <row r="1226">
@@ -13921,7 +13921,7 @@
         <v>626</v>
       </c>
       <c r="C1226" t="n">
-        <v>1471908.42</v>
+        <v>1549377.28</v>
       </c>
     </row>
     <row r="1227">
@@ -13932,7 +13932,7 @@
         <v>1465</v>
       </c>
       <c r="C1227" t="n">
-        <v>310726</v>
+        <v>327080</v>
       </c>
     </row>
     <row r="1228">
@@ -13943,7 +13943,7 @@
         <v>2758</v>
       </c>
       <c r="C1228" t="n">
-        <v>51818.19</v>
+        <v>54545.46</v>
       </c>
     </row>
     <row r="1229">
@@ -13954,7 +13954,7 @@
         <v>2742</v>
       </c>
       <c r="C1229" t="n">
-        <v>51818.19</v>
+        <v>54545.46</v>
       </c>
     </row>
     <row r="1230">
@@ -13976,7 +13976,7 @@
         <v>1873</v>
       </c>
       <c r="C1231" t="n">
-        <v>276355</v>
+        <v>290900</v>
       </c>
     </row>
     <row r="1232">
@@ -13987,7 +13987,7 @@
         <v>2163</v>
       </c>
       <c r="C1232" t="n">
-        <v>129542</v>
+        <v>136360</v>
       </c>
     </row>
     <row r="1233">
@@ -13998,7 +13998,7 @@
         <v>2394</v>
       </c>
       <c r="C1233" t="n">
-        <v>133038</v>
+        <v>140040</v>
       </c>
     </row>
     <row r="1234">
@@ -14009,7 +14009,7 @@
         <v>33</v>
       </c>
       <c r="C1234" t="n">
-        <v>335084</v>
+        <v>352720</v>
       </c>
     </row>
     <row r="1235">
@@ -14020,7 +14020,7 @@
         <v>2421</v>
       </c>
       <c r="C1235" t="n">
-        <v>56126</v>
+        <v>59080</v>
       </c>
     </row>
     <row r="1236">
@@ -14031,7 +14031,7 @@
         <v>2663</v>
       </c>
       <c r="C1236" t="n">
-        <v>237500</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="1237">
@@ -14042,7 +14042,7 @@
         <v>2413</v>
       </c>
       <c r="C1237" t="n">
-        <v>104538</v>
+        <v>110040</v>
       </c>
     </row>
     <row r="1238">
@@ -14053,7 +14053,7 @@
         <v>351</v>
       </c>
       <c r="C1238" t="n">
-        <v>158897</v>
+        <v>167260</v>
       </c>
     </row>
     <row r="1239">
@@ -14064,7 +14064,7 @@
         <v>1298</v>
       </c>
       <c r="C1239" t="n">
-        <v>1099397</v>
+        <v>1157260</v>
       </c>
     </row>
     <row r="1240">
@@ -14075,7 +14075,7 @@
         <v>2491</v>
       </c>
       <c r="C1240" t="n">
-        <v>88844</v>
+        <v>93520</v>
       </c>
     </row>
     <row r="1241">
@@ -14086,7 +14086,7 @@
         <v>2571</v>
       </c>
       <c r="C1241" t="n">
-        <v>125457</v>
+        <v>132060</v>
       </c>
     </row>
     <row r="1242">
@@ -14097,7 +14097,7 @@
         <v>2507</v>
       </c>
       <c r="C1242" t="n">
-        <v>76228</v>
+        <v>80240</v>
       </c>
     </row>
     <row r="1243">
@@ -14108,7 +14108,7 @@
         <v>2799</v>
       </c>
       <c r="C1243" t="n">
-        <v>98116</v>
+        <v>103280</v>
       </c>
     </row>
     <row r="1244">
@@ -14130,7 +14130,7 @@
         <v>2582</v>
       </c>
       <c r="C1245" t="n">
-        <v>74746</v>
+        <v>78680</v>
       </c>
     </row>
     <row r="1246">
@@ -14141,7 +14141,7 @@
         <v>2637</v>
       </c>
       <c r="C1246" t="n">
-        <v>54359</v>
+        <v>57220</v>
       </c>
     </row>
     <row r="1247">
@@ -14152,7 +14152,7 @@
         <v>630</v>
       </c>
       <c r="C1247" t="n">
-        <v>129276</v>
+        <v>136080</v>
       </c>
     </row>
     <row r="1248">
@@ -14163,7 +14163,7 @@
         <v>525</v>
       </c>
       <c r="C1248" t="n">
-        <v>194313</v>
+        <v>204540</v>
       </c>
     </row>
     <row r="1249">
@@ -14174,7 +14174,7 @@
         <v>2727</v>
       </c>
       <c r="C1249" t="n">
-        <v>34960</v>
+        <v>36800</v>
       </c>
     </row>
     <row r="1250">
@@ -14185,7 +14185,7 @@
         <v>2707</v>
       </c>
       <c r="C1250" t="n">
-        <v>27664</v>
+        <v>29120</v>
       </c>
     </row>
     <row r="1251">
@@ -14196,7 +14196,7 @@
         <v>2834</v>
       </c>
       <c r="C1251" t="n">
-        <v>14291.46</v>
+        <v>15043.64</v>
       </c>
     </row>
     <row r="1252">
@@ -14207,7 +14207,7 @@
         <v>2773</v>
       </c>
       <c r="C1252" t="n">
-        <v>69688.57000000001</v>
+        <v>73356.38</v>
       </c>
     </row>
     <row r="1253">
@@ -14218,7 +14218,7 @@
         <v>2341</v>
       </c>
       <c r="C1253" t="n">
-        <v>122550</v>
+        <v>129000</v>
       </c>
     </row>
     <row r="1254">
@@ -14229,7 +14229,7 @@
         <v>1374</v>
       </c>
       <c r="C1254" t="n">
-        <v>155439</v>
+        <v>163620</v>
       </c>
     </row>
     <row r="1255">
@@ -14240,7 +14240,7 @@
         <v>793</v>
       </c>
       <c r="C1255" t="n">
-        <v>35929</v>
+        <v>37820</v>
       </c>
     </row>
     <row r="1256">
@@ -14251,7 +14251,7 @@
         <v>794</v>
       </c>
       <c r="C1256" t="n">
-        <v>35929</v>
+        <v>37820</v>
       </c>
     </row>
     <row r="1257">
@@ -14262,7 +14262,7 @@
         <v>1834</v>
       </c>
       <c r="C1257" t="n">
-        <v>101042</v>
+        <v>106360</v>
       </c>
     </row>
     <row r="1258">
@@ -14273,7 +14273,7 @@
         <v>802</v>
       </c>
       <c r="C1258" t="n">
-        <v>64771</v>
+        <v>68180</v>
       </c>
     </row>
     <row r="1259">
@@ -14284,7 +14284,7 @@
         <v>1344</v>
       </c>
       <c r="C1259" t="n">
-        <v>129542</v>
+        <v>136360</v>
       </c>
     </row>
     <row r="1260">
@@ -14295,7 +14295,7 @@
         <v>1881</v>
       </c>
       <c r="C1260" t="n">
-        <v>59318</v>
+        <v>62440</v>
       </c>
     </row>
     <row r="1261">
@@ -14306,7 +14306,7 @@
         <v>2365</v>
       </c>
       <c r="C1261" t="n">
-        <v>68799</v>
+        <v>72420</v>
       </c>
     </row>
     <row r="1262">
@@ -14317,7 +14317,7 @@
         <v>2411</v>
       </c>
       <c r="C1262" t="n">
-        <v>122550</v>
+        <v>129000</v>
       </c>
     </row>
     <row r="1263">
@@ -14328,7 +14328,7 @@
         <v>2363</v>
       </c>
       <c r="C1263" t="n">
-        <v>129542</v>
+        <v>136360</v>
       </c>
     </row>
     <row r="1264">
@@ -14339,7 +14339,7 @@
         <v>2124</v>
       </c>
       <c r="C1264" t="n">
-        <v>302271</v>
+        <v>318180</v>
       </c>
     </row>
     <row r="1265">
@@ -14350,7 +14350,7 @@
         <v>1937</v>
       </c>
       <c r="C1265" t="n">
-        <v>220210</v>
+        <v>231800</v>
       </c>
     </row>
     <row r="1266">
@@ -14361,7 +14361,7 @@
         <v>2709</v>
       </c>
       <c r="C1266" t="n">
-        <v>155439</v>
+        <v>163620</v>
       </c>
     </row>
     <row r="1267">
@@ -14372,7 +14372,7 @@
         <v>2558</v>
       </c>
       <c r="C1267" t="n">
-        <v>25954</v>
+        <v>27320</v>
       </c>
     </row>
     <row r="1268">
@@ -14383,7 +14383,7 @@
         <v>663</v>
       </c>
       <c r="C1268" t="n">
-        <v>220210</v>
+        <v>231800</v>
       </c>
     </row>
     <row r="1269">
@@ -14394,7 +14394,7 @@
         <v>40</v>
       </c>
       <c r="C1269" t="n">
-        <v>190000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="1270">
@@ -14405,7 +14405,7 @@
         <v>2833</v>
       </c>
       <c r="C1270" t="n">
-        <v>60454.57</v>
+        <v>63636.38</v>
       </c>
     </row>
     <row r="1271">
@@ -14416,7 +14416,7 @@
         <v>1756</v>
       </c>
       <c r="C1271" t="n">
-        <v>376979</v>
+        <v>396820</v>
       </c>
     </row>
     <row r="1272">
@@ -14427,7 +14427,7 @@
         <v>1116</v>
       </c>
       <c r="C1272" t="n">
-        <v>219051</v>
+        <v>230580</v>
       </c>
     </row>
     <row r="1273">
@@ -14438,7 +14438,7 @@
         <v>636</v>
       </c>
       <c r="C1273" t="n">
-        <v>215897</v>
+        <v>227260</v>
       </c>
     </row>
     <row r="1274">
@@ -14449,7 +14449,7 @@
         <v>1800</v>
       </c>
       <c r="C1274" t="n">
-        <v>24168</v>
+        <v>25440</v>
       </c>
     </row>
     <row r="1275">
@@ -14460,7 +14460,7 @@
         <v>2815</v>
       </c>
       <c r="C1275" t="n">
-        <v>51818.19</v>
+        <v>54545.46</v>
       </c>
     </row>
     <row r="1276">
@@ -14471,7 +14471,7 @@
         <v>1658</v>
       </c>
       <c r="C1276" t="n">
-        <v>114000</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="1277">
@@ -14482,7 +14482,7 @@
         <v>2635</v>
       </c>
       <c r="C1277" t="n">
-        <v>112271</v>
+        <v>118180</v>
       </c>
     </row>
     <row r="1278">
@@ -14493,7 +14493,7 @@
         <v>2402</v>
       </c>
       <c r="C1278" t="n">
-        <v>563084</v>
+        <v>592720</v>
       </c>
     </row>
     <row r="1279">
@@ -14504,7 +14504,7 @@
         <v>452</v>
       </c>
       <c r="C1279" t="n">
-        <v>233168</v>
+        <v>245440</v>
       </c>
     </row>
     <row r="1280">
@@ -14515,7 +14515,7 @@
         <v>2085</v>
       </c>
       <c r="C1280" t="n">
-        <v>114038</v>
+        <v>120040</v>
       </c>
     </row>
     <row r="1281">
@@ -14526,7 +14526,7 @@
         <v>2568</v>
       </c>
       <c r="C1281" t="n">
-        <v>176548</v>
+        <v>185840</v>
       </c>
     </row>
     <row r="1282">
@@ -14537,7 +14537,7 @@
         <v>1906</v>
       </c>
       <c r="C1282" t="n">
-        <v>100206</v>
+        <v>105480</v>
       </c>
     </row>
     <row r="1283">
@@ -14548,7 +14548,7 @@
         <v>2821</v>
       </c>
       <c r="C1283" t="n">
-        <v>87134</v>
+        <v>91720</v>
       </c>
     </row>
     <row r="1284">
@@ -14559,7 +14559,7 @@
         <v>2698</v>
       </c>
       <c r="C1284" t="n">
-        <v>106799</v>
+        <v>112420</v>
       </c>
     </row>
     <row r="1285">
@@ -14570,7 +14570,7 @@
         <v>2118</v>
       </c>
       <c r="C1285" t="n">
-        <v>204820</v>
+        <v>215600</v>
       </c>
     </row>
     <row r="1286">
@@ -14581,7 +14581,7 @@
         <v>2383</v>
       </c>
       <c r="C1286" t="n">
-        <v>119586</v>
+        <v>125880</v>
       </c>
     </row>
     <row r="1287">
@@ -14592,7 +14592,7 @@
         <v>2813</v>
       </c>
       <c r="C1287" t="n">
-        <v>54359</v>
+        <v>57220</v>
       </c>
     </row>
     <row r="1288">
@@ -14603,7 +14603,7 @@
         <v>925</v>
       </c>
       <c r="C1288" t="n">
-        <v>67944</v>
+        <v>71520</v>
       </c>
     </row>
     <row r="1289">
@@ -14614,7 +14614,7 @@
         <v>2689</v>
       </c>
       <c r="C1289" t="n">
-        <v>54359</v>
+        <v>57220</v>
       </c>
     </row>
     <row r="1290">
@@ -14625,7 +14625,7 @@
         <v>2716</v>
       </c>
       <c r="C1290" t="n">
-        <v>74746</v>
+        <v>78680</v>
       </c>
     </row>
     <row r="1291">
@@ -14636,7 +14636,7 @@
         <v>2831</v>
       </c>
       <c r="C1291" t="n">
-        <v>51813</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1292">
@@ -14647,7 +14647,7 @@
         <v>2045</v>
       </c>
       <c r="C1292" t="n">
-        <v>290575.33</v>
+        <v>305868.76</v>
       </c>
     </row>
     <row r="1293">
@@ -14658,7 +14658,7 @@
         <v>580</v>
       </c>
       <c r="C1293" t="n">
-        <v>116584</v>
+        <v>122720</v>
       </c>
     </row>
     <row r="1294">
@@ -14669,7 +14669,7 @@
         <v>438</v>
       </c>
       <c r="C1294" t="n">
-        <v>133855</v>
+        <v>140900</v>
       </c>
     </row>
     <row r="1295">
@@ -14680,7 +14680,7 @@
         <v>1539</v>
       </c>
       <c r="C1295" t="n">
-        <v>146813</v>
+        <v>154540</v>
       </c>
     </row>
     <row r="1296">
@@ -14691,7 +14691,7 @@
         <v>2817</v>
       </c>
       <c r="C1296" t="n">
-        <v>51813</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1297">
@@ -14702,7 +14702,7 @@
         <v>2816</v>
       </c>
       <c r="C1297" t="n">
-        <v>112271</v>
+        <v>118180</v>
       </c>
     </row>
     <row r="1298">
@@ -14713,7 +14713,7 @@
         <v>2146</v>
       </c>
       <c r="C1298" t="n">
-        <v>174154</v>
+        <v>183320</v>
       </c>
     </row>
     <row r="1299">
@@ -14724,7 +14724,7 @@
         <v>2276</v>
       </c>
       <c r="C1299" t="n">
-        <v>193496</v>
+        <v>203680</v>
       </c>
     </row>
     <row r="1300">
@@ -14735,7 +14735,7 @@
         <v>1381</v>
       </c>
       <c r="C1300" t="n">
-        <v>254771</v>
+        <v>268180</v>
       </c>
     </row>
     <row r="1301">
@@ -14746,7 +14746,7 @@
         <v>2081</v>
       </c>
       <c r="C1301" t="n">
-        <v>129542</v>
+        <v>136360</v>
       </c>
     </row>
     <row r="1302">
@@ -14757,7 +14757,7 @@
         <v>14</v>
       </c>
       <c r="C1302" t="n">
-        <v>375668</v>
+        <v>395440</v>
       </c>
     </row>
     <row r="1303">
@@ -14768,7 +14768,7 @@
         <v>766</v>
       </c>
       <c r="C1303" t="n">
-        <v>59318</v>
+        <v>62440</v>
       </c>
     </row>
     <row r="1304">
@@ -14779,7 +14779,7 @@
         <v>2547</v>
       </c>
       <c r="C1304" t="n">
-        <v>35511</v>
+        <v>37380</v>
       </c>
     </row>
     <row r="1305">
@@ -14790,7 +14790,7 @@
         <v>2552</v>
       </c>
       <c r="C1305" t="n">
-        <v>25536</v>
+        <v>26880</v>
       </c>
     </row>
     <row r="1306">
@@ -14801,7 +14801,7 @@
         <v>131</v>
       </c>
       <c r="C1306" t="n">
-        <v>353210</v>
+        <v>371800</v>
       </c>
     </row>
     <row r="1307">
@@ -14812,7 +14812,7 @@
         <v>2250</v>
       </c>
       <c r="C1307" t="n">
-        <v>285779</v>
+        <v>300820</v>
       </c>
     </row>
     <row r="1308">
@@ -14823,7 +14823,7 @@
         <v>89</v>
       </c>
       <c r="C1308" t="n">
-        <v>292068</v>
+        <v>307440</v>
       </c>
     </row>
     <row r="1309">
@@ -14834,7 +14834,7 @@
         <v>2141</v>
       </c>
       <c r="C1309" t="n">
-        <v>27322</v>
+        <v>28760</v>
       </c>
     </row>
     <row r="1310">
@@ -14845,7 +14845,7 @@
         <v>2798</v>
       </c>
       <c r="C1310" t="n">
-        <v>51818.19</v>
+        <v>54545.46</v>
       </c>
     </row>
     <row r="1311">
@@ -14856,7 +14856,7 @@
         <v>2797</v>
       </c>
       <c r="C1311" t="n">
-        <v>51818.19</v>
+        <v>54545.46</v>
       </c>
     </row>
     <row r="1312">
@@ -14867,7 +14867,7 @@
         <v>2266</v>
       </c>
       <c r="C1312" t="n">
-        <v>69090.92</v>
+        <v>72727.28</v>
       </c>
     </row>
     <row r="1313">
@@ -14878,7 +14878,7 @@
         <v>1499</v>
       </c>
       <c r="C1313" t="n">
-        <v>120897</v>
+        <v>127260</v>
       </c>
     </row>
     <row r="1314">
@@ -14889,7 +14889,7 @@
         <v>2496</v>
       </c>
       <c r="C1314" t="n">
-        <v>138168</v>
+        <v>145440</v>
       </c>
     </row>
     <row r="1315">
@@ -14900,7 +14900,7 @@
         <v>949</v>
       </c>
       <c r="C1315" t="n">
-        <v>84759</v>
+        <v>89220</v>
       </c>
     </row>
     <row r="1316">
@@ -14911,7 +14911,7 @@
         <v>1853</v>
       </c>
       <c r="C1316" t="n">
-        <v>103626</v>
+        <v>109080</v>
       </c>
     </row>
     <row r="1317">
@@ -14922,7 +14922,7 @@
         <v>854</v>
       </c>
       <c r="C1317" t="n">
-        <v>95000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1318">
@@ -14933,7 +14933,7 @@
         <v>2674</v>
       </c>
       <c r="C1318" t="n">
-        <v>224542</v>
+        <v>236360</v>
       </c>
     </row>
     <row r="1319">
@@ -14944,7 +14944,7 @@
         <v>2803</v>
       </c>
       <c r="C1319" t="n">
-        <v>103626</v>
+        <v>109080</v>
       </c>
     </row>
     <row r="1320">
@@ -14955,7 +14955,7 @@
         <v>2599</v>
       </c>
       <c r="C1320" t="n">
-        <v>164084</v>
+        <v>172720</v>
       </c>
     </row>
     <row r="1321">
@@ -14966,7 +14966,7 @@
         <v>783</v>
       </c>
       <c r="C1321" t="n">
-        <v>44897</v>
+        <v>47260</v>
       </c>
     </row>
     <row r="1322">
@@ -14977,7 +14977,7 @@
         <v>27</v>
       </c>
       <c r="C1322" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1323">
@@ -14988,7 +14988,7 @@
         <v>531</v>
       </c>
       <c r="C1323" t="n">
-        <v>302271</v>
+        <v>318180</v>
       </c>
     </row>
     <row r="1324">
@@ -14999,7 +14999,7 @@
         <v>1308</v>
       </c>
       <c r="C1324" t="n">
-        <v>139498</v>
+        <v>146840</v>
       </c>
     </row>
     <row r="1325">
@@ -15010,7 +15010,7 @@
         <v>2792</v>
       </c>
       <c r="C1325" t="n">
-        <v>100605</v>
+        <v>105900</v>
       </c>
     </row>
     <row r="1326">
@@ -15032,7 +15032,7 @@
         <v>2823</v>
       </c>
       <c r="C1327" t="n">
-        <v>80750</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="1328">
@@ -15043,7 +15043,7 @@
         <v>2584</v>
       </c>
       <c r="C1328" t="n">
-        <v>54359</v>
+        <v>57220</v>
       </c>
     </row>
     <row r="1329">
@@ -15054,7 +15054,7 @@
         <v>945</v>
       </c>
       <c r="C1329" t="n">
-        <v>244682</v>
+        <v>257560</v>
       </c>
     </row>
     <row r="1330">
@@ -15065,7 +15065,7 @@
         <v>2660</v>
       </c>
       <c r="C1330" t="n">
-        <v>267710</v>
+        <v>281800</v>
       </c>
     </row>
     <row r="1331">
@@ -15076,7 +15076,7 @@
         <v>1317</v>
       </c>
       <c r="C1331" t="n">
-        <v>259084</v>
+        <v>272720</v>
       </c>
     </row>
     <row r="1332">
@@ -15087,7 +15087,7 @@
         <v>2790</v>
       </c>
       <c r="C1332" t="n">
-        <v>55005</v>
+        <v>57900</v>
       </c>
     </row>
     <row r="1333">
@@ -15098,7 +15098,7 @@
         <v>2711</v>
       </c>
       <c r="C1333" t="n">
-        <v>74866.92</v>
+        <v>78807.28</v>
       </c>
     </row>
     <row r="1334">
@@ -15109,7 +15109,7 @@
         <v>2607</v>
       </c>
       <c r="C1334" t="n">
-        <v>42908.92</v>
+        <v>45167.28</v>
       </c>
     </row>
     <row r="1335">
@@ -15120,7 +15120,7 @@
         <v>2667</v>
       </c>
       <c r="C1335" t="n">
-        <v>39468.19</v>
+        <v>41545.46</v>
       </c>
     </row>
     <row r="1336">
@@ -15131,7 +15131,7 @@
         <v>2706</v>
       </c>
       <c r="C1336" t="n">
-        <v>19027.65</v>
+        <v>20029.1</v>
       </c>
     </row>
     <row r="1337">
@@ -15142,7 +15142,7 @@
         <v>2657</v>
       </c>
       <c r="C1337" t="n">
-        <v>68396.57000000001</v>
+        <v>71996.38</v>
       </c>
     </row>
     <row r="1338">
@@ -15153,7 +15153,7 @@
         <v>1278</v>
       </c>
       <c r="C1338" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1339">
@@ -15164,7 +15164,7 @@
         <v>2745</v>
       </c>
       <c r="C1339" t="n">
-        <v>95000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1340">
@@ -15175,7 +15175,7 @@
         <v>2753</v>
       </c>
       <c r="C1340" t="n">
-        <v>64771</v>
+        <v>68180</v>
       </c>
     </row>
     <row r="1341">
@@ -15186,7 +15186,7 @@
         <v>2183</v>
       </c>
       <c r="C1341" t="n">
-        <v>316046</v>
+        <v>332680</v>
       </c>
     </row>
     <row r="1342">
@@ -15197,7 +15197,7 @@
         <v>1340</v>
       </c>
       <c r="C1342" t="n">
-        <v>125210</v>
+        <v>131800</v>
       </c>
     </row>
     <row r="1343">
@@ -15208,7 +15208,7 @@
         <v>2583</v>
       </c>
       <c r="C1343" t="n">
-        <v>35929</v>
+        <v>37820</v>
       </c>
     </row>
     <row r="1344">
@@ -15219,7 +15219,7 @@
         <v>2090</v>
       </c>
       <c r="C1344" t="n">
-        <v>35929</v>
+        <v>37820</v>
       </c>
     </row>
     <row r="1345">
@@ -15230,7 +15230,7 @@
         <v>1277</v>
       </c>
       <c r="C1345" t="n">
-        <v>190000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="1346">
@@ -15241,7 +15241,7 @@
         <v>1501</v>
       </c>
       <c r="C1346" t="n">
-        <v>82042</v>
+        <v>86360</v>
       </c>
     </row>
     <row r="1347">
@@ -15252,7 +15252,7 @@
         <v>703</v>
       </c>
       <c r="C1347" t="n">
-        <v>215897</v>
+        <v>227260</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:01:43
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -11292,7 +11292,7 @@
         <v>931</v>
       </c>
       <c r="C987" t="n">
-        <v>85840</v>
+        <v>90132</v>
       </c>
     </row>
     <row r="988">
@@ -11303,7 +11303,7 @@
         <v>947</v>
       </c>
       <c r="C988" t="n">
-        <v>395020</v>
+        <v>414771</v>
       </c>
     </row>
     <row r="989">
@@ -11314,7 +11314,7 @@
         <v>1956</v>
       </c>
       <c r="C989" t="n">
-        <v>229520</v>
+        <v>240996</v>
       </c>
     </row>
     <row r="990">
@@ -11325,7 +11325,7 @@
         <v>2824</v>
       </c>
       <c r="C990" t="n">
-        <v>100000</v>
+        <v>105000</v>
       </c>
     </row>
     <row r="991">
@@ -11336,7 +11336,7 @@
         <v>2787</v>
       </c>
       <c r="C991" t="n">
-        <v>118180</v>
+        <v>124089</v>
       </c>
     </row>
     <row r="992">
@@ -11347,7 +11347,7 @@
         <v>2830</v>
       </c>
       <c r="C992" t="n">
-        <v>81800</v>
+        <v>85890</v>
       </c>
     </row>
     <row r="993">
@@ -11358,7 +11358,7 @@
         <v>1254</v>
       </c>
       <c r="C993" t="n">
-        <v>176541.82</v>
+        <v>185368.91</v>
       </c>
     </row>
     <row r="994">
@@ -11369,7 +11369,7 @@
         <v>816</v>
       </c>
       <c r="C994" t="n">
-        <v>243500</v>
+        <v>255675</v>
       </c>
     </row>
     <row r="995">
@@ -11380,7 +11380,7 @@
         <v>2671</v>
       </c>
       <c r="C995" t="n">
-        <v>72720</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="996">
@@ -11391,7 +11391,7 @@
         <v>2705</v>
       </c>
       <c r="C996" t="n">
-        <v>162900</v>
+        <v>171045</v>
       </c>
     </row>
     <row r="997">
@@ -11402,7 +11402,7 @@
         <v>2333</v>
       </c>
       <c r="C997" t="n">
-        <v>140320</v>
+        <v>147336</v>
       </c>
     </row>
     <row r="998">
@@ -11413,7 +11413,7 @@
         <v>2440</v>
       </c>
       <c r="C998" t="n">
-        <v>81800</v>
+        <v>85890</v>
       </c>
     </row>
     <row r="999">
@@ -11424,7 +11424,7 @@
         <v>2448</v>
       </c>
       <c r="C999" t="n">
-        <v>18180</v>
+        <v>19089</v>
       </c>
     </row>
     <row r="1000">
@@ -11435,7 +11435,7 @@
         <v>2310</v>
       </c>
       <c r="C1000" t="n">
-        <v>62440</v>
+        <v>65562</v>
       </c>
     </row>
     <row r="1001">
@@ -11446,7 +11446,7 @@
         <v>2809</v>
       </c>
       <c r="C1001" t="n">
-        <v>62440</v>
+        <v>65562</v>
       </c>
     </row>
     <row r="1002">
@@ -11457,7 +11457,7 @@
         <v>2548</v>
       </c>
       <c r="C1002" t="n">
-        <v>53200</v>
+        <v>55860</v>
       </c>
     </row>
     <row r="1003">
@@ -11468,7 +11468,7 @@
         <v>451</v>
       </c>
       <c r="C1003" t="n">
-        <v>218180</v>
+        <v>229089</v>
       </c>
     </row>
     <row r="1004">
@@ -11479,7 +11479,7 @@
         <v>933</v>
       </c>
       <c r="C1004" t="n">
-        <v>74080</v>
+        <v>77784</v>
       </c>
     </row>
     <row r="1005">
@@ -11490,7 +11490,7 @@
         <v>2702</v>
       </c>
       <c r="C1005" t="n">
-        <v>74080</v>
+        <v>77784</v>
       </c>
     </row>
     <row r="1006">
@@ -11501,7 +11501,7 @@
         <v>2549</v>
       </c>
       <c r="C1006" t="n">
-        <v>25760</v>
+        <v>27048</v>
       </c>
     </row>
     <row r="1007">
@@ -11512,7 +11512,7 @@
         <v>535</v>
       </c>
       <c r="C1007" t="n">
-        <v>336360</v>
+        <v>353178</v>
       </c>
     </row>
     <row r="1008">
@@ -11523,7 +11523,7 @@
         <v>1117</v>
       </c>
       <c r="C1008" t="n">
-        <v>316260</v>
+        <v>332073</v>
       </c>
     </row>
     <row r="1009">
@@ -11545,7 +11545,7 @@
         <v>530</v>
       </c>
       <c r="C1010" t="n">
-        <v>221880</v>
+        <v>232974</v>
       </c>
     </row>
     <row r="1011">
@@ -11556,7 +11556,7 @@
         <v>358</v>
       </c>
       <c r="C1011" t="n">
-        <v>309080</v>
+        <v>324534</v>
       </c>
     </row>
     <row r="1012">
@@ -11567,7 +11567,7 @@
         <v>2498</v>
       </c>
       <c r="C1012" t="n">
-        <v>50480</v>
+        <v>53004</v>
       </c>
     </row>
     <row r="1013">
@@ -11578,7 +11578,7 @@
         <v>2381</v>
       </c>
       <c r="C1013" t="n">
-        <v>72120</v>
+        <v>75726</v>
       </c>
     </row>
     <row r="1014">
@@ -11589,7 +11589,7 @@
         <v>2695</v>
       </c>
       <c r="C1014" t="n">
-        <v>43380</v>
+        <v>45549</v>
       </c>
     </row>
     <row r="1015">
@@ -11600,7 +11600,7 @@
         <v>2744</v>
       </c>
       <c r="C1015" t="n">
-        <v>54545.46</v>
+        <v>57272.73</v>
       </c>
     </row>
     <row r="1016">
@@ -11611,7 +11611,7 @@
         <v>2750</v>
       </c>
       <c r="C1016" t="n">
-        <v>54540</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1017">
@@ -11622,7 +11622,7 @@
         <v>2131</v>
       </c>
       <c r="C1017" t="n">
-        <v>109080</v>
+        <v>114534</v>
       </c>
     </row>
     <row r="1018">
@@ -11633,7 +11633,7 @@
         <v>818</v>
       </c>
       <c r="C1018" t="n">
-        <v>363620</v>
+        <v>381801</v>
       </c>
     </row>
     <row r="1019">
@@ -11644,7 +11644,7 @@
         <v>2566</v>
       </c>
       <c r="C1019" t="n">
-        <v>72720</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1020">
@@ -11655,7 +11655,7 @@
         <v>132</v>
       </c>
       <c r="C1020" t="n">
-        <v>681800</v>
+        <v>715890</v>
       </c>
     </row>
     <row r="1021">
@@ -11666,7 +11666,7 @@
         <v>2431</v>
       </c>
       <c r="C1021" t="n">
-        <v>167260</v>
+        <v>175623</v>
       </c>
     </row>
     <row r="1022">
@@ -11677,7 +11677,7 @@
         <v>2249</v>
       </c>
       <c r="C1022" t="n">
-        <v>177560</v>
+        <v>186438</v>
       </c>
     </row>
     <row r="1023">
@@ -11688,7 +11688,7 @@
         <v>1585</v>
       </c>
       <c r="C1023" t="n">
-        <v>150040</v>
+        <v>157542</v>
       </c>
     </row>
     <row r="1024">
@@ -11699,7 +11699,7 @@
         <v>2325</v>
       </c>
       <c r="C1024" t="n">
-        <v>145040</v>
+        <v>152292</v>
       </c>
     </row>
     <row r="1025">
@@ -11710,7 +11710,7 @@
         <v>2190</v>
       </c>
       <c r="C1025" t="n">
-        <v>204540</v>
+        <v>214767</v>
       </c>
     </row>
     <row r="1026">
@@ -11721,7 +11721,7 @@
         <v>1466</v>
       </c>
       <c r="C1026" t="n">
-        <v>368180</v>
+        <v>386589</v>
       </c>
     </row>
     <row r="1027">
@@ -11732,7 +11732,7 @@
         <v>2659</v>
       </c>
       <c r="C1027" t="n">
-        <v>111820</v>
+        <v>117411</v>
       </c>
     </row>
     <row r="1028">
@@ -11743,7 +11743,7 @@
         <v>1384</v>
       </c>
       <c r="C1028" t="n">
-        <v>409080</v>
+        <v>429534</v>
       </c>
     </row>
     <row r="1029">
@@ -11754,7 +11754,7 @@
         <v>634</v>
       </c>
       <c r="C1029" t="n">
-        <v>500000</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="1030">
@@ -11765,7 +11765,7 @@
         <v>2804</v>
       </c>
       <c r="C1030" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1031">
@@ -11776,7 +11776,7 @@
         <v>2375</v>
       </c>
       <c r="C1031" t="n">
-        <v>300000</v>
+        <v>315000</v>
       </c>
     </row>
     <row r="1032">
@@ -11787,7 +11787,7 @@
         <v>2601</v>
       </c>
       <c r="C1032" t="n">
-        <v>250000</v>
+        <v>262500</v>
       </c>
     </row>
     <row r="1033">
@@ -11798,7 +11798,7 @@
         <v>952</v>
       </c>
       <c r="C1033" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1034">
@@ -11809,7 +11809,7 @@
         <v>571</v>
       </c>
       <c r="C1034" t="n">
-        <v>578620</v>
+        <v>607551</v>
       </c>
     </row>
     <row r="1035">
@@ -11820,7 +11820,7 @@
         <v>2697</v>
       </c>
       <c r="C1035" t="n">
-        <v>176300</v>
+        <v>185115</v>
       </c>
     </row>
     <row r="1036">
@@ -11831,7 +11831,7 @@
         <v>2678</v>
       </c>
       <c r="C1036" t="n">
-        <v>305020</v>
+        <v>320271</v>
       </c>
     </row>
     <row r="1037">
@@ -11842,7 +11842,7 @@
         <v>2768</v>
       </c>
       <c r="C1037" t="n">
-        <v>319220</v>
+        <v>335181</v>
       </c>
     </row>
     <row r="1038">
@@ -11853,7 +11853,7 @@
         <v>2359</v>
       </c>
       <c r="C1038" t="n">
-        <v>96820</v>
+        <v>101661</v>
       </c>
     </row>
     <row r="1039">
@@ -11864,7 +11864,7 @@
         <v>353</v>
       </c>
       <c r="C1039" t="n">
-        <v>314532.01</v>
+        <v>330258.6</v>
       </c>
     </row>
     <row r="1040">
@@ -11875,7 +11875,7 @@
         <v>2026</v>
       </c>
       <c r="C1040" t="n">
-        <v>260612.23</v>
+        <v>273642.84</v>
       </c>
     </row>
     <row r="1041">
@@ -11897,7 +11897,7 @@
         <v>2345</v>
       </c>
       <c r="C1042" t="n">
-        <v>57220</v>
+        <v>60081</v>
       </c>
     </row>
     <row r="1043">
@@ -11908,7 +11908,7 @@
         <v>2789</v>
       </c>
       <c r="C1043" t="n">
-        <v>154540</v>
+        <v>162267</v>
       </c>
     </row>
     <row r="1044">
@@ -11919,7 +11919,7 @@
         <v>569</v>
       </c>
       <c r="C1044" t="n">
-        <v>2603560</v>
+        <v>2733738</v>
       </c>
     </row>
     <row r="1045">
@@ -11930,7 +11930,7 @@
         <v>2822</v>
       </c>
       <c r="C1045" t="n">
-        <v>122720</v>
+        <v>128856</v>
       </c>
     </row>
     <row r="1046">
@@ -11941,7 +11941,7 @@
         <v>2728</v>
       </c>
       <c r="C1046" t="n">
-        <v>9080</v>
+        <v>9534</v>
       </c>
     </row>
     <row r="1047">
@@ -11952,7 +11952,7 @@
         <v>2488</v>
       </c>
       <c r="C1047" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1048">
@@ -11963,7 +11963,7 @@
         <v>2791</v>
       </c>
       <c r="C1048" t="n">
-        <v>89718.2</v>
+        <v>94204.10000000001</v>
       </c>
     </row>
     <row r="1049">
@@ -11974,7 +11974,7 @@
         <v>2577</v>
       </c>
       <c r="C1049" t="n">
-        <v>81063.73</v>
+        <v>85116.91</v>
       </c>
     </row>
     <row r="1050">
@@ -11985,7 +11985,7 @@
         <v>2069</v>
       </c>
       <c r="C1050" t="n">
-        <v>163620</v>
+        <v>171801</v>
       </c>
     </row>
     <row r="1051">
@@ -11996,7 +11996,7 @@
         <v>2082</v>
       </c>
       <c r="C1051" t="n">
-        <v>151420</v>
+        <v>158991</v>
       </c>
     </row>
     <row r="1052">
@@ -12007,7 +12007,7 @@
         <v>781</v>
       </c>
       <c r="C1052" t="n">
-        <v>118180</v>
+        <v>124089</v>
       </c>
     </row>
     <row r="1053">
@@ -12018,7 +12018,7 @@
         <v>744</v>
       </c>
       <c r="C1053" t="n">
-        <v>37820</v>
+        <v>39711</v>
       </c>
     </row>
     <row r="1054">
@@ -12029,7 +12029,7 @@
         <v>2223</v>
       </c>
       <c r="C1054" t="n">
-        <v>119940</v>
+        <v>125937</v>
       </c>
     </row>
     <row r="1055">
@@ -12040,7 +12040,7 @@
         <v>2452</v>
       </c>
       <c r="C1055" t="n">
-        <v>63620</v>
+        <v>66801</v>
       </c>
     </row>
     <row r="1056">
@@ -12051,7 +12051,7 @@
         <v>970</v>
       </c>
       <c r="C1056" t="n">
-        <v>62440</v>
+        <v>65562</v>
       </c>
     </row>
     <row r="1057">
@@ -12062,7 +12062,7 @@
         <v>2550</v>
       </c>
       <c r="C1057" t="n">
-        <v>55440</v>
+        <v>58212</v>
       </c>
     </row>
     <row r="1058">
@@ -12073,7 +12073,7 @@
         <v>768</v>
       </c>
       <c r="C1058" t="n">
-        <v>118180</v>
+        <v>124089</v>
       </c>
     </row>
     <row r="1059">
@@ -12084,7 +12084,7 @@
         <v>1075</v>
       </c>
       <c r="C1059" t="n">
-        <v>411800</v>
+        <v>432390</v>
       </c>
     </row>
     <row r="1060">
@@ -12095,7 +12095,7 @@
         <v>664</v>
       </c>
       <c r="C1060" t="n">
-        <v>235440</v>
+        <v>247212</v>
       </c>
     </row>
     <row r="1061">
@@ -12106,7 +12106,7 @@
         <v>2555</v>
       </c>
       <c r="C1061" t="n">
-        <v>37740</v>
+        <v>39627</v>
       </c>
     </row>
     <row r="1062">
@@ -12117,7 +12117,7 @@
         <v>2627</v>
       </c>
       <c r="C1062" t="n">
-        <v>22160</v>
+        <v>23268</v>
       </c>
     </row>
     <row r="1063">
@@ -12128,7 +12128,7 @@
         <v>2557</v>
       </c>
       <c r="C1063" t="n">
-        <v>23440</v>
+        <v>24612</v>
       </c>
     </row>
     <row r="1064">
@@ -12139,7 +12139,7 @@
         <v>2551</v>
       </c>
       <c r="C1064" t="n">
-        <v>18620</v>
+        <v>19551</v>
       </c>
     </row>
     <row r="1065">
@@ -12150,7 +12150,7 @@
         <v>2463</v>
       </c>
       <c r="C1065" t="n">
-        <v>291100</v>
+        <v>305655</v>
       </c>
     </row>
     <row r="1066">
@@ -12161,7 +12161,7 @@
         <v>2279</v>
       </c>
       <c r="C1066" t="n">
-        <v>219620</v>
+        <v>230601</v>
       </c>
     </row>
     <row r="1067">
@@ -12172,7 +12172,7 @@
         <v>631</v>
       </c>
       <c r="C1067" t="n">
-        <v>318180</v>
+        <v>334089</v>
       </c>
     </row>
     <row r="1068">
@@ -12183,7 +12183,7 @@
         <v>2251</v>
       </c>
       <c r="C1068" t="n">
-        <v>194840</v>
+        <v>204582</v>
       </c>
     </row>
     <row r="1069">
@@ -12194,7 +12194,7 @@
         <v>1653</v>
       </c>
       <c r="C1069" t="n">
-        <v>295440</v>
+        <v>310212</v>
       </c>
     </row>
     <row r="1070">
@@ -12205,7 +12205,7 @@
         <v>1293</v>
       </c>
       <c r="C1070" t="n">
-        <v>377260</v>
+        <v>396123</v>
       </c>
     </row>
     <row r="1071">
@@ -12216,7 +12216,7 @@
         <v>360</v>
       </c>
       <c r="C1071" t="n">
-        <v>454540</v>
+        <v>477267</v>
       </c>
     </row>
     <row r="1072">
@@ -12227,7 +12227,7 @@
         <v>1063</v>
       </c>
       <c r="C1072" t="n">
-        <v>330500</v>
+        <v>347025</v>
       </c>
     </row>
     <row r="1073">
@@ -12238,7 +12238,7 @@
         <v>2273</v>
       </c>
       <c r="C1073" t="n">
-        <v>192800</v>
+        <v>202440</v>
       </c>
     </row>
     <row r="1074">
@@ -12249,7 +12249,7 @@
         <v>2757</v>
       </c>
       <c r="C1074" t="n">
-        <v>63636.38</v>
+        <v>66818.19</v>
       </c>
     </row>
     <row r="1075">
@@ -12260,7 +12260,7 @@
         <v>2795</v>
       </c>
       <c r="C1075" t="n">
-        <v>54545.46</v>
+        <v>57272.73</v>
       </c>
     </row>
     <row r="1076">
@@ -12271,7 +12271,7 @@
         <v>2722</v>
       </c>
       <c r="C1076" t="n">
-        <v>54540</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1077">
@@ -12282,7 +12282,7 @@
         <v>2718</v>
       </c>
       <c r="C1077" t="n">
-        <v>72720</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1078">
@@ -12293,7 +12293,7 @@
         <v>595</v>
       </c>
       <c r="C1078" t="n">
-        <v>500000</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="1079">
@@ -12304,7 +12304,7 @@
         <v>890</v>
       </c>
       <c r="C1079" t="n">
-        <v>636360</v>
+        <v>668178</v>
       </c>
     </row>
     <row r="1080">
@@ -12315,7 +12315,7 @@
         <v>2652</v>
       </c>
       <c r="C1080" t="n">
-        <v>118180</v>
+        <v>124089</v>
       </c>
     </row>
     <row r="1081">
@@ -12326,7 +12326,7 @@
         <v>2714</v>
       </c>
       <c r="C1081" t="n">
-        <v>327260</v>
+        <v>343623</v>
       </c>
     </row>
     <row r="1082">
@@ -12337,7 +12337,7 @@
         <v>1869</v>
       </c>
       <c r="C1082" t="n">
-        <v>209080</v>
+        <v>219534</v>
       </c>
     </row>
     <row r="1083">
@@ -12348,7 +12348,7 @@
         <v>400</v>
       </c>
       <c r="C1083" t="n">
-        <v>172720</v>
+        <v>181356</v>
       </c>
     </row>
     <row r="1084">
@@ -12359,7 +12359,7 @@
         <v>1907</v>
       </c>
       <c r="C1084" t="n">
-        <v>337260</v>
+        <v>354123</v>
       </c>
     </row>
     <row r="1085">
@@ -12370,7 +12370,7 @@
         <v>1996</v>
       </c>
       <c r="C1085" t="n">
-        <v>213180</v>
+        <v>223839</v>
       </c>
     </row>
     <row r="1086">
@@ -12381,7 +12381,7 @@
         <v>1890</v>
       </c>
       <c r="C1086" t="n">
-        <v>287402.41</v>
+        <v>301772.52</v>
       </c>
     </row>
     <row r="1087">
@@ -12392,7 +12392,7 @@
         <v>2114</v>
       </c>
       <c r="C1087" t="n">
-        <v>167000</v>
+        <v>175350</v>
       </c>
     </row>
     <row r="1088">
@@ -12403,7 +12403,7 @@
         <v>2330</v>
       </c>
       <c r="C1088" t="n">
-        <v>244340</v>
+        <v>256557</v>
       </c>
     </row>
     <row r="1089">
@@ -12447,7 +12447,7 @@
         <v>2629</v>
       </c>
       <c r="C1092" t="n">
-        <v>62440</v>
+        <v>65562</v>
       </c>
     </row>
     <row r="1093">
@@ -12458,7 +12458,7 @@
         <v>951</v>
       </c>
       <c r="C1093" t="n">
-        <v>104540</v>
+        <v>109767</v>
       </c>
     </row>
     <row r="1094">
@@ -12469,7 +12469,7 @@
         <v>2449</v>
       </c>
       <c r="C1094" t="n">
-        <v>36360</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1095">
@@ -12480,7 +12480,7 @@
         <v>610</v>
       </c>
       <c r="C1095" t="n">
-        <v>740900</v>
+        <v>777945</v>
       </c>
     </row>
     <row r="1096">
@@ -12491,7 +12491,7 @@
         <v>2761</v>
       </c>
       <c r="C1096" t="n">
-        <v>74080</v>
+        <v>77784</v>
       </c>
     </row>
     <row r="1097">
@@ -12502,7 +12502,7 @@
         <v>483</v>
       </c>
       <c r="C1097" t="n">
-        <v>402720</v>
+        <v>422856</v>
       </c>
     </row>
     <row r="1098">
@@ -12513,7 +12513,7 @@
         <v>2015</v>
       </c>
       <c r="C1098" t="n">
-        <v>336360</v>
+        <v>353178</v>
       </c>
     </row>
     <row r="1099">
@@ -12524,7 +12524,7 @@
         <v>1478</v>
       </c>
       <c r="C1099" t="n">
-        <v>491960</v>
+        <v>516558</v>
       </c>
     </row>
     <row r="1100">
@@ -12535,7 +12535,7 @@
         <v>424</v>
       </c>
       <c r="C1100" t="n">
-        <v>219620</v>
+        <v>230601</v>
       </c>
     </row>
     <row r="1101">
@@ -12557,7 +12557,7 @@
         <v>477</v>
       </c>
       <c r="C1102" t="n">
-        <v>235140</v>
+        <v>246897</v>
       </c>
     </row>
     <row r="1103">
@@ -12568,7 +12568,7 @@
         <v>1810</v>
       </c>
       <c r="C1103" t="n">
-        <v>36420</v>
+        <v>38241</v>
       </c>
     </row>
     <row r="1104">
@@ -12579,7 +12579,7 @@
         <v>2826</v>
       </c>
       <c r="C1104" t="n">
-        <v>63636.38</v>
+        <v>66818.19</v>
       </c>
     </row>
     <row r="1105">
@@ -12590,7 +12590,7 @@
         <v>2561</v>
       </c>
       <c r="C1105" t="n">
-        <v>13360</v>
+        <v>14028</v>
       </c>
     </row>
     <row r="1106">
@@ -12601,7 +12601,7 @@
         <v>2653</v>
       </c>
       <c r="C1106" t="n">
-        <v>54545.46</v>
+        <v>57272.73</v>
       </c>
     </row>
     <row r="1107">
@@ -12612,7 +12612,7 @@
         <v>2829</v>
       </c>
       <c r="C1107" t="n">
-        <v>54545.46</v>
+        <v>57272.73</v>
       </c>
     </row>
     <row r="1108">
@@ -12623,7 +12623,7 @@
         <v>2643</v>
       </c>
       <c r="C1108" t="n">
-        <v>26840</v>
+        <v>28182</v>
       </c>
     </row>
     <row r="1109">
@@ -12634,7 +12634,7 @@
         <v>2794</v>
       </c>
       <c r="C1109" t="n">
-        <v>81800</v>
+        <v>85890</v>
       </c>
     </row>
     <row r="1110">
@@ -12645,7 +12645,7 @@
         <v>2655</v>
       </c>
       <c r="C1110" t="n">
-        <v>100000</v>
+        <v>105000</v>
       </c>
     </row>
     <row r="1111">
@@ -12656,7 +12656,7 @@
         <v>1456</v>
       </c>
       <c r="C1111" t="n">
-        <v>700260</v>
+        <v>735273</v>
       </c>
     </row>
     <row r="1112">
@@ -12667,7 +12667,7 @@
         <v>2606</v>
       </c>
       <c r="C1112" t="n">
-        <v>215080</v>
+        <v>225834</v>
       </c>
     </row>
     <row r="1113">
@@ -12678,7 +12678,7 @@
         <v>1142</v>
       </c>
       <c r="C1113" t="n">
-        <v>390040</v>
+        <v>409542</v>
       </c>
     </row>
     <row r="1114">
@@ -12689,7 +12689,7 @@
         <v>1450</v>
       </c>
       <c r="C1114" t="n">
-        <v>247780</v>
+        <v>260169</v>
       </c>
     </row>
     <row r="1115">
@@ -12700,7 +12700,7 @@
         <v>2133</v>
       </c>
       <c r="C1115" t="n">
-        <v>578620</v>
+        <v>607551</v>
       </c>
     </row>
     <row r="1116">
@@ -12711,7 +12711,7 @@
         <v>522</v>
       </c>
       <c r="C1116" t="n">
-        <v>177260</v>
+        <v>186123</v>
       </c>
     </row>
     <row r="1117">
@@ -12722,7 +12722,7 @@
         <v>2696</v>
       </c>
       <c r="C1117" t="n">
-        <v>239200</v>
+        <v>251160</v>
       </c>
     </row>
     <row r="1118">
@@ -12744,7 +12744,7 @@
         <v>2692</v>
       </c>
       <c r="C1119" t="n">
-        <v>68180</v>
+        <v>71589</v>
       </c>
     </row>
     <row r="1120">
@@ -12755,7 +12755,7 @@
         <v>2691</v>
       </c>
       <c r="C1120" t="n">
-        <v>122720</v>
+        <v>128856</v>
       </c>
     </row>
     <row r="1121">
@@ -12766,7 +12766,7 @@
         <v>1632</v>
       </c>
       <c r="C1121" t="n">
-        <v>227260</v>
+        <v>238623</v>
       </c>
     </row>
     <row r="1122">
@@ -12777,7 +12777,7 @@
         <v>2641</v>
       </c>
       <c r="C1122" t="n">
-        <v>72720</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1123">
@@ -12788,7 +12788,7 @@
         <v>2197</v>
       </c>
       <c r="C1123" t="n">
-        <v>181800</v>
+        <v>190890</v>
       </c>
     </row>
     <row r="1124">
@@ -12799,7 +12799,7 @@
         <v>609</v>
       </c>
       <c r="C1124" t="n">
-        <v>200000</v>
+        <v>210000</v>
       </c>
     </row>
     <row r="1125">
@@ -12810,7 +12810,7 @@
         <v>1380</v>
       </c>
       <c r="C1125" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1126">
@@ -12821,7 +12821,7 @@
         <v>104</v>
       </c>
       <c r="C1126" t="n">
-        <v>272720</v>
+        <v>286356</v>
       </c>
     </row>
     <row r="1127">
@@ -12832,7 +12832,7 @@
         <v>2621</v>
       </c>
       <c r="C1127" t="n">
-        <v>63620</v>
+        <v>66801</v>
       </c>
     </row>
     <row r="1128">
@@ -12843,7 +12843,7 @@
         <v>2786</v>
       </c>
       <c r="C1128" t="n">
-        <v>63620</v>
+        <v>66801</v>
       </c>
     </row>
     <row r="1129">
@@ -12854,7 +12854,7 @@
         <v>2784</v>
       </c>
       <c r="C1129" t="n">
-        <v>37820</v>
+        <v>39711</v>
       </c>
     </row>
     <row r="1130">
@@ -12865,7 +12865,7 @@
         <v>2586</v>
       </c>
       <c r="C1130" t="n">
-        <v>37820</v>
+        <v>39711</v>
       </c>
     </row>
     <row r="1131">
@@ -12876,7 +12876,7 @@
         <v>2145</v>
       </c>
       <c r="C1131" t="n">
-        <v>117680</v>
+        <v>123564</v>
       </c>
     </row>
     <row r="1132">
@@ -12887,7 +12887,7 @@
         <v>2574</v>
       </c>
       <c r="C1132" t="n">
-        <v>117680</v>
+        <v>123564</v>
       </c>
     </row>
     <row r="1133">
@@ -12898,7 +12898,7 @@
         <v>2492</v>
       </c>
       <c r="C1133" t="n">
-        <v>129000</v>
+        <v>135450</v>
       </c>
     </row>
     <row r="1134">
@@ -12909,7 +12909,7 @@
         <v>629</v>
       </c>
       <c r="C1134" t="n">
-        <v>401800</v>
+        <v>421890</v>
       </c>
     </row>
     <row r="1135">
@@ -12920,7 +12920,7 @@
         <v>966</v>
       </c>
       <c r="C1135" t="n">
-        <v>74080</v>
+        <v>77784</v>
       </c>
     </row>
     <row r="1136">
@@ -12931,7 +12931,7 @@
         <v>2721</v>
       </c>
       <c r="C1136" t="n">
-        <v>74080</v>
+        <v>77784</v>
       </c>
     </row>
     <row r="1137">
@@ -12942,7 +12942,7 @@
         <v>2554</v>
       </c>
       <c r="C1137" t="n">
-        <v>22320</v>
+        <v>23436</v>
       </c>
     </row>
     <row r="1138">
@@ -12953,7 +12953,7 @@
         <v>2556</v>
       </c>
       <c r="C1138" t="n">
-        <v>32820</v>
+        <v>34461</v>
       </c>
     </row>
     <row r="1139">
@@ -12964,7 +12964,7 @@
         <v>2546</v>
       </c>
       <c r="C1139" t="n">
-        <v>21680</v>
+        <v>22764</v>
       </c>
     </row>
     <row r="1140">
@@ -12975,7 +12975,7 @@
         <v>42</v>
       </c>
       <c r="C1140" t="n">
-        <v>1718180</v>
+        <v>1804089</v>
       </c>
     </row>
     <row r="1141">
@@ -12986,7 +12986,7 @@
         <v>953</v>
       </c>
       <c r="C1141" t="n">
-        <v>620600</v>
+        <v>651630</v>
       </c>
     </row>
     <row r="1142">
@@ -12997,7 +12997,7 @@
         <v>1137</v>
       </c>
       <c r="C1142" t="n">
-        <v>581800</v>
+        <v>610890</v>
       </c>
     </row>
     <row r="1143">
@@ -13008,7 +13008,7 @@
         <v>675</v>
       </c>
       <c r="C1143" t="n">
-        <v>181800</v>
+        <v>190890</v>
       </c>
     </row>
     <row r="1144">
@@ -13019,7 +13019,7 @@
         <v>619</v>
       </c>
       <c r="C1144" t="n">
-        <v>281120</v>
+        <v>295176</v>
       </c>
     </row>
     <row r="1145">
@@ -13030,7 +13030,7 @@
         <v>1299</v>
       </c>
       <c r="C1145" t="n">
-        <v>473040</v>
+        <v>496692</v>
       </c>
     </row>
     <row r="1146">
@@ -13041,7 +13041,7 @@
         <v>1064</v>
       </c>
       <c r="C1146" t="n">
-        <v>544880</v>
+        <v>572124</v>
       </c>
     </row>
     <row r="1147">
@@ -13052,7 +13052,7 @@
         <v>2308</v>
       </c>
       <c r="C1147" t="n">
-        <v>186360</v>
+        <v>195678</v>
       </c>
     </row>
     <row r="1148">
@@ -13063,7 +13063,7 @@
         <v>2747</v>
       </c>
       <c r="C1148" t="n">
-        <v>54545.46</v>
+        <v>57272.73</v>
       </c>
     </row>
     <row r="1149">
@@ -13074,7 +13074,7 @@
         <v>2819</v>
       </c>
       <c r="C1149" t="n">
-        <v>54545.46</v>
+        <v>57272.73</v>
       </c>
     </row>
     <row r="1150">
@@ -13085,7 +13085,7 @@
         <v>1259</v>
       </c>
       <c r="C1150" t="n">
-        <v>90909.10000000001</v>
+        <v>95454.55</v>
       </c>
     </row>
     <row r="1151">
@@ -13096,7 +13096,7 @@
         <v>2544</v>
       </c>
       <c r="C1151" t="n">
-        <v>72720</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1152">
@@ -13107,7 +13107,7 @@
         <v>2261</v>
       </c>
       <c r="C1152" t="n">
-        <v>136360</v>
+        <v>143178</v>
       </c>
     </row>
     <row r="1153">
@@ -13118,7 +13118,7 @@
         <v>2729</v>
       </c>
       <c r="C1153" t="n">
-        <v>72720</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1154">
@@ -13129,7 +13129,7 @@
         <v>2649</v>
       </c>
       <c r="C1154" t="n">
-        <v>26840</v>
+        <v>28182</v>
       </c>
     </row>
     <row r="1155">
@@ -13140,7 +13140,7 @@
         <v>2494</v>
       </c>
       <c r="C1155" t="n">
-        <v>118180</v>
+        <v>124089</v>
       </c>
     </row>
     <row r="1156">
@@ -13162,7 +13162,7 @@
         <v>2802</v>
       </c>
       <c r="C1157" t="n">
-        <v>64380</v>
+        <v>67599</v>
       </c>
     </row>
     <row r="1158">
@@ -13173,7 +13173,7 @@
         <v>2726</v>
       </c>
       <c r="C1158" t="n">
-        <v>136360</v>
+        <v>143178</v>
       </c>
     </row>
     <row r="1159">
@@ -13184,7 +13184,7 @@
         <v>2820</v>
       </c>
       <c r="C1159" t="n">
-        <v>163620</v>
+        <v>171801</v>
       </c>
     </row>
     <row r="1160">
@@ -13195,7 +13195,7 @@
         <v>1007</v>
       </c>
       <c r="C1160" t="n">
-        <v>172720</v>
+        <v>181356</v>
       </c>
     </row>
     <row r="1161">
@@ -13206,7 +13206,7 @@
         <v>20</v>
       </c>
       <c r="C1161" t="n">
-        <v>350000</v>
+        <v>367500</v>
       </c>
     </row>
     <row r="1162">
@@ -13217,7 +13217,7 @@
         <v>1372</v>
       </c>
       <c r="C1162" t="n">
-        <v>263620</v>
+        <v>276801</v>
       </c>
     </row>
     <row r="1163">
@@ -13228,7 +13228,7 @@
         <v>2735</v>
       </c>
       <c r="C1163" t="n">
-        <v>109080</v>
+        <v>114534</v>
       </c>
     </row>
     <row r="1164">
@@ -13239,7 +13239,7 @@
         <v>2811</v>
       </c>
       <c r="C1164" t="n">
-        <v>37820</v>
+        <v>39711</v>
       </c>
     </row>
     <row r="1165">
@@ -13250,7 +13250,7 @@
         <v>1871</v>
       </c>
       <c r="C1165" t="n">
-        <v>160680</v>
+        <v>168714</v>
       </c>
     </row>
     <row r="1166">
@@ -13261,7 +13261,7 @@
         <v>2541</v>
       </c>
       <c r="C1166" t="n">
-        <v>192360</v>
+        <v>201978</v>
       </c>
     </row>
     <row r="1167">
@@ -13272,7 +13272,7 @@
         <v>2362</v>
       </c>
       <c r="C1167" t="n">
-        <v>68180</v>
+        <v>71589</v>
       </c>
     </row>
     <row r="1168">
@@ -13283,7 +13283,7 @@
         <v>1324</v>
       </c>
       <c r="C1168" t="n">
-        <v>254540</v>
+        <v>267267</v>
       </c>
     </row>
     <row r="1169">
@@ -13294,7 +13294,7 @@
         <v>2323</v>
       </c>
       <c r="C1169" t="n">
-        <v>62440</v>
+        <v>65562</v>
       </c>
     </row>
     <row r="1170">
@@ -13305,7 +13305,7 @@
         <v>2647</v>
       </c>
       <c r="C1170" t="n">
-        <v>129000</v>
+        <v>135450</v>
       </c>
     </row>
     <row r="1171">
@@ -13316,7 +13316,7 @@
         <v>559</v>
       </c>
       <c r="C1171" t="n">
-        <v>208580</v>
+        <v>219009</v>
       </c>
     </row>
     <row r="1172">
@@ -13327,7 +13327,7 @@
         <v>2762</v>
       </c>
       <c r="C1172" t="n">
-        <v>74080</v>
+        <v>77784</v>
       </c>
     </row>
     <row r="1173">
@@ -13338,7 +13338,7 @@
         <v>2501</v>
       </c>
       <c r="C1173" t="n">
-        <v>74080</v>
+        <v>77784</v>
       </c>
     </row>
     <row r="1174">
@@ -13349,7 +13349,7 @@
         <v>2562</v>
       </c>
       <c r="C1174" t="n">
-        <v>14380</v>
+        <v>15099</v>
       </c>
     </row>
     <row r="1175">
@@ -13360,7 +13360,7 @@
         <v>429</v>
       </c>
       <c r="C1175" t="n">
-        <v>354540</v>
+        <v>372267</v>
       </c>
     </row>
     <row r="1176">
@@ -13371,7 +13371,7 @@
         <v>58</v>
       </c>
       <c r="C1176" t="n">
-        <v>245980</v>
+        <v>258279</v>
       </c>
     </row>
     <row r="1177">
@@ -13382,7 +13382,7 @@
         <v>2245</v>
       </c>
       <c r="C1177" t="n">
-        <v>219620</v>
+        <v>230601</v>
       </c>
     </row>
     <row r="1178">
@@ -13393,7 +13393,7 @@
         <v>285</v>
       </c>
       <c r="C1178" t="n">
-        <v>491960</v>
+        <v>516558</v>
       </c>
     </row>
     <row r="1179">
@@ -13415,7 +13415,7 @@
         <v>363</v>
       </c>
       <c r="C1180" t="n">
-        <v>272720</v>
+        <v>286356</v>
       </c>
     </row>
     <row r="1181">
@@ -13426,7 +13426,7 @@
         <v>2651</v>
       </c>
       <c r="C1181" t="n">
-        <v>153740</v>
+        <v>161427</v>
       </c>
     </row>
     <row r="1182">
@@ -13437,7 +13437,7 @@
         <v>2142</v>
       </c>
       <c r="C1182" t="n">
-        <v>48520</v>
+        <v>50946</v>
       </c>
     </row>
     <row r="1183">
@@ -13448,7 +13448,7 @@
         <v>2258</v>
       </c>
       <c r="C1183" t="n">
-        <v>72727.28</v>
+        <v>76363.64</v>
       </c>
     </row>
     <row r="1184">
@@ -13459,7 +13459,7 @@
         <v>2772</v>
       </c>
       <c r="C1184" t="n">
-        <v>54545.46</v>
+        <v>57272.73</v>
       </c>
     </row>
     <row r="1185">
@@ -13470,7 +13470,7 @@
         <v>2346</v>
       </c>
       <c r="C1185" t="n">
-        <v>100000</v>
+        <v>105000</v>
       </c>
     </row>
     <row r="1186">
@@ -13481,7 +13481,7 @@
         <v>2442</v>
       </c>
       <c r="C1186" t="n">
-        <v>72720</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1187">
@@ -13492,7 +13492,7 @@
         <v>772</v>
       </c>
       <c r="C1187" t="n">
-        <v>300000</v>
+        <v>315000</v>
       </c>
     </row>
     <row r="1188">
@@ -13503,7 +13503,7 @@
         <v>2684</v>
       </c>
       <c r="C1188" t="n">
-        <v>86360</v>
+        <v>90678</v>
       </c>
     </row>
     <row r="1189">
@@ -13514,7 +13514,7 @@
         <v>2765</v>
       </c>
       <c r="C1189" t="n">
-        <v>81800</v>
+        <v>85890</v>
       </c>
     </row>
     <row r="1190">
@@ -13525,7 +13525,7 @@
         <v>2567</v>
       </c>
       <c r="C1190" t="n">
-        <v>150040</v>
+        <v>157542</v>
       </c>
     </row>
     <row r="1191">
@@ -13536,7 +13536,7 @@
         <v>2178</v>
       </c>
       <c r="C1191" t="n">
-        <v>254540</v>
+        <v>267267</v>
       </c>
     </row>
     <row r="1192">
@@ -13547,7 +13547,7 @@
         <v>2827</v>
       </c>
       <c r="C1192" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1193">
@@ -13558,7 +13558,7 @@
         <v>2510</v>
       </c>
       <c r="C1193" t="n">
-        <v>504760</v>
+        <v>529998</v>
       </c>
     </row>
     <row r="1194">
@@ -13569,7 +13569,7 @@
         <v>2392</v>
       </c>
       <c r="C1194" t="n">
-        <v>151420</v>
+        <v>158991</v>
       </c>
     </row>
     <row r="1195">
@@ -13580,7 +13580,7 @@
         <v>415</v>
       </c>
       <c r="C1195" t="n">
-        <v>517720</v>
+        <v>543606</v>
       </c>
     </row>
     <row r="1196">
@@ -13591,7 +13591,7 @@
         <v>2107</v>
       </c>
       <c r="C1196" t="n">
-        <v>267340</v>
+        <v>280707</v>
       </c>
     </row>
     <row r="1197">
@@ -13602,7 +13602,7 @@
         <v>2211</v>
       </c>
       <c r="C1197" t="n">
-        <v>221640</v>
+        <v>232722</v>
       </c>
     </row>
     <row r="1198">
@@ -13613,7 +13613,7 @@
         <v>2682</v>
       </c>
       <c r="C1198" t="n">
-        <v>136340</v>
+        <v>143157</v>
       </c>
     </row>
     <row r="1199">
@@ -13646,7 +13646,7 @@
         <v>2755</v>
       </c>
       <c r="C1201" t="n">
-        <v>54540</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1202">
@@ -13657,7 +13657,7 @@
         <v>941</v>
       </c>
       <c r="C1202" t="n">
-        <v>323518.63</v>
+        <v>339694.56</v>
       </c>
     </row>
     <row r="1203">
@@ -13668,7 +13668,7 @@
         <v>2734</v>
       </c>
       <c r="C1203" t="n">
-        <v>50060</v>
+        <v>52563</v>
       </c>
     </row>
     <row r="1204">
@@ -13690,7 +13690,7 @@
         <v>1289</v>
       </c>
       <c r="C1205" t="n">
-        <v>227260</v>
+        <v>238623</v>
       </c>
     </row>
     <row r="1206">
@@ -13701,7 +13701,7 @@
         <v>2801</v>
       </c>
       <c r="C1206" t="n">
-        <v>72720</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1207">
@@ -13712,7 +13712,7 @@
         <v>2810</v>
       </c>
       <c r="C1207" t="n">
-        <v>122720</v>
+        <v>128856</v>
       </c>
     </row>
     <row r="1208">
@@ -13723,7 +13723,7 @@
         <v>767</v>
       </c>
       <c r="C1208" t="n">
-        <v>163620</v>
+        <v>171801</v>
       </c>
     </row>
     <row r="1209">
@@ -13734,7 +13734,7 @@
         <v>2687</v>
       </c>
       <c r="C1209" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1210">
@@ -13745,7 +13745,7 @@
         <v>2686</v>
       </c>
       <c r="C1210" t="n">
-        <v>118180</v>
+        <v>124089</v>
       </c>
     </row>
     <row r="1211">
@@ -13756,7 +13756,7 @@
         <v>2730</v>
       </c>
       <c r="C1211" t="n">
-        <v>81800</v>
+        <v>85890</v>
       </c>
     </row>
     <row r="1212">
@@ -13767,7 +13767,7 @@
         <v>2580</v>
       </c>
       <c r="C1212" t="n">
-        <v>30500</v>
+        <v>32025</v>
       </c>
     </row>
     <row r="1213">
@@ -13778,7 +13778,7 @@
         <v>2472</v>
       </c>
       <c r="C1213" t="n">
-        <v>48129.1</v>
+        <v>50535.55</v>
       </c>
     </row>
     <row r="1214">
@@ -13789,7 +13789,7 @@
         <v>2631</v>
       </c>
       <c r="C1214" t="n">
-        <v>22301.82</v>
+        <v>23416.91</v>
       </c>
     </row>
     <row r="1215">
@@ -13800,7 +13800,7 @@
         <v>1642</v>
       </c>
       <c r="C1215" t="n">
-        <v>240900</v>
+        <v>252945</v>
       </c>
     </row>
     <row r="1216">
@@ -13811,7 +13811,7 @@
         <v>2613</v>
       </c>
       <c r="C1216" t="n">
-        <v>162900</v>
+        <v>171045</v>
       </c>
     </row>
     <row r="1217">
@@ -13822,7 +13822,7 @@
         <v>1020</v>
       </c>
       <c r="C1217" t="n">
-        <v>81800</v>
+        <v>85890</v>
       </c>
     </row>
     <row r="1218">
@@ -13833,7 +13833,7 @@
         <v>2785</v>
       </c>
       <c r="C1218" t="n">
-        <v>37820</v>
+        <v>39711</v>
       </c>
     </row>
     <row r="1219">
@@ -13844,7 +13844,7 @@
         <v>1327</v>
       </c>
       <c r="C1219" t="n">
-        <v>54540</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1220">
@@ -13855,7 +13855,7 @@
         <v>749</v>
       </c>
       <c r="C1220" t="n">
-        <v>74080</v>
+        <v>77784</v>
       </c>
     </row>
     <row r="1221">
@@ -13866,7 +13866,7 @@
         <v>1983</v>
       </c>
       <c r="C1221" t="n">
-        <v>491960</v>
+        <v>516558</v>
       </c>
     </row>
     <row r="1222">
@@ -13877,7 +13877,7 @@
         <v>1993</v>
       </c>
       <c r="C1222" t="n">
-        <v>316260</v>
+        <v>332073</v>
       </c>
     </row>
     <row r="1223">
@@ -13888,7 +13888,7 @@
         <v>2767</v>
       </c>
       <c r="C1223" t="n">
-        <v>175380</v>
+        <v>184149</v>
       </c>
     </row>
     <row r="1224">
@@ -13910,7 +13910,7 @@
         <v>1102</v>
       </c>
       <c r="C1225" t="n">
-        <v>219620</v>
+        <v>230601</v>
       </c>
     </row>
     <row r="1226">
@@ -13921,7 +13921,7 @@
         <v>626</v>
       </c>
       <c r="C1226" t="n">
-        <v>1549377.28</v>
+        <v>1626846.14</v>
       </c>
     </row>
     <row r="1227">
@@ -13932,7 +13932,7 @@
         <v>1465</v>
       </c>
       <c r="C1227" t="n">
-        <v>327080</v>
+        <v>343434</v>
       </c>
     </row>
     <row r="1228">
@@ -13943,7 +13943,7 @@
         <v>2758</v>
       </c>
       <c r="C1228" t="n">
-        <v>54545.46</v>
+        <v>57272.73</v>
       </c>
     </row>
     <row r="1229">
@@ -13954,7 +13954,7 @@
         <v>2742</v>
       </c>
       <c r="C1229" t="n">
-        <v>54545.46</v>
+        <v>57272.73</v>
       </c>
     </row>
     <row r="1230">
@@ -13976,7 +13976,7 @@
         <v>1873</v>
       </c>
       <c r="C1231" t="n">
-        <v>290900</v>
+        <v>305445</v>
       </c>
     </row>
     <row r="1232">
@@ -13987,7 +13987,7 @@
         <v>2163</v>
       </c>
       <c r="C1232" t="n">
-        <v>136360</v>
+        <v>143178</v>
       </c>
     </row>
     <row r="1233">
@@ -13998,7 +13998,7 @@
         <v>2394</v>
       </c>
       <c r="C1233" t="n">
-        <v>140040</v>
+        <v>147042</v>
       </c>
     </row>
     <row r="1234">
@@ -14009,7 +14009,7 @@
         <v>33</v>
       </c>
       <c r="C1234" t="n">
-        <v>352720</v>
+        <v>370356</v>
       </c>
     </row>
     <row r="1235">
@@ -14020,7 +14020,7 @@
         <v>2421</v>
       </c>
       <c r="C1235" t="n">
-        <v>59080</v>
+        <v>62034</v>
       </c>
     </row>
     <row r="1236">
@@ -14031,7 +14031,7 @@
         <v>2663</v>
       </c>
       <c r="C1236" t="n">
-        <v>250000</v>
+        <v>262500</v>
       </c>
     </row>
     <row r="1237">
@@ -14042,7 +14042,7 @@
         <v>2413</v>
       </c>
       <c r="C1237" t="n">
-        <v>110040</v>
+        <v>115542</v>
       </c>
     </row>
     <row r="1238">
@@ -14053,7 +14053,7 @@
         <v>351</v>
       </c>
       <c r="C1238" t="n">
-        <v>167260</v>
+        <v>175623</v>
       </c>
     </row>
     <row r="1239">
@@ -14064,7 +14064,7 @@
         <v>1298</v>
       </c>
       <c r="C1239" t="n">
-        <v>1157260</v>
+        <v>1215123</v>
       </c>
     </row>
     <row r="1240">
@@ -14075,7 +14075,7 @@
         <v>2491</v>
       </c>
       <c r="C1240" t="n">
-        <v>93520</v>
+        <v>98196</v>
       </c>
     </row>
     <row r="1241">
@@ -14086,7 +14086,7 @@
         <v>2571</v>
       </c>
       <c r="C1241" t="n">
-        <v>132060</v>
+        <v>138663</v>
       </c>
     </row>
     <row r="1242">
@@ -14097,7 +14097,7 @@
         <v>2507</v>
       </c>
       <c r="C1242" t="n">
-        <v>80240</v>
+        <v>84252</v>
       </c>
     </row>
     <row r="1243">
@@ -14108,7 +14108,7 @@
         <v>2799</v>
       </c>
       <c r="C1243" t="n">
-        <v>103280</v>
+        <v>108444</v>
       </c>
     </row>
     <row r="1244">
@@ -14130,7 +14130,7 @@
         <v>2582</v>
       </c>
       <c r="C1245" t="n">
-        <v>78680</v>
+        <v>82614</v>
       </c>
     </row>
     <row r="1246">
@@ -14141,7 +14141,7 @@
         <v>2637</v>
       </c>
       <c r="C1246" t="n">
-        <v>57220</v>
+        <v>60081</v>
       </c>
     </row>
     <row r="1247">
@@ -14152,7 +14152,7 @@
         <v>630</v>
       </c>
       <c r="C1247" t="n">
-        <v>136080</v>
+        <v>142884</v>
       </c>
     </row>
     <row r="1248">
@@ -14163,7 +14163,7 @@
         <v>525</v>
       </c>
       <c r="C1248" t="n">
-        <v>204540</v>
+        <v>214767</v>
       </c>
     </row>
     <row r="1249">
@@ -14174,7 +14174,7 @@
         <v>2727</v>
       </c>
       <c r="C1249" t="n">
-        <v>36800</v>
+        <v>38640</v>
       </c>
     </row>
     <row r="1250">
@@ -14185,7 +14185,7 @@
         <v>2707</v>
       </c>
       <c r="C1250" t="n">
-        <v>29120</v>
+        <v>30576</v>
       </c>
     </row>
     <row r="1251">
@@ -14196,7 +14196,7 @@
         <v>2834</v>
       </c>
       <c r="C1251" t="n">
-        <v>15043.64</v>
+        <v>15795.82</v>
       </c>
     </row>
     <row r="1252">
@@ -14207,7 +14207,7 @@
         <v>2773</v>
       </c>
       <c r="C1252" t="n">
-        <v>73356.38</v>
+        <v>77024.19</v>
       </c>
     </row>
     <row r="1253">
@@ -14218,7 +14218,7 @@
         <v>2341</v>
       </c>
       <c r="C1253" t="n">
-        <v>129000</v>
+        <v>135450</v>
       </c>
     </row>
     <row r="1254">
@@ -14229,7 +14229,7 @@
         <v>1374</v>
       </c>
       <c r="C1254" t="n">
-        <v>163620</v>
+        <v>171801</v>
       </c>
     </row>
     <row r="1255">
@@ -14240,7 +14240,7 @@
         <v>793</v>
       </c>
       <c r="C1255" t="n">
-        <v>37820</v>
+        <v>39711</v>
       </c>
     </row>
     <row r="1256">
@@ -14251,7 +14251,7 @@
         <v>794</v>
       </c>
       <c r="C1256" t="n">
-        <v>37820</v>
+        <v>39711</v>
       </c>
     </row>
     <row r="1257">
@@ -14262,7 +14262,7 @@
         <v>1834</v>
       </c>
       <c r="C1257" t="n">
-        <v>106360</v>
+        <v>111678</v>
       </c>
     </row>
     <row r="1258">
@@ -14273,7 +14273,7 @@
         <v>802</v>
       </c>
       <c r="C1258" t="n">
-        <v>68180</v>
+        <v>71589</v>
       </c>
     </row>
     <row r="1259">
@@ -14284,7 +14284,7 @@
         <v>1344</v>
       </c>
       <c r="C1259" t="n">
-        <v>136360</v>
+        <v>143178</v>
       </c>
     </row>
     <row r="1260">
@@ -14295,7 +14295,7 @@
         <v>1881</v>
       </c>
       <c r="C1260" t="n">
-        <v>62440</v>
+        <v>65562</v>
       </c>
     </row>
     <row r="1261">
@@ -14306,7 +14306,7 @@
         <v>2365</v>
       </c>
       <c r="C1261" t="n">
-        <v>72420</v>
+        <v>76041</v>
       </c>
     </row>
     <row r="1262">
@@ -14317,7 +14317,7 @@
         <v>2411</v>
       </c>
       <c r="C1262" t="n">
-        <v>129000</v>
+        <v>135450</v>
       </c>
     </row>
     <row r="1263">
@@ -14328,7 +14328,7 @@
         <v>2363</v>
       </c>
       <c r="C1263" t="n">
-        <v>136360</v>
+        <v>143178</v>
       </c>
     </row>
     <row r="1264">
@@ -14339,7 +14339,7 @@
         <v>2124</v>
       </c>
       <c r="C1264" t="n">
-        <v>318180</v>
+        <v>334089</v>
       </c>
     </row>
     <row r="1265">
@@ -14350,7 +14350,7 @@
         <v>1937</v>
       </c>
       <c r="C1265" t="n">
-        <v>231800</v>
+        <v>243390</v>
       </c>
     </row>
     <row r="1266">
@@ -14361,7 +14361,7 @@
         <v>2709</v>
       </c>
       <c r="C1266" t="n">
-        <v>163620</v>
+        <v>171801</v>
       </c>
     </row>
     <row r="1267">
@@ -14372,7 +14372,7 @@
         <v>2558</v>
       </c>
       <c r="C1267" t="n">
-        <v>27320</v>
+        <v>28686</v>
       </c>
     </row>
     <row r="1268">
@@ -14383,7 +14383,7 @@
         <v>663</v>
       </c>
       <c r="C1268" t="n">
-        <v>231800</v>
+        <v>243390</v>
       </c>
     </row>
     <row r="1269">
@@ -14394,7 +14394,7 @@
         <v>40</v>
       </c>
       <c r="C1269" t="n">
-        <v>200000</v>
+        <v>210000</v>
       </c>
     </row>
     <row r="1270">
@@ -14405,7 +14405,7 @@
         <v>2833</v>
       </c>
       <c r="C1270" t="n">
-        <v>63636.38</v>
+        <v>66818.19</v>
       </c>
     </row>
     <row r="1271">
@@ -14416,7 +14416,7 @@
         <v>1756</v>
       </c>
       <c r="C1271" t="n">
-        <v>396820</v>
+        <v>416661</v>
       </c>
     </row>
     <row r="1272">
@@ -14427,7 +14427,7 @@
         <v>1116</v>
       </c>
       <c r="C1272" t="n">
-        <v>230580</v>
+        <v>242109</v>
       </c>
     </row>
     <row r="1273">
@@ -14438,7 +14438,7 @@
         <v>636</v>
       </c>
       <c r="C1273" t="n">
-        <v>227260</v>
+        <v>238623</v>
       </c>
     </row>
     <row r="1274">
@@ -14449,7 +14449,7 @@
         <v>1800</v>
       </c>
       <c r="C1274" t="n">
-        <v>25440</v>
+        <v>26712</v>
       </c>
     </row>
     <row r="1275">
@@ -14460,7 +14460,7 @@
         <v>2815</v>
       </c>
       <c r="C1275" t="n">
-        <v>54545.46</v>
+        <v>57272.73</v>
       </c>
     </row>
     <row r="1276">
@@ -14471,7 +14471,7 @@
         <v>1658</v>
       </c>
       <c r="C1276" t="n">
-        <v>120000</v>
+        <v>126000</v>
       </c>
     </row>
     <row r="1277">
@@ -14482,7 +14482,7 @@
         <v>2635</v>
       </c>
       <c r="C1277" t="n">
-        <v>118180</v>
+        <v>124089</v>
       </c>
     </row>
     <row r="1278">
@@ -14493,7 +14493,7 @@
         <v>2402</v>
       </c>
       <c r="C1278" t="n">
-        <v>592720</v>
+        <v>622356</v>
       </c>
     </row>
     <row r="1279">
@@ -14504,7 +14504,7 @@
         <v>452</v>
       </c>
       <c r="C1279" t="n">
-        <v>245440</v>
+        <v>257712</v>
       </c>
     </row>
     <row r="1280">
@@ -14515,7 +14515,7 @@
         <v>2085</v>
       </c>
       <c r="C1280" t="n">
-        <v>120040</v>
+        <v>126042</v>
       </c>
     </row>
     <row r="1281">
@@ -14526,7 +14526,7 @@
         <v>2568</v>
       </c>
       <c r="C1281" t="n">
-        <v>185840</v>
+        <v>195132</v>
       </c>
     </row>
     <row r="1282">
@@ -14537,7 +14537,7 @@
         <v>1906</v>
       </c>
       <c r="C1282" t="n">
-        <v>105480</v>
+        <v>110754</v>
       </c>
     </row>
     <row r="1283">
@@ -14548,7 +14548,7 @@
         <v>2821</v>
       </c>
       <c r="C1283" t="n">
-        <v>91720</v>
+        <v>96306</v>
       </c>
     </row>
     <row r="1284">
@@ -14559,7 +14559,7 @@
         <v>2698</v>
       </c>
       <c r="C1284" t="n">
-        <v>112420</v>
+        <v>118041</v>
       </c>
     </row>
     <row r="1285">
@@ -14570,7 +14570,7 @@
         <v>2118</v>
       </c>
       <c r="C1285" t="n">
-        <v>215600</v>
+        <v>226380</v>
       </c>
     </row>
     <row r="1286">
@@ -14581,7 +14581,7 @@
         <v>2383</v>
       </c>
       <c r="C1286" t="n">
-        <v>125880</v>
+        <v>132174</v>
       </c>
     </row>
     <row r="1287">
@@ -14592,7 +14592,7 @@
         <v>2813</v>
       </c>
       <c r="C1287" t="n">
-        <v>57220</v>
+        <v>60081</v>
       </c>
     </row>
     <row r="1288">
@@ -14603,7 +14603,7 @@
         <v>925</v>
       </c>
       <c r="C1288" t="n">
-        <v>71520</v>
+        <v>75096</v>
       </c>
     </row>
     <row r="1289">
@@ -14614,7 +14614,7 @@
         <v>2689</v>
       </c>
       <c r="C1289" t="n">
-        <v>57220</v>
+        <v>60081</v>
       </c>
     </row>
     <row r="1290">
@@ -14625,7 +14625,7 @@
         <v>2716</v>
       </c>
       <c r="C1290" t="n">
-        <v>78680</v>
+        <v>82614</v>
       </c>
     </row>
     <row r="1291">
@@ -14636,7 +14636,7 @@
         <v>2831</v>
       </c>
       <c r="C1291" t="n">
-        <v>54540</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1292">
@@ -14647,7 +14647,7 @@
         <v>2045</v>
       </c>
       <c r="C1292" t="n">
-        <v>305868.76</v>
+        <v>321162.19</v>
       </c>
     </row>
     <row r="1293">
@@ -14658,7 +14658,7 @@
         <v>580</v>
       </c>
       <c r="C1293" t="n">
-        <v>122720</v>
+        <v>128856</v>
       </c>
     </row>
     <row r="1294">
@@ -14669,7 +14669,7 @@
         <v>438</v>
       </c>
       <c r="C1294" t="n">
-        <v>140900</v>
+        <v>147945</v>
       </c>
     </row>
     <row r="1295">
@@ -14680,7 +14680,7 @@
         <v>1539</v>
       </c>
       <c r="C1295" t="n">
-        <v>154540</v>
+        <v>162267</v>
       </c>
     </row>
     <row r="1296">
@@ -14691,7 +14691,7 @@
         <v>2817</v>
       </c>
       <c r="C1296" t="n">
-        <v>54540</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1297">
@@ -14702,7 +14702,7 @@
         <v>2816</v>
       </c>
       <c r="C1297" t="n">
-        <v>118180</v>
+        <v>124089</v>
       </c>
     </row>
     <row r="1298">
@@ -14713,7 +14713,7 @@
         <v>2146</v>
       </c>
       <c r="C1298" t="n">
-        <v>183320</v>
+        <v>192486</v>
       </c>
     </row>
     <row r="1299">
@@ -14724,7 +14724,7 @@
         <v>2276</v>
       </c>
       <c r="C1299" t="n">
-        <v>203680</v>
+        <v>213864</v>
       </c>
     </row>
     <row r="1300">
@@ -14735,7 +14735,7 @@
         <v>1381</v>
       </c>
       <c r="C1300" t="n">
-        <v>268180</v>
+        <v>281589</v>
       </c>
     </row>
     <row r="1301">
@@ -14746,7 +14746,7 @@
         <v>2081</v>
       </c>
       <c r="C1301" t="n">
-        <v>136360</v>
+        <v>143178</v>
       </c>
     </row>
     <row r="1302">
@@ -14757,7 +14757,7 @@
         <v>14</v>
       </c>
       <c r="C1302" t="n">
-        <v>395440</v>
+        <v>415212</v>
       </c>
     </row>
     <row r="1303">
@@ -14768,7 +14768,7 @@
         <v>766</v>
       </c>
       <c r="C1303" t="n">
-        <v>62440</v>
+        <v>65562</v>
       </c>
     </row>
     <row r="1304">
@@ -14779,7 +14779,7 @@
         <v>2547</v>
       </c>
       <c r="C1304" t="n">
-        <v>37380</v>
+        <v>39249</v>
       </c>
     </row>
     <row r="1305">
@@ -14790,7 +14790,7 @@
         <v>2552</v>
       </c>
       <c r="C1305" t="n">
-        <v>26880</v>
+        <v>28224</v>
       </c>
     </row>
     <row r="1306">
@@ -14801,7 +14801,7 @@
         <v>131</v>
       </c>
       <c r="C1306" t="n">
-        <v>371800</v>
+        <v>390390</v>
       </c>
     </row>
     <row r="1307">
@@ -14812,7 +14812,7 @@
         <v>2250</v>
       </c>
       <c r="C1307" t="n">
-        <v>300820</v>
+        <v>315861</v>
       </c>
     </row>
     <row r="1308">
@@ -14823,7 +14823,7 @@
         <v>89</v>
       </c>
       <c r="C1308" t="n">
-        <v>307440</v>
+        <v>322812</v>
       </c>
     </row>
     <row r="1309">
@@ -14834,7 +14834,7 @@
         <v>2141</v>
       </c>
       <c r="C1309" t="n">
-        <v>28760</v>
+        <v>30198</v>
       </c>
     </row>
     <row r="1310">
@@ -14845,7 +14845,7 @@
         <v>2798</v>
       </c>
       <c r="C1310" t="n">
-        <v>54545.46</v>
+        <v>57272.73</v>
       </c>
     </row>
     <row r="1311">
@@ -14856,7 +14856,7 @@
         <v>2797</v>
       </c>
       <c r="C1311" t="n">
-        <v>54545.46</v>
+        <v>57272.73</v>
       </c>
     </row>
     <row r="1312">
@@ -14867,7 +14867,7 @@
         <v>2266</v>
       </c>
       <c r="C1312" t="n">
-        <v>72727.28</v>
+        <v>76363.64</v>
       </c>
     </row>
     <row r="1313">
@@ -14878,7 +14878,7 @@
         <v>1499</v>
       </c>
       <c r="C1313" t="n">
-        <v>127260</v>
+        <v>133623</v>
       </c>
     </row>
     <row r="1314">
@@ -14889,7 +14889,7 @@
         <v>2496</v>
       </c>
       <c r="C1314" t="n">
-        <v>145440</v>
+        <v>152712</v>
       </c>
     </row>
     <row r="1315">
@@ -14900,7 +14900,7 @@
         <v>949</v>
       </c>
       <c r="C1315" t="n">
-        <v>89220</v>
+        <v>93681</v>
       </c>
     </row>
     <row r="1316">
@@ -14911,7 +14911,7 @@
         <v>1853</v>
       </c>
       <c r="C1316" t="n">
-        <v>109080</v>
+        <v>114534</v>
       </c>
     </row>
     <row r="1317">
@@ -14922,7 +14922,7 @@
         <v>854</v>
       </c>
       <c r="C1317" t="n">
-        <v>100000</v>
+        <v>105000</v>
       </c>
     </row>
     <row r="1318">
@@ -14933,7 +14933,7 @@
         <v>2674</v>
       </c>
       <c r="C1318" t="n">
-        <v>236360</v>
+        <v>248178</v>
       </c>
     </row>
     <row r="1319">
@@ -14944,7 +14944,7 @@
         <v>2803</v>
       </c>
       <c r="C1319" t="n">
-        <v>109080</v>
+        <v>114534</v>
       </c>
     </row>
     <row r="1320">
@@ -14955,7 +14955,7 @@
         <v>2599</v>
       </c>
       <c r="C1320" t="n">
-        <v>172720</v>
+        <v>181356</v>
       </c>
     </row>
     <row r="1321">
@@ -14966,7 +14966,7 @@
         <v>783</v>
       </c>
       <c r="C1321" t="n">
-        <v>47260</v>
+        <v>49623</v>
       </c>
     </row>
     <row r="1322">
@@ -14977,7 +14977,7 @@
         <v>27</v>
       </c>
       <c r="C1322" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1323">
@@ -14988,7 +14988,7 @@
         <v>531</v>
       </c>
       <c r="C1323" t="n">
-        <v>318180</v>
+        <v>334089</v>
       </c>
     </row>
     <row r="1324">
@@ -14999,7 +14999,7 @@
         <v>1308</v>
       </c>
       <c r="C1324" t="n">
-        <v>146840</v>
+        <v>154182</v>
       </c>
     </row>
     <row r="1325">
@@ -15010,7 +15010,7 @@
         <v>2792</v>
       </c>
       <c r="C1325" t="n">
-        <v>105900</v>
+        <v>111195</v>
       </c>
     </row>
     <row r="1326">
@@ -15032,7 +15032,7 @@
         <v>2823</v>
       </c>
       <c r="C1327" t="n">
-        <v>85000</v>
+        <v>89250</v>
       </c>
     </row>
     <row r="1328">
@@ -15043,7 +15043,7 @@
         <v>2584</v>
       </c>
       <c r="C1328" t="n">
-        <v>57220</v>
+        <v>60081</v>
       </c>
     </row>
     <row r="1329">
@@ -15054,7 +15054,7 @@
         <v>945</v>
       </c>
       <c r="C1329" t="n">
-        <v>257560</v>
+        <v>270438</v>
       </c>
     </row>
     <row r="1330">
@@ -15065,7 +15065,7 @@
         <v>2660</v>
       </c>
       <c r="C1330" t="n">
-        <v>281800</v>
+        <v>295890</v>
       </c>
     </row>
     <row r="1331">
@@ -15076,7 +15076,7 @@
         <v>1317</v>
       </c>
       <c r="C1331" t="n">
-        <v>272720</v>
+        <v>286356</v>
       </c>
     </row>
     <row r="1332">
@@ -15087,7 +15087,7 @@
         <v>2790</v>
       </c>
       <c r="C1332" t="n">
-        <v>57900</v>
+        <v>60795</v>
       </c>
     </row>
     <row r="1333">
@@ -15098,7 +15098,7 @@
         <v>2711</v>
       </c>
       <c r="C1333" t="n">
-        <v>78807.28</v>
+        <v>82747.64</v>
       </c>
     </row>
     <row r="1334">
@@ -15109,7 +15109,7 @@
         <v>2607</v>
       </c>
       <c r="C1334" t="n">
-        <v>45167.28</v>
+        <v>47425.64</v>
       </c>
     </row>
     <row r="1335">
@@ -15120,7 +15120,7 @@
         <v>2667</v>
       </c>
       <c r="C1335" t="n">
-        <v>41545.46</v>
+        <v>43622.73</v>
       </c>
     </row>
     <row r="1336">
@@ -15131,7 +15131,7 @@
         <v>2706</v>
       </c>
       <c r="C1336" t="n">
-        <v>20029.1</v>
+        <v>21030.55</v>
       </c>
     </row>
     <row r="1337">
@@ -15142,7 +15142,7 @@
         <v>2657</v>
       </c>
       <c r="C1337" t="n">
-        <v>71996.38</v>
+        <v>75596.19</v>
       </c>
     </row>
     <row r="1338">
@@ -15153,7 +15153,7 @@
         <v>1278</v>
       </c>
       <c r="C1338" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1339">
@@ -15164,7 +15164,7 @@
         <v>2745</v>
       </c>
       <c r="C1339" t="n">
-        <v>100000</v>
+        <v>105000</v>
       </c>
     </row>
     <row r="1340">
@@ -15175,7 +15175,7 @@
         <v>2753</v>
       </c>
       <c r="C1340" t="n">
-        <v>68180</v>
+        <v>71589</v>
       </c>
     </row>
     <row r="1341">
@@ -15186,7 +15186,7 @@
         <v>2183</v>
       </c>
       <c r="C1341" t="n">
-        <v>332680</v>
+        <v>349314</v>
       </c>
     </row>
     <row r="1342">
@@ -15197,7 +15197,7 @@
         <v>1340</v>
       </c>
       <c r="C1342" t="n">
-        <v>131800</v>
+        <v>138390</v>
       </c>
     </row>
     <row r="1343">
@@ -15208,7 +15208,7 @@
         <v>2583</v>
       </c>
       <c r="C1343" t="n">
-        <v>37820</v>
+        <v>39711</v>
       </c>
     </row>
     <row r="1344">
@@ -15219,7 +15219,7 @@
         <v>2090</v>
       </c>
       <c r="C1344" t="n">
-        <v>37820</v>
+        <v>39711</v>
       </c>
     </row>
     <row r="1345">
@@ -15230,7 +15230,7 @@
         <v>1277</v>
       </c>
       <c r="C1345" t="n">
-        <v>200000</v>
+        <v>210000</v>
       </c>
     </row>
     <row r="1346">
@@ -15241,7 +15241,7 @@
         <v>1501</v>
       </c>
       <c r="C1346" t="n">
-        <v>86360</v>
+        <v>90678</v>
       </c>
     </row>
     <row r="1347">
@@ -15252,7 +15252,7 @@
         <v>703</v>
       </c>
       <c r="C1347" t="n">
-        <v>227260</v>
+        <v>238623</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:02:50
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1347"/>
+  <dimension ref="A1:C1373"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11289,10 +11289,10 @@
         <v>46266</v>
       </c>
       <c r="B987" t="n">
-        <v>931</v>
+        <v>2190</v>
       </c>
       <c r="C987" t="n">
-        <v>90132</v>
+        <v>225000</v>
       </c>
     </row>
     <row r="988">
@@ -11300,10 +11300,10 @@
         <v>46266</v>
       </c>
       <c r="B988" t="n">
-        <v>947</v>
+        <v>1466</v>
       </c>
       <c r="C988" t="n">
-        <v>414771</v>
+        <v>405000</v>
       </c>
     </row>
     <row r="989">
@@ -11311,10 +11311,10 @@
         <v>46266</v>
       </c>
       <c r="B989" t="n">
-        <v>1956</v>
+        <v>2659</v>
       </c>
       <c r="C989" t="n">
-        <v>240996</v>
+        <v>123018.07</v>
       </c>
     </row>
     <row r="990">
@@ -11322,10 +11322,10 @@
         <v>46266</v>
       </c>
       <c r="B990" t="n">
-        <v>2824</v>
+        <v>360</v>
       </c>
       <c r="C990" t="n">
-        <v>105000</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="991">
@@ -11333,10 +11333,10 @@
         <v>46266</v>
       </c>
       <c r="B991" t="n">
-        <v>2787</v>
+        <v>1063</v>
       </c>
       <c r="C991" t="n">
-        <v>124089</v>
+        <v>363550.99</v>
       </c>
     </row>
     <row r="992">
@@ -11344,10 +11344,10 @@
         <v>46266</v>
       </c>
       <c r="B992" t="n">
-        <v>2830</v>
+        <v>2273</v>
       </c>
       <c r="C992" t="n">
-        <v>85890</v>
+        <v>212081.7</v>
       </c>
     </row>
     <row r="993">
@@ -11355,10 +11355,10 @@
         <v>46266</v>
       </c>
       <c r="B993" t="n">
-        <v>1254</v>
+        <v>2757</v>
       </c>
       <c r="C993" t="n">
-        <v>185368.91</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="994">
@@ -11366,10 +11366,10 @@
         <v>46266</v>
       </c>
       <c r="B994" t="n">
-        <v>816</v>
+        <v>2795</v>
       </c>
       <c r="C994" t="n">
-        <v>255675</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="995">
@@ -11377,10 +11377,10 @@
         <v>46266</v>
       </c>
       <c r="B995" t="n">
-        <v>2671</v>
+        <v>2722</v>
       </c>
       <c r="C995" t="n">
-        <v>76356</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="996">
@@ -11388,10 +11388,10 @@
         <v>46266</v>
       </c>
       <c r="B996" t="n">
-        <v>2705</v>
+        <v>2718</v>
       </c>
       <c r="C996" t="n">
-        <v>171045</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="997">
@@ -11399,10 +11399,10 @@
         <v>46266</v>
       </c>
       <c r="B997" t="n">
-        <v>2333</v>
+        <v>595</v>
       </c>
       <c r="C997" t="n">
-        <v>147336</v>
+        <v>550000</v>
       </c>
     </row>
     <row r="998">
@@ -11410,10 +11410,10 @@
         <v>46266</v>
       </c>
       <c r="B998" t="n">
-        <v>2440</v>
+        <v>890</v>
       </c>
       <c r="C998" t="n">
-        <v>85890</v>
+        <v>700000</v>
       </c>
     </row>
     <row r="999">
@@ -11421,10 +11421,10 @@
         <v>46266</v>
       </c>
       <c r="B999" t="n">
-        <v>2448</v>
+        <v>2652</v>
       </c>
       <c r="C999" t="n">
-        <v>19089</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="1000">
@@ -11432,10 +11432,10 @@
         <v>46266</v>
       </c>
       <c r="B1000" t="n">
-        <v>2310</v>
+        <v>2714</v>
       </c>
       <c r="C1000" t="n">
-        <v>65562</v>
+        <v>360000</v>
       </c>
     </row>
     <row r="1001">
@@ -11443,10 +11443,10 @@
         <v>46266</v>
       </c>
       <c r="B1001" t="n">
-        <v>2809</v>
+        <v>1869</v>
       </c>
       <c r="C1001" t="n">
-        <v>65562</v>
+        <v>230000</v>
       </c>
     </row>
     <row r="1002">
@@ -11454,10 +11454,10 @@
         <v>46266</v>
       </c>
       <c r="B1002" t="n">
-        <v>2548</v>
+        <v>400</v>
       </c>
       <c r="C1002" t="n">
-        <v>55860</v>
+        <v>190000</v>
       </c>
     </row>
     <row r="1003">
@@ -11465,10 +11465,10 @@
         <v>46266</v>
       </c>
       <c r="B1003" t="n">
-        <v>451</v>
+        <v>1907</v>
       </c>
       <c r="C1003" t="n">
-        <v>229089</v>
+        <v>371004</v>
       </c>
     </row>
     <row r="1004">
@@ -11476,10 +11476,10 @@
         <v>46266</v>
       </c>
       <c r="B1004" t="n">
-        <v>933</v>
+        <v>1996</v>
       </c>
       <c r="C1004" t="n">
-        <v>77784</v>
+        <v>234500</v>
       </c>
     </row>
     <row r="1005">
@@ -11487,10 +11487,10 @@
         <v>46266</v>
       </c>
       <c r="B1005" t="n">
-        <v>2702</v>
+        <v>1890</v>
       </c>
       <c r="C1005" t="n">
-        <v>77784</v>
+        <v>316150.63</v>
       </c>
     </row>
     <row r="1006">
@@ -11498,10 +11498,10 @@
         <v>46266</v>
       </c>
       <c r="B1006" t="n">
-        <v>2549</v>
+        <v>2114</v>
       </c>
       <c r="C1006" t="n">
-        <v>27048</v>
+        <v>181834.85</v>
       </c>
     </row>
     <row r="1007">
@@ -11509,10 +11509,10 @@
         <v>46266</v>
       </c>
       <c r="B1007" t="n">
-        <v>535</v>
+        <v>2330</v>
       </c>
       <c r="C1007" t="n">
-        <v>353178</v>
+        <v>266920.09</v>
       </c>
     </row>
     <row r="1008">
@@ -11520,10 +11520,10 @@
         <v>46266</v>
       </c>
       <c r="B1008" t="n">
-        <v>1117</v>
+        <v>2000</v>
       </c>
       <c r="C1008" t="n">
-        <v>332073</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1009">
@@ -11531,7 +11531,7 @@
         <v>46266</v>
       </c>
       <c r="B1009" t="n">
-        <v>2109</v>
+        <v>2591</v>
       </c>
       <c r="C1009" t="n">
         <v>0</v>
@@ -11542,10 +11542,10 @@
         <v>46266</v>
       </c>
       <c r="B1010" t="n">
-        <v>530</v>
+        <v>2639</v>
       </c>
       <c r="C1010" t="n">
-        <v>232974</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1011">
@@ -11553,10 +11553,10 @@
         <v>46266</v>
       </c>
       <c r="B1011" t="n">
-        <v>358</v>
+        <v>2109</v>
       </c>
       <c r="C1011" t="n">
-        <v>324534</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1012">
@@ -11564,10 +11564,10 @@
         <v>46266</v>
       </c>
       <c r="B1012" t="n">
-        <v>2498</v>
+        <v>931</v>
       </c>
       <c r="C1012" t="n">
-        <v>53004</v>
+        <v>94424.85000000001</v>
       </c>
     </row>
     <row r="1013">
@@ -11575,10 +11575,10 @@
         <v>46266</v>
       </c>
       <c r="B1013" t="n">
-        <v>2381</v>
+        <v>1108</v>
       </c>
       <c r="C1013" t="n">
-        <v>75726</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1014">
@@ -11586,10 +11586,10 @@
         <v>46266</v>
       </c>
       <c r="B1014" t="n">
-        <v>2695</v>
+        <v>947</v>
       </c>
       <c r="C1014" t="n">
-        <v>45549</v>
+        <v>434540.65</v>
       </c>
     </row>
     <row r="1015">
@@ -11597,10 +11597,10 @@
         <v>46266</v>
       </c>
       <c r="B1015" t="n">
-        <v>2744</v>
+        <v>1956</v>
       </c>
       <c r="C1015" t="n">
-        <v>57272.73</v>
+        <v>252480.18</v>
       </c>
     </row>
     <row r="1016">
@@ -11608,10 +11608,10 @@
         <v>46266</v>
       </c>
       <c r="B1016" t="n">
-        <v>2750</v>
+        <v>2832</v>
       </c>
       <c r="C1016" t="n">
-        <v>57267</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="1017">
@@ -11619,10 +11619,10 @@
         <v>46266</v>
       </c>
       <c r="B1017" t="n">
-        <v>2131</v>
+        <v>1271</v>
       </c>
       <c r="C1017" t="n">
-        <v>114534</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1018">
@@ -11630,10 +11630,10 @@
         <v>46266</v>
       </c>
       <c r="B1018" t="n">
-        <v>818</v>
+        <v>2712</v>
       </c>
       <c r="C1018" t="n">
-        <v>381801</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1019">
@@ -11641,10 +11641,10 @@
         <v>46266</v>
       </c>
       <c r="B1019" t="n">
-        <v>2566</v>
+        <v>2824</v>
       </c>
       <c r="C1019" t="n">
-        <v>76356</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="1020">
@@ -11652,10 +11652,10 @@
         <v>46266</v>
       </c>
       <c r="B1020" t="n">
-        <v>132</v>
+        <v>2787</v>
       </c>
       <c r="C1020" t="n">
-        <v>715890</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="1021">
@@ -11663,10 +11663,10 @@
         <v>46266</v>
       </c>
       <c r="B1021" t="n">
-        <v>2431</v>
+        <v>2830</v>
       </c>
       <c r="C1021" t="n">
-        <v>175623</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="1022">
@@ -11674,10 +11674,10 @@
         <v>46266</v>
       </c>
       <c r="B1022" t="n">
-        <v>2249</v>
+        <v>2777</v>
       </c>
       <c r="C1022" t="n">
-        <v>186438</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1023">
@@ -11685,10 +11685,10 @@
         <v>46266</v>
       </c>
       <c r="B1023" t="n">
-        <v>1585</v>
+        <v>1254</v>
       </c>
       <c r="C1023" t="n">
-        <v>157542</v>
+        <v>194200</v>
       </c>
     </row>
     <row r="1024">
@@ -11696,10 +11696,10 @@
         <v>46266</v>
       </c>
       <c r="B1024" t="n">
-        <v>2325</v>
+        <v>816</v>
       </c>
       <c r="C1024" t="n">
-        <v>152292</v>
+        <v>267863</v>
       </c>
     </row>
     <row r="1025">
@@ -11707,10 +11707,10 @@
         <v>46266</v>
       </c>
       <c r="B1025" t="n">
-        <v>2190</v>
+        <v>2671</v>
       </c>
       <c r="C1025" t="n">
-        <v>214767</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="1026">
@@ -11718,10 +11718,10 @@
         <v>46266</v>
       </c>
       <c r="B1026" t="n">
-        <v>1466</v>
+        <v>2705</v>
       </c>
       <c r="C1026" t="n">
-        <v>386589</v>
+        <v>179192.41</v>
       </c>
     </row>
     <row r="1027">
@@ -11729,10 +11729,10 @@
         <v>46266</v>
       </c>
       <c r="B1027" t="n">
-        <v>2659</v>
+        <v>2333</v>
       </c>
       <c r="C1027" t="n">
-        <v>117411</v>
+        <v>154354.21</v>
       </c>
     </row>
     <row r="1028">
@@ -11740,10 +11740,10 @@
         <v>46266</v>
       </c>
       <c r="B1028" t="n">
-        <v>1384</v>
+        <v>2440</v>
       </c>
       <c r="C1028" t="n">
-        <v>429534</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="1029">
@@ -11751,10 +11751,10 @@
         <v>46266</v>
       </c>
       <c r="B1029" t="n">
-        <v>634</v>
+        <v>2448</v>
       </c>
       <c r="C1029" t="n">
-        <v>525000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="1030">
@@ -11762,10 +11762,10 @@
         <v>46266</v>
       </c>
       <c r="B1030" t="n">
-        <v>2804</v>
+        <v>2310</v>
       </c>
       <c r="C1030" t="n">
-        <v>95445</v>
+        <v>68705.64999999999</v>
       </c>
     </row>
     <row r="1031">
@@ -11773,10 +11773,10 @@
         <v>46266</v>
       </c>
       <c r="B1031" t="n">
-        <v>2375</v>
+        <v>2809</v>
       </c>
       <c r="C1031" t="n">
-        <v>315000</v>
+        <v>68705.64999999999</v>
       </c>
     </row>
     <row r="1032">
@@ -11784,10 +11784,10 @@
         <v>46266</v>
       </c>
       <c r="B1032" t="n">
-        <v>2601</v>
+        <v>2548</v>
       </c>
       <c r="C1032" t="n">
-        <v>262500</v>
+        <v>58526.51</v>
       </c>
     </row>
     <row r="1033">
@@ -11795,10 +11795,10 @@
         <v>46266</v>
       </c>
       <c r="B1033" t="n">
-        <v>952</v>
+        <v>451</v>
       </c>
       <c r="C1033" t="n">
-        <v>95445</v>
+        <v>240000</v>
       </c>
     </row>
     <row r="1034">
@@ -11806,10 +11806,10 @@
         <v>46266</v>
       </c>
       <c r="B1034" t="n">
-        <v>571</v>
+        <v>933</v>
       </c>
       <c r="C1034" t="n">
-        <v>607551</v>
+        <v>81489.46000000001</v>
       </c>
     </row>
     <row r="1035">
@@ -11817,10 +11817,10 @@
         <v>46266</v>
       </c>
       <c r="B1035" t="n">
-        <v>2697</v>
+        <v>2702</v>
       </c>
       <c r="C1035" t="n">
-        <v>185115</v>
+        <v>81489.46000000001</v>
       </c>
     </row>
     <row r="1036">
@@ -11828,10 +11828,10 @@
         <v>46266</v>
       </c>
       <c r="B1036" t="n">
-        <v>2678</v>
+        <v>2549</v>
       </c>
       <c r="C1036" t="n">
-        <v>320271</v>
+        <v>28353.8</v>
       </c>
     </row>
     <row r="1037">
@@ -11839,10 +11839,10 @@
         <v>46266</v>
       </c>
       <c r="B1037" t="n">
-        <v>2768</v>
+        <v>535</v>
       </c>
       <c r="C1037" t="n">
-        <v>335181</v>
+        <v>370000</v>
       </c>
     </row>
     <row r="1038">
@@ -11850,10 +11850,10 @@
         <v>46266</v>
       </c>
       <c r="B1038" t="n">
-        <v>2359</v>
+        <v>1117</v>
       </c>
       <c r="C1038" t="n">
-        <v>101661</v>
+        <v>347896.96</v>
       </c>
     </row>
     <row r="1039">
@@ -11861,10 +11861,10 @@
         <v>46266</v>
       </c>
       <c r="B1039" t="n">
-        <v>353</v>
+        <v>530</v>
       </c>
       <c r="C1039" t="n">
-        <v>330258.6</v>
+        <v>244071.88</v>
       </c>
     </row>
     <row r="1040">
@@ -11872,10 +11872,10 @@
         <v>46266</v>
       </c>
       <c r="B1040" t="n">
-        <v>2026</v>
+        <v>358</v>
       </c>
       <c r="C1040" t="n">
-        <v>273642.84</v>
+        <v>340000</v>
       </c>
     </row>
     <row r="1041">
@@ -11883,10 +11883,10 @@
         <v>46266</v>
       </c>
       <c r="B1041" t="n">
-        <v>1105</v>
+        <v>2498</v>
       </c>
       <c r="C1041" t="n">
-        <v>0</v>
+        <v>55536.48</v>
       </c>
     </row>
     <row r="1042">
@@ -11894,10 +11894,10 @@
         <v>46266</v>
       </c>
       <c r="B1042" t="n">
-        <v>2345</v>
+        <v>2381</v>
       </c>
       <c r="C1042" t="n">
-        <v>60081</v>
+        <v>79332.77</v>
       </c>
     </row>
     <row r="1043">
@@ -11905,10 +11905,10 @@
         <v>46266</v>
       </c>
       <c r="B1043" t="n">
-        <v>2789</v>
+        <v>2695</v>
       </c>
       <c r="C1043" t="n">
-        <v>162267</v>
+        <v>47738.38</v>
       </c>
     </row>
     <row r="1044">
@@ -11916,10 +11916,10 @@
         <v>46266</v>
       </c>
       <c r="B1044" t="n">
-        <v>569</v>
+        <v>2744</v>
       </c>
       <c r="C1044" t="n">
-        <v>2733738</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1045">
@@ -11927,10 +11927,10 @@
         <v>46266</v>
       </c>
       <c r="B1045" t="n">
-        <v>2822</v>
+        <v>2750</v>
       </c>
       <c r="C1045" t="n">
-        <v>128856</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1046">
@@ -11938,10 +11938,10 @@
         <v>46266</v>
       </c>
       <c r="B1046" t="n">
-        <v>2728</v>
+        <v>2131</v>
       </c>
       <c r="C1046" t="n">
-        <v>9534</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="1047">
@@ -11949,10 +11949,10 @@
         <v>46266</v>
       </c>
       <c r="B1047" t="n">
-        <v>2488</v>
+        <v>818</v>
       </c>
       <c r="C1047" t="n">
-        <v>95445</v>
+        <v>400000</v>
       </c>
     </row>
     <row r="1048">
@@ -11960,10 +11960,10 @@
         <v>46266</v>
       </c>
       <c r="B1048" t="n">
-        <v>2791</v>
+        <v>2566</v>
       </c>
       <c r="C1048" t="n">
-        <v>94204.10000000001</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="1049">
@@ -11971,10 +11971,10 @@
         <v>46266</v>
       </c>
       <c r="B1049" t="n">
-        <v>2577</v>
+        <v>132</v>
       </c>
       <c r="C1049" t="n">
-        <v>85116.91</v>
+        <v>750000</v>
       </c>
     </row>
     <row r="1050">
@@ -11982,10 +11982,10 @@
         <v>46266</v>
       </c>
       <c r="B1050" t="n">
-        <v>2069</v>
+        <v>2431</v>
       </c>
       <c r="C1050" t="n">
-        <v>171801</v>
+        <v>184000</v>
       </c>
     </row>
     <row r="1051">
@@ -11993,10 +11993,10 @@
         <v>46266</v>
       </c>
       <c r="B1051" t="n">
-        <v>2082</v>
+        <v>2249</v>
       </c>
       <c r="C1051" t="n">
-        <v>158991</v>
+        <v>195323.18</v>
       </c>
     </row>
     <row r="1052">
@@ -12004,10 +12004,10 @@
         <v>46266</v>
       </c>
       <c r="B1052" t="n">
-        <v>781</v>
+        <v>1585</v>
       </c>
       <c r="C1052" t="n">
-        <v>124089</v>
+        <v>165061.84</v>
       </c>
     </row>
     <row r="1053">
@@ -12015,10 +12015,10 @@
         <v>46266</v>
       </c>
       <c r="B1053" t="n">
-        <v>744</v>
+        <v>2325</v>
       </c>
       <c r="C1053" t="n">
-        <v>39711</v>
+        <v>159559.78</v>
       </c>
     </row>
     <row r="1054">
@@ -12026,10 +12026,10 @@
         <v>46266</v>
       </c>
       <c r="B1054" t="n">
-        <v>2223</v>
+        <v>2554</v>
       </c>
       <c r="C1054" t="n">
-        <v>125937</v>
+        <v>24555.46</v>
       </c>
     </row>
     <row r="1055">
@@ -12037,10 +12037,10 @@
         <v>46266</v>
       </c>
       <c r="B1055" t="n">
-        <v>2452</v>
+        <v>2556</v>
       </c>
       <c r="C1055" t="n">
-        <v>66801</v>
+        <v>36110.97</v>
       </c>
     </row>
     <row r="1056">
@@ -12048,10 +12048,10 @@
         <v>46266</v>
       </c>
       <c r="B1056" t="n">
-        <v>970</v>
+        <v>2546</v>
       </c>
       <c r="C1056" t="n">
-        <v>65562</v>
+        <v>23859.99</v>
       </c>
     </row>
     <row r="1057">
@@ -12059,10 +12059,10 @@
         <v>46266</v>
       </c>
       <c r="B1057" t="n">
-        <v>2550</v>
+        <v>42</v>
       </c>
       <c r="C1057" t="n">
-        <v>58212</v>
+        <v>1890000</v>
       </c>
     </row>
     <row r="1058">
@@ -12070,10 +12070,10 @@
         <v>46266</v>
       </c>
       <c r="B1058" t="n">
-        <v>768</v>
+        <v>953</v>
       </c>
       <c r="C1058" t="n">
-        <v>124089</v>
+        <v>682665.38</v>
       </c>
     </row>
     <row r="1059">
@@ -12081,10 +12081,10 @@
         <v>46266</v>
       </c>
       <c r="B1059" t="n">
-        <v>1075</v>
+        <v>1137</v>
       </c>
       <c r="C1059" t="n">
-        <v>432390</v>
+        <v>640000</v>
       </c>
     </row>
     <row r="1060">
@@ -12092,10 +12092,10 @@
         <v>46266</v>
       </c>
       <c r="B1060" t="n">
-        <v>664</v>
+        <v>675</v>
       </c>
       <c r="C1060" t="n">
-        <v>247212</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="1061">
@@ -12103,10 +12103,10 @@
         <v>46266</v>
       </c>
       <c r="B1061" t="n">
-        <v>2555</v>
+        <v>619</v>
       </c>
       <c r="C1061" t="n">
-        <v>39627</v>
+        <v>309241.74</v>
       </c>
     </row>
     <row r="1062">
@@ -12114,10 +12114,10 @@
         <v>46266</v>
       </c>
       <c r="B1062" t="n">
-        <v>2627</v>
+        <v>1299</v>
       </c>
       <c r="C1062" t="n">
-        <v>23268</v>
+        <v>520358.7</v>
       </c>
     </row>
     <row r="1063">
@@ -12125,10 +12125,10 @@
         <v>46266</v>
       </c>
       <c r="B1063" t="n">
-        <v>2557</v>
+        <v>1064</v>
       </c>
       <c r="C1063" t="n">
-        <v>24612</v>
+        <v>599374.29</v>
       </c>
     </row>
     <row r="1064">
@@ -12136,10 +12136,10 @@
         <v>46266</v>
       </c>
       <c r="B1064" t="n">
-        <v>2551</v>
+        <v>2308</v>
       </c>
       <c r="C1064" t="n">
-        <v>19551</v>
+        <v>205000</v>
       </c>
     </row>
     <row r="1065">
@@ -12147,10 +12147,10 @@
         <v>46266</v>
       </c>
       <c r="B1065" t="n">
-        <v>2463</v>
+        <v>2747</v>
       </c>
       <c r="C1065" t="n">
-        <v>305655</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1066">
@@ -12158,10 +12158,10 @@
         <v>46266</v>
       </c>
       <c r="B1066" t="n">
-        <v>2279</v>
+        <v>2819</v>
       </c>
       <c r="C1066" t="n">
-        <v>230601</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1067">
@@ -12169,10 +12169,10 @@
         <v>46266</v>
       </c>
       <c r="B1067" t="n">
-        <v>631</v>
+        <v>1259</v>
       </c>
       <c r="C1067" t="n">
-        <v>334089</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1068">
@@ -12180,10 +12180,10 @@
         <v>46266</v>
       </c>
       <c r="B1068" t="n">
-        <v>2251</v>
+        <v>2544</v>
       </c>
       <c r="C1068" t="n">
-        <v>204582</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="1069">
@@ -12191,10 +12191,10 @@
         <v>46266</v>
       </c>
       <c r="B1069" t="n">
-        <v>1653</v>
+        <v>2261</v>
       </c>
       <c r="C1069" t="n">
-        <v>310212</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="1070">
@@ -12202,10 +12202,10 @@
         <v>46266</v>
       </c>
       <c r="B1070" t="n">
-        <v>1293</v>
+        <v>2729</v>
       </c>
       <c r="C1070" t="n">
-        <v>396123</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="1071">
@@ -12213,10 +12213,10 @@
         <v>46266</v>
       </c>
       <c r="B1071" t="n">
-        <v>360</v>
+        <v>2649</v>
       </c>
       <c r="C1071" t="n">
-        <v>477267</v>
+        <v>29530.75</v>
       </c>
     </row>
     <row r="1072">
@@ -12224,10 +12224,10 @@
         <v>46266</v>
       </c>
       <c r="B1072" t="n">
-        <v>1063</v>
+        <v>2494</v>
       </c>
       <c r="C1072" t="n">
-        <v>347025</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="1073">
@@ -12235,10 +12235,10 @@
         <v>46266</v>
       </c>
       <c r="B1073" t="n">
-        <v>2273</v>
+        <v>1384</v>
       </c>
       <c r="C1073" t="n">
-        <v>202440</v>
+        <v>450000</v>
       </c>
     </row>
     <row r="1074">
@@ -12246,10 +12246,10 @@
         <v>46266</v>
       </c>
       <c r="B1074" t="n">
-        <v>2757</v>
+        <v>634</v>
       </c>
       <c r="C1074" t="n">
-        <v>66818.19</v>
+        <v>550000</v>
       </c>
     </row>
     <row r="1075">
@@ -12257,10 +12257,10 @@
         <v>46266</v>
       </c>
       <c r="B1075" t="n">
-        <v>2795</v>
+        <v>2804</v>
       </c>
       <c r="C1075" t="n">
-        <v>57272.73</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1076">
@@ -12268,10 +12268,10 @@
         <v>46266</v>
       </c>
       <c r="B1076" t="n">
-        <v>2722</v>
+        <v>2375</v>
       </c>
       <c r="C1076" t="n">
-        <v>57267</v>
+        <v>330000</v>
       </c>
     </row>
     <row r="1077">
@@ -12279,10 +12279,10 @@
         <v>46266</v>
       </c>
       <c r="B1077" t="n">
-        <v>2718</v>
+        <v>2601</v>
       </c>
       <c r="C1077" t="n">
-        <v>76356</v>
+        <v>275000</v>
       </c>
     </row>
     <row r="1078">
@@ -12290,10 +12290,10 @@
         <v>46266</v>
       </c>
       <c r="B1078" t="n">
-        <v>595</v>
+        <v>952</v>
       </c>
       <c r="C1078" t="n">
-        <v>525000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1079">
@@ -12301,10 +12301,10 @@
         <v>46266</v>
       </c>
       <c r="B1079" t="n">
-        <v>890</v>
+        <v>571</v>
       </c>
       <c r="C1079" t="n">
-        <v>668178</v>
+        <v>636500</v>
       </c>
     </row>
     <row r="1080">
@@ -12312,10 +12312,10 @@
         <v>46266</v>
       </c>
       <c r="B1080" t="n">
-        <v>2652</v>
+        <v>2697</v>
       </c>
       <c r="C1080" t="n">
-        <v>124089</v>
+        <v>192075.77</v>
       </c>
     </row>
     <row r="1081">
@@ -12323,10 +12323,10 @@
         <v>46266</v>
       </c>
       <c r="B1081" t="n">
-        <v>2714</v>
+        <v>2678</v>
       </c>
       <c r="C1081" t="n">
-        <v>343623</v>
+        <v>335540.59</v>
       </c>
     </row>
     <row r="1082">
@@ -12334,10 +12334,10 @@
         <v>46266</v>
       </c>
       <c r="B1082" t="n">
-        <v>1869</v>
+        <v>2768</v>
       </c>
       <c r="C1082" t="n">
-        <v>219534</v>
+        <v>349289.06</v>
       </c>
     </row>
     <row r="1083">
@@ -12345,10 +12345,10 @@
         <v>46266</v>
       </c>
       <c r="B1083" t="n">
-        <v>400</v>
+        <v>2359</v>
       </c>
       <c r="C1083" t="n">
-        <v>181356</v>
+        <v>104635.75</v>
       </c>
     </row>
     <row r="1084">
@@ -12356,10 +12356,10 @@
         <v>46266</v>
       </c>
       <c r="B1084" t="n">
-        <v>1907</v>
+        <v>353</v>
       </c>
       <c r="C1084" t="n">
-        <v>354123</v>
+        <v>345985.19</v>
       </c>
     </row>
     <row r="1085">
@@ -12367,10 +12367,10 @@
         <v>46266</v>
       </c>
       <c r="B1085" t="n">
-        <v>1996</v>
+        <v>2026</v>
       </c>
       <c r="C1085" t="n">
-        <v>223839</v>
+        <v>286673.45</v>
       </c>
     </row>
     <row r="1086">
@@ -12378,10 +12378,10 @@
         <v>46266</v>
       </c>
       <c r="B1086" t="n">
-        <v>1890</v>
+        <v>1105</v>
       </c>
       <c r="C1086" t="n">
-        <v>301772.52</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1087">
@@ -12389,10 +12389,10 @@
         <v>46266</v>
       </c>
       <c r="B1087" t="n">
-        <v>2114</v>
+        <v>2345</v>
       </c>
       <c r="C1087" t="n">
-        <v>175350</v>
+        <v>62949.9</v>
       </c>
     </row>
     <row r="1088">
@@ -12400,10 +12400,10 @@
         <v>46266</v>
       </c>
       <c r="B1088" t="n">
-        <v>2330</v>
+        <v>2789</v>
       </c>
       <c r="C1088" t="n">
-        <v>256557</v>
+        <v>170000</v>
       </c>
     </row>
     <row r="1089">
@@ -12411,10 +12411,10 @@
         <v>46266</v>
       </c>
       <c r="B1089" t="n">
-        <v>2000</v>
+        <v>569</v>
       </c>
       <c r="C1089" t="n">
-        <v>0</v>
+        <v>2863931.44</v>
       </c>
     </row>
     <row r="1090">
@@ -12422,7 +12422,7 @@
         <v>46266</v>
       </c>
       <c r="B1090" t="n">
-        <v>2591</v>
+        <v>2680</v>
       </c>
       <c r="C1090" t="n">
         <v>0</v>
@@ -12433,10 +12433,10 @@
         <v>46266</v>
       </c>
       <c r="B1091" t="n">
-        <v>2639</v>
+        <v>2822</v>
       </c>
       <c r="C1091" t="n">
-        <v>0</v>
+        <v>135000</v>
       </c>
     </row>
     <row r="1092">
@@ -12444,10 +12444,10 @@
         <v>46266</v>
       </c>
       <c r="B1092" t="n">
-        <v>2629</v>
+        <v>2728</v>
       </c>
       <c r="C1092" t="n">
-        <v>65562</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="1093">
@@ -12455,10 +12455,10 @@
         <v>46266</v>
       </c>
       <c r="B1093" t="n">
-        <v>951</v>
+        <v>2738</v>
       </c>
       <c r="C1093" t="n">
-        <v>109767</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1094">
@@ -12466,10 +12466,10 @@
         <v>46266</v>
       </c>
       <c r="B1094" t="n">
-        <v>2449</v>
+        <v>2488</v>
       </c>
       <c r="C1094" t="n">
-        <v>38178</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1095">
@@ -12477,10 +12477,10 @@
         <v>46266</v>
       </c>
       <c r="B1095" t="n">
-        <v>610</v>
+        <v>2791</v>
       </c>
       <c r="C1095" t="n">
-        <v>777945</v>
+        <v>98700</v>
       </c>
     </row>
     <row r="1096">
@@ -12488,10 +12488,10 @@
         <v>46266</v>
       </c>
       <c r="B1096" t="n">
-        <v>2761</v>
+        <v>2577</v>
       </c>
       <c r="C1096" t="n">
-        <v>77784</v>
+        <v>89186.09</v>
       </c>
     </row>
     <row r="1097">
@@ -12499,10 +12499,10 @@
         <v>46266</v>
       </c>
       <c r="B1097" t="n">
-        <v>483</v>
+        <v>2069</v>
       </c>
       <c r="C1097" t="n">
-        <v>422856</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="1098">
@@ -12510,10 +12510,10 @@
         <v>46266</v>
       </c>
       <c r="B1098" t="n">
-        <v>2015</v>
+        <v>2082</v>
       </c>
       <c r="C1098" t="n">
-        <v>353178</v>
+        <v>166573.23</v>
       </c>
     </row>
     <row r="1099">
@@ -12521,10 +12521,10 @@
         <v>46266</v>
       </c>
       <c r="B1099" t="n">
-        <v>1478</v>
+        <v>781</v>
       </c>
       <c r="C1099" t="n">
-        <v>516558</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="1100">
@@ -12532,10 +12532,10 @@
         <v>46266</v>
       </c>
       <c r="B1100" t="n">
-        <v>424</v>
+        <v>744</v>
       </c>
       <c r="C1100" t="n">
-        <v>230601</v>
+        <v>41610.33</v>
       </c>
     </row>
     <row r="1101">
@@ -12543,10 +12543,10 @@
         <v>46266</v>
       </c>
       <c r="B1101" t="n">
-        <v>1261</v>
+        <v>2223</v>
       </c>
       <c r="C1101" t="n">
-        <v>0</v>
+        <v>131947.96</v>
       </c>
     </row>
     <row r="1102">
@@ -12554,10 +12554,10 @@
         <v>46266</v>
       </c>
       <c r="B1102" t="n">
-        <v>477</v>
+        <v>2452</v>
       </c>
       <c r="C1102" t="n">
-        <v>246897</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="1103">
@@ -12565,10 +12565,10 @@
         <v>46266</v>
       </c>
       <c r="B1103" t="n">
-        <v>1810</v>
+        <v>970</v>
       </c>
       <c r="C1103" t="n">
-        <v>38241</v>
+        <v>68705.64999999999</v>
       </c>
     </row>
     <row r="1104">
@@ -12576,10 +12576,10 @@
         <v>46266</v>
       </c>
       <c r="B1104" t="n">
-        <v>2826</v>
+        <v>2550</v>
       </c>
       <c r="C1104" t="n">
-        <v>66818.19</v>
+        <v>60987.41</v>
       </c>
     </row>
     <row r="1105">
@@ -12587,10 +12587,10 @@
         <v>46266</v>
       </c>
       <c r="B1105" t="n">
-        <v>2561</v>
+        <v>768</v>
       </c>
       <c r="C1105" t="n">
-        <v>14028</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="1106">
@@ -12598,10 +12598,10 @@
         <v>46266</v>
       </c>
       <c r="B1106" t="n">
-        <v>2653</v>
+        <v>1075</v>
       </c>
       <c r="C1106" t="n">
-        <v>57272.73</v>
+        <v>453000</v>
       </c>
     </row>
     <row r="1107">
@@ -12609,10 +12609,10 @@
         <v>46266</v>
       </c>
       <c r="B1107" t="n">
-        <v>2829</v>
+        <v>664</v>
       </c>
       <c r="C1107" t="n">
-        <v>57272.73</v>
+        <v>259000</v>
       </c>
     </row>
     <row r="1108">
@@ -12620,10 +12620,10 @@
         <v>46266</v>
       </c>
       <c r="B1108" t="n">
-        <v>2643</v>
+        <v>2555</v>
       </c>
       <c r="C1108" t="n">
-        <v>28182</v>
+        <v>41514.24</v>
       </c>
     </row>
     <row r="1109">
@@ -12631,10 +12631,10 @@
         <v>46266</v>
       </c>
       <c r="B1109" t="n">
-        <v>2794</v>
+        <v>2627</v>
       </c>
       <c r="C1109" t="n">
-        <v>85890</v>
+        <v>24394.96</v>
       </c>
     </row>
     <row r="1110">
@@ -12642,10 +12642,10 @@
         <v>46266</v>
       </c>
       <c r="B1110" t="n">
-        <v>2655</v>
+        <v>2557</v>
       </c>
       <c r="C1110" t="n">
-        <v>105000</v>
+        <v>25785.9</v>
       </c>
     </row>
     <row r="1111">
@@ -12653,10 +12653,10 @@
         <v>46266</v>
       </c>
       <c r="B1111" t="n">
-        <v>1456</v>
+        <v>2551</v>
       </c>
       <c r="C1111" t="n">
-        <v>735273</v>
+        <v>20489.63</v>
       </c>
     </row>
     <row r="1112">
@@ -12664,10 +12664,10 @@
         <v>46266</v>
       </c>
       <c r="B1112" t="n">
-        <v>2606</v>
+        <v>2463</v>
       </c>
       <c r="C1112" t="n">
-        <v>225834</v>
+        <v>320224.87</v>
       </c>
     </row>
     <row r="1113">
@@ -12675,10 +12675,10 @@
         <v>46266</v>
       </c>
       <c r="B1113" t="n">
-        <v>1142</v>
+        <v>2279</v>
       </c>
       <c r="C1113" t="n">
-        <v>409542</v>
+        <v>241595.11</v>
       </c>
     </row>
     <row r="1114">
@@ -12686,10 +12686,10 @@
         <v>46266</v>
       </c>
       <c r="B1114" t="n">
-        <v>1450</v>
+        <v>631</v>
       </c>
       <c r="C1114" t="n">
-        <v>260169</v>
+        <v>350000</v>
       </c>
     </row>
     <row r="1115">
@@ -12697,10 +12697,10 @@
         <v>46266</v>
       </c>
       <c r="B1115" t="n">
-        <v>2133</v>
+        <v>2251</v>
       </c>
       <c r="C1115" t="n">
-        <v>607551</v>
+        <v>214342.76</v>
       </c>
     </row>
     <row r="1116">
@@ -12708,10 +12708,10 @@
         <v>46266</v>
       </c>
       <c r="B1116" t="n">
-        <v>522</v>
+        <v>1653</v>
       </c>
       <c r="C1116" t="n">
-        <v>186123</v>
+        <v>325000</v>
       </c>
     </row>
     <row r="1117">
@@ -12719,10 +12719,10 @@
         <v>46266</v>
       </c>
       <c r="B1117" t="n">
-        <v>2696</v>
+        <v>1293</v>
       </c>
       <c r="C1117" t="n">
-        <v>251160</v>
+        <v>415000</v>
       </c>
     </row>
     <row r="1118">
@@ -12730,10 +12730,10 @@
         <v>46266</v>
       </c>
       <c r="B1118" t="n">
-        <v>2693</v>
+        <v>767</v>
       </c>
       <c r="C1118" t="n">
-        <v>0</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="1119">
@@ -12741,10 +12741,10 @@
         <v>46266</v>
       </c>
       <c r="B1119" t="n">
-        <v>2692</v>
+        <v>2687</v>
       </c>
       <c r="C1119" t="n">
-        <v>71589</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1120">
@@ -12752,10 +12752,10 @@
         <v>46266</v>
       </c>
       <c r="B1120" t="n">
-        <v>2691</v>
+        <v>2648</v>
       </c>
       <c r="C1120" t="n">
-        <v>128856</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1121">
@@ -12763,10 +12763,10 @@
         <v>46266</v>
       </c>
       <c r="B1121" t="n">
-        <v>1632</v>
+        <v>2686</v>
       </c>
       <c r="C1121" t="n">
-        <v>238623</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="1122">
@@ -12774,10 +12774,10 @@
         <v>46266</v>
       </c>
       <c r="B1122" t="n">
-        <v>2641</v>
+        <v>2730</v>
       </c>
       <c r="C1122" t="n">
-        <v>76356</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="1123">
@@ -12785,10 +12785,10 @@
         <v>46266</v>
       </c>
       <c r="B1123" t="n">
-        <v>2197</v>
+        <v>2760</v>
       </c>
       <c r="C1123" t="n">
-        <v>190890</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1124">
@@ -12796,10 +12796,10 @@
         <v>46266</v>
       </c>
       <c r="B1124" t="n">
-        <v>609</v>
+        <v>2776</v>
       </c>
       <c r="C1124" t="n">
-        <v>210000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1125">
@@ -12807,10 +12807,10 @@
         <v>46266</v>
       </c>
       <c r="B1125" t="n">
-        <v>1380</v>
+        <v>2778</v>
       </c>
       <c r="C1125" t="n">
-        <v>95445</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1126">
@@ -12818,10 +12818,10 @@
         <v>46266</v>
       </c>
       <c r="B1126" t="n">
-        <v>104</v>
+        <v>2580</v>
       </c>
       <c r="C1126" t="n">
-        <v>286356</v>
+        <v>33550</v>
       </c>
     </row>
     <row r="1127">
@@ -12829,10 +12829,10 @@
         <v>46266</v>
       </c>
       <c r="B1127" t="n">
-        <v>2621</v>
+        <v>2472</v>
       </c>
       <c r="C1127" t="n">
-        <v>66801</v>
+        <v>52950</v>
       </c>
     </row>
     <row r="1128">
@@ -12840,10 +12840,10 @@
         <v>46266</v>
       </c>
       <c r="B1128" t="n">
-        <v>2786</v>
+        <v>2631</v>
       </c>
       <c r="C1128" t="n">
-        <v>66801</v>
+        <v>24550</v>
       </c>
     </row>
     <row r="1129">
@@ -12851,10 +12851,10 @@
         <v>46266</v>
       </c>
       <c r="B1129" t="n">
-        <v>2784</v>
+        <v>1642</v>
       </c>
       <c r="C1129" t="n">
-        <v>39711</v>
+        <v>265000</v>
       </c>
     </row>
     <row r="1130">
@@ -12862,10 +12862,10 @@
         <v>46266</v>
       </c>
       <c r="B1130" t="n">
-        <v>2586</v>
+        <v>2613</v>
       </c>
       <c r="C1130" t="n">
-        <v>39711</v>
+        <v>179192.41</v>
       </c>
     </row>
     <row r="1131">
@@ -12873,10 +12873,10 @@
         <v>46266</v>
       </c>
       <c r="B1131" t="n">
-        <v>2145</v>
+        <v>1020</v>
       </c>
       <c r="C1131" t="n">
-        <v>123564</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="1132">
@@ -12884,10 +12884,10 @@
         <v>46266</v>
       </c>
       <c r="B1132" t="n">
-        <v>2574</v>
+        <v>2785</v>
       </c>
       <c r="C1132" t="n">
-        <v>123564</v>
+        <v>41610.33</v>
       </c>
     </row>
     <row r="1133">
@@ -12895,10 +12895,10 @@
         <v>46266</v>
       </c>
       <c r="B1133" t="n">
-        <v>2492</v>
+        <v>1327</v>
       </c>
       <c r="C1133" t="n">
-        <v>135450</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1134">
@@ -12906,10 +12906,10 @@
         <v>46266</v>
       </c>
       <c r="B1134" t="n">
-        <v>629</v>
+        <v>2629</v>
       </c>
       <c r="C1134" t="n">
-        <v>421890</v>
+        <v>68705.63</v>
       </c>
     </row>
     <row r="1135">
@@ -12917,10 +12917,10 @@
         <v>46266</v>
       </c>
       <c r="B1135" t="n">
-        <v>966</v>
+        <v>951</v>
       </c>
       <c r="C1135" t="n">
-        <v>77784</v>
+        <v>115000</v>
       </c>
     </row>
     <row r="1136">
@@ -12928,10 +12928,10 @@
         <v>46266</v>
       </c>
       <c r="B1136" t="n">
-        <v>2721</v>
+        <v>2449</v>
       </c>
       <c r="C1136" t="n">
-        <v>77784</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="1137">
@@ -12939,10 +12939,10 @@
         <v>46266</v>
       </c>
       <c r="B1137" t="n">
-        <v>2554</v>
+        <v>610</v>
       </c>
       <c r="C1137" t="n">
-        <v>23436</v>
+        <v>815000</v>
       </c>
     </row>
     <row r="1138">
@@ -12950,10 +12950,10 @@
         <v>46266</v>
       </c>
       <c r="B1138" t="n">
-        <v>2556</v>
+        <v>2761</v>
       </c>
       <c r="C1138" t="n">
-        <v>34461</v>
+        <v>81489.46000000001</v>
       </c>
     </row>
     <row r="1139">
@@ -12961,10 +12961,10 @@
         <v>46266</v>
       </c>
       <c r="B1139" t="n">
-        <v>2546</v>
+        <v>483</v>
       </c>
       <c r="C1139" t="n">
-        <v>22764</v>
+        <v>443000</v>
       </c>
     </row>
     <row r="1140">
@@ -12972,10 +12972,10 @@
         <v>46266</v>
       </c>
       <c r="B1140" t="n">
-        <v>42</v>
+        <v>2015</v>
       </c>
       <c r="C1140" t="n">
-        <v>1804089</v>
+        <v>370000</v>
       </c>
     </row>
     <row r="1141">
@@ -12983,10 +12983,10 @@
         <v>46266</v>
       </c>
       <c r="B1141" t="n">
-        <v>953</v>
+        <v>1478</v>
       </c>
       <c r="C1141" t="n">
-        <v>651630</v>
+        <v>541173.05</v>
       </c>
     </row>
     <row r="1142">
@@ -12994,10 +12994,10 @@
         <v>46266</v>
       </c>
       <c r="B1142" t="n">
-        <v>1137</v>
+        <v>424</v>
       </c>
       <c r="C1142" t="n">
-        <v>610890</v>
+        <v>241595.11</v>
       </c>
     </row>
     <row r="1143">
@@ -13005,10 +13005,10 @@
         <v>46266</v>
       </c>
       <c r="B1143" t="n">
-        <v>675</v>
+        <v>1261</v>
       </c>
       <c r="C1143" t="n">
-        <v>190890</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1144">
@@ -13016,10 +13016,10 @@
         <v>46266</v>
       </c>
       <c r="B1144" t="n">
-        <v>619</v>
+        <v>477</v>
       </c>
       <c r="C1144" t="n">
-        <v>295176</v>
+        <v>258659.79</v>
       </c>
     </row>
     <row r="1145">
@@ -13027,10 +13027,10 @@
         <v>46266</v>
       </c>
       <c r="B1145" t="n">
-        <v>1299</v>
+        <v>1810</v>
       </c>
       <c r="C1145" t="n">
-        <v>496692</v>
+        <v>40077.59</v>
       </c>
     </row>
     <row r="1146">
@@ -13038,10 +13038,10 @@
         <v>46266</v>
       </c>
       <c r="B1146" t="n">
-        <v>1064</v>
+        <v>2826</v>
       </c>
       <c r="C1146" t="n">
-        <v>572124</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="1147">
@@ -13049,10 +13049,10 @@
         <v>46266</v>
       </c>
       <c r="B1147" t="n">
-        <v>2308</v>
+        <v>2561</v>
       </c>
       <c r="C1147" t="n">
-        <v>195678</v>
+        <v>14711.88</v>
       </c>
     </row>
     <row r="1148">
@@ -13060,10 +13060,10 @@
         <v>46266</v>
       </c>
       <c r="B1148" t="n">
-        <v>2747</v>
+        <v>2653</v>
       </c>
       <c r="C1148" t="n">
-        <v>57272.73</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1149">
@@ -13071,10 +13071,10 @@
         <v>46266</v>
       </c>
       <c r="B1149" t="n">
-        <v>2819</v>
+        <v>2829</v>
       </c>
       <c r="C1149" t="n">
-        <v>57272.73</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1150">
@@ -13082,10 +13082,10 @@
         <v>46266</v>
       </c>
       <c r="B1150" t="n">
-        <v>1259</v>
+        <v>2643</v>
       </c>
       <c r="C1150" t="n">
-        <v>95454.55</v>
+        <v>29530.75</v>
       </c>
     </row>
     <row r="1151">
@@ -13093,10 +13093,10 @@
         <v>46266</v>
       </c>
       <c r="B1151" t="n">
-        <v>2544</v>
+        <v>2794</v>
       </c>
       <c r="C1151" t="n">
-        <v>76356</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="1152">
@@ -13104,10 +13104,10 @@
         <v>46266</v>
       </c>
       <c r="B1152" t="n">
-        <v>2261</v>
+        <v>2655</v>
       </c>
       <c r="C1152" t="n">
-        <v>143178</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="1153">
@@ -13115,10 +13115,10 @@
         <v>46266</v>
       </c>
       <c r="B1153" t="n">
-        <v>2729</v>
+        <v>1456</v>
       </c>
       <c r="C1153" t="n">
-        <v>76356</v>
+        <v>770288.58</v>
       </c>
     </row>
     <row r="1154">
@@ -13126,10 +13126,10 @@
         <v>46266</v>
       </c>
       <c r="B1154" t="n">
-        <v>2649</v>
+        <v>2606</v>
       </c>
       <c r="C1154" t="n">
-        <v>28182</v>
+        <v>236588.64</v>
       </c>
     </row>
     <row r="1155">
@@ -13137,10 +13137,10 @@
         <v>46266</v>
       </c>
       <c r="B1155" t="n">
-        <v>2494</v>
+        <v>1142</v>
       </c>
       <c r="C1155" t="n">
-        <v>124089</v>
+        <v>429052.25</v>
       </c>
     </row>
     <row r="1156">
@@ -13148,10 +13148,10 @@
         <v>46266</v>
       </c>
       <c r="B1156" t="n">
-        <v>2633</v>
+        <v>1450</v>
       </c>
       <c r="C1156" t="n">
-        <v>0</v>
+        <v>272574.37</v>
       </c>
     </row>
     <row r="1157">
@@ -13159,10 +13159,10 @@
         <v>46266</v>
       </c>
       <c r="B1157" t="n">
-        <v>2802</v>
+        <v>2133</v>
       </c>
       <c r="C1157" t="n">
-        <v>67599</v>
+        <v>636500</v>
       </c>
     </row>
     <row r="1158">
@@ -13170,10 +13170,10 @@
         <v>46266</v>
       </c>
       <c r="B1158" t="n">
-        <v>2726</v>
+        <v>522</v>
       </c>
       <c r="C1158" t="n">
-        <v>143178</v>
+        <v>195000</v>
       </c>
     </row>
     <row r="1159">
@@ -13181,10 +13181,10 @@
         <v>46266</v>
       </c>
       <c r="B1159" t="n">
-        <v>2820</v>
+        <v>2696</v>
       </c>
       <c r="C1159" t="n">
-        <v>171801</v>
+        <v>261273.45</v>
       </c>
     </row>
     <row r="1160">
@@ -13192,10 +13192,10 @@
         <v>46266</v>
       </c>
       <c r="B1160" t="n">
-        <v>1007</v>
+        <v>2693</v>
       </c>
       <c r="C1160" t="n">
-        <v>181356</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1161">
@@ -13203,10 +13203,10 @@
         <v>46266</v>
       </c>
       <c r="B1161" t="n">
-        <v>20</v>
+        <v>2692</v>
       </c>
       <c r="C1161" t="n">
-        <v>367500</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="1162">
@@ -13214,10 +13214,10 @@
         <v>46266</v>
       </c>
       <c r="B1162" t="n">
-        <v>1372</v>
+        <v>2691</v>
       </c>
       <c r="C1162" t="n">
-        <v>276801</v>
+        <v>135000</v>
       </c>
     </row>
     <row r="1163">
@@ -13225,10 +13225,10 @@
         <v>46266</v>
       </c>
       <c r="B1163" t="n">
-        <v>2735</v>
+        <v>1632</v>
       </c>
       <c r="C1163" t="n">
-        <v>114534</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="1164">
@@ -13236,10 +13236,10 @@
         <v>46266</v>
       </c>
       <c r="B1164" t="n">
-        <v>2811</v>
+        <v>2641</v>
       </c>
       <c r="C1164" t="n">
-        <v>39711</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1165">
@@ -13247,10 +13247,10 @@
         <v>46266</v>
       </c>
       <c r="B1165" t="n">
-        <v>1871</v>
+        <v>2197</v>
       </c>
       <c r="C1165" t="n">
-        <v>168714</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="1166">
@@ -13258,10 +13258,10 @@
         <v>46266</v>
       </c>
       <c r="B1166" t="n">
-        <v>2541</v>
+        <v>2185</v>
       </c>
       <c r="C1166" t="n">
-        <v>201978</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1167">
@@ -13269,10 +13269,10 @@
         <v>46266</v>
       </c>
       <c r="B1167" t="n">
-        <v>2362</v>
+        <v>2710</v>
       </c>
       <c r="C1167" t="n">
-        <v>71589</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1168">
@@ -13280,10 +13280,10 @@
         <v>46266</v>
       </c>
       <c r="B1168" t="n">
-        <v>1324</v>
+        <v>2708</v>
       </c>
       <c r="C1168" t="n">
-        <v>267267</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1169">
@@ -13291,10 +13291,10 @@
         <v>46266</v>
       </c>
       <c r="B1169" t="n">
-        <v>2323</v>
+        <v>609</v>
       </c>
       <c r="C1169" t="n">
-        <v>65562</v>
+        <v>220000</v>
       </c>
     </row>
     <row r="1170">
@@ -13302,10 +13302,10 @@
         <v>46266</v>
       </c>
       <c r="B1170" t="n">
-        <v>2647</v>
+        <v>1380</v>
       </c>
       <c r="C1170" t="n">
-        <v>135450</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1171">
@@ -13313,10 +13313,10 @@
         <v>46266</v>
       </c>
       <c r="B1171" t="n">
-        <v>559</v>
+        <v>104</v>
       </c>
       <c r="C1171" t="n">
-        <v>219009</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="1172">
@@ -13324,10 +13324,10 @@
         <v>46266</v>
       </c>
       <c r="B1172" t="n">
-        <v>2762</v>
+        <v>2621</v>
       </c>
       <c r="C1172" t="n">
-        <v>77784</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="1173">
@@ -13335,10 +13335,10 @@
         <v>46266</v>
       </c>
       <c r="B1173" t="n">
-        <v>2501</v>
+        <v>2786</v>
       </c>
       <c r="C1173" t="n">
-        <v>77784</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="1174">
@@ -13346,10 +13346,10 @@
         <v>46266</v>
       </c>
       <c r="B1174" t="n">
-        <v>2562</v>
+        <v>2784</v>
       </c>
       <c r="C1174" t="n">
-        <v>15099</v>
+        <v>41610.33</v>
       </c>
     </row>
     <row r="1175">
@@ -13357,10 +13357,10 @@
         <v>46266</v>
       </c>
       <c r="B1175" t="n">
-        <v>429</v>
+        <v>2586</v>
       </c>
       <c r="C1175" t="n">
-        <v>372267</v>
+        <v>41610.33</v>
       </c>
     </row>
     <row r="1176">
@@ -13368,10 +13368,10 @@
         <v>46266</v>
       </c>
       <c r="B1176" t="n">
-        <v>58</v>
+        <v>2145</v>
       </c>
       <c r="C1176" t="n">
-        <v>258279</v>
+        <v>129458.37</v>
       </c>
     </row>
     <row r="1177">
@@ -13379,10 +13379,10 @@
         <v>46266</v>
       </c>
       <c r="B1177" t="n">
-        <v>2245</v>
+        <v>2574</v>
       </c>
       <c r="C1177" t="n">
-        <v>230601</v>
+        <v>129458.37</v>
       </c>
     </row>
     <row r="1178">
@@ -13390,10 +13390,10 @@
         <v>46266</v>
       </c>
       <c r="B1178" t="n">
-        <v>285</v>
+        <v>2492</v>
       </c>
       <c r="C1178" t="n">
-        <v>516558</v>
+        <v>141906.29</v>
       </c>
     </row>
     <row r="1179">
@@ -13401,10 +13401,10 @@
         <v>46266</v>
       </c>
       <c r="B1179" t="n">
-        <v>1464</v>
+        <v>629</v>
       </c>
       <c r="C1179" t="n">
-        <v>0</v>
+        <v>442000</v>
       </c>
     </row>
     <row r="1180">
@@ -13412,10 +13412,10 @@
         <v>46266</v>
       </c>
       <c r="B1180" t="n">
-        <v>363</v>
+        <v>966</v>
       </c>
       <c r="C1180" t="n">
-        <v>286356</v>
+        <v>81489.46000000001</v>
       </c>
     </row>
     <row r="1181">
@@ -13423,10 +13423,10 @@
         <v>46266</v>
       </c>
       <c r="B1181" t="n">
-        <v>2651</v>
+        <v>2721</v>
       </c>
       <c r="C1181" t="n">
-        <v>161427</v>
+        <v>81489.46000000001</v>
       </c>
     </row>
     <row r="1182">
@@ -13434,10 +13434,10 @@
         <v>46266</v>
       </c>
       <c r="B1182" t="n">
-        <v>2142</v>
+        <v>2635</v>
       </c>
       <c r="C1182" t="n">
-        <v>50946</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="1183">
@@ -13445,10 +13445,10 @@
         <v>46266</v>
       </c>
       <c r="B1183" t="n">
-        <v>2258</v>
+        <v>2402</v>
       </c>
       <c r="C1183" t="n">
-        <v>76363.64</v>
+        <v>651994.26</v>
       </c>
     </row>
     <row r="1184">
@@ -13456,10 +13456,10 @@
         <v>46266</v>
       </c>
       <c r="B1184" t="n">
-        <v>2772</v>
+        <v>452</v>
       </c>
       <c r="C1184" t="n">
-        <v>57272.73</v>
+        <v>270000</v>
       </c>
     </row>
     <row r="1185">
@@ -13467,10 +13467,10 @@
         <v>46266</v>
       </c>
       <c r="B1185" t="n">
-        <v>2346</v>
+        <v>2085</v>
       </c>
       <c r="C1185" t="n">
-        <v>105000</v>
+        <v>132049.47</v>
       </c>
     </row>
     <row r="1186">
@@ -13478,10 +13478,10 @@
         <v>46266</v>
       </c>
       <c r="B1186" t="n">
-        <v>2442</v>
+        <v>1906</v>
       </c>
       <c r="C1186" t="n">
-        <v>76356</v>
+        <v>114176.74</v>
       </c>
     </row>
     <row r="1187">
@@ -13489,10 +13489,10 @@
         <v>46266</v>
       </c>
       <c r="B1187" t="n">
-        <v>772</v>
+        <v>2821</v>
       </c>
       <c r="C1187" t="n">
-        <v>315000</v>
+        <v>99046.03999999999</v>
       </c>
     </row>
     <row r="1188">
@@ -13500,10 +13500,10 @@
         <v>46266</v>
       </c>
       <c r="B1188" t="n">
-        <v>2684</v>
+        <v>2633</v>
       </c>
       <c r="C1188" t="n">
-        <v>90678</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1189">
@@ -13511,10 +13511,10 @@
         <v>46266</v>
       </c>
       <c r="B1189" t="n">
-        <v>2765</v>
+        <v>2802</v>
       </c>
       <c r="C1189" t="n">
-        <v>85890</v>
+        <v>70818.63</v>
       </c>
     </row>
     <row r="1190">
@@ -13522,10 +13522,10 @@
         <v>46266</v>
       </c>
       <c r="B1190" t="n">
-        <v>2567</v>
+        <v>841</v>
       </c>
       <c r="C1190" t="n">
-        <v>157542</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1191">
@@ -13533,10 +13533,10 @@
         <v>46266</v>
       </c>
       <c r="B1191" t="n">
-        <v>2178</v>
+        <v>1045</v>
       </c>
       <c r="C1191" t="n">
-        <v>267267</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1192">
@@ -13544,10 +13544,10 @@
         <v>46266</v>
       </c>
       <c r="B1192" t="n">
-        <v>2827</v>
+        <v>2530</v>
       </c>
       <c r="C1192" t="n">
-        <v>95445</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1193">
@@ -13555,10 +13555,10 @@
         <v>46266</v>
       </c>
       <c r="B1193" t="n">
-        <v>2510</v>
+        <v>2717</v>
       </c>
       <c r="C1193" t="n">
-        <v>529998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1194">
@@ -13566,10 +13566,10 @@
         <v>46266</v>
       </c>
       <c r="B1194" t="n">
-        <v>2392</v>
+        <v>2726</v>
       </c>
       <c r="C1194" t="n">
-        <v>158991</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="1195">
@@ -13577,10 +13577,10 @@
         <v>46266</v>
       </c>
       <c r="B1195" t="n">
-        <v>415</v>
+        <v>2820</v>
       </c>
       <c r="C1195" t="n">
-        <v>543606</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="1196">
@@ -13588,10 +13588,10 @@
         <v>46266</v>
       </c>
       <c r="B1196" t="n">
-        <v>2107</v>
+        <v>2739</v>
       </c>
       <c r="C1196" t="n">
-        <v>280707</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1197">
@@ -13599,10 +13599,10 @@
         <v>46266</v>
       </c>
       <c r="B1197" t="n">
-        <v>2211</v>
+        <v>2741</v>
       </c>
       <c r="C1197" t="n">
-        <v>232722</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1198">
@@ -13610,10 +13610,10 @@
         <v>46266</v>
       </c>
       <c r="B1198" t="n">
-        <v>2682</v>
+        <v>1007</v>
       </c>
       <c r="C1198" t="n">
-        <v>143157</v>
+        <v>190000</v>
       </c>
     </row>
     <row r="1199">
@@ -13621,10 +13621,10 @@
         <v>46266</v>
       </c>
       <c r="B1199" t="n">
-        <v>2781</v>
+        <v>20</v>
       </c>
       <c r="C1199" t="n">
-        <v>0</v>
+        <v>385000</v>
       </c>
     </row>
     <row r="1200">
@@ -13632,10 +13632,10 @@
         <v>46266</v>
       </c>
       <c r="B1200" t="n">
-        <v>2576</v>
+        <v>1372</v>
       </c>
       <c r="C1200" t="n">
-        <v>0</v>
+        <v>290000</v>
       </c>
     </row>
     <row r="1201">
@@ -13643,10 +13643,10 @@
         <v>46266</v>
       </c>
       <c r="B1201" t="n">
-        <v>2755</v>
+        <v>2735</v>
       </c>
       <c r="C1201" t="n">
-        <v>57267</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="1202">
@@ -13654,10 +13654,10 @@
         <v>46266</v>
       </c>
       <c r="B1202" t="n">
-        <v>941</v>
+        <v>2811</v>
       </c>
       <c r="C1202" t="n">
-        <v>339694.56</v>
+        <v>41610.33</v>
       </c>
     </row>
     <row r="1203">
@@ -13665,10 +13665,10 @@
         <v>46266</v>
       </c>
       <c r="B1203" t="n">
-        <v>2734</v>
+        <v>1871</v>
       </c>
       <c r="C1203" t="n">
-        <v>52563</v>
+        <v>176760.47</v>
       </c>
     </row>
     <row r="1204">
@@ -13676,10 +13676,10 @@
         <v>46266</v>
       </c>
       <c r="B1204" t="n">
-        <v>1840</v>
+        <v>2541</v>
       </c>
       <c r="C1204" t="n">
-        <v>0</v>
+        <v>211614.65</v>
       </c>
     </row>
     <row r="1205">
@@ -13687,10 +13687,10 @@
         <v>46266</v>
       </c>
       <c r="B1205" t="n">
-        <v>1289</v>
+        <v>2362</v>
       </c>
       <c r="C1205" t="n">
-        <v>238623</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="1206">
@@ -13698,10 +13698,10 @@
         <v>46266</v>
       </c>
       <c r="B1206" t="n">
-        <v>2801</v>
+        <v>1324</v>
       </c>
       <c r="C1206" t="n">
-        <v>76356</v>
+        <v>280000</v>
       </c>
     </row>
     <row r="1207">
@@ -13709,10 +13709,10 @@
         <v>46266</v>
       </c>
       <c r="B1207" t="n">
-        <v>2810</v>
+        <v>2323</v>
       </c>
       <c r="C1207" t="n">
-        <v>128856</v>
+        <v>68705.64999999999</v>
       </c>
     </row>
     <row r="1208">
@@ -13720,10 +13720,10 @@
         <v>46266</v>
       </c>
       <c r="B1208" t="n">
-        <v>767</v>
+        <v>2647</v>
       </c>
       <c r="C1208" t="n">
-        <v>171801</v>
+        <v>141906.29</v>
       </c>
     </row>
     <row r="1209">
@@ -13731,10 +13731,10 @@
         <v>46266</v>
       </c>
       <c r="B1209" t="n">
-        <v>2687</v>
+        <v>559</v>
       </c>
       <c r="C1209" t="n">
-        <v>95445</v>
+        <v>229446.83</v>
       </c>
     </row>
     <row r="1210">
@@ -13742,10 +13742,10 @@
         <v>46266</v>
       </c>
       <c r="B1210" t="n">
-        <v>2686</v>
+        <v>2762</v>
       </c>
       <c r="C1210" t="n">
-        <v>124089</v>
+        <v>81489.49000000001</v>
       </c>
     </row>
     <row r="1211">
@@ -13753,10 +13753,10 @@
         <v>46266</v>
       </c>
       <c r="B1211" t="n">
-        <v>2730</v>
+        <v>2501</v>
       </c>
       <c r="C1211" t="n">
-        <v>85890</v>
+        <v>81489.46000000001</v>
       </c>
     </row>
     <row r="1212">
@@ -13764,10 +13764,10 @@
         <v>46266</v>
       </c>
       <c r="B1212" t="n">
-        <v>2580</v>
+        <v>2562</v>
       </c>
       <c r="C1212" t="n">
-        <v>32025</v>
+        <v>15835.33</v>
       </c>
     </row>
     <row r="1213">
@@ -13775,10 +13775,10 @@
         <v>46266</v>
       </c>
       <c r="B1213" t="n">
-        <v>2472</v>
+        <v>429</v>
       </c>
       <c r="C1213" t="n">
-        <v>50535.55</v>
+        <v>390000</v>
       </c>
     </row>
     <row r="1214">
@@ -13786,10 +13786,10 @@
         <v>46266</v>
       </c>
       <c r="B1214" t="n">
-        <v>2631</v>
+        <v>58</v>
       </c>
       <c r="C1214" t="n">
-        <v>23416.91</v>
+        <v>270586.53</v>
       </c>
     </row>
     <row r="1215">
@@ -13797,10 +13797,10 @@
         <v>46266</v>
       </c>
       <c r="B1215" t="n">
-        <v>1642</v>
+        <v>2245</v>
       </c>
       <c r="C1215" t="n">
-        <v>252945</v>
+        <v>241595.11</v>
       </c>
     </row>
     <row r="1216">
@@ -13808,10 +13808,10 @@
         <v>46266</v>
       </c>
       <c r="B1216" t="n">
-        <v>2613</v>
+        <v>285</v>
       </c>
       <c r="C1216" t="n">
-        <v>171045</v>
+        <v>541173.05</v>
       </c>
     </row>
     <row r="1217">
@@ -13819,10 +13819,10 @@
         <v>46266</v>
       </c>
       <c r="B1217" t="n">
-        <v>1020</v>
+        <v>1464</v>
       </c>
       <c r="C1217" t="n">
-        <v>85890</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1218">
@@ -13830,10 +13830,10 @@
         <v>46266</v>
       </c>
       <c r="B1218" t="n">
-        <v>2785</v>
+        <v>363</v>
       </c>
       <c r="C1218" t="n">
-        <v>39711</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="1219">
@@ -13841,10 +13841,10 @@
         <v>46266</v>
       </c>
       <c r="B1219" t="n">
-        <v>1327</v>
+        <v>2651</v>
       </c>
       <c r="C1219" t="n">
-        <v>57267</v>
+        <v>169120.47</v>
       </c>
     </row>
     <row r="1220">
@@ -13852,10 +13852,10 @@
         <v>46266</v>
       </c>
       <c r="B1220" t="n">
-        <v>749</v>
+        <v>2142</v>
       </c>
       <c r="C1220" t="n">
-        <v>77784</v>
+        <v>53386.01</v>
       </c>
     </row>
     <row r="1221">
@@ -13863,10 +13863,10 @@
         <v>46266</v>
       </c>
       <c r="B1221" t="n">
-        <v>1983</v>
+        <v>2258</v>
       </c>
       <c r="C1221" t="n">
-        <v>516558</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="1222">
@@ -13874,10 +13874,10 @@
         <v>46266</v>
       </c>
       <c r="B1222" t="n">
-        <v>1993</v>
+        <v>2772</v>
       </c>
       <c r="C1222" t="n">
-        <v>332073</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1223">
@@ -13885,10 +13885,10 @@
         <v>46266</v>
       </c>
       <c r="B1223" t="n">
-        <v>2767</v>
+        <v>2346</v>
       </c>
       <c r="C1223" t="n">
-        <v>184149</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="1224">
@@ -13896,10 +13896,10 @@
         <v>46266</v>
       </c>
       <c r="B1224" t="n">
-        <v>2646</v>
+        <v>2442</v>
       </c>
       <c r="C1224" t="n">
-        <v>0</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="1225">
@@ -13907,10 +13907,10 @@
         <v>46266</v>
       </c>
       <c r="B1225" t="n">
-        <v>1102</v>
+        <v>772</v>
       </c>
       <c r="C1225" t="n">
-        <v>230601</v>
+        <v>330000</v>
       </c>
     </row>
     <row r="1226">
@@ -13918,10 +13918,10 @@
         <v>46266</v>
       </c>
       <c r="B1226" t="n">
-        <v>626</v>
+        <v>2684</v>
       </c>
       <c r="C1226" t="n">
-        <v>1626846.14</v>
+        <v>95000</v>
       </c>
     </row>
     <row r="1227">
@@ -13929,10 +13929,10 @@
         <v>46266</v>
       </c>
       <c r="B1227" t="n">
-        <v>1465</v>
+        <v>2765</v>
       </c>
       <c r="C1227" t="n">
-        <v>343434</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="1228">
@@ -13940,10 +13940,10 @@
         <v>46266</v>
       </c>
       <c r="B1228" t="n">
-        <v>2758</v>
+        <v>2567</v>
       </c>
       <c r="C1228" t="n">
-        <v>57272.73</v>
+        <v>165061.84</v>
       </c>
     </row>
     <row r="1229">
@@ -13951,10 +13951,10 @@
         <v>46266</v>
       </c>
       <c r="B1229" t="n">
-        <v>2742</v>
+        <v>2178</v>
       </c>
       <c r="C1229" t="n">
-        <v>57272.73</v>
+        <v>280000</v>
       </c>
     </row>
     <row r="1230">
@@ -13962,10 +13962,10 @@
         <v>46266</v>
       </c>
       <c r="B1230" t="n">
-        <v>2748</v>
+        <v>2827</v>
       </c>
       <c r="C1230" t="n">
-        <v>0</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1231">
@@ -13973,10 +13973,10 @@
         <v>46266</v>
       </c>
       <c r="B1231" t="n">
-        <v>1873</v>
+        <v>2510</v>
       </c>
       <c r="C1231" t="n">
-        <v>305445</v>
+        <v>555244.09</v>
       </c>
     </row>
     <row r="1232">
@@ -13984,10 +13984,10 @@
         <v>46266</v>
       </c>
       <c r="B1232" t="n">
-        <v>2163</v>
+        <v>2392</v>
       </c>
       <c r="C1232" t="n">
-        <v>143178</v>
+        <v>166573.23</v>
       </c>
     </row>
     <row r="1233">
@@ -13995,10 +13995,10 @@
         <v>46266</v>
       </c>
       <c r="B1233" t="n">
-        <v>2394</v>
+        <v>415</v>
       </c>
       <c r="C1233" t="n">
-        <v>147042</v>
+        <v>569500</v>
       </c>
     </row>
     <row r="1234">
@@ -14006,10 +14006,10 @@
         <v>46266</v>
       </c>
       <c r="B1234" t="n">
-        <v>33</v>
+        <v>2107</v>
       </c>
       <c r="C1234" t="n">
-        <v>370356</v>
+        <v>292211.87</v>
       </c>
     </row>
     <row r="1235">
@@ -14017,10 +14017,10 @@
         <v>46266</v>
       </c>
       <c r="B1235" t="n">
-        <v>2421</v>
+        <v>2211</v>
       </c>
       <c r="C1235" t="n">
-        <v>62034</v>
+        <v>241954.32</v>
       </c>
     </row>
     <row r="1236">
@@ -14028,10 +14028,10 @@
         <v>46266</v>
       </c>
       <c r="B1236" t="n">
-        <v>2663</v>
+        <v>2682</v>
       </c>
       <c r="C1236" t="n">
-        <v>262500</v>
+        <v>149990.08</v>
       </c>
     </row>
     <row r="1237">
@@ -14039,10 +14039,10 @@
         <v>46266</v>
       </c>
       <c r="B1237" t="n">
-        <v>2413</v>
+        <v>2781</v>
       </c>
       <c r="C1237" t="n">
-        <v>115542</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1238">
@@ -14050,10 +14050,10 @@
         <v>46266</v>
       </c>
       <c r="B1238" t="n">
-        <v>351</v>
+        <v>2576</v>
       </c>
       <c r="C1238" t="n">
-        <v>175623</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1239">
@@ -14061,10 +14061,10 @@
         <v>46266</v>
       </c>
       <c r="B1239" t="n">
-        <v>1298</v>
+        <v>2755</v>
       </c>
       <c r="C1239" t="n">
-        <v>1215123</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1240">
@@ -14072,10 +14072,10 @@
         <v>46266</v>
       </c>
       <c r="B1240" t="n">
-        <v>2491</v>
+        <v>941</v>
       </c>
       <c r="C1240" t="n">
-        <v>98196</v>
+        <v>355870.49</v>
       </c>
     </row>
     <row r="1241">
@@ -14083,10 +14083,10 @@
         <v>46266</v>
       </c>
       <c r="B1241" t="n">
-        <v>2571</v>
+        <v>2734</v>
       </c>
       <c r="C1241" t="n">
-        <v>138663</v>
+        <v>55081.16</v>
       </c>
     </row>
     <row r="1242">
@@ -14094,10 +14094,10 @@
         <v>46266</v>
       </c>
       <c r="B1242" t="n">
-        <v>2507</v>
+        <v>1840</v>
       </c>
       <c r="C1242" t="n">
-        <v>84252</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1243">
@@ -14105,10 +14105,10 @@
         <v>46266</v>
       </c>
       <c r="B1243" t="n">
-        <v>2799</v>
+        <v>1289</v>
       </c>
       <c r="C1243" t="n">
-        <v>108444</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="1244">
@@ -14116,10 +14116,10 @@
         <v>46266</v>
       </c>
       <c r="B1244" t="n">
-        <v>2253</v>
+        <v>2801</v>
       </c>
       <c r="C1244" t="n">
-        <v>0</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="1245">
@@ -14127,10 +14127,10 @@
         <v>46266</v>
       </c>
       <c r="B1245" t="n">
-        <v>2582</v>
+        <v>2810</v>
       </c>
       <c r="C1245" t="n">
-        <v>82614</v>
+        <v>135000</v>
       </c>
     </row>
     <row r="1246">
@@ -14138,10 +14138,10 @@
         <v>46266</v>
       </c>
       <c r="B1246" t="n">
-        <v>2637</v>
+        <v>1501</v>
       </c>
       <c r="C1246" t="n">
-        <v>60081</v>
+        <v>95000</v>
       </c>
     </row>
     <row r="1247">
@@ -14149,10 +14149,10 @@
         <v>46266</v>
       </c>
       <c r="B1247" t="n">
-        <v>630</v>
+        <v>703</v>
       </c>
       <c r="C1247" t="n">
-        <v>142884</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="1248">
@@ -14160,10 +14160,10 @@
         <v>46266</v>
       </c>
       <c r="B1248" t="n">
-        <v>525</v>
+        <v>749</v>
       </c>
       <c r="C1248" t="n">
-        <v>214767</v>
+        <v>81489.46000000001</v>
       </c>
     </row>
     <row r="1249">
@@ -14171,10 +14171,10 @@
         <v>46266</v>
       </c>
       <c r="B1249" t="n">
-        <v>2727</v>
+        <v>1983</v>
       </c>
       <c r="C1249" t="n">
-        <v>38640</v>
+        <v>541173.05</v>
       </c>
     </row>
     <row r="1250">
@@ -14182,10 +14182,10 @@
         <v>46266</v>
       </c>
       <c r="B1250" t="n">
-        <v>2707</v>
+        <v>1993</v>
       </c>
       <c r="C1250" t="n">
-        <v>30576</v>
+        <v>347896.96</v>
       </c>
     </row>
     <row r="1251">
@@ -14193,10 +14193,10 @@
         <v>46266</v>
       </c>
       <c r="B1251" t="n">
-        <v>2834</v>
+        <v>2767</v>
       </c>
       <c r="C1251" t="n">
-        <v>15795.82</v>
+        <v>192936.84</v>
       </c>
     </row>
     <row r="1252">
@@ -14204,10 +14204,10 @@
         <v>46266</v>
       </c>
       <c r="B1252" t="n">
-        <v>2773</v>
+        <v>2646</v>
       </c>
       <c r="C1252" t="n">
-        <v>77024.19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1253">
@@ -14215,10 +14215,10 @@
         <v>46266</v>
       </c>
       <c r="B1253" t="n">
-        <v>2341</v>
+        <v>1102</v>
       </c>
       <c r="C1253" t="n">
-        <v>135450</v>
+        <v>241595.11</v>
       </c>
     </row>
     <row r="1254">
@@ -14226,10 +14226,10 @@
         <v>46266</v>
       </c>
       <c r="B1254" t="n">
-        <v>1374</v>
+        <v>626</v>
       </c>
       <c r="C1254" t="n">
-        <v>171801</v>
+        <v>1704315</v>
       </c>
     </row>
     <row r="1255">
@@ -14237,10 +14237,10 @@
         <v>46266</v>
       </c>
       <c r="B1255" t="n">
-        <v>793</v>
+        <v>1465</v>
       </c>
       <c r="C1255" t="n">
-        <v>39711</v>
+        <v>359789.28</v>
       </c>
     </row>
     <row r="1256">
@@ -14248,10 +14248,10 @@
         <v>46266</v>
       </c>
       <c r="B1256" t="n">
-        <v>794</v>
+        <v>2758</v>
       </c>
       <c r="C1256" t="n">
-        <v>39711</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1257">
@@ -14259,10 +14259,10 @@
         <v>46266</v>
       </c>
       <c r="B1257" t="n">
-        <v>1834</v>
+        <v>2742</v>
       </c>
       <c r="C1257" t="n">
-        <v>111678</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1258">
@@ -14270,10 +14270,10 @@
         <v>46266</v>
       </c>
       <c r="B1258" t="n">
-        <v>802</v>
+        <v>2748</v>
       </c>
       <c r="C1258" t="n">
-        <v>71589</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1259">
@@ -14281,10 +14281,10 @@
         <v>46266</v>
       </c>
       <c r="B1259" t="n">
-        <v>1344</v>
+        <v>1873</v>
       </c>
       <c r="C1259" t="n">
-        <v>143178</v>
+        <v>320000</v>
       </c>
     </row>
     <row r="1260">
@@ -14292,10 +14292,10 @@
         <v>46266</v>
       </c>
       <c r="B1260" t="n">
-        <v>1881</v>
+        <v>2163</v>
       </c>
       <c r="C1260" t="n">
-        <v>65562</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="1261">
@@ -14303,10 +14303,10 @@
         <v>46266</v>
       </c>
       <c r="B1261" t="n">
-        <v>2365</v>
+        <v>2394</v>
       </c>
       <c r="C1261" t="n">
-        <v>76041</v>
+        <v>154057.72</v>
       </c>
     </row>
     <row r="1262">
@@ -14314,10 +14314,10 @@
         <v>46266</v>
       </c>
       <c r="B1262" t="n">
-        <v>2411</v>
+        <v>33</v>
       </c>
       <c r="C1262" t="n">
-        <v>135450</v>
+        <v>388000</v>
       </c>
     </row>
     <row r="1263">
@@ -14325,10 +14325,10 @@
         <v>46266</v>
       </c>
       <c r="B1263" t="n">
-        <v>2363</v>
+        <v>2421</v>
       </c>
       <c r="C1263" t="n">
-        <v>143178</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="1264">
@@ -14336,10 +14336,10 @@
         <v>46266</v>
       </c>
       <c r="B1264" t="n">
-        <v>2124</v>
+        <v>2663</v>
       </c>
       <c r="C1264" t="n">
-        <v>334089</v>
+        <v>275000</v>
       </c>
     </row>
     <row r="1265">
@@ -14347,10 +14347,10 @@
         <v>46266</v>
       </c>
       <c r="B1265" t="n">
-        <v>1937</v>
+        <v>2413</v>
       </c>
       <c r="C1265" t="n">
-        <v>243390</v>
+        <v>121045.35</v>
       </c>
     </row>
     <row r="1266">
@@ -14358,10 +14358,10 @@
         <v>46266</v>
       </c>
       <c r="B1266" t="n">
-        <v>2709</v>
+        <v>351</v>
       </c>
       <c r="C1266" t="n">
-        <v>171801</v>
+        <v>184000</v>
       </c>
     </row>
     <row r="1267">
@@ -14369,10 +14369,10 @@
         <v>46266</v>
       </c>
       <c r="B1267" t="n">
-        <v>2558</v>
+        <v>1298</v>
       </c>
       <c r="C1267" t="n">
-        <v>28686</v>
+        <v>1273000</v>
       </c>
     </row>
     <row r="1268">
@@ -14380,10 +14380,10 @@
         <v>46266</v>
       </c>
       <c r="B1268" t="n">
-        <v>663</v>
+        <v>2491</v>
       </c>
       <c r="C1268" t="n">
-        <v>243390</v>
+        <v>102895.07</v>
       </c>
     </row>
     <row r="1269">
@@ -14391,10 +14391,10 @@
         <v>46266</v>
       </c>
       <c r="B1269" t="n">
-        <v>40</v>
+        <v>2571</v>
       </c>
       <c r="C1269" t="n">
-        <v>210000</v>
+        <v>145281.04</v>
       </c>
     </row>
     <row r="1270">
@@ -14402,10 +14402,10 @@
         <v>46266</v>
       </c>
       <c r="B1270" t="n">
-        <v>2833</v>
+        <v>2507</v>
       </c>
       <c r="C1270" t="n">
-        <v>66818.19</v>
+        <v>86421.14</v>
       </c>
     </row>
     <row r="1271">
@@ -14413,10 +14413,10 @@
         <v>46266</v>
       </c>
       <c r="B1271" t="n">
-        <v>1756</v>
+        <v>2799</v>
       </c>
       <c r="C1271" t="n">
-        <v>416661</v>
+        <v>113633.63</v>
       </c>
     </row>
     <row r="1272">
@@ -14424,10 +14424,10 @@
         <v>46266</v>
       </c>
       <c r="B1272" t="n">
-        <v>1116</v>
+        <v>2253</v>
       </c>
       <c r="C1272" t="n">
-        <v>242109</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1273">
@@ -14435,10 +14435,10 @@
         <v>46266</v>
       </c>
       <c r="B1273" t="n">
-        <v>636</v>
+        <v>2834</v>
       </c>
       <c r="C1273" t="n">
-        <v>238623</v>
+        <v>16550</v>
       </c>
     </row>
     <row r="1274">
@@ -14446,10 +14446,10 @@
         <v>46266</v>
       </c>
       <c r="B1274" t="n">
-        <v>1800</v>
+        <v>2582</v>
       </c>
       <c r="C1274" t="n">
-        <v>26712</v>
+        <v>86556.11</v>
       </c>
     </row>
     <row r="1275">
@@ -14457,10 +14457,10 @@
         <v>46266</v>
       </c>
       <c r="B1275" t="n">
-        <v>2815</v>
+        <v>2637</v>
       </c>
       <c r="C1275" t="n">
-        <v>57272.73</v>
+        <v>62949.9</v>
       </c>
     </row>
     <row r="1276">
@@ -14468,10 +14468,10 @@
         <v>46266</v>
       </c>
       <c r="B1276" t="n">
-        <v>1658</v>
+        <v>630</v>
       </c>
       <c r="C1276" t="n">
-        <v>126000</v>
+        <v>149700.41</v>
       </c>
     </row>
     <row r="1277">
@@ -14479,10 +14479,10 @@
         <v>46266</v>
       </c>
       <c r="B1277" t="n">
-        <v>2635</v>
+        <v>1638</v>
       </c>
       <c r="C1277" t="n">
-        <v>124089</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1278">
@@ -14490,10 +14490,10 @@
         <v>46266</v>
       </c>
       <c r="B1278" t="n">
-        <v>2402</v>
+        <v>2681</v>
       </c>
       <c r="C1278" t="n">
-        <v>622356</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1279">
@@ -14501,10 +14501,10 @@
         <v>46266</v>
       </c>
       <c r="B1279" t="n">
-        <v>452</v>
+        <v>525</v>
       </c>
       <c r="C1279" t="n">
-        <v>257712</v>
+        <v>225000</v>
       </c>
     </row>
     <row r="1280">
@@ -14512,10 +14512,10 @@
         <v>46266</v>
       </c>
       <c r="B1280" t="n">
-        <v>2085</v>
+        <v>2727</v>
       </c>
       <c r="C1280" t="n">
-        <v>126042</v>
+        <v>40496.2</v>
       </c>
     </row>
     <row r="1281">
@@ -14523,10 +14523,10 @@
         <v>46266</v>
       </c>
       <c r="B1281" t="n">
-        <v>2568</v>
+        <v>2049</v>
       </c>
       <c r="C1281" t="n">
-        <v>195132</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1282">
@@ -14534,10 +14534,10 @@
         <v>46266</v>
       </c>
       <c r="B1282" t="n">
-        <v>1906</v>
+        <v>2740</v>
       </c>
       <c r="C1282" t="n">
-        <v>110754</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1283">
@@ -14545,10 +14545,10 @@
         <v>46266</v>
       </c>
       <c r="B1283" t="n">
-        <v>2821</v>
+        <v>2707</v>
       </c>
       <c r="C1283" t="n">
-        <v>96306</v>
+        <v>32050</v>
       </c>
     </row>
     <row r="1284">
@@ -14556,10 +14556,10 @@
         <v>46266</v>
       </c>
       <c r="B1284" t="n">
-        <v>2698</v>
+        <v>2773</v>
       </c>
       <c r="C1284" t="n">
-        <v>118041</v>
+        <v>80700</v>
       </c>
     </row>
     <row r="1285">
@@ -14567,10 +14567,10 @@
         <v>46266</v>
       </c>
       <c r="B1285" t="n">
-        <v>2118</v>
+        <v>2568</v>
       </c>
       <c r="C1285" t="n">
-        <v>226380</v>
+        <v>204430.78</v>
       </c>
     </row>
     <row r="1286">
@@ -14578,10 +14578,10 @@
         <v>46266</v>
       </c>
       <c r="B1286" t="n">
-        <v>2383</v>
+        <v>2341</v>
       </c>
       <c r="C1286" t="n">
-        <v>132174</v>
+        <v>141906.29</v>
       </c>
     </row>
     <row r="1287">
@@ -14589,10 +14589,10 @@
         <v>46266</v>
       </c>
       <c r="B1287" t="n">
-        <v>2813</v>
+        <v>1374</v>
       </c>
       <c r="C1287" t="n">
-        <v>60081</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="1288">
@@ -14600,10 +14600,10 @@
         <v>46266</v>
       </c>
       <c r="B1288" t="n">
-        <v>925</v>
+        <v>793</v>
       </c>
       <c r="C1288" t="n">
-        <v>75096</v>
+        <v>41610.33</v>
       </c>
     </row>
     <row r="1289">
@@ -14611,10 +14611,10 @@
         <v>46266</v>
       </c>
       <c r="B1289" t="n">
-        <v>2689</v>
+        <v>794</v>
       </c>
       <c r="C1289" t="n">
-        <v>60081</v>
+        <v>41610.33</v>
       </c>
     </row>
     <row r="1290">
@@ -14622,10 +14622,10 @@
         <v>46266</v>
       </c>
       <c r="B1290" t="n">
-        <v>2716</v>
+        <v>1834</v>
       </c>
       <c r="C1290" t="n">
-        <v>82614</v>
+        <v>117010.45</v>
       </c>
     </row>
     <row r="1291">
@@ -14633,10 +14633,10 @@
         <v>46266</v>
       </c>
       <c r="B1291" t="n">
-        <v>2831</v>
+        <v>802</v>
       </c>
       <c r="C1291" t="n">
-        <v>57267</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="1292">
@@ -14644,10 +14644,10 @@
         <v>46266</v>
       </c>
       <c r="B1292" t="n">
-        <v>2045</v>
+        <v>1344</v>
       </c>
       <c r="C1292" t="n">
-        <v>321162.19</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="1293">
@@ -14655,10 +14655,10 @@
         <v>46266</v>
       </c>
       <c r="B1293" t="n">
-        <v>580</v>
+        <v>1881</v>
       </c>
       <c r="C1293" t="n">
-        <v>128856</v>
+        <v>68705.64999999999</v>
       </c>
     </row>
     <row r="1294">
@@ -14666,10 +14666,10 @@
         <v>46266</v>
       </c>
       <c r="B1294" t="n">
-        <v>438</v>
+        <v>2365</v>
       </c>
       <c r="C1294" t="n">
-        <v>147945</v>
+        <v>79666.69</v>
       </c>
     </row>
     <row r="1295">
@@ -14677,10 +14677,10 @@
         <v>46266</v>
       </c>
       <c r="B1295" t="n">
-        <v>1539</v>
+        <v>2411</v>
       </c>
       <c r="C1295" t="n">
-        <v>162267</v>
+        <v>141906.29</v>
       </c>
     </row>
     <row r="1296">
@@ -14688,10 +14688,10 @@
         <v>46266</v>
       </c>
       <c r="B1296" t="n">
-        <v>2817</v>
+        <v>2363</v>
       </c>
       <c r="C1296" t="n">
-        <v>57267</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="1297">
@@ -14699,10 +14699,10 @@
         <v>46266</v>
       </c>
       <c r="B1297" t="n">
-        <v>2816</v>
+        <v>2124</v>
       </c>
       <c r="C1297" t="n">
-        <v>124089</v>
+        <v>350000</v>
       </c>
     </row>
     <row r="1298">
@@ -14710,10 +14710,10 @@
         <v>46266</v>
       </c>
       <c r="B1298" t="n">
-        <v>2146</v>
+        <v>1937</v>
       </c>
       <c r="C1298" t="n">
-        <v>192486</v>
+        <v>255000</v>
       </c>
     </row>
     <row r="1299">
@@ -14721,10 +14721,10 @@
         <v>46266</v>
       </c>
       <c r="B1299" t="n">
-        <v>2276</v>
+        <v>2709</v>
       </c>
       <c r="C1299" t="n">
-        <v>213864</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="1300">
@@ -14732,10 +14732,10 @@
         <v>46266</v>
       </c>
       <c r="B1300" t="n">
-        <v>1381</v>
+        <v>2558</v>
       </c>
       <c r="C1300" t="n">
-        <v>281589</v>
+        <v>30065.72</v>
       </c>
     </row>
     <row r="1301">
@@ -14743,10 +14743,10 @@
         <v>46266</v>
       </c>
       <c r="B1301" t="n">
-        <v>2081</v>
+        <v>663</v>
       </c>
       <c r="C1301" t="n">
-        <v>143178</v>
+        <v>255000</v>
       </c>
     </row>
     <row r="1302">
@@ -14754,10 +14754,10 @@
         <v>46266</v>
       </c>
       <c r="B1302" t="n">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="C1302" t="n">
-        <v>415212</v>
+        <v>220000</v>
       </c>
     </row>
     <row r="1303">
@@ -14765,10 +14765,10 @@
         <v>46266</v>
       </c>
       <c r="B1303" t="n">
-        <v>766</v>
+        <v>2833</v>
       </c>
       <c r="C1303" t="n">
-        <v>65562</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="1304">
@@ -14776,10 +14776,10 @@
         <v>46266</v>
       </c>
       <c r="B1304" t="n">
-        <v>2547</v>
+        <v>1756</v>
       </c>
       <c r="C1304" t="n">
-        <v>39249</v>
+        <v>436523.6</v>
       </c>
     </row>
     <row r="1305">
@@ -14787,10 +14787,10 @@
         <v>46266</v>
       </c>
       <c r="B1305" t="n">
-        <v>2552</v>
+        <v>1116</v>
       </c>
       <c r="C1305" t="n">
-        <v>28224</v>
+        <v>253640.38</v>
       </c>
     </row>
     <row r="1306">
@@ -14798,10 +14798,10 @@
         <v>46266</v>
       </c>
       <c r="B1306" t="n">
-        <v>131</v>
+        <v>636</v>
       </c>
       <c r="C1306" t="n">
-        <v>390390</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="1307">
@@ -14809,10 +14809,10 @@
         <v>46266</v>
       </c>
       <c r="B1307" t="n">
-        <v>2250</v>
+        <v>1800</v>
       </c>
       <c r="C1307" t="n">
-        <v>315861</v>
+        <v>27984.92</v>
       </c>
     </row>
     <row r="1308">
@@ -14820,10 +14820,10 @@
         <v>46266</v>
       </c>
       <c r="B1308" t="n">
-        <v>89</v>
+        <v>2815</v>
       </c>
       <c r="C1308" t="n">
-        <v>322812</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1309">
@@ -14831,10 +14831,10 @@
         <v>46266</v>
       </c>
       <c r="B1309" t="n">
-        <v>2141</v>
+        <v>1658</v>
       </c>
       <c r="C1309" t="n">
-        <v>30198</v>
+        <v>132000</v>
       </c>
     </row>
     <row r="1310">
@@ -14842,10 +14842,10 @@
         <v>46266</v>
       </c>
       <c r="B1310" t="n">
-        <v>2798</v>
+        <v>2698</v>
       </c>
       <c r="C1310" t="n">
-        <v>57272.73</v>
+        <v>121811.41</v>
       </c>
     </row>
     <row r="1311">
@@ -14853,10 +14853,10 @@
         <v>46266</v>
       </c>
       <c r="B1311" t="n">
-        <v>2797</v>
+        <v>2118</v>
       </c>
       <c r="C1311" t="n">
-        <v>57272.73</v>
+        <v>235302.9</v>
       </c>
     </row>
     <row r="1312">
@@ -14864,10 +14864,10 @@
         <v>46266</v>
       </c>
       <c r="B1312" t="n">
-        <v>2266</v>
+        <v>2383</v>
       </c>
       <c r="C1312" t="n">
-        <v>76363.64</v>
+        <v>136601.72</v>
       </c>
     </row>
     <row r="1313">
@@ -14875,10 +14875,10 @@
         <v>46266</v>
       </c>
       <c r="B1313" t="n">
-        <v>1499</v>
+        <v>2813</v>
       </c>
       <c r="C1313" t="n">
-        <v>133623</v>
+        <v>62949.9</v>
       </c>
     </row>
     <row r="1314">
@@ -14886,10 +14886,10 @@
         <v>46266</v>
       </c>
       <c r="B1314" t="n">
-        <v>2496</v>
+        <v>925</v>
       </c>
       <c r="C1314" t="n">
-        <v>152712</v>
+        <v>78687.37</v>
       </c>
     </row>
     <row r="1315">
@@ -14897,10 +14897,10 @@
         <v>46266</v>
       </c>
       <c r="B1315" t="n">
-        <v>949</v>
+        <v>2689</v>
       </c>
       <c r="C1315" t="n">
-        <v>93681</v>
+        <v>62949.9</v>
       </c>
     </row>
     <row r="1316">
@@ -14908,10 +14908,10 @@
         <v>46266</v>
       </c>
       <c r="B1316" t="n">
-        <v>1853</v>
+        <v>2716</v>
       </c>
       <c r="C1316" t="n">
-        <v>114534</v>
+        <v>86556.11</v>
       </c>
     </row>
     <row r="1317">
@@ -14919,10 +14919,10 @@
         <v>46266</v>
       </c>
       <c r="B1317" t="n">
-        <v>854</v>
+        <v>2831</v>
       </c>
       <c r="C1317" t="n">
-        <v>105000</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1318">
@@ -14930,10 +14930,10 @@
         <v>46266</v>
       </c>
       <c r="B1318" t="n">
-        <v>2674</v>
+        <v>2775</v>
       </c>
       <c r="C1318" t="n">
-        <v>248178</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1319">
@@ -14941,10 +14941,10 @@
         <v>46266</v>
       </c>
       <c r="B1319" t="n">
-        <v>2803</v>
+        <v>2045</v>
       </c>
       <c r="C1319" t="n">
-        <v>114534</v>
+        <v>336471.62</v>
       </c>
     </row>
     <row r="1320">
@@ -14952,10 +14952,10 @@
         <v>46266</v>
       </c>
       <c r="B1320" t="n">
-        <v>2599</v>
+        <v>580</v>
       </c>
       <c r="C1320" t="n">
-        <v>181356</v>
+        <v>135000</v>
       </c>
     </row>
     <row r="1321">
@@ -14963,10 +14963,10 @@
         <v>46266</v>
       </c>
       <c r="B1321" t="n">
-        <v>783</v>
+        <v>438</v>
       </c>
       <c r="C1321" t="n">
-        <v>49623</v>
+        <v>155000</v>
       </c>
     </row>
     <row r="1322">
@@ -14974,10 +14974,10 @@
         <v>46266</v>
       </c>
       <c r="B1322" t="n">
-        <v>27</v>
+        <v>1539</v>
       </c>
       <c r="C1322" t="n">
-        <v>95445</v>
+        <v>170000</v>
       </c>
     </row>
     <row r="1323">
@@ -14985,10 +14985,10 @@
         <v>46266</v>
       </c>
       <c r="B1323" t="n">
-        <v>531</v>
+        <v>2817</v>
       </c>
       <c r="C1323" t="n">
-        <v>334089</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1324">
@@ -14996,10 +14996,10 @@
         <v>46266</v>
       </c>
       <c r="B1324" t="n">
-        <v>1308</v>
+        <v>2816</v>
       </c>
       <c r="C1324" t="n">
-        <v>154182</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="1325">
@@ -15007,10 +15007,10 @@
         <v>46266</v>
       </c>
       <c r="B1325" t="n">
-        <v>2792</v>
+        <v>2146</v>
       </c>
       <c r="C1325" t="n">
-        <v>111195</v>
+        <v>201656.31</v>
       </c>
     </row>
     <row r="1326">
@@ -15018,10 +15018,10 @@
         <v>46266</v>
       </c>
       <c r="B1326" t="n">
-        <v>2828</v>
+        <v>2276</v>
       </c>
       <c r="C1326" t="n">
-        <v>0</v>
+        <v>224062.57</v>
       </c>
     </row>
     <row r="1327">
@@ -15029,10 +15029,10 @@
         <v>46266</v>
       </c>
       <c r="B1327" t="n">
-        <v>2823</v>
+        <v>1381</v>
       </c>
       <c r="C1327" t="n">
-        <v>89250</v>
+        <v>295000</v>
       </c>
     </row>
     <row r="1328">
@@ -15040,10 +15040,10 @@
         <v>46266</v>
       </c>
       <c r="B1328" t="n">
-        <v>2584</v>
+        <v>2081</v>
       </c>
       <c r="C1328" t="n">
-        <v>60081</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="1329">
@@ -15051,10 +15051,10 @@
         <v>46266</v>
       </c>
       <c r="B1329" t="n">
-        <v>945</v>
+        <v>14</v>
       </c>
       <c r="C1329" t="n">
-        <v>270438</v>
+        <v>435000</v>
       </c>
     </row>
     <row r="1330">
@@ -15062,10 +15062,10 @@
         <v>46266</v>
       </c>
       <c r="B1330" t="n">
-        <v>2660</v>
+        <v>766</v>
       </c>
       <c r="C1330" t="n">
-        <v>295890</v>
+        <v>68705.64999999999</v>
       </c>
     </row>
     <row r="1331">
@@ -15073,10 +15073,10 @@
         <v>46266</v>
       </c>
       <c r="B1331" t="n">
-        <v>1317</v>
+        <v>2547</v>
       </c>
       <c r="C1331" t="n">
-        <v>286356</v>
+        <v>41139.75</v>
       </c>
     </row>
     <row r="1332">
@@ -15084,10 +15084,10 @@
         <v>46266</v>
       </c>
       <c r="B1332" t="n">
-        <v>2790</v>
+        <v>2552</v>
       </c>
       <c r="C1332" t="n">
-        <v>60795</v>
+        <v>29584.24</v>
       </c>
     </row>
     <row r="1333">
@@ -15095,10 +15095,10 @@
         <v>46266</v>
       </c>
       <c r="B1333" t="n">
-        <v>2711</v>
+        <v>131</v>
       </c>
       <c r="C1333" t="n">
-        <v>82747.64</v>
+        <v>409000</v>
       </c>
     </row>
     <row r="1334">
@@ -15106,10 +15106,10 @@
         <v>46266</v>
       </c>
       <c r="B1334" t="n">
-        <v>2607</v>
+        <v>2250</v>
       </c>
       <c r="C1334" t="n">
-        <v>47425.64</v>
+        <v>330913.83</v>
       </c>
     </row>
     <row r="1335">
@@ -15117,10 +15117,10 @@
         <v>46266</v>
       </c>
       <c r="B1335" t="n">
-        <v>2667</v>
+        <v>89</v>
       </c>
       <c r="C1335" t="n">
-        <v>43622.73</v>
+        <v>338186.71</v>
       </c>
     </row>
     <row r="1336">
@@ -15128,10 +15128,10 @@
         <v>46266</v>
       </c>
       <c r="B1336" t="n">
-        <v>2706</v>
+        <v>2141</v>
       </c>
       <c r="C1336" t="n">
-        <v>21030.55</v>
+        <v>31645.3</v>
       </c>
     </row>
     <row r="1337">
@@ -15139,10 +15139,10 @@
         <v>46266</v>
       </c>
       <c r="B1337" t="n">
-        <v>2657</v>
+        <v>2798</v>
       </c>
       <c r="C1337" t="n">
-        <v>75596.19</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1338">
@@ -15150,10 +15150,10 @@
         <v>46266</v>
       </c>
       <c r="B1338" t="n">
-        <v>1278</v>
+        <v>2797</v>
       </c>
       <c r="C1338" t="n">
-        <v>95445</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1339">
@@ -15161,10 +15161,10 @@
         <v>46266</v>
       </c>
       <c r="B1339" t="n">
-        <v>2745</v>
+        <v>2266</v>
       </c>
       <c r="C1339" t="n">
-        <v>105000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="1340">
@@ -15172,10 +15172,10 @@
         <v>46266</v>
       </c>
       <c r="B1340" t="n">
-        <v>2753</v>
+        <v>1499</v>
       </c>
       <c r="C1340" t="n">
-        <v>71589</v>
+        <v>140000</v>
       </c>
     </row>
     <row r="1341">
@@ -15183,10 +15183,10 @@
         <v>46266</v>
       </c>
       <c r="B1341" t="n">
-        <v>2183</v>
+        <v>2496</v>
       </c>
       <c r="C1341" t="n">
-        <v>349314</v>
+        <v>160000</v>
       </c>
     </row>
     <row r="1342">
@@ -15194,10 +15194,10 @@
         <v>46266</v>
       </c>
       <c r="B1342" t="n">
-        <v>1340</v>
+        <v>949</v>
       </c>
       <c r="C1342" t="n">
-        <v>138390</v>
+        <v>98163.42</v>
       </c>
     </row>
     <row r="1343">
@@ -15205,10 +15205,10 @@
         <v>46266</v>
       </c>
       <c r="B1343" t="n">
-        <v>2583</v>
+        <v>1853</v>
       </c>
       <c r="C1343" t="n">
-        <v>39711</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="1344">
@@ -15216,10 +15216,10 @@
         <v>46266</v>
       </c>
       <c r="B1344" t="n">
-        <v>2090</v>
+        <v>854</v>
       </c>
       <c r="C1344" t="n">
-        <v>39711</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="1345">
@@ -15227,10 +15227,10 @@
         <v>46266</v>
       </c>
       <c r="B1345" t="n">
-        <v>1277</v>
+        <v>2674</v>
       </c>
       <c r="C1345" t="n">
-        <v>210000</v>
+        <v>260000</v>
       </c>
     </row>
     <row r="1346">
@@ -15238,10 +15238,10 @@
         <v>46266</v>
       </c>
       <c r="B1346" t="n">
-        <v>1501</v>
+        <v>2803</v>
       </c>
       <c r="C1346" t="n">
-        <v>90678</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="1347">
@@ -15249,10 +15249,296 @@
         <v>46266</v>
       </c>
       <c r="B1347" t="n">
-        <v>703</v>
+        <v>2599</v>
       </c>
       <c r="C1347" t="n">
-        <v>238623</v>
+        <v>190000</v>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1348" t="n">
+        <v>783</v>
+      </c>
+      <c r="C1348" t="n">
+        <v>52000</v>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1349" t="n">
+        <v>27</v>
+      </c>
+      <c r="C1349" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1350" t="n">
+        <v>531</v>
+      </c>
+      <c r="C1350" t="n">
+        <v>350000</v>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1351" t="n">
+        <v>1308</v>
+      </c>
+      <c r="C1351" t="n">
+        <v>159657.08</v>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1352" t="n">
+        <v>2792</v>
+      </c>
+      <c r="C1352" t="n">
+        <v>114633.65</v>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1353" t="n">
+        <v>2828</v>
+      </c>
+      <c r="C1353" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1354" t="n">
+        <v>2823</v>
+      </c>
+      <c r="C1354" t="n">
+        <v>93500</v>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1355" t="n">
+        <v>2584</v>
+      </c>
+      <c r="C1355" t="n">
+        <v>62949.9</v>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1356" t="n">
+        <v>945</v>
+      </c>
+      <c r="C1356" t="n">
+        <v>283334.51</v>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1357" t="n">
+        <v>2660</v>
+      </c>
+      <c r="C1357" t="n">
+        <v>310000</v>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1358" t="n">
+        <v>1317</v>
+      </c>
+      <c r="C1358" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1359" t="n">
+        <v>2839</v>
+      </c>
+      <c r="C1359" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1360" t="n">
+        <v>2790</v>
+      </c>
+      <c r="C1360" t="n">
+        <v>63700</v>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1361" t="n">
+        <v>2711</v>
+      </c>
+      <c r="C1361" t="n">
+        <v>86709.92</v>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1362" t="n">
+        <v>2607</v>
+      </c>
+      <c r="C1362" t="n">
+        <v>49700</v>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1363" t="n">
+        <v>2667</v>
+      </c>
+      <c r="C1363" t="n">
+        <v>45700</v>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1364" t="n">
+        <v>2706</v>
+      </c>
+      <c r="C1364" t="n">
+        <v>22050</v>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1365" t="n">
+        <v>2657</v>
+      </c>
+      <c r="C1365" t="n">
+        <v>79200</v>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1366" t="n">
+        <v>1278</v>
+      </c>
+      <c r="C1366" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1367" t="n">
+        <v>2745</v>
+      </c>
+      <c r="C1367" t="n">
+        <v>110000</v>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1368" t="n">
+        <v>2753</v>
+      </c>
+      <c r="C1368" t="n">
+        <v>75000</v>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1369" t="n">
+        <v>2183</v>
+      </c>
+      <c r="C1369" t="n">
+        <v>365968.86</v>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1370" t="n">
+        <v>1340</v>
+      </c>
+      <c r="C1370" t="n">
+        <v>145000</v>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1371" t="n">
+        <v>2583</v>
+      </c>
+      <c r="C1371" t="n">
+        <v>41610.39</v>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1372" t="n">
+        <v>2090</v>
+      </c>
+      <c r="C1372" t="n">
+        <v>41610.33</v>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1373" t="n">
+        <v>1277</v>
+      </c>
+      <c r="C1373" t="n">
+        <v>220000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:01:23
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1577"/>
+  <dimension ref="A1:C1598"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15557,10 +15557,10 @@
         <v>46296</v>
       </c>
       <c r="B1375" t="n">
-        <v>2785</v>
+        <v>675</v>
       </c>
       <c r="C1375" t="n">
-        <v>11346</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1376">
@@ -15568,10 +15568,10 @@
         <v>46296</v>
       </c>
       <c r="B1376" t="n">
-        <v>2809</v>
+        <v>2804</v>
       </c>
       <c r="C1376" t="n">
-        <v>18732</v>
+        <v>31815</v>
       </c>
     </row>
     <row r="1377">
@@ -15579,10 +15579,10 @@
         <v>46296</v>
       </c>
       <c r="B1377" t="n">
-        <v>2494</v>
+        <v>2714</v>
       </c>
       <c r="C1377" t="n">
-        <v>40908</v>
+        <v>114541</v>
       </c>
     </row>
     <row r="1378">
@@ -15590,10 +15590,10 @@
         <v>46296</v>
       </c>
       <c r="B1378" t="n">
-        <v>2652</v>
+        <v>2765</v>
       </c>
       <c r="C1378" t="n">
-        <v>38178</v>
+        <v>28630</v>
       </c>
     </row>
     <row r="1379">
@@ -15601,10 +15601,10 @@
         <v>46296</v>
       </c>
       <c r="B1379" t="n">
-        <v>360</v>
+        <v>2359</v>
       </c>
       <c r="C1379" t="n">
-        <v>136362</v>
+        <v>33194</v>
       </c>
     </row>
     <row r="1380">
@@ -15612,10 +15612,10 @@
         <v>46296</v>
       </c>
       <c r="B1380" t="n">
-        <v>2767</v>
+        <v>2678</v>
       </c>
       <c r="C1380" t="n">
-        <v>51816</v>
+        <v>31486</v>
       </c>
     </row>
     <row r="1381">
@@ -15623,10 +15623,10 @@
         <v>46296</v>
       </c>
       <c r="B1381" t="n">
-        <v>2711</v>
+        <v>2697</v>
       </c>
       <c r="C1381" t="n">
-        <v>23610</v>
+        <v>47782</v>
       </c>
     </row>
     <row r="1382">
@@ -15634,10 +15634,10 @@
         <v>46296</v>
       </c>
       <c r="B1382" t="n">
-        <v>1102</v>
+        <v>2498</v>
       </c>
       <c r="C1382" t="n">
-        <v>64122</v>
+        <v>17913</v>
       </c>
     </row>
     <row r="1383">
@@ -15645,10 +15645,10 @@
         <v>46296</v>
       </c>
       <c r="B1383" t="n">
-        <v>353</v>
+        <v>2641</v>
       </c>
       <c r="C1383" t="n">
-        <v>79782</v>
+        <v>47726</v>
       </c>
     </row>
     <row r="1384">
@@ -15656,10 +15656,10 @@
         <v>46296</v>
       </c>
       <c r="B1384" t="n">
-        <v>2250</v>
+        <v>2801</v>
       </c>
       <c r="C1384" t="n">
-        <v>92724</v>
+        <v>31815</v>
       </c>
     </row>
     <row r="1385">
@@ -15667,10 +15667,10 @@
         <v>46296</v>
       </c>
       <c r="B1385" t="n">
-        <v>1800</v>
+        <v>2810</v>
       </c>
       <c r="C1385" t="n">
-        <v>7734</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1386">
@@ -15678,10 +15678,10 @@
         <v>46296</v>
       </c>
       <c r="B1386" t="n">
-        <v>2726</v>
+        <v>2245</v>
       </c>
       <c r="C1386" t="n">
-        <v>42270</v>
+        <v>70448</v>
       </c>
     </row>
     <row r="1387">
@@ -15689,10 +15689,10 @@
         <v>46296</v>
       </c>
       <c r="B1387" t="n">
-        <v>2729</v>
+        <v>2251</v>
       </c>
       <c r="C1387" t="n">
-        <v>24540</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1388">
@@ -15700,10 +15700,10 @@
         <v>46296</v>
       </c>
       <c r="B1388" t="n">
-        <v>2830</v>
+        <v>2142</v>
       </c>
       <c r="C1388" t="n">
-        <v>24540</v>
+        <v>17220</v>
       </c>
     </row>
     <row r="1389">
@@ -15711,10 +15711,10 @@
         <v>46296</v>
       </c>
       <c r="B1389" t="n">
-        <v>2674</v>
+        <v>664</v>
       </c>
       <c r="C1389" t="n">
-        <v>70908</v>
+        <v>83363</v>
       </c>
     </row>
     <row r="1390">
@@ -15722,10 +15722,10 @@
         <v>46296</v>
       </c>
       <c r="B1390" t="n">
-        <v>2308</v>
+        <v>2472</v>
       </c>
       <c r="C1390" t="n">
-        <v>54540</v>
+        <v>16842</v>
       </c>
     </row>
     <row r="1391">
@@ -15733,10 +15733,10 @@
         <v>46296</v>
       </c>
       <c r="B1391" t="n">
-        <v>2601</v>
+        <v>2659</v>
       </c>
       <c r="C1391" t="n">
-        <v>75000</v>
+        <v>39137</v>
       </c>
     </row>
     <row r="1392">
@@ -15744,10 +15744,10 @@
         <v>46296</v>
       </c>
       <c r="B1392" t="n">
-        <v>2015</v>
+        <v>2583</v>
       </c>
       <c r="C1392" t="n">
-        <v>100908</v>
+        <v>13237</v>
       </c>
     </row>
     <row r="1393">
@@ -15755,10 +15755,10 @@
         <v>46296</v>
       </c>
       <c r="B1393" t="n">
-        <v>2607</v>
+        <v>2692</v>
       </c>
       <c r="C1393" t="n">
-        <v>13548</v>
+        <v>19782</v>
       </c>
     </row>
     <row r="1394">
@@ -15766,10 +15766,10 @@
         <v>46296</v>
       </c>
       <c r="B1394" t="n">
-        <v>2707</v>
+        <v>2691</v>
       </c>
       <c r="C1394" t="n">
-        <v>11778</v>
+        <v>31815</v>
       </c>
     </row>
     <row r="1395">
@@ -15777,10 +15777,10 @@
         <v>46296</v>
       </c>
       <c r="B1395" t="n">
-        <v>569</v>
+        <v>2785</v>
       </c>
       <c r="C1395" t="n">
-        <v>791844</v>
+        <v>13237</v>
       </c>
     </row>
     <row r="1396">
@@ -15788,10 +15788,10 @@
         <v>46296</v>
       </c>
       <c r="B1396" t="n">
-        <v>2660</v>
+        <v>2809</v>
       </c>
       <c r="C1396" t="n">
-        <v>95454</v>
+        <v>21854</v>
       </c>
     </row>
     <row r="1397">
@@ -15799,10 +15799,10 @@
         <v>46296</v>
       </c>
       <c r="B1397" t="n">
-        <v>1632</v>
+        <v>2494</v>
       </c>
       <c r="C1397" t="n">
-        <v>70908</v>
+        <v>47726</v>
       </c>
     </row>
     <row r="1398">
@@ -15810,10 +15810,10 @@
         <v>46296</v>
       </c>
       <c r="B1398" t="n">
-        <v>1756</v>
+        <v>2652</v>
       </c>
       <c r="C1398" t="n">
-        <v>114540</v>
+        <v>44541</v>
       </c>
     </row>
     <row r="1399">
@@ -15821,10 +15821,10 @@
         <v>46296</v>
       </c>
       <c r="B1399" t="n">
-        <v>58</v>
+        <v>360</v>
       </c>
       <c r="C1399" t="n">
-        <v>68400</v>
+        <v>159089</v>
       </c>
     </row>
     <row r="1400">
@@ -15832,10 +15832,10 @@
         <v>46296</v>
       </c>
       <c r="B1400" t="n">
-        <v>40</v>
+        <v>2767</v>
       </c>
       <c r="C1400" t="n">
-        <v>60840</v>
+        <v>60452</v>
       </c>
     </row>
     <row r="1401">
@@ -15843,10 +15843,10 @@
         <v>46296</v>
       </c>
       <c r="B1401" t="n">
-        <v>559</v>
+        <v>2107</v>
       </c>
       <c r="C1401" t="n">
-        <v>63816</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1402">
@@ -15854,10 +15854,10 @@
         <v>46296</v>
       </c>
       <c r="B1402" t="n">
-        <v>2773</v>
+        <v>2711</v>
       </c>
       <c r="C1402" t="n">
-        <v>22002</v>
+        <v>27545</v>
       </c>
     </row>
     <row r="1403">
@@ -15865,10 +15865,10 @@
         <v>46296</v>
       </c>
       <c r="B1403" t="n">
-        <v>2631</v>
+        <v>1102</v>
       </c>
       <c r="C1403" t="n">
-        <v>10566</v>
+        <v>74809</v>
       </c>
     </row>
     <row r="1404">
@@ -15876,10 +15876,10 @@
         <v>46296</v>
       </c>
       <c r="B1404" t="n">
-        <v>1642</v>
+        <v>353</v>
       </c>
       <c r="C1404" t="n">
-        <v>72270</v>
+        <v>93079</v>
       </c>
     </row>
     <row r="1405">
@@ -15887,10 +15887,10 @@
         <v>46296</v>
       </c>
       <c r="B1405" t="n">
-        <v>2621</v>
+        <v>2250</v>
       </c>
       <c r="C1405" t="n">
-        <v>19086</v>
+        <v>108178</v>
       </c>
     </row>
     <row r="1406">
@@ -15898,10 +15898,10 @@
         <v>46296</v>
       </c>
       <c r="B1406" t="n">
-        <v>2735</v>
+        <v>1800</v>
       </c>
       <c r="C1406" t="n">
-        <v>32724</v>
+        <v>9023</v>
       </c>
     </row>
     <row r="1407">
@@ -15909,10 +15909,10 @@
         <v>46296</v>
       </c>
       <c r="B1407" t="n">
-        <v>945</v>
+        <v>2682</v>
       </c>
       <c r="C1407" t="n">
-        <v>95640</v>
+        <v>44541</v>
       </c>
     </row>
     <row r="1408">
@@ -15920,10 +15920,10 @@
         <v>46296</v>
       </c>
       <c r="B1408" t="n">
-        <v>2629</v>
+        <v>2786</v>
       </c>
       <c r="C1408" t="n">
-        <v>18732</v>
+        <v>22267</v>
       </c>
     </row>
     <row r="1409">
@@ -15931,10 +15931,10 @@
         <v>46296</v>
       </c>
       <c r="B1409" t="n">
-        <v>933</v>
+        <v>2816</v>
       </c>
       <c r="C1409" t="n">
-        <v>22224</v>
+        <v>41363</v>
       </c>
     </row>
     <row r="1410">
@@ -15942,10 +15942,10 @@
         <v>46296</v>
       </c>
       <c r="B1410" t="n">
-        <v>2721</v>
+        <v>2090</v>
       </c>
       <c r="C1410" t="n">
-        <v>22224</v>
+        <v>13237</v>
       </c>
     </row>
     <row r="1411">
@@ -15953,10 +15953,10 @@
         <v>46296</v>
       </c>
       <c r="B1411" t="n">
-        <v>2826</v>
+        <v>766</v>
       </c>
       <c r="C1411" t="n">
-        <v>19086</v>
+        <v>21854</v>
       </c>
     </row>
     <row r="1412">
@@ -15964,10 +15964,10 @@
         <v>46296</v>
       </c>
       <c r="B1412" t="n">
-        <v>2346</v>
+        <v>2702</v>
       </c>
       <c r="C1412" t="n">
-        <v>19086</v>
+        <v>25928</v>
       </c>
     </row>
     <row r="1413">
@@ -15975,10 +15975,10 @@
         <v>46296</v>
       </c>
       <c r="B1413" t="n">
-        <v>2686</v>
+        <v>2772</v>
       </c>
       <c r="C1413" t="n">
-        <v>38178</v>
+        <v>19089</v>
       </c>
     </row>
     <row r="1414">
@@ -15986,10 +15986,10 @@
         <v>46296</v>
       </c>
       <c r="B1414" t="n">
-        <v>2566</v>
+        <v>767</v>
       </c>
       <c r="C1414" t="n">
-        <v>21816</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1415">
@@ -15997,10 +15997,10 @@
         <v>46296</v>
       </c>
       <c r="B1415" t="n">
-        <v>2684</v>
+        <v>2727</v>
       </c>
       <c r="C1415" t="n">
-        <v>25908</v>
+        <v>12880</v>
       </c>
     </row>
     <row r="1416">
@@ -16008,10 +16008,10 @@
         <v>46296</v>
       </c>
       <c r="B1416" t="n">
-        <v>2375</v>
+        <v>2846</v>
       </c>
       <c r="C1416" t="n">
-        <v>90000</v>
+        <v>82726</v>
       </c>
     </row>
     <row r="1417">
@@ -16019,10 +16019,10 @@
         <v>46296</v>
       </c>
       <c r="B1417" t="n">
-        <v>525</v>
+        <v>609</v>
       </c>
       <c r="C1417" t="n">
-        <v>64086</v>
+        <v>71589</v>
       </c>
     </row>
     <row r="1418">
@@ -16030,10 +16030,10 @@
         <v>46296</v>
       </c>
       <c r="B1418" t="n">
-        <v>1064</v>
+        <v>2726</v>
       </c>
       <c r="C1418" t="n">
-        <v>163632</v>
+        <v>49315</v>
       </c>
     </row>
     <row r="1419">
@@ -16041,10 +16041,10 @@
         <v>46296</v>
       </c>
       <c r="B1419" t="n">
-        <v>1810</v>
+        <v>2729</v>
       </c>
       <c r="C1419" t="n">
-        <v>11076</v>
+        <v>28630</v>
       </c>
     </row>
     <row r="1420">
@@ -16052,10 +16052,10 @@
         <v>46296</v>
       </c>
       <c r="B1420" t="n">
-        <v>1937</v>
+        <v>2830</v>
       </c>
       <c r="C1420" t="n">
-        <v>70632</v>
+        <v>28630</v>
       </c>
     </row>
     <row r="1421">
@@ -16063,10 +16063,10 @@
         <v>46296</v>
       </c>
       <c r="B1421" t="n">
-        <v>483</v>
+        <v>2674</v>
       </c>
       <c r="C1421" t="n">
-        <v>123270</v>
+        <v>82726</v>
       </c>
     </row>
     <row r="1422">
@@ -16074,10 +16074,10 @@
         <v>46296</v>
       </c>
       <c r="B1422" t="n">
-        <v>2580</v>
+        <v>2308</v>
       </c>
       <c r="C1422" t="n">
-        <v>9186</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1423">
@@ -16085,10 +16085,10 @@
         <v>46296</v>
       </c>
       <c r="B1423" t="n">
-        <v>2706</v>
+        <v>2601</v>
       </c>
       <c r="C1423" t="n">
-        <v>7176</v>
+        <v>87500</v>
       </c>
     </row>
     <row r="1424">
@@ -16096,10 +16096,10 @@
         <v>46296</v>
       </c>
       <c r="B1424" t="n">
-        <v>2633</v>
+        <v>2015</v>
       </c>
       <c r="C1424" t="n">
-        <v>5256</v>
+        <v>117726</v>
       </c>
     </row>
     <row r="1425">
@@ -16107,10 +16107,10 @@
         <v>46296</v>
       </c>
       <c r="B1425" t="n">
-        <v>2811</v>
+        <v>1308</v>
       </c>
       <c r="C1425" t="n">
-        <v>11346</v>
+        <v>49952</v>
       </c>
     </row>
     <row r="1426">
@@ -16118,10 +16118,10 @@
         <v>46296</v>
       </c>
       <c r="B1426" t="n">
-        <v>1881</v>
+        <v>2118</v>
       </c>
       <c r="C1426" t="n">
-        <v>18732</v>
+        <v>66871</v>
       </c>
     </row>
     <row r="1427">
@@ -16129,10 +16129,10 @@
         <v>46296</v>
       </c>
       <c r="B1427" t="n">
-        <v>970</v>
+        <v>2607</v>
       </c>
       <c r="C1427" t="n">
-        <v>18732</v>
+        <v>15806</v>
       </c>
     </row>
     <row r="1428">
@@ -16140,10 +16140,10 @@
         <v>46296</v>
       </c>
       <c r="B1428" t="n">
-        <v>2761</v>
+        <v>2707</v>
       </c>
       <c r="C1428" t="n">
-        <v>22224</v>
+        <v>13741</v>
       </c>
     </row>
     <row r="1429">
@@ -16151,10 +16151,10 @@
         <v>46296</v>
       </c>
       <c r="B1429" t="n">
-        <v>2747</v>
+        <v>2383</v>
       </c>
       <c r="C1429" t="n">
-        <v>19086</v>
+        <v>42294</v>
       </c>
     </row>
     <row r="1430">
@@ -16162,10 +16162,10 @@
         <v>46296</v>
       </c>
       <c r="B1430" t="n">
-        <v>2544</v>
+        <v>2821</v>
       </c>
       <c r="C1430" t="n">
-        <v>19086</v>
+        <v>42427</v>
       </c>
     </row>
     <row r="1431">
@@ -16173,10 +16173,10 @@
         <v>46296</v>
       </c>
       <c r="B1431" t="n">
-        <v>358</v>
+        <v>569</v>
       </c>
       <c r="C1431" t="n">
-        <v>85908</v>
+        <v>923818</v>
       </c>
     </row>
     <row r="1432">
@@ -16184,10 +16184,10 @@
         <v>46296</v>
       </c>
       <c r="B1432" t="n">
-        <v>1653</v>
+        <v>2660</v>
       </c>
       <c r="C1432" t="n">
-        <v>85908</v>
+        <v>111363</v>
       </c>
     </row>
     <row r="1433">
@@ -16195,10 +16195,10 @@
         <v>46296</v>
       </c>
       <c r="B1433" t="n">
-        <v>675</v>
+        <v>1632</v>
       </c>
       <c r="C1433" t="n">
-        <v>54540</v>
+        <v>82726</v>
       </c>
     </row>
     <row r="1434">
@@ -16206,10 +16206,10 @@
         <v>46296</v>
       </c>
       <c r="B1434" t="n">
-        <v>2804</v>
+        <v>1756</v>
       </c>
       <c r="C1434" t="n">
-        <v>27270</v>
+        <v>133630</v>
       </c>
     </row>
     <row r="1435">
@@ -16217,10 +16217,10 @@
         <v>46296</v>
       </c>
       <c r="B1435" t="n">
-        <v>2714</v>
+        <v>58</v>
       </c>
       <c r="C1435" t="n">
-        <v>98178</v>
+        <v>79800</v>
       </c>
     </row>
     <row r="1436">
@@ -16228,10 +16228,10 @@
         <v>46296</v>
       </c>
       <c r="B1436" t="n">
-        <v>2765</v>
+        <v>40</v>
       </c>
       <c r="C1436" t="n">
-        <v>24540</v>
+        <v>70980</v>
       </c>
     </row>
     <row r="1437">
@@ -16239,10 +16239,10 @@
         <v>46296</v>
       </c>
       <c r="B1437" t="n">
-        <v>2498</v>
+        <v>559</v>
       </c>
       <c r="C1437" t="n">
-        <v>15354</v>
+        <v>74452</v>
       </c>
     </row>
     <row r="1438">
@@ -16250,10 +16250,10 @@
         <v>46296</v>
       </c>
       <c r="B1438" t="n">
-        <v>2641</v>
+        <v>2773</v>
       </c>
       <c r="C1438" t="n">
-        <v>40908</v>
+        <v>25669</v>
       </c>
     </row>
     <row r="1439">
@@ -16261,10 +16261,10 @@
         <v>46296</v>
       </c>
       <c r="B1439" t="n">
-        <v>2801</v>
+        <v>2631</v>
       </c>
       <c r="C1439" t="n">
-        <v>27270</v>
+        <v>12327</v>
       </c>
     </row>
     <row r="1440">
@@ -16272,10 +16272,10 @@
         <v>46296</v>
       </c>
       <c r="B1440" t="n">
-        <v>2810</v>
+        <v>1642</v>
       </c>
       <c r="C1440" t="n">
-        <v>43632</v>
+        <v>84315</v>
       </c>
     </row>
     <row r="1441">
@@ -16283,10 +16283,10 @@
         <v>46296</v>
       </c>
       <c r="B1441" t="n">
-        <v>2245</v>
+        <v>2621</v>
       </c>
       <c r="C1441" t="n">
-        <v>60384</v>
+        <v>22267</v>
       </c>
     </row>
     <row r="1442">
@@ -16294,10 +16294,10 @@
         <v>46296</v>
       </c>
       <c r="B1442" t="n">
-        <v>2251</v>
+        <v>2735</v>
       </c>
       <c r="C1442" t="n">
-        <v>54540</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1443">
@@ -16305,10 +16305,10 @@
         <v>46296</v>
       </c>
       <c r="B1443" t="n">
-        <v>2142</v>
+        <v>945</v>
       </c>
       <c r="C1443" t="n">
-        <v>14760</v>
+        <v>111580</v>
       </c>
     </row>
     <row r="1444">
@@ -16316,10 +16316,10 @@
         <v>46296</v>
       </c>
       <c r="B1444" t="n">
-        <v>664</v>
+        <v>2629</v>
       </c>
       <c r="C1444" t="n">
-        <v>71454</v>
+        <v>21854</v>
       </c>
     </row>
     <row r="1445">
@@ -16327,10 +16327,10 @@
         <v>46296</v>
       </c>
       <c r="B1445" t="n">
-        <v>2472</v>
+        <v>933</v>
       </c>
       <c r="C1445" t="n">
-        <v>14436</v>
+        <v>25928</v>
       </c>
     </row>
     <row r="1446">
@@ -16338,10 +16338,10 @@
         <v>46296</v>
       </c>
       <c r="B1446" t="n">
-        <v>2659</v>
+        <v>2721</v>
       </c>
       <c r="C1446" t="n">
-        <v>33546</v>
+        <v>25928</v>
       </c>
     </row>
     <row r="1447">
@@ -16349,10 +16349,10 @@
         <v>46296</v>
       </c>
       <c r="B1447" t="n">
-        <v>2583</v>
+        <v>2826</v>
       </c>
       <c r="C1447" t="n">
-        <v>11346</v>
+        <v>22267</v>
       </c>
     </row>
     <row r="1448">
@@ -16360,10 +16360,10 @@
         <v>46296</v>
       </c>
       <c r="B1448" t="n">
-        <v>2692</v>
+        <v>2346</v>
       </c>
       <c r="C1448" t="n">
-        <v>16956</v>
+        <v>22267</v>
       </c>
     </row>
     <row r="1449">
@@ -16371,10 +16371,10 @@
         <v>46296</v>
       </c>
       <c r="B1449" t="n">
-        <v>2691</v>
+        <v>2686</v>
       </c>
       <c r="C1449" t="n">
-        <v>27270</v>
+        <v>44541</v>
       </c>
     </row>
     <row r="1450">
@@ -16382,10 +16382,10 @@
         <v>46296</v>
       </c>
       <c r="B1450" t="n">
-        <v>953</v>
+        <v>2566</v>
       </c>
       <c r="C1450" t="n">
-        <v>188178</v>
+        <v>25452</v>
       </c>
     </row>
     <row r="1451">
@@ -16393,10 +16393,10 @@
         <v>46296</v>
       </c>
       <c r="B1451" t="n">
-        <v>610</v>
+        <v>2684</v>
       </c>
       <c r="C1451" t="n">
-        <v>224124</v>
+        <v>30226</v>
       </c>
     </row>
     <row r="1452">
@@ -16404,10 +16404,10 @@
         <v>46296</v>
       </c>
       <c r="B1452" t="n">
-        <v>2834</v>
+        <v>2375</v>
       </c>
       <c r="C1452" t="n">
-        <v>10164</v>
+        <v>105000</v>
       </c>
     </row>
     <row r="1453">
@@ -16415,10 +16415,10 @@
         <v>46296</v>
       </c>
       <c r="B1453" t="n">
-        <v>952</v>
+        <v>2507</v>
       </c>
       <c r="C1453" t="n">
-        <v>27270</v>
+        <v>28420</v>
       </c>
     </row>
     <row r="1454">
@@ -16426,10 +16426,10 @@
         <v>46296</v>
       </c>
       <c r="B1454" t="n">
-        <v>1539</v>
+        <v>1906</v>
       </c>
       <c r="C1454" t="n">
-        <v>46362</v>
+        <v>34545</v>
       </c>
     </row>
     <row r="1455">
@@ -16437,10 +16437,10 @@
         <v>46296</v>
       </c>
       <c r="B1455" t="n">
-        <v>793</v>
+        <v>525</v>
       </c>
       <c r="C1455" t="n">
-        <v>11346</v>
+        <v>74767</v>
       </c>
     </row>
     <row r="1456">
@@ -16448,10 +16448,10 @@
         <v>46296</v>
       </c>
       <c r="B1456" t="n">
-        <v>794</v>
+        <v>1064</v>
       </c>
       <c r="C1456" t="n">
-        <v>11346</v>
+        <v>190904</v>
       </c>
     </row>
     <row r="1457">
@@ -16459,10 +16459,10 @@
         <v>46296</v>
       </c>
       <c r="B1457" t="n">
-        <v>2838</v>
+        <v>1810</v>
       </c>
       <c r="C1457" t="n">
-        <v>13632</v>
+        <v>12922</v>
       </c>
     </row>
     <row r="1458">
@@ -16470,10 +16470,10 @@
         <v>46296</v>
       </c>
       <c r="B1458" t="n">
-        <v>2762</v>
+        <v>1937</v>
       </c>
       <c r="C1458" t="n">
-        <v>22224</v>
+        <v>82404</v>
       </c>
     </row>
     <row r="1459">
@@ -16481,10 +16481,10 @@
         <v>46296</v>
       </c>
       <c r="B1459" t="n">
-        <v>749</v>
+        <v>483</v>
       </c>
       <c r="C1459" t="n">
-        <v>22224</v>
+        <v>143815</v>
       </c>
     </row>
     <row r="1460">
@@ -16492,10 +16492,10 @@
         <v>46296</v>
       </c>
       <c r="B1460" t="n">
-        <v>2258</v>
+        <v>2580</v>
       </c>
       <c r="C1460" t="n">
-        <v>21816</v>
+        <v>10717</v>
       </c>
     </row>
     <row r="1461">
@@ -16503,10 +16503,10 @@
         <v>46296</v>
       </c>
       <c r="B1461" t="n">
-        <v>2744</v>
+        <v>2706</v>
       </c>
       <c r="C1461" t="n">
-        <v>16362</v>
+        <v>8372</v>
       </c>
     </row>
     <row r="1462">
@@ -16514,10 +16514,10 @@
         <v>46296</v>
       </c>
       <c r="B1462" t="n">
-        <v>2653</v>
+        <v>2633</v>
       </c>
       <c r="C1462" t="n">
-        <v>16362</v>
+        <v>6132</v>
       </c>
     </row>
     <row r="1463">
@@ -16525,10 +16525,10 @@
         <v>46296</v>
       </c>
       <c r="B1463" t="n">
-        <v>2742</v>
+        <v>2811</v>
       </c>
       <c r="C1463" t="n">
-        <v>16362</v>
+        <v>13237</v>
       </c>
     </row>
     <row r="1464">
@@ -16536,10 +16536,10 @@
         <v>46296</v>
       </c>
       <c r="B1464" t="n">
-        <v>1499</v>
+        <v>1881</v>
       </c>
       <c r="C1464" t="n">
-        <v>24540</v>
+        <v>21854</v>
       </c>
     </row>
     <row r="1465">
@@ -16547,10 +16547,10 @@
         <v>46296</v>
       </c>
       <c r="B1465" t="n">
-        <v>2261</v>
+        <v>970</v>
       </c>
       <c r="C1465" t="n">
-        <v>49086</v>
+        <v>21854</v>
       </c>
     </row>
     <row r="1466">
@@ -16558,10 +16558,10 @@
         <v>46296</v>
       </c>
       <c r="B1466" t="n">
-        <v>2709</v>
+        <v>2761</v>
       </c>
       <c r="C1466" t="n">
-        <v>49086</v>
+        <v>25928</v>
       </c>
     </row>
     <row r="1467">
@@ -16569,10 +16569,10 @@
         <v>46296</v>
       </c>
       <c r="B1467" t="n">
-        <v>1137</v>
+        <v>2747</v>
       </c>
       <c r="C1467" t="n">
-        <v>174540</v>
+        <v>22267</v>
       </c>
     </row>
     <row r="1468">
@@ -16580,10 +16580,10 @@
         <v>46296</v>
       </c>
       <c r="B1468" t="n">
-        <v>429</v>
+        <v>2544</v>
       </c>
       <c r="C1468" t="n">
-        <v>103632</v>
+        <v>22267</v>
       </c>
     </row>
     <row r="1469">
@@ -16591,10 +16591,10 @@
         <v>46296</v>
       </c>
       <c r="B1469" t="n">
-        <v>2695</v>
+        <v>358</v>
       </c>
       <c r="C1469" t="n">
-        <v>13194</v>
+        <v>100226</v>
       </c>
     </row>
     <row r="1470">
@@ -16602,10 +16602,10 @@
         <v>46296</v>
       </c>
       <c r="B1470" t="n">
-        <v>1289</v>
+        <v>1653</v>
       </c>
       <c r="C1470" t="n">
-        <v>75000</v>
+        <v>100226</v>
       </c>
     </row>
     <row r="1471">
@@ -16613,10 +16613,10 @@
         <v>46296</v>
       </c>
       <c r="B1471" t="n">
-        <v>2789</v>
+        <v>1317</v>
       </c>
       <c r="C1471" t="n">
-        <v>49086</v>
+        <v>100226</v>
       </c>
     </row>
     <row r="1472">
@@ -16624,10 +16624,10 @@
         <v>46296</v>
       </c>
       <c r="B1472" t="n">
-        <v>2197</v>
+        <v>2822</v>
       </c>
       <c r="C1472" t="n">
-        <v>58632</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1473">
@@ -16635,10 +16635,10 @@
         <v>46296</v>
       </c>
       <c r="B1473" t="n">
-        <v>947</v>
+        <v>1117</v>
       </c>
       <c r="C1473" t="n">
-        <v>120948</v>
+        <v>127309</v>
       </c>
     </row>
     <row r="1474">
@@ -16646,10 +16646,10 @@
         <v>46296</v>
       </c>
       <c r="B1474" t="n">
-        <v>2279</v>
+        <v>1299</v>
       </c>
       <c r="C1474" t="n">
-        <v>66798</v>
+        <v>167853</v>
       </c>
     </row>
     <row r="1475">
@@ -16657,10 +16657,10 @@
         <v>46296</v>
       </c>
       <c r="B1475" t="n">
-        <v>1465</v>
+        <v>477</v>
       </c>
       <c r="C1475" t="n">
-        <v>105000</v>
+        <v>69174</v>
       </c>
     </row>
     <row r="1476">
@@ -16668,10 +16668,10 @@
         <v>46296</v>
       </c>
       <c r="B1476" t="n">
-        <v>2651</v>
+        <v>530</v>
       </c>
       <c r="C1476" t="n">
-        <v>46362</v>
+        <v>95452</v>
       </c>
     </row>
     <row r="1477">
@@ -16679,10 +16679,10 @@
         <v>46296</v>
       </c>
       <c r="B1477" t="n">
-        <v>42</v>
+        <v>953</v>
       </c>
       <c r="C1477" t="n">
-        <v>519816</v>
+        <v>219541</v>
       </c>
     </row>
     <row r="1478">
@@ -16690,10 +16690,10 @@
         <v>46296</v>
       </c>
       <c r="B1478" t="n">
-        <v>2045</v>
+        <v>610</v>
       </c>
       <c r="C1478" t="n">
-        <v>86856</v>
+        <v>261478</v>
       </c>
     </row>
     <row r="1479">
@@ -16701,10 +16701,10 @@
         <v>46296</v>
       </c>
       <c r="B1479" t="n">
-        <v>2663</v>
+        <v>2792</v>
       </c>
       <c r="C1479" t="n">
-        <v>75000</v>
+        <v>65667</v>
       </c>
     </row>
     <row r="1480">
@@ -16712,10 +16712,10 @@
         <v>46296</v>
       </c>
       <c r="B1480" t="n">
-        <v>2823</v>
+        <v>2834</v>
       </c>
       <c r="C1480" t="n">
-        <v>19362</v>
+        <v>11858</v>
       </c>
     </row>
     <row r="1481">
@@ -16723,10 +16723,10 @@
         <v>46296</v>
       </c>
       <c r="B1481" t="n">
-        <v>2757</v>
+        <v>952</v>
       </c>
       <c r="C1481" t="n">
-        <v>21816</v>
+        <v>31815</v>
       </c>
     </row>
     <row r="1482">
@@ -16734,10 +16734,10 @@
         <v>46296</v>
       </c>
       <c r="B1482" t="n">
-        <v>2815</v>
+        <v>1539</v>
       </c>
       <c r="C1482" t="n">
-        <v>16362</v>
+        <v>54089</v>
       </c>
     </row>
     <row r="1483">
@@ -16745,10 +16745,10 @@
         <v>46296</v>
       </c>
       <c r="B1483" t="n">
-        <v>2829</v>
+        <v>793</v>
       </c>
       <c r="C1483" t="n">
-        <v>16362</v>
+        <v>13237</v>
       </c>
     </row>
     <row r="1484">
@@ -16756,10 +16756,10 @@
         <v>46296</v>
       </c>
       <c r="B1484" t="n">
-        <v>2496</v>
+        <v>794</v>
       </c>
       <c r="C1484" t="n">
-        <v>54540</v>
+        <v>13237</v>
       </c>
     </row>
     <row r="1485">
@@ -16767,10 +16767,10 @@
         <v>46296</v>
       </c>
       <c r="B1485" t="n">
-        <v>2131</v>
+        <v>2838</v>
       </c>
       <c r="C1485" t="n">
-        <v>27270</v>
+        <v>15904</v>
       </c>
     </row>
     <row r="1486">
@@ -16778,10 +16778,10 @@
         <v>46296</v>
       </c>
       <c r="B1486" t="n">
-        <v>2847</v>
+        <v>2762</v>
       </c>
       <c r="C1486" t="n">
-        <v>36816</v>
+        <v>25928</v>
       </c>
     </row>
     <row r="1487">
@@ -16789,10 +16789,10 @@
         <v>46296</v>
       </c>
       <c r="B1487" t="n">
-        <v>1293</v>
+        <v>749</v>
       </c>
       <c r="C1487" t="n">
-        <v>105000</v>
+        <v>25928</v>
       </c>
     </row>
     <row r="1488">
@@ -16800,10 +16800,10 @@
         <v>46296</v>
       </c>
       <c r="B1488" t="n">
-        <v>631</v>
+        <v>2258</v>
       </c>
       <c r="C1488" t="n">
-        <v>95454</v>
+        <v>25452</v>
       </c>
     </row>
     <row r="1489">
@@ -16811,10 +16811,10 @@
         <v>46296</v>
       </c>
       <c r="B1489" t="n">
-        <v>2791</v>
+        <v>2744</v>
       </c>
       <c r="C1489" t="n">
-        <v>28002</v>
+        <v>19089</v>
       </c>
     </row>
     <row r="1490">
@@ -16822,10 +16822,10 @@
         <v>46296</v>
       </c>
       <c r="B1490" t="n">
-        <v>2273</v>
+        <v>2653</v>
       </c>
       <c r="C1490" t="n">
-        <v>58638</v>
+        <v>19089</v>
       </c>
     </row>
     <row r="1491">
@@ -16833,10 +16833,10 @@
         <v>46296</v>
       </c>
       <c r="B1491" t="n">
-        <v>2381</v>
+        <v>2742</v>
       </c>
       <c r="C1491" t="n">
-        <v>21930</v>
+        <v>19089</v>
       </c>
     </row>
     <row r="1492">
@@ -16844,10 +16844,10 @@
         <v>46296</v>
       </c>
       <c r="B1492" t="n">
-        <v>630</v>
+        <v>1499</v>
       </c>
       <c r="C1492" t="n">
-        <v>22506</v>
+        <v>28630</v>
       </c>
     </row>
     <row r="1493">
@@ -16855,10 +16855,10 @@
         <v>46296</v>
       </c>
       <c r="B1493" t="n">
-        <v>1983</v>
+        <v>2261</v>
       </c>
       <c r="C1493" t="n">
-        <v>149520</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1494">
@@ -16866,10 +16866,10 @@
         <v>46296</v>
       </c>
       <c r="B1494" t="n">
-        <v>1993</v>
+        <v>2709</v>
       </c>
       <c r="C1494" t="n">
-        <v>101532</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1495">
@@ -16877,10 +16877,10 @@
         <v>46296</v>
       </c>
       <c r="B1495" t="n">
-        <v>89</v>
+        <v>1137</v>
       </c>
       <c r="C1495" t="n">
-        <v>95454</v>
+        <v>203630</v>
       </c>
     </row>
     <row r="1496">
@@ -16888,10 +16888,10 @@
         <v>46296</v>
       </c>
       <c r="B1496" t="n">
-        <v>1063</v>
+        <v>429</v>
       </c>
       <c r="C1496" t="n">
-        <v>105000</v>
+        <v>120904</v>
       </c>
     </row>
     <row r="1497">
@@ -16899,10 +16899,10 @@
         <v>46296</v>
       </c>
       <c r="B1497" t="n">
-        <v>1116</v>
+        <v>2114</v>
       </c>
       <c r="C1497" t="n">
-        <v>68178</v>
+        <v>54131</v>
       </c>
     </row>
     <row r="1498">
@@ -16910,10 +16910,10 @@
         <v>46296</v>
       </c>
       <c r="B1498" t="n">
-        <v>941</v>
+        <v>2211</v>
       </c>
       <c r="C1498" t="n">
-        <v>82062</v>
+        <v>76629</v>
       </c>
     </row>
     <row r="1499">
@@ -16921,10 +16921,10 @@
         <v>46296</v>
       </c>
       <c r="B1499" t="n">
-        <v>2141</v>
+        <v>1108</v>
       </c>
       <c r="C1499" t="n">
-        <v>8748</v>
+        <v>97482</v>
       </c>
     </row>
     <row r="1500">
@@ -16932,10 +16932,10 @@
         <v>46296</v>
       </c>
       <c r="B1500" t="n">
-        <v>2463</v>
+        <v>2695</v>
       </c>
       <c r="C1500" t="n">
-        <v>89952</v>
+        <v>15393</v>
       </c>
     </row>
     <row r="1501">
@@ -16943,10 +16943,10 @@
         <v>46296</v>
       </c>
       <c r="B1501" t="n">
-        <v>1890</v>
+        <v>1289</v>
       </c>
       <c r="C1501" t="n">
-        <v>66882</v>
+        <v>87500</v>
       </c>
     </row>
     <row r="1502">
@@ -16954,10 +16954,10 @@
         <v>46296</v>
       </c>
       <c r="B1502" t="n">
-        <v>2639</v>
+        <v>2789</v>
       </c>
       <c r="C1502" t="n">
-        <v>10926</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1503">
@@ -16965,10 +16965,10 @@
         <v>46296</v>
       </c>
       <c r="B1503" t="n">
-        <v>2682</v>
+        <v>2197</v>
       </c>
       <c r="C1503" t="n">
-        <v>38178</v>
+        <v>68404</v>
       </c>
     </row>
     <row r="1504">
@@ -16976,10 +16976,10 @@
         <v>46296</v>
       </c>
       <c r="B1504" t="n">
-        <v>2786</v>
+        <v>947</v>
       </c>
       <c r="C1504" t="n">
-        <v>19086</v>
+        <v>141106</v>
       </c>
     </row>
     <row r="1505">
@@ -16987,10 +16987,10 @@
         <v>46296</v>
       </c>
       <c r="B1505" t="n">
-        <v>2816</v>
+        <v>2279</v>
       </c>
       <c r="C1505" t="n">
-        <v>35454</v>
+        <v>77931</v>
       </c>
     </row>
     <row r="1506">
@@ -16998,10 +16998,10 @@
         <v>46296</v>
       </c>
       <c r="B1506" t="n">
-        <v>2090</v>
+        <v>1465</v>
       </c>
       <c r="C1506" t="n">
-        <v>11346</v>
+        <v>122500</v>
       </c>
     </row>
     <row r="1507">
@@ -17009,10 +17009,10 @@
         <v>46296</v>
       </c>
       <c r="B1507" t="n">
-        <v>766</v>
+        <v>2651</v>
       </c>
       <c r="C1507" t="n">
-        <v>18732</v>
+        <v>54089</v>
       </c>
     </row>
     <row r="1508">
@@ -17020,10 +17020,10 @@
         <v>46296</v>
       </c>
       <c r="B1508" t="n">
-        <v>2702</v>
+        <v>42</v>
       </c>
       <c r="C1508" t="n">
-        <v>22224</v>
+        <v>606452</v>
       </c>
     </row>
     <row r="1509">
@@ -17031,10 +17031,10 @@
         <v>46296</v>
       </c>
       <c r="B1509" t="n">
-        <v>2772</v>
+        <v>2045</v>
       </c>
       <c r="C1509" t="n">
-        <v>16362</v>
+        <v>101332</v>
       </c>
     </row>
     <row r="1510">
@@ -17042,10 +17042,10 @@
         <v>46296</v>
       </c>
       <c r="B1510" t="n">
-        <v>767</v>
+        <v>2663</v>
       </c>
       <c r="C1510" t="n">
-        <v>54540</v>
+        <v>87500</v>
       </c>
     </row>
     <row r="1511">
@@ -17053,10 +17053,10 @@
         <v>46296</v>
       </c>
       <c r="B1511" t="n">
-        <v>2727</v>
+        <v>2823</v>
       </c>
       <c r="C1511" t="n">
-        <v>11040</v>
+        <v>22589</v>
       </c>
     </row>
     <row r="1512">
@@ -17064,10 +17064,10 @@
         <v>46296</v>
       </c>
       <c r="B1512" t="n">
-        <v>2846</v>
+        <v>2757</v>
       </c>
       <c r="C1512" t="n">
-        <v>70908</v>
+        <v>25452</v>
       </c>
     </row>
     <row r="1513">
@@ -17075,10 +17075,10 @@
         <v>46296</v>
       </c>
       <c r="B1513" t="n">
-        <v>609</v>
+        <v>2815</v>
       </c>
       <c r="C1513" t="n">
-        <v>61362</v>
+        <v>19089</v>
       </c>
     </row>
     <row r="1514">
@@ -17086,10 +17086,10 @@
         <v>46296</v>
       </c>
       <c r="B1514" t="n">
-        <v>1075</v>
+        <v>2829</v>
       </c>
       <c r="C1514" t="n">
-        <v>125178</v>
+        <v>19089</v>
       </c>
     </row>
     <row r="1515">
@@ -17097,10 +17097,10 @@
         <v>46296</v>
       </c>
       <c r="B1515" t="n">
-        <v>131</v>
+        <v>2496</v>
       </c>
       <c r="C1515" t="n">
-        <v>113454</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1516">
@@ -17108,10 +17108,10 @@
         <v>46296</v>
       </c>
       <c r="B1516" t="n">
-        <v>2667</v>
+        <v>2131</v>
       </c>
       <c r="C1516" t="n">
-        <v>12462</v>
+        <v>31815</v>
       </c>
     </row>
     <row r="1517">
@@ -17119,10 +17119,10 @@
         <v>46296</v>
       </c>
       <c r="B1517" t="n">
-        <v>2577</v>
+        <v>2847</v>
       </c>
       <c r="C1517" t="n">
-        <v>24318</v>
+        <v>42952</v>
       </c>
     </row>
     <row r="1518">
@@ -17130,10 +17130,10 @@
         <v>46296</v>
       </c>
       <c r="B1518" t="n">
-        <v>2745</v>
+        <v>1293</v>
       </c>
       <c r="C1518" t="n">
-        <v>30000</v>
+        <v>122500</v>
       </c>
     </row>
     <row r="1519">
@@ -17141,10 +17141,10 @@
         <v>46296</v>
       </c>
       <c r="B1519" t="n">
-        <v>2817</v>
+        <v>631</v>
       </c>
       <c r="C1519" t="n">
-        <v>16362</v>
+        <v>111363</v>
       </c>
     </row>
     <row r="1520">
@@ -17152,10 +17152,10 @@
         <v>46296</v>
       </c>
       <c r="B1520" t="n">
-        <v>2784</v>
+        <v>2791</v>
       </c>
       <c r="C1520" t="n">
-        <v>11346</v>
+        <v>32669</v>
       </c>
     </row>
     <row r="1521">
@@ -17163,10 +17163,10 @@
         <v>46296</v>
       </c>
       <c r="B1521" t="n">
-        <v>626</v>
+        <v>2571</v>
       </c>
       <c r="C1521" t="n">
-        <v>471222</v>
+        <v>84819</v>
       </c>
     </row>
     <row r="1522">
@@ -17174,10 +17174,10 @@
         <v>46296</v>
       </c>
       <c r="B1522" t="n">
-        <v>2586</v>
+        <v>2273</v>
       </c>
       <c r="C1522" t="n">
-        <v>11346</v>
+        <v>68411</v>
       </c>
     </row>
     <row r="1523">
@@ -17185,10 +17185,10 @@
         <v>46296</v>
       </c>
       <c r="B1523" t="n">
-        <v>966</v>
+        <v>2381</v>
       </c>
       <c r="C1523" t="n">
-        <v>22224</v>
+        <v>25585</v>
       </c>
     </row>
     <row r="1524">
@@ -17196,10 +17196,10 @@
         <v>46296</v>
       </c>
       <c r="B1524" t="n">
-        <v>2798</v>
+        <v>630</v>
       </c>
       <c r="C1524" t="n">
-        <v>16362</v>
+        <v>26257</v>
       </c>
     </row>
     <row r="1525">
@@ -17207,10 +17207,10 @@
         <v>46296</v>
       </c>
       <c r="B1525" t="n">
-        <v>2797</v>
+        <v>1983</v>
       </c>
       <c r="C1525" t="n">
-        <v>16362</v>
+        <v>174440</v>
       </c>
     </row>
     <row r="1526">
@@ -17218,10 +17218,10 @@
         <v>46296</v>
       </c>
       <c r="B1526" t="n">
-        <v>2819</v>
+        <v>1993</v>
       </c>
       <c r="C1526" t="n">
-        <v>16362</v>
+        <v>118454</v>
       </c>
     </row>
     <row r="1527">
@@ -17229,10 +17229,10 @@
         <v>46296</v>
       </c>
       <c r="B1527" t="n">
-        <v>2266</v>
+        <v>89</v>
       </c>
       <c r="C1527" t="n">
-        <v>21816</v>
+        <v>111363</v>
       </c>
     </row>
     <row r="1528">
@@ -17240,10 +17240,10 @@
         <v>46296</v>
       </c>
       <c r="B1528" t="n">
-        <v>2795</v>
+        <v>1063</v>
       </c>
       <c r="C1528" t="n">
-        <v>16362</v>
+        <v>122500</v>
       </c>
     </row>
     <row r="1529">
@@ -17251,10 +17251,10 @@
         <v>46296</v>
       </c>
       <c r="B1529" t="n">
-        <v>2722</v>
+        <v>1116</v>
       </c>
       <c r="C1529" t="n">
-        <v>5454</v>
+        <v>79541</v>
       </c>
     </row>
     <row r="1530">
@@ -17262,10 +17262,10 @@
         <v>46296</v>
       </c>
       <c r="B1530" t="n">
-        <v>1853</v>
+        <v>941</v>
       </c>
       <c r="C1530" t="n">
-        <v>32724</v>
+        <v>95739</v>
       </c>
     </row>
     <row r="1531">
@@ -17273,10 +17273,10 @@
         <v>46296</v>
       </c>
       <c r="B1531" t="n">
-        <v>2842</v>
+        <v>2141</v>
       </c>
       <c r="C1531" t="n">
-        <v>49086</v>
+        <v>10206</v>
       </c>
     </row>
     <row r="1532">
@@ -17284,10 +17284,10 @@
         <v>46296</v>
       </c>
       <c r="B1532" t="n">
-        <v>2831</v>
+        <v>2463</v>
       </c>
       <c r="C1532" t="n">
-        <v>16362</v>
+        <v>104944</v>
       </c>
     </row>
     <row r="1533">
@@ -17295,10 +17295,10 @@
         <v>46296</v>
       </c>
       <c r="B1533" t="n">
-        <v>818</v>
+        <v>1890</v>
       </c>
       <c r="C1533" t="n">
-        <v>109086</v>
+        <v>78029</v>
       </c>
     </row>
     <row r="1534">
@@ -17306,10 +17306,10 @@
         <v>46296</v>
       </c>
       <c r="B1534" t="n">
-        <v>619</v>
+        <v>2639</v>
       </c>
       <c r="C1534" t="n">
-        <v>85500</v>
+        <v>12747</v>
       </c>
     </row>
     <row r="1535">
@@ -17317,10 +17317,10 @@
         <v>46296</v>
       </c>
       <c r="B1535" t="n">
-        <v>1478</v>
+        <v>1075</v>
       </c>
       <c r="C1535" t="n">
-        <v>149628</v>
+        <v>146041</v>
       </c>
     </row>
     <row r="1536">
@@ -17328,10 +17328,10 @@
         <v>46296</v>
       </c>
       <c r="B1536" t="n">
-        <v>2026</v>
+        <v>131</v>
       </c>
       <c r="C1536" t="n">
-        <v>66108</v>
+        <v>132363</v>
       </c>
     </row>
     <row r="1537">
@@ -17339,10 +17339,10 @@
         <v>46296</v>
       </c>
       <c r="B1537" t="n">
-        <v>285</v>
+        <v>2667</v>
       </c>
       <c r="C1537" t="n">
-        <v>149628</v>
+        <v>14539</v>
       </c>
     </row>
     <row r="1538">
@@ -17350,10 +17350,10 @@
         <v>46296</v>
       </c>
       <c r="B1538" t="n">
-        <v>424</v>
+        <v>2330</v>
       </c>
       <c r="C1538" t="n">
-        <v>64122</v>
+        <v>28301</v>
       </c>
     </row>
     <row r="1539">
@@ -17361,10 +17361,10 @@
         <v>46296</v>
       </c>
       <c r="B1539" t="n">
-        <v>451</v>
+        <v>2577</v>
       </c>
       <c r="C1539" t="n">
-        <v>66270</v>
+        <v>28371</v>
       </c>
     </row>
     <row r="1540">
@@ -17372,10 +17372,10 @@
         <v>46296</v>
       </c>
       <c r="B1540" t="n">
-        <v>629</v>
+        <v>2745</v>
       </c>
       <c r="C1540" t="n">
-        <v>123816</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="1541">
@@ -17383,10 +17383,10 @@
         <v>46296</v>
       </c>
       <c r="B1541" t="n">
-        <v>663</v>
+        <v>2817</v>
       </c>
       <c r="C1541" t="n">
-        <v>70632</v>
+        <v>19089</v>
       </c>
     </row>
     <row r="1542">
@@ -17394,10 +17394,10 @@
         <v>46296</v>
       </c>
       <c r="B1542" t="n">
-        <v>2657</v>
+        <v>2784</v>
       </c>
       <c r="C1542" t="n">
-        <v>21594</v>
+        <v>13237</v>
       </c>
     </row>
     <row r="1543">
@@ -17405,10 +17405,10 @@
         <v>46296</v>
       </c>
       <c r="B1543" t="n">
-        <v>1254</v>
+        <v>626</v>
       </c>
       <c r="C1543" t="n">
-        <v>52962</v>
+        <v>549759</v>
       </c>
     </row>
     <row r="1544">
@@ -17416,10 +17416,10 @@
         <v>46296</v>
       </c>
       <c r="B1544" t="n">
-        <v>2671</v>
+        <v>2586</v>
       </c>
       <c r="C1544" t="n">
-        <v>21816</v>
+        <v>13237</v>
       </c>
     </row>
     <row r="1545">
@@ -17427,10 +17427,10 @@
         <v>46296</v>
       </c>
       <c r="B1545" t="n">
-        <v>2753</v>
+        <v>966</v>
       </c>
       <c r="C1545" t="n">
-        <v>20454</v>
+        <v>25928</v>
       </c>
     </row>
     <row r="1546">
@@ -17438,10 +17438,10 @@
         <v>46296</v>
       </c>
       <c r="B1546" t="n">
-        <v>744</v>
+        <v>2798</v>
       </c>
       <c r="C1546" t="n">
-        <v>11346</v>
+        <v>19089</v>
       </c>
     </row>
     <row r="1547">
@@ -17449,10 +17449,10 @@
         <v>46296</v>
       </c>
       <c r="B1547" t="n">
-        <v>2323</v>
+        <v>2797</v>
       </c>
       <c r="C1547" t="n">
-        <v>18732</v>
+        <v>19089</v>
       </c>
     </row>
     <row r="1548">
@@ -17460,10 +17460,10 @@
         <v>46296</v>
       </c>
       <c r="B1548" t="n">
-        <v>2310</v>
+        <v>2819</v>
       </c>
       <c r="C1548" t="n">
-        <v>18732</v>
+        <v>19089</v>
       </c>
     </row>
     <row r="1549">
@@ -17471,10 +17471,10 @@
         <v>46296</v>
       </c>
       <c r="B1549" t="n">
-        <v>2501</v>
+        <v>2266</v>
       </c>
       <c r="C1549" t="n">
-        <v>22224</v>
+        <v>25452</v>
       </c>
     </row>
     <row r="1550">
@@ -17482,10 +17482,10 @@
         <v>46296</v>
       </c>
       <c r="B1550" t="n">
-        <v>716</v>
+        <v>2795</v>
       </c>
       <c r="C1550" t="n">
-        <v>34956</v>
+        <v>19089</v>
       </c>
     </row>
     <row r="1551">
@@ -17493,10 +17493,10 @@
         <v>46296</v>
       </c>
       <c r="B1551" t="n">
-        <v>2758</v>
+        <v>2722</v>
       </c>
       <c r="C1551" t="n">
-        <v>16362</v>
+        <v>6363</v>
       </c>
     </row>
     <row r="1552">
@@ -17504,10 +17504,10 @@
         <v>46296</v>
       </c>
       <c r="B1552" t="n">
-        <v>1259</v>
+        <v>1853</v>
       </c>
       <c r="C1552" t="n">
-        <v>30000</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1553">
@@ -17515,10 +17515,10 @@
         <v>46296</v>
       </c>
       <c r="B1553" t="n">
-        <v>2833</v>
+        <v>2842</v>
       </c>
       <c r="C1553" t="n">
-        <v>21816</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1554">
@@ -17526,10 +17526,10 @@
         <v>46296</v>
       </c>
       <c r="B1554" t="n">
-        <v>2687</v>
+        <v>2831</v>
       </c>
       <c r="C1554" t="n">
-        <v>21816</v>
+        <v>19089</v>
       </c>
     </row>
     <row r="1555">
@@ -17537,10 +17537,10 @@
         <v>46296</v>
       </c>
       <c r="B1555" t="n">
-        <v>2824</v>
+        <v>818</v>
       </c>
       <c r="C1555" t="n">
-        <v>30792</v>
+        <v>127267</v>
       </c>
     </row>
     <row r="1556">
@@ -17548,10 +17548,10 @@
         <v>46296</v>
       </c>
       <c r="B1556" t="n">
-        <v>2730</v>
+        <v>2696</v>
       </c>
       <c r="C1556" t="n">
-        <v>24540</v>
+        <v>68236</v>
       </c>
     </row>
     <row r="1557">
@@ -17559,10 +17559,10 @@
         <v>46296</v>
       </c>
       <c r="B1557" t="n">
-        <v>2718</v>
+        <v>2698</v>
       </c>
       <c r="C1557" t="n">
-        <v>35454</v>
+        <v>34972</v>
       </c>
     </row>
     <row r="1558">
@@ -17570,10 +17570,10 @@
         <v>46296</v>
       </c>
       <c r="B1558" t="n">
-        <v>2750</v>
+        <v>619</v>
       </c>
       <c r="C1558" t="n">
-        <v>8178</v>
+        <v>99750</v>
       </c>
     </row>
     <row r="1559">
@@ -17581,10 +17581,10 @@
         <v>46296</v>
       </c>
       <c r="B1559" t="n">
-        <v>854</v>
+        <v>1478</v>
       </c>
       <c r="C1559" t="n">
-        <v>38178</v>
+        <v>174566</v>
       </c>
     </row>
     <row r="1560">
@@ -17592,10 +17592,10 @@
         <v>46296</v>
       </c>
       <c r="B1560" t="n">
-        <v>2794</v>
+        <v>2026</v>
       </c>
       <c r="C1560" t="n">
-        <v>32724</v>
+        <v>77126</v>
       </c>
     </row>
     <row r="1561">
@@ -17603,10 +17603,10 @@
         <v>46296</v>
       </c>
       <c r="B1561" t="n">
-        <v>2488</v>
+        <v>285</v>
       </c>
       <c r="C1561" t="n">
-        <v>27270</v>
+        <v>174566</v>
       </c>
     </row>
     <row r="1562">
@@ -17614,10 +17614,10 @@
         <v>46296</v>
       </c>
       <c r="B1562" t="n">
-        <v>363</v>
+        <v>424</v>
       </c>
       <c r="C1562" t="n">
-        <v>81816</v>
+        <v>74809</v>
       </c>
     </row>
     <row r="1563">
@@ -17625,10 +17625,10 @@
         <v>46296</v>
       </c>
       <c r="B1563" t="n">
-        <v>2655</v>
+        <v>451</v>
       </c>
       <c r="C1563" t="n">
-        <v>30000</v>
+        <v>77315</v>
       </c>
     </row>
     <row r="1564">
@@ -17636,10 +17636,10 @@
         <v>46296</v>
       </c>
       <c r="B1564" t="n">
-        <v>1873</v>
+        <v>629</v>
       </c>
       <c r="C1564" t="n">
-        <v>87270</v>
+        <v>144452</v>
       </c>
     </row>
     <row r="1565">
@@ -17647,10 +17647,10 @@
         <v>46296</v>
       </c>
       <c r="B1565" t="n">
-        <v>2635</v>
+        <v>663</v>
       </c>
       <c r="C1565" t="n">
-        <v>35454</v>
+        <v>82404</v>
       </c>
     </row>
     <row r="1566">
@@ -17658,10 +17658,10 @@
         <v>46296</v>
       </c>
       <c r="B1566" t="n">
-        <v>636</v>
+        <v>2657</v>
       </c>
       <c r="C1566" t="n">
-        <v>68178</v>
+        <v>25193</v>
       </c>
     </row>
     <row r="1567">
@@ -17669,10 +17669,10 @@
         <v>46296</v>
       </c>
       <c r="B1567" t="n">
-        <v>2803</v>
+        <v>1254</v>
       </c>
       <c r="C1567" t="n">
-        <v>32724</v>
+        <v>61789</v>
       </c>
     </row>
     <row r="1568">
@@ -17680,10 +17680,10 @@
         <v>46296</v>
       </c>
       <c r="B1568" t="n">
-        <v>2163</v>
+        <v>2671</v>
       </c>
       <c r="C1568" t="n">
-        <v>49086</v>
+        <v>25452</v>
       </c>
     </row>
     <row r="1569">
@@ -17691,10 +17691,10 @@
         <v>46296</v>
       </c>
       <c r="B1569" t="n">
-        <v>1466</v>
+        <v>2753</v>
       </c>
       <c r="C1569" t="n">
-        <v>110454</v>
+        <v>23863</v>
       </c>
     </row>
     <row r="1570">
@@ -17702,10 +17702,10 @@
         <v>46296</v>
       </c>
       <c r="B1570" t="n">
-        <v>535</v>
+        <v>744</v>
       </c>
       <c r="C1570" t="n">
-        <v>97140</v>
+        <v>13237</v>
       </c>
     </row>
     <row r="1571">
@@ -17713,10 +17713,10 @@
         <v>46296</v>
       </c>
       <c r="B1571" t="n">
-        <v>2790</v>
+        <v>2323</v>
       </c>
       <c r="C1571" t="n">
-        <v>17226</v>
+        <v>21854</v>
       </c>
     </row>
     <row r="1572">
@@ -17724,10 +17724,10 @@
         <v>46296</v>
       </c>
       <c r="B1572" t="n">
-        <v>1317</v>
+        <v>2310</v>
       </c>
       <c r="C1572" t="n">
-        <v>85908</v>
+        <v>21854</v>
       </c>
     </row>
     <row r="1573">
@@ -17735,10 +17735,10 @@
         <v>46296</v>
       </c>
       <c r="B1573" t="n">
-        <v>2822</v>
+        <v>2501</v>
       </c>
       <c r="C1573" t="n">
-        <v>43632</v>
+        <v>25928</v>
       </c>
     </row>
     <row r="1574">
@@ -17746,10 +17746,10 @@
         <v>46296</v>
       </c>
       <c r="B1574" t="n">
-        <v>1117</v>
+        <v>716</v>
       </c>
       <c r="C1574" t="n">
-        <v>109122</v>
+        <v>40782</v>
       </c>
     </row>
     <row r="1575">
@@ -17757,10 +17757,10 @@
         <v>46296</v>
       </c>
       <c r="B1575" t="n">
-        <v>1299</v>
+        <v>2758</v>
       </c>
       <c r="C1575" t="n">
-        <v>143874</v>
+        <v>19089</v>
       </c>
     </row>
     <row r="1576">
@@ -17768,10 +17768,10 @@
         <v>46296</v>
       </c>
       <c r="B1576" t="n">
-        <v>477</v>
+        <v>1259</v>
       </c>
       <c r="C1576" t="n">
-        <v>59292</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="1577">
@@ -17779,10 +17779,241 @@
         <v>46296</v>
       </c>
       <c r="B1577" t="n">
-        <v>530</v>
+        <v>2833</v>
       </c>
       <c r="C1577" t="n">
-        <v>81816</v>
+        <v>25452</v>
+      </c>
+    </row>
+    <row r="1578">
+      <c r="A1578" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1578" t="n">
+        <v>2687</v>
+      </c>
+      <c r="C1578" t="n">
+        <v>25452</v>
+      </c>
+    </row>
+    <row r="1579">
+      <c r="A1579" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1579" t="n">
+        <v>2824</v>
+      </c>
+      <c r="C1579" t="n">
+        <v>35924</v>
+      </c>
+    </row>
+    <row r="1580">
+      <c r="A1580" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1580" t="n">
+        <v>2730</v>
+      </c>
+      <c r="C1580" t="n">
+        <v>28630</v>
+      </c>
+    </row>
+    <row r="1581">
+      <c r="A1581" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1581" t="n">
+        <v>2718</v>
+      </c>
+      <c r="C1581" t="n">
+        <v>41363</v>
+      </c>
+    </row>
+    <row r="1582">
+      <c r="A1582" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1582" t="n">
+        <v>2750</v>
+      </c>
+      <c r="C1582" t="n">
+        <v>9541</v>
+      </c>
+    </row>
+    <row r="1583">
+      <c r="A1583" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1583" t="n">
+        <v>854</v>
+      </c>
+      <c r="C1583" t="n">
+        <v>44541</v>
+      </c>
+    </row>
+    <row r="1584">
+      <c r="A1584" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1584" t="n">
+        <v>2794</v>
+      </c>
+      <c r="C1584" t="n">
+        <v>38178</v>
+      </c>
+    </row>
+    <row r="1585">
+      <c r="A1585" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1585" t="n">
+        <v>2488</v>
+      </c>
+      <c r="C1585" t="n">
+        <v>31815</v>
+      </c>
+    </row>
+    <row r="1586">
+      <c r="A1586" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1586" t="n">
+        <v>363</v>
+      </c>
+      <c r="C1586" t="n">
+        <v>95452</v>
+      </c>
+    </row>
+    <row r="1587">
+      <c r="A1587" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1587" t="n">
+        <v>2655</v>
+      </c>
+      <c r="C1587" t="n">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="1588">
+      <c r="A1588" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1588" t="n">
+        <v>1873</v>
+      </c>
+      <c r="C1588" t="n">
+        <v>101815</v>
+      </c>
+    </row>
+    <row r="1589">
+      <c r="A1589" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1589" t="n">
+        <v>2635</v>
+      </c>
+      <c r="C1589" t="n">
+        <v>41363</v>
+      </c>
+    </row>
+    <row r="1590">
+      <c r="A1590" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1590" t="n">
+        <v>636</v>
+      </c>
+      <c r="C1590" t="n">
+        <v>79541</v>
+      </c>
+    </row>
+    <row r="1591">
+      <c r="A1591" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1591" t="n">
+        <v>2803</v>
+      </c>
+      <c r="C1591" t="n">
+        <v>38178</v>
+      </c>
+    </row>
+    <row r="1592">
+      <c r="A1592" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1592" t="n">
+        <v>2163</v>
+      </c>
+      <c r="C1592" t="n">
+        <v>57267</v>
+      </c>
+    </row>
+    <row r="1593">
+      <c r="A1593" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1593" t="n">
+        <v>1466</v>
+      </c>
+      <c r="C1593" t="n">
+        <v>128863</v>
+      </c>
+    </row>
+    <row r="1594">
+      <c r="A1594" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1594" t="n">
+        <v>535</v>
+      </c>
+      <c r="C1594" t="n">
+        <v>113330</v>
+      </c>
+    </row>
+    <row r="1595">
+      <c r="A1595" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1595" t="n">
+        <v>2790</v>
+      </c>
+      <c r="C1595" t="n">
+        <v>20097</v>
+      </c>
+    </row>
+    <row r="1596">
+      <c r="A1596" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1596" t="n">
+        <v>2768</v>
+      </c>
+      <c r="C1596" t="n">
+        <v>96299</v>
+      </c>
+    </row>
+    <row r="1597">
+      <c r="A1597" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1597" t="n">
+        <v>2491</v>
+      </c>
+      <c r="C1597" t="n">
+        <v>77273</v>
+      </c>
+    </row>
+    <row r="1598">
+      <c r="A1598" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1598" t="n">
+        <v>2799</v>
+      </c>
+      <c r="C1598" t="n">
+        <v>34783</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:02:02
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1598"/>
+  <dimension ref="A1:C1726"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15557,10 +15557,10 @@
         <v>46296</v>
       </c>
       <c r="B1375" t="n">
-        <v>675</v>
+        <v>2245</v>
       </c>
       <c r="C1375" t="n">
-        <v>63630</v>
+        <v>80512</v>
       </c>
     </row>
     <row r="1376">
@@ -15568,10 +15568,10 @@
         <v>46296</v>
       </c>
       <c r="B1376" t="n">
-        <v>2804</v>
+        <v>2251</v>
       </c>
       <c r="C1376" t="n">
-        <v>31815</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1377">
@@ -15579,10 +15579,10 @@
         <v>46296</v>
       </c>
       <c r="B1377" t="n">
-        <v>2714</v>
+        <v>2142</v>
       </c>
       <c r="C1377" t="n">
-        <v>114541</v>
+        <v>19680</v>
       </c>
     </row>
     <row r="1378">
@@ -15590,10 +15590,10 @@
         <v>46296</v>
       </c>
       <c r="B1378" t="n">
-        <v>2765</v>
+        <v>664</v>
       </c>
       <c r="C1378" t="n">
-        <v>28630</v>
+        <v>95272</v>
       </c>
     </row>
     <row r="1379">
@@ -15601,10 +15601,10 @@
         <v>46296</v>
       </c>
       <c r="B1379" t="n">
-        <v>2359</v>
+        <v>2472</v>
       </c>
       <c r="C1379" t="n">
-        <v>33194</v>
+        <v>19248</v>
       </c>
     </row>
     <row r="1380">
@@ -15612,10 +15612,10 @@
         <v>46296</v>
       </c>
       <c r="B1380" t="n">
-        <v>2678</v>
+        <v>1456</v>
       </c>
       <c r="C1380" t="n">
-        <v>31486</v>
+        <v>290176</v>
       </c>
     </row>
     <row r="1381">
@@ -15623,10 +15623,10 @@
         <v>46296</v>
       </c>
       <c r="B1381" t="n">
-        <v>2697</v>
+        <v>1585</v>
       </c>
       <c r="C1381" t="n">
-        <v>47782</v>
+        <v>65816</v>
       </c>
     </row>
     <row r="1382">
@@ -15634,10 +15634,10 @@
         <v>46296</v>
       </c>
       <c r="B1382" t="n">
-        <v>2498</v>
+        <v>1907</v>
       </c>
       <c r="C1382" t="n">
-        <v>17913</v>
+        <v>200192</v>
       </c>
     </row>
     <row r="1383">
@@ -15645,10 +15645,10 @@
         <v>46296</v>
       </c>
       <c r="B1383" t="n">
-        <v>2641</v>
+        <v>2659</v>
       </c>
       <c r="C1383" t="n">
-        <v>47726</v>
+        <v>44728</v>
       </c>
     </row>
     <row r="1384">
@@ -15656,10 +15656,10 @@
         <v>46296</v>
       </c>
       <c r="B1384" t="n">
-        <v>2801</v>
+        <v>2583</v>
       </c>
       <c r="C1384" t="n">
-        <v>31815</v>
+        <v>15128</v>
       </c>
     </row>
     <row r="1385">
@@ -15667,10 +15667,10 @@
         <v>46296</v>
       </c>
       <c r="B1385" t="n">
-        <v>2810</v>
+        <v>2692</v>
       </c>
       <c r="C1385" t="n">
-        <v>50904</v>
+        <v>25454.66</v>
       </c>
     </row>
     <row r="1386">
@@ -15678,10 +15678,10 @@
         <v>46296</v>
       </c>
       <c r="B1386" t="n">
-        <v>2245</v>
+        <v>2691</v>
       </c>
       <c r="C1386" t="n">
-        <v>70448</v>
+        <v>44430.66</v>
       </c>
     </row>
     <row r="1387">
@@ -15689,10 +15689,10 @@
         <v>46296</v>
       </c>
       <c r="B1387" t="n">
-        <v>2251</v>
+        <v>931</v>
       </c>
       <c r="C1387" t="n">
-        <v>63630</v>
+        <v>34808</v>
       </c>
     </row>
     <row r="1388">
@@ -15700,10 +15700,10 @@
         <v>46296</v>
       </c>
       <c r="B1388" t="n">
-        <v>2142</v>
+        <v>2785</v>
       </c>
       <c r="C1388" t="n">
-        <v>17220</v>
+        <v>15128</v>
       </c>
     </row>
     <row r="1389">
@@ -15711,10 +15711,10 @@
         <v>46296</v>
       </c>
       <c r="B1389" t="n">
-        <v>664</v>
+        <v>2411</v>
       </c>
       <c r="C1389" t="n">
-        <v>83363</v>
+        <v>36360</v>
       </c>
     </row>
     <row r="1390">
@@ -15722,10 +15722,10 @@
         <v>46296</v>
       </c>
       <c r="B1390" t="n">
-        <v>2472</v>
+        <v>2716</v>
       </c>
       <c r="C1390" t="n">
-        <v>16842</v>
+        <v>31904</v>
       </c>
     </row>
     <row r="1391">
@@ -15733,10 +15733,10 @@
         <v>46296</v>
       </c>
       <c r="B1391" t="n">
-        <v>2659</v>
+        <v>2809</v>
       </c>
       <c r="C1391" t="n">
-        <v>39137</v>
+        <v>24976</v>
       </c>
     </row>
     <row r="1392">
@@ -15744,10 +15744,10 @@
         <v>46296</v>
       </c>
       <c r="B1392" t="n">
-        <v>2583</v>
+        <v>104</v>
       </c>
       <c r="C1392" t="n">
-        <v>13237</v>
+        <v>109088</v>
       </c>
     </row>
     <row r="1393">
@@ -15755,10 +15755,10 @@
         <v>46296</v>
       </c>
       <c r="B1393" t="n">
-        <v>2692</v>
+        <v>781</v>
       </c>
       <c r="C1393" t="n">
-        <v>19782</v>
+        <v>47272</v>
       </c>
     </row>
     <row r="1394">
@@ -15766,10 +15766,10 @@
         <v>46296</v>
       </c>
       <c r="B1394" t="n">
-        <v>2691</v>
+        <v>2494</v>
       </c>
       <c r="C1394" t="n">
-        <v>31815</v>
+        <v>54544</v>
       </c>
     </row>
     <row r="1395">
@@ -15777,10 +15777,10 @@
         <v>46296</v>
       </c>
       <c r="B1395" t="n">
-        <v>2785</v>
+        <v>2652</v>
       </c>
       <c r="C1395" t="n">
-        <v>13237</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1396">
@@ -15788,10 +15788,10 @@
         <v>46296</v>
       </c>
       <c r="B1396" t="n">
-        <v>2809</v>
+        <v>1384</v>
       </c>
       <c r="C1396" t="n">
-        <v>21854</v>
+        <v>127272</v>
       </c>
     </row>
     <row r="1397">
@@ -15799,10 +15799,10 @@
         <v>46296</v>
       </c>
       <c r="B1397" t="n">
-        <v>2494</v>
+        <v>360</v>
       </c>
       <c r="C1397" t="n">
-        <v>47726</v>
+        <v>181816</v>
       </c>
     </row>
     <row r="1398">
@@ -15810,10 +15810,10 @@
         <v>46296</v>
       </c>
       <c r="B1398" t="n">
-        <v>2652</v>
+        <v>2767</v>
       </c>
       <c r="C1398" t="n">
-        <v>44541</v>
+        <v>69088</v>
       </c>
     </row>
     <row r="1399">
@@ -15821,10 +15821,10 @@
         <v>46296</v>
       </c>
       <c r="B1399" t="n">
-        <v>360</v>
+        <v>2178</v>
       </c>
       <c r="C1399" t="n">
-        <v>159089</v>
+        <v>99632</v>
       </c>
     </row>
     <row r="1400">
@@ -15832,10 +15832,10 @@
         <v>46296</v>
       </c>
       <c r="B1400" t="n">
-        <v>2767</v>
+        <v>2107</v>
       </c>
       <c r="C1400" t="n">
-        <v>60452</v>
+        <v>109080</v>
       </c>
     </row>
     <row r="1401">
@@ -15843,10 +15843,10 @@
         <v>46296</v>
       </c>
       <c r="B1401" t="n">
-        <v>2107</v>
+        <v>2711</v>
       </c>
       <c r="C1401" t="n">
-        <v>95445</v>
+        <v>31480</v>
       </c>
     </row>
     <row r="1402">
@@ -15854,10 +15854,10 @@
         <v>46296</v>
       </c>
       <c r="B1402" t="n">
-        <v>2711</v>
+        <v>2845</v>
       </c>
       <c r="C1402" t="n">
-        <v>27545</v>
+        <v>18176</v>
       </c>
     </row>
     <row r="1403">
@@ -15868,7 +15868,7 @@
         <v>1102</v>
       </c>
       <c r="C1403" t="n">
-        <v>74809</v>
+        <v>85496</v>
       </c>
     </row>
     <row r="1404">
@@ -15879,7 +15879,7 @@
         <v>353</v>
       </c>
       <c r="C1404" t="n">
-        <v>93079</v>
+        <v>106376</v>
       </c>
     </row>
     <row r="1405">
@@ -15890,7 +15890,7 @@
         <v>2250</v>
       </c>
       <c r="C1405" t="n">
-        <v>108178</v>
+        <v>123632</v>
       </c>
     </row>
     <row r="1406">
@@ -15901,7 +15901,7 @@
         <v>1800</v>
       </c>
       <c r="C1406" t="n">
-        <v>9023</v>
+        <v>10312</v>
       </c>
     </row>
     <row r="1407">
@@ -15909,10 +15909,10 @@
         <v>46296</v>
       </c>
       <c r="B1407" t="n">
-        <v>2682</v>
+        <v>2555</v>
       </c>
       <c r="C1407" t="n">
-        <v>44541</v>
+        <v>14216</v>
       </c>
     </row>
     <row r="1408">
@@ -15920,10 +15920,10 @@
         <v>46296</v>
       </c>
       <c r="B1408" t="n">
-        <v>2786</v>
+        <v>2558</v>
       </c>
       <c r="C1408" t="n">
-        <v>22267</v>
+        <v>14216</v>
       </c>
     </row>
     <row r="1409">
@@ -15931,10 +15931,10 @@
         <v>46296</v>
       </c>
       <c r="B1409" t="n">
-        <v>2816</v>
+        <v>2721</v>
       </c>
       <c r="C1409" t="n">
-        <v>41363</v>
+        <v>29632</v>
       </c>
     </row>
     <row r="1410">
@@ -15942,10 +15942,10 @@
         <v>46296</v>
       </c>
       <c r="B1410" t="n">
-        <v>2090</v>
+        <v>2556</v>
       </c>
       <c r="C1410" t="n">
-        <v>13237</v>
+        <v>14216</v>
       </c>
     </row>
     <row r="1411">
@@ -15953,10 +15953,10 @@
         <v>46296</v>
       </c>
       <c r="B1411" t="n">
-        <v>766</v>
+        <v>2826</v>
       </c>
       <c r="C1411" t="n">
-        <v>21854</v>
+        <v>25448</v>
       </c>
     </row>
     <row r="1412">
@@ -15964,10 +15964,10 @@
         <v>46296</v>
       </c>
       <c r="B1412" t="n">
-        <v>2702</v>
+        <v>2346</v>
       </c>
       <c r="C1412" t="n">
-        <v>25928</v>
+        <v>25448</v>
       </c>
     </row>
     <row r="1413">
@@ -15975,10 +15975,10 @@
         <v>46296</v>
       </c>
       <c r="B1413" t="n">
-        <v>2772</v>
+        <v>595</v>
       </c>
       <c r="C1413" t="n">
-        <v>19089</v>
+        <v>90904</v>
       </c>
     </row>
     <row r="1414">
@@ -15986,10 +15986,10 @@
         <v>46296</v>
       </c>
       <c r="B1414" t="n">
-        <v>767</v>
+        <v>1278</v>
       </c>
       <c r="C1414" t="n">
-        <v>63630</v>
+        <v>63632</v>
       </c>
     </row>
     <row r="1415">
@@ -15997,10 +15997,10 @@
         <v>46296</v>
       </c>
       <c r="B1415" t="n">
-        <v>2727</v>
+        <v>2686</v>
       </c>
       <c r="C1415" t="n">
-        <v>12880</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1416">
@@ -16008,10 +16008,10 @@
         <v>46296</v>
       </c>
       <c r="B1416" t="n">
-        <v>2846</v>
+        <v>1344</v>
       </c>
       <c r="C1416" t="n">
-        <v>82726</v>
+        <v>54544</v>
       </c>
     </row>
     <row r="1417">
@@ -16019,10 +16019,10 @@
         <v>46296</v>
       </c>
       <c r="B1417" t="n">
-        <v>609</v>
+        <v>2566</v>
       </c>
       <c r="C1417" t="n">
-        <v>71589</v>
+        <v>29088</v>
       </c>
     </row>
     <row r="1418">
@@ -16030,10 +16030,10 @@
         <v>46296</v>
       </c>
       <c r="B1418" t="n">
-        <v>2726</v>
+        <v>2684</v>
       </c>
       <c r="C1418" t="n">
-        <v>49315</v>
+        <v>34544</v>
       </c>
     </row>
     <row r="1419">
@@ -16041,10 +16041,10 @@
         <v>46296</v>
       </c>
       <c r="B1419" t="n">
-        <v>2729</v>
+        <v>2375</v>
       </c>
       <c r="C1419" t="n">
-        <v>28630</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="1420">
@@ -16052,10 +16052,10 @@
         <v>46296</v>
       </c>
       <c r="B1420" t="n">
-        <v>2830</v>
+        <v>2362</v>
       </c>
       <c r="C1420" t="n">
-        <v>28630</v>
+        <v>27272</v>
       </c>
     </row>
     <row r="1421">
@@ -16063,10 +16063,10 @@
         <v>46296</v>
       </c>
       <c r="B1421" t="n">
-        <v>2674</v>
+        <v>2449</v>
       </c>
       <c r="C1421" t="n">
-        <v>82726</v>
+        <v>34544</v>
       </c>
     </row>
     <row r="1422">
@@ -16074,10 +16074,10 @@
         <v>46296</v>
       </c>
       <c r="B1422" t="n">
-        <v>2308</v>
+        <v>2844</v>
       </c>
       <c r="C1422" t="n">
-        <v>63630</v>
+        <v>18176</v>
       </c>
     </row>
     <row r="1423">
@@ -16085,10 +16085,10 @@
         <v>46296</v>
       </c>
       <c r="B1423" t="n">
-        <v>2601</v>
+        <v>2507</v>
       </c>
       <c r="C1423" t="n">
-        <v>87500</v>
+        <v>32480</v>
       </c>
     </row>
     <row r="1424">
@@ -16096,10 +16096,10 @@
         <v>46296</v>
       </c>
       <c r="B1424" t="n">
-        <v>2015</v>
+        <v>1906</v>
       </c>
       <c r="C1424" t="n">
-        <v>117726</v>
+        <v>39480</v>
       </c>
     </row>
     <row r="1425">
@@ -16107,10 +16107,10 @@
         <v>46296</v>
       </c>
       <c r="B1425" t="n">
-        <v>1308</v>
+        <v>525</v>
       </c>
       <c r="C1425" t="n">
-        <v>49952</v>
+        <v>85448</v>
       </c>
     </row>
     <row r="1426">
@@ -16118,10 +16118,10 @@
         <v>46296</v>
       </c>
       <c r="B1426" t="n">
-        <v>2118</v>
+        <v>1261</v>
       </c>
       <c r="C1426" t="n">
-        <v>66871</v>
+        <v>25818.22</v>
       </c>
     </row>
     <row r="1427">
@@ -16129,10 +16129,10 @@
         <v>46296</v>
       </c>
       <c r="B1427" t="n">
-        <v>2607</v>
+        <v>2755</v>
       </c>
       <c r="C1427" t="n">
-        <v>15806</v>
+        <v>18181.92</v>
       </c>
     </row>
     <row r="1428">
@@ -16140,10 +16140,10 @@
         <v>46296</v>
       </c>
       <c r="B1428" t="n">
-        <v>2707</v>
+        <v>1064</v>
       </c>
       <c r="C1428" t="n">
-        <v>13741</v>
+        <v>218176</v>
       </c>
     </row>
     <row r="1429">
@@ -16151,10 +16151,10 @@
         <v>46296</v>
       </c>
       <c r="B1429" t="n">
-        <v>2383</v>
+        <v>1810</v>
       </c>
       <c r="C1429" t="n">
-        <v>42294</v>
+        <v>14768</v>
       </c>
     </row>
     <row r="1430">
@@ -16162,10 +16162,10 @@
         <v>46296</v>
       </c>
       <c r="B1430" t="n">
-        <v>2821</v>
+        <v>1937</v>
       </c>
       <c r="C1430" t="n">
-        <v>42427</v>
+        <v>94176</v>
       </c>
     </row>
     <row r="1431">
@@ -16173,10 +16173,10 @@
         <v>46296</v>
       </c>
       <c r="B1431" t="n">
-        <v>569</v>
+        <v>483</v>
       </c>
       <c r="C1431" t="n">
-        <v>923818</v>
+        <v>164360</v>
       </c>
     </row>
     <row r="1432">
@@ -16184,10 +16184,10 @@
         <v>46296</v>
       </c>
       <c r="B1432" t="n">
-        <v>2660</v>
+        <v>2580</v>
       </c>
       <c r="C1432" t="n">
-        <v>111363</v>
+        <v>12248</v>
       </c>
     </row>
     <row r="1433">
@@ -16195,10 +16195,10 @@
         <v>46296</v>
       </c>
       <c r="B1433" t="n">
-        <v>1632</v>
+        <v>2706</v>
       </c>
       <c r="C1433" t="n">
-        <v>82726</v>
+        <v>9568</v>
       </c>
     </row>
     <row r="1434">
@@ -16206,10 +16206,10 @@
         <v>46296</v>
       </c>
       <c r="B1434" t="n">
-        <v>1756</v>
+        <v>2633</v>
       </c>
       <c r="C1434" t="n">
-        <v>133630</v>
+        <v>7008</v>
       </c>
     </row>
     <row r="1435">
@@ -16217,10 +16217,10 @@
         <v>46296</v>
       </c>
       <c r="B1435" t="n">
-        <v>58</v>
+        <v>2392</v>
       </c>
       <c r="C1435" t="n">
-        <v>79800</v>
+        <v>75424</v>
       </c>
     </row>
     <row r="1436">
@@ -16228,10 +16228,10 @@
         <v>46296</v>
       </c>
       <c r="B1436" t="n">
-        <v>40</v>
+        <v>2613</v>
       </c>
       <c r="C1436" t="n">
-        <v>70980</v>
+        <v>53104</v>
       </c>
     </row>
     <row r="1437">
@@ -16239,10 +16239,10 @@
         <v>46296</v>
       </c>
       <c r="B1437" t="n">
-        <v>559</v>
+        <v>2183</v>
       </c>
       <c r="C1437" t="n">
-        <v>74452</v>
+        <v>191208</v>
       </c>
     </row>
     <row r="1438">
@@ -16250,10 +16250,10 @@
         <v>46296</v>
       </c>
       <c r="B1438" t="n">
-        <v>2773</v>
+        <v>2541</v>
       </c>
       <c r="C1438" t="n">
-        <v>25669</v>
+        <v>85960</v>
       </c>
     </row>
     <row r="1439">
@@ -16261,10 +16261,10 @@
         <v>46296</v>
       </c>
       <c r="B1439" t="n">
-        <v>2631</v>
+        <v>2333</v>
       </c>
       <c r="C1439" t="n">
-        <v>12327</v>
+        <v>58032</v>
       </c>
     </row>
     <row r="1440">
@@ -16272,10 +16272,10 @@
         <v>46296</v>
       </c>
       <c r="B1440" t="n">
-        <v>1642</v>
+        <v>2813</v>
       </c>
       <c r="C1440" t="n">
-        <v>84315</v>
+        <v>23200</v>
       </c>
     </row>
     <row r="1441">
@@ -16283,10 +16283,10 @@
         <v>46296</v>
       </c>
       <c r="B1441" t="n">
-        <v>2621</v>
+        <v>2811</v>
       </c>
       <c r="C1441" t="n">
-        <v>22267</v>
+        <v>15128</v>
       </c>
     </row>
     <row r="1442">
@@ -16294,10 +16294,10 @@
         <v>46296</v>
       </c>
       <c r="B1442" t="n">
-        <v>2735</v>
+        <v>1881</v>
       </c>
       <c r="C1442" t="n">
-        <v>38178</v>
+        <v>24976</v>
       </c>
     </row>
     <row r="1443">
@@ -16305,10 +16305,10 @@
         <v>46296</v>
       </c>
       <c r="B1443" t="n">
-        <v>945</v>
+        <v>2825</v>
       </c>
       <c r="C1443" t="n">
-        <v>111580</v>
+        <v>20304</v>
       </c>
     </row>
     <row r="1444">
@@ -16316,10 +16316,10 @@
         <v>46296</v>
       </c>
       <c r="B1444" t="n">
-        <v>2629</v>
+        <v>970</v>
       </c>
       <c r="C1444" t="n">
-        <v>21854</v>
+        <v>24976</v>
       </c>
     </row>
     <row r="1445">
@@ -16327,10 +16327,10 @@
         <v>46296</v>
       </c>
       <c r="B1445" t="n">
-        <v>933</v>
+        <v>2552</v>
       </c>
       <c r="C1445" t="n">
-        <v>25928</v>
+        <v>14216</v>
       </c>
     </row>
     <row r="1446">
@@ -16338,10 +16338,10 @@
         <v>46296</v>
       </c>
       <c r="B1446" t="n">
-        <v>2721</v>
+        <v>2562</v>
       </c>
       <c r="C1446" t="n">
-        <v>25928</v>
+        <v>14216</v>
       </c>
     </row>
     <row r="1447">
@@ -16349,10 +16349,10 @@
         <v>46296</v>
       </c>
       <c r="B1447" t="n">
-        <v>2826</v>
+        <v>2761</v>
       </c>
       <c r="C1447" t="n">
-        <v>22267</v>
+        <v>29632</v>
       </c>
     </row>
     <row r="1448">
@@ -16360,10 +16360,10 @@
         <v>46296</v>
       </c>
       <c r="B1448" t="n">
-        <v>2346</v>
+        <v>2747</v>
       </c>
       <c r="C1448" t="n">
-        <v>22267</v>
+        <v>25448</v>
       </c>
     </row>
     <row r="1449">
@@ -16371,10 +16371,10 @@
         <v>46296</v>
       </c>
       <c r="B1449" t="n">
-        <v>2686</v>
+        <v>415</v>
       </c>
       <c r="C1449" t="n">
-        <v>44541</v>
+        <v>90904</v>
       </c>
     </row>
     <row r="1450">
@@ -16382,10 +16382,10 @@
         <v>46296</v>
       </c>
       <c r="B1450" t="n">
-        <v>2566</v>
+        <v>2544</v>
       </c>
       <c r="C1450" t="n">
-        <v>25452</v>
+        <v>25448</v>
       </c>
     </row>
     <row r="1451">
@@ -16393,10 +16393,10 @@
         <v>46296</v>
       </c>
       <c r="B1451" t="n">
-        <v>2684</v>
+        <v>816</v>
       </c>
       <c r="C1451" t="n">
-        <v>30226</v>
+        <v>109088</v>
       </c>
     </row>
     <row r="1452">
@@ -16404,10 +16404,10 @@
         <v>46296</v>
       </c>
       <c r="B1452" t="n">
-        <v>2375</v>
+        <v>890</v>
       </c>
       <c r="C1452" t="n">
-        <v>105000</v>
+        <v>327272</v>
       </c>
     </row>
     <row r="1453">
@@ -16415,10 +16415,10 @@
         <v>46296</v>
       </c>
       <c r="B1453" t="n">
-        <v>2507</v>
+        <v>1298</v>
       </c>
       <c r="C1453" t="n">
-        <v>28420</v>
+        <v>460000</v>
       </c>
     </row>
     <row r="1454">
@@ -16426,10 +16426,10 @@
         <v>46296</v>
       </c>
       <c r="B1454" t="n">
-        <v>1906</v>
+        <v>1372</v>
       </c>
       <c r="C1454" t="n">
-        <v>34545</v>
+        <v>109088</v>
       </c>
     </row>
     <row r="1455">
@@ -16437,10 +16437,10 @@
         <v>46296</v>
       </c>
       <c r="B1455" t="n">
-        <v>525</v>
+        <v>358</v>
       </c>
       <c r="C1455" t="n">
-        <v>74767</v>
+        <v>114544</v>
       </c>
     </row>
     <row r="1456">
@@ -16448,10 +16448,10 @@
         <v>46296</v>
       </c>
       <c r="B1456" t="n">
-        <v>1064</v>
+        <v>1653</v>
       </c>
       <c r="C1456" t="n">
-        <v>190904</v>
+        <v>114544</v>
       </c>
     </row>
     <row r="1457">
@@ -16459,10 +16459,10 @@
         <v>46296</v>
       </c>
       <c r="B1457" t="n">
-        <v>1810</v>
+        <v>675</v>
       </c>
       <c r="C1457" t="n">
-        <v>12922</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1458">
@@ -16470,10 +16470,10 @@
         <v>46296</v>
       </c>
       <c r="B1458" t="n">
-        <v>1937</v>
+        <v>2804</v>
       </c>
       <c r="C1458" t="n">
-        <v>82404</v>
+        <v>36360</v>
       </c>
     </row>
     <row r="1459">
@@ -16481,10 +16481,10 @@
         <v>46296</v>
       </c>
       <c r="B1459" t="n">
-        <v>483</v>
+        <v>2714</v>
       </c>
       <c r="C1459" t="n">
-        <v>143815</v>
+        <v>130904</v>
       </c>
     </row>
     <row r="1460">
@@ -16492,10 +16492,10 @@
         <v>46296</v>
       </c>
       <c r="B1460" t="n">
-        <v>2580</v>
+        <v>2765</v>
       </c>
       <c r="C1460" t="n">
-        <v>10717</v>
+        <v>32720</v>
       </c>
     </row>
     <row r="1461">
@@ -16503,10 +16503,10 @@
         <v>46296</v>
       </c>
       <c r="B1461" t="n">
-        <v>2706</v>
+        <v>2421</v>
       </c>
       <c r="C1461" t="n">
-        <v>8372</v>
+        <v>22176</v>
       </c>
     </row>
     <row r="1462">
@@ -16514,10 +16514,10 @@
         <v>46296</v>
       </c>
       <c r="B1462" t="n">
-        <v>2633</v>
+        <v>2359</v>
       </c>
       <c r="C1462" t="n">
-        <v>6132</v>
+        <v>37936</v>
       </c>
     </row>
     <row r="1463">
@@ -16525,10 +16525,10 @@
         <v>46296</v>
       </c>
       <c r="B1463" t="n">
-        <v>2811</v>
+        <v>2678</v>
       </c>
       <c r="C1463" t="n">
-        <v>13237</v>
+        <v>35984</v>
       </c>
     </row>
     <row r="1464">
@@ -16536,10 +16536,10 @@
         <v>46296</v>
       </c>
       <c r="B1464" t="n">
-        <v>1881</v>
+        <v>2697</v>
       </c>
       <c r="C1464" t="n">
-        <v>21854</v>
+        <v>54608</v>
       </c>
     </row>
     <row r="1465">
@@ -16547,10 +16547,10 @@
         <v>46296</v>
       </c>
       <c r="B1465" t="n">
-        <v>970</v>
+        <v>2498</v>
       </c>
       <c r="C1465" t="n">
-        <v>21854</v>
+        <v>20472</v>
       </c>
     </row>
     <row r="1466">
@@ -16558,10 +16558,10 @@
         <v>46296</v>
       </c>
       <c r="B1466" t="n">
-        <v>2761</v>
+        <v>2641</v>
       </c>
       <c r="C1466" t="n">
-        <v>25928</v>
+        <v>54544</v>
       </c>
     </row>
     <row r="1467">
@@ -16569,10 +16569,10 @@
         <v>46296</v>
       </c>
       <c r="B1467" t="n">
-        <v>2747</v>
+        <v>2801</v>
       </c>
       <c r="C1467" t="n">
-        <v>22267</v>
+        <v>36360</v>
       </c>
     </row>
     <row r="1468">
@@ -16580,10 +16580,10 @@
         <v>46296</v>
       </c>
       <c r="B1468" t="n">
-        <v>2544</v>
+        <v>2810</v>
       </c>
       <c r="C1468" t="n">
-        <v>22267</v>
+        <v>58176</v>
       </c>
     </row>
     <row r="1469">
@@ -16591,10 +16591,10 @@
         <v>46296</v>
       </c>
       <c r="B1469" t="n">
-        <v>358</v>
+        <v>2109</v>
       </c>
       <c r="C1469" t="n">
-        <v>100226</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1470">
@@ -16602,10 +16602,10 @@
         <v>46296</v>
       </c>
       <c r="B1470" t="n">
-        <v>1653</v>
+        <v>2693</v>
       </c>
       <c r="C1470" t="n">
-        <v>100226</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1471">
@@ -16613,10 +16613,10 @@
         <v>46296</v>
       </c>
       <c r="B1471" t="n">
-        <v>1317</v>
+        <v>1142</v>
       </c>
       <c r="C1471" t="n">
-        <v>100226</v>
+        <v>166576</v>
       </c>
     </row>
     <row r="1472">
@@ -16624,10 +16624,10 @@
         <v>46296</v>
       </c>
       <c r="B1472" t="n">
-        <v>2822</v>
+        <v>2082</v>
       </c>
       <c r="C1472" t="n">
-        <v>50904</v>
+        <v>36360</v>
       </c>
     </row>
     <row r="1473">
@@ -16635,10 +16635,10 @@
         <v>46296</v>
       </c>
       <c r="B1473" t="n">
-        <v>1117</v>
+        <v>2276</v>
       </c>
       <c r="C1473" t="n">
-        <v>127309</v>
+        <v>72336</v>
       </c>
     </row>
     <row r="1474">
@@ -16646,10 +16646,10 @@
         <v>46296</v>
       </c>
       <c r="B1474" t="n">
-        <v>1299</v>
+        <v>2786</v>
       </c>
       <c r="C1474" t="n">
-        <v>167853</v>
+        <v>25448</v>
       </c>
     </row>
     <row r="1475">
@@ -16657,10 +16657,10 @@
         <v>46296</v>
       </c>
       <c r="B1475" t="n">
-        <v>477</v>
+        <v>2816</v>
       </c>
       <c r="C1475" t="n">
-        <v>69174</v>
+        <v>47272</v>
       </c>
     </row>
     <row r="1476">
@@ -16668,10 +16668,10 @@
         <v>46296</v>
       </c>
       <c r="B1476" t="n">
-        <v>530</v>
+        <v>1871</v>
       </c>
       <c r="C1476" t="n">
-        <v>95452</v>
+        <v>52184</v>
       </c>
     </row>
     <row r="1477">
@@ -16679,10 +16679,10 @@
         <v>46296</v>
       </c>
       <c r="B1477" t="n">
-        <v>953</v>
+        <v>2345</v>
       </c>
       <c r="C1477" t="n">
-        <v>219541</v>
+        <v>23200</v>
       </c>
     </row>
     <row r="1478">
@@ -16690,10 +16690,10 @@
         <v>46296</v>
       </c>
       <c r="B1478" t="n">
-        <v>610</v>
+        <v>2802</v>
       </c>
       <c r="C1478" t="n">
-        <v>261478</v>
+        <v>26104</v>
       </c>
     </row>
     <row r="1479">
@@ -16701,10 +16701,10 @@
         <v>46296</v>
       </c>
       <c r="B1479" t="n">
-        <v>2792</v>
+        <v>2090</v>
       </c>
       <c r="C1479" t="n">
-        <v>65667</v>
+        <v>15128</v>
       </c>
     </row>
     <row r="1480">
@@ -16712,10 +16712,10 @@
         <v>46296</v>
       </c>
       <c r="B1480" t="n">
-        <v>2834</v>
+        <v>2647</v>
       </c>
       <c r="C1480" t="n">
-        <v>11858</v>
+        <v>51000</v>
       </c>
     </row>
     <row r="1481">
@@ -16723,10 +16723,10 @@
         <v>46296</v>
       </c>
       <c r="B1481" t="n">
-        <v>952</v>
+        <v>2365</v>
       </c>
       <c r="C1481" t="n">
-        <v>31815</v>
+        <v>36360</v>
       </c>
     </row>
     <row r="1482">
@@ -16734,10 +16734,10 @@
         <v>46296</v>
       </c>
       <c r="B1482" t="n">
-        <v>1539</v>
+        <v>766</v>
       </c>
       <c r="C1482" t="n">
-        <v>54089</v>
+        <v>24976</v>
       </c>
     </row>
     <row r="1483">
@@ -16745,10 +16745,10 @@
         <v>46296</v>
       </c>
       <c r="B1483" t="n">
-        <v>793</v>
+        <v>2702</v>
       </c>
       <c r="C1483" t="n">
-        <v>13237</v>
+        <v>29632</v>
       </c>
     </row>
     <row r="1484">
@@ -16756,10 +16756,10 @@
         <v>46296</v>
       </c>
       <c r="B1484" t="n">
-        <v>794</v>
+        <v>20</v>
       </c>
       <c r="C1484" t="n">
-        <v>13237</v>
+        <v>163632</v>
       </c>
     </row>
     <row r="1485">
@@ -16767,10 +16767,10 @@
         <v>46296</v>
       </c>
       <c r="B1485" t="n">
-        <v>2838</v>
+        <v>27</v>
       </c>
       <c r="C1485" t="n">
-        <v>15904</v>
+        <v>54544</v>
       </c>
     </row>
     <row r="1486">
@@ -16778,10 +16778,10 @@
         <v>46296</v>
       </c>
       <c r="B1486" t="n">
-        <v>2762</v>
+        <v>33</v>
       </c>
       <c r="C1486" t="n">
-        <v>25928</v>
+        <v>144720</v>
       </c>
     </row>
     <row r="1487">
@@ -16789,10 +16789,10 @@
         <v>46296</v>
       </c>
       <c r="B1487" t="n">
-        <v>749</v>
+        <v>2554</v>
       </c>
       <c r="C1487" t="n">
-        <v>25928</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1488">
@@ -16800,10 +16800,10 @@
         <v>46296</v>
       </c>
       <c r="B1488" t="n">
-        <v>2258</v>
+        <v>2561</v>
       </c>
       <c r="C1488" t="n">
-        <v>25452</v>
+        <v>14216</v>
       </c>
     </row>
     <row r="1489">
@@ -16811,10 +16811,10 @@
         <v>46296</v>
       </c>
       <c r="B1489" t="n">
-        <v>2744</v>
+        <v>2772</v>
       </c>
       <c r="C1489" t="n">
-        <v>19089</v>
+        <v>21816</v>
       </c>
     </row>
     <row r="1490">
@@ -16822,10 +16822,10 @@
         <v>46296</v>
       </c>
       <c r="B1490" t="n">
-        <v>2653</v>
+        <v>132</v>
       </c>
       <c r="C1490" t="n">
-        <v>19089</v>
+        <v>127272</v>
       </c>
     </row>
     <row r="1491">
@@ -16833,10 +16833,10 @@
         <v>46296</v>
       </c>
       <c r="B1491" t="n">
-        <v>2742</v>
+        <v>580</v>
       </c>
       <c r="C1491" t="n">
-        <v>19089</v>
+        <v>63632</v>
       </c>
     </row>
     <row r="1492">
@@ -16844,10 +16844,10 @@
         <v>46296</v>
       </c>
       <c r="B1492" t="n">
-        <v>1499</v>
+        <v>634</v>
       </c>
       <c r="C1492" t="n">
-        <v>28630</v>
+        <v>181816</v>
       </c>
     </row>
     <row r="1493">
@@ -16855,10 +16855,10 @@
         <v>46296</v>
       </c>
       <c r="B1493" t="n">
-        <v>2261</v>
+        <v>1277</v>
       </c>
       <c r="C1493" t="n">
-        <v>57267</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="1494">
@@ -16866,10 +16866,10 @@
         <v>46296</v>
       </c>
       <c r="B1494" t="n">
-        <v>2709</v>
+        <v>767</v>
       </c>
       <c r="C1494" t="n">
-        <v>57267</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1495">
@@ -16877,10 +16877,10 @@
         <v>46296</v>
       </c>
       <c r="B1495" t="n">
-        <v>1137</v>
+        <v>2727</v>
       </c>
       <c r="C1495" t="n">
-        <v>203630</v>
+        <v>14720</v>
       </c>
     </row>
     <row r="1496">
@@ -16888,10 +16888,10 @@
         <v>46296</v>
       </c>
       <c r="B1496" t="n">
-        <v>429</v>
+        <v>2846</v>
       </c>
       <c r="C1496" t="n">
-        <v>120904</v>
+        <v>94544</v>
       </c>
     </row>
     <row r="1497">
@@ -16899,10 +16899,10 @@
         <v>46296</v>
       </c>
       <c r="B1497" t="n">
-        <v>2114</v>
+        <v>609</v>
       </c>
       <c r="C1497" t="n">
-        <v>54131</v>
+        <v>81816</v>
       </c>
     </row>
     <row r="1498">
@@ -16910,10 +16910,10 @@
         <v>46296</v>
       </c>
       <c r="B1498" t="n">
-        <v>2211</v>
+        <v>2726</v>
       </c>
       <c r="C1498" t="n">
-        <v>76629</v>
+        <v>56360</v>
       </c>
     </row>
     <row r="1499">
@@ -16921,10 +16921,10 @@
         <v>46296</v>
       </c>
       <c r="B1499" t="n">
-        <v>1108</v>
+        <v>2729</v>
       </c>
       <c r="C1499" t="n">
-        <v>97482</v>
+        <v>32720</v>
       </c>
     </row>
     <row r="1500">
@@ -16932,10 +16932,10 @@
         <v>46296</v>
       </c>
       <c r="B1500" t="n">
-        <v>2695</v>
+        <v>1340</v>
       </c>
       <c r="C1500" t="n">
-        <v>15393</v>
+        <v>54544</v>
       </c>
     </row>
     <row r="1501">
@@ -16943,10 +16943,10 @@
         <v>46296</v>
       </c>
       <c r="B1501" t="n">
-        <v>1289</v>
+        <v>2830</v>
       </c>
       <c r="C1501" t="n">
-        <v>87500</v>
+        <v>32720</v>
       </c>
     </row>
     <row r="1502">
@@ -16954,10 +16954,10 @@
         <v>46296</v>
       </c>
       <c r="B1502" t="n">
-        <v>2789</v>
+        <v>2674</v>
       </c>
       <c r="C1502" t="n">
-        <v>57267</v>
+        <v>94544</v>
       </c>
     </row>
     <row r="1503">
@@ -16965,10 +16965,10 @@
         <v>46296</v>
       </c>
       <c r="B1503" t="n">
-        <v>2197</v>
+        <v>2308</v>
       </c>
       <c r="C1503" t="n">
-        <v>68404</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1504">
@@ -16976,10 +16976,10 @@
         <v>46296</v>
       </c>
       <c r="B1504" t="n">
-        <v>947</v>
+        <v>2601</v>
       </c>
       <c r="C1504" t="n">
-        <v>141106</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1505">
@@ -16987,10 +16987,10 @@
         <v>46296</v>
       </c>
       <c r="B1505" t="n">
-        <v>2279</v>
+        <v>2190</v>
       </c>
       <c r="C1505" t="n">
-        <v>77931</v>
+        <v>76360</v>
       </c>
     </row>
     <row r="1506">
@@ -16998,10 +16998,10 @@
         <v>46296</v>
       </c>
       <c r="B1506" t="n">
-        <v>1465</v>
+        <v>2015</v>
       </c>
       <c r="C1506" t="n">
-        <v>122500</v>
+        <v>134544</v>
       </c>
     </row>
     <row r="1507">
@@ -17009,10 +17009,10 @@
         <v>46296</v>
       </c>
       <c r="B1507" t="n">
-        <v>2651</v>
+        <v>1308</v>
       </c>
       <c r="C1507" t="n">
-        <v>54089</v>
+        <v>57088</v>
       </c>
     </row>
     <row r="1508">
@@ -17020,10 +17020,10 @@
         <v>46296</v>
       </c>
       <c r="B1508" t="n">
-        <v>42</v>
+        <v>2118</v>
       </c>
       <c r="C1508" t="n">
-        <v>606452</v>
+        <v>76424</v>
       </c>
     </row>
     <row r="1509">
@@ -17031,10 +17031,10 @@
         <v>46296</v>
       </c>
       <c r="B1509" t="n">
-        <v>2045</v>
+        <v>2607</v>
       </c>
       <c r="C1509" t="n">
-        <v>101332</v>
+        <v>18064</v>
       </c>
     </row>
     <row r="1510">
@@ -17042,10 +17042,10 @@
         <v>46296</v>
       </c>
       <c r="B1510" t="n">
-        <v>2663</v>
+        <v>2707</v>
       </c>
       <c r="C1510" t="n">
-        <v>87500</v>
+        <v>15704</v>
       </c>
     </row>
     <row r="1511">
@@ -17053,10 +17053,10 @@
         <v>46296</v>
       </c>
       <c r="B1511" t="n">
-        <v>2823</v>
+        <v>2383</v>
       </c>
       <c r="C1511" t="n">
-        <v>22589</v>
+        <v>48336</v>
       </c>
     </row>
     <row r="1512">
@@ -17064,10 +17064,10 @@
         <v>46296</v>
       </c>
       <c r="B1512" t="n">
-        <v>2757</v>
+        <v>2821</v>
       </c>
       <c r="C1512" t="n">
-        <v>25452</v>
+        <v>48488</v>
       </c>
     </row>
     <row r="1513">
@@ -17075,10 +17075,10 @@
         <v>46296</v>
       </c>
       <c r="B1513" t="n">
-        <v>2815</v>
+        <v>569</v>
       </c>
       <c r="C1513" t="n">
-        <v>19089</v>
+        <v>1055792</v>
       </c>
     </row>
     <row r="1514">
@@ -17086,10 +17086,10 @@
         <v>46296</v>
       </c>
       <c r="B1514" t="n">
-        <v>2829</v>
+        <v>2660</v>
       </c>
       <c r="C1514" t="n">
-        <v>19089</v>
+        <v>127272</v>
       </c>
     </row>
     <row r="1515">
@@ -17097,10 +17097,10 @@
         <v>46296</v>
       </c>
       <c r="B1515" t="n">
-        <v>2496</v>
+        <v>1632</v>
       </c>
       <c r="C1515" t="n">
-        <v>63630</v>
+        <v>94544</v>
       </c>
     </row>
     <row r="1516">
@@ -17108,10 +17108,10 @@
         <v>46296</v>
       </c>
       <c r="B1516" t="n">
-        <v>2131</v>
+        <v>1756</v>
       </c>
       <c r="C1516" t="n">
-        <v>31815</v>
+        <v>152720</v>
       </c>
     </row>
     <row r="1517">
@@ -17119,10 +17119,10 @@
         <v>46296</v>
       </c>
       <c r="B1517" t="n">
-        <v>2847</v>
+        <v>58</v>
       </c>
       <c r="C1517" t="n">
-        <v>42952</v>
+        <v>91200</v>
       </c>
     </row>
     <row r="1518">
@@ -17130,10 +17130,10 @@
         <v>46296</v>
       </c>
       <c r="B1518" t="n">
-        <v>1293</v>
+        <v>40</v>
       </c>
       <c r="C1518" t="n">
-        <v>122500</v>
+        <v>81120</v>
       </c>
     </row>
     <row r="1519">
@@ -17141,10 +17141,10 @@
         <v>46296</v>
       </c>
       <c r="B1519" t="n">
-        <v>631</v>
+        <v>559</v>
       </c>
       <c r="C1519" t="n">
-        <v>111363</v>
+        <v>85088</v>
       </c>
     </row>
     <row r="1520">
@@ -17152,10 +17152,10 @@
         <v>46296</v>
       </c>
       <c r="B1520" t="n">
-        <v>2791</v>
+        <v>2773</v>
       </c>
       <c r="C1520" t="n">
-        <v>32669</v>
+        <v>29336</v>
       </c>
     </row>
     <row r="1521">
@@ -17163,10 +17163,10 @@
         <v>46296</v>
       </c>
       <c r="B1521" t="n">
-        <v>2571</v>
+        <v>2631</v>
       </c>
       <c r="C1521" t="n">
-        <v>84819</v>
+        <v>14088</v>
       </c>
     </row>
     <row r="1522">
@@ -17174,10 +17174,10 @@
         <v>46296</v>
       </c>
       <c r="B1522" t="n">
-        <v>2273</v>
+        <v>2085</v>
       </c>
       <c r="C1522" t="n">
-        <v>68411</v>
+        <v>36360</v>
       </c>
     </row>
     <row r="1523">
@@ -17185,10 +17185,10 @@
         <v>46296</v>
       </c>
       <c r="B1523" t="n">
-        <v>2381</v>
+        <v>1642</v>
       </c>
       <c r="C1523" t="n">
-        <v>25585</v>
+        <v>96360</v>
       </c>
     </row>
     <row r="1524">
@@ -17196,10 +17196,10 @@
         <v>46296</v>
       </c>
       <c r="B1524" t="n">
-        <v>630</v>
+        <v>2621</v>
       </c>
       <c r="C1524" t="n">
-        <v>26257</v>
+        <v>25448</v>
       </c>
     </row>
     <row r="1525">
@@ -17207,10 +17207,10 @@
         <v>46296</v>
       </c>
       <c r="B1525" t="n">
-        <v>1983</v>
+        <v>2705</v>
       </c>
       <c r="C1525" t="n">
-        <v>174440</v>
+        <v>73008</v>
       </c>
     </row>
     <row r="1526">
@@ -17218,10 +17218,10 @@
         <v>46296</v>
       </c>
       <c r="B1526" t="n">
-        <v>1993</v>
+        <v>2735</v>
       </c>
       <c r="C1526" t="n">
-        <v>118454</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1527">
@@ -17229,10 +17229,10 @@
         <v>46296</v>
       </c>
       <c r="B1527" t="n">
-        <v>89</v>
+        <v>945</v>
       </c>
       <c r="C1527" t="n">
-        <v>111363</v>
+        <v>127520</v>
       </c>
     </row>
     <row r="1528">
@@ -17240,10 +17240,10 @@
         <v>46296</v>
       </c>
       <c r="B1528" t="n">
-        <v>1063</v>
+        <v>2582</v>
       </c>
       <c r="C1528" t="n">
-        <v>122500</v>
+        <v>31904</v>
       </c>
     </row>
     <row r="1529">
@@ -17251,10 +17251,10 @@
         <v>46296</v>
       </c>
       <c r="B1529" t="n">
-        <v>1116</v>
+        <v>2584</v>
       </c>
       <c r="C1529" t="n">
-        <v>79541</v>
+        <v>23200</v>
       </c>
     </row>
     <row r="1530">
@@ -17262,10 +17262,10 @@
         <v>46296</v>
       </c>
       <c r="B1530" t="n">
-        <v>941</v>
+        <v>2689</v>
       </c>
       <c r="C1530" t="n">
-        <v>95739</v>
+        <v>23200</v>
       </c>
     </row>
     <row r="1531">
@@ -17273,10 +17273,10 @@
         <v>46296</v>
       </c>
       <c r="B1531" t="n">
-        <v>2141</v>
+        <v>2574</v>
       </c>
       <c r="C1531" t="n">
-        <v>10206</v>
+        <v>50992</v>
       </c>
     </row>
     <row r="1532">
@@ -17284,10 +17284,10 @@
         <v>46296</v>
       </c>
       <c r="B1532" t="n">
-        <v>2463</v>
+        <v>1834</v>
       </c>
       <c r="C1532" t="n">
-        <v>104944</v>
+        <v>42800</v>
       </c>
     </row>
     <row r="1533">
@@ -17295,10 +17295,10 @@
         <v>46296</v>
       </c>
       <c r="B1533" t="n">
-        <v>1890</v>
+        <v>2629</v>
       </c>
       <c r="C1533" t="n">
-        <v>78029</v>
+        <v>24976</v>
       </c>
     </row>
     <row r="1534">
@@ -17306,10 +17306,10 @@
         <v>46296</v>
       </c>
       <c r="B1534" t="n">
-        <v>2639</v>
+        <v>933</v>
       </c>
       <c r="C1534" t="n">
-        <v>12747</v>
+        <v>29632</v>
       </c>
     </row>
     <row r="1535">
@@ -17317,10 +17317,10 @@
         <v>46296</v>
       </c>
       <c r="B1535" t="n">
-        <v>1075</v>
+        <v>1499</v>
       </c>
       <c r="C1535" t="n">
-        <v>146041</v>
+        <v>32720</v>
       </c>
     </row>
     <row r="1536">
@@ -17328,10 +17328,10 @@
         <v>46296</v>
       </c>
       <c r="B1536" t="n">
-        <v>131</v>
+        <v>2261</v>
       </c>
       <c r="C1536" t="n">
-        <v>132363</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1537">
@@ -17339,10 +17339,10 @@
         <v>46296</v>
       </c>
       <c r="B1537" t="n">
-        <v>2667</v>
+        <v>1324</v>
       </c>
       <c r="C1537" t="n">
-        <v>14539</v>
+        <v>101816</v>
       </c>
     </row>
     <row r="1538">
@@ -17350,10 +17350,10 @@
         <v>46296</v>
       </c>
       <c r="B1538" t="n">
-        <v>2330</v>
+        <v>2709</v>
       </c>
       <c r="C1538" t="n">
-        <v>28301</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1539">
@@ -17361,10 +17361,10 @@
         <v>46296</v>
       </c>
       <c r="B1539" t="n">
-        <v>2577</v>
+        <v>1137</v>
       </c>
       <c r="C1539" t="n">
-        <v>28371</v>
+        <v>232720</v>
       </c>
     </row>
     <row r="1540">
@@ -17372,10 +17372,10 @@
         <v>46296</v>
       </c>
       <c r="B1540" t="n">
-        <v>2745</v>
+        <v>2440</v>
       </c>
       <c r="C1540" t="n">
-        <v>35000</v>
+        <v>29088</v>
       </c>
     </row>
     <row r="1541">
@@ -17383,10 +17383,10 @@
         <v>46296</v>
       </c>
       <c r="B1541" t="n">
-        <v>2817</v>
+        <v>429</v>
       </c>
       <c r="C1541" t="n">
-        <v>19089</v>
+        <v>138176</v>
       </c>
     </row>
     <row r="1542">
@@ -17394,10 +17394,10 @@
         <v>46296</v>
       </c>
       <c r="B1542" t="n">
-        <v>2784</v>
+        <v>2114</v>
       </c>
       <c r="C1542" t="n">
-        <v>13237</v>
+        <v>61864</v>
       </c>
     </row>
     <row r="1543">
@@ -17405,10 +17405,10 @@
         <v>46296</v>
       </c>
       <c r="B1543" t="n">
-        <v>626</v>
+        <v>2211</v>
       </c>
       <c r="C1543" t="n">
-        <v>549759</v>
+        <v>87576</v>
       </c>
     </row>
     <row r="1544">
@@ -17416,10 +17416,10 @@
         <v>46296</v>
       </c>
       <c r="B1544" t="n">
-        <v>2586</v>
+        <v>1108</v>
       </c>
       <c r="C1544" t="n">
-        <v>13237</v>
+        <v>111408</v>
       </c>
     </row>
     <row r="1545">
@@ -17427,10 +17427,10 @@
         <v>46296</v>
       </c>
       <c r="B1545" t="n">
-        <v>966</v>
+        <v>2695</v>
       </c>
       <c r="C1545" t="n">
-        <v>25928</v>
+        <v>17592</v>
       </c>
     </row>
     <row r="1546">
@@ -17438,10 +17438,10 @@
         <v>46296</v>
       </c>
       <c r="B1546" t="n">
-        <v>2798</v>
+        <v>1289</v>
       </c>
       <c r="C1546" t="n">
-        <v>19089</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1547">
@@ -17449,10 +17449,10 @@
         <v>46296</v>
       </c>
       <c r="B1547" t="n">
-        <v>2797</v>
+        <v>2789</v>
       </c>
       <c r="C1547" t="n">
-        <v>19089</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1548">
@@ -17460,10 +17460,10 @@
         <v>46296</v>
       </c>
       <c r="B1548" t="n">
-        <v>2819</v>
+        <v>2197</v>
       </c>
       <c r="C1548" t="n">
-        <v>19089</v>
+        <v>78176</v>
       </c>
     </row>
     <row r="1549">
@@ -17471,10 +17471,10 @@
         <v>46296</v>
       </c>
       <c r="B1549" t="n">
-        <v>2266</v>
+        <v>947</v>
       </c>
       <c r="C1549" t="n">
-        <v>25452</v>
+        <v>161264</v>
       </c>
     </row>
     <row r="1550">
@@ -17482,10 +17482,10 @@
         <v>46296</v>
       </c>
       <c r="B1550" t="n">
-        <v>2795</v>
+        <v>2279</v>
       </c>
       <c r="C1550" t="n">
-        <v>19089</v>
+        <v>89064</v>
       </c>
     </row>
     <row r="1551">
@@ -17493,10 +17493,10 @@
         <v>46296</v>
       </c>
       <c r="B1551" t="n">
-        <v>2722</v>
+        <v>1465</v>
       </c>
       <c r="C1551" t="n">
-        <v>6363</v>
+        <v>140000</v>
       </c>
     </row>
     <row r="1552">
@@ -17504,10 +17504,10 @@
         <v>46296</v>
       </c>
       <c r="B1552" t="n">
-        <v>1853</v>
+        <v>2651</v>
       </c>
       <c r="C1552" t="n">
-        <v>38178</v>
+        <v>61816</v>
       </c>
     </row>
     <row r="1553">
@@ -17515,10 +17515,10 @@
         <v>46296</v>
       </c>
       <c r="B1553" t="n">
-        <v>2842</v>
+        <v>42</v>
       </c>
       <c r="C1553" t="n">
-        <v>57267</v>
+        <v>693088</v>
       </c>
     </row>
     <row r="1554">
@@ -17526,10 +17526,10 @@
         <v>46296</v>
       </c>
       <c r="B1554" t="n">
-        <v>2831</v>
+        <v>949</v>
       </c>
       <c r="C1554" t="n">
-        <v>19089</v>
+        <v>36168</v>
       </c>
     </row>
     <row r="1555">
@@ -17537,10 +17537,10 @@
         <v>46296</v>
       </c>
       <c r="B1555" t="n">
-        <v>818</v>
+        <v>2606</v>
       </c>
       <c r="C1555" t="n">
-        <v>127267</v>
+        <v>93360</v>
       </c>
     </row>
     <row r="1556">
@@ -17548,10 +17548,10 @@
         <v>46296</v>
       </c>
       <c r="B1556" t="n">
-        <v>2696</v>
+        <v>2249</v>
       </c>
       <c r="C1556" t="n">
-        <v>68236</v>
+        <v>79320</v>
       </c>
     </row>
     <row r="1557">
@@ -17559,10 +17559,10 @@
         <v>46296</v>
       </c>
       <c r="B1557" t="n">
-        <v>2698</v>
+        <v>2045</v>
       </c>
       <c r="C1557" t="n">
-        <v>34972</v>
+        <v>115808</v>
       </c>
     </row>
     <row r="1558">
@@ -17570,10 +17570,10 @@
         <v>46296</v>
       </c>
       <c r="B1558" t="n">
-        <v>619</v>
+        <v>2663</v>
       </c>
       <c r="C1558" t="n">
-        <v>99750</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1559">
@@ -17581,10 +17581,10 @@
         <v>46296</v>
       </c>
       <c r="B1559" t="n">
-        <v>1478</v>
+        <v>2823</v>
       </c>
       <c r="C1559" t="n">
-        <v>174566</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1560">
@@ -17592,10 +17592,10 @@
         <v>46296</v>
       </c>
       <c r="B1560" t="n">
-        <v>2026</v>
+        <v>2341</v>
       </c>
       <c r="C1560" t="n">
-        <v>77126</v>
+        <v>63600</v>
       </c>
     </row>
     <row r="1561">
@@ -17603,10 +17603,10 @@
         <v>46296</v>
       </c>
       <c r="B1561" t="n">
-        <v>285</v>
+        <v>2637</v>
       </c>
       <c r="C1561" t="n">
-        <v>174566</v>
+        <v>23200</v>
       </c>
     </row>
     <row r="1562">
@@ -17614,10 +17614,10 @@
         <v>46296</v>
       </c>
       <c r="B1562" t="n">
-        <v>424</v>
+        <v>2492</v>
       </c>
       <c r="C1562" t="n">
-        <v>74809</v>
+        <v>36424</v>
       </c>
     </row>
     <row r="1563">
@@ -17625,10 +17625,10 @@
         <v>46296</v>
       </c>
       <c r="B1563" t="n">
-        <v>451</v>
+        <v>2548</v>
       </c>
       <c r="C1563" t="n">
-        <v>77315</v>
+        <v>14216</v>
       </c>
     </row>
     <row r="1564">
@@ -17636,10 +17636,10 @@
         <v>46296</v>
       </c>
       <c r="B1564" t="n">
-        <v>629</v>
+        <v>351</v>
       </c>
       <c r="C1564" t="n">
-        <v>144452</v>
+        <v>77448</v>
       </c>
     </row>
     <row r="1565">
@@ -17647,10 +17647,10 @@
         <v>46296</v>
       </c>
       <c r="B1565" t="n">
-        <v>663</v>
+        <v>531</v>
       </c>
       <c r="C1565" t="n">
-        <v>82404</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1566">
@@ -17658,10 +17658,10 @@
         <v>46296</v>
       </c>
       <c r="B1566" t="n">
-        <v>2657</v>
+        <v>2757</v>
       </c>
       <c r="C1566" t="n">
-        <v>25193</v>
+        <v>29088</v>
       </c>
     </row>
     <row r="1567">
@@ -17669,10 +17669,10 @@
         <v>46296</v>
       </c>
       <c r="B1567" t="n">
-        <v>1254</v>
+        <v>2815</v>
       </c>
       <c r="C1567" t="n">
-        <v>61789</v>
+        <v>21816</v>
       </c>
     </row>
     <row r="1568">
@@ -17680,10 +17680,10 @@
         <v>46296</v>
       </c>
       <c r="B1568" t="n">
-        <v>2671</v>
+        <v>2829</v>
       </c>
       <c r="C1568" t="n">
-        <v>25452</v>
+        <v>21816</v>
       </c>
     </row>
     <row r="1569">
@@ -17691,10 +17691,10 @@
         <v>46296</v>
       </c>
       <c r="B1569" t="n">
-        <v>2753</v>
+        <v>768</v>
       </c>
       <c r="C1569" t="n">
-        <v>23863</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1570">
@@ -17702,10 +17702,10 @@
         <v>46296</v>
       </c>
       <c r="B1570" t="n">
-        <v>744</v>
+        <v>772</v>
       </c>
       <c r="C1570" t="n">
-        <v>13237</v>
+        <v>118176</v>
       </c>
     </row>
     <row r="1571">
@@ -17713,10 +17713,10 @@
         <v>46296</v>
       </c>
       <c r="B1571" t="n">
-        <v>2323</v>
+        <v>2496</v>
       </c>
       <c r="C1571" t="n">
-        <v>21854</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1572">
@@ -17724,10 +17724,10 @@
         <v>46296</v>
       </c>
       <c r="B1572" t="n">
-        <v>2310</v>
+        <v>802</v>
       </c>
       <c r="C1572" t="n">
-        <v>21854</v>
+        <v>27272</v>
       </c>
     </row>
     <row r="1573">
@@ -17735,10 +17735,10 @@
         <v>46296</v>
       </c>
       <c r="B1573" t="n">
-        <v>2501</v>
+        <v>2131</v>
       </c>
       <c r="C1573" t="n">
-        <v>25928</v>
+        <v>36360</v>
       </c>
     </row>
     <row r="1574">
@@ -17746,10 +17746,10 @@
         <v>46296</v>
       </c>
       <c r="B1574" t="n">
-        <v>716</v>
+        <v>1381</v>
       </c>
       <c r="C1574" t="n">
-        <v>40782</v>
+        <v>109088</v>
       </c>
     </row>
     <row r="1575">
@@ -17757,10 +17757,10 @@
         <v>46296</v>
       </c>
       <c r="B1575" t="n">
-        <v>2758</v>
+        <v>2847</v>
       </c>
       <c r="C1575" t="n">
-        <v>19089</v>
+        <v>49088</v>
       </c>
     </row>
     <row r="1576">
@@ -17768,10 +17768,10 @@
         <v>46296</v>
       </c>
       <c r="B1576" t="n">
-        <v>1259</v>
+        <v>1293</v>
       </c>
       <c r="C1576" t="n">
-        <v>35000</v>
+        <v>140000</v>
       </c>
     </row>
     <row r="1577">
@@ -17779,10 +17779,10 @@
         <v>46296</v>
       </c>
       <c r="B1577" t="n">
-        <v>2833</v>
+        <v>2363</v>
       </c>
       <c r="C1577" t="n">
-        <v>25452</v>
+        <v>61816</v>
       </c>
     </row>
     <row r="1578">
@@ -17790,10 +17790,10 @@
         <v>46296</v>
       </c>
       <c r="B1578" t="n">
-        <v>2687</v>
+        <v>631</v>
       </c>
       <c r="C1578" t="n">
-        <v>25452</v>
+        <v>127272</v>
       </c>
     </row>
     <row r="1579">
@@ -17801,10 +17801,10 @@
         <v>46296</v>
       </c>
       <c r="B1579" t="n">
-        <v>2824</v>
+        <v>2791</v>
       </c>
       <c r="C1579" t="n">
-        <v>35924</v>
+        <v>37336</v>
       </c>
     </row>
     <row r="1580">
@@ -17812,10 +17812,10 @@
         <v>46296</v>
       </c>
       <c r="B1580" t="n">
-        <v>2730</v>
+        <v>1380</v>
       </c>
       <c r="C1580" t="n">
-        <v>28630</v>
+        <v>18176</v>
       </c>
     </row>
     <row r="1581">
@@ -17823,10 +17823,10 @@
         <v>46296</v>
       </c>
       <c r="B1581" t="n">
-        <v>2718</v>
+        <v>2841</v>
       </c>
       <c r="C1581" t="n">
-        <v>41363</v>
+        <v>18176</v>
       </c>
     </row>
     <row r="1582">
@@ -17834,10 +17834,10 @@
         <v>46296</v>
       </c>
       <c r="B1582" t="n">
-        <v>2750</v>
+        <v>2571</v>
       </c>
       <c r="C1582" t="n">
-        <v>9541</v>
+        <v>96936</v>
       </c>
     </row>
     <row r="1583">
@@ -17845,10 +17845,10 @@
         <v>46296</v>
       </c>
       <c r="B1583" t="n">
-        <v>854</v>
+        <v>2273</v>
       </c>
       <c r="C1583" t="n">
-        <v>44541</v>
+        <v>78184</v>
       </c>
     </row>
     <row r="1584">
@@ -17856,10 +17856,10 @@
         <v>46296</v>
       </c>
       <c r="B1584" t="n">
-        <v>2794</v>
+        <v>2381</v>
       </c>
       <c r="C1584" t="n">
-        <v>38178</v>
+        <v>29240</v>
       </c>
     </row>
     <row r="1585">
@@ -17867,10 +17867,10 @@
         <v>46296</v>
       </c>
       <c r="B1585" t="n">
-        <v>2488</v>
+        <v>630</v>
       </c>
       <c r="C1585" t="n">
-        <v>31815</v>
+        <v>30008</v>
       </c>
     </row>
     <row r="1586">
@@ -17878,10 +17878,10 @@
         <v>46296</v>
       </c>
       <c r="B1586" t="n">
-        <v>363</v>
+        <v>2576</v>
       </c>
       <c r="C1586" t="n">
-        <v>95452</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1587">
@@ -17889,10 +17889,10 @@
         <v>46296</v>
       </c>
       <c r="B1587" t="n">
-        <v>2655</v>
+        <v>1983</v>
       </c>
       <c r="C1587" t="n">
-        <v>35000</v>
+        <v>199360</v>
       </c>
     </row>
     <row r="1588">
@@ -17900,10 +17900,10 @@
         <v>46296</v>
       </c>
       <c r="B1588" t="n">
-        <v>1873</v>
+        <v>1993</v>
       </c>
       <c r="C1588" t="n">
-        <v>101815</v>
+        <v>135376</v>
       </c>
     </row>
     <row r="1589">
@@ -17911,10 +17911,10 @@
         <v>46296</v>
       </c>
       <c r="B1589" t="n">
-        <v>2635</v>
+        <v>89</v>
       </c>
       <c r="C1589" t="n">
-        <v>41363</v>
+        <v>127272</v>
       </c>
     </row>
     <row r="1590">
@@ -17922,10 +17922,10 @@
         <v>46296</v>
       </c>
       <c r="B1590" t="n">
-        <v>636</v>
+        <v>1063</v>
       </c>
       <c r="C1590" t="n">
-        <v>79541</v>
+        <v>140000</v>
       </c>
     </row>
     <row r="1591">
@@ -17933,10 +17933,10 @@
         <v>46296</v>
       </c>
       <c r="B1591" t="n">
-        <v>2803</v>
+        <v>1116</v>
       </c>
       <c r="C1591" t="n">
-        <v>38178</v>
+        <v>90904</v>
       </c>
     </row>
     <row r="1592">
@@ -17944,10 +17944,10 @@
         <v>46296</v>
       </c>
       <c r="B1592" t="n">
-        <v>2163</v>
+        <v>941</v>
       </c>
       <c r="C1592" t="n">
-        <v>57267</v>
+        <v>109416</v>
       </c>
     </row>
     <row r="1593">
@@ -17955,10 +17955,10 @@
         <v>46296</v>
       </c>
       <c r="B1593" t="n">
-        <v>1466</v>
+        <v>2141</v>
       </c>
       <c r="C1593" t="n">
-        <v>128863</v>
+        <v>11664</v>
       </c>
     </row>
     <row r="1594">
@@ -17966,10 +17966,10 @@
         <v>46296</v>
       </c>
       <c r="B1594" t="n">
-        <v>535</v>
+        <v>2463</v>
       </c>
       <c r="C1594" t="n">
-        <v>113330</v>
+        <v>119936</v>
       </c>
     </row>
     <row r="1595">
@@ -17977,10 +17977,10 @@
         <v>46296</v>
       </c>
       <c r="B1595" t="n">
-        <v>2790</v>
+        <v>2325</v>
       </c>
       <c r="C1595" t="n">
-        <v>20097</v>
+        <v>41952</v>
       </c>
     </row>
     <row r="1596">
@@ -17988,10 +17988,10 @@
         <v>46296</v>
       </c>
       <c r="B1596" t="n">
-        <v>2768</v>
+        <v>1890</v>
       </c>
       <c r="C1596" t="n">
-        <v>96299</v>
+        <v>89176</v>
       </c>
     </row>
     <row r="1597">
@@ -17999,10 +17999,10 @@
         <v>46296</v>
       </c>
       <c r="B1597" t="n">
-        <v>2491</v>
+        <v>2639</v>
       </c>
       <c r="C1597" t="n">
-        <v>77273</v>
+        <v>14568</v>
       </c>
     </row>
     <row r="1598">
@@ -18010,10 +18010,1418 @@
         <v>46296</v>
       </c>
       <c r="B1598" t="n">
+        <v>2682</v>
+      </c>
+      <c r="C1598" t="n">
+        <v>50904</v>
+      </c>
+    </row>
+    <row r="1599">
+      <c r="A1599" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1599" t="n">
+        <v>703</v>
+      </c>
+      <c r="C1599" t="n">
+        <v>90904</v>
+      </c>
+    </row>
+    <row r="1600">
+      <c r="A1600" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1600" t="n">
+        <v>2833</v>
+      </c>
+      <c r="C1600" t="n">
+        <v>29088</v>
+      </c>
+    </row>
+    <row r="1601">
+      <c r="A1601" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1601" t="n">
+        <v>1007</v>
+      </c>
+      <c r="C1601" t="n">
+        <v>72720</v>
+      </c>
+    </row>
+    <row r="1602">
+      <c r="A1602" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1602" t="n">
+        <v>2687</v>
+      </c>
+      <c r="C1602" t="n">
+        <v>29088</v>
+      </c>
+    </row>
+    <row r="1603">
+      <c r="A1603" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1603" t="n">
+        <v>2824</v>
+      </c>
+      <c r="C1603" t="n">
+        <v>41056</v>
+      </c>
+    </row>
+    <row r="1604">
+      <c r="A1604" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1604" t="n">
+        <v>2730</v>
+      </c>
+      <c r="C1604" t="n">
+        <v>32720</v>
+      </c>
+    </row>
+    <row r="1605">
+      <c r="A1605" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1605" t="n">
+        <v>2718</v>
+      </c>
+      <c r="C1605" t="n">
+        <v>47272</v>
+      </c>
+    </row>
+    <row r="1606">
+      <c r="A1606" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1606" t="n">
+        <v>2750</v>
+      </c>
+      <c r="C1606" t="n">
+        <v>10904</v>
+      </c>
+    </row>
+    <row r="1607">
+      <c r="A1607" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1607" t="n">
+        <v>854</v>
+      </c>
+      <c r="C1607" t="n">
+        <v>50904</v>
+      </c>
+    </row>
+    <row r="1608">
+      <c r="A1608" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1608" t="n">
+        <v>2794</v>
+      </c>
+      <c r="C1608" t="n">
+        <v>43632</v>
+      </c>
+    </row>
+    <row r="1609">
+      <c r="A1609" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1609" t="n">
+        <v>1374</v>
+      </c>
+      <c r="C1609" t="n">
+        <v>72720</v>
+      </c>
+    </row>
+    <row r="1610">
+      <c r="A1610" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1610" t="n">
+        <v>2488</v>
+      </c>
+      <c r="C1610" t="n">
+        <v>36360</v>
+      </c>
+    </row>
+    <row r="1611">
+      <c r="A1611" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1611" t="n">
+        <v>363</v>
+      </c>
+      <c r="C1611" t="n">
+        <v>109088</v>
+      </c>
+    </row>
+    <row r="1612">
+      <c r="A1612" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1612" t="n">
+        <v>2655</v>
+      </c>
+      <c r="C1612" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="1613">
+      <c r="A1613" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1613" t="n">
+        <v>1873</v>
+      </c>
+      <c r="C1613" t="n">
+        <v>116360</v>
+      </c>
+    </row>
+    <row r="1614">
+      <c r="A1614" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1614" t="n">
+        <v>2635</v>
+      </c>
+      <c r="C1614" t="n">
+        <v>47272</v>
+      </c>
+    </row>
+    <row r="1615">
+      <c r="A1615" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1615" t="n">
+        <v>1658</v>
+      </c>
+      <c r="C1615" t="n">
+        <v>55632</v>
+      </c>
+    </row>
+    <row r="1616">
+      <c r="A1616" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1616" t="n">
+        <v>2069</v>
+      </c>
+      <c r="C1616" t="n">
+        <v>72720</v>
+      </c>
+    </row>
+    <row r="1617">
+      <c r="A1617" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1617" t="n">
+        <v>2081</v>
+      </c>
+      <c r="C1617" t="n">
+        <v>54544</v>
+      </c>
+    </row>
+    <row r="1618">
+      <c r="A1618" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1618" t="n">
+        <v>2124</v>
+      </c>
+      <c r="C1618" t="n">
+        <v>127272</v>
+      </c>
+    </row>
+    <row r="1619">
+      <c r="A1619" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1619" t="n">
+        <v>636</v>
+      </c>
+      <c r="C1619" t="n">
+        <v>90904</v>
+      </c>
+    </row>
+    <row r="1620">
+      <c r="A1620" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1620" t="n">
+        <v>2803</v>
+      </c>
+      <c r="C1620" t="n">
+        <v>43632</v>
+      </c>
+    </row>
+    <row r="1621">
+      <c r="A1621" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1621" t="n">
+        <v>2163</v>
+      </c>
+      <c r="C1621" t="n">
+        <v>65448</v>
+      </c>
+    </row>
+    <row r="1622">
+      <c r="A1622" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1622" t="n">
+        <v>1466</v>
+      </c>
+      <c r="C1622" t="n">
+        <v>147272</v>
+      </c>
+    </row>
+    <row r="1623">
+      <c r="A1623" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1623" t="n">
+        <v>2133</v>
+      </c>
+      <c r="C1623" t="n">
+        <v>127272</v>
+      </c>
+    </row>
+    <row r="1624">
+      <c r="A1624" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1624" t="n">
+        <v>2431</v>
+      </c>
+      <c r="C1624" t="n">
+        <v>54544</v>
+      </c>
+    </row>
+    <row r="1625">
+      <c r="A1625" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1625" t="n">
+        <v>535</v>
+      </c>
+      <c r="C1625" t="n">
+        <v>129520</v>
+      </c>
+    </row>
+    <row r="1626">
+      <c r="A1626" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1626" t="n">
+        <v>2790</v>
+      </c>
+      <c r="C1626" t="n">
+        <v>22968</v>
+      </c>
+    </row>
+    <row r="1627">
+      <c r="A1627" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1627" t="n">
+        <v>2442</v>
+      </c>
+      <c r="C1627" t="n">
+        <v>94176</v>
+      </c>
+    </row>
+    <row r="1628">
+      <c r="A1628" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1628" t="n">
+        <v>2376</v>
+      </c>
+      <c r="C1628" t="n">
+        <v>363632</v>
+      </c>
+    </row>
+    <row r="1629">
+      <c r="A1629" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1629" t="n">
+        <v>2768</v>
+      </c>
+      <c r="C1629" t="n">
+        <v>110056</v>
+      </c>
+    </row>
+    <row r="1630">
+      <c r="A1630" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1630" t="n">
+        <v>2491</v>
+      </c>
+      <c r="C1630" t="n">
+        <v>88312</v>
+      </c>
+    </row>
+    <row r="1631">
+      <c r="A1631" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1631" t="n">
         <v>2799</v>
       </c>
-      <c r="C1598" t="n">
-        <v>34783</v>
+      <c r="C1631" t="n">
+        <v>39752</v>
+      </c>
+    </row>
+    <row r="1632">
+      <c r="A1632" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1632" t="n">
+        <v>1317</v>
+      </c>
+      <c r="C1632" t="n">
+        <v>114544</v>
+      </c>
+    </row>
+    <row r="1633">
+      <c r="A1633" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1633" t="n">
+        <v>2822</v>
+      </c>
+      <c r="C1633" t="n">
+        <v>58176</v>
+      </c>
+    </row>
+    <row r="1634">
+      <c r="A1634" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1634" t="n">
+        <v>1117</v>
+      </c>
+      <c r="C1634" t="n">
+        <v>145496</v>
+      </c>
+    </row>
+    <row r="1635">
+      <c r="A1635" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1635" t="n">
+        <v>1299</v>
+      </c>
+      <c r="C1635" t="n">
+        <v>191832</v>
+      </c>
+    </row>
+    <row r="1636">
+      <c r="A1636" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1636" t="n">
+        <v>477</v>
+      </c>
+      <c r="C1636" t="n">
+        <v>79056</v>
+      </c>
+    </row>
+    <row r="1637">
+      <c r="A1637" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1637" t="n">
+        <v>530</v>
+      </c>
+      <c r="C1637" t="n">
+        <v>109088</v>
+      </c>
+    </row>
+    <row r="1638">
+      <c r="A1638" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1638" t="n">
+        <v>953</v>
+      </c>
+      <c r="C1638" t="n">
+        <v>250904</v>
+      </c>
+    </row>
+    <row r="1639">
+      <c r="A1639" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1639" t="n">
+        <v>610</v>
+      </c>
+      <c r="C1639" t="n">
+        <v>298832</v>
+      </c>
+    </row>
+    <row r="1640">
+      <c r="A1640" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1640" t="n">
+        <v>2792</v>
+      </c>
+      <c r="C1640" t="n">
+        <v>75048</v>
+      </c>
+    </row>
+    <row r="1641">
+      <c r="A1641" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1641" t="n">
+        <v>2834</v>
+      </c>
+      <c r="C1641" t="n">
+        <v>13552</v>
+      </c>
+    </row>
+    <row r="1642">
+      <c r="A1642" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1642" t="n">
+        <v>2394</v>
+      </c>
+      <c r="C1642" t="n">
+        <v>41256</v>
+      </c>
+    </row>
+    <row r="1643">
+      <c r="A1643" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1643" t="n">
+        <v>2567</v>
+      </c>
+      <c r="C1643" t="n">
+        <v>36360</v>
+      </c>
+    </row>
+    <row r="1644">
+      <c r="A1644" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1644" t="n">
+        <v>952</v>
+      </c>
+      <c r="C1644" t="n">
+        <v>36360</v>
+      </c>
+    </row>
+    <row r="1645">
+      <c r="A1645" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1645" t="n">
+        <v>1539</v>
+      </c>
+      <c r="C1645" t="n">
+        <v>61816</v>
+      </c>
+    </row>
+    <row r="1646">
+      <c r="A1646" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1646" t="n">
+        <v>793</v>
+      </c>
+      <c r="C1646" t="n">
+        <v>15128</v>
+      </c>
+    </row>
+    <row r="1647">
+      <c r="A1647" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1647" t="n">
+        <v>794</v>
+      </c>
+      <c r="C1647" t="n">
+        <v>15128</v>
+      </c>
+    </row>
+    <row r="1648">
+      <c r="A1648" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1648" t="n">
+        <v>2838</v>
+      </c>
+      <c r="C1648" t="n">
+        <v>21818.22</v>
+      </c>
+    </row>
+    <row r="1649">
+      <c r="A1649" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1649" t="n">
+        <v>2223</v>
+      </c>
+      <c r="C1649" t="n">
+        <v>42584</v>
+      </c>
+    </row>
+    <row r="1650">
+      <c r="A1650" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1650" t="n">
+        <v>2547</v>
+      </c>
+      <c r="C1650" t="n">
+        <v>12320</v>
+      </c>
+    </row>
+    <row r="1651">
+      <c r="A1651" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1651" t="n">
+        <v>2762</v>
+      </c>
+      <c r="C1651" t="n">
+        <v>29632</v>
+      </c>
+    </row>
+    <row r="1652">
+      <c r="A1652" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1652" t="n">
+        <v>2550</v>
+      </c>
+      <c r="C1652" t="n">
+        <v>14216</v>
+      </c>
+    </row>
+    <row r="1653">
+      <c r="A1653" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1653" t="n">
+        <v>2627</v>
+      </c>
+      <c r="C1653" t="n">
+        <v>14216</v>
+      </c>
+    </row>
+    <row r="1654">
+      <c r="A1654" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1654" t="n">
+        <v>2551</v>
+      </c>
+      <c r="C1654" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1655">
+      <c r="A1655" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1655" t="n">
+        <v>749</v>
+      </c>
+      <c r="C1655" t="n">
+        <v>29632</v>
+      </c>
+    </row>
+    <row r="1656">
+      <c r="A1656" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1656" t="n">
+        <v>2549</v>
+      </c>
+      <c r="C1656" t="n">
+        <v>14216</v>
+      </c>
+    </row>
+    <row r="1657">
+      <c r="A1657" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1657" t="n">
+        <v>2649</v>
+      </c>
+      <c r="C1657" t="n">
+        <v>14216</v>
+      </c>
+    </row>
+    <row r="1658">
+      <c r="A1658" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1658" t="n">
+        <v>2258</v>
+      </c>
+      <c r="C1658" t="n">
+        <v>29088</v>
+      </c>
+    </row>
+    <row r="1659">
+      <c r="A1659" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1659" t="n">
+        <v>2744</v>
+      </c>
+      <c r="C1659" t="n">
+        <v>21816</v>
+      </c>
+    </row>
+    <row r="1660">
+      <c r="A1660" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1660" t="n">
+        <v>452</v>
+      </c>
+      <c r="C1660" t="n">
+        <v>102904</v>
+      </c>
+    </row>
+    <row r="1661">
+      <c r="A1661" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1661" t="n">
+        <v>2653</v>
+      </c>
+      <c r="C1661" t="n">
+        <v>21816</v>
+      </c>
+    </row>
+    <row r="1662">
+      <c r="A1662" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1662" t="n">
+        <v>2742</v>
+      </c>
+      <c r="C1662" t="n">
+        <v>21816</v>
+      </c>
+    </row>
+    <row r="1663">
+      <c r="A1663" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1663" t="n">
+        <v>1075</v>
+      </c>
+      <c r="C1663" t="n">
+        <v>166904</v>
+      </c>
+    </row>
+    <row r="1664">
+      <c r="A1664" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1664" t="n">
+        <v>131</v>
+      </c>
+      <c r="C1664" t="n">
+        <v>151272</v>
+      </c>
+    </row>
+    <row r="1665">
+      <c r="A1665" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1665" t="n">
+        <v>2667</v>
+      </c>
+      <c r="C1665" t="n">
+        <v>16616</v>
+      </c>
+    </row>
+    <row r="1666">
+      <c r="A1666" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1666" t="n">
+        <v>2330</v>
+      </c>
+      <c r="C1666" t="n">
+        <v>32344</v>
+      </c>
+    </row>
+    <row r="1667">
+      <c r="A1667" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1667" t="n">
+        <v>2577</v>
+      </c>
+      <c r="C1667" t="n">
+        <v>32424</v>
+      </c>
+    </row>
+    <row r="1668">
+      <c r="A1668" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1668" t="n">
+        <v>2510</v>
+      </c>
+      <c r="C1668" t="n">
+        <v>230272</v>
+      </c>
+    </row>
+    <row r="1669">
+      <c r="A1669" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1669" t="n">
+        <v>2745</v>
+      </c>
+      <c r="C1669" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="1670">
+      <c r="A1670" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1670" t="n">
+        <v>2817</v>
+      </c>
+      <c r="C1670" t="n">
+        <v>21816</v>
+      </c>
+    </row>
+    <row r="1671">
+      <c r="A1671" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1671" t="n">
+        <v>2784</v>
+      </c>
+      <c r="C1671" t="n">
+        <v>15128</v>
+      </c>
+    </row>
+    <row r="1672">
+      <c r="A1672" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1672" t="n">
+        <v>626</v>
+      </c>
+      <c r="C1672" t="n">
+        <v>628296</v>
+      </c>
+    </row>
+    <row r="1673">
+      <c r="A1673" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1673" t="n">
+        <v>925</v>
+      </c>
+      <c r="C1673" t="n">
+        <v>29008</v>
+      </c>
+    </row>
+    <row r="1674">
+      <c r="A1674" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1674" t="n">
+        <v>2586</v>
+      </c>
+      <c r="C1674" t="n">
+        <v>15128</v>
+      </c>
+    </row>
+    <row r="1675">
+      <c r="A1675" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1675" t="n">
+        <v>966</v>
+      </c>
+      <c r="C1675" t="n">
+        <v>29632</v>
+      </c>
+    </row>
+    <row r="1676">
+      <c r="A1676" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1676" t="n">
+        <v>2557</v>
+      </c>
+      <c r="C1676" t="n">
+        <v>14216</v>
+      </c>
+    </row>
+    <row r="1677">
+      <c r="A1677" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1677" t="n">
+        <v>14</v>
+      </c>
+      <c r="C1677" t="n">
+        <v>163632</v>
+      </c>
+    </row>
+    <row r="1678">
+      <c r="A1678" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1678" t="n">
+        <v>2798</v>
+      </c>
+      <c r="C1678" t="n">
+        <v>21816</v>
+      </c>
+    </row>
+    <row r="1679">
+      <c r="A1679" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1679" t="n">
+        <v>2797</v>
+      </c>
+      <c r="C1679" t="n">
+        <v>21816</v>
+      </c>
+    </row>
+    <row r="1680">
+      <c r="A1680" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1680" t="n">
+        <v>522</v>
+      </c>
+      <c r="C1680" t="n">
+        <v>72720</v>
+      </c>
+    </row>
+    <row r="1681">
+      <c r="A1681" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1681" t="n">
+        <v>2819</v>
+      </c>
+      <c r="C1681" t="n">
+        <v>21816</v>
+      </c>
+    </row>
+    <row r="1682">
+      <c r="A1682" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1682" t="n">
+        <v>2266</v>
+      </c>
+      <c r="C1682" t="n">
+        <v>29088</v>
+      </c>
+    </row>
+    <row r="1683">
+      <c r="A1683" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1683" t="n">
+        <v>2795</v>
+      </c>
+      <c r="C1683" t="n">
+        <v>21816</v>
+      </c>
+    </row>
+    <row r="1684">
+      <c r="A1684" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1684" t="n">
+        <v>2722</v>
+      </c>
+      <c r="C1684" t="n">
+        <v>7272</v>
+      </c>
+    </row>
+    <row r="1685">
+      <c r="A1685" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1685" t="n">
+        <v>951</v>
+      </c>
+      <c r="C1685" t="n">
+        <v>41816</v>
+      </c>
+    </row>
+    <row r="1686">
+      <c r="A1686" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1686" t="n">
+        <v>1020</v>
+      </c>
+      <c r="C1686" t="n">
+        <v>36360</v>
+      </c>
+    </row>
+    <row r="1687">
+      <c r="A1687" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1687" t="n">
+        <v>1853</v>
+      </c>
+      <c r="C1687" t="n">
+        <v>43632</v>
+      </c>
+    </row>
+    <row r="1688">
+      <c r="A1688" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1688" t="n">
+        <v>1327</v>
+      </c>
+      <c r="C1688" t="n">
+        <v>25448</v>
+      </c>
+    </row>
+    <row r="1689">
+      <c r="A1689" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1689" t="n">
+        <v>2842</v>
+      </c>
+      <c r="C1689" t="n">
+        <v>65448</v>
+      </c>
+    </row>
+    <row r="1690">
+      <c r="A1690" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1690" t="n">
+        <v>2831</v>
+      </c>
+      <c r="C1690" t="n">
+        <v>21816</v>
+      </c>
+    </row>
+    <row r="1691">
+      <c r="A1691" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1691" t="n">
+        <v>818</v>
+      </c>
+      <c r="C1691" t="n">
+        <v>145448</v>
+      </c>
+    </row>
+    <row r="1692">
+      <c r="A1692" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1692" t="n">
+        <v>1501</v>
+      </c>
+      <c r="C1692" t="n">
+        <v>36360</v>
+      </c>
+    </row>
+    <row r="1693">
+      <c r="A1693" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1693" t="n">
+        <v>1869</v>
+      </c>
+      <c r="C1693" t="n">
+        <v>88720</v>
+      </c>
+    </row>
+    <row r="1694">
+      <c r="A1694" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1694" t="n">
+        <v>1996</v>
+      </c>
+      <c r="C1694" t="n">
+        <v>90904</v>
+      </c>
+    </row>
+    <row r="1695">
+      <c r="A1695" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1695" t="n">
+        <v>2462</v>
+      </c>
+      <c r="C1695" t="n">
+        <v>20592</v>
+      </c>
+    </row>
+    <row r="1696">
+      <c r="A1696" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1696" t="n">
+        <v>2696</v>
+      </c>
+      <c r="C1696" t="n">
+        <v>77984</v>
+      </c>
+    </row>
+    <row r="1697">
+      <c r="A1697" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1697" t="n">
+        <v>2698</v>
+      </c>
+      <c r="C1697" t="n">
+        <v>39968</v>
+      </c>
+    </row>
+    <row r="1698">
+      <c r="A1698" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1698" t="n">
+        <v>2828</v>
+      </c>
+      <c r="C1698" t="n">
+        <v>21818.22</v>
+      </c>
+    </row>
+    <row r="1699">
+      <c r="A1699" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1699" t="n">
+        <v>619</v>
+      </c>
+      <c r="C1699" t="n">
+        <v>114000</v>
+      </c>
+    </row>
+    <row r="1700">
+      <c r="A1700" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1700" t="n">
+        <v>1478</v>
+      </c>
+      <c r="C1700" t="n">
+        <v>199504</v>
+      </c>
+    </row>
+    <row r="1701">
+      <c r="A1701" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1701" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1701" t="n">
+        <v>88144</v>
+      </c>
+    </row>
+    <row r="1702">
+      <c r="A1702" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1702" t="n">
+        <v>285</v>
+      </c>
+      <c r="C1702" t="n">
+        <v>199504</v>
+      </c>
+    </row>
+    <row r="1703">
+      <c r="A1703" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1703" t="n">
+        <v>424</v>
+      </c>
+      <c r="C1703" t="n">
+        <v>85496</v>
+      </c>
+    </row>
+    <row r="1704">
+      <c r="A1704" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1704" t="n">
+        <v>451</v>
+      </c>
+      <c r="C1704" t="n">
+        <v>88360</v>
+      </c>
+    </row>
+    <row r="1705">
+      <c r="A1705" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1705" t="n">
+        <v>629</v>
+      </c>
+      <c r="C1705" t="n">
+        <v>165088</v>
+      </c>
+    </row>
+    <row r="1706">
+      <c r="A1706" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1706" t="n">
+        <v>663</v>
+      </c>
+      <c r="C1706" t="n">
+        <v>94176</v>
+      </c>
+    </row>
+    <row r="1707">
+      <c r="A1707" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1707" t="n">
+        <v>2657</v>
+      </c>
+      <c r="C1707" t="n">
+        <v>28792</v>
+      </c>
+    </row>
+    <row r="1708">
+      <c r="A1708" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1708" t="n">
+        <v>1254</v>
+      </c>
+      <c r="C1708" t="n">
+        <v>70616</v>
+      </c>
+    </row>
+    <row r="1709">
+      <c r="A1709" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1709" t="n">
+        <v>2402</v>
+      </c>
+      <c r="C1709" t="n">
+        <v>177616</v>
+      </c>
+    </row>
+    <row r="1710">
+      <c r="A1710" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1710" t="n">
+        <v>2413</v>
+      </c>
+      <c r="C1710" t="n">
+        <v>50120</v>
+      </c>
+    </row>
+    <row r="1711">
+      <c r="A1711" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1711" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C1711" t="n">
+        <v>129816</v>
+      </c>
+    </row>
+    <row r="1712">
+      <c r="A1712" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1712" t="n">
+        <v>2671</v>
+      </c>
+      <c r="C1712" t="n">
+        <v>29088</v>
+      </c>
+    </row>
+    <row r="1713">
+      <c r="A1713" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1713" t="n">
+        <v>2568</v>
+      </c>
+      <c r="C1713" t="n">
+        <v>58344</v>
+      </c>
+    </row>
+    <row r="1714">
+      <c r="A1714" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1714" t="n">
+        <v>2146</v>
+      </c>
+      <c r="C1714" t="n">
+        <v>70648</v>
+      </c>
+    </row>
+    <row r="1715">
+      <c r="A1715" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1715" t="n">
+        <v>2753</v>
+      </c>
+      <c r="C1715" t="n">
+        <v>27272</v>
+      </c>
+    </row>
+    <row r="1716">
+      <c r="A1716" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1716" t="n">
+        <v>744</v>
+      </c>
+      <c r="C1716" t="n">
+        <v>15128</v>
+      </c>
+    </row>
+    <row r="1717">
+      <c r="A1717" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1717" t="n">
+        <v>2323</v>
+      </c>
+      <c r="C1717" t="n">
+        <v>24976</v>
+      </c>
+    </row>
+    <row r="1718">
+      <c r="A1718" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1718" t="n">
+        <v>2310</v>
+      </c>
+      <c r="C1718" t="n">
+        <v>24976</v>
+      </c>
+    </row>
+    <row r="1719">
+      <c r="A1719" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1719" t="n">
+        <v>2145</v>
+      </c>
+      <c r="C1719" t="n">
+        <v>36360</v>
+      </c>
+    </row>
+    <row r="1720">
+      <c r="A1720" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1720" t="n">
+        <v>2501</v>
+      </c>
+      <c r="C1720" t="n">
+        <v>29632</v>
+      </c>
+    </row>
+    <row r="1721">
+      <c r="A1721" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1721" t="n">
+        <v>2546</v>
+      </c>
+      <c r="C1721" t="n">
+        <v>14216</v>
+      </c>
+    </row>
+    <row r="1722">
+      <c r="A1722" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1722" t="n">
+        <v>716</v>
+      </c>
+      <c r="C1722" t="n">
+        <v>46608</v>
+      </c>
+    </row>
+    <row r="1723">
+      <c r="A1723" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1723" t="n">
+        <v>2758</v>
+      </c>
+      <c r="C1723" t="n">
+        <v>21816</v>
+      </c>
+    </row>
+    <row r="1724">
+      <c r="A1724" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1724" t="n">
+        <v>400</v>
+      </c>
+      <c r="C1724" t="n">
+        <v>65448</v>
+      </c>
+    </row>
+    <row r="1725">
+      <c r="A1725" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1725" t="n">
+        <v>1259</v>
+      </c>
+      <c r="C1725" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="1726">
+      <c r="A1726" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1726" t="n">
+        <v>571</v>
+      </c>
+      <c r="C1726" t="n">
+        <v>340000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:01:24
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -15557,10 +15557,10 @@
         <v>46296</v>
       </c>
       <c r="B1375" t="n">
-        <v>2245</v>
+        <v>2693</v>
       </c>
       <c r="C1375" t="n">
-        <v>80512</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1376">
@@ -15568,10 +15568,10 @@
         <v>46296</v>
       </c>
       <c r="B1376" t="n">
-        <v>2251</v>
+        <v>2245</v>
       </c>
       <c r="C1376" t="n">
-        <v>72720</v>
+        <v>90576</v>
       </c>
     </row>
     <row r="1377">
@@ -15579,10 +15579,10 @@
         <v>46296</v>
       </c>
       <c r="B1377" t="n">
-        <v>2142</v>
+        <v>2251</v>
       </c>
       <c r="C1377" t="n">
-        <v>19680</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1378">
@@ -15593,7 +15593,7 @@
         <v>664</v>
       </c>
       <c r="C1378" t="n">
-        <v>95272</v>
+        <v>107181</v>
       </c>
     </row>
     <row r="1379">
@@ -15604,7 +15604,7 @@
         <v>2472</v>
       </c>
       <c r="C1379" t="n">
-        <v>19248</v>
+        <v>21654</v>
       </c>
     </row>
     <row r="1380">
@@ -15615,7 +15615,7 @@
         <v>1456</v>
       </c>
       <c r="C1380" t="n">
-        <v>290176</v>
+        <v>326448</v>
       </c>
     </row>
     <row r="1381">
@@ -15626,7 +15626,7 @@
         <v>1585</v>
       </c>
       <c r="C1381" t="n">
-        <v>65816</v>
+        <v>74043</v>
       </c>
     </row>
     <row r="1382">
@@ -15637,7 +15637,7 @@
         <v>1907</v>
       </c>
       <c r="C1382" t="n">
-        <v>200192</v>
+        <v>225216</v>
       </c>
     </row>
     <row r="1383">
@@ -15648,7 +15648,7 @@
         <v>2659</v>
       </c>
       <c r="C1383" t="n">
-        <v>44728</v>
+        <v>50319</v>
       </c>
     </row>
     <row r="1384">
@@ -15659,7 +15659,7 @@
         <v>2583</v>
       </c>
       <c r="C1384" t="n">
-        <v>15128</v>
+        <v>17019</v>
       </c>
     </row>
     <row r="1385">
@@ -15670,7 +15670,7 @@
         <v>2692</v>
       </c>
       <c r="C1385" t="n">
-        <v>25454.66</v>
+        <v>28636.47</v>
       </c>
     </row>
     <row r="1386">
@@ -15681,7 +15681,7 @@
         <v>2691</v>
       </c>
       <c r="C1386" t="n">
-        <v>44430.66</v>
+        <v>49984.47</v>
       </c>
     </row>
     <row r="1387">
@@ -15692,7 +15692,7 @@
         <v>931</v>
       </c>
       <c r="C1387" t="n">
-        <v>34808</v>
+        <v>39159</v>
       </c>
     </row>
     <row r="1388">
@@ -15703,7 +15703,7 @@
         <v>2785</v>
       </c>
       <c r="C1388" t="n">
-        <v>15128</v>
+        <v>17019</v>
       </c>
     </row>
     <row r="1389">
@@ -15714,7 +15714,7 @@
         <v>2411</v>
       </c>
       <c r="C1389" t="n">
-        <v>36360</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1390">
@@ -15725,7 +15725,7 @@
         <v>2716</v>
       </c>
       <c r="C1390" t="n">
-        <v>31904</v>
+        <v>35892</v>
       </c>
     </row>
     <row r="1391">
@@ -15736,7 +15736,7 @@
         <v>2809</v>
       </c>
       <c r="C1391" t="n">
-        <v>24976</v>
+        <v>28098</v>
       </c>
     </row>
     <row r="1392">
@@ -15747,7 +15747,7 @@
         <v>104</v>
       </c>
       <c r="C1392" t="n">
-        <v>109088</v>
+        <v>122724</v>
       </c>
     </row>
     <row r="1393">
@@ -15758,7 +15758,7 @@
         <v>781</v>
       </c>
       <c r="C1393" t="n">
-        <v>47272</v>
+        <v>53181</v>
       </c>
     </row>
     <row r="1394">
@@ -15769,7 +15769,7 @@
         <v>2494</v>
       </c>
       <c r="C1394" t="n">
-        <v>54544</v>
+        <v>61362</v>
       </c>
     </row>
     <row r="1395">
@@ -15780,7 +15780,7 @@
         <v>2652</v>
       </c>
       <c r="C1395" t="n">
-        <v>50904</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1396">
@@ -15791,7 +15791,7 @@
         <v>1384</v>
       </c>
       <c r="C1396" t="n">
-        <v>127272</v>
+        <v>143181</v>
       </c>
     </row>
     <row r="1397">
@@ -15802,7 +15802,7 @@
         <v>360</v>
       </c>
       <c r="C1397" t="n">
-        <v>181816</v>
+        <v>204543</v>
       </c>
     </row>
     <row r="1398">
@@ -15813,7 +15813,7 @@
         <v>2767</v>
       </c>
       <c r="C1398" t="n">
-        <v>69088</v>
+        <v>77724</v>
       </c>
     </row>
     <row r="1399">
@@ -15824,7 +15824,7 @@
         <v>2178</v>
       </c>
       <c r="C1399" t="n">
-        <v>99632</v>
+        <v>112086</v>
       </c>
     </row>
     <row r="1400">
@@ -15835,7 +15835,7 @@
         <v>2107</v>
       </c>
       <c r="C1400" t="n">
-        <v>109080</v>
+        <v>122715</v>
       </c>
     </row>
     <row r="1401">
@@ -15846,7 +15846,7 @@
         <v>2711</v>
       </c>
       <c r="C1401" t="n">
-        <v>31480</v>
+        <v>35415</v>
       </c>
     </row>
     <row r="1402">
@@ -15857,7 +15857,7 @@
         <v>2845</v>
       </c>
       <c r="C1402" t="n">
-        <v>18176</v>
+        <v>20448</v>
       </c>
     </row>
     <row r="1403">
@@ -15868,7 +15868,7 @@
         <v>1102</v>
       </c>
       <c r="C1403" t="n">
-        <v>85496</v>
+        <v>96183</v>
       </c>
     </row>
     <row r="1404">
@@ -15879,7 +15879,7 @@
         <v>353</v>
       </c>
       <c r="C1404" t="n">
-        <v>106376</v>
+        <v>119673</v>
       </c>
     </row>
     <row r="1405">
@@ -15890,7 +15890,7 @@
         <v>2250</v>
       </c>
       <c r="C1405" t="n">
-        <v>123632</v>
+        <v>139086</v>
       </c>
     </row>
     <row r="1406">
@@ -15901,7 +15901,7 @@
         <v>1800</v>
       </c>
       <c r="C1406" t="n">
-        <v>10312</v>
+        <v>11601</v>
       </c>
     </row>
     <row r="1407">
@@ -15912,7 +15912,7 @@
         <v>2555</v>
       </c>
       <c r="C1407" t="n">
-        <v>14216</v>
+        <v>15993</v>
       </c>
     </row>
     <row r="1408">
@@ -15923,7 +15923,7 @@
         <v>2558</v>
       </c>
       <c r="C1408" t="n">
-        <v>14216</v>
+        <v>15993</v>
       </c>
     </row>
     <row r="1409">
@@ -15934,7 +15934,7 @@
         <v>2721</v>
       </c>
       <c r="C1409" t="n">
-        <v>29632</v>
+        <v>33336</v>
       </c>
     </row>
     <row r="1410">
@@ -15945,7 +15945,7 @@
         <v>2556</v>
       </c>
       <c r="C1410" t="n">
-        <v>14216</v>
+        <v>15993</v>
       </c>
     </row>
     <row r="1411">
@@ -15956,7 +15956,7 @@
         <v>2826</v>
       </c>
       <c r="C1411" t="n">
-        <v>25448</v>
+        <v>28629</v>
       </c>
     </row>
     <row r="1412">
@@ -15967,7 +15967,7 @@
         <v>2346</v>
       </c>
       <c r="C1412" t="n">
-        <v>25448</v>
+        <v>28629</v>
       </c>
     </row>
     <row r="1413">
@@ -15978,7 +15978,7 @@
         <v>595</v>
       </c>
       <c r="C1413" t="n">
-        <v>90904</v>
+        <v>102267</v>
       </c>
     </row>
     <row r="1414">
@@ -15989,7 +15989,7 @@
         <v>1278</v>
       </c>
       <c r="C1414" t="n">
-        <v>63632</v>
+        <v>71586</v>
       </c>
     </row>
     <row r="1415">
@@ -16000,7 +16000,7 @@
         <v>2686</v>
       </c>
       <c r="C1415" t="n">
-        <v>50904</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1416">
@@ -16011,7 +16011,7 @@
         <v>1344</v>
       </c>
       <c r="C1416" t="n">
-        <v>54544</v>
+        <v>61362</v>
       </c>
     </row>
     <row r="1417">
@@ -16022,7 +16022,7 @@
         <v>2566</v>
       </c>
       <c r="C1417" t="n">
-        <v>29088</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1418">
@@ -16033,7 +16033,7 @@
         <v>2684</v>
       </c>
       <c r="C1418" t="n">
-        <v>34544</v>
+        <v>38862</v>
       </c>
     </row>
     <row r="1419">
@@ -16044,7 +16044,7 @@
         <v>2375</v>
       </c>
       <c r="C1419" t="n">
-        <v>120000</v>
+        <v>135000</v>
       </c>
     </row>
     <row r="1420">
@@ -16055,7 +16055,7 @@
         <v>2362</v>
       </c>
       <c r="C1420" t="n">
-        <v>27272</v>
+        <v>30681</v>
       </c>
     </row>
     <row r="1421">
@@ -16066,7 +16066,7 @@
         <v>2449</v>
       </c>
       <c r="C1421" t="n">
-        <v>34544</v>
+        <v>38862</v>
       </c>
     </row>
     <row r="1422">
@@ -16077,7 +16077,7 @@
         <v>2844</v>
       </c>
       <c r="C1422" t="n">
-        <v>18176</v>
+        <v>20448</v>
       </c>
     </row>
     <row r="1423">
@@ -16088,7 +16088,7 @@
         <v>2507</v>
       </c>
       <c r="C1423" t="n">
-        <v>32480</v>
+        <v>36540</v>
       </c>
     </row>
     <row r="1424">
@@ -16099,7 +16099,7 @@
         <v>1906</v>
       </c>
       <c r="C1424" t="n">
-        <v>39480</v>
+        <v>44415</v>
       </c>
     </row>
     <row r="1425">
@@ -16110,7 +16110,7 @@
         <v>525</v>
       </c>
       <c r="C1425" t="n">
-        <v>85448</v>
+        <v>96129</v>
       </c>
     </row>
     <row r="1426">
@@ -16121,7 +16121,7 @@
         <v>1261</v>
       </c>
       <c r="C1426" t="n">
-        <v>25818.22</v>
+        <v>29045.49</v>
       </c>
     </row>
     <row r="1427">
@@ -16132,7 +16132,7 @@
         <v>2755</v>
       </c>
       <c r="C1427" t="n">
-        <v>18181.92</v>
+        <v>20454.64</v>
       </c>
     </row>
     <row r="1428">
@@ -16143,7 +16143,7 @@
         <v>1064</v>
       </c>
       <c r="C1428" t="n">
-        <v>218176</v>
+        <v>245448</v>
       </c>
     </row>
     <row r="1429">
@@ -16154,7 +16154,7 @@
         <v>1810</v>
       </c>
       <c r="C1429" t="n">
-        <v>14768</v>
+        <v>16614</v>
       </c>
     </row>
     <row r="1430">
@@ -16165,7 +16165,7 @@
         <v>1937</v>
       </c>
       <c r="C1430" t="n">
-        <v>94176</v>
+        <v>105948</v>
       </c>
     </row>
     <row r="1431">
@@ -16176,7 +16176,7 @@
         <v>483</v>
       </c>
       <c r="C1431" t="n">
-        <v>164360</v>
+        <v>184905</v>
       </c>
     </row>
     <row r="1432">
@@ -16187,7 +16187,7 @@
         <v>2580</v>
       </c>
       <c r="C1432" t="n">
-        <v>12248</v>
+        <v>13779</v>
       </c>
     </row>
     <row r="1433">
@@ -16198,7 +16198,7 @@
         <v>2706</v>
       </c>
       <c r="C1433" t="n">
-        <v>9568</v>
+        <v>10764</v>
       </c>
     </row>
     <row r="1434">
@@ -16209,7 +16209,7 @@
         <v>2633</v>
       </c>
       <c r="C1434" t="n">
-        <v>7008</v>
+        <v>7884</v>
       </c>
     </row>
     <row r="1435">
@@ -16220,7 +16220,7 @@
         <v>2392</v>
       </c>
       <c r="C1435" t="n">
-        <v>75424</v>
+        <v>84852</v>
       </c>
     </row>
     <row r="1436">
@@ -16231,7 +16231,7 @@
         <v>2613</v>
       </c>
       <c r="C1436" t="n">
-        <v>53104</v>
+        <v>59742</v>
       </c>
     </row>
     <row r="1437">
@@ -16242,7 +16242,7 @@
         <v>2183</v>
       </c>
       <c r="C1437" t="n">
-        <v>191208</v>
+        <v>215109</v>
       </c>
     </row>
     <row r="1438">
@@ -16253,7 +16253,7 @@
         <v>2541</v>
       </c>
       <c r="C1438" t="n">
-        <v>85960</v>
+        <v>96705</v>
       </c>
     </row>
     <row r="1439">
@@ -16264,7 +16264,7 @@
         <v>2333</v>
       </c>
       <c r="C1439" t="n">
-        <v>58032</v>
+        <v>65286</v>
       </c>
     </row>
     <row r="1440">
@@ -16275,7 +16275,7 @@
         <v>2813</v>
       </c>
       <c r="C1440" t="n">
-        <v>23200</v>
+        <v>26100</v>
       </c>
     </row>
     <row r="1441">
@@ -16286,7 +16286,7 @@
         <v>2811</v>
       </c>
       <c r="C1441" t="n">
-        <v>15128</v>
+        <v>17019</v>
       </c>
     </row>
     <row r="1442">
@@ -16297,7 +16297,7 @@
         <v>1881</v>
       </c>
       <c r="C1442" t="n">
-        <v>24976</v>
+        <v>28098</v>
       </c>
     </row>
     <row r="1443">
@@ -16308,7 +16308,7 @@
         <v>2825</v>
       </c>
       <c r="C1443" t="n">
-        <v>20304</v>
+        <v>22842</v>
       </c>
     </row>
     <row r="1444">
@@ -16319,7 +16319,7 @@
         <v>970</v>
       </c>
       <c r="C1444" t="n">
-        <v>24976</v>
+        <v>28098</v>
       </c>
     </row>
     <row r="1445">
@@ -16330,7 +16330,7 @@
         <v>2552</v>
       </c>
       <c r="C1445" t="n">
-        <v>14216</v>
+        <v>15993</v>
       </c>
     </row>
     <row r="1446">
@@ -16341,7 +16341,7 @@
         <v>2562</v>
       </c>
       <c r="C1446" t="n">
-        <v>14216</v>
+        <v>15993</v>
       </c>
     </row>
     <row r="1447">
@@ -16352,7 +16352,7 @@
         <v>2761</v>
       </c>
       <c r="C1447" t="n">
-        <v>29632</v>
+        <v>33336</v>
       </c>
     </row>
     <row r="1448">
@@ -16363,7 +16363,7 @@
         <v>2747</v>
       </c>
       <c r="C1448" t="n">
-        <v>25448</v>
+        <v>28629</v>
       </c>
     </row>
     <row r="1449">
@@ -16374,7 +16374,7 @@
         <v>415</v>
       </c>
       <c r="C1449" t="n">
-        <v>90904</v>
+        <v>102267</v>
       </c>
     </row>
     <row r="1450">
@@ -16385,7 +16385,7 @@
         <v>2544</v>
       </c>
       <c r="C1450" t="n">
-        <v>25448</v>
+        <v>28629</v>
       </c>
     </row>
     <row r="1451">
@@ -16396,7 +16396,7 @@
         <v>816</v>
       </c>
       <c r="C1451" t="n">
-        <v>109088</v>
+        <v>122724</v>
       </c>
     </row>
     <row r="1452">
@@ -16407,7 +16407,7 @@
         <v>890</v>
       </c>
       <c r="C1452" t="n">
-        <v>327272</v>
+        <v>368181</v>
       </c>
     </row>
     <row r="1453">
@@ -16418,7 +16418,7 @@
         <v>1298</v>
       </c>
       <c r="C1453" t="n">
-        <v>460000</v>
+        <v>517500</v>
       </c>
     </row>
     <row r="1454">
@@ -16429,7 +16429,7 @@
         <v>1372</v>
       </c>
       <c r="C1454" t="n">
-        <v>109088</v>
+        <v>122724</v>
       </c>
     </row>
     <row r="1455">
@@ -16440,7 +16440,7 @@
         <v>358</v>
       </c>
       <c r="C1455" t="n">
-        <v>114544</v>
+        <v>128862</v>
       </c>
     </row>
     <row r="1456">
@@ -16451,7 +16451,7 @@
         <v>1653</v>
       </c>
       <c r="C1456" t="n">
-        <v>114544</v>
+        <v>128862</v>
       </c>
     </row>
     <row r="1457">
@@ -16462,7 +16462,7 @@
         <v>675</v>
       </c>
       <c r="C1457" t="n">
-        <v>72720</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1458">
@@ -16473,7 +16473,7 @@
         <v>2804</v>
       </c>
       <c r="C1458" t="n">
-        <v>36360</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1459">
@@ -16484,7 +16484,7 @@
         <v>2714</v>
       </c>
       <c r="C1459" t="n">
-        <v>130904</v>
+        <v>147267</v>
       </c>
     </row>
     <row r="1460">
@@ -16495,7 +16495,7 @@
         <v>2765</v>
       </c>
       <c r="C1460" t="n">
-        <v>32720</v>
+        <v>36810</v>
       </c>
     </row>
     <row r="1461">
@@ -16506,7 +16506,7 @@
         <v>2421</v>
       </c>
       <c r="C1461" t="n">
-        <v>22176</v>
+        <v>24948</v>
       </c>
     </row>
     <row r="1462">
@@ -16517,7 +16517,7 @@
         <v>2359</v>
       </c>
       <c r="C1462" t="n">
-        <v>37936</v>
+        <v>42678</v>
       </c>
     </row>
     <row r="1463">
@@ -16528,7 +16528,7 @@
         <v>2678</v>
       </c>
       <c r="C1463" t="n">
-        <v>35984</v>
+        <v>40482</v>
       </c>
     </row>
     <row r="1464">
@@ -16539,7 +16539,7 @@
         <v>2697</v>
       </c>
       <c r="C1464" t="n">
-        <v>54608</v>
+        <v>61434</v>
       </c>
     </row>
     <row r="1465">
@@ -16547,10 +16547,10 @@
         <v>46296</v>
       </c>
       <c r="B1465" t="n">
-        <v>2498</v>
+        <v>2142</v>
       </c>
       <c r="C1465" t="n">
-        <v>20472</v>
+        <v>22140</v>
       </c>
     </row>
     <row r="1466">
@@ -16558,10 +16558,10 @@
         <v>46296</v>
       </c>
       <c r="B1466" t="n">
-        <v>2641</v>
+        <v>2498</v>
       </c>
       <c r="C1466" t="n">
-        <v>54544</v>
+        <v>23031</v>
       </c>
     </row>
     <row r="1467">
@@ -16569,10 +16569,10 @@
         <v>46296</v>
       </c>
       <c r="B1467" t="n">
-        <v>2801</v>
+        <v>2641</v>
       </c>
       <c r="C1467" t="n">
-        <v>36360</v>
+        <v>61362</v>
       </c>
     </row>
     <row r="1468">
@@ -16580,10 +16580,10 @@
         <v>46296</v>
       </c>
       <c r="B1468" t="n">
-        <v>2810</v>
+        <v>2801</v>
       </c>
       <c r="C1468" t="n">
-        <v>58176</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1469">
@@ -16591,10 +16591,10 @@
         <v>46296</v>
       </c>
       <c r="B1469" t="n">
-        <v>2109</v>
+        <v>2810</v>
       </c>
       <c r="C1469" t="n">
-        <v>0</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1470">
@@ -16602,7 +16602,7 @@
         <v>46296</v>
       </c>
       <c r="B1470" t="n">
-        <v>2693</v>
+        <v>2109</v>
       </c>
       <c r="C1470" t="n">
         <v>0</v>
@@ -16616,7 +16616,7 @@
         <v>1142</v>
       </c>
       <c r="C1471" t="n">
-        <v>166576</v>
+        <v>187398</v>
       </c>
     </row>
     <row r="1472">
@@ -16627,7 +16627,7 @@
         <v>2082</v>
       </c>
       <c r="C1472" t="n">
-        <v>36360</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1473">
@@ -16638,7 +16638,7 @@
         <v>2276</v>
       </c>
       <c r="C1473" t="n">
-        <v>72336</v>
+        <v>81378</v>
       </c>
     </row>
     <row r="1474">
@@ -16649,7 +16649,7 @@
         <v>2786</v>
       </c>
       <c r="C1474" t="n">
-        <v>25448</v>
+        <v>28629</v>
       </c>
     </row>
     <row r="1475">
@@ -16660,7 +16660,7 @@
         <v>2816</v>
       </c>
       <c r="C1475" t="n">
-        <v>47272</v>
+        <v>53181</v>
       </c>
     </row>
     <row r="1476">
@@ -16671,7 +16671,7 @@
         <v>1871</v>
       </c>
       <c r="C1476" t="n">
-        <v>52184</v>
+        <v>58707</v>
       </c>
     </row>
     <row r="1477">
@@ -16682,7 +16682,7 @@
         <v>2345</v>
       </c>
       <c r="C1477" t="n">
-        <v>23200</v>
+        <v>26100</v>
       </c>
     </row>
     <row r="1478">
@@ -16693,7 +16693,7 @@
         <v>2802</v>
       </c>
       <c r="C1478" t="n">
-        <v>26104</v>
+        <v>29367</v>
       </c>
     </row>
     <row r="1479">
@@ -16704,7 +16704,7 @@
         <v>2090</v>
       </c>
       <c r="C1479" t="n">
-        <v>15128</v>
+        <v>17019</v>
       </c>
     </row>
     <row r="1480">
@@ -16715,7 +16715,7 @@
         <v>2647</v>
       </c>
       <c r="C1480" t="n">
-        <v>51000</v>
+        <v>57375</v>
       </c>
     </row>
     <row r="1481">
@@ -16726,7 +16726,7 @@
         <v>2365</v>
       </c>
       <c r="C1481" t="n">
-        <v>36360</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1482">
@@ -16737,7 +16737,7 @@
         <v>766</v>
       </c>
       <c r="C1482" t="n">
-        <v>24976</v>
+        <v>28098</v>
       </c>
     </row>
     <row r="1483">
@@ -16748,7 +16748,7 @@
         <v>2702</v>
       </c>
       <c r="C1483" t="n">
-        <v>29632</v>
+        <v>33336</v>
       </c>
     </row>
     <row r="1484">
@@ -16759,7 +16759,7 @@
         <v>20</v>
       </c>
       <c r="C1484" t="n">
-        <v>163632</v>
+        <v>184086</v>
       </c>
     </row>
     <row r="1485">
@@ -16770,7 +16770,7 @@
         <v>27</v>
       </c>
       <c r="C1485" t="n">
-        <v>54544</v>
+        <v>61362</v>
       </c>
     </row>
     <row r="1486">
@@ -16781,7 +16781,7 @@
         <v>33</v>
       </c>
       <c r="C1486" t="n">
-        <v>144720</v>
+        <v>162810</v>
       </c>
     </row>
     <row r="1487">
@@ -16803,7 +16803,7 @@
         <v>2561</v>
       </c>
       <c r="C1488" t="n">
-        <v>14216</v>
+        <v>15993</v>
       </c>
     </row>
     <row r="1489">
@@ -16814,7 +16814,7 @@
         <v>2772</v>
       </c>
       <c r="C1489" t="n">
-        <v>21816</v>
+        <v>24543</v>
       </c>
     </row>
     <row r="1490">
@@ -16825,7 +16825,7 @@
         <v>132</v>
       </c>
       <c r="C1490" t="n">
-        <v>127272</v>
+        <v>143181</v>
       </c>
     </row>
     <row r="1491">
@@ -16836,7 +16836,7 @@
         <v>580</v>
       </c>
       <c r="C1491" t="n">
-        <v>63632</v>
+        <v>71586</v>
       </c>
     </row>
     <row r="1492">
@@ -16847,7 +16847,7 @@
         <v>634</v>
       </c>
       <c r="C1492" t="n">
-        <v>181816</v>
+        <v>204543</v>
       </c>
     </row>
     <row r="1493">
@@ -16858,7 +16858,7 @@
         <v>1277</v>
       </c>
       <c r="C1493" t="n">
-        <v>80000</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="1494">
@@ -16869,7 +16869,7 @@
         <v>767</v>
       </c>
       <c r="C1494" t="n">
-        <v>72720</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1495">
@@ -16880,7 +16880,7 @@
         <v>2727</v>
       </c>
       <c r="C1495" t="n">
-        <v>14720</v>
+        <v>16560</v>
       </c>
     </row>
     <row r="1496">
@@ -16891,7 +16891,7 @@
         <v>2846</v>
       </c>
       <c r="C1496" t="n">
-        <v>94544</v>
+        <v>106362</v>
       </c>
     </row>
     <row r="1497">
@@ -16902,7 +16902,7 @@
         <v>609</v>
       </c>
       <c r="C1497" t="n">
-        <v>81816</v>
+        <v>92043</v>
       </c>
     </row>
     <row r="1498">
@@ -16913,7 +16913,7 @@
         <v>2726</v>
       </c>
       <c r="C1498" t="n">
-        <v>56360</v>
+        <v>63405</v>
       </c>
     </row>
     <row r="1499">
@@ -16924,7 +16924,7 @@
         <v>2729</v>
       </c>
       <c r="C1499" t="n">
-        <v>32720</v>
+        <v>36810</v>
       </c>
     </row>
     <row r="1500">
@@ -16935,7 +16935,7 @@
         <v>1340</v>
       </c>
       <c r="C1500" t="n">
-        <v>54544</v>
+        <v>61362</v>
       </c>
     </row>
     <row r="1501">
@@ -16946,7 +16946,7 @@
         <v>2830</v>
       </c>
       <c r="C1501" t="n">
-        <v>32720</v>
+        <v>36810</v>
       </c>
     </row>
     <row r="1502">
@@ -16957,7 +16957,7 @@
         <v>2674</v>
       </c>
       <c r="C1502" t="n">
-        <v>94544</v>
+        <v>106362</v>
       </c>
     </row>
     <row r="1503">
@@ -16968,7 +16968,7 @@
         <v>2308</v>
       </c>
       <c r="C1503" t="n">
-        <v>72720</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1504">
@@ -16979,7 +16979,7 @@
         <v>2601</v>
       </c>
       <c r="C1504" t="n">
-        <v>100000</v>
+        <v>112500</v>
       </c>
     </row>
     <row r="1505">
@@ -16990,7 +16990,7 @@
         <v>2190</v>
       </c>
       <c r="C1505" t="n">
-        <v>76360</v>
+        <v>85905</v>
       </c>
     </row>
     <row r="1506">
@@ -17001,7 +17001,7 @@
         <v>2015</v>
       </c>
       <c r="C1506" t="n">
-        <v>134544</v>
+        <v>151362</v>
       </c>
     </row>
     <row r="1507">
@@ -17012,7 +17012,7 @@
         <v>1308</v>
       </c>
       <c r="C1507" t="n">
-        <v>57088</v>
+        <v>64224</v>
       </c>
     </row>
     <row r="1508">
@@ -17023,7 +17023,7 @@
         <v>2118</v>
       </c>
       <c r="C1508" t="n">
-        <v>76424</v>
+        <v>85977</v>
       </c>
     </row>
     <row r="1509">
@@ -17034,7 +17034,7 @@
         <v>2607</v>
       </c>
       <c r="C1509" t="n">
-        <v>18064</v>
+        <v>20322</v>
       </c>
     </row>
     <row r="1510">
@@ -17045,7 +17045,7 @@
         <v>2707</v>
       </c>
       <c r="C1510" t="n">
-        <v>15704</v>
+        <v>17667</v>
       </c>
     </row>
     <row r="1511">
@@ -17056,7 +17056,7 @@
         <v>2383</v>
       </c>
       <c r="C1511" t="n">
-        <v>48336</v>
+        <v>54378</v>
       </c>
     </row>
     <row r="1512">
@@ -17067,7 +17067,7 @@
         <v>2821</v>
       </c>
       <c r="C1512" t="n">
-        <v>48488</v>
+        <v>54549</v>
       </c>
     </row>
     <row r="1513">
@@ -17078,7 +17078,7 @@
         <v>569</v>
       </c>
       <c r="C1513" t="n">
-        <v>1055792</v>
+        <v>1187766</v>
       </c>
     </row>
     <row r="1514">
@@ -17089,7 +17089,7 @@
         <v>2660</v>
       </c>
       <c r="C1514" t="n">
-        <v>127272</v>
+        <v>143181</v>
       </c>
     </row>
     <row r="1515">
@@ -17100,7 +17100,7 @@
         <v>1632</v>
       </c>
       <c r="C1515" t="n">
-        <v>94544</v>
+        <v>106362</v>
       </c>
     </row>
     <row r="1516">
@@ -17111,7 +17111,7 @@
         <v>1756</v>
       </c>
       <c r="C1516" t="n">
-        <v>152720</v>
+        <v>171810</v>
       </c>
     </row>
     <row r="1517">
@@ -17122,7 +17122,7 @@
         <v>58</v>
       </c>
       <c r="C1517" t="n">
-        <v>91200</v>
+        <v>102600</v>
       </c>
     </row>
     <row r="1518">
@@ -17133,7 +17133,7 @@
         <v>40</v>
       </c>
       <c r="C1518" t="n">
-        <v>81120</v>
+        <v>91260</v>
       </c>
     </row>
     <row r="1519">
@@ -17144,7 +17144,7 @@
         <v>559</v>
       </c>
       <c r="C1519" t="n">
-        <v>85088</v>
+        <v>95724</v>
       </c>
     </row>
     <row r="1520">
@@ -17155,7 +17155,7 @@
         <v>2773</v>
       </c>
       <c r="C1520" t="n">
-        <v>29336</v>
+        <v>33003</v>
       </c>
     </row>
     <row r="1521">
@@ -17166,7 +17166,7 @@
         <v>2631</v>
       </c>
       <c r="C1521" t="n">
-        <v>14088</v>
+        <v>15849</v>
       </c>
     </row>
     <row r="1522">
@@ -17177,7 +17177,7 @@
         <v>2085</v>
       </c>
       <c r="C1522" t="n">
-        <v>36360</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1523">
@@ -17188,7 +17188,7 @@
         <v>1642</v>
       </c>
       <c r="C1523" t="n">
-        <v>96360</v>
+        <v>108405</v>
       </c>
     </row>
     <row r="1524">
@@ -17199,7 +17199,7 @@
         <v>2621</v>
       </c>
       <c r="C1524" t="n">
-        <v>25448</v>
+        <v>28629</v>
       </c>
     </row>
     <row r="1525">
@@ -17210,7 +17210,7 @@
         <v>2705</v>
       </c>
       <c r="C1525" t="n">
-        <v>73008</v>
+        <v>82134</v>
       </c>
     </row>
     <row r="1526">
@@ -17221,7 +17221,7 @@
         <v>2735</v>
       </c>
       <c r="C1526" t="n">
-        <v>43632</v>
+        <v>49086</v>
       </c>
     </row>
     <row r="1527">
@@ -17232,7 +17232,7 @@
         <v>945</v>
       </c>
       <c r="C1527" t="n">
-        <v>127520</v>
+        <v>143460</v>
       </c>
     </row>
     <row r="1528">
@@ -17243,7 +17243,7 @@
         <v>2582</v>
       </c>
       <c r="C1528" t="n">
-        <v>31904</v>
+        <v>35892</v>
       </c>
     </row>
     <row r="1529">
@@ -17254,7 +17254,7 @@
         <v>2584</v>
       </c>
       <c r="C1529" t="n">
-        <v>23200</v>
+        <v>26100</v>
       </c>
     </row>
     <row r="1530">
@@ -17265,7 +17265,7 @@
         <v>2689</v>
       </c>
       <c r="C1530" t="n">
-        <v>23200</v>
+        <v>26100</v>
       </c>
     </row>
     <row r="1531">
@@ -17276,7 +17276,7 @@
         <v>2574</v>
       </c>
       <c r="C1531" t="n">
-        <v>50992</v>
+        <v>57366</v>
       </c>
     </row>
     <row r="1532">
@@ -17287,7 +17287,7 @@
         <v>1834</v>
       </c>
       <c r="C1532" t="n">
-        <v>42800</v>
+        <v>48150</v>
       </c>
     </row>
     <row r="1533">
@@ -17298,7 +17298,7 @@
         <v>2629</v>
       </c>
       <c r="C1533" t="n">
-        <v>24976</v>
+        <v>28098</v>
       </c>
     </row>
     <row r="1534">
@@ -17309,7 +17309,7 @@
         <v>933</v>
       </c>
       <c r="C1534" t="n">
-        <v>29632</v>
+        <v>33336</v>
       </c>
     </row>
     <row r="1535">
@@ -17320,7 +17320,7 @@
         <v>1499</v>
       </c>
       <c r="C1535" t="n">
-        <v>32720</v>
+        <v>36810</v>
       </c>
     </row>
     <row r="1536">
@@ -17331,7 +17331,7 @@
         <v>2261</v>
       </c>
       <c r="C1536" t="n">
-        <v>65448</v>
+        <v>73629</v>
       </c>
     </row>
     <row r="1537">
@@ -17342,7 +17342,7 @@
         <v>1324</v>
       </c>
       <c r="C1537" t="n">
-        <v>101816</v>
+        <v>114543</v>
       </c>
     </row>
     <row r="1538">
@@ -17353,7 +17353,7 @@
         <v>2709</v>
       </c>
       <c r="C1538" t="n">
-        <v>65448</v>
+        <v>73629</v>
       </c>
     </row>
     <row r="1539">
@@ -17364,7 +17364,7 @@
         <v>1137</v>
       </c>
       <c r="C1539" t="n">
-        <v>232720</v>
+        <v>261810</v>
       </c>
     </row>
     <row r="1540">
@@ -17375,7 +17375,7 @@
         <v>2440</v>
       </c>
       <c r="C1540" t="n">
-        <v>29088</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1541">
@@ -17386,7 +17386,7 @@
         <v>429</v>
       </c>
       <c r="C1541" t="n">
-        <v>138176</v>
+        <v>155448</v>
       </c>
     </row>
     <row r="1542">
@@ -17397,7 +17397,7 @@
         <v>2114</v>
       </c>
       <c r="C1542" t="n">
-        <v>61864</v>
+        <v>69597</v>
       </c>
     </row>
     <row r="1543">
@@ -17408,7 +17408,7 @@
         <v>2211</v>
       </c>
       <c r="C1543" t="n">
-        <v>87576</v>
+        <v>98523</v>
       </c>
     </row>
     <row r="1544">
@@ -17419,7 +17419,7 @@
         <v>1108</v>
       </c>
       <c r="C1544" t="n">
-        <v>111408</v>
+        <v>125334</v>
       </c>
     </row>
     <row r="1545">
@@ -17430,7 +17430,7 @@
         <v>2695</v>
       </c>
       <c r="C1545" t="n">
-        <v>17592</v>
+        <v>19791</v>
       </c>
     </row>
     <row r="1546">
@@ -17441,7 +17441,7 @@
         <v>1289</v>
       </c>
       <c r="C1546" t="n">
-        <v>100000</v>
+        <v>112500</v>
       </c>
     </row>
     <row r="1547">
@@ -17452,7 +17452,7 @@
         <v>2789</v>
       </c>
       <c r="C1547" t="n">
-        <v>65448</v>
+        <v>73629</v>
       </c>
     </row>
     <row r="1548">
@@ -17463,7 +17463,7 @@
         <v>2197</v>
       </c>
       <c r="C1548" t="n">
-        <v>78176</v>
+        <v>87948</v>
       </c>
     </row>
     <row r="1549">
@@ -17474,7 +17474,7 @@
         <v>947</v>
       </c>
       <c r="C1549" t="n">
-        <v>161264</v>
+        <v>181422</v>
       </c>
     </row>
     <row r="1550">
@@ -17485,7 +17485,7 @@
         <v>2279</v>
       </c>
       <c r="C1550" t="n">
-        <v>89064</v>
+        <v>100197</v>
       </c>
     </row>
     <row r="1551">
@@ -17496,7 +17496,7 @@
         <v>1465</v>
       </c>
       <c r="C1551" t="n">
-        <v>140000</v>
+        <v>157500</v>
       </c>
     </row>
     <row r="1552">
@@ -17507,7 +17507,7 @@
         <v>2651</v>
       </c>
       <c r="C1552" t="n">
-        <v>61816</v>
+        <v>69543</v>
       </c>
     </row>
     <row r="1553">
@@ -17518,7 +17518,7 @@
         <v>42</v>
       </c>
       <c r="C1553" t="n">
-        <v>693088</v>
+        <v>779724</v>
       </c>
     </row>
     <row r="1554">
@@ -17529,7 +17529,7 @@
         <v>949</v>
       </c>
       <c r="C1554" t="n">
-        <v>36168</v>
+        <v>40689</v>
       </c>
     </row>
     <row r="1555">
@@ -17540,7 +17540,7 @@
         <v>2606</v>
       </c>
       <c r="C1555" t="n">
-        <v>93360</v>
+        <v>105030</v>
       </c>
     </row>
     <row r="1556">
@@ -17551,7 +17551,7 @@
         <v>2249</v>
       </c>
       <c r="C1556" t="n">
-        <v>79320</v>
+        <v>89235</v>
       </c>
     </row>
     <row r="1557">
@@ -17562,7 +17562,7 @@
         <v>2045</v>
       </c>
       <c r="C1557" t="n">
-        <v>115808</v>
+        <v>130284</v>
       </c>
     </row>
     <row r="1558">
@@ -17573,7 +17573,7 @@
         <v>2663</v>
       </c>
       <c r="C1558" t="n">
-        <v>100000</v>
+        <v>112500</v>
       </c>
     </row>
     <row r="1559">
@@ -17595,7 +17595,7 @@
         <v>2341</v>
       </c>
       <c r="C1560" t="n">
-        <v>63600</v>
+        <v>71550</v>
       </c>
     </row>
     <row r="1561">
@@ -17606,7 +17606,7 @@
         <v>2637</v>
       </c>
       <c r="C1561" t="n">
-        <v>23200</v>
+        <v>26100</v>
       </c>
     </row>
     <row r="1562">
@@ -17617,7 +17617,7 @@
         <v>2492</v>
       </c>
       <c r="C1562" t="n">
-        <v>36424</v>
+        <v>40977</v>
       </c>
     </row>
     <row r="1563">
@@ -17628,7 +17628,7 @@
         <v>2548</v>
       </c>
       <c r="C1563" t="n">
-        <v>14216</v>
+        <v>15993</v>
       </c>
     </row>
     <row r="1564">
@@ -17639,7 +17639,7 @@
         <v>351</v>
       </c>
       <c r="C1564" t="n">
-        <v>77448</v>
+        <v>87129</v>
       </c>
     </row>
     <row r="1565">
@@ -17650,7 +17650,7 @@
         <v>531</v>
       </c>
       <c r="C1565" t="n">
-        <v>72720</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1566">
@@ -17661,7 +17661,7 @@
         <v>2757</v>
       </c>
       <c r="C1566" t="n">
-        <v>29088</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1567">
@@ -17672,7 +17672,7 @@
         <v>2815</v>
       </c>
       <c r="C1567" t="n">
-        <v>21816</v>
+        <v>24543</v>
       </c>
     </row>
     <row r="1568">
@@ -17683,7 +17683,7 @@
         <v>2829</v>
       </c>
       <c r="C1568" t="n">
-        <v>21816</v>
+        <v>24543</v>
       </c>
     </row>
     <row r="1569">
@@ -17694,7 +17694,7 @@
         <v>768</v>
       </c>
       <c r="C1569" t="n">
-        <v>50904</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1570">
@@ -17705,7 +17705,7 @@
         <v>772</v>
       </c>
       <c r="C1570" t="n">
-        <v>118176</v>
+        <v>132948</v>
       </c>
     </row>
     <row r="1571">
@@ -17716,7 +17716,7 @@
         <v>2496</v>
       </c>
       <c r="C1571" t="n">
-        <v>72720</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1572">
@@ -17727,7 +17727,7 @@
         <v>802</v>
       </c>
       <c r="C1572" t="n">
-        <v>27272</v>
+        <v>30681</v>
       </c>
     </row>
     <row r="1573">
@@ -17738,7 +17738,7 @@
         <v>2131</v>
       </c>
       <c r="C1573" t="n">
-        <v>36360</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1574">
@@ -17749,7 +17749,7 @@
         <v>1381</v>
       </c>
       <c r="C1574" t="n">
-        <v>109088</v>
+        <v>122724</v>
       </c>
     </row>
     <row r="1575">
@@ -17760,7 +17760,7 @@
         <v>2847</v>
       </c>
       <c r="C1575" t="n">
-        <v>49088</v>
+        <v>55224</v>
       </c>
     </row>
     <row r="1576">
@@ -17771,7 +17771,7 @@
         <v>1293</v>
       </c>
       <c r="C1576" t="n">
-        <v>140000</v>
+        <v>157500</v>
       </c>
     </row>
     <row r="1577">
@@ -17782,7 +17782,7 @@
         <v>2363</v>
       </c>
       <c r="C1577" t="n">
-        <v>61816</v>
+        <v>69543</v>
       </c>
     </row>
     <row r="1578">
@@ -17793,7 +17793,7 @@
         <v>631</v>
       </c>
       <c r="C1578" t="n">
-        <v>127272</v>
+        <v>143181</v>
       </c>
     </row>
     <row r="1579">
@@ -17804,7 +17804,7 @@
         <v>2791</v>
       </c>
       <c r="C1579" t="n">
-        <v>37336</v>
+        <v>42003</v>
       </c>
     </row>
     <row r="1580">
@@ -17815,7 +17815,7 @@
         <v>1380</v>
       </c>
       <c r="C1580" t="n">
-        <v>18176</v>
+        <v>20448</v>
       </c>
     </row>
     <row r="1581">
@@ -17826,7 +17826,7 @@
         <v>2841</v>
       </c>
       <c r="C1581" t="n">
-        <v>18176</v>
+        <v>20448</v>
       </c>
     </row>
     <row r="1582">
@@ -17837,7 +17837,7 @@
         <v>2571</v>
       </c>
       <c r="C1582" t="n">
-        <v>96936</v>
+        <v>109053</v>
       </c>
     </row>
     <row r="1583">
@@ -17848,7 +17848,7 @@
         <v>2273</v>
       </c>
       <c r="C1583" t="n">
-        <v>78184</v>
+        <v>87957</v>
       </c>
     </row>
     <row r="1584">
@@ -17859,7 +17859,7 @@
         <v>2381</v>
       </c>
       <c r="C1584" t="n">
-        <v>29240</v>
+        <v>32895</v>
       </c>
     </row>
     <row r="1585">
@@ -17870,7 +17870,7 @@
         <v>630</v>
       </c>
       <c r="C1585" t="n">
-        <v>30008</v>
+        <v>33759</v>
       </c>
     </row>
     <row r="1586">
@@ -17892,7 +17892,7 @@
         <v>1983</v>
       </c>
       <c r="C1587" t="n">
-        <v>199360</v>
+        <v>224280</v>
       </c>
     </row>
     <row r="1588">
@@ -17903,7 +17903,7 @@
         <v>1993</v>
       </c>
       <c r="C1588" t="n">
-        <v>135376</v>
+        <v>152298</v>
       </c>
     </row>
     <row r="1589">
@@ -17914,7 +17914,7 @@
         <v>89</v>
       </c>
       <c r="C1589" t="n">
-        <v>127272</v>
+        <v>143181</v>
       </c>
     </row>
     <row r="1590">
@@ -17925,7 +17925,7 @@
         <v>1063</v>
       </c>
       <c r="C1590" t="n">
-        <v>140000</v>
+        <v>157500</v>
       </c>
     </row>
     <row r="1591">
@@ -17936,7 +17936,7 @@
         <v>1116</v>
       </c>
       <c r="C1591" t="n">
-        <v>90904</v>
+        <v>102267</v>
       </c>
     </row>
     <row r="1592">
@@ -17947,7 +17947,7 @@
         <v>941</v>
       </c>
       <c r="C1592" t="n">
-        <v>109416</v>
+        <v>123093</v>
       </c>
     </row>
     <row r="1593">
@@ -17958,7 +17958,7 @@
         <v>2141</v>
       </c>
       <c r="C1593" t="n">
-        <v>11664</v>
+        <v>13122</v>
       </c>
     </row>
     <row r="1594">
@@ -17969,7 +17969,7 @@
         <v>2463</v>
       </c>
       <c r="C1594" t="n">
-        <v>119936</v>
+        <v>134928</v>
       </c>
     </row>
     <row r="1595">
@@ -17980,7 +17980,7 @@
         <v>2325</v>
       </c>
       <c r="C1595" t="n">
-        <v>41952</v>
+        <v>47196</v>
       </c>
     </row>
     <row r="1596">
@@ -17991,7 +17991,7 @@
         <v>1890</v>
       </c>
       <c r="C1596" t="n">
-        <v>89176</v>
+        <v>100323</v>
       </c>
     </row>
     <row r="1597">
@@ -18002,7 +18002,7 @@
         <v>2639</v>
       </c>
       <c r="C1597" t="n">
-        <v>14568</v>
+        <v>16389</v>
       </c>
     </row>
     <row r="1598">
@@ -18013,7 +18013,7 @@
         <v>2682</v>
       </c>
       <c r="C1598" t="n">
-        <v>50904</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1599">
@@ -18024,7 +18024,7 @@
         <v>703</v>
       </c>
       <c r="C1599" t="n">
-        <v>90904</v>
+        <v>102267</v>
       </c>
     </row>
     <row r="1600">
@@ -18035,7 +18035,7 @@
         <v>2833</v>
       </c>
       <c r="C1600" t="n">
-        <v>29088</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1601">
@@ -18046,7 +18046,7 @@
         <v>1007</v>
       </c>
       <c r="C1601" t="n">
-        <v>72720</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1602">
@@ -18057,7 +18057,7 @@
         <v>2687</v>
       </c>
       <c r="C1602" t="n">
-        <v>29088</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1603">
@@ -18068,7 +18068,7 @@
         <v>2824</v>
       </c>
       <c r="C1603" t="n">
-        <v>41056</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="1604">
@@ -18079,7 +18079,7 @@
         <v>2730</v>
       </c>
       <c r="C1604" t="n">
-        <v>32720</v>
+        <v>36810</v>
       </c>
     </row>
     <row r="1605">
@@ -18090,7 +18090,7 @@
         <v>2718</v>
       </c>
       <c r="C1605" t="n">
-        <v>47272</v>
+        <v>53181</v>
       </c>
     </row>
     <row r="1606">
@@ -18101,7 +18101,7 @@
         <v>2750</v>
       </c>
       <c r="C1606" t="n">
-        <v>10904</v>
+        <v>12267</v>
       </c>
     </row>
     <row r="1607">
@@ -18112,7 +18112,7 @@
         <v>854</v>
       </c>
       <c r="C1607" t="n">
-        <v>50904</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1608">
@@ -18123,7 +18123,7 @@
         <v>2794</v>
       </c>
       <c r="C1608" t="n">
-        <v>43632</v>
+        <v>49086</v>
       </c>
     </row>
     <row r="1609">
@@ -18134,7 +18134,7 @@
         <v>1374</v>
       </c>
       <c r="C1609" t="n">
-        <v>72720</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1610">
@@ -18145,7 +18145,7 @@
         <v>2488</v>
       </c>
       <c r="C1610" t="n">
-        <v>36360</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1611">
@@ -18156,7 +18156,7 @@
         <v>363</v>
       </c>
       <c r="C1611" t="n">
-        <v>109088</v>
+        <v>122724</v>
       </c>
     </row>
     <row r="1612">
@@ -18167,7 +18167,7 @@
         <v>2655</v>
       </c>
       <c r="C1612" t="n">
-        <v>40000</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="1613">
@@ -18178,7 +18178,7 @@
         <v>1873</v>
       </c>
       <c r="C1613" t="n">
-        <v>116360</v>
+        <v>130905</v>
       </c>
     </row>
     <row r="1614">
@@ -18189,7 +18189,7 @@
         <v>2635</v>
       </c>
       <c r="C1614" t="n">
-        <v>47272</v>
+        <v>53181</v>
       </c>
     </row>
     <row r="1615">
@@ -18200,7 +18200,7 @@
         <v>1658</v>
       </c>
       <c r="C1615" t="n">
-        <v>55632</v>
+        <v>62586</v>
       </c>
     </row>
     <row r="1616">
@@ -18211,7 +18211,7 @@
         <v>2069</v>
       </c>
       <c r="C1616" t="n">
-        <v>72720</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1617">
@@ -18222,7 +18222,7 @@
         <v>2081</v>
       </c>
       <c r="C1617" t="n">
-        <v>54544</v>
+        <v>61362</v>
       </c>
     </row>
     <row r="1618">
@@ -18233,7 +18233,7 @@
         <v>2124</v>
       </c>
       <c r="C1618" t="n">
-        <v>127272</v>
+        <v>143181</v>
       </c>
     </row>
     <row r="1619">
@@ -18244,7 +18244,7 @@
         <v>636</v>
       </c>
       <c r="C1619" t="n">
-        <v>90904</v>
+        <v>102267</v>
       </c>
     </row>
     <row r="1620">
@@ -18255,7 +18255,7 @@
         <v>2803</v>
       </c>
       <c r="C1620" t="n">
-        <v>43632</v>
+        <v>49086</v>
       </c>
     </row>
     <row r="1621">
@@ -18266,7 +18266,7 @@
         <v>2163</v>
       </c>
       <c r="C1621" t="n">
-        <v>65448</v>
+        <v>73629</v>
       </c>
     </row>
     <row r="1622">
@@ -18277,7 +18277,7 @@
         <v>1466</v>
       </c>
       <c r="C1622" t="n">
-        <v>147272</v>
+        <v>165681</v>
       </c>
     </row>
     <row r="1623">
@@ -18288,7 +18288,7 @@
         <v>2133</v>
       </c>
       <c r="C1623" t="n">
-        <v>127272</v>
+        <v>143181</v>
       </c>
     </row>
     <row r="1624">
@@ -18299,7 +18299,7 @@
         <v>2431</v>
       </c>
       <c r="C1624" t="n">
-        <v>54544</v>
+        <v>61362</v>
       </c>
     </row>
     <row r="1625">
@@ -18310,7 +18310,7 @@
         <v>535</v>
       </c>
       <c r="C1625" t="n">
-        <v>129520</v>
+        <v>145710</v>
       </c>
     </row>
     <row r="1626">
@@ -18321,7 +18321,7 @@
         <v>2790</v>
       </c>
       <c r="C1626" t="n">
-        <v>22968</v>
+        <v>25839</v>
       </c>
     </row>
     <row r="1627">
@@ -18332,7 +18332,7 @@
         <v>2442</v>
       </c>
       <c r="C1627" t="n">
-        <v>94176</v>
+        <v>105948</v>
       </c>
     </row>
     <row r="1628">
@@ -18343,7 +18343,7 @@
         <v>2376</v>
       </c>
       <c r="C1628" t="n">
-        <v>363632</v>
+        <v>409086</v>
       </c>
     </row>
     <row r="1629">
@@ -18354,7 +18354,7 @@
         <v>2768</v>
       </c>
       <c r="C1629" t="n">
-        <v>110056</v>
+        <v>123813</v>
       </c>
     </row>
     <row r="1630">
@@ -18365,7 +18365,7 @@
         <v>2491</v>
       </c>
       <c r="C1630" t="n">
-        <v>88312</v>
+        <v>99351</v>
       </c>
     </row>
     <row r="1631">
@@ -18376,7 +18376,7 @@
         <v>2799</v>
       </c>
       <c r="C1631" t="n">
-        <v>39752</v>
+        <v>44721</v>
       </c>
     </row>
     <row r="1632">
@@ -18387,7 +18387,7 @@
         <v>1317</v>
       </c>
       <c r="C1632" t="n">
-        <v>114544</v>
+        <v>128862</v>
       </c>
     </row>
     <row r="1633">
@@ -18398,7 +18398,7 @@
         <v>2822</v>
       </c>
       <c r="C1633" t="n">
-        <v>58176</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1634">
@@ -18409,7 +18409,7 @@
         <v>1117</v>
       </c>
       <c r="C1634" t="n">
-        <v>145496</v>
+        <v>163683</v>
       </c>
     </row>
     <row r="1635">
@@ -18420,7 +18420,7 @@
         <v>1299</v>
       </c>
       <c r="C1635" t="n">
-        <v>191832</v>
+        <v>215811</v>
       </c>
     </row>
     <row r="1636">
@@ -18431,7 +18431,7 @@
         <v>477</v>
       </c>
       <c r="C1636" t="n">
-        <v>79056</v>
+        <v>88938</v>
       </c>
     </row>
     <row r="1637">
@@ -18442,7 +18442,7 @@
         <v>530</v>
       </c>
       <c r="C1637" t="n">
-        <v>109088</v>
+        <v>122724</v>
       </c>
     </row>
     <row r="1638">
@@ -18453,7 +18453,7 @@
         <v>953</v>
       </c>
       <c r="C1638" t="n">
-        <v>250904</v>
+        <v>282267</v>
       </c>
     </row>
     <row r="1639">
@@ -18464,7 +18464,7 @@
         <v>610</v>
       </c>
       <c r="C1639" t="n">
-        <v>298832</v>
+        <v>336186</v>
       </c>
     </row>
     <row r="1640">
@@ -18475,7 +18475,7 @@
         <v>2792</v>
       </c>
       <c r="C1640" t="n">
-        <v>75048</v>
+        <v>84429</v>
       </c>
     </row>
     <row r="1641">
@@ -18486,7 +18486,7 @@
         <v>2834</v>
       </c>
       <c r="C1641" t="n">
-        <v>13552</v>
+        <v>15246</v>
       </c>
     </row>
     <row r="1642">
@@ -18497,7 +18497,7 @@
         <v>2394</v>
       </c>
       <c r="C1642" t="n">
-        <v>41256</v>
+        <v>46413</v>
       </c>
     </row>
     <row r="1643">
@@ -18508,7 +18508,7 @@
         <v>2567</v>
       </c>
       <c r="C1643" t="n">
-        <v>36360</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1644">
@@ -18519,7 +18519,7 @@
         <v>952</v>
       </c>
       <c r="C1644" t="n">
-        <v>36360</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1645">
@@ -18530,7 +18530,7 @@
         <v>1539</v>
       </c>
       <c r="C1645" t="n">
-        <v>61816</v>
+        <v>69543</v>
       </c>
     </row>
     <row r="1646">
@@ -18541,7 +18541,7 @@
         <v>793</v>
       </c>
       <c r="C1646" t="n">
-        <v>15128</v>
+        <v>17019</v>
       </c>
     </row>
     <row r="1647">
@@ -18552,7 +18552,7 @@
         <v>794</v>
       </c>
       <c r="C1647" t="n">
-        <v>15128</v>
+        <v>17019</v>
       </c>
     </row>
     <row r="1648">
@@ -18563,7 +18563,7 @@
         <v>2838</v>
       </c>
       <c r="C1648" t="n">
-        <v>21818.22</v>
+        <v>24545.49</v>
       </c>
     </row>
     <row r="1649">
@@ -18574,7 +18574,7 @@
         <v>2223</v>
       </c>
       <c r="C1649" t="n">
-        <v>42584</v>
+        <v>47907</v>
       </c>
     </row>
     <row r="1650">
@@ -18585,7 +18585,7 @@
         <v>2547</v>
       </c>
       <c r="C1650" t="n">
-        <v>12320</v>
+        <v>13860</v>
       </c>
     </row>
     <row r="1651">
@@ -18596,7 +18596,7 @@
         <v>2762</v>
       </c>
       <c r="C1651" t="n">
-        <v>29632</v>
+        <v>33336</v>
       </c>
     </row>
     <row r="1652">
@@ -18607,7 +18607,7 @@
         <v>2550</v>
       </c>
       <c r="C1652" t="n">
-        <v>14216</v>
+        <v>15993</v>
       </c>
     </row>
     <row r="1653">
@@ -18618,7 +18618,7 @@
         <v>2627</v>
       </c>
       <c r="C1653" t="n">
-        <v>14216</v>
+        <v>15993</v>
       </c>
     </row>
     <row r="1654">
@@ -18640,7 +18640,7 @@
         <v>749</v>
       </c>
       <c r="C1655" t="n">
-        <v>29632</v>
+        <v>33336</v>
       </c>
     </row>
     <row r="1656">
@@ -18651,7 +18651,7 @@
         <v>2549</v>
       </c>
       <c r="C1656" t="n">
-        <v>14216</v>
+        <v>15993</v>
       </c>
     </row>
     <row r="1657">
@@ -18662,7 +18662,7 @@
         <v>2649</v>
       </c>
       <c r="C1657" t="n">
-        <v>14216</v>
+        <v>15993</v>
       </c>
     </row>
     <row r="1658">
@@ -18673,7 +18673,7 @@
         <v>2258</v>
       </c>
       <c r="C1658" t="n">
-        <v>29088</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1659">
@@ -18684,7 +18684,7 @@
         <v>2744</v>
       </c>
       <c r="C1659" t="n">
-        <v>21816</v>
+        <v>24543</v>
       </c>
     </row>
     <row r="1660">
@@ -18695,7 +18695,7 @@
         <v>452</v>
       </c>
       <c r="C1660" t="n">
-        <v>102904</v>
+        <v>115767</v>
       </c>
     </row>
     <row r="1661">
@@ -18706,7 +18706,7 @@
         <v>2653</v>
       </c>
       <c r="C1661" t="n">
-        <v>21816</v>
+        <v>24543</v>
       </c>
     </row>
     <row r="1662">
@@ -18717,7 +18717,7 @@
         <v>2742</v>
       </c>
       <c r="C1662" t="n">
-        <v>21816</v>
+        <v>24543</v>
       </c>
     </row>
     <row r="1663">
@@ -18728,7 +18728,7 @@
         <v>1075</v>
       </c>
       <c r="C1663" t="n">
-        <v>166904</v>
+        <v>187767</v>
       </c>
     </row>
     <row r="1664">
@@ -18739,7 +18739,7 @@
         <v>131</v>
       </c>
       <c r="C1664" t="n">
-        <v>151272</v>
+        <v>170181</v>
       </c>
     </row>
     <row r="1665">
@@ -18750,7 +18750,7 @@
         <v>2667</v>
       </c>
       <c r="C1665" t="n">
-        <v>16616</v>
+        <v>18693</v>
       </c>
     </row>
     <row r="1666">
@@ -18761,7 +18761,7 @@
         <v>2330</v>
       </c>
       <c r="C1666" t="n">
-        <v>32344</v>
+        <v>36387</v>
       </c>
     </row>
     <row r="1667">
@@ -18772,7 +18772,7 @@
         <v>2577</v>
       </c>
       <c r="C1667" t="n">
-        <v>32424</v>
+        <v>36477</v>
       </c>
     </row>
     <row r="1668">
@@ -18783,7 +18783,7 @@
         <v>2510</v>
       </c>
       <c r="C1668" t="n">
-        <v>230272</v>
+        <v>259056</v>
       </c>
     </row>
     <row r="1669">
@@ -18794,7 +18794,7 @@
         <v>2745</v>
       </c>
       <c r="C1669" t="n">
-        <v>40000</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="1670">
@@ -18805,7 +18805,7 @@
         <v>2817</v>
       </c>
       <c r="C1670" t="n">
-        <v>21816</v>
+        <v>24543</v>
       </c>
     </row>
     <row r="1671">
@@ -18816,7 +18816,7 @@
         <v>2784</v>
       </c>
       <c r="C1671" t="n">
-        <v>15128</v>
+        <v>17019</v>
       </c>
     </row>
     <row r="1672">
@@ -18827,7 +18827,7 @@
         <v>626</v>
       </c>
       <c r="C1672" t="n">
-        <v>628296</v>
+        <v>706833</v>
       </c>
     </row>
     <row r="1673">
@@ -18838,7 +18838,7 @@
         <v>925</v>
       </c>
       <c r="C1673" t="n">
-        <v>29008</v>
+        <v>32634</v>
       </c>
     </row>
     <row r="1674">
@@ -18849,7 +18849,7 @@
         <v>2586</v>
       </c>
       <c r="C1674" t="n">
-        <v>15128</v>
+        <v>17019</v>
       </c>
     </row>
     <row r="1675">
@@ -18860,7 +18860,7 @@
         <v>966</v>
       </c>
       <c r="C1675" t="n">
-        <v>29632</v>
+        <v>33336</v>
       </c>
     </row>
     <row r="1676">
@@ -18871,7 +18871,7 @@
         <v>2557</v>
       </c>
       <c r="C1676" t="n">
-        <v>14216</v>
+        <v>15993</v>
       </c>
     </row>
     <row r="1677">
@@ -18882,7 +18882,7 @@
         <v>14</v>
       </c>
       <c r="C1677" t="n">
-        <v>163632</v>
+        <v>184086</v>
       </c>
     </row>
     <row r="1678">
@@ -18893,7 +18893,7 @@
         <v>2798</v>
       </c>
       <c r="C1678" t="n">
-        <v>21816</v>
+        <v>24543</v>
       </c>
     </row>
     <row r="1679">
@@ -18904,7 +18904,7 @@
         <v>2797</v>
       </c>
       <c r="C1679" t="n">
-        <v>21816</v>
+        <v>24543</v>
       </c>
     </row>
     <row r="1680">
@@ -18915,7 +18915,7 @@
         <v>522</v>
       </c>
       <c r="C1680" t="n">
-        <v>72720</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1681">
@@ -18926,7 +18926,7 @@
         <v>2819</v>
       </c>
       <c r="C1681" t="n">
-        <v>21816</v>
+        <v>24543</v>
       </c>
     </row>
     <row r="1682">
@@ -18937,7 +18937,7 @@
         <v>2266</v>
       </c>
       <c r="C1682" t="n">
-        <v>29088</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1683">
@@ -18948,7 +18948,7 @@
         <v>2795</v>
       </c>
       <c r="C1683" t="n">
-        <v>21816</v>
+        <v>24543</v>
       </c>
     </row>
     <row r="1684">
@@ -18959,7 +18959,7 @@
         <v>2722</v>
       </c>
       <c r="C1684" t="n">
-        <v>7272</v>
+        <v>8181</v>
       </c>
     </row>
     <row r="1685">
@@ -18970,7 +18970,7 @@
         <v>951</v>
       </c>
       <c r="C1685" t="n">
-        <v>41816</v>
+        <v>47043</v>
       </c>
     </row>
     <row r="1686">
@@ -18981,7 +18981,7 @@
         <v>1020</v>
       </c>
       <c r="C1686" t="n">
-        <v>36360</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1687">
@@ -18992,7 +18992,7 @@
         <v>1853</v>
       </c>
       <c r="C1687" t="n">
-        <v>43632</v>
+        <v>49086</v>
       </c>
     </row>
     <row r="1688">
@@ -19003,7 +19003,7 @@
         <v>1327</v>
       </c>
       <c r="C1688" t="n">
-        <v>25448</v>
+        <v>28629</v>
       </c>
     </row>
     <row r="1689">
@@ -19014,7 +19014,7 @@
         <v>2842</v>
       </c>
       <c r="C1689" t="n">
-        <v>65448</v>
+        <v>73629</v>
       </c>
     </row>
     <row r="1690">
@@ -19025,7 +19025,7 @@
         <v>2831</v>
       </c>
       <c r="C1690" t="n">
-        <v>21816</v>
+        <v>24543</v>
       </c>
     </row>
     <row r="1691">
@@ -19036,7 +19036,7 @@
         <v>818</v>
       </c>
       <c r="C1691" t="n">
-        <v>145448</v>
+        <v>163629</v>
       </c>
     </row>
     <row r="1692">
@@ -19047,7 +19047,7 @@
         <v>1501</v>
       </c>
       <c r="C1692" t="n">
-        <v>36360</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1693">
@@ -19058,7 +19058,7 @@
         <v>1869</v>
       </c>
       <c r="C1693" t="n">
-        <v>88720</v>
+        <v>99810</v>
       </c>
     </row>
     <row r="1694">
@@ -19069,7 +19069,7 @@
         <v>1996</v>
       </c>
       <c r="C1694" t="n">
-        <v>90904</v>
+        <v>102267</v>
       </c>
     </row>
     <row r="1695">
@@ -19080,7 +19080,7 @@
         <v>2462</v>
       </c>
       <c r="C1695" t="n">
-        <v>20592</v>
+        <v>23166</v>
       </c>
     </row>
     <row r="1696">
@@ -19091,7 +19091,7 @@
         <v>2696</v>
       </c>
       <c r="C1696" t="n">
-        <v>77984</v>
+        <v>87732</v>
       </c>
     </row>
     <row r="1697">
@@ -19102,7 +19102,7 @@
         <v>2698</v>
       </c>
       <c r="C1697" t="n">
-        <v>39968</v>
+        <v>44964</v>
       </c>
     </row>
     <row r="1698">
@@ -19113,7 +19113,7 @@
         <v>2828</v>
       </c>
       <c r="C1698" t="n">
-        <v>21818.22</v>
+        <v>24545.49</v>
       </c>
     </row>
     <row r="1699">
@@ -19124,7 +19124,7 @@
         <v>619</v>
       </c>
       <c r="C1699" t="n">
-        <v>114000</v>
+        <v>128250</v>
       </c>
     </row>
     <row r="1700">
@@ -19135,7 +19135,7 @@
         <v>1478</v>
       </c>
       <c r="C1700" t="n">
-        <v>199504</v>
+        <v>224442</v>
       </c>
     </row>
     <row r="1701">
@@ -19146,7 +19146,7 @@
         <v>2026</v>
       </c>
       <c r="C1701" t="n">
-        <v>88144</v>
+        <v>99162</v>
       </c>
     </row>
     <row r="1702">
@@ -19154,10 +19154,10 @@
         <v>46296</v>
       </c>
       <c r="B1702" t="n">
-        <v>285</v>
+        <v>663</v>
       </c>
       <c r="C1702" t="n">
-        <v>199504</v>
+        <v>105948</v>
       </c>
     </row>
     <row r="1703">
@@ -19165,10 +19165,10 @@
         <v>46296</v>
       </c>
       <c r="B1703" t="n">
-        <v>424</v>
+        <v>285</v>
       </c>
       <c r="C1703" t="n">
-        <v>85496</v>
+        <v>224442</v>
       </c>
     </row>
     <row r="1704">
@@ -19176,10 +19176,10 @@
         <v>46296</v>
       </c>
       <c r="B1704" t="n">
-        <v>451</v>
+        <v>424</v>
       </c>
       <c r="C1704" t="n">
-        <v>88360</v>
+        <v>96183</v>
       </c>
     </row>
     <row r="1705">
@@ -19187,10 +19187,10 @@
         <v>46296</v>
       </c>
       <c r="B1705" t="n">
-        <v>629</v>
+        <v>451</v>
       </c>
       <c r="C1705" t="n">
-        <v>165088</v>
+        <v>99405</v>
       </c>
     </row>
     <row r="1706">
@@ -19198,10 +19198,10 @@
         <v>46296</v>
       </c>
       <c r="B1706" t="n">
-        <v>663</v>
+        <v>629</v>
       </c>
       <c r="C1706" t="n">
-        <v>94176</v>
+        <v>185724</v>
       </c>
     </row>
     <row r="1707">
@@ -19212,7 +19212,7 @@
         <v>2657</v>
       </c>
       <c r="C1707" t="n">
-        <v>28792</v>
+        <v>32391</v>
       </c>
     </row>
     <row r="1708">
@@ -19223,7 +19223,7 @@
         <v>1254</v>
       </c>
       <c r="C1708" t="n">
-        <v>70616</v>
+        <v>79443</v>
       </c>
     </row>
     <row r="1709">
@@ -19234,7 +19234,7 @@
         <v>2402</v>
       </c>
       <c r="C1709" t="n">
-        <v>177616</v>
+        <v>199818</v>
       </c>
     </row>
     <row r="1710">
@@ -19245,7 +19245,7 @@
         <v>2413</v>
       </c>
       <c r="C1710" t="n">
-        <v>50120</v>
+        <v>56385</v>
       </c>
     </row>
     <row r="1711">
@@ -19256,7 +19256,7 @@
         <v>1450</v>
       </c>
       <c r="C1711" t="n">
-        <v>129816</v>
+        <v>146043</v>
       </c>
     </row>
     <row r="1712">
@@ -19267,7 +19267,7 @@
         <v>2671</v>
       </c>
       <c r="C1712" t="n">
-        <v>29088</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1713">
@@ -19278,7 +19278,7 @@
         <v>2568</v>
       </c>
       <c r="C1713" t="n">
-        <v>58344</v>
+        <v>65637</v>
       </c>
     </row>
     <row r="1714">
@@ -19289,7 +19289,7 @@
         <v>2146</v>
       </c>
       <c r="C1714" t="n">
-        <v>70648</v>
+        <v>79479</v>
       </c>
     </row>
     <row r="1715">
@@ -19300,7 +19300,7 @@
         <v>2753</v>
       </c>
       <c r="C1715" t="n">
-        <v>27272</v>
+        <v>30681</v>
       </c>
     </row>
     <row r="1716">
@@ -19311,7 +19311,7 @@
         <v>744</v>
       </c>
       <c r="C1716" t="n">
-        <v>15128</v>
+        <v>17019</v>
       </c>
     </row>
     <row r="1717">
@@ -19322,7 +19322,7 @@
         <v>2323</v>
       </c>
       <c r="C1717" t="n">
-        <v>24976</v>
+        <v>28098</v>
       </c>
     </row>
     <row r="1718">
@@ -19333,7 +19333,7 @@
         <v>2310</v>
       </c>
       <c r="C1718" t="n">
-        <v>24976</v>
+        <v>28098</v>
       </c>
     </row>
     <row r="1719">
@@ -19344,7 +19344,7 @@
         <v>2145</v>
       </c>
       <c r="C1719" t="n">
-        <v>36360</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1720">
@@ -19355,7 +19355,7 @@
         <v>2501</v>
       </c>
       <c r="C1720" t="n">
-        <v>29632</v>
+        <v>33336</v>
       </c>
     </row>
     <row r="1721">
@@ -19366,7 +19366,7 @@
         <v>2546</v>
       </c>
       <c r="C1721" t="n">
-        <v>14216</v>
+        <v>15993</v>
       </c>
     </row>
     <row r="1722">
@@ -19377,7 +19377,7 @@
         <v>716</v>
       </c>
       <c r="C1722" t="n">
-        <v>46608</v>
+        <v>52434</v>
       </c>
     </row>
     <row r="1723">
@@ -19388,7 +19388,7 @@
         <v>2758</v>
       </c>
       <c r="C1723" t="n">
-        <v>21816</v>
+        <v>24543</v>
       </c>
     </row>
     <row r="1724">
@@ -19399,7 +19399,7 @@
         <v>400</v>
       </c>
       <c r="C1724" t="n">
-        <v>65448</v>
+        <v>73629</v>
       </c>
     </row>
     <row r="1725">
@@ -19410,7 +19410,7 @@
         <v>1259</v>
       </c>
       <c r="C1725" t="n">
-        <v>40000</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="1726">
@@ -19421,7 +19421,7 @@
         <v>571</v>
       </c>
       <c r="C1726" t="n">
-        <v>340000</v>
+        <v>382500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:02:21
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -15560,7 +15560,7 @@
         <v>2853</v>
       </c>
       <c r="C1375" t="n">
-        <v>37030</v>
+        <v>40733</v>
       </c>
     </row>
     <row r="1376">
@@ -15571,7 +15571,7 @@
         <v>2245</v>
       </c>
       <c r="C1376" t="n">
-        <v>100640</v>
+        <v>110704</v>
       </c>
     </row>
     <row r="1377">
@@ -15582,7 +15582,7 @@
         <v>2251</v>
       </c>
       <c r="C1377" t="n">
-        <v>90900</v>
+        <v>99990</v>
       </c>
     </row>
     <row r="1378">
@@ -15593,7 +15593,7 @@
         <v>664</v>
       </c>
       <c r="C1378" t="n">
-        <v>119090</v>
+        <v>130999</v>
       </c>
     </row>
     <row r="1379">
@@ -15604,7 +15604,7 @@
         <v>2472</v>
       </c>
       <c r="C1379" t="n">
-        <v>24060</v>
+        <v>26466</v>
       </c>
     </row>
     <row r="1380">
@@ -15615,7 +15615,7 @@
         <v>1456</v>
       </c>
       <c r="C1380" t="n">
-        <v>362720</v>
+        <v>398992</v>
       </c>
     </row>
     <row r="1381">
@@ -15626,7 +15626,7 @@
         <v>1585</v>
       </c>
       <c r="C1381" t="n">
-        <v>82270</v>
+        <v>90497</v>
       </c>
     </row>
     <row r="1382">
@@ -15670,7 +15670,7 @@
         <v>1907</v>
       </c>
       <c r="C1385" t="n">
-        <v>250240</v>
+        <v>275264</v>
       </c>
     </row>
     <row r="1386">
@@ -15703,7 +15703,7 @@
         <v>2659</v>
       </c>
       <c r="C1388" t="n">
-        <v>55910</v>
+        <v>61501</v>
       </c>
     </row>
     <row r="1389">
@@ -15714,7 +15714,7 @@
         <v>2583</v>
       </c>
       <c r="C1389" t="n">
-        <v>18910</v>
+        <v>20801</v>
       </c>
     </row>
     <row r="1390">
@@ -15725,7 +15725,7 @@
         <v>2692</v>
       </c>
       <c r="C1390" t="n">
-        <v>31818.28</v>
+        <v>35000.09</v>
       </c>
     </row>
     <row r="1391">
@@ -15736,7 +15736,7 @@
         <v>2691</v>
       </c>
       <c r="C1391" t="n">
-        <v>55538.28</v>
+        <v>61092.09</v>
       </c>
     </row>
     <row r="1392">
@@ -15747,7 +15747,7 @@
         <v>931</v>
       </c>
       <c r="C1392" t="n">
-        <v>43510</v>
+        <v>47861</v>
       </c>
     </row>
     <row r="1393">
@@ -15758,7 +15758,7 @@
         <v>2785</v>
       </c>
       <c r="C1393" t="n">
-        <v>18910</v>
+        <v>20801</v>
       </c>
     </row>
     <row r="1394">
@@ -15769,7 +15769,7 @@
         <v>2411</v>
       </c>
       <c r="C1394" t="n">
-        <v>45450</v>
+        <v>49995</v>
       </c>
     </row>
     <row r="1395">
@@ -15780,7 +15780,7 @@
         <v>2716</v>
       </c>
       <c r="C1395" t="n">
-        <v>39880</v>
+        <v>43868</v>
       </c>
     </row>
     <row r="1396">
@@ -15791,7 +15791,7 @@
         <v>2809</v>
       </c>
       <c r="C1396" t="n">
-        <v>31220</v>
+        <v>34342</v>
       </c>
     </row>
     <row r="1397">
@@ -15802,7 +15802,7 @@
         <v>104</v>
       </c>
       <c r="C1397" t="n">
-        <v>136363.68</v>
+        <v>150000.04</v>
       </c>
     </row>
     <row r="1398">
@@ -15835,7 +15835,7 @@
         <v>781</v>
       </c>
       <c r="C1400" t="n">
-        <v>59090</v>
+        <v>64999</v>
       </c>
     </row>
     <row r="1401">
@@ -15857,7 +15857,7 @@
         <v>2494</v>
       </c>
       <c r="C1402" t="n">
-        <v>68180</v>
+        <v>74998</v>
       </c>
     </row>
     <row r="1403">
@@ -15868,7 +15868,7 @@
         <v>2652</v>
       </c>
       <c r="C1403" t="n">
-        <v>63630</v>
+        <v>69993</v>
       </c>
     </row>
     <row r="1404">
@@ -15879,7 +15879,7 @@
         <v>1384</v>
       </c>
       <c r="C1404" t="n">
-        <v>159090.92</v>
+        <v>175000.01</v>
       </c>
     </row>
     <row r="1405">
@@ -15890,7 +15890,7 @@
         <v>360</v>
       </c>
       <c r="C1405" t="n">
-        <v>227270</v>
+        <v>249997</v>
       </c>
     </row>
     <row r="1406">
@@ -15901,7 +15901,7 @@
         <v>2767</v>
       </c>
       <c r="C1406" t="n">
-        <v>86360</v>
+        <v>94996</v>
       </c>
     </row>
     <row r="1407">
@@ -15912,7 +15912,7 @@
         <v>2178</v>
       </c>
       <c r="C1407" t="n">
-        <v>124540</v>
+        <v>136994</v>
       </c>
     </row>
     <row r="1408">
@@ -15923,7 +15923,7 @@
         <v>2107</v>
       </c>
       <c r="C1408" t="n">
-        <v>136350</v>
+        <v>149985</v>
       </c>
     </row>
     <row r="1409">
@@ -15934,7 +15934,7 @@
         <v>2711</v>
       </c>
       <c r="C1409" t="n">
-        <v>39350</v>
+        <v>43285</v>
       </c>
     </row>
     <row r="1410">
@@ -15945,7 +15945,7 @@
         <v>2845</v>
       </c>
       <c r="C1410" t="n">
-        <v>22720</v>
+        <v>24992</v>
       </c>
     </row>
     <row r="1411">
@@ -15989,7 +15989,7 @@
         <v>1102</v>
       </c>
       <c r="C1414" t="n">
-        <v>106870</v>
+        <v>117557</v>
       </c>
     </row>
     <row r="1415">
@@ -16000,7 +16000,7 @@
         <v>353</v>
       </c>
       <c r="C1415" t="n">
-        <v>132970</v>
+        <v>146267</v>
       </c>
     </row>
     <row r="1416">
@@ -16011,7 +16011,7 @@
         <v>2250</v>
       </c>
       <c r="C1416" t="n">
-        <v>154540</v>
+        <v>169994</v>
       </c>
     </row>
     <row r="1417">
@@ -16022,7 +16022,7 @@
         <v>1800</v>
       </c>
       <c r="C1417" t="n">
-        <v>12890</v>
+        <v>14179</v>
       </c>
     </row>
     <row r="1418">
@@ -16033,7 +16033,7 @@
         <v>2362</v>
       </c>
       <c r="C1418" t="n">
-        <v>34090</v>
+        <v>37499</v>
       </c>
     </row>
     <row r="1419">
@@ -16044,7 +16044,7 @@
         <v>2449</v>
       </c>
       <c r="C1419" t="n">
-        <v>43180</v>
+        <v>47498</v>
       </c>
     </row>
     <row r="1420">
@@ -16055,7 +16055,7 @@
         <v>2844</v>
       </c>
       <c r="C1420" t="n">
-        <v>22720</v>
+        <v>24992</v>
       </c>
     </row>
     <row r="1421">
@@ -16066,7 +16066,7 @@
         <v>2507</v>
       </c>
       <c r="C1421" t="n">
-        <v>40600</v>
+        <v>44660</v>
       </c>
     </row>
     <row r="1422">
@@ -16077,7 +16077,7 @@
         <v>1906</v>
       </c>
       <c r="C1422" t="n">
-        <v>49350</v>
+        <v>54285</v>
       </c>
     </row>
     <row r="1423">
@@ -16099,7 +16099,7 @@
         <v>525</v>
       </c>
       <c r="C1424" t="n">
-        <v>106818.28</v>
+        <v>117500.09</v>
       </c>
     </row>
     <row r="1425">
@@ -16110,7 +16110,7 @@
         <v>1261</v>
       </c>
       <c r="C1425" t="n">
-        <v>32272.76</v>
+        <v>35500.03</v>
       </c>
     </row>
     <row r="1426">
@@ -16121,7 +16121,7 @@
         <v>2755</v>
       </c>
       <c r="C1426" t="n">
-        <v>22727.36</v>
+        <v>25000.08</v>
       </c>
     </row>
     <row r="1427">
@@ -16143,7 +16143,7 @@
         <v>1064</v>
       </c>
       <c r="C1428" t="n">
-        <v>272720</v>
+        <v>299992</v>
       </c>
     </row>
     <row r="1429">
@@ -16154,7 +16154,7 @@
         <v>1810</v>
       </c>
       <c r="C1429" t="n">
-        <v>18460</v>
+        <v>20306</v>
       </c>
     </row>
     <row r="1430">
@@ -16165,7 +16165,7 @@
         <v>1937</v>
       </c>
       <c r="C1430" t="n">
-        <v>117720</v>
+        <v>129492</v>
       </c>
     </row>
     <row r="1431">
@@ -16176,7 +16176,7 @@
         <v>483</v>
       </c>
       <c r="C1431" t="n">
-        <v>205450</v>
+        <v>225995</v>
       </c>
     </row>
     <row r="1432">
@@ -16187,7 +16187,7 @@
         <v>2580</v>
       </c>
       <c r="C1432" t="n">
-        <v>15310</v>
+        <v>16841</v>
       </c>
     </row>
     <row r="1433">
@@ -16198,7 +16198,7 @@
         <v>2706</v>
       </c>
       <c r="C1433" t="n">
-        <v>11960</v>
+        <v>13156</v>
       </c>
     </row>
     <row r="1434">
@@ -16209,7 +16209,7 @@
         <v>2633</v>
       </c>
       <c r="C1434" t="n">
-        <v>8760</v>
+        <v>9636</v>
       </c>
     </row>
     <row r="1435">
@@ -16242,7 +16242,7 @@
         <v>2392</v>
       </c>
       <c r="C1437" t="n">
-        <v>94280</v>
+        <v>103708</v>
       </c>
     </row>
     <row r="1438">
@@ -16264,7 +16264,7 @@
         <v>2613</v>
       </c>
       <c r="C1439" t="n">
-        <v>66380</v>
+        <v>73018</v>
       </c>
     </row>
     <row r="1440">
@@ -16275,7 +16275,7 @@
         <v>2183</v>
       </c>
       <c r="C1440" t="n">
-        <v>239010</v>
+        <v>262911</v>
       </c>
     </row>
     <row r="1441">
@@ -16286,7 +16286,7 @@
         <v>2541</v>
       </c>
       <c r="C1441" t="n">
-        <v>107450</v>
+        <v>118195</v>
       </c>
     </row>
     <row r="1442">
@@ -16297,7 +16297,7 @@
         <v>2333</v>
       </c>
       <c r="C1442" t="n">
-        <v>72540</v>
+        <v>79794</v>
       </c>
     </row>
     <row r="1443">
@@ -16308,7 +16308,7 @@
         <v>2813</v>
       </c>
       <c r="C1443" t="n">
-        <v>29000</v>
+        <v>31900</v>
       </c>
     </row>
     <row r="1444">
@@ -16319,7 +16319,7 @@
         <v>2811</v>
       </c>
       <c r="C1444" t="n">
-        <v>18910</v>
+        <v>20801</v>
       </c>
     </row>
     <row r="1445">
@@ -16330,7 +16330,7 @@
         <v>1881</v>
       </c>
       <c r="C1445" t="n">
-        <v>31220</v>
+        <v>34342</v>
       </c>
     </row>
     <row r="1446">
@@ -16341,7 +16341,7 @@
         <v>2825</v>
       </c>
       <c r="C1446" t="n">
-        <v>25380</v>
+        <v>27918</v>
       </c>
     </row>
     <row r="1447">
@@ -16352,7 +16352,7 @@
         <v>970</v>
       </c>
       <c r="C1447" t="n">
-        <v>31220</v>
+        <v>34342</v>
       </c>
     </row>
     <row r="1448">
@@ -16363,7 +16363,7 @@
         <v>2552</v>
       </c>
       <c r="C1448" t="n">
-        <v>17770</v>
+        <v>19547</v>
       </c>
     </row>
     <row r="1449">
@@ -16374,7 +16374,7 @@
         <v>2562</v>
       </c>
       <c r="C1449" t="n">
-        <v>17770</v>
+        <v>19547</v>
       </c>
     </row>
     <row r="1450">
@@ -16407,7 +16407,7 @@
         <v>2747</v>
       </c>
       <c r="C1452" t="n">
-        <v>31810</v>
+        <v>34991</v>
       </c>
     </row>
     <row r="1453">
@@ -16418,7 +16418,7 @@
         <v>415</v>
       </c>
       <c r="C1453" t="n">
-        <v>113636.44</v>
+        <v>125000.07</v>
       </c>
     </row>
     <row r="1454">
@@ -16462,7 +16462,7 @@
         <v>2544</v>
       </c>
       <c r="C1457" t="n">
-        <v>31810</v>
+        <v>34991</v>
       </c>
     </row>
     <row r="1458">
@@ -16473,7 +16473,7 @@
         <v>816</v>
       </c>
       <c r="C1458" t="n">
-        <v>136363.68</v>
+        <v>150000.04</v>
       </c>
     </row>
     <row r="1459">
@@ -16484,7 +16484,7 @@
         <v>890</v>
       </c>
       <c r="C1459" t="n">
-        <v>409090.92</v>
+        <v>450000.01</v>
       </c>
     </row>
     <row r="1460">
@@ -16495,7 +16495,7 @@
         <v>1298</v>
       </c>
       <c r="C1460" t="n">
-        <v>575000</v>
+        <v>632500</v>
       </c>
     </row>
     <row r="1461">
@@ -16506,7 +16506,7 @@
         <v>1372</v>
       </c>
       <c r="C1461" t="n">
-        <v>136363.68</v>
+        <v>150000.04</v>
       </c>
     </row>
     <row r="1462">
@@ -16517,7 +16517,7 @@
         <v>358</v>
       </c>
       <c r="C1462" t="n">
-        <v>143180</v>
+        <v>157498</v>
       </c>
     </row>
     <row r="1463">
@@ -16528,7 +16528,7 @@
         <v>1653</v>
       </c>
       <c r="C1463" t="n">
-        <v>143180</v>
+        <v>157498</v>
       </c>
     </row>
     <row r="1464">
@@ -16539,7 +16539,7 @@
         <v>675</v>
       </c>
       <c r="C1464" t="n">
-        <v>90900</v>
+        <v>99990</v>
       </c>
     </row>
     <row r="1465">
@@ -16550,7 +16550,7 @@
         <v>2804</v>
       </c>
       <c r="C1465" t="n">
-        <v>45450</v>
+        <v>49995</v>
       </c>
     </row>
     <row r="1466">
@@ -16561,7 +16561,7 @@
         <v>2714</v>
       </c>
       <c r="C1466" t="n">
-        <v>163630</v>
+        <v>179993</v>
       </c>
     </row>
     <row r="1467">
@@ -16572,7 +16572,7 @@
         <v>2765</v>
       </c>
       <c r="C1467" t="n">
-        <v>40900</v>
+        <v>44990</v>
       </c>
     </row>
     <row r="1468">
@@ -16583,7 +16583,7 @@
         <v>2421</v>
       </c>
       <c r="C1468" t="n">
-        <v>27720</v>
+        <v>30492</v>
       </c>
     </row>
     <row r="1469">
@@ -16594,7 +16594,7 @@
         <v>2359</v>
       </c>
       <c r="C1469" t="n">
-        <v>47420</v>
+        <v>52162</v>
       </c>
     </row>
     <row r="1470">
@@ -16605,7 +16605,7 @@
         <v>2678</v>
       </c>
       <c r="C1470" t="n">
-        <v>44980</v>
+        <v>49478</v>
       </c>
     </row>
     <row r="1471">
@@ -16616,7 +16616,7 @@
         <v>2697</v>
       </c>
       <c r="C1471" t="n">
-        <v>68260</v>
+        <v>75086</v>
       </c>
     </row>
     <row r="1472">
@@ -16649,7 +16649,7 @@
         <v>2142</v>
       </c>
       <c r="C1474" t="n">
-        <v>24600</v>
+        <v>27060</v>
       </c>
     </row>
     <row r="1475">
@@ -16660,7 +16660,7 @@
         <v>2498</v>
       </c>
       <c r="C1475" t="n">
-        <v>25590</v>
+        <v>28149</v>
       </c>
     </row>
     <row r="1476">
@@ -16682,7 +16682,7 @@
         <v>2801</v>
       </c>
       <c r="C1477" t="n">
-        <v>45454.6</v>
+        <v>50000.05</v>
       </c>
     </row>
     <row r="1478">
@@ -16693,7 +16693,7 @@
         <v>2810</v>
       </c>
       <c r="C1478" t="n">
-        <v>72727.36</v>
+        <v>80000.08</v>
       </c>
     </row>
     <row r="1479">
@@ -16734,10 +16734,10 @@
         <v>46296</v>
       </c>
       <c r="B1482" t="n">
-        <v>580</v>
+        <v>1433</v>
       </c>
       <c r="C1482" t="n">
-        <v>79545.52</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1483">
@@ -16745,10 +16745,10 @@
         <v>46296</v>
       </c>
       <c r="B1483" t="n">
-        <v>634</v>
+        <v>580</v>
       </c>
       <c r="C1483" t="n">
-        <v>227272.76</v>
+        <v>87500.06</v>
       </c>
     </row>
     <row r="1484">
@@ -16756,10 +16756,10 @@
         <v>46296</v>
       </c>
       <c r="B1484" t="n">
-        <v>2437</v>
+        <v>634</v>
       </c>
       <c r="C1484" t="n">
-        <v>0</v>
+        <v>250000.03</v>
       </c>
     </row>
     <row r="1485">
@@ -16767,10 +16767,10 @@
         <v>46296</v>
       </c>
       <c r="B1485" t="n">
-        <v>1277</v>
+        <v>2437</v>
       </c>
       <c r="C1485" t="n">
-        <v>100000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1486">
@@ -16778,10 +16778,10 @@
         <v>46296</v>
       </c>
       <c r="B1486" t="n">
-        <v>767</v>
+        <v>1277</v>
       </c>
       <c r="C1486" t="n">
-        <v>90900</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="1487">
@@ -16789,10 +16789,10 @@
         <v>46296</v>
       </c>
       <c r="B1487" t="n">
-        <v>2727</v>
+        <v>767</v>
       </c>
       <c r="C1487" t="n">
-        <v>18400</v>
+        <v>99990</v>
       </c>
     </row>
     <row r="1488">
@@ -16800,10 +16800,10 @@
         <v>46296</v>
       </c>
       <c r="B1488" t="n">
-        <v>2846</v>
+        <v>2727</v>
       </c>
       <c r="C1488" t="n">
-        <v>118180</v>
+        <v>20240</v>
       </c>
     </row>
     <row r="1489">
@@ -16811,10 +16811,10 @@
         <v>46296</v>
       </c>
       <c r="B1489" t="n">
-        <v>609</v>
+        <v>2846</v>
       </c>
       <c r="C1489" t="n">
-        <v>102270</v>
+        <v>129998</v>
       </c>
     </row>
     <row r="1490">
@@ -16822,10 +16822,10 @@
         <v>46296</v>
       </c>
       <c r="B1490" t="n">
-        <v>2726</v>
+        <v>609</v>
       </c>
       <c r="C1490" t="n">
-        <v>70450</v>
+        <v>112497</v>
       </c>
     </row>
     <row r="1491">
@@ -16833,10 +16833,10 @@
         <v>46296</v>
       </c>
       <c r="B1491" t="n">
-        <v>2729</v>
+        <v>2726</v>
       </c>
       <c r="C1491" t="n">
-        <v>40900</v>
+        <v>77495</v>
       </c>
     </row>
     <row r="1492">
@@ -16844,10 +16844,10 @@
         <v>46296</v>
       </c>
       <c r="B1492" t="n">
-        <v>1340</v>
+        <v>2729</v>
       </c>
       <c r="C1492" t="n">
-        <v>68180</v>
+        <v>44990</v>
       </c>
     </row>
     <row r="1493">
@@ -16855,10 +16855,10 @@
         <v>46296</v>
       </c>
       <c r="B1493" t="n">
-        <v>2830</v>
+        <v>1340</v>
       </c>
       <c r="C1493" t="n">
-        <v>40900</v>
+        <v>74998</v>
       </c>
     </row>
     <row r="1494">
@@ -16866,10 +16866,10 @@
         <v>46296</v>
       </c>
       <c r="B1494" t="n">
-        <v>2674</v>
+        <v>2830</v>
       </c>
       <c r="C1494" t="n">
-        <v>118180</v>
+        <v>44990</v>
       </c>
     </row>
     <row r="1495">
@@ -16877,10 +16877,10 @@
         <v>46296</v>
       </c>
       <c r="B1495" t="n">
-        <v>2308</v>
+        <v>2674</v>
       </c>
       <c r="C1495" t="n">
-        <v>90900</v>
+        <v>129998</v>
       </c>
     </row>
     <row r="1496">
@@ -16888,10 +16888,10 @@
         <v>46296</v>
       </c>
       <c r="B1496" t="n">
-        <v>2601</v>
+        <v>2308</v>
       </c>
       <c r="C1496" t="n">
-        <v>125000</v>
+        <v>99990</v>
       </c>
     </row>
     <row r="1497">
@@ -16902,7 +16902,7 @@
         <v>2190</v>
       </c>
       <c r="C1497" t="n">
-        <v>95450</v>
+        <v>104995</v>
       </c>
     </row>
     <row r="1498">
@@ -16913,7 +16913,7 @@
         <v>2015</v>
       </c>
       <c r="C1498" t="n">
-        <v>168180</v>
+        <v>184998</v>
       </c>
     </row>
     <row r="1499">
@@ -16924,7 +16924,7 @@
         <v>1308</v>
       </c>
       <c r="C1499" t="n">
-        <v>71360</v>
+        <v>78496</v>
       </c>
     </row>
     <row r="1500">
@@ -16935,7 +16935,7 @@
         <v>2118</v>
       </c>
       <c r="C1500" t="n">
-        <v>95530</v>
+        <v>105083</v>
       </c>
     </row>
     <row r="1501">
@@ -16946,7 +16946,7 @@
         <v>2607</v>
       </c>
       <c r="C1501" t="n">
-        <v>22580</v>
+        <v>24838</v>
       </c>
     </row>
     <row r="1502">
@@ -16957,7 +16957,7 @@
         <v>2707</v>
       </c>
       <c r="C1502" t="n">
-        <v>19630</v>
+        <v>21593</v>
       </c>
     </row>
     <row r="1503">
@@ -16968,7 +16968,7 @@
         <v>2832</v>
       </c>
       <c r="C1503" t="n">
-        <v>68181.84</v>
+        <v>75000.02</v>
       </c>
     </row>
     <row r="1504">
@@ -16979,7 +16979,7 @@
         <v>2383</v>
       </c>
       <c r="C1504" t="n">
-        <v>60420</v>
+        <v>66462</v>
       </c>
     </row>
     <row r="1505">
@@ -17012,7 +17012,7 @@
         <v>2821</v>
       </c>
       <c r="C1507" t="n">
-        <v>60610</v>
+        <v>66671</v>
       </c>
     </row>
     <row r="1508">
@@ -17034,7 +17034,7 @@
         <v>569</v>
       </c>
       <c r="C1509" t="n">
-        <v>1319740</v>
+        <v>1451714</v>
       </c>
     </row>
     <row r="1510">
@@ -17045,7 +17045,7 @@
         <v>2660</v>
       </c>
       <c r="C1510" t="n">
-        <v>159090.92</v>
+        <v>175000.01</v>
       </c>
     </row>
     <row r="1511">
@@ -17056,7 +17056,7 @@
         <v>1632</v>
       </c>
       <c r="C1511" t="n">
-        <v>118181.84</v>
+        <v>130000.02</v>
       </c>
     </row>
     <row r="1512">
@@ -17067,7 +17067,7 @@
         <v>1756</v>
       </c>
       <c r="C1512" t="n">
-        <v>190900</v>
+        <v>209990</v>
       </c>
     </row>
     <row r="1513">
@@ -17078,7 +17078,7 @@
         <v>58</v>
       </c>
       <c r="C1513" t="n">
-        <v>114000</v>
+        <v>125400</v>
       </c>
     </row>
     <row r="1514">
@@ -17089,7 +17089,7 @@
         <v>40</v>
       </c>
       <c r="C1514" t="n">
-        <v>101400</v>
+        <v>111540</v>
       </c>
     </row>
     <row r="1515">
@@ -17100,7 +17100,7 @@
         <v>559</v>
       </c>
       <c r="C1515" t="n">
-        <v>106360</v>
+        <v>116996</v>
       </c>
     </row>
     <row r="1516">
@@ -17111,7 +17111,7 @@
         <v>2773</v>
       </c>
       <c r="C1516" t="n">
-        <v>36670</v>
+        <v>40337</v>
       </c>
     </row>
     <row r="1517">
@@ -17122,7 +17122,7 @@
         <v>2631</v>
       </c>
       <c r="C1517" t="n">
-        <v>17610</v>
+        <v>19371</v>
       </c>
     </row>
     <row r="1518">
@@ -17133,7 +17133,7 @@
         <v>2085</v>
       </c>
       <c r="C1518" t="n">
-        <v>45450</v>
+        <v>49995</v>
       </c>
     </row>
     <row r="1519">
@@ -17155,7 +17155,7 @@
         <v>1642</v>
       </c>
       <c r="C1520" t="n">
-        <v>120450</v>
+        <v>132495</v>
       </c>
     </row>
     <row r="1521">
@@ -17166,7 +17166,7 @@
         <v>2621</v>
       </c>
       <c r="C1521" t="n">
-        <v>31810</v>
+        <v>34991</v>
       </c>
     </row>
     <row r="1522">
@@ -17177,7 +17177,7 @@
         <v>2705</v>
       </c>
       <c r="C1522" t="n">
-        <v>91260</v>
+        <v>100386</v>
       </c>
     </row>
     <row r="1523">
@@ -17188,7 +17188,7 @@
         <v>2735</v>
       </c>
       <c r="C1523" t="n">
-        <v>54540</v>
+        <v>59994</v>
       </c>
     </row>
     <row r="1524">
@@ -17199,7 +17199,7 @@
         <v>945</v>
       </c>
       <c r="C1524" t="n">
-        <v>159400</v>
+        <v>175340</v>
       </c>
     </row>
     <row r="1525">
@@ -17210,7 +17210,7 @@
         <v>2582</v>
       </c>
       <c r="C1525" t="n">
-        <v>39880</v>
+        <v>43868</v>
       </c>
     </row>
     <row r="1526">
@@ -17221,7 +17221,7 @@
         <v>2584</v>
       </c>
       <c r="C1526" t="n">
-        <v>29000</v>
+        <v>31900</v>
       </c>
     </row>
     <row r="1527">
@@ -17232,7 +17232,7 @@
         <v>2689</v>
       </c>
       <c r="C1527" t="n">
-        <v>29000</v>
+        <v>31900</v>
       </c>
     </row>
     <row r="1528">
@@ -17243,7 +17243,7 @@
         <v>2574</v>
       </c>
       <c r="C1528" t="n">
-        <v>63740</v>
+        <v>70114</v>
       </c>
     </row>
     <row r="1529">
@@ -17254,7 +17254,7 @@
         <v>1834</v>
       </c>
       <c r="C1529" t="n">
-        <v>53500</v>
+        <v>58850</v>
       </c>
     </row>
     <row r="1530">
@@ -17265,7 +17265,7 @@
         <v>2629</v>
       </c>
       <c r="C1530" t="n">
-        <v>31220</v>
+        <v>34342</v>
       </c>
     </row>
     <row r="1531">
@@ -17276,7 +17276,7 @@
         <v>933</v>
       </c>
       <c r="C1531" t="n">
-        <v>37030</v>
+        <v>40733</v>
       </c>
     </row>
     <row r="1532">
@@ -17287,7 +17287,7 @@
         <v>2555</v>
       </c>
       <c r="C1532" t="n">
-        <v>17770</v>
+        <v>19547</v>
       </c>
     </row>
     <row r="1533">
@@ -17298,7 +17298,7 @@
         <v>2558</v>
       </c>
       <c r="C1533" t="n">
-        <v>17770</v>
+        <v>19547</v>
       </c>
     </row>
     <row r="1534">
@@ -17309,7 +17309,7 @@
         <v>2721</v>
       </c>
       <c r="C1534" t="n">
-        <v>37030</v>
+        <v>40733</v>
       </c>
     </row>
     <row r="1535">
@@ -17320,7 +17320,7 @@
         <v>2556</v>
       </c>
       <c r="C1535" t="n">
-        <v>17770</v>
+        <v>19547</v>
       </c>
     </row>
     <row r="1536">
@@ -17331,7 +17331,7 @@
         <v>2826</v>
       </c>
       <c r="C1536" t="n">
-        <v>31810</v>
+        <v>34991</v>
       </c>
     </row>
     <row r="1537">
@@ -17353,7 +17353,7 @@
         <v>2346</v>
       </c>
       <c r="C1538" t="n">
-        <v>31810</v>
+        <v>34991</v>
       </c>
     </row>
     <row r="1539">
@@ -17364,7 +17364,7 @@
         <v>595</v>
       </c>
       <c r="C1539" t="n">
-        <v>113636.44</v>
+        <v>125000.07</v>
       </c>
     </row>
     <row r="1540">
@@ -17375,7 +17375,7 @@
         <v>1278</v>
       </c>
       <c r="C1540" t="n">
-        <v>79545.52</v>
+        <v>87500.06</v>
       </c>
     </row>
     <row r="1541">
@@ -17386,7 +17386,7 @@
         <v>2686</v>
       </c>
       <c r="C1541" t="n">
-        <v>63630</v>
+        <v>69993</v>
       </c>
     </row>
     <row r="1542">
@@ -17397,7 +17397,7 @@
         <v>1344</v>
       </c>
       <c r="C1542" t="n">
-        <v>68180</v>
+        <v>74998</v>
       </c>
     </row>
     <row r="1543">
@@ -17408,7 +17408,7 @@
         <v>2566</v>
       </c>
       <c r="C1543" t="n">
-        <v>36360</v>
+        <v>39996</v>
       </c>
     </row>
     <row r="1544">
@@ -17419,7 +17419,7 @@
         <v>2684</v>
       </c>
       <c r="C1544" t="n">
-        <v>43180</v>
+        <v>47498</v>
       </c>
     </row>
     <row r="1545">
@@ -17430,7 +17430,7 @@
         <v>2375</v>
       </c>
       <c r="C1545" t="n">
-        <v>150000</v>
+        <v>165000</v>
       </c>
     </row>
     <row r="1546">
@@ -17441,7 +17441,7 @@
         <v>2829</v>
       </c>
       <c r="C1546" t="n">
-        <v>27270</v>
+        <v>29997</v>
       </c>
     </row>
     <row r="1547">
@@ -17452,7 +17452,7 @@
         <v>768</v>
       </c>
       <c r="C1547" t="n">
-        <v>63630</v>
+        <v>69993</v>
       </c>
     </row>
     <row r="1548">
@@ -17463,7 +17463,7 @@
         <v>772</v>
       </c>
       <c r="C1548" t="n">
-        <v>147720</v>
+        <v>162492</v>
       </c>
     </row>
     <row r="1549">
@@ -17474,7 +17474,7 @@
         <v>2496</v>
       </c>
       <c r="C1549" t="n">
-        <v>90900</v>
+        <v>99990</v>
       </c>
     </row>
     <row r="1550">
@@ -17485,7 +17485,7 @@
         <v>802</v>
       </c>
       <c r="C1550" t="n">
-        <v>34090</v>
+        <v>37499</v>
       </c>
     </row>
     <row r="1551">
@@ -17496,7 +17496,7 @@
         <v>2131</v>
       </c>
       <c r="C1551" t="n">
-        <v>45450</v>
+        <v>49995</v>
       </c>
     </row>
     <row r="1552">
@@ -17507,7 +17507,7 @@
         <v>1381</v>
       </c>
       <c r="C1552" t="n">
-        <v>136363.68</v>
+        <v>150000.04</v>
       </c>
     </row>
     <row r="1553">
@@ -17518,7 +17518,7 @@
         <v>2847</v>
       </c>
       <c r="C1553" t="n">
-        <v>61360</v>
+        <v>67496</v>
       </c>
     </row>
     <row r="1554">
@@ -17529,7 +17529,7 @@
         <v>1293</v>
       </c>
       <c r="C1554" t="n">
-        <v>175000</v>
+        <v>192500</v>
       </c>
     </row>
     <row r="1555">
@@ -17540,7 +17540,7 @@
         <v>2363</v>
       </c>
       <c r="C1555" t="n">
-        <v>77270</v>
+        <v>84997</v>
       </c>
     </row>
     <row r="1556">
@@ -17551,7 +17551,7 @@
         <v>631</v>
       </c>
       <c r="C1556" t="n">
-        <v>159090</v>
+        <v>174999</v>
       </c>
     </row>
     <row r="1557">
@@ -17562,7 +17562,7 @@
         <v>2791</v>
       </c>
       <c r="C1557" t="n">
-        <v>46670</v>
+        <v>51337</v>
       </c>
     </row>
     <row r="1558">
@@ -17584,7 +17584,7 @@
         <v>2841</v>
       </c>
       <c r="C1559" t="n">
-        <v>22720</v>
+        <v>24992</v>
       </c>
     </row>
     <row r="1560">
@@ -17595,7 +17595,7 @@
         <v>2571</v>
       </c>
       <c r="C1560" t="n">
-        <v>121170</v>
+        <v>133287</v>
       </c>
     </row>
     <row r="1561">
@@ -17661,7 +17661,7 @@
         <v>2273</v>
       </c>
       <c r="C1566" t="n">
-        <v>97730</v>
+        <v>107503</v>
       </c>
     </row>
     <row r="1567">
@@ -17672,7 +17672,7 @@
         <v>2381</v>
       </c>
       <c r="C1567" t="n">
-        <v>36550</v>
+        <v>40205</v>
       </c>
     </row>
     <row r="1568">
@@ -17683,7 +17683,7 @@
         <v>630</v>
       </c>
       <c r="C1568" t="n">
-        <v>37513.63</v>
+        <v>41264.99</v>
       </c>
     </row>
     <row r="1569">
@@ -17705,7 +17705,7 @@
         <v>1983</v>
       </c>
       <c r="C1570" t="n">
-        <v>249200</v>
+        <v>274120</v>
       </c>
     </row>
     <row r="1571">
@@ -17716,7 +17716,7 @@
         <v>1993</v>
       </c>
       <c r="C1571" t="n">
-        <v>169220</v>
+        <v>186142</v>
       </c>
     </row>
     <row r="1572">
@@ -17727,7 +17727,7 @@
         <v>89</v>
       </c>
       <c r="C1572" t="n">
-        <v>159090</v>
+        <v>174999</v>
       </c>
     </row>
     <row r="1573">
@@ -17738,7 +17738,7 @@
         <v>1063</v>
       </c>
       <c r="C1573" t="n">
-        <v>175000</v>
+        <v>192500</v>
       </c>
     </row>
     <row r="1574">
@@ -17749,7 +17749,7 @@
         <v>1116</v>
       </c>
       <c r="C1574" t="n">
-        <v>113630</v>
+        <v>124993</v>
       </c>
     </row>
     <row r="1575">
@@ -17760,7 +17760,7 @@
         <v>941</v>
       </c>
       <c r="C1575" t="n">
-        <v>136770</v>
+        <v>150447</v>
       </c>
     </row>
     <row r="1576">
@@ -17771,7 +17771,7 @@
         <v>2141</v>
       </c>
       <c r="C1576" t="n">
-        <v>14580</v>
+        <v>16038</v>
       </c>
     </row>
     <row r="1577">
@@ -17782,7 +17782,7 @@
         <v>2463</v>
       </c>
       <c r="C1577" t="n">
-        <v>149920</v>
+        <v>164912</v>
       </c>
     </row>
     <row r="1578">
@@ -17793,7 +17793,7 @@
         <v>2325</v>
       </c>
       <c r="C1578" t="n">
-        <v>52440</v>
+        <v>57684</v>
       </c>
     </row>
     <row r="1579">
@@ -17837,7 +17837,7 @@
         <v>1890</v>
       </c>
       <c r="C1582" t="n">
-        <v>111470</v>
+        <v>122617</v>
       </c>
     </row>
     <row r="1583">
@@ -17848,7 +17848,7 @@
         <v>2639</v>
       </c>
       <c r="C1583" t="n">
-        <v>18210</v>
+        <v>20031</v>
       </c>
     </row>
     <row r="1584">
@@ -17859,7 +17859,7 @@
         <v>2682</v>
       </c>
       <c r="C1584" t="n">
-        <v>63630</v>
+        <v>69993</v>
       </c>
     </row>
     <row r="1585">
@@ -17867,10 +17867,10 @@
         <v>46296</v>
       </c>
       <c r="B1585" t="n">
-        <v>1142</v>
+        <v>2601</v>
       </c>
       <c r="C1585" t="n">
-        <v>208220</v>
+        <v>137500</v>
       </c>
     </row>
     <row r="1586">
@@ -17878,10 +17878,10 @@
         <v>46296</v>
       </c>
       <c r="B1586" t="n">
-        <v>628</v>
+        <v>1142</v>
       </c>
       <c r="C1586" t="n">
-        <v>0</v>
+        <v>229042</v>
       </c>
     </row>
     <row r="1587">
@@ -17889,7 +17889,7 @@
         <v>46296</v>
       </c>
       <c r="B1587" t="n">
-        <v>2046</v>
+        <v>628</v>
       </c>
       <c r="C1587" t="n">
         <v>0</v>
@@ -17900,7 +17900,7 @@
         <v>46296</v>
       </c>
       <c r="B1588" t="n">
-        <v>2189</v>
+        <v>2046</v>
       </c>
       <c r="C1588" t="n">
         <v>0</v>
@@ -17911,10 +17911,10 @@
         <v>46296</v>
       </c>
       <c r="B1589" t="n">
-        <v>2082</v>
+        <v>2189</v>
       </c>
       <c r="C1589" t="n">
-        <v>45450</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1590">
@@ -17922,10 +17922,10 @@
         <v>46296</v>
       </c>
       <c r="B1590" t="n">
-        <v>2276</v>
+        <v>2082</v>
       </c>
       <c r="C1590" t="n">
-        <v>90420</v>
+        <v>49995</v>
       </c>
     </row>
     <row r="1591">
@@ -17933,10 +17933,10 @@
         <v>46296</v>
       </c>
       <c r="B1591" t="n">
-        <v>2786</v>
+        <v>2276</v>
       </c>
       <c r="C1591" t="n">
-        <v>31810</v>
+        <v>99462</v>
       </c>
     </row>
     <row r="1592">
@@ -17944,10 +17944,10 @@
         <v>46296</v>
       </c>
       <c r="B1592" t="n">
-        <v>2816</v>
+        <v>2786</v>
       </c>
       <c r="C1592" t="n">
-        <v>59090</v>
+        <v>34991</v>
       </c>
     </row>
     <row r="1593">
@@ -17955,10 +17955,10 @@
         <v>46296</v>
       </c>
       <c r="B1593" t="n">
-        <v>1871</v>
+        <v>2816</v>
       </c>
       <c r="C1593" t="n">
-        <v>65230</v>
+        <v>64999</v>
       </c>
     </row>
     <row r="1594">
@@ -17966,10 +17966,10 @@
         <v>46296</v>
       </c>
       <c r="B1594" t="n">
-        <v>2345</v>
+        <v>1871</v>
       </c>
       <c r="C1594" t="n">
-        <v>29000</v>
+        <v>71753</v>
       </c>
     </row>
     <row r="1595">
@@ -17977,10 +17977,10 @@
         <v>46296</v>
       </c>
       <c r="B1595" t="n">
-        <v>2802</v>
+        <v>2345</v>
       </c>
       <c r="C1595" t="n">
-        <v>32630</v>
+        <v>31900</v>
       </c>
     </row>
     <row r="1596">
@@ -17988,10 +17988,10 @@
         <v>46296</v>
       </c>
       <c r="B1596" t="n">
-        <v>2090</v>
+        <v>2802</v>
       </c>
       <c r="C1596" t="n">
-        <v>18910</v>
+        <v>35893</v>
       </c>
     </row>
     <row r="1597">
@@ -17999,10 +17999,10 @@
         <v>46296</v>
       </c>
       <c r="B1597" t="n">
-        <v>2647</v>
+        <v>2090</v>
       </c>
       <c r="C1597" t="n">
-        <v>63750</v>
+        <v>20801</v>
       </c>
     </row>
     <row r="1598">
@@ -18010,10 +18010,10 @@
         <v>46296</v>
       </c>
       <c r="B1598" t="n">
-        <v>2365</v>
+        <v>2647</v>
       </c>
       <c r="C1598" t="n">
-        <v>45450</v>
+        <v>70125</v>
       </c>
     </row>
     <row r="1599">
@@ -18021,10 +18021,10 @@
         <v>46296</v>
       </c>
       <c r="B1599" t="n">
-        <v>766</v>
+        <v>2365</v>
       </c>
       <c r="C1599" t="n">
-        <v>31220</v>
+        <v>49995</v>
       </c>
     </row>
     <row r="1600">
@@ -18032,10 +18032,10 @@
         <v>46296</v>
       </c>
       <c r="B1600" t="n">
-        <v>2702</v>
+        <v>766</v>
       </c>
       <c r="C1600" t="n">
-        <v>37030</v>
+        <v>34342</v>
       </c>
     </row>
     <row r="1601">
@@ -18043,10 +18043,10 @@
         <v>46296</v>
       </c>
       <c r="B1601" t="n">
-        <v>20</v>
+        <v>2702</v>
       </c>
       <c r="C1601" t="n">
-        <v>204545.52</v>
+        <v>40733</v>
       </c>
     </row>
     <row r="1602">
@@ -18054,10 +18054,10 @@
         <v>46296</v>
       </c>
       <c r="B1602" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C1602" t="n">
-        <v>68181.84</v>
+        <v>225000.06</v>
       </c>
     </row>
     <row r="1603">
@@ -18065,10 +18065,10 @@
         <v>46296</v>
       </c>
       <c r="B1603" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C1603" t="n">
-        <v>180900</v>
+        <v>75000.02</v>
       </c>
     </row>
     <row r="1604">
@@ -18076,10 +18076,10 @@
         <v>46296</v>
       </c>
       <c r="B1604" t="n">
-        <v>2554</v>
+        <v>33</v>
       </c>
       <c r="C1604" t="n">
-        <v>0</v>
+        <v>198990</v>
       </c>
     </row>
     <row r="1605">
@@ -18087,10 +18087,10 @@
         <v>46296</v>
       </c>
       <c r="B1605" t="n">
-        <v>2561</v>
+        <v>2554</v>
       </c>
       <c r="C1605" t="n">
-        <v>17770</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1606">
@@ -18098,10 +18098,10 @@
         <v>46296</v>
       </c>
       <c r="B1606" t="n">
-        <v>934</v>
+        <v>2561</v>
       </c>
       <c r="C1606" t="n">
-        <v>0</v>
+        <v>19547</v>
       </c>
     </row>
     <row r="1607">
@@ -18109,10 +18109,10 @@
         <v>46296</v>
       </c>
       <c r="B1607" t="n">
-        <v>2772</v>
+        <v>934</v>
       </c>
       <c r="C1607" t="n">
-        <v>27270</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1608">
@@ -18120,10 +18120,10 @@
         <v>46296</v>
       </c>
       <c r="B1608" t="n">
-        <v>132</v>
+        <v>2772</v>
       </c>
       <c r="C1608" t="n">
-        <v>159090.92</v>
+        <v>29997</v>
       </c>
     </row>
     <row r="1609">
@@ -18131,10 +18131,10 @@
         <v>46296</v>
       </c>
       <c r="B1609" t="n">
-        <v>1433</v>
+        <v>132</v>
       </c>
       <c r="C1609" t="n">
-        <v>0</v>
+        <v>175000.01</v>
       </c>
     </row>
     <row r="1610">
@@ -18145,7 +18145,7 @@
         <v>2834</v>
       </c>
       <c r="C1610" t="n">
-        <v>16940</v>
+        <v>18634</v>
       </c>
     </row>
     <row r="1611">
@@ -18156,7 +18156,7 @@
         <v>2394</v>
       </c>
       <c r="C1611" t="n">
-        <v>51570</v>
+        <v>56727</v>
       </c>
     </row>
     <row r="1612">
@@ -18167,7 +18167,7 @@
         <v>2567</v>
       </c>
       <c r="C1612" t="n">
-        <v>45450</v>
+        <v>49995</v>
       </c>
     </row>
     <row r="1613">
@@ -18178,7 +18178,7 @@
         <v>952</v>
       </c>
       <c r="C1613" t="n">
-        <v>45450</v>
+        <v>49995</v>
       </c>
     </row>
     <row r="1614">
@@ -18189,7 +18189,7 @@
         <v>1539</v>
       </c>
       <c r="C1614" t="n">
-        <v>77270</v>
+        <v>84997</v>
       </c>
     </row>
     <row r="1615">
@@ -18200,7 +18200,7 @@
         <v>793</v>
       </c>
       <c r="C1615" t="n">
-        <v>18910</v>
+        <v>20801</v>
       </c>
     </row>
     <row r="1616">
@@ -18211,7 +18211,7 @@
         <v>794</v>
       </c>
       <c r="C1616" t="n">
-        <v>18910</v>
+        <v>20801</v>
       </c>
     </row>
     <row r="1617">
@@ -18222,7 +18222,7 @@
         <v>2838</v>
       </c>
       <c r="C1617" t="n">
-        <v>27272.76</v>
+        <v>30000.03</v>
       </c>
     </row>
     <row r="1618">
@@ -18233,7 +18233,7 @@
         <v>2223</v>
       </c>
       <c r="C1618" t="n">
-        <v>53230</v>
+        <v>58553</v>
       </c>
     </row>
     <row r="1619">
@@ -18244,7 +18244,7 @@
         <v>2547</v>
       </c>
       <c r="C1619" t="n">
-        <v>15400</v>
+        <v>16940</v>
       </c>
     </row>
     <row r="1620">
@@ -18255,7 +18255,7 @@
         <v>2762</v>
       </c>
       <c r="C1620" t="n">
-        <v>37030</v>
+        <v>40733</v>
       </c>
     </row>
     <row r="1621">
@@ -18266,7 +18266,7 @@
         <v>2550</v>
       </c>
       <c r="C1621" t="n">
-        <v>17770</v>
+        <v>19547</v>
       </c>
     </row>
     <row r="1622">
@@ -18277,7 +18277,7 @@
         <v>2627</v>
       </c>
       <c r="C1622" t="n">
-        <v>17770</v>
+        <v>19547</v>
       </c>
     </row>
     <row r="1623">
@@ -18299,7 +18299,7 @@
         <v>749</v>
       </c>
       <c r="C1624" t="n">
-        <v>37030</v>
+        <v>40733</v>
       </c>
     </row>
     <row r="1625">
@@ -18310,7 +18310,7 @@
         <v>2549</v>
       </c>
       <c r="C1625" t="n">
-        <v>17770</v>
+        <v>19547</v>
       </c>
     </row>
     <row r="1626">
@@ -18321,7 +18321,7 @@
         <v>2649</v>
       </c>
       <c r="C1626" t="n">
-        <v>17770</v>
+        <v>19547</v>
       </c>
     </row>
     <row r="1627">
@@ -18332,7 +18332,7 @@
         <v>2258</v>
       </c>
       <c r="C1627" t="n">
-        <v>36360</v>
+        <v>39996</v>
       </c>
     </row>
     <row r="1628">
@@ -18343,7 +18343,7 @@
         <v>2744</v>
       </c>
       <c r="C1628" t="n">
-        <v>27270</v>
+        <v>29997</v>
       </c>
     </row>
     <row r="1629">
@@ -18354,7 +18354,7 @@
         <v>452</v>
       </c>
       <c r="C1629" t="n">
-        <v>128630</v>
+        <v>141493</v>
       </c>
     </row>
     <row r="1630">
@@ -18376,7 +18376,7 @@
         <v>2653</v>
       </c>
       <c r="C1631" t="n">
-        <v>27270</v>
+        <v>29997</v>
       </c>
     </row>
     <row r="1632">
@@ -18409,7 +18409,7 @@
         <v>2742</v>
       </c>
       <c r="C1634" t="n">
-        <v>9090</v>
+        <v>9999</v>
       </c>
     </row>
     <row r="1635">
@@ -18420,7 +18420,7 @@
         <v>1499</v>
       </c>
       <c r="C1635" t="n">
-        <v>40900</v>
+        <v>44990</v>
       </c>
     </row>
     <row r="1636">
@@ -18431,7 +18431,7 @@
         <v>2261</v>
       </c>
       <c r="C1636" t="n">
-        <v>81810</v>
+        <v>89991</v>
       </c>
     </row>
     <row r="1637">
@@ -18442,7 +18442,7 @@
         <v>1324</v>
       </c>
       <c r="C1637" t="n">
-        <v>127270</v>
+        <v>139997</v>
       </c>
     </row>
     <row r="1638">
@@ -18453,7 +18453,7 @@
         <v>2709</v>
       </c>
       <c r="C1638" t="n">
-        <v>81810</v>
+        <v>89991</v>
       </c>
     </row>
     <row r="1639">
@@ -18464,7 +18464,7 @@
         <v>1137</v>
       </c>
       <c r="C1639" t="n">
-        <v>290900</v>
+        <v>319990</v>
       </c>
     </row>
     <row r="1640">
@@ -18475,7 +18475,7 @@
         <v>2440</v>
       </c>
       <c r="C1640" t="n">
-        <v>36360</v>
+        <v>39996</v>
       </c>
     </row>
     <row r="1641">
@@ -18486,7 +18486,7 @@
         <v>429</v>
       </c>
       <c r="C1641" t="n">
-        <v>172720</v>
+        <v>189992</v>
       </c>
     </row>
     <row r="1642">
@@ -18497,7 +18497,7 @@
         <v>2114</v>
       </c>
       <c r="C1642" t="n">
-        <v>77330</v>
+        <v>85063</v>
       </c>
     </row>
     <row r="1643">
@@ -18508,7 +18508,7 @@
         <v>2211</v>
       </c>
       <c r="C1643" t="n">
-        <v>109470</v>
+        <v>120417</v>
       </c>
     </row>
     <row r="1644">
@@ -18519,7 +18519,7 @@
         <v>1108</v>
       </c>
       <c r="C1644" t="n">
-        <v>139260</v>
+        <v>153186</v>
       </c>
     </row>
     <row r="1645">
@@ -18530,7 +18530,7 @@
         <v>2695</v>
       </c>
       <c r="C1645" t="n">
-        <v>21990</v>
+        <v>24189</v>
       </c>
     </row>
     <row r="1646">
@@ -18541,7 +18541,7 @@
         <v>1289</v>
       </c>
       <c r="C1646" t="n">
-        <v>125000</v>
+        <v>137500</v>
       </c>
     </row>
     <row r="1647">
@@ -18552,7 +18552,7 @@
         <v>2789</v>
       </c>
       <c r="C1647" t="n">
-        <v>81818.28</v>
+        <v>90000.09</v>
       </c>
     </row>
     <row r="1648">
@@ -18563,7 +18563,7 @@
         <v>2197</v>
       </c>
       <c r="C1648" t="n">
-        <v>97727.36</v>
+        <v>107500.08</v>
       </c>
     </row>
     <row r="1649">
@@ -18574,7 +18574,7 @@
         <v>947</v>
       </c>
       <c r="C1649" t="n">
-        <v>201580</v>
+        <v>221738</v>
       </c>
     </row>
     <row r="1650">
@@ -18585,7 +18585,7 @@
         <v>2279</v>
       </c>
       <c r="C1650" t="n">
-        <v>111330</v>
+        <v>122463</v>
       </c>
     </row>
     <row r="1651">
@@ -18596,7 +18596,7 @@
         <v>1465</v>
       </c>
       <c r="C1651" t="n">
-        <v>175000</v>
+        <v>192500</v>
       </c>
     </row>
     <row r="1652">
@@ -18607,7 +18607,7 @@
         <v>2651</v>
       </c>
       <c r="C1652" t="n">
-        <v>77270</v>
+        <v>84997</v>
       </c>
     </row>
     <row r="1653">
@@ -18618,7 +18618,7 @@
         <v>42</v>
       </c>
       <c r="C1653" t="n">
-        <v>866360</v>
+        <v>952996</v>
       </c>
     </row>
     <row r="1654">
@@ -18629,7 +18629,7 @@
         <v>949</v>
       </c>
       <c r="C1654" t="n">
-        <v>45210</v>
+        <v>49731</v>
       </c>
     </row>
     <row r="1655">
@@ -18640,7 +18640,7 @@
         <v>2606</v>
       </c>
       <c r="C1655" t="n">
-        <v>116700</v>
+        <v>128370</v>
       </c>
     </row>
     <row r="1656">
@@ -18651,7 +18651,7 @@
         <v>2249</v>
       </c>
       <c r="C1656" t="n">
-        <v>99150</v>
+        <v>109065</v>
       </c>
     </row>
     <row r="1657">
@@ -18695,7 +18695,7 @@
         <v>2045</v>
       </c>
       <c r="C1660" t="n">
-        <v>144760</v>
+        <v>159236</v>
       </c>
     </row>
     <row r="1661">
@@ -18706,7 +18706,7 @@
         <v>2663</v>
       </c>
       <c r="C1661" t="n">
-        <v>125000</v>
+        <v>137500</v>
       </c>
     </row>
     <row r="1662">
@@ -18728,7 +18728,7 @@
         <v>2854</v>
       </c>
       <c r="C1663" t="n">
-        <v>18180</v>
+        <v>19998</v>
       </c>
     </row>
     <row r="1664">
@@ -18750,7 +18750,7 @@
         <v>2341</v>
       </c>
       <c r="C1665" t="n">
-        <v>79500</v>
+        <v>87450</v>
       </c>
     </row>
     <row r="1666">
@@ -18761,7 +18761,7 @@
         <v>2637</v>
       </c>
       <c r="C1666" t="n">
-        <v>29000</v>
+        <v>31900</v>
       </c>
     </row>
     <row r="1667">
@@ -18772,7 +18772,7 @@
         <v>2492</v>
       </c>
       <c r="C1667" t="n">
-        <v>45530</v>
+        <v>50083</v>
       </c>
     </row>
     <row r="1668">
@@ -18783,7 +18783,7 @@
         <v>2548</v>
       </c>
       <c r="C1668" t="n">
-        <v>17770</v>
+        <v>19547</v>
       </c>
     </row>
     <row r="1669">
@@ -18794,7 +18794,7 @@
         <v>351</v>
       </c>
       <c r="C1669" t="n">
-        <v>96810</v>
+        <v>106491</v>
       </c>
     </row>
     <row r="1670">
@@ -18827,7 +18827,7 @@
         <v>2757</v>
       </c>
       <c r="C1672" t="n">
-        <v>36360</v>
+        <v>39996</v>
       </c>
     </row>
     <row r="1673">
@@ -18838,7 +18838,7 @@
         <v>2815</v>
       </c>
       <c r="C1673" t="n">
-        <v>27270</v>
+        <v>29997</v>
       </c>
     </row>
     <row r="1674">
@@ -18849,7 +18849,7 @@
         <v>2323</v>
       </c>
       <c r="C1674" t="n">
-        <v>31220</v>
+        <v>34342</v>
       </c>
     </row>
     <row r="1675">
@@ -18860,7 +18860,7 @@
         <v>2310</v>
       </c>
       <c r="C1675" t="n">
-        <v>31220</v>
+        <v>34342</v>
       </c>
     </row>
     <row r="1676">
@@ -18871,7 +18871,7 @@
         <v>2145</v>
       </c>
       <c r="C1676" t="n">
-        <v>45450</v>
+        <v>49995</v>
       </c>
     </row>
     <row r="1677">
@@ -18882,7 +18882,7 @@
         <v>2501</v>
       </c>
       <c r="C1677" t="n">
-        <v>37030</v>
+        <v>40733</v>
       </c>
     </row>
     <row r="1678">
@@ -18893,7 +18893,7 @@
         <v>2546</v>
       </c>
       <c r="C1678" t="n">
-        <v>17770</v>
+        <v>19547</v>
       </c>
     </row>
     <row r="1679">
@@ -18904,7 +18904,7 @@
         <v>716</v>
       </c>
       <c r="C1679" t="n">
-        <v>58260</v>
+        <v>64086</v>
       </c>
     </row>
     <row r="1680">
@@ -18915,7 +18915,7 @@
         <v>2758</v>
       </c>
       <c r="C1680" t="n">
-        <v>27270</v>
+        <v>29997</v>
       </c>
     </row>
     <row r="1681">
@@ -18926,7 +18926,7 @@
         <v>400</v>
       </c>
       <c r="C1681" t="n">
-        <v>81810</v>
+        <v>89991</v>
       </c>
     </row>
     <row r="1682">
@@ -18937,7 +18937,7 @@
         <v>6</v>
       </c>
       <c r="C1682" t="n">
-        <v>22727.36</v>
+        <v>25000.08</v>
       </c>
     </row>
     <row r="1683">
@@ -18970,7 +18970,7 @@
         <v>1259</v>
       </c>
       <c r="C1685" t="n">
-        <v>50000</v>
+        <v>55000</v>
       </c>
     </row>
     <row r="1686">
@@ -18981,7 +18981,7 @@
         <v>571</v>
       </c>
       <c r="C1686" t="n">
-        <v>470454.6</v>
+        <v>517500.05</v>
       </c>
     </row>
     <row r="1687">
@@ -18992,7 +18992,7 @@
         <v>703</v>
       </c>
       <c r="C1687" t="n">
-        <v>113630</v>
+        <v>124993</v>
       </c>
     </row>
     <row r="1688">
@@ -19014,7 +19014,7 @@
         <v>2833</v>
       </c>
       <c r="C1689" t="n">
-        <v>36360</v>
+        <v>39996</v>
       </c>
     </row>
     <row r="1690">
@@ -19025,7 +19025,7 @@
         <v>1007</v>
       </c>
       <c r="C1690" t="n">
-        <v>90909.2</v>
+        <v>100000.1</v>
       </c>
     </row>
     <row r="1691">
@@ -19036,7 +19036,7 @@
         <v>2687</v>
       </c>
       <c r="C1691" t="n">
-        <v>36360</v>
+        <v>39996</v>
       </c>
     </row>
     <row r="1692">
@@ -19047,7 +19047,7 @@
         <v>2824</v>
       </c>
       <c r="C1692" t="n">
-        <v>51320</v>
+        <v>56452</v>
       </c>
     </row>
     <row r="1693">
@@ -19058,7 +19058,7 @@
         <v>2730</v>
       </c>
       <c r="C1693" t="n">
-        <v>40900</v>
+        <v>44990</v>
       </c>
     </row>
     <row r="1694">
@@ -19069,7 +19069,7 @@
         <v>2718</v>
       </c>
       <c r="C1694" t="n">
-        <v>59090</v>
+        <v>64999</v>
       </c>
     </row>
     <row r="1695">
@@ -19080,7 +19080,7 @@
         <v>2750</v>
       </c>
       <c r="C1695" t="n">
-        <v>13630</v>
+        <v>14993</v>
       </c>
     </row>
     <row r="1696">
@@ -19091,7 +19091,7 @@
         <v>854</v>
       </c>
       <c r="C1696" t="n">
-        <v>63630</v>
+        <v>69993</v>
       </c>
     </row>
     <row r="1697">
@@ -19102,7 +19102,7 @@
         <v>2794</v>
       </c>
       <c r="C1697" t="n">
-        <v>54540</v>
+        <v>59994</v>
       </c>
     </row>
     <row r="1698">
@@ -19113,7 +19113,7 @@
         <v>1374</v>
       </c>
       <c r="C1698" t="n">
-        <v>90900</v>
+        <v>99990</v>
       </c>
     </row>
     <row r="1699">
@@ -19124,7 +19124,7 @@
         <v>2488</v>
       </c>
       <c r="C1699" t="n">
-        <v>45450</v>
+        <v>49995</v>
       </c>
     </row>
     <row r="1700">
@@ -19135,7 +19135,7 @@
         <v>363</v>
       </c>
       <c r="C1700" t="n">
-        <v>136360</v>
+        <v>149996</v>
       </c>
     </row>
     <row r="1701">
@@ -19146,7 +19146,7 @@
         <v>2655</v>
       </c>
       <c r="C1701" t="n">
-        <v>50000</v>
+        <v>55000</v>
       </c>
     </row>
     <row r="1702">
@@ -19157,7 +19157,7 @@
         <v>1873</v>
       </c>
       <c r="C1702" t="n">
-        <v>145450</v>
+        <v>159995</v>
       </c>
     </row>
     <row r="1703">
@@ -19168,7 +19168,7 @@
         <v>2635</v>
       </c>
       <c r="C1703" t="n">
-        <v>59090</v>
+        <v>64999</v>
       </c>
     </row>
     <row r="1704">
@@ -19179,7 +19179,7 @@
         <v>1658</v>
       </c>
       <c r="C1704" t="n">
-        <v>69540</v>
+        <v>76494</v>
       </c>
     </row>
     <row r="1705">
@@ -19190,7 +19190,7 @@
         <v>2069</v>
       </c>
       <c r="C1705" t="n">
-        <v>90909.2</v>
+        <v>100000.1</v>
       </c>
     </row>
     <row r="1706">
@@ -19201,7 +19201,7 @@
         <v>2081</v>
       </c>
       <c r="C1706" t="n">
-        <v>68180</v>
+        <v>74998</v>
       </c>
     </row>
     <row r="1707">
@@ -19212,7 +19212,7 @@
         <v>2124</v>
       </c>
       <c r="C1707" t="n">
-        <v>159090</v>
+        <v>174999</v>
       </c>
     </row>
     <row r="1708">
@@ -19223,7 +19223,7 @@
         <v>636</v>
       </c>
       <c r="C1708" t="n">
-        <v>113630</v>
+        <v>124993</v>
       </c>
     </row>
     <row r="1709">
@@ -19234,7 +19234,7 @@
         <v>2803</v>
       </c>
       <c r="C1709" t="n">
-        <v>54540</v>
+        <v>59994</v>
       </c>
     </row>
     <row r="1710">
@@ -19245,7 +19245,7 @@
         <v>2163</v>
       </c>
       <c r="C1710" t="n">
-        <v>81810</v>
+        <v>89991</v>
       </c>
     </row>
     <row r="1711">
@@ -19256,7 +19256,7 @@
         <v>1466</v>
       </c>
       <c r="C1711" t="n">
-        <v>184090</v>
+        <v>202499</v>
       </c>
     </row>
     <row r="1712">
@@ -19267,7 +19267,7 @@
         <v>2133</v>
       </c>
       <c r="C1712" t="n">
-        <v>159090.92</v>
+        <v>175000.01</v>
       </c>
     </row>
     <row r="1713">
@@ -19278,7 +19278,7 @@
         <v>2431</v>
       </c>
       <c r="C1713" t="n">
-        <v>68180</v>
+        <v>74998</v>
       </c>
     </row>
     <row r="1714">
@@ -19289,7 +19289,7 @@
         <v>535</v>
       </c>
       <c r="C1714" t="n">
-        <v>161900</v>
+        <v>178090</v>
       </c>
     </row>
     <row r="1715">
@@ -19300,7 +19300,7 @@
         <v>2790</v>
       </c>
       <c r="C1715" t="n">
-        <v>28710</v>
+        <v>31581</v>
       </c>
     </row>
     <row r="1716">
@@ -19311,7 +19311,7 @@
         <v>2442</v>
       </c>
       <c r="C1716" t="n">
-        <v>117720</v>
+        <v>129492</v>
       </c>
     </row>
     <row r="1717">
@@ -19322,7 +19322,7 @@
         <v>2376</v>
       </c>
       <c r="C1717" t="n">
-        <v>500000</v>
+        <v>550000</v>
       </c>
     </row>
     <row r="1718">
@@ -19333,7 +19333,7 @@
         <v>2768</v>
       </c>
       <c r="C1718" t="n">
-        <v>137570</v>
+        <v>151327</v>
       </c>
     </row>
     <row r="1719">
@@ -19344,7 +19344,7 @@
         <v>2491</v>
       </c>
       <c r="C1719" t="n">
-        <v>110390</v>
+        <v>121429</v>
       </c>
     </row>
     <row r="1720">
@@ -19355,7 +19355,7 @@
         <v>2799</v>
       </c>
       <c r="C1720" t="n">
-        <v>49690</v>
+        <v>54659</v>
       </c>
     </row>
     <row r="1721">
@@ -19388,7 +19388,7 @@
         <v>1317</v>
       </c>
       <c r="C1723" t="n">
-        <v>143181.84</v>
+        <v>157500.02</v>
       </c>
     </row>
     <row r="1724">
@@ -19399,7 +19399,7 @@
         <v>2822</v>
       </c>
       <c r="C1724" t="n">
-        <v>72727.36</v>
+        <v>80000.08</v>
       </c>
     </row>
     <row r="1725">
@@ -19410,7 +19410,7 @@
         <v>1117</v>
       </c>
       <c r="C1725" t="n">
-        <v>181870</v>
+        <v>200057</v>
       </c>
     </row>
     <row r="1726">
@@ -19421,7 +19421,7 @@
         <v>1299</v>
       </c>
       <c r="C1726" t="n">
-        <v>239790</v>
+        <v>263769</v>
       </c>
     </row>
     <row r="1727">
@@ -19432,7 +19432,7 @@
         <v>477</v>
       </c>
       <c r="C1727" t="n">
-        <v>98820</v>
+        <v>108702</v>
       </c>
     </row>
     <row r="1728">
@@ -19443,7 +19443,7 @@
         <v>530</v>
       </c>
       <c r="C1728" t="n">
-        <v>136360</v>
+        <v>149996</v>
       </c>
     </row>
     <row r="1729">
@@ -19454,7 +19454,7 @@
         <v>953</v>
       </c>
       <c r="C1729" t="n">
-        <v>313630</v>
+        <v>344993</v>
       </c>
     </row>
     <row r="1730">
@@ -19465,7 +19465,7 @@
         <v>610</v>
       </c>
       <c r="C1730" t="n">
-        <v>373540</v>
+        <v>410894</v>
       </c>
     </row>
     <row r="1731">
@@ -19476,7 +19476,7 @@
         <v>2792</v>
       </c>
       <c r="C1731" t="n">
-        <v>93810</v>
+        <v>103191</v>
       </c>
     </row>
     <row r="1732">
@@ -19553,7 +19553,7 @@
         <v>1075</v>
       </c>
       <c r="C1738" t="n">
-        <v>208630</v>
+        <v>229493</v>
       </c>
     </row>
     <row r="1739">
@@ -19564,7 +19564,7 @@
         <v>131</v>
       </c>
       <c r="C1739" t="n">
-        <v>189090</v>
+        <v>207999</v>
       </c>
     </row>
     <row r="1740">
@@ -19575,7 +19575,7 @@
         <v>2667</v>
       </c>
       <c r="C1740" t="n">
-        <v>20770</v>
+        <v>22847</v>
       </c>
     </row>
     <row r="1741">
@@ -19586,7 +19586,7 @@
         <v>2330</v>
       </c>
       <c r="C1741" t="n">
-        <v>40430</v>
+        <v>44473</v>
       </c>
     </row>
     <row r="1742">
@@ -19608,7 +19608,7 @@
         <v>2577</v>
       </c>
       <c r="C1743" t="n">
-        <v>40530</v>
+        <v>44583</v>
       </c>
     </row>
     <row r="1744">
@@ -19619,7 +19619,7 @@
         <v>2510</v>
       </c>
       <c r="C1744" t="n">
-        <v>287840</v>
+        <v>316624</v>
       </c>
     </row>
     <row r="1745">
@@ -19641,7 +19641,7 @@
         <v>2850</v>
       </c>
       <c r="C1746" t="n">
-        <v>27270</v>
+        <v>29997</v>
       </c>
     </row>
     <row r="1747">
@@ -19663,7 +19663,7 @@
         <v>2745</v>
       </c>
       <c r="C1748" t="n">
-        <v>50000</v>
+        <v>55000</v>
       </c>
     </row>
     <row r="1749">
@@ -19674,7 +19674,7 @@
         <v>2817</v>
       </c>
       <c r="C1749" t="n">
-        <v>27270</v>
+        <v>29997</v>
       </c>
     </row>
     <row r="1750">
@@ -19685,7 +19685,7 @@
         <v>2784</v>
       </c>
       <c r="C1750" t="n">
-        <v>18910</v>
+        <v>20801</v>
       </c>
     </row>
     <row r="1751">
@@ -19696,7 +19696,7 @@
         <v>626</v>
       </c>
       <c r="C1751" t="n">
-        <v>785370</v>
+        <v>863907</v>
       </c>
     </row>
     <row r="1752">
@@ -19707,7 +19707,7 @@
         <v>925</v>
       </c>
       <c r="C1752" t="n">
-        <v>36260</v>
+        <v>39886</v>
       </c>
     </row>
     <row r="1753">
@@ -19718,7 +19718,7 @@
         <v>2586</v>
       </c>
       <c r="C1753" t="n">
-        <v>18910</v>
+        <v>20801</v>
       </c>
     </row>
     <row r="1754">
@@ -19729,7 +19729,7 @@
         <v>966</v>
       </c>
       <c r="C1754" t="n">
-        <v>37030</v>
+        <v>40733</v>
       </c>
     </row>
     <row r="1755">
@@ -19740,7 +19740,7 @@
         <v>2557</v>
       </c>
       <c r="C1755" t="n">
-        <v>17770</v>
+        <v>19547</v>
       </c>
     </row>
     <row r="1756">
@@ -19751,7 +19751,7 @@
         <v>14</v>
       </c>
       <c r="C1756" t="n">
-        <v>204540</v>
+        <v>224994</v>
       </c>
     </row>
     <row r="1757">
@@ -19762,7 +19762,7 @@
         <v>2798</v>
       </c>
       <c r="C1757" t="n">
-        <v>27270</v>
+        <v>29997</v>
       </c>
     </row>
     <row r="1758">
@@ -19784,7 +19784,7 @@
         <v>522</v>
       </c>
       <c r="C1759" t="n">
-        <v>90909.2</v>
+        <v>100000.1</v>
       </c>
     </row>
     <row r="1760">
@@ -19806,7 +19806,7 @@
         <v>2819</v>
       </c>
       <c r="C1761" t="n">
-        <v>27270</v>
+        <v>29997</v>
       </c>
     </row>
     <row r="1762">
@@ -19817,7 +19817,7 @@
         <v>2266</v>
       </c>
       <c r="C1762" t="n">
-        <v>36360</v>
+        <v>39996</v>
       </c>
     </row>
     <row r="1763">
@@ -19850,7 +19850,7 @@
         <v>2795</v>
       </c>
       <c r="C1765" t="n">
-        <v>27270</v>
+        <v>29997</v>
       </c>
     </row>
     <row r="1766">
@@ -19861,7 +19861,7 @@
         <v>2722</v>
       </c>
       <c r="C1766" t="n">
-        <v>9090</v>
+        <v>9999</v>
       </c>
     </row>
     <row r="1767">
@@ -19872,7 +19872,7 @@
         <v>951</v>
       </c>
       <c r="C1767" t="n">
-        <v>52270</v>
+        <v>57497</v>
       </c>
     </row>
     <row r="1768">
@@ -19883,7 +19883,7 @@
         <v>1020</v>
       </c>
       <c r="C1768" t="n">
-        <v>45450</v>
+        <v>49995</v>
       </c>
     </row>
     <row r="1769">
@@ -19894,7 +19894,7 @@
         <v>1853</v>
       </c>
       <c r="C1769" t="n">
-        <v>54540</v>
+        <v>59994</v>
       </c>
     </row>
     <row r="1770">
@@ -19905,7 +19905,7 @@
         <v>1327</v>
       </c>
       <c r="C1770" t="n">
-        <v>31810</v>
+        <v>34991</v>
       </c>
     </row>
     <row r="1771">
@@ -19916,7 +19916,7 @@
         <v>2842</v>
       </c>
       <c r="C1771" t="n">
-        <v>81810</v>
+        <v>89991</v>
       </c>
     </row>
     <row r="1772">
@@ -19927,7 +19927,7 @@
         <v>2831</v>
       </c>
       <c r="C1772" t="n">
-        <v>27270</v>
+        <v>29997</v>
       </c>
     </row>
     <row r="1773">
@@ -19938,7 +19938,7 @@
         <v>818</v>
       </c>
       <c r="C1773" t="n">
-        <v>181810</v>
+        <v>199991</v>
       </c>
     </row>
     <row r="1774">
@@ -19949,7 +19949,7 @@
         <v>1501</v>
       </c>
       <c r="C1774" t="n">
-        <v>45450</v>
+        <v>49995</v>
       </c>
     </row>
     <row r="1775">
@@ -19960,7 +19960,7 @@
         <v>1869</v>
       </c>
       <c r="C1775" t="n">
-        <v>110900</v>
+        <v>121990</v>
       </c>
     </row>
     <row r="1776">
@@ -19971,7 +19971,7 @@
         <v>1996</v>
       </c>
       <c r="C1776" t="n">
-        <v>113636.44</v>
+        <v>125000.07</v>
       </c>
     </row>
     <row r="1777">
@@ -19982,7 +19982,7 @@
         <v>2462</v>
       </c>
       <c r="C1777" t="n">
-        <v>25743.28</v>
+        <v>28317.59</v>
       </c>
     </row>
     <row r="1778">
@@ -19993,7 +19993,7 @@
         <v>2696</v>
       </c>
       <c r="C1778" t="n">
-        <v>97480</v>
+        <v>107228</v>
       </c>
     </row>
     <row r="1779">
@@ -20004,7 +20004,7 @@
         <v>2698</v>
       </c>
       <c r="C1779" t="n">
-        <v>49960</v>
+        <v>54956</v>
       </c>
     </row>
     <row r="1780">
@@ -20026,7 +20026,7 @@
         <v>2828</v>
       </c>
       <c r="C1781" t="n">
-        <v>27272.76</v>
+        <v>30000.03</v>
       </c>
     </row>
     <row r="1782">
@@ -20037,7 +20037,7 @@
         <v>2843</v>
       </c>
       <c r="C1782" t="n">
-        <v>31810</v>
+        <v>34991</v>
       </c>
     </row>
     <row r="1783">
@@ -20048,7 +20048,7 @@
         <v>619</v>
       </c>
       <c r="C1783" t="n">
-        <v>142500</v>
+        <v>156750</v>
       </c>
     </row>
     <row r="1784">
@@ -20059,7 +20059,7 @@
         <v>1478</v>
       </c>
       <c r="C1784" t="n">
-        <v>249380</v>
+        <v>274318</v>
       </c>
     </row>
     <row r="1785">
@@ -20070,7 +20070,7 @@
         <v>2026</v>
       </c>
       <c r="C1785" t="n">
-        <v>110180</v>
+        <v>121198</v>
       </c>
     </row>
     <row r="1786">
@@ -20081,7 +20081,7 @@
         <v>663</v>
       </c>
       <c r="C1786" t="n">
-        <v>117720</v>
+        <v>129492</v>
       </c>
     </row>
     <row r="1787">
@@ -20092,7 +20092,7 @@
         <v>285</v>
       </c>
       <c r="C1787" t="n">
-        <v>249380</v>
+        <v>274318</v>
       </c>
     </row>
     <row r="1788">
@@ -20103,7 +20103,7 @@
         <v>424</v>
       </c>
       <c r="C1788" t="n">
-        <v>106870</v>
+        <v>117557</v>
       </c>
     </row>
     <row r="1789">
@@ -20114,7 +20114,7 @@
         <v>451</v>
       </c>
       <c r="C1789" t="n">
-        <v>110450</v>
+        <v>121495</v>
       </c>
     </row>
     <row r="1790">
@@ -20125,7 +20125,7 @@
         <v>629</v>
       </c>
       <c r="C1790" t="n">
-        <v>206360</v>
+        <v>226996</v>
       </c>
     </row>
     <row r="1791">
@@ -20136,7 +20136,7 @@
         <v>2657</v>
       </c>
       <c r="C1791" t="n">
-        <v>35990</v>
+        <v>39589</v>
       </c>
     </row>
     <row r="1792">
@@ -20147,7 +20147,7 @@
         <v>1254</v>
       </c>
       <c r="C1792" t="n">
-        <v>88270</v>
+        <v>97097</v>
       </c>
     </row>
     <row r="1793">
@@ -20158,7 +20158,7 @@
         <v>2402</v>
       </c>
       <c r="C1793" t="n">
-        <v>222020</v>
+        <v>244222</v>
       </c>
     </row>
     <row r="1794">
@@ -20169,7 +20169,7 @@
         <v>2413</v>
       </c>
       <c r="C1794" t="n">
-        <v>62650</v>
+        <v>68915</v>
       </c>
     </row>
     <row r="1795">
@@ -20180,7 +20180,7 @@
         <v>1450</v>
       </c>
       <c r="C1795" t="n">
-        <v>162270</v>
+        <v>178497</v>
       </c>
     </row>
     <row r="1796">
@@ -20202,7 +20202,7 @@
         <v>2671</v>
       </c>
       <c r="C1797" t="n">
-        <v>36360</v>
+        <v>39996</v>
       </c>
     </row>
     <row r="1798">
@@ -20213,7 +20213,7 @@
         <v>2568</v>
       </c>
       <c r="C1798" t="n">
-        <v>72930</v>
+        <v>80223</v>
       </c>
     </row>
     <row r="1799">
@@ -20224,7 +20224,7 @@
         <v>2146</v>
       </c>
       <c r="C1799" t="n">
-        <v>88310</v>
+        <v>97141</v>
       </c>
     </row>
     <row r="1800">
@@ -20235,7 +20235,7 @@
         <v>2753</v>
       </c>
       <c r="C1800" t="n">
-        <v>34090</v>
+        <v>37499</v>
       </c>
     </row>
     <row r="1801">
@@ -20246,7 +20246,7 @@
         <v>744</v>
       </c>
       <c r="C1801" t="n">
-        <v>18910</v>
+        <v>20801</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:01:50
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -15560,7 +15560,7 @@
         <v>2853</v>
       </c>
       <c r="C1375" t="n">
-        <v>40733</v>
+        <v>44436</v>
       </c>
     </row>
     <row r="1376">
@@ -15571,7 +15571,7 @@
         <v>2245</v>
       </c>
       <c r="C1376" t="n">
-        <v>110704</v>
+        <v>120768</v>
       </c>
     </row>
     <row r="1377">
@@ -15582,7 +15582,7 @@
         <v>2251</v>
       </c>
       <c r="C1377" t="n">
-        <v>99990</v>
+        <v>109080</v>
       </c>
     </row>
     <row r="1378">
@@ -15593,7 +15593,7 @@
         <v>664</v>
       </c>
       <c r="C1378" t="n">
-        <v>130999</v>
+        <v>142908</v>
       </c>
     </row>
     <row r="1379">
@@ -15604,7 +15604,7 @@
         <v>2472</v>
       </c>
       <c r="C1379" t="n">
-        <v>26466</v>
+        <v>28872</v>
       </c>
     </row>
     <row r="1380">
@@ -15615,7 +15615,7 @@
         <v>1456</v>
       </c>
       <c r="C1380" t="n">
-        <v>398992</v>
+        <v>435264</v>
       </c>
     </row>
     <row r="1381">
@@ -15626,7 +15626,7 @@
         <v>1585</v>
       </c>
       <c r="C1381" t="n">
-        <v>90497</v>
+        <v>98724</v>
       </c>
     </row>
     <row r="1382">
@@ -15670,7 +15670,7 @@
         <v>1907</v>
       </c>
       <c r="C1385" t="n">
-        <v>275264</v>
+        <v>300288</v>
       </c>
     </row>
     <row r="1386">
@@ -15703,7 +15703,7 @@
         <v>2659</v>
       </c>
       <c r="C1388" t="n">
-        <v>61501</v>
+        <v>67092</v>
       </c>
     </row>
     <row r="1389">
@@ -15714,7 +15714,7 @@
         <v>2583</v>
       </c>
       <c r="C1389" t="n">
-        <v>20801</v>
+        <v>22692</v>
       </c>
     </row>
     <row r="1390">
@@ -15725,7 +15725,7 @@
         <v>2692</v>
       </c>
       <c r="C1390" t="n">
-        <v>35000.09</v>
+        <v>38181.9</v>
       </c>
     </row>
     <row r="1391">
@@ -15736,7 +15736,7 @@
         <v>2691</v>
       </c>
       <c r="C1391" t="n">
-        <v>61092.09</v>
+        <v>66645.89999999999</v>
       </c>
     </row>
     <row r="1392">
@@ -15747,7 +15747,7 @@
         <v>931</v>
       </c>
       <c r="C1392" t="n">
-        <v>47861</v>
+        <v>52212</v>
       </c>
     </row>
     <row r="1393">
@@ -15758,7 +15758,7 @@
         <v>2785</v>
       </c>
       <c r="C1393" t="n">
-        <v>20801</v>
+        <v>22692</v>
       </c>
     </row>
     <row r="1394">
@@ -15769,7 +15769,7 @@
         <v>2411</v>
       </c>
       <c r="C1394" t="n">
-        <v>49995</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1395">
@@ -15780,7 +15780,7 @@
         <v>2716</v>
       </c>
       <c r="C1395" t="n">
-        <v>43868</v>
+        <v>47856</v>
       </c>
     </row>
     <row r="1396">
@@ -15791,7 +15791,7 @@
         <v>2809</v>
       </c>
       <c r="C1396" t="n">
-        <v>34342</v>
+        <v>37464</v>
       </c>
     </row>
     <row r="1397">
@@ -15802,7 +15802,7 @@
         <v>104</v>
       </c>
       <c r="C1397" t="n">
-        <v>150000.04</v>
+        <v>163636.4</v>
       </c>
     </row>
     <row r="1398">
@@ -15835,7 +15835,7 @@
         <v>781</v>
       </c>
       <c r="C1400" t="n">
-        <v>64999</v>
+        <v>70908</v>
       </c>
     </row>
     <row r="1401">
@@ -15857,7 +15857,7 @@
         <v>2494</v>
       </c>
       <c r="C1402" t="n">
-        <v>74998</v>
+        <v>81816</v>
       </c>
     </row>
     <row r="1403">
@@ -15868,7 +15868,7 @@
         <v>2652</v>
       </c>
       <c r="C1403" t="n">
-        <v>69993</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1404">
@@ -15879,7 +15879,7 @@
         <v>1384</v>
       </c>
       <c r="C1404" t="n">
-        <v>175000.01</v>
+        <v>190909.1</v>
       </c>
     </row>
     <row r="1405">
@@ -15890,7 +15890,7 @@
         <v>360</v>
       </c>
       <c r="C1405" t="n">
-        <v>249997</v>
+        <v>272724</v>
       </c>
     </row>
     <row r="1406">
@@ -15901,7 +15901,7 @@
         <v>2767</v>
       </c>
       <c r="C1406" t="n">
-        <v>94996</v>
+        <v>103632</v>
       </c>
     </row>
     <row r="1407">
@@ -15912,7 +15912,7 @@
         <v>2178</v>
       </c>
       <c r="C1407" t="n">
-        <v>136994</v>
+        <v>149448</v>
       </c>
     </row>
     <row r="1408">
@@ -15923,7 +15923,7 @@
         <v>2107</v>
       </c>
       <c r="C1408" t="n">
-        <v>149985</v>
+        <v>163620</v>
       </c>
     </row>
     <row r="1409">
@@ -15934,7 +15934,7 @@
         <v>2711</v>
       </c>
       <c r="C1409" t="n">
-        <v>43285</v>
+        <v>47220</v>
       </c>
     </row>
     <row r="1410">
@@ -15945,7 +15945,7 @@
         <v>2845</v>
       </c>
       <c r="C1410" t="n">
-        <v>24992</v>
+        <v>27264</v>
       </c>
     </row>
     <row r="1411">
@@ -15989,7 +15989,7 @@
         <v>1102</v>
       </c>
       <c r="C1414" t="n">
-        <v>117557</v>
+        <v>128244</v>
       </c>
     </row>
     <row r="1415">
@@ -16000,7 +16000,7 @@
         <v>353</v>
       </c>
       <c r="C1415" t="n">
-        <v>146267</v>
+        <v>159564</v>
       </c>
     </row>
     <row r="1416">
@@ -16011,7 +16011,7 @@
         <v>2250</v>
       </c>
       <c r="C1416" t="n">
-        <v>169994</v>
+        <v>185448</v>
       </c>
     </row>
     <row r="1417">
@@ -16022,7 +16022,7 @@
         <v>1800</v>
       </c>
       <c r="C1417" t="n">
-        <v>14179</v>
+        <v>15468</v>
       </c>
     </row>
     <row r="1418">
@@ -16033,7 +16033,7 @@
         <v>2362</v>
       </c>
       <c r="C1418" t="n">
-        <v>37499</v>
+        <v>40908</v>
       </c>
     </row>
     <row r="1419">
@@ -16044,7 +16044,7 @@
         <v>2449</v>
       </c>
       <c r="C1419" t="n">
-        <v>47498</v>
+        <v>51816</v>
       </c>
     </row>
     <row r="1420">
@@ -16055,7 +16055,7 @@
         <v>2844</v>
       </c>
       <c r="C1420" t="n">
-        <v>24992</v>
+        <v>27264</v>
       </c>
     </row>
     <row r="1421">
@@ -16066,7 +16066,7 @@
         <v>2507</v>
       </c>
       <c r="C1421" t="n">
-        <v>44660</v>
+        <v>48720</v>
       </c>
     </row>
     <row r="1422">
@@ -16077,7 +16077,7 @@
         <v>1906</v>
       </c>
       <c r="C1422" t="n">
-        <v>54285</v>
+        <v>59220</v>
       </c>
     </row>
     <row r="1423">
@@ -16099,7 +16099,7 @@
         <v>525</v>
       </c>
       <c r="C1424" t="n">
-        <v>117500.09</v>
+        <v>128181.9</v>
       </c>
     </row>
     <row r="1425">
@@ -16110,7 +16110,7 @@
         <v>1261</v>
       </c>
       <c r="C1425" t="n">
-        <v>35500.03</v>
+        <v>38727.3</v>
       </c>
     </row>
     <row r="1426">
@@ -16121,7 +16121,7 @@
         <v>2755</v>
       </c>
       <c r="C1426" t="n">
-        <v>25000.08</v>
+        <v>27272.8</v>
       </c>
     </row>
     <row r="1427">
@@ -16143,7 +16143,7 @@
         <v>1064</v>
       </c>
       <c r="C1428" t="n">
-        <v>299992</v>
+        <v>327264</v>
       </c>
     </row>
     <row r="1429">
@@ -16154,7 +16154,7 @@
         <v>1810</v>
       </c>
       <c r="C1429" t="n">
-        <v>20306</v>
+        <v>22152</v>
       </c>
     </row>
     <row r="1430">
@@ -16165,7 +16165,7 @@
         <v>1937</v>
       </c>
       <c r="C1430" t="n">
-        <v>129492</v>
+        <v>141264</v>
       </c>
     </row>
     <row r="1431">
@@ -16176,7 +16176,7 @@
         <v>483</v>
       </c>
       <c r="C1431" t="n">
-        <v>225995</v>
+        <v>246540</v>
       </c>
     </row>
     <row r="1432">
@@ -16187,7 +16187,7 @@
         <v>2580</v>
       </c>
       <c r="C1432" t="n">
-        <v>16841</v>
+        <v>18372</v>
       </c>
     </row>
     <row r="1433">
@@ -16198,7 +16198,7 @@
         <v>2706</v>
       </c>
       <c r="C1433" t="n">
-        <v>13156</v>
+        <v>14352</v>
       </c>
     </row>
     <row r="1434">
@@ -16209,7 +16209,7 @@
         <v>2633</v>
       </c>
       <c r="C1434" t="n">
-        <v>9636</v>
+        <v>10512</v>
       </c>
     </row>
     <row r="1435">
@@ -16242,7 +16242,7 @@
         <v>2392</v>
       </c>
       <c r="C1437" t="n">
-        <v>103708</v>
+        <v>113136</v>
       </c>
     </row>
     <row r="1438">
@@ -16264,7 +16264,7 @@
         <v>2613</v>
       </c>
       <c r="C1439" t="n">
-        <v>73018</v>
+        <v>79656</v>
       </c>
     </row>
     <row r="1440">
@@ -16275,7 +16275,7 @@
         <v>2183</v>
       </c>
       <c r="C1440" t="n">
-        <v>262911</v>
+        <v>286812</v>
       </c>
     </row>
     <row r="1441">
@@ -16286,7 +16286,7 @@
         <v>2541</v>
       </c>
       <c r="C1441" t="n">
-        <v>118195</v>
+        <v>128940</v>
       </c>
     </row>
     <row r="1442">
@@ -16297,7 +16297,7 @@
         <v>2333</v>
       </c>
       <c r="C1442" t="n">
-        <v>79794</v>
+        <v>87048</v>
       </c>
     </row>
     <row r="1443">
@@ -16308,7 +16308,7 @@
         <v>2813</v>
       </c>
       <c r="C1443" t="n">
-        <v>31900</v>
+        <v>34800</v>
       </c>
     </row>
     <row r="1444">
@@ -16319,7 +16319,7 @@
         <v>2811</v>
       </c>
       <c r="C1444" t="n">
-        <v>20801</v>
+        <v>22692</v>
       </c>
     </row>
     <row r="1445">
@@ -16330,7 +16330,7 @@
         <v>1881</v>
       </c>
       <c r="C1445" t="n">
-        <v>34342</v>
+        <v>37464</v>
       </c>
     </row>
     <row r="1446">
@@ -16341,7 +16341,7 @@
         <v>2825</v>
       </c>
       <c r="C1446" t="n">
-        <v>27918</v>
+        <v>30456</v>
       </c>
     </row>
     <row r="1447">
@@ -16352,7 +16352,7 @@
         <v>970</v>
       </c>
       <c r="C1447" t="n">
-        <v>34342</v>
+        <v>37464</v>
       </c>
     </row>
     <row r="1448">
@@ -16363,7 +16363,7 @@
         <v>2552</v>
       </c>
       <c r="C1448" t="n">
-        <v>19547</v>
+        <v>21324</v>
       </c>
     </row>
     <row r="1449">
@@ -16374,7 +16374,7 @@
         <v>2562</v>
       </c>
       <c r="C1449" t="n">
-        <v>19547</v>
+        <v>21324</v>
       </c>
     </row>
     <row r="1450">
@@ -16407,7 +16407,7 @@
         <v>2747</v>
       </c>
       <c r="C1452" t="n">
-        <v>34991</v>
+        <v>38172</v>
       </c>
     </row>
     <row r="1453">
@@ -16418,7 +16418,7 @@
         <v>415</v>
       </c>
       <c r="C1453" t="n">
-        <v>125000.07</v>
+        <v>136363.7</v>
       </c>
     </row>
     <row r="1454">
@@ -16462,7 +16462,7 @@
         <v>2544</v>
       </c>
       <c r="C1457" t="n">
-        <v>34991</v>
+        <v>38172</v>
       </c>
     </row>
     <row r="1458">
@@ -16473,7 +16473,7 @@
         <v>816</v>
       </c>
       <c r="C1458" t="n">
-        <v>150000.04</v>
+        <v>163636.4</v>
       </c>
     </row>
     <row r="1459">
@@ -16484,7 +16484,7 @@
         <v>890</v>
       </c>
       <c r="C1459" t="n">
-        <v>450000.01</v>
+        <v>490909.1</v>
       </c>
     </row>
     <row r="1460">
@@ -16495,7 +16495,7 @@
         <v>1298</v>
       </c>
       <c r="C1460" t="n">
-        <v>632500</v>
+        <v>690000</v>
       </c>
     </row>
     <row r="1461">
@@ -16506,7 +16506,7 @@
         <v>1372</v>
       </c>
       <c r="C1461" t="n">
-        <v>150000.04</v>
+        <v>163636.4</v>
       </c>
     </row>
     <row r="1462">
@@ -16517,7 +16517,7 @@
         <v>358</v>
       </c>
       <c r="C1462" t="n">
-        <v>157498</v>
+        <v>171816</v>
       </c>
     </row>
     <row r="1463">
@@ -16528,7 +16528,7 @@
         <v>1653</v>
       </c>
       <c r="C1463" t="n">
-        <v>157498</v>
+        <v>171816</v>
       </c>
     </row>
     <row r="1464">
@@ -16539,7 +16539,7 @@
         <v>675</v>
       </c>
       <c r="C1464" t="n">
-        <v>99990</v>
+        <v>109080</v>
       </c>
     </row>
     <row r="1465">
@@ -16550,7 +16550,7 @@
         <v>2804</v>
       </c>
       <c r="C1465" t="n">
-        <v>49995</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1466">
@@ -16561,7 +16561,7 @@
         <v>2714</v>
       </c>
       <c r="C1466" t="n">
-        <v>179993</v>
+        <v>196356</v>
       </c>
     </row>
     <row r="1467">
@@ -16572,7 +16572,7 @@
         <v>2765</v>
       </c>
       <c r="C1467" t="n">
-        <v>44990</v>
+        <v>49080</v>
       </c>
     </row>
     <row r="1468">
@@ -16583,7 +16583,7 @@
         <v>2421</v>
       </c>
       <c r="C1468" t="n">
-        <v>30492</v>
+        <v>33264</v>
       </c>
     </row>
     <row r="1469">
@@ -16594,7 +16594,7 @@
         <v>2359</v>
       </c>
       <c r="C1469" t="n">
-        <v>52162</v>
+        <v>56904</v>
       </c>
     </row>
     <row r="1470">
@@ -16605,7 +16605,7 @@
         <v>2678</v>
       </c>
       <c r="C1470" t="n">
-        <v>49478</v>
+        <v>53976</v>
       </c>
     </row>
     <row r="1471">
@@ -16616,7 +16616,7 @@
         <v>2697</v>
       </c>
       <c r="C1471" t="n">
-        <v>75086</v>
+        <v>81912</v>
       </c>
     </row>
     <row r="1472">
@@ -16649,7 +16649,7 @@
         <v>2142</v>
       </c>
       <c r="C1474" t="n">
-        <v>27060</v>
+        <v>29520</v>
       </c>
     </row>
     <row r="1475">
@@ -16660,7 +16660,7 @@
         <v>2498</v>
       </c>
       <c r="C1475" t="n">
-        <v>28149</v>
+        <v>30708</v>
       </c>
     </row>
     <row r="1476">
@@ -16682,7 +16682,7 @@
         <v>2801</v>
       </c>
       <c r="C1477" t="n">
-        <v>50000.05</v>
+        <v>54545.5</v>
       </c>
     </row>
     <row r="1478">
@@ -16693,7 +16693,7 @@
         <v>2810</v>
       </c>
       <c r="C1478" t="n">
-        <v>80000.08</v>
+        <v>87272.8</v>
       </c>
     </row>
     <row r="1479">
@@ -16734,10 +16734,10 @@
         <v>46296</v>
       </c>
       <c r="B1482" t="n">
-        <v>1433</v>
+        <v>132</v>
       </c>
       <c r="C1482" t="n">
-        <v>0</v>
+        <v>190909.1</v>
       </c>
     </row>
     <row r="1483">
@@ -16745,10 +16745,10 @@
         <v>46296</v>
       </c>
       <c r="B1483" t="n">
-        <v>580</v>
+        <v>1433</v>
       </c>
       <c r="C1483" t="n">
-        <v>87500.06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1484">
@@ -16756,10 +16756,10 @@
         <v>46296</v>
       </c>
       <c r="B1484" t="n">
-        <v>634</v>
+        <v>580</v>
       </c>
       <c r="C1484" t="n">
-        <v>250000.03</v>
+        <v>95454.60000000001</v>
       </c>
     </row>
     <row r="1485">
@@ -16767,10 +16767,10 @@
         <v>46296</v>
       </c>
       <c r="B1485" t="n">
-        <v>2437</v>
+        <v>634</v>
       </c>
       <c r="C1485" t="n">
-        <v>0</v>
+        <v>272727.3</v>
       </c>
     </row>
     <row r="1486">
@@ -16778,10 +16778,10 @@
         <v>46296</v>
       </c>
       <c r="B1486" t="n">
-        <v>1277</v>
+        <v>2437</v>
       </c>
       <c r="C1486" t="n">
-        <v>110000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1487">
@@ -16789,10 +16789,10 @@
         <v>46296</v>
       </c>
       <c r="B1487" t="n">
-        <v>767</v>
+        <v>1277</v>
       </c>
       <c r="C1487" t="n">
-        <v>99990</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="1488">
@@ -16800,10 +16800,10 @@
         <v>46296</v>
       </c>
       <c r="B1488" t="n">
-        <v>2727</v>
+        <v>767</v>
       </c>
       <c r="C1488" t="n">
-        <v>20240</v>
+        <v>109080</v>
       </c>
     </row>
     <row r="1489">
@@ -16811,10 +16811,10 @@
         <v>46296</v>
       </c>
       <c r="B1489" t="n">
-        <v>2846</v>
+        <v>2727</v>
       </c>
       <c r="C1489" t="n">
-        <v>129998</v>
+        <v>22080</v>
       </c>
     </row>
     <row r="1490">
@@ -16822,10 +16822,10 @@
         <v>46296</v>
       </c>
       <c r="B1490" t="n">
-        <v>609</v>
+        <v>2846</v>
       </c>
       <c r="C1490" t="n">
-        <v>112497</v>
+        <v>141816</v>
       </c>
     </row>
     <row r="1491">
@@ -16833,10 +16833,10 @@
         <v>46296</v>
       </c>
       <c r="B1491" t="n">
-        <v>2726</v>
+        <v>609</v>
       </c>
       <c r="C1491" t="n">
-        <v>77495</v>
+        <v>122724</v>
       </c>
     </row>
     <row r="1492">
@@ -16844,10 +16844,10 @@
         <v>46296</v>
       </c>
       <c r="B1492" t="n">
-        <v>2729</v>
+        <v>2726</v>
       </c>
       <c r="C1492" t="n">
-        <v>44990</v>
+        <v>84540</v>
       </c>
     </row>
     <row r="1493">
@@ -16855,10 +16855,10 @@
         <v>46296</v>
       </c>
       <c r="B1493" t="n">
-        <v>1340</v>
+        <v>2729</v>
       </c>
       <c r="C1493" t="n">
-        <v>74998</v>
+        <v>49080</v>
       </c>
     </row>
     <row r="1494">
@@ -16866,10 +16866,10 @@
         <v>46296</v>
       </c>
       <c r="B1494" t="n">
-        <v>2830</v>
+        <v>1340</v>
       </c>
       <c r="C1494" t="n">
-        <v>44990</v>
+        <v>81816</v>
       </c>
     </row>
     <row r="1495">
@@ -16877,10 +16877,10 @@
         <v>46296</v>
       </c>
       <c r="B1495" t="n">
-        <v>2674</v>
+        <v>2830</v>
       </c>
       <c r="C1495" t="n">
-        <v>129998</v>
+        <v>49080</v>
       </c>
     </row>
     <row r="1496">
@@ -16888,10 +16888,10 @@
         <v>46296</v>
       </c>
       <c r="B1496" t="n">
-        <v>2308</v>
+        <v>2674</v>
       </c>
       <c r="C1496" t="n">
-        <v>99990</v>
+        <v>141816</v>
       </c>
     </row>
     <row r="1497">
@@ -16899,10 +16899,10 @@
         <v>46296</v>
       </c>
       <c r="B1497" t="n">
-        <v>2190</v>
+        <v>2308</v>
       </c>
       <c r="C1497" t="n">
-        <v>104995</v>
+        <v>109080</v>
       </c>
     </row>
     <row r="1498">
@@ -16910,10 +16910,10 @@
         <v>46296</v>
       </c>
       <c r="B1498" t="n">
-        <v>2015</v>
+        <v>2190</v>
       </c>
       <c r="C1498" t="n">
-        <v>184998</v>
+        <v>114540</v>
       </c>
     </row>
     <row r="1499">
@@ -16921,10 +16921,10 @@
         <v>46296</v>
       </c>
       <c r="B1499" t="n">
-        <v>1308</v>
+        <v>2015</v>
       </c>
       <c r="C1499" t="n">
-        <v>78496</v>
+        <v>201816</v>
       </c>
     </row>
     <row r="1500">
@@ -16932,10 +16932,10 @@
         <v>46296</v>
       </c>
       <c r="B1500" t="n">
-        <v>2118</v>
+        <v>1308</v>
       </c>
       <c r="C1500" t="n">
-        <v>105083</v>
+        <v>85632</v>
       </c>
     </row>
     <row r="1501">
@@ -16943,10 +16943,10 @@
         <v>46296</v>
       </c>
       <c r="B1501" t="n">
-        <v>2607</v>
+        <v>2118</v>
       </c>
       <c r="C1501" t="n">
-        <v>24838</v>
+        <v>114636</v>
       </c>
     </row>
     <row r="1502">
@@ -16954,10 +16954,10 @@
         <v>46296</v>
       </c>
       <c r="B1502" t="n">
-        <v>2707</v>
+        <v>2607</v>
       </c>
       <c r="C1502" t="n">
-        <v>21593</v>
+        <v>27096</v>
       </c>
     </row>
     <row r="1503">
@@ -16968,7 +16968,7 @@
         <v>2832</v>
       </c>
       <c r="C1503" t="n">
-        <v>75000.02</v>
+        <v>81818.2</v>
       </c>
     </row>
     <row r="1504">
@@ -16979,7 +16979,7 @@
         <v>2383</v>
       </c>
       <c r="C1504" t="n">
-        <v>66462</v>
+        <v>72504</v>
       </c>
     </row>
     <row r="1505">
@@ -17012,7 +17012,7 @@
         <v>2821</v>
       </c>
       <c r="C1507" t="n">
-        <v>66671</v>
+        <v>72732</v>
       </c>
     </row>
     <row r="1508">
@@ -17034,7 +17034,7 @@
         <v>569</v>
       </c>
       <c r="C1509" t="n">
-        <v>1451714</v>
+        <v>1583688</v>
       </c>
     </row>
     <row r="1510">
@@ -17045,7 +17045,7 @@
         <v>2660</v>
       </c>
       <c r="C1510" t="n">
-        <v>175000.01</v>
+        <v>190909.1</v>
       </c>
     </row>
     <row r="1511">
@@ -17056,7 +17056,7 @@
         <v>1632</v>
       </c>
       <c r="C1511" t="n">
-        <v>130000.02</v>
+        <v>141818.2</v>
       </c>
     </row>
     <row r="1512">
@@ -17067,7 +17067,7 @@
         <v>1756</v>
       </c>
       <c r="C1512" t="n">
-        <v>209990</v>
+        <v>229080</v>
       </c>
     </row>
     <row r="1513">
@@ -17078,7 +17078,7 @@
         <v>58</v>
       </c>
       <c r="C1513" t="n">
-        <v>125400</v>
+        <v>136800</v>
       </c>
     </row>
     <row r="1514">
@@ -17089,7 +17089,7 @@
         <v>40</v>
       </c>
       <c r="C1514" t="n">
-        <v>111540</v>
+        <v>121680</v>
       </c>
     </row>
     <row r="1515">
@@ -17100,7 +17100,7 @@
         <v>559</v>
       </c>
       <c r="C1515" t="n">
-        <v>116996</v>
+        <v>127632</v>
       </c>
     </row>
     <row r="1516">
@@ -17111,7 +17111,7 @@
         <v>2773</v>
       </c>
       <c r="C1516" t="n">
-        <v>40337</v>
+        <v>44004</v>
       </c>
     </row>
     <row r="1517">
@@ -17122,7 +17122,7 @@
         <v>2631</v>
       </c>
       <c r="C1517" t="n">
-        <v>19371</v>
+        <v>21132</v>
       </c>
     </row>
     <row r="1518">
@@ -17133,7 +17133,7 @@
         <v>2085</v>
       </c>
       <c r="C1518" t="n">
-        <v>49995</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1519">
@@ -17155,7 +17155,7 @@
         <v>1642</v>
       </c>
       <c r="C1520" t="n">
-        <v>132495</v>
+        <v>144540</v>
       </c>
     </row>
     <row r="1521">
@@ -17166,7 +17166,7 @@
         <v>2621</v>
       </c>
       <c r="C1521" t="n">
-        <v>34991</v>
+        <v>38172</v>
       </c>
     </row>
     <row r="1522">
@@ -17177,7 +17177,7 @@
         <v>2705</v>
       </c>
       <c r="C1522" t="n">
-        <v>100386</v>
+        <v>109512</v>
       </c>
     </row>
     <row r="1523">
@@ -17188,7 +17188,7 @@
         <v>2735</v>
       </c>
       <c r="C1523" t="n">
-        <v>59994</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1524">
@@ -17199,7 +17199,7 @@
         <v>945</v>
       </c>
       <c r="C1524" t="n">
-        <v>175340</v>
+        <v>191280</v>
       </c>
     </row>
     <row r="1525">
@@ -17210,7 +17210,7 @@
         <v>2582</v>
       </c>
       <c r="C1525" t="n">
-        <v>43868</v>
+        <v>47856</v>
       </c>
     </row>
     <row r="1526">
@@ -17221,7 +17221,7 @@
         <v>2584</v>
       </c>
       <c r="C1526" t="n">
-        <v>31900</v>
+        <v>34800</v>
       </c>
     </row>
     <row r="1527">
@@ -17232,7 +17232,7 @@
         <v>2689</v>
       </c>
       <c r="C1527" t="n">
-        <v>31900</v>
+        <v>34800</v>
       </c>
     </row>
     <row r="1528">
@@ -17243,7 +17243,7 @@
         <v>2574</v>
       </c>
       <c r="C1528" t="n">
-        <v>70114</v>
+        <v>76488</v>
       </c>
     </row>
     <row r="1529">
@@ -17254,7 +17254,7 @@
         <v>1834</v>
       </c>
       <c r="C1529" t="n">
-        <v>58850</v>
+        <v>64200</v>
       </c>
     </row>
     <row r="1530">
@@ -17265,7 +17265,7 @@
         <v>2629</v>
       </c>
       <c r="C1530" t="n">
-        <v>34342</v>
+        <v>37464</v>
       </c>
     </row>
     <row r="1531">
@@ -17276,7 +17276,7 @@
         <v>933</v>
       </c>
       <c r="C1531" t="n">
-        <v>40733</v>
+        <v>44436</v>
       </c>
     </row>
     <row r="1532">
@@ -17287,7 +17287,7 @@
         <v>2555</v>
       </c>
       <c r="C1532" t="n">
-        <v>19547</v>
+        <v>21324</v>
       </c>
     </row>
     <row r="1533">
@@ -17298,7 +17298,7 @@
         <v>2558</v>
       </c>
       <c r="C1533" t="n">
-        <v>19547</v>
+        <v>21324</v>
       </c>
     </row>
     <row r="1534">
@@ -17309,7 +17309,7 @@
         <v>2721</v>
       </c>
       <c r="C1534" t="n">
-        <v>40733</v>
+        <v>44436</v>
       </c>
     </row>
     <row r="1535">
@@ -17320,7 +17320,7 @@
         <v>2556</v>
       </c>
       <c r="C1535" t="n">
-        <v>19547</v>
+        <v>21324</v>
       </c>
     </row>
     <row r="1536">
@@ -17331,7 +17331,7 @@
         <v>2826</v>
       </c>
       <c r="C1536" t="n">
-        <v>34991</v>
+        <v>38172</v>
       </c>
     </row>
     <row r="1537">
@@ -17353,7 +17353,7 @@
         <v>2346</v>
       </c>
       <c r="C1538" t="n">
-        <v>34991</v>
+        <v>38172</v>
       </c>
     </row>
     <row r="1539">
@@ -17364,7 +17364,7 @@
         <v>595</v>
       </c>
       <c r="C1539" t="n">
-        <v>125000.07</v>
+        <v>136363.7</v>
       </c>
     </row>
     <row r="1540">
@@ -17375,7 +17375,7 @@
         <v>1278</v>
       </c>
       <c r="C1540" t="n">
-        <v>87500.06</v>
+        <v>95454.60000000001</v>
       </c>
     </row>
     <row r="1541">
@@ -17386,7 +17386,7 @@
         <v>2686</v>
       </c>
       <c r="C1541" t="n">
-        <v>69993</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1542">
@@ -17397,7 +17397,7 @@
         <v>1344</v>
       </c>
       <c r="C1542" t="n">
-        <v>74998</v>
+        <v>81816</v>
       </c>
     </row>
     <row r="1543">
@@ -17408,7 +17408,7 @@
         <v>2566</v>
       </c>
       <c r="C1543" t="n">
-        <v>39996</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1544">
@@ -17419,7 +17419,7 @@
         <v>2684</v>
       </c>
       <c r="C1544" t="n">
-        <v>47498</v>
+        <v>51816</v>
       </c>
     </row>
     <row r="1545">
@@ -17430,7 +17430,7 @@
         <v>2375</v>
       </c>
       <c r="C1545" t="n">
-        <v>165000</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="1546">
@@ -17441,7 +17441,7 @@
         <v>2829</v>
       </c>
       <c r="C1546" t="n">
-        <v>29997</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1547">
@@ -17452,7 +17452,7 @@
         <v>768</v>
       </c>
       <c r="C1547" t="n">
-        <v>69993</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1548">
@@ -17463,7 +17463,7 @@
         <v>772</v>
       </c>
       <c r="C1548" t="n">
-        <v>162492</v>
+        <v>177264</v>
       </c>
     </row>
     <row r="1549">
@@ -17474,7 +17474,7 @@
         <v>2496</v>
       </c>
       <c r="C1549" t="n">
-        <v>99990</v>
+        <v>109080</v>
       </c>
     </row>
     <row r="1550">
@@ -17485,7 +17485,7 @@
         <v>802</v>
       </c>
       <c r="C1550" t="n">
-        <v>37499</v>
+        <v>40908</v>
       </c>
     </row>
     <row r="1551">
@@ -17496,7 +17496,7 @@
         <v>2131</v>
       </c>
       <c r="C1551" t="n">
-        <v>49995</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1552">
@@ -17507,7 +17507,7 @@
         <v>1381</v>
       </c>
       <c r="C1552" t="n">
-        <v>150000.04</v>
+        <v>163636.4</v>
       </c>
     </row>
     <row r="1553">
@@ -17518,7 +17518,7 @@
         <v>2847</v>
       </c>
       <c r="C1553" t="n">
-        <v>67496</v>
+        <v>73632</v>
       </c>
     </row>
     <row r="1554">
@@ -17529,7 +17529,7 @@
         <v>1293</v>
       </c>
       <c r="C1554" t="n">
-        <v>192500</v>
+        <v>210000</v>
       </c>
     </row>
     <row r="1555">
@@ -17540,7 +17540,7 @@
         <v>2363</v>
       </c>
       <c r="C1555" t="n">
-        <v>84997</v>
+        <v>92724</v>
       </c>
     </row>
     <row r="1556">
@@ -17551,7 +17551,7 @@
         <v>631</v>
       </c>
       <c r="C1556" t="n">
-        <v>174999</v>
+        <v>190908</v>
       </c>
     </row>
     <row r="1557">
@@ -17562,7 +17562,7 @@
         <v>2791</v>
       </c>
       <c r="C1557" t="n">
-        <v>51337</v>
+        <v>56004</v>
       </c>
     </row>
     <row r="1558">
@@ -17584,7 +17584,7 @@
         <v>2841</v>
       </c>
       <c r="C1559" t="n">
-        <v>24992</v>
+        <v>27264</v>
       </c>
     </row>
     <row r="1560">
@@ -17595,7 +17595,7 @@
         <v>2571</v>
       </c>
       <c r="C1560" t="n">
-        <v>133287</v>
+        <v>145404</v>
       </c>
     </row>
     <row r="1561">
@@ -17661,7 +17661,7 @@
         <v>2273</v>
       </c>
       <c r="C1566" t="n">
-        <v>107503</v>
+        <v>117276</v>
       </c>
     </row>
     <row r="1567">
@@ -17672,7 +17672,7 @@
         <v>2381</v>
       </c>
       <c r="C1567" t="n">
-        <v>40205</v>
+        <v>43860</v>
       </c>
     </row>
     <row r="1568">
@@ -17683,7 +17683,7 @@
         <v>630</v>
       </c>
       <c r="C1568" t="n">
-        <v>41264.99</v>
+        <v>45016.35</v>
       </c>
     </row>
     <row r="1569">
@@ -17705,7 +17705,7 @@
         <v>1983</v>
       </c>
       <c r="C1570" t="n">
-        <v>274120</v>
+        <v>299040</v>
       </c>
     </row>
     <row r="1571">
@@ -17716,7 +17716,7 @@
         <v>1993</v>
       </c>
       <c r="C1571" t="n">
-        <v>186142</v>
+        <v>203064</v>
       </c>
     </row>
     <row r="1572">
@@ -17727,7 +17727,7 @@
         <v>89</v>
       </c>
       <c r="C1572" t="n">
-        <v>174999</v>
+        <v>190908</v>
       </c>
     </row>
     <row r="1573">
@@ -17738,7 +17738,7 @@
         <v>1063</v>
       </c>
       <c r="C1573" t="n">
-        <v>192500</v>
+        <v>210000</v>
       </c>
     </row>
     <row r="1574">
@@ -17749,7 +17749,7 @@
         <v>1116</v>
       </c>
       <c r="C1574" t="n">
-        <v>124993</v>
+        <v>136356</v>
       </c>
     </row>
     <row r="1575">
@@ -17760,7 +17760,7 @@
         <v>941</v>
       </c>
       <c r="C1575" t="n">
-        <v>150447</v>
+        <v>164124</v>
       </c>
     </row>
     <row r="1576">
@@ -17771,7 +17771,7 @@
         <v>2141</v>
       </c>
       <c r="C1576" t="n">
-        <v>16038</v>
+        <v>17496</v>
       </c>
     </row>
     <row r="1577">
@@ -17782,7 +17782,7 @@
         <v>2463</v>
       </c>
       <c r="C1577" t="n">
-        <v>164912</v>
+        <v>179904</v>
       </c>
     </row>
     <row r="1578">
@@ -17790,10 +17790,10 @@
         <v>46296</v>
       </c>
       <c r="B1578" t="n">
-        <v>2325</v>
+        <v>2707</v>
       </c>
       <c r="C1578" t="n">
-        <v>57684</v>
+        <v>23556</v>
       </c>
     </row>
     <row r="1579">
@@ -17801,10 +17801,10 @@
         <v>46296</v>
       </c>
       <c r="B1579" t="n">
-        <v>2049</v>
+        <v>2325</v>
       </c>
       <c r="C1579" t="n">
-        <v>0</v>
+        <v>62928</v>
       </c>
     </row>
     <row r="1580">
@@ -17812,7 +17812,7 @@
         <v>46296</v>
       </c>
       <c r="B1580" t="n">
-        <v>2740</v>
+        <v>2049</v>
       </c>
       <c r="C1580" t="n">
         <v>0</v>
@@ -17823,7 +17823,7 @@
         <v>46296</v>
       </c>
       <c r="B1581" t="n">
-        <v>2741</v>
+        <v>2740</v>
       </c>
       <c r="C1581" t="n">
         <v>0</v>
@@ -17834,10 +17834,10 @@
         <v>46296</v>
       </c>
       <c r="B1582" t="n">
-        <v>1890</v>
+        <v>2741</v>
       </c>
       <c r="C1582" t="n">
-        <v>122617</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1583">
@@ -17845,10 +17845,10 @@
         <v>46296</v>
       </c>
       <c r="B1583" t="n">
-        <v>2639</v>
+        <v>1890</v>
       </c>
       <c r="C1583" t="n">
-        <v>20031</v>
+        <v>133764</v>
       </c>
     </row>
     <row r="1584">
@@ -17856,10 +17856,10 @@
         <v>46296</v>
       </c>
       <c r="B1584" t="n">
-        <v>2682</v>
+        <v>2639</v>
       </c>
       <c r="C1584" t="n">
-        <v>69993</v>
+        <v>21852</v>
       </c>
     </row>
     <row r="1585">
@@ -17867,10 +17867,10 @@
         <v>46296</v>
       </c>
       <c r="B1585" t="n">
-        <v>2601</v>
+        <v>2682</v>
       </c>
       <c r="C1585" t="n">
-        <v>137500</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1586">
@@ -17878,10 +17878,10 @@
         <v>46296</v>
       </c>
       <c r="B1586" t="n">
-        <v>1142</v>
+        <v>2601</v>
       </c>
       <c r="C1586" t="n">
-        <v>229042</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="1587">
@@ -17889,10 +17889,10 @@
         <v>46296</v>
       </c>
       <c r="B1587" t="n">
-        <v>628</v>
+        <v>1142</v>
       </c>
       <c r="C1587" t="n">
-        <v>0</v>
+        <v>249864</v>
       </c>
     </row>
     <row r="1588">
@@ -17900,7 +17900,7 @@
         <v>46296</v>
       </c>
       <c r="B1588" t="n">
-        <v>2046</v>
+        <v>628</v>
       </c>
       <c r="C1588" t="n">
         <v>0</v>
@@ -17911,7 +17911,7 @@
         <v>46296</v>
       </c>
       <c r="B1589" t="n">
-        <v>2189</v>
+        <v>2046</v>
       </c>
       <c r="C1589" t="n">
         <v>0</v>
@@ -17922,10 +17922,10 @@
         <v>46296</v>
       </c>
       <c r="B1590" t="n">
-        <v>2082</v>
+        <v>2189</v>
       </c>
       <c r="C1590" t="n">
-        <v>49995</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1591">
@@ -17933,10 +17933,10 @@
         <v>46296</v>
       </c>
       <c r="B1591" t="n">
-        <v>2276</v>
+        <v>2082</v>
       </c>
       <c r="C1591" t="n">
-        <v>99462</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1592">
@@ -17944,10 +17944,10 @@
         <v>46296</v>
       </c>
       <c r="B1592" t="n">
-        <v>2786</v>
+        <v>2276</v>
       </c>
       <c r="C1592" t="n">
-        <v>34991</v>
+        <v>108504</v>
       </c>
     </row>
     <row r="1593">
@@ -17955,10 +17955,10 @@
         <v>46296</v>
       </c>
       <c r="B1593" t="n">
-        <v>2816</v>
+        <v>2786</v>
       </c>
       <c r="C1593" t="n">
-        <v>64999</v>
+        <v>38172</v>
       </c>
     </row>
     <row r="1594">
@@ -17966,10 +17966,10 @@
         <v>46296</v>
       </c>
       <c r="B1594" t="n">
-        <v>1871</v>
+        <v>2816</v>
       </c>
       <c r="C1594" t="n">
-        <v>71753</v>
+        <v>70908</v>
       </c>
     </row>
     <row r="1595">
@@ -17977,10 +17977,10 @@
         <v>46296</v>
       </c>
       <c r="B1595" t="n">
-        <v>2345</v>
+        <v>1871</v>
       </c>
       <c r="C1595" t="n">
-        <v>31900</v>
+        <v>78276</v>
       </c>
     </row>
     <row r="1596">
@@ -17988,10 +17988,10 @@
         <v>46296</v>
       </c>
       <c r="B1596" t="n">
-        <v>2802</v>
+        <v>2345</v>
       </c>
       <c r="C1596" t="n">
-        <v>35893</v>
+        <v>34800</v>
       </c>
     </row>
     <row r="1597">
@@ -17999,10 +17999,10 @@
         <v>46296</v>
       </c>
       <c r="B1597" t="n">
-        <v>2090</v>
+        <v>2802</v>
       </c>
       <c r="C1597" t="n">
-        <v>20801</v>
+        <v>39156</v>
       </c>
     </row>
     <row r="1598">
@@ -18010,10 +18010,10 @@
         <v>46296</v>
       </c>
       <c r="B1598" t="n">
-        <v>2647</v>
+        <v>2090</v>
       </c>
       <c r="C1598" t="n">
-        <v>70125</v>
+        <v>22692</v>
       </c>
     </row>
     <row r="1599">
@@ -18021,10 +18021,10 @@
         <v>46296</v>
       </c>
       <c r="B1599" t="n">
-        <v>2365</v>
+        <v>2647</v>
       </c>
       <c r="C1599" t="n">
-        <v>49995</v>
+        <v>76500</v>
       </c>
     </row>
     <row r="1600">
@@ -18032,10 +18032,10 @@
         <v>46296</v>
       </c>
       <c r="B1600" t="n">
-        <v>766</v>
+        <v>2365</v>
       </c>
       <c r="C1600" t="n">
-        <v>34342</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1601">
@@ -18043,10 +18043,10 @@
         <v>46296</v>
       </c>
       <c r="B1601" t="n">
-        <v>2702</v>
+        <v>766</v>
       </c>
       <c r="C1601" t="n">
-        <v>40733</v>
+        <v>37464</v>
       </c>
     </row>
     <row r="1602">
@@ -18054,10 +18054,10 @@
         <v>46296</v>
       </c>
       <c r="B1602" t="n">
-        <v>20</v>
+        <v>2702</v>
       </c>
       <c r="C1602" t="n">
-        <v>225000.06</v>
+        <v>44436</v>
       </c>
     </row>
     <row r="1603">
@@ -18065,10 +18065,10 @@
         <v>46296</v>
       </c>
       <c r="B1603" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C1603" t="n">
-        <v>75000.02</v>
+        <v>245454.6</v>
       </c>
     </row>
     <row r="1604">
@@ -18076,10 +18076,10 @@
         <v>46296</v>
       </c>
       <c r="B1604" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C1604" t="n">
-        <v>198990</v>
+        <v>81818.2</v>
       </c>
     </row>
     <row r="1605">
@@ -18087,10 +18087,10 @@
         <v>46296</v>
       </c>
       <c r="B1605" t="n">
-        <v>2554</v>
+        <v>33</v>
       </c>
       <c r="C1605" t="n">
-        <v>0</v>
+        <v>217080</v>
       </c>
     </row>
     <row r="1606">
@@ -18098,10 +18098,10 @@
         <v>46296</v>
       </c>
       <c r="B1606" t="n">
-        <v>2561</v>
+        <v>2554</v>
       </c>
       <c r="C1606" t="n">
-        <v>19547</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1607">
@@ -18109,10 +18109,10 @@
         <v>46296</v>
       </c>
       <c r="B1607" t="n">
-        <v>934</v>
+        <v>2561</v>
       </c>
       <c r="C1607" t="n">
-        <v>0</v>
+        <v>21324</v>
       </c>
     </row>
     <row r="1608">
@@ -18120,10 +18120,10 @@
         <v>46296</v>
       </c>
       <c r="B1608" t="n">
-        <v>2772</v>
+        <v>934</v>
       </c>
       <c r="C1608" t="n">
-        <v>29997</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1609">
@@ -18131,10 +18131,10 @@
         <v>46296</v>
       </c>
       <c r="B1609" t="n">
-        <v>132</v>
+        <v>2772</v>
       </c>
       <c r="C1609" t="n">
-        <v>175000.01</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1610">
@@ -18145,7 +18145,7 @@
         <v>2834</v>
       </c>
       <c r="C1610" t="n">
-        <v>18634</v>
+        <v>20328</v>
       </c>
     </row>
     <row r="1611">
@@ -18156,7 +18156,7 @@
         <v>2394</v>
       </c>
       <c r="C1611" t="n">
-        <v>56727</v>
+        <v>61884</v>
       </c>
     </row>
     <row r="1612">
@@ -18167,7 +18167,7 @@
         <v>2567</v>
       </c>
       <c r="C1612" t="n">
-        <v>49995</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1613">
@@ -18178,7 +18178,7 @@
         <v>952</v>
       </c>
       <c r="C1613" t="n">
-        <v>49995</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1614">
@@ -18189,7 +18189,7 @@
         <v>1539</v>
       </c>
       <c r="C1614" t="n">
-        <v>84997</v>
+        <v>92724</v>
       </c>
     </row>
     <row r="1615">
@@ -18200,7 +18200,7 @@
         <v>793</v>
       </c>
       <c r="C1615" t="n">
-        <v>20801</v>
+        <v>22692</v>
       </c>
     </row>
     <row r="1616">
@@ -18211,7 +18211,7 @@
         <v>794</v>
       </c>
       <c r="C1616" t="n">
-        <v>20801</v>
+        <v>22692</v>
       </c>
     </row>
     <row r="1617">
@@ -18222,7 +18222,7 @@
         <v>2838</v>
       </c>
       <c r="C1617" t="n">
-        <v>30000.03</v>
+        <v>32727.3</v>
       </c>
     </row>
     <row r="1618">
@@ -18233,7 +18233,7 @@
         <v>2223</v>
       </c>
       <c r="C1618" t="n">
-        <v>58553</v>
+        <v>63876</v>
       </c>
     </row>
     <row r="1619">
@@ -18244,7 +18244,7 @@
         <v>2547</v>
       </c>
       <c r="C1619" t="n">
-        <v>16940</v>
+        <v>18480</v>
       </c>
     </row>
     <row r="1620">
@@ -18255,7 +18255,7 @@
         <v>2762</v>
       </c>
       <c r="C1620" t="n">
-        <v>40733</v>
+        <v>44436</v>
       </c>
     </row>
     <row r="1621">
@@ -18266,7 +18266,7 @@
         <v>2550</v>
       </c>
       <c r="C1621" t="n">
-        <v>19547</v>
+        <v>21324</v>
       </c>
     </row>
     <row r="1622">
@@ -18277,7 +18277,7 @@
         <v>2627</v>
       </c>
       <c r="C1622" t="n">
-        <v>19547</v>
+        <v>21324</v>
       </c>
     </row>
     <row r="1623">
@@ -18299,7 +18299,7 @@
         <v>749</v>
       </c>
       <c r="C1624" t="n">
-        <v>40733</v>
+        <v>44436</v>
       </c>
     </row>
     <row r="1625">
@@ -18310,7 +18310,7 @@
         <v>2549</v>
       </c>
       <c r="C1625" t="n">
-        <v>19547</v>
+        <v>21324</v>
       </c>
     </row>
     <row r="1626">
@@ -18321,7 +18321,7 @@
         <v>2649</v>
       </c>
       <c r="C1626" t="n">
-        <v>19547</v>
+        <v>21324</v>
       </c>
     </row>
     <row r="1627">
@@ -18332,7 +18332,7 @@
         <v>2258</v>
       </c>
       <c r="C1627" t="n">
-        <v>39996</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1628">
@@ -18343,7 +18343,7 @@
         <v>2744</v>
       </c>
       <c r="C1628" t="n">
-        <v>29997</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1629">
@@ -18354,7 +18354,7 @@
         <v>452</v>
       </c>
       <c r="C1629" t="n">
-        <v>141493</v>
+        <v>154356</v>
       </c>
     </row>
     <row r="1630">
@@ -18376,7 +18376,7 @@
         <v>2653</v>
       </c>
       <c r="C1631" t="n">
-        <v>29997</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1632">
@@ -18409,7 +18409,7 @@
         <v>2742</v>
       </c>
       <c r="C1634" t="n">
-        <v>9999</v>
+        <v>10908</v>
       </c>
     </row>
     <row r="1635">
@@ -18420,7 +18420,7 @@
         <v>1499</v>
       </c>
       <c r="C1635" t="n">
-        <v>44990</v>
+        <v>49080</v>
       </c>
     </row>
     <row r="1636">
@@ -18431,7 +18431,7 @@
         <v>2261</v>
       </c>
       <c r="C1636" t="n">
-        <v>89991</v>
+        <v>98172</v>
       </c>
     </row>
     <row r="1637">
@@ -18442,7 +18442,7 @@
         <v>1324</v>
       </c>
       <c r="C1637" t="n">
-        <v>139997</v>
+        <v>152724</v>
       </c>
     </row>
     <row r="1638">
@@ -18453,7 +18453,7 @@
         <v>2709</v>
       </c>
       <c r="C1638" t="n">
-        <v>89991</v>
+        <v>98172</v>
       </c>
     </row>
     <row r="1639">
@@ -18464,7 +18464,7 @@
         <v>1137</v>
       </c>
       <c r="C1639" t="n">
-        <v>319990</v>
+        <v>349080</v>
       </c>
     </row>
     <row r="1640">
@@ -18475,7 +18475,7 @@
         <v>2440</v>
       </c>
       <c r="C1640" t="n">
-        <v>39996</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1641">
@@ -18486,7 +18486,7 @@
         <v>429</v>
       </c>
       <c r="C1641" t="n">
-        <v>189992</v>
+        <v>207264</v>
       </c>
     </row>
     <row r="1642">
@@ -18497,7 +18497,7 @@
         <v>2114</v>
       </c>
       <c r="C1642" t="n">
-        <v>85063</v>
+        <v>92796</v>
       </c>
     </row>
     <row r="1643">
@@ -18508,7 +18508,7 @@
         <v>2211</v>
       </c>
       <c r="C1643" t="n">
-        <v>120417</v>
+        <v>131364</v>
       </c>
     </row>
     <row r="1644">
@@ -18519,7 +18519,7 @@
         <v>1108</v>
       </c>
       <c r="C1644" t="n">
-        <v>153186</v>
+        <v>167112</v>
       </c>
     </row>
     <row r="1645">
@@ -18530,7 +18530,7 @@
         <v>2695</v>
       </c>
       <c r="C1645" t="n">
-        <v>24189</v>
+        <v>26388</v>
       </c>
     </row>
     <row r="1646">
@@ -18541,7 +18541,7 @@
         <v>1289</v>
       </c>
       <c r="C1646" t="n">
-        <v>137500</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="1647">
@@ -18552,7 +18552,7 @@
         <v>2789</v>
       </c>
       <c r="C1647" t="n">
-        <v>90000.09</v>
+        <v>98181.89999999999</v>
       </c>
     </row>
     <row r="1648">
@@ -18563,7 +18563,7 @@
         <v>2197</v>
       </c>
       <c r="C1648" t="n">
-        <v>107500.08</v>
+        <v>117272.8</v>
       </c>
     </row>
     <row r="1649">
@@ -18574,7 +18574,7 @@
         <v>947</v>
       </c>
       <c r="C1649" t="n">
-        <v>221738</v>
+        <v>241896</v>
       </c>
     </row>
     <row r="1650">
@@ -18585,7 +18585,7 @@
         <v>2279</v>
       </c>
       <c r="C1650" t="n">
-        <v>122463</v>
+        <v>133596</v>
       </c>
     </row>
     <row r="1651">
@@ -18596,7 +18596,7 @@
         <v>1465</v>
       </c>
       <c r="C1651" t="n">
-        <v>192500</v>
+        <v>210000</v>
       </c>
     </row>
     <row r="1652">
@@ -18607,7 +18607,7 @@
         <v>2651</v>
       </c>
       <c r="C1652" t="n">
-        <v>84997</v>
+        <v>92724</v>
       </c>
     </row>
     <row r="1653">
@@ -18618,7 +18618,7 @@
         <v>42</v>
       </c>
       <c r="C1653" t="n">
-        <v>952996</v>
+        <v>1039632</v>
       </c>
     </row>
     <row r="1654">
@@ -18629,7 +18629,7 @@
         <v>949</v>
       </c>
       <c r="C1654" t="n">
-        <v>49731</v>
+        <v>54252</v>
       </c>
     </row>
     <row r="1655">
@@ -18640,7 +18640,7 @@
         <v>2606</v>
       </c>
       <c r="C1655" t="n">
-        <v>128370</v>
+        <v>140040</v>
       </c>
     </row>
     <row r="1656">
@@ -18651,7 +18651,7 @@
         <v>2249</v>
       </c>
       <c r="C1656" t="n">
-        <v>109065</v>
+        <v>118980</v>
       </c>
     </row>
     <row r="1657">
@@ -18695,7 +18695,7 @@
         <v>2045</v>
       </c>
       <c r="C1660" t="n">
-        <v>159236</v>
+        <v>173712</v>
       </c>
     </row>
     <row r="1661">
@@ -18706,7 +18706,7 @@
         <v>2663</v>
       </c>
       <c r="C1661" t="n">
-        <v>137500</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="1662">
@@ -18728,7 +18728,7 @@
         <v>2854</v>
       </c>
       <c r="C1663" t="n">
-        <v>19998</v>
+        <v>21816</v>
       </c>
     </row>
     <row r="1664">
@@ -18750,7 +18750,7 @@
         <v>2341</v>
       </c>
       <c r="C1665" t="n">
-        <v>87450</v>
+        <v>95400</v>
       </c>
     </row>
     <row r="1666">
@@ -18761,7 +18761,7 @@
         <v>2637</v>
       </c>
       <c r="C1666" t="n">
-        <v>31900</v>
+        <v>34800</v>
       </c>
     </row>
     <row r="1667">
@@ -18772,7 +18772,7 @@
         <v>2492</v>
       </c>
       <c r="C1667" t="n">
-        <v>50083</v>
+        <v>54636</v>
       </c>
     </row>
     <row r="1668">
@@ -18783,7 +18783,7 @@
         <v>2548</v>
       </c>
       <c r="C1668" t="n">
-        <v>19547</v>
+        <v>21324</v>
       </c>
     </row>
     <row r="1669">
@@ -18794,7 +18794,7 @@
         <v>351</v>
       </c>
       <c r="C1669" t="n">
-        <v>106491</v>
+        <v>116172</v>
       </c>
     </row>
     <row r="1670">
@@ -18827,7 +18827,7 @@
         <v>2757</v>
       </c>
       <c r="C1672" t="n">
-        <v>39996</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1673">
@@ -18838,7 +18838,7 @@
         <v>2815</v>
       </c>
       <c r="C1673" t="n">
-        <v>29997</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1674">
@@ -18849,7 +18849,7 @@
         <v>2323</v>
       </c>
       <c r="C1674" t="n">
-        <v>34342</v>
+        <v>37464</v>
       </c>
     </row>
     <row r="1675">
@@ -18860,7 +18860,7 @@
         <v>2310</v>
       </c>
       <c r="C1675" t="n">
-        <v>34342</v>
+        <v>37464</v>
       </c>
     </row>
     <row r="1676">
@@ -18871,7 +18871,7 @@
         <v>2145</v>
       </c>
       <c r="C1676" t="n">
-        <v>49995</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1677">
@@ -18882,7 +18882,7 @@
         <v>2501</v>
       </c>
       <c r="C1677" t="n">
-        <v>40733</v>
+        <v>44436</v>
       </c>
     </row>
     <row r="1678">
@@ -18893,7 +18893,7 @@
         <v>2546</v>
       </c>
       <c r="C1678" t="n">
-        <v>19547</v>
+        <v>21324</v>
       </c>
     </row>
     <row r="1679">
@@ -18904,7 +18904,7 @@
         <v>716</v>
       </c>
       <c r="C1679" t="n">
-        <v>64086</v>
+        <v>69912</v>
       </c>
     </row>
     <row r="1680">
@@ -18915,7 +18915,7 @@
         <v>2758</v>
       </c>
       <c r="C1680" t="n">
-        <v>29997</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1681">
@@ -18926,7 +18926,7 @@
         <v>400</v>
       </c>
       <c r="C1681" t="n">
-        <v>89991</v>
+        <v>98172</v>
       </c>
     </row>
     <row r="1682">
@@ -18937,7 +18937,7 @@
         <v>6</v>
       </c>
       <c r="C1682" t="n">
-        <v>25000.08</v>
+        <v>27272.8</v>
       </c>
     </row>
     <row r="1683">
@@ -18970,7 +18970,7 @@
         <v>1259</v>
       </c>
       <c r="C1685" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1686">
@@ -18981,7 +18981,7 @@
         <v>571</v>
       </c>
       <c r="C1686" t="n">
-        <v>517500.05</v>
+        <v>564545.5</v>
       </c>
     </row>
     <row r="1687">
@@ -18992,7 +18992,7 @@
         <v>703</v>
       </c>
       <c r="C1687" t="n">
-        <v>124993</v>
+        <v>136356</v>
       </c>
     </row>
     <row r="1688">
@@ -19014,7 +19014,7 @@
         <v>2833</v>
       </c>
       <c r="C1689" t="n">
-        <v>39996</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1690">
@@ -19025,7 +19025,7 @@
         <v>1007</v>
       </c>
       <c r="C1690" t="n">
-        <v>100000.1</v>
+        <v>109091</v>
       </c>
     </row>
     <row r="1691">
@@ -19036,7 +19036,7 @@
         <v>2687</v>
       </c>
       <c r="C1691" t="n">
-        <v>39996</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1692">
@@ -19047,7 +19047,7 @@
         <v>2824</v>
       </c>
       <c r="C1692" t="n">
-        <v>56452</v>
+        <v>61584</v>
       </c>
     </row>
     <row r="1693">
@@ -19058,7 +19058,7 @@
         <v>2730</v>
       </c>
       <c r="C1693" t="n">
-        <v>44990</v>
+        <v>49080</v>
       </c>
     </row>
     <row r="1694">
@@ -19069,7 +19069,7 @@
         <v>2718</v>
       </c>
       <c r="C1694" t="n">
-        <v>64999</v>
+        <v>70908</v>
       </c>
     </row>
     <row r="1695">
@@ -19080,7 +19080,7 @@
         <v>2750</v>
       </c>
       <c r="C1695" t="n">
-        <v>14993</v>
+        <v>16356</v>
       </c>
     </row>
     <row r="1696">
@@ -19091,7 +19091,7 @@
         <v>854</v>
       </c>
       <c r="C1696" t="n">
-        <v>69993</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1697">
@@ -19102,7 +19102,7 @@
         <v>2794</v>
       </c>
       <c r="C1697" t="n">
-        <v>59994</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1698">
@@ -19113,7 +19113,7 @@
         <v>1374</v>
       </c>
       <c r="C1698" t="n">
-        <v>99990</v>
+        <v>109080</v>
       </c>
     </row>
     <row r="1699">
@@ -19124,7 +19124,7 @@
         <v>2488</v>
       </c>
       <c r="C1699" t="n">
-        <v>49995</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1700">
@@ -19135,7 +19135,7 @@
         <v>363</v>
       </c>
       <c r="C1700" t="n">
-        <v>149996</v>
+        <v>163632</v>
       </c>
     </row>
     <row r="1701">
@@ -19146,7 +19146,7 @@
         <v>2655</v>
       </c>
       <c r="C1701" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1702">
@@ -19157,7 +19157,7 @@
         <v>1873</v>
       </c>
       <c r="C1702" t="n">
-        <v>159995</v>
+        <v>174540</v>
       </c>
     </row>
     <row r="1703">
@@ -19168,7 +19168,7 @@
         <v>2635</v>
       </c>
       <c r="C1703" t="n">
-        <v>64999</v>
+        <v>70908</v>
       </c>
     </row>
     <row r="1704">
@@ -19179,7 +19179,7 @@
         <v>1658</v>
       </c>
       <c r="C1704" t="n">
-        <v>76494</v>
+        <v>83448</v>
       </c>
     </row>
     <row r="1705">
@@ -19190,7 +19190,7 @@
         <v>2069</v>
       </c>
       <c r="C1705" t="n">
-        <v>100000.1</v>
+        <v>109091</v>
       </c>
     </row>
     <row r="1706">
@@ -19201,7 +19201,7 @@
         <v>2081</v>
       </c>
       <c r="C1706" t="n">
-        <v>74998</v>
+        <v>81816</v>
       </c>
     </row>
     <row r="1707">
@@ -19212,7 +19212,7 @@
         <v>2124</v>
       </c>
       <c r="C1707" t="n">
-        <v>174999</v>
+        <v>190908</v>
       </c>
     </row>
     <row r="1708">
@@ -19223,7 +19223,7 @@
         <v>636</v>
       </c>
       <c r="C1708" t="n">
-        <v>124993</v>
+        <v>136356</v>
       </c>
     </row>
     <row r="1709">
@@ -19234,7 +19234,7 @@
         <v>2803</v>
       </c>
       <c r="C1709" t="n">
-        <v>59994</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1710">
@@ -19245,7 +19245,7 @@
         <v>2163</v>
       </c>
       <c r="C1710" t="n">
-        <v>89991</v>
+        <v>98172</v>
       </c>
     </row>
     <row r="1711">
@@ -19256,7 +19256,7 @@
         <v>1466</v>
       </c>
       <c r="C1711" t="n">
-        <v>202499</v>
+        <v>220908</v>
       </c>
     </row>
     <row r="1712">
@@ -19267,7 +19267,7 @@
         <v>2133</v>
       </c>
       <c r="C1712" t="n">
-        <v>175000.01</v>
+        <v>190909.1</v>
       </c>
     </row>
     <row r="1713">
@@ -19278,7 +19278,7 @@
         <v>2431</v>
       </c>
       <c r="C1713" t="n">
-        <v>74998</v>
+        <v>81816</v>
       </c>
     </row>
     <row r="1714">
@@ -19289,7 +19289,7 @@
         <v>535</v>
       </c>
       <c r="C1714" t="n">
-        <v>178090</v>
+        <v>194280</v>
       </c>
     </row>
     <row r="1715">
@@ -19300,7 +19300,7 @@
         <v>2790</v>
       </c>
       <c r="C1715" t="n">
-        <v>31581</v>
+        <v>34452</v>
       </c>
     </row>
     <row r="1716">
@@ -19311,7 +19311,7 @@
         <v>2442</v>
       </c>
       <c r="C1716" t="n">
-        <v>129492</v>
+        <v>141264</v>
       </c>
     </row>
     <row r="1717">
@@ -19322,7 +19322,7 @@
         <v>2376</v>
       </c>
       <c r="C1717" t="n">
-        <v>550000</v>
+        <v>600000</v>
       </c>
     </row>
     <row r="1718">
@@ -19333,7 +19333,7 @@
         <v>2768</v>
       </c>
       <c r="C1718" t="n">
-        <v>151327</v>
+        <v>165084</v>
       </c>
     </row>
     <row r="1719">
@@ -19344,7 +19344,7 @@
         <v>2491</v>
       </c>
       <c r="C1719" t="n">
-        <v>121429</v>
+        <v>132468</v>
       </c>
     </row>
     <row r="1720">
@@ -19355,7 +19355,7 @@
         <v>2799</v>
       </c>
       <c r="C1720" t="n">
-        <v>54659</v>
+        <v>59628</v>
       </c>
     </row>
     <row r="1721">
@@ -19388,7 +19388,7 @@
         <v>1317</v>
       </c>
       <c r="C1723" t="n">
-        <v>157500.02</v>
+        <v>171818.2</v>
       </c>
     </row>
     <row r="1724">
@@ -19399,7 +19399,7 @@
         <v>2822</v>
       </c>
       <c r="C1724" t="n">
-        <v>80000.08</v>
+        <v>87272.8</v>
       </c>
     </row>
     <row r="1725">
@@ -19410,7 +19410,7 @@
         <v>1117</v>
       </c>
       <c r="C1725" t="n">
-        <v>200057</v>
+        <v>218244</v>
       </c>
     </row>
     <row r="1726">
@@ -19421,7 +19421,7 @@
         <v>1299</v>
       </c>
       <c r="C1726" t="n">
-        <v>263769</v>
+        <v>287748</v>
       </c>
     </row>
     <row r="1727">
@@ -19432,7 +19432,7 @@
         <v>477</v>
       </c>
       <c r="C1727" t="n">
-        <v>108702</v>
+        <v>118584</v>
       </c>
     </row>
     <row r="1728">
@@ -19443,7 +19443,7 @@
         <v>530</v>
       </c>
       <c r="C1728" t="n">
-        <v>149996</v>
+        <v>163632</v>
       </c>
     </row>
     <row r="1729">
@@ -19454,7 +19454,7 @@
         <v>953</v>
       </c>
       <c r="C1729" t="n">
-        <v>344993</v>
+        <v>376356</v>
       </c>
     </row>
     <row r="1730">
@@ -19465,7 +19465,7 @@
         <v>610</v>
       </c>
       <c r="C1730" t="n">
-        <v>410894</v>
+        <v>448248</v>
       </c>
     </row>
     <row r="1731">
@@ -19476,7 +19476,7 @@
         <v>2792</v>
       </c>
       <c r="C1731" t="n">
-        <v>103191</v>
+        <v>112572</v>
       </c>
     </row>
     <row r="1732">
@@ -19553,7 +19553,7 @@
         <v>1075</v>
       </c>
       <c r="C1738" t="n">
-        <v>229493</v>
+        <v>250356</v>
       </c>
     </row>
     <row r="1739">
@@ -19564,7 +19564,7 @@
         <v>131</v>
       </c>
       <c r="C1739" t="n">
-        <v>207999</v>
+        <v>226908</v>
       </c>
     </row>
     <row r="1740">
@@ -19575,7 +19575,7 @@
         <v>2667</v>
       </c>
       <c r="C1740" t="n">
-        <v>22847</v>
+        <v>24924</v>
       </c>
     </row>
     <row r="1741">
@@ -19586,7 +19586,7 @@
         <v>2330</v>
       </c>
       <c r="C1741" t="n">
-        <v>44473</v>
+        <v>48516</v>
       </c>
     </row>
     <row r="1742">
@@ -19608,7 +19608,7 @@
         <v>2577</v>
       </c>
       <c r="C1743" t="n">
-        <v>44583</v>
+        <v>48636</v>
       </c>
     </row>
     <row r="1744">
@@ -19619,7 +19619,7 @@
         <v>2510</v>
       </c>
       <c r="C1744" t="n">
-        <v>316624</v>
+        <v>345408</v>
       </c>
     </row>
     <row r="1745">
@@ -19641,7 +19641,7 @@
         <v>2850</v>
       </c>
       <c r="C1746" t="n">
-        <v>29997</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1747">
@@ -19663,7 +19663,7 @@
         <v>2745</v>
       </c>
       <c r="C1748" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="1749">
@@ -19674,7 +19674,7 @@
         <v>2817</v>
       </c>
       <c r="C1749" t="n">
-        <v>29997</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1750">
@@ -19685,7 +19685,7 @@
         <v>2784</v>
       </c>
       <c r="C1750" t="n">
-        <v>20801</v>
+        <v>22692</v>
       </c>
     </row>
     <row r="1751">
@@ -19696,7 +19696,7 @@
         <v>626</v>
       </c>
       <c r="C1751" t="n">
-        <v>863907</v>
+        <v>942444</v>
       </c>
     </row>
     <row r="1752">
@@ -19707,7 +19707,7 @@
         <v>925</v>
       </c>
       <c r="C1752" t="n">
-        <v>39886</v>
+        <v>43512</v>
       </c>
     </row>
     <row r="1753">
@@ -19718,7 +19718,7 @@
         <v>2586</v>
       </c>
       <c r="C1753" t="n">
-        <v>20801</v>
+        <v>22692</v>
       </c>
     </row>
     <row r="1754">
@@ -19729,7 +19729,7 @@
         <v>966</v>
       </c>
       <c r="C1754" t="n">
-        <v>40733</v>
+        <v>44436</v>
       </c>
     </row>
     <row r="1755">
@@ -19740,7 +19740,7 @@
         <v>2557</v>
       </c>
       <c r="C1755" t="n">
-        <v>19547</v>
+        <v>21324</v>
       </c>
     </row>
     <row r="1756">
@@ -19751,7 +19751,7 @@
         <v>14</v>
       </c>
       <c r="C1756" t="n">
-        <v>224994</v>
+        <v>245448</v>
       </c>
     </row>
     <row r="1757">
@@ -19762,7 +19762,7 @@
         <v>2798</v>
       </c>
       <c r="C1757" t="n">
-        <v>29997</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1758">
@@ -19784,7 +19784,7 @@
         <v>522</v>
       </c>
       <c r="C1759" t="n">
-        <v>100000.1</v>
+        <v>109091</v>
       </c>
     </row>
     <row r="1760">
@@ -19806,7 +19806,7 @@
         <v>2819</v>
       </c>
       <c r="C1761" t="n">
-        <v>29997</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1762">
@@ -19817,7 +19817,7 @@
         <v>2266</v>
       </c>
       <c r="C1762" t="n">
-        <v>39996</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1763">
@@ -19850,7 +19850,7 @@
         <v>2795</v>
       </c>
       <c r="C1765" t="n">
-        <v>29997</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1766">
@@ -19861,7 +19861,7 @@
         <v>2722</v>
       </c>
       <c r="C1766" t="n">
-        <v>9999</v>
+        <v>10908</v>
       </c>
     </row>
     <row r="1767">
@@ -19872,7 +19872,7 @@
         <v>951</v>
       </c>
       <c r="C1767" t="n">
-        <v>57497</v>
+        <v>62724</v>
       </c>
     </row>
     <row r="1768">
@@ -19883,7 +19883,7 @@
         <v>1020</v>
       </c>
       <c r="C1768" t="n">
-        <v>49995</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1769">
@@ -19894,7 +19894,7 @@
         <v>1853</v>
       </c>
       <c r="C1769" t="n">
-        <v>59994</v>
+        <v>65448</v>
       </c>
     </row>
     <row r="1770">
@@ -19905,7 +19905,7 @@
         <v>1327</v>
       </c>
       <c r="C1770" t="n">
-        <v>34991</v>
+        <v>38172</v>
       </c>
     </row>
     <row r="1771">
@@ -19916,7 +19916,7 @@
         <v>2842</v>
       </c>
       <c r="C1771" t="n">
-        <v>89991</v>
+        <v>98172</v>
       </c>
     </row>
     <row r="1772">
@@ -19927,7 +19927,7 @@
         <v>2831</v>
       </c>
       <c r="C1772" t="n">
-        <v>29997</v>
+        <v>32724</v>
       </c>
     </row>
     <row r="1773">
@@ -19938,7 +19938,7 @@
         <v>818</v>
       </c>
       <c r="C1773" t="n">
-        <v>199991</v>
+        <v>218172</v>
       </c>
     </row>
     <row r="1774">
@@ -19949,7 +19949,7 @@
         <v>1501</v>
       </c>
       <c r="C1774" t="n">
-        <v>49995</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1775">
@@ -19960,7 +19960,7 @@
         <v>1869</v>
       </c>
       <c r="C1775" t="n">
-        <v>121990</v>
+        <v>133080</v>
       </c>
     </row>
     <row r="1776">
@@ -19971,7 +19971,7 @@
         <v>1996</v>
       </c>
       <c r="C1776" t="n">
-        <v>125000.07</v>
+        <v>136363.7</v>
       </c>
     </row>
     <row r="1777">
@@ -19982,7 +19982,7 @@
         <v>2462</v>
       </c>
       <c r="C1777" t="n">
-        <v>28317.59</v>
+        <v>30891.9</v>
       </c>
     </row>
     <row r="1778">
@@ -19993,7 +19993,7 @@
         <v>2696</v>
       </c>
       <c r="C1778" t="n">
-        <v>107228</v>
+        <v>116976</v>
       </c>
     </row>
     <row r="1779">
@@ -20004,7 +20004,7 @@
         <v>2698</v>
       </c>
       <c r="C1779" t="n">
-        <v>54956</v>
+        <v>59952</v>
       </c>
     </row>
     <row r="1780">
@@ -20026,7 +20026,7 @@
         <v>2828</v>
       </c>
       <c r="C1781" t="n">
-        <v>30000.03</v>
+        <v>32727.3</v>
       </c>
     </row>
     <row r="1782">
@@ -20037,7 +20037,7 @@
         <v>2843</v>
       </c>
       <c r="C1782" t="n">
-        <v>34991</v>
+        <v>38172</v>
       </c>
     </row>
     <row r="1783">
@@ -20048,7 +20048,7 @@
         <v>619</v>
       </c>
       <c r="C1783" t="n">
-        <v>156750</v>
+        <v>171000</v>
       </c>
     </row>
     <row r="1784">
@@ -20059,7 +20059,7 @@
         <v>1478</v>
       </c>
       <c r="C1784" t="n">
-        <v>274318</v>
+        <v>299256</v>
       </c>
     </row>
     <row r="1785">
@@ -20070,7 +20070,7 @@
         <v>2026</v>
       </c>
       <c r="C1785" t="n">
-        <v>121198</v>
+        <v>132216</v>
       </c>
     </row>
     <row r="1786">
@@ -20081,7 +20081,7 @@
         <v>663</v>
       </c>
       <c r="C1786" t="n">
-        <v>129492</v>
+        <v>141264</v>
       </c>
     </row>
     <row r="1787">
@@ -20092,7 +20092,7 @@
         <v>285</v>
       </c>
       <c r="C1787" t="n">
-        <v>274318</v>
+        <v>299256</v>
       </c>
     </row>
     <row r="1788">
@@ -20103,7 +20103,7 @@
         <v>424</v>
       </c>
       <c r="C1788" t="n">
-        <v>117557</v>
+        <v>128244</v>
       </c>
     </row>
     <row r="1789">
@@ -20114,7 +20114,7 @@
         <v>451</v>
       </c>
       <c r="C1789" t="n">
-        <v>121495</v>
+        <v>132540</v>
       </c>
     </row>
     <row r="1790">
@@ -20125,7 +20125,7 @@
         <v>629</v>
       </c>
       <c r="C1790" t="n">
-        <v>226996</v>
+        <v>247632</v>
       </c>
     </row>
     <row r="1791">
@@ -20136,7 +20136,7 @@
         <v>2657</v>
       </c>
       <c r="C1791" t="n">
-        <v>39589</v>
+        <v>43188</v>
       </c>
     </row>
     <row r="1792">
@@ -20147,7 +20147,7 @@
         <v>1254</v>
       </c>
       <c r="C1792" t="n">
-        <v>97097</v>
+        <v>105924</v>
       </c>
     </row>
     <row r="1793">
@@ -20158,7 +20158,7 @@
         <v>2402</v>
       </c>
       <c r="C1793" t="n">
-        <v>244222</v>
+        <v>266424</v>
       </c>
     </row>
     <row r="1794">
@@ -20169,7 +20169,7 @@
         <v>2413</v>
       </c>
       <c r="C1794" t="n">
-        <v>68915</v>
+        <v>75180</v>
       </c>
     </row>
     <row r="1795">
@@ -20180,7 +20180,7 @@
         <v>1450</v>
       </c>
       <c r="C1795" t="n">
-        <v>178497</v>
+        <v>194724</v>
       </c>
     </row>
     <row r="1796">
@@ -20202,7 +20202,7 @@
         <v>2671</v>
       </c>
       <c r="C1797" t="n">
-        <v>39996</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1798">
@@ -20213,7 +20213,7 @@
         <v>2568</v>
       </c>
       <c r="C1798" t="n">
-        <v>80223</v>
+        <v>87516</v>
       </c>
     </row>
     <row r="1799">
@@ -20224,7 +20224,7 @@
         <v>2146</v>
       </c>
       <c r="C1799" t="n">
-        <v>97141</v>
+        <v>105972</v>
       </c>
     </row>
     <row r="1800">
@@ -20235,7 +20235,7 @@
         <v>2753</v>
       </c>
       <c r="C1800" t="n">
-        <v>37499</v>
+        <v>40908</v>
       </c>
     </row>
     <row r="1801">
@@ -20246,7 +20246,7 @@
         <v>744</v>
       </c>
       <c r="C1801" t="n">
-        <v>20801</v>
+        <v>22692</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:01:21
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -15560,7 +15560,7 @@
         <v>2853</v>
       </c>
       <c r="C1375" t="n">
-        <v>44436</v>
+        <v>48139</v>
       </c>
     </row>
     <row r="1376">
@@ -15571,7 +15571,7 @@
         <v>2245</v>
       </c>
       <c r="C1376" t="n">
-        <v>120768</v>
+        <v>130832</v>
       </c>
     </row>
     <row r="1377">
@@ -15582,7 +15582,7 @@
         <v>2251</v>
       </c>
       <c r="C1377" t="n">
-        <v>109080</v>
+        <v>118170</v>
       </c>
     </row>
     <row r="1378">
@@ -15593,7 +15593,7 @@
         <v>664</v>
       </c>
       <c r="C1378" t="n">
-        <v>142908</v>
+        <v>154817</v>
       </c>
     </row>
     <row r="1379">
@@ -15604,7 +15604,7 @@
         <v>2472</v>
       </c>
       <c r="C1379" t="n">
-        <v>28872</v>
+        <v>31278</v>
       </c>
     </row>
     <row r="1380">
@@ -15615,7 +15615,7 @@
         <v>1456</v>
       </c>
       <c r="C1380" t="n">
-        <v>435264</v>
+        <v>471536</v>
       </c>
     </row>
     <row r="1381">
@@ -15626,7 +15626,7 @@
         <v>1585</v>
       </c>
       <c r="C1381" t="n">
-        <v>98724</v>
+        <v>106951</v>
       </c>
     </row>
     <row r="1382">
@@ -15670,7 +15670,7 @@
         <v>1907</v>
       </c>
       <c r="C1385" t="n">
-        <v>300288</v>
+        <v>325312</v>
       </c>
     </row>
     <row r="1386">
@@ -15703,7 +15703,7 @@
         <v>2659</v>
       </c>
       <c r="C1388" t="n">
-        <v>67092</v>
+        <v>72683</v>
       </c>
     </row>
     <row r="1389">
@@ -15714,7 +15714,7 @@
         <v>2583</v>
       </c>
       <c r="C1389" t="n">
-        <v>22692</v>
+        <v>24583</v>
       </c>
     </row>
     <row r="1390">
@@ -15725,7 +15725,7 @@
         <v>2692</v>
       </c>
       <c r="C1390" t="n">
-        <v>38181.9</v>
+        <v>41363.71</v>
       </c>
     </row>
     <row r="1391">
@@ -15736,7 +15736,7 @@
         <v>2691</v>
       </c>
       <c r="C1391" t="n">
-        <v>66645.89999999999</v>
+        <v>72199.71000000001</v>
       </c>
     </row>
     <row r="1392">
@@ -15747,7 +15747,7 @@
         <v>931</v>
       </c>
       <c r="C1392" t="n">
-        <v>52212</v>
+        <v>56563</v>
       </c>
     </row>
     <row r="1393">
@@ -15758,7 +15758,7 @@
         <v>2785</v>
       </c>
       <c r="C1393" t="n">
-        <v>22692</v>
+        <v>24583</v>
       </c>
     </row>
     <row r="1394">
@@ -15769,7 +15769,7 @@
         <v>2411</v>
       </c>
       <c r="C1394" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1395">
@@ -15780,7 +15780,7 @@
         <v>2716</v>
       </c>
       <c r="C1395" t="n">
-        <v>47856</v>
+        <v>51844</v>
       </c>
     </row>
     <row r="1396">
@@ -15791,7 +15791,7 @@
         <v>2809</v>
       </c>
       <c r="C1396" t="n">
-        <v>37464</v>
+        <v>40586</v>
       </c>
     </row>
     <row r="1397">
@@ -15802,7 +15802,7 @@
         <v>104</v>
       </c>
       <c r="C1397" t="n">
-        <v>163636.4</v>
+        <v>177272.76</v>
       </c>
     </row>
     <row r="1398">
@@ -15835,7 +15835,7 @@
         <v>781</v>
       </c>
       <c r="C1400" t="n">
-        <v>70908</v>
+        <v>76817</v>
       </c>
     </row>
     <row r="1401">
@@ -15857,7 +15857,7 @@
         <v>2494</v>
       </c>
       <c r="C1402" t="n">
-        <v>81816</v>
+        <v>88634</v>
       </c>
     </row>
     <row r="1403">
@@ -15868,7 +15868,7 @@
         <v>2652</v>
       </c>
       <c r="C1403" t="n">
-        <v>76356</v>
+        <v>82719</v>
       </c>
     </row>
     <row r="1404">
@@ -15879,7 +15879,7 @@
         <v>1384</v>
       </c>
       <c r="C1404" t="n">
-        <v>190909.1</v>
+        <v>206818.19</v>
       </c>
     </row>
     <row r="1405">
@@ -15890,7 +15890,7 @@
         <v>360</v>
       </c>
       <c r="C1405" t="n">
-        <v>272724</v>
+        <v>295451</v>
       </c>
     </row>
     <row r="1406">
@@ -15901,7 +15901,7 @@
         <v>2767</v>
       </c>
       <c r="C1406" t="n">
-        <v>103632</v>
+        <v>112268</v>
       </c>
     </row>
     <row r="1407">
@@ -15912,7 +15912,7 @@
         <v>2178</v>
       </c>
       <c r="C1407" t="n">
-        <v>149448</v>
+        <v>161902</v>
       </c>
     </row>
     <row r="1408">
@@ -15923,7 +15923,7 @@
         <v>2107</v>
       </c>
       <c r="C1408" t="n">
-        <v>163620</v>
+        <v>177255</v>
       </c>
     </row>
     <row r="1409">
@@ -15934,7 +15934,7 @@
         <v>2711</v>
       </c>
       <c r="C1409" t="n">
-        <v>47220</v>
+        <v>51155</v>
       </c>
     </row>
     <row r="1410">
@@ -15945,7 +15945,7 @@
         <v>2845</v>
       </c>
       <c r="C1410" t="n">
-        <v>27264</v>
+        <v>29536</v>
       </c>
     </row>
     <row r="1411">
@@ -15989,7 +15989,7 @@
         <v>1102</v>
       </c>
       <c r="C1414" t="n">
-        <v>128244</v>
+        <v>138931</v>
       </c>
     </row>
     <row r="1415">
@@ -16000,7 +16000,7 @@
         <v>353</v>
       </c>
       <c r="C1415" t="n">
-        <v>159564</v>
+        <v>172861</v>
       </c>
     </row>
     <row r="1416">
@@ -16011,7 +16011,7 @@
         <v>2250</v>
       </c>
       <c r="C1416" t="n">
-        <v>185448</v>
+        <v>200902</v>
       </c>
     </row>
     <row r="1417">
@@ -16022,7 +16022,7 @@
         <v>1800</v>
       </c>
       <c r="C1417" t="n">
-        <v>15468</v>
+        <v>16757</v>
       </c>
     </row>
     <row r="1418">
@@ -16033,7 +16033,7 @@
         <v>2362</v>
       </c>
       <c r="C1418" t="n">
-        <v>40908</v>
+        <v>44317</v>
       </c>
     </row>
     <row r="1419">
@@ -16044,7 +16044,7 @@
         <v>2449</v>
       </c>
       <c r="C1419" t="n">
-        <v>51816</v>
+        <v>56134</v>
       </c>
     </row>
     <row r="1420">
@@ -16055,7 +16055,7 @@
         <v>2844</v>
       </c>
       <c r="C1420" t="n">
-        <v>27264</v>
+        <v>29536</v>
       </c>
     </row>
     <row r="1421">
@@ -16066,7 +16066,7 @@
         <v>2507</v>
       </c>
       <c r="C1421" t="n">
-        <v>48720</v>
+        <v>52780</v>
       </c>
     </row>
     <row r="1422">
@@ -16077,7 +16077,7 @@
         <v>1906</v>
       </c>
       <c r="C1422" t="n">
-        <v>59220</v>
+        <v>64155</v>
       </c>
     </row>
     <row r="1423">
@@ -16099,7 +16099,7 @@
         <v>525</v>
       </c>
       <c r="C1424" t="n">
-        <v>128181.9</v>
+        <v>138863.71</v>
       </c>
     </row>
     <row r="1425">
@@ -16110,7 +16110,7 @@
         <v>1261</v>
       </c>
       <c r="C1425" t="n">
-        <v>38727.3</v>
+        <v>41954.57</v>
       </c>
     </row>
     <row r="1426">
@@ -16121,7 +16121,7 @@
         <v>2755</v>
       </c>
       <c r="C1426" t="n">
-        <v>27272.8</v>
+        <v>29545.52</v>
       </c>
     </row>
     <row r="1427">
@@ -16143,7 +16143,7 @@
         <v>1064</v>
       </c>
       <c r="C1428" t="n">
-        <v>327264</v>
+        <v>354536</v>
       </c>
     </row>
     <row r="1429">
@@ -16154,7 +16154,7 @@
         <v>1810</v>
       </c>
       <c r="C1429" t="n">
-        <v>22152</v>
+        <v>23998</v>
       </c>
     </row>
     <row r="1430">
@@ -16165,7 +16165,7 @@
         <v>1937</v>
       </c>
       <c r="C1430" t="n">
-        <v>141264</v>
+        <v>153036</v>
       </c>
     </row>
     <row r="1431">
@@ -16176,7 +16176,7 @@
         <v>483</v>
       </c>
       <c r="C1431" t="n">
-        <v>246540</v>
+        <v>267085</v>
       </c>
     </row>
     <row r="1432">
@@ -16187,7 +16187,7 @@
         <v>2580</v>
       </c>
       <c r="C1432" t="n">
-        <v>18372</v>
+        <v>19903</v>
       </c>
     </row>
     <row r="1433">
@@ -16198,7 +16198,7 @@
         <v>2706</v>
       </c>
       <c r="C1433" t="n">
-        <v>14352</v>
+        <v>15548</v>
       </c>
     </row>
     <row r="1434">
@@ -16209,7 +16209,7 @@
         <v>2633</v>
       </c>
       <c r="C1434" t="n">
-        <v>10512</v>
+        <v>11388</v>
       </c>
     </row>
     <row r="1435">
@@ -16242,7 +16242,7 @@
         <v>2392</v>
       </c>
       <c r="C1437" t="n">
-        <v>113136</v>
+        <v>122564</v>
       </c>
     </row>
     <row r="1438">
@@ -16264,7 +16264,7 @@
         <v>2613</v>
       </c>
       <c r="C1439" t="n">
-        <v>79656</v>
+        <v>86294</v>
       </c>
     </row>
     <row r="1440">
@@ -16275,7 +16275,7 @@
         <v>2183</v>
       </c>
       <c r="C1440" t="n">
-        <v>286812</v>
+        <v>310713</v>
       </c>
     </row>
     <row r="1441">
@@ -16286,7 +16286,7 @@
         <v>2541</v>
       </c>
       <c r="C1441" t="n">
-        <v>128940</v>
+        <v>139685</v>
       </c>
     </row>
     <row r="1442">
@@ -16297,7 +16297,7 @@
         <v>2333</v>
       </c>
       <c r="C1442" t="n">
-        <v>87048</v>
+        <v>94302</v>
       </c>
     </row>
     <row r="1443">
@@ -16308,7 +16308,7 @@
         <v>2813</v>
       </c>
       <c r="C1443" t="n">
-        <v>34800</v>
+        <v>37700</v>
       </c>
     </row>
     <row r="1444">
@@ -16319,7 +16319,7 @@
         <v>2811</v>
       </c>
       <c r="C1444" t="n">
-        <v>22692</v>
+        <v>24583</v>
       </c>
     </row>
     <row r="1445">
@@ -16330,7 +16330,7 @@
         <v>1881</v>
       </c>
       <c r="C1445" t="n">
-        <v>37464</v>
+        <v>40586</v>
       </c>
     </row>
     <row r="1446">
@@ -16341,7 +16341,7 @@
         <v>2825</v>
       </c>
       <c r="C1446" t="n">
-        <v>30456</v>
+        <v>32994</v>
       </c>
     </row>
     <row r="1447">
@@ -16352,7 +16352,7 @@
         <v>970</v>
       </c>
       <c r="C1447" t="n">
-        <v>37464</v>
+        <v>40586</v>
       </c>
     </row>
     <row r="1448">
@@ -16363,7 +16363,7 @@
         <v>2552</v>
       </c>
       <c r="C1448" t="n">
-        <v>21324</v>
+        <v>23101</v>
       </c>
     </row>
     <row r="1449">
@@ -16374,7 +16374,7 @@
         <v>2562</v>
       </c>
       <c r="C1449" t="n">
-        <v>21324</v>
+        <v>23101</v>
       </c>
     </row>
     <row r="1450">
@@ -16407,7 +16407,7 @@
         <v>2747</v>
       </c>
       <c r="C1452" t="n">
-        <v>38172</v>
+        <v>41353</v>
       </c>
     </row>
     <row r="1453">
@@ -16418,7 +16418,7 @@
         <v>415</v>
       </c>
       <c r="C1453" t="n">
-        <v>136363.7</v>
+        <v>147727.33</v>
       </c>
     </row>
     <row r="1454">
@@ -16462,7 +16462,7 @@
         <v>2544</v>
       </c>
       <c r="C1457" t="n">
-        <v>38172</v>
+        <v>41353</v>
       </c>
     </row>
     <row r="1458">
@@ -16473,7 +16473,7 @@
         <v>816</v>
       </c>
       <c r="C1458" t="n">
-        <v>163636.4</v>
+        <v>177272.76</v>
       </c>
     </row>
     <row r="1459">
@@ -16484,7 +16484,7 @@
         <v>890</v>
       </c>
       <c r="C1459" t="n">
-        <v>490909.1</v>
+        <v>531818.1899999999</v>
       </c>
     </row>
     <row r="1460">
@@ -16495,7 +16495,7 @@
         <v>1298</v>
       </c>
       <c r="C1460" t="n">
-        <v>690000</v>
+        <v>747500</v>
       </c>
     </row>
     <row r="1461">
@@ -16506,7 +16506,7 @@
         <v>1372</v>
       </c>
       <c r="C1461" t="n">
-        <v>163636.4</v>
+        <v>177272.76</v>
       </c>
     </row>
     <row r="1462">
@@ -16517,7 +16517,7 @@
         <v>358</v>
       </c>
       <c r="C1462" t="n">
-        <v>171816</v>
+        <v>186134</v>
       </c>
     </row>
     <row r="1463">
@@ -16528,7 +16528,7 @@
         <v>1653</v>
       </c>
       <c r="C1463" t="n">
-        <v>171816</v>
+        <v>186134</v>
       </c>
     </row>
     <row r="1464">
@@ -16539,7 +16539,7 @@
         <v>675</v>
       </c>
       <c r="C1464" t="n">
-        <v>109080</v>
+        <v>118170</v>
       </c>
     </row>
     <row r="1465">
@@ -16550,7 +16550,7 @@
         <v>2804</v>
       </c>
       <c r="C1465" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1466">
@@ -16561,7 +16561,7 @@
         <v>2714</v>
       </c>
       <c r="C1466" t="n">
-        <v>196356</v>
+        <v>212719</v>
       </c>
     </row>
     <row r="1467">
@@ -16572,7 +16572,7 @@
         <v>2765</v>
       </c>
       <c r="C1467" t="n">
-        <v>49080</v>
+        <v>53170</v>
       </c>
     </row>
     <row r="1468">
@@ -16583,7 +16583,7 @@
         <v>2421</v>
       </c>
       <c r="C1468" t="n">
-        <v>33264</v>
+        <v>36036</v>
       </c>
     </row>
     <row r="1469">
@@ -16594,7 +16594,7 @@
         <v>2359</v>
       </c>
       <c r="C1469" t="n">
-        <v>56904</v>
+        <v>61646</v>
       </c>
     </row>
     <row r="1470">
@@ -16605,7 +16605,7 @@
         <v>2678</v>
       </c>
       <c r="C1470" t="n">
-        <v>53976</v>
+        <v>58474</v>
       </c>
     </row>
     <row r="1471">
@@ -16616,7 +16616,7 @@
         <v>2697</v>
       </c>
       <c r="C1471" t="n">
-        <v>81912</v>
+        <v>88738</v>
       </c>
     </row>
     <row r="1472">
@@ -16649,7 +16649,7 @@
         <v>2142</v>
       </c>
       <c r="C1474" t="n">
-        <v>29520</v>
+        <v>31980</v>
       </c>
     </row>
     <row r="1475">
@@ -16660,7 +16660,7 @@
         <v>2498</v>
       </c>
       <c r="C1475" t="n">
-        <v>30708</v>
+        <v>33267</v>
       </c>
     </row>
     <row r="1476">
@@ -16682,7 +16682,7 @@
         <v>2801</v>
       </c>
       <c r="C1477" t="n">
-        <v>54545.5</v>
+        <v>59090.95</v>
       </c>
     </row>
     <row r="1478">
@@ -16693,7 +16693,7 @@
         <v>2810</v>
       </c>
       <c r="C1478" t="n">
-        <v>87272.8</v>
+        <v>94545.52</v>
       </c>
     </row>
     <row r="1479">
@@ -16737,7 +16737,7 @@
         <v>132</v>
       </c>
       <c r="C1482" t="n">
-        <v>190909.1</v>
+        <v>206818.19</v>
       </c>
     </row>
     <row r="1483">
@@ -16759,7 +16759,7 @@
         <v>580</v>
       </c>
       <c r="C1484" t="n">
-        <v>95454.60000000001</v>
+        <v>103409.14</v>
       </c>
     </row>
     <row r="1485">
@@ -16770,7 +16770,7 @@
         <v>634</v>
       </c>
       <c r="C1485" t="n">
-        <v>272727.3</v>
+        <v>295454.57</v>
       </c>
     </row>
     <row r="1486">
@@ -16792,7 +16792,7 @@
         <v>1277</v>
       </c>
       <c r="C1487" t="n">
-        <v>120000</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="1488">
@@ -16803,7 +16803,7 @@
         <v>767</v>
       </c>
       <c r="C1488" t="n">
-        <v>109080</v>
+        <v>118170</v>
       </c>
     </row>
     <row r="1489">
@@ -16814,7 +16814,7 @@
         <v>2727</v>
       </c>
       <c r="C1489" t="n">
-        <v>22080</v>
+        <v>23920</v>
       </c>
     </row>
     <row r="1490">
@@ -16825,7 +16825,7 @@
         <v>2846</v>
       </c>
       <c r="C1490" t="n">
-        <v>141816</v>
+        <v>153634</v>
       </c>
     </row>
     <row r="1491">
@@ -16836,7 +16836,7 @@
         <v>609</v>
       </c>
       <c r="C1491" t="n">
-        <v>122724</v>
+        <v>132951</v>
       </c>
     </row>
     <row r="1492">
@@ -16847,7 +16847,7 @@
         <v>2726</v>
       </c>
       <c r="C1492" t="n">
-        <v>84540</v>
+        <v>91585</v>
       </c>
     </row>
     <row r="1493">
@@ -16858,7 +16858,7 @@
         <v>2729</v>
       </c>
       <c r="C1493" t="n">
-        <v>49080</v>
+        <v>53170</v>
       </c>
     </row>
     <row r="1494">
@@ -16869,7 +16869,7 @@
         <v>1340</v>
       </c>
       <c r="C1494" t="n">
-        <v>81816</v>
+        <v>88634</v>
       </c>
     </row>
     <row r="1495">
@@ -16880,7 +16880,7 @@
         <v>2830</v>
       </c>
       <c r="C1495" t="n">
-        <v>49080</v>
+        <v>53170</v>
       </c>
     </row>
     <row r="1496">
@@ -16891,7 +16891,7 @@
         <v>2674</v>
       </c>
       <c r="C1496" t="n">
-        <v>141816</v>
+        <v>153634</v>
       </c>
     </row>
     <row r="1497">
@@ -16902,7 +16902,7 @@
         <v>2308</v>
       </c>
       <c r="C1497" t="n">
-        <v>109080</v>
+        <v>118170</v>
       </c>
     </row>
     <row r="1498">
@@ -16913,7 +16913,7 @@
         <v>2190</v>
       </c>
       <c r="C1498" t="n">
-        <v>114540</v>
+        <v>124085</v>
       </c>
     </row>
     <row r="1499">
@@ -16924,7 +16924,7 @@
         <v>2015</v>
       </c>
       <c r="C1499" t="n">
-        <v>201816</v>
+        <v>218634</v>
       </c>
     </row>
     <row r="1500">
@@ -16935,7 +16935,7 @@
         <v>1308</v>
       </c>
       <c r="C1500" t="n">
-        <v>85632</v>
+        <v>92768</v>
       </c>
     </row>
     <row r="1501">
@@ -16946,7 +16946,7 @@
         <v>2118</v>
       </c>
       <c r="C1501" t="n">
-        <v>114636</v>
+        <v>124189</v>
       </c>
     </row>
     <row r="1502">
@@ -16957,7 +16957,7 @@
         <v>2607</v>
       </c>
       <c r="C1502" t="n">
-        <v>27096</v>
+        <v>29354</v>
       </c>
     </row>
     <row r="1503">
@@ -16968,7 +16968,7 @@
         <v>2832</v>
       </c>
       <c r="C1503" t="n">
-        <v>81818.2</v>
+        <v>88636.38</v>
       </c>
     </row>
     <row r="1504">
@@ -16979,7 +16979,7 @@
         <v>2383</v>
       </c>
       <c r="C1504" t="n">
-        <v>72504</v>
+        <v>78546</v>
       </c>
     </row>
     <row r="1505">
@@ -17012,7 +17012,7 @@
         <v>2821</v>
       </c>
       <c r="C1507" t="n">
-        <v>72732</v>
+        <v>78793</v>
       </c>
     </row>
     <row r="1508">
@@ -17034,7 +17034,7 @@
         <v>569</v>
       </c>
       <c r="C1509" t="n">
-        <v>1583688</v>
+        <v>1715662</v>
       </c>
     </row>
     <row r="1510">
@@ -17045,7 +17045,7 @@
         <v>2660</v>
       </c>
       <c r="C1510" t="n">
-        <v>190909.1</v>
+        <v>206818.19</v>
       </c>
     </row>
     <row r="1511">
@@ -17056,7 +17056,7 @@
         <v>1632</v>
       </c>
       <c r="C1511" t="n">
-        <v>141818.2</v>
+        <v>153636.38</v>
       </c>
     </row>
     <row r="1512">
@@ -17067,7 +17067,7 @@
         <v>1756</v>
       </c>
       <c r="C1512" t="n">
-        <v>229080</v>
+        <v>248170</v>
       </c>
     </row>
     <row r="1513">
@@ -17078,7 +17078,7 @@
         <v>58</v>
       </c>
       <c r="C1513" t="n">
-        <v>136800</v>
+        <v>148200</v>
       </c>
     </row>
     <row r="1514">
@@ -17089,7 +17089,7 @@
         <v>40</v>
       </c>
       <c r="C1514" t="n">
-        <v>121680</v>
+        <v>131820</v>
       </c>
     </row>
     <row r="1515">
@@ -17100,7 +17100,7 @@
         <v>559</v>
       </c>
       <c r="C1515" t="n">
-        <v>127632</v>
+        <v>138268</v>
       </c>
     </row>
     <row r="1516">
@@ -17111,7 +17111,7 @@
         <v>2773</v>
       </c>
       <c r="C1516" t="n">
-        <v>44004</v>
+        <v>47671</v>
       </c>
     </row>
     <row r="1517">
@@ -17122,7 +17122,7 @@
         <v>2631</v>
       </c>
       <c r="C1517" t="n">
-        <v>21132</v>
+        <v>22893</v>
       </c>
     </row>
     <row r="1518">
@@ -17133,7 +17133,7 @@
         <v>2085</v>
       </c>
       <c r="C1518" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1519">
@@ -17155,7 +17155,7 @@
         <v>1642</v>
       </c>
       <c r="C1520" t="n">
-        <v>144540</v>
+        <v>156585</v>
       </c>
     </row>
     <row r="1521">
@@ -17166,7 +17166,7 @@
         <v>2621</v>
       </c>
       <c r="C1521" t="n">
-        <v>38172</v>
+        <v>41353</v>
       </c>
     </row>
     <row r="1522">
@@ -17177,7 +17177,7 @@
         <v>2705</v>
       </c>
       <c r="C1522" t="n">
-        <v>109512</v>
+        <v>118638</v>
       </c>
     </row>
     <row r="1523">
@@ -17188,7 +17188,7 @@
         <v>2735</v>
       </c>
       <c r="C1523" t="n">
-        <v>65448</v>
+        <v>70902</v>
       </c>
     </row>
     <row r="1524">
@@ -17199,7 +17199,7 @@
         <v>945</v>
       </c>
       <c r="C1524" t="n">
-        <v>191280</v>
+        <v>207220</v>
       </c>
     </row>
     <row r="1525">
@@ -17210,7 +17210,7 @@
         <v>2582</v>
       </c>
       <c r="C1525" t="n">
-        <v>47856</v>
+        <v>51844</v>
       </c>
     </row>
     <row r="1526">
@@ -17221,7 +17221,7 @@
         <v>2584</v>
       </c>
       <c r="C1526" t="n">
-        <v>34800</v>
+        <v>37700</v>
       </c>
     </row>
     <row r="1527">
@@ -17232,7 +17232,7 @@
         <v>2689</v>
       </c>
       <c r="C1527" t="n">
-        <v>34800</v>
+        <v>37700</v>
       </c>
     </row>
     <row r="1528">
@@ -17243,7 +17243,7 @@
         <v>2574</v>
       </c>
       <c r="C1528" t="n">
-        <v>76488</v>
+        <v>82862</v>
       </c>
     </row>
     <row r="1529">
@@ -17254,7 +17254,7 @@
         <v>1834</v>
       </c>
       <c r="C1529" t="n">
-        <v>64200</v>
+        <v>69550</v>
       </c>
     </row>
     <row r="1530">
@@ -17265,7 +17265,7 @@
         <v>2629</v>
       </c>
       <c r="C1530" t="n">
-        <v>37464</v>
+        <v>40586</v>
       </c>
     </row>
     <row r="1531">
@@ -17276,7 +17276,7 @@
         <v>933</v>
       </c>
       <c r="C1531" t="n">
-        <v>44436</v>
+        <v>48139</v>
       </c>
     </row>
     <row r="1532">
@@ -17287,7 +17287,7 @@
         <v>2555</v>
       </c>
       <c r="C1532" t="n">
-        <v>21324</v>
+        <v>23101</v>
       </c>
     </row>
     <row r="1533">
@@ -17298,7 +17298,7 @@
         <v>2558</v>
       </c>
       <c r="C1533" t="n">
-        <v>21324</v>
+        <v>23101</v>
       </c>
     </row>
     <row r="1534">
@@ -17309,7 +17309,7 @@
         <v>2721</v>
       </c>
       <c r="C1534" t="n">
-        <v>44436</v>
+        <v>48139</v>
       </c>
     </row>
     <row r="1535">
@@ -17320,7 +17320,7 @@
         <v>2556</v>
       </c>
       <c r="C1535" t="n">
-        <v>21324</v>
+        <v>23101</v>
       </c>
     </row>
     <row r="1536">
@@ -17331,7 +17331,7 @@
         <v>2826</v>
       </c>
       <c r="C1536" t="n">
-        <v>38172</v>
+        <v>41353</v>
       </c>
     </row>
     <row r="1537">
@@ -17353,7 +17353,7 @@
         <v>2346</v>
       </c>
       <c r="C1538" t="n">
-        <v>38172</v>
+        <v>41353</v>
       </c>
     </row>
     <row r="1539">
@@ -17364,7 +17364,7 @@
         <v>595</v>
       </c>
       <c r="C1539" t="n">
-        <v>136363.7</v>
+        <v>147727.33</v>
       </c>
     </row>
     <row r="1540">
@@ -17375,7 +17375,7 @@
         <v>1278</v>
       </c>
       <c r="C1540" t="n">
-        <v>95454.60000000001</v>
+        <v>103409.14</v>
       </c>
     </row>
     <row r="1541">
@@ -17386,7 +17386,7 @@
         <v>2686</v>
       </c>
       <c r="C1541" t="n">
-        <v>76356</v>
+        <v>82719</v>
       </c>
     </row>
     <row r="1542">
@@ -17397,7 +17397,7 @@
         <v>1344</v>
       </c>
       <c r="C1542" t="n">
-        <v>81816</v>
+        <v>88634</v>
       </c>
     </row>
     <row r="1543">
@@ -17408,7 +17408,7 @@
         <v>2566</v>
       </c>
       <c r="C1543" t="n">
-        <v>43632</v>
+        <v>47268</v>
       </c>
     </row>
     <row r="1544">
@@ -17419,7 +17419,7 @@
         <v>2684</v>
       </c>
       <c r="C1544" t="n">
-        <v>51816</v>
+        <v>56134</v>
       </c>
     </row>
     <row r="1545">
@@ -17430,7 +17430,7 @@
         <v>2375</v>
       </c>
       <c r="C1545" t="n">
-        <v>180000</v>
+        <v>195000</v>
       </c>
     </row>
     <row r="1546">
@@ -17441,7 +17441,7 @@
         <v>2829</v>
       </c>
       <c r="C1546" t="n">
-        <v>32724</v>
+        <v>35451</v>
       </c>
     </row>
     <row r="1547">
@@ -17452,7 +17452,7 @@
         <v>768</v>
       </c>
       <c r="C1547" t="n">
-        <v>76356</v>
+        <v>82719</v>
       </c>
     </row>
     <row r="1548">
@@ -17463,7 +17463,7 @@
         <v>772</v>
       </c>
       <c r="C1548" t="n">
-        <v>177264</v>
+        <v>192036</v>
       </c>
     </row>
     <row r="1549">
@@ -17474,7 +17474,7 @@
         <v>2496</v>
       </c>
       <c r="C1549" t="n">
-        <v>109080</v>
+        <v>118170</v>
       </c>
     </row>
     <row r="1550">
@@ -17485,7 +17485,7 @@
         <v>802</v>
       </c>
       <c r="C1550" t="n">
-        <v>40908</v>
+        <v>44317</v>
       </c>
     </row>
     <row r="1551">
@@ -17496,7 +17496,7 @@
         <v>2131</v>
       </c>
       <c r="C1551" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1552">
@@ -17507,7 +17507,7 @@
         <v>1381</v>
       </c>
       <c r="C1552" t="n">
-        <v>163636.4</v>
+        <v>177272.76</v>
       </c>
     </row>
     <row r="1553">
@@ -17518,7 +17518,7 @@
         <v>2847</v>
       </c>
       <c r="C1553" t="n">
-        <v>73632</v>
+        <v>79768</v>
       </c>
     </row>
     <row r="1554">
@@ -17529,7 +17529,7 @@
         <v>1293</v>
       </c>
       <c r="C1554" t="n">
-        <v>210000</v>
+        <v>227500</v>
       </c>
     </row>
     <row r="1555">
@@ -17540,7 +17540,7 @@
         <v>2363</v>
       </c>
       <c r="C1555" t="n">
-        <v>92724</v>
+        <v>100451</v>
       </c>
     </row>
     <row r="1556">
@@ -17551,7 +17551,7 @@
         <v>631</v>
       </c>
       <c r="C1556" t="n">
-        <v>190908</v>
+        <v>206817</v>
       </c>
     </row>
     <row r="1557">
@@ -17562,7 +17562,7 @@
         <v>2791</v>
       </c>
       <c r="C1557" t="n">
-        <v>56004</v>
+        <v>60671</v>
       </c>
     </row>
     <row r="1558">
@@ -17584,7 +17584,7 @@
         <v>2841</v>
       </c>
       <c r="C1559" t="n">
-        <v>27264</v>
+        <v>29536</v>
       </c>
     </row>
     <row r="1560">
@@ -17595,7 +17595,7 @@
         <v>2571</v>
       </c>
       <c r="C1560" t="n">
-        <v>145404</v>
+        <v>157521</v>
       </c>
     </row>
     <row r="1561">
@@ -17661,7 +17661,7 @@
         <v>2273</v>
       </c>
       <c r="C1566" t="n">
-        <v>117276</v>
+        <v>127049</v>
       </c>
     </row>
     <row r="1567">
@@ -17672,7 +17672,7 @@
         <v>2381</v>
       </c>
       <c r="C1567" t="n">
-        <v>43860</v>
+        <v>47515</v>
       </c>
     </row>
     <row r="1568">
@@ -17683,7 +17683,7 @@
         <v>630</v>
       </c>
       <c r="C1568" t="n">
-        <v>45016.35</v>
+        <v>48767.71</v>
       </c>
     </row>
     <row r="1569">
@@ -17705,7 +17705,7 @@
         <v>1983</v>
       </c>
       <c r="C1570" t="n">
-        <v>299040</v>
+        <v>323960</v>
       </c>
     </row>
     <row r="1571">
@@ -17716,7 +17716,7 @@
         <v>1993</v>
       </c>
       <c r="C1571" t="n">
-        <v>203064</v>
+        <v>219986</v>
       </c>
     </row>
     <row r="1572">
@@ -17727,7 +17727,7 @@
         <v>89</v>
       </c>
       <c r="C1572" t="n">
-        <v>190908</v>
+        <v>206817</v>
       </c>
     </row>
     <row r="1573">
@@ -17738,7 +17738,7 @@
         <v>1063</v>
       </c>
       <c r="C1573" t="n">
-        <v>210000</v>
+        <v>227500</v>
       </c>
     </row>
     <row r="1574">
@@ -17749,7 +17749,7 @@
         <v>1116</v>
       </c>
       <c r="C1574" t="n">
-        <v>136356</v>
+        <v>147719</v>
       </c>
     </row>
     <row r="1575">
@@ -17760,7 +17760,7 @@
         <v>941</v>
       </c>
       <c r="C1575" t="n">
-        <v>164124</v>
+        <v>177801</v>
       </c>
     </row>
     <row r="1576">
@@ -17771,7 +17771,7 @@
         <v>2141</v>
       </c>
       <c r="C1576" t="n">
-        <v>17496</v>
+        <v>18954</v>
       </c>
     </row>
     <row r="1577">
@@ -17782,7 +17782,7 @@
         <v>2463</v>
       </c>
       <c r="C1577" t="n">
-        <v>179904</v>
+        <v>194896</v>
       </c>
     </row>
     <row r="1578">
@@ -17793,7 +17793,7 @@
         <v>2707</v>
       </c>
       <c r="C1578" t="n">
-        <v>23556</v>
+        <v>25519</v>
       </c>
     </row>
     <row r="1579">
@@ -17804,7 +17804,7 @@
         <v>2325</v>
       </c>
       <c r="C1579" t="n">
-        <v>62928</v>
+        <v>68172</v>
       </c>
     </row>
     <row r="1580">
@@ -17848,7 +17848,7 @@
         <v>1890</v>
       </c>
       <c r="C1583" t="n">
-        <v>133764</v>
+        <v>144911</v>
       </c>
     </row>
     <row r="1584">
@@ -17859,7 +17859,7 @@
         <v>2639</v>
       </c>
       <c r="C1584" t="n">
-        <v>21852</v>
+        <v>23673</v>
       </c>
     </row>
     <row r="1585">
@@ -17870,7 +17870,7 @@
         <v>2682</v>
       </c>
       <c r="C1585" t="n">
-        <v>76356</v>
+        <v>82719</v>
       </c>
     </row>
     <row r="1586">
@@ -17881,7 +17881,7 @@
         <v>2601</v>
       </c>
       <c r="C1586" t="n">
-        <v>150000</v>
+        <v>162500</v>
       </c>
     </row>
     <row r="1587">
@@ -17892,7 +17892,7 @@
         <v>1142</v>
       </c>
       <c r="C1587" t="n">
-        <v>249864</v>
+        <v>270686</v>
       </c>
     </row>
     <row r="1588">
@@ -17936,7 +17936,7 @@
         <v>2082</v>
       </c>
       <c r="C1591" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1592">
@@ -17947,7 +17947,7 @@
         <v>2276</v>
       </c>
       <c r="C1592" t="n">
-        <v>108504</v>
+        <v>117546</v>
       </c>
     </row>
     <row r="1593">
@@ -17958,7 +17958,7 @@
         <v>2786</v>
       </c>
       <c r="C1593" t="n">
-        <v>38172</v>
+        <v>41353</v>
       </c>
     </row>
     <row r="1594">
@@ -17969,7 +17969,7 @@
         <v>2816</v>
       </c>
       <c r="C1594" t="n">
-        <v>70908</v>
+        <v>76817</v>
       </c>
     </row>
     <row r="1595">
@@ -17980,7 +17980,7 @@
         <v>1871</v>
       </c>
       <c r="C1595" t="n">
-        <v>78276</v>
+        <v>84799</v>
       </c>
     </row>
     <row r="1596">
@@ -17991,7 +17991,7 @@
         <v>2345</v>
       </c>
       <c r="C1596" t="n">
-        <v>34800</v>
+        <v>37700</v>
       </c>
     </row>
     <row r="1597">
@@ -18002,7 +18002,7 @@
         <v>2802</v>
       </c>
       <c r="C1597" t="n">
-        <v>39156</v>
+        <v>42419</v>
       </c>
     </row>
     <row r="1598">
@@ -18013,7 +18013,7 @@
         <v>2090</v>
       </c>
       <c r="C1598" t="n">
-        <v>22692</v>
+        <v>24583</v>
       </c>
     </row>
     <row r="1599">
@@ -18024,7 +18024,7 @@
         <v>2647</v>
       </c>
       <c r="C1599" t="n">
-        <v>76500</v>
+        <v>82875</v>
       </c>
     </row>
     <row r="1600">
@@ -18035,7 +18035,7 @@
         <v>2365</v>
       </c>
       <c r="C1600" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1601">
@@ -18046,7 +18046,7 @@
         <v>766</v>
       </c>
       <c r="C1601" t="n">
-        <v>37464</v>
+        <v>40586</v>
       </c>
     </row>
     <row r="1602">
@@ -18057,7 +18057,7 @@
         <v>2702</v>
       </c>
       <c r="C1602" t="n">
-        <v>44436</v>
+        <v>48139</v>
       </c>
     </row>
     <row r="1603">
@@ -18068,7 +18068,7 @@
         <v>20</v>
       </c>
       <c r="C1603" t="n">
-        <v>245454.6</v>
+        <v>265909.14</v>
       </c>
     </row>
     <row r="1604">
@@ -18079,7 +18079,7 @@
         <v>27</v>
       </c>
       <c r="C1604" t="n">
-        <v>81818.2</v>
+        <v>88636.38</v>
       </c>
     </row>
     <row r="1605">
@@ -18090,7 +18090,7 @@
         <v>33</v>
       </c>
       <c r="C1605" t="n">
-        <v>217080</v>
+        <v>235170</v>
       </c>
     </row>
     <row r="1606">
@@ -18112,7 +18112,7 @@
         <v>2561</v>
       </c>
       <c r="C1607" t="n">
-        <v>21324</v>
+        <v>23101</v>
       </c>
     </row>
     <row r="1608">
@@ -18134,7 +18134,7 @@
         <v>2772</v>
       </c>
       <c r="C1609" t="n">
-        <v>32724</v>
+        <v>35451</v>
       </c>
     </row>
     <row r="1610">
@@ -18145,7 +18145,7 @@
         <v>2834</v>
       </c>
       <c r="C1610" t="n">
-        <v>20328</v>
+        <v>22022</v>
       </c>
     </row>
     <row r="1611">
@@ -18156,7 +18156,7 @@
         <v>2394</v>
       </c>
       <c r="C1611" t="n">
-        <v>61884</v>
+        <v>67041</v>
       </c>
     </row>
     <row r="1612">
@@ -18167,7 +18167,7 @@
         <v>2567</v>
       </c>
       <c r="C1612" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1613">
@@ -18178,7 +18178,7 @@
         <v>952</v>
       </c>
       <c r="C1613" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1614">
@@ -18189,7 +18189,7 @@
         <v>1539</v>
       </c>
       <c r="C1614" t="n">
-        <v>92724</v>
+        <v>100451</v>
       </c>
     </row>
     <row r="1615">
@@ -18200,7 +18200,7 @@
         <v>793</v>
       </c>
       <c r="C1615" t="n">
-        <v>22692</v>
+        <v>24583</v>
       </c>
     </row>
     <row r="1616">
@@ -18211,7 +18211,7 @@
         <v>794</v>
       </c>
       <c r="C1616" t="n">
-        <v>22692</v>
+        <v>24583</v>
       </c>
     </row>
     <row r="1617">
@@ -18222,7 +18222,7 @@
         <v>2838</v>
       </c>
       <c r="C1617" t="n">
-        <v>32727.3</v>
+        <v>35454.57</v>
       </c>
     </row>
     <row r="1618">
@@ -18233,7 +18233,7 @@
         <v>2223</v>
       </c>
       <c r="C1618" t="n">
-        <v>63876</v>
+        <v>69199</v>
       </c>
     </row>
     <row r="1619">
@@ -18244,7 +18244,7 @@
         <v>2547</v>
       </c>
       <c r="C1619" t="n">
-        <v>18480</v>
+        <v>20020</v>
       </c>
     </row>
     <row r="1620">
@@ -18255,7 +18255,7 @@
         <v>2762</v>
       </c>
       <c r="C1620" t="n">
-        <v>44436</v>
+        <v>48139</v>
       </c>
     </row>
     <row r="1621">
@@ -18266,7 +18266,7 @@
         <v>2550</v>
       </c>
       <c r="C1621" t="n">
-        <v>21324</v>
+        <v>23101</v>
       </c>
     </row>
     <row r="1622">
@@ -18277,7 +18277,7 @@
         <v>2627</v>
       </c>
       <c r="C1622" t="n">
-        <v>21324</v>
+        <v>23101</v>
       </c>
     </row>
     <row r="1623">
@@ -18299,7 +18299,7 @@
         <v>749</v>
       </c>
       <c r="C1624" t="n">
-        <v>44436</v>
+        <v>48139</v>
       </c>
     </row>
     <row r="1625">
@@ -18310,7 +18310,7 @@
         <v>2549</v>
       </c>
       <c r="C1625" t="n">
-        <v>21324</v>
+        <v>23101</v>
       </c>
     </row>
     <row r="1626">
@@ -18321,7 +18321,7 @@
         <v>2649</v>
       </c>
       <c r="C1626" t="n">
-        <v>21324</v>
+        <v>23101</v>
       </c>
     </row>
     <row r="1627">
@@ -18332,7 +18332,7 @@
         <v>2258</v>
       </c>
       <c r="C1627" t="n">
-        <v>43632</v>
+        <v>47268</v>
       </c>
     </row>
     <row r="1628">
@@ -18343,7 +18343,7 @@
         <v>2744</v>
       </c>
       <c r="C1628" t="n">
-        <v>32724</v>
+        <v>35451</v>
       </c>
     </row>
     <row r="1629">
@@ -18354,7 +18354,7 @@
         <v>452</v>
       </c>
       <c r="C1629" t="n">
-        <v>154356</v>
+        <v>167219</v>
       </c>
     </row>
     <row r="1630">
@@ -18376,7 +18376,7 @@
         <v>2653</v>
       </c>
       <c r="C1631" t="n">
-        <v>32724</v>
+        <v>35451</v>
       </c>
     </row>
     <row r="1632">
@@ -18409,7 +18409,7 @@
         <v>2742</v>
       </c>
       <c r="C1634" t="n">
-        <v>10908</v>
+        <v>11817</v>
       </c>
     </row>
     <row r="1635">
@@ -18420,7 +18420,7 @@
         <v>1499</v>
       </c>
       <c r="C1635" t="n">
-        <v>49080</v>
+        <v>53170</v>
       </c>
     </row>
     <row r="1636">
@@ -18431,7 +18431,7 @@
         <v>2261</v>
       </c>
       <c r="C1636" t="n">
-        <v>98172</v>
+        <v>106353</v>
       </c>
     </row>
     <row r="1637">
@@ -18442,7 +18442,7 @@
         <v>1324</v>
       </c>
       <c r="C1637" t="n">
-        <v>152724</v>
+        <v>165451</v>
       </c>
     </row>
     <row r="1638">
@@ -18453,7 +18453,7 @@
         <v>2709</v>
       </c>
       <c r="C1638" t="n">
-        <v>98172</v>
+        <v>106353</v>
       </c>
     </row>
     <row r="1639">
@@ -18464,7 +18464,7 @@
         <v>1137</v>
       </c>
       <c r="C1639" t="n">
-        <v>349080</v>
+        <v>378170</v>
       </c>
     </row>
     <row r="1640">
@@ -18475,7 +18475,7 @@
         <v>2440</v>
       </c>
       <c r="C1640" t="n">
-        <v>43632</v>
+        <v>47268</v>
       </c>
     </row>
     <row r="1641">
@@ -18486,7 +18486,7 @@
         <v>429</v>
       </c>
       <c r="C1641" t="n">
-        <v>207264</v>
+        <v>224536</v>
       </c>
     </row>
     <row r="1642">
@@ -18497,7 +18497,7 @@
         <v>2114</v>
       </c>
       <c r="C1642" t="n">
-        <v>92796</v>
+        <v>100529</v>
       </c>
     </row>
     <row r="1643">
@@ -18508,7 +18508,7 @@
         <v>2211</v>
       </c>
       <c r="C1643" t="n">
-        <v>131364</v>
+        <v>142311</v>
       </c>
     </row>
     <row r="1644">
@@ -18519,7 +18519,7 @@
         <v>1108</v>
       </c>
       <c r="C1644" t="n">
-        <v>167112</v>
+        <v>181038</v>
       </c>
     </row>
     <row r="1645">
@@ -18530,7 +18530,7 @@
         <v>2695</v>
       </c>
       <c r="C1645" t="n">
-        <v>26388</v>
+        <v>28587</v>
       </c>
     </row>
     <row r="1646">
@@ -18541,7 +18541,7 @@
         <v>1289</v>
       </c>
       <c r="C1646" t="n">
-        <v>150000</v>
+        <v>162500</v>
       </c>
     </row>
     <row r="1647">
@@ -18552,7 +18552,7 @@
         <v>2789</v>
       </c>
       <c r="C1647" t="n">
-        <v>98181.89999999999</v>
+        <v>106363.71</v>
       </c>
     </row>
     <row r="1648">
@@ -18563,7 +18563,7 @@
         <v>2197</v>
       </c>
       <c r="C1648" t="n">
-        <v>117272.8</v>
+        <v>127045.52</v>
       </c>
     </row>
     <row r="1649">
@@ -18574,7 +18574,7 @@
         <v>947</v>
       </c>
       <c r="C1649" t="n">
-        <v>241896</v>
+        <v>262054</v>
       </c>
     </row>
     <row r="1650">
@@ -18585,7 +18585,7 @@
         <v>2279</v>
       </c>
       <c r="C1650" t="n">
-        <v>133596</v>
+        <v>144729</v>
       </c>
     </row>
     <row r="1651">
@@ -18596,7 +18596,7 @@
         <v>1465</v>
       </c>
       <c r="C1651" t="n">
-        <v>210000</v>
+        <v>227500</v>
       </c>
     </row>
     <row r="1652">
@@ -18607,7 +18607,7 @@
         <v>2651</v>
       </c>
       <c r="C1652" t="n">
-        <v>92724</v>
+        <v>100451</v>
       </c>
     </row>
     <row r="1653">
@@ -18618,7 +18618,7 @@
         <v>42</v>
       </c>
       <c r="C1653" t="n">
-        <v>1039632</v>
+        <v>1126268</v>
       </c>
     </row>
     <row r="1654">
@@ -18629,7 +18629,7 @@
         <v>949</v>
       </c>
       <c r="C1654" t="n">
-        <v>54252</v>
+        <v>58773</v>
       </c>
     </row>
     <row r="1655">
@@ -18640,7 +18640,7 @@
         <v>2606</v>
       </c>
       <c r="C1655" t="n">
-        <v>140040</v>
+        <v>151710</v>
       </c>
     </row>
     <row r="1656">
@@ -18651,7 +18651,7 @@
         <v>2249</v>
       </c>
       <c r="C1656" t="n">
-        <v>118980</v>
+        <v>128895</v>
       </c>
     </row>
     <row r="1657">
@@ -18695,7 +18695,7 @@
         <v>2045</v>
       </c>
       <c r="C1660" t="n">
-        <v>173712</v>
+        <v>188188</v>
       </c>
     </row>
     <row r="1661">
@@ -18706,7 +18706,7 @@
         <v>2663</v>
       </c>
       <c r="C1661" t="n">
-        <v>150000</v>
+        <v>162500</v>
       </c>
     </row>
     <row r="1662">
@@ -18728,7 +18728,7 @@
         <v>2854</v>
       </c>
       <c r="C1663" t="n">
-        <v>21816</v>
+        <v>23634</v>
       </c>
     </row>
     <row r="1664">
@@ -18750,7 +18750,7 @@
         <v>2341</v>
       </c>
       <c r="C1665" t="n">
-        <v>95400</v>
+        <v>103350</v>
       </c>
     </row>
     <row r="1666">
@@ -18761,7 +18761,7 @@
         <v>2637</v>
       </c>
       <c r="C1666" t="n">
-        <v>34800</v>
+        <v>37700</v>
       </c>
     </row>
     <row r="1667">
@@ -18772,7 +18772,7 @@
         <v>2492</v>
       </c>
       <c r="C1667" t="n">
-        <v>54636</v>
+        <v>59189</v>
       </c>
     </row>
     <row r="1668">
@@ -18783,7 +18783,7 @@
         <v>2548</v>
       </c>
       <c r="C1668" t="n">
-        <v>21324</v>
+        <v>23101</v>
       </c>
     </row>
     <row r="1669">
@@ -18794,7 +18794,7 @@
         <v>351</v>
       </c>
       <c r="C1669" t="n">
-        <v>116172</v>
+        <v>125853</v>
       </c>
     </row>
     <row r="1670">
@@ -18827,7 +18827,7 @@
         <v>2757</v>
       </c>
       <c r="C1672" t="n">
-        <v>43632</v>
+        <v>47268</v>
       </c>
     </row>
     <row r="1673">
@@ -18838,7 +18838,7 @@
         <v>2815</v>
       </c>
       <c r="C1673" t="n">
-        <v>32724</v>
+        <v>35451</v>
       </c>
     </row>
     <row r="1674">
@@ -18849,7 +18849,7 @@
         <v>2323</v>
       </c>
       <c r="C1674" t="n">
-        <v>37464</v>
+        <v>40586</v>
       </c>
     </row>
     <row r="1675">
@@ -18860,7 +18860,7 @@
         <v>2310</v>
       </c>
       <c r="C1675" t="n">
-        <v>37464</v>
+        <v>40586</v>
       </c>
     </row>
     <row r="1676">
@@ -18871,7 +18871,7 @@
         <v>2145</v>
       </c>
       <c r="C1676" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1677">
@@ -18882,7 +18882,7 @@
         <v>2501</v>
       </c>
       <c r="C1677" t="n">
-        <v>44436</v>
+        <v>48139</v>
       </c>
     </row>
     <row r="1678">
@@ -18893,7 +18893,7 @@
         <v>2546</v>
       </c>
       <c r="C1678" t="n">
-        <v>21324</v>
+        <v>23101</v>
       </c>
     </row>
     <row r="1679">
@@ -18904,7 +18904,7 @@
         <v>716</v>
       </c>
       <c r="C1679" t="n">
-        <v>69912</v>
+        <v>75738</v>
       </c>
     </row>
     <row r="1680">
@@ -18915,7 +18915,7 @@
         <v>2758</v>
       </c>
       <c r="C1680" t="n">
-        <v>32724</v>
+        <v>35451</v>
       </c>
     </row>
     <row r="1681">
@@ -18926,7 +18926,7 @@
         <v>400</v>
       </c>
       <c r="C1681" t="n">
-        <v>98172</v>
+        <v>106353</v>
       </c>
     </row>
     <row r="1682">
@@ -18937,7 +18937,7 @@
         <v>6</v>
       </c>
       <c r="C1682" t="n">
-        <v>27272.8</v>
+        <v>29545.52</v>
       </c>
     </row>
     <row r="1683">
@@ -18970,7 +18970,7 @@
         <v>1259</v>
       </c>
       <c r="C1685" t="n">
-        <v>60000</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="1686">
@@ -18981,7 +18981,7 @@
         <v>571</v>
       </c>
       <c r="C1686" t="n">
-        <v>564545.5</v>
+        <v>611590.95</v>
       </c>
     </row>
     <row r="1687">
@@ -18992,7 +18992,7 @@
         <v>703</v>
       </c>
       <c r="C1687" t="n">
-        <v>136356</v>
+        <v>147719</v>
       </c>
     </row>
     <row r="1688">
@@ -19014,7 +19014,7 @@
         <v>2833</v>
       </c>
       <c r="C1689" t="n">
-        <v>43632</v>
+        <v>47268</v>
       </c>
     </row>
     <row r="1690">
@@ -19025,7 +19025,7 @@
         <v>1007</v>
       </c>
       <c r="C1690" t="n">
-        <v>109091</v>
+        <v>118181.9</v>
       </c>
     </row>
     <row r="1691">
@@ -19036,7 +19036,7 @@
         <v>2687</v>
       </c>
       <c r="C1691" t="n">
-        <v>43632</v>
+        <v>47268</v>
       </c>
     </row>
     <row r="1692">
@@ -19047,7 +19047,7 @@
         <v>2824</v>
       </c>
       <c r="C1692" t="n">
-        <v>61584</v>
+        <v>66716</v>
       </c>
     </row>
     <row r="1693">
@@ -19058,7 +19058,7 @@
         <v>2730</v>
       </c>
       <c r="C1693" t="n">
-        <v>49080</v>
+        <v>53170</v>
       </c>
     </row>
     <row r="1694">
@@ -19069,7 +19069,7 @@
         <v>2718</v>
       </c>
       <c r="C1694" t="n">
-        <v>70908</v>
+        <v>76817</v>
       </c>
     </row>
     <row r="1695">
@@ -19080,7 +19080,7 @@
         <v>2750</v>
       </c>
       <c r="C1695" t="n">
-        <v>16356</v>
+        <v>17719</v>
       </c>
     </row>
     <row r="1696">
@@ -19091,7 +19091,7 @@
         <v>854</v>
       </c>
       <c r="C1696" t="n">
-        <v>76356</v>
+        <v>82719</v>
       </c>
     </row>
     <row r="1697">
@@ -19102,7 +19102,7 @@
         <v>2794</v>
       </c>
       <c r="C1697" t="n">
-        <v>65448</v>
+        <v>70902</v>
       </c>
     </row>
     <row r="1698">
@@ -19113,7 +19113,7 @@
         <v>1374</v>
       </c>
       <c r="C1698" t="n">
-        <v>109080</v>
+        <v>118170</v>
       </c>
     </row>
     <row r="1699">
@@ -19124,7 +19124,7 @@
         <v>2488</v>
       </c>
       <c r="C1699" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1700">
@@ -19135,7 +19135,7 @@
         <v>363</v>
       </c>
       <c r="C1700" t="n">
-        <v>163632</v>
+        <v>177268</v>
       </c>
     </row>
     <row r="1701">
@@ -19146,7 +19146,7 @@
         <v>2655</v>
       </c>
       <c r="C1701" t="n">
-        <v>60000</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="1702">
@@ -19157,7 +19157,7 @@
         <v>1873</v>
       </c>
       <c r="C1702" t="n">
-        <v>174540</v>
+        <v>189085</v>
       </c>
     </row>
     <row r="1703">
@@ -19168,7 +19168,7 @@
         <v>2635</v>
       </c>
       <c r="C1703" t="n">
-        <v>70908</v>
+        <v>76817</v>
       </c>
     </row>
     <row r="1704">
@@ -19179,7 +19179,7 @@
         <v>1658</v>
       </c>
       <c r="C1704" t="n">
-        <v>83448</v>
+        <v>90402</v>
       </c>
     </row>
     <row r="1705">
@@ -19190,7 +19190,7 @@
         <v>2069</v>
       </c>
       <c r="C1705" t="n">
-        <v>109091</v>
+        <v>118181.9</v>
       </c>
     </row>
     <row r="1706">
@@ -19201,7 +19201,7 @@
         <v>2081</v>
       </c>
       <c r="C1706" t="n">
-        <v>81816</v>
+        <v>88634</v>
       </c>
     </row>
     <row r="1707">
@@ -19212,7 +19212,7 @@
         <v>2124</v>
       </c>
       <c r="C1707" t="n">
-        <v>190908</v>
+        <v>206817</v>
       </c>
     </row>
     <row r="1708">
@@ -19223,7 +19223,7 @@
         <v>636</v>
       </c>
       <c r="C1708" t="n">
-        <v>136356</v>
+        <v>147719</v>
       </c>
     </row>
     <row r="1709">
@@ -19234,7 +19234,7 @@
         <v>2803</v>
       </c>
       <c r="C1709" t="n">
-        <v>65448</v>
+        <v>70902</v>
       </c>
     </row>
     <row r="1710">
@@ -19245,7 +19245,7 @@
         <v>2163</v>
       </c>
       <c r="C1710" t="n">
-        <v>98172</v>
+        <v>106353</v>
       </c>
     </row>
     <row r="1711">
@@ -19256,7 +19256,7 @@
         <v>1466</v>
       </c>
       <c r="C1711" t="n">
-        <v>220908</v>
+        <v>239317</v>
       </c>
     </row>
     <row r="1712">
@@ -19267,7 +19267,7 @@
         <v>2133</v>
       </c>
       <c r="C1712" t="n">
-        <v>190909.1</v>
+        <v>206818.19</v>
       </c>
     </row>
     <row r="1713">
@@ -19278,7 +19278,7 @@
         <v>2431</v>
       </c>
       <c r="C1713" t="n">
-        <v>81816</v>
+        <v>88634</v>
       </c>
     </row>
     <row r="1714">
@@ -19289,7 +19289,7 @@
         <v>535</v>
       </c>
       <c r="C1714" t="n">
-        <v>194280</v>
+        <v>210470</v>
       </c>
     </row>
     <row r="1715">
@@ -19300,7 +19300,7 @@
         <v>2790</v>
       </c>
       <c r="C1715" t="n">
-        <v>34452</v>
+        <v>37323</v>
       </c>
     </row>
     <row r="1716">
@@ -19311,7 +19311,7 @@
         <v>2442</v>
       </c>
       <c r="C1716" t="n">
-        <v>141264</v>
+        <v>153036</v>
       </c>
     </row>
     <row r="1717">
@@ -19322,7 +19322,7 @@
         <v>2376</v>
       </c>
       <c r="C1717" t="n">
-        <v>600000</v>
+        <v>650000</v>
       </c>
     </row>
     <row r="1718">
@@ -19333,7 +19333,7 @@
         <v>2768</v>
       </c>
       <c r="C1718" t="n">
-        <v>165084</v>
+        <v>178841</v>
       </c>
     </row>
     <row r="1719">
@@ -19344,7 +19344,7 @@
         <v>2491</v>
       </c>
       <c r="C1719" t="n">
-        <v>132468</v>
+        <v>143507</v>
       </c>
     </row>
     <row r="1720">
@@ -19355,7 +19355,7 @@
         <v>2799</v>
       </c>
       <c r="C1720" t="n">
-        <v>59628</v>
+        <v>64597</v>
       </c>
     </row>
     <row r="1721">
@@ -19388,7 +19388,7 @@
         <v>1317</v>
       </c>
       <c r="C1723" t="n">
-        <v>171818.2</v>
+        <v>186136.38</v>
       </c>
     </row>
     <row r="1724">
@@ -19399,7 +19399,7 @@
         <v>2822</v>
       </c>
       <c r="C1724" t="n">
-        <v>87272.8</v>
+        <v>94545.52</v>
       </c>
     </row>
     <row r="1725">
@@ -19410,7 +19410,7 @@
         <v>1117</v>
       </c>
       <c r="C1725" t="n">
-        <v>218244</v>
+        <v>236431</v>
       </c>
     </row>
     <row r="1726">
@@ -19421,7 +19421,7 @@
         <v>1299</v>
       </c>
       <c r="C1726" t="n">
-        <v>287748</v>
+        <v>311727</v>
       </c>
     </row>
     <row r="1727">
@@ -19432,7 +19432,7 @@
         <v>477</v>
       </c>
       <c r="C1727" t="n">
-        <v>118584</v>
+        <v>128466</v>
       </c>
     </row>
     <row r="1728">
@@ -19443,7 +19443,7 @@
         <v>530</v>
       </c>
       <c r="C1728" t="n">
-        <v>163632</v>
+        <v>177268</v>
       </c>
     </row>
     <row r="1729">
@@ -19454,7 +19454,7 @@
         <v>953</v>
       </c>
       <c r="C1729" t="n">
-        <v>376356</v>
+        <v>407719</v>
       </c>
     </row>
     <row r="1730">
@@ -19465,7 +19465,7 @@
         <v>610</v>
       </c>
       <c r="C1730" t="n">
-        <v>448248</v>
+        <v>485602</v>
       </c>
     </row>
     <row r="1731">
@@ -19476,7 +19476,7 @@
         <v>2792</v>
       </c>
       <c r="C1731" t="n">
-        <v>112572</v>
+        <v>121953</v>
       </c>
     </row>
     <row r="1732">
@@ -19553,7 +19553,7 @@
         <v>1075</v>
       </c>
       <c r="C1738" t="n">
-        <v>250356</v>
+        <v>271219</v>
       </c>
     </row>
     <row r="1739">
@@ -19564,7 +19564,7 @@
         <v>131</v>
       </c>
       <c r="C1739" t="n">
-        <v>226908</v>
+        <v>245817</v>
       </c>
     </row>
     <row r="1740">
@@ -19575,7 +19575,7 @@
         <v>2667</v>
       </c>
       <c r="C1740" t="n">
-        <v>24924</v>
+        <v>27001</v>
       </c>
     </row>
     <row r="1741">
@@ -19586,7 +19586,7 @@
         <v>2330</v>
       </c>
       <c r="C1741" t="n">
-        <v>48516</v>
+        <v>52559</v>
       </c>
     </row>
     <row r="1742">
@@ -19608,7 +19608,7 @@
         <v>2577</v>
       </c>
       <c r="C1743" t="n">
-        <v>48636</v>
+        <v>52689</v>
       </c>
     </row>
     <row r="1744">
@@ -19619,7 +19619,7 @@
         <v>2510</v>
       </c>
       <c r="C1744" t="n">
-        <v>345408</v>
+        <v>374192</v>
       </c>
     </row>
     <row r="1745">
@@ -19641,7 +19641,7 @@
         <v>2850</v>
       </c>
       <c r="C1746" t="n">
-        <v>32724</v>
+        <v>35451</v>
       </c>
     </row>
     <row r="1747">
@@ -19663,7 +19663,7 @@
         <v>2745</v>
       </c>
       <c r="C1748" t="n">
-        <v>60000</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="1749">
@@ -19674,7 +19674,7 @@
         <v>2817</v>
       </c>
       <c r="C1749" t="n">
-        <v>32724</v>
+        <v>35451</v>
       </c>
     </row>
     <row r="1750">
@@ -19685,7 +19685,7 @@
         <v>2784</v>
       </c>
       <c r="C1750" t="n">
-        <v>22692</v>
+        <v>24583</v>
       </c>
     </row>
     <row r="1751">
@@ -19696,7 +19696,7 @@
         <v>626</v>
       </c>
       <c r="C1751" t="n">
-        <v>942444</v>
+        <v>1020981</v>
       </c>
     </row>
     <row r="1752">
@@ -19707,7 +19707,7 @@
         <v>925</v>
       </c>
       <c r="C1752" t="n">
-        <v>43512</v>
+        <v>47138</v>
       </c>
     </row>
     <row r="1753">
@@ -19718,7 +19718,7 @@
         <v>2586</v>
       </c>
       <c r="C1753" t="n">
-        <v>22692</v>
+        <v>24583</v>
       </c>
     </row>
     <row r="1754">
@@ -19729,7 +19729,7 @@
         <v>966</v>
       </c>
       <c r="C1754" t="n">
-        <v>44436</v>
+        <v>48139</v>
       </c>
     </row>
     <row r="1755">
@@ -19740,7 +19740,7 @@
         <v>2557</v>
       </c>
       <c r="C1755" t="n">
-        <v>21324</v>
+        <v>23101</v>
       </c>
     </row>
     <row r="1756">
@@ -19751,7 +19751,7 @@
         <v>14</v>
       </c>
       <c r="C1756" t="n">
-        <v>245448</v>
+        <v>265902</v>
       </c>
     </row>
     <row r="1757">
@@ -19762,7 +19762,7 @@
         <v>2798</v>
       </c>
       <c r="C1757" t="n">
-        <v>32724</v>
+        <v>35451</v>
       </c>
     </row>
     <row r="1758">
@@ -19784,7 +19784,7 @@
         <v>522</v>
       </c>
       <c r="C1759" t="n">
-        <v>109091</v>
+        <v>118181.9</v>
       </c>
     </row>
     <row r="1760">
@@ -19806,7 +19806,7 @@
         <v>2819</v>
       </c>
       <c r="C1761" t="n">
-        <v>32724</v>
+        <v>35451</v>
       </c>
     </row>
     <row r="1762">
@@ -19817,7 +19817,7 @@
         <v>2266</v>
       </c>
       <c r="C1762" t="n">
-        <v>43632</v>
+        <v>47268</v>
       </c>
     </row>
     <row r="1763">
@@ -19850,7 +19850,7 @@
         <v>2795</v>
       </c>
       <c r="C1765" t="n">
-        <v>32724</v>
+        <v>35451</v>
       </c>
     </row>
     <row r="1766">
@@ -19861,7 +19861,7 @@
         <v>2722</v>
       </c>
       <c r="C1766" t="n">
-        <v>10908</v>
+        <v>11817</v>
       </c>
     </row>
     <row r="1767">
@@ -19872,7 +19872,7 @@
         <v>951</v>
       </c>
       <c r="C1767" t="n">
-        <v>62724</v>
+        <v>67951</v>
       </c>
     </row>
     <row r="1768">
@@ -19883,7 +19883,7 @@
         <v>1020</v>
       </c>
       <c r="C1768" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1769">
@@ -19894,7 +19894,7 @@
         <v>1853</v>
       </c>
       <c r="C1769" t="n">
-        <v>65448</v>
+        <v>70902</v>
       </c>
     </row>
     <row r="1770">
@@ -19905,7 +19905,7 @@
         <v>1327</v>
       </c>
       <c r="C1770" t="n">
-        <v>38172</v>
+        <v>41353</v>
       </c>
     </row>
     <row r="1771">
@@ -19916,7 +19916,7 @@
         <v>2842</v>
       </c>
       <c r="C1771" t="n">
-        <v>98172</v>
+        <v>106353</v>
       </c>
     </row>
     <row r="1772">
@@ -19927,7 +19927,7 @@
         <v>2831</v>
       </c>
       <c r="C1772" t="n">
-        <v>32724</v>
+        <v>35451</v>
       </c>
     </row>
     <row r="1773">
@@ -19938,7 +19938,7 @@
         <v>818</v>
       </c>
       <c r="C1773" t="n">
-        <v>218172</v>
+        <v>236353</v>
       </c>
     </row>
     <row r="1774">
@@ -19949,7 +19949,7 @@
         <v>1501</v>
       </c>
       <c r="C1774" t="n">
-        <v>54540</v>
+        <v>59085</v>
       </c>
     </row>
     <row r="1775">
@@ -19960,7 +19960,7 @@
         <v>1869</v>
       </c>
       <c r="C1775" t="n">
-        <v>133080</v>
+        <v>144170</v>
       </c>
     </row>
     <row r="1776">
@@ -19971,7 +19971,7 @@
         <v>1996</v>
       </c>
       <c r="C1776" t="n">
-        <v>136363.7</v>
+        <v>147727.33</v>
       </c>
     </row>
     <row r="1777">
@@ -19982,7 +19982,7 @@
         <v>2462</v>
       </c>
       <c r="C1777" t="n">
-        <v>30891.9</v>
+        <v>33466.21</v>
       </c>
     </row>
     <row r="1778">
@@ -19993,7 +19993,7 @@
         <v>2696</v>
       </c>
       <c r="C1778" t="n">
-        <v>116976</v>
+        <v>126724</v>
       </c>
     </row>
     <row r="1779">
@@ -20004,7 +20004,7 @@
         <v>2698</v>
       </c>
       <c r="C1779" t="n">
-        <v>59952</v>
+        <v>64948</v>
       </c>
     </row>
     <row r="1780">
@@ -20026,7 +20026,7 @@
         <v>2828</v>
       </c>
       <c r="C1781" t="n">
-        <v>32727.3</v>
+        <v>35454.57</v>
       </c>
     </row>
     <row r="1782">
@@ -20037,7 +20037,7 @@
         <v>2843</v>
       </c>
       <c r="C1782" t="n">
-        <v>38172</v>
+        <v>41353</v>
       </c>
     </row>
     <row r="1783">
@@ -20048,7 +20048,7 @@
         <v>619</v>
       </c>
       <c r="C1783" t="n">
-        <v>171000</v>
+        <v>185250</v>
       </c>
     </row>
     <row r="1784">
@@ -20059,7 +20059,7 @@
         <v>1478</v>
       </c>
       <c r="C1784" t="n">
-        <v>299256</v>
+        <v>324194</v>
       </c>
     </row>
     <row r="1785">
@@ -20070,7 +20070,7 @@
         <v>2026</v>
       </c>
       <c r="C1785" t="n">
-        <v>132216</v>
+        <v>143234</v>
       </c>
     </row>
     <row r="1786">
@@ -20081,7 +20081,7 @@
         <v>663</v>
       </c>
       <c r="C1786" t="n">
-        <v>141264</v>
+        <v>153036</v>
       </c>
     </row>
     <row r="1787">
@@ -20092,7 +20092,7 @@
         <v>285</v>
       </c>
       <c r="C1787" t="n">
-        <v>299256</v>
+        <v>324194</v>
       </c>
     </row>
     <row r="1788">
@@ -20103,7 +20103,7 @@
         <v>424</v>
       </c>
       <c r="C1788" t="n">
-        <v>128244</v>
+        <v>138931</v>
       </c>
     </row>
     <row r="1789">
@@ -20114,7 +20114,7 @@
         <v>451</v>
       </c>
       <c r="C1789" t="n">
-        <v>132540</v>
+        <v>143585</v>
       </c>
     </row>
     <row r="1790">
@@ -20125,7 +20125,7 @@
         <v>629</v>
       </c>
       <c r="C1790" t="n">
-        <v>247632</v>
+        <v>268268</v>
       </c>
     </row>
     <row r="1791">
@@ -20136,7 +20136,7 @@
         <v>2657</v>
       </c>
       <c r="C1791" t="n">
-        <v>43188</v>
+        <v>46787</v>
       </c>
     </row>
     <row r="1792">
@@ -20147,7 +20147,7 @@
         <v>1254</v>
       </c>
       <c r="C1792" t="n">
-        <v>105924</v>
+        <v>114751</v>
       </c>
     </row>
     <row r="1793">
@@ -20158,7 +20158,7 @@
         <v>2402</v>
       </c>
       <c r="C1793" t="n">
-        <v>266424</v>
+        <v>288626</v>
       </c>
     </row>
     <row r="1794">
@@ -20169,7 +20169,7 @@
         <v>2413</v>
       </c>
       <c r="C1794" t="n">
-        <v>75180</v>
+        <v>81445</v>
       </c>
     </row>
     <row r="1795">
@@ -20180,7 +20180,7 @@
         <v>1450</v>
       </c>
       <c r="C1795" t="n">
-        <v>194724</v>
+        <v>210951</v>
       </c>
     </row>
     <row r="1796">
@@ -20202,7 +20202,7 @@
         <v>2671</v>
       </c>
       <c r="C1797" t="n">
-        <v>43632</v>
+        <v>47268</v>
       </c>
     </row>
     <row r="1798">
@@ -20213,7 +20213,7 @@
         <v>2568</v>
       </c>
       <c r="C1798" t="n">
-        <v>87516</v>
+        <v>94809</v>
       </c>
     </row>
     <row r="1799">
@@ -20224,7 +20224,7 @@
         <v>2146</v>
       </c>
       <c r="C1799" t="n">
-        <v>105972</v>
+        <v>114803</v>
       </c>
     </row>
     <row r="1800">
@@ -20235,7 +20235,7 @@
         <v>2753</v>
       </c>
       <c r="C1800" t="n">
-        <v>40908</v>
+        <v>44317</v>
       </c>
     </row>
     <row r="1801">
@@ -20246,7 +20246,7 @@
         <v>744</v>
       </c>
       <c r="C1801" t="n">
-        <v>22692</v>
+        <v>24583</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:02:23
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -15560,7 +15560,7 @@
         <v>2853</v>
       </c>
       <c r="C1375" t="n">
-        <v>48139</v>
+        <v>51842</v>
       </c>
     </row>
     <row r="1376">
@@ -15571,7 +15571,7 @@
         <v>2245</v>
       </c>
       <c r="C1376" t="n">
-        <v>130832</v>
+        <v>140896</v>
       </c>
     </row>
     <row r="1377">
@@ -15582,7 +15582,7 @@
         <v>2251</v>
       </c>
       <c r="C1377" t="n">
-        <v>118170</v>
+        <v>127260</v>
       </c>
     </row>
     <row r="1378">
@@ -15593,7 +15593,7 @@
         <v>664</v>
       </c>
       <c r="C1378" t="n">
-        <v>154817</v>
+        <v>166726</v>
       </c>
     </row>
     <row r="1379">
@@ -15604,7 +15604,7 @@
         <v>2472</v>
       </c>
       <c r="C1379" t="n">
-        <v>31278</v>
+        <v>33684</v>
       </c>
     </row>
     <row r="1380">
@@ -15615,7 +15615,7 @@
         <v>1456</v>
       </c>
       <c r="C1380" t="n">
-        <v>471536</v>
+        <v>507808</v>
       </c>
     </row>
     <row r="1381">
@@ -15626,7 +15626,7 @@
         <v>1585</v>
       </c>
       <c r="C1381" t="n">
-        <v>106951</v>
+        <v>115178</v>
       </c>
     </row>
     <row r="1382">
@@ -15670,7 +15670,7 @@
         <v>1907</v>
       </c>
       <c r="C1385" t="n">
-        <v>325312</v>
+        <v>350336</v>
       </c>
     </row>
     <row r="1386">
@@ -15703,7 +15703,7 @@
         <v>2659</v>
       </c>
       <c r="C1388" t="n">
-        <v>72683</v>
+        <v>78274</v>
       </c>
     </row>
     <row r="1389">
@@ -15714,7 +15714,7 @@
         <v>2583</v>
       </c>
       <c r="C1389" t="n">
-        <v>24583</v>
+        <v>26474</v>
       </c>
     </row>
     <row r="1390">
@@ -15725,7 +15725,7 @@
         <v>2692</v>
       </c>
       <c r="C1390" t="n">
-        <v>41363.71</v>
+        <v>44545.52</v>
       </c>
     </row>
     <row r="1391">
@@ -15736,7 +15736,7 @@
         <v>2691</v>
       </c>
       <c r="C1391" t="n">
-        <v>72199.71000000001</v>
+        <v>77753.52</v>
       </c>
     </row>
     <row r="1392">
@@ -15747,7 +15747,7 @@
         <v>931</v>
       </c>
       <c r="C1392" t="n">
-        <v>56563</v>
+        <v>60914</v>
       </c>
     </row>
     <row r="1393">
@@ -15758,7 +15758,7 @@
         <v>2785</v>
       </c>
       <c r="C1393" t="n">
-        <v>24583</v>
+        <v>26474</v>
       </c>
     </row>
     <row r="1394">
@@ -15769,7 +15769,7 @@
         <v>2411</v>
       </c>
       <c r="C1394" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1395">
@@ -15780,7 +15780,7 @@
         <v>2716</v>
       </c>
       <c r="C1395" t="n">
-        <v>51844</v>
+        <v>55832</v>
       </c>
     </row>
     <row r="1396">
@@ -15791,7 +15791,7 @@
         <v>2809</v>
       </c>
       <c r="C1396" t="n">
-        <v>40586</v>
+        <v>43708</v>
       </c>
     </row>
     <row r="1397">
@@ -15802,7 +15802,7 @@
         <v>104</v>
       </c>
       <c r="C1397" t="n">
-        <v>177272.76</v>
+        <v>190909.12</v>
       </c>
     </row>
     <row r="1398">
@@ -15835,7 +15835,7 @@
         <v>781</v>
       </c>
       <c r="C1400" t="n">
-        <v>76817</v>
+        <v>82726</v>
       </c>
     </row>
     <row r="1401">
@@ -15857,7 +15857,7 @@
         <v>2494</v>
       </c>
       <c r="C1402" t="n">
-        <v>88634</v>
+        <v>95452</v>
       </c>
     </row>
     <row r="1403">
@@ -15868,7 +15868,7 @@
         <v>2652</v>
       </c>
       <c r="C1403" t="n">
-        <v>82719</v>
+        <v>89082</v>
       </c>
     </row>
     <row r="1404">
@@ -15879,7 +15879,7 @@
         <v>1384</v>
       </c>
       <c r="C1404" t="n">
-        <v>206818.19</v>
+        <v>222727.28</v>
       </c>
     </row>
     <row r="1405">
@@ -15890,7 +15890,7 @@
         <v>360</v>
       </c>
       <c r="C1405" t="n">
-        <v>295451</v>
+        <v>318178</v>
       </c>
     </row>
     <row r="1406">
@@ -15901,7 +15901,7 @@
         <v>2767</v>
       </c>
       <c r="C1406" t="n">
-        <v>112268</v>
+        <v>120904</v>
       </c>
     </row>
     <row r="1407">
@@ -15912,7 +15912,7 @@
         <v>2178</v>
       </c>
       <c r="C1407" t="n">
-        <v>161902</v>
+        <v>174356</v>
       </c>
     </row>
     <row r="1408">
@@ -15923,7 +15923,7 @@
         <v>2107</v>
       </c>
       <c r="C1408" t="n">
-        <v>177255</v>
+        <v>190890</v>
       </c>
     </row>
     <row r="1409">
@@ -15934,7 +15934,7 @@
         <v>2711</v>
       </c>
       <c r="C1409" t="n">
-        <v>51155</v>
+        <v>55090</v>
       </c>
     </row>
     <row r="1410">
@@ -15945,7 +15945,7 @@
         <v>2845</v>
       </c>
       <c r="C1410" t="n">
-        <v>29536</v>
+        <v>31808</v>
       </c>
     </row>
     <row r="1411">
@@ -15989,7 +15989,7 @@
         <v>1102</v>
       </c>
       <c r="C1414" t="n">
-        <v>138931</v>
+        <v>149618</v>
       </c>
     </row>
     <row r="1415">
@@ -16000,7 +16000,7 @@
         <v>353</v>
       </c>
       <c r="C1415" t="n">
-        <v>172861</v>
+        <v>186158</v>
       </c>
     </row>
     <row r="1416">
@@ -16011,7 +16011,7 @@
         <v>2250</v>
       </c>
       <c r="C1416" t="n">
-        <v>200902</v>
+        <v>216356</v>
       </c>
     </row>
     <row r="1417">
@@ -16022,7 +16022,7 @@
         <v>1800</v>
       </c>
       <c r="C1417" t="n">
-        <v>16757</v>
+        <v>18046</v>
       </c>
     </row>
     <row r="1418">
@@ -16033,7 +16033,7 @@
         <v>2362</v>
       </c>
       <c r="C1418" t="n">
-        <v>44317</v>
+        <v>47726</v>
       </c>
     </row>
     <row r="1419">
@@ -16044,7 +16044,7 @@
         <v>2449</v>
       </c>
       <c r="C1419" t="n">
-        <v>56134</v>
+        <v>60452</v>
       </c>
     </row>
     <row r="1420">
@@ -16055,7 +16055,7 @@
         <v>2844</v>
       </c>
       <c r="C1420" t="n">
-        <v>29536</v>
+        <v>31808</v>
       </c>
     </row>
     <row r="1421">
@@ -16066,7 +16066,7 @@
         <v>2507</v>
       </c>
       <c r="C1421" t="n">
-        <v>52780</v>
+        <v>56840</v>
       </c>
     </row>
     <row r="1422">
@@ -16077,7 +16077,7 @@
         <v>1906</v>
       </c>
       <c r="C1422" t="n">
-        <v>64155</v>
+        <v>69090</v>
       </c>
     </row>
     <row r="1423">
@@ -16099,7 +16099,7 @@
         <v>525</v>
       </c>
       <c r="C1424" t="n">
-        <v>138863.71</v>
+        <v>149545.52</v>
       </c>
     </row>
     <row r="1425">
@@ -16110,7 +16110,7 @@
         <v>1261</v>
       </c>
       <c r="C1425" t="n">
-        <v>41954.57</v>
+        <v>45181.84</v>
       </c>
     </row>
     <row r="1426">
@@ -16121,7 +16121,7 @@
         <v>2755</v>
       </c>
       <c r="C1426" t="n">
-        <v>29545.52</v>
+        <v>31818.24</v>
       </c>
     </row>
     <row r="1427">
@@ -16143,7 +16143,7 @@
         <v>1064</v>
       </c>
       <c r="C1428" t="n">
-        <v>354536</v>
+        <v>381808</v>
       </c>
     </row>
     <row r="1429">
@@ -16154,7 +16154,7 @@
         <v>1810</v>
       </c>
       <c r="C1429" t="n">
-        <v>23998</v>
+        <v>25844</v>
       </c>
     </row>
     <row r="1430">
@@ -16165,7 +16165,7 @@
         <v>1937</v>
       </c>
       <c r="C1430" t="n">
-        <v>153036</v>
+        <v>164808</v>
       </c>
     </row>
     <row r="1431">
@@ -16176,7 +16176,7 @@
         <v>483</v>
       </c>
       <c r="C1431" t="n">
-        <v>267085</v>
+        <v>287630</v>
       </c>
     </row>
     <row r="1432">
@@ -16187,7 +16187,7 @@
         <v>2580</v>
       </c>
       <c r="C1432" t="n">
-        <v>19903</v>
+        <v>21434</v>
       </c>
     </row>
     <row r="1433">
@@ -16198,7 +16198,7 @@
         <v>2706</v>
       </c>
       <c r="C1433" t="n">
-        <v>15548</v>
+        <v>16744</v>
       </c>
     </row>
     <row r="1434">
@@ -16209,7 +16209,7 @@
         <v>2633</v>
       </c>
       <c r="C1434" t="n">
-        <v>11388</v>
+        <v>12264</v>
       </c>
     </row>
     <row r="1435">
@@ -16242,7 +16242,7 @@
         <v>2392</v>
       </c>
       <c r="C1437" t="n">
-        <v>122564</v>
+        <v>131992</v>
       </c>
     </row>
     <row r="1438">
@@ -16264,7 +16264,7 @@
         <v>2613</v>
       </c>
       <c r="C1439" t="n">
-        <v>86294</v>
+        <v>92932</v>
       </c>
     </row>
     <row r="1440">
@@ -16275,7 +16275,7 @@
         <v>2183</v>
       </c>
       <c r="C1440" t="n">
-        <v>310713</v>
+        <v>334614</v>
       </c>
     </row>
     <row r="1441">
@@ -16286,7 +16286,7 @@
         <v>2541</v>
       </c>
       <c r="C1441" t="n">
-        <v>139685</v>
+        <v>150430</v>
       </c>
     </row>
     <row r="1442">
@@ -16297,7 +16297,7 @@
         <v>2333</v>
       </c>
       <c r="C1442" t="n">
-        <v>94302</v>
+        <v>101556</v>
       </c>
     </row>
     <row r="1443">
@@ -16308,7 +16308,7 @@
         <v>2813</v>
       </c>
       <c r="C1443" t="n">
-        <v>37700</v>
+        <v>40600</v>
       </c>
     </row>
     <row r="1444">
@@ -16319,7 +16319,7 @@
         <v>2811</v>
       </c>
       <c r="C1444" t="n">
-        <v>24583</v>
+        <v>26474</v>
       </c>
     </row>
     <row r="1445">
@@ -16330,7 +16330,7 @@
         <v>1881</v>
       </c>
       <c r="C1445" t="n">
-        <v>40586</v>
+        <v>43708</v>
       </c>
     </row>
     <row r="1446">
@@ -16341,7 +16341,7 @@
         <v>2825</v>
       </c>
       <c r="C1446" t="n">
-        <v>32994</v>
+        <v>35532</v>
       </c>
     </row>
     <row r="1447">
@@ -16352,7 +16352,7 @@
         <v>970</v>
       </c>
       <c r="C1447" t="n">
-        <v>40586</v>
+        <v>43708</v>
       </c>
     </row>
     <row r="1448">
@@ -16363,7 +16363,7 @@
         <v>2552</v>
       </c>
       <c r="C1448" t="n">
-        <v>23101</v>
+        <v>24878</v>
       </c>
     </row>
     <row r="1449">
@@ -16374,7 +16374,7 @@
         <v>2562</v>
       </c>
       <c r="C1449" t="n">
-        <v>23101</v>
+        <v>24878</v>
       </c>
     </row>
     <row r="1450">
@@ -16407,7 +16407,7 @@
         <v>2747</v>
       </c>
       <c r="C1452" t="n">
-        <v>41353</v>
+        <v>44534</v>
       </c>
     </row>
     <row r="1453">
@@ -16418,7 +16418,7 @@
         <v>415</v>
       </c>
       <c r="C1453" t="n">
-        <v>147727.33</v>
+        <v>159090.96</v>
       </c>
     </row>
     <row r="1454">
@@ -16462,7 +16462,7 @@
         <v>2544</v>
       </c>
       <c r="C1457" t="n">
-        <v>41353</v>
+        <v>44534</v>
       </c>
     </row>
     <row r="1458">
@@ -16473,7 +16473,7 @@
         <v>816</v>
       </c>
       <c r="C1458" t="n">
-        <v>177272.76</v>
+        <v>190909.12</v>
       </c>
     </row>
     <row r="1459">
@@ -16484,7 +16484,7 @@
         <v>890</v>
       </c>
       <c r="C1459" t="n">
-        <v>531818.1899999999</v>
+        <v>572727.28</v>
       </c>
     </row>
     <row r="1460">
@@ -16495,7 +16495,7 @@
         <v>1298</v>
       </c>
       <c r="C1460" t="n">
-        <v>747500</v>
+        <v>805000</v>
       </c>
     </row>
     <row r="1461">
@@ -16506,7 +16506,7 @@
         <v>1372</v>
       </c>
       <c r="C1461" t="n">
-        <v>177272.76</v>
+        <v>190909.12</v>
       </c>
     </row>
     <row r="1462">
@@ -16517,7 +16517,7 @@
         <v>358</v>
       </c>
       <c r="C1462" t="n">
-        <v>186134</v>
+        <v>200452</v>
       </c>
     </row>
     <row r="1463">
@@ -16528,7 +16528,7 @@
         <v>1653</v>
       </c>
       <c r="C1463" t="n">
-        <v>186134</v>
+        <v>200452</v>
       </c>
     </row>
     <row r="1464">
@@ -16539,7 +16539,7 @@
         <v>675</v>
       </c>
       <c r="C1464" t="n">
-        <v>118170</v>
+        <v>127260</v>
       </c>
     </row>
     <row r="1465">
@@ -16550,7 +16550,7 @@
         <v>2804</v>
       </c>
       <c r="C1465" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1466">
@@ -16561,7 +16561,7 @@
         <v>2714</v>
       </c>
       <c r="C1466" t="n">
-        <v>212719</v>
+        <v>229082</v>
       </c>
     </row>
     <row r="1467">
@@ -16572,7 +16572,7 @@
         <v>2765</v>
       </c>
       <c r="C1467" t="n">
-        <v>53170</v>
+        <v>57260</v>
       </c>
     </row>
     <row r="1468">
@@ -16583,7 +16583,7 @@
         <v>2421</v>
       </c>
       <c r="C1468" t="n">
-        <v>36036</v>
+        <v>38808</v>
       </c>
     </row>
     <row r="1469">
@@ -16594,7 +16594,7 @@
         <v>2359</v>
       </c>
       <c r="C1469" t="n">
-        <v>61646</v>
+        <v>66388</v>
       </c>
     </row>
     <row r="1470">
@@ -16605,7 +16605,7 @@
         <v>2678</v>
       </c>
       <c r="C1470" t="n">
-        <v>58474</v>
+        <v>62972</v>
       </c>
     </row>
     <row r="1471">
@@ -16616,7 +16616,7 @@
         <v>2697</v>
       </c>
       <c r="C1471" t="n">
-        <v>88738</v>
+        <v>95564</v>
       </c>
     </row>
     <row r="1472">
@@ -16649,7 +16649,7 @@
         <v>2142</v>
       </c>
       <c r="C1474" t="n">
-        <v>31980</v>
+        <v>34440</v>
       </c>
     </row>
     <row r="1475">
@@ -16660,7 +16660,7 @@
         <v>2498</v>
       </c>
       <c r="C1475" t="n">
-        <v>33267</v>
+        <v>35826</v>
       </c>
     </row>
     <row r="1476">
@@ -16682,7 +16682,7 @@
         <v>2801</v>
       </c>
       <c r="C1477" t="n">
-        <v>59090.95</v>
+        <v>63636.4</v>
       </c>
     </row>
     <row r="1478">
@@ -16693,7 +16693,7 @@
         <v>2810</v>
       </c>
       <c r="C1478" t="n">
-        <v>94545.52</v>
+        <v>101818.24</v>
       </c>
     </row>
     <row r="1479">
@@ -16737,7 +16737,7 @@
         <v>132</v>
       </c>
       <c r="C1482" t="n">
-        <v>206818.19</v>
+        <v>222727.28</v>
       </c>
     </row>
     <row r="1483">
@@ -16759,7 +16759,7 @@
         <v>580</v>
       </c>
       <c r="C1484" t="n">
-        <v>103409.14</v>
+        <v>111363.68</v>
       </c>
     </row>
     <row r="1485">
@@ -16770,7 +16770,7 @@
         <v>634</v>
       </c>
       <c r="C1485" t="n">
-        <v>295454.57</v>
+        <v>318181.84</v>
       </c>
     </row>
     <row r="1486">
@@ -16792,7 +16792,7 @@
         <v>1277</v>
       </c>
       <c r="C1487" t="n">
-        <v>130000</v>
+        <v>140000</v>
       </c>
     </row>
     <row r="1488">
@@ -16803,7 +16803,7 @@
         <v>767</v>
       </c>
       <c r="C1488" t="n">
-        <v>118170</v>
+        <v>127260</v>
       </c>
     </row>
     <row r="1489">
@@ -16814,7 +16814,7 @@
         <v>2727</v>
       </c>
       <c r="C1489" t="n">
-        <v>23920</v>
+        <v>25760</v>
       </c>
     </row>
     <row r="1490">
@@ -16825,7 +16825,7 @@
         <v>2846</v>
       </c>
       <c r="C1490" t="n">
-        <v>153634</v>
+        <v>165452</v>
       </c>
     </row>
     <row r="1491">
@@ -16836,7 +16836,7 @@
         <v>609</v>
       </c>
       <c r="C1491" t="n">
-        <v>132951</v>
+        <v>143178</v>
       </c>
     </row>
     <row r="1492">
@@ -16847,7 +16847,7 @@
         <v>2726</v>
       </c>
       <c r="C1492" t="n">
-        <v>91585</v>
+        <v>98630</v>
       </c>
     </row>
     <row r="1493">
@@ -16858,7 +16858,7 @@
         <v>2729</v>
       </c>
       <c r="C1493" t="n">
-        <v>53170</v>
+        <v>57260</v>
       </c>
     </row>
     <row r="1494">
@@ -16869,7 +16869,7 @@
         <v>1340</v>
       </c>
       <c r="C1494" t="n">
-        <v>88634</v>
+        <v>95452</v>
       </c>
     </row>
     <row r="1495">
@@ -16880,7 +16880,7 @@
         <v>2830</v>
       </c>
       <c r="C1495" t="n">
-        <v>53170</v>
+        <v>57260</v>
       </c>
     </row>
     <row r="1496">
@@ -16891,7 +16891,7 @@
         <v>2674</v>
       </c>
       <c r="C1496" t="n">
-        <v>153634</v>
+        <v>165452</v>
       </c>
     </row>
     <row r="1497">
@@ -16902,7 +16902,7 @@
         <v>2308</v>
       </c>
       <c r="C1497" t="n">
-        <v>118170</v>
+        <v>127260</v>
       </c>
     </row>
     <row r="1498">
@@ -16913,7 +16913,7 @@
         <v>2190</v>
       </c>
       <c r="C1498" t="n">
-        <v>124085</v>
+        <v>133630</v>
       </c>
     </row>
     <row r="1499">
@@ -16924,7 +16924,7 @@
         <v>2015</v>
       </c>
       <c r="C1499" t="n">
-        <v>218634</v>
+        <v>235452</v>
       </c>
     </row>
     <row r="1500">
@@ -16935,7 +16935,7 @@
         <v>1308</v>
       </c>
       <c r="C1500" t="n">
-        <v>92768</v>
+        <v>99904</v>
       </c>
     </row>
     <row r="1501">
@@ -16946,7 +16946,7 @@
         <v>2118</v>
       </c>
       <c r="C1501" t="n">
-        <v>124189</v>
+        <v>133742</v>
       </c>
     </row>
     <row r="1502">
@@ -16957,7 +16957,7 @@
         <v>2607</v>
       </c>
       <c r="C1502" t="n">
-        <v>29354</v>
+        <v>31612</v>
       </c>
     </row>
     <row r="1503">
@@ -16968,7 +16968,7 @@
         <v>2832</v>
       </c>
       <c r="C1503" t="n">
-        <v>88636.38</v>
+        <v>95454.56</v>
       </c>
     </row>
     <row r="1504">
@@ -16979,7 +16979,7 @@
         <v>2383</v>
       </c>
       <c r="C1504" t="n">
-        <v>78546</v>
+        <v>84588</v>
       </c>
     </row>
     <row r="1505">
@@ -17012,7 +17012,7 @@
         <v>2821</v>
       </c>
       <c r="C1507" t="n">
-        <v>78793</v>
+        <v>84854</v>
       </c>
     </row>
     <row r="1508">
@@ -17034,7 +17034,7 @@
         <v>569</v>
       </c>
       <c r="C1509" t="n">
-        <v>1715662</v>
+        <v>1847636</v>
       </c>
     </row>
     <row r="1510">
@@ -17045,7 +17045,7 @@
         <v>2660</v>
       </c>
       <c r="C1510" t="n">
-        <v>206818.19</v>
+        <v>222727.28</v>
       </c>
     </row>
     <row r="1511">
@@ -17056,7 +17056,7 @@
         <v>1632</v>
       </c>
       <c r="C1511" t="n">
-        <v>153636.38</v>
+        <v>165454.56</v>
       </c>
     </row>
     <row r="1512">
@@ -17067,7 +17067,7 @@
         <v>1756</v>
       </c>
       <c r="C1512" t="n">
-        <v>248170</v>
+        <v>267260</v>
       </c>
     </row>
     <row r="1513">
@@ -17078,7 +17078,7 @@
         <v>58</v>
       </c>
       <c r="C1513" t="n">
-        <v>148200</v>
+        <v>159600</v>
       </c>
     </row>
     <row r="1514">
@@ -17089,7 +17089,7 @@
         <v>40</v>
       </c>
       <c r="C1514" t="n">
-        <v>131820</v>
+        <v>141960</v>
       </c>
     </row>
     <row r="1515">
@@ -17100,7 +17100,7 @@
         <v>559</v>
       </c>
       <c r="C1515" t="n">
-        <v>138268</v>
+        <v>148904</v>
       </c>
     </row>
     <row r="1516">
@@ -17111,7 +17111,7 @@
         <v>2773</v>
       </c>
       <c r="C1516" t="n">
-        <v>47671</v>
+        <v>51338</v>
       </c>
     </row>
     <row r="1517">
@@ -17122,7 +17122,7 @@
         <v>2631</v>
       </c>
       <c r="C1517" t="n">
-        <v>22893</v>
+        <v>24654</v>
       </c>
     </row>
     <row r="1518">
@@ -17133,7 +17133,7 @@
         <v>2085</v>
       </c>
       <c r="C1518" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1519">
@@ -17155,7 +17155,7 @@
         <v>1642</v>
       </c>
       <c r="C1520" t="n">
-        <v>156585</v>
+        <v>168630</v>
       </c>
     </row>
     <row r="1521">
@@ -17166,7 +17166,7 @@
         <v>2621</v>
       </c>
       <c r="C1521" t="n">
-        <v>41353</v>
+        <v>44534</v>
       </c>
     </row>
     <row r="1522">
@@ -17177,7 +17177,7 @@
         <v>2705</v>
       </c>
       <c r="C1522" t="n">
-        <v>118638</v>
+        <v>127764</v>
       </c>
     </row>
     <row r="1523">
@@ -17188,7 +17188,7 @@
         <v>2735</v>
       </c>
       <c r="C1523" t="n">
-        <v>70902</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1524">
@@ -17199,7 +17199,7 @@
         <v>945</v>
       </c>
       <c r="C1524" t="n">
-        <v>207220</v>
+        <v>223160</v>
       </c>
     </row>
     <row r="1525">
@@ -17210,7 +17210,7 @@
         <v>2582</v>
       </c>
       <c r="C1525" t="n">
-        <v>51844</v>
+        <v>55832</v>
       </c>
     </row>
     <row r="1526">
@@ -17221,7 +17221,7 @@
         <v>2584</v>
       </c>
       <c r="C1526" t="n">
-        <v>37700</v>
+        <v>40600</v>
       </c>
     </row>
     <row r="1527">
@@ -17232,7 +17232,7 @@
         <v>2689</v>
       </c>
       <c r="C1527" t="n">
-        <v>37700</v>
+        <v>40600</v>
       </c>
     </row>
     <row r="1528">
@@ -17243,7 +17243,7 @@
         <v>2574</v>
       </c>
       <c r="C1528" t="n">
-        <v>82862</v>
+        <v>89236</v>
       </c>
     </row>
     <row r="1529">
@@ -17254,7 +17254,7 @@
         <v>1834</v>
       </c>
       <c r="C1529" t="n">
-        <v>69550</v>
+        <v>74900</v>
       </c>
     </row>
     <row r="1530">
@@ -17265,7 +17265,7 @@
         <v>2629</v>
       </c>
       <c r="C1530" t="n">
-        <v>40586</v>
+        <v>43708</v>
       </c>
     </row>
     <row r="1531">
@@ -17276,7 +17276,7 @@
         <v>933</v>
       </c>
       <c r="C1531" t="n">
-        <v>48139</v>
+        <v>51842</v>
       </c>
     </row>
     <row r="1532">
@@ -17287,7 +17287,7 @@
         <v>2555</v>
       </c>
       <c r="C1532" t="n">
-        <v>23101</v>
+        <v>24878</v>
       </c>
     </row>
     <row r="1533">
@@ -17298,7 +17298,7 @@
         <v>2558</v>
       </c>
       <c r="C1533" t="n">
-        <v>23101</v>
+        <v>24878</v>
       </c>
     </row>
     <row r="1534">
@@ -17309,7 +17309,7 @@
         <v>2721</v>
       </c>
       <c r="C1534" t="n">
-        <v>48139</v>
+        <v>51842</v>
       </c>
     </row>
     <row r="1535">
@@ -17320,7 +17320,7 @@
         <v>2556</v>
       </c>
       <c r="C1535" t="n">
-        <v>23101</v>
+        <v>24878</v>
       </c>
     </row>
     <row r="1536">
@@ -17331,7 +17331,7 @@
         <v>2826</v>
       </c>
       <c r="C1536" t="n">
-        <v>41353</v>
+        <v>44534</v>
       </c>
     </row>
     <row r="1537">
@@ -17353,7 +17353,7 @@
         <v>2346</v>
       </c>
       <c r="C1538" t="n">
-        <v>41353</v>
+        <v>44534</v>
       </c>
     </row>
     <row r="1539">
@@ -17364,7 +17364,7 @@
         <v>595</v>
       </c>
       <c r="C1539" t="n">
-        <v>147727.33</v>
+        <v>159090.96</v>
       </c>
     </row>
     <row r="1540">
@@ -17375,7 +17375,7 @@
         <v>1278</v>
       </c>
       <c r="C1540" t="n">
-        <v>103409.14</v>
+        <v>111363.68</v>
       </c>
     </row>
     <row r="1541">
@@ -17386,7 +17386,7 @@
         <v>2686</v>
       </c>
       <c r="C1541" t="n">
-        <v>82719</v>
+        <v>89082</v>
       </c>
     </row>
     <row r="1542">
@@ -17397,7 +17397,7 @@
         <v>1344</v>
       </c>
       <c r="C1542" t="n">
-        <v>88634</v>
+        <v>95452</v>
       </c>
     </row>
     <row r="1543">
@@ -17408,7 +17408,7 @@
         <v>2566</v>
       </c>
       <c r="C1543" t="n">
-        <v>47268</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1544">
@@ -17419,7 +17419,7 @@
         <v>2684</v>
       </c>
       <c r="C1544" t="n">
-        <v>56134</v>
+        <v>60452</v>
       </c>
     </row>
     <row r="1545">
@@ -17430,7 +17430,7 @@
         <v>2375</v>
       </c>
       <c r="C1545" t="n">
-        <v>195000</v>
+        <v>210000</v>
       </c>
     </row>
     <row r="1546">
@@ -17441,7 +17441,7 @@
         <v>2829</v>
       </c>
       <c r="C1546" t="n">
-        <v>35451</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1547">
@@ -17452,7 +17452,7 @@
         <v>768</v>
       </c>
       <c r="C1547" t="n">
-        <v>82719</v>
+        <v>89082</v>
       </c>
     </row>
     <row r="1548">
@@ -17463,7 +17463,7 @@
         <v>772</v>
       </c>
       <c r="C1548" t="n">
-        <v>192036</v>
+        <v>206808</v>
       </c>
     </row>
     <row r="1549">
@@ -17474,7 +17474,7 @@
         <v>2496</v>
       </c>
       <c r="C1549" t="n">
-        <v>118170</v>
+        <v>127260</v>
       </c>
     </row>
     <row r="1550">
@@ -17485,7 +17485,7 @@
         <v>802</v>
       </c>
       <c r="C1550" t="n">
-        <v>44317</v>
+        <v>47726</v>
       </c>
     </row>
     <row r="1551">
@@ -17496,7 +17496,7 @@
         <v>2131</v>
       </c>
       <c r="C1551" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1552">
@@ -17507,7 +17507,7 @@
         <v>1381</v>
       </c>
       <c r="C1552" t="n">
-        <v>177272.76</v>
+        <v>190909.12</v>
       </c>
     </row>
     <row r="1553">
@@ -17518,7 +17518,7 @@
         <v>2847</v>
       </c>
       <c r="C1553" t="n">
-        <v>79768</v>
+        <v>85904</v>
       </c>
     </row>
     <row r="1554">
@@ -17529,7 +17529,7 @@
         <v>1293</v>
       </c>
       <c r="C1554" t="n">
-        <v>227500</v>
+        <v>245000</v>
       </c>
     </row>
     <row r="1555">
@@ -17540,7 +17540,7 @@
         <v>2363</v>
       </c>
       <c r="C1555" t="n">
-        <v>100451</v>
+        <v>108178</v>
       </c>
     </row>
     <row r="1556">
@@ -17551,7 +17551,7 @@
         <v>631</v>
       </c>
       <c r="C1556" t="n">
-        <v>206817</v>
+        <v>222726</v>
       </c>
     </row>
     <row r="1557">
@@ -17562,7 +17562,7 @@
         <v>2791</v>
       </c>
       <c r="C1557" t="n">
-        <v>60671</v>
+        <v>65338</v>
       </c>
     </row>
     <row r="1558">
@@ -17584,7 +17584,7 @@
         <v>2841</v>
       </c>
       <c r="C1559" t="n">
-        <v>29536</v>
+        <v>31808</v>
       </c>
     </row>
     <row r="1560">
@@ -17595,7 +17595,7 @@
         <v>2571</v>
       </c>
       <c r="C1560" t="n">
-        <v>157521</v>
+        <v>169638</v>
       </c>
     </row>
     <row r="1561">
@@ -17661,7 +17661,7 @@
         <v>2273</v>
       </c>
       <c r="C1566" t="n">
-        <v>127049</v>
+        <v>136822</v>
       </c>
     </row>
     <row r="1567">
@@ -17672,7 +17672,7 @@
         <v>2381</v>
       </c>
       <c r="C1567" t="n">
-        <v>47515</v>
+        <v>51170</v>
       </c>
     </row>
     <row r="1568">
@@ -17683,7 +17683,7 @@
         <v>630</v>
       </c>
       <c r="C1568" t="n">
-        <v>48767.71</v>
+        <v>52519.07</v>
       </c>
     </row>
     <row r="1569">
@@ -17705,7 +17705,7 @@
         <v>1983</v>
       </c>
       <c r="C1570" t="n">
-        <v>323960</v>
+        <v>348880</v>
       </c>
     </row>
     <row r="1571">
@@ -17716,7 +17716,7 @@
         <v>1993</v>
       </c>
       <c r="C1571" t="n">
-        <v>219986</v>
+        <v>236908</v>
       </c>
     </row>
     <row r="1572">
@@ -17727,7 +17727,7 @@
         <v>89</v>
       </c>
       <c r="C1572" t="n">
-        <v>206817</v>
+        <v>222726</v>
       </c>
     </row>
     <row r="1573">
@@ -17738,7 +17738,7 @@
         <v>1063</v>
       </c>
       <c r="C1573" t="n">
-        <v>227500</v>
+        <v>245000</v>
       </c>
     </row>
     <row r="1574">
@@ -17749,7 +17749,7 @@
         <v>1116</v>
       </c>
       <c r="C1574" t="n">
-        <v>147719</v>
+        <v>159082</v>
       </c>
     </row>
     <row r="1575">
@@ -17760,7 +17760,7 @@
         <v>941</v>
       </c>
       <c r="C1575" t="n">
-        <v>177801</v>
+        <v>191478</v>
       </c>
     </row>
     <row r="1576">
@@ -17771,7 +17771,7 @@
         <v>2141</v>
       </c>
       <c r="C1576" t="n">
-        <v>18954</v>
+        <v>20412</v>
       </c>
     </row>
     <row r="1577">
@@ -17782,7 +17782,7 @@
         <v>2463</v>
       </c>
       <c r="C1577" t="n">
-        <v>194896</v>
+        <v>209888</v>
       </c>
     </row>
     <row r="1578">
@@ -17793,7 +17793,7 @@
         <v>2707</v>
       </c>
       <c r="C1578" t="n">
-        <v>25519</v>
+        <v>27482</v>
       </c>
     </row>
     <row r="1579">
@@ -17804,7 +17804,7 @@
         <v>2325</v>
       </c>
       <c r="C1579" t="n">
-        <v>68172</v>
+        <v>73416</v>
       </c>
     </row>
     <row r="1580">
@@ -17848,7 +17848,7 @@
         <v>1890</v>
       </c>
       <c r="C1583" t="n">
-        <v>144911</v>
+        <v>156058</v>
       </c>
     </row>
     <row r="1584">
@@ -17859,7 +17859,7 @@
         <v>2639</v>
       </c>
       <c r="C1584" t="n">
-        <v>23673</v>
+        <v>25494</v>
       </c>
     </row>
     <row r="1585">
@@ -17870,7 +17870,7 @@
         <v>2682</v>
       </c>
       <c r="C1585" t="n">
-        <v>82719</v>
+        <v>89082</v>
       </c>
     </row>
     <row r="1586">
@@ -17881,7 +17881,7 @@
         <v>2601</v>
       </c>
       <c r="C1586" t="n">
-        <v>162500</v>
+        <v>175000</v>
       </c>
     </row>
     <row r="1587">
@@ -17892,7 +17892,7 @@
         <v>1142</v>
       </c>
       <c r="C1587" t="n">
-        <v>270686</v>
+        <v>291508</v>
       </c>
     </row>
     <row r="1588">
@@ -17936,7 +17936,7 @@
         <v>2082</v>
       </c>
       <c r="C1591" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1592">
@@ -17947,7 +17947,7 @@
         <v>2276</v>
       </c>
       <c r="C1592" t="n">
-        <v>117546</v>
+        <v>126588</v>
       </c>
     </row>
     <row r="1593">
@@ -17958,7 +17958,7 @@
         <v>2786</v>
       </c>
       <c r="C1593" t="n">
-        <v>41353</v>
+        <v>44534</v>
       </c>
     </row>
     <row r="1594">
@@ -17969,7 +17969,7 @@
         <v>2816</v>
       </c>
       <c r="C1594" t="n">
-        <v>76817</v>
+        <v>82726</v>
       </c>
     </row>
     <row r="1595">
@@ -17980,7 +17980,7 @@
         <v>1871</v>
       </c>
       <c r="C1595" t="n">
-        <v>84799</v>
+        <v>91322</v>
       </c>
     </row>
     <row r="1596">
@@ -17991,7 +17991,7 @@
         <v>2345</v>
       </c>
       <c r="C1596" t="n">
-        <v>37700</v>
+        <v>40600</v>
       </c>
     </row>
     <row r="1597">
@@ -18002,7 +18002,7 @@
         <v>2802</v>
       </c>
       <c r="C1597" t="n">
-        <v>42419</v>
+        <v>45682</v>
       </c>
     </row>
     <row r="1598">
@@ -18013,7 +18013,7 @@
         <v>2090</v>
       </c>
       <c r="C1598" t="n">
-        <v>24583</v>
+        <v>26474</v>
       </c>
     </row>
     <row r="1599">
@@ -18024,7 +18024,7 @@
         <v>2647</v>
       </c>
       <c r="C1599" t="n">
-        <v>82875</v>
+        <v>89250</v>
       </c>
     </row>
     <row r="1600">
@@ -18035,7 +18035,7 @@
         <v>2365</v>
       </c>
       <c r="C1600" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1601">
@@ -18046,7 +18046,7 @@
         <v>766</v>
       </c>
       <c r="C1601" t="n">
-        <v>40586</v>
+        <v>43708</v>
       </c>
     </row>
     <row r="1602">
@@ -18057,7 +18057,7 @@
         <v>2702</v>
       </c>
       <c r="C1602" t="n">
-        <v>48139</v>
+        <v>51842</v>
       </c>
     </row>
     <row r="1603">
@@ -18068,7 +18068,7 @@
         <v>20</v>
       </c>
       <c r="C1603" t="n">
-        <v>265909.14</v>
+        <v>286363.68</v>
       </c>
     </row>
     <row r="1604">
@@ -18079,7 +18079,7 @@
         <v>27</v>
       </c>
       <c r="C1604" t="n">
-        <v>88636.38</v>
+        <v>95454.56</v>
       </c>
     </row>
     <row r="1605">
@@ -18090,7 +18090,7 @@
         <v>33</v>
       </c>
       <c r="C1605" t="n">
-        <v>235170</v>
+        <v>253260</v>
       </c>
     </row>
     <row r="1606">
@@ -18112,7 +18112,7 @@
         <v>2561</v>
       </c>
       <c r="C1607" t="n">
-        <v>23101</v>
+        <v>24878</v>
       </c>
     </row>
     <row r="1608">
@@ -18134,7 +18134,7 @@
         <v>2772</v>
       </c>
       <c r="C1609" t="n">
-        <v>35451</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1610">
@@ -18145,7 +18145,7 @@
         <v>2834</v>
       </c>
       <c r="C1610" t="n">
-        <v>22022</v>
+        <v>23716</v>
       </c>
     </row>
     <row r="1611">
@@ -18156,7 +18156,7 @@
         <v>2394</v>
       </c>
       <c r="C1611" t="n">
-        <v>67041</v>
+        <v>72198</v>
       </c>
     </row>
     <row r="1612">
@@ -18167,7 +18167,7 @@
         <v>2567</v>
       </c>
       <c r="C1612" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1613">
@@ -18178,7 +18178,7 @@
         <v>952</v>
       </c>
       <c r="C1613" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1614">
@@ -18189,7 +18189,7 @@
         <v>1539</v>
       </c>
       <c r="C1614" t="n">
-        <v>100451</v>
+        <v>108178</v>
       </c>
     </row>
     <row r="1615">
@@ -18200,7 +18200,7 @@
         <v>793</v>
       </c>
       <c r="C1615" t="n">
-        <v>24583</v>
+        <v>26474</v>
       </c>
     </row>
     <row r="1616">
@@ -18211,7 +18211,7 @@
         <v>794</v>
       </c>
       <c r="C1616" t="n">
-        <v>24583</v>
+        <v>26474</v>
       </c>
     </row>
     <row r="1617">
@@ -18222,7 +18222,7 @@
         <v>2838</v>
       </c>
       <c r="C1617" t="n">
-        <v>35454.57</v>
+        <v>38181.84</v>
       </c>
     </row>
     <row r="1618">
@@ -18233,7 +18233,7 @@
         <v>2223</v>
       </c>
       <c r="C1618" t="n">
-        <v>69199</v>
+        <v>74522</v>
       </c>
     </row>
     <row r="1619">
@@ -18244,7 +18244,7 @@
         <v>2547</v>
       </c>
       <c r="C1619" t="n">
-        <v>20020</v>
+        <v>21560</v>
       </c>
     </row>
     <row r="1620">
@@ -18255,7 +18255,7 @@
         <v>2762</v>
       </c>
       <c r="C1620" t="n">
-        <v>48139</v>
+        <v>51842</v>
       </c>
     </row>
     <row r="1621">
@@ -18266,7 +18266,7 @@
         <v>2550</v>
       </c>
       <c r="C1621" t="n">
-        <v>23101</v>
+        <v>24878</v>
       </c>
     </row>
     <row r="1622">
@@ -18277,7 +18277,7 @@
         <v>2627</v>
       </c>
       <c r="C1622" t="n">
-        <v>23101</v>
+        <v>24878</v>
       </c>
     </row>
     <row r="1623">
@@ -18299,7 +18299,7 @@
         <v>749</v>
       </c>
       <c r="C1624" t="n">
-        <v>48139</v>
+        <v>51842</v>
       </c>
     </row>
     <row r="1625">
@@ -18310,7 +18310,7 @@
         <v>2549</v>
       </c>
       <c r="C1625" t="n">
-        <v>23101</v>
+        <v>24878</v>
       </c>
     </row>
     <row r="1626">
@@ -18321,7 +18321,7 @@
         <v>2649</v>
       </c>
       <c r="C1626" t="n">
-        <v>23101</v>
+        <v>24878</v>
       </c>
     </row>
     <row r="1627">
@@ -18332,7 +18332,7 @@
         <v>2258</v>
       </c>
       <c r="C1627" t="n">
-        <v>47268</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1628">
@@ -18343,7 +18343,7 @@
         <v>2744</v>
       </c>
       <c r="C1628" t="n">
-        <v>35451</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1629">
@@ -18354,7 +18354,7 @@
         <v>452</v>
       </c>
       <c r="C1629" t="n">
-        <v>167219</v>
+        <v>180082</v>
       </c>
     </row>
     <row r="1630">
@@ -18376,7 +18376,7 @@
         <v>2653</v>
       </c>
       <c r="C1631" t="n">
-        <v>35451</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1632">
@@ -18409,7 +18409,7 @@
         <v>2742</v>
       </c>
       <c r="C1634" t="n">
-        <v>11817</v>
+        <v>12726</v>
       </c>
     </row>
     <row r="1635">
@@ -18420,7 +18420,7 @@
         <v>1499</v>
       </c>
       <c r="C1635" t="n">
-        <v>53170</v>
+        <v>57260</v>
       </c>
     </row>
     <row r="1636">
@@ -18431,7 +18431,7 @@
         <v>2261</v>
       </c>
       <c r="C1636" t="n">
-        <v>106353</v>
+        <v>114534</v>
       </c>
     </row>
     <row r="1637">
@@ -18442,7 +18442,7 @@
         <v>1324</v>
       </c>
       <c r="C1637" t="n">
-        <v>165451</v>
+        <v>178178</v>
       </c>
     </row>
     <row r="1638">
@@ -18453,7 +18453,7 @@
         <v>2709</v>
       </c>
       <c r="C1638" t="n">
-        <v>106353</v>
+        <v>114534</v>
       </c>
     </row>
     <row r="1639">
@@ -18464,7 +18464,7 @@
         <v>1137</v>
       </c>
       <c r="C1639" t="n">
-        <v>378170</v>
+        <v>407260</v>
       </c>
     </row>
     <row r="1640">
@@ -18475,7 +18475,7 @@
         <v>2440</v>
       </c>
       <c r="C1640" t="n">
-        <v>47268</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1641">
@@ -18486,7 +18486,7 @@
         <v>429</v>
       </c>
       <c r="C1641" t="n">
-        <v>224536</v>
+        <v>241808</v>
       </c>
     </row>
     <row r="1642">
@@ -18497,7 +18497,7 @@
         <v>2114</v>
       </c>
       <c r="C1642" t="n">
-        <v>100529</v>
+        <v>108262</v>
       </c>
     </row>
     <row r="1643">
@@ -18508,7 +18508,7 @@
         <v>2211</v>
       </c>
       <c r="C1643" t="n">
-        <v>142311</v>
+        <v>153258</v>
       </c>
     </row>
     <row r="1644">
@@ -18519,7 +18519,7 @@
         <v>1108</v>
       </c>
       <c r="C1644" t="n">
-        <v>181038</v>
+        <v>194964</v>
       </c>
     </row>
     <row r="1645">
@@ -18530,7 +18530,7 @@
         <v>2695</v>
       </c>
       <c r="C1645" t="n">
-        <v>28587</v>
+        <v>30786</v>
       </c>
     </row>
     <row r="1646">
@@ -18541,7 +18541,7 @@
         <v>1289</v>
       </c>
       <c r="C1646" t="n">
-        <v>162500</v>
+        <v>175000</v>
       </c>
     </row>
     <row r="1647">
@@ -18552,7 +18552,7 @@
         <v>2789</v>
       </c>
       <c r="C1647" t="n">
-        <v>106363.71</v>
+        <v>114545.52</v>
       </c>
     </row>
     <row r="1648">
@@ -18563,7 +18563,7 @@
         <v>2197</v>
       </c>
       <c r="C1648" t="n">
-        <v>127045.52</v>
+        <v>136818.24</v>
       </c>
     </row>
     <row r="1649">
@@ -18574,7 +18574,7 @@
         <v>947</v>
       </c>
       <c r="C1649" t="n">
-        <v>262054</v>
+        <v>282212</v>
       </c>
     </row>
     <row r="1650">
@@ -18585,7 +18585,7 @@
         <v>2279</v>
       </c>
       <c r="C1650" t="n">
-        <v>144729</v>
+        <v>155862</v>
       </c>
     </row>
     <row r="1651">
@@ -18596,7 +18596,7 @@
         <v>1465</v>
       </c>
       <c r="C1651" t="n">
-        <v>227500</v>
+        <v>245000</v>
       </c>
     </row>
     <row r="1652">
@@ -18607,7 +18607,7 @@
         <v>2651</v>
       </c>
       <c r="C1652" t="n">
-        <v>100451</v>
+        <v>108178</v>
       </c>
     </row>
     <row r="1653">
@@ -18618,7 +18618,7 @@
         <v>42</v>
       </c>
       <c r="C1653" t="n">
-        <v>1126268</v>
+        <v>1212904</v>
       </c>
     </row>
     <row r="1654">
@@ -18629,7 +18629,7 @@
         <v>949</v>
       </c>
       <c r="C1654" t="n">
-        <v>58773</v>
+        <v>63294</v>
       </c>
     </row>
     <row r="1655">
@@ -18640,7 +18640,7 @@
         <v>2606</v>
       </c>
       <c r="C1655" t="n">
-        <v>151710</v>
+        <v>163380</v>
       </c>
     </row>
     <row r="1656">
@@ -18651,7 +18651,7 @@
         <v>2249</v>
       </c>
       <c r="C1656" t="n">
-        <v>128895</v>
+        <v>138810</v>
       </c>
     </row>
     <row r="1657">
@@ -18695,7 +18695,7 @@
         <v>2045</v>
       </c>
       <c r="C1660" t="n">
-        <v>188188</v>
+        <v>202664</v>
       </c>
     </row>
     <row r="1661">
@@ -18706,7 +18706,7 @@
         <v>2663</v>
       </c>
       <c r="C1661" t="n">
-        <v>162500</v>
+        <v>175000</v>
       </c>
     </row>
     <row r="1662">
@@ -18728,7 +18728,7 @@
         <v>2854</v>
       </c>
       <c r="C1663" t="n">
-        <v>23634</v>
+        <v>25452</v>
       </c>
     </row>
     <row r="1664">
@@ -18750,7 +18750,7 @@
         <v>2341</v>
       </c>
       <c r="C1665" t="n">
-        <v>103350</v>
+        <v>111300</v>
       </c>
     </row>
     <row r="1666">
@@ -18761,7 +18761,7 @@
         <v>2637</v>
       </c>
       <c r="C1666" t="n">
-        <v>37700</v>
+        <v>40600</v>
       </c>
     </row>
     <row r="1667">
@@ -18772,7 +18772,7 @@
         <v>2492</v>
       </c>
       <c r="C1667" t="n">
-        <v>59189</v>
+        <v>63742</v>
       </c>
     </row>
     <row r="1668">
@@ -18783,7 +18783,7 @@
         <v>2548</v>
       </c>
       <c r="C1668" t="n">
-        <v>23101</v>
+        <v>24878</v>
       </c>
     </row>
     <row r="1669">
@@ -18794,7 +18794,7 @@
         <v>351</v>
       </c>
       <c r="C1669" t="n">
-        <v>125853</v>
+        <v>135534</v>
       </c>
     </row>
     <row r="1670">
@@ -18827,7 +18827,7 @@
         <v>2757</v>
       </c>
       <c r="C1672" t="n">
-        <v>47268</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1673">
@@ -18838,7 +18838,7 @@
         <v>2815</v>
       </c>
       <c r="C1673" t="n">
-        <v>35451</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1674">
@@ -18849,7 +18849,7 @@
         <v>2323</v>
       </c>
       <c r="C1674" t="n">
-        <v>40586</v>
+        <v>43708</v>
       </c>
     </row>
     <row r="1675">
@@ -18860,7 +18860,7 @@
         <v>2310</v>
       </c>
       <c r="C1675" t="n">
-        <v>40586</v>
+        <v>43708</v>
       </c>
     </row>
     <row r="1676">
@@ -18871,7 +18871,7 @@
         <v>2145</v>
       </c>
       <c r="C1676" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1677">
@@ -18882,7 +18882,7 @@
         <v>2501</v>
       </c>
       <c r="C1677" t="n">
-        <v>48139</v>
+        <v>51842</v>
       </c>
     </row>
     <row r="1678">
@@ -18893,7 +18893,7 @@
         <v>2546</v>
       </c>
       <c r="C1678" t="n">
-        <v>23101</v>
+        <v>24878</v>
       </c>
     </row>
     <row r="1679">
@@ -18904,7 +18904,7 @@
         <v>716</v>
       </c>
       <c r="C1679" t="n">
-        <v>75738</v>
+        <v>81564</v>
       </c>
     </row>
     <row r="1680">
@@ -18915,7 +18915,7 @@
         <v>2758</v>
       </c>
       <c r="C1680" t="n">
-        <v>35451</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1681">
@@ -18926,7 +18926,7 @@
         <v>400</v>
       </c>
       <c r="C1681" t="n">
-        <v>106353</v>
+        <v>114534</v>
       </c>
     </row>
     <row r="1682">
@@ -18937,7 +18937,7 @@
         <v>6</v>
       </c>
       <c r="C1682" t="n">
-        <v>29545.52</v>
+        <v>31818.24</v>
       </c>
     </row>
     <row r="1683">
@@ -18970,7 +18970,7 @@
         <v>1259</v>
       </c>
       <c r="C1685" t="n">
-        <v>65000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="1686">
@@ -18981,7 +18981,7 @@
         <v>571</v>
       </c>
       <c r="C1686" t="n">
-        <v>611590.95</v>
+        <v>658636.4</v>
       </c>
     </row>
     <row r="1687">
@@ -18992,7 +18992,7 @@
         <v>703</v>
       </c>
       <c r="C1687" t="n">
-        <v>147719</v>
+        <v>159082</v>
       </c>
     </row>
     <row r="1688">
@@ -19014,7 +19014,7 @@
         <v>2833</v>
       </c>
       <c r="C1689" t="n">
-        <v>47268</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1690">
@@ -19025,7 +19025,7 @@
         <v>1007</v>
       </c>
       <c r="C1690" t="n">
-        <v>118181.9</v>
+        <v>127272.8</v>
       </c>
     </row>
     <row r="1691">
@@ -19036,7 +19036,7 @@
         <v>2687</v>
       </c>
       <c r="C1691" t="n">
-        <v>47268</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1692">
@@ -19047,7 +19047,7 @@
         <v>2824</v>
       </c>
       <c r="C1692" t="n">
-        <v>66716</v>
+        <v>71848</v>
       </c>
     </row>
     <row r="1693">
@@ -19058,7 +19058,7 @@
         <v>2730</v>
       </c>
       <c r="C1693" t="n">
-        <v>53170</v>
+        <v>57260</v>
       </c>
     </row>
     <row r="1694">
@@ -19069,7 +19069,7 @@
         <v>2718</v>
       </c>
       <c r="C1694" t="n">
-        <v>76817</v>
+        <v>82726</v>
       </c>
     </row>
     <row r="1695">
@@ -19080,7 +19080,7 @@
         <v>2750</v>
       </c>
       <c r="C1695" t="n">
-        <v>17719</v>
+        <v>19082</v>
       </c>
     </row>
     <row r="1696">
@@ -19091,7 +19091,7 @@
         <v>854</v>
       </c>
       <c r="C1696" t="n">
-        <v>82719</v>
+        <v>89082</v>
       </c>
     </row>
     <row r="1697">
@@ -19102,7 +19102,7 @@
         <v>2794</v>
       </c>
       <c r="C1697" t="n">
-        <v>70902</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1698">
@@ -19113,7 +19113,7 @@
         <v>1374</v>
       </c>
       <c r="C1698" t="n">
-        <v>118170</v>
+        <v>127260</v>
       </c>
     </row>
     <row r="1699">
@@ -19124,7 +19124,7 @@
         <v>2488</v>
       </c>
       <c r="C1699" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1700">
@@ -19135,7 +19135,7 @@
         <v>363</v>
       </c>
       <c r="C1700" t="n">
-        <v>177268</v>
+        <v>190904</v>
       </c>
     </row>
     <row r="1701">
@@ -19146,7 +19146,7 @@
         <v>2655</v>
       </c>
       <c r="C1701" t="n">
-        <v>65000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="1702">
@@ -19157,7 +19157,7 @@
         <v>1873</v>
       </c>
       <c r="C1702" t="n">
-        <v>189085</v>
+        <v>203630</v>
       </c>
     </row>
     <row r="1703">
@@ -19168,7 +19168,7 @@
         <v>2635</v>
       </c>
       <c r="C1703" t="n">
-        <v>76817</v>
+        <v>82726</v>
       </c>
     </row>
     <row r="1704">
@@ -19179,7 +19179,7 @@
         <v>1658</v>
       </c>
       <c r="C1704" t="n">
-        <v>90402</v>
+        <v>97356</v>
       </c>
     </row>
     <row r="1705">
@@ -19190,7 +19190,7 @@
         <v>2069</v>
       </c>
       <c r="C1705" t="n">
-        <v>118181.9</v>
+        <v>127272.8</v>
       </c>
     </row>
     <row r="1706">
@@ -19201,7 +19201,7 @@
         <v>2081</v>
       </c>
       <c r="C1706" t="n">
-        <v>88634</v>
+        <v>95452</v>
       </c>
     </row>
     <row r="1707">
@@ -19212,7 +19212,7 @@
         <v>2124</v>
       </c>
       <c r="C1707" t="n">
-        <v>206817</v>
+        <v>222726</v>
       </c>
     </row>
     <row r="1708">
@@ -19223,7 +19223,7 @@
         <v>636</v>
       </c>
       <c r="C1708" t="n">
-        <v>147719</v>
+        <v>159082</v>
       </c>
     </row>
     <row r="1709">
@@ -19234,7 +19234,7 @@
         <v>2803</v>
       </c>
       <c r="C1709" t="n">
-        <v>70902</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1710">
@@ -19245,7 +19245,7 @@
         <v>2163</v>
       </c>
       <c r="C1710" t="n">
-        <v>106353</v>
+        <v>114534</v>
       </c>
     </row>
     <row r="1711">
@@ -19256,7 +19256,7 @@
         <v>1466</v>
       </c>
       <c r="C1711" t="n">
-        <v>239317</v>
+        <v>257726</v>
       </c>
     </row>
     <row r="1712">
@@ -19267,7 +19267,7 @@
         <v>2133</v>
       </c>
       <c r="C1712" t="n">
-        <v>206818.19</v>
+        <v>222727.28</v>
       </c>
     </row>
     <row r="1713">
@@ -19278,7 +19278,7 @@
         <v>2431</v>
       </c>
       <c r="C1713" t="n">
-        <v>88634</v>
+        <v>95452</v>
       </c>
     </row>
     <row r="1714">
@@ -19289,7 +19289,7 @@
         <v>535</v>
       </c>
       <c r="C1714" t="n">
-        <v>210470</v>
+        <v>226660</v>
       </c>
     </row>
     <row r="1715">
@@ -19300,7 +19300,7 @@
         <v>2790</v>
       </c>
       <c r="C1715" t="n">
-        <v>37323</v>
+        <v>40194</v>
       </c>
     </row>
     <row r="1716">
@@ -19311,7 +19311,7 @@
         <v>2442</v>
       </c>
       <c r="C1716" t="n">
-        <v>153036</v>
+        <v>164808</v>
       </c>
     </row>
     <row r="1717">
@@ -19322,7 +19322,7 @@
         <v>2376</v>
       </c>
       <c r="C1717" t="n">
-        <v>650000</v>
+        <v>700000</v>
       </c>
     </row>
     <row r="1718">
@@ -19333,7 +19333,7 @@
         <v>2768</v>
       </c>
       <c r="C1718" t="n">
-        <v>178841</v>
+        <v>192598</v>
       </c>
     </row>
     <row r="1719">
@@ -19344,7 +19344,7 @@
         <v>2491</v>
       </c>
       <c r="C1719" t="n">
-        <v>143507</v>
+        <v>154546</v>
       </c>
     </row>
     <row r="1720">
@@ -19355,7 +19355,7 @@
         <v>2799</v>
       </c>
       <c r="C1720" t="n">
-        <v>64597</v>
+        <v>69566</v>
       </c>
     </row>
     <row r="1721">
@@ -19388,7 +19388,7 @@
         <v>1317</v>
       </c>
       <c r="C1723" t="n">
-        <v>186136.38</v>
+        <v>200454.56</v>
       </c>
     </row>
     <row r="1724">
@@ -19399,7 +19399,7 @@
         <v>2822</v>
       </c>
       <c r="C1724" t="n">
-        <v>94545.52</v>
+        <v>101818.24</v>
       </c>
     </row>
     <row r="1725">
@@ -19410,7 +19410,7 @@
         <v>1117</v>
       </c>
       <c r="C1725" t="n">
-        <v>236431</v>
+        <v>254618</v>
       </c>
     </row>
     <row r="1726">
@@ -19421,7 +19421,7 @@
         <v>1299</v>
       </c>
       <c r="C1726" t="n">
-        <v>311727</v>
+        <v>335706</v>
       </c>
     </row>
     <row r="1727">
@@ -19432,7 +19432,7 @@
         <v>477</v>
       </c>
       <c r="C1727" t="n">
-        <v>128466</v>
+        <v>138348</v>
       </c>
     </row>
     <row r="1728">
@@ -19443,7 +19443,7 @@
         <v>530</v>
       </c>
       <c r="C1728" t="n">
-        <v>177268</v>
+        <v>190904</v>
       </c>
     </row>
     <row r="1729">
@@ -19454,7 +19454,7 @@
         <v>953</v>
       </c>
       <c r="C1729" t="n">
-        <v>407719</v>
+        <v>439082</v>
       </c>
     </row>
     <row r="1730">
@@ -19465,7 +19465,7 @@
         <v>610</v>
       </c>
       <c r="C1730" t="n">
-        <v>485602</v>
+        <v>522956</v>
       </c>
     </row>
     <row r="1731">
@@ -19476,7 +19476,7 @@
         <v>2792</v>
       </c>
       <c r="C1731" t="n">
-        <v>121953</v>
+        <v>131334</v>
       </c>
     </row>
     <row r="1732">
@@ -19553,7 +19553,7 @@
         <v>1075</v>
       </c>
       <c r="C1738" t="n">
-        <v>271219</v>
+        <v>292082</v>
       </c>
     </row>
     <row r="1739">
@@ -19564,7 +19564,7 @@
         <v>131</v>
       </c>
       <c r="C1739" t="n">
-        <v>245817</v>
+        <v>264726</v>
       </c>
     </row>
     <row r="1740">
@@ -19575,7 +19575,7 @@
         <v>2667</v>
       </c>
       <c r="C1740" t="n">
-        <v>27001</v>
+        <v>29078</v>
       </c>
     </row>
     <row r="1741">
@@ -19586,7 +19586,7 @@
         <v>2330</v>
       </c>
       <c r="C1741" t="n">
-        <v>52559</v>
+        <v>56602</v>
       </c>
     </row>
     <row r="1742">
@@ -19608,7 +19608,7 @@
         <v>2577</v>
       </c>
       <c r="C1743" t="n">
-        <v>52689</v>
+        <v>56742</v>
       </c>
     </row>
     <row r="1744">
@@ -19619,7 +19619,7 @@
         <v>2510</v>
       </c>
       <c r="C1744" t="n">
-        <v>374192</v>
+        <v>402976</v>
       </c>
     </row>
     <row r="1745">
@@ -19641,7 +19641,7 @@
         <v>2850</v>
       </c>
       <c r="C1746" t="n">
-        <v>35451</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1747">
@@ -19663,7 +19663,7 @@
         <v>2745</v>
       </c>
       <c r="C1748" t="n">
-        <v>65000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="1749">
@@ -19674,7 +19674,7 @@
         <v>2817</v>
       </c>
       <c r="C1749" t="n">
-        <v>35451</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1750">
@@ -19685,7 +19685,7 @@
         <v>2784</v>
       </c>
       <c r="C1750" t="n">
-        <v>24583</v>
+        <v>26474</v>
       </c>
     </row>
     <row r="1751">
@@ -19696,7 +19696,7 @@
         <v>626</v>
       </c>
       <c r="C1751" t="n">
-        <v>1020981</v>
+        <v>1099518</v>
       </c>
     </row>
     <row r="1752">
@@ -19707,7 +19707,7 @@
         <v>925</v>
       </c>
       <c r="C1752" t="n">
-        <v>47138</v>
+        <v>50764</v>
       </c>
     </row>
     <row r="1753">
@@ -19718,7 +19718,7 @@
         <v>2586</v>
       </c>
       <c r="C1753" t="n">
-        <v>24583</v>
+        <v>26474</v>
       </c>
     </row>
     <row r="1754">
@@ -19729,7 +19729,7 @@
         <v>966</v>
       </c>
       <c r="C1754" t="n">
-        <v>48139</v>
+        <v>51842</v>
       </c>
     </row>
     <row r="1755">
@@ -19740,7 +19740,7 @@
         <v>2557</v>
       </c>
       <c r="C1755" t="n">
-        <v>23101</v>
+        <v>24878</v>
       </c>
     </row>
     <row r="1756">
@@ -19751,7 +19751,7 @@
         <v>14</v>
       </c>
       <c r="C1756" t="n">
-        <v>265902</v>
+        <v>286356</v>
       </c>
     </row>
     <row r="1757">
@@ -19762,7 +19762,7 @@
         <v>2798</v>
       </c>
       <c r="C1757" t="n">
-        <v>35451</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1758">
@@ -19784,7 +19784,7 @@
         <v>522</v>
       </c>
       <c r="C1759" t="n">
-        <v>118181.9</v>
+        <v>127272.8</v>
       </c>
     </row>
     <row r="1760">
@@ -19806,7 +19806,7 @@
         <v>2819</v>
       </c>
       <c r="C1761" t="n">
-        <v>35451</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1762">
@@ -19817,7 +19817,7 @@
         <v>2266</v>
       </c>
       <c r="C1762" t="n">
-        <v>47268</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1763">
@@ -19850,7 +19850,7 @@
         <v>2795</v>
       </c>
       <c r="C1765" t="n">
-        <v>35451</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1766">
@@ -19861,7 +19861,7 @@
         <v>2722</v>
       </c>
       <c r="C1766" t="n">
-        <v>11817</v>
+        <v>12726</v>
       </c>
     </row>
     <row r="1767">
@@ -19872,7 +19872,7 @@
         <v>951</v>
       </c>
       <c r="C1767" t="n">
-        <v>67951</v>
+        <v>73178</v>
       </c>
     </row>
     <row r="1768">
@@ -19883,7 +19883,7 @@
         <v>1020</v>
       </c>
       <c r="C1768" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1769">
@@ -19894,7 +19894,7 @@
         <v>1853</v>
       </c>
       <c r="C1769" t="n">
-        <v>70902</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1770">
@@ -19905,7 +19905,7 @@
         <v>1327</v>
       </c>
       <c r="C1770" t="n">
-        <v>41353</v>
+        <v>44534</v>
       </c>
     </row>
     <row r="1771">
@@ -19916,7 +19916,7 @@
         <v>2842</v>
       </c>
       <c r="C1771" t="n">
-        <v>106353</v>
+        <v>114534</v>
       </c>
     </row>
     <row r="1772">
@@ -19927,7 +19927,7 @@
         <v>2831</v>
       </c>
       <c r="C1772" t="n">
-        <v>35451</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1773">
@@ -19938,7 +19938,7 @@
         <v>818</v>
       </c>
       <c r="C1773" t="n">
-        <v>236353</v>
+        <v>254534</v>
       </c>
     </row>
     <row r="1774">
@@ -19949,7 +19949,7 @@
         <v>1501</v>
       </c>
       <c r="C1774" t="n">
-        <v>59085</v>
+        <v>63630</v>
       </c>
     </row>
     <row r="1775">
@@ -19960,7 +19960,7 @@
         <v>1869</v>
       </c>
       <c r="C1775" t="n">
-        <v>144170</v>
+        <v>155260</v>
       </c>
     </row>
     <row r="1776">
@@ -19971,7 +19971,7 @@
         <v>1996</v>
       </c>
       <c r="C1776" t="n">
-        <v>147727.33</v>
+        <v>159090.96</v>
       </c>
     </row>
     <row r="1777">
@@ -19982,7 +19982,7 @@
         <v>2462</v>
       </c>
       <c r="C1777" t="n">
-        <v>33466.21</v>
+        <v>36040.52</v>
       </c>
     </row>
     <row r="1778">
@@ -19993,7 +19993,7 @@
         <v>2696</v>
       </c>
       <c r="C1778" t="n">
-        <v>126724</v>
+        <v>136472</v>
       </c>
     </row>
     <row r="1779">
@@ -20004,7 +20004,7 @@
         <v>2698</v>
       </c>
       <c r="C1779" t="n">
-        <v>64948</v>
+        <v>69944</v>
       </c>
     </row>
     <row r="1780">
@@ -20026,7 +20026,7 @@
         <v>2828</v>
       </c>
       <c r="C1781" t="n">
-        <v>35454.57</v>
+        <v>38181.84</v>
       </c>
     </row>
     <row r="1782">
@@ -20037,7 +20037,7 @@
         <v>2843</v>
       </c>
       <c r="C1782" t="n">
-        <v>41353</v>
+        <v>44534</v>
       </c>
     </row>
     <row r="1783">
@@ -20048,7 +20048,7 @@
         <v>619</v>
       </c>
       <c r="C1783" t="n">
-        <v>185250</v>
+        <v>199500</v>
       </c>
     </row>
     <row r="1784">
@@ -20059,7 +20059,7 @@
         <v>1478</v>
       </c>
       <c r="C1784" t="n">
-        <v>324194</v>
+        <v>349132</v>
       </c>
     </row>
     <row r="1785">
@@ -20070,7 +20070,7 @@
         <v>2026</v>
       </c>
       <c r="C1785" t="n">
-        <v>143234</v>
+        <v>154252</v>
       </c>
     </row>
     <row r="1786">
@@ -20081,7 +20081,7 @@
         <v>663</v>
       </c>
       <c r="C1786" t="n">
-        <v>153036</v>
+        <v>164808</v>
       </c>
     </row>
     <row r="1787">
@@ -20092,7 +20092,7 @@
         <v>285</v>
       </c>
       <c r="C1787" t="n">
-        <v>324194</v>
+        <v>349132</v>
       </c>
     </row>
     <row r="1788">
@@ -20103,7 +20103,7 @@
         <v>424</v>
       </c>
       <c r="C1788" t="n">
-        <v>138931</v>
+        <v>149618</v>
       </c>
     </row>
     <row r="1789">
@@ -20114,7 +20114,7 @@
         <v>451</v>
       </c>
       <c r="C1789" t="n">
-        <v>143585</v>
+        <v>154630</v>
       </c>
     </row>
     <row r="1790">
@@ -20125,7 +20125,7 @@
         <v>629</v>
       </c>
       <c r="C1790" t="n">
-        <v>268268</v>
+        <v>288904</v>
       </c>
     </row>
     <row r="1791">
@@ -20136,7 +20136,7 @@
         <v>2657</v>
       </c>
       <c r="C1791" t="n">
-        <v>46787</v>
+        <v>50386</v>
       </c>
     </row>
     <row r="1792">
@@ -20147,7 +20147,7 @@
         <v>1254</v>
       </c>
       <c r="C1792" t="n">
-        <v>114751</v>
+        <v>123578</v>
       </c>
     </row>
     <row r="1793">
@@ -20158,7 +20158,7 @@
         <v>2402</v>
       </c>
       <c r="C1793" t="n">
-        <v>288626</v>
+        <v>310828</v>
       </c>
     </row>
     <row r="1794">
@@ -20169,7 +20169,7 @@
         <v>2413</v>
       </c>
       <c r="C1794" t="n">
-        <v>81445</v>
+        <v>87710</v>
       </c>
     </row>
     <row r="1795">
@@ -20180,7 +20180,7 @@
         <v>1450</v>
       </c>
       <c r="C1795" t="n">
-        <v>210951</v>
+        <v>227178</v>
       </c>
     </row>
     <row r="1796">
@@ -20202,7 +20202,7 @@
         <v>2671</v>
       </c>
       <c r="C1797" t="n">
-        <v>47268</v>
+        <v>50904</v>
       </c>
     </row>
     <row r="1798">
@@ -20213,7 +20213,7 @@
         <v>2568</v>
       </c>
       <c r="C1798" t="n">
-        <v>94809</v>
+        <v>102102</v>
       </c>
     </row>
     <row r="1799">
@@ -20224,7 +20224,7 @@
         <v>2146</v>
       </c>
       <c r="C1799" t="n">
-        <v>114803</v>
+        <v>123634</v>
       </c>
     </row>
     <row r="1800">
@@ -20235,7 +20235,7 @@
         <v>2753</v>
       </c>
       <c r="C1800" t="n">
-        <v>44317</v>
+        <v>47726</v>
       </c>
     </row>
     <row r="1801">
@@ -20246,7 +20246,7 @@
         <v>744</v>
       </c>
       <c r="C1801" t="n">
-        <v>24583</v>
+        <v>26474</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:02:15
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -15560,7 +15560,7 @@
         <v>2853</v>
       </c>
       <c r="C1375" t="n">
-        <v>51842</v>
+        <v>55545</v>
       </c>
     </row>
     <row r="1376">
@@ -15571,7 +15571,7 @@
         <v>2245</v>
       </c>
       <c r="C1376" t="n">
-        <v>140896</v>
+        <v>150960</v>
       </c>
     </row>
     <row r="1377">
@@ -15582,7 +15582,7 @@
         <v>2251</v>
       </c>
       <c r="C1377" t="n">
-        <v>127260</v>
+        <v>136350</v>
       </c>
     </row>
     <row r="1378">
@@ -15593,7 +15593,7 @@
         <v>664</v>
       </c>
       <c r="C1378" t="n">
-        <v>166726</v>
+        <v>178635</v>
       </c>
     </row>
     <row r="1379">
@@ -15604,7 +15604,7 @@
         <v>2472</v>
       </c>
       <c r="C1379" t="n">
-        <v>33684</v>
+        <v>36090</v>
       </c>
     </row>
     <row r="1380">
@@ -15615,7 +15615,7 @@
         <v>1456</v>
       </c>
       <c r="C1380" t="n">
-        <v>507808</v>
+        <v>544080</v>
       </c>
     </row>
     <row r="1381">
@@ -15626,7 +15626,7 @@
         <v>1585</v>
       </c>
       <c r="C1381" t="n">
-        <v>115178</v>
+        <v>123405</v>
       </c>
     </row>
     <row r="1382">
@@ -15670,7 +15670,7 @@
         <v>1907</v>
       </c>
       <c r="C1385" t="n">
-        <v>350336</v>
+        <v>375360</v>
       </c>
     </row>
     <row r="1386">
@@ -15703,7 +15703,7 @@
         <v>2659</v>
       </c>
       <c r="C1388" t="n">
-        <v>78274</v>
+        <v>83865</v>
       </c>
     </row>
     <row r="1389">
@@ -15714,7 +15714,7 @@
         <v>2583</v>
       </c>
       <c r="C1389" t="n">
-        <v>26474</v>
+        <v>28365</v>
       </c>
     </row>
     <row r="1390">
@@ -15725,7 +15725,7 @@
         <v>2692</v>
       </c>
       <c r="C1390" t="n">
-        <v>44545.52</v>
+        <v>47727.33</v>
       </c>
     </row>
     <row r="1391">
@@ -15736,7 +15736,7 @@
         <v>2691</v>
       </c>
       <c r="C1391" t="n">
-        <v>77753.52</v>
+        <v>83307.33</v>
       </c>
     </row>
     <row r="1392">
@@ -15747,7 +15747,7 @@
         <v>931</v>
       </c>
       <c r="C1392" t="n">
-        <v>60914</v>
+        <v>65265</v>
       </c>
     </row>
     <row r="1393">
@@ -15758,7 +15758,7 @@
         <v>2785</v>
       </c>
       <c r="C1393" t="n">
-        <v>26474</v>
+        <v>28365</v>
       </c>
     </row>
     <row r="1394">
@@ -15769,7 +15769,7 @@
         <v>2411</v>
       </c>
       <c r="C1394" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1395">
@@ -15780,7 +15780,7 @@
         <v>2716</v>
       </c>
       <c r="C1395" t="n">
-        <v>55832</v>
+        <v>59820</v>
       </c>
     </row>
     <row r="1396">
@@ -15791,7 +15791,7 @@
         <v>2809</v>
       </c>
       <c r="C1396" t="n">
-        <v>43708</v>
+        <v>46830</v>
       </c>
     </row>
     <row r="1397">
@@ -15802,7 +15802,7 @@
         <v>104</v>
       </c>
       <c r="C1397" t="n">
-        <v>190909.12</v>
+        <v>204545.48</v>
       </c>
     </row>
     <row r="1398">
@@ -15835,7 +15835,7 @@
         <v>781</v>
       </c>
       <c r="C1400" t="n">
-        <v>82726</v>
+        <v>88635</v>
       </c>
     </row>
     <row r="1401">
@@ -15857,7 +15857,7 @@
         <v>2494</v>
       </c>
       <c r="C1402" t="n">
-        <v>95452</v>
+        <v>102270</v>
       </c>
     </row>
     <row r="1403">
@@ -15868,7 +15868,7 @@
         <v>2652</v>
       </c>
       <c r="C1403" t="n">
-        <v>89082</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1404">
@@ -15879,7 +15879,7 @@
         <v>1384</v>
       </c>
       <c r="C1404" t="n">
-        <v>222727.28</v>
+        <v>238636.37</v>
       </c>
     </row>
     <row r="1405">
@@ -15890,7 +15890,7 @@
         <v>360</v>
       </c>
       <c r="C1405" t="n">
-        <v>318178</v>
+        <v>340905</v>
       </c>
     </row>
     <row r="1406">
@@ -15901,7 +15901,7 @@
         <v>2767</v>
       </c>
       <c r="C1406" t="n">
-        <v>120904</v>
+        <v>129540</v>
       </c>
     </row>
     <row r="1407">
@@ -15912,7 +15912,7 @@
         <v>2178</v>
       </c>
       <c r="C1407" t="n">
-        <v>174356</v>
+        <v>186810</v>
       </c>
     </row>
     <row r="1408">
@@ -15923,7 +15923,7 @@
         <v>2107</v>
       </c>
       <c r="C1408" t="n">
-        <v>190890</v>
+        <v>204525</v>
       </c>
     </row>
     <row r="1409">
@@ -15934,7 +15934,7 @@
         <v>2711</v>
       </c>
       <c r="C1409" t="n">
-        <v>55090</v>
+        <v>59025</v>
       </c>
     </row>
     <row r="1410">
@@ -15945,7 +15945,7 @@
         <v>2845</v>
       </c>
       <c r="C1410" t="n">
-        <v>31808</v>
+        <v>34080</v>
       </c>
     </row>
     <row r="1411">
@@ -15989,7 +15989,7 @@
         <v>1102</v>
       </c>
       <c r="C1414" t="n">
-        <v>149618</v>
+        <v>160305</v>
       </c>
     </row>
     <row r="1415">
@@ -16000,7 +16000,7 @@
         <v>353</v>
       </c>
       <c r="C1415" t="n">
-        <v>186158</v>
+        <v>199455</v>
       </c>
     </row>
     <row r="1416">
@@ -16011,7 +16011,7 @@
         <v>2250</v>
       </c>
       <c r="C1416" t="n">
-        <v>216356</v>
+        <v>231810</v>
       </c>
     </row>
     <row r="1417">
@@ -16022,7 +16022,7 @@
         <v>1800</v>
       </c>
       <c r="C1417" t="n">
-        <v>18046</v>
+        <v>19335</v>
       </c>
     </row>
     <row r="1418">
@@ -16033,7 +16033,7 @@
         <v>2362</v>
       </c>
       <c r="C1418" t="n">
-        <v>47726</v>
+        <v>51135</v>
       </c>
     </row>
     <row r="1419">
@@ -16044,7 +16044,7 @@
         <v>2449</v>
       </c>
       <c r="C1419" t="n">
-        <v>60452</v>
+        <v>64770</v>
       </c>
     </row>
     <row r="1420">
@@ -16055,7 +16055,7 @@
         <v>2844</v>
       </c>
       <c r="C1420" t="n">
-        <v>31808</v>
+        <v>34080</v>
       </c>
     </row>
     <row r="1421">
@@ -16066,7 +16066,7 @@
         <v>2507</v>
       </c>
       <c r="C1421" t="n">
-        <v>56840</v>
+        <v>60900</v>
       </c>
     </row>
     <row r="1422">
@@ -16077,7 +16077,7 @@
         <v>1906</v>
       </c>
       <c r="C1422" t="n">
-        <v>69090</v>
+        <v>74025</v>
       </c>
     </row>
     <row r="1423">
@@ -16099,7 +16099,7 @@
         <v>525</v>
       </c>
       <c r="C1424" t="n">
-        <v>149545.52</v>
+        <v>160227.33</v>
       </c>
     </row>
     <row r="1425">
@@ -16110,7 +16110,7 @@
         <v>1261</v>
       </c>
       <c r="C1425" t="n">
-        <v>45181.84</v>
+        <v>48409.11</v>
       </c>
     </row>
     <row r="1426">
@@ -16121,7 +16121,7 @@
         <v>2755</v>
       </c>
       <c r="C1426" t="n">
-        <v>31818.24</v>
+        <v>34090.96</v>
       </c>
     </row>
     <row r="1427">
@@ -16143,7 +16143,7 @@
         <v>1064</v>
       </c>
       <c r="C1428" t="n">
-        <v>381808</v>
+        <v>409080</v>
       </c>
     </row>
     <row r="1429">
@@ -16154,7 +16154,7 @@
         <v>1810</v>
       </c>
       <c r="C1429" t="n">
-        <v>25844</v>
+        <v>27690</v>
       </c>
     </row>
     <row r="1430">
@@ -16165,7 +16165,7 @@
         <v>1937</v>
       </c>
       <c r="C1430" t="n">
-        <v>164808</v>
+        <v>176580</v>
       </c>
     </row>
     <row r="1431">
@@ -16176,7 +16176,7 @@
         <v>483</v>
       </c>
       <c r="C1431" t="n">
-        <v>287630</v>
+        <v>308175</v>
       </c>
     </row>
     <row r="1432">
@@ -16187,7 +16187,7 @@
         <v>2580</v>
       </c>
       <c r="C1432" t="n">
-        <v>21434</v>
+        <v>22965</v>
       </c>
     </row>
     <row r="1433">
@@ -16198,7 +16198,7 @@
         <v>2706</v>
       </c>
       <c r="C1433" t="n">
-        <v>16744</v>
+        <v>17940</v>
       </c>
     </row>
     <row r="1434">
@@ -16209,7 +16209,7 @@
         <v>2633</v>
       </c>
       <c r="C1434" t="n">
-        <v>12264</v>
+        <v>13140</v>
       </c>
     </row>
     <row r="1435">
@@ -16242,7 +16242,7 @@
         <v>2392</v>
       </c>
       <c r="C1437" t="n">
-        <v>131992</v>
+        <v>141420</v>
       </c>
     </row>
     <row r="1438">
@@ -16264,7 +16264,7 @@
         <v>2613</v>
       </c>
       <c r="C1439" t="n">
-        <v>92932</v>
+        <v>99570</v>
       </c>
     </row>
     <row r="1440">
@@ -16275,7 +16275,7 @@
         <v>2183</v>
       </c>
       <c r="C1440" t="n">
-        <v>334614</v>
+        <v>358515</v>
       </c>
     </row>
     <row r="1441">
@@ -16286,7 +16286,7 @@
         <v>2541</v>
       </c>
       <c r="C1441" t="n">
-        <v>150430</v>
+        <v>161175</v>
       </c>
     </row>
     <row r="1442">
@@ -16297,7 +16297,7 @@
         <v>2333</v>
       </c>
       <c r="C1442" t="n">
-        <v>101556</v>
+        <v>108810</v>
       </c>
     </row>
     <row r="1443">
@@ -16308,7 +16308,7 @@
         <v>2813</v>
       </c>
       <c r="C1443" t="n">
-        <v>40600</v>
+        <v>43500</v>
       </c>
     </row>
     <row r="1444">
@@ -16319,7 +16319,7 @@
         <v>2811</v>
       </c>
       <c r="C1444" t="n">
-        <v>26474</v>
+        <v>28365</v>
       </c>
     </row>
     <row r="1445">
@@ -16330,7 +16330,7 @@
         <v>1881</v>
       </c>
       <c r="C1445" t="n">
-        <v>43708</v>
+        <v>46830</v>
       </c>
     </row>
     <row r="1446">
@@ -16341,7 +16341,7 @@
         <v>2825</v>
       </c>
       <c r="C1446" t="n">
-        <v>35532</v>
+        <v>38070</v>
       </c>
     </row>
     <row r="1447">
@@ -16352,7 +16352,7 @@
         <v>970</v>
       </c>
       <c r="C1447" t="n">
-        <v>43708</v>
+        <v>46830</v>
       </c>
     </row>
     <row r="1448">
@@ -16363,7 +16363,7 @@
         <v>2552</v>
       </c>
       <c r="C1448" t="n">
-        <v>24878</v>
+        <v>26655</v>
       </c>
     </row>
     <row r="1449">
@@ -16374,7 +16374,7 @@
         <v>2562</v>
       </c>
       <c r="C1449" t="n">
-        <v>24878</v>
+        <v>26655</v>
       </c>
     </row>
     <row r="1450">
@@ -16407,7 +16407,7 @@
         <v>2747</v>
       </c>
       <c r="C1452" t="n">
-        <v>44534</v>
+        <v>47715</v>
       </c>
     </row>
     <row r="1453">
@@ -16418,7 +16418,7 @@
         <v>415</v>
       </c>
       <c r="C1453" t="n">
-        <v>159090.96</v>
+        <v>170454.59</v>
       </c>
     </row>
     <row r="1454">
@@ -16462,7 +16462,7 @@
         <v>2544</v>
       </c>
       <c r="C1457" t="n">
-        <v>44534</v>
+        <v>47715</v>
       </c>
     </row>
     <row r="1458">
@@ -16473,7 +16473,7 @@
         <v>816</v>
       </c>
       <c r="C1458" t="n">
-        <v>190909.12</v>
+        <v>204545.48</v>
       </c>
     </row>
     <row r="1459">
@@ -16484,7 +16484,7 @@
         <v>890</v>
       </c>
       <c r="C1459" t="n">
-        <v>572727.28</v>
+        <v>613636.37</v>
       </c>
     </row>
     <row r="1460">
@@ -16495,7 +16495,7 @@
         <v>1298</v>
       </c>
       <c r="C1460" t="n">
-        <v>805000</v>
+        <v>862500</v>
       </c>
     </row>
     <row r="1461">
@@ -16506,7 +16506,7 @@
         <v>1372</v>
       </c>
       <c r="C1461" t="n">
-        <v>190909.12</v>
+        <v>204545.48</v>
       </c>
     </row>
     <row r="1462">
@@ -16517,7 +16517,7 @@
         <v>358</v>
       </c>
       <c r="C1462" t="n">
-        <v>200452</v>
+        <v>214770</v>
       </c>
     </row>
     <row r="1463">
@@ -16528,7 +16528,7 @@
         <v>1653</v>
       </c>
       <c r="C1463" t="n">
-        <v>200452</v>
+        <v>214770</v>
       </c>
     </row>
     <row r="1464">
@@ -16539,7 +16539,7 @@
         <v>675</v>
       </c>
       <c r="C1464" t="n">
-        <v>127260</v>
+        <v>136350</v>
       </c>
     </row>
     <row r="1465">
@@ -16550,7 +16550,7 @@
         <v>2804</v>
       </c>
       <c r="C1465" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1466">
@@ -16561,7 +16561,7 @@
         <v>2714</v>
       </c>
       <c r="C1466" t="n">
-        <v>229082</v>
+        <v>245445</v>
       </c>
     </row>
     <row r="1467">
@@ -16572,7 +16572,7 @@
         <v>2765</v>
       </c>
       <c r="C1467" t="n">
-        <v>57260</v>
+        <v>61350</v>
       </c>
     </row>
     <row r="1468">
@@ -16583,7 +16583,7 @@
         <v>2421</v>
       </c>
       <c r="C1468" t="n">
-        <v>38808</v>
+        <v>41580</v>
       </c>
     </row>
     <row r="1469">
@@ -16594,7 +16594,7 @@
         <v>2359</v>
       </c>
       <c r="C1469" t="n">
-        <v>66388</v>
+        <v>71130</v>
       </c>
     </row>
     <row r="1470">
@@ -16605,7 +16605,7 @@
         <v>2678</v>
       </c>
       <c r="C1470" t="n">
-        <v>62972</v>
+        <v>67470</v>
       </c>
     </row>
     <row r="1471">
@@ -16616,7 +16616,7 @@
         <v>2697</v>
       </c>
       <c r="C1471" t="n">
-        <v>95564</v>
+        <v>102390</v>
       </c>
     </row>
     <row r="1472">
@@ -16649,7 +16649,7 @@
         <v>2142</v>
       </c>
       <c r="C1474" t="n">
-        <v>34440</v>
+        <v>36900</v>
       </c>
     </row>
     <row r="1475">
@@ -16660,7 +16660,7 @@
         <v>2498</v>
       </c>
       <c r="C1475" t="n">
-        <v>35826</v>
+        <v>38385</v>
       </c>
     </row>
     <row r="1476">
@@ -16682,7 +16682,7 @@
         <v>2801</v>
       </c>
       <c r="C1477" t="n">
-        <v>63636.4</v>
+        <v>68181.85000000001</v>
       </c>
     </row>
     <row r="1478">
@@ -16693,7 +16693,7 @@
         <v>2810</v>
       </c>
       <c r="C1478" t="n">
-        <v>101818.24</v>
+        <v>109090.96</v>
       </c>
     </row>
     <row r="1479">
@@ -16737,7 +16737,7 @@
         <v>132</v>
       </c>
       <c r="C1482" t="n">
-        <v>222727.28</v>
+        <v>238636.37</v>
       </c>
     </row>
     <row r="1483">
@@ -16759,7 +16759,7 @@
         <v>580</v>
       </c>
       <c r="C1484" t="n">
-        <v>111363.68</v>
+        <v>119318.22</v>
       </c>
     </row>
     <row r="1485">
@@ -16770,7 +16770,7 @@
         <v>634</v>
       </c>
       <c r="C1485" t="n">
-        <v>318181.84</v>
+        <v>340909.11</v>
       </c>
     </row>
     <row r="1486">
@@ -16792,7 +16792,7 @@
         <v>1277</v>
       </c>
       <c r="C1487" t="n">
-        <v>140000</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="1488">
@@ -16803,7 +16803,7 @@
         <v>767</v>
       </c>
       <c r="C1488" t="n">
-        <v>127260</v>
+        <v>136350</v>
       </c>
     </row>
     <row r="1489">
@@ -16814,7 +16814,7 @@
         <v>2727</v>
       </c>
       <c r="C1489" t="n">
-        <v>25760</v>
+        <v>27600</v>
       </c>
     </row>
     <row r="1490">
@@ -16825,7 +16825,7 @@
         <v>2846</v>
       </c>
       <c r="C1490" t="n">
-        <v>165452</v>
+        <v>177270</v>
       </c>
     </row>
     <row r="1491">
@@ -16836,7 +16836,7 @@
         <v>609</v>
       </c>
       <c r="C1491" t="n">
-        <v>143178</v>
+        <v>153405</v>
       </c>
     </row>
     <row r="1492">
@@ -16847,7 +16847,7 @@
         <v>2726</v>
       </c>
       <c r="C1492" t="n">
-        <v>98630</v>
+        <v>105675</v>
       </c>
     </row>
     <row r="1493">
@@ -16858,7 +16858,7 @@
         <v>2729</v>
       </c>
       <c r="C1493" t="n">
-        <v>57260</v>
+        <v>61350</v>
       </c>
     </row>
     <row r="1494">
@@ -16869,7 +16869,7 @@
         <v>1340</v>
       </c>
       <c r="C1494" t="n">
-        <v>95452</v>
+        <v>102270</v>
       </c>
     </row>
     <row r="1495">
@@ -16880,7 +16880,7 @@
         <v>2830</v>
       </c>
       <c r="C1495" t="n">
-        <v>57260</v>
+        <v>61350</v>
       </c>
     </row>
     <row r="1496">
@@ -16891,7 +16891,7 @@
         <v>2674</v>
       </c>
       <c r="C1496" t="n">
-        <v>165452</v>
+        <v>177270</v>
       </c>
     </row>
     <row r="1497">
@@ -16902,7 +16902,7 @@
         <v>2308</v>
       </c>
       <c r="C1497" t="n">
-        <v>127260</v>
+        <v>136350</v>
       </c>
     </row>
     <row r="1498">
@@ -16913,7 +16913,7 @@
         <v>2190</v>
       </c>
       <c r="C1498" t="n">
-        <v>133630</v>
+        <v>143175</v>
       </c>
     </row>
     <row r="1499">
@@ -16924,7 +16924,7 @@
         <v>2015</v>
       </c>
       <c r="C1499" t="n">
-        <v>235452</v>
+        <v>252270</v>
       </c>
     </row>
     <row r="1500">
@@ -16935,7 +16935,7 @@
         <v>1308</v>
       </c>
       <c r="C1500" t="n">
-        <v>99904</v>
+        <v>107040</v>
       </c>
     </row>
     <row r="1501">
@@ -16946,7 +16946,7 @@
         <v>2118</v>
       </c>
       <c r="C1501" t="n">
-        <v>133742</v>
+        <v>143295</v>
       </c>
     </row>
     <row r="1502">
@@ -16957,7 +16957,7 @@
         <v>2607</v>
       </c>
       <c r="C1502" t="n">
-        <v>31612</v>
+        <v>33870</v>
       </c>
     </row>
     <row r="1503">
@@ -16968,7 +16968,7 @@
         <v>2832</v>
       </c>
       <c r="C1503" t="n">
-        <v>95454.56</v>
+        <v>102272.74</v>
       </c>
     </row>
     <row r="1504">
@@ -16979,7 +16979,7 @@
         <v>2383</v>
       </c>
       <c r="C1504" t="n">
-        <v>84588</v>
+        <v>90630</v>
       </c>
     </row>
     <row r="1505">
@@ -17012,7 +17012,7 @@
         <v>2821</v>
       </c>
       <c r="C1507" t="n">
-        <v>84854</v>
+        <v>90915</v>
       </c>
     </row>
     <row r="1508">
@@ -17034,7 +17034,7 @@
         <v>569</v>
       </c>
       <c r="C1509" t="n">
-        <v>1847636</v>
+        <v>1979610</v>
       </c>
     </row>
     <row r="1510">
@@ -17045,7 +17045,7 @@
         <v>2660</v>
       </c>
       <c r="C1510" t="n">
-        <v>222727.28</v>
+        <v>238636.37</v>
       </c>
     </row>
     <row r="1511">
@@ -17056,7 +17056,7 @@
         <v>1632</v>
       </c>
       <c r="C1511" t="n">
-        <v>165454.56</v>
+        <v>177272.74</v>
       </c>
     </row>
     <row r="1512">
@@ -17067,7 +17067,7 @@
         <v>1756</v>
       </c>
       <c r="C1512" t="n">
-        <v>267260</v>
+        <v>286350</v>
       </c>
     </row>
     <row r="1513">
@@ -17078,7 +17078,7 @@
         <v>58</v>
       </c>
       <c r="C1513" t="n">
-        <v>159600</v>
+        <v>171000</v>
       </c>
     </row>
     <row r="1514">
@@ -17089,7 +17089,7 @@
         <v>40</v>
       </c>
       <c r="C1514" t="n">
-        <v>141960</v>
+        <v>152100</v>
       </c>
     </row>
     <row r="1515">
@@ -17100,7 +17100,7 @@
         <v>559</v>
       </c>
       <c r="C1515" t="n">
-        <v>148904</v>
+        <v>159540</v>
       </c>
     </row>
     <row r="1516">
@@ -17111,7 +17111,7 @@
         <v>2773</v>
       </c>
       <c r="C1516" t="n">
-        <v>51338</v>
+        <v>55005</v>
       </c>
     </row>
     <row r="1517">
@@ -17122,7 +17122,7 @@
         <v>2631</v>
       </c>
       <c r="C1517" t="n">
-        <v>24654</v>
+        <v>26415</v>
       </c>
     </row>
     <row r="1518">
@@ -17133,7 +17133,7 @@
         <v>2085</v>
       </c>
       <c r="C1518" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1519">
@@ -17155,7 +17155,7 @@
         <v>1642</v>
       </c>
       <c r="C1520" t="n">
-        <v>168630</v>
+        <v>180675</v>
       </c>
     </row>
     <row r="1521">
@@ -17166,7 +17166,7 @@
         <v>2621</v>
       </c>
       <c r="C1521" t="n">
-        <v>44534</v>
+        <v>47715</v>
       </c>
     </row>
     <row r="1522">
@@ -17177,7 +17177,7 @@
         <v>2705</v>
       </c>
       <c r="C1522" t="n">
-        <v>127764</v>
+        <v>136890</v>
       </c>
     </row>
     <row r="1523">
@@ -17188,7 +17188,7 @@
         <v>2735</v>
       </c>
       <c r="C1523" t="n">
-        <v>76356</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1524">
@@ -17199,7 +17199,7 @@
         <v>945</v>
       </c>
       <c r="C1524" t="n">
-        <v>223160</v>
+        <v>239100</v>
       </c>
     </row>
     <row r="1525">
@@ -17210,7 +17210,7 @@
         <v>2582</v>
       </c>
       <c r="C1525" t="n">
-        <v>55832</v>
+        <v>59820</v>
       </c>
     </row>
     <row r="1526">
@@ -17221,7 +17221,7 @@
         <v>2584</v>
       </c>
       <c r="C1526" t="n">
-        <v>40600</v>
+        <v>43500</v>
       </c>
     </row>
     <row r="1527">
@@ -17232,7 +17232,7 @@
         <v>2689</v>
       </c>
       <c r="C1527" t="n">
-        <v>40600</v>
+        <v>43500</v>
       </c>
     </row>
     <row r="1528">
@@ -17243,7 +17243,7 @@
         <v>2574</v>
       </c>
       <c r="C1528" t="n">
-        <v>89236</v>
+        <v>95610</v>
       </c>
     </row>
     <row r="1529">
@@ -17254,7 +17254,7 @@
         <v>1834</v>
       </c>
       <c r="C1529" t="n">
-        <v>74900</v>
+        <v>80250</v>
       </c>
     </row>
     <row r="1530">
@@ -17265,7 +17265,7 @@
         <v>2629</v>
       </c>
       <c r="C1530" t="n">
-        <v>43708</v>
+        <v>46830</v>
       </c>
     </row>
     <row r="1531">
@@ -17276,7 +17276,7 @@
         <v>933</v>
       </c>
       <c r="C1531" t="n">
-        <v>51842</v>
+        <v>55545</v>
       </c>
     </row>
     <row r="1532">
@@ -17287,7 +17287,7 @@
         <v>2555</v>
       </c>
       <c r="C1532" t="n">
-        <v>24878</v>
+        <v>26655</v>
       </c>
     </row>
     <row r="1533">
@@ -17298,7 +17298,7 @@
         <v>2558</v>
       </c>
       <c r="C1533" t="n">
-        <v>24878</v>
+        <v>26655</v>
       </c>
     </row>
     <row r="1534">
@@ -17309,7 +17309,7 @@
         <v>2721</v>
       </c>
       <c r="C1534" t="n">
-        <v>51842</v>
+        <v>55545</v>
       </c>
     </row>
     <row r="1535">
@@ -17320,7 +17320,7 @@
         <v>2556</v>
       </c>
       <c r="C1535" t="n">
-        <v>24878</v>
+        <v>26655</v>
       </c>
     </row>
     <row r="1536">
@@ -17331,7 +17331,7 @@
         <v>2826</v>
       </c>
       <c r="C1536" t="n">
-        <v>44534</v>
+        <v>47715</v>
       </c>
     </row>
     <row r="1537">
@@ -17353,7 +17353,7 @@
         <v>2346</v>
       </c>
       <c r="C1538" t="n">
-        <v>44534</v>
+        <v>47715</v>
       </c>
     </row>
     <row r="1539">
@@ -17364,7 +17364,7 @@
         <v>595</v>
       </c>
       <c r="C1539" t="n">
-        <v>159090.96</v>
+        <v>170454.59</v>
       </c>
     </row>
     <row r="1540">
@@ -17375,7 +17375,7 @@
         <v>1278</v>
       </c>
       <c r="C1540" t="n">
-        <v>111363.68</v>
+        <v>119318.22</v>
       </c>
     </row>
     <row r="1541">
@@ -17386,7 +17386,7 @@
         <v>2686</v>
       </c>
       <c r="C1541" t="n">
-        <v>89082</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1542">
@@ -17397,7 +17397,7 @@
         <v>1344</v>
       </c>
       <c r="C1542" t="n">
-        <v>95452</v>
+        <v>102270</v>
       </c>
     </row>
     <row r="1543">
@@ -17408,7 +17408,7 @@
         <v>2566</v>
       </c>
       <c r="C1543" t="n">
-        <v>50904</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1544">
@@ -17419,7 +17419,7 @@
         <v>2684</v>
       </c>
       <c r="C1544" t="n">
-        <v>60452</v>
+        <v>64770</v>
       </c>
     </row>
     <row r="1545">
@@ -17430,7 +17430,7 @@
         <v>2375</v>
       </c>
       <c r="C1545" t="n">
-        <v>210000</v>
+        <v>225000</v>
       </c>
     </row>
     <row r="1546">
@@ -17441,7 +17441,7 @@
         <v>2829</v>
       </c>
       <c r="C1546" t="n">
-        <v>38178</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1547">
@@ -17452,7 +17452,7 @@
         <v>768</v>
       </c>
       <c r="C1547" t="n">
-        <v>89082</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1548">
@@ -17463,7 +17463,7 @@
         <v>772</v>
       </c>
       <c r="C1548" t="n">
-        <v>206808</v>
+        <v>221580</v>
       </c>
     </row>
     <row r="1549">
@@ -17474,7 +17474,7 @@
         <v>2496</v>
       </c>
       <c r="C1549" t="n">
-        <v>127260</v>
+        <v>136350</v>
       </c>
     </row>
     <row r="1550">
@@ -17485,7 +17485,7 @@
         <v>802</v>
       </c>
       <c r="C1550" t="n">
-        <v>47726</v>
+        <v>51135</v>
       </c>
     </row>
     <row r="1551">
@@ -17496,7 +17496,7 @@
         <v>2131</v>
       </c>
       <c r="C1551" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1552">
@@ -17507,7 +17507,7 @@
         <v>1381</v>
       </c>
       <c r="C1552" t="n">
-        <v>190909.12</v>
+        <v>204545.48</v>
       </c>
     </row>
     <row r="1553">
@@ -17518,7 +17518,7 @@
         <v>2847</v>
       </c>
       <c r="C1553" t="n">
-        <v>85904</v>
+        <v>92040</v>
       </c>
     </row>
     <row r="1554">
@@ -17529,7 +17529,7 @@
         <v>1293</v>
       </c>
       <c r="C1554" t="n">
-        <v>245000</v>
+        <v>262500</v>
       </c>
     </row>
     <row r="1555">
@@ -17540,7 +17540,7 @@
         <v>2363</v>
       </c>
       <c r="C1555" t="n">
-        <v>108178</v>
+        <v>115905</v>
       </c>
     </row>
     <row r="1556">
@@ -17551,7 +17551,7 @@
         <v>631</v>
       </c>
       <c r="C1556" t="n">
-        <v>222726</v>
+        <v>238635</v>
       </c>
     </row>
     <row r="1557">
@@ -17562,7 +17562,7 @@
         <v>2791</v>
       </c>
       <c r="C1557" t="n">
-        <v>65338</v>
+        <v>70005</v>
       </c>
     </row>
     <row r="1558">
@@ -17584,7 +17584,7 @@
         <v>2841</v>
       </c>
       <c r="C1559" t="n">
-        <v>31808</v>
+        <v>34080</v>
       </c>
     </row>
     <row r="1560">
@@ -17595,7 +17595,7 @@
         <v>2571</v>
       </c>
       <c r="C1560" t="n">
-        <v>169638</v>
+        <v>181755</v>
       </c>
     </row>
     <row r="1561">
@@ -17661,7 +17661,7 @@
         <v>2273</v>
       </c>
       <c r="C1566" t="n">
-        <v>136822</v>
+        <v>146595</v>
       </c>
     </row>
     <row r="1567">
@@ -17672,7 +17672,7 @@
         <v>2381</v>
       </c>
       <c r="C1567" t="n">
-        <v>51170</v>
+        <v>54825</v>
       </c>
     </row>
     <row r="1568">
@@ -17683,7 +17683,7 @@
         <v>630</v>
       </c>
       <c r="C1568" t="n">
-        <v>52519.07</v>
+        <v>56270.43</v>
       </c>
     </row>
     <row r="1569">
@@ -17705,7 +17705,7 @@
         <v>1983</v>
       </c>
       <c r="C1570" t="n">
-        <v>348880</v>
+        <v>373800</v>
       </c>
     </row>
     <row r="1571">
@@ -17716,7 +17716,7 @@
         <v>1993</v>
       </c>
       <c r="C1571" t="n">
-        <v>236908</v>
+        <v>253830</v>
       </c>
     </row>
     <row r="1572">
@@ -17727,7 +17727,7 @@
         <v>89</v>
       </c>
       <c r="C1572" t="n">
-        <v>222726</v>
+        <v>238635</v>
       </c>
     </row>
     <row r="1573">
@@ -17738,7 +17738,7 @@
         <v>1063</v>
       </c>
       <c r="C1573" t="n">
-        <v>245000</v>
+        <v>262500</v>
       </c>
     </row>
     <row r="1574">
@@ -17749,7 +17749,7 @@
         <v>1116</v>
       </c>
       <c r="C1574" t="n">
-        <v>159082</v>
+        <v>170445</v>
       </c>
     </row>
     <row r="1575">
@@ -17760,7 +17760,7 @@
         <v>941</v>
       </c>
       <c r="C1575" t="n">
-        <v>191478</v>
+        <v>205155</v>
       </c>
     </row>
     <row r="1576">
@@ -17771,7 +17771,7 @@
         <v>2141</v>
       </c>
       <c r="C1576" t="n">
-        <v>20412</v>
+        <v>21870</v>
       </c>
     </row>
     <row r="1577">
@@ -17782,7 +17782,7 @@
         <v>2463</v>
       </c>
       <c r="C1577" t="n">
-        <v>209888</v>
+        <v>224880</v>
       </c>
     </row>
     <row r="1578">
@@ -17793,7 +17793,7 @@
         <v>2707</v>
       </c>
       <c r="C1578" t="n">
-        <v>27482</v>
+        <v>29445</v>
       </c>
     </row>
     <row r="1579">
@@ -17804,7 +17804,7 @@
         <v>2325</v>
       </c>
       <c r="C1579" t="n">
-        <v>73416</v>
+        <v>78660</v>
       </c>
     </row>
     <row r="1580">
@@ -17848,7 +17848,7 @@
         <v>1890</v>
       </c>
       <c r="C1583" t="n">
-        <v>156058</v>
+        <v>167205</v>
       </c>
     </row>
     <row r="1584">
@@ -17859,7 +17859,7 @@
         <v>2639</v>
       </c>
       <c r="C1584" t="n">
-        <v>25494</v>
+        <v>27315</v>
       </c>
     </row>
     <row r="1585">
@@ -17870,7 +17870,7 @@
         <v>2682</v>
       </c>
       <c r="C1585" t="n">
-        <v>89082</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1586">
@@ -17881,7 +17881,7 @@
         <v>2601</v>
       </c>
       <c r="C1586" t="n">
-        <v>175000</v>
+        <v>187500</v>
       </c>
     </row>
     <row r="1587">
@@ -17892,7 +17892,7 @@
         <v>1142</v>
       </c>
       <c r="C1587" t="n">
-        <v>291508</v>
+        <v>312330</v>
       </c>
     </row>
     <row r="1588">
@@ -17936,7 +17936,7 @@
         <v>2082</v>
       </c>
       <c r="C1591" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1592">
@@ -17947,7 +17947,7 @@
         <v>2276</v>
       </c>
       <c r="C1592" t="n">
-        <v>126588</v>
+        <v>135630</v>
       </c>
     </row>
     <row r="1593">
@@ -17958,7 +17958,7 @@
         <v>2786</v>
       </c>
       <c r="C1593" t="n">
-        <v>44534</v>
+        <v>47715</v>
       </c>
     </row>
     <row r="1594">
@@ -17969,7 +17969,7 @@
         <v>2816</v>
       </c>
       <c r="C1594" t="n">
-        <v>82726</v>
+        <v>88635</v>
       </c>
     </row>
     <row r="1595">
@@ -17980,7 +17980,7 @@
         <v>1871</v>
       </c>
       <c r="C1595" t="n">
-        <v>91322</v>
+        <v>97845</v>
       </c>
     </row>
     <row r="1596">
@@ -17991,7 +17991,7 @@
         <v>2345</v>
       </c>
       <c r="C1596" t="n">
-        <v>40600</v>
+        <v>43500</v>
       </c>
     </row>
     <row r="1597">
@@ -18002,7 +18002,7 @@
         <v>2802</v>
       </c>
       <c r="C1597" t="n">
-        <v>45682</v>
+        <v>48945</v>
       </c>
     </row>
     <row r="1598">
@@ -18013,7 +18013,7 @@
         <v>2090</v>
       </c>
       <c r="C1598" t="n">
-        <v>26474</v>
+        <v>28365</v>
       </c>
     </row>
     <row r="1599">
@@ -18024,7 +18024,7 @@
         <v>2647</v>
       </c>
       <c r="C1599" t="n">
-        <v>89250</v>
+        <v>95625</v>
       </c>
     </row>
     <row r="1600">
@@ -18035,7 +18035,7 @@
         <v>2365</v>
       </c>
       <c r="C1600" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1601">
@@ -18046,7 +18046,7 @@
         <v>766</v>
       </c>
       <c r="C1601" t="n">
-        <v>43708</v>
+        <v>46830</v>
       </c>
     </row>
     <row r="1602">
@@ -18057,7 +18057,7 @@
         <v>2702</v>
       </c>
       <c r="C1602" t="n">
-        <v>51842</v>
+        <v>55545</v>
       </c>
     </row>
     <row r="1603">
@@ -18068,7 +18068,7 @@
         <v>20</v>
       </c>
       <c r="C1603" t="n">
-        <v>286363.68</v>
+        <v>306818.22</v>
       </c>
     </row>
     <row r="1604">
@@ -18079,7 +18079,7 @@
         <v>27</v>
       </c>
       <c r="C1604" t="n">
-        <v>95454.56</v>
+        <v>102272.74</v>
       </c>
     </row>
     <row r="1605">
@@ -18090,7 +18090,7 @@
         <v>33</v>
       </c>
       <c r="C1605" t="n">
-        <v>253260</v>
+        <v>271350</v>
       </c>
     </row>
     <row r="1606">
@@ -18112,7 +18112,7 @@
         <v>2561</v>
       </c>
       <c r="C1607" t="n">
-        <v>24878</v>
+        <v>26655</v>
       </c>
     </row>
     <row r="1608">
@@ -18134,7 +18134,7 @@
         <v>2772</v>
       </c>
       <c r="C1609" t="n">
-        <v>38178</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1610">
@@ -18145,7 +18145,7 @@
         <v>2834</v>
       </c>
       <c r="C1610" t="n">
-        <v>23716</v>
+        <v>25410</v>
       </c>
     </row>
     <row r="1611">
@@ -18156,7 +18156,7 @@
         <v>2394</v>
       </c>
       <c r="C1611" t="n">
-        <v>72198</v>
+        <v>77355</v>
       </c>
     </row>
     <row r="1612">
@@ -18167,7 +18167,7 @@
         <v>2567</v>
       </c>
       <c r="C1612" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1613">
@@ -18178,7 +18178,7 @@
         <v>952</v>
       </c>
       <c r="C1613" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1614">
@@ -18189,7 +18189,7 @@
         <v>1539</v>
       </c>
       <c r="C1614" t="n">
-        <v>108178</v>
+        <v>115905</v>
       </c>
     </row>
     <row r="1615">
@@ -18200,7 +18200,7 @@
         <v>793</v>
       </c>
       <c r="C1615" t="n">
-        <v>26474</v>
+        <v>28365</v>
       </c>
     </row>
     <row r="1616">
@@ -18211,7 +18211,7 @@
         <v>794</v>
       </c>
       <c r="C1616" t="n">
-        <v>26474</v>
+        <v>28365</v>
       </c>
     </row>
     <row r="1617">
@@ -18222,7 +18222,7 @@
         <v>2838</v>
       </c>
       <c r="C1617" t="n">
-        <v>38181.84</v>
+        <v>40909.11</v>
       </c>
     </row>
     <row r="1618">
@@ -18233,7 +18233,7 @@
         <v>2223</v>
       </c>
       <c r="C1618" t="n">
-        <v>74522</v>
+        <v>79845</v>
       </c>
     </row>
     <row r="1619">
@@ -18244,7 +18244,7 @@
         <v>2547</v>
       </c>
       <c r="C1619" t="n">
-        <v>21560</v>
+        <v>23100</v>
       </c>
     </row>
     <row r="1620">
@@ -18255,7 +18255,7 @@
         <v>2762</v>
       </c>
       <c r="C1620" t="n">
-        <v>51842</v>
+        <v>55545</v>
       </c>
     </row>
     <row r="1621">
@@ -18266,7 +18266,7 @@
         <v>2550</v>
       </c>
       <c r="C1621" t="n">
-        <v>24878</v>
+        <v>26655</v>
       </c>
     </row>
     <row r="1622">
@@ -18277,7 +18277,7 @@
         <v>2627</v>
       </c>
       <c r="C1622" t="n">
-        <v>24878</v>
+        <v>26655</v>
       </c>
     </row>
     <row r="1623">
@@ -18299,7 +18299,7 @@
         <v>749</v>
       </c>
       <c r="C1624" t="n">
-        <v>51842</v>
+        <v>55545</v>
       </c>
     </row>
     <row r="1625">
@@ -18310,7 +18310,7 @@
         <v>2549</v>
       </c>
       <c r="C1625" t="n">
-        <v>24878</v>
+        <v>26655</v>
       </c>
     </row>
     <row r="1626">
@@ -18321,7 +18321,7 @@
         <v>2649</v>
       </c>
       <c r="C1626" t="n">
-        <v>24878</v>
+        <v>26655</v>
       </c>
     </row>
     <row r="1627">
@@ -18332,7 +18332,7 @@
         <v>2258</v>
       </c>
       <c r="C1627" t="n">
-        <v>50904</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1628">
@@ -18343,7 +18343,7 @@
         <v>2744</v>
       </c>
       <c r="C1628" t="n">
-        <v>38178</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1629">
@@ -18354,7 +18354,7 @@
         <v>452</v>
       </c>
       <c r="C1629" t="n">
-        <v>180082</v>
+        <v>192945</v>
       </c>
     </row>
     <row r="1630">
@@ -18376,7 +18376,7 @@
         <v>2653</v>
       </c>
       <c r="C1631" t="n">
-        <v>38178</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1632">
@@ -18409,7 +18409,7 @@
         <v>2742</v>
       </c>
       <c r="C1634" t="n">
-        <v>12726</v>
+        <v>13635</v>
       </c>
     </row>
     <row r="1635">
@@ -18420,7 +18420,7 @@
         <v>1499</v>
       </c>
       <c r="C1635" t="n">
-        <v>57260</v>
+        <v>61350</v>
       </c>
     </row>
     <row r="1636">
@@ -18431,7 +18431,7 @@
         <v>2261</v>
       </c>
       <c r="C1636" t="n">
-        <v>114534</v>
+        <v>122715</v>
       </c>
     </row>
     <row r="1637">
@@ -18442,7 +18442,7 @@
         <v>1324</v>
       </c>
       <c r="C1637" t="n">
-        <v>178178</v>
+        <v>190905</v>
       </c>
     </row>
     <row r="1638">
@@ -18453,7 +18453,7 @@
         <v>2709</v>
       </c>
       <c r="C1638" t="n">
-        <v>114534</v>
+        <v>122715</v>
       </c>
     </row>
     <row r="1639">
@@ -18464,7 +18464,7 @@
         <v>1137</v>
       </c>
       <c r="C1639" t="n">
-        <v>407260</v>
+        <v>436350</v>
       </c>
     </row>
     <row r="1640">
@@ -18475,7 +18475,7 @@
         <v>2440</v>
       </c>
       <c r="C1640" t="n">
-        <v>50904</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1641">
@@ -18486,7 +18486,7 @@
         <v>429</v>
       </c>
       <c r="C1641" t="n">
-        <v>241808</v>
+        <v>259080</v>
       </c>
     </row>
     <row r="1642">
@@ -18497,7 +18497,7 @@
         <v>2114</v>
       </c>
       <c r="C1642" t="n">
-        <v>108262</v>
+        <v>115995</v>
       </c>
     </row>
     <row r="1643">
@@ -18508,7 +18508,7 @@
         <v>2211</v>
       </c>
       <c r="C1643" t="n">
-        <v>153258</v>
+        <v>164205</v>
       </c>
     </row>
     <row r="1644">
@@ -18519,7 +18519,7 @@
         <v>1108</v>
       </c>
       <c r="C1644" t="n">
-        <v>194964</v>
+        <v>208890</v>
       </c>
     </row>
     <row r="1645">
@@ -18530,7 +18530,7 @@
         <v>2695</v>
       </c>
       <c r="C1645" t="n">
-        <v>30786</v>
+        <v>32985</v>
       </c>
     </row>
     <row r="1646">
@@ -18541,7 +18541,7 @@
         <v>1289</v>
       </c>
       <c r="C1646" t="n">
-        <v>175000</v>
+        <v>187500</v>
       </c>
     </row>
     <row r="1647">
@@ -18552,7 +18552,7 @@
         <v>2789</v>
       </c>
       <c r="C1647" t="n">
-        <v>114545.52</v>
+        <v>122727.33</v>
       </c>
     </row>
     <row r="1648">
@@ -18563,7 +18563,7 @@
         <v>2197</v>
       </c>
       <c r="C1648" t="n">
-        <v>136818.24</v>
+        <v>146590.96</v>
       </c>
     </row>
     <row r="1649">
@@ -18574,7 +18574,7 @@
         <v>947</v>
       </c>
       <c r="C1649" t="n">
-        <v>282212</v>
+        <v>302370</v>
       </c>
     </row>
     <row r="1650">
@@ -18585,7 +18585,7 @@
         <v>2279</v>
       </c>
       <c r="C1650" t="n">
-        <v>155862</v>
+        <v>166995</v>
       </c>
     </row>
     <row r="1651">
@@ -18596,7 +18596,7 @@
         <v>1465</v>
       </c>
       <c r="C1651" t="n">
-        <v>245000</v>
+        <v>262500</v>
       </c>
     </row>
     <row r="1652">
@@ -18607,7 +18607,7 @@
         <v>2651</v>
       </c>
       <c r="C1652" t="n">
-        <v>108178</v>
+        <v>115905</v>
       </c>
     </row>
     <row r="1653">
@@ -18618,7 +18618,7 @@
         <v>42</v>
       </c>
       <c r="C1653" t="n">
-        <v>1212904</v>
+        <v>1299540</v>
       </c>
     </row>
     <row r="1654">
@@ -18629,7 +18629,7 @@
         <v>949</v>
       </c>
       <c r="C1654" t="n">
-        <v>63294</v>
+        <v>67815</v>
       </c>
     </row>
     <row r="1655">
@@ -18640,7 +18640,7 @@
         <v>2606</v>
       </c>
       <c r="C1655" t="n">
-        <v>163380</v>
+        <v>175050</v>
       </c>
     </row>
     <row r="1656">
@@ -18651,7 +18651,7 @@
         <v>2249</v>
       </c>
       <c r="C1656" t="n">
-        <v>138810</v>
+        <v>148725</v>
       </c>
     </row>
     <row r="1657">
@@ -18695,7 +18695,7 @@
         <v>2045</v>
       </c>
       <c r="C1660" t="n">
-        <v>202664</v>
+        <v>217140</v>
       </c>
     </row>
     <row r="1661">
@@ -18706,7 +18706,7 @@
         <v>2663</v>
       </c>
       <c r="C1661" t="n">
-        <v>175000</v>
+        <v>187500</v>
       </c>
     </row>
     <row r="1662">
@@ -18728,7 +18728,7 @@
         <v>2854</v>
       </c>
       <c r="C1663" t="n">
-        <v>25452</v>
+        <v>27270</v>
       </c>
     </row>
     <row r="1664">
@@ -18750,7 +18750,7 @@
         <v>2341</v>
       </c>
       <c r="C1665" t="n">
-        <v>111300</v>
+        <v>119250</v>
       </c>
     </row>
     <row r="1666">
@@ -18761,7 +18761,7 @@
         <v>2637</v>
       </c>
       <c r="C1666" t="n">
-        <v>40600</v>
+        <v>43500</v>
       </c>
     </row>
     <row r="1667">
@@ -18772,7 +18772,7 @@
         <v>2492</v>
       </c>
       <c r="C1667" t="n">
-        <v>63742</v>
+        <v>68295</v>
       </c>
     </row>
     <row r="1668">
@@ -18783,7 +18783,7 @@
         <v>2548</v>
       </c>
       <c r="C1668" t="n">
-        <v>24878</v>
+        <v>26655</v>
       </c>
     </row>
     <row r="1669">
@@ -18794,7 +18794,7 @@
         <v>351</v>
       </c>
       <c r="C1669" t="n">
-        <v>135534</v>
+        <v>145215</v>
       </c>
     </row>
     <row r="1670">
@@ -18827,7 +18827,7 @@
         <v>2757</v>
       </c>
       <c r="C1672" t="n">
-        <v>50904</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1673">
@@ -18838,7 +18838,7 @@
         <v>2815</v>
       </c>
       <c r="C1673" t="n">
-        <v>38178</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1674">
@@ -18849,7 +18849,7 @@
         <v>2323</v>
       </c>
       <c r="C1674" t="n">
-        <v>43708</v>
+        <v>46830</v>
       </c>
     </row>
     <row r="1675">
@@ -18860,7 +18860,7 @@
         <v>2310</v>
       </c>
       <c r="C1675" t="n">
-        <v>43708</v>
+        <v>46830</v>
       </c>
     </row>
     <row r="1676">
@@ -18871,7 +18871,7 @@
         <v>2145</v>
       </c>
       <c r="C1676" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1677">
@@ -18882,7 +18882,7 @@
         <v>2501</v>
       </c>
       <c r="C1677" t="n">
-        <v>51842</v>
+        <v>55545</v>
       </c>
     </row>
     <row r="1678">
@@ -18893,7 +18893,7 @@
         <v>2546</v>
       </c>
       <c r="C1678" t="n">
-        <v>24878</v>
+        <v>26655</v>
       </c>
     </row>
     <row r="1679">
@@ -18904,7 +18904,7 @@
         <v>716</v>
       </c>
       <c r="C1679" t="n">
-        <v>81564</v>
+        <v>87390</v>
       </c>
     </row>
     <row r="1680">
@@ -18915,7 +18915,7 @@
         <v>2758</v>
       </c>
       <c r="C1680" t="n">
-        <v>38178</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1681">
@@ -18926,7 +18926,7 @@
         <v>400</v>
       </c>
       <c r="C1681" t="n">
-        <v>114534</v>
+        <v>122715</v>
       </c>
     </row>
     <row r="1682">
@@ -18937,7 +18937,7 @@
         <v>6</v>
       </c>
       <c r="C1682" t="n">
-        <v>31818.24</v>
+        <v>34090.96</v>
       </c>
     </row>
     <row r="1683">
@@ -18970,7 +18970,7 @@
         <v>1259</v>
       </c>
       <c r="C1685" t="n">
-        <v>70000</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="1686">
@@ -18981,7 +18981,7 @@
         <v>571</v>
       </c>
       <c r="C1686" t="n">
-        <v>658636.4</v>
+        <v>705681.85</v>
       </c>
     </row>
     <row r="1687">
@@ -18992,7 +18992,7 @@
         <v>703</v>
       </c>
       <c r="C1687" t="n">
-        <v>159082</v>
+        <v>170445</v>
       </c>
     </row>
     <row r="1688">
@@ -19014,7 +19014,7 @@
         <v>2833</v>
       </c>
       <c r="C1689" t="n">
-        <v>50904</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1690">
@@ -19025,7 +19025,7 @@
         <v>1007</v>
       </c>
       <c r="C1690" t="n">
-        <v>127272.8</v>
+        <v>136363.7</v>
       </c>
     </row>
     <row r="1691">
@@ -19036,7 +19036,7 @@
         <v>2687</v>
       </c>
       <c r="C1691" t="n">
-        <v>50904</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1692">
@@ -19047,7 +19047,7 @@
         <v>2824</v>
       </c>
       <c r="C1692" t="n">
-        <v>71848</v>
+        <v>76980</v>
       </c>
     </row>
     <row r="1693">
@@ -19058,7 +19058,7 @@
         <v>2730</v>
       </c>
       <c r="C1693" t="n">
-        <v>57260</v>
+        <v>61350</v>
       </c>
     </row>
     <row r="1694">
@@ -19069,7 +19069,7 @@
         <v>2718</v>
       </c>
       <c r="C1694" t="n">
-        <v>82726</v>
+        <v>88635</v>
       </c>
     </row>
     <row r="1695">
@@ -19080,7 +19080,7 @@
         <v>2750</v>
       </c>
       <c r="C1695" t="n">
-        <v>19082</v>
+        <v>20445</v>
       </c>
     </row>
     <row r="1696">
@@ -19091,7 +19091,7 @@
         <v>854</v>
       </c>
       <c r="C1696" t="n">
-        <v>89082</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1697">
@@ -19102,7 +19102,7 @@
         <v>2794</v>
       </c>
       <c r="C1697" t="n">
-        <v>76356</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1698">
@@ -19113,7 +19113,7 @@
         <v>1374</v>
       </c>
       <c r="C1698" t="n">
-        <v>127260</v>
+        <v>136350</v>
       </c>
     </row>
     <row r="1699">
@@ -19124,7 +19124,7 @@
         <v>2488</v>
       </c>
       <c r="C1699" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1700">
@@ -19135,7 +19135,7 @@
         <v>363</v>
       </c>
       <c r="C1700" t="n">
-        <v>190904</v>
+        <v>204540</v>
       </c>
     </row>
     <row r="1701">
@@ -19146,7 +19146,7 @@
         <v>2655</v>
       </c>
       <c r="C1701" t="n">
-        <v>70000</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="1702">
@@ -19157,7 +19157,7 @@
         <v>1873</v>
       </c>
       <c r="C1702" t="n">
-        <v>203630</v>
+        <v>218175</v>
       </c>
     </row>
     <row r="1703">
@@ -19168,7 +19168,7 @@
         <v>2635</v>
       </c>
       <c r="C1703" t="n">
-        <v>82726</v>
+        <v>88635</v>
       </c>
     </row>
     <row r="1704">
@@ -19179,7 +19179,7 @@
         <v>1658</v>
       </c>
       <c r="C1704" t="n">
-        <v>97356</v>
+        <v>104310</v>
       </c>
     </row>
     <row r="1705">
@@ -19190,7 +19190,7 @@
         <v>2069</v>
       </c>
       <c r="C1705" t="n">
-        <v>127272.8</v>
+        <v>136363.7</v>
       </c>
     </row>
     <row r="1706">
@@ -19201,7 +19201,7 @@
         <v>2081</v>
       </c>
       <c r="C1706" t="n">
-        <v>95452</v>
+        <v>102270</v>
       </c>
     </row>
     <row r="1707">
@@ -19212,7 +19212,7 @@
         <v>2124</v>
       </c>
       <c r="C1707" t="n">
-        <v>222726</v>
+        <v>238635</v>
       </c>
     </row>
     <row r="1708">
@@ -19223,7 +19223,7 @@
         <v>636</v>
       </c>
       <c r="C1708" t="n">
-        <v>159082</v>
+        <v>170445</v>
       </c>
     </row>
     <row r="1709">
@@ -19234,7 +19234,7 @@
         <v>2803</v>
       </c>
       <c r="C1709" t="n">
-        <v>76356</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1710">
@@ -19245,7 +19245,7 @@
         <v>2163</v>
       </c>
       <c r="C1710" t="n">
-        <v>114534</v>
+        <v>122715</v>
       </c>
     </row>
     <row r="1711">
@@ -19256,7 +19256,7 @@
         <v>1466</v>
       </c>
       <c r="C1711" t="n">
-        <v>257726</v>
+        <v>276135</v>
       </c>
     </row>
     <row r="1712">
@@ -19267,7 +19267,7 @@
         <v>2133</v>
       </c>
       <c r="C1712" t="n">
-        <v>222727.28</v>
+        <v>238636.37</v>
       </c>
     </row>
     <row r="1713">
@@ -19278,7 +19278,7 @@
         <v>2431</v>
       </c>
       <c r="C1713" t="n">
-        <v>95452</v>
+        <v>102270</v>
       </c>
     </row>
     <row r="1714">
@@ -19289,7 +19289,7 @@
         <v>535</v>
       </c>
       <c r="C1714" t="n">
-        <v>226660</v>
+        <v>242850</v>
       </c>
     </row>
     <row r="1715">
@@ -19300,7 +19300,7 @@
         <v>2790</v>
       </c>
       <c r="C1715" t="n">
-        <v>40194</v>
+        <v>43065</v>
       </c>
     </row>
     <row r="1716">
@@ -19311,7 +19311,7 @@
         <v>2442</v>
       </c>
       <c r="C1716" t="n">
-        <v>164808</v>
+        <v>176580</v>
       </c>
     </row>
     <row r="1717">
@@ -19322,7 +19322,7 @@
         <v>2376</v>
       </c>
       <c r="C1717" t="n">
-        <v>700000</v>
+        <v>750000</v>
       </c>
     </row>
     <row r="1718">
@@ -19333,7 +19333,7 @@
         <v>2768</v>
       </c>
       <c r="C1718" t="n">
-        <v>192598</v>
+        <v>206355</v>
       </c>
     </row>
     <row r="1719">
@@ -19344,7 +19344,7 @@
         <v>2491</v>
       </c>
       <c r="C1719" t="n">
-        <v>154546</v>
+        <v>165585</v>
       </c>
     </row>
     <row r="1720">
@@ -19355,7 +19355,7 @@
         <v>2799</v>
       </c>
       <c r="C1720" t="n">
-        <v>69566</v>
+        <v>74535</v>
       </c>
     </row>
     <row r="1721">
@@ -19388,7 +19388,7 @@
         <v>1317</v>
       </c>
       <c r="C1723" t="n">
-        <v>200454.56</v>
+        <v>214772.74</v>
       </c>
     </row>
     <row r="1724">
@@ -19399,7 +19399,7 @@
         <v>2822</v>
       </c>
       <c r="C1724" t="n">
-        <v>101818.24</v>
+        <v>109090.96</v>
       </c>
     </row>
     <row r="1725">
@@ -19410,7 +19410,7 @@
         <v>1117</v>
       </c>
       <c r="C1725" t="n">
-        <v>254618</v>
+        <v>272805</v>
       </c>
     </row>
     <row r="1726">
@@ -19421,7 +19421,7 @@
         <v>1299</v>
       </c>
       <c r="C1726" t="n">
-        <v>335706</v>
+        <v>359685</v>
       </c>
     </row>
     <row r="1727">
@@ -19432,7 +19432,7 @@
         <v>477</v>
       </c>
       <c r="C1727" t="n">
-        <v>138348</v>
+        <v>148230</v>
       </c>
     </row>
     <row r="1728">
@@ -19443,7 +19443,7 @@
         <v>530</v>
       </c>
       <c r="C1728" t="n">
-        <v>190904</v>
+        <v>204540</v>
       </c>
     </row>
     <row r="1729">
@@ -19454,7 +19454,7 @@
         <v>953</v>
       </c>
       <c r="C1729" t="n">
-        <v>439082</v>
+        <v>470445</v>
       </c>
     </row>
     <row r="1730">
@@ -19465,7 +19465,7 @@
         <v>610</v>
       </c>
       <c r="C1730" t="n">
-        <v>522956</v>
+        <v>560310</v>
       </c>
     </row>
     <row r="1731">
@@ -19476,7 +19476,7 @@
         <v>2792</v>
       </c>
       <c r="C1731" t="n">
-        <v>131334</v>
+        <v>140715</v>
       </c>
     </row>
     <row r="1732">
@@ -19553,7 +19553,7 @@
         <v>1075</v>
       </c>
       <c r="C1738" t="n">
-        <v>292082</v>
+        <v>312945</v>
       </c>
     </row>
     <row r="1739">
@@ -19564,7 +19564,7 @@
         <v>131</v>
       </c>
       <c r="C1739" t="n">
-        <v>264726</v>
+        <v>283635</v>
       </c>
     </row>
     <row r="1740">
@@ -19575,7 +19575,7 @@
         <v>2667</v>
       </c>
       <c r="C1740" t="n">
-        <v>29078</v>
+        <v>31155</v>
       </c>
     </row>
     <row r="1741">
@@ -19586,7 +19586,7 @@
         <v>2330</v>
       </c>
       <c r="C1741" t="n">
-        <v>56602</v>
+        <v>60645</v>
       </c>
     </row>
     <row r="1742">
@@ -19608,7 +19608,7 @@
         <v>2577</v>
       </c>
       <c r="C1743" t="n">
-        <v>56742</v>
+        <v>60795</v>
       </c>
     </row>
     <row r="1744">
@@ -19619,7 +19619,7 @@
         <v>2510</v>
       </c>
       <c r="C1744" t="n">
-        <v>402976</v>
+        <v>431760</v>
       </c>
     </row>
     <row r="1745">
@@ -19641,7 +19641,7 @@
         <v>2850</v>
       </c>
       <c r="C1746" t="n">
-        <v>38178</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1747">
@@ -19663,7 +19663,7 @@
         <v>2745</v>
       </c>
       <c r="C1748" t="n">
-        <v>70000</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="1749">
@@ -19674,7 +19674,7 @@
         <v>2817</v>
       </c>
       <c r="C1749" t="n">
-        <v>38178</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1750">
@@ -19685,7 +19685,7 @@
         <v>2784</v>
       </c>
       <c r="C1750" t="n">
-        <v>26474</v>
+        <v>28365</v>
       </c>
     </row>
     <row r="1751">
@@ -19696,7 +19696,7 @@
         <v>626</v>
       </c>
       <c r="C1751" t="n">
-        <v>1099518</v>
+        <v>1178055</v>
       </c>
     </row>
     <row r="1752">
@@ -19707,7 +19707,7 @@
         <v>925</v>
       </c>
       <c r="C1752" t="n">
-        <v>50764</v>
+        <v>54390</v>
       </c>
     </row>
     <row r="1753">
@@ -19718,7 +19718,7 @@
         <v>2586</v>
       </c>
       <c r="C1753" t="n">
-        <v>26474</v>
+        <v>28365</v>
       </c>
     </row>
     <row r="1754">
@@ -19729,7 +19729,7 @@
         <v>966</v>
       </c>
       <c r="C1754" t="n">
-        <v>51842</v>
+        <v>55545</v>
       </c>
     </row>
     <row r="1755">
@@ -19740,7 +19740,7 @@
         <v>2557</v>
       </c>
       <c r="C1755" t="n">
-        <v>24878</v>
+        <v>26655</v>
       </c>
     </row>
     <row r="1756">
@@ -19751,7 +19751,7 @@
         <v>14</v>
       </c>
       <c r="C1756" t="n">
-        <v>286356</v>
+        <v>306810</v>
       </c>
     </row>
     <row r="1757">
@@ -19762,7 +19762,7 @@
         <v>2798</v>
       </c>
       <c r="C1757" t="n">
-        <v>38178</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1758">
@@ -19784,7 +19784,7 @@
         <v>522</v>
       </c>
       <c r="C1759" t="n">
-        <v>127272.8</v>
+        <v>136363.7</v>
       </c>
     </row>
     <row r="1760">
@@ -19806,7 +19806,7 @@
         <v>2819</v>
       </c>
       <c r="C1761" t="n">
-        <v>38178</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1762">
@@ -19817,7 +19817,7 @@
         <v>2266</v>
       </c>
       <c r="C1762" t="n">
-        <v>50904</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1763">
@@ -19850,7 +19850,7 @@
         <v>2795</v>
       </c>
       <c r="C1765" t="n">
-        <v>38178</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1766">
@@ -19861,7 +19861,7 @@
         <v>2722</v>
       </c>
       <c r="C1766" t="n">
-        <v>12726</v>
+        <v>13635</v>
       </c>
     </row>
     <row r="1767">
@@ -19872,7 +19872,7 @@
         <v>951</v>
       </c>
       <c r="C1767" t="n">
-        <v>73178</v>
+        <v>78405</v>
       </c>
     </row>
     <row r="1768">
@@ -19883,7 +19883,7 @@
         <v>1020</v>
       </c>
       <c r="C1768" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1769">
@@ -19894,7 +19894,7 @@
         <v>1853</v>
       </c>
       <c r="C1769" t="n">
-        <v>76356</v>
+        <v>81810</v>
       </c>
     </row>
     <row r="1770">
@@ -19905,7 +19905,7 @@
         <v>1327</v>
       </c>
       <c r="C1770" t="n">
-        <v>44534</v>
+        <v>47715</v>
       </c>
     </row>
     <row r="1771">
@@ -19916,7 +19916,7 @@
         <v>2842</v>
       </c>
       <c r="C1771" t="n">
-        <v>114534</v>
+        <v>122715</v>
       </c>
     </row>
     <row r="1772">
@@ -19927,7 +19927,7 @@
         <v>2831</v>
       </c>
       <c r="C1772" t="n">
-        <v>38178</v>
+        <v>40905</v>
       </c>
     </row>
     <row r="1773">
@@ -19938,7 +19938,7 @@
         <v>818</v>
       </c>
       <c r="C1773" t="n">
-        <v>254534</v>
+        <v>272715</v>
       </c>
     </row>
     <row r="1774">
@@ -19949,7 +19949,7 @@
         <v>1501</v>
       </c>
       <c r="C1774" t="n">
-        <v>63630</v>
+        <v>68175</v>
       </c>
     </row>
     <row r="1775">
@@ -19960,7 +19960,7 @@
         <v>1869</v>
       </c>
       <c r="C1775" t="n">
-        <v>155260</v>
+        <v>166350</v>
       </c>
     </row>
     <row r="1776">
@@ -19971,7 +19971,7 @@
         <v>1996</v>
       </c>
       <c r="C1776" t="n">
-        <v>159090.96</v>
+        <v>170454.59</v>
       </c>
     </row>
     <row r="1777">
@@ -19982,7 +19982,7 @@
         <v>2462</v>
       </c>
       <c r="C1777" t="n">
-        <v>36040.52</v>
+        <v>38614.83</v>
       </c>
     </row>
     <row r="1778">
@@ -19993,7 +19993,7 @@
         <v>2696</v>
       </c>
       <c r="C1778" t="n">
-        <v>136472</v>
+        <v>146220</v>
       </c>
     </row>
     <row r="1779">
@@ -20004,7 +20004,7 @@
         <v>2698</v>
       </c>
       <c r="C1779" t="n">
-        <v>69944</v>
+        <v>74940</v>
       </c>
     </row>
     <row r="1780">
@@ -20026,7 +20026,7 @@
         <v>2828</v>
       </c>
       <c r="C1781" t="n">
-        <v>38181.84</v>
+        <v>40909.11</v>
       </c>
     </row>
     <row r="1782">
@@ -20037,7 +20037,7 @@
         <v>2843</v>
       </c>
       <c r="C1782" t="n">
-        <v>44534</v>
+        <v>47715</v>
       </c>
     </row>
     <row r="1783">
@@ -20048,7 +20048,7 @@
         <v>619</v>
       </c>
       <c r="C1783" t="n">
-        <v>199500</v>
+        <v>213750</v>
       </c>
     </row>
     <row r="1784">
@@ -20059,7 +20059,7 @@
         <v>1478</v>
       </c>
       <c r="C1784" t="n">
-        <v>349132</v>
+        <v>374070</v>
       </c>
     </row>
     <row r="1785">
@@ -20070,7 +20070,7 @@
         <v>2026</v>
       </c>
       <c r="C1785" t="n">
-        <v>154252</v>
+        <v>165270</v>
       </c>
     </row>
     <row r="1786">
@@ -20081,7 +20081,7 @@
         <v>663</v>
       </c>
       <c r="C1786" t="n">
-        <v>164808</v>
+        <v>176580</v>
       </c>
     </row>
     <row r="1787">
@@ -20092,7 +20092,7 @@
         <v>285</v>
       </c>
       <c r="C1787" t="n">
-        <v>349132</v>
+        <v>374070</v>
       </c>
     </row>
     <row r="1788">
@@ -20103,7 +20103,7 @@
         <v>424</v>
       </c>
       <c r="C1788" t="n">
-        <v>149618</v>
+        <v>160305</v>
       </c>
     </row>
     <row r="1789">
@@ -20114,7 +20114,7 @@
         <v>451</v>
       </c>
       <c r="C1789" t="n">
-        <v>154630</v>
+        <v>165675</v>
       </c>
     </row>
     <row r="1790">
@@ -20125,7 +20125,7 @@
         <v>629</v>
       </c>
       <c r="C1790" t="n">
-        <v>288904</v>
+        <v>309540</v>
       </c>
     </row>
     <row r="1791">
@@ -20136,7 +20136,7 @@
         <v>2657</v>
       </c>
       <c r="C1791" t="n">
-        <v>50386</v>
+        <v>53985</v>
       </c>
     </row>
     <row r="1792">
@@ -20147,7 +20147,7 @@
         <v>1254</v>
       </c>
       <c r="C1792" t="n">
-        <v>123578</v>
+        <v>132405</v>
       </c>
     </row>
     <row r="1793">
@@ -20158,7 +20158,7 @@
         <v>2402</v>
       </c>
       <c r="C1793" t="n">
-        <v>310828</v>
+        <v>333030</v>
       </c>
     </row>
     <row r="1794">
@@ -20169,7 +20169,7 @@
         <v>2413</v>
       </c>
       <c r="C1794" t="n">
-        <v>87710</v>
+        <v>93975</v>
       </c>
     </row>
     <row r="1795">
@@ -20180,7 +20180,7 @@
         <v>1450</v>
       </c>
       <c r="C1795" t="n">
-        <v>227178</v>
+        <v>243405</v>
       </c>
     </row>
     <row r="1796">
@@ -20202,7 +20202,7 @@
         <v>2671</v>
       </c>
       <c r="C1797" t="n">
-        <v>50904</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1798">
@@ -20213,7 +20213,7 @@
         <v>2568</v>
       </c>
       <c r="C1798" t="n">
-        <v>102102</v>
+        <v>109395</v>
       </c>
     </row>
     <row r="1799">
@@ -20224,7 +20224,7 @@
         <v>2146</v>
       </c>
       <c r="C1799" t="n">
-        <v>123634</v>
+        <v>132465</v>
       </c>
     </row>
     <row r="1800">
@@ -20235,7 +20235,7 @@
         <v>2753</v>
       </c>
       <c r="C1800" t="n">
-        <v>47726</v>
+        <v>51135</v>
       </c>
     </row>
     <row r="1801">
@@ -20246,7 +20246,7 @@
         <v>744</v>
       </c>
       <c r="C1801" t="n">
-        <v>26474</v>
+        <v>28365</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:02:13
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -15560,7 +15560,7 @@
         <v>2853</v>
       </c>
       <c r="C1375" t="n">
-        <v>55545</v>
+        <v>59248</v>
       </c>
     </row>
     <row r="1376">
@@ -15571,7 +15571,7 @@
         <v>2245</v>
       </c>
       <c r="C1376" t="n">
-        <v>150960</v>
+        <v>161024</v>
       </c>
     </row>
     <row r="1377">
@@ -15582,7 +15582,7 @@
         <v>2251</v>
       </c>
       <c r="C1377" t="n">
-        <v>136350</v>
+        <v>145440</v>
       </c>
     </row>
     <row r="1378">
@@ -15593,7 +15593,7 @@
         <v>664</v>
       </c>
       <c r="C1378" t="n">
-        <v>178635</v>
+        <v>190544</v>
       </c>
     </row>
     <row r="1379">
@@ -15604,7 +15604,7 @@
         <v>2472</v>
       </c>
       <c r="C1379" t="n">
-        <v>36090</v>
+        <v>38496</v>
       </c>
     </row>
     <row r="1380">
@@ -15615,7 +15615,7 @@
         <v>1456</v>
       </c>
       <c r="C1380" t="n">
-        <v>544080</v>
+        <v>580352</v>
       </c>
     </row>
     <row r="1381">
@@ -15626,7 +15626,7 @@
         <v>1585</v>
       </c>
       <c r="C1381" t="n">
-        <v>123405</v>
+        <v>131632</v>
       </c>
     </row>
     <row r="1382">
@@ -15670,7 +15670,7 @@
         <v>1907</v>
       </c>
       <c r="C1385" t="n">
-        <v>375360</v>
+        <v>400384</v>
       </c>
     </row>
     <row r="1386">
@@ -15703,7 +15703,7 @@
         <v>2659</v>
       </c>
       <c r="C1388" t="n">
-        <v>83865</v>
+        <v>89456</v>
       </c>
     </row>
     <row r="1389">
@@ -15714,7 +15714,7 @@
         <v>2583</v>
       </c>
       <c r="C1389" t="n">
-        <v>28365</v>
+        <v>30256</v>
       </c>
     </row>
     <row r="1390">
@@ -15725,7 +15725,7 @@
         <v>2692</v>
       </c>
       <c r="C1390" t="n">
-        <v>47727.33</v>
+        <v>50909.14</v>
       </c>
     </row>
     <row r="1391">
@@ -15736,7 +15736,7 @@
         <v>2691</v>
       </c>
       <c r="C1391" t="n">
-        <v>83307.33</v>
+        <v>88861.14</v>
       </c>
     </row>
     <row r="1392">
@@ -15747,7 +15747,7 @@
         <v>931</v>
       </c>
       <c r="C1392" t="n">
-        <v>65265</v>
+        <v>69616</v>
       </c>
     </row>
     <row r="1393">
@@ -15758,7 +15758,7 @@
         <v>2785</v>
       </c>
       <c r="C1393" t="n">
-        <v>28365</v>
+        <v>30256</v>
       </c>
     </row>
     <row r="1394">
@@ -15769,7 +15769,7 @@
         <v>2411</v>
       </c>
       <c r="C1394" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1395">
@@ -15780,7 +15780,7 @@
         <v>2716</v>
       </c>
       <c r="C1395" t="n">
-        <v>59820</v>
+        <v>63808</v>
       </c>
     </row>
     <row r="1396">
@@ -15791,7 +15791,7 @@
         <v>2809</v>
       </c>
       <c r="C1396" t="n">
-        <v>46830</v>
+        <v>49952</v>
       </c>
     </row>
     <row r="1397">
@@ -15802,7 +15802,7 @@
         <v>104</v>
       </c>
       <c r="C1397" t="n">
-        <v>204545.48</v>
+        <v>218181.84</v>
       </c>
     </row>
     <row r="1398">
@@ -15835,7 +15835,7 @@
         <v>781</v>
       </c>
       <c r="C1400" t="n">
-        <v>88635</v>
+        <v>94544</v>
       </c>
     </row>
     <row r="1401">
@@ -15857,7 +15857,7 @@
         <v>2494</v>
       </c>
       <c r="C1402" t="n">
-        <v>102270</v>
+        <v>109088</v>
       </c>
     </row>
     <row r="1403">
@@ -15868,7 +15868,7 @@
         <v>2652</v>
       </c>
       <c r="C1403" t="n">
-        <v>95445</v>
+        <v>101808</v>
       </c>
     </row>
     <row r="1404">
@@ -15879,7 +15879,7 @@
         <v>1384</v>
       </c>
       <c r="C1404" t="n">
-        <v>238636.37</v>
+        <v>254545.46</v>
       </c>
     </row>
     <row r="1405">
@@ -15890,7 +15890,7 @@
         <v>360</v>
       </c>
       <c r="C1405" t="n">
-        <v>340905</v>
+        <v>363632</v>
       </c>
     </row>
     <row r="1406">
@@ -15901,7 +15901,7 @@
         <v>2767</v>
       </c>
       <c r="C1406" t="n">
-        <v>129540</v>
+        <v>138176</v>
       </c>
     </row>
     <row r="1407">
@@ -15912,7 +15912,7 @@
         <v>2178</v>
       </c>
       <c r="C1407" t="n">
-        <v>186810</v>
+        <v>199264</v>
       </c>
     </row>
     <row r="1408">
@@ -15923,7 +15923,7 @@
         <v>2107</v>
       </c>
       <c r="C1408" t="n">
-        <v>204525</v>
+        <v>218160</v>
       </c>
     </row>
     <row r="1409">
@@ -15934,7 +15934,7 @@
         <v>2711</v>
       </c>
       <c r="C1409" t="n">
-        <v>59025</v>
+        <v>62960</v>
       </c>
     </row>
     <row r="1410">
@@ -15945,7 +15945,7 @@
         <v>2845</v>
       </c>
       <c r="C1410" t="n">
-        <v>34080</v>
+        <v>36352</v>
       </c>
     </row>
     <row r="1411">
@@ -15989,7 +15989,7 @@
         <v>1102</v>
       </c>
       <c r="C1414" t="n">
-        <v>160305</v>
+        <v>170992</v>
       </c>
     </row>
     <row r="1415">
@@ -16000,7 +16000,7 @@
         <v>353</v>
       </c>
       <c r="C1415" t="n">
-        <v>199455</v>
+        <v>212752</v>
       </c>
     </row>
     <row r="1416">
@@ -16011,7 +16011,7 @@
         <v>2250</v>
       </c>
       <c r="C1416" t="n">
-        <v>231810</v>
+        <v>247264</v>
       </c>
     </row>
     <row r="1417">
@@ -16022,7 +16022,7 @@
         <v>1800</v>
       </c>
       <c r="C1417" t="n">
-        <v>19335</v>
+        <v>20624</v>
       </c>
     </row>
     <row r="1418">
@@ -16033,7 +16033,7 @@
         <v>2362</v>
       </c>
       <c r="C1418" t="n">
-        <v>51135</v>
+        <v>54544</v>
       </c>
     </row>
     <row r="1419">
@@ -16044,7 +16044,7 @@
         <v>2449</v>
       </c>
       <c r="C1419" t="n">
-        <v>64770</v>
+        <v>69088</v>
       </c>
     </row>
     <row r="1420">
@@ -16055,7 +16055,7 @@
         <v>2844</v>
       </c>
       <c r="C1420" t="n">
-        <v>34080</v>
+        <v>36352</v>
       </c>
     </row>
     <row r="1421">
@@ -16066,7 +16066,7 @@
         <v>2507</v>
       </c>
       <c r="C1421" t="n">
-        <v>60900</v>
+        <v>64960</v>
       </c>
     </row>
     <row r="1422">
@@ -16077,7 +16077,7 @@
         <v>1906</v>
       </c>
       <c r="C1422" t="n">
-        <v>74025</v>
+        <v>78960</v>
       </c>
     </row>
     <row r="1423">
@@ -16099,7 +16099,7 @@
         <v>525</v>
       </c>
       <c r="C1424" t="n">
-        <v>160227.33</v>
+        <v>170909.14</v>
       </c>
     </row>
     <row r="1425">
@@ -16110,7 +16110,7 @@
         <v>1261</v>
       </c>
       <c r="C1425" t="n">
-        <v>48409.11</v>
+        <v>51636.38</v>
       </c>
     </row>
     <row r="1426">
@@ -16121,7 +16121,7 @@
         <v>2755</v>
       </c>
       <c r="C1426" t="n">
-        <v>34090.96</v>
+        <v>36363.68</v>
       </c>
     </row>
     <row r="1427">
@@ -16143,7 +16143,7 @@
         <v>1064</v>
       </c>
       <c r="C1428" t="n">
-        <v>409080</v>
+        <v>436352</v>
       </c>
     </row>
     <row r="1429">
@@ -16154,7 +16154,7 @@
         <v>1810</v>
       </c>
       <c r="C1429" t="n">
-        <v>27690</v>
+        <v>29536</v>
       </c>
     </row>
     <row r="1430">
@@ -16165,7 +16165,7 @@
         <v>1937</v>
       </c>
       <c r="C1430" t="n">
-        <v>176580</v>
+        <v>188352</v>
       </c>
     </row>
     <row r="1431">
@@ -16176,7 +16176,7 @@
         <v>483</v>
       </c>
       <c r="C1431" t="n">
-        <v>308175</v>
+        <v>328720</v>
       </c>
     </row>
     <row r="1432">
@@ -16187,7 +16187,7 @@
         <v>2580</v>
       </c>
       <c r="C1432" t="n">
-        <v>22965</v>
+        <v>24496</v>
       </c>
     </row>
     <row r="1433">
@@ -16198,7 +16198,7 @@
         <v>2706</v>
       </c>
       <c r="C1433" t="n">
-        <v>17940</v>
+        <v>19136</v>
       </c>
     </row>
     <row r="1434">
@@ -16209,7 +16209,7 @@
         <v>2633</v>
       </c>
       <c r="C1434" t="n">
-        <v>13140</v>
+        <v>14016</v>
       </c>
     </row>
     <row r="1435">
@@ -16242,7 +16242,7 @@
         <v>2392</v>
       </c>
       <c r="C1437" t="n">
-        <v>141420</v>
+        <v>150848</v>
       </c>
     </row>
     <row r="1438">
@@ -16264,7 +16264,7 @@
         <v>2613</v>
       </c>
       <c r="C1439" t="n">
-        <v>99570</v>
+        <v>106208</v>
       </c>
     </row>
     <row r="1440">
@@ -16275,7 +16275,7 @@
         <v>2183</v>
       </c>
       <c r="C1440" t="n">
-        <v>358515</v>
+        <v>382416</v>
       </c>
     </row>
     <row r="1441">
@@ -16286,7 +16286,7 @@
         <v>2541</v>
       </c>
       <c r="C1441" t="n">
-        <v>161175</v>
+        <v>171920</v>
       </c>
     </row>
     <row r="1442">
@@ -16297,7 +16297,7 @@
         <v>2333</v>
       </c>
       <c r="C1442" t="n">
-        <v>108810</v>
+        <v>116064</v>
       </c>
     </row>
     <row r="1443">
@@ -16308,7 +16308,7 @@
         <v>2813</v>
       </c>
       <c r="C1443" t="n">
-        <v>43500</v>
+        <v>46400</v>
       </c>
     </row>
     <row r="1444">
@@ -16319,7 +16319,7 @@
         <v>2811</v>
       </c>
       <c r="C1444" t="n">
-        <v>28365</v>
+        <v>30256</v>
       </c>
     </row>
     <row r="1445">
@@ -16330,7 +16330,7 @@
         <v>1881</v>
       </c>
       <c r="C1445" t="n">
-        <v>46830</v>
+        <v>49952</v>
       </c>
     </row>
     <row r="1446">
@@ -16341,7 +16341,7 @@
         <v>2825</v>
       </c>
       <c r="C1446" t="n">
-        <v>38070</v>
+        <v>40608</v>
       </c>
     </row>
     <row r="1447">
@@ -16352,7 +16352,7 @@
         <v>970</v>
       </c>
       <c r="C1447" t="n">
-        <v>46830</v>
+        <v>49952</v>
       </c>
     </row>
     <row r="1448">
@@ -16363,7 +16363,7 @@
         <v>2552</v>
       </c>
       <c r="C1448" t="n">
-        <v>26655</v>
+        <v>28432</v>
       </c>
     </row>
     <row r="1449">
@@ -16374,7 +16374,7 @@
         <v>2562</v>
       </c>
       <c r="C1449" t="n">
-        <v>26655</v>
+        <v>28432</v>
       </c>
     </row>
     <row r="1450">
@@ -16407,7 +16407,7 @@
         <v>2747</v>
       </c>
       <c r="C1452" t="n">
-        <v>47715</v>
+        <v>50896</v>
       </c>
     </row>
     <row r="1453">
@@ -16418,7 +16418,7 @@
         <v>415</v>
       </c>
       <c r="C1453" t="n">
-        <v>170454.59</v>
+        <v>181818.22</v>
       </c>
     </row>
     <row r="1454">
@@ -16462,7 +16462,7 @@
         <v>2544</v>
       </c>
       <c r="C1457" t="n">
-        <v>47715</v>
+        <v>50896</v>
       </c>
     </row>
     <row r="1458">
@@ -16473,7 +16473,7 @@
         <v>816</v>
       </c>
       <c r="C1458" t="n">
-        <v>204545.48</v>
+        <v>218181.84</v>
       </c>
     </row>
     <row r="1459">
@@ -16484,7 +16484,7 @@
         <v>890</v>
       </c>
       <c r="C1459" t="n">
-        <v>613636.37</v>
+        <v>654545.46</v>
       </c>
     </row>
     <row r="1460">
@@ -16495,7 +16495,7 @@
         <v>1298</v>
       </c>
       <c r="C1460" t="n">
-        <v>862500</v>
+        <v>920000</v>
       </c>
     </row>
     <row r="1461">
@@ -16506,7 +16506,7 @@
         <v>1372</v>
       </c>
       <c r="C1461" t="n">
-        <v>204545.48</v>
+        <v>218181.84</v>
       </c>
     </row>
     <row r="1462">
@@ -16517,7 +16517,7 @@
         <v>358</v>
       </c>
       <c r="C1462" t="n">
-        <v>214770</v>
+        <v>229088</v>
       </c>
     </row>
     <row r="1463">
@@ -16528,7 +16528,7 @@
         <v>1653</v>
       </c>
       <c r="C1463" t="n">
-        <v>214770</v>
+        <v>229088</v>
       </c>
     </row>
     <row r="1464">
@@ -16539,7 +16539,7 @@
         <v>675</v>
       </c>
       <c r="C1464" t="n">
-        <v>136350</v>
+        <v>145440</v>
       </c>
     </row>
     <row r="1465">
@@ -16550,7 +16550,7 @@
         <v>2804</v>
       </c>
       <c r="C1465" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1466">
@@ -16561,7 +16561,7 @@
         <v>2714</v>
       </c>
       <c r="C1466" t="n">
-        <v>245445</v>
+        <v>261808</v>
       </c>
     </row>
     <row r="1467">
@@ -16572,7 +16572,7 @@
         <v>2765</v>
       </c>
       <c r="C1467" t="n">
-        <v>61350</v>
+        <v>65440</v>
       </c>
     </row>
     <row r="1468">
@@ -16583,7 +16583,7 @@
         <v>2421</v>
       </c>
       <c r="C1468" t="n">
-        <v>41580</v>
+        <v>44352</v>
       </c>
     </row>
     <row r="1469">
@@ -16594,7 +16594,7 @@
         <v>2359</v>
       </c>
       <c r="C1469" t="n">
-        <v>71130</v>
+        <v>75872</v>
       </c>
     </row>
     <row r="1470">
@@ -16605,7 +16605,7 @@
         <v>2678</v>
       </c>
       <c r="C1470" t="n">
-        <v>67470</v>
+        <v>71968</v>
       </c>
     </row>
     <row r="1471">
@@ -16616,7 +16616,7 @@
         <v>2697</v>
       </c>
       <c r="C1471" t="n">
-        <v>102390</v>
+        <v>109216</v>
       </c>
     </row>
     <row r="1472">
@@ -16649,7 +16649,7 @@
         <v>2142</v>
       </c>
       <c r="C1474" t="n">
-        <v>36900</v>
+        <v>39360</v>
       </c>
     </row>
     <row r="1475">
@@ -16660,7 +16660,7 @@
         <v>2498</v>
       </c>
       <c r="C1475" t="n">
-        <v>38385</v>
+        <v>40944</v>
       </c>
     </row>
     <row r="1476">
@@ -16682,7 +16682,7 @@
         <v>2801</v>
       </c>
       <c r="C1477" t="n">
-        <v>68181.85000000001</v>
+        <v>72727.3</v>
       </c>
     </row>
     <row r="1478">
@@ -16693,7 +16693,7 @@
         <v>2810</v>
       </c>
       <c r="C1478" t="n">
-        <v>109090.96</v>
+        <v>116363.68</v>
       </c>
     </row>
     <row r="1479">
@@ -16737,7 +16737,7 @@
         <v>132</v>
       </c>
       <c r="C1482" t="n">
-        <v>238636.37</v>
+        <v>254545.46</v>
       </c>
     </row>
     <row r="1483">
@@ -16759,7 +16759,7 @@
         <v>580</v>
       </c>
       <c r="C1484" t="n">
-        <v>119318.22</v>
+        <v>127272.76</v>
       </c>
     </row>
     <row r="1485">
@@ -16770,7 +16770,7 @@
         <v>634</v>
       </c>
       <c r="C1485" t="n">
-        <v>340909.11</v>
+        <v>363636.38</v>
       </c>
     </row>
     <row r="1486">
@@ -16792,7 +16792,7 @@
         <v>1277</v>
       </c>
       <c r="C1487" t="n">
-        <v>150000</v>
+        <v>160000</v>
       </c>
     </row>
     <row r="1488">
@@ -16803,7 +16803,7 @@
         <v>767</v>
       </c>
       <c r="C1488" t="n">
-        <v>136350</v>
+        <v>145440</v>
       </c>
     </row>
     <row r="1489">
@@ -16814,7 +16814,7 @@
         <v>2727</v>
       </c>
       <c r="C1489" t="n">
-        <v>27600</v>
+        <v>29440</v>
       </c>
     </row>
     <row r="1490">
@@ -16825,7 +16825,7 @@
         <v>2846</v>
       </c>
       <c r="C1490" t="n">
-        <v>177270</v>
+        <v>189088</v>
       </c>
     </row>
     <row r="1491">
@@ -16836,7 +16836,7 @@
         <v>609</v>
       </c>
       <c r="C1491" t="n">
-        <v>153405</v>
+        <v>163632</v>
       </c>
     </row>
     <row r="1492">
@@ -16847,7 +16847,7 @@
         <v>2726</v>
       </c>
       <c r="C1492" t="n">
-        <v>105675</v>
+        <v>112720</v>
       </c>
     </row>
     <row r="1493">
@@ -16858,7 +16858,7 @@
         <v>2729</v>
       </c>
       <c r="C1493" t="n">
-        <v>61350</v>
+        <v>65440</v>
       </c>
     </row>
     <row r="1494">
@@ -16869,7 +16869,7 @@
         <v>1340</v>
       </c>
       <c r="C1494" t="n">
-        <v>102270</v>
+        <v>109088</v>
       </c>
     </row>
     <row r="1495">
@@ -16880,7 +16880,7 @@
         <v>2830</v>
       </c>
       <c r="C1495" t="n">
-        <v>61350</v>
+        <v>65440</v>
       </c>
     </row>
     <row r="1496">
@@ -16891,7 +16891,7 @@
         <v>2674</v>
       </c>
       <c r="C1496" t="n">
-        <v>177270</v>
+        <v>189088</v>
       </c>
     </row>
     <row r="1497">
@@ -16902,7 +16902,7 @@
         <v>2308</v>
       </c>
       <c r="C1497" t="n">
-        <v>136350</v>
+        <v>145440</v>
       </c>
     </row>
     <row r="1498">
@@ -16913,7 +16913,7 @@
         <v>2190</v>
       </c>
       <c r="C1498" t="n">
-        <v>143175</v>
+        <v>152720</v>
       </c>
     </row>
     <row r="1499">
@@ -16924,7 +16924,7 @@
         <v>2015</v>
       </c>
       <c r="C1499" t="n">
-        <v>252270</v>
+        <v>269088</v>
       </c>
     </row>
     <row r="1500">
@@ -16935,7 +16935,7 @@
         <v>1308</v>
       </c>
       <c r="C1500" t="n">
-        <v>107040</v>
+        <v>114176</v>
       </c>
     </row>
     <row r="1501">
@@ -16946,7 +16946,7 @@
         <v>2118</v>
       </c>
       <c r="C1501" t="n">
-        <v>143295</v>
+        <v>152848</v>
       </c>
     </row>
     <row r="1502">
@@ -16957,7 +16957,7 @@
         <v>2607</v>
       </c>
       <c r="C1502" t="n">
-        <v>33870</v>
+        <v>36128</v>
       </c>
     </row>
     <row r="1503">
@@ -16968,7 +16968,7 @@
         <v>2832</v>
       </c>
       <c r="C1503" t="n">
-        <v>102272.74</v>
+        <v>109090.92</v>
       </c>
     </row>
     <row r="1504">
@@ -16979,7 +16979,7 @@
         <v>2383</v>
       </c>
       <c r="C1504" t="n">
-        <v>90630</v>
+        <v>96672</v>
       </c>
     </row>
     <row r="1505">
@@ -17012,7 +17012,7 @@
         <v>2821</v>
       </c>
       <c r="C1507" t="n">
-        <v>90915</v>
+        <v>96976</v>
       </c>
     </row>
     <row r="1508">
@@ -17034,7 +17034,7 @@
         <v>569</v>
       </c>
       <c r="C1509" t="n">
-        <v>1979610</v>
+        <v>2111584</v>
       </c>
     </row>
     <row r="1510">
@@ -17045,7 +17045,7 @@
         <v>2660</v>
       </c>
       <c r="C1510" t="n">
-        <v>238636.37</v>
+        <v>254545.46</v>
       </c>
     </row>
     <row r="1511">
@@ -17056,7 +17056,7 @@
         <v>1632</v>
       </c>
       <c r="C1511" t="n">
-        <v>177272.74</v>
+        <v>189090.92</v>
       </c>
     </row>
     <row r="1512">
@@ -17067,7 +17067,7 @@
         <v>1756</v>
       </c>
       <c r="C1512" t="n">
-        <v>286350</v>
+        <v>305440</v>
       </c>
     </row>
     <row r="1513">
@@ -17078,7 +17078,7 @@
         <v>58</v>
       </c>
       <c r="C1513" t="n">
-        <v>171000</v>
+        <v>182400</v>
       </c>
     </row>
     <row r="1514">
@@ -17089,7 +17089,7 @@
         <v>40</v>
       </c>
       <c r="C1514" t="n">
-        <v>152100</v>
+        <v>162240</v>
       </c>
     </row>
     <row r="1515">
@@ -17100,7 +17100,7 @@
         <v>559</v>
       </c>
       <c r="C1515" t="n">
-        <v>159540</v>
+        <v>170176</v>
       </c>
     </row>
     <row r="1516">
@@ -17111,7 +17111,7 @@
         <v>2773</v>
       </c>
       <c r="C1516" t="n">
-        <v>55005</v>
+        <v>58672</v>
       </c>
     </row>
     <row r="1517">
@@ -17122,7 +17122,7 @@
         <v>2631</v>
       </c>
       <c r="C1517" t="n">
-        <v>26415</v>
+        <v>28176</v>
       </c>
     </row>
     <row r="1518">
@@ -17133,7 +17133,7 @@
         <v>2085</v>
       </c>
       <c r="C1518" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1519">
@@ -17155,7 +17155,7 @@
         <v>1642</v>
       </c>
       <c r="C1520" t="n">
-        <v>180675</v>
+        <v>192720</v>
       </c>
     </row>
     <row r="1521">
@@ -17166,7 +17166,7 @@
         <v>2621</v>
       </c>
       <c r="C1521" t="n">
-        <v>47715</v>
+        <v>50896</v>
       </c>
     </row>
     <row r="1522">
@@ -17177,7 +17177,7 @@
         <v>2705</v>
       </c>
       <c r="C1522" t="n">
-        <v>136890</v>
+        <v>146016</v>
       </c>
     </row>
     <row r="1523">
@@ -17188,7 +17188,7 @@
         <v>2735</v>
       </c>
       <c r="C1523" t="n">
-        <v>81810</v>
+        <v>87264</v>
       </c>
     </row>
     <row r="1524">
@@ -17199,7 +17199,7 @@
         <v>945</v>
       </c>
       <c r="C1524" t="n">
-        <v>239100</v>
+        <v>255040</v>
       </c>
     </row>
     <row r="1525">
@@ -17210,7 +17210,7 @@
         <v>2582</v>
       </c>
       <c r="C1525" t="n">
-        <v>59820</v>
+        <v>63808</v>
       </c>
     </row>
     <row r="1526">
@@ -17221,7 +17221,7 @@
         <v>2584</v>
       </c>
       <c r="C1526" t="n">
-        <v>43500</v>
+        <v>46400</v>
       </c>
     </row>
     <row r="1527">
@@ -17232,7 +17232,7 @@
         <v>2689</v>
       </c>
       <c r="C1527" t="n">
-        <v>43500</v>
+        <v>46400</v>
       </c>
     </row>
     <row r="1528">
@@ -17243,7 +17243,7 @@
         <v>2574</v>
       </c>
       <c r="C1528" t="n">
-        <v>95610</v>
+        <v>101984</v>
       </c>
     </row>
     <row r="1529">
@@ -17254,7 +17254,7 @@
         <v>1834</v>
       </c>
       <c r="C1529" t="n">
-        <v>80250</v>
+        <v>85600</v>
       </c>
     </row>
     <row r="1530">
@@ -17265,7 +17265,7 @@
         <v>2629</v>
       </c>
       <c r="C1530" t="n">
-        <v>46830</v>
+        <v>49952</v>
       </c>
     </row>
     <row r="1531">
@@ -17276,7 +17276,7 @@
         <v>933</v>
       </c>
       <c r="C1531" t="n">
-        <v>55545</v>
+        <v>59248</v>
       </c>
     </row>
     <row r="1532">
@@ -17287,7 +17287,7 @@
         <v>2555</v>
       </c>
       <c r="C1532" t="n">
-        <v>26655</v>
+        <v>28432</v>
       </c>
     </row>
     <row r="1533">
@@ -17298,7 +17298,7 @@
         <v>2558</v>
       </c>
       <c r="C1533" t="n">
-        <v>26655</v>
+        <v>28432</v>
       </c>
     </row>
     <row r="1534">
@@ -17309,7 +17309,7 @@
         <v>2721</v>
       </c>
       <c r="C1534" t="n">
-        <v>55545</v>
+        <v>59248</v>
       </c>
     </row>
     <row r="1535">
@@ -17320,7 +17320,7 @@
         <v>2556</v>
       </c>
       <c r="C1535" t="n">
-        <v>26655</v>
+        <v>28432</v>
       </c>
     </row>
     <row r="1536">
@@ -17331,7 +17331,7 @@
         <v>2826</v>
       </c>
       <c r="C1536" t="n">
-        <v>47715</v>
+        <v>50896</v>
       </c>
     </row>
     <row r="1537">
@@ -17353,7 +17353,7 @@
         <v>2346</v>
       </c>
       <c r="C1538" t="n">
-        <v>47715</v>
+        <v>50896</v>
       </c>
     </row>
     <row r="1539">
@@ -17364,7 +17364,7 @@
         <v>595</v>
       </c>
       <c r="C1539" t="n">
-        <v>170454.59</v>
+        <v>181818.22</v>
       </c>
     </row>
     <row r="1540">
@@ -17375,7 +17375,7 @@
         <v>1278</v>
       </c>
       <c r="C1540" t="n">
-        <v>119318.22</v>
+        <v>127272.76</v>
       </c>
     </row>
     <row r="1541">
@@ -17386,7 +17386,7 @@
         <v>2686</v>
       </c>
       <c r="C1541" t="n">
-        <v>95445</v>
+        <v>101808</v>
       </c>
     </row>
     <row r="1542">
@@ -17397,7 +17397,7 @@
         <v>1344</v>
       </c>
       <c r="C1542" t="n">
-        <v>102270</v>
+        <v>109088</v>
       </c>
     </row>
     <row r="1543">
@@ -17408,7 +17408,7 @@
         <v>2566</v>
       </c>
       <c r="C1543" t="n">
-        <v>54540</v>
+        <v>58176</v>
       </c>
     </row>
     <row r="1544">
@@ -17419,7 +17419,7 @@
         <v>2684</v>
       </c>
       <c r="C1544" t="n">
-        <v>64770</v>
+        <v>69088</v>
       </c>
     </row>
     <row r="1545">
@@ -17430,7 +17430,7 @@
         <v>2375</v>
       </c>
       <c r="C1545" t="n">
-        <v>225000</v>
+        <v>240000</v>
       </c>
     </row>
     <row r="1546">
@@ -17441,7 +17441,7 @@
         <v>2829</v>
       </c>
       <c r="C1546" t="n">
-        <v>40905</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1547">
@@ -17452,7 +17452,7 @@
         <v>768</v>
       </c>
       <c r="C1547" t="n">
-        <v>95445</v>
+        <v>101808</v>
       </c>
     </row>
     <row r="1548">
@@ -17463,7 +17463,7 @@
         <v>772</v>
       </c>
       <c r="C1548" t="n">
-        <v>221580</v>
+        <v>236352</v>
       </c>
     </row>
     <row r="1549">
@@ -17474,7 +17474,7 @@
         <v>2496</v>
       </c>
       <c r="C1549" t="n">
-        <v>136350</v>
+        <v>145440</v>
       </c>
     </row>
     <row r="1550">
@@ -17485,7 +17485,7 @@
         <v>802</v>
       </c>
       <c r="C1550" t="n">
-        <v>51135</v>
+        <v>54544</v>
       </c>
     </row>
     <row r="1551">
@@ -17496,7 +17496,7 @@
         <v>2131</v>
       </c>
       <c r="C1551" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1552">
@@ -17507,7 +17507,7 @@
         <v>1381</v>
       </c>
       <c r="C1552" t="n">
-        <v>204545.48</v>
+        <v>218181.84</v>
       </c>
     </row>
     <row r="1553">
@@ -17518,7 +17518,7 @@
         <v>2847</v>
       </c>
       <c r="C1553" t="n">
-        <v>92040</v>
+        <v>98176</v>
       </c>
     </row>
     <row r="1554">
@@ -17529,7 +17529,7 @@
         <v>1293</v>
       </c>
       <c r="C1554" t="n">
-        <v>262500</v>
+        <v>280000</v>
       </c>
     </row>
     <row r="1555">
@@ -17540,7 +17540,7 @@
         <v>2363</v>
       </c>
       <c r="C1555" t="n">
-        <v>115905</v>
+        <v>123632</v>
       </c>
     </row>
     <row r="1556">
@@ -17551,7 +17551,7 @@
         <v>631</v>
       </c>
       <c r="C1556" t="n">
-        <v>238635</v>
+        <v>254544</v>
       </c>
     </row>
     <row r="1557">
@@ -17562,7 +17562,7 @@
         <v>2791</v>
       </c>
       <c r="C1557" t="n">
-        <v>70005</v>
+        <v>74672</v>
       </c>
     </row>
     <row r="1558">
@@ -17584,7 +17584,7 @@
         <v>2841</v>
       </c>
       <c r="C1559" t="n">
-        <v>34080</v>
+        <v>36352</v>
       </c>
     </row>
     <row r="1560">
@@ -17595,7 +17595,7 @@
         <v>2571</v>
       </c>
       <c r="C1560" t="n">
-        <v>181755</v>
+        <v>193872</v>
       </c>
     </row>
     <row r="1561">
@@ -17661,7 +17661,7 @@
         <v>2273</v>
       </c>
       <c r="C1566" t="n">
-        <v>146595</v>
+        <v>156368</v>
       </c>
     </row>
     <row r="1567">
@@ -17672,7 +17672,7 @@
         <v>2381</v>
       </c>
       <c r="C1567" t="n">
-        <v>54825</v>
+        <v>58480</v>
       </c>
     </row>
     <row r="1568">
@@ -17683,7 +17683,7 @@
         <v>630</v>
       </c>
       <c r="C1568" t="n">
-        <v>56270.43</v>
+        <v>60021.79</v>
       </c>
     </row>
     <row r="1569">
@@ -17705,7 +17705,7 @@
         <v>1983</v>
       </c>
       <c r="C1570" t="n">
-        <v>373800</v>
+        <v>398720</v>
       </c>
     </row>
     <row r="1571">
@@ -17716,7 +17716,7 @@
         <v>1993</v>
       </c>
       <c r="C1571" t="n">
-        <v>253830</v>
+        <v>270752</v>
       </c>
     </row>
     <row r="1572">
@@ -17727,7 +17727,7 @@
         <v>89</v>
       </c>
       <c r="C1572" t="n">
-        <v>238635</v>
+        <v>254544</v>
       </c>
     </row>
     <row r="1573">
@@ -17738,7 +17738,7 @@
         <v>1063</v>
       </c>
       <c r="C1573" t="n">
-        <v>262500</v>
+        <v>280000</v>
       </c>
     </row>
     <row r="1574">
@@ -17749,7 +17749,7 @@
         <v>1116</v>
       </c>
       <c r="C1574" t="n">
-        <v>170445</v>
+        <v>181808</v>
       </c>
     </row>
     <row r="1575">
@@ -17760,7 +17760,7 @@
         <v>941</v>
       </c>
       <c r="C1575" t="n">
-        <v>205155</v>
+        <v>218832</v>
       </c>
     </row>
     <row r="1576">
@@ -17771,7 +17771,7 @@
         <v>2141</v>
       </c>
       <c r="C1576" t="n">
-        <v>21870</v>
+        <v>23328</v>
       </c>
     </row>
     <row r="1577">
@@ -17782,7 +17782,7 @@
         <v>2463</v>
       </c>
       <c r="C1577" t="n">
-        <v>224880</v>
+        <v>239872</v>
       </c>
     </row>
     <row r="1578">
@@ -17793,7 +17793,7 @@
         <v>2707</v>
       </c>
       <c r="C1578" t="n">
-        <v>29445</v>
+        <v>31408</v>
       </c>
     </row>
     <row r="1579">
@@ -17804,7 +17804,7 @@
         <v>2325</v>
       </c>
       <c r="C1579" t="n">
-        <v>78660</v>
+        <v>83904</v>
       </c>
     </row>
     <row r="1580">
@@ -17848,7 +17848,7 @@
         <v>1890</v>
       </c>
       <c r="C1583" t="n">
-        <v>167205</v>
+        <v>178352</v>
       </c>
     </row>
     <row r="1584">
@@ -17859,7 +17859,7 @@
         <v>2639</v>
       </c>
       <c r="C1584" t="n">
-        <v>27315</v>
+        <v>29136</v>
       </c>
     </row>
     <row r="1585">
@@ -17870,7 +17870,7 @@
         <v>2682</v>
       </c>
       <c r="C1585" t="n">
-        <v>95445</v>
+        <v>101808</v>
       </c>
     </row>
     <row r="1586">
@@ -17881,7 +17881,7 @@
         <v>2601</v>
       </c>
       <c r="C1586" t="n">
-        <v>187500</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="1587">
@@ -17892,7 +17892,7 @@
         <v>1142</v>
       </c>
       <c r="C1587" t="n">
-        <v>312330</v>
+        <v>333152</v>
       </c>
     </row>
     <row r="1588">
@@ -17936,7 +17936,7 @@
         <v>2082</v>
       </c>
       <c r="C1591" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1592">
@@ -17947,7 +17947,7 @@
         <v>2276</v>
       </c>
       <c r="C1592" t="n">
-        <v>135630</v>
+        <v>144672</v>
       </c>
     </row>
     <row r="1593">
@@ -17958,7 +17958,7 @@
         <v>2786</v>
       </c>
       <c r="C1593" t="n">
-        <v>47715</v>
+        <v>50896</v>
       </c>
     </row>
     <row r="1594">
@@ -17969,7 +17969,7 @@
         <v>2816</v>
       </c>
       <c r="C1594" t="n">
-        <v>88635</v>
+        <v>94544</v>
       </c>
     </row>
     <row r="1595">
@@ -17980,7 +17980,7 @@
         <v>1871</v>
       </c>
       <c r="C1595" t="n">
-        <v>97845</v>
+        <v>104368</v>
       </c>
     </row>
     <row r="1596">
@@ -17991,7 +17991,7 @@
         <v>2345</v>
       </c>
       <c r="C1596" t="n">
-        <v>43500</v>
+        <v>46400</v>
       </c>
     </row>
     <row r="1597">
@@ -18002,7 +18002,7 @@
         <v>2802</v>
       </c>
       <c r="C1597" t="n">
-        <v>48945</v>
+        <v>52208</v>
       </c>
     </row>
     <row r="1598">
@@ -18013,7 +18013,7 @@
         <v>2090</v>
       </c>
       <c r="C1598" t="n">
-        <v>28365</v>
+        <v>30256</v>
       </c>
     </row>
     <row r="1599">
@@ -18024,7 +18024,7 @@
         <v>2647</v>
       </c>
       <c r="C1599" t="n">
-        <v>95625</v>
+        <v>102000</v>
       </c>
     </row>
     <row r="1600">
@@ -18035,7 +18035,7 @@
         <v>2365</v>
       </c>
       <c r="C1600" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1601">
@@ -18046,7 +18046,7 @@
         <v>766</v>
       </c>
       <c r="C1601" t="n">
-        <v>46830</v>
+        <v>49952</v>
       </c>
     </row>
     <row r="1602">
@@ -18057,7 +18057,7 @@
         <v>2702</v>
       </c>
       <c r="C1602" t="n">
-        <v>55545</v>
+        <v>59248</v>
       </c>
     </row>
     <row r="1603">
@@ -18068,7 +18068,7 @@
         <v>20</v>
       </c>
       <c r="C1603" t="n">
-        <v>306818.22</v>
+        <v>327272.76</v>
       </c>
     </row>
     <row r="1604">
@@ -18079,7 +18079,7 @@
         <v>27</v>
       </c>
       <c r="C1604" t="n">
-        <v>102272.74</v>
+        <v>109090.92</v>
       </c>
     </row>
     <row r="1605">
@@ -18090,7 +18090,7 @@
         <v>33</v>
       </c>
       <c r="C1605" t="n">
-        <v>271350</v>
+        <v>289440</v>
       </c>
     </row>
     <row r="1606">
@@ -18112,7 +18112,7 @@
         <v>2561</v>
       </c>
       <c r="C1607" t="n">
-        <v>26655</v>
+        <v>28432</v>
       </c>
     </row>
     <row r="1608">
@@ -18134,7 +18134,7 @@
         <v>2772</v>
       </c>
       <c r="C1609" t="n">
-        <v>40905</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1610">
@@ -18145,7 +18145,7 @@
         <v>2834</v>
       </c>
       <c r="C1610" t="n">
-        <v>25410</v>
+        <v>27104</v>
       </c>
     </row>
     <row r="1611">
@@ -18156,7 +18156,7 @@
         <v>2394</v>
       </c>
       <c r="C1611" t="n">
-        <v>77355</v>
+        <v>82512</v>
       </c>
     </row>
     <row r="1612">
@@ -18167,7 +18167,7 @@
         <v>2567</v>
       </c>
       <c r="C1612" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1613">
@@ -18178,7 +18178,7 @@
         <v>952</v>
       </c>
       <c r="C1613" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1614">
@@ -18189,7 +18189,7 @@
         <v>1539</v>
       </c>
       <c r="C1614" t="n">
-        <v>115905</v>
+        <v>123632</v>
       </c>
     </row>
     <row r="1615">
@@ -18200,7 +18200,7 @@
         <v>793</v>
       </c>
       <c r="C1615" t="n">
-        <v>28365</v>
+        <v>30256</v>
       </c>
     </row>
     <row r="1616">
@@ -18211,7 +18211,7 @@
         <v>794</v>
       </c>
       <c r="C1616" t="n">
-        <v>28365</v>
+        <v>30256</v>
       </c>
     </row>
     <row r="1617">
@@ -18222,7 +18222,7 @@
         <v>2838</v>
       </c>
       <c r="C1617" t="n">
-        <v>40909.11</v>
+        <v>43636.38</v>
       </c>
     </row>
     <row r="1618">
@@ -18233,7 +18233,7 @@
         <v>2223</v>
       </c>
       <c r="C1618" t="n">
-        <v>79845</v>
+        <v>85168</v>
       </c>
     </row>
     <row r="1619">
@@ -18244,7 +18244,7 @@
         <v>2547</v>
       </c>
       <c r="C1619" t="n">
-        <v>23100</v>
+        <v>24640</v>
       </c>
     </row>
     <row r="1620">
@@ -18255,7 +18255,7 @@
         <v>2762</v>
       </c>
       <c r="C1620" t="n">
-        <v>55545</v>
+        <v>59248</v>
       </c>
     </row>
     <row r="1621">
@@ -18266,7 +18266,7 @@
         <v>2550</v>
       </c>
       <c r="C1621" t="n">
-        <v>26655</v>
+        <v>28432</v>
       </c>
     </row>
     <row r="1622">
@@ -18277,7 +18277,7 @@
         <v>2627</v>
       </c>
       <c r="C1622" t="n">
-        <v>26655</v>
+        <v>28432</v>
       </c>
     </row>
     <row r="1623">
@@ -18299,7 +18299,7 @@
         <v>749</v>
       </c>
       <c r="C1624" t="n">
-        <v>55545</v>
+        <v>59248</v>
       </c>
     </row>
     <row r="1625">
@@ -18310,7 +18310,7 @@
         <v>2549</v>
       </c>
       <c r="C1625" t="n">
-        <v>26655</v>
+        <v>28432</v>
       </c>
     </row>
     <row r="1626">
@@ -18321,7 +18321,7 @@
         <v>2649</v>
       </c>
       <c r="C1626" t="n">
-        <v>26655</v>
+        <v>28432</v>
       </c>
     </row>
     <row r="1627">
@@ -18332,7 +18332,7 @@
         <v>2258</v>
       </c>
       <c r="C1627" t="n">
-        <v>54540</v>
+        <v>58176</v>
       </c>
     </row>
     <row r="1628">
@@ -18343,7 +18343,7 @@
         <v>2744</v>
       </c>
       <c r="C1628" t="n">
-        <v>40905</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1629">
@@ -18354,7 +18354,7 @@
         <v>452</v>
       </c>
       <c r="C1629" t="n">
-        <v>192945</v>
+        <v>205808</v>
       </c>
     </row>
     <row r="1630">
@@ -18376,7 +18376,7 @@
         <v>2653</v>
       </c>
       <c r="C1631" t="n">
-        <v>40905</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1632">
@@ -18409,7 +18409,7 @@
         <v>2742</v>
       </c>
       <c r="C1634" t="n">
-        <v>13635</v>
+        <v>14544</v>
       </c>
     </row>
     <row r="1635">
@@ -18420,7 +18420,7 @@
         <v>1499</v>
       </c>
       <c r="C1635" t="n">
-        <v>61350</v>
+        <v>65440</v>
       </c>
     </row>
     <row r="1636">
@@ -18431,7 +18431,7 @@
         <v>2261</v>
       </c>
       <c r="C1636" t="n">
-        <v>122715</v>
+        <v>130896</v>
       </c>
     </row>
     <row r="1637">
@@ -18442,7 +18442,7 @@
         <v>1324</v>
       </c>
       <c r="C1637" t="n">
-        <v>190905</v>
+        <v>203632</v>
       </c>
     </row>
     <row r="1638">
@@ -18453,7 +18453,7 @@
         <v>2709</v>
       </c>
       <c r="C1638" t="n">
-        <v>122715</v>
+        <v>130896</v>
       </c>
     </row>
     <row r="1639">
@@ -18464,7 +18464,7 @@
         <v>1137</v>
       </c>
       <c r="C1639" t="n">
-        <v>436350</v>
+        <v>465440</v>
       </c>
     </row>
     <row r="1640">
@@ -18475,7 +18475,7 @@
         <v>2440</v>
       </c>
       <c r="C1640" t="n">
-        <v>54540</v>
+        <v>58176</v>
       </c>
     </row>
     <row r="1641">
@@ -18486,7 +18486,7 @@
         <v>429</v>
       </c>
       <c r="C1641" t="n">
-        <v>259080</v>
+        <v>276352</v>
       </c>
     </row>
     <row r="1642">
@@ -18497,7 +18497,7 @@
         <v>2114</v>
       </c>
       <c r="C1642" t="n">
-        <v>115995</v>
+        <v>123728</v>
       </c>
     </row>
     <row r="1643">
@@ -18508,7 +18508,7 @@
         <v>2211</v>
       </c>
       <c r="C1643" t="n">
-        <v>164205</v>
+        <v>175152</v>
       </c>
     </row>
     <row r="1644">
@@ -18519,7 +18519,7 @@
         <v>1108</v>
       </c>
       <c r="C1644" t="n">
-        <v>208890</v>
+        <v>222816</v>
       </c>
     </row>
     <row r="1645">
@@ -18530,7 +18530,7 @@
         <v>2695</v>
       </c>
       <c r="C1645" t="n">
-        <v>32985</v>
+        <v>35184</v>
       </c>
     </row>
     <row r="1646">
@@ -18541,7 +18541,7 @@
         <v>1289</v>
       </c>
       <c r="C1646" t="n">
-        <v>187500</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="1647">
@@ -18552,7 +18552,7 @@
         <v>2789</v>
       </c>
       <c r="C1647" t="n">
-        <v>122727.33</v>
+        <v>130909.14</v>
       </c>
     </row>
     <row r="1648">
@@ -18563,7 +18563,7 @@
         <v>2197</v>
       </c>
       <c r="C1648" t="n">
-        <v>146590.96</v>
+        <v>156363.68</v>
       </c>
     </row>
     <row r="1649">
@@ -18574,7 +18574,7 @@
         <v>947</v>
       </c>
       <c r="C1649" t="n">
-        <v>302370</v>
+        <v>322528</v>
       </c>
     </row>
     <row r="1650">
@@ -18585,7 +18585,7 @@
         <v>2279</v>
       </c>
       <c r="C1650" t="n">
-        <v>166995</v>
+        <v>178128</v>
       </c>
     </row>
     <row r="1651">
@@ -18596,7 +18596,7 @@
         <v>1465</v>
       </c>
       <c r="C1651" t="n">
-        <v>262500</v>
+        <v>280000</v>
       </c>
     </row>
     <row r="1652">
@@ -18607,7 +18607,7 @@
         <v>2651</v>
       </c>
       <c r="C1652" t="n">
-        <v>115905</v>
+        <v>123632</v>
       </c>
     </row>
     <row r="1653">
@@ -18618,7 +18618,7 @@
         <v>42</v>
       </c>
       <c r="C1653" t="n">
-        <v>1299540</v>
+        <v>1386176</v>
       </c>
     </row>
     <row r="1654">
@@ -18629,7 +18629,7 @@
         <v>949</v>
       </c>
       <c r="C1654" t="n">
-        <v>67815</v>
+        <v>72336</v>
       </c>
     </row>
     <row r="1655">
@@ -18640,7 +18640,7 @@
         <v>2606</v>
       </c>
       <c r="C1655" t="n">
-        <v>175050</v>
+        <v>186720</v>
       </c>
     </row>
     <row r="1656">
@@ -18651,7 +18651,7 @@
         <v>2249</v>
       </c>
       <c r="C1656" t="n">
-        <v>148725</v>
+        <v>158640</v>
       </c>
     </row>
     <row r="1657">
@@ -18695,7 +18695,7 @@
         <v>2045</v>
       </c>
       <c r="C1660" t="n">
-        <v>217140</v>
+        <v>231616</v>
       </c>
     </row>
     <row r="1661">
@@ -18706,7 +18706,7 @@
         <v>2663</v>
       </c>
       <c r="C1661" t="n">
-        <v>187500</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="1662">
@@ -18728,7 +18728,7 @@
         <v>2854</v>
       </c>
       <c r="C1663" t="n">
-        <v>27270</v>
+        <v>29088</v>
       </c>
     </row>
     <row r="1664">
@@ -18750,7 +18750,7 @@
         <v>2341</v>
       </c>
       <c r="C1665" t="n">
-        <v>119250</v>
+        <v>127200</v>
       </c>
     </row>
     <row r="1666">
@@ -18761,7 +18761,7 @@
         <v>2637</v>
       </c>
       <c r="C1666" t="n">
-        <v>43500</v>
+        <v>46400</v>
       </c>
     </row>
     <row r="1667">
@@ -18772,7 +18772,7 @@
         <v>2492</v>
       </c>
       <c r="C1667" t="n">
-        <v>68295</v>
+        <v>72848</v>
       </c>
     </row>
     <row r="1668">
@@ -18783,7 +18783,7 @@
         <v>2548</v>
       </c>
       <c r="C1668" t="n">
-        <v>26655</v>
+        <v>28432</v>
       </c>
     </row>
     <row r="1669">
@@ -18794,7 +18794,7 @@
         <v>351</v>
       </c>
       <c r="C1669" t="n">
-        <v>145215</v>
+        <v>154896</v>
       </c>
     </row>
     <row r="1670">
@@ -18827,7 +18827,7 @@
         <v>2757</v>
       </c>
       <c r="C1672" t="n">
-        <v>54540</v>
+        <v>58176</v>
       </c>
     </row>
     <row r="1673">
@@ -18838,7 +18838,7 @@
         <v>2815</v>
       </c>
       <c r="C1673" t="n">
-        <v>40905</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1674">
@@ -18849,7 +18849,7 @@
         <v>2323</v>
       </c>
       <c r="C1674" t="n">
-        <v>46830</v>
+        <v>49952</v>
       </c>
     </row>
     <row r="1675">
@@ -18860,7 +18860,7 @@
         <v>2310</v>
       </c>
       <c r="C1675" t="n">
-        <v>46830</v>
+        <v>49952</v>
       </c>
     </row>
     <row r="1676">
@@ -18871,7 +18871,7 @@
         <v>2145</v>
       </c>
       <c r="C1676" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1677">
@@ -18882,7 +18882,7 @@
         <v>2501</v>
       </c>
       <c r="C1677" t="n">
-        <v>55545</v>
+        <v>59248</v>
       </c>
     </row>
     <row r="1678">
@@ -18893,7 +18893,7 @@
         <v>2546</v>
       </c>
       <c r="C1678" t="n">
-        <v>26655</v>
+        <v>28432</v>
       </c>
     </row>
     <row r="1679">
@@ -18904,7 +18904,7 @@
         <v>716</v>
       </c>
       <c r="C1679" t="n">
-        <v>87390</v>
+        <v>93216</v>
       </c>
     </row>
     <row r="1680">
@@ -18915,7 +18915,7 @@
         <v>2758</v>
       </c>
       <c r="C1680" t="n">
-        <v>40905</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1681">
@@ -18926,7 +18926,7 @@
         <v>400</v>
       </c>
       <c r="C1681" t="n">
-        <v>122715</v>
+        <v>130896</v>
       </c>
     </row>
     <row r="1682">
@@ -18937,7 +18937,7 @@
         <v>6</v>
       </c>
       <c r="C1682" t="n">
-        <v>34090.96</v>
+        <v>36363.68</v>
       </c>
     </row>
     <row r="1683">
@@ -18970,7 +18970,7 @@
         <v>1259</v>
       </c>
       <c r="C1685" t="n">
-        <v>75000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="1686">
@@ -18981,7 +18981,7 @@
         <v>571</v>
       </c>
       <c r="C1686" t="n">
-        <v>705681.85</v>
+        <v>752727.3</v>
       </c>
     </row>
     <row r="1687">
@@ -18992,7 +18992,7 @@
         <v>703</v>
       </c>
       <c r="C1687" t="n">
-        <v>170445</v>
+        <v>181808</v>
       </c>
     </row>
     <row r="1688">
@@ -19014,7 +19014,7 @@
         <v>2833</v>
       </c>
       <c r="C1689" t="n">
-        <v>54540</v>
+        <v>58176</v>
       </c>
     </row>
     <row r="1690">
@@ -19025,7 +19025,7 @@
         <v>1007</v>
       </c>
       <c r="C1690" t="n">
-        <v>136363.7</v>
+        <v>145454.6</v>
       </c>
     </row>
     <row r="1691">
@@ -19036,7 +19036,7 @@
         <v>2687</v>
       </c>
       <c r="C1691" t="n">
-        <v>54540</v>
+        <v>58176</v>
       </c>
     </row>
     <row r="1692">
@@ -19047,7 +19047,7 @@
         <v>2824</v>
       </c>
       <c r="C1692" t="n">
-        <v>76980</v>
+        <v>82112</v>
       </c>
     </row>
     <row r="1693">
@@ -19058,7 +19058,7 @@
         <v>2730</v>
       </c>
       <c r="C1693" t="n">
-        <v>61350</v>
+        <v>65440</v>
       </c>
     </row>
     <row r="1694">
@@ -19069,7 +19069,7 @@
         <v>2718</v>
       </c>
       <c r="C1694" t="n">
-        <v>88635</v>
+        <v>94544</v>
       </c>
     </row>
     <row r="1695">
@@ -19080,7 +19080,7 @@
         <v>2750</v>
       </c>
       <c r="C1695" t="n">
-        <v>20445</v>
+        <v>21808</v>
       </c>
     </row>
     <row r="1696">
@@ -19091,7 +19091,7 @@
         <v>854</v>
       </c>
       <c r="C1696" t="n">
-        <v>95445</v>
+        <v>101808</v>
       </c>
     </row>
     <row r="1697">
@@ -19102,7 +19102,7 @@
         <v>2794</v>
       </c>
       <c r="C1697" t="n">
-        <v>81810</v>
+        <v>87264</v>
       </c>
     </row>
     <row r="1698">
@@ -19113,7 +19113,7 @@
         <v>1374</v>
       </c>
       <c r="C1698" t="n">
-        <v>136350</v>
+        <v>145440</v>
       </c>
     </row>
     <row r="1699">
@@ -19124,7 +19124,7 @@
         <v>2488</v>
       </c>
       <c r="C1699" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1700">
@@ -19135,7 +19135,7 @@
         <v>363</v>
       </c>
       <c r="C1700" t="n">
-        <v>204540</v>
+        <v>218176</v>
       </c>
     </row>
     <row r="1701">
@@ -19146,7 +19146,7 @@
         <v>2655</v>
       </c>
       <c r="C1701" t="n">
-        <v>75000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="1702">
@@ -19157,7 +19157,7 @@
         <v>1873</v>
       </c>
       <c r="C1702" t="n">
-        <v>218175</v>
+        <v>232720</v>
       </c>
     </row>
     <row r="1703">
@@ -19168,7 +19168,7 @@
         <v>2635</v>
       </c>
       <c r="C1703" t="n">
-        <v>88635</v>
+        <v>94544</v>
       </c>
     </row>
     <row r="1704">
@@ -19179,7 +19179,7 @@
         <v>1658</v>
       </c>
       <c r="C1704" t="n">
-        <v>104310</v>
+        <v>111264</v>
       </c>
     </row>
     <row r="1705">
@@ -19190,7 +19190,7 @@
         <v>2069</v>
       </c>
       <c r="C1705" t="n">
-        <v>136363.7</v>
+        <v>145454.6</v>
       </c>
     </row>
     <row r="1706">
@@ -19201,7 +19201,7 @@
         <v>2081</v>
       </c>
       <c r="C1706" t="n">
-        <v>102270</v>
+        <v>109088</v>
       </c>
     </row>
     <row r="1707">
@@ -19212,7 +19212,7 @@
         <v>2124</v>
       </c>
       <c r="C1707" t="n">
-        <v>238635</v>
+        <v>254544</v>
       </c>
     </row>
     <row r="1708">
@@ -19223,7 +19223,7 @@
         <v>636</v>
       </c>
       <c r="C1708" t="n">
-        <v>170445</v>
+        <v>181808</v>
       </c>
     </row>
     <row r="1709">
@@ -19234,7 +19234,7 @@
         <v>2803</v>
       </c>
       <c r="C1709" t="n">
-        <v>81810</v>
+        <v>87264</v>
       </c>
     </row>
     <row r="1710">
@@ -19245,7 +19245,7 @@
         <v>2163</v>
       </c>
       <c r="C1710" t="n">
-        <v>122715</v>
+        <v>130896</v>
       </c>
     </row>
     <row r="1711">
@@ -19256,7 +19256,7 @@
         <v>1466</v>
       </c>
       <c r="C1711" t="n">
-        <v>276135</v>
+        <v>294544</v>
       </c>
     </row>
     <row r="1712">
@@ -19267,7 +19267,7 @@
         <v>2133</v>
       </c>
       <c r="C1712" t="n">
-        <v>238636.37</v>
+        <v>254545.46</v>
       </c>
     </row>
     <row r="1713">
@@ -19278,7 +19278,7 @@
         <v>2431</v>
       </c>
       <c r="C1713" t="n">
-        <v>102270</v>
+        <v>109088</v>
       </c>
     </row>
     <row r="1714">
@@ -19289,7 +19289,7 @@
         <v>535</v>
       </c>
       <c r="C1714" t="n">
-        <v>242850</v>
+        <v>259040</v>
       </c>
     </row>
     <row r="1715">
@@ -19300,7 +19300,7 @@
         <v>2790</v>
       </c>
       <c r="C1715" t="n">
-        <v>43065</v>
+        <v>45936</v>
       </c>
     </row>
     <row r="1716">
@@ -19311,7 +19311,7 @@
         <v>2442</v>
       </c>
       <c r="C1716" t="n">
-        <v>176580</v>
+        <v>188352</v>
       </c>
     </row>
     <row r="1717">
@@ -19322,7 +19322,7 @@
         <v>2376</v>
       </c>
       <c r="C1717" t="n">
-        <v>750000</v>
+        <v>800000</v>
       </c>
     </row>
     <row r="1718">
@@ -19333,7 +19333,7 @@
         <v>2768</v>
       </c>
       <c r="C1718" t="n">
-        <v>206355</v>
+        <v>220112</v>
       </c>
     </row>
     <row r="1719">
@@ -19344,7 +19344,7 @@
         <v>2491</v>
       </c>
       <c r="C1719" t="n">
-        <v>165585</v>
+        <v>176624</v>
       </c>
     </row>
     <row r="1720">
@@ -19355,7 +19355,7 @@
         <v>2799</v>
       </c>
       <c r="C1720" t="n">
-        <v>74535</v>
+        <v>79504</v>
       </c>
     </row>
     <row r="1721">
@@ -19388,7 +19388,7 @@
         <v>1317</v>
       </c>
       <c r="C1723" t="n">
-        <v>214772.74</v>
+        <v>229090.92</v>
       </c>
     </row>
     <row r="1724">
@@ -19399,7 +19399,7 @@
         <v>2822</v>
       </c>
       <c r="C1724" t="n">
-        <v>109090.96</v>
+        <v>116363.68</v>
       </c>
     </row>
     <row r="1725">
@@ -19410,7 +19410,7 @@
         <v>1117</v>
       </c>
       <c r="C1725" t="n">
-        <v>272805</v>
+        <v>290992</v>
       </c>
     </row>
     <row r="1726">
@@ -19421,7 +19421,7 @@
         <v>1299</v>
       </c>
       <c r="C1726" t="n">
-        <v>359685</v>
+        <v>383664</v>
       </c>
     </row>
     <row r="1727">
@@ -19432,7 +19432,7 @@
         <v>477</v>
       </c>
       <c r="C1727" t="n">
-        <v>148230</v>
+        <v>158112</v>
       </c>
     </row>
     <row r="1728">
@@ -19443,7 +19443,7 @@
         <v>530</v>
       </c>
       <c r="C1728" t="n">
-        <v>204540</v>
+        <v>218176</v>
       </c>
     </row>
     <row r="1729">
@@ -19454,7 +19454,7 @@
         <v>953</v>
       </c>
       <c r="C1729" t="n">
-        <v>470445</v>
+        <v>501808</v>
       </c>
     </row>
     <row r="1730">
@@ -19465,7 +19465,7 @@
         <v>610</v>
       </c>
       <c r="C1730" t="n">
-        <v>560310</v>
+        <v>597664</v>
       </c>
     </row>
     <row r="1731">
@@ -19476,7 +19476,7 @@
         <v>2792</v>
       </c>
       <c r="C1731" t="n">
-        <v>140715</v>
+        <v>150096</v>
       </c>
     </row>
     <row r="1732">
@@ -19553,7 +19553,7 @@
         <v>1075</v>
       </c>
       <c r="C1738" t="n">
-        <v>312945</v>
+        <v>333808</v>
       </c>
     </row>
     <row r="1739">
@@ -19564,7 +19564,7 @@
         <v>131</v>
       </c>
       <c r="C1739" t="n">
-        <v>283635</v>
+        <v>302544</v>
       </c>
     </row>
     <row r="1740">
@@ -19575,7 +19575,7 @@
         <v>2667</v>
       </c>
       <c r="C1740" t="n">
-        <v>31155</v>
+        <v>33232</v>
       </c>
     </row>
     <row r="1741">
@@ -19586,7 +19586,7 @@
         <v>2330</v>
       </c>
       <c r="C1741" t="n">
-        <v>60645</v>
+        <v>64688</v>
       </c>
     </row>
     <row r="1742">
@@ -19608,7 +19608,7 @@
         <v>2577</v>
       </c>
       <c r="C1743" t="n">
-        <v>60795</v>
+        <v>64848</v>
       </c>
     </row>
     <row r="1744">
@@ -19619,7 +19619,7 @@
         <v>2510</v>
       </c>
       <c r="C1744" t="n">
-        <v>431760</v>
+        <v>460544</v>
       </c>
     </row>
     <row r="1745">
@@ -19641,7 +19641,7 @@
         <v>2850</v>
       </c>
       <c r="C1746" t="n">
-        <v>40905</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1747">
@@ -19663,7 +19663,7 @@
         <v>2745</v>
       </c>
       <c r="C1748" t="n">
-        <v>75000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="1749">
@@ -19674,7 +19674,7 @@
         <v>2817</v>
       </c>
       <c r="C1749" t="n">
-        <v>40905</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1750">
@@ -19685,7 +19685,7 @@
         <v>2784</v>
       </c>
       <c r="C1750" t="n">
-        <v>28365</v>
+        <v>30256</v>
       </c>
     </row>
     <row r="1751">
@@ -19696,7 +19696,7 @@
         <v>626</v>
       </c>
       <c r="C1751" t="n">
-        <v>1178055</v>
+        <v>1256592</v>
       </c>
     </row>
     <row r="1752">
@@ -19707,7 +19707,7 @@
         <v>925</v>
       </c>
       <c r="C1752" t="n">
-        <v>54390</v>
+        <v>58016</v>
       </c>
     </row>
     <row r="1753">
@@ -19718,7 +19718,7 @@
         <v>2586</v>
       </c>
       <c r="C1753" t="n">
-        <v>28365</v>
+        <v>30256</v>
       </c>
     </row>
     <row r="1754">
@@ -19729,7 +19729,7 @@
         <v>966</v>
       </c>
       <c r="C1754" t="n">
-        <v>55545</v>
+        <v>59248</v>
       </c>
     </row>
     <row r="1755">
@@ -19740,7 +19740,7 @@
         <v>2557</v>
       </c>
       <c r="C1755" t="n">
-        <v>26655</v>
+        <v>28432</v>
       </c>
     </row>
     <row r="1756">
@@ -19751,7 +19751,7 @@
         <v>14</v>
       </c>
       <c r="C1756" t="n">
-        <v>306810</v>
+        <v>327264</v>
       </c>
     </row>
     <row r="1757">
@@ -19762,7 +19762,7 @@
         <v>2798</v>
       </c>
       <c r="C1757" t="n">
-        <v>40905</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1758">
@@ -19784,7 +19784,7 @@
         <v>522</v>
       </c>
       <c r="C1759" t="n">
-        <v>136363.7</v>
+        <v>145454.6</v>
       </c>
     </row>
     <row r="1760">
@@ -19806,7 +19806,7 @@
         <v>2819</v>
       </c>
       <c r="C1761" t="n">
-        <v>40905</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1762">
@@ -19817,7 +19817,7 @@
         <v>2266</v>
       </c>
       <c r="C1762" t="n">
-        <v>54540</v>
+        <v>58176</v>
       </c>
     </row>
     <row r="1763">
@@ -19850,7 +19850,7 @@
         <v>2795</v>
       </c>
       <c r="C1765" t="n">
-        <v>40905</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1766">
@@ -19861,7 +19861,7 @@
         <v>2722</v>
       </c>
       <c r="C1766" t="n">
-        <v>13635</v>
+        <v>14544</v>
       </c>
     </row>
     <row r="1767">
@@ -19872,7 +19872,7 @@
         <v>951</v>
       </c>
       <c r="C1767" t="n">
-        <v>78405</v>
+        <v>83632</v>
       </c>
     </row>
     <row r="1768">
@@ -19883,7 +19883,7 @@
         <v>1020</v>
       </c>
       <c r="C1768" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1769">
@@ -19894,7 +19894,7 @@
         <v>1853</v>
       </c>
       <c r="C1769" t="n">
-        <v>81810</v>
+        <v>87264</v>
       </c>
     </row>
     <row r="1770">
@@ -19905,7 +19905,7 @@
         <v>1327</v>
       </c>
       <c r="C1770" t="n">
-        <v>47715</v>
+        <v>50896</v>
       </c>
     </row>
     <row r="1771">
@@ -19916,7 +19916,7 @@
         <v>2842</v>
       </c>
       <c r="C1771" t="n">
-        <v>122715</v>
+        <v>130896</v>
       </c>
     </row>
     <row r="1772">
@@ -19927,7 +19927,7 @@
         <v>2831</v>
       </c>
       <c r="C1772" t="n">
-        <v>40905</v>
+        <v>43632</v>
       </c>
     </row>
     <row r="1773">
@@ -19938,7 +19938,7 @@
         <v>818</v>
       </c>
       <c r="C1773" t="n">
-        <v>272715</v>
+        <v>290896</v>
       </c>
     </row>
     <row r="1774">
@@ -19949,7 +19949,7 @@
         <v>1501</v>
       </c>
       <c r="C1774" t="n">
-        <v>68175</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1775">
@@ -19960,7 +19960,7 @@
         <v>1869</v>
       </c>
       <c r="C1775" t="n">
-        <v>166350</v>
+        <v>177440</v>
       </c>
     </row>
     <row r="1776">
@@ -19971,7 +19971,7 @@
         <v>1996</v>
       </c>
       <c r="C1776" t="n">
-        <v>170454.59</v>
+        <v>181818.22</v>
       </c>
     </row>
     <row r="1777">
@@ -19982,7 +19982,7 @@
         <v>2462</v>
       </c>
       <c r="C1777" t="n">
-        <v>38614.83</v>
+        <v>41189.14</v>
       </c>
     </row>
     <row r="1778">
@@ -19993,7 +19993,7 @@
         <v>2696</v>
       </c>
       <c r="C1778" t="n">
-        <v>146220</v>
+        <v>155968</v>
       </c>
     </row>
     <row r="1779">
@@ -20004,7 +20004,7 @@
         <v>2698</v>
       </c>
       <c r="C1779" t="n">
-        <v>74940</v>
+        <v>79936</v>
       </c>
     </row>
     <row r="1780">
@@ -20026,7 +20026,7 @@
         <v>2828</v>
       </c>
       <c r="C1781" t="n">
-        <v>40909.11</v>
+        <v>43636.38</v>
       </c>
     </row>
     <row r="1782">
@@ -20037,7 +20037,7 @@
         <v>2843</v>
       </c>
       <c r="C1782" t="n">
-        <v>47715</v>
+        <v>50896</v>
       </c>
     </row>
     <row r="1783">
@@ -20048,7 +20048,7 @@
         <v>619</v>
       </c>
       <c r="C1783" t="n">
-        <v>213750</v>
+        <v>228000</v>
       </c>
     </row>
     <row r="1784">
@@ -20059,7 +20059,7 @@
         <v>1478</v>
       </c>
       <c r="C1784" t="n">
-        <v>374070</v>
+        <v>399008</v>
       </c>
     </row>
     <row r="1785">
@@ -20070,7 +20070,7 @@
         <v>2026</v>
       </c>
       <c r="C1785" t="n">
-        <v>165270</v>
+        <v>176288</v>
       </c>
     </row>
     <row r="1786">
@@ -20081,7 +20081,7 @@
         <v>663</v>
       </c>
       <c r="C1786" t="n">
-        <v>176580</v>
+        <v>188352</v>
       </c>
     </row>
     <row r="1787">
@@ -20092,7 +20092,7 @@
         <v>285</v>
       </c>
       <c r="C1787" t="n">
-        <v>374070</v>
+        <v>399008</v>
       </c>
     </row>
     <row r="1788">
@@ -20103,7 +20103,7 @@
         <v>424</v>
       </c>
       <c r="C1788" t="n">
-        <v>160305</v>
+        <v>170992</v>
       </c>
     </row>
     <row r="1789">
@@ -20114,7 +20114,7 @@
         <v>451</v>
       </c>
       <c r="C1789" t="n">
-        <v>165675</v>
+        <v>176720</v>
       </c>
     </row>
     <row r="1790">
@@ -20125,7 +20125,7 @@
         <v>629</v>
       </c>
       <c r="C1790" t="n">
-        <v>309540</v>
+        <v>330176</v>
       </c>
     </row>
     <row r="1791">
@@ -20136,7 +20136,7 @@
         <v>2657</v>
       </c>
       <c r="C1791" t="n">
-        <v>53985</v>
+        <v>57584</v>
       </c>
     </row>
     <row r="1792">
@@ -20147,7 +20147,7 @@
         <v>1254</v>
       </c>
       <c r="C1792" t="n">
-        <v>132405</v>
+        <v>141232</v>
       </c>
     </row>
     <row r="1793">
@@ -20158,7 +20158,7 @@
         <v>2402</v>
       </c>
       <c r="C1793" t="n">
-        <v>333030</v>
+        <v>355232</v>
       </c>
     </row>
     <row r="1794">
@@ -20169,7 +20169,7 @@
         <v>2413</v>
       </c>
       <c r="C1794" t="n">
-        <v>93975</v>
+        <v>100240</v>
       </c>
     </row>
     <row r="1795">
@@ -20180,7 +20180,7 @@
         <v>1450</v>
       </c>
       <c r="C1795" t="n">
-        <v>243405</v>
+        <v>259632</v>
       </c>
     </row>
     <row r="1796">
@@ -20202,7 +20202,7 @@
         <v>2671</v>
       </c>
       <c r="C1797" t="n">
-        <v>54540</v>
+        <v>58176</v>
       </c>
     </row>
     <row r="1798">
@@ -20213,7 +20213,7 @@
         <v>2568</v>
       </c>
       <c r="C1798" t="n">
-        <v>109395</v>
+        <v>116688</v>
       </c>
     </row>
     <row r="1799">
@@ -20224,7 +20224,7 @@
         <v>2146</v>
       </c>
       <c r="C1799" t="n">
-        <v>132465</v>
+        <v>141296</v>
       </c>
     </row>
     <row r="1800">
@@ -20235,7 +20235,7 @@
         <v>2753</v>
       </c>
       <c r="C1800" t="n">
-        <v>51135</v>
+        <v>54544</v>
       </c>
     </row>
     <row r="1801">
@@ -20246,7 +20246,7 @@
         <v>744</v>
       </c>
       <c r="C1801" t="n">
-        <v>28365</v>
+        <v>30256</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:02:58
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -15560,7 +15560,7 @@
         <v>2853</v>
       </c>
       <c r="C1375" t="n">
-        <v>59248</v>
+        <v>62951</v>
       </c>
     </row>
     <row r="1376">
@@ -15571,7 +15571,7 @@
         <v>2245</v>
       </c>
       <c r="C1376" t="n">
-        <v>161024</v>
+        <v>171088</v>
       </c>
     </row>
     <row r="1377">
@@ -15582,7 +15582,7 @@
         <v>2251</v>
       </c>
       <c r="C1377" t="n">
-        <v>145440</v>
+        <v>154530</v>
       </c>
     </row>
     <row r="1378">
@@ -15593,7 +15593,7 @@
         <v>664</v>
       </c>
       <c r="C1378" t="n">
-        <v>190544</v>
+        <v>202453</v>
       </c>
     </row>
     <row r="1379">
@@ -15604,7 +15604,7 @@
         <v>2472</v>
       </c>
       <c r="C1379" t="n">
-        <v>38496</v>
+        <v>40902</v>
       </c>
     </row>
     <row r="1380">
@@ -15615,7 +15615,7 @@
         <v>1456</v>
       </c>
       <c r="C1380" t="n">
-        <v>580352</v>
+        <v>616624</v>
       </c>
     </row>
     <row r="1381">
@@ -15626,7 +15626,7 @@
         <v>1585</v>
       </c>
       <c r="C1381" t="n">
-        <v>131632</v>
+        <v>139859</v>
       </c>
     </row>
     <row r="1382">
@@ -15670,7 +15670,7 @@
         <v>1907</v>
       </c>
       <c r="C1385" t="n">
-        <v>400384</v>
+        <v>425408</v>
       </c>
     </row>
     <row r="1386">
@@ -15703,7 +15703,7 @@
         <v>2659</v>
       </c>
       <c r="C1388" t="n">
-        <v>89456</v>
+        <v>95047</v>
       </c>
     </row>
     <row r="1389">
@@ -15714,7 +15714,7 @@
         <v>2583</v>
       </c>
       <c r="C1389" t="n">
-        <v>30256</v>
+        <v>32147</v>
       </c>
     </row>
     <row r="1390">
@@ -15725,7 +15725,7 @@
         <v>2692</v>
       </c>
       <c r="C1390" t="n">
-        <v>50909.14</v>
+        <v>54090.95</v>
       </c>
     </row>
     <row r="1391">
@@ -15736,7 +15736,7 @@
         <v>2691</v>
       </c>
       <c r="C1391" t="n">
-        <v>88861.14</v>
+        <v>94414.95</v>
       </c>
     </row>
     <row r="1392">
@@ -15747,7 +15747,7 @@
         <v>931</v>
       </c>
       <c r="C1392" t="n">
-        <v>69616</v>
+        <v>73967</v>
       </c>
     </row>
     <row r="1393">
@@ -15758,7 +15758,7 @@
         <v>2785</v>
       </c>
       <c r="C1393" t="n">
-        <v>30256</v>
+        <v>32147</v>
       </c>
     </row>
     <row r="1394">
@@ -15769,7 +15769,7 @@
         <v>2411</v>
       </c>
       <c r="C1394" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1395">
@@ -15780,7 +15780,7 @@
         <v>2716</v>
       </c>
       <c r="C1395" t="n">
-        <v>63808</v>
+        <v>67796</v>
       </c>
     </row>
     <row r="1396">
@@ -15791,7 +15791,7 @@
         <v>2809</v>
       </c>
       <c r="C1396" t="n">
-        <v>49952</v>
+        <v>53074</v>
       </c>
     </row>
     <row r="1397">
@@ -15802,7 +15802,7 @@
         <v>104</v>
       </c>
       <c r="C1397" t="n">
-        <v>218181.84</v>
+        <v>231818.2</v>
       </c>
     </row>
     <row r="1398">
@@ -15835,7 +15835,7 @@
         <v>781</v>
       </c>
       <c r="C1400" t="n">
-        <v>94544</v>
+        <v>100453</v>
       </c>
     </row>
     <row r="1401">
@@ -15857,7 +15857,7 @@
         <v>2494</v>
       </c>
       <c r="C1402" t="n">
-        <v>109088</v>
+        <v>115906</v>
       </c>
     </row>
     <row r="1403">
@@ -15868,7 +15868,7 @@
         <v>2652</v>
       </c>
       <c r="C1403" t="n">
-        <v>101808</v>
+        <v>108171</v>
       </c>
     </row>
     <row r="1404">
@@ -15879,7 +15879,7 @@
         <v>1384</v>
       </c>
       <c r="C1404" t="n">
-        <v>254545.46</v>
+        <v>270454.55</v>
       </c>
     </row>
     <row r="1405">
@@ -15890,7 +15890,7 @@
         <v>360</v>
       </c>
       <c r="C1405" t="n">
-        <v>363632</v>
+        <v>386359</v>
       </c>
     </row>
     <row r="1406">
@@ -15901,7 +15901,7 @@
         <v>2767</v>
       </c>
       <c r="C1406" t="n">
-        <v>138176</v>
+        <v>146812</v>
       </c>
     </row>
     <row r="1407">
@@ -15912,7 +15912,7 @@
         <v>2178</v>
       </c>
       <c r="C1407" t="n">
-        <v>199264</v>
+        <v>211718</v>
       </c>
     </row>
     <row r="1408">
@@ -15923,7 +15923,7 @@
         <v>2107</v>
       </c>
       <c r="C1408" t="n">
-        <v>218160</v>
+        <v>231795</v>
       </c>
     </row>
     <row r="1409">
@@ -15934,7 +15934,7 @@
         <v>2711</v>
       </c>
       <c r="C1409" t="n">
-        <v>62960</v>
+        <v>66895</v>
       </c>
     </row>
     <row r="1410">
@@ -15945,7 +15945,7 @@
         <v>2845</v>
       </c>
       <c r="C1410" t="n">
-        <v>36352</v>
+        <v>38624</v>
       </c>
     </row>
     <row r="1411">
@@ -15989,7 +15989,7 @@
         <v>1102</v>
       </c>
       <c r="C1414" t="n">
-        <v>170992</v>
+        <v>181679</v>
       </c>
     </row>
     <row r="1415">
@@ -16000,7 +16000,7 @@
         <v>353</v>
       </c>
       <c r="C1415" t="n">
-        <v>212752</v>
+        <v>226049</v>
       </c>
     </row>
     <row r="1416">
@@ -16011,7 +16011,7 @@
         <v>2250</v>
       </c>
       <c r="C1416" t="n">
-        <v>247264</v>
+        <v>262718</v>
       </c>
     </row>
     <row r="1417">
@@ -16022,7 +16022,7 @@
         <v>1800</v>
       </c>
       <c r="C1417" t="n">
-        <v>20624</v>
+        <v>21913</v>
       </c>
     </row>
     <row r="1418">
@@ -16033,7 +16033,7 @@
         <v>2362</v>
       </c>
       <c r="C1418" t="n">
-        <v>54544</v>
+        <v>57953</v>
       </c>
     </row>
     <row r="1419">
@@ -16044,7 +16044,7 @@
         <v>2449</v>
       </c>
       <c r="C1419" t="n">
-        <v>69088</v>
+        <v>73406</v>
       </c>
     </row>
     <row r="1420">
@@ -16055,7 +16055,7 @@
         <v>2844</v>
       </c>
       <c r="C1420" t="n">
-        <v>36352</v>
+        <v>38624</v>
       </c>
     </row>
     <row r="1421">
@@ -16066,7 +16066,7 @@
         <v>2507</v>
       </c>
       <c r="C1421" t="n">
-        <v>64960</v>
+        <v>69020</v>
       </c>
     </row>
     <row r="1422">
@@ -16077,7 +16077,7 @@
         <v>1906</v>
       </c>
       <c r="C1422" t="n">
-        <v>78960</v>
+        <v>83895</v>
       </c>
     </row>
     <row r="1423">
@@ -16099,7 +16099,7 @@
         <v>525</v>
       </c>
       <c r="C1424" t="n">
-        <v>170909.14</v>
+        <v>181590.95</v>
       </c>
     </row>
     <row r="1425">
@@ -16110,7 +16110,7 @@
         <v>1261</v>
       </c>
       <c r="C1425" t="n">
-        <v>51636.38</v>
+        <v>54863.65</v>
       </c>
     </row>
     <row r="1426">
@@ -16121,7 +16121,7 @@
         <v>2755</v>
       </c>
       <c r="C1426" t="n">
-        <v>36363.68</v>
+        <v>38636.4</v>
       </c>
     </row>
     <row r="1427">
@@ -16143,7 +16143,7 @@
         <v>1064</v>
       </c>
       <c r="C1428" t="n">
-        <v>436352</v>
+        <v>463624</v>
       </c>
     </row>
     <row r="1429">
@@ -16154,7 +16154,7 @@
         <v>1810</v>
       </c>
       <c r="C1429" t="n">
-        <v>29536</v>
+        <v>31382</v>
       </c>
     </row>
     <row r="1430">
@@ -16165,7 +16165,7 @@
         <v>1937</v>
       </c>
       <c r="C1430" t="n">
-        <v>188352</v>
+        <v>200124</v>
       </c>
     </row>
     <row r="1431">
@@ -16176,7 +16176,7 @@
         <v>483</v>
       </c>
       <c r="C1431" t="n">
-        <v>328720</v>
+        <v>349265</v>
       </c>
     </row>
     <row r="1432">
@@ -16187,7 +16187,7 @@
         <v>2580</v>
       </c>
       <c r="C1432" t="n">
-        <v>24496</v>
+        <v>26027</v>
       </c>
     </row>
     <row r="1433">
@@ -16198,7 +16198,7 @@
         <v>2706</v>
       </c>
       <c r="C1433" t="n">
-        <v>19136</v>
+        <v>20332</v>
       </c>
     </row>
     <row r="1434">
@@ -16209,7 +16209,7 @@
         <v>2633</v>
       </c>
       <c r="C1434" t="n">
-        <v>14016</v>
+        <v>14892</v>
       </c>
     </row>
     <row r="1435">
@@ -16242,7 +16242,7 @@
         <v>2392</v>
       </c>
       <c r="C1437" t="n">
-        <v>150848</v>
+        <v>160276</v>
       </c>
     </row>
     <row r="1438">
@@ -16264,7 +16264,7 @@
         <v>2613</v>
       </c>
       <c r="C1439" t="n">
-        <v>106208</v>
+        <v>112846</v>
       </c>
     </row>
     <row r="1440">
@@ -16275,7 +16275,7 @@
         <v>2183</v>
       </c>
       <c r="C1440" t="n">
-        <v>382416</v>
+        <v>406317</v>
       </c>
     </row>
     <row r="1441">
@@ -16286,7 +16286,7 @@
         <v>2541</v>
       </c>
       <c r="C1441" t="n">
-        <v>171920</v>
+        <v>182665</v>
       </c>
     </row>
     <row r="1442">
@@ -16297,7 +16297,7 @@
         <v>2333</v>
       </c>
       <c r="C1442" t="n">
-        <v>116064</v>
+        <v>123318</v>
       </c>
     </row>
     <row r="1443">
@@ -16308,7 +16308,7 @@
         <v>2813</v>
       </c>
       <c r="C1443" t="n">
-        <v>46400</v>
+        <v>49300</v>
       </c>
     </row>
     <row r="1444">
@@ -16319,7 +16319,7 @@
         <v>2811</v>
       </c>
       <c r="C1444" t="n">
-        <v>30256</v>
+        <v>32147</v>
       </c>
     </row>
     <row r="1445">
@@ -16330,7 +16330,7 @@
         <v>1881</v>
       </c>
       <c r="C1445" t="n">
-        <v>49952</v>
+        <v>53074</v>
       </c>
     </row>
     <row r="1446">
@@ -16341,7 +16341,7 @@
         <v>2825</v>
       </c>
       <c r="C1446" t="n">
-        <v>40608</v>
+        <v>43146</v>
       </c>
     </row>
     <row r="1447">
@@ -16352,7 +16352,7 @@
         <v>970</v>
       </c>
       <c r="C1447" t="n">
-        <v>49952</v>
+        <v>53074</v>
       </c>
     </row>
     <row r="1448">
@@ -16363,7 +16363,7 @@
         <v>2552</v>
       </c>
       <c r="C1448" t="n">
-        <v>28432</v>
+        <v>30209</v>
       </c>
     </row>
     <row r="1449">
@@ -16374,7 +16374,7 @@
         <v>2562</v>
       </c>
       <c r="C1449" t="n">
-        <v>28432</v>
+        <v>30209</v>
       </c>
     </row>
     <row r="1450">
@@ -16407,7 +16407,7 @@
         <v>2747</v>
       </c>
       <c r="C1452" t="n">
-        <v>50896</v>
+        <v>54077</v>
       </c>
     </row>
     <row r="1453">
@@ -16418,7 +16418,7 @@
         <v>415</v>
       </c>
       <c r="C1453" t="n">
-        <v>181818.22</v>
+        <v>193181.85</v>
       </c>
     </row>
     <row r="1454">
@@ -16462,7 +16462,7 @@
         <v>2544</v>
       </c>
       <c r="C1457" t="n">
-        <v>50896</v>
+        <v>54077</v>
       </c>
     </row>
     <row r="1458">
@@ -16473,7 +16473,7 @@
         <v>816</v>
       </c>
       <c r="C1458" t="n">
-        <v>218181.84</v>
+        <v>231818.2</v>
       </c>
     </row>
     <row r="1459">
@@ -16484,7 +16484,7 @@
         <v>890</v>
       </c>
       <c r="C1459" t="n">
-        <v>654545.46</v>
+        <v>695454.55</v>
       </c>
     </row>
     <row r="1460">
@@ -16495,7 +16495,7 @@
         <v>1298</v>
       </c>
       <c r="C1460" t="n">
-        <v>920000</v>
+        <v>977500</v>
       </c>
     </row>
     <row r="1461">
@@ -16506,7 +16506,7 @@
         <v>1372</v>
       </c>
       <c r="C1461" t="n">
-        <v>218181.84</v>
+        <v>231818.2</v>
       </c>
     </row>
     <row r="1462">
@@ -16517,7 +16517,7 @@
         <v>358</v>
       </c>
       <c r="C1462" t="n">
-        <v>229088</v>
+        <v>243406</v>
       </c>
     </row>
     <row r="1463">
@@ -16528,7 +16528,7 @@
         <v>1653</v>
       </c>
       <c r="C1463" t="n">
-        <v>229088</v>
+        <v>243406</v>
       </c>
     </row>
     <row r="1464">
@@ -16539,7 +16539,7 @@
         <v>675</v>
       </c>
       <c r="C1464" t="n">
-        <v>145440</v>
+        <v>154530</v>
       </c>
     </row>
     <row r="1465">
@@ -16550,7 +16550,7 @@
         <v>2804</v>
       </c>
       <c r="C1465" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1466">
@@ -16561,7 +16561,7 @@
         <v>2714</v>
       </c>
       <c r="C1466" t="n">
-        <v>261808</v>
+        <v>278171</v>
       </c>
     </row>
     <row r="1467">
@@ -16572,7 +16572,7 @@
         <v>2765</v>
       </c>
       <c r="C1467" t="n">
-        <v>65440</v>
+        <v>69530</v>
       </c>
     </row>
     <row r="1468">
@@ -16583,7 +16583,7 @@
         <v>2421</v>
       </c>
       <c r="C1468" t="n">
-        <v>44352</v>
+        <v>47124</v>
       </c>
     </row>
     <row r="1469">
@@ -16594,7 +16594,7 @@
         <v>2359</v>
       </c>
       <c r="C1469" t="n">
-        <v>75872</v>
+        <v>80614</v>
       </c>
     </row>
     <row r="1470">
@@ -16605,7 +16605,7 @@
         <v>2678</v>
       </c>
       <c r="C1470" t="n">
-        <v>71968</v>
+        <v>76466</v>
       </c>
     </row>
     <row r="1471">
@@ -16616,7 +16616,7 @@
         <v>2697</v>
       </c>
       <c r="C1471" t="n">
-        <v>109216</v>
+        <v>116042</v>
       </c>
     </row>
     <row r="1472">
@@ -16649,7 +16649,7 @@
         <v>2142</v>
       </c>
       <c r="C1474" t="n">
-        <v>39360</v>
+        <v>41820</v>
       </c>
     </row>
     <row r="1475">
@@ -16660,7 +16660,7 @@
         <v>2498</v>
       </c>
       <c r="C1475" t="n">
-        <v>40944</v>
+        <v>43503</v>
       </c>
     </row>
     <row r="1476">
@@ -16682,7 +16682,7 @@
         <v>2801</v>
       </c>
       <c r="C1477" t="n">
-        <v>72727.3</v>
+        <v>77272.75</v>
       </c>
     </row>
     <row r="1478">
@@ -16693,7 +16693,7 @@
         <v>2810</v>
       </c>
       <c r="C1478" t="n">
-        <v>116363.68</v>
+        <v>123636.4</v>
       </c>
     </row>
     <row r="1479">
@@ -16737,7 +16737,7 @@
         <v>132</v>
       </c>
       <c r="C1482" t="n">
-        <v>254545.46</v>
+        <v>270454.55</v>
       </c>
     </row>
     <row r="1483">
@@ -16759,7 +16759,7 @@
         <v>580</v>
       </c>
       <c r="C1484" t="n">
-        <v>127272.76</v>
+        <v>135227.3</v>
       </c>
     </row>
     <row r="1485">
@@ -16770,7 +16770,7 @@
         <v>634</v>
       </c>
       <c r="C1485" t="n">
-        <v>363636.38</v>
+        <v>386363.65</v>
       </c>
     </row>
     <row r="1486">
@@ -16792,7 +16792,7 @@
         <v>1277</v>
       </c>
       <c r="C1487" t="n">
-        <v>160000</v>
+        <v>170000</v>
       </c>
     </row>
     <row r="1488">
@@ -16803,7 +16803,7 @@
         <v>767</v>
       </c>
       <c r="C1488" t="n">
-        <v>145440</v>
+        <v>154530</v>
       </c>
     </row>
     <row r="1489">
@@ -16814,7 +16814,7 @@
         <v>2727</v>
       </c>
       <c r="C1489" t="n">
-        <v>29440</v>
+        <v>31280</v>
       </c>
     </row>
     <row r="1490">
@@ -16825,7 +16825,7 @@
         <v>2846</v>
       </c>
       <c r="C1490" t="n">
-        <v>189088</v>
+        <v>200906</v>
       </c>
     </row>
     <row r="1491">
@@ -16836,7 +16836,7 @@
         <v>609</v>
       </c>
       <c r="C1491" t="n">
-        <v>163632</v>
+        <v>173859</v>
       </c>
     </row>
     <row r="1492">
@@ -16847,7 +16847,7 @@
         <v>2726</v>
       </c>
       <c r="C1492" t="n">
-        <v>112720</v>
+        <v>119765</v>
       </c>
     </row>
     <row r="1493">
@@ -16858,7 +16858,7 @@
         <v>2729</v>
       </c>
       <c r="C1493" t="n">
-        <v>65440</v>
+        <v>69530</v>
       </c>
     </row>
     <row r="1494">
@@ -16869,7 +16869,7 @@
         <v>1340</v>
       </c>
       <c r="C1494" t="n">
-        <v>109088</v>
+        <v>115906</v>
       </c>
     </row>
     <row r="1495">
@@ -16880,7 +16880,7 @@
         <v>2830</v>
       </c>
       <c r="C1495" t="n">
-        <v>65440</v>
+        <v>69530</v>
       </c>
     </row>
     <row r="1496">
@@ -16891,7 +16891,7 @@
         <v>2674</v>
       </c>
       <c r="C1496" t="n">
-        <v>189088</v>
+        <v>200906</v>
       </c>
     </row>
     <row r="1497">
@@ -16902,7 +16902,7 @@
         <v>2308</v>
       </c>
       <c r="C1497" t="n">
-        <v>145440</v>
+        <v>154530</v>
       </c>
     </row>
     <row r="1498">
@@ -16913,7 +16913,7 @@
         <v>2190</v>
       </c>
       <c r="C1498" t="n">
-        <v>152720</v>
+        <v>162265</v>
       </c>
     </row>
     <row r="1499">
@@ -16924,7 +16924,7 @@
         <v>2015</v>
       </c>
       <c r="C1499" t="n">
-        <v>269088</v>
+        <v>285906</v>
       </c>
     </row>
     <row r="1500">
@@ -16935,7 +16935,7 @@
         <v>1308</v>
       </c>
       <c r="C1500" t="n">
-        <v>114176</v>
+        <v>121312</v>
       </c>
     </row>
     <row r="1501">
@@ -16946,7 +16946,7 @@
         <v>2118</v>
       </c>
       <c r="C1501" t="n">
-        <v>152848</v>
+        <v>162401</v>
       </c>
     </row>
     <row r="1502">
@@ -16957,7 +16957,7 @@
         <v>2607</v>
       </c>
       <c r="C1502" t="n">
-        <v>36128</v>
+        <v>38386</v>
       </c>
     </row>
     <row r="1503">
@@ -16968,7 +16968,7 @@
         <v>2832</v>
       </c>
       <c r="C1503" t="n">
-        <v>109090.92</v>
+        <v>115909.1</v>
       </c>
     </row>
     <row r="1504">
@@ -16979,7 +16979,7 @@
         <v>2383</v>
       </c>
       <c r="C1504" t="n">
-        <v>96672</v>
+        <v>102714</v>
       </c>
     </row>
     <row r="1505">
@@ -17012,7 +17012,7 @@
         <v>2821</v>
       </c>
       <c r="C1507" t="n">
-        <v>96976</v>
+        <v>103037</v>
       </c>
     </row>
     <row r="1508">
@@ -17034,7 +17034,7 @@
         <v>569</v>
       </c>
       <c r="C1509" t="n">
-        <v>2111584</v>
+        <v>2243558</v>
       </c>
     </row>
     <row r="1510">
@@ -17045,7 +17045,7 @@
         <v>2660</v>
       </c>
       <c r="C1510" t="n">
-        <v>254545.46</v>
+        <v>270454.55</v>
       </c>
     </row>
     <row r="1511">
@@ -17056,7 +17056,7 @@
         <v>1632</v>
       </c>
       <c r="C1511" t="n">
-        <v>189090.92</v>
+        <v>200909.1</v>
       </c>
     </row>
     <row r="1512">
@@ -17067,7 +17067,7 @@
         <v>1756</v>
       </c>
       <c r="C1512" t="n">
-        <v>305440</v>
+        <v>324530</v>
       </c>
     </row>
     <row r="1513">
@@ -17078,7 +17078,7 @@
         <v>58</v>
       </c>
       <c r="C1513" t="n">
-        <v>182400</v>
+        <v>193800</v>
       </c>
     </row>
     <row r="1514">
@@ -17089,7 +17089,7 @@
         <v>40</v>
       </c>
       <c r="C1514" t="n">
-        <v>162240</v>
+        <v>172380</v>
       </c>
     </row>
     <row r="1515">
@@ -17100,7 +17100,7 @@
         <v>559</v>
       </c>
       <c r="C1515" t="n">
-        <v>170176</v>
+        <v>180812</v>
       </c>
     </row>
     <row r="1516">
@@ -17111,7 +17111,7 @@
         <v>2773</v>
       </c>
       <c r="C1516" t="n">
-        <v>58672</v>
+        <v>62339</v>
       </c>
     </row>
     <row r="1517">
@@ -17122,7 +17122,7 @@
         <v>2631</v>
       </c>
       <c r="C1517" t="n">
-        <v>28176</v>
+        <v>29937</v>
       </c>
     </row>
     <row r="1518">
@@ -17133,7 +17133,7 @@
         <v>2085</v>
       </c>
       <c r="C1518" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1519">
@@ -17155,7 +17155,7 @@
         <v>1642</v>
       </c>
       <c r="C1520" t="n">
-        <v>192720</v>
+        <v>204765</v>
       </c>
     </row>
     <row r="1521">
@@ -17166,7 +17166,7 @@
         <v>2621</v>
       </c>
       <c r="C1521" t="n">
-        <v>50896</v>
+        <v>54077</v>
       </c>
     </row>
     <row r="1522">
@@ -17177,7 +17177,7 @@
         <v>2705</v>
       </c>
       <c r="C1522" t="n">
-        <v>146016</v>
+        <v>155142</v>
       </c>
     </row>
     <row r="1523">
@@ -17188,7 +17188,7 @@
         <v>2735</v>
       </c>
       <c r="C1523" t="n">
-        <v>87264</v>
+        <v>92718</v>
       </c>
     </row>
     <row r="1524">
@@ -17199,7 +17199,7 @@
         <v>945</v>
       </c>
       <c r="C1524" t="n">
-        <v>255040</v>
+        <v>270980</v>
       </c>
     </row>
     <row r="1525">
@@ -17210,7 +17210,7 @@
         <v>2582</v>
       </c>
       <c r="C1525" t="n">
-        <v>63808</v>
+        <v>67796</v>
       </c>
     </row>
     <row r="1526">
@@ -17221,7 +17221,7 @@
         <v>2584</v>
       </c>
       <c r="C1526" t="n">
-        <v>46400</v>
+        <v>49300</v>
       </c>
     </row>
     <row r="1527">
@@ -17232,7 +17232,7 @@
         <v>2689</v>
       </c>
       <c r="C1527" t="n">
-        <v>46400</v>
+        <v>49300</v>
       </c>
     </row>
     <row r="1528">
@@ -17243,7 +17243,7 @@
         <v>2574</v>
       </c>
       <c r="C1528" t="n">
-        <v>101984</v>
+        <v>108358</v>
       </c>
     </row>
     <row r="1529">
@@ -17254,7 +17254,7 @@
         <v>1834</v>
       </c>
       <c r="C1529" t="n">
-        <v>85600</v>
+        <v>90950</v>
       </c>
     </row>
     <row r="1530">
@@ -17265,7 +17265,7 @@
         <v>2629</v>
       </c>
       <c r="C1530" t="n">
-        <v>49952</v>
+        <v>53074</v>
       </c>
     </row>
     <row r="1531">
@@ -17276,7 +17276,7 @@
         <v>933</v>
       </c>
       <c r="C1531" t="n">
-        <v>59248</v>
+        <v>62951</v>
       </c>
     </row>
     <row r="1532">
@@ -17287,7 +17287,7 @@
         <v>2555</v>
       </c>
       <c r="C1532" t="n">
-        <v>28432</v>
+        <v>30209</v>
       </c>
     </row>
     <row r="1533">
@@ -17298,7 +17298,7 @@
         <v>2558</v>
       </c>
       <c r="C1533" t="n">
-        <v>28432</v>
+        <v>30209</v>
       </c>
     </row>
     <row r="1534">
@@ -17309,7 +17309,7 @@
         <v>2721</v>
       </c>
       <c r="C1534" t="n">
-        <v>59248</v>
+        <v>62951</v>
       </c>
     </row>
     <row r="1535">
@@ -17320,7 +17320,7 @@
         <v>2556</v>
       </c>
       <c r="C1535" t="n">
-        <v>28432</v>
+        <v>30209</v>
       </c>
     </row>
     <row r="1536">
@@ -17331,7 +17331,7 @@
         <v>2826</v>
       </c>
       <c r="C1536" t="n">
-        <v>50896</v>
+        <v>54077</v>
       </c>
     </row>
     <row r="1537">
@@ -17353,7 +17353,7 @@
         <v>2346</v>
       </c>
       <c r="C1538" t="n">
-        <v>50896</v>
+        <v>54077</v>
       </c>
     </row>
     <row r="1539">
@@ -17364,7 +17364,7 @@
         <v>595</v>
       </c>
       <c r="C1539" t="n">
-        <v>181818.22</v>
+        <v>193181.85</v>
       </c>
     </row>
     <row r="1540">
@@ -17375,7 +17375,7 @@
         <v>1278</v>
       </c>
       <c r="C1540" t="n">
-        <v>127272.76</v>
+        <v>135227.3</v>
       </c>
     </row>
     <row r="1541">
@@ -17386,7 +17386,7 @@
         <v>2686</v>
       </c>
       <c r="C1541" t="n">
-        <v>101808</v>
+        <v>108171</v>
       </c>
     </row>
     <row r="1542">
@@ -17397,7 +17397,7 @@
         <v>1344</v>
       </c>
       <c r="C1542" t="n">
-        <v>109088</v>
+        <v>115906</v>
       </c>
     </row>
     <row r="1543">
@@ -17408,7 +17408,7 @@
         <v>2566</v>
       </c>
       <c r="C1543" t="n">
-        <v>58176</v>
+        <v>61812</v>
       </c>
     </row>
     <row r="1544">
@@ -17419,7 +17419,7 @@
         <v>2684</v>
       </c>
       <c r="C1544" t="n">
-        <v>69088</v>
+        <v>73406</v>
       </c>
     </row>
     <row r="1545">
@@ -17430,7 +17430,7 @@
         <v>2375</v>
       </c>
       <c r="C1545" t="n">
-        <v>240000</v>
+        <v>255000</v>
       </c>
     </row>
     <row r="1546">
@@ -17441,7 +17441,7 @@
         <v>2829</v>
       </c>
       <c r="C1546" t="n">
-        <v>43632</v>
+        <v>46359</v>
       </c>
     </row>
     <row r="1547">
@@ -17452,7 +17452,7 @@
         <v>768</v>
       </c>
       <c r="C1547" t="n">
-        <v>101808</v>
+        <v>108171</v>
       </c>
     </row>
     <row r="1548">
@@ -17463,7 +17463,7 @@
         <v>772</v>
       </c>
       <c r="C1548" t="n">
-        <v>236352</v>
+        <v>251124</v>
       </c>
     </row>
     <row r="1549">
@@ -17474,7 +17474,7 @@
         <v>2496</v>
       </c>
       <c r="C1549" t="n">
-        <v>145440</v>
+        <v>154530</v>
       </c>
     </row>
     <row r="1550">
@@ -17485,7 +17485,7 @@
         <v>802</v>
       </c>
       <c r="C1550" t="n">
-        <v>54544</v>
+        <v>57953</v>
       </c>
     </row>
     <row r="1551">
@@ -17496,7 +17496,7 @@
         <v>2131</v>
       </c>
       <c r="C1551" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1552">
@@ -17507,7 +17507,7 @@
         <v>1381</v>
       </c>
       <c r="C1552" t="n">
-        <v>218181.84</v>
+        <v>231818.2</v>
       </c>
     </row>
     <row r="1553">
@@ -17518,7 +17518,7 @@
         <v>2847</v>
       </c>
       <c r="C1553" t="n">
-        <v>98176</v>
+        <v>104312</v>
       </c>
     </row>
     <row r="1554">
@@ -17529,7 +17529,7 @@
         <v>1293</v>
       </c>
       <c r="C1554" t="n">
-        <v>280000</v>
+        <v>297500</v>
       </c>
     </row>
     <row r="1555">
@@ -17540,7 +17540,7 @@
         <v>2363</v>
       </c>
       <c r="C1555" t="n">
-        <v>123632</v>
+        <v>131359</v>
       </c>
     </row>
     <row r="1556">
@@ -17551,7 +17551,7 @@
         <v>631</v>
       </c>
       <c r="C1556" t="n">
-        <v>254544</v>
+        <v>270453</v>
       </c>
     </row>
     <row r="1557">
@@ -17562,7 +17562,7 @@
         <v>2791</v>
       </c>
       <c r="C1557" t="n">
-        <v>74672</v>
+        <v>79339</v>
       </c>
     </row>
     <row r="1558">
@@ -17584,7 +17584,7 @@
         <v>2841</v>
       </c>
       <c r="C1559" t="n">
-        <v>36352</v>
+        <v>38624</v>
       </c>
     </row>
     <row r="1560">
@@ -17595,7 +17595,7 @@
         <v>2571</v>
       </c>
       <c r="C1560" t="n">
-        <v>193872</v>
+        <v>205989</v>
       </c>
     </row>
     <row r="1561">
@@ -17661,7 +17661,7 @@
         <v>2273</v>
       </c>
       <c r="C1566" t="n">
-        <v>156368</v>
+        <v>166141</v>
       </c>
     </row>
     <row r="1567">
@@ -17672,7 +17672,7 @@
         <v>2381</v>
       </c>
       <c r="C1567" t="n">
-        <v>58480</v>
+        <v>62135</v>
       </c>
     </row>
     <row r="1568">
@@ -17683,7 +17683,7 @@
         <v>630</v>
       </c>
       <c r="C1568" t="n">
-        <v>60021.79</v>
+        <v>63773.15</v>
       </c>
     </row>
     <row r="1569">
@@ -17705,7 +17705,7 @@
         <v>1983</v>
       </c>
       <c r="C1570" t="n">
-        <v>398720</v>
+        <v>423640</v>
       </c>
     </row>
     <row r="1571">
@@ -17716,7 +17716,7 @@
         <v>1993</v>
       </c>
       <c r="C1571" t="n">
-        <v>270752</v>
+        <v>287674</v>
       </c>
     </row>
     <row r="1572">
@@ -17727,7 +17727,7 @@
         <v>89</v>
       </c>
       <c r="C1572" t="n">
-        <v>254544</v>
+        <v>270453</v>
       </c>
     </row>
     <row r="1573">
@@ -17738,7 +17738,7 @@
         <v>1063</v>
       </c>
       <c r="C1573" t="n">
-        <v>280000</v>
+        <v>297500</v>
       </c>
     </row>
     <row r="1574">
@@ -17749,7 +17749,7 @@
         <v>1116</v>
       </c>
       <c r="C1574" t="n">
-        <v>181808</v>
+        <v>193171</v>
       </c>
     </row>
     <row r="1575">
@@ -17760,7 +17760,7 @@
         <v>941</v>
       </c>
       <c r="C1575" t="n">
-        <v>218832</v>
+        <v>232509</v>
       </c>
     </row>
     <row r="1576">
@@ -17771,7 +17771,7 @@
         <v>2141</v>
       </c>
       <c r="C1576" t="n">
-        <v>23328</v>
+        <v>24786</v>
       </c>
     </row>
     <row r="1577">
@@ -17782,7 +17782,7 @@
         <v>2463</v>
       </c>
       <c r="C1577" t="n">
-        <v>239872</v>
+        <v>254864</v>
       </c>
     </row>
     <row r="1578">
@@ -17793,7 +17793,7 @@
         <v>2707</v>
       </c>
       <c r="C1578" t="n">
-        <v>31408</v>
+        <v>33371</v>
       </c>
     </row>
     <row r="1579">
@@ -17804,7 +17804,7 @@
         <v>2325</v>
       </c>
       <c r="C1579" t="n">
-        <v>83904</v>
+        <v>89148</v>
       </c>
     </row>
     <row r="1580">
@@ -17848,7 +17848,7 @@
         <v>1890</v>
       </c>
       <c r="C1583" t="n">
-        <v>178352</v>
+        <v>189499</v>
       </c>
     </row>
     <row r="1584">
@@ -17859,7 +17859,7 @@
         <v>2639</v>
       </c>
       <c r="C1584" t="n">
-        <v>29136</v>
+        <v>30957</v>
       </c>
     </row>
     <row r="1585">
@@ -17870,7 +17870,7 @@
         <v>2682</v>
       </c>
       <c r="C1585" t="n">
-        <v>101808</v>
+        <v>108171</v>
       </c>
     </row>
     <row r="1586">
@@ -17881,7 +17881,7 @@
         <v>2601</v>
       </c>
       <c r="C1586" t="n">
-        <v>200000</v>
+        <v>212500</v>
       </c>
     </row>
     <row r="1587">
@@ -17892,7 +17892,7 @@
         <v>1142</v>
       </c>
       <c r="C1587" t="n">
-        <v>333152</v>
+        <v>353974</v>
       </c>
     </row>
     <row r="1588">
@@ -17936,7 +17936,7 @@
         <v>2082</v>
       </c>
       <c r="C1591" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1592">
@@ -17947,7 +17947,7 @@
         <v>2276</v>
       </c>
       <c r="C1592" t="n">
-        <v>144672</v>
+        <v>153714</v>
       </c>
     </row>
     <row r="1593">
@@ -17958,7 +17958,7 @@
         <v>2786</v>
       </c>
       <c r="C1593" t="n">
-        <v>50896</v>
+        <v>54077</v>
       </c>
     </row>
     <row r="1594">
@@ -17969,7 +17969,7 @@
         <v>2816</v>
       </c>
       <c r="C1594" t="n">
-        <v>94544</v>
+        <v>100453</v>
       </c>
     </row>
     <row r="1595">
@@ -17980,7 +17980,7 @@
         <v>1871</v>
       </c>
       <c r="C1595" t="n">
-        <v>104368</v>
+        <v>110891</v>
       </c>
     </row>
     <row r="1596">
@@ -17991,7 +17991,7 @@
         <v>2345</v>
       </c>
       <c r="C1596" t="n">
-        <v>46400</v>
+        <v>49300</v>
       </c>
     </row>
     <row r="1597">
@@ -18002,7 +18002,7 @@
         <v>2802</v>
       </c>
       <c r="C1597" t="n">
-        <v>52208</v>
+        <v>55471</v>
       </c>
     </row>
     <row r="1598">
@@ -18013,7 +18013,7 @@
         <v>2090</v>
       </c>
       <c r="C1598" t="n">
-        <v>30256</v>
+        <v>32147</v>
       </c>
     </row>
     <row r="1599">
@@ -18024,7 +18024,7 @@
         <v>2647</v>
       </c>
       <c r="C1599" t="n">
-        <v>102000</v>
+        <v>108375</v>
       </c>
     </row>
     <row r="1600">
@@ -18035,7 +18035,7 @@
         <v>2365</v>
       </c>
       <c r="C1600" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1601">
@@ -18046,7 +18046,7 @@
         <v>766</v>
       </c>
       <c r="C1601" t="n">
-        <v>49952</v>
+        <v>53074</v>
       </c>
     </row>
     <row r="1602">
@@ -18057,7 +18057,7 @@
         <v>2702</v>
       </c>
       <c r="C1602" t="n">
-        <v>59248</v>
+        <v>62951</v>
       </c>
     </row>
     <row r="1603">
@@ -18068,7 +18068,7 @@
         <v>20</v>
       </c>
       <c r="C1603" t="n">
-        <v>327272.76</v>
+        <v>347727.3</v>
       </c>
     </row>
     <row r="1604">
@@ -18079,7 +18079,7 @@
         <v>27</v>
       </c>
       <c r="C1604" t="n">
-        <v>109090.92</v>
+        <v>115909.1</v>
       </c>
     </row>
     <row r="1605">
@@ -18090,7 +18090,7 @@
         <v>33</v>
       </c>
       <c r="C1605" t="n">
-        <v>289440</v>
+        <v>307530</v>
       </c>
     </row>
     <row r="1606">
@@ -18112,7 +18112,7 @@
         <v>2561</v>
       </c>
       <c r="C1607" t="n">
-        <v>28432</v>
+        <v>30209</v>
       </c>
     </row>
     <row r="1608">
@@ -18134,7 +18134,7 @@
         <v>2772</v>
       </c>
       <c r="C1609" t="n">
-        <v>43632</v>
+        <v>46359</v>
       </c>
     </row>
     <row r="1610">
@@ -18145,7 +18145,7 @@
         <v>2834</v>
       </c>
       <c r="C1610" t="n">
-        <v>27104</v>
+        <v>28798</v>
       </c>
     </row>
     <row r="1611">
@@ -18156,7 +18156,7 @@
         <v>2394</v>
       </c>
       <c r="C1611" t="n">
-        <v>82512</v>
+        <v>87669</v>
       </c>
     </row>
     <row r="1612">
@@ -18167,7 +18167,7 @@
         <v>2567</v>
       </c>
       <c r="C1612" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1613">
@@ -18178,7 +18178,7 @@
         <v>952</v>
       </c>
       <c r="C1613" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1614">
@@ -18189,7 +18189,7 @@
         <v>1539</v>
       </c>
       <c r="C1614" t="n">
-        <v>123632</v>
+        <v>131359</v>
       </c>
     </row>
     <row r="1615">
@@ -18200,7 +18200,7 @@
         <v>793</v>
       </c>
       <c r="C1615" t="n">
-        <v>30256</v>
+        <v>32147</v>
       </c>
     </row>
     <row r="1616">
@@ -18211,7 +18211,7 @@
         <v>794</v>
       </c>
       <c r="C1616" t="n">
-        <v>30256</v>
+        <v>32147</v>
       </c>
     </row>
     <row r="1617">
@@ -18222,7 +18222,7 @@
         <v>2838</v>
       </c>
       <c r="C1617" t="n">
-        <v>43636.38</v>
+        <v>46363.65</v>
       </c>
     </row>
     <row r="1618">
@@ -18233,7 +18233,7 @@
         <v>2223</v>
       </c>
       <c r="C1618" t="n">
-        <v>85168</v>
+        <v>90491</v>
       </c>
     </row>
     <row r="1619">
@@ -18244,7 +18244,7 @@
         <v>2547</v>
       </c>
       <c r="C1619" t="n">
-        <v>24640</v>
+        <v>26180</v>
       </c>
     </row>
     <row r="1620">
@@ -18255,7 +18255,7 @@
         <v>2762</v>
       </c>
       <c r="C1620" t="n">
-        <v>59248</v>
+        <v>62951</v>
       </c>
     </row>
     <row r="1621">
@@ -18266,7 +18266,7 @@
         <v>2550</v>
       </c>
       <c r="C1621" t="n">
-        <v>28432</v>
+        <v>30209</v>
       </c>
     </row>
     <row r="1622">
@@ -18277,7 +18277,7 @@
         <v>2627</v>
       </c>
       <c r="C1622" t="n">
-        <v>28432</v>
+        <v>30209</v>
       </c>
     </row>
     <row r="1623">
@@ -18299,7 +18299,7 @@
         <v>749</v>
       </c>
       <c r="C1624" t="n">
-        <v>59248</v>
+        <v>62951</v>
       </c>
     </row>
     <row r="1625">
@@ -18310,7 +18310,7 @@
         <v>2549</v>
       </c>
       <c r="C1625" t="n">
-        <v>28432</v>
+        <v>30209</v>
       </c>
     </row>
     <row r="1626">
@@ -18321,7 +18321,7 @@
         <v>2649</v>
       </c>
       <c r="C1626" t="n">
-        <v>28432</v>
+        <v>30209</v>
       </c>
     </row>
     <row r="1627">
@@ -18332,7 +18332,7 @@
         <v>2258</v>
       </c>
       <c r="C1627" t="n">
-        <v>58176</v>
+        <v>61812</v>
       </c>
     </row>
     <row r="1628">
@@ -18343,7 +18343,7 @@
         <v>2744</v>
       </c>
       <c r="C1628" t="n">
-        <v>43632</v>
+        <v>46359</v>
       </c>
     </row>
     <row r="1629">
@@ -18354,7 +18354,7 @@
         <v>452</v>
       </c>
       <c r="C1629" t="n">
-        <v>205808</v>
+        <v>218671</v>
       </c>
     </row>
     <row r="1630">
@@ -18376,7 +18376,7 @@
         <v>2653</v>
       </c>
       <c r="C1631" t="n">
-        <v>43632</v>
+        <v>46359</v>
       </c>
     </row>
     <row r="1632">
@@ -18409,7 +18409,7 @@
         <v>2742</v>
       </c>
       <c r="C1634" t="n">
-        <v>14544</v>
+        <v>15453</v>
       </c>
     </row>
     <row r="1635">
@@ -18420,7 +18420,7 @@
         <v>1499</v>
       </c>
       <c r="C1635" t="n">
-        <v>65440</v>
+        <v>69530</v>
       </c>
     </row>
     <row r="1636">
@@ -18431,7 +18431,7 @@
         <v>2261</v>
       </c>
       <c r="C1636" t="n">
-        <v>130896</v>
+        <v>139077</v>
       </c>
     </row>
     <row r="1637">
@@ -18442,7 +18442,7 @@
         <v>1324</v>
       </c>
       <c r="C1637" t="n">
-        <v>203632</v>
+        <v>216359</v>
       </c>
     </row>
     <row r="1638">
@@ -18453,7 +18453,7 @@
         <v>2709</v>
       </c>
       <c r="C1638" t="n">
-        <v>130896</v>
+        <v>139077</v>
       </c>
     </row>
     <row r="1639">
@@ -18464,7 +18464,7 @@
         <v>1137</v>
       </c>
       <c r="C1639" t="n">
-        <v>465440</v>
+        <v>494530</v>
       </c>
     </row>
     <row r="1640">
@@ -18475,7 +18475,7 @@
         <v>2440</v>
       </c>
       <c r="C1640" t="n">
-        <v>58176</v>
+        <v>61812</v>
       </c>
     </row>
     <row r="1641">
@@ -18486,7 +18486,7 @@
         <v>429</v>
       </c>
       <c r="C1641" t="n">
-        <v>276352</v>
+        <v>293624</v>
       </c>
     </row>
     <row r="1642">
@@ -18497,7 +18497,7 @@
         <v>2114</v>
       </c>
       <c r="C1642" t="n">
-        <v>123728</v>
+        <v>131461</v>
       </c>
     </row>
     <row r="1643">
@@ -18508,7 +18508,7 @@
         <v>2211</v>
       </c>
       <c r="C1643" t="n">
-        <v>175152</v>
+        <v>186099</v>
       </c>
     </row>
     <row r="1644">
@@ -18519,7 +18519,7 @@
         <v>1108</v>
       </c>
       <c r="C1644" t="n">
-        <v>222816</v>
+        <v>236742</v>
       </c>
     </row>
     <row r="1645">
@@ -18530,7 +18530,7 @@
         <v>2695</v>
       </c>
       <c r="C1645" t="n">
-        <v>35184</v>
+        <v>37383</v>
       </c>
     </row>
     <row r="1646">
@@ -18541,7 +18541,7 @@
         <v>1289</v>
       </c>
       <c r="C1646" t="n">
-        <v>200000</v>
+        <v>212500</v>
       </c>
     </row>
     <row r="1647">
@@ -18552,7 +18552,7 @@
         <v>2789</v>
       </c>
       <c r="C1647" t="n">
-        <v>130909.14</v>
+        <v>139090.95</v>
       </c>
     </row>
     <row r="1648">
@@ -18563,7 +18563,7 @@
         <v>2197</v>
       </c>
       <c r="C1648" t="n">
-        <v>156363.68</v>
+        <v>166136.4</v>
       </c>
     </row>
     <row r="1649">
@@ -18574,7 +18574,7 @@
         <v>947</v>
       </c>
       <c r="C1649" t="n">
-        <v>322528</v>
+        <v>342686</v>
       </c>
     </row>
     <row r="1650">
@@ -18585,7 +18585,7 @@
         <v>2279</v>
       </c>
       <c r="C1650" t="n">
-        <v>178128</v>
+        <v>189261</v>
       </c>
     </row>
     <row r="1651">
@@ -18596,7 +18596,7 @@
         <v>1465</v>
       </c>
       <c r="C1651" t="n">
-        <v>280000</v>
+        <v>297500</v>
       </c>
     </row>
     <row r="1652">
@@ -18607,7 +18607,7 @@
         <v>2651</v>
       </c>
       <c r="C1652" t="n">
-        <v>123632</v>
+        <v>131359</v>
       </c>
     </row>
     <row r="1653">
@@ -18618,7 +18618,7 @@
         <v>42</v>
       </c>
       <c r="C1653" t="n">
-        <v>1386176</v>
+        <v>1472812</v>
       </c>
     </row>
     <row r="1654">
@@ -18629,7 +18629,7 @@
         <v>949</v>
       </c>
       <c r="C1654" t="n">
-        <v>72336</v>
+        <v>76857</v>
       </c>
     </row>
     <row r="1655">
@@ -18640,7 +18640,7 @@
         <v>2606</v>
       </c>
       <c r="C1655" t="n">
-        <v>186720</v>
+        <v>198390</v>
       </c>
     </row>
     <row r="1656">
@@ -18651,7 +18651,7 @@
         <v>2249</v>
       </c>
       <c r="C1656" t="n">
-        <v>158640</v>
+        <v>168555</v>
       </c>
     </row>
     <row r="1657">
@@ -18695,7 +18695,7 @@
         <v>2045</v>
       </c>
       <c r="C1660" t="n">
-        <v>231616</v>
+        <v>246092</v>
       </c>
     </row>
     <row r="1661">
@@ -18706,7 +18706,7 @@
         <v>2663</v>
       </c>
       <c r="C1661" t="n">
-        <v>200000</v>
+        <v>212500</v>
       </c>
     </row>
     <row r="1662">
@@ -18728,7 +18728,7 @@
         <v>2854</v>
       </c>
       <c r="C1663" t="n">
-        <v>29088</v>
+        <v>30906</v>
       </c>
     </row>
     <row r="1664">
@@ -18750,7 +18750,7 @@
         <v>2341</v>
       </c>
       <c r="C1665" t="n">
-        <v>127200</v>
+        <v>135150</v>
       </c>
     </row>
     <row r="1666">
@@ -18761,7 +18761,7 @@
         <v>2637</v>
       </c>
       <c r="C1666" t="n">
-        <v>46400</v>
+        <v>49300</v>
       </c>
     </row>
     <row r="1667">
@@ -18772,7 +18772,7 @@
         <v>2492</v>
       </c>
       <c r="C1667" t="n">
-        <v>72848</v>
+        <v>77401</v>
       </c>
     </row>
     <row r="1668">
@@ -18783,7 +18783,7 @@
         <v>2548</v>
       </c>
       <c r="C1668" t="n">
-        <v>28432</v>
+        <v>30209</v>
       </c>
     </row>
     <row r="1669">
@@ -18794,7 +18794,7 @@
         <v>351</v>
       </c>
       <c r="C1669" t="n">
-        <v>154896</v>
+        <v>164577</v>
       </c>
     </row>
     <row r="1670">
@@ -18827,7 +18827,7 @@
         <v>2757</v>
       </c>
       <c r="C1672" t="n">
-        <v>58176</v>
+        <v>61812</v>
       </c>
     </row>
     <row r="1673">
@@ -18838,7 +18838,7 @@
         <v>2815</v>
       </c>
       <c r="C1673" t="n">
-        <v>43632</v>
+        <v>46359</v>
       </c>
     </row>
     <row r="1674">
@@ -18849,7 +18849,7 @@
         <v>2323</v>
       </c>
       <c r="C1674" t="n">
-        <v>49952</v>
+        <v>53074</v>
       </c>
     </row>
     <row r="1675">
@@ -18860,7 +18860,7 @@
         <v>2310</v>
       </c>
       <c r="C1675" t="n">
-        <v>49952</v>
+        <v>53074</v>
       </c>
     </row>
     <row r="1676">
@@ -18871,7 +18871,7 @@
         <v>2145</v>
       </c>
       <c r="C1676" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1677">
@@ -18882,7 +18882,7 @@
         <v>2501</v>
       </c>
       <c r="C1677" t="n">
-        <v>59248</v>
+        <v>62951</v>
       </c>
     </row>
     <row r="1678">
@@ -18893,7 +18893,7 @@
         <v>2546</v>
       </c>
       <c r="C1678" t="n">
-        <v>28432</v>
+        <v>30209</v>
       </c>
     </row>
     <row r="1679">
@@ -18904,7 +18904,7 @@
         <v>716</v>
       </c>
       <c r="C1679" t="n">
-        <v>93216</v>
+        <v>99042</v>
       </c>
     </row>
     <row r="1680">
@@ -18915,7 +18915,7 @@
         <v>2758</v>
       </c>
       <c r="C1680" t="n">
-        <v>43632</v>
+        <v>46359</v>
       </c>
     </row>
     <row r="1681">
@@ -18926,7 +18926,7 @@
         <v>400</v>
       </c>
       <c r="C1681" t="n">
-        <v>130896</v>
+        <v>139077</v>
       </c>
     </row>
     <row r="1682">
@@ -18937,7 +18937,7 @@
         <v>6</v>
       </c>
       <c r="C1682" t="n">
-        <v>36363.68</v>
+        <v>38636.4</v>
       </c>
     </row>
     <row r="1683">
@@ -18970,7 +18970,7 @@
         <v>1259</v>
       </c>
       <c r="C1685" t="n">
-        <v>80000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="1686">
@@ -18981,7 +18981,7 @@
         <v>571</v>
       </c>
       <c r="C1686" t="n">
-        <v>752727.3</v>
+        <v>799772.75</v>
       </c>
     </row>
     <row r="1687">
@@ -18992,7 +18992,7 @@
         <v>703</v>
       </c>
       <c r="C1687" t="n">
-        <v>181808</v>
+        <v>193171</v>
       </c>
     </row>
     <row r="1688">
@@ -19014,7 +19014,7 @@
         <v>2833</v>
       </c>
       <c r="C1689" t="n">
-        <v>58176</v>
+        <v>61812</v>
       </c>
     </row>
     <row r="1690">
@@ -19025,7 +19025,7 @@
         <v>1007</v>
       </c>
       <c r="C1690" t="n">
-        <v>145454.6</v>
+        <v>154545.5</v>
       </c>
     </row>
     <row r="1691">
@@ -19036,7 +19036,7 @@
         <v>2687</v>
       </c>
       <c r="C1691" t="n">
-        <v>58176</v>
+        <v>61812</v>
       </c>
     </row>
     <row r="1692">
@@ -19047,7 +19047,7 @@
         <v>2824</v>
       </c>
       <c r="C1692" t="n">
-        <v>82112</v>
+        <v>87244</v>
       </c>
     </row>
     <row r="1693">
@@ -19058,7 +19058,7 @@
         <v>2730</v>
       </c>
       <c r="C1693" t="n">
-        <v>65440</v>
+        <v>69530</v>
       </c>
     </row>
     <row r="1694">
@@ -19069,7 +19069,7 @@
         <v>2718</v>
       </c>
       <c r="C1694" t="n">
-        <v>94544</v>
+        <v>100453</v>
       </c>
     </row>
     <row r="1695">
@@ -19080,7 +19080,7 @@
         <v>2750</v>
       </c>
       <c r="C1695" t="n">
-        <v>21808</v>
+        <v>23171</v>
       </c>
     </row>
     <row r="1696">
@@ -19091,7 +19091,7 @@
         <v>854</v>
       </c>
       <c r="C1696" t="n">
-        <v>101808</v>
+        <v>108171</v>
       </c>
     </row>
     <row r="1697">
@@ -19102,7 +19102,7 @@
         <v>2794</v>
       </c>
       <c r="C1697" t="n">
-        <v>87264</v>
+        <v>92718</v>
       </c>
     </row>
     <row r="1698">
@@ -19113,7 +19113,7 @@
         <v>1374</v>
       </c>
       <c r="C1698" t="n">
-        <v>145440</v>
+        <v>154530</v>
       </c>
     </row>
     <row r="1699">
@@ -19124,7 +19124,7 @@
         <v>2488</v>
       </c>
       <c r="C1699" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1700">
@@ -19135,7 +19135,7 @@
         <v>363</v>
       </c>
       <c r="C1700" t="n">
-        <v>218176</v>
+        <v>231812</v>
       </c>
     </row>
     <row r="1701">
@@ -19146,7 +19146,7 @@
         <v>2655</v>
       </c>
       <c r="C1701" t="n">
-        <v>80000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="1702">
@@ -19157,7 +19157,7 @@
         <v>1873</v>
       </c>
       <c r="C1702" t="n">
-        <v>232720</v>
+        <v>247265</v>
       </c>
     </row>
     <row r="1703">
@@ -19168,7 +19168,7 @@
         <v>2635</v>
       </c>
       <c r="C1703" t="n">
-        <v>94544</v>
+        <v>100453</v>
       </c>
     </row>
     <row r="1704">
@@ -19179,7 +19179,7 @@
         <v>1658</v>
       </c>
       <c r="C1704" t="n">
-        <v>111264</v>
+        <v>118218</v>
       </c>
     </row>
     <row r="1705">
@@ -19190,7 +19190,7 @@
         <v>2069</v>
       </c>
       <c r="C1705" t="n">
-        <v>145454.6</v>
+        <v>154545.5</v>
       </c>
     </row>
     <row r="1706">
@@ -19201,7 +19201,7 @@
         <v>2081</v>
       </c>
       <c r="C1706" t="n">
-        <v>109088</v>
+        <v>115906</v>
       </c>
     </row>
     <row r="1707">
@@ -19212,7 +19212,7 @@
         <v>2124</v>
       </c>
       <c r="C1707" t="n">
-        <v>254544</v>
+        <v>270453</v>
       </c>
     </row>
     <row r="1708">
@@ -19223,7 +19223,7 @@
         <v>636</v>
       </c>
       <c r="C1708" t="n">
-        <v>181808</v>
+        <v>193171</v>
       </c>
     </row>
     <row r="1709">
@@ -19234,7 +19234,7 @@
         <v>2803</v>
       </c>
       <c r="C1709" t="n">
-        <v>87264</v>
+        <v>92718</v>
       </c>
     </row>
     <row r="1710">
@@ -19245,7 +19245,7 @@
         <v>2163</v>
       </c>
       <c r="C1710" t="n">
-        <v>130896</v>
+        <v>139077</v>
       </c>
     </row>
     <row r="1711">
@@ -19256,7 +19256,7 @@
         <v>1466</v>
       </c>
       <c r="C1711" t="n">
-        <v>294544</v>
+        <v>312953</v>
       </c>
     </row>
     <row r="1712">
@@ -19267,7 +19267,7 @@
         <v>2133</v>
       </c>
       <c r="C1712" t="n">
-        <v>254545.46</v>
+        <v>270454.55</v>
       </c>
     </row>
     <row r="1713">
@@ -19278,7 +19278,7 @@
         <v>2431</v>
       </c>
       <c r="C1713" t="n">
-        <v>109088</v>
+        <v>115906</v>
       </c>
     </row>
     <row r="1714">
@@ -19289,7 +19289,7 @@
         <v>535</v>
       </c>
       <c r="C1714" t="n">
-        <v>259040</v>
+        <v>275230</v>
       </c>
     </row>
     <row r="1715">
@@ -19300,7 +19300,7 @@
         <v>2790</v>
       </c>
       <c r="C1715" t="n">
-        <v>45936</v>
+        <v>48807</v>
       </c>
     </row>
     <row r="1716">
@@ -19311,7 +19311,7 @@
         <v>2442</v>
       </c>
       <c r="C1716" t="n">
-        <v>188352</v>
+        <v>200124</v>
       </c>
     </row>
     <row r="1717">
@@ -19322,7 +19322,7 @@
         <v>2376</v>
       </c>
       <c r="C1717" t="n">
-        <v>800000</v>
+        <v>850000</v>
       </c>
     </row>
     <row r="1718">
@@ -19333,7 +19333,7 @@
         <v>2768</v>
       </c>
       <c r="C1718" t="n">
-        <v>220112</v>
+        <v>233869</v>
       </c>
     </row>
     <row r="1719">
@@ -19344,7 +19344,7 @@
         <v>2491</v>
       </c>
       <c r="C1719" t="n">
-        <v>176624</v>
+        <v>187663</v>
       </c>
     </row>
     <row r="1720">
@@ -19355,7 +19355,7 @@
         <v>2799</v>
       </c>
       <c r="C1720" t="n">
-        <v>79504</v>
+        <v>84473</v>
       </c>
     </row>
     <row r="1721">
@@ -19388,7 +19388,7 @@
         <v>1317</v>
       </c>
       <c r="C1723" t="n">
-        <v>229090.92</v>
+        <v>243409.1</v>
       </c>
     </row>
     <row r="1724">
@@ -19399,7 +19399,7 @@
         <v>2822</v>
       </c>
       <c r="C1724" t="n">
-        <v>116363.68</v>
+        <v>123636.4</v>
       </c>
     </row>
     <row r="1725">
@@ -19410,7 +19410,7 @@
         <v>1117</v>
       </c>
       <c r="C1725" t="n">
-        <v>290992</v>
+        <v>309179</v>
       </c>
     </row>
     <row r="1726">
@@ -19421,7 +19421,7 @@
         <v>1299</v>
       </c>
       <c r="C1726" t="n">
-        <v>383664</v>
+        <v>407643</v>
       </c>
     </row>
     <row r="1727">
@@ -19432,7 +19432,7 @@
         <v>477</v>
       </c>
       <c r="C1727" t="n">
-        <v>158112</v>
+        <v>167994</v>
       </c>
     </row>
     <row r="1728">
@@ -19443,7 +19443,7 @@
         <v>530</v>
       </c>
       <c r="C1728" t="n">
-        <v>218176</v>
+        <v>231812</v>
       </c>
     </row>
     <row r="1729">
@@ -19454,7 +19454,7 @@
         <v>953</v>
       </c>
       <c r="C1729" t="n">
-        <v>501808</v>
+        <v>533171</v>
       </c>
     </row>
     <row r="1730">
@@ -19465,7 +19465,7 @@
         <v>610</v>
       </c>
       <c r="C1730" t="n">
-        <v>597664</v>
+        <v>635018</v>
       </c>
     </row>
     <row r="1731">
@@ -19476,7 +19476,7 @@
         <v>2792</v>
       </c>
       <c r="C1731" t="n">
-        <v>150096</v>
+        <v>159477</v>
       </c>
     </row>
     <row r="1732">
@@ -19553,7 +19553,7 @@
         <v>1075</v>
       </c>
       <c r="C1738" t="n">
-        <v>333808</v>
+        <v>354671</v>
       </c>
     </row>
     <row r="1739">
@@ -19564,7 +19564,7 @@
         <v>131</v>
       </c>
       <c r="C1739" t="n">
-        <v>302544</v>
+        <v>321453</v>
       </c>
     </row>
     <row r="1740">
@@ -19575,7 +19575,7 @@
         <v>2667</v>
       </c>
       <c r="C1740" t="n">
-        <v>33232</v>
+        <v>35309</v>
       </c>
     </row>
     <row r="1741">
@@ -19586,7 +19586,7 @@
         <v>2330</v>
       </c>
       <c r="C1741" t="n">
-        <v>64688</v>
+        <v>68731</v>
       </c>
     </row>
     <row r="1742">
@@ -19608,7 +19608,7 @@
         <v>2577</v>
       </c>
       <c r="C1743" t="n">
-        <v>64848</v>
+        <v>68901</v>
       </c>
     </row>
     <row r="1744">
@@ -19619,7 +19619,7 @@
         <v>2510</v>
       </c>
       <c r="C1744" t="n">
-        <v>460544</v>
+        <v>489328</v>
       </c>
     </row>
     <row r="1745">
@@ -19641,7 +19641,7 @@
         <v>2850</v>
       </c>
       <c r="C1746" t="n">
-        <v>43632</v>
+        <v>46359</v>
       </c>
     </row>
     <row r="1747">
@@ -19663,7 +19663,7 @@
         <v>2745</v>
       </c>
       <c r="C1748" t="n">
-        <v>80000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="1749">
@@ -19674,7 +19674,7 @@
         <v>2817</v>
       </c>
       <c r="C1749" t="n">
-        <v>43632</v>
+        <v>46359</v>
       </c>
     </row>
     <row r="1750">
@@ -19685,7 +19685,7 @@
         <v>2784</v>
       </c>
       <c r="C1750" t="n">
-        <v>30256</v>
+        <v>32147</v>
       </c>
     </row>
     <row r="1751">
@@ -19696,7 +19696,7 @@
         <v>626</v>
       </c>
       <c r="C1751" t="n">
-        <v>1256592</v>
+        <v>1335129</v>
       </c>
     </row>
     <row r="1752">
@@ -19707,7 +19707,7 @@
         <v>925</v>
       </c>
       <c r="C1752" t="n">
-        <v>58016</v>
+        <v>61642</v>
       </c>
     </row>
     <row r="1753">
@@ -19718,7 +19718,7 @@
         <v>2586</v>
       </c>
       <c r="C1753" t="n">
-        <v>30256</v>
+        <v>32147</v>
       </c>
     </row>
     <row r="1754">
@@ -19729,7 +19729,7 @@
         <v>966</v>
       </c>
       <c r="C1754" t="n">
-        <v>59248</v>
+        <v>62951</v>
       </c>
     </row>
     <row r="1755">
@@ -19740,7 +19740,7 @@
         <v>2557</v>
       </c>
       <c r="C1755" t="n">
-        <v>28432</v>
+        <v>30209</v>
       </c>
     </row>
     <row r="1756">
@@ -19751,7 +19751,7 @@
         <v>14</v>
       </c>
       <c r="C1756" t="n">
-        <v>327264</v>
+        <v>347718</v>
       </c>
     </row>
     <row r="1757">
@@ -19762,7 +19762,7 @@
         <v>2798</v>
       </c>
       <c r="C1757" t="n">
-        <v>43632</v>
+        <v>46359</v>
       </c>
     </row>
     <row r="1758">
@@ -19784,7 +19784,7 @@
         <v>522</v>
       </c>
       <c r="C1759" t="n">
-        <v>145454.6</v>
+        <v>154545.5</v>
       </c>
     </row>
     <row r="1760">
@@ -19806,7 +19806,7 @@
         <v>2819</v>
       </c>
       <c r="C1761" t="n">
-        <v>43632</v>
+        <v>46359</v>
       </c>
     </row>
     <row r="1762">
@@ -19817,7 +19817,7 @@
         <v>2266</v>
       </c>
       <c r="C1762" t="n">
-        <v>58176</v>
+        <v>61812</v>
       </c>
     </row>
     <row r="1763">
@@ -19850,7 +19850,7 @@
         <v>2795</v>
       </c>
       <c r="C1765" t="n">
-        <v>43632</v>
+        <v>46359</v>
       </c>
     </row>
     <row r="1766">
@@ -19861,7 +19861,7 @@
         <v>2722</v>
       </c>
       <c r="C1766" t="n">
-        <v>14544</v>
+        <v>15453</v>
       </c>
     </row>
     <row r="1767">
@@ -19872,7 +19872,7 @@
         <v>951</v>
       </c>
       <c r="C1767" t="n">
-        <v>83632</v>
+        <v>88859</v>
       </c>
     </row>
     <row r="1768">
@@ -19883,7 +19883,7 @@
         <v>1020</v>
       </c>
       <c r="C1768" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1769">
@@ -19894,7 +19894,7 @@
         <v>1853</v>
       </c>
       <c r="C1769" t="n">
-        <v>87264</v>
+        <v>92718</v>
       </c>
     </row>
     <row r="1770">
@@ -19905,7 +19905,7 @@
         <v>1327</v>
       </c>
       <c r="C1770" t="n">
-        <v>50896</v>
+        <v>54077</v>
       </c>
     </row>
     <row r="1771">
@@ -19916,7 +19916,7 @@
         <v>2842</v>
       </c>
       <c r="C1771" t="n">
-        <v>130896</v>
+        <v>139077</v>
       </c>
     </row>
     <row r="1772">
@@ -19927,7 +19927,7 @@
         <v>2831</v>
       </c>
       <c r="C1772" t="n">
-        <v>43632</v>
+        <v>46359</v>
       </c>
     </row>
     <row r="1773">
@@ -19938,7 +19938,7 @@
         <v>818</v>
       </c>
       <c r="C1773" t="n">
-        <v>290896</v>
+        <v>309077</v>
       </c>
     </row>
     <row r="1774">
@@ -19949,7 +19949,7 @@
         <v>1501</v>
       </c>
       <c r="C1774" t="n">
-        <v>72720</v>
+        <v>77265</v>
       </c>
     </row>
     <row r="1775">
@@ -19960,7 +19960,7 @@
         <v>1869</v>
       </c>
       <c r="C1775" t="n">
-        <v>177440</v>
+        <v>188530</v>
       </c>
     </row>
     <row r="1776">
@@ -19971,7 +19971,7 @@
         <v>1996</v>
       </c>
       <c r="C1776" t="n">
-        <v>181818.22</v>
+        <v>193181.85</v>
       </c>
     </row>
     <row r="1777">
@@ -19982,7 +19982,7 @@
         <v>2462</v>
       </c>
       <c r="C1777" t="n">
-        <v>41189.14</v>
+        <v>43763.45</v>
       </c>
     </row>
     <row r="1778">
@@ -19993,7 +19993,7 @@
         <v>2696</v>
       </c>
       <c r="C1778" t="n">
-        <v>155968</v>
+        <v>165716</v>
       </c>
     </row>
     <row r="1779">
@@ -20004,7 +20004,7 @@
         <v>2698</v>
       </c>
       <c r="C1779" t="n">
-        <v>79936</v>
+        <v>84932</v>
       </c>
     </row>
     <row r="1780">
@@ -20026,7 +20026,7 @@
         <v>2828</v>
       </c>
       <c r="C1781" t="n">
-        <v>43636.38</v>
+        <v>46363.65</v>
       </c>
     </row>
     <row r="1782">
@@ -20037,7 +20037,7 @@
         <v>2843</v>
       </c>
       <c r="C1782" t="n">
-        <v>50896</v>
+        <v>54077</v>
       </c>
     </row>
     <row r="1783">
@@ -20048,7 +20048,7 @@
         <v>619</v>
       </c>
       <c r="C1783" t="n">
-        <v>228000</v>
+        <v>242250</v>
       </c>
     </row>
     <row r="1784">
@@ -20059,7 +20059,7 @@
         <v>1478</v>
       </c>
       <c r="C1784" t="n">
-        <v>399008</v>
+        <v>423946</v>
       </c>
     </row>
     <row r="1785">
@@ -20070,7 +20070,7 @@
         <v>2026</v>
       </c>
       <c r="C1785" t="n">
-        <v>176288</v>
+        <v>187306</v>
       </c>
     </row>
     <row r="1786">
@@ -20081,7 +20081,7 @@
         <v>663</v>
       </c>
       <c r="C1786" t="n">
-        <v>188352</v>
+        <v>200124</v>
       </c>
     </row>
     <row r="1787">
@@ -20092,7 +20092,7 @@
         <v>285</v>
       </c>
       <c r="C1787" t="n">
-        <v>399008</v>
+        <v>423946</v>
       </c>
     </row>
     <row r="1788">
@@ -20103,7 +20103,7 @@
         <v>424</v>
       </c>
       <c r="C1788" t="n">
-        <v>170992</v>
+        <v>181679</v>
       </c>
     </row>
     <row r="1789">
@@ -20114,7 +20114,7 @@
         <v>451</v>
       </c>
       <c r="C1789" t="n">
-        <v>176720</v>
+        <v>187765</v>
       </c>
     </row>
     <row r="1790">
@@ -20125,7 +20125,7 @@
         <v>629</v>
       </c>
       <c r="C1790" t="n">
-        <v>330176</v>
+        <v>350812</v>
       </c>
     </row>
     <row r="1791">
@@ -20136,7 +20136,7 @@
         <v>2657</v>
       </c>
       <c r="C1791" t="n">
-        <v>57584</v>
+        <v>61183</v>
       </c>
     </row>
     <row r="1792">
@@ -20147,7 +20147,7 @@
         <v>1254</v>
       </c>
       <c r="C1792" t="n">
-        <v>141232</v>
+        <v>150059</v>
       </c>
     </row>
     <row r="1793">
@@ -20158,7 +20158,7 @@
         <v>2402</v>
       </c>
       <c r="C1793" t="n">
-        <v>355232</v>
+        <v>377434</v>
       </c>
     </row>
     <row r="1794">
@@ -20169,7 +20169,7 @@
         <v>2413</v>
       </c>
       <c r="C1794" t="n">
-        <v>100240</v>
+        <v>106505</v>
       </c>
     </row>
     <row r="1795">
@@ -20180,7 +20180,7 @@
         <v>1450</v>
       </c>
       <c r="C1795" t="n">
-        <v>259632</v>
+        <v>275859</v>
       </c>
     </row>
     <row r="1796">
@@ -20202,7 +20202,7 @@
         <v>2671</v>
       </c>
       <c r="C1797" t="n">
-        <v>58176</v>
+        <v>61812</v>
       </c>
     </row>
     <row r="1798">
@@ -20213,7 +20213,7 @@
         <v>2568</v>
       </c>
       <c r="C1798" t="n">
-        <v>116688</v>
+        <v>123981</v>
       </c>
     </row>
     <row r="1799">
@@ -20224,7 +20224,7 @@
         <v>2146</v>
       </c>
       <c r="C1799" t="n">
-        <v>141296</v>
+        <v>150127</v>
       </c>
     </row>
     <row r="1800">
@@ -20235,7 +20235,7 @@
         <v>2753</v>
       </c>
       <c r="C1800" t="n">
-        <v>54544</v>
+        <v>57953</v>
       </c>
     </row>
     <row r="1801">
@@ -20246,7 +20246,7 @@
         <v>744</v>
       </c>
       <c r="C1801" t="n">
-        <v>30256</v>
+        <v>32147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:03:07
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -15560,7 +15560,7 @@
         <v>353</v>
       </c>
       <c r="C1375" t="n">
-        <v>239346</v>
+        <v>252643</v>
       </c>
     </row>
     <row r="1376">
@@ -15571,7 +15571,7 @@
         <v>2250</v>
       </c>
       <c r="C1376" t="n">
-        <v>278172</v>
+        <v>293626</v>
       </c>
     </row>
     <row r="1377">
@@ -15582,7 +15582,7 @@
         <v>1800</v>
       </c>
       <c r="C1377" t="n">
-        <v>23202</v>
+        <v>24491</v>
       </c>
     </row>
     <row r="1378">
@@ -15593,7 +15593,7 @@
         <v>2142</v>
       </c>
       <c r="C1378" t="n">
-        <v>46666.26</v>
+        <v>49258.82</v>
       </c>
     </row>
     <row r="1379">
@@ -15604,7 +15604,7 @@
         <v>2498</v>
       </c>
       <c r="C1379" t="n">
-        <v>48545.63</v>
+        <v>51242.6</v>
       </c>
     </row>
     <row r="1380">
@@ -15626,7 +15626,7 @@
         <v>2801</v>
       </c>
       <c r="C1381" t="n">
-        <v>81818.2</v>
+        <v>86363.64999999999</v>
       </c>
     </row>
     <row r="1382">
@@ -15637,7 +15637,7 @@
         <v>2810</v>
       </c>
       <c r="C1382" t="n">
-        <v>130909.12</v>
+        <v>138181.84</v>
       </c>
     </row>
     <row r="1383">
@@ -15681,7 +15681,7 @@
         <v>2853</v>
       </c>
       <c r="C1386" t="n">
-        <v>66654</v>
+        <v>70357</v>
       </c>
     </row>
     <row r="1387">
@@ -15692,7 +15692,7 @@
         <v>2245</v>
       </c>
       <c r="C1387" t="n">
-        <v>181152</v>
+        <v>191216</v>
       </c>
     </row>
     <row r="1388">
@@ -15703,7 +15703,7 @@
         <v>2251</v>
       </c>
       <c r="C1388" t="n">
-        <v>163620</v>
+        <v>172710</v>
       </c>
     </row>
     <row r="1389">
@@ -15714,7 +15714,7 @@
         <v>664</v>
       </c>
       <c r="C1389" t="n">
-        <v>214362</v>
+        <v>226271</v>
       </c>
     </row>
     <row r="1390">
@@ -15725,7 +15725,7 @@
         <v>2472</v>
       </c>
       <c r="C1390" t="n">
-        <v>43308</v>
+        <v>45714</v>
       </c>
     </row>
     <row r="1391">
@@ -15736,7 +15736,7 @@
         <v>1456</v>
       </c>
       <c r="C1391" t="n">
-        <v>652896</v>
+        <v>689168</v>
       </c>
     </row>
     <row r="1392">
@@ -15747,7 +15747,7 @@
         <v>1585</v>
       </c>
       <c r="C1392" t="n">
-        <v>148086</v>
+        <v>156313</v>
       </c>
     </row>
     <row r="1393">
@@ -15791,7 +15791,7 @@
         <v>1907</v>
       </c>
       <c r="C1396" t="n">
-        <v>450432</v>
+        <v>475456</v>
       </c>
     </row>
     <row r="1397">
@@ -15824,7 +15824,7 @@
         <v>2659</v>
       </c>
       <c r="C1399" t="n">
-        <v>100638</v>
+        <v>106229</v>
       </c>
     </row>
     <row r="1400">
@@ -15868,7 +15868,7 @@
         <v>2583</v>
       </c>
       <c r="C1403" t="n">
-        <v>34038</v>
+        <v>35929</v>
       </c>
     </row>
     <row r="1404">
@@ -15879,7 +15879,7 @@
         <v>2692</v>
       </c>
       <c r="C1404" t="n">
-        <v>57272.76</v>
+        <v>60454.57</v>
       </c>
     </row>
     <row r="1405">
@@ -15890,7 +15890,7 @@
         <v>2691</v>
       </c>
       <c r="C1405" t="n">
-        <v>99968.75999999999</v>
+        <v>105522.57</v>
       </c>
     </row>
     <row r="1406">
@@ -15923,7 +15923,7 @@
         <v>931</v>
       </c>
       <c r="C1408" t="n">
-        <v>78318</v>
+        <v>82669</v>
       </c>
     </row>
     <row r="1409">
@@ -15934,7 +15934,7 @@
         <v>2785</v>
       </c>
       <c r="C1409" t="n">
-        <v>34038</v>
+        <v>35929</v>
       </c>
     </row>
     <row r="1410">
@@ -15945,7 +15945,7 @@
         <v>2411</v>
       </c>
       <c r="C1410" t="n">
-        <v>81810</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1411">
@@ -15978,7 +15978,7 @@
         <v>2716</v>
       </c>
       <c r="C1413" t="n">
-        <v>71784</v>
+        <v>75772</v>
       </c>
     </row>
     <row r="1414">
@@ -15989,7 +15989,7 @@
         <v>2809</v>
       </c>
       <c r="C1414" t="n">
-        <v>56196</v>
+        <v>59318</v>
       </c>
     </row>
     <row r="1415">
@@ -16033,7 +16033,7 @@
         <v>104</v>
       </c>
       <c r="C1418" t="n">
-        <v>245454.56</v>
+        <v>259090.92</v>
       </c>
     </row>
     <row r="1419">
@@ -16088,7 +16088,7 @@
         <v>781</v>
       </c>
       <c r="C1423" t="n">
-        <v>106362</v>
+        <v>112271</v>
       </c>
     </row>
     <row r="1424">
@@ -16132,7 +16132,7 @@
         <v>2494</v>
       </c>
       <c r="C1427" t="n">
-        <v>122724</v>
+        <v>129542</v>
       </c>
     </row>
     <row r="1428">
@@ -16165,7 +16165,7 @@
         <v>2652</v>
       </c>
       <c r="C1430" t="n">
-        <v>114534</v>
+        <v>120897</v>
       </c>
     </row>
     <row r="1431">
@@ -16176,7 +16176,7 @@
         <v>1384</v>
       </c>
       <c r="C1431" t="n">
-        <v>286363.64</v>
+        <v>302272.73</v>
       </c>
     </row>
     <row r="1432">
@@ -16187,7 +16187,7 @@
         <v>360</v>
       </c>
       <c r="C1432" t="n">
-        <v>409086</v>
+        <v>431813</v>
       </c>
     </row>
     <row r="1433">
@@ -16198,7 +16198,7 @@
         <v>2767</v>
       </c>
       <c r="C1433" t="n">
-        <v>155448</v>
+        <v>164084</v>
       </c>
     </row>
     <row r="1434">
@@ -16209,7 +16209,7 @@
         <v>2178</v>
       </c>
       <c r="C1434" t="n">
-        <v>224181.84</v>
+        <v>236636.38</v>
       </c>
     </row>
     <row r="1435">
@@ -16220,7 +16220,7 @@
         <v>2107</v>
       </c>
       <c r="C1435" t="n">
-        <v>245430</v>
+        <v>259065</v>
       </c>
     </row>
     <row r="1436">
@@ -16231,7 +16231,7 @@
         <v>2711</v>
       </c>
       <c r="C1436" t="n">
-        <v>70830</v>
+        <v>74765</v>
       </c>
     </row>
     <row r="1437">
@@ -16242,7 +16242,7 @@
         <v>2845</v>
       </c>
       <c r="C1437" t="n">
-        <v>24545.48</v>
+        <v>25909.11</v>
       </c>
     </row>
     <row r="1438">
@@ -16286,7 +16286,7 @@
         <v>1102</v>
       </c>
       <c r="C1441" t="n">
-        <v>192366</v>
+        <v>203053</v>
       </c>
     </row>
     <row r="1442">
@@ -16297,7 +16297,7 @@
         <v>525</v>
       </c>
       <c r="C1442" t="n">
-        <v>192272.76</v>
+        <v>202954.57</v>
       </c>
     </row>
     <row r="1443">
@@ -16308,7 +16308,7 @@
         <v>1261</v>
       </c>
       <c r="C1443" t="n">
-        <v>58090.92</v>
+        <v>61318.19</v>
       </c>
     </row>
     <row r="1444">
@@ -16319,7 +16319,7 @@
         <v>2755</v>
       </c>
       <c r="C1444" t="n">
-        <v>40909.12</v>
+        <v>43181.84</v>
       </c>
     </row>
     <row r="1445">
@@ -16341,7 +16341,7 @@
         <v>783</v>
       </c>
       <c r="C1446" t="n">
-        <v>32727.28</v>
+        <v>34545.46</v>
       </c>
     </row>
     <row r="1447">
@@ -16352,7 +16352,7 @@
         <v>1064</v>
       </c>
       <c r="C1447" t="n">
-        <v>490896</v>
+        <v>518168</v>
       </c>
     </row>
     <row r="1448">
@@ -16363,7 +16363,7 @@
         <v>1810</v>
       </c>
       <c r="C1448" t="n">
-        <v>35033.34</v>
+        <v>36979.63</v>
       </c>
     </row>
     <row r="1449">
@@ -16374,7 +16374,7 @@
         <v>1937</v>
       </c>
       <c r="C1449" t="n">
-        <v>211896</v>
+        <v>223668</v>
       </c>
     </row>
     <row r="1450">
@@ -16385,7 +16385,7 @@
         <v>483</v>
       </c>
       <c r="C1450" t="n">
-        <v>369810</v>
+        <v>390355</v>
       </c>
     </row>
     <row r="1451">
@@ -16396,7 +16396,7 @@
         <v>2580</v>
       </c>
       <c r="C1451" t="n">
-        <v>27558</v>
+        <v>29089</v>
       </c>
     </row>
     <row r="1452">
@@ -16407,7 +16407,7 @@
         <v>2706</v>
       </c>
       <c r="C1452" t="n">
-        <v>21528</v>
+        <v>22724</v>
       </c>
     </row>
     <row r="1453">
@@ -16418,7 +16418,7 @@
         <v>2633</v>
       </c>
       <c r="C1453" t="n">
-        <v>15768</v>
+        <v>16644</v>
       </c>
     </row>
     <row r="1454">
@@ -16451,7 +16451,7 @@
         <v>2392</v>
       </c>
       <c r="C1456" t="n">
-        <v>169704</v>
+        <v>179132</v>
       </c>
     </row>
     <row r="1457">
@@ -16473,7 +16473,7 @@
         <v>2613</v>
       </c>
       <c r="C1458" t="n">
-        <v>119484</v>
+        <v>126122</v>
       </c>
     </row>
     <row r="1459">
@@ -16484,7 +16484,7 @@
         <v>2183</v>
       </c>
       <c r="C1459" t="n">
-        <v>430218</v>
+        <v>454119</v>
       </c>
     </row>
     <row r="1460">
@@ -16495,7 +16495,7 @@
         <v>2541</v>
       </c>
       <c r="C1460" t="n">
-        <v>193410</v>
+        <v>204155</v>
       </c>
     </row>
     <row r="1461">
@@ -16517,7 +16517,7 @@
         <v>2333</v>
       </c>
       <c r="C1462" t="n">
-        <v>130572</v>
+        <v>137826</v>
       </c>
     </row>
     <row r="1463">
@@ -16561,7 +16561,7 @@
         <v>2813</v>
       </c>
       <c r="C1466" t="n">
-        <v>52200</v>
+        <v>55100</v>
       </c>
     </row>
     <row r="1467">
@@ -16572,7 +16572,7 @@
         <v>2811</v>
       </c>
       <c r="C1467" t="n">
-        <v>34038</v>
+        <v>35929</v>
       </c>
     </row>
     <row r="1468">
@@ -16583,7 +16583,7 @@
         <v>1881</v>
       </c>
       <c r="C1468" t="n">
-        <v>56196</v>
+        <v>59318</v>
       </c>
     </row>
     <row r="1469">
@@ -16594,7 +16594,7 @@
         <v>2825</v>
       </c>
       <c r="C1469" t="n">
-        <v>45684</v>
+        <v>48222</v>
       </c>
     </row>
     <row r="1470">
@@ -16605,7 +16605,7 @@
         <v>970</v>
       </c>
       <c r="C1470" t="n">
-        <v>56196</v>
+        <v>59318</v>
       </c>
     </row>
     <row r="1471">
@@ -16616,7 +16616,7 @@
         <v>2552</v>
       </c>
       <c r="C1471" t="n">
-        <v>31986</v>
+        <v>33763</v>
       </c>
     </row>
     <row r="1472">
@@ -16627,7 +16627,7 @@
         <v>2562</v>
       </c>
       <c r="C1472" t="n">
-        <v>31986</v>
+        <v>33763</v>
       </c>
     </row>
     <row r="1473">
@@ -16704,7 +16704,7 @@
         <v>2747</v>
       </c>
       <c r="C1479" t="n">
-        <v>57258</v>
+        <v>60439</v>
       </c>
     </row>
     <row r="1480">
@@ -16792,7 +16792,7 @@
         <v>2544</v>
       </c>
       <c r="C1487" t="n">
-        <v>57258</v>
+        <v>60439</v>
       </c>
     </row>
     <row r="1488">
@@ -16803,7 +16803,7 @@
         <v>816</v>
       </c>
       <c r="C1488" t="n">
-        <v>245454.56</v>
+        <v>259090.92</v>
       </c>
     </row>
     <row r="1489">
@@ -16814,7 +16814,7 @@
         <v>890</v>
       </c>
       <c r="C1489" t="n">
-        <v>593181.84</v>
+        <v>626136.38</v>
       </c>
     </row>
     <row r="1490">
@@ -16836,7 +16836,7 @@
         <v>1298</v>
       </c>
       <c r="C1491" t="n">
-        <v>1035000</v>
+        <v>1092500</v>
       </c>
     </row>
     <row r="1492">
@@ -16847,7 +16847,7 @@
         <v>1372</v>
       </c>
       <c r="C1492" t="n">
-        <v>245454.56</v>
+        <v>259090.92</v>
       </c>
     </row>
     <row r="1493">
@@ -16858,7 +16858,7 @@
         <v>358</v>
       </c>
       <c r="C1493" t="n">
-        <v>257724</v>
+        <v>272042</v>
       </c>
     </row>
     <row r="1494">
@@ -16880,7 +16880,7 @@
         <v>1653</v>
       </c>
       <c r="C1495" t="n">
-        <v>257724</v>
+        <v>272042</v>
       </c>
     </row>
     <row r="1496">
@@ -16891,7 +16891,7 @@
         <v>675</v>
       </c>
       <c r="C1496" t="n">
-        <v>163620</v>
+        <v>172710</v>
       </c>
     </row>
     <row r="1497">
@@ -16902,7 +16902,7 @@
         <v>2804</v>
       </c>
       <c r="C1497" t="n">
-        <v>81810</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1498">
@@ -16913,7 +16913,7 @@
         <v>2714</v>
       </c>
       <c r="C1498" t="n">
-        <v>294534</v>
+        <v>310897</v>
       </c>
     </row>
     <row r="1499">
@@ -16924,7 +16924,7 @@
         <v>2765</v>
       </c>
       <c r="C1499" t="n">
-        <v>73620</v>
+        <v>77710</v>
       </c>
     </row>
     <row r="1500">
@@ -16935,7 +16935,7 @@
         <v>2421</v>
       </c>
       <c r="C1500" t="n">
-        <v>49909.12</v>
+        <v>52681.84</v>
       </c>
     </row>
     <row r="1501">
@@ -16946,7 +16946,7 @@
         <v>2359</v>
       </c>
       <c r="C1501" t="n">
-        <v>85356</v>
+        <v>90098</v>
       </c>
     </row>
     <row r="1502">
@@ -16957,7 +16957,7 @@
         <v>2678</v>
       </c>
       <c r="C1502" t="n">
-        <v>80964</v>
+        <v>85462</v>
       </c>
     </row>
     <row r="1503">
@@ -16968,7 +16968,7 @@
         <v>2697</v>
       </c>
       <c r="C1503" t="n">
-        <v>122868</v>
+        <v>129694</v>
       </c>
     </row>
     <row r="1504">
@@ -17001,7 +17001,7 @@
         <v>1308</v>
       </c>
       <c r="C1506" t="n">
-        <v>128448</v>
+        <v>135584</v>
       </c>
     </row>
     <row r="1507">
@@ -17012,7 +17012,7 @@
         <v>2118</v>
       </c>
       <c r="C1507" t="n">
-        <v>171954</v>
+        <v>181507</v>
       </c>
     </row>
     <row r="1508">
@@ -17023,7 +17023,7 @@
         <v>2607</v>
       </c>
       <c r="C1508" t="n">
-        <v>40644</v>
+        <v>42902</v>
       </c>
     </row>
     <row r="1509">
@@ -17034,7 +17034,7 @@
         <v>2832</v>
       </c>
       <c r="C1509" t="n">
-        <v>122727.28</v>
+        <v>129545.46</v>
       </c>
     </row>
     <row r="1510">
@@ -17045,7 +17045,7 @@
         <v>2383</v>
       </c>
       <c r="C1510" t="n">
-        <v>108756</v>
+        <v>114798</v>
       </c>
     </row>
     <row r="1511">
@@ -17078,7 +17078,7 @@
         <v>2821</v>
       </c>
       <c r="C1513" t="n">
-        <v>109098</v>
+        <v>115159</v>
       </c>
     </row>
     <row r="1514">
@@ -17100,7 +17100,7 @@
         <v>569</v>
       </c>
       <c r="C1515" t="n">
-        <v>2375532</v>
+        <v>2507506</v>
       </c>
     </row>
     <row r="1516">
@@ -17111,7 +17111,7 @@
         <v>2660</v>
       </c>
       <c r="C1516" t="n">
-        <v>286363.64</v>
+        <v>302272.73</v>
       </c>
     </row>
     <row r="1517">
@@ -17122,7 +17122,7 @@
         <v>1632</v>
       </c>
       <c r="C1517" t="n">
-        <v>212727.28</v>
+        <v>224545.46</v>
       </c>
     </row>
     <row r="1518">
@@ -17133,7 +17133,7 @@
         <v>1756</v>
       </c>
       <c r="C1518" t="n">
-        <v>343620</v>
+        <v>362710</v>
       </c>
     </row>
     <row r="1519">
@@ -17144,7 +17144,7 @@
         <v>58</v>
       </c>
       <c r="C1519" t="n">
-        <v>205200</v>
+        <v>216600</v>
       </c>
     </row>
     <row r="1520">
@@ -17155,7 +17155,7 @@
         <v>40</v>
       </c>
       <c r="C1520" t="n">
-        <v>182520</v>
+        <v>192660</v>
       </c>
     </row>
     <row r="1521">
@@ -17166,7 +17166,7 @@
         <v>559</v>
       </c>
       <c r="C1521" t="n">
-        <v>191448</v>
+        <v>202084</v>
       </c>
     </row>
     <row r="1522">
@@ -17177,7 +17177,7 @@
         <v>2773</v>
       </c>
       <c r="C1522" t="n">
-        <v>66006</v>
+        <v>69673</v>
       </c>
     </row>
     <row r="1523">
@@ -17188,7 +17188,7 @@
         <v>2631</v>
       </c>
       <c r="C1523" t="n">
-        <v>31698</v>
+        <v>33459</v>
       </c>
     </row>
     <row r="1524">
@@ -17199,7 +17199,7 @@
         <v>2085</v>
       </c>
       <c r="C1524" t="n">
-        <v>81810</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1525">
@@ -17221,7 +17221,7 @@
         <v>1642</v>
       </c>
       <c r="C1526" t="n">
-        <v>216810</v>
+        <v>228855</v>
       </c>
     </row>
     <row r="1527">
@@ -17232,7 +17232,7 @@
         <v>2621</v>
       </c>
       <c r="C1527" t="n">
-        <v>57258</v>
+        <v>60439</v>
       </c>
     </row>
     <row r="1528">
@@ -17243,7 +17243,7 @@
         <v>2705</v>
       </c>
       <c r="C1528" t="n">
-        <v>164268</v>
+        <v>173394</v>
       </c>
     </row>
     <row r="1529">
@@ -17276,7 +17276,7 @@
         <v>2735</v>
       </c>
       <c r="C1531" t="n">
-        <v>98172</v>
+        <v>103626</v>
       </c>
     </row>
     <row r="1532">
@@ -17287,7 +17287,7 @@
         <v>945</v>
       </c>
       <c r="C1532" t="n">
-        <v>286920</v>
+        <v>302860</v>
       </c>
     </row>
     <row r="1533">
@@ -17309,7 +17309,7 @@
         <v>2582</v>
       </c>
       <c r="C1534" t="n">
-        <v>71784</v>
+        <v>75772</v>
       </c>
     </row>
     <row r="1535">
@@ -17320,7 +17320,7 @@
         <v>2584</v>
       </c>
       <c r="C1535" t="n">
-        <v>52200</v>
+        <v>55100</v>
       </c>
     </row>
     <row r="1536">
@@ -17331,7 +17331,7 @@
         <v>2689</v>
       </c>
       <c r="C1536" t="n">
-        <v>52200</v>
+        <v>55100</v>
       </c>
     </row>
     <row r="1537">
@@ -17342,7 +17342,7 @@
         <v>2574</v>
       </c>
       <c r="C1537" t="n">
-        <v>114732</v>
+        <v>121106</v>
       </c>
     </row>
     <row r="1538">
@@ -17353,7 +17353,7 @@
         <v>1834</v>
       </c>
       <c r="C1538" t="n">
-        <v>96300</v>
+        <v>101650</v>
       </c>
     </row>
     <row r="1539">
@@ -17375,7 +17375,7 @@
         <v>2629</v>
       </c>
       <c r="C1540" t="n">
-        <v>56196</v>
+        <v>59318</v>
       </c>
     </row>
     <row r="1541">
@@ -17386,7 +17386,7 @@
         <v>933</v>
       </c>
       <c r="C1541" t="n">
-        <v>66654</v>
+        <v>70357</v>
       </c>
     </row>
     <row r="1542">
@@ -17397,7 +17397,7 @@
         <v>2555</v>
       </c>
       <c r="C1542" t="n">
-        <v>31986</v>
+        <v>33763</v>
       </c>
     </row>
     <row r="1543">
@@ -17408,7 +17408,7 @@
         <v>2558</v>
       </c>
       <c r="C1543" t="n">
-        <v>31986</v>
+        <v>33763</v>
       </c>
     </row>
     <row r="1544">
@@ -17430,7 +17430,7 @@
         <v>2721</v>
       </c>
       <c r="C1545" t="n">
-        <v>66654</v>
+        <v>70357</v>
       </c>
     </row>
     <row r="1546">
@@ -17441,7 +17441,7 @@
         <v>2556</v>
       </c>
       <c r="C1546" t="n">
-        <v>31986</v>
+        <v>33763</v>
       </c>
     </row>
     <row r="1547">
@@ -17463,7 +17463,7 @@
         <v>2826</v>
       </c>
       <c r="C1548" t="n">
-        <v>57258</v>
+        <v>60439</v>
       </c>
     </row>
     <row r="1549">
@@ -17485,7 +17485,7 @@
         <v>2346</v>
       </c>
       <c r="C1550" t="n">
-        <v>57258</v>
+        <v>60439</v>
       </c>
     </row>
     <row r="1551">
@@ -17496,7 +17496,7 @@
         <v>595</v>
       </c>
       <c r="C1551" t="n">
-        <v>204545.48</v>
+        <v>215909.11</v>
       </c>
     </row>
     <row r="1552">
@@ -17529,7 +17529,7 @@
         <v>1278</v>
       </c>
       <c r="C1554" t="n">
-        <v>143181.84</v>
+        <v>151136.38</v>
       </c>
     </row>
     <row r="1555">
@@ -17540,7 +17540,7 @@
         <v>2686</v>
       </c>
       <c r="C1555" t="n">
-        <v>114534</v>
+        <v>120897</v>
       </c>
     </row>
     <row r="1556">
@@ -17551,7 +17551,7 @@
         <v>1344</v>
       </c>
       <c r="C1556" t="n">
-        <v>122724</v>
+        <v>129542</v>
       </c>
     </row>
     <row r="1557">
@@ -17606,7 +17606,7 @@
         <v>2566</v>
       </c>
       <c r="C1561" t="n">
-        <v>65448</v>
+        <v>69084</v>
       </c>
     </row>
     <row r="1562">
@@ -17617,7 +17617,7 @@
         <v>2684</v>
       </c>
       <c r="C1562" t="n">
-        <v>77724</v>
+        <v>82042</v>
       </c>
     </row>
     <row r="1563">
@@ -17628,7 +17628,7 @@
         <v>2375</v>
       </c>
       <c r="C1563" t="n">
-        <v>270000</v>
+        <v>285000</v>
       </c>
     </row>
     <row r="1564">
@@ -17639,7 +17639,7 @@
         <v>2362</v>
       </c>
       <c r="C1564" t="n">
-        <v>61362</v>
+        <v>64771</v>
       </c>
     </row>
     <row r="1565">
@@ -17650,7 +17650,7 @@
         <v>2449</v>
       </c>
       <c r="C1565" t="n">
-        <v>77724</v>
+        <v>82042</v>
       </c>
     </row>
     <row r="1566">
@@ -17661,7 +17661,7 @@
         <v>2844</v>
       </c>
       <c r="C1566" t="n">
-        <v>24545.48</v>
+        <v>25909.11</v>
       </c>
     </row>
     <row r="1567">
@@ -17672,7 +17672,7 @@
         <v>2507</v>
       </c>
       <c r="C1567" t="n">
-        <v>73080</v>
+        <v>77140</v>
       </c>
     </row>
     <row r="1568">
@@ -17683,7 +17683,7 @@
         <v>1906</v>
       </c>
       <c r="C1568" t="n">
-        <v>88830</v>
+        <v>93765</v>
       </c>
     </row>
     <row r="1569">
@@ -17705,7 +17705,7 @@
         <v>1983</v>
       </c>
       <c r="C1570" t="n">
-        <v>448560</v>
+        <v>473480</v>
       </c>
     </row>
     <row r="1571">
@@ -17716,7 +17716,7 @@
         <v>1993</v>
       </c>
       <c r="C1571" t="n">
-        <v>304596</v>
+        <v>321518</v>
       </c>
     </row>
     <row r="1572">
@@ -17727,7 +17727,7 @@
         <v>89</v>
       </c>
       <c r="C1572" t="n">
-        <v>286362</v>
+        <v>302271</v>
       </c>
     </row>
     <row r="1573">
@@ -17738,7 +17738,7 @@
         <v>1063</v>
       </c>
       <c r="C1573" t="n">
-        <v>315000</v>
+        <v>332500</v>
       </c>
     </row>
     <row r="1574">
@@ -17749,7 +17749,7 @@
         <v>1116</v>
       </c>
       <c r="C1574" t="n">
-        <v>204534</v>
+        <v>215897</v>
       </c>
     </row>
     <row r="1575">
@@ -17760,7 +17760,7 @@
         <v>941</v>
       </c>
       <c r="C1575" t="n">
-        <v>246186</v>
+        <v>259863</v>
       </c>
     </row>
     <row r="1576">
@@ -17771,7 +17771,7 @@
         <v>2141</v>
       </c>
       <c r="C1576" t="n">
-        <v>27661.82</v>
+        <v>29198.58</v>
       </c>
     </row>
     <row r="1577">
@@ -17782,7 +17782,7 @@
         <v>2463</v>
       </c>
       <c r="C1577" t="n">
-        <v>269856</v>
+        <v>284848</v>
       </c>
     </row>
     <row r="1578">
@@ -17793,7 +17793,7 @@
         <v>2707</v>
       </c>
       <c r="C1578" t="n">
-        <v>35334</v>
+        <v>37297</v>
       </c>
     </row>
     <row r="1579">
@@ -17804,7 +17804,7 @@
         <v>2325</v>
       </c>
       <c r="C1579" t="n">
-        <v>94392</v>
+        <v>99636</v>
       </c>
     </row>
     <row r="1580">
@@ -17848,7 +17848,7 @@
         <v>1890</v>
       </c>
       <c r="C1583" t="n">
-        <v>200646</v>
+        <v>211793</v>
       </c>
     </row>
     <row r="1584">
@@ -17859,7 +17859,7 @@
         <v>2639</v>
       </c>
       <c r="C1584" t="n">
-        <v>32778</v>
+        <v>34599</v>
       </c>
     </row>
     <row r="1585">
@@ -17870,7 +17870,7 @@
         <v>2682</v>
       </c>
       <c r="C1585" t="n">
-        <v>114534</v>
+        <v>120897</v>
       </c>
     </row>
     <row r="1586">
@@ -17881,7 +17881,7 @@
         <v>2601</v>
       </c>
       <c r="C1586" t="n">
-        <v>225000</v>
+        <v>237500</v>
       </c>
     </row>
     <row r="1587">
@@ -17892,7 +17892,7 @@
         <v>1142</v>
       </c>
       <c r="C1587" t="n">
-        <v>374796</v>
+        <v>395618</v>
       </c>
     </row>
     <row r="1588">
@@ -17936,7 +17936,7 @@
         <v>2082</v>
       </c>
       <c r="C1591" t="n">
-        <v>81810</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1592">
@@ -17947,7 +17947,7 @@
         <v>2276</v>
       </c>
       <c r="C1592" t="n">
-        <v>162756</v>
+        <v>171798</v>
       </c>
     </row>
     <row r="1593">
@@ -17969,7 +17969,7 @@
         <v>2786</v>
       </c>
       <c r="C1594" t="n">
-        <v>57258</v>
+        <v>60439</v>
       </c>
     </row>
     <row r="1595">
@@ -17980,7 +17980,7 @@
         <v>2816</v>
       </c>
       <c r="C1595" t="n">
-        <v>106362</v>
+        <v>112271</v>
       </c>
     </row>
     <row r="1596">
@@ -17991,7 +17991,7 @@
         <v>1871</v>
       </c>
       <c r="C1596" t="n">
-        <v>117414</v>
+        <v>123937</v>
       </c>
     </row>
     <row r="1597">
@@ -18002,7 +18002,7 @@
         <v>2345</v>
       </c>
       <c r="C1597" t="n">
-        <v>52200</v>
+        <v>55100</v>
       </c>
     </row>
     <row r="1598">
@@ -18013,7 +18013,7 @@
         <v>2802</v>
       </c>
       <c r="C1598" t="n">
-        <v>58734</v>
+        <v>61997</v>
       </c>
     </row>
     <row r="1599">
@@ -18024,7 +18024,7 @@
         <v>2090</v>
       </c>
       <c r="C1599" t="n">
-        <v>34038</v>
+        <v>35929</v>
       </c>
     </row>
     <row r="1600">
@@ -18035,7 +18035,7 @@
         <v>2647</v>
       </c>
       <c r="C1600" t="n">
-        <v>114750</v>
+        <v>121125</v>
       </c>
     </row>
     <row r="1601">
@@ -18046,7 +18046,7 @@
         <v>2365</v>
       </c>
       <c r="C1601" t="n">
-        <v>81810</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1602">
@@ -18057,7 +18057,7 @@
         <v>766</v>
       </c>
       <c r="C1602" t="n">
-        <v>56196</v>
+        <v>59318</v>
       </c>
     </row>
     <row r="1603">
@@ -18068,7 +18068,7 @@
         <v>2702</v>
       </c>
       <c r="C1603" t="n">
-        <v>66654</v>
+        <v>70357</v>
       </c>
     </row>
     <row r="1604">
@@ -18090,7 +18090,7 @@
         <v>20</v>
       </c>
       <c r="C1605" t="n">
-        <v>368181.84</v>
+        <v>388636.38</v>
       </c>
     </row>
     <row r="1606">
@@ -18101,7 +18101,7 @@
         <v>27</v>
       </c>
       <c r="C1606" t="n">
-        <v>122727.28</v>
+        <v>129545.46</v>
       </c>
     </row>
     <row r="1607">
@@ -18112,7 +18112,7 @@
         <v>33</v>
       </c>
       <c r="C1607" t="n">
-        <v>325636.4</v>
+        <v>343727.3</v>
       </c>
     </row>
     <row r="1608">
@@ -18134,7 +18134,7 @@
         <v>2561</v>
       </c>
       <c r="C1609" t="n">
-        <v>31986</v>
+        <v>33763</v>
       </c>
     </row>
     <row r="1610">
@@ -18178,7 +18178,7 @@
         <v>2772</v>
       </c>
       <c r="C1613" t="n">
-        <v>49086</v>
+        <v>51813</v>
       </c>
     </row>
     <row r="1614">
@@ -18189,7 +18189,7 @@
         <v>132</v>
       </c>
       <c r="C1614" t="n">
-        <v>286363.64</v>
+        <v>302272.73</v>
       </c>
     </row>
     <row r="1615">
@@ -18211,7 +18211,7 @@
         <v>580</v>
       </c>
       <c r="C1616" t="n">
-        <v>143181.84</v>
+        <v>151136.38</v>
       </c>
     </row>
     <row r="1617">
@@ -18222,7 +18222,7 @@
         <v>634</v>
       </c>
       <c r="C1617" t="n">
-        <v>409090.92</v>
+        <v>431818.19</v>
       </c>
     </row>
     <row r="1618">
@@ -18244,7 +18244,7 @@
         <v>1277</v>
       </c>
       <c r="C1619" t="n">
-        <v>180000</v>
+        <v>190000</v>
       </c>
     </row>
     <row r="1620">
@@ -18255,7 +18255,7 @@
         <v>767</v>
       </c>
       <c r="C1620" t="n">
-        <v>163620</v>
+        <v>172710</v>
       </c>
     </row>
     <row r="1621">
@@ -18266,7 +18266,7 @@
         <v>2727</v>
       </c>
       <c r="C1621" t="n">
-        <v>33120</v>
+        <v>34960</v>
       </c>
     </row>
     <row r="1622">
@@ -18277,7 +18277,7 @@
         <v>2846</v>
       </c>
       <c r="C1622" t="n">
-        <v>212724</v>
+        <v>224542</v>
       </c>
     </row>
     <row r="1623">
@@ -18288,7 +18288,7 @@
         <v>609</v>
       </c>
       <c r="C1623" t="n">
-        <v>184086</v>
+        <v>194313</v>
       </c>
     </row>
     <row r="1624">
@@ -18299,7 +18299,7 @@
         <v>2726</v>
       </c>
       <c r="C1624" t="n">
-        <v>126810</v>
+        <v>133855</v>
       </c>
     </row>
     <row r="1625">
@@ -18321,7 +18321,7 @@
         <v>2729</v>
       </c>
       <c r="C1626" t="n">
-        <v>73620</v>
+        <v>77710</v>
       </c>
     </row>
     <row r="1627">
@@ -18332,7 +18332,7 @@
         <v>1340</v>
       </c>
       <c r="C1627" t="n">
-        <v>122724</v>
+        <v>129542</v>
       </c>
     </row>
     <row r="1628">
@@ -18343,7 +18343,7 @@
         <v>2830</v>
       </c>
       <c r="C1628" t="n">
-        <v>73620</v>
+        <v>77710</v>
       </c>
     </row>
     <row r="1629">
@@ -18365,7 +18365,7 @@
         <v>2674</v>
       </c>
       <c r="C1630" t="n">
-        <v>212724</v>
+        <v>224542</v>
       </c>
     </row>
     <row r="1631">
@@ -18376,7 +18376,7 @@
         <v>2308</v>
       </c>
       <c r="C1631" t="n">
-        <v>163620</v>
+        <v>172710</v>
       </c>
     </row>
     <row r="1632">
@@ -18387,7 +18387,7 @@
         <v>2190</v>
       </c>
       <c r="C1632" t="n">
-        <v>171818.2</v>
+        <v>181363.65</v>
       </c>
     </row>
     <row r="1633">
@@ -18398,7 +18398,7 @@
         <v>2015</v>
       </c>
       <c r="C1633" t="n">
-        <v>302724</v>
+        <v>319542</v>
       </c>
     </row>
     <row r="1634">
@@ -18409,7 +18409,7 @@
         <v>429</v>
       </c>
       <c r="C1634" t="n">
-        <v>310896</v>
+        <v>328168</v>
       </c>
     </row>
     <row r="1635">
@@ -18420,7 +18420,7 @@
         <v>2114</v>
       </c>
       <c r="C1635" t="n">
-        <v>139194</v>
+        <v>146927</v>
       </c>
     </row>
     <row r="1636">
@@ -18431,7 +18431,7 @@
         <v>2211</v>
       </c>
       <c r="C1636" t="n">
-        <v>197046</v>
+        <v>207993</v>
       </c>
     </row>
     <row r="1637">
@@ -18442,7 +18442,7 @@
         <v>1108</v>
       </c>
       <c r="C1637" t="n">
-        <v>250668</v>
+        <v>264594</v>
       </c>
     </row>
     <row r="1638">
@@ -18453,7 +18453,7 @@
         <v>2695</v>
       </c>
       <c r="C1638" t="n">
-        <v>41729.16</v>
+        <v>44047.44</v>
       </c>
     </row>
     <row r="1639">
@@ -18464,7 +18464,7 @@
         <v>1289</v>
       </c>
       <c r="C1639" t="n">
-        <v>225000</v>
+        <v>237500</v>
       </c>
     </row>
     <row r="1640">
@@ -18475,7 +18475,7 @@
         <v>2789</v>
       </c>
       <c r="C1640" t="n">
-        <v>147272.76</v>
+        <v>155454.57</v>
       </c>
     </row>
     <row r="1641">
@@ -18486,7 +18486,7 @@
         <v>2197</v>
       </c>
       <c r="C1641" t="n">
-        <v>175909.12</v>
+        <v>185681.84</v>
       </c>
     </row>
     <row r="1642">
@@ -18497,7 +18497,7 @@
         <v>947</v>
       </c>
       <c r="C1642" t="n">
-        <v>362844</v>
+        <v>383002</v>
       </c>
     </row>
     <row r="1643">
@@ -18508,7 +18508,7 @@
         <v>2279</v>
       </c>
       <c r="C1643" t="n">
-        <v>200394</v>
+        <v>211527</v>
       </c>
     </row>
     <row r="1644">
@@ -18519,7 +18519,7 @@
         <v>1465</v>
       </c>
       <c r="C1644" t="n">
-        <v>315000</v>
+        <v>332500</v>
       </c>
     </row>
     <row r="1645">
@@ -18530,7 +18530,7 @@
         <v>2651</v>
       </c>
       <c r="C1645" t="n">
-        <v>139086</v>
+        <v>146813</v>
       </c>
     </row>
     <row r="1646">
@@ -18541,7 +18541,7 @@
         <v>42</v>
       </c>
       <c r="C1646" t="n">
-        <v>1559448</v>
+        <v>1646084</v>
       </c>
     </row>
     <row r="1647">
@@ -18552,7 +18552,7 @@
         <v>949</v>
       </c>
       <c r="C1647" t="n">
-        <v>81378</v>
+        <v>85899</v>
       </c>
     </row>
     <row r="1648">
@@ -18563,7 +18563,7 @@
         <v>2606</v>
       </c>
       <c r="C1648" t="n">
-        <v>210060</v>
+        <v>221730</v>
       </c>
     </row>
     <row r="1649">
@@ -18574,7 +18574,7 @@
         <v>2249</v>
       </c>
       <c r="C1649" t="n">
-        <v>178470</v>
+        <v>188385</v>
       </c>
     </row>
     <row r="1650">
@@ -18618,7 +18618,7 @@
         <v>2045</v>
       </c>
       <c r="C1653" t="n">
-        <v>260568</v>
+        <v>275044</v>
       </c>
     </row>
     <row r="1654">
@@ -18629,7 +18629,7 @@
         <v>2663</v>
       </c>
       <c r="C1654" t="n">
-        <v>225000</v>
+        <v>237500</v>
       </c>
     </row>
     <row r="1655">
@@ -18651,7 +18651,7 @@
         <v>2854</v>
       </c>
       <c r="C1656" t="n">
-        <v>32724</v>
+        <v>34542</v>
       </c>
     </row>
     <row r="1657">
@@ -18684,7 +18684,7 @@
         <v>2341</v>
       </c>
       <c r="C1659" t="n">
-        <v>143100</v>
+        <v>151050</v>
       </c>
     </row>
     <row r="1660">
@@ -18695,7 +18695,7 @@
         <v>2637</v>
       </c>
       <c r="C1660" t="n">
-        <v>52200</v>
+        <v>55100</v>
       </c>
     </row>
     <row r="1661">
@@ -18706,7 +18706,7 @@
         <v>2492</v>
       </c>
       <c r="C1661" t="n">
-        <v>81954</v>
+        <v>86507</v>
       </c>
     </row>
     <row r="1662">
@@ -18739,7 +18739,7 @@
         <v>2548</v>
       </c>
       <c r="C1664" t="n">
-        <v>31986</v>
+        <v>33763</v>
       </c>
     </row>
     <row r="1665">
@@ -18750,7 +18750,7 @@
         <v>351</v>
       </c>
       <c r="C1665" t="n">
-        <v>174272.76</v>
+        <v>183954.57</v>
       </c>
     </row>
     <row r="1666">
@@ -18783,7 +18783,7 @@
         <v>2757</v>
       </c>
       <c r="C1668" t="n">
-        <v>65448</v>
+        <v>69084</v>
       </c>
     </row>
     <row r="1669">
@@ -18794,7 +18794,7 @@
         <v>2815</v>
       </c>
       <c r="C1669" t="n">
-        <v>49086</v>
+        <v>51813</v>
       </c>
     </row>
     <row r="1670">
@@ -18805,7 +18805,7 @@
         <v>2829</v>
       </c>
       <c r="C1670" t="n">
-        <v>49086</v>
+        <v>51813</v>
       </c>
     </row>
     <row r="1671">
@@ -18816,7 +18816,7 @@
         <v>768</v>
       </c>
       <c r="C1671" t="n">
-        <v>114534</v>
+        <v>120897</v>
       </c>
     </row>
     <row r="1672">
@@ -18827,7 +18827,7 @@
         <v>772</v>
       </c>
       <c r="C1672" t="n">
-        <v>265909.12</v>
+        <v>280681.84</v>
       </c>
     </row>
     <row r="1673">
@@ -18860,7 +18860,7 @@
         <v>2496</v>
       </c>
       <c r="C1675" t="n">
-        <v>163620</v>
+        <v>172710</v>
       </c>
     </row>
     <row r="1676">
@@ -18871,7 +18871,7 @@
         <v>802</v>
       </c>
       <c r="C1676" t="n">
-        <v>61362</v>
+        <v>64771</v>
       </c>
     </row>
     <row r="1677">
@@ -18893,7 +18893,7 @@
         <v>2131</v>
       </c>
       <c r="C1678" t="n">
-        <v>81810</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1679">
@@ -18904,7 +18904,7 @@
         <v>1381</v>
       </c>
       <c r="C1679" t="n">
-        <v>245454.56</v>
+        <v>259090.92</v>
       </c>
     </row>
     <row r="1680">
@@ -18915,7 +18915,7 @@
         <v>2847</v>
       </c>
       <c r="C1680" t="n">
-        <v>110448</v>
+        <v>116584</v>
       </c>
     </row>
     <row r="1681">
@@ -18926,7 +18926,7 @@
         <v>1293</v>
       </c>
       <c r="C1681" t="n">
-        <v>315000</v>
+        <v>332500</v>
       </c>
     </row>
     <row r="1682">
@@ -18948,7 +18948,7 @@
         <v>2363</v>
       </c>
       <c r="C1683" t="n">
-        <v>139086</v>
+        <v>146813</v>
       </c>
     </row>
     <row r="1684">
@@ -18959,7 +18959,7 @@
         <v>631</v>
       </c>
       <c r="C1684" t="n">
-        <v>286362</v>
+        <v>302271</v>
       </c>
     </row>
     <row r="1685">
@@ -18970,7 +18970,7 @@
         <v>2791</v>
       </c>
       <c r="C1685" t="n">
-        <v>84006</v>
+        <v>88673</v>
       </c>
     </row>
     <row r="1686">
@@ -18992,7 +18992,7 @@
         <v>2841</v>
       </c>
       <c r="C1687" t="n">
-        <v>40896</v>
+        <v>43168</v>
       </c>
     </row>
     <row r="1688">
@@ -19003,7 +19003,7 @@
         <v>2571</v>
       </c>
       <c r="C1688" t="n">
-        <v>218106</v>
+        <v>230223</v>
       </c>
     </row>
     <row r="1689">
@@ -19069,7 +19069,7 @@
         <v>2273</v>
       </c>
       <c r="C1694" t="n">
-        <v>185386.92</v>
+        <v>195686.19</v>
       </c>
     </row>
     <row r="1695">
@@ -19080,7 +19080,7 @@
         <v>2381</v>
       </c>
       <c r="C1695" t="n">
-        <v>69347.24000000001</v>
+        <v>73199.86</v>
       </c>
     </row>
     <row r="1696">
@@ -19091,7 +19091,7 @@
         <v>630</v>
       </c>
       <c r="C1696" t="n">
-        <v>67524.50999999999</v>
+        <v>71275.87</v>
       </c>
     </row>
     <row r="1697">
@@ -19113,7 +19113,7 @@
         <v>2768</v>
       </c>
       <c r="C1698" t="n">
-        <v>247626</v>
+        <v>261383</v>
       </c>
     </row>
     <row r="1699">
@@ -19124,7 +19124,7 @@
         <v>2491</v>
       </c>
       <c r="C1699" t="n">
-        <v>198702</v>
+        <v>209741</v>
       </c>
     </row>
     <row r="1700">
@@ -19135,7 +19135,7 @@
         <v>2799</v>
       </c>
       <c r="C1700" t="n">
-        <v>89442</v>
+        <v>94411</v>
       </c>
     </row>
     <row r="1701">
@@ -19168,7 +19168,7 @@
         <v>1317</v>
       </c>
       <c r="C1703" t="n">
-        <v>257727.28</v>
+        <v>272045.46</v>
       </c>
     </row>
     <row r="1704">
@@ -19179,7 +19179,7 @@
         <v>2822</v>
       </c>
       <c r="C1704" t="n">
-        <v>130909.12</v>
+        <v>138181.84</v>
       </c>
     </row>
     <row r="1705">
@@ -19190,7 +19190,7 @@
         <v>1117</v>
       </c>
       <c r="C1705" t="n">
-        <v>327366</v>
+        <v>345553</v>
       </c>
     </row>
     <row r="1706">
@@ -19201,7 +19201,7 @@
         <v>1299</v>
       </c>
       <c r="C1706" t="n">
-        <v>431622</v>
+        <v>455601</v>
       </c>
     </row>
     <row r="1707">
@@ -19212,7 +19212,7 @@
         <v>477</v>
       </c>
       <c r="C1707" t="n">
-        <v>177876</v>
+        <v>187758</v>
       </c>
     </row>
     <row r="1708">
@@ -19223,7 +19223,7 @@
         <v>530</v>
       </c>
       <c r="C1708" t="n">
-        <v>245448</v>
+        <v>259084</v>
       </c>
     </row>
     <row r="1709">
@@ -19234,7 +19234,7 @@
         <v>953</v>
       </c>
       <c r="C1709" t="n">
-        <v>564534</v>
+        <v>595897</v>
       </c>
     </row>
     <row r="1710">
@@ -19245,7 +19245,7 @@
         <v>610</v>
       </c>
       <c r="C1710" t="n">
-        <v>672372</v>
+        <v>709726</v>
       </c>
     </row>
     <row r="1711">
@@ -19256,7 +19256,7 @@
         <v>2792</v>
       </c>
       <c r="C1711" t="n">
-        <v>168858</v>
+        <v>178239</v>
       </c>
     </row>
     <row r="1712">
@@ -19333,7 +19333,7 @@
         <v>2834</v>
       </c>
       <c r="C1718" t="n">
-        <v>30492</v>
+        <v>32186</v>
       </c>
     </row>
     <row r="1719">
@@ -19344,7 +19344,7 @@
         <v>2394</v>
       </c>
       <c r="C1719" t="n">
-        <v>92826</v>
+        <v>97983</v>
       </c>
     </row>
     <row r="1720">
@@ -19355,7 +19355,7 @@
         <v>2567</v>
       </c>
       <c r="C1720" t="n">
-        <v>81810</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1721">
@@ -19366,7 +19366,7 @@
         <v>952</v>
       </c>
       <c r="C1721" t="n">
-        <v>81810</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1722">
@@ -19377,7 +19377,7 @@
         <v>1539</v>
       </c>
       <c r="C1722" t="n">
-        <v>139086</v>
+        <v>146813</v>
       </c>
     </row>
     <row r="1723">
@@ -19388,7 +19388,7 @@
         <v>793</v>
       </c>
       <c r="C1723" t="n">
-        <v>34038</v>
+        <v>35929</v>
       </c>
     </row>
     <row r="1724">
@@ -19399,7 +19399,7 @@
         <v>794</v>
       </c>
       <c r="C1724" t="n">
-        <v>34038</v>
+        <v>35929</v>
       </c>
     </row>
     <row r="1725">
@@ -19410,7 +19410,7 @@
         <v>2838</v>
       </c>
       <c r="C1725" t="n">
-        <v>49090.92</v>
+        <v>51818.19</v>
       </c>
     </row>
     <row r="1726">
@@ -19432,7 +19432,7 @@
         <v>2223</v>
       </c>
       <c r="C1727" t="n">
-        <v>95814</v>
+        <v>101137</v>
       </c>
     </row>
     <row r="1728">
@@ -19443,7 +19443,7 @@
         <v>2547</v>
       </c>
       <c r="C1728" t="n">
-        <v>27720</v>
+        <v>29260</v>
       </c>
     </row>
     <row r="1729">
@@ -19465,7 +19465,7 @@
         <v>2762</v>
       </c>
       <c r="C1730" t="n">
-        <v>66654</v>
+        <v>70357</v>
       </c>
     </row>
     <row r="1731">
@@ -19476,7 +19476,7 @@
         <v>2550</v>
       </c>
       <c r="C1731" t="n">
-        <v>31986</v>
+        <v>33763</v>
       </c>
     </row>
     <row r="1732">
@@ -19487,7 +19487,7 @@
         <v>2627</v>
       </c>
       <c r="C1732" t="n">
-        <v>31986</v>
+        <v>33763</v>
       </c>
     </row>
     <row r="1733">
@@ -19542,7 +19542,7 @@
         <v>749</v>
       </c>
       <c r="C1737" t="n">
-        <v>66654</v>
+        <v>70357</v>
       </c>
     </row>
     <row r="1738">
@@ -19553,7 +19553,7 @@
         <v>2549</v>
       </c>
       <c r="C1738" t="n">
-        <v>31986</v>
+        <v>33763</v>
       </c>
     </row>
     <row r="1739">
@@ -19564,7 +19564,7 @@
         <v>2649</v>
       </c>
       <c r="C1739" t="n">
-        <v>31986</v>
+        <v>33763</v>
       </c>
     </row>
     <row r="1740">
@@ -19575,7 +19575,7 @@
         <v>2258</v>
       </c>
       <c r="C1740" t="n">
-        <v>65448</v>
+        <v>69084</v>
       </c>
     </row>
     <row r="1741">
@@ -19586,7 +19586,7 @@
         <v>2744</v>
       </c>
       <c r="C1741" t="n">
-        <v>49086</v>
+        <v>51813</v>
       </c>
     </row>
     <row r="1742">
@@ -19597,7 +19597,7 @@
         <v>452</v>
       </c>
       <c r="C1742" t="n">
-        <v>231545.48</v>
+        <v>244409.11</v>
       </c>
     </row>
     <row r="1743">
@@ -19652,7 +19652,7 @@
         <v>2653</v>
       </c>
       <c r="C1747" t="n">
-        <v>49086</v>
+        <v>51813</v>
       </c>
     </row>
     <row r="1748">
@@ -19696,7 +19696,7 @@
         <v>2742</v>
       </c>
       <c r="C1751" t="n">
-        <v>16362</v>
+        <v>17271</v>
       </c>
     </row>
     <row r="1752">
@@ -19707,7 +19707,7 @@
         <v>1499</v>
       </c>
       <c r="C1752" t="n">
-        <v>73620</v>
+        <v>77710</v>
       </c>
     </row>
     <row r="1753">
@@ -19718,7 +19718,7 @@
         <v>2261</v>
       </c>
       <c r="C1753" t="n">
-        <v>147258</v>
+        <v>155439</v>
       </c>
     </row>
     <row r="1754">
@@ -19762,7 +19762,7 @@
         <v>1324</v>
       </c>
       <c r="C1757" t="n">
-        <v>229086</v>
+        <v>241813</v>
       </c>
     </row>
     <row r="1758">
@@ -19773,7 +19773,7 @@
         <v>2709</v>
       </c>
       <c r="C1758" t="n">
-        <v>147258</v>
+        <v>155439</v>
       </c>
     </row>
     <row r="1759">
@@ -19795,7 +19795,7 @@
         <v>1137</v>
       </c>
       <c r="C1760" t="n">
-        <v>523620</v>
+        <v>552710</v>
       </c>
     </row>
     <row r="1761">
@@ -19806,7 +19806,7 @@
         <v>2440</v>
       </c>
       <c r="C1761" t="n">
-        <v>65448</v>
+        <v>69084</v>
       </c>
     </row>
     <row r="1762">
@@ -19817,7 +19817,7 @@
         <v>2413</v>
       </c>
       <c r="C1762" t="n">
-        <v>112770</v>
+        <v>119035</v>
       </c>
     </row>
     <row r="1763">
@@ -19828,7 +19828,7 @@
         <v>1450</v>
       </c>
       <c r="C1763" t="n">
-        <v>292086</v>
+        <v>308313</v>
       </c>
     </row>
     <row r="1764">
@@ -19850,7 +19850,7 @@
         <v>2671</v>
       </c>
       <c r="C1765" t="n">
-        <v>65448</v>
+        <v>69084</v>
       </c>
     </row>
     <row r="1766">
@@ -19861,7 +19861,7 @@
         <v>2568</v>
       </c>
       <c r="C1766" t="n">
-        <v>131274</v>
+        <v>138567</v>
       </c>
     </row>
     <row r="1767">
@@ -19872,7 +19872,7 @@
         <v>2146</v>
       </c>
       <c r="C1767" t="n">
-        <v>158958</v>
+        <v>167789</v>
       </c>
     </row>
     <row r="1768">
@@ -19883,7 +19883,7 @@
         <v>2753</v>
       </c>
       <c r="C1768" t="n">
-        <v>61362</v>
+        <v>64771</v>
       </c>
     </row>
     <row r="1769">
@@ -19916,7 +19916,7 @@
         <v>744</v>
       </c>
       <c r="C1771" t="n">
-        <v>34038</v>
+        <v>35929</v>
       </c>
     </row>
     <row r="1772">
@@ -19927,7 +19927,7 @@
         <v>2323</v>
       </c>
       <c r="C1772" t="n">
-        <v>56196</v>
+        <v>59318</v>
       </c>
     </row>
     <row r="1773">
@@ -19938,7 +19938,7 @@
         <v>2310</v>
       </c>
       <c r="C1773" t="n">
-        <v>56196</v>
+        <v>59318</v>
       </c>
     </row>
     <row r="1774">
@@ -19949,7 +19949,7 @@
         <v>2145</v>
       </c>
       <c r="C1774" t="n">
-        <v>81810</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1775">
@@ -19960,7 +19960,7 @@
         <v>2858</v>
       </c>
       <c r="C1775" t="n">
-        <v>40909.12</v>
+        <v>43181.84</v>
       </c>
     </row>
     <row r="1776">
@@ -19993,7 +19993,7 @@
         <v>2501</v>
       </c>
       <c r="C1778" t="n">
-        <v>66654</v>
+        <v>70357</v>
       </c>
     </row>
     <row r="1779">
@@ -20004,7 +20004,7 @@
         <v>2546</v>
       </c>
       <c r="C1779" t="n">
-        <v>31986</v>
+        <v>33763</v>
       </c>
     </row>
     <row r="1780">
@@ -20026,7 +20026,7 @@
         <v>716</v>
       </c>
       <c r="C1781" t="n">
-        <v>104868</v>
+        <v>110694</v>
       </c>
     </row>
     <row r="1782">
@@ -20037,7 +20037,7 @@
         <v>2758</v>
       </c>
       <c r="C1782" t="n">
-        <v>49086</v>
+        <v>51813</v>
       </c>
     </row>
     <row r="1783">
@@ -20048,7 +20048,7 @@
         <v>400</v>
       </c>
       <c r="C1783" t="n">
-        <v>147272.76</v>
+        <v>155454.57</v>
       </c>
     </row>
     <row r="1784">
@@ -20059,7 +20059,7 @@
         <v>6</v>
       </c>
       <c r="C1784" t="n">
-        <v>40909.12</v>
+        <v>43181.84</v>
       </c>
     </row>
     <row r="1785">
@@ -20114,7 +20114,7 @@
         <v>1259</v>
       </c>
       <c r="C1789" t="n">
-        <v>90000</v>
+        <v>95000</v>
       </c>
     </row>
     <row r="1790">
@@ -20125,7 +20125,7 @@
         <v>571</v>
       </c>
       <c r="C1790" t="n">
-        <v>846818.2</v>
+        <v>893863.65</v>
       </c>
     </row>
     <row r="1791">
@@ -20136,7 +20136,7 @@
         <v>703</v>
       </c>
       <c r="C1791" t="n">
-        <v>204534</v>
+        <v>215897</v>
       </c>
     </row>
     <row r="1792">
@@ -20191,7 +20191,7 @@
         <v>2833</v>
       </c>
       <c r="C1796" t="n">
-        <v>65448</v>
+        <v>69084</v>
       </c>
     </row>
     <row r="1797">
@@ -20202,7 +20202,7 @@
         <v>1007</v>
       </c>
       <c r="C1797" t="n">
-        <v>163636.4</v>
+        <v>172727.3</v>
       </c>
     </row>
     <row r="1798">
@@ -20213,7 +20213,7 @@
         <v>2687</v>
       </c>
       <c r="C1798" t="n">
-        <v>65448</v>
+        <v>69084</v>
       </c>
     </row>
     <row r="1799">
@@ -20224,7 +20224,7 @@
         <v>2824</v>
       </c>
       <c r="C1799" t="n">
-        <v>92376</v>
+        <v>97508</v>
       </c>
     </row>
     <row r="1800">
@@ -20235,7 +20235,7 @@
         <v>2730</v>
       </c>
       <c r="C1800" t="n">
-        <v>73620</v>
+        <v>77710</v>
       </c>
     </row>
     <row r="1801">
@@ -20257,7 +20257,7 @@
         <v>2718</v>
       </c>
       <c r="C1802" t="n">
-        <v>106362</v>
+        <v>112271</v>
       </c>
     </row>
     <row r="1803">
@@ -20268,7 +20268,7 @@
         <v>2750</v>
       </c>
       <c r="C1803" t="n">
-        <v>24534</v>
+        <v>25897</v>
       </c>
     </row>
     <row r="1804">
@@ -20279,7 +20279,7 @@
         <v>854</v>
       </c>
       <c r="C1804" t="n">
-        <v>114534</v>
+        <v>120897</v>
       </c>
     </row>
     <row r="1805">
@@ -20290,7 +20290,7 @@
         <v>2794</v>
       </c>
       <c r="C1805" t="n">
-        <v>98172</v>
+        <v>103626</v>
       </c>
     </row>
     <row r="1806">
@@ -20301,7 +20301,7 @@
         <v>1374</v>
       </c>
       <c r="C1806" t="n">
-        <v>163620</v>
+        <v>172710</v>
       </c>
     </row>
     <row r="1807">
@@ -20312,7 +20312,7 @@
         <v>2488</v>
       </c>
       <c r="C1807" t="n">
-        <v>81810</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1808">
@@ -20323,7 +20323,7 @@
         <v>363</v>
       </c>
       <c r="C1808" t="n">
-        <v>245448</v>
+        <v>259084</v>
       </c>
     </row>
     <row r="1809">
@@ -20334,7 +20334,7 @@
         <v>2655</v>
       </c>
       <c r="C1809" t="n">
-        <v>90000</v>
+        <v>95000</v>
       </c>
     </row>
     <row r="1810">
@@ -20345,7 +20345,7 @@
         <v>1873</v>
       </c>
       <c r="C1810" t="n">
-        <v>261810</v>
+        <v>276355</v>
       </c>
     </row>
     <row r="1811">
@@ -20356,7 +20356,7 @@
         <v>2635</v>
       </c>
       <c r="C1811" t="n">
-        <v>106362</v>
+        <v>112271</v>
       </c>
     </row>
     <row r="1812">
@@ -20367,7 +20367,7 @@
         <v>1658</v>
       </c>
       <c r="C1812" t="n">
-        <v>125181.84</v>
+        <v>132136.38</v>
       </c>
     </row>
     <row r="1813">
@@ -20378,7 +20378,7 @@
         <v>2069</v>
       </c>
       <c r="C1813" t="n">
-        <v>163636.4</v>
+        <v>172727.3</v>
       </c>
     </row>
     <row r="1814">
@@ -20389,7 +20389,7 @@
         <v>2081</v>
       </c>
       <c r="C1814" t="n">
-        <v>122724</v>
+        <v>129542</v>
       </c>
     </row>
     <row r="1815">
@@ -20400,7 +20400,7 @@
         <v>2124</v>
       </c>
       <c r="C1815" t="n">
-        <v>286362</v>
+        <v>302271</v>
       </c>
     </row>
     <row r="1816">
@@ -20411,7 +20411,7 @@
         <v>636</v>
       </c>
       <c r="C1816" t="n">
-        <v>204534</v>
+        <v>215897</v>
       </c>
     </row>
     <row r="1817">
@@ -20422,7 +20422,7 @@
         <v>2803</v>
       </c>
       <c r="C1817" t="n">
-        <v>98172</v>
+        <v>103626</v>
       </c>
     </row>
     <row r="1818">
@@ -20433,7 +20433,7 @@
         <v>2163</v>
       </c>
       <c r="C1818" t="n">
-        <v>147258</v>
+        <v>155439</v>
       </c>
     </row>
     <row r="1819">
@@ -20444,7 +20444,7 @@
         <v>1466</v>
       </c>
       <c r="C1819" t="n">
-        <v>331362</v>
+        <v>349771</v>
       </c>
     </row>
     <row r="1820">
@@ -20455,7 +20455,7 @@
         <v>2133</v>
       </c>
       <c r="C1820" t="n">
-        <v>593181.84</v>
+        <v>626136.38</v>
       </c>
     </row>
     <row r="1821">
@@ -20466,7 +20466,7 @@
         <v>2431</v>
       </c>
       <c r="C1821" t="n">
-        <v>122727.28</v>
+        <v>129545.46</v>
       </c>
     </row>
     <row r="1822">
@@ -20477,7 +20477,7 @@
         <v>535</v>
       </c>
       <c r="C1822" t="n">
-        <v>291420</v>
+        <v>307610</v>
       </c>
     </row>
     <row r="1823">
@@ -20488,7 +20488,7 @@
         <v>2790</v>
       </c>
       <c r="C1823" t="n">
-        <v>51678</v>
+        <v>54549</v>
       </c>
     </row>
     <row r="1824">
@@ -20499,7 +20499,7 @@
         <v>2442</v>
       </c>
       <c r="C1824" t="n">
-        <v>211909.12</v>
+        <v>223681.84</v>
       </c>
     </row>
     <row r="1825">
@@ -20510,7 +20510,7 @@
         <v>2376</v>
       </c>
       <c r="C1825" t="n">
-        <v>900000</v>
+        <v>950000</v>
       </c>
     </row>
     <row r="1826">
@@ -20521,7 +20521,7 @@
         <v>1075</v>
       </c>
       <c r="C1826" t="n">
-        <v>375534</v>
+        <v>396397</v>
       </c>
     </row>
     <row r="1827">
@@ -20532,7 +20532,7 @@
         <v>131</v>
       </c>
       <c r="C1827" t="n">
-        <v>340362</v>
+        <v>359271</v>
       </c>
     </row>
     <row r="1828">
@@ -20543,7 +20543,7 @@
         <v>2667</v>
       </c>
       <c r="C1828" t="n">
-        <v>37386</v>
+        <v>39463</v>
       </c>
     </row>
     <row r="1829">
@@ -20554,7 +20554,7 @@
         <v>2330</v>
       </c>
       <c r="C1829" t="n">
-        <v>72774</v>
+        <v>76817</v>
       </c>
     </row>
     <row r="1830">
@@ -20576,7 +20576,7 @@
         <v>2577</v>
       </c>
       <c r="C1831" t="n">
-        <v>72954</v>
+        <v>77007</v>
       </c>
     </row>
     <row r="1832">
@@ -20587,7 +20587,7 @@
         <v>2510</v>
       </c>
       <c r="C1832" t="n">
-        <v>518112</v>
+        <v>546896</v>
       </c>
     </row>
     <row r="1833">
@@ -20609,7 +20609,7 @@
         <v>2850</v>
       </c>
       <c r="C1834" t="n">
-        <v>49086</v>
+        <v>51813</v>
       </c>
     </row>
     <row r="1835">
@@ -20631,7 +20631,7 @@
         <v>2745</v>
       </c>
       <c r="C1836" t="n">
-        <v>90000</v>
+        <v>95000</v>
       </c>
     </row>
     <row r="1837">
@@ -20642,7 +20642,7 @@
         <v>2817</v>
       </c>
       <c r="C1837" t="n">
-        <v>49086</v>
+        <v>51813</v>
       </c>
     </row>
     <row r="1838">
@@ -20664,7 +20664,7 @@
         <v>2784</v>
       </c>
       <c r="C1839" t="n">
-        <v>34038</v>
+        <v>35929</v>
       </c>
     </row>
     <row r="1840">
@@ -20686,7 +20686,7 @@
         <v>626</v>
       </c>
       <c r="C1841" t="n">
-        <v>1413666</v>
+        <v>1492203</v>
       </c>
     </row>
     <row r="1842">
@@ -20697,7 +20697,7 @@
         <v>925</v>
       </c>
       <c r="C1842" t="n">
-        <v>65268</v>
+        <v>68894</v>
       </c>
     </row>
     <row r="1843">
@@ -20708,7 +20708,7 @@
         <v>2586</v>
       </c>
       <c r="C1843" t="n">
-        <v>34038</v>
+        <v>35929</v>
       </c>
     </row>
     <row r="1844">
@@ -20741,7 +20741,7 @@
         <v>966</v>
       </c>
       <c r="C1846" t="n">
-        <v>66654</v>
+        <v>70357</v>
       </c>
     </row>
     <row r="1847">
@@ -20752,7 +20752,7 @@
         <v>2557</v>
       </c>
       <c r="C1847" t="n">
-        <v>31986</v>
+        <v>33763</v>
       </c>
     </row>
     <row r="1848">
@@ -20774,7 +20774,7 @@
         <v>14</v>
       </c>
       <c r="C1849" t="n">
-        <v>368172</v>
+        <v>388626</v>
       </c>
     </row>
     <row r="1850">
@@ -20796,7 +20796,7 @@
         <v>2798</v>
       </c>
       <c r="C1851" t="n">
-        <v>49086</v>
+        <v>51813</v>
       </c>
     </row>
     <row r="1852">
@@ -20818,7 +20818,7 @@
         <v>522</v>
       </c>
       <c r="C1853" t="n">
-        <v>163636.4</v>
+        <v>172727.3</v>
       </c>
     </row>
     <row r="1854">
@@ -20840,7 +20840,7 @@
         <v>2819</v>
       </c>
       <c r="C1855" t="n">
-        <v>49086</v>
+        <v>51813</v>
       </c>
     </row>
     <row r="1856">
@@ -20851,7 +20851,7 @@
         <v>2266</v>
       </c>
       <c r="C1856" t="n">
-        <v>65448</v>
+        <v>69084</v>
       </c>
     </row>
     <row r="1857">
@@ -20895,7 +20895,7 @@
         <v>2795</v>
       </c>
       <c r="C1860" t="n">
-        <v>49086</v>
+        <v>51813</v>
       </c>
     </row>
     <row r="1861">
@@ -20906,7 +20906,7 @@
         <v>2722</v>
       </c>
       <c r="C1861" t="n">
-        <v>16362</v>
+        <v>17271</v>
       </c>
     </row>
     <row r="1862">
@@ -20917,7 +20917,7 @@
         <v>951</v>
       </c>
       <c r="C1862" t="n">
-        <v>94086</v>
+        <v>99313</v>
       </c>
     </row>
     <row r="1863">
@@ -20928,7 +20928,7 @@
         <v>1020</v>
       </c>
       <c r="C1863" t="n">
-        <v>81810</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1864">
@@ -20950,7 +20950,7 @@
         <v>1853</v>
       </c>
       <c r="C1865" t="n">
-        <v>98172</v>
+        <v>103626</v>
       </c>
     </row>
     <row r="1866">
@@ -20961,7 +20961,7 @@
         <v>1327</v>
       </c>
       <c r="C1866" t="n">
-        <v>57258</v>
+        <v>60439</v>
       </c>
     </row>
     <row r="1867">
@@ -20972,7 +20972,7 @@
         <v>2842</v>
       </c>
       <c r="C1867" t="n">
-        <v>147258</v>
+        <v>155439</v>
       </c>
     </row>
     <row r="1868">
@@ -20983,7 +20983,7 @@
         <v>2831</v>
       </c>
       <c r="C1868" t="n">
-        <v>49086</v>
+        <v>51813</v>
       </c>
     </row>
     <row r="1869">
@@ -20994,7 +20994,7 @@
         <v>818</v>
       </c>
       <c r="C1869" t="n">
-        <v>327258</v>
+        <v>345439</v>
       </c>
     </row>
     <row r="1870">
@@ -21005,7 +21005,7 @@
         <v>1501</v>
       </c>
       <c r="C1870" t="n">
-        <v>81810</v>
+        <v>86355</v>
       </c>
     </row>
     <row r="1871">
@@ -21016,7 +21016,7 @@
         <v>1869</v>
       </c>
       <c r="C1871" t="n">
-        <v>199636.4</v>
+        <v>210727.3</v>
       </c>
     </row>
     <row r="1872">
@@ -21027,7 +21027,7 @@
         <v>1996</v>
       </c>
       <c r="C1872" t="n">
-        <v>204545.48</v>
+        <v>215909.11</v>
       </c>
     </row>
     <row r="1873">
@@ -21038,7 +21038,7 @@
         <v>2462</v>
       </c>
       <c r="C1873" t="n">
-        <v>46337.76</v>
+        <v>48912.07</v>
       </c>
     </row>
     <row r="1874">
@@ -21049,7 +21049,7 @@
         <v>2696</v>
       </c>
       <c r="C1874" t="n">
-        <v>175464</v>
+        <v>185212</v>
       </c>
     </row>
     <row r="1875">
@@ -21060,7 +21060,7 @@
         <v>2698</v>
       </c>
       <c r="C1875" t="n">
-        <v>89928</v>
+        <v>94924</v>
       </c>
     </row>
     <row r="1876">
@@ -21082,7 +21082,7 @@
         <v>2828</v>
       </c>
       <c r="C1877" t="n">
-        <v>49090.92</v>
+        <v>51818.19</v>
       </c>
     </row>
     <row r="1878">
@@ -21093,7 +21093,7 @@
         <v>2843</v>
       </c>
       <c r="C1878" t="n">
-        <v>57258</v>
+        <v>60439</v>
       </c>
     </row>
     <row r="1879">
@@ -21104,7 +21104,7 @@
         <v>619</v>
       </c>
       <c r="C1879" t="n">
-        <v>256500</v>
+        <v>270750</v>
       </c>
     </row>
     <row r="1880">
@@ -21115,7 +21115,7 @@
         <v>1478</v>
       </c>
       <c r="C1880" t="n">
-        <v>448884</v>
+        <v>473822</v>
       </c>
     </row>
     <row r="1881">
@@ -21126,7 +21126,7 @@
         <v>2026</v>
       </c>
       <c r="C1881" t="n">
-        <v>198324</v>
+        <v>209342</v>
       </c>
     </row>
     <row r="1882">
@@ -21137,7 +21137,7 @@
         <v>663</v>
       </c>
       <c r="C1882" t="n">
-        <v>211896</v>
+        <v>223668</v>
       </c>
     </row>
     <row r="1883">
@@ -21148,7 +21148,7 @@
         <v>285</v>
       </c>
       <c r="C1883" t="n">
-        <v>448884</v>
+        <v>473822</v>
       </c>
     </row>
     <row r="1884">
@@ -21159,7 +21159,7 @@
         <v>424</v>
       </c>
       <c r="C1884" t="n">
-        <v>192366</v>
+        <v>203053</v>
       </c>
     </row>
     <row r="1885">
@@ -21170,7 +21170,7 @@
         <v>451</v>
       </c>
       <c r="C1885" t="n">
-        <v>198810</v>
+        <v>209855</v>
       </c>
     </row>
     <row r="1886">
@@ -21181,7 +21181,7 @@
         <v>629</v>
       </c>
       <c r="C1886" t="n">
-        <v>371448</v>
+        <v>392084</v>
       </c>
     </row>
     <row r="1887">
@@ -21192,7 +21192,7 @@
         <v>2657</v>
       </c>
       <c r="C1887" t="n">
-        <v>64782</v>
+        <v>68381</v>
       </c>
     </row>
     <row r="1888">
@@ -21203,7 +21203,7 @@
         <v>1254</v>
       </c>
       <c r="C1888" t="n">
-        <v>158886</v>
+        <v>167713</v>
       </c>
     </row>
     <row r="1889">
@@ -21214,7 +21214,7 @@
         <v>2402</v>
       </c>
       <c r="C1889" t="n">
-        <v>399636</v>
+        <v>421838</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:02:38
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -15560,7 +15560,7 @@
         <v>353</v>
       </c>
       <c r="C1375" t="n">
-        <v>252643</v>
+        <v>265940</v>
       </c>
     </row>
     <row r="1376">
@@ -15571,7 +15571,7 @@
         <v>2250</v>
       </c>
       <c r="C1376" t="n">
-        <v>293626</v>
+        <v>309080</v>
       </c>
     </row>
     <row r="1377">
@@ -15582,7 +15582,7 @@
         <v>1800</v>
       </c>
       <c r="C1377" t="n">
-        <v>24491</v>
+        <v>25780</v>
       </c>
     </row>
     <row r="1378">
@@ -15593,7 +15593,7 @@
         <v>2142</v>
       </c>
       <c r="C1378" t="n">
-        <v>49258.82</v>
+        <v>51851.38</v>
       </c>
     </row>
     <row r="1379">
@@ -15604,7 +15604,7 @@
         <v>2498</v>
       </c>
       <c r="C1379" t="n">
-        <v>51242.6</v>
+        <v>53939.57</v>
       </c>
     </row>
     <row r="1380">
@@ -15626,7 +15626,7 @@
         <v>2801</v>
       </c>
       <c r="C1381" t="n">
-        <v>86363.64999999999</v>
+        <v>90909.10000000001</v>
       </c>
     </row>
     <row r="1382">
@@ -15637,7 +15637,7 @@
         <v>2810</v>
       </c>
       <c r="C1382" t="n">
-        <v>138181.84</v>
+        <v>145454.56</v>
       </c>
     </row>
     <row r="1383">
@@ -15681,7 +15681,7 @@
         <v>2853</v>
       </c>
       <c r="C1386" t="n">
-        <v>70357</v>
+        <v>74060</v>
       </c>
     </row>
     <row r="1387">
@@ -15692,7 +15692,7 @@
         <v>2245</v>
       </c>
       <c r="C1387" t="n">
-        <v>191216</v>
+        <v>201280</v>
       </c>
     </row>
     <row r="1388">
@@ -15703,7 +15703,7 @@
         <v>2251</v>
       </c>
       <c r="C1388" t="n">
-        <v>172710</v>
+        <v>181800</v>
       </c>
     </row>
     <row r="1389">
@@ -15714,7 +15714,7 @@
         <v>664</v>
       </c>
       <c r="C1389" t="n">
-        <v>226271</v>
+        <v>238180</v>
       </c>
     </row>
     <row r="1390">
@@ -15725,7 +15725,7 @@
         <v>2472</v>
       </c>
       <c r="C1390" t="n">
-        <v>45714</v>
+        <v>48120</v>
       </c>
     </row>
     <row r="1391">
@@ -15736,7 +15736,7 @@
         <v>1456</v>
       </c>
       <c r="C1391" t="n">
-        <v>689168</v>
+        <v>725440</v>
       </c>
     </row>
     <row r="1392">
@@ -15747,7 +15747,7 @@
         <v>1585</v>
       </c>
       <c r="C1392" t="n">
-        <v>156313</v>
+        <v>164540</v>
       </c>
     </row>
     <row r="1393">
@@ -15791,7 +15791,7 @@
         <v>1907</v>
       </c>
       <c r="C1396" t="n">
-        <v>475456</v>
+        <v>500480</v>
       </c>
     </row>
     <row r="1397">
@@ -15824,7 +15824,7 @@
         <v>2659</v>
       </c>
       <c r="C1399" t="n">
-        <v>106229</v>
+        <v>111820</v>
       </c>
     </row>
     <row r="1400">
@@ -15868,7 +15868,7 @@
         <v>2583</v>
       </c>
       <c r="C1403" t="n">
-        <v>35929</v>
+        <v>37820</v>
       </c>
     </row>
     <row r="1404">
@@ -15879,7 +15879,7 @@
         <v>2692</v>
       </c>
       <c r="C1404" t="n">
-        <v>60454.57</v>
+        <v>63636.38</v>
       </c>
     </row>
     <row r="1405">
@@ -15890,7 +15890,7 @@
         <v>2691</v>
       </c>
       <c r="C1405" t="n">
-        <v>105522.57</v>
+        <v>111076.38</v>
       </c>
     </row>
     <row r="1406">
@@ -15923,7 +15923,7 @@
         <v>931</v>
       </c>
       <c r="C1408" t="n">
-        <v>82669</v>
+        <v>87020</v>
       </c>
     </row>
     <row r="1409">
@@ -15934,7 +15934,7 @@
         <v>2785</v>
       </c>
       <c r="C1409" t="n">
-        <v>35929</v>
+        <v>37820</v>
       </c>
     </row>
     <row r="1410">
@@ -15945,7 +15945,7 @@
         <v>2411</v>
       </c>
       <c r="C1410" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1411">
@@ -15978,7 +15978,7 @@
         <v>2716</v>
       </c>
       <c r="C1413" t="n">
-        <v>75772</v>
+        <v>79760</v>
       </c>
     </row>
     <row r="1414">
@@ -15989,7 +15989,7 @@
         <v>2809</v>
       </c>
       <c r="C1414" t="n">
-        <v>59318</v>
+        <v>62440</v>
       </c>
     </row>
     <row r="1415">
@@ -16033,7 +16033,7 @@
         <v>104</v>
       </c>
       <c r="C1418" t="n">
-        <v>259090.92</v>
+        <v>272727.28</v>
       </c>
     </row>
     <row r="1419">
@@ -16088,7 +16088,7 @@
         <v>781</v>
       </c>
       <c r="C1423" t="n">
-        <v>112271</v>
+        <v>118180</v>
       </c>
     </row>
     <row r="1424">
@@ -16132,7 +16132,7 @@
         <v>2494</v>
       </c>
       <c r="C1427" t="n">
-        <v>129542</v>
+        <v>136360</v>
       </c>
     </row>
     <row r="1428">
@@ -16165,7 +16165,7 @@
         <v>2652</v>
       </c>
       <c r="C1430" t="n">
-        <v>120897</v>
+        <v>127260</v>
       </c>
     </row>
     <row r="1431">
@@ -16176,7 +16176,7 @@
         <v>1384</v>
       </c>
       <c r="C1431" t="n">
-        <v>302272.73</v>
+        <v>318181.82</v>
       </c>
     </row>
     <row r="1432">
@@ -16187,7 +16187,7 @@
         <v>360</v>
       </c>
       <c r="C1432" t="n">
-        <v>431813</v>
+        <v>454540</v>
       </c>
     </row>
     <row r="1433">
@@ -16198,7 +16198,7 @@
         <v>2767</v>
       </c>
       <c r="C1433" t="n">
-        <v>164084</v>
+        <v>172720</v>
       </c>
     </row>
     <row r="1434">
@@ -16209,7 +16209,7 @@
         <v>2178</v>
       </c>
       <c r="C1434" t="n">
-        <v>236636.38</v>
+        <v>249090.92</v>
       </c>
     </row>
     <row r="1435">
@@ -16220,7 +16220,7 @@
         <v>2107</v>
       </c>
       <c r="C1435" t="n">
-        <v>259065</v>
+        <v>272700</v>
       </c>
     </row>
     <row r="1436">
@@ -16231,7 +16231,7 @@
         <v>2711</v>
       </c>
       <c r="C1436" t="n">
-        <v>74765</v>
+        <v>78700</v>
       </c>
     </row>
     <row r="1437">
@@ -16242,7 +16242,7 @@
         <v>2845</v>
       </c>
       <c r="C1437" t="n">
-        <v>25909.11</v>
+        <v>27272.74</v>
       </c>
     </row>
     <row r="1438">
@@ -16286,7 +16286,7 @@
         <v>1102</v>
       </c>
       <c r="C1441" t="n">
-        <v>203053</v>
+        <v>213740</v>
       </c>
     </row>
     <row r="1442">
@@ -16297,7 +16297,7 @@
         <v>525</v>
       </c>
       <c r="C1442" t="n">
-        <v>202954.57</v>
+        <v>213636.38</v>
       </c>
     </row>
     <row r="1443">
@@ -16308,7 +16308,7 @@
         <v>1261</v>
       </c>
       <c r="C1443" t="n">
-        <v>61318.19</v>
+        <v>64545.46</v>
       </c>
     </row>
     <row r="1444">
@@ -16319,7 +16319,7 @@
         <v>2755</v>
       </c>
       <c r="C1444" t="n">
-        <v>43181.84</v>
+        <v>45454.56</v>
       </c>
     </row>
     <row r="1445">
@@ -16341,7 +16341,7 @@
         <v>783</v>
       </c>
       <c r="C1446" t="n">
-        <v>34545.46</v>
+        <v>36363.64</v>
       </c>
     </row>
     <row r="1447">
@@ -16352,7 +16352,7 @@
         <v>1064</v>
       </c>
       <c r="C1447" t="n">
-        <v>518168</v>
+        <v>545440</v>
       </c>
     </row>
     <row r="1448">
@@ -16363,7 +16363,7 @@
         <v>1810</v>
       </c>
       <c r="C1448" t="n">
-        <v>36979.63</v>
+        <v>38925.92</v>
       </c>
     </row>
     <row r="1449">
@@ -16374,7 +16374,7 @@
         <v>1937</v>
       </c>
       <c r="C1449" t="n">
-        <v>223668</v>
+        <v>235440</v>
       </c>
     </row>
     <row r="1450">
@@ -16385,7 +16385,7 @@
         <v>483</v>
       </c>
       <c r="C1450" t="n">
-        <v>390355</v>
+        <v>410900</v>
       </c>
     </row>
     <row r="1451">
@@ -16396,7 +16396,7 @@
         <v>2580</v>
       </c>
       <c r="C1451" t="n">
-        <v>29089</v>
+        <v>30620</v>
       </c>
     </row>
     <row r="1452">
@@ -16407,7 +16407,7 @@
         <v>2706</v>
       </c>
       <c r="C1452" t="n">
-        <v>22724</v>
+        <v>23920</v>
       </c>
     </row>
     <row r="1453">
@@ -16418,7 +16418,7 @@
         <v>2633</v>
       </c>
       <c r="C1453" t="n">
-        <v>16644</v>
+        <v>17520</v>
       </c>
     </row>
     <row r="1454">
@@ -16451,7 +16451,7 @@
         <v>2392</v>
       </c>
       <c r="C1456" t="n">
-        <v>179132</v>
+        <v>188560</v>
       </c>
     </row>
     <row r="1457">
@@ -16473,7 +16473,7 @@
         <v>2613</v>
       </c>
       <c r="C1458" t="n">
-        <v>126122</v>
+        <v>132760</v>
       </c>
     </row>
     <row r="1459">
@@ -16484,7 +16484,7 @@
         <v>2183</v>
       </c>
       <c r="C1459" t="n">
-        <v>454119</v>
+        <v>478020</v>
       </c>
     </row>
     <row r="1460">
@@ -16495,7 +16495,7 @@
         <v>2541</v>
       </c>
       <c r="C1460" t="n">
-        <v>204155</v>
+        <v>214900</v>
       </c>
     </row>
     <row r="1461">
@@ -16517,7 +16517,7 @@
         <v>2333</v>
       </c>
       <c r="C1462" t="n">
-        <v>137826</v>
+        <v>145080</v>
       </c>
     </row>
     <row r="1463">
@@ -16561,7 +16561,7 @@
         <v>2813</v>
       </c>
       <c r="C1466" t="n">
-        <v>55100</v>
+        <v>58000</v>
       </c>
     </row>
     <row r="1467">
@@ -16572,7 +16572,7 @@
         <v>2811</v>
       </c>
       <c r="C1467" t="n">
-        <v>35929</v>
+        <v>37820</v>
       </c>
     </row>
     <row r="1468">
@@ -16583,7 +16583,7 @@
         <v>1881</v>
       </c>
       <c r="C1468" t="n">
-        <v>59318</v>
+        <v>62440</v>
       </c>
     </row>
     <row r="1469">
@@ -16594,7 +16594,7 @@
         <v>2825</v>
       </c>
       <c r="C1469" t="n">
-        <v>48222</v>
+        <v>50760</v>
       </c>
     </row>
     <row r="1470">
@@ -16605,7 +16605,7 @@
         <v>970</v>
       </c>
       <c r="C1470" t="n">
-        <v>59318</v>
+        <v>62440</v>
       </c>
     </row>
     <row r="1471">
@@ -16616,7 +16616,7 @@
         <v>2552</v>
       </c>
       <c r="C1471" t="n">
-        <v>33763</v>
+        <v>35540</v>
       </c>
     </row>
     <row r="1472">
@@ -16627,7 +16627,7 @@
         <v>2562</v>
       </c>
       <c r="C1472" t="n">
-        <v>33763</v>
+        <v>35540</v>
       </c>
     </row>
     <row r="1473">
@@ -16704,7 +16704,7 @@
         <v>2747</v>
       </c>
       <c r="C1479" t="n">
-        <v>60439</v>
+        <v>63620</v>
       </c>
     </row>
     <row r="1480">
@@ -16792,7 +16792,7 @@
         <v>2544</v>
       </c>
       <c r="C1487" t="n">
-        <v>60439</v>
+        <v>63620</v>
       </c>
     </row>
     <row r="1488">
@@ -16803,7 +16803,7 @@
         <v>816</v>
       </c>
       <c r="C1488" t="n">
-        <v>259090.92</v>
+        <v>272727.28</v>
       </c>
     </row>
     <row r="1489">
@@ -16814,7 +16814,7 @@
         <v>890</v>
       </c>
       <c r="C1489" t="n">
-        <v>626136.38</v>
+        <v>659090.92</v>
       </c>
     </row>
     <row r="1490">
@@ -16836,7 +16836,7 @@
         <v>1298</v>
       </c>
       <c r="C1491" t="n">
-        <v>1092500</v>
+        <v>1150000</v>
       </c>
     </row>
     <row r="1492">
@@ -16847,7 +16847,7 @@
         <v>1372</v>
       </c>
       <c r="C1492" t="n">
-        <v>259090.92</v>
+        <v>272727.28</v>
       </c>
     </row>
     <row r="1493">
@@ -16858,7 +16858,7 @@
         <v>358</v>
       </c>
       <c r="C1493" t="n">
-        <v>272042</v>
+        <v>286360</v>
       </c>
     </row>
     <row r="1494">
@@ -16880,7 +16880,7 @@
         <v>1653</v>
       </c>
       <c r="C1495" t="n">
-        <v>272042</v>
+        <v>286360</v>
       </c>
     </row>
     <row r="1496">
@@ -16891,7 +16891,7 @@
         <v>675</v>
       </c>
       <c r="C1496" t="n">
-        <v>172710</v>
+        <v>181800</v>
       </c>
     </row>
     <row r="1497">
@@ -16902,7 +16902,7 @@
         <v>2804</v>
       </c>
       <c r="C1497" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1498">
@@ -16913,7 +16913,7 @@
         <v>2714</v>
       </c>
       <c r="C1498" t="n">
-        <v>310897</v>
+        <v>327260</v>
       </c>
     </row>
     <row r="1499">
@@ -16924,7 +16924,7 @@
         <v>2765</v>
       </c>
       <c r="C1499" t="n">
-        <v>77710</v>
+        <v>81800</v>
       </c>
     </row>
     <row r="1500">
@@ -16935,7 +16935,7 @@
         <v>2421</v>
       </c>
       <c r="C1500" t="n">
-        <v>52681.84</v>
+        <v>55454.56</v>
       </c>
     </row>
     <row r="1501">
@@ -16946,7 +16946,7 @@
         <v>2359</v>
       </c>
       <c r="C1501" t="n">
-        <v>90098</v>
+        <v>94840</v>
       </c>
     </row>
     <row r="1502">
@@ -16957,7 +16957,7 @@
         <v>2678</v>
       </c>
       <c r="C1502" t="n">
-        <v>85462</v>
+        <v>89960</v>
       </c>
     </row>
     <row r="1503">
@@ -16968,7 +16968,7 @@
         <v>2697</v>
       </c>
       <c r="C1503" t="n">
-        <v>129694</v>
+        <v>136520</v>
       </c>
     </row>
     <row r="1504">
@@ -17001,7 +17001,7 @@
         <v>1308</v>
       </c>
       <c r="C1506" t="n">
-        <v>135584</v>
+        <v>142720</v>
       </c>
     </row>
     <row r="1507">
@@ -17012,7 +17012,7 @@
         <v>2118</v>
       </c>
       <c r="C1507" t="n">
-        <v>181507</v>
+        <v>191060</v>
       </c>
     </row>
     <row r="1508">
@@ -17023,7 +17023,7 @@
         <v>2607</v>
       </c>
       <c r="C1508" t="n">
-        <v>42902</v>
+        <v>45160</v>
       </c>
     </row>
     <row r="1509">
@@ -17034,7 +17034,7 @@
         <v>2832</v>
       </c>
       <c r="C1509" t="n">
-        <v>129545.46</v>
+        <v>136363.64</v>
       </c>
     </row>
     <row r="1510">
@@ -17045,7 +17045,7 @@
         <v>2383</v>
       </c>
       <c r="C1510" t="n">
-        <v>114798</v>
+        <v>120840</v>
       </c>
     </row>
     <row r="1511">
@@ -17078,7 +17078,7 @@
         <v>2821</v>
       </c>
       <c r="C1513" t="n">
-        <v>115159</v>
+        <v>121220</v>
       </c>
     </row>
     <row r="1514">
@@ -17100,7 +17100,7 @@
         <v>569</v>
       </c>
       <c r="C1515" t="n">
-        <v>2507506</v>
+        <v>2639480</v>
       </c>
     </row>
     <row r="1516">
@@ -17111,7 +17111,7 @@
         <v>2660</v>
       </c>
       <c r="C1516" t="n">
-        <v>302272.73</v>
+        <v>318181.82</v>
       </c>
     </row>
     <row r="1517">
@@ -17122,7 +17122,7 @@
         <v>1632</v>
       </c>
       <c r="C1517" t="n">
-        <v>224545.46</v>
+        <v>236363.64</v>
       </c>
     </row>
     <row r="1518">
@@ -17133,7 +17133,7 @@
         <v>1756</v>
       </c>
       <c r="C1518" t="n">
-        <v>362710</v>
+        <v>381800</v>
       </c>
     </row>
     <row r="1519">
@@ -17144,7 +17144,7 @@
         <v>58</v>
       </c>
       <c r="C1519" t="n">
-        <v>216600</v>
+        <v>228000</v>
       </c>
     </row>
     <row r="1520">
@@ -17155,7 +17155,7 @@
         <v>40</v>
       </c>
       <c r="C1520" t="n">
-        <v>192660</v>
+        <v>202800</v>
       </c>
     </row>
     <row r="1521">
@@ -17166,7 +17166,7 @@
         <v>559</v>
       </c>
       <c r="C1521" t="n">
-        <v>202084</v>
+        <v>212720</v>
       </c>
     </row>
     <row r="1522">
@@ -17177,7 +17177,7 @@
         <v>2773</v>
       </c>
       <c r="C1522" t="n">
-        <v>69673</v>
+        <v>73340</v>
       </c>
     </row>
     <row r="1523">
@@ -17188,7 +17188,7 @@
         <v>2631</v>
       </c>
       <c r="C1523" t="n">
-        <v>33459</v>
+        <v>35220</v>
       </c>
     </row>
     <row r="1524">
@@ -17199,7 +17199,7 @@
         <v>2085</v>
       </c>
       <c r="C1524" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1525">
@@ -17221,7 +17221,7 @@
         <v>1642</v>
       </c>
       <c r="C1526" t="n">
-        <v>228855</v>
+        <v>240900</v>
       </c>
     </row>
     <row r="1527">
@@ -17232,7 +17232,7 @@
         <v>2621</v>
       </c>
       <c r="C1527" t="n">
-        <v>60439</v>
+        <v>63620</v>
       </c>
     </row>
     <row r="1528">
@@ -17243,7 +17243,7 @@
         <v>2705</v>
       </c>
       <c r="C1528" t="n">
-        <v>173394</v>
+        <v>182520</v>
       </c>
     </row>
     <row r="1529">
@@ -17276,7 +17276,7 @@
         <v>2735</v>
       </c>
       <c r="C1531" t="n">
-        <v>103626</v>
+        <v>109080</v>
       </c>
     </row>
     <row r="1532">
@@ -17287,7 +17287,7 @@
         <v>945</v>
       </c>
       <c r="C1532" t="n">
-        <v>302860</v>
+        <v>318800</v>
       </c>
     </row>
     <row r="1533">
@@ -17309,7 +17309,7 @@
         <v>2582</v>
       </c>
       <c r="C1534" t="n">
-        <v>75772</v>
+        <v>79760</v>
       </c>
     </row>
     <row r="1535">
@@ -17320,7 +17320,7 @@
         <v>2584</v>
       </c>
       <c r="C1535" t="n">
-        <v>55100</v>
+        <v>58000</v>
       </c>
     </row>
     <row r="1536">
@@ -17331,7 +17331,7 @@
         <v>2689</v>
       </c>
       <c r="C1536" t="n">
-        <v>55100</v>
+        <v>58000</v>
       </c>
     </row>
     <row r="1537">
@@ -17342,7 +17342,7 @@
         <v>2574</v>
       </c>
       <c r="C1537" t="n">
-        <v>121106</v>
+        <v>127480</v>
       </c>
     </row>
     <row r="1538">
@@ -17353,7 +17353,7 @@
         <v>1834</v>
       </c>
       <c r="C1538" t="n">
-        <v>101650</v>
+        <v>107000</v>
       </c>
     </row>
     <row r="1539">
@@ -17375,7 +17375,7 @@
         <v>2629</v>
       </c>
       <c r="C1540" t="n">
-        <v>59318</v>
+        <v>62440</v>
       </c>
     </row>
     <row r="1541">
@@ -17386,7 +17386,7 @@
         <v>933</v>
       </c>
       <c r="C1541" t="n">
-        <v>70357</v>
+        <v>74060</v>
       </c>
     </row>
     <row r="1542">
@@ -17397,7 +17397,7 @@
         <v>2555</v>
       </c>
       <c r="C1542" t="n">
-        <v>33763</v>
+        <v>35540</v>
       </c>
     </row>
     <row r="1543">
@@ -17408,7 +17408,7 @@
         <v>2558</v>
       </c>
       <c r="C1543" t="n">
-        <v>33763</v>
+        <v>35540</v>
       </c>
     </row>
     <row r="1544">
@@ -17430,7 +17430,7 @@
         <v>2721</v>
       </c>
       <c r="C1545" t="n">
-        <v>70357</v>
+        <v>74060</v>
       </c>
     </row>
     <row r="1546">
@@ -17441,7 +17441,7 @@
         <v>2556</v>
       </c>
       <c r="C1546" t="n">
-        <v>33763</v>
+        <v>35540</v>
       </c>
     </row>
     <row r="1547">
@@ -17463,7 +17463,7 @@
         <v>2826</v>
       </c>
       <c r="C1548" t="n">
-        <v>60439</v>
+        <v>63620</v>
       </c>
     </row>
     <row r="1549">
@@ -17485,7 +17485,7 @@
         <v>2346</v>
       </c>
       <c r="C1550" t="n">
-        <v>60439</v>
+        <v>63620</v>
       </c>
     </row>
     <row r="1551">
@@ -17496,7 +17496,7 @@
         <v>595</v>
       </c>
       <c r="C1551" t="n">
-        <v>215909.11</v>
+        <v>227272.74</v>
       </c>
     </row>
     <row r="1552">
@@ -17529,7 +17529,7 @@
         <v>1278</v>
       </c>
       <c r="C1554" t="n">
-        <v>151136.38</v>
+        <v>159090.92</v>
       </c>
     </row>
     <row r="1555">
@@ -17540,7 +17540,7 @@
         <v>2686</v>
       </c>
       <c r="C1555" t="n">
-        <v>120897</v>
+        <v>127260</v>
       </c>
     </row>
     <row r="1556">
@@ -17551,7 +17551,7 @@
         <v>1344</v>
       </c>
       <c r="C1556" t="n">
-        <v>129542</v>
+        <v>136360</v>
       </c>
     </row>
     <row r="1557">
@@ -17606,7 +17606,7 @@
         <v>2566</v>
       </c>
       <c r="C1561" t="n">
-        <v>69084</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1562">
@@ -17617,7 +17617,7 @@
         <v>2684</v>
       </c>
       <c r="C1562" t="n">
-        <v>82042</v>
+        <v>86360</v>
       </c>
     </row>
     <row r="1563">
@@ -17628,7 +17628,7 @@
         <v>2375</v>
       </c>
       <c r="C1563" t="n">
-        <v>285000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="1564">
@@ -17639,7 +17639,7 @@
         <v>2362</v>
       </c>
       <c r="C1564" t="n">
-        <v>64771</v>
+        <v>68180</v>
       </c>
     </row>
     <row r="1565">
@@ -17650,7 +17650,7 @@
         <v>2449</v>
       </c>
       <c r="C1565" t="n">
-        <v>82042</v>
+        <v>86360</v>
       </c>
     </row>
     <row r="1566">
@@ -17661,7 +17661,7 @@
         <v>2844</v>
       </c>
       <c r="C1566" t="n">
-        <v>25909.11</v>
+        <v>27272.74</v>
       </c>
     </row>
     <row r="1567">
@@ -17672,7 +17672,7 @@
         <v>2507</v>
       </c>
       <c r="C1567" t="n">
-        <v>77140</v>
+        <v>81200</v>
       </c>
     </row>
     <row r="1568">
@@ -17683,7 +17683,7 @@
         <v>1906</v>
       </c>
       <c r="C1568" t="n">
-        <v>93765</v>
+        <v>98700</v>
       </c>
     </row>
     <row r="1569">
@@ -17705,7 +17705,7 @@
         <v>1983</v>
       </c>
       <c r="C1570" t="n">
-        <v>473480</v>
+        <v>498400</v>
       </c>
     </row>
     <row r="1571">
@@ -17716,7 +17716,7 @@
         <v>1993</v>
       </c>
       <c r="C1571" t="n">
-        <v>321518</v>
+        <v>338440</v>
       </c>
     </row>
     <row r="1572">
@@ -17727,7 +17727,7 @@
         <v>89</v>
       </c>
       <c r="C1572" t="n">
-        <v>302271</v>
+        <v>318180</v>
       </c>
     </row>
     <row r="1573">
@@ -17738,7 +17738,7 @@
         <v>1063</v>
       </c>
       <c r="C1573" t="n">
-        <v>332500</v>
+        <v>350000</v>
       </c>
     </row>
     <row r="1574">
@@ -17749,7 +17749,7 @@
         <v>1116</v>
       </c>
       <c r="C1574" t="n">
-        <v>215897</v>
+        <v>227260</v>
       </c>
     </row>
     <row r="1575">
@@ -17760,7 +17760,7 @@
         <v>941</v>
       </c>
       <c r="C1575" t="n">
-        <v>259863</v>
+        <v>273540</v>
       </c>
     </row>
     <row r="1576">
@@ -17771,7 +17771,7 @@
         <v>2141</v>
       </c>
       <c r="C1576" t="n">
-        <v>29198.58</v>
+        <v>30735.34</v>
       </c>
     </row>
     <row r="1577">
@@ -17782,7 +17782,7 @@
         <v>2463</v>
       </c>
       <c r="C1577" t="n">
-        <v>284848</v>
+        <v>299840</v>
       </c>
     </row>
     <row r="1578">
@@ -17793,7 +17793,7 @@
         <v>2707</v>
       </c>
       <c r="C1578" t="n">
-        <v>37297</v>
+        <v>39260</v>
       </c>
     </row>
     <row r="1579">
@@ -17804,7 +17804,7 @@
         <v>2325</v>
       </c>
       <c r="C1579" t="n">
-        <v>99636</v>
+        <v>104880</v>
       </c>
     </row>
     <row r="1580">
@@ -17848,7 +17848,7 @@
         <v>1890</v>
       </c>
       <c r="C1583" t="n">
-        <v>211793</v>
+        <v>222940</v>
       </c>
     </row>
     <row r="1584">
@@ -17859,7 +17859,7 @@
         <v>2639</v>
       </c>
       <c r="C1584" t="n">
-        <v>34599</v>
+        <v>36420</v>
       </c>
     </row>
     <row r="1585">
@@ -17870,7 +17870,7 @@
         <v>2682</v>
       </c>
       <c r="C1585" t="n">
-        <v>120897</v>
+        <v>127260</v>
       </c>
     </row>
     <row r="1586">
@@ -17881,7 +17881,7 @@
         <v>2601</v>
       </c>
       <c r="C1586" t="n">
-        <v>237500</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="1587">
@@ -17892,7 +17892,7 @@
         <v>1142</v>
       </c>
       <c r="C1587" t="n">
-        <v>395618</v>
+        <v>416440</v>
       </c>
     </row>
     <row r="1588">
@@ -17936,7 +17936,7 @@
         <v>2082</v>
       </c>
       <c r="C1591" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1592">
@@ -17947,7 +17947,7 @@
         <v>2276</v>
       </c>
       <c r="C1592" t="n">
-        <v>171798</v>
+        <v>180840</v>
       </c>
     </row>
     <row r="1593">
@@ -17969,7 +17969,7 @@
         <v>2786</v>
       </c>
       <c r="C1594" t="n">
-        <v>60439</v>
+        <v>63620</v>
       </c>
     </row>
     <row r="1595">
@@ -17980,7 +17980,7 @@
         <v>2816</v>
       </c>
       <c r="C1595" t="n">
-        <v>112271</v>
+        <v>118180</v>
       </c>
     </row>
     <row r="1596">
@@ -17991,7 +17991,7 @@
         <v>1871</v>
       </c>
       <c r="C1596" t="n">
-        <v>123937</v>
+        <v>130460</v>
       </c>
     </row>
     <row r="1597">
@@ -18002,7 +18002,7 @@
         <v>2345</v>
       </c>
       <c r="C1597" t="n">
-        <v>55100</v>
+        <v>58000</v>
       </c>
     </row>
     <row r="1598">
@@ -18013,7 +18013,7 @@
         <v>2802</v>
       </c>
       <c r="C1598" t="n">
-        <v>61997</v>
+        <v>65260</v>
       </c>
     </row>
     <row r="1599">
@@ -18024,7 +18024,7 @@
         <v>2090</v>
       </c>
       <c r="C1599" t="n">
-        <v>35929</v>
+        <v>37820</v>
       </c>
     </row>
     <row r="1600">
@@ -18035,7 +18035,7 @@
         <v>2647</v>
       </c>
       <c r="C1600" t="n">
-        <v>121125</v>
+        <v>127500</v>
       </c>
     </row>
     <row r="1601">
@@ -18046,7 +18046,7 @@
         <v>2365</v>
       </c>
       <c r="C1601" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1602">
@@ -18057,7 +18057,7 @@
         <v>766</v>
       </c>
       <c r="C1602" t="n">
-        <v>59318</v>
+        <v>62440</v>
       </c>
     </row>
     <row r="1603">
@@ -18068,7 +18068,7 @@
         <v>2702</v>
       </c>
       <c r="C1603" t="n">
-        <v>70357</v>
+        <v>74060</v>
       </c>
     </row>
     <row r="1604">
@@ -18090,7 +18090,7 @@
         <v>20</v>
       </c>
       <c r="C1605" t="n">
-        <v>388636.38</v>
+        <v>409090.92</v>
       </c>
     </row>
     <row r="1606">
@@ -18101,7 +18101,7 @@
         <v>27</v>
       </c>
       <c r="C1606" t="n">
-        <v>129545.46</v>
+        <v>136363.64</v>
       </c>
     </row>
     <row r="1607">
@@ -18112,7 +18112,7 @@
         <v>33</v>
       </c>
       <c r="C1607" t="n">
-        <v>343727.3</v>
+        <v>361818.2</v>
       </c>
     </row>
     <row r="1608">
@@ -18134,7 +18134,7 @@
         <v>2561</v>
       </c>
       <c r="C1609" t="n">
-        <v>33763</v>
+        <v>35540</v>
       </c>
     </row>
     <row r="1610">
@@ -18178,7 +18178,7 @@
         <v>2772</v>
       </c>
       <c r="C1613" t="n">
-        <v>51813</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1614">
@@ -18189,7 +18189,7 @@
         <v>132</v>
       </c>
       <c r="C1614" t="n">
-        <v>302272.73</v>
+        <v>318181.82</v>
       </c>
     </row>
     <row r="1615">
@@ -18211,7 +18211,7 @@
         <v>580</v>
       </c>
       <c r="C1616" t="n">
-        <v>151136.38</v>
+        <v>159090.92</v>
       </c>
     </row>
     <row r="1617">
@@ -18222,7 +18222,7 @@
         <v>634</v>
       </c>
       <c r="C1617" t="n">
-        <v>431818.19</v>
+        <v>454545.46</v>
       </c>
     </row>
     <row r="1618">
@@ -18244,7 +18244,7 @@
         <v>1277</v>
       </c>
       <c r="C1619" t="n">
-        <v>190000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="1620">
@@ -18255,7 +18255,7 @@
         <v>767</v>
       </c>
       <c r="C1620" t="n">
-        <v>172710</v>
+        <v>181800</v>
       </c>
     </row>
     <row r="1621">
@@ -18266,7 +18266,7 @@
         <v>2727</v>
       </c>
       <c r="C1621" t="n">
-        <v>34960</v>
+        <v>36800</v>
       </c>
     </row>
     <row r="1622">
@@ -18277,7 +18277,7 @@
         <v>2846</v>
       </c>
       <c r="C1622" t="n">
-        <v>224542</v>
+        <v>236360</v>
       </c>
     </row>
     <row r="1623">
@@ -18288,7 +18288,7 @@
         <v>609</v>
       </c>
       <c r="C1623" t="n">
-        <v>194313</v>
+        <v>204540</v>
       </c>
     </row>
     <row r="1624">
@@ -18299,7 +18299,7 @@
         <v>2726</v>
       </c>
       <c r="C1624" t="n">
-        <v>133855</v>
+        <v>140900</v>
       </c>
     </row>
     <row r="1625">
@@ -18321,7 +18321,7 @@
         <v>2729</v>
       </c>
       <c r="C1626" t="n">
-        <v>77710</v>
+        <v>81800</v>
       </c>
     </row>
     <row r="1627">
@@ -18332,7 +18332,7 @@
         <v>1340</v>
       </c>
       <c r="C1627" t="n">
-        <v>129542</v>
+        <v>136360</v>
       </c>
     </row>
     <row r="1628">
@@ -18343,7 +18343,7 @@
         <v>2830</v>
       </c>
       <c r="C1628" t="n">
-        <v>77710</v>
+        <v>81800</v>
       </c>
     </row>
     <row r="1629">
@@ -18365,7 +18365,7 @@
         <v>2674</v>
       </c>
       <c r="C1630" t="n">
-        <v>224542</v>
+        <v>236360</v>
       </c>
     </row>
     <row r="1631">
@@ -18376,7 +18376,7 @@
         <v>2308</v>
       </c>
       <c r="C1631" t="n">
-        <v>172710</v>
+        <v>181800</v>
       </c>
     </row>
     <row r="1632">
@@ -18387,7 +18387,7 @@
         <v>2190</v>
       </c>
       <c r="C1632" t="n">
-        <v>181363.65</v>
+        <v>190909.1</v>
       </c>
     </row>
     <row r="1633">
@@ -18398,7 +18398,7 @@
         <v>2015</v>
       </c>
       <c r="C1633" t="n">
-        <v>319542</v>
+        <v>336360</v>
       </c>
     </row>
     <row r="1634">
@@ -18409,7 +18409,7 @@
         <v>429</v>
       </c>
       <c r="C1634" t="n">
-        <v>328168</v>
+        <v>345440</v>
       </c>
     </row>
     <row r="1635">
@@ -18420,7 +18420,7 @@
         <v>2114</v>
       </c>
       <c r="C1635" t="n">
-        <v>146927</v>
+        <v>154660</v>
       </c>
     </row>
     <row r="1636">
@@ -18431,7 +18431,7 @@
         <v>2211</v>
       </c>
       <c r="C1636" t="n">
-        <v>207993</v>
+        <v>218940</v>
       </c>
     </row>
     <row r="1637">
@@ -18442,7 +18442,7 @@
         <v>1108</v>
       </c>
       <c r="C1637" t="n">
-        <v>264594</v>
+        <v>278520</v>
       </c>
     </row>
     <row r="1638">
@@ -18453,7 +18453,7 @@
         <v>2695</v>
       </c>
       <c r="C1638" t="n">
-        <v>44047.44</v>
+        <v>46365.72</v>
       </c>
     </row>
     <row r="1639">
@@ -18464,7 +18464,7 @@
         <v>1289</v>
       </c>
       <c r="C1639" t="n">
-        <v>237500</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="1640">
@@ -18475,7 +18475,7 @@
         <v>2789</v>
       </c>
       <c r="C1640" t="n">
-        <v>155454.57</v>
+        <v>163636.38</v>
       </c>
     </row>
     <row r="1641">
@@ -18486,7 +18486,7 @@
         <v>2197</v>
       </c>
       <c r="C1641" t="n">
-        <v>185681.84</v>
+        <v>195454.56</v>
       </c>
     </row>
     <row r="1642">
@@ -18497,7 +18497,7 @@
         <v>947</v>
       </c>
       <c r="C1642" t="n">
-        <v>383002</v>
+        <v>403160</v>
       </c>
     </row>
     <row r="1643">
@@ -18508,7 +18508,7 @@
         <v>2279</v>
       </c>
       <c r="C1643" t="n">
-        <v>211527</v>
+        <v>222660</v>
       </c>
     </row>
     <row r="1644">
@@ -18519,7 +18519,7 @@
         <v>1465</v>
       </c>
       <c r="C1644" t="n">
-        <v>332500</v>
+        <v>350000</v>
       </c>
     </row>
     <row r="1645">
@@ -18530,7 +18530,7 @@
         <v>2651</v>
       </c>
       <c r="C1645" t="n">
-        <v>146813</v>
+        <v>154540</v>
       </c>
     </row>
     <row r="1646">
@@ -18541,7 +18541,7 @@
         <v>42</v>
       </c>
       <c r="C1646" t="n">
-        <v>1646084</v>
+        <v>1732720</v>
       </c>
     </row>
     <row r="1647">
@@ -18552,7 +18552,7 @@
         <v>949</v>
       </c>
       <c r="C1647" t="n">
-        <v>85899</v>
+        <v>90420</v>
       </c>
     </row>
     <row r="1648">
@@ -18563,7 +18563,7 @@
         <v>2606</v>
       </c>
       <c r="C1648" t="n">
-        <v>221730</v>
+        <v>233400</v>
       </c>
     </row>
     <row r="1649">
@@ -18574,7 +18574,7 @@
         <v>2249</v>
       </c>
       <c r="C1649" t="n">
-        <v>188385</v>
+        <v>198300</v>
       </c>
     </row>
     <row r="1650">
@@ -18618,7 +18618,7 @@
         <v>2045</v>
       </c>
       <c r="C1653" t="n">
-        <v>275044</v>
+        <v>289520</v>
       </c>
     </row>
     <row r="1654">
@@ -18629,7 +18629,7 @@
         <v>2663</v>
       </c>
       <c r="C1654" t="n">
-        <v>237500</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="1655">
@@ -18651,7 +18651,7 @@
         <v>2854</v>
       </c>
       <c r="C1656" t="n">
-        <v>34542</v>
+        <v>36360</v>
       </c>
     </row>
     <row r="1657">
@@ -18684,7 +18684,7 @@
         <v>2341</v>
       </c>
       <c r="C1659" t="n">
-        <v>151050</v>
+        <v>159000</v>
       </c>
     </row>
     <row r="1660">
@@ -18695,7 +18695,7 @@
         <v>2637</v>
       </c>
       <c r="C1660" t="n">
-        <v>55100</v>
+        <v>58000</v>
       </c>
     </row>
     <row r="1661">
@@ -18706,7 +18706,7 @@
         <v>2492</v>
       </c>
       <c r="C1661" t="n">
-        <v>86507</v>
+        <v>91060</v>
       </c>
     </row>
     <row r="1662">
@@ -18739,7 +18739,7 @@
         <v>2548</v>
       </c>
       <c r="C1664" t="n">
-        <v>33763</v>
+        <v>35540</v>
       </c>
     </row>
     <row r="1665">
@@ -18750,7 +18750,7 @@
         <v>351</v>
       </c>
       <c r="C1665" t="n">
-        <v>183954.57</v>
+        <v>193636.38</v>
       </c>
     </row>
     <row r="1666">
@@ -18783,7 +18783,7 @@
         <v>2757</v>
       </c>
       <c r="C1668" t="n">
-        <v>69084</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1669">
@@ -18794,7 +18794,7 @@
         <v>2815</v>
       </c>
       <c r="C1669" t="n">
-        <v>51813</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1670">
@@ -18805,7 +18805,7 @@
         <v>2829</v>
       </c>
       <c r="C1670" t="n">
-        <v>51813</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1671">
@@ -18816,7 +18816,7 @@
         <v>768</v>
       </c>
       <c r="C1671" t="n">
-        <v>120897</v>
+        <v>127260</v>
       </c>
     </row>
     <row r="1672">
@@ -18827,7 +18827,7 @@
         <v>772</v>
       </c>
       <c r="C1672" t="n">
-        <v>280681.84</v>
+        <v>295454.56</v>
       </c>
     </row>
     <row r="1673">
@@ -18860,7 +18860,7 @@
         <v>2496</v>
       </c>
       <c r="C1675" t="n">
-        <v>172710</v>
+        <v>181800</v>
       </c>
     </row>
     <row r="1676">
@@ -18871,7 +18871,7 @@
         <v>802</v>
       </c>
       <c r="C1676" t="n">
-        <v>64771</v>
+        <v>68180</v>
       </c>
     </row>
     <row r="1677">
@@ -18893,7 +18893,7 @@
         <v>2131</v>
       </c>
       <c r="C1678" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1679">
@@ -18904,7 +18904,7 @@
         <v>1381</v>
       </c>
       <c r="C1679" t="n">
-        <v>259090.92</v>
+        <v>272727.28</v>
       </c>
     </row>
     <row r="1680">
@@ -18915,7 +18915,7 @@
         <v>2847</v>
       </c>
       <c r="C1680" t="n">
-        <v>116584</v>
+        <v>122720</v>
       </c>
     </row>
     <row r="1681">
@@ -18926,7 +18926,7 @@
         <v>1293</v>
       </c>
       <c r="C1681" t="n">
-        <v>332500</v>
+        <v>350000</v>
       </c>
     </row>
     <row r="1682">
@@ -18948,7 +18948,7 @@
         <v>2363</v>
       </c>
       <c r="C1683" t="n">
-        <v>146813</v>
+        <v>154540</v>
       </c>
     </row>
     <row r="1684">
@@ -18959,7 +18959,7 @@
         <v>631</v>
       </c>
       <c r="C1684" t="n">
-        <v>302271</v>
+        <v>318180</v>
       </c>
     </row>
     <row r="1685">
@@ -18970,7 +18970,7 @@
         <v>2791</v>
       </c>
       <c r="C1685" t="n">
-        <v>88673</v>
+        <v>93340</v>
       </c>
     </row>
     <row r="1686">
@@ -18992,7 +18992,7 @@
         <v>2841</v>
       </c>
       <c r="C1687" t="n">
-        <v>43168</v>
+        <v>45440</v>
       </c>
     </row>
     <row r="1688">
@@ -19003,7 +19003,7 @@
         <v>2571</v>
       </c>
       <c r="C1688" t="n">
-        <v>230223</v>
+        <v>242340</v>
       </c>
     </row>
     <row r="1689">
@@ -19069,7 +19069,7 @@
         <v>2273</v>
       </c>
       <c r="C1694" t="n">
-        <v>195686.19</v>
+        <v>205985.46</v>
       </c>
     </row>
     <row r="1695">
@@ -19080,7 +19080,7 @@
         <v>2381</v>
       </c>
       <c r="C1695" t="n">
-        <v>73199.86</v>
+        <v>77052.48</v>
       </c>
     </row>
     <row r="1696">
@@ -19091,7 +19091,7 @@
         <v>630</v>
       </c>
       <c r="C1696" t="n">
-        <v>71275.87</v>
+        <v>75027.23</v>
       </c>
     </row>
     <row r="1697">
@@ -19113,7 +19113,7 @@
         <v>2768</v>
       </c>
       <c r="C1698" t="n">
-        <v>261383</v>
+        <v>275140</v>
       </c>
     </row>
     <row r="1699">
@@ -19124,7 +19124,7 @@
         <v>2491</v>
       </c>
       <c r="C1699" t="n">
-        <v>209741</v>
+        <v>220780</v>
       </c>
     </row>
     <row r="1700">
@@ -19135,7 +19135,7 @@
         <v>2799</v>
       </c>
       <c r="C1700" t="n">
-        <v>94411</v>
+        <v>99380</v>
       </c>
     </row>
     <row r="1701">
@@ -19168,7 +19168,7 @@
         <v>1317</v>
       </c>
       <c r="C1703" t="n">
-        <v>272045.46</v>
+        <v>286363.64</v>
       </c>
     </row>
     <row r="1704">
@@ -19179,7 +19179,7 @@
         <v>2822</v>
       </c>
       <c r="C1704" t="n">
-        <v>138181.84</v>
+        <v>145454.56</v>
       </c>
     </row>
     <row r="1705">
@@ -19190,7 +19190,7 @@
         <v>1117</v>
       </c>
       <c r="C1705" t="n">
-        <v>345553</v>
+        <v>363740</v>
       </c>
     </row>
     <row r="1706">
@@ -19201,7 +19201,7 @@
         <v>1299</v>
       </c>
       <c r="C1706" t="n">
-        <v>455601</v>
+        <v>479580</v>
       </c>
     </row>
     <row r="1707">
@@ -19212,7 +19212,7 @@
         <v>477</v>
       </c>
       <c r="C1707" t="n">
-        <v>187758</v>
+        <v>197640</v>
       </c>
     </row>
     <row r="1708">
@@ -19223,7 +19223,7 @@
         <v>530</v>
       </c>
       <c r="C1708" t="n">
-        <v>259084</v>
+        <v>272720</v>
       </c>
     </row>
     <row r="1709">
@@ -19234,7 +19234,7 @@
         <v>953</v>
       </c>
       <c r="C1709" t="n">
-        <v>595897</v>
+        <v>627260</v>
       </c>
     </row>
     <row r="1710">
@@ -19245,7 +19245,7 @@
         <v>610</v>
       </c>
       <c r="C1710" t="n">
-        <v>709726</v>
+        <v>747080</v>
       </c>
     </row>
     <row r="1711">
@@ -19256,7 +19256,7 @@
         <v>2792</v>
       </c>
       <c r="C1711" t="n">
-        <v>178239</v>
+        <v>187620</v>
       </c>
     </row>
     <row r="1712">
@@ -19333,7 +19333,7 @@
         <v>2834</v>
       </c>
       <c r="C1718" t="n">
-        <v>32186</v>
+        <v>33880</v>
       </c>
     </row>
     <row r="1719">
@@ -19344,7 +19344,7 @@
         <v>2394</v>
       </c>
       <c r="C1719" t="n">
-        <v>97983</v>
+        <v>103140</v>
       </c>
     </row>
     <row r="1720">
@@ -19355,7 +19355,7 @@
         <v>2567</v>
       </c>
       <c r="C1720" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1721">
@@ -19366,7 +19366,7 @@
         <v>952</v>
       </c>
       <c r="C1721" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1722">
@@ -19377,7 +19377,7 @@
         <v>1539</v>
       </c>
       <c r="C1722" t="n">
-        <v>146813</v>
+        <v>154540</v>
       </c>
     </row>
     <row r="1723">
@@ -19388,7 +19388,7 @@
         <v>793</v>
       </c>
       <c r="C1723" t="n">
-        <v>35929</v>
+        <v>37820</v>
       </c>
     </row>
     <row r="1724">
@@ -19399,7 +19399,7 @@
         <v>794</v>
       </c>
       <c r="C1724" t="n">
-        <v>35929</v>
+        <v>37820</v>
       </c>
     </row>
     <row r="1725">
@@ -19410,7 +19410,7 @@
         <v>2838</v>
       </c>
       <c r="C1725" t="n">
-        <v>51818.19</v>
+        <v>54545.46</v>
       </c>
     </row>
     <row r="1726">
@@ -19432,7 +19432,7 @@
         <v>2223</v>
       </c>
       <c r="C1727" t="n">
-        <v>101137</v>
+        <v>106460</v>
       </c>
     </row>
     <row r="1728">
@@ -19443,7 +19443,7 @@
         <v>2547</v>
       </c>
       <c r="C1728" t="n">
-        <v>29260</v>
+        <v>30800</v>
       </c>
     </row>
     <row r="1729">
@@ -19465,7 +19465,7 @@
         <v>2762</v>
       </c>
       <c r="C1730" t="n">
-        <v>70357</v>
+        <v>74060</v>
       </c>
     </row>
     <row r="1731">
@@ -19476,7 +19476,7 @@
         <v>2550</v>
       </c>
       <c r="C1731" t="n">
-        <v>33763</v>
+        <v>35540</v>
       </c>
     </row>
     <row r="1732">
@@ -19487,7 +19487,7 @@
         <v>2627</v>
       </c>
       <c r="C1732" t="n">
-        <v>33763</v>
+        <v>35540</v>
       </c>
     </row>
     <row r="1733">
@@ -19542,7 +19542,7 @@
         <v>749</v>
       </c>
       <c r="C1737" t="n">
-        <v>70357</v>
+        <v>74060</v>
       </c>
     </row>
     <row r="1738">
@@ -19553,7 +19553,7 @@
         <v>2549</v>
       </c>
       <c r="C1738" t="n">
-        <v>33763</v>
+        <v>35540</v>
       </c>
     </row>
     <row r="1739">
@@ -19564,7 +19564,7 @@
         <v>2649</v>
       </c>
       <c r="C1739" t="n">
-        <v>33763</v>
+        <v>35540</v>
       </c>
     </row>
     <row r="1740">
@@ -19575,7 +19575,7 @@
         <v>2258</v>
       </c>
       <c r="C1740" t="n">
-        <v>69084</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1741">
@@ -19586,7 +19586,7 @@
         <v>2744</v>
       </c>
       <c r="C1741" t="n">
-        <v>51813</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1742">
@@ -19597,7 +19597,7 @@
         <v>452</v>
       </c>
       <c r="C1742" t="n">
-        <v>244409.11</v>
+        <v>257272.74</v>
       </c>
     </row>
     <row r="1743">
@@ -19652,7 +19652,7 @@
         <v>2653</v>
       </c>
       <c r="C1747" t="n">
-        <v>51813</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1748">
@@ -19696,7 +19696,7 @@
         <v>2742</v>
       </c>
       <c r="C1751" t="n">
-        <v>17271</v>
+        <v>18180</v>
       </c>
     </row>
     <row r="1752">
@@ -19707,7 +19707,7 @@
         <v>1499</v>
       </c>
       <c r="C1752" t="n">
-        <v>77710</v>
+        <v>81800</v>
       </c>
     </row>
     <row r="1753">
@@ -19718,7 +19718,7 @@
         <v>2261</v>
       </c>
       <c r="C1753" t="n">
-        <v>155439</v>
+        <v>163620</v>
       </c>
     </row>
     <row r="1754">
@@ -19762,7 +19762,7 @@
         <v>1324</v>
       </c>
       <c r="C1757" t="n">
-        <v>241813</v>
+        <v>254540</v>
       </c>
     </row>
     <row r="1758">
@@ -19773,7 +19773,7 @@
         <v>2709</v>
       </c>
       <c r="C1758" t="n">
-        <v>155439</v>
+        <v>163620</v>
       </c>
     </row>
     <row r="1759">
@@ -19795,7 +19795,7 @@
         <v>1137</v>
       </c>
       <c r="C1760" t="n">
-        <v>552710</v>
+        <v>581800</v>
       </c>
     </row>
     <row r="1761">
@@ -19806,7 +19806,7 @@
         <v>2440</v>
       </c>
       <c r="C1761" t="n">
-        <v>69084</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1762">
@@ -19817,7 +19817,7 @@
         <v>2413</v>
       </c>
       <c r="C1762" t="n">
-        <v>119035</v>
+        <v>125300</v>
       </c>
     </row>
     <row r="1763">
@@ -19828,7 +19828,7 @@
         <v>1450</v>
       </c>
       <c r="C1763" t="n">
-        <v>308313</v>
+        <v>324540</v>
       </c>
     </row>
     <row r="1764">
@@ -19850,7 +19850,7 @@
         <v>2671</v>
       </c>
       <c r="C1765" t="n">
-        <v>69084</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1766">
@@ -19861,7 +19861,7 @@
         <v>2568</v>
       </c>
       <c r="C1766" t="n">
-        <v>138567</v>
+        <v>145860</v>
       </c>
     </row>
     <row r="1767">
@@ -19872,7 +19872,7 @@
         <v>2146</v>
       </c>
       <c r="C1767" t="n">
-        <v>167789</v>
+        <v>176620</v>
       </c>
     </row>
     <row r="1768">
@@ -19883,7 +19883,7 @@
         <v>2753</v>
       </c>
       <c r="C1768" t="n">
-        <v>64771</v>
+        <v>68180</v>
       </c>
     </row>
     <row r="1769">
@@ -19916,7 +19916,7 @@
         <v>744</v>
       </c>
       <c r="C1771" t="n">
-        <v>35929</v>
+        <v>37820</v>
       </c>
     </row>
     <row r="1772">
@@ -19927,7 +19927,7 @@
         <v>2323</v>
       </c>
       <c r="C1772" t="n">
-        <v>59318</v>
+        <v>62440</v>
       </c>
     </row>
     <row r="1773">
@@ -19938,7 +19938,7 @@
         <v>2310</v>
       </c>
       <c r="C1773" t="n">
-        <v>59318</v>
+        <v>62440</v>
       </c>
     </row>
     <row r="1774">
@@ -19949,7 +19949,7 @@
         <v>2145</v>
       </c>
       <c r="C1774" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1775">
@@ -19960,7 +19960,7 @@
         <v>2858</v>
       </c>
       <c r="C1775" t="n">
-        <v>43181.84</v>
+        <v>45454.56</v>
       </c>
     </row>
     <row r="1776">
@@ -19993,7 +19993,7 @@
         <v>2501</v>
       </c>
       <c r="C1778" t="n">
-        <v>70357</v>
+        <v>74060</v>
       </c>
     </row>
     <row r="1779">
@@ -20004,7 +20004,7 @@
         <v>2546</v>
       </c>
       <c r="C1779" t="n">
-        <v>33763</v>
+        <v>35540</v>
       </c>
     </row>
     <row r="1780">
@@ -20026,7 +20026,7 @@
         <v>716</v>
       </c>
       <c r="C1781" t="n">
-        <v>110694</v>
+        <v>116520</v>
       </c>
     </row>
     <row r="1782">
@@ -20037,7 +20037,7 @@
         <v>2758</v>
       </c>
       <c r="C1782" t="n">
-        <v>51813</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1783">
@@ -20048,7 +20048,7 @@
         <v>400</v>
       </c>
       <c r="C1783" t="n">
-        <v>155454.57</v>
+        <v>163636.38</v>
       </c>
     </row>
     <row r="1784">
@@ -20059,7 +20059,7 @@
         <v>6</v>
       </c>
       <c r="C1784" t="n">
-        <v>43181.84</v>
+        <v>45454.56</v>
       </c>
     </row>
     <row r="1785">
@@ -20114,7 +20114,7 @@
         <v>1259</v>
       </c>
       <c r="C1789" t="n">
-        <v>95000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1790">
@@ -20125,7 +20125,7 @@
         <v>571</v>
       </c>
       <c r="C1790" t="n">
-        <v>893863.65</v>
+        <v>940909.1</v>
       </c>
     </row>
     <row r="1791">
@@ -20136,7 +20136,7 @@
         <v>703</v>
       </c>
       <c r="C1791" t="n">
-        <v>215897</v>
+        <v>227260</v>
       </c>
     </row>
     <row r="1792">
@@ -20191,7 +20191,7 @@
         <v>2833</v>
       </c>
       <c r="C1796" t="n">
-        <v>69084</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1797">
@@ -20202,7 +20202,7 @@
         <v>1007</v>
       </c>
       <c r="C1797" t="n">
-        <v>172727.3</v>
+        <v>181818.2</v>
       </c>
     </row>
     <row r="1798">
@@ -20213,7 +20213,7 @@
         <v>2687</v>
       </c>
       <c r="C1798" t="n">
-        <v>69084</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1799">
@@ -20224,7 +20224,7 @@
         <v>2824</v>
       </c>
       <c r="C1799" t="n">
-        <v>97508</v>
+        <v>102640</v>
       </c>
     </row>
     <row r="1800">
@@ -20235,7 +20235,7 @@
         <v>2730</v>
       </c>
       <c r="C1800" t="n">
-        <v>77710</v>
+        <v>81800</v>
       </c>
     </row>
     <row r="1801">
@@ -20257,7 +20257,7 @@
         <v>2718</v>
       </c>
       <c r="C1802" t="n">
-        <v>112271</v>
+        <v>118180</v>
       </c>
     </row>
     <row r="1803">
@@ -20268,7 +20268,7 @@
         <v>2750</v>
       </c>
       <c r="C1803" t="n">
-        <v>25897</v>
+        <v>27260</v>
       </c>
     </row>
     <row r="1804">
@@ -20279,7 +20279,7 @@
         <v>854</v>
       </c>
       <c r="C1804" t="n">
-        <v>120897</v>
+        <v>127260</v>
       </c>
     </row>
     <row r="1805">
@@ -20290,7 +20290,7 @@
         <v>2794</v>
       </c>
       <c r="C1805" t="n">
-        <v>103626</v>
+        <v>109080</v>
       </c>
     </row>
     <row r="1806">
@@ -20301,7 +20301,7 @@
         <v>1374</v>
       </c>
       <c r="C1806" t="n">
-        <v>172710</v>
+        <v>181800</v>
       </c>
     </row>
     <row r="1807">
@@ -20312,7 +20312,7 @@
         <v>2488</v>
       </c>
       <c r="C1807" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1808">
@@ -20323,7 +20323,7 @@
         <v>363</v>
       </c>
       <c r="C1808" t="n">
-        <v>259084</v>
+        <v>272720</v>
       </c>
     </row>
     <row r="1809">
@@ -20334,7 +20334,7 @@
         <v>2655</v>
       </c>
       <c r="C1809" t="n">
-        <v>95000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1810">
@@ -20345,7 +20345,7 @@
         <v>1873</v>
       </c>
       <c r="C1810" t="n">
-        <v>276355</v>
+        <v>290900</v>
       </c>
     </row>
     <row r="1811">
@@ -20356,7 +20356,7 @@
         <v>2635</v>
       </c>
       <c r="C1811" t="n">
-        <v>112271</v>
+        <v>118180</v>
       </c>
     </row>
     <row r="1812">
@@ -20367,7 +20367,7 @@
         <v>1658</v>
       </c>
       <c r="C1812" t="n">
-        <v>132136.38</v>
+        <v>139090.92</v>
       </c>
     </row>
     <row r="1813">
@@ -20378,7 +20378,7 @@
         <v>2069</v>
       </c>
       <c r="C1813" t="n">
-        <v>172727.3</v>
+        <v>181818.2</v>
       </c>
     </row>
     <row r="1814">
@@ -20389,7 +20389,7 @@
         <v>2081</v>
       </c>
       <c r="C1814" t="n">
-        <v>129542</v>
+        <v>136360</v>
       </c>
     </row>
     <row r="1815">
@@ -20400,7 +20400,7 @@
         <v>2124</v>
       </c>
       <c r="C1815" t="n">
-        <v>302271</v>
+        <v>318180</v>
       </c>
     </row>
     <row r="1816">
@@ -20411,7 +20411,7 @@
         <v>636</v>
       </c>
       <c r="C1816" t="n">
-        <v>215897</v>
+        <v>227260</v>
       </c>
     </row>
     <row r="1817">
@@ -20422,7 +20422,7 @@
         <v>2803</v>
       </c>
       <c r="C1817" t="n">
-        <v>103626</v>
+        <v>109080</v>
       </c>
     </row>
     <row r="1818">
@@ -20433,7 +20433,7 @@
         <v>2163</v>
       </c>
       <c r="C1818" t="n">
-        <v>155439</v>
+        <v>163620</v>
       </c>
     </row>
     <row r="1819">
@@ -20444,7 +20444,7 @@
         <v>1466</v>
       </c>
       <c r="C1819" t="n">
-        <v>349771</v>
+        <v>368180</v>
       </c>
     </row>
     <row r="1820">
@@ -20455,7 +20455,7 @@
         <v>2133</v>
       </c>
       <c r="C1820" t="n">
-        <v>626136.38</v>
+        <v>659090.92</v>
       </c>
     </row>
     <row r="1821">
@@ -20466,7 +20466,7 @@
         <v>2431</v>
       </c>
       <c r="C1821" t="n">
-        <v>129545.46</v>
+        <v>136363.64</v>
       </c>
     </row>
     <row r="1822">
@@ -20477,7 +20477,7 @@
         <v>535</v>
       </c>
       <c r="C1822" t="n">
-        <v>307610</v>
+        <v>323800</v>
       </c>
     </row>
     <row r="1823">
@@ -20488,7 +20488,7 @@
         <v>2790</v>
       </c>
       <c r="C1823" t="n">
-        <v>54549</v>
+        <v>57420</v>
       </c>
     </row>
     <row r="1824">
@@ -20499,7 +20499,7 @@
         <v>2442</v>
       </c>
       <c r="C1824" t="n">
-        <v>223681.84</v>
+        <v>235454.56</v>
       </c>
     </row>
     <row r="1825">
@@ -20510,7 +20510,7 @@
         <v>2376</v>
       </c>
       <c r="C1825" t="n">
-        <v>950000</v>
+        <v>1000000</v>
       </c>
     </row>
     <row r="1826">
@@ -20521,7 +20521,7 @@
         <v>1075</v>
       </c>
       <c r="C1826" t="n">
-        <v>396397</v>
+        <v>417260</v>
       </c>
     </row>
     <row r="1827">
@@ -20532,7 +20532,7 @@
         <v>131</v>
       </c>
       <c r="C1827" t="n">
-        <v>359271</v>
+        <v>378180</v>
       </c>
     </row>
     <row r="1828">
@@ -20543,7 +20543,7 @@
         <v>2667</v>
       </c>
       <c r="C1828" t="n">
-        <v>39463</v>
+        <v>41540</v>
       </c>
     </row>
     <row r="1829">
@@ -20554,7 +20554,7 @@
         <v>2330</v>
       </c>
       <c r="C1829" t="n">
-        <v>76817</v>
+        <v>80860</v>
       </c>
     </row>
     <row r="1830">
@@ -20576,7 +20576,7 @@
         <v>2577</v>
       </c>
       <c r="C1831" t="n">
-        <v>77007</v>
+        <v>81060</v>
       </c>
     </row>
     <row r="1832">
@@ -20587,7 +20587,7 @@
         <v>2510</v>
       </c>
       <c r="C1832" t="n">
-        <v>546896</v>
+        <v>575680</v>
       </c>
     </row>
     <row r="1833">
@@ -20609,7 +20609,7 @@
         <v>2850</v>
       </c>
       <c r="C1834" t="n">
-        <v>51813</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1835">
@@ -20631,7 +20631,7 @@
         <v>2745</v>
       </c>
       <c r="C1836" t="n">
-        <v>95000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="1837">
@@ -20642,7 +20642,7 @@
         <v>2817</v>
       </c>
       <c r="C1837" t="n">
-        <v>51813</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1838">
@@ -20664,7 +20664,7 @@
         <v>2784</v>
       </c>
       <c r="C1839" t="n">
-        <v>35929</v>
+        <v>37820</v>
       </c>
     </row>
     <row r="1840">
@@ -20686,7 +20686,7 @@
         <v>626</v>
       </c>
       <c r="C1841" t="n">
-        <v>1492203</v>
+        <v>1570740</v>
       </c>
     </row>
     <row r="1842">
@@ -20697,7 +20697,7 @@
         <v>925</v>
       </c>
       <c r="C1842" t="n">
-        <v>68894</v>
+        <v>72520</v>
       </c>
     </row>
     <row r="1843">
@@ -20708,7 +20708,7 @@
         <v>2586</v>
       </c>
       <c r="C1843" t="n">
-        <v>35929</v>
+        <v>37820</v>
       </c>
     </row>
     <row r="1844">
@@ -20741,7 +20741,7 @@
         <v>966</v>
       </c>
       <c r="C1846" t="n">
-        <v>70357</v>
+        <v>74060</v>
       </c>
     </row>
     <row r="1847">
@@ -20752,7 +20752,7 @@
         <v>2557</v>
       </c>
       <c r="C1847" t="n">
-        <v>33763</v>
+        <v>35540</v>
       </c>
     </row>
     <row r="1848">
@@ -20774,7 +20774,7 @@
         <v>14</v>
       </c>
       <c r="C1849" t="n">
-        <v>388626</v>
+        <v>409080</v>
       </c>
     </row>
     <row r="1850">
@@ -20796,7 +20796,7 @@
         <v>2798</v>
       </c>
       <c r="C1851" t="n">
-        <v>51813</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1852">
@@ -20818,7 +20818,7 @@
         <v>522</v>
       </c>
       <c r="C1853" t="n">
-        <v>172727.3</v>
+        <v>181818.2</v>
       </c>
     </row>
     <row r="1854">
@@ -20840,7 +20840,7 @@
         <v>2819</v>
       </c>
       <c r="C1855" t="n">
-        <v>51813</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1856">
@@ -20851,7 +20851,7 @@
         <v>2266</v>
       </c>
       <c r="C1856" t="n">
-        <v>69084</v>
+        <v>72720</v>
       </c>
     </row>
     <row r="1857">
@@ -20895,7 +20895,7 @@
         <v>2795</v>
       </c>
       <c r="C1860" t="n">
-        <v>51813</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1861">
@@ -20906,7 +20906,7 @@
         <v>2722</v>
       </c>
       <c r="C1861" t="n">
-        <v>17271</v>
+        <v>18180</v>
       </c>
     </row>
     <row r="1862">
@@ -20917,7 +20917,7 @@
         <v>951</v>
       </c>
       <c r="C1862" t="n">
-        <v>99313</v>
+        <v>104540</v>
       </c>
     </row>
     <row r="1863">
@@ -20928,7 +20928,7 @@
         <v>1020</v>
       </c>
       <c r="C1863" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1864">
@@ -20950,7 +20950,7 @@
         <v>1853</v>
       </c>
       <c r="C1865" t="n">
-        <v>103626</v>
+        <v>109080</v>
       </c>
     </row>
     <row r="1866">
@@ -20961,7 +20961,7 @@
         <v>1327</v>
       </c>
       <c r="C1866" t="n">
-        <v>60439</v>
+        <v>63620</v>
       </c>
     </row>
     <row r="1867">
@@ -20972,7 +20972,7 @@
         <v>2842</v>
       </c>
       <c r="C1867" t="n">
-        <v>155439</v>
+        <v>163620</v>
       </c>
     </row>
     <row r="1868">
@@ -20983,7 +20983,7 @@
         <v>2831</v>
       </c>
       <c r="C1868" t="n">
-        <v>51813</v>
+        <v>54540</v>
       </c>
     </row>
     <row r="1869">
@@ -20994,7 +20994,7 @@
         <v>818</v>
       </c>
       <c r="C1869" t="n">
-        <v>345439</v>
+        <v>363620</v>
       </c>
     </row>
     <row r="1870">
@@ -21005,7 +21005,7 @@
         <v>1501</v>
       </c>
       <c r="C1870" t="n">
-        <v>86355</v>
+        <v>90900</v>
       </c>
     </row>
     <row r="1871">
@@ -21016,7 +21016,7 @@
         <v>1869</v>
       </c>
       <c r="C1871" t="n">
-        <v>210727.3</v>
+        <v>221818.2</v>
       </c>
     </row>
     <row r="1872">
@@ -21027,7 +21027,7 @@
         <v>1996</v>
       </c>
       <c r="C1872" t="n">
-        <v>215909.11</v>
+        <v>227272.74</v>
       </c>
     </row>
     <row r="1873">
@@ -21038,7 +21038,7 @@
         <v>2462</v>
       </c>
       <c r="C1873" t="n">
-        <v>48912.07</v>
+        <v>51486.38</v>
       </c>
     </row>
     <row r="1874">
@@ -21049,7 +21049,7 @@
         <v>2696</v>
       </c>
       <c r="C1874" t="n">
-        <v>185212</v>
+        <v>194960</v>
       </c>
     </row>
     <row r="1875">
@@ -21060,7 +21060,7 @@
         <v>2698</v>
       </c>
       <c r="C1875" t="n">
-        <v>94924</v>
+        <v>99920</v>
       </c>
     </row>
     <row r="1876">
@@ -21082,7 +21082,7 @@
         <v>2828</v>
       </c>
       <c r="C1877" t="n">
-        <v>51818.19</v>
+        <v>54545.46</v>
       </c>
     </row>
     <row r="1878">
@@ -21093,7 +21093,7 @@
         <v>2843</v>
       </c>
       <c r="C1878" t="n">
-        <v>60439</v>
+        <v>63620</v>
       </c>
     </row>
     <row r="1879">
@@ -21104,7 +21104,7 @@
         <v>619</v>
       </c>
       <c r="C1879" t="n">
-        <v>270750</v>
+        <v>285000</v>
       </c>
     </row>
     <row r="1880">
@@ -21115,7 +21115,7 @@
         <v>1478</v>
       </c>
       <c r="C1880" t="n">
-        <v>473822</v>
+        <v>498760</v>
       </c>
     </row>
     <row r="1881">
@@ -21126,7 +21126,7 @@
         <v>2026</v>
       </c>
       <c r="C1881" t="n">
-        <v>209342</v>
+        <v>220360</v>
       </c>
     </row>
     <row r="1882">
@@ -21137,7 +21137,7 @@
         <v>663</v>
       </c>
       <c r="C1882" t="n">
-        <v>223668</v>
+        <v>235440</v>
       </c>
     </row>
     <row r="1883">
@@ -21148,7 +21148,7 @@
         <v>285</v>
       </c>
       <c r="C1883" t="n">
-        <v>473822</v>
+        <v>498760</v>
       </c>
     </row>
     <row r="1884">
@@ -21159,7 +21159,7 @@
         <v>424</v>
       </c>
       <c r="C1884" t="n">
-        <v>203053</v>
+        <v>213740</v>
       </c>
     </row>
     <row r="1885">
@@ -21170,7 +21170,7 @@
         <v>451</v>
       </c>
       <c r="C1885" t="n">
-        <v>209855</v>
+        <v>220900</v>
       </c>
     </row>
     <row r="1886">
@@ -21181,7 +21181,7 @@
         <v>629</v>
       </c>
       <c r="C1886" t="n">
-        <v>392084</v>
+        <v>412720</v>
       </c>
     </row>
     <row r="1887">
@@ -21192,7 +21192,7 @@
         <v>2657</v>
       </c>
       <c r="C1887" t="n">
-        <v>68381</v>
+        <v>71980</v>
       </c>
     </row>
     <row r="1888">
@@ -21203,7 +21203,7 @@
         <v>1254</v>
       </c>
       <c r="C1888" t="n">
-        <v>167713</v>
+        <v>176540</v>
       </c>
     </row>
     <row r="1889">
@@ -21214,7 +21214,7 @@
         <v>2402</v>
       </c>
       <c r="C1889" t="n">
-        <v>421838</v>
+        <v>444040</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:03:17
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -15560,7 +15560,7 @@
         <v>353</v>
       </c>
       <c r="C1375" t="n">
-        <v>265940</v>
+        <v>279237</v>
       </c>
     </row>
     <row r="1376">
@@ -15571,7 +15571,7 @@
         <v>2250</v>
       </c>
       <c r="C1376" t="n">
-        <v>309080</v>
+        <v>324534</v>
       </c>
     </row>
     <row r="1377">
@@ -15582,7 +15582,7 @@
         <v>1800</v>
       </c>
       <c r="C1377" t="n">
-        <v>25780</v>
+        <v>27069</v>
       </c>
     </row>
     <row r="1378">
@@ -15593,7 +15593,7 @@
         <v>2142</v>
       </c>
       <c r="C1378" t="n">
-        <v>51851.38</v>
+        <v>54443.94</v>
       </c>
     </row>
     <row r="1379">
@@ -15604,7 +15604,7 @@
         <v>2498</v>
       </c>
       <c r="C1379" t="n">
-        <v>53939.57</v>
+        <v>56636.54</v>
       </c>
     </row>
     <row r="1380">
@@ -15626,7 +15626,7 @@
         <v>2801</v>
       </c>
       <c r="C1381" t="n">
-        <v>90909.10000000001</v>
+        <v>95454.55</v>
       </c>
     </row>
     <row r="1382">
@@ -15637,7 +15637,7 @@
         <v>2810</v>
       </c>
       <c r="C1382" t="n">
-        <v>145454.56</v>
+        <v>152727.28</v>
       </c>
     </row>
     <row r="1383">
@@ -15681,7 +15681,7 @@
         <v>2853</v>
       </c>
       <c r="C1386" t="n">
-        <v>74060</v>
+        <v>77763</v>
       </c>
     </row>
     <row r="1387">
@@ -15692,7 +15692,7 @@
         <v>2245</v>
       </c>
       <c r="C1387" t="n">
-        <v>201280</v>
+        <v>211344</v>
       </c>
     </row>
     <row r="1388">
@@ -15703,7 +15703,7 @@
         <v>2251</v>
       </c>
       <c r="C1388" t="n">
-        <v>181800</v>
+        <v>190890</v>
       </c>
     </row>
     <row r="1389">
@@ -15714,7 +15714,7 @@
         <v>664</v>
       </c>
       <c r="C1389" t="n">
-        <v>238180</v>
+        <v>250089</v>
       </c>
     </row>
     <row r="1390">
@@ -15725,7 +15725,7 @@
         <v>2472</v>
       </c>
       <c r="C1390" t="n">
-        <v>48120</v>
+        <v>50526</v>
       </c>
     </row>
     <row r="1391">
@@ -15736,7 +15736,7 @@
         <v>1456</v>
       </c>
       <c r="C1391" t="n">
-        <v>725440</v>
+        <v>761712</v>
       </c>
     </row>
     <row r="1392">
@@ -15747,7 +15747,7 @@
         <v>1585</v>
       </c>
       <c r="C1392" t="n">
-        <v>164540</v>
+        <v>172767</v>
       </c>
     </row>
     <row r="1393">
@@ -15791,7 +15791,7 @@
         <v>1907</v>
       </c>
       <c r="C1396" t="n">
-        <v>500480</v>
+        <v>525504</v>
       </c>
     </row>
     <row r="1397">
@@ -15824,7 +15824,7 @@
         <v>2659</v>
       </c>
       <c r="C1399" t="n">
-        <v>111820</v>
+        <v>117411</v>
       </c>
     </row>
     <row r="1400">
@@ -15868,7 +15868,7 @@
         <v>2583</v>
       </c>
       <c r="C1403" t="n">
-        <v>37820</v>
+        <v>39711</v>
       </c>
     </row>
     <row r="1404">
@@ -15879,7 +15879,7 @@
         <v>2692</v>
       </c>
       <c r="C1404" t="n">
-        <v>63636.38</v>
+        <v>66818.19</v>
       </c>
     </row>
     <row r="1405">
@@ -15890,7 +15890,7 @@
         <v>2691</v>
       </c>
       <c r="C1405" t="n">
-        <v>111076.38</v>
+        <v>116630.19</v>
       </c>
     </row>
     <row r="1406">
@@ -15923,7 +15923,7 @@
         <v>931</v>
       </c>
       <c r="C1408" t="n">
-        <v>87020</v>
+        <v>91371</v>
       </c>
     </row>
     <row r="1409">
@@ -15934,7 +15934,7 @@
         <v>2785</v>
       </c>
       <c r="C1409" t="n">
-        <v>37820</v>
+        <v>39711</v>
       </c>
     </row>
     <row r="1410">
@@ -15945,7 +15945,7 @@
         <v>2411</v>
       </c>
       <c r="C1410" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1411">
@@ -15978,7 +15978,7 @@
         <v>2716</v>
       </c>
       <c r="C1413" t="n">
-        <v>79760</v>
+        <v>83748</v>
       </c>
     </row>
     <row r="1414">
@@ -15989,7 +15989,7 @@
         <v>2809</v>
       </c>
       <c r="C1414" t="n">
-        <v>62440</v>
+        <v>65562</v>
       </c>
     </row>
     <row r="1415">
@@ -16033,7 +16033,7 @@
         <v>104</v>
       </c>
       <c r="C1418" t="n">
-        <v>272727.28</v>
+        <v>286363.64</v>
       </c>
     </row>
     <row r="1419">
@@ -16088,7 +16088,7 @@
         <v>781</v>
       </c>
       <c r="C1423" t="n">
-        <v>118180</v>
+        <v>124089</v>
       </c>
     </row>
     <row r="1424">
@@ -16132,7 +16132,7 @@
         <v>2494</v>
       </c>
       <c r="C1427" t="n">
-        <v>136360</v>
+        <v>143178</v>
       </c>
     </row>
     <row r="1428">
@@ -16165,7 +16165,7 @@
         <v>2652</v>
       </c>
       <c r="C1430" t="n">
-        <v>127260</v>
+        <v>133623</v>
       </c>
     </row>
     <row r="1431">
@@ -16176,7 +16176,7 @@
         <v>1384</v>
       </c>
       <c r="C1431" t="n">
-        <v>318181.82</v>
+        <v>334090.91</v>
       </c>
     </row>
     <row r="1432">
@@ -16187,7 +16187,7 @@
         <v>360</v>
       </c>
       <c r="C1432" t="n">
-        <v>454540</v>
+        <v>477267</v>
       </c>
     </row>
     <row r="1433">
@@ -16198,7 +16198,7 @@
         <v>2767</v>
       </c>
       <c r="C1433" t="n">
-        <v>172720</v>
+        <v>181356</v>
       </c>
     </row>
     <row r="1434">
@@ -16209,7 +16209,7 @@
         <v>2178</v>
       </c>
       <c r="C1434" t="n">
-        <v>249090.92</v>
+        <v>261545.46</v>
       </c>
     </row>
     <row r="1435">
@@ -16220,7 +16220,7 @@
         <v>2107</v>
       </c>
       <c r="C1435" t="n">
-        <v>272700</v>
+        <v>286335</v>
       </c>
     </row>
     <row r="1436">
@@ -16231,7 +16231,7 @@
         <v>2711</v>
       </c>
       <c r="C1436" t="n">
-        <v>78700</v>
+        <v>82635</v>
       </c>
     </row>
     <row r="1437">
@@ -16242,7 +16242,7 @@
         <v>2845</v>
       </c>
       <c r="C1437" t="n">
-        <v>27272.74</v>
+        <v>28636.37</v>
       </c>
     </row>
     <row r="1438">
@@ -16286,7 +16286,7 @@
         <v>1102</v>
       </c>
       <c r="C1441" t="n">
-        <v>213740</v>
+        <v>224427</v>
       </c>
     </row>
     <row r="1442">
@@ -16297,7 +16297,7 @@
         <v>525</v>
       </c>
       <c r="C1442" t="n">
-        <v>213636.38</v>
+        <v>224318.19</v>
       </c>
     </row>
     <row r="1443">
@@ -16308,7 +16308,7 @@
         <v>1261</v>
       </c>
       <c r="C1443" t="n">
-        <v>64545.46</v>
+        <v>67772.73</v>
       </c>
     </row>
     <row r="1444">
@@ -16319,7 +16319,7 @@
         <v>2755</v>
       </c>
       <c r="C1444" t="n">
-        <v>45454.56</v>
+        <v>47727.28</v>
       </c>
     </row>
     <row r="1445">
@@ -16341,7 +16341,7 @@
         <v>783</v>
       </c>
       <c r="C1446" t="n">
-        <v>36363.64</v>
+        <v>38181.82</v>
       </c>
     </row>
     <row r="1447">
@@ -16352,7 +16352,7 @@
         <v>1064</v>
       </c>
       <c r="C1447" t="n">
-        <v>545440</v>
+        <v>572712</v>
       </c>
     </row>
     <row r="1448">
@@ -16363,7 +16363,7 @@
         <v>1810</v>
       </c>
       <c r="C1448" t="n">
-        <v>38925.92</v>
+        <v>40872.21</v>
       </c>
     </row>
     <row r="1449">
@@ -16374,7 +16374,7 @@
         <v>1937</v>
       </c>
       <c r="C1449" t="n">
-        <v>235440</v>
+        <v>247212</v>
       </c>
     </row>
     <row r="1450">
@@ -16385,7 +16385,7 @@
         <v>483</v>
       </c>
       <c r="C1450" t="n">
-        <v>410900</v>
+        <v>431445</v>
       </c>
     </row>
     <row r="1451">
@@ -16396,7 +16396,7 @@
         <v>2580</v>
       </c>
       <c r="C1451" t="n">
-        <v>30620</v>
+        <v>32151</v>
       </c>
     </row>
     <row r="1452">
@@ -16407,7 +16407,7 @@
         <v>2706</v>
       </c>
       <c r="C1452" t="n">
-        <v>23920</v>
+        <v>25116</v>
       </c>
     </row>
     <row r="1453">
@@ -16418,7 +16418,7 @@
         <v>2633</v>
       </c>
       <c r="C1453" t="n">
-        <v>17520</v>
+        <v>18396</v>
       </c>
     </row>
     <row r="1454">
@@ -16451,7 +16451,7 @@
         <v>2392</v>
       </c>
       <c r="C1456" t="n">
-        <v>188560</v>
+        <v>197988</v>
       </c>
     </row>
     <row r="1457">
@@ -16473,7 +16473,7 @@
         <v>2613</v>
       </c>
       <c r="C1458" t="n">
-        <v>132760</v>
+        <v>139398</v>
       </c>
     </row>
     <row r="1459">
@@ -16484,7 +16484,7 @@
         <v>2183</v>
       </c>
       <c r="C1459" t="n">
-        <v>478020</v>
+        <v>501921</v>
       </c>
     </row>
     <row r="1460">
@@ -16495,7 +16495,7 @@
         <v>2541</v>
       </c>
       <c r="C1460" t="n">
-        <v>214900</v>
+        <v>225645</v>
       </c>
     </row>
     <row r="1461">
@@ -16517,7 +16517,7 @@
         <v>2333</v>
       </c>
       <c r="C1462" t="n">
-        <v>145080</v>
+        <v>152334</v>
       </c>
     </row>
     <row r="1463">
@@ -16561,7 +16561,7 @@
         <v>2813</v>
       </c>
       <c r="C1466" t="n">
-        <v>58000</v>
+        <v>60900</v>
       </c>
     </row>
     <row r="1467">
@@ -16572,7 +16572,7 @@
         <v>2811</v>
       </c>
       <c r="C1467" t="n">
-        <v>37820</v>
+        <v>39711</v>
       </c>
     </row>
     <row r="1468">
@@ -16583,7 +16583,7 @@
         <v>1881</v>
       </c>
       <c r="C1468" t="n">
-        <v>62440</v>
+        <v>65562</v>
       </c>
     </row>
     <row r="1469">
@@ -16594,7 +16594,7 @@
         <v>2825</v>
       </c>
       <c r="C1469" t="n">
-        <v>50760</v>
+        <v>53298</v>
       </c>
     </row>
     <row r="1470">
@@ -16605,7 +16605,7 @@
         <v>970</v>
       </c>
       <c r="C1470" t="n">
-        <v>62440</v>
+        <v>65562</v>
       </c>
     </row>
     <row r="1471">
@@ -16616,7 +16616,7 @@
         <v>2552</v>
       </c>
       <c r="C1471" t="n">
-        <v>35540</v>
+        <v>37317</v>
       </c>
     </row>
     <row r="1472">
@@ -16627,7 +16627,7 @@
         <v>2562</v>
       </c>
       <c r="C1472" t="n">
-        <v>35540</v>
+        <v>37317</v>
       </c>
     </row>
     <row r="1473">
@@ -16704,7 +16704,7 @@
         <v>2747</v>
       </c>
       <c r="C1479" t="n">
-        <v>63620</v>
+        <v>66801</v>
       </c>
     </row>
     <row r="1480">
@@ -16792,7 +16792,7 @@
         <v>2544</v>
       </c>
       <c r="C1487" t="n">
-        <v>63620</v>
+        <v>66801</v>
       </c>
     </row>
     <row r="1488">
@@ -16803,7 +16803,7 @@
         <v>816</v>
       </c>
       <c r="C1488" t="n">
-        <v>272727.28</v>
+        <v>286363.64</v>
       </c>
     </row>
     <row r="1489">
@@ -16814,7 +16814,7 @@
         <v>890</v>
       </c>
       <c r="C1489" t="n">
-        <v>659090.92</v>
+        <v>692045.46</v>
       </c>
     </row>
     <row r="1490">
@@ -16836,7 +16836,7 @@
         <v>1298</v>
       </c>
       <c r="C1491" t="n">
-        <v>1150000</v>
+        <v>1207500</v>
       </c>
     </row>
     <row r="1492">
@@ -16847,7 +16847,7 @@
         <v>1372</v>
       </c>
       <c r="C1492" t="n">
-        <v>272727.28</v>
+        <v>286363.64</v>
       </c>
     </row>
     <row r="1493">
@@ -16858,7 +16858,7 @@
         <v>358</v>
       </c>
       <c r="C1493" t="n">
-        <v>286360</v>
+        <v>300678</v>
       </c>
     </row>
     <row r="1494">
@@ -16880,7 +16880,7 @@
         <v>1653</v>
       </c>
       <c r="C1495" t="n">
-        <v>286360</v>
+        <v>300678</v>
       </c>
     </row>
     <row r="1496">
@@ -16891,7 +16891,7 @@
         <v>675</v>
       </c>
       <c r="C1496" t="n">
-        <v>181800</v>
+        <v>190890</v>
       </c>
     </row>
     <row r="1497">
@@ -16902,7 +16902,7 @@
         <v>2804</v>
       </c>
       <c r="C1497" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1498">
@@ -16913,7 +16913,7 @@
         <v>2714</v>
       </c>
       <c r="C1498" t="n">
-        <v>327260</v>
+        <v>343623</v>
       </c>
     </row>
     <row r="1499">
@@ -16924,7 +16924,7 @@
         <v>2765</v>
       </c>
       <c r="C1499" t="n">
-        <v>81800</v>
+        <v>85890</v>
       </c>
     </row>
     <row r="1500">
@@ -16935,7 +16935,7 @@
         <v>2421</v>
       </c>
       <c r="C1500" t="n">
-        <v>55454.56</v>
+        <v>58227.28</v>
       </c>
     </row>
     <row r="1501">
@@ -16946,7 +16946,7 @@
         <v>2359</v>
       </c>
       <c r="C1501" t="n">
-        <v>94840</v>
+        <v>99582</v>
       </c>
     </row>
     <row r="1502">
@@ -16957,7 +16957,7 @@
         <v>2678</v>
       </c>
       <c r="C1502" t="n">
-        <v>89960</v>
+        <v>94458</v>
       </c>
     </row>
     <row r="1503">
@@ -16968,7 +16968,7 @@
         <v>2697</v>
       </c>
       <c r="C1503" t="n">
-        <v>136520</v>
+        <v>143346</v>
       </c>
     </row>
     <row r="1504">
@@ -17001,7 +17001,7 @@
         <v>1308</v>
       </c>
       <c r="C1506" t="n">
-        <v>142720</v>
+        <v>149856</v>
       </c>
     </row>
     <row r="1507">
@@ -17012,7 +17012,7 @@
         <v>2118</v>
       </c>
       <c r="C1507" t="n">
-        <v>191060</v>
+        <v>200613</v>
       </c>
     </row>
     <row r="1508">
@@ -17023,7 +17023,7 @@
         <v>2607</v>
       </c>
       <c r="C1508" t="n">
-        <v>45160</v>
+        <v>47418</v>
       </c>
     </row>
     <row r="1509">
@@ -17034,7 +17034,7 @@
         <v>2832</v>
       </c>
       <c r="C1509" t="n">
-        <v>136363.64</v>
+        <v>143181.82</v>
       </c>
     </row>
     <row r="1510">
@@ -17045,7 +17045,7 @@
         <v>2383</v>
       </c>
       <c r="C1510" t="n">
-        <v>120840</v>
+        <v>126882</v>
       </c>
     </row>
     <row r="1511">
@@ -17078,7 +17078,7 @@
         <v>2821</v>
       </c>
       <c r="C1513" t="n">
-        <v>121220</v>
+        <v>127281</v>
       </c>
     </row>
     <row r="1514">
@@ -17100,7 +17100,7 @@
         <v>569</v>
       </c>
       <c r="C1515" t="n">
-        <v>2639480</v>
+        <v>2771454</v>
       </c>
     </row>
     <row r="1516">
@@ -17111,7 +17111,7 @@
         <v>2660</v>
       </c>
       <c r="C1516" t="n">
-        <v>318181.82</v>
+        <v>334090.91</v>
       </c>
     </row>
     <row r="1517">
@@ -17122,7 +17122,7 @@
         <v>1632</v>
       </c>
       <c r="C1517" t="n">
-        <v>236363.64</v>
+        <v>248181.82</v>
       </c>
     </row>
     <row r="1518">
@@ -17133,7 +17133,7 @@
         <v>1756</v>
       </c>
       <c r="C1518" t="n">
-        <v>381800</v>
+        <v>400890</v>
       </c>
     </row>
     <row r="1519">
@@ -17144,7 +17144,7 @@
         <v>58</v>
       </c>
       <c r="C1519" t="n">
-        <v>228000</v>
+        <v>239400</v>
       </c>
     </row>
     <row r="1520">
@@ -17155,7 +17155,7 @@
         <v>40</v>
       </c>
       <c r="C1520" t="n">
-        <v>202800</v>
+        <v>212940</v>
       </c>
     </row>
     <row r="1521">
@@ -17166,7 +17166,7 @@
         <v>559</v>
       </c>
       <c r="C1521" t="n">
-        <v>212720</v>
+        <v>223356</v>
       </c>
     </row>
     <row r="1522">
@@ -17177,7 +17177,7 @@
         <v>2773</v>
       </c>
       <c r="C1522" t="n">
-        <v>73340</v>
+        <v>77007</v>
       </c>
     </row>
     <row r="1523">
@@ -17188,7 +17188,7 @@
         <v>2631</v>
       </c>
       <c r="C1523" t="n">
-        <v>35220</v>
+        <v>36981</v>
       </c>
     </row>
     <row r="1524">
@@ -17199,7 +17199,7 @@
         <v>2085</v>
       </c>
       <c r="C1524" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1525">
@@ -17221,7 +17221,7 @@
         <v>1642</v>
       </c>
       <c r="C1526" t="n">
-        <v>240900</v>
+        <v>252945</v>
       </c>
     </row>
     <row r="1527">
@@ -17232,7 +17232,7 @@
         <v>2621</v>
       </c>
       <c r="C1527" t="n">
-        <v>63620</v>
+        <v>66801</v>
       </c>
     </row>
     <row r="1528">
@@ -17243,7 +17243,7 @@
         <v>2705</v>
       </c>
       <c r="C1528" t="n">
-        <v>182520</v>
+        <v>191646</v>
       </c>
     </row>
     <row r="1529">
@@ -17276,7 +17276,7 @@
         <v>2735</v>
       </c>
       <c r="C1531" t="n">
-        <v>109080</v>
+        <v>114534</v>
       </c>
     </row>
     <row r="1532">
@@ -17287,7 +17287,7 @@
         <v>945</v>
       </c>
       <c r="C1532" t="n">
-        <v>318800</v>
+        <v>334740</v>
       </c>
     </row>
     <row r="1533">
@@ -17309,7 +17309,7 @@
         <v>2582</v>
       </c>
       <c r="C1534" t="n">
-        <v>79760</v>
+        <v>83748</v>
       </c>
     </row>
     <row r="1535">
@@ -17320,7 +17320,7 @@
         <v>2584</v>
       </c>
       <c r="C1535" t="n">
-        <v>58000</v>
+        <v>60900</v>
       </c>
     </row>
     <row r="1536">
@@ -17331,7 +17331,7 @@
         <v>2689</v>
       </c>
       <c r="C1536" t="n">
-        <v>58000</v>
+        <v>60900</v>
       </c>
     </row>
     <row r="1537">
@@ -17342,7 +17342,7 @@
         <v>2574</v>
       </c>
       <c r="C1537" t="n">
-        <v>127480</v>
+        <v>133854</v>
       </c>
     </row>
     <row r="1538">
@@ -17353,7 +17353,7 @@
         <v>1834</v>
       </c>
       <c r="C1538" t="n">
-        <v>107000</v>
+        <v>112350</v>
       </c>
     </row>
     <row r="1539">
@@ -17375,7 +17375,7 @@
         <v>2629</v>
       </c>
       <c r="C1540" t="n">
-        <v>62440</v>
+        <v>65562</v>
       </c>
     </row>
     <row r="1541">
@@ -17386,7 +17386,7 @@
         <v>933</v>
       </c>
       <c r="C1541" t="n">
-        <v>74060</v>
+        <v>77763</v>
       </c>
     </row>
     <row r="1542">
@@ -17397,7 +17397,7 @@
         <v>2555</v>
       </c>
       <c r="C1542" t="n">
-        <v>35540</v>
+        <v>37317</v>
       </c>
     </row>
     <row r="1543">
@@ -17408,7 +17408,7 @@
         <v>2558</v>
       </c>
       <c r="C1543" t="n">
-        <v>35540</v>
+        <v>37317</v>
       </c>
     </row>
     <row r="1544">
@@ -17430,7 +17430,7 @@
         <v>2721</v>
       </c>
       <c r="C1545" t="n">
-        <v>74060</v>
+        <v>77763</v>
       </c>
     </row>
     <row r="1546">
@@ -17441,7 +17441,7 @@
         <v>2556</v>
       </c>
       <c r="C1546" t="n">
-        <v>35540</v>
+        <v>37317</v>
       </c>
     </row>
     <row r="1547">
@@ -17463,7 +17463,7 @@
         <v>2826</v>
       </c>
       <c r="C1548" t="n">
-        <v>63620</v>
+        <v>66801</v>
       </c>
     </row>
     <row r="1549">
@@ -17485,7 +17485,7 @@
         <v>2346</v>
       </c>
       <c r="C1550" t="n">
-        <v>63620</v>
+        <v>66801</v>
       </c>
     </row>
     <row r="1551">
@@ -17496,7 +17496,7 @@
         <v>595</v>
       </c>
       <c r="C1551" t="n">
-        <v>227272.74</v>
+        <v>238636.37</v>
       </c>
     </row>
     <row r="1552">
@@ -17529,7 +17529,7 @@
         <v>1278</v>
       </c>
       <c r="C1554" t="n">
-        <v>159090.92</v>
+        <v>167045.46</v>
       </c>
     </row>
     <row r="1555">
@@ -17540,7 +17540,7 @@
         <v>2686</v>
       </c>
       <c r="C1555" t="n">
-        <v>127260</v>
+        <v>133623</v>
       </c>
     </row>
     <row r="1556">
@@ -17551,7 +17551,7 @@
         <v>1344</v>
       </c>
       <c r="C1556" t="n">
-        <v>136360</v>
+        <v>143178</v>
       </c>
     </row>
     <row r="1557">
@@ -17606,7 +17606,7 @@
         <v>2566</v>
       </c>
       <c r="C1561" t="n">
-        <v>72720</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1562">
@@ -17617,7 +17617,7 @@
         <v>2684</v>
       </c>
       <c r="C1562" t="n">
-        <v>86360</v>
+        <v>90678</v>
       </c>
     </row>
     <row r="1563">
@@ -17628,7 +17628,7 @@
         <v>2375</v>
       </c>
       <c r="C1563" t="n">
-        <v>300000</v>
+        <v>315000</v>
       </c>
     </row>
     <row r="1564">
@@ -17639,7 +17639,7 @@
         <v>2362</v>
       </c>
       <c r="C1564" t="n">
-        <v>68180</v>
+        <v>71589</v>
       </c>
     </row>
     <row r="1565">
@@ -17650,7 +17650,7 @@
         <v>2449</v>
       </c>
       <c r="C1565" t="n">
-        <v>86360</v>
+        <v>90678</v>
       </c>
     </row>
     <row r="1566">
@@ -17661,7 +17661,7 @@
         <v>2844</v>
       </c>
       <c r="C1566" t="n">
-        <v>27272.74</v>
+        <v>28636.37</v>
       </c>
     </row>
     <row r="1567">
@@ -17672,7 +17672,7 @@
         <v>2507</v>
       </c>
       <c r="C1567" t="n">
-        <v>81200</v>
+        <v>85260</v>
       </c>
     </row>
     <row r="1568">
@@ -17683,7 +17683,7 @@
         <v>1906</v>
       </c>
       <c r="C1568" t="n">
-        <v>98700</v>
+        <v>103635</v>
       </c>
     </row>
     <row r="1569">
@@ -17705,7 +17705,7 @@
         <v>1983</v>
       </c>
       <c r="C1570" t="n">
-        <v>498400</v>
+        <v>523320</v>
       </c>
     </row>
     <row r="1571">
@@ -17716,7 +17716,7 @@
         <v>1993</v>
       </c>
       <c r="C1571" t="n">
-        <v>338440</v>
+        <v>355362</v>
       </c>
     </row>
     <row r="1572">
@@ -17727,7 +17727,7 @@
         <v>89</v>
       </c>
       <c r="C1572" t="n">
-        <v>318180</v>
+        <v>334089</v>
       </c>
     </row>
     <row r="1573">
@@ -17738,7 +17738,7 @@
         <v>1063</v>
       </c>
       <c r="C1573" t="n">
-        <v>350000</v>
+        <v>367500</v>
       </c>
     </row>
     <row r="1574">
@@ -17749,7 +17749,7 @@
         <v>1116</v>
       </c>
       <c r="C1574" t="n">
-        <v>227260</v>
+        <v>238623</v>
       </c>
     </row>
     <row r="1575">
@@ -17760,7 +17760,7 @@
         <v>941</v>
       </c>
       <c r="C1575" t="n">
-        <v>273540</v>
+        <v>287217</v>
       </c>
     </row>
     <row r="1576">
@@ -17771,7 +17771,7 @@
         <v>2141</v>
       </c>
       <c r="C1576" t="n">
-        <v>30735.34</v>
+        <v>32272.1</v>
       </c>
     </row>
     <row r="1577">
@@ -17782,7 +17782,7 @@
         <v>2463</v>
       </c>
       <c r="C1577" t="n">
-        <v>299840</v>
+        <v>314832</v>
       </c>
     </row>
     <row r="1578">
@@ -17793,7 +17793,7 @@
         <v>2707</v>
       </c>
       <c r="C1578" t="n">
-        <v>39260</v>
+        <v>41223</v>
       </c>
     </row>
     <row r="1579">
@@ -17804,7 +17804,7 @@
         <v>2325</v>
       </c>
       <c r="C1579" t="n">
-        <v>104880</v>
+        <v>110124</v>
       </c>
     </row>
     <row r="1580">
@@ -17848,7 +17848,7 @@
         <v>1890</v>
       </c>
       <c r="C1583" t="n">
-        <v>222940</v>
+        <v>234087</v>
       </c>
     </row>
     <row r="1584">
@@ -17859,7 +17859,7 @@
         <v>2639</v>
       </c>
       <c r="C1584" t="n">
-        <v>36420</v>
+        <v>38241</v>
       </c>
     </row>
     <row r="1585">
@@ -17870,7 +17870,7 @@
         <v>2682</v>
       </c>
       <c r="C1585" t="n">
-        <v>127260</v>
+        <v>133623</v>
       </c>
     </row>
     <row r="1586">
@@ -17881,7 +17881,7 @@
         <v>2601</v>
       </c>
       <c r="C1586" t="n">
-        <v>250000</v>
+        <v>262500</v>
       </c>
     </row>
     <row r="1587">
@@ -17892,7 +17892,7 @@
         <v>1142</v>
       </c>
       <c r="C1587" t="n">
-        <v>416440</v>
+        <v>437262</v>
       </c>
     </row>
     <row r="1588">
@@ -17936,7 +17936,7 @@
         <v>2082</v>
       </c>
       <c r="C1591" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1592">
@@ -17947,7 +17947,7 @@
         <v>2276</v>
       </c>
       <c r="C1592" t="n">
-        <v>180840</v>
+        <v>189882</v>
       </c>
     </row>
     <row r="1593">
@@ -17969,7 +17969,7 @@
         <v>2786</v>
       </c>
       <c r="C1594" t="n">
-        <v>63620</v>
+        <v>66801</v>
       </c>
     </row>
     <row r="1595">
@@ -17980,7 +17980,7 @@
         <v>2816</v>
       </c>
       <c r="C1595" t="n">
-        <v>118180</v>
+        <v>124089</v>
       </c>
     </row>
     <row r="1596">
@@ -17991,7 +17991,7 @@
         <v>1871</v>
       </c>
       <c r="C1596" t="n">
-        <v>130460</v>
+        <v>136983</v>
       </c>
     </row>
     <row r="1597">
@@ -18002,7 +18002,7 @@
         <v>2345</v>
       </c>
       <c r="C1597" t="n">
-        <v>58000</v>
+        <v>60900</v>
       </c>
     </row>
     <row r="1598">
@@ -18013,7 +18013,7 @@
         <v>2802</v>
       </c>
       <c r="C1598" t="n">
-        <v>65260</v>
+        <v>68523</v>
       </c>
     </row>
     <row r="1599">
@@ -18024,7 +18024,7 @@
         <v>2090</v>
       </c>
       <c r="C1599" t="n">
-        <v>37820</v>
+        <v>39711</v>
       </c>
     </row>
     <row r="1600">
@@ -18035,7 +18035,7 @@
         <v>2647</v>
       </c>
       <c r="C1600" t="n">
-        <v>127500</v>
+        <v>133875</v>
       </c>
     </row>
     <row r="1601">
@@ -18046,7 +18046,7 @@
         <v>2365</v>
       </c>
       <c r="C1601" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1602">
@@ -18057,7 +18057,7 @@
         <v>766</v>
       </c>
       <c r="C1602" t="n">
-        <v>62440</v>
+        <v>65562</v>
       </c>
     </row>
     <row r="1603">
@@ -18068,7 +18068,7 @@
         <v>2702</v>
       </c>
       <c r="C1603" t="n">
-        <v>74060</v>
+        <v>77763</v>
       </c>
     </row>
     <row r="1604">
@@ -18090,7 +18090,7 @@
         <v>20</v>
       </c>
       <c r="C1605" t="n">
-        <v>409090.92</v>
+        <v>429545.46</v>
       </c>
     </row>
     <row r="1606">
@@ -18101,7 +18101,7 @@
         <v>27</v>
       </c>
       <c r="C1606" t="n">
-        <v>136363.64</v>
+        <v>143181.82</v>
       </c>
     </row>
     <row r="1607">
@@ -18112,7 +18112,7 @@
         <v>33</v>
       </c>
       <c r="C1607" t="n">
-        <v>361818.2</v>
+        <v>379909.1</v>
       </c>
     </row>
     <row r="1608">
@@ -18134,7 +18134,7 @@
         <v>2561</v>
       </c>
       <c r="C1609" t="n">
-        <v>35540</v>
+        <v>37317</v>
       </c>
     </row>
     <row r="1610">
@@ -18178,7 +18178,7 @@
         <v>2772</v>
       </c>
       <c r="C1613" t="n">
-        <v>54540</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1614">
@@ -18189,7 +18189,7 @@
         <v>132</v>
       </c>
       <c r="C1614" t="n">
-        <v>318181.82</v>
+        <v>334090.91</v>
       </c>
     </row>
     <row r="1615">
@@ -18211,7 +18211,7 @@
         <v>580</v>
       </c>
       <c r="C1616" t="n">
-        <v>159090.92</v>
+        <v>167045.46</v>
       </c>
     </row>
     <row r="1617">
@@ -18222,7 +18222,7 @@
         <v>634</v>
       </c>
       <c r="C1617" t="n">
-        <v>454545.46</v>
+        <v>477272.73</v>
       </c>
     </row>
     <row r="1618">
@@ -18244,7 +18244,7 @@
         <v>1277</v>
       </c>
       <c r="C1619" t="n">
-        <v>200000</v>
+        <v>210000</v>
       </c>
     </row>
     <row r="1620">
@@ -18255,7 +18255,7 @@
         <v>767</v>
       </c>
       <c r="C1620" t="n">
-        <v>181800</v>
+        <v>190890</v>
       </c>
     </row>
     <row r="1621">
@@ -18266,7 +18266,7 @@
         <v>2727</v>
       </c>
       <c r="C1621" t="n">
-        <v>36800</v>
+        <v>38640</v>
       </c>
     </row>
     <row r="1622">
@@ -18277,7 +18277,7 @@
         <v>2846</v>
       </c>
       <c r="C1622" t="n">
-        <v>236360</v>
+        <v>248178</v>
       </c>
     </row>
     <row r="1623">
@@ -18288,7 +18288,7 @@
         <v>609</v>
       </c>
       <c r="C1623" t="n">
-        <v>204540</v>
+        <v>214767</v>
       </c>
     </row>
     <row r="1624">
@@ -18299,7 +18299,7 @@
         <v>2726</v>
       </c>
       <c r="C1624" t="n">
-        <v>140900</v>
+        <v>147945</v>
       </c>
     </row>
     <row r="1625">
@@ -18321,7 +18321,7 @@
         <v>2729</v>
       </c>
       <c r="C1626" t="n">
-        <v>81800</v>
+        <v>85890</v>
       </c>
     </row>
     <row r="1627">
@@ -18332,7 +18332,7 @@
         <v>1340</v>
       </c>
       <c r="C1627" t="n">
-        <v>136360</v>
+        <v>143178</v>
       </c>
     </row>
     <row r="1628">
@@ -18343,7 +18343,7 @@
         <v>2830</v>
       </c>
       <c r="C1628" t="n">
-        <v>81800</v>
+        <v>85890</v>
       </c>
     </row>
     <row r="1629">
@@ -18365,7 +18365,7 @@
         <v>2674</v>
       </c>
       <c r="C1630" t="n">
-        <v>236360</v>
+        <v>248178</v>
       </c>
     </row>
     <row r="1631">
@@ -18376,7 +18376,7 @@
         <v>2308</v>
       </c>
       <c r="C1631" t="n">
-        <v>181800</v>
+        <v>190890</v>
       </c>
     </row>
     <row r="1632">
@@ -18387,7 +18387,7 @@
         <v>2190</v>
       </c>
       <c r="C1632" t="n">
-        <v>190909.1</v>
+        <v>200454.55</v>
       </c>
     </row>
     <row r="1633">
@@ -18398,7 +18398,7 @@
         <v>2015</v>
       </c>
       <c r="C1633" t="n">
-        <v>336360</v>
+        <v>353178</v>
       </c>
     </row>
     <row r="1634">
@@ -18409,7 +18409,7 @@
         <v>429</v>
       </c>
       <c r="C1634" t="n">
-        <v>345440</v>
+        <v>362712</v>
       </c>
     </row>
     <row r="1635">
@@ -18420,7 +18420,7 @@
         <v>2114</v>
       </c>
       <c r="C1635" t="n">
-        <v>154660</v>
+        <v>162393</v>
       </c>
     </row>
     <row r="1636">
@@ -18431,7 +18431,7 @@
         <v>2211</v>
       </c>
       <c r="C1636" t="n">
-        <v>218940</v>
+        <v>229887</v>
       </c>
     </row>
     <row r="1637">
@@ -18442,7 +18442,7 @@
         <v>1108</v>
       </c>
       <c r="C1637" t="n">
-        <v>278520</v>
+        <v>292446</v>
       </c>
     </row>
     <row r="1638">
@@ -18453,7 +18453,7 @@
         <v>2695</v>
       </c>
       <c r="C1638" t="n">
-        <v>46365.72</v>
+        <v>48684</v>
       </c>
     </row>
     <row r="1639">
@@ -18464,7 +18464,7 @@
         <v>1289</v>
       </c>
       <c r="C1639" t="n">
-        <v>250000</v>
+        <v>262500</v>
       </c>
     </row>
     <row r="1640">
@@ -18475,7 +18475,7 @@
         <v>2789</v>
       </c>
       <c r="C1640" t="n">
-        <v>163636.38</v>
+        <v>171818.19</v>
       </c>
     </row>
     <row r="1641">
@@ -18486,7 +18486,7 @@
         <v>2197</v>
       </c>
       <c r="C1641" t="n">
-        <v>195454.56</v>
+        <v>205227.28</v>
       </c>
     </row>
     <row r="1642">
@@ -18497,7 +18497,7 @@
         <v>947</v>
       </c>
       <c r="C1642" t="n">
-        <v>403160</v>
+        <v>423318</v>
       </c>
     </row>
     <row r="1643">
@@ -18508,7 +18508,7 @@
         <v>2279</v>
       </c>
       <c r="C1643" t="n">
-        <v>222660</v>
+        <v>233793</v>
       </c>
     </row>
     <row r="1644">
@@ -18519,7 +18519,7 @@
         <v>1465</v>
       </c>
       <c r="C1644" t="n">
-        <v>350000</v>
+        <v>367500</v>
       </c>
     </row>
     <row r="1645">
@@ -18530,7 +18530,7 @@
         <v>2651</v>
       </c>
       <c r="C1645" t="n">
-        <v>154540</v>
+        <v>162267</v>
       </c>
     </row>
     <row r="1646">
@@ -18541,7 +18541,7 @@
         <v>42</v>
       </c>
       <c r="C1646" t="n">
-        <v>1732720</v>
+        <v>1819356</v>
       </c>
     </row>
     <row r="1647">
@@ -18552,7 +18552,7 @@
         <v>949</v>
       </c>
       <c r="C1647" t="n">
-        <v>90420</v>
+        <v>94941</v>
       </c>
     </row>
     <row r="1648">
@@ -18563,7 +18563,7 @@
         <v>2606</v>
       </c>
       <c r="C1648" t="n">
-        <v>233400</v>
+        <v>245070</v>
       </c>
     </row>
     <row r="1649">
@@ -18574,7 +18574,7 @@
         <v>2249</v>
       </c>
       <c r="C1649" t="n">
-        <v>198300</v>
+        <v>208215</v>
       </c>
     </row>
     <row r="1650">
@@ -18618,7 +18618,7 @@
         <v>2045</v>
       </c>
       <c r="C1653" t="n">
-        <v>289520</v>
+        <v>303996</v>
       </c>
     </row>
     <row r="1654">
@@ -18629,7 +18629,7 @@
         <v>2663</v>
       </c>
       <c r="C1654" t="n">
-        <v>250000</v>
+        <v>262500</v>
       </c>
     </row>
     <row r="1655">
@@ -18651,7 +18651,7 @@
         <v>2854</v>
       </c>
       <c r="C1656" t="n">
-        <v>36360</v>
+        <v>38178</v>
       </c>
     </row>
     <row r="1657">
@@ -18684,7 +18684,7 @@
         <v>2341</v>
       </c>
       <c r="C1659" t="n">
-        <v>159000</v>
+        <v>166950</v>
       </c>
     </row>
     <row r="1660">
@@ -18695,7 +18695,7 @@
         <v>2637</v>
       </c>
       <c r="C1660" t="n">
-        <v>58000</v>
+        <v>60900</v>
       </c>
     </row>
     <row r="1661">
@@ -18706,7 +18706,7 @@
         <v>2492</v>
       </c>
       <c r="C1661" t="n">
-        <v>91060</v>
+        <v>95613</v>
       </c>
     </row>
     <row r="1662">
@@ -18739,7 +18739,7 @@
         <v>2548</v>
       </c>
       <c r="C1664" t="n">
-        <v>35540</v>
+        <v>37317</v>
       </c>
     </row>
     <row r="1665">
@@ -18750,7 +18750,7 @@
         <v>351</v>
       </c>
       <c r="C1665" t="n">
-        <v>193636.38</v>
+        <v>203318.19</v>
       </c>
     </row>
     <row r="1666">
@@ -18783,7 +18783,7 @@
         <v>2757</v>
       </c>
       <c r="C1668" t="n">
-        <v>72720</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1669">
@@ -18794,7 +18794,7 @@
         <v>2815</v>
       </c>
       <c r="C1669" t="n">
-        <v>54540</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1670">
@@ -18805,7 +18805,7 @@
         <v>2829</v>
       </c>
       <c r="C1670" t="n">
-        <v>54540</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1671">
@@ -18816,7 +18816,7 @@
         <v>768</v>
       </c>
       <c r="C1671" t="n">
-        <v>127260</v>
+        <v>133623</v>
       </c>
     </row>
     <row r="1672">
@@ -18827,7 +18827,7 @@
         <v>772</v>
       </c>
       <c r="C1672" t="n">
-        <v>295454.56</v>
+        <v>310227.28</v>
       </c>
     </row>
     <row r="1673">
@@ -18860,7 +18860,7 @@
         <v>2496</v>
       </c>
       <c r="C1675" t="n">
-        <v>181800</v>
+        <v>190890</v>
       </c>
     </row>
     <row r="1676">
@@ -18871,7 +18871,7 @@
         <v>802</v>
       </c>
       <c r="C1676" t="n">
-        <v>68180</v>
+        <v>71589</v>
       </c>
     </row>
     <row r="1677">
@@ -18893,7 +18893,7 @@
         <v>2131</v>
       </c>
       <c r="C1678" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1679">
@@ -18904,7 +18904,7 @@
         <v>1381</v>
       </c>
       <c r="C1679" t="n">
-        <v>272727.28</v>
+        <v>286363.64</v>
       </c>
     </row>
     <row r="1680">
@@ -18915,7 +18915,7 @@
         <v>2847</v>
       </c>
       <c r="C1680" t="n">
-        <v>122720</v>
+        <v>128856</v>
       </c>
     </row>
     <row r="1681">
@@ -18926,7 +18926,7 @@
         <v>1293</v>
       </c>
       <c r="C1681" t="n">
-        <v>350000</v>
+        <v>367500</v>
       </c>
     </row>
     <row r="1682">
@@ -18948,7 +18948,7 @@
         <v>2363</v>
       </c>
       <c r="C1683" t="n">
-        <v>154540</v>
+        <v>162267</v>
       </c>
     </row>
     <row r="1684">
@@ -18959,7 +18959,7 @@
         <v>631</v>
       </c>
       <c r="C1684" t="n">
-        <v>318180</v>
+        <v>334089</v>
       </c>
     </row>
     <row r="1685">
@@ -18970,7 +18970,7 @@
         <v>2791</v>
       </c>
       <c r="C1685" t="n">
-        <v>93340</v>
+        <v>98007</v>
       </c>
     </row>
     <row r="1686">
@@ -18992,7 +18992,7 @@
         <v>2841</v>
       </c>
       <c r="C1687" t="n">
-        <v>45440</v>
+        <v>47712</v>
       </c>
     </row>
     <row r="1688">
@@ -19003,7 +19003,7 @@
         <v>2571</v>
       </c>
       <c r="C1688" t="n">
-        <v>242340</v>
+        <v>254457</v>
       </c>
     </row>
     <row r="1689">
@@ -19069,7 +19069,7 @@
         <v>2273</v>
       </c>
       <c r="C1694" t="n">
-        <v>205985.46</v>
+        <v>216284.73</v>
       </c>
     </row>
     <row r="1695">
@@ -19080,7 +19080,7 @@
         <v>2381</v>
       </c>
       <c r="C1695" t="n">
-        <v>77052.48</v>
+        <v>80905.10000000001</v>
       </c>
     </row>
     <row r="1696">
@@ -19091,7 +19091,7 @@
         <v>630</v>
       </c>
       <c r="C1696" t="n">
-        <v>75027.23</v>
+        <v>78778.59</v>
       </c>
     </row>
     <row r="1697">
@@ -19113,7 +19113,7 @@
         <v>2768</v>
       </c>
       <c r="C1698" t="n">
-        <v>275140</v>
+        <v>288897</v>
       </c>
     </row>
     <row r="1699">
@@ -19124,7 +19124,7 @@
         <v>2491</v>
       </c>
       <c r="C1699" t="n">
-        <v>220780</v>
+        <v>231819</v>
       </c>
     </row>
     <row r="1700">
@@ -19135,7 +19135,7 @@
         <v>2799</v>
       </c>
       <c r="C1700" t="n">
-        <v>99380</v>
+        <v>104349</v>
       </c>
     </row>
     <row r="1701">
@@ -19168,7 +19168,7 @@
         <v>1317</v>
       </c>
       <c r="C1703" t="n">
-        <v>286363.64</v>
+        <v>300681.82</v>
       </c>
     </row>
     <row r="1704">
@@ -19179,7 +19179,7 @@
         <v>2822</v>
       </c>
       <c r="C1704" t="n">
-        <v>145454.56</v>
+        <v>152727.28</v>
       </c>
     </row>
     <row r="1705">
@@ -19190,7 +19190,7 @@
         <v>1117</v>
       </c>
       <c r="C1705" t="n">
-        <v>363740</v>
+        <v>381927</v>
       </c>
     </row>
     <row r="1706">
@@ -19201,7 +19201,7 @@
         <v>1299</v>
       </c>
       <c r="C1706" t="n">
-        <v>479580</v>
+        <v>503559</v>
       </c>
     </row>
     <row r="1707">
@@ -19212,7 +19212,7 @@
         <v>477</v>
       </c>
       <c r="C1707" t="n">
-        <v>197640</v>
+        <v>207522</v>
       </c>
     </row>
     <row r="1708">
@@ -19223,7 +19223,7 @@
         <v>530</v>
       </c>
       <c r="C1708" t="n">
-        <v>272720</v>
+        <v>286356</v>
       </c>
     </row>
     <row r="1709">
@@ -19234,7 +19234,7 @@
         <v>953</v>
       </c>
       <c r="C1709" t="n">
-        <v>627260</v>
+        <v>658623</v>
       </c>
     </row>
     <row r="1710">
@@ -19245,7 +19245,7 @@
         <v>610</v>
       </c>
       <c r="C1710" t="n">
-        <v>747080</v>
+        <v>784434</v>
       </c>
     </row>
     <row r="1711">
@@ -19256,7 +19256,7 @@
         <v>2792</v>
       </c>
       <c r="C1711" t="n">
-        <v>187620</v>
+        <v>197001</v>
       </c>
     </row>
     <row r="1712">
@@ -19333,7 +19333,7 @@
         <v>2834</v>
       </c>
       <c r="C1718" t="n">
-        <v>33880</v>
+        <v>35574</v>
       </c>
     </row>
     <row r="1719">
@@ -19344,7 +19344,7 @@
         <v>2394</v>
       </c>
       <c r="C1719" t="n">
-        <v>103140</v>
+        <v>108297</v>
       </c>
     </row>
     <row r="1720">
@@ -19355,7 +19355,7 @@
         <v>2567</v>
       </c>
       <c r="C1720" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1721">
@@ -19366,7 +19366,7 @@
         <v>952</v>
       </c>
       <c r="C1721" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1722">
@@ -19377,7 +19377,7 @@
         <v>1539</v>
       </c>
       <c r="C1722" t="n">
-        <v>154540</v>
+        <v>162267</v>
       </c>
     </row>
     <row r="1723">
@@ -19388,7 +19388,7 @@
         <v>793</v>
       </c>
       <c r="C1723" t="n">
-        <v>37820</v>
+        <v>39711</v>
       </c>
     </row>
     <row r="1724">
@@ -19399,7 +19399,7 @@
         <v>794</v>
       </c>
       <c r="C1724" t="n">
-        <v>37820</v>
+        <v>39711</v>
       </c>
     </row>
     <row r="1725">
@@ -19410,7 +19410,7 @@
         <v>2838</v>
       </c>
       <c r="C1725" t="n">
-        <v>54545.46</v>
+        <v>57272.73</v>
       </c>
     </row>
     <row r="1726">
@@ -19432,7 +19432,7 @@
         <v>2223</v>
       </c>
       <c r="C1727" t="n">
-        <v>106460</v>
+        <v>111783</v>
       </c>
     </row>
     <row r="1728">
@@ -19443,7 +19443,7 @@
         <v>2547</v>
       </c>
       <c r="C1728" t="n">
-        <v>30800</v>
+        <v>32340</v>
       </c>
     </row>
     <row r="1729">
@@ -19465,7 +19465,7 @@
         <v>2762</v>
       </c>
       <c r="C1730" t="n">
-        <v>74060</v>
+        <v>77763</v>
       </c>
     </row>
     <row r="1731">
@@ -19476,7 +19476,7 @@
         <v>2550</v>
       </c>
       <c r="C1731" t="n">
-        <v>35540</v>
+        <v>37317</v>
       </c>
     </row>
     <row r="1732">
@@ -19487,7 +19487,7 @@
         <v>2627</v>
       </c>
       <c r="C1732" t="n">
-        <v>35540</v>
+        <v>37317</v>
       </c>
     </row>
     <row r="1733">
@@ -19542,7 +19542,7 @@
         <v>749</v>
       </c>
       <c r="C1737" t="n">
-        <v>74060</v>
+        <v>77763</v>
       </c>
     </row>
     <row r="1738">
@@ -19553,7 +19553,7 @@
         <v>2549</v>
       </c>
       <c r="C1738" t="n">
-        <v>35540</v>
+        <v>37317</v>
       </c>
     </row>
     <row r="1739">
@@ -19564,7 +19564,7 @@
         <v>2649</v>
       </c>
       <c r="C1739" t="n">
-        <v>35540</v>
+        <v>37317</v>
       </c>
     </row>
     <row r="1740">
@@ -19575,7 +19575,7 @@
         <v>2258</v>
       </c>
       <c r="C1740" t="n">
-        <v>72720</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1741">
@@ -19586,7 +19586,7 @@
         <v>2744</v>
       </c>
       <c r="C1741" t="n">
-        <v>54540</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1742">
@@ -19597,7 +19597,7 @@
         <v>452</v>
       </c>
       <c r="C1742" t="n">
-        <v>257272.74</v>
+        <v>270136.37</v>
       </c>
     </row>
     <row r="1743">
@@ -19652,7 +19652,7 @@
         <v>2653</v>
       </c>
       <c r="C1747" t="n">
-        <v>54540</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1748">
@@ -19696,7 +19696,7 @@
         <v>2742</v>
       </c>
       <c r="C1751" t="n">
-        <v>18180</v>
+        <v>19089</v>
       </c>
     </row>
     <row r="1752">
@@ -19707,7 +19707,7 @@
         <v>1499</v>
       </c>
       <c r="C1752" t="n">
-        <v>81800</v>
+        <v>85890</v>
       </c>
     </row>
     <row r="1753">
@@ -19718,7 +19718,7 @@
         <v>2261</v>
       </c>
       <c r="C1753" t="n">
-        <v>163620</v>
+        <v>171801</v>
       </c>
     </row>
     <row r="1754">
@@ -19762,7 +19762,7 @@
         <v>1324</v>
       </c>
       <c r="C1757" t="n">
-        <v>254540</v>
+        <v>267267</v>
       </c>
     </row>
     <row r="1758">
@@ -19773,7 +19773,7 @@
         <v>2709</v>
       </c>
       <c r="C1758" t="n">
-        <v>163620</v>
+        <v>171801</v>
       </c>
     </row>
     <row r="1759">
@@ -19795,7 +19795,7 @@
         <v>1137</v>
       </c>
       <c r="C1760" t="n">
-        <v>581800</v>
+        <v>610890</v>
       </c>
     </row>
     <row r="1761">
@@ -19806,7 +19806,7 @@
         <v>2440</v>
       </c>
       <c r="C1761" t="n">
-        <v>72720</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1762">
@@ -19817,7 +19817,7 @@
         <v>2413</v>
       </c>
       <c r="C1762" t="n">
-        <v>125300</v>
+        <v>131565</v>
       </c>
     </row>
     <row r="1763">
@@ -19828,7 +19828,7 @@
         <v>1450</v>
       </c>
       <c r="C1763" t="n">
-        <v>324540</v>
+        <v>340767</v>
       </c>
     </row>
     <row r="1764">
@@ -19850,7 +19850,7 @@
         <v>2671</v>
       </c>
       <c r="C1765" t="n">
-        <v>72720</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1766">
@@ -19861,7 +19861,7 @@
         <v>2568</v>
       </c>
       <c r="C1766" t="n">
-        <v>145860</v>
+        <v>153153</v>
       </c>
     </row>
     <row r="1767">
@@ -19872,7 +19872,7 @@
         <v>2146</v>
       </c>
       <c r="C1767" t="n">
-        <v>176620</v>
+        <v>185451</v>
       </c>
     </row>
     <row r="1768">
@@ -19883,7 +19883,7 @@
         <v>2753</v>
       </c>
       <c r="C1768" t="n">
-        <v>68180</v>
+        <v>71589</v>
       </c>
     </row>
     <row r="1769">
@@ -19916,7 +19916,7 @@
         <v>744</v>
       </c>
       <c r="C1771" t="n">
-        <v>37820</v>
+        <v>39711</v>
       </c>
     </row>
     <row r="1772">
@@ -19927,7 +19927,7 @@
         <v>2323</v>
       </c>
       <c r="C1772" t="n">
-        <v>62440</v>
+        <v>65562</v>
       </c>
     </row>
     <row r="1773">
@@ -19938,7 +19938,7 @@
         <v>2310</v>
       </c>
       <c r="C1773" t="n">
-        <v>62440</v>
+        <v>65562</v>
       </c>
     </row>
     <row r="1774">
@@ -19949,7 +19949,7 @@
         <v>2145</v>
       </c>
       <c r="C1774" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1775">
@@ -19960,7 +19960,7 @@
         <v>2858</v>
       </c>
       <c r="C1775" t="n">
-        <v>45454.56</v>
+        <v>47727.28</v>
       </c>
     </row>
     <row r="1776">
@@ -19993,7 +19993,7 @@
         <v>2501</v>
       </c>
       <c r="C1778" t="n">
-        <v>74060</v>
+        <v>77763</v>
       </c>
     </row>
     <row r="1779">
@@ -20004,7 +20004,7 @@
         <v>2546</v>
       </c>
       <c r="C1779" t="n">
-        <v>35540</v>
+        <v>37317</v>
       </c>
     </row>
     <row r="1780">
@@ -20026,7 +20026,7 @@
         <v>716</v>
       </c>
       <c r="C1781" t="n">
-        <v>116520</v>
+        <v>122346</v>
       </c>
     </row>
     <row r="1782">
@@ -20037,7 +20037,7 @@
         <v>2758</v>
       </c>
       <c r="C1782" t="n">
-        <v>54540</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1783">
@@ -20048,7 +20048,7 @@
         <v>400</v>
       </c>
       <c r="C1783" t="n">
-        <v>163636.38</v>
+        <v>171818.19</v>
       </c>
     </row>
     <row r="1784">
@@ -20059,7 +20059,7 @@
         <v>6</v>
       </c>
       <c r="C1784" t="n">
-        <v>45454.56</v>
+        <v>47727.28</v>
       </c>
     </row>
     <row r="1785">
@@ -20114,7 +20114,7 @@
         <v>1259</v>
       </c>
       <c r="C1789" t="n">
-        <v>100000</v>
+        <v>105000</v>
       </c>
     </row>
     <row r="1790">
@@ -20125,7 +20125,7 @@
         <v>571</v>
       </c>
       <c r="C1790" t="n">
-        <v>940909.1</v>
+        <v>987954.55</v>
       </c>
     </row>
     <row r="1791">
@@ -20136,7 +20136,7 @@
         <v>703</v>
       </c>
       <c r="C1791" t="n">
-        <v>227260</v>
+        <v>238623</v>
       </c>
     </row>
     <row r="1792">
@@ -20191,7 +20191,7 @@
         <v>2833</v>
       </c>
       <c r="C1796" t="n">
-        <v>72720</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1797">
@@ -20202,7 +20202,7 @@
         <v>1007</v>
       </c>
       <c r="C1797" t="n">
-        <v>181818.2</v>
+        <v>190909.1</v>
       </c>
     </row>
     <row r="1798">
@@ -20213,7 +20213,7 @@
         <v>2687</v>
       </c>
       <c r="C1798" t="n">
-        <v>72720</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1799">
@@ -20224,7 +20224,7 @@
         <v>2824</v>
       </c>
       <c r="C1799" t="n">
-        <v>102640</v>
+        <v>107772</v>
       </c>
     </row>
     <row r="1800">
@@ -20235,7 +20235,7 @@
         <v>2730</v>
       </c>
       <c r="C1800" t="n">
-        <v>81800</v>
+        <v>85890</v>
       </c>
     </row>
     <row r="1801">
@@ -20257,7 +20257,7 @@
         <v>2718</v>
       </c>
       <c r="C1802" t="n">
-        <v>118180</v>
+        <v>124089</v>
       </c>
     </row>
     <row r="1803">
@@ -20268,7 +20268,7 @@
         <v>2750</v>
       </c>
       <c r="C1803" t="n">
-        <v>27260</v>
+        <v>28623</v>
       </c>
     </row>
     <row r="1804">
@@ -20279,7 +20279,7 @@
         <v>854</v>
       </c>
       <c r="C1804" t="n">
-        <v>127260</v>
+        <v>133623</v>
       </c>
     </row>
     <row r="1805">
@@ -20290,7 +20290,7 @@
         <v>2794</v>
       </c>
       <c r="C1805" t="n">
-        <v>109080</v>
+        <v>114534</v>
       </c>
     </row>
     <row r="1806">
@@ -20301,7 +20301,7 @@
         <v>1374</v>
       </c>
       <c r="C1806" t="n">
-        <v>181800</v>
+        <v>190890</v>
       </c>
     </row>
     <row r="1807">
@@ -20312,7 +20312,7 @@
         <v>2488</v>
       </c>
       <c r="C1807" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1808">
@@ -20323,7 +20323,7 @@
         <v>363</v>
       </c>
       <c r="C1808" t="n">
-        <v>272720</v>
+        <v>286356</v>
       </c>
     </row>
     <row r="1809">
@@ -20334,7 +20334,7 @@
         <v>2655</v>
       </c>
       <c r="C1809" t="n">
-        <v>100000</v>
+        <v>105000</v>
       </c>
     </row>
     <row r="1810">
@@ -20345,7 +20345,7 @@
         <v>1873</v>
       </c>
       <c r="C1810" t="n">
-        <v>290900</v>
+        <v>305445</v>
       </c>
     </row>
     <row r="1811">
@@ -20356,7 +20356,7 @@
         <v>2635</v>
       </c>
       <c r="C1811" t="n">
-        <v>118180</v>
+        <v>124089</v>
       </c>
     </row>
     <row r="1812">
@@ -20367,7 +20367,7 @@
         <v>1658</v>
       </c>
       <c r="C1812" t="n">
-        <v>139090.92</v>
+        <v>146045.46</v>
       </c>
     </row>
     <row r="1813">
@@ -20378,7 +20378,7 @@
         <v>2069</v>
       </c>
       <c r="C1813" t="n">
-        <v>181818.2</v>
+        <v>190909.1</v>
       </c>
     </row>
     <row r="1814">
@@ -20389,7 +20389,7 @@
         <v>2081</v>
       </c>
       <c r="C1814" t="n">
-        <v>136360</v>
+        <v>143178</v>
       </c>
     </row>
     <row r="1815">
@@ -20400,7 +20400,7 @@
         <v>2124</v>
       </c>
       <c r="C1815" t="n">
-        <v>318180</v>
+        <v>334089</v>
       </c>
     </row>
     <row r="1816">
@@ -20411,7 +20411,7 @@
         <v>636</v>
       </c>
       <c r="C1816" t="n">
-        <v>227260</v>
+        <v>238623</v>
       </c>
     </row>
     <row r="1817">
@@ -20422,7 +20422,7 @@
         <v>2803</v>
       </c>
       <c r="C1817" t="n">
-        <v>109080</v>
+        <v>114534</v>
       </c>
     </row>
     <row r="1818">
@@ -20433,7 +20433,7 @@
         <v>2163</v>
       </c>
       <c r="C1818" t="n">
-        <v>163620</v>
+        <v>171801</v>
       </c>
     </row>
     <row r="1819">
@@ -20444,7 +20444,7 @@
         <v>1466</v>
       </c>
       <c r="C1819" t="n">
-        <v>368180</v>
+        <v>386589</v>
       </c>
     </row>
     <row r="1820">
@@ -20455,7 +20455,7 @@
         <v>2133</v>
       </c>
       <c r="C1820" t="n">
-        <v>659090.92</v>
+        <v>692045.46</v>
       </c>
     </row>
     <row r="1821">
@@ -20466,7 +20466,7 @@
         <v>2431</v>
       </c>
       <c r="C1821" t="n">
-        <v>136363.64</v>
+        <v>143181.82</v>
       </c>
     </row>
     <row r="1822">
@@ -20477,7 +20477,7 @@
         <v>535</v>
       </c>
       <c r="C1822" t="n">
-        <v>323800</v>
+        <v>339990</v>
       </c>
     </row>
     <row r="1823">
@@ -20488,7 +20488,7 @@
         <v>2790</v>
       </c>
       <c r="C1823" t="n">
-        <v>57420</v>
+        <v>60291</v>
       </c>
     </row>
     <row r="1824">
@@ -20499,7 +20499,7 @@
         <v>2442</v>
       </c>
       <c r="C1824" t="n">
-        <v>235454.56</v>
+        <v>247227.28</v>
       </c>
     </row>
     <row r="1825">
@@ -20510,7 +20510,7 @@
         <v>2376</v>
       </c>
       <c r="C1825" t="n">
-        <v>1000000</v>
+        <v>1050000</v>
       </c>
     </row>
     <row r="1826">
@@ -20521,7 +20521,7 @@
         <v>1075</v>
       </c>
       <c r="C1826" t="n">
-        <v>417260</v>
+        <v>438123</v>
       </c>
     </row>
     <row r="1827">
@@ -20532,7 +20532,7 @@
         <v>131</v>
       </c>
       <c r="C1827" t="n">
-        <v>378180</v>
+        <v>397089</v>
       </c>
     </row>
     <row r="1828">
@@ -20543,7 +20543,7 @@
         <v>2667</v>
       </c>
       <c r="C1828" t="n">
-        <v>41540</v>
+        <v>43617</v>
       </c>
     </row>
     <row r="1829">
@@ -20554,7 +20554,7 @@
         <v>2330</v>
       </c>
       <c r="C1829" t="n">
-        <v>80860</v>
+        <v>84903</v>
       </c>
     </row>
     <row r="1830">
@@ -20576,7 +20576,7 @@
         <v>2577</v>
       </c>
       <c r="C1831" t="n">
-        <v>81060</v>
+        <v>85113</v>
       </c>
     </row>
     <row r="1832">
@@ -20587,7 +20587,7 @@
         <v>2510</v>
       </c>
       <c r="C1832" t="n">
-        <v>575680</v>
+        <v>604464</v>
       </c>
     </row>
     <row r="1833">
@@ -20609,7 +20609,7 @@
         <v>2850</v>
       </c>
       <c r="C1834" t="n">
-        <v>54540</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1835">
@@ -20631,7 +20631,7 @@
         <v>2745</v>
       </c>
       <c r="C1836" t="n">
-        <v>100000</v>
+        <v>105000</v>
       </c>
     </row>
     <row r="1837">
@@ -20642,7 +20642,7 @@
         <v>2817</v>
       </c>
       <c r="C1837" t="n">
-        <v>54540</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1838">
@@ -20664,7 +20664,7 @@
         <v>2784</v>
       </c>
       <c r="C1839" t="n">
-        <v>37820</v>
+        <v>39711</v>
       </c>
     </row>
     <row r="1840">
@@ -20686,7 +20686,7 @@
         <v>626</v>
       </c>
       <c r="C1841" t="n">
-        <v>1570740</v>
+        <v>1649277</v>
       </c>
     </row>
     <row r="1842">
@@ -20697,7 +20697,7 @@
         <v>925</v>
       </c>
       <c r="C1842" t="n">
-        <v>72520</v>
+        <v>76146</v>
       </c>
     </row>
     <row r="1843">
@@ -20708,7 +20708,7 @@
         <v>2586</v>
       </c>
       <c r="C1843" t="n">
-        <v>37820</v>
+        <v>39711</v>
       </c>
     </row>
     <row r="1844">
@@ -20741,7 +20741,7 @@
         <v>966</v>
       </c>
       <c r="C1846" t="n">
-        <v>74060</v>
+        <v>77763</v>
       </c>
     </row>
     <row r="1847">
@@ -20752,7 +20752,7 @@
         <v>2557</v>
       </c>
       <c r="C1847" t="n">
-        <v>35540</v>
+        <v>37317</v>
       </c>
     </row>
     <row r="1848">
@@ -20774,7 +20774,7 @@
         <v>14</v>
       </c>
       <c r="C1849" t="n">
-        <v>409080</v>
+        <v>429534</v>
       </c>
     </row>
     <row r="1850">
@@ -20796,7 +20796,7 @@
         <v>2798</v>
       </c>
       <c r="C1851" t="n">
-        <v>54540</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1852">
@@ -20818,7 +20818,7 @@
         <v>522</v>
       </c>
       <c r="C1853" t="n">
-        <v>181818.2</v>
+        <v>190909.1</v>
       </c>
     </row>
     <row r="1854">
@@ -20840,7 +20840,7 @@
         <v>2819</v>
       </c>
       <c r="C1855" t="n">
-        <v>54540</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1856">
@@ -20851,7 +20851,7 @@
         <v>2266</v>
       </c>
       <c r="C1856" t="n">
-        <v>72720</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="1857">
@@ -20895,7 +20895,7 @@
         <v>2795</v>
       </c>
       <c r="C1860" t="n">
-        <v>54540</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1861">
@@ -20906,7 +20906,7 @@
         <v>2722</v>
       </c>
       <c r="C1861" t="n">
-        <v>18180</v>
+        <v>19089</v>
       </c>
     </row>
     <row r="1862">
@@ -20917,7 +20917,7 @@
         <v>951</v>
       </c>
       <c r="C1862" t="n">
-        <v>104540</v>
+        <v>109767</v>
       </c>
     </row>
     <row r="1863">
@@ -20928,7 +20928,7 @@
         <v>1020</v>
       </c>
       <c r="C1863" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1864">
@@ -20950,7 +20950,7 @@
         <v>1853</v>
       </c>
       <c r="C1865" t="n">
-        <v>109080</v>
+        <v>114534</v>
       </c>
     </row>
     <row r="1866">
@@ -20961,7 +20961,7 @@
         <v>1327</v>
       </c>
       <c r="C1866" t="n">
-        <v>63620</v>
+        <v>66801</v>
       </c>
     </row>
     <row r="1867">
@@ -20972,7 +20972,7 @@
         <v>2842</v>
       </c>
       <c r="C1867" t="n">
-        <v>163620</v>
+        <v>171801</v>
       </c>
     </row>
     <row r="1868">
@@ -20983,7 +20983,7 @@
         <v>2831</v>
       </c>
       <c r="C1868" t="n">
-        <v>54540</v>
+        <v>57267</v>
       </c>
     </row>
     <row r="1869">
@@ -20994,7 +20994,7 @@
         <v>818</v>
       </c>
       <c r="C1869" t="n">
-        <v>363620</v>
+        <v>381801</v>
       </c>
     </row>
     <row r="1870">
@@ -21005,7 +21005,7 @@
         <v>1501</v>
       </c>
       <c r="C1870" t="n">
-        <v>90900</v>
+        <v>95445</v>
       </c>
     </row>
     <row r="1871">
@@ -21016,7 +21016,7 @@
         <v>1869</v>
       </c>
       <c r="C1871" t="n">
-        <v>221818.2</v>
+        <v>232909.1</v>
       </c>
     </row>
     <row r="1872">
@@ -21027,7 +21027,7 @@
         <v>1996</v>
       </c>
       <c r="C1872" t="n">
-        <v>227272.74</v>
+        <v>238636.37</v>
       </c>
     </row>
     <row r="1873">
@@ -21038,7 +21038,7 @@
         <v>2462</v>
       </c>
       <c r="C1873" t="n">
-        <v>51486.38</v>
+        <v>54060.69</v>
       </c>
     </row>
     <row r="1874">
@@ -21049,7 +21049,7 @@
         <v>2696</v>
       </c>
       <c r="C1874" t="n">
-        <v>194960</v>
+        <v>204708</v>
       </c>
     </row>
     <row r="1875">
@@ -21060,7 +21060,7 @@
         <v>2698</v>
       </c>
       <c r="C1875" t="n">
-        <v>99920</v>
+        <v>104916</v>
       </c>
     </row>
     <row r="1876">
@@ -21082,7 +21082,7 @@
         <v>2828</v>
       </c>
       <c r="C1877" t="n">
-        <v>54545.46</v>
+        <v>57272.73</v>
       </c>
     </row>
     <row r="1878">
@@ -21093,7 +21093,7 @@
         <v>2843</v>
       </c>
       <c r="C1878" t="n">
-        <v>63620</v>
+        <v>66801</v>
       </c>
     </row>
     <row r="1879">
@@ -21104,7 +21104,7 @@
         <v>619</v>
       </c>
       <c r="C1879" t="n">
-        <v>285000</v>
+        <v>299250</v>
       </c>
     </row>
     <row r="1880">
@@ -21115,7 +21115,7 @@
         <v>1478</v>
       </c>
       <c r="C1880" t="n">
-        <v>498760</v>
+        <v>523698</v>
       </c>
     </row>
     <row r="1881">
@@ -21126,7 +21126,7 @@
         <v>2026</v>
       </c>
       <c r="C1881" t="n">
-        <v>220360</v>
+        <v>231378</v>
       </c>
     </row>
     <row r="1882">
@@ -21137,7 +21137,7 @@
         <v>663</v>
       </c>
       <c r="C1882" t="n">
-        <v>235440</v>
+        <v>247212</v>
       </c>
     </row>
     <row r="1883">
@@ -21148,7 +21148,7 @@
         <v>285</v>
       </c>
       <c r="C1883" t="n">
-        <v>498760</v>
+        <v>523698</v>
       </c>
     </row>
     <row r="1884">
@@ -21159,7 +21159,7 @@
         <v>424</v>
       </c>
       <c r="C1884" t="n">
-        <v>213740</v>
+        <v>224427</v>
       </c>
     </row>
     <row r="1885">
@@ -21170,7 +21170,7 @@
         <v>451</v>
       </c>
       <c r="C1885" t="n">
-        <v>220900</v>
+        <v>231945</v>
       </c>
     </row>
     <row r="1886">
@@ -21181,7 +21181,7 @@
         <v>629</v>
       </c>
       <c r="C1886" t="n">
-        <v>412720</v>
+        <v>433356</v>
       </c>
     </row>
     <row r="1887">
@@ -21192,7 +21192,7 @@
         <v>2657</v>
       </c>
       <c r="C1887" t="n">
-        <v>71980</v>
+        <v>75579</v>
       </c>
     </row>
     <row r="1888">
@@ -21203,7 +21203,7 @@
         <v>1254</v>
       </c>
       <c r="C1888" t="n">
-        <v>176540</v>
+        <v>185367</v>
       </c>
     </row>
     <row r="1889">
@@ -21214,7 +21214,7 @@
         <v>2402</v>
       </c>
       <c r="C1889" t="n">
-        <v>444040</v>
+        <v>466242</v>
       </c>
     </row>
   </sheetData>

</xml_diff>